<commit_message>
Gas model: measured vial headspace feeds Geometry D49; blank-safe calibration columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -580,6 +580,8 @@
     <definedName name="z_e_H2" localSheetId="2">Electrochemistry!$D$16</definedName>
     <definedName name="z_e_O2" localSheetId="2">Electrochemistry!$D$17</definedName>
     <definedName name="z_e_ORR" localSheetId="2">Electrochemistry!$D$27</definedName>
+    <definedName name="cal_hs">Calibrations!$D$76</definedName>
+    <definedName name="cal_hs_fill">Calibrations!$D$77</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8147,8 +8149,10 @@
         <f>HYPERLINK("#Geometry!D90","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
-      <c r="F19" s="21" t="s">
-        <v>71</v>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Red until the vial headspace is measured (vial-geometry.md); while red, the pulse above is provisional (~4x uncertain). After the headspace runs it reads HEADSPACE MEASURED until the body volume is measured too.</t>
+        </is>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -10455,11 +10459,13 @@
         <v>57</v>
       </c>
       <c r="D49" s="42">
-        <f>V_vial_total-V_charge-V_inserts</f>
+        <f>IF(AND(ISNUMBER(cal_hs),ISNUMBER(cal_hs_fill)),cal_hs-(V_charge-cal_hs_fill),V_vial_total-V_charge-V_inserts)</f>
         <v>2.612428455917</v>
       </c>
-      <c r="E49" s="37" t="s">
-        <v>253</v>
+      <c r="E49" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measured when the Calibrations vial-geometry runs exist for this reactor type (headspace at the measured working fill, shifted by any difference between that fill and V_charge); otherwise total vial volume − liquid charged − inserts.</t>
+        </is>
       </c>
       <c r="F49" s="20"/>
       <c r="G49" s="20"/>
@@ -11144,7 +11150,7 @@
       </c>
       <c r="C90" s="20"/>
       <c r="D90" s="24" t="str">
-        <f>IF(ABS(A_x*D_int/1000-V_vial_total)&gt;3,"VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth","OK")</f>
+        <f>IF(ABS(A_x*D_int/1000-V_vial_total)&lt;=3,"OK",IF(AND(ISNUMBER(cal_hs),ISNUMBER(cal_hs_fill)),"HEADSPACE MEASURED - bore depth still inconsistent (measure body volume)","VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth"))</f>
         <v>VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth</v>
       </c>
       <c r="E90" s="20"/>
@@ -24860,7 +24866,7 @@
       <c r="L64" s="97"/>
       <c r="M64" s="97"/>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="65" x14ac:dyDescent="0.2">
       <c r="A65" s="128" t="s">
         <v>1397</v>
       </c>
@@ -24894,23 +24900,36 @@
       <c r="K65" s="128" t="s">
         <v>1403</v>
       </c>
-      <c r="L65" s="97"/>
-      <c r="M65" s="97"/>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L65" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace (computed)</t>
+        </is>
+      </c>
+      <c r="M65" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Working-fill mass</t>
+        </is>
+      </c>
+      <c r="N65" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Working fill (computed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" x14ac:dyDescent="0.2">
       <c r="A66" s="122"/>
       <c r="B66" s="123"/>
       <c r="C66" s="122"/>
       <c r="D66" s="123"/>
       <c r="E66" s="123"/>
       <c r="F66" s="123"/>
-      <c r="G66" s="129">
-        <f t="shared" ref="G66:G73" si="1">IFERROR(E66/(0.99705-0.00028*(F66-25)),"")</f>
-        <v>0.0</v>
-      </c>
-      <c r="H66" s="129">
-        <f>IFERROR((E66/(0.99705-0.00028*(F66-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G66" s="129" t="str">
+        <f>IF(E66="","",IFERROR(E66/(0.99705-0.00028*(F66-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H66" s="129" t="str">
+        <f>IF(E66="","",IFERROR((E66/(0.99705-0.00028*(F66-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I66" s="129" t="str">
         <f>IFERROR(VLOOKUP(C66,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -24918,23 +24937,30 @@
       </c>
       <c r="J66" s="122"/>
       <c r="K66" s="122"/>
-      <c r="L66" s="97"/>
-      <c r="M66" s="97"/>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L66" s="129" t="str">
+        <f>IF(D66="","",IFERROR(D66/(0.99705-0.00028*(F66-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M66" s="123"/>
+      <c r="N66" s="129" t="str">
+        <f>IF(M66="","",IFERROR(M66/(0.99705-0.00028*(F66-25)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" x14ac:dyDescent="0.2">
       <c r="A67" s="122"/>
       <c r="B67" s="123"/>
       <c r="C67" s="122"/>
       <c r="D67" s="123"/>
       <c r="E67" s="123"/>
       <c r="F67" s="123"/>
-      <c r="G67" s="129">
-        <f t="shared" si="1"/>
-        <v>0.0</v>
-      </c>
-      <c r="H67" s="129">
-        <f>IFERROR((E67/(0.99705-0.00028*(F67-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G67" s="129" t="str">
+        <f>IF(E67="","",IFERROR(E67/(0.99705-0.00028*(F67-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H67" s="129" t="str">
+        <f>IF(E67="","",IFERROR((E67/(0.99705-0.00028*(F67-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I67" s="129" t="str">
         <f>IFERROR(VLOOKUP(C67,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -24942,23 +24968,30 @@
       </c>
       <c r="J67" s="122"/>
       <c r="K67" s="122"/>
-      <c r="L67" s="97"/>
-      <c r="M67" s="97"/>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L67" s="129" t="str">
+        <f>IF(D67="","",IFERROR(D67/(0.99705-0.00028*(F67-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M67" s="123"/>
+      <c r="N67" s="129" t="str">
+        <f>IF(M67="","",IFERROR(M67/(0.99705-0.00028*(F67-25)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" x14ac:dyDescent="0.2">
       <c r="A68" s="122"/>
       <c r="B68" s="123"/>
       <c r="C68" s="122"/>
       <c r="D68" s="123"/>
       <c r="E68" s="123"/>
       <c r="F68" s="123"/>
-      <c r="G68" s="129">
-        <f t="shared" si="1"/>
-        <v>0.0</v>
-      </c>
-      <c r="H68" s="129">
-        <f>IFERROR((E68/(0.99705-0.00028*(F68-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G68" s="129" t="str">
+        <f>IF(E68="","",IFERROR(E68/(0.99705-0.00028*(F68-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H68" s="129" t="str">
+        <f>IF(E68="","",IFERROR((E68/(0.99705-0.00028*(F68-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I68" s="129" t="str">
         <f>IFERROR(VLOOKUP(C68,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -24966,23 +24999,30 @@
       </c>
       <c r="J68" s="122"/>
       <c r="K68" s="122"/>
-      <c r="L68" s="97"/>
-      <c r="M68" s="97"/>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L68" s="129" t="str">
+        <f>IF(D68="","",IFERROR(D68/(0.99705-0.00028*(F68-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M68" s="123"/>
+      <c r="N68" s="129" t="str">
+        <f>IF(M68="","",IFERROR(M68/(0.99705-0.00028*(F68-25)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" x14ac:dyDescent="0.2">
       <c r="A69" s="122"/>
       <c r="B69" s="123"/>
       <c r="C69" s="122"/>
       <c r="D69" s="123"/>
       <c r="E69" s="123"/>
       <c r="F69" s="123"/>
-      <c r="G69" s="129">
-        <f t="shared" si="1"/>
-        <v>0.0</v>
-      </c>
-      <c r="H69" s="129">
-        <f>IFERROR((E69/(0.99705-0.00028*(F69-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G69" s="129" t="str">
+        <f>IF(E69="","",IFERROR(E69/(0.99705-0.00028*(F69-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H69" s="129" t="str">
+        <f>IF(E69="","",IFERROR((E69/(0.99705-0.00028*(F69-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I69" s="129" t="str">
         <f>IFERROR(VLOOKUP(C69,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -24990,23 +25030,30 @@
       </c>
       <c r="J69" s="122"/>
       <c r="K69" s="122"/>
-      <c r="L69" s="97"/>
-      <c r="M69" s="97"/>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L69" s="129" t="str">
+        <f>IF(D69="","",IFERROR(D69/(0.99705-0.00028*(F69-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M69" s="123"/>
+      <c r="N69" s="129" t="str">
+        <f>IF(M69="","",IFERROR(M69/(0.99705-0.00028*(F69-25)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" x14ac:dyDescent="0.2">
       <c r="A70" s="122"/>
       <c r="B70" s="123"/>
       <c r="C70" s="122"/>
       <c r="D70" s="123"/>
       <c r="E70" s="123"/>
       <c r="F70" s="123"/>
-      <c r="G70" s="129">
-        <f t="shared" si="1"/>
-        <v>0.0</v>
-      </c>
-      <c r="H70" s="129">
-        <f>IFERROR((E70/(0.99705-0.00028*(F70-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G70" s="129" t="str">
+        <f>IF(E70="","",IFERROR(E70/(0.99705-0.00028*(F70-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H70" s="129" t="str">
+        <f>IF(E70="","",IFERROR((E70/(0.99705-0.00028*(F70-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I70" s="129" t="str">
         <f>IFERROR(VLOOKUP(C70,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -25014,23 +25061,30 @@
       </c>
       <c r="J70" s="122"/>
       <c r="K70" s="122"/>
-      <c r="L70" s="97"/>
-      <c r="M70" s="97"/>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L70" s="129" t="str">
+        <f>IF(D70="","",IFERROR(D70/(0.99705-0.00028*(F70-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M70" s="123"/>
+      <c r="N70" s="129" t="str">
+        <f>IF(M70="","",IFERROR(M70/(0.99705-0.00028*(F70-25)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" x14ac:dyDescent="0.2">
       <c r="A71" s="122"/>
       <c r="B71" s="123"/>
       <c r="C71" s="122"/>
       <c r="D71" s="123"/>
       <c r="E71" s="123"/>
       <c r="F71" s="123"/>
-      <c r="G71" s="129">
-        <f t="shared" si="1"/>
-        <v>0.0</v>
-      </c>
-      <c r="H71" s="129">
-        <f>IFERROR((E71/(0.99705-0.00028*(F71-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G71" s="129" t="str">
+        <f>IF(E71="","",IFERROR(E71/(0.99705-0.00028*(F71-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H71" s="129" t="str">
+        <f>IF(E71="","",IFERROR((E71/(0.99705-0.00028*(F71-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I71" s="129" t="str">
         <f>IFERROR(VLOOKUP(C71,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -25038,23 +25092,30 @@
       </c>
       <c r="J71" s="122"/>
       <c r="K71" s="122"/>
-      <c r="L71" s="97"/>
-      <c r="M71" s="97"/>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L71" s="129" t="str">
+        <f>IF(D71="","",IFERROR(D71/(0.99705-0.00028*(F71-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M71" s="123"/>
+      <c r="N71" s="129" t="str">
+        <f>IF(M71="","",IFERROR(M71/(0.99705-0.00028*(F71-25)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" x14ac:dyDescent="0.2">
       <c r="A72" s="122"/>
       <c r="B72" s="123"/>
       <c r="C72" s="122"/>
       <c r="D72" s="123"/>
       <c r="E72" s="123"/>
       <c r="F72" s="123"/>
-      <c r="G72" s="129">
-        <f t="shared" si="1"/>
-        <v>0.0</v>
-      </c>
-      <c r="H72" s="129">
-        <f>IFERROR((E72/(0.99705-0.00028*(F72-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G72" s="129" t="str">
+        <f>IF(E72="","",IFERROR(E72/(0.99705-0.00028*(F72-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H72" s="129" t="str">
+        <f>IF(E72="","",IFERROR((E72/(0.99705-0.00028*(F72-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I72" s="129" t="str">
         <f>IFERROR(VLOOKUP(C72,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -25062,23 +25123,30 @@
       </c>
       <c r="J72" s="122"/>
       <c r="K72" s="122"/>
-      <c r="L72" s="97"/>
-      <c r="M72" s="97"/>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="L72" s="129" t="str">
+        <f>IF(D72="","",IFERROR(D72/(0.99705-0.00028*(F72-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M72" s="123"/>
+      <c r="N72" s="129" t="str">
+        <f>IF(M72="","",IFERROR(M72/(0.99705-0.00028*(F72-25)),""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" x14ac:dyDescent="0.2">
       <c r="A73" s="122"/>
       <c r="B73" s="123"/>
       <c r="C73" s="122"/>
       <c r="D73" s="123"/>
       <c r="E73" s="123"/>
       <c r="F73" s="123"/>
-      <c r="G73" s="129">
-        <f t="shared" si="1"/>
-        <v>0.0</v>
-      </c>
-      <c r="H73" s="129">
-        <f>IFERROR((E73/(0.99705-0.00028*(F73-25)))*1000/Geometry!$D$21,"")</f>
-        <v>0.0</v>
+      <c r="G73" s="129" t="str">
+        <f>IF(E73="","",IFERROR(E73/(0.99705-0.00028*(F73-25)),""))</f>
+        <v/>
+      </c>
+      <c r="H73" s="129" t="str">
+        <f>IF(E73="","",IFERROR((E73/(0.99705-0.00028*(F73-25)))*1000/Geometry!$D$21,""))</f>
+        <v/>
       </c>
       <c r="I73" s="129" t="str">
         <f>IFERROR(VLOOKUP(C73,Geometry!$A$59:$B$80,2,FALSE),"")</f>
@@ -25086,8 +25154,15 @@
       </c>
       <c r="J73" s="122"/>
       <c r="K73" s="122"/>
-      <c r="L73" s="97"/>
-      <c r="M73" s="97"/>
+      <c r="L73" s="129" t="str">
+        <f>IF(D73="","",IFERROR(D73/(0.99705-0.00028*(F73-25)),""))</f>
+        <v/>
+      </c>
+      <c r="M73" s="123"/>
+      <c r="N73" s="129" t="str">
+        <f>IF(M73="","",IFERROR(M73/(0.99705-0.00028*(F73-25)),""))</f>
+        <v/>
+      </c>
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A74" s="125" t="s">
@@ -25134,10 +25209,21 @@
       <c r="M75" s="97"/>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A76" s="97"/>
+      <c r="A76" s="125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - headspace at working fill</t>
+        </is>
+      </c>
       <c r="B76" s="97"/>
-      <c r="C76" s="97"/>
-      <c r="D76" s="97"/>
+      <c r="C76" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D76" s="124" t="str">
+        <f>IFERROR(AVERAGEIFS(L66:L73,I66:I73,Geometry!$D$51,J66:J73,"y"),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
       <c r="E76" s="97"/>
       <c r="F76" s="97"/>
       <c r="G76" s="97"/>
@@ -25149,10 +25235,21 @@
       <c r="M76" s="97"/>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A77" s="97"/>
+      <c r="A77" s="125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - working fill behind that headspace</t>
+        </is>
+      </c>
       <c r="B77" s="97"/>
-      <c r="C77" s="97"/>
-      <c r="D77" s="97"/>
+      <c r="C77" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D77" s="124" t="str">
+        <f>IFERROR(AVERAGEIFS(N66:N73,I66:I73,Geometry!$D$51,J66:J73,"y"),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
       <c r="E77" s="97"/>
       <c r="F77" s="97"/>
       <c r="G77" s="97"/>

</xml_diff>

<commit_message>
Gas model: protocol hyperlinks point at AEP02, not the retired CO2-modular branch
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -8847,7 +8847,7 @@
         <v>1015</v>
       </c>
       <c r="D66" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/surface-kla.md","surface-kla.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/surface-kla.md","surface-kla.md →")</f>
         <v>surface-kla.md →</v>
       </c>
       <c r="E66" s="103"/>
@@ -8866,7 +8866,7 @@
         <v>1018</v>
       </c>
       <c r="D67" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/vial-geometry.md","vial-geometry.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/vial-geometry.md","vial-geometry.md →")</f>
         <v>vial-geometry.md →</v>
       </c>
       <c r="E67" s="103"/>
@@ -8885,7 +8885,7 @@
         <v>1022</v>
       </c>
       <c r="D68" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/faradaic-efficiency.md","faradaic-efficiency.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/faradaic-efficiency.md","faradaic-efficiency.md →")</f>
         <v>faradaic-efficiency.md →</v>
       </c>
       <c r="E68" s="103"/>
@@ -8904,7 +8904,7 @@
         <v>1025</v>
       </c>
       <c r="D69" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/knallgas-stoichiometry.md","knallgas-stoichiometry.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/knallgas-stoichiometry.md","knallgas-stoichiometry.md →")</f>
         <v>knallgas-stoichiometry.md →</v>
       </c>
       <c r="E69" s="103"/>
@@ -8923,7 +8923,7 @@
         <v>1029</v>
       </c>
       <c r="D70" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/faradaic-efficiency.md","faradaic-efficiency.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/faradaic-efficiency.md","faradaic-efficiency.md →")</f>
         <v>faradaic-efficiency.md →</v>
       </c>
       <c r="E70" s="103"/>
@@ -8942,7 +8942,7 @@
         <v>1032</v>
       </c>
       <c r="D71" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/vial-geometry.md","vial-geometry.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/vial-geometry.md","vial-geometry.md →")</f>
         <v>vial-geometry.md →</v>
       </c>
       <c r="E71" s="103"/>
@@ -8961,7 +8961,7 @@
         <v>1036</v>
       </c>
       <c r="D72" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/flow-calibration.md","flow-calibration.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/flow-calibration.md","flow-calibration.md →")</f>
         <v>flow-calibration.md →</v>
       </c>
       <c r="E72" s="103"/>
@@ -8980,7 +8980,7 @@
         <v>1040</v>
       </c>
       <c r="D73" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/dissolved-oxygen.md","dissolved-oxygen.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/dissolved-oxygen.md","dissolved-oxygen.md →")</f>
         <v>dissolved-oxygen.md →</v>
       </c>
       <c r="E73" s="103"/>
@@ -8999,7 +8999,7 @@
         <v>1044</v>
       </c>
       <c r="D74" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/flow-calibration.md","flow-calibration.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/flow-calibration.md","flow-calibration.md →")</f>
         <v>flow-calibration.md →</v>
       </c>
       <c r="E74" s="103"/>
@@ -9018,7 +9018,7 @@
         <v>1048</v>
       </c>
       <c r="D75" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/sinter-porosity.md","sinter-porosity.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/sinter-porosity.md","sinter-porosity.md →")</f>
         <v>sinter-porosity.md →</v>
       </c>
       <c r="E75" s="103"/>
@@ -9037,7 +9037,7 @@
         <v>1052</v>
       </c>
       <c r="D76" s="36" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/README.md","README.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/README.md","README.md →")</f>
         <v>README.md →</v>
       </c>
       <c r="E76" s="103"/>
@@ -9056,7 +9056,7 @@
         <v>1052</v>
       </c>
       <c r="D77" s="23" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/current-density-screen.md","current-density-screen.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/current-density-screen.md","current-density-screen.md →")</f>
         <v>current-density-screen.md →</v>
       </c>
       <c r="E77" s="20"/>
@@ -9075,7 +9075,7 @@
         <v>1052</v>
       </c>
       <c r="D78" s="23" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/vial-geometry.md","vial-geometry.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/vial-geometry.md","vial-geometry.md →")</f>
         <v>vial-geometry.md →</v>
       </c>
       <c r="E78" s="20"/>
@@ -9094,7 +9094,7 @@
         <v>1052</v>
       </c>
       <c r="D79" s="23" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/gerrit-current.md","gerrit-current.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/gerrit-current.md","gerrit-current.md →")</f>
         <v>gerrit-current.md →</v>
       </c>
       <c r="E79" s="20"/>
@@ -9113,7 +9113,7 @@
         <v>1029</v>
       </c>
       <c r="D80" s="23" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/README.md","README.md →")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/README.md","README.md →")</f>
         <v>README.md →</v>
       </c>
       <c r="F80" t="s">
@@ -23829,7 +23829,7 @@
     </row>
     <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/gerrit-current.md","ELECTROLYSIS CURRENT")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/gerrit-current.md","ELECTROLYSIS CURRENT")</f>
         <v>ELECTROLYSIS CURRENT</v>
       </c>
     </row>
@@ -23994,7 +23994,7 @@
     </row>
     <row r="20" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/faradaic-efficiency.md","FARADAIC EFFICIENCY  (cathodic etaF, anodic etaF_OER)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/faradaic-efficiency.md","FARADAIC EFFICIENCY  (cathodic etaF, anodic etaF_OER)")</f>
         <v>FARADAIC EFFICIENCY  (cathodic etaF, anodic etaF_OER)</v>
       </c>
     </row>
@@ -24285,7 +24285,7 @@
     </row>
     <row r="35" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="127" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/surface-kla.md","SURFACE kLa  (oxygen surface transfer)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/surface-kla.md","SURFACE kLa  (oxygen surface transfer)")</f>
         <v>SURFACE kLa  (oxygen surface transfer)</v>
       </c>
       <c r="B35" s="97"/>
@@ -24545,7 +24545,7 @@
     </row>
     <row r="49" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="127" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/flow-calibration.md","CO2 FLOW  (dosing flow rate)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/flow-calibration.md","CO2 FLOW  (dosing flow rate)")</f>
         <v>CO2 FLOW  (dosing flow rate)</v>
       </c>
       <c r="B49" s="97"/>
@@ -24833,7 +24833,7 @@
     </row>
     <row r="63" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="127" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/vial-geometry.md","VIAL GEOMETRY  (true volume &amp; bore depth)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/vial-geometry.md","VIAL GEOMETRY  (true volume &amp; bore depth)")</f>
         <v>VIAL GEOMETRY  (true volume &amp; bore depth)</v>
       </c>
       <c r="B63" s="97"/>
@@ -25262,7 +25262,7 @@
     </row>
     <row r="78" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A78" s="127" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/sinter-porosity.md","SINTER POROSITY  (sparger frit grade)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/sinter-porosity.md","SINTER POROSITY  (sparger frit grade)")</f>
         <v>SINTER POROSITY  (sparger frit grade)</v>
       </c>
       <c r="B78" s="97"/>
@@ -25548,7 +25548,7 @@
     </row>
     <row r="92" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A92" s="127" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/dissolved-oxygen.md","DISSOLVED-OXYGEN THRESHOLDS  (per organism)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/dissolved-oxygen.md","DISSOLVED-OXYGEN THRESHOLDS  (per organism)")</f>
         <v>DISSOLVED-OXYGEN THRESHOLDS  (per organism)</v>
       </c>
       <c r="B92" s="97"/>
@@ -25854,7 +25854,7 @@
     </row>
     <row r="109" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A109" s="127" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/knallgas-stoichiometry.md","KNALLGAS UPTAKE RATIO  (per organism)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/knallgas-stoichiometry.md","KNALLGAS UPTAKE RATIO  (per organism)")</f>
         <v>KNALLGAS UPTAKE RATIO  (per organism)</v>
       </c>
       <c r="B109" s="97"/>
@@ -26136,7 +26136,7 @@
     </row>
     <row r="125" spans="1:13" ht="16" x14ac:dyDescent="0.2">
       <c r="A125" s="127" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/CO2-modular/Media/protocols/current-density-screen.md","CURRENT-DENSITY TOLERANCE  (per organism)")</f>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/current-density-screen.md","CURRENT-DENSITY TOLERANCE  (per organism)")</f>
         <v>CURRENT-DENSITY TOLERANCE  (per organism)</v>
       </c>
       <c r="B125" s="97"/>

</xml_diff>

<commit_message>
Gas model: strip Excel's embedded absolute path from workbook.xml
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martincurrie/andeye Dropbox/andeye/Projects/electroPioreactor/Media/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96CC8FD1-785B-AC4D-8121-CAB29CA67389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4720" yWindow="9920" windowWidth="25160" windowHeight="18060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>

</xml_diff>

<commit_message>
Gas model: buffer, chlorine and flammability verdicts corrected; unsafe carbon-relax advisory removed; kLa protocol units
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -577,6 +577,31 @@
     <definedName name="z_e_ORR" localSheetId="2">Electrochemistry!$D$27</definedName>
     <definedName name="cal_hs">Calibrations!$D$76</definedName>
     <definedName name="cal_hs_fill">Calibrations!$D$77</definedName>
+    <definedName name="D_HCO3" localSheetId="3">Chemistry!$D$251</definedName>
+    <definedName name="HCO3_op" localSheetId="3">Chemistry!$D$252</definedName>
+    <definedName name="HPO4_op" localSheetId="3">Chemistry!$D$253</definedName>
+    <definedName name="eta_anode_c" localSheetId="3">Chemistry!$D$254</definedName>
+    <definedName name="pcet_credit_c" localSheetId="3">Chemistry!$D$255</definedName>
+    <definedName name="E_anode_op" localSheetId="3">Chemistry!$D$256</definedName>
+    <definedName name="E0_HOCl" localSheetId="3">Chemistry!$D$257</definedName>
+    <definedName name="E_HOCl_Cl" localSheetId="3">Chemistry!$D$258</definedName>
+    <definedName name="C_eff_lo_Cl2" localSheetId="3">Chemistry!$D$259</definedName>
+    <definedName name="C_eff_hi_Cl2" localSheetId="3">Chemistry!$D$260</definedName>
+    <definedName name="M_O2" localSheetId="5">'Mass Transfer'!$D$231</definedName>
+    <definedName name="DO_at_carbon" localSheetId="5">'Mass Transfer'!$D$232</definedName>
+    <definedName name="CO2_supply_b" localSheetId="4">Biology!$D$76</definedName>
+    <definedName name="CO2_rate_full_b" localSheetId="4">Biology!$D$77</definedName>
+    <definedName name="spg_dur_b" localSheetId="4">Biology!$D$78</definedName>
+    <definedName name="R_gas_b" localSheetId="4">Biology!$D$79</definedName>
+    <definedName name="H2_LFL" localSheetId="4">Biology!$D$80</definedName>
+    <definedName name="O2_LOC_H2" localSheetId="4">Biology!$D$81</definedName>
+    <definedName name="LOC_margin" localSheetId="4">Biology!$D$82</definedName>
+    <definedName name="n_flamm_src" localSheetId="4">Biology!$D$83</definedName>
+    <definedName name="y_H2_hs_lag" localSheetId="4">Biology!$D$84</definedName>
+    <definedName name="y_O2_hs_lag" localSheetId="4">Biology!$D$85</definedName>
+    <definedName name="duty_H2safe" localSheetId="4">Biology!$D$86</definedName>
+    <definedName name="spg_int_H2safe" localSheetId="4">Biology!$D$87</definedName>
+    <definedName name="N2_sweep_H2safe" localSheetId="4">Biology!$D$88</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8043,7 +8068,7 @@
         <v>13</v>
       </c>
       <c r="D13" s="90">
-        <f>IFERROR('Mass Transfer'!$D$90,"calibrate this reactor first (see CO2 flows)")</f>
+        <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$90)</f>
         <v>0.784513049825</v>
       </c>
       <c r="E13" s="23" t="str">
@@ -8079,7 +8104,7 @@
         <v>67</v>
       </c>
       <c r="D15" s="90">
-        <f>IFERROR('Mass Transfer'!$D$91,"calibrate this reactor first (see CO2 flows)")</f>
+        <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$91)</f>
         <v>16.46036421628</v>
       </c>
       <c r="E15" s="23" t="str">
@@ -8205,39 +8230,47 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="89" t="s">
-        <v>78</v>
+      <c r="A23" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Can the interval relax to the carbon-limited one?</t>
+        </is>
       </c>
       <c r="B23" s="20"/>
       <c r="C23" s="20"/>
       <c r="D23" s="90" t="str">
         <f>'Mass Transfer'!$D$113</f>
-        <v>organism DO unknown</v>
+        <v>Do NOT relax: at the carbon-limited interval (185 min) DO would be 12.9 mg/L against a 2.6 mg/L target</v>
       </c>
       <c r="E23" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F23" s="21" t="s">
-        <v>79</v>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Green only if CO₂ dosed for carbon alone would still hold dissolved O₂ at the target; otherwise it states the DO the longer interval would give.</t>
+        </is>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="89" t="s">
-        <v>80</v>
+      <c r="A24" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ headspace flammable?</t>
+        </is>
       </c>
       <c r="B24" s="20"/>
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
-        <v>EXPLOSIVE</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 19%, O₂ 9% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="23" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
         <v>→ Biology</v>
       </c>
-      <c r="F24" s="21" t="s">
-        <v>81</v>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag-phase headspace (electrolysis on, no H₂ uptake) against the H₂ flammability limit and the O₂ limiting concentration; the text names the remedy.</t>
+        </is>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -8445,14 +8478,16 @@
       </c>
       <c r="D36" s="121">
         <f>Chemistry!$D$226</f>
-        <v>0.500655956628</v>
+        <v>0.500804384457</v>
       </c>
       <c r="E36" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F36" s="21" t="s">
-        <v>1930</v>
+      <c r="F36" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effective biocidal chlorine from the medium’s chloride, as Cl₂ (the basis of the thresholds). Onset 0.1 mg/L, kill 2 mg/L (Chemistry D146/D147); colour: green below 0.1, red above 1. Zero for chloride-free media.</t>
+        </is>
       </c>
     </row>
     <row r="37" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -8475,7 +8510,7 @@
       </c>
       <c r="D38" s="90">
         <f>'Mass Transfer'!$D$108</f>
-        <v>2.639031652174</v>
+        <v>2.638866712696</v>
       </c>
       <c r="E38" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D108","→ Mass")</f>
@@ -9111,8 +9146,10 @@
         <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/README.md","README.md →")</f>
         <v>README.md →</v>
       </c>
-      <c r="F80" t="s">
-        <v>1911</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cu/Ni/Fe by ICP or a colorimetric kit. The operating anode sits well above the Cu²⁺/Cu equilibrium (row 88), so dissolution is thermodynamically allowed; this is the unmodelled prime suspect for the Exp-2 death and it also closes the anodic charge budget.</t>
+        </is>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
@@ -9205,7 +9242,7 @@
       </c>
       <c r="D86" s="22" t="str">
         <f>Chemistry!$D$219</f>
-        <v>BUFFER EXCEEDED — anode surface acidifies (local pH ~1 unit below bulk); the pH solved above is the bulk value only</v>
+        <v>OK — buffer holds the electrode surfaces at the bulk pH</v>
       </c>
       <c r="E86" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D219","→ Chemistry")</f>
@@ -9216,22 +9253,26 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>1593</v>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOCl/Cl⁻ couple minus anode potential</t>
+        </is>
       </c>
       <c r="C87" s="19" t="s">
         <v>1595</v>
       </c>
       <c r="D87" s="22">
         <f>Chemistry!$D$209</f>
-        <v>0.741190671663</v>
+        <v>-0.422483519032</v>
       </c>
       <c r="E87" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D209","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F87" t="s">
-        <v>1872</v>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negative = the anode is above the chloride-oxidation couple: chlorine forms, limited by chloride transport (Chemistry D132).</t>
+        </is>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
@@ -9243,14 +9284,16 @@
       </c>
       <c r="D88" s="22">
         <f>Chemistry!$D$211</f>
-        <v>0.49641463654</v>
+        <v>1.240557060036</v>
       </c>
       <c r="E88" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F88" t="s">
-        <v>1873</v>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How far the operating anode sits above the Cu²⁺/Cu standard potential; positive = copper dissolution thermodynamically allowed.</t>
+        </is>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.2">
@@ -14966,8 +15009,8 @@
         <v>956</v>
       </c>
       <c r="D104" s="62">
-        <f>1/(1+10^(pH_meas-pKa_HOCl))</f>
-        <v>0.896166326878</v>
+        <f>1/(1+KaHOCl_c/10^-pH_op)</f>
+        <v>0.870210730329</v>
       </c>
       <c r="E104" s="51" t="s">
         <v>1879</v>
@@ -15053,8 +15096,8 @@
         <v>966</v>
       </c>
       <c r="D109" s="64" t="str">
-        <f>IF(C_eff&lt;Cl_onset,"negligible free chlorine ("&amp;TEXT(C_eff,"0.00")&amp;" mg/L &lt; onset); does NOT account for the Exp-2 death - see metal_flag",IF(C_eff&lt;Cl_kill,"sub-lethal "&amp;TEXT(C_eff,"0.00")&amp;" mg/L (band "&amp;TEXT(C_eff_lo,"0.00")&amp;"-"&amp;TEXT(C_eff_hi,"0.00")&amp;"); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag","SEVERE free chlorine: "&amp;TEXT(C_eff,"0.0")&amp;" mg/L biofilm/electrode damage (Baek 2021)"))</f>
-        <v>sub-lethal 0.37 mg/L (band 0.00-0.53); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
+        <f>IF(C_eff_Cl2&lt;Cl_onset,"negligible free chlorine ("&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ &lt; onset); does NOT account for the Exp-2 death - see metal_flag",IF(C_eff_Cl2&lt;Cl_kill,"sub-lethal "&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ (band "&amp;TEXT(C_eff_lo_Cl2,"0.00")&amp;"-"&amp;TEXT(C_eff_hi_Cl2,"0.00")&amp;"); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag","SEVERE free chlorine: "&amp;TEXT(C_eff_Cl2,"0.0")&amp;" mg/L as Cl₂ - biofilm/electrode damage (Baek 2021)"))</f>
+        <v>sub-lethal 0.50 mg/L as Cl₂ (band 0.00-0.71); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
       </c>
       <c r="E109" s="51" t="s">
         <v>1127</v>
@@ -15157,7 +15200,7 @@
       </c>
       <c r="D125" s="62">
         <f>pH_Cl*pH_fHOCl*M_HOCl</f>
-        <v>8.472316725176</v>
+        <v>8.22693366608</v>
       </c>
       <c r="E125" s="51" t="s">
         <v>1460</v>
@@ -15356,8 +15399,8 @@
         <v>1098</v>
       </c>
       <c r="D138" s="62">
-        <f>pH_NT/(1+10^(pKa_NH4-pH_meas))</f>
-        <v>1.5968172298e-05</v>
+        <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
+        <v>1.241103645704e-05</v>
       </c>
       <c r="E138" s="51" t="s">
         <v>1099</v>
@@ -15375,7 +15418,7 @@
       </c>
       <c r="D139" s="62">
         <f>P_HOCl/(k1_NH2Cl*NH3_free)</f>
-        <v>7.303649900372e-10</v>
+        <v>9.396954107506e-10</v>
       </c>
       <c r="E139" s="51" t="s">
         <v>1102</v>
@@ -15393,7 +15436,7 @@
       </c>
       <c r="D140" s="62">
         <f>HOCl_ss*M_HOCl</f>
-        <v>3.831494737735e-05</v>
+        <v>4.929642124798e-05</v>
       </c>
       <c r="E140" s="51" t="s">
         <v>1105</v>
@@ -15480,7 +15523,7 @@
       </c>
       <c r="D145" s="62">
         <f>f_local*HOCl_ss_mgL+NH2Cl_mgL/R_chloramine</f>
-        <v>0.37041169273</v>
+        <v>0.370521507469</v>
       </c>
       <c r="E145" s="51" t="s">
         <v>1464</v>
@@ -15672,7 +15715,7 @@
       </c>
       <c r="D156" s="62">
         <f>f_local*HOCl_ss_mgL+NH2Cl_lo/R_chloramine_hi</f>
-        <v>0.002585700326</v>
+        <v>0.002695515065</v>
       </c>
       <c r="E156" s="51" t="s">
         <v>1247</v>
@@ -15690,7 +15733,7 @@
       </c>
       <c r="D157" s="62">
         <f>f_local*HOCl_ss_mgL+NH2Cl_hi/R_chloramine_lo</f>
-        <v>0.52560290879</v>
+        <v>0.525712723528</v>
       </c>
       <c r="E157" s="51" t="s">
         <v>1251</v>
@@ -16481,8 +16524,10 @@
       </c>
     </row>
     <row r="208" spans="1:5" ht="24" x14ac:dyDescent="0.2">
-      <c r="A208" t="s">
-        <v>1590</v>
+      <c r="A208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cl₂/Cl⁻ potential at the medium chloride (Cl₂ gas at 1 atm, reference only)</t>
+        </is>
       </c>
       <c r="B208" s="18" t="s">
         <v>1591</v>
@@ -16499,8 +16544,10 @@
       </c>
     </row>
     <row r="209" spans="1:5" ht="60" x14ac:dyDescent="0.2">
-      <c r="A209" t="s">
-        <v>1593</v>
+      <c r="A209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOCl/Cl⁻ couple minus operating anode potential</t>
+        </is>
       </c>
       <c r="B209" s="18" t="s">
         <v>1594</v>
@@ -16509,11 +16556,13 @@
         <v>1595</v>
       </c>
       <c r="D209" s="22">
-        <f>E_Cl2-E_OER</f>
-        <v>0.741190671663</v>
-      </c>
-      <c r="E209" s="67" t="s">
-        <v>1596</v>
+        <f>E_HOCl_Cl-E_anode_op</f>
+        <v>-0.422483519032</v>
+      </c>
+      <c r="E209" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Negative = the anode sits above the HOCl/Cl⁻ couple, so chloride oxidation is thermodynamically accessible and, on Pt, transport-limited (Chemistry D132). Cl₂ gas at 1 atm (D208) is a reference only: at trace chloride the product is HOCl.</t>
+        </is>
       </c>
     </row>
     <row r="210" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -16535,8 +16584,10 @@
       </c>
     </row>
     <row r="211" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A211" t="s">
-        <v>1600</v>
+      <c r="A211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operating anode potential above Cu²⁺/Cu</t>
+        </is>
       </c>
       <c r="B211" s="18" t="s">
         <v>1601</v>
@@ -16545,8 +16596,8 @@
         <v>1595</v>
       </c>
       <c r="D211" s="22">
-        <f>E_OER-E0_Cu</f>
-        <v>0.49641463654</v>
+        <f>E_anode_op-E0_Cu</f>
+        <v>1.240557060036</v>
       </c>
       <c r="E211" s="67" t="s">
         <v>1602</v>
@@ -16602,11 +16653,13 @@
         <v>1282</v>
       </c>
       <c r="D216" s="22">
-        <f>Fcc*D_HPO4*(pH_PT*(1-1/(1+10^(pH_meas-(-LOG10(Ka2p_c))))))*1000/(delta_diff/1000000)/10</f>
-        <v>2.804749298695</v>
-      </c>
-      <c r="E216" s="67" t="s">
-        <v>1612</v>
+        <f>Fcc*(D_HPO4*HPO4_op+D_HCO3*HCO3_op)*1000/(delta_diff/1000000)/10</f>
+        <v>8.049160263403</v>
+      </c>
+      <c r="E216" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">j_lim = F·Σ(D·C)/δ over the proton acceptors reaching the anode: hydrogen phosphate and bicarbonate (D251–D253). At the CO₂-dosed operating point bicarbonate is the larger term; at air equilibrium it falls to ~0.4 mM and the phosphate term alone applies, so re-read this verdict whenever the schedule changes.</t>
+        </is>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.2">
@@ -16639,7 +16692,7 @@
       </c>
       <c r="D218" s="22">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>1.007610801297</v>
+        <v>0.35110441286</v>
       </c>
       <c r="E218" s="67" t="s">
         <v>1618</v>
@@ -16657,7 +16710,7 @@
       </c>
       <c r="D219" s="22" t="str">
         <f>IF(j_buffer_ratio&gt;1,"BUFFER EXCEEDED — anode surface acidifies (local pH ~1 unit below bulk); the pH solved above is the bulk value only",IF(j_buffer_ratio&gt;0.5,"watch — running at "&amp;TEXT(j_buffer_ratio,"0%")&amp;" of the phosphate buffer limit; expect a 0.4–1.0 unit excursion at each electrode surface","OK — buffer holds the electrode surfaces at the bulk pH"))</f>
-        <v>BUFFER EXCEEDED — anode surface acidifies (local pH ~1 unit below bulk); the pH solved above is the bulk value only</v>
+        <v>OK — buffer holds the electrode surfaces at the bulk pH</v>
       </c>
       <c r="E219" s="67" t="s">
         <v>1621</v>
@@ -16766,10 +16819,275 @@
       </c>
       <c r="D226" s="22">
         <f>C_eff*M_Cl2/M_HOCl</f>
-        <v>0.500655956628</v>
+        <v>0.500804384457</v>
       </c>
       <c r="E226" s="67" t="s">
         <v>1899</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELECTRODE-SURFACE CHEMISTRY AT THE OPERATING POINT</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diffusion coefficient — HCO₃⁻</t>
+        </is>
+      </c>
+      <c r="B251" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D_HCO3</t>
+        </is>
+      </c>
+      <c r="C251" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m²/s</t>
+        </is>
+      </c>
+      <c r="D251" s="52">
+        <v>1.185e-09</v>
+      </c>
+      <c r="E251" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRC Handbook (Vanýsek), ionic diffusion coefficient at 25 °C, 1.185×10⁻⁵ cm²/s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bicarbonate at the operating point</t>
+        </is>
+      </c>
+      <c r="B252" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HCO3_op</t>
+        </is>
+      </c>
+      <c r="C252" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D252" s="22">
+        <f>Ka1c_c*CO2aqc/10^-pH_op</f>
+        <v>0.01976870305</v>
+      </c>
+      <c r="E252" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concentration scale, same speciation the charge balance solves (Ka1c_c with pH_op).</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hydrogen phosphate at the operating point</t>
+        </is>
+      </c>
+      <c r="B253" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HPO4_op</t>
+        </is>
+      </c>
+      <c r="C253" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D253" s="22">
+        <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
+        <v>0.013100861499</v>
+      </c>
+      <c r="E253" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concentration scale: HPO₄²⁻ share of total phosphate at pH_op with the concentration-scale pKa2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) anode overpotential</t>
+        </is>
+      </c>
+      <c r="B254" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eta_anode_c</t>
+        </is>
+      </c>
+      <c r="C254" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="D254" s="22">
+        <f>Electrochemistry!$D$111</f>
+        <v>0.894142423496</v>
+      </c>
+      <c r="E254" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D111 (Tafel, at the operating current density).</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) proton-coupled credit</t>
+        </is>
+      </c>
+      <c r="B255" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pcet_credit_c</t>
+        </is>
+      </c>
+      <c r="C255" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="D255" s="22">
+        <f>Electrochemistry!$D$113</f>
+        <v>-0.15</v>
+      </c>
+      <c r="E255" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D113.</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operating anode potential</t>
+        </is>
+      </c>
+      <c r="B256" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E_anode_op</t>
+        </is>
+      </c>
+      <c r="C256" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V vs SHE</t>
+        </is>
+      </c>
+      <c r="D256" s="22">
+        <f>E_OER+eta_anode_c+pcet_credit_c</f>
+        <v>1.582457060036</v>
+      </c>
+      <c r="E256" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reversible O₂/H₂O potential at the bulk pH plus the anode overpotential and the proton-coupled credit from the cell-voltage budget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard potential — HOCl + H⁺ + 2e⁻ → Cl⁻ + H₂O</t>
+        </is>
+      </c>
+      <c r="B257" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E0_HOCl</t>
+        </is>
+      </c>
+      <c r="C257" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="D257" s="52">
+        <v>1.482</v>
+      </c>
+      <c r="E257" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRC Handbook §5, ±0.002 V.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOCl/Cl⁻ potential at the operating point</t>
+        </is>
+      </c>
+      <c r="B258" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E_HOCl_Cl</t>
+        </is>
+      </c>
+      <c r="C258" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V vs SHE</t>
+        </is>
+      </c>
+      <c r="D258" s="22">
+        <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,1E-12))-pH_meas-LOG10(MAX(pH_Cl,1E-12)))</f>
+        <v>1.159973541004</v>
+      </c>
+      <c r="E258" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nernst for the couple actually formed at trace chloride (HOCl at nanomolar level, not Cl₂ gas at 1 atm), at the electrode-enriched HOCl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Free chlorine low end, as Cl₂</t>
+        </is>
+      </c>
+      <c r="B259" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C_eff_lo_Cl2</t>
+        </is>
+      </c>
+      <c r="C259" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D259" s="22">
+        <f>C_eff_lo*M_Cl2/M_HOCl</f>
+        <v>0.003643312833</v>
+      </c>
+      <c r="E259" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C_eff_lo on the as-Cl₂ basis the thresholds use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Free chlorine high end, as Cl₂</t>
+        </is>
+      </c>
+      <c r="B260" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C_eff_hi_Cl2</t>
+        </is>
+      </c>
+      <c r="C260" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D260" s="22">
+        <f>C_eff_hi*M_Cl2/M_HOCl</f>
+        <v>0.710563979689</v>
+      </c>
+      <c r="E260" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C_eff_hi on the as-Cl₂ basis the thresholds use.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -17581,8 +17899,10 @@
       <c r="F43" s="20"/>
     </row>
     <row r="44" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="17" t="s">
-        <v>509</v>
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ headspace flammability verdict</t>
+        </is>
       </c>
       <c r="B44" s="18" t="s">
         <v>510</v>
@@ -17591,11 +17911,13 @@
         <v>135</v>
       </c>
       <c r="D44" s="48" t="str">
-        <f>IF(H2_turnover&gt;1,"EXPLOSIVE","watch")</f>
-        <v>EXPLOSIVE</v>
-      </c>
-      <c r="E44" s="70" t="s">
-        <v>511</v>
+        <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;", O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag basis)")</f>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 19%, O₂ 9% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+      </c>
+      <c r="E44" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tests the lag-phase headspace mix (rows 84–85) against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin. Replaces a dissolved-H₂ turnover proxy, which said nothing about flammability.</t>
+        </is>
       </c>
       <c r="F44" s="101" t="s">
         <v>512</v>
@@ -17873,6 +18195,348 @@
       </c>
       <c r="E61" s="68" t="s">
         <v>1928</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEADSPACE FLAMMABILITY (lag phase: electrolysis running, no H₂ uptake yet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) average CO₂ supply rate</t>
+        </is>
+      </c>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_supply_b</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D76" s="27">
+        <f>'Mass Transfer'!$D$100</f>
+        <v>0.0003892277799716</v>
+      </c>
+      <c r="E76" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D100 (schedule in use).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) CO₂ rate while the valve is open</t>
+        </is>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_rate_full_b</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D77" s="27">
+        <f>'Mass Transfer'!$D$178</f>
+        <v>0.489998045758</v>
+      </c>
+      <c r="E77" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D178.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) pulse duration</t>
+        </is>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_dur_b</t>
+        </is>
+      </c>
+      <c r="C78" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D78" s="27">
+        <f>'Mass Transfer'!$D$90</f>
+        <v>0.784513049825</v>
+      </c>
+      <c r="E78" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D90.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) ideal gas constant</t>
+        </is>
+      </c>
+      <c r="B79" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R_gas_b</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">J/(mol·K)</t>
+        </is>
+      </c>
+      <c r="D79" s="27">
+        <f>'Mass Transfer'!$D$101</f>
+        <v>8.314462618</v>
+      </c>
+      <c r="E79" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D101.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ lower flammability limit</t>
+        </is>
+      </c>
+      <c r="B80" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_LFL</t>
+        </is>
+      </c>
+      <c r="C80" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D80" s="52">
+        <v>0.04</v>
+      </c>
+      <c r="E80" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.0 vol% in air or O₂ (Coward &amp; Jones 1952; Zabetakis 1965, USBM Bulletin 627).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limiting O₂ concentration for H₂, CO₂ diluent</t>
+        </is>
+      </c>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_LOC_H2</t>
+        </is>
+      </c>
+      <c r="C81" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D81" s="52">
+        <v>0.052</v>
+      </c>
+      <c r="E81" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">About 5.2 vol% O₂ with CO₂ as diluent (5.0 % with N₂): Zabetakis 1965; NFPA 69 annex table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design margin on the LOC</t>
+        </is>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOC_margin</t>
+        </is>
+      </c>
+      <c r="C82" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D82" s="52">
+        <v>0.6</v>
+      </c>
+      <c r="E82" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFPA 69: hold O₂ at or below 60 % of the LOC when it is not monitored continuously (check the edition in force).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas evolved into the headspace (lag)</t>
+        </is>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n_flamm_src</t>
+        </is>
+      </c>
+      <c r="C83" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D83" s="48">
+        <f>rH2_gen+O2_net_gen</f>
+        <v>0.0001531217041947</v>
+      </c>
+      <c r="E83" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag phase: no uptake, so all electrolytic H₂ and net O₂ reach the headspace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace H₂ fraction (lag, mean-field)</t>
+        </is>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_H2_hs_lag</t>
+        </is>
+      </c>
+      <c r="C84" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D84" s="48">
+        <f>rH2_gen/(n_flamm_src+CO2_supply_b)</f>
+        <v>0.191315446335</v>
+      </c>
+      <c r="E84" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outflow-only mean-field balance: H₂ over all gas entering the headspace. Air ingress through the vent would lower H₂ and raise O₂.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ fraction (lag, mean-field)</t>
+        </is>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_hs_lag</t>
+        </is>
+      </c>
+      <c r="C85" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D85" s="48">
+        <f>O2_net_gen/(n_flamm_src+CO2_supply_b)</f>
+        <v>0.0910148751</v>
+      </c>
+      <c r="E85" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above, for O₂.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ duty that makes the lag headspace non-flammable</t>
+        </is>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">duty_H2safe</t>
+        </is>
+      </c>
+      <c r="C86" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D86" s="48">
+        <f>MAX(0,MIN(rH2_gen/H2_LFL-n_flamm_src,O2_net_gen/(O2_LOC_H2*LOC_margin)-n_flamm_src))/CO2_rate_full_b</f>
+        <v>0.002916316798</v>
+      </c>
+      <c r="E86" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Least valve-open fraction that brings H₂ below the LFL or O₂ below the LOC margin, whichever needs less CO₂.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval that makes the lag headspace non-flammable</t>
+        </is>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_H2safe</t>
+        </is>
+      </c>
+      <c r="C87" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D87" s="48">
+        <f>IF(duty_H2safe&gt;0,spg_dur_b/(60*duty_H2safe),NA())</f>
+        <v>4.483469527972</v>
+      </c>
+      <c r="E87" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field; the pulse-to-pulse sawtooth peaks need roughly half this interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ sweep that keeps lag H₂ below the LFL</t>
+        </is>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N2_sweep_H2safe</t>
+        </is>
+      </c>
+      <c r="C88" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D88" s="48">
+        <f>MAX(0,rH2_gen/H2_LFL-n_flamm_src)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
+        <v>0.995282852087</v>
+      </c>
+      <c r="E88" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Continuous inert headspace sweep that dilutes H₂ below the LFL with no CO₂ at all.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -19902,8 +20566,8 @@
         <v>102</v>
       </c>
       <c r="D108" s="24">
-        <f>(DO_hs_floor+DO_surf_excess)*32</f>
-        <v>2.639031652174</v>
+        <f>(DO_hs_floor+DO_surf_excess)*M_O2</f>
+        <v>2.638866712696</v>
       </c>
       <c r="E108" s="20" t="s">
         <v>1929</v>
@@ -19983,11 +20647,13 @@
       </c>
       <c r="C113" s="20"/>
       <c r="D113" s="24" t="str">
-        <f>IF(AND(ISNUMBER(DO_ss),ISNUMBER(DO_impair)),IF(DO_ss&lt;DO_impair,"Surface stripping holds DO under impairment - sparge is CARBON-limited (long interval); the O2-limited interval is the conservative fallback until kL_surf is measured","Surface stripping insufficient - sparge must vent O2 - use the O2-limited interval"),"organism DO unknown")</f>
-        <v>organism DO unknown</v>
-      </c>
-      <c r="E113" s="82" t="s">
-        <v>795</v>
+        <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) DO would be "&amp;TEXT(DO_at_carbon*M_O2,"0.0")&amp;" mg/L against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")</f>
+        <v>Do NOT relax: at the carbon-limited interval (185 min) DO would be 12.9 mg/L against a 2.6 mg/L target</v>
+      </c>
+      <c r="E113" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tests the carbon-limited interval against the same DO balance the schedule uses (D232). Replaces a test of DO_ss against the impairment level, which was circular (DO_ss sits at the target by construction) and invited an unsafe 185 min interval.</t>
+        </is>
       </c>
       <c r="F113" s="20"/>
     </row>
@@ -21185,7 +21851,7 @@
         <v>962</v>
       </c>
       <c r="D185" s="22">
-        <f>IF(ISNUMBER(duty_DO),spg_dur_opt/(60*duty_DO),NA())</f>
+        <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_opt/(60*duty_DO),spg_int_carbon),NA())</f>
         <v>16.46036421628</v>
       </c>
       <c r="E185" s="67" t="s">
@@ -21503,6 +22169,64 @@
       </c>
       <c r="E206" s="99" t="s">
         <v>1922</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CARBON-LIMITED INTERVAL: IS IT SAFE?</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ molar mass</t>
+        </is>
+      </c>
+      <c r="B231" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M_O2</t>
+        </is>
+      </c>
+      <c r="C231" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g/mol</t>
+        </is>
+      </c>
+      <c r="D231" s="52">
+        <v>31.998</v>
+      </c>
+      <c r="E231" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IUPAC standard atomic weights: 2 × 15.999.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO if the interval relaxed to the carbon-limited one</t>
+        </is>
+      </c>
+      <c r="B232" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_at_carbon</t>
+        </is>
+      </c>
+      <c r="C232" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D232" s="22">
+        <f>H_O2_T*P_atm*O2_excess/(O2_excess+CO2_rate_full*duty_carbon)+DO_surf_excess</f>
+        <v>0.401951360368</v>
+      </c>
+      <c r="E232" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same headspace back-pressure + surface-excess balance as D188/D180, evaluated at the carbon-limited duty instead of the DO-limited one.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gas model: house-rule hygiene (stale notes, named constants); values verified identical in Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -602,6 +602,42 @@
     <definedName name="duty_H2safe" localSheetId="4">Biology!$D$86</definedName>
     <definedName name="spg_int_H2safe" localSheetId="4">Biology!$D$87</definedName>
     <definedName name="N2_sweep_H2safe" localSheetId="4">Biology!$D$88</definedName>
+    <definedName name="knall_H2_default" localSheetId="4">Biology!$D$63</definedName>
+    <definedName name="knall_O2_default" localSheetId="4">Biology!$D$64</definedName>
+    <definedName name="knall_CO2_default" localSheetId="4">Biology!$D$65</definedName>
+    <definedName name="T_zero_C" localSheetId="4">Biology!$D$66</definedName>
+    <definedName name="P_atm_set" localSheetId="4">Biology!$D$67</definedName>
+    <definedName name="gerrit_slope_default" localSheetId="2">Electrochemistry!$D$125</definedName>
+    <definedName name="gerrit_int_default" localSheetId="2">Electrochemistry!$D$126</definedName>
+    <definedName name="V_headroom_min" localSheetId="2">Electrochemistry!$D$127</definedName>
+    <definedName name="T_ref" localSheetId="3">Chemistry!$D$229</definedName>
+    <definedName name="DH_const" localSheetId="3">Chemistry!$D$230</definedName>
+    <definedName name="eps_water_298" localSheetId="3">Chemistry!$D$231</definedName>
+    <definedName name="eps_T_exp" localSheetId="3">Chemistry!$D$232</definedName>
+    <definedName name="davies_c" localSheetId="3">Chemistry!$D$233</definedName>
+    <definedName name="Cl_floor_molL" localSheetId="3">Chemistry!$D$234</definedName>
+    <definedName name="pH_step" localSheetId="3">Chemistry!$D$235</definedName>
+    <definedName name="pH_band_lo" localSheetId="3">Chemistry!$D$236</definedName>
+    <definedName name="pH_band_hi" localSheetId="3">Chemistry!$D$237</definedName>
+    <definedName name="buffer_caution_frac" localSheetId="3">Chemistry!$D$238</definedName>
+    <definedName name="T_ref" localSheetId="5">'Mass Transfer'!$D$209</definedName>
+    <definedName name="T_zero_C" localSheetId="5">'Mass Transfer'!$D$210</definedName>
+    <definedName name="d_bubble_min_m" localSheetId="5">'Mass Transfer'!$D$211</definedName>
+    <definedName name="We_static_max" localSheetId="5">'Mass Transfer'!$D$212</definedName>
+    <definedName name="cleared_min" localSheetId="5">'Mass Transfer'!$D$213</definedName>
+    <definedName name="od_gap_min_s" localSheetId="5">'Mass Transfer'!$D$214</definedName>
+    <definedName name="tip_speed_max" localSheetId="5">'Mass Transfer'!$D$216</definedName>
+    <definedName name="geom_tol_mL" localSheetId="1">Geometry!$D$96</definedName>
+    <definedName name="round_split" localSheetId="0">Summary!$D$93</definedName>
+    <definedName name="bp_const" localSheetId="7">Calibrations!$D$140</definedName>
+    <definedName name="por_break_1" localSheetId="7">Calibrations!$D$141</definedName>
+    <definedName name="por_break_2" localSheetId="7">Calibrations!$D$142</definedName>
+    <definedName name="por_break_3" localSheetId="7">Calibrations!$D$143</definedName>
+    <definedName name="por_break_4" localSheetId="7">Calibrations!$D$144</definedName>
+    <definedName name="por_break_5" localSheetId="7">Calibrations!$D$145</definedName>
+    <definedName name="z_e_H2" localSheetId="7">Calibrations!$D$146</definedName>
+    <definedName name="z_e_O2" localSheetId="7">Calibrations!$D$147</definedName>
+    <definedName name="T_zero_C" localSheetId="7">Calibrations!$D$148</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -7890,8 +7926,10 @@
       <c r="E3" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="21" t="s">
-        <v>36</v>
+      <c r="F3" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anode material and sparger. Choose from the list (Electrochemistry A35:A38). Dropdown.</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -8089,7 +8127,7 @@
         <v>13</v>
       </c>
       <c r="D14" s="91">
-        <f>IF(AND(ISNUMBER($G$13),$G$13&gt;0),$G$13,IF(NOT(ISNUMBER(D13)),D13,IF(D13&gt;0.5,ROUND(D13,0),ROUND(D13,1-(1+INT(LOG10(ABS(D13))))))))</f>
+        <f>IF(AND(ISNUMBER($G$13),$G$13&gt;0),$G$13,IF(NOT(ISNUMBER(D13)),D13,IF(D13&gt;round_split,ROUND(D13,0),ROUND(D13,1-(1+INT(LOG10(ABS(D13))))))))</f>
         <v>1.0</v>
       </c>
       <c r="E14" s="20"/>
@@ -8111,8 +8149,10 @@
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F15" s="21" t="s">
-        <v>68</v>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time between doses: the shorter of the carbon-limited interval and the headspace-O₂-dilution interval (binding constraint on Mass Transfer D94). Credits surface O₂ stripping via the kL_surf estimate; measuring kL_surf refines it.</t>
+        </is>
       </c>
       <c r="G15" s="36"/>
     </row>
@@ -8125,7 +8165,7 @@
         <v>67</v>
       </c>
       <c r="D16" s="91">
-        <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,IF(D15&gt;0.5,ROUND(D15,0),ROUND(D15,1-(1+INT(LOG10(ABS(D15))))))))</f>
+        <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,IF(D15&gt;round_split,ROUND(D15,0),ROUND(D15,1-(1+INT(LOG10(ABS(D15))))))))</f>
         <v>16.0</v>
       </c>
       <c r="E16" s="92"/>
@@ -8453,8 +8493,10 @@
       </c>
     </row>
     <row r="35" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="89" t="s">
-        <v>988</v>
+      <c r="A35" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-average pH (activity scale, as a probe reads)</t>
+        </is>
       </c>
       <c r="C35" s="20"/>
       <c r="D35" s="121">
@@ -8462,11 +8504,13 @@
         <v>6.603949596052</v>
       </c>
       <c r="E35" s="23" t="str">
-        <f>HYPERLINK("#Chemistry!D103","→ Chemistry")</f>
+        <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F35" s="21" t="s">
-        <v>1881</v>
+      <c r="F35" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH at the cycle-average dissolved CO₂ of the schedule in use, on the activity scale a probe reads; the trough just after a pulse is lower. Green 6.5–7.5; red outside 6–8.</t>
+        </is>
       </c>
     </row>
     <row r="36" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -8521,8 +8565,10 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A39" s="89" t="s">
-        <v>104</v>
+      <c r="A39" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carbon-limited sparge interval</t>
+        </is>
       </c>
       <c r="B39" s="102"/>
       <c r="C39" s="20" t="s">
@@ -8536,8 +8582,10 @@
         <f>HYPERLINK("#'Mass Transfer'!D112","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F39" s="21" t="s">
-        <v>105</v>
+      <c r="F39" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval set by CO₂ supply alone. The schedule uses it only when it is shorter than the O₂-dilution interval.</t>
+        </is>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -8881,8 +8929,10 @@
         <v>surface-kla.md →</v>
       </c>
       <c r="E66" s="103"/>
-      <c r="F66" s="21" t="s">
-        <v>1901</v>
+      <c r="F66" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sets how far dissolved O₂ must sit above the headspace to shed the surplus, and the feasibility margin behind the whole DO strategy (kLa in use ÷ kLa required). It moves the answer continuously.</t>
+        </is>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
@@ -8919,8 +8969,10 @@
         <v>faradaic-efficiency.md →</v>
       </c>
       <c r="E68" s="103"/>
-      <c r="F68" s="21" t="s">
-        <v>1902</v>
+      <c r="F68" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated from the cathodic O₂ flux, but the calculation rests on an estimated electrode mass-transfer coefficient. Measuring it settles the H₂/O₂ split and the peroxide source at once.</t>
+        </is>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
@@ -9153,8 +9205,10 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A81" s="5" t="s">
-        <v>1865</v>
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELECTROCHEMISTRY – CALCULATED (hand these to an electrochemist)</t>
+        </is>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
@@ -9172,8 +9226,10 @@
         <f>HYPERLINK("#Electrochemistry!D88","→ Electrochemistry")</f>
         <v>→ Electrochemistry</v>
       </c>
-      <c r="F82" t="s">
-        <v>1866</v>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fraction of cathode current making H₂ rather than reducing dissolved O₂.</t>
+        </is>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
@@ -9332,6 +9388,38 @@
       </c>
       <c r="F90" t="s">
         <v>1876</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DISPLAY SETTINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rounding split</t>
+        </is>
+      </c>
+      <c r="B93" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">round_split</t>
+        </is>
+      </c>
+      <c r="C93" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s or min</t>
+        </is>
+      </c>
+      <c r="D93" s="36">
+        <v>0.5</v>
+      </c>
+      <c r="E93" s="87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined display rule for rows 14 and 16: whole units above this value, else two significant figures.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -11188,20 +11276,24 @@
       </c>
       <c r="C90" s="20"/>
       <c r="D90" s="24" t="str">
-        <f>IF(ABS(A_x*D_int/1000-V_vial_total)&lt;=3,"OK",IF(AND(ISNUMBER(cal_hs),ISNUMBER(cal_hs_fill)),"HEADSPACE MEASURED - bore depth still inconsistent (measure body volume)","VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth"))</f>
+        <f>IF(ABS(A_x*D_int/1000-V_vial_total)&lt;=geom_tol_mL,"OK",IF(AND(ISNUMBER(cal_hs),ISNUMBER(cal_hs_fill)),"HEADSPACE MEASURED - bore depth still inconsistent (measure body volume)","VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth"))</f>
         <v>VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth</v>
       </c>
       <c r="E90" s="20"/>
-      <c r="F90" s="101" t="s">
-        <v>305</v>
+      <c r="F90" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fires INCONSISTENT for the 20 mL vial because the bare cylinder (A_x x usable depth ~28 mL) overestimates the true 20 mL vial (it tapers/necks, not a full cylinder to 55 mm). Expected tolerance artefact, not a data error - resolved by measuring true bore depth (protocols/vial-geometry.md).</t>
+        </is>
       </c>
       <c r="G90" s="20"/>
       <c r="H90" s="20"/>
       <c r="I90" s="20"/>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A91" s="5" t="s">
-        <v>1465</v>
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ELECTRODE GEOMETRY FOR THE OHMIC DROP</t>
+        </is>
       </c>
     </row>
     <row r="92" spans="1:9" ht="36" x14ac:dyDescent="0.2">
@@ -11237,6 +11329,38 @@
       </c>
       <c r="E93" s="99" t="s">
         <v>1471</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONSISTENCY-CHECK TOLERANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vial volume consistency tolerance</t>
+        </is>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">geom_tol_mL</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D96" s="36">
+        <v>3</v>
+      </c>
+      <c r="E96" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: allowed gap between the bare-cylinder volume (A_x × D_int) and the total vial volume.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -11459,7 +11583,7 @@
         <v>321</v>
       </c>
       <c r="D11" s="22">
-        <f>IF(ISNUMBER(cal_gerrit_slope),cal_gerrit_slope,1.03)</f>
+        <f>IF(ISNUMBER(cal_gerrit_slope),cal_gerrit_slope,gerrit_slope_default)</f>
         <v>1.03</v>
       </c>
       <c r="E11" s="109" t="s">
@@ -11481,7 +11605,7 @@
         <v>325</v>
       </c>
       <c r="D12" s="22">
-        <f>IF(ISNUMBER(cal_gerrit_int),cal_gerrit_int,2.6)</f>
+        <f>IF(ISNUMBER(cal_gerrit_int),cal_gerrit_int,gerrit_int_default)</f>
         <v>2.6</v>
       </c>
       <c r="E12" s="109" t="s">
@@ -11611,8 +11735,10 @@
         <f>IF(ISNUMBER(cal_etaF),cal_etaF,etaF_calc)</f>
         <v>0.977475298652</v>
       </c>
-      <c r="E18" s="67" t="s">
-        <v>1754</v>
+      <c r="E18" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cathodic H₂ faradaic efficiency: a measured value from the Calibrations tab if there is one, otherwise CALCULATED (D88, etaF_calc) from the cathodic O₂ reduction competing for the current. Neutral-pH HER on stainless peaks near 97% before that competition is counted, so the calculated value remains an upper bound.</t>
+        </is>
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20"/>
@@ -11787,8 +11913,10 @@
         <f>IF(ISNUMBER(cal_etaF_OER),cal_etaF_OER,etaF_OER_calc)</f>
         <v>0.975081911036</v>
       </c>
-      <c r="E26" s="67" t="s">
-        <v>1755</v>
+      <c r="E26" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anodic O₂ faradaic efficiency: measured if available, otherwise CALCULATED (etaF_OER_calc) as 1 − the chlorine share − the metal-dissolution share. UdG contains chloride, so the chlorine current is modelled explicitly (D101).</t>
+        </is>
       </c>
       <c r="F26" s="20"/>
       <c r="G26" s="20"/>
@@ -12247,8 +12375,10 @@
         <f>Geometry!$D$93</f>
         <v>9.18130412738</v>
       </c>
-      <c r="E45" s="99" t="s">
-        <v>1472</v>
+      <c r="E45" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Submerged length at the achieved liquid level (Geometry D93), not the bare datum (Geometry D35), which would overstate the wetted area by about 6.5% and understate every current density by the same factor.</t>
+        </is>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
@@ -12772,8 +12902,10 @@
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A78" s="5" t="s">
-        <v>1625</v>
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CALCULATED FARADAIC SPLIT – the cathode competes with dissolved O₂</t>
+        </is>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -12950,8 +13082,10 @@
         <f>MAX(0,1-i_ORR_design/I_app)</f>
         <v>0.977475298652</v>
       </c>
-      <c r="E88" s="67" t="s">
-        <v>1654</v>
+      <c r="E88" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 − (cathodic O₂ current)/(applied current). Neutral-pH HER on stainless also has its own kinetic losses; this accounts only for the O₂ that competes for the current.</t>
+        </is>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
@@ -13025,8 +13159,10 @@
         <f>f_HOOH*i_ORR_design/(2*F_const)*M_H2O2*1000*3600/ec_V_L</f>
         <v>0.813296984002</v>
       </c>
-      <c r="E93" s="67" t="s">
-        <v>1667</v>
+      <c r="E93" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 electrons per H₂O₂. This source runs whenever there is current and dissolved O₂.</t>
+        </is>
       </c>
     </row>
     <row r="94" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -13208,8 +13344,10 @@
         <f>MAX(0,1-f_Cl_anode-IF(ISNUMBER(ec_corr_I),ec_corr_I,0))</f>
         <v>0.975081911036</v>
       </c>
-      <c r="E104" s="67" t="s">
-        <v>1698</v>
+      <c r="E104" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 − chlorine share − metal-dissolution share. It remains an UPPER BOUND while the metal-dissolution charge is unmeasured: a corroding anode takes current that this cell still credits to oxygen.</t>
+        </is>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
@@ -13509,11 +13647,93 @@
         <v>1274</v>
       </c>
       <c r="D122" s="22" t="str">
-        <f>IF(V_headroom&lt;0,"OVER RAIL — the drive cannot deliver this current; the linear current law will not hold",IF(V_headroom&lt;1,"watch — within 1 V of the rail ("&amp;TEXT(V_cell_est,"0.00")&amp;" V of "&amp;TEXT(V_rail,"0")&amp;" V); expect the current law to bend","OK — "&amp;TEXT(V_cell_est,"0.00")&amp;" V estimated against a "&amp;TEXT(V_rail,"0")&amp;" V rail"))</f>
+        <f>IF(V_headroom&lt;0,"OVER RAIL — the drive cannot deliver this current; the linear current law will not hold",IF(V_headroom&lt;V_headroom_min,"watch — within "&amp;TEXT(V_headroom_min,"0")&amp;" V of the rail ("&amp;TEXT(V_cell_est,"0.00")&amp;" V of "&amp;TEXT(V_rail,"0")&amp;" V); expect the current law to bend","OK — "&amp;TEXT(V_cell_est,"0.00")&amp;" V estimated against a "&amp;TEXT(V_rail,"0")&amp;" V rail"))</f>
         <v>OK — 3.26 V estimated against a 5 V rail</v>
       </c>
       <c r="E122" s="67" t="s">
         <v>1753</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAMED DEFAULTS AND THRESHOLDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gerrit's Law slope (default)</t>
+        </is>
+      </c>
+      <c r="B125" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gerrit_slope_default</t>
+        </is>
+      </c>
+      <c r="C125" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mA/%</t>
+        </is>
+      </c>
+      <c r="D125" s="36">
+        <v>1.03</v>
+      </c>
+      <c r="E125" s="109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gerrit's Law fit, LED_D current calibration (protocols/gerrit-current.md); used when no Calibrations run is included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gerrit's Law intercept (default)</t>
+        </is>
+      </c>
+      <c r="B126" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gerrit_int_default</t>
+        </is>
+      </c>
+      <c r="C126" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mA</t>
+        </is>
+      </c>
+      <c r="D126" s="36">
+        <v>2.6</v>
+      </c>
+      <c r="E126" s="109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gerrit's Law fit, LED_D current calibration (protocols/gerrit-current.md); used when no Calibrations run is included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voltage headroom caution margin</t>
+        </is>
+      </c>
+      <c r="B127" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_headroom_min</t>
+        </is>
+      </c>
+      <c r="C127" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="D127" s="36">
+        <v>1</v>
+      </c>
+      <c r="E127" s="114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: the current law starts to bend within this margin of the drive rail.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -13612,8 +13832,10 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="36" x14ac:dyDescent="0.2">
-      <c r="A5" s="17" t="s">
-        <v>845</v>
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Dissolved CO₂ (cycle average)</t>
+        </is>
       </c>
       <c r="B5" s="18" t="s">
         <v>846</v>
@@ -13625,8 +13847,10 @@
         <f>'Mass Transfer'!$D$162</f>
         <v>0.008590210622</v>
       </c>
-      <c r="E5" s="51" t="s">
-        <v>1158</v>
+      <c r="E5" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Schedule-dependent cycle-average dissolved CO₂ (mass-conserving limit cycle, bounded by air equilibrium and pure-CO₂ saturation).</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -13697,8 +13921,10 @@
         <f>'Mass Transfer'!$D$101</f>
         <v>8.314462618</v>
       </c>
-      <c r="E9" s="84" t="s">
-        <v>1900</v>
+      <c r="E9" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Mass Transfer (R_gas).</t>
+        </is>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -13737,7 +13963,7 @@
         <v>9.15</v>
       </c>
       <c r="D13" s="64">
-        <f t="shared" ref="D13:D20" si="0">B13*EXP(-C13*1000/R_gas*(1/TKc-1/298.15))</f>
+        <f>B13*EXP(-C13*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>4.45e-07</v>
       </c>
       <c r="E13" s="84" t="s">
@@ -13755,7 +13981,7 @@
         <v>14.9</v>
       </c>
       <c r="D14" s="64">
-        <f t="shared" si="0"/>
+        <f>B14*EXP(-C14*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>4.69e-11</v>
       </c>
       <c r="E14" s="84" t="s">
@@ -13773,7 +13999,7 @@
         <v>-8</v>
       </c>
       <c r="D15" s="64">
-        <f t="shared" si="0"/>
+        <f>B15*EXP(-C15*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>0.0071</v>
       </c>
       <c r="E15" s="84" t="s">
@@ -13791,7 +14017,7 @@
         <v>3.6</v>
       </c>
       <c r="D16" s="64">
-        <f t="shared" si="0"/>
+        <f>B16*EXP(-C16*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>6.31e-08</v>
       </c>
       <c r="E16" s="84" t="s">
@@ -13809,7 +14035,7 @@
         <v>16</v>
       </c>
       <c r="D17" s="64">
-        <f t="shared" si="0"/>
+        <f>B17*EXP(-C17*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>4.2e-13</v>
       </c>
       <c r="E17" s="84" t="s">
@@ -13827,7 +14053,7 @@
         <v>52.2</v>
       </c>
       <c r="D18" s="64">
-        <f t="shared" si="0"/>
+        <f>B18*EXP(-C18*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>5.6e-10</v>
       </c>
       <c r="E18" s="84" t="s">
@@ -13845,7 +14071,7 @@
         <v>55.8</v>
       </c>
       <c r="D19" s="64">
-        <f t="shared" si="0"/>
+        <f>B19*EXP(-C19*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>1e-14</v>
       </c>
       <c r="E19" s="84" t="s">
@@ -13863,7 +14089,7 @@
         <v>13.8</v>
       </c>
       <c r="D20" s="64">
-        <f t="shared" si="0"/>
+        <f>B20*EXP(-C20*1000/R_gas*(1/TKc-1/T_ref))</f>
         <v>2.884031503127e-08</v>
       </c>
       <c r="E20" s="84" t="s">
@@ -14302,7 +14528,7 @@
         <v>0.033213926229</v>
       </c>
       <c r="C50" s="64">
-        <f t="shared" ref="C50:C81" si="2">IF(AND(B50&gt;=0,B51&lt;0),A50+0.1*B50/(B50-B51),0)</f>
+        <f>IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14315,7 +14541,7 @@
         <v>0.033095991179</v>
       </c>
       <c r="C51" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B51&gt;=0,B52&lt;0),A51+pH_step*B51/(B51-B52),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14328,7 +14554,7 @@
         <v>0.032986799309</v>
       </c>
       <c r="C52" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B52&gt;=0,B53&lt;0),A52+pH_step*B52/(B52-B53),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14341,7 +14567,7 @@
         <v>0.032880652062</v>
       </c>
       <c r="C53" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B53&gt;=0,B54&lt;0),A53+pH_step*B53/(B53-B54),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14354,7 +14580,7 @@
         <v>0.032771986272</v>
       </c>
       <c r="C54" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B54&gt;=0,B55&lt;0),A54+pH_step*B54/(B54-B55),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14367,7 +14593,7 @@
         <v>0.032655096798</v>
       </c>
       <c r="C55" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B55&gt;=0,B56&lt;0),A55+pH_step*B55/(B55-B56),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14380,7 +14606,7 @@
         <v>0.032523849984</v>
       </c>
       <c r="C56" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B56&gt;=0,B57&lt;0),A56+pH_step*B56/(B56-B57),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14393,7 +14619,7 @@
         <v>0.032371376227</v>
       </c>
       <c r="C57" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B57&gt;=0,B58&lt;0),A57+pH_step*B57/(B57-B58),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14406,7 +14632,7 @@
         <v>0.032189729231</v>
       </c>
       <c r="C58" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B58&gt;=0,B59&lt;0),A58+pH_step*B58/(B58-B59),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14419,7 +14645,7 @@
         <v>0.031969498815</v>
       </c>
       <c r="C59" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B59&gt;=0,B60&lt;0),A59+pH_step*B59/(B59-B60),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14432,7 +14658,7 @@
         <v>0.031699363744</v>
       </c>
       <c r="C60" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B60&gt;=0,B61&lt;0),A60+pH_step*B60/(B60-B61),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14445,7 +14671,7 @@
         <v>0.031365571066</v>
       </c>
       <c r="C61" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B61&gt;=0,B62&lt;0),A61+pH_step*B61/(B61-B62),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14458,7 +14684,7 @@
         <v>0.030951329376</v>
       </c>
       <c r="C62" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B62&gt;=0,B63&lt;0),A62+pH_step*B62/(B62-B63),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14471,7 +14697,7 @@
         <v>0.030436105853</v>
       </c>
       <c r="C63" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B63&gt;=0,B64&lt;0),A63+pH_step*B63/(B63-B64),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14484,7 +14710,7 @@
         <v>0.029794821411</v>
       </c>
       <c r="C64" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B64&gt;=0,B65&lt;0),A64+pH_step*B64/(B64-B65),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14497,7 +14723,7 @@
         <v>0.028996945562</v>
       </c>
       <c r="C65" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B65&gt;=0,B66&lt;0),A65+pH_step*B65/(B65-B66),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14510,7 +14736,7 @@
         <v>0.028005502639</v>
       </c>
       <c r="C66" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B66&gt;=0,B67&lt;0),A66+pH_step*B66/(B66-B67),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14523,7 +14749,7 @@
         <v>0.026776012764</v>
       </c>
       <c r="C67" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B67&gt;=0,B68&lt;0),A67+pH_step*B67/(B67-B68),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14536,7 +14762,7 @@
         <v>0.025255400836</v>
       </c>
       <c r="C68" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B68&gt;=0,B69&lt;0),A68+pH_step*B68/(B68-B69),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14549,7 +14775,7 @@
         <v>0.02338090709</v>
       </c>
       <c r="C69" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B69&gt;=0,B70&lt;0),A69+pH_step*B69/(B69-B70),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14562,7 +14788,7 @@
         <v>0.021079010121</v>
       </c>
       <c r="C70" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B70&gt;=0,B71&lt;0),A70+pH_step*B70/(B70-B71),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14575,7 +14801,7 @@
         <v>0.01826430841</v>
       </c>
       <c r="C71" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B71&gt;=0,B72&lt;0),A71+pH_step*B71/(B71-B72),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14588,7 +14814,7 @@
         <v>0.014838178095</v>
       </c>
       <c r="C72" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B72&gt;=0,B73&lt;0),A72+pH_step*B72/(B72-B73),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14601,7 +14827,7 @@
         <v>0.010686819787</v>
       </c>
       <c r="C73" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B73&gt;=0,B74&lt;0),A73+pH_step*B73/(B73-B74),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14614,7 +14840,7 @@
         <v>0.005678038225</v>
       </c>
       <c r="C74" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B74&gt;=0,B75&lt;0),A74+pH_step*B74/(B74-B75),0)</f>
         <v>6.494284837612</v>
       </c>
     </row>
@@ -14627,7 +14853,7 @@
         <v>-0.0003441795237407</v>
       </c>
       <c r="C75" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B75&gt;=0,B76&lt;0),A75+pH_step*B75/(B75-B76),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14640,7 +14866,7 @@
         <v>-0.00756840932</v>
       </c>
       <c r="C76" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B76&gt;=0,B77&lt;0),A76+pH_step*B76/(B76-B77),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14653,7 +14879,7 @@
         <v>-0.016228970854</v>
       </c>
       <c r="C77" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B77&gt;=0,B78&lt;0),A77+pH_step*B77/(B77-B78),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14666,7 +14892,7 @@
         <v>-0.02662440719</v>
       </c>
       <c r="C78" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B78&gt;=0,B79&lt;0),A78+pH_step*B78/(B78-B79),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14679,7 +14905,7 @@
         <v>-0.039141735033</v>
       </c>
       <c r="C79" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B79&gt;=0,B80&lt;0),A79+pH_step*B79/(B79-B80),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14692,7 +14918,7 @@
         <v>-0.054286645726</v>
       </c>
       <c r="C80" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B80&gt;=0,B81&lt;0),A80+pH_step*B80/(B80-B81),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14705,7 +14931,7 @@
         <v>-0.072719923595</v>
       </c>
       <c r="C81" s="64">
-        <f t="shared" si="2"/>
+        <f>IF(AND(B81&gt;=0,B82&lt;0),A81+pH_step*B81/(B81-B82),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14718,7 +14944,7 @@
         <v>-0.095300976728</v>
       </c>
       <c r="C82" s="64">
-        <f t="shared" ref="C82:C99" si="4">IF(AND(B82&gt;=0,B83&lt;0),A82+0.1*B82/(B82-B83),0)</f>
+        <f>IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14731,7 +14957,7 @@
         <v>-0.123140508482</v>
       </c>
       <c r="C83" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B83&gt;=0,B84&lt;0),A83+pH_step*B83/(B83-B84),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14744,7 +14970,7 @@
         <v>-0.157665823938</v>
       </c>
       <c r="C84" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B84&gt;=0,B85&lt;0),A84+pH_step*B84/(B84-B85),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14757,7 +14983,7 @@
         <v>-0.200703923131</v>
       </c>
       <c r="C85" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B85&gt;=0,B86&lt;0),A85+pH_step*B85/(B85-B86),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14770,7 +14996,7 @@
         <v>-0.2545894166</v>
       </c>
       <c r="C86" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B86&gt;=0,B87&lt;0),A86+pH_step*B86/(B86-B87),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14783,7 +15009,7 @@
         <v>-0.322306667774</v>
       </c>
       <c r="C87" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B87&gt;=0,B88&lt;0),A87+pH_step*B87/(B87-B88),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14796,7 +15022,7 @@
         <v>-0.407678885978</v>
       </c>
       <c r="C88" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B88&gt;=0,B89&lt;0),A88+pH_step*B88/(B88-B89),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14809,7 +15035,7 @@
         <v>-0.515621824235</v>
       </c>
       <c r="C89" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B89&gt;=0,B90&lt;0),A89+pH_step*B89/(B89-B90),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14822,7 +15048,7 @@
         <v>-0.65248719742</v>
       </c>
       <c r="C90" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B90&gt;=0,B91&lt;0),A90+pH_step*B90/(B90-B91),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14835,7 +15061,7 @@
         <v>-0.826532271905</v>
       </c>
       <c r="C91" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B91&gt;=0,B92&lt;0),A91+pH_step*B91/(B91-B92),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14848,7 +15074,7 @@
         <v>-1.048569336646</v>
       </c>
       <c r="C92" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B92&gt;=0,B93&lt;0),A92+pH_step*B92/(B92-B93),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14861,7 +15087,7 @@
         <v>-1.332875144027</v>
       </c>
       <c r="C93" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B93&gt;=0,B94&lt;0),A93+pH_step*B93/(B93-B94),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14874,7 +15100,7 @@
         <v>-1.698480927379</v>
       </c>
       <c r="C94" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B94&gt;=0,B95&lt;0),A94+pH_step*B94/(B94-B95),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14887,7 +15113,7 @@
         <v>-2.171026165161</v>
       </c>
       <c r="C95" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B95&gt;=0,B96&lt;0),A95+pH_step*B95/(B95-B96),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14900,7 +15126,7 @@
         <v>-2.785456321043</v>
       </c>
       <c r="C96" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B96&gt;=0,B97&lt;0),A96+pH_step*B96/(B96-B97),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14913,7 +15139,7 @@
         <v>-3.589995975505</v>
       </c>
       <c r="C97" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B97&gt;=0,B98&lt;0),A97+pH_step*B97/(B97-B98),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14926,7 +15152,7 @@
         <v>-4.652065051273</v>
       </c>
       <c r="C98" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B98&gt;=0,B99&lt;0),A98+pH_step*B98/(B98-B99),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14939,7 +15165,7 @@
         <v>-6.067176130696</v>
       </c>
       <c r="C99" s="64">
-        <f t="shared" si="4"/>
+        <f>IF(AND(B99&gt;=0,B100&lt;0),A99+pH_step*B99/(B99-B100),0)</f>
         <v>0.0</v>
       </c>
     </row>
@@ -14978,8 +15204,10 @@
       </c>
     </row>
     <row r="103" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A103" s="17" t="s">
-        <v>950</v>
+      <c r="A103" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPERATING pH (buffered, cycle average)</t>
+        </is>
       </c>
       <c r="B103" s="18" t="s">
         <v>951</v>
@@ -14994,8 +15222,10 @@
       <c r="E103" s="51" t="s">
         <v>1878</v>
       </c>
-      <c r="F103" s="101" t="s">
-        <v>953</v>
+      <c r="F103" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH at the cycle-average dissolved CO₂ of the schedule in use. The trough just after a CO₂ pulse is lower; a probe with response lag reads near this value, not the trough.</t>
+        </is>
       </c>
     </row>
     <row r="104" spans="1:7" ht="36" x14ac:dyDescent="0.2">
@@ -15057,8 +15287,10 @@
         <f>Iappc/(2*Fcc)*M_HOCl*3600/VLc</f>
         <v>371.244905447914</v>
       </c>
-      <c r="E107" s="51" t="s">
-        <v>1459</v>
+      <c r="E107" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Naïve FE=1 upper bound (all anode current → Cl₂). Superseded by the mass-transport-limited chlorine current I_Cl (D133) and the production rate P_HOCl (D134). Kept only to show the overstatement (~40× at the current operating point).</t>
+        </is>
       </c>
       <c r="G107" s="69" t="s">
         <v>1009</v>
@@ -15117,7 +15349,7 @@
         <v>969</v>
       </c>
       <c r="D110" s="64" t="str">
-        <f>IF(pH_meas&lt;6.5,"pH BELOW HOB optimum (&lt;6.5) — reduce the CO₂ dose or lengthen the interval",IF(pH_meas&gt;7.5,"pH above optimum (&gt;7.5)","pH in HOB band 6.5–7.5"))</f>
+        <f>IF(pH_meas&lt;pH_band_lo,"pH BELOW HOB optimum (&lt;"&amp;TEXT(pH_band_lo,"0.0")&amp;") — reduce the CO₂ dose or lengthen the interval",IF(pH_meas&gt;pH_band_hi,"pH above optimum (&gt;"&amp;TEXT(pH_band_hi,"0.0")&amp;")","pH in HOB band "&amp;TEXT(pH_band_lo,"0.0")&amp;"–"&amp;TEXT(pH_band_hi,"0.0")))</f>
         <v>pH in HOB band 6.5–7.5</v>
       </c>
       <c r="E110" s="51" t="s">
@@ -15295,8 +15527,10 @@
         <f>Fcc*km_Cl*(pH_Cl/1000)*A_anode</f>
         <v>0.0001417839262056</v>
       </c>
-      <c r="E132" s="51" t="s">
-        <v>1462</v>
+      <c r="E132" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">i_lim = n·F·k_m·[Cl⁻]·A, n = 1 per ARRIVING chloride; [Cl⁻] in mol/cm³ = pH_Cl/1000. Caps chlorine at the chloride flux; it binds at trace Cl⁻ such as UdG, so production scales with chloride.</t>
+        </is>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
@@ -16097,7 +16331,7 @@
         <v>1507</v>
       </c>
       <c r="D180" s="22">
-        <f>IF(Summary!$D$5="MC02",kappa0_mc02,IF(Summary!$D$5="UdG phosphate",kappa0_udg,NA()))*kappa_fI*(1+kappa_TC*(TKc-298.15))</f>
+        <f>IF(Summary!$D$5="MC02",kappa0_mc02,IF(Summary!$D$5="UdG phosphate",kappa0_udg,NA()))*kappa_fI*(1+kappa_TC*(TKc-T_ref))</f>
         <v>0.706946657056</v>
       </c>
       <c r="E180" s="67" t="s">
@@ -16174,7 +16408,7 @@
         <v>1274</v>
       </c>
       <c r="D186" s="22">
-        <f>1820000*(78.54*(298.15/TKc)^1.368)^-1.5*TKc^-1.5</f>
+        <f>DH_const*(eps_water_298*(T_ref/TKc)^eps_T_exp)^-1.5*TKc^-1.5</f>
         <v>0.507905390447</v>
       </c>
       <c r="E186" s="67" t="s">
@@ -16192,7 +16426,7 @@
         <v>1274</v>
       </c>
       <c r="D187" s="22">
-        <f>10^(-A_DH*1*(SQRT(I_ionic)/(1+SQRT(I_ionic))-0.3*I_ionic))</f>
+        <f>10^(-A_DH*1*(SQRT(I_ionic)/(1+SQRT(I_ionic))-davies_c*I_ionic))</f>
         <v>0.776846550354</v>
       </c>
       <c r="E187" s="67" t="s">
@@ -16210,7 +16444,7 @@
         <v>1274</v>
       </c>
       <c r="D188" s="22">
-        <f>10^(-A_DH*4*(SQRT(I_ionic)/(1+SQRT(I_ionic))-0.3*I_ionic))</f>
+        <f>10^(-A_DH*4*(SQRT(I_ionic)/(1+SQRT(I_ionic))-davies_c*I_ionic))</f>
         <v>0.364200859384</v>
       </c>
       <c r="E188" s="67" t="s">
@@ -16228,7 +16462,7 @@
         <v>1274</v>
       </c>
       <c r="D189" s="22">
-        <f>10^(-A_DH*9*(SQRT(I_ionic)/(1+SQRT(I_ionic))-0.3*I_ionic))</f>
+        <f>10^(-A_DH*9*(SQRT(I_ionic)/(1+SQRT(I_ionic))-davies_c*I_ionic))</f>
         <v>0.103042686755</v>
       </c>
       <c r="E189" s="67" t="s">
@@ -16536,7 +16770,7 @@
         <v>1571</v>
       </c>
       <c r="D208" s="22">
-        <f>E0_Cl2+nernst_slope*(-LOG10(MAX(pH_Cl,0.000000000001)))</f>
+        <f>E0_Cl2+nernst_slope*(-LOG10(MAX(pH_Cl,Cl_floor_molL)))</f>
         <v>1.579505308204</v>
       </c>
       <c r="E208" s="67" t="s">
@@ -16709,7 +16943,7 @@
         <v>1274</v>
       </c>
       <c r="D219" s="22" t="str">
-        <f>IF(j_buffer_ratio&gt;1,"BUFFER EXCEEDED — anode surface acidifies (local pH ~1 unit below bulk); the pH solved above is the bulk value only",IF(j_buffer_ratio&gt;0.5,"watch — running at "&amp;TEXT(j_buffer_ratio,"0%")&amp;" of the phosphate buffer limit; expect a 0.4–1.0 unit excursion at each electrode surface","OK — buffer holds the electrode surfaces at the bulk pH"))</f>
+        <f>IF(j_buffer_ratio&gt;1,"BUFFER EXCEEDED — anode surface acidifies (local pH ~1 unit below bulk); the pH solved above is the bulk value only",IF(j_buffer_ratio&gt;buffer_caution_frac,"watch — running at "&amp;TEXT(j_buffer_ratio,"0%")&amp;" of the phosphate buffer limit; expect a 0.4–1.0 unit excursion at each electrode surface","OK — buffer holds the electrode surfaces at the bulk pH"))</f>
         <v>OK — buffer holds the electrode surfaces at the bulk pH</v>
       </c>
       <c r="E219" s="67" t="s">
@@ -16735,8 +16969,10 @@
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A221" s="5" t="s">
-        <v>1882</v>
+      <c r="A221" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNIT CONSTANTS</t>
+        </is>
       </c>
     </row>
     <row r="222" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -16823,6 +17059,264 @@
       </c>
       <c r="E226" s="67" t="s">
         <v>1899</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAMED CONSTANTS, THRESHOLDS AND IMPORTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Reference temperature (25 °C)</t>
+        </is>
+      </c>
+      <c r="B229" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T_ref</t>
+        </is>
+      </c>
+      <c r="C229" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K</t>
+        </is>
+      </c>
+      <c r="D229" s="22">
+        <f>Biology!$D$23</f>
+        <v>298.15</v>
+      </c>
+      <c r="E229" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D23</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debye–Hückel A coefficient constant</t>
+        </is>
+      </c>
+      <c r="B230" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DH_const</t>
+        </is>
+      </c>
+      <c r="C230" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K^1.5</t>
+        </is>
+      </c>
+      <c r="D230" s="36">
+        <v>1820000</v>
+      </c>
+      <c r="E230" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A = 1.82×10⁶·(εT)^-1.5 (standard Debye–Hückel form; gives 0.509 at 25 °C).</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relative permittivity of water at 298.15 K</t>
+        </is>
+      </c>
+      <c r="B231" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eps_water_298</t>
+        </is>
+      </c>
+      <c r="C231" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D231" s="36">
+        <v>78.54</v>
+      </c>
+      <c r="E231" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRC Handbook, water dielectric constant at 25 °C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Permittivity temperature exponent</t>
+        </is>
+      </c>
+      <c r="B232" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eps_T_exp</t>
+        </is>
+      </c>
+      <c r="C232" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D232" s="36">
+        <v>1.368</v>
+      </c>
+      <c r="E232" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ε(T) = ε₂₉₈·(298.15/T)^n, power-law fit to the water permittivity (as in E186).</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Davies equation linear coefficient</t>
+        </is>
+      </c>
+      <c r="B233" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">davies_c</t>
+        </is>
+      </c>
+      <c r="C233" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D233" s="36">
+        <v>0.3</v>
+      </c>
+      <c r="E233" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Davies (1962): log γ = −A z²(√I/(1+√I) − 0.3 I).</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chloride numerical floor</t>
+        </is>
+      </c>
+      <c r="B234" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cl_floor_molL</t>
+        </is>
+      </c>
+      <c r="C234" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D234" s="36">
+        <v>1e-12</v>
+      </c>
+      <c r="E234" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined: numerical floor so LOG10 never sees zero chloride; far below any real chloride level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH solve grid step</t>
+        </is>
+      </c>
+      <c r="B235" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH_step</t>
+        </is>
+      </c>
+      <c r="C235" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D235" s="36">
+        <v>0.1</v>
+      </c>
+      <c r="E235" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined: spacing of the typed pH grid A50:A100 (4.0 to 9.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOB pH band, lower edge</t>
+        </is>
+      </c>
+      <c r="B236" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH_band_lo</t>
+        </is>
+      </c>
+      <c r="C236" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D236" s="36">
+        <v>6.5</v>
+      </c>
+      <c r="E236" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOB optimum 6.5–7.5 (Pous 2022/23; Rovira-Alsina 2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOB pH band, upper edge</t>
+        </is>
+      </c>
+      <c r="B237" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH_band_hi</t>
+        </is>
+      </c>
+      <c r="C237" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D237" s="36">
+        <v>7.5</v>
+      </c>
+      <c r="E237" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HOB optimum 6.5–7.5 (Pous 2022/23; Rovira-Alsina 2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Buffer caution fraction</t>
+        </is>
+      </c>
+      <c r="B238" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">buffer_caution_frac</t>
+        </is>
+      </c>
+      <c r="C238" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D238" s="36">
+        <v>0.5</v>
+      </c>
+      <c r="E238" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coarse estimate: flag "watch" above this fraction of the buffer-limited current density.</t>
+        </is>
       </c>
     </row>
     <row r="250">
@@ -17274,7 +17768,7 @@
         <v>135</v>
       </c>
       <c r="D10" s="105">
-        <f>IF(ISNUMBER(cal_knall_H2),cal_knall_H2,6)</f>
+        <f>IF(ISNUMBER(cal_knall_H2),cal_knall_H2,knall_H2_default)</f>
         <v>6.0</v>
       </c>
       <c r="E10" s="61" t="s">
@@ -17293,7 +17787,7 @@
         <v>135</v>
       </c>
       <c r="D11" s="105">
-        <f>IF(ISNUMBER(cal_knall_O2),cal_knall_O2,2)</f>
+        <f>IF(ISNUMBER(cal_knall_O2),cal_knall_O2,knall_O2_default)</f>
         <v>2.0</v>
       </c>
       <c r="E11" s="61" t="s">
@@ -17312,7 +17806,7 @@
         <v>135</v>
       </c>
       <c r="D12" s="105">
-        <f>IF(ISNUMBER(cal_knall_CO2),cal_knall_CO2,1)</f>
+        <f>IF(ISNUMBER(cal_knall_CO2),cal_knall_CO2,knall_CO2_default)</f>
         <v>1.0</v>
       </c>
       <c r="E12" s="61" t="s">
@@ -17426,7 +17920,7 @@
         <v>309</v>
       </c>
       <c r="D18" s="42">
-        <f>T_C+273.15</f>
+        <f>T_C+T_zero_C</f>
         <v>298.15</v>
       </c>
       <c r="E18" s="99" t="s">
@@ -17445,7 +17939,7 @@
         <v>62</v>
       </c>
       <c r="D19" s="63">
-        <f>IF(Summary!$D$10&gt;0,Summary!$D$10,101325)</f>
+        <f>IF(P_atm_set&gt;0,P_atm_set,Pa_per_atm)</f>
         <v>101325.0</v>
       </c>
       <c r="E19" s="37" t="s">
@@ -17919,8 +18413,10 @@
           <t xml:space="preserve">Tests the lag-phase headspace mix (rows 84–85) against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin. Replaces a dissolved-H₂ turnover proxy, which said nothing about flammability.</t>
         </is>
       </c>
-      <c r="F44" s="101" t="s">
-        <v>512</v>
+      <c r="F44" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hazard verdict (lag-phase headspace flammability), not a data gap.</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
@@ -18158,8 +18654,10 @@
       <c r="F58" s="20"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A59" s="5" t="s">
-        <v>1473</v>
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TARGET DISSOLVED-OXYGEN FRACTION (one definition, used by every guard)</t>
+        </is>
       </c>
     </row>
     <row r="60" spans="1:6" ht="24" x14ac:dyDescent="0.2">
@@ -18193,8 +18691,143 @@
       <c r="D61" s="52">
         <v>0.22608695652173899</v>
       </c>
-      <c r="E61" s="68" t="s">
-        <v>1928</v>
+      <c r="E61" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C. necator DO_opt 2.6 ÷ DO_toxic 11.5 mg/L (row 52), the only organism in the table with a measured band, used as the stand-in for the rest. Same optimum ÷ ceiling ratio the row above computes, so the fallback is consistent with the definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAMED DEFAULTS, CONSTANTS AND IMPORTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Default H₂ uptake ratio (no calibration)</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">knall_H2_default</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D63" s="36">
+        <v>6</v>
+      </c>
+      <c r="E63" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Used when no Calibrations knallgas run is included. 6:2:1 = mid-range central uptake ratio (Lu &amp; Yu 2019; feed optimum 7:2:1, Ishizaki 2001).</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Default O₂ uptake ratio (no calibration)</t>
+        </is>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">knall_O2_default</t>
+        </is>
+      </c>
+      <c r="C64" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D64" s="36">
+        <v>2</v>
+      </c>
+      <c r="E64" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above: O₂:H₂ uptake 0.29–0.35 (×6 → 1.75–2.1), 2 = central.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Default CO₂ uptake ratio (no calibration)</t>
+        </is>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">knall_CO2_default</t>
+        </is>
+      </c>
+      <c r="C65" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D65" s="36">
+        <v>1</v>
+      </c>
+      <c r="E65" s="61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above: CO₂:H₂ uptake 0.15–0.19 (×6 → 0.9–1.15), 1 = central.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Celsius-to-kelvin offset</t>
+        </is>
+      </c>
+      <c r="B66" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T_zero_C</t>
+        </is>
+      </c>
+      <c r="C66" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K</t>
+        </is>
+      </c>
+      <c r="D66" s="36">
+        <v>273.15</v>
+      </c>
+      <c r="E66" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined (SI): 0 °C = 273.15 K exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Ambient pressure setpoint</t>
+        </is>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P_atm_set</t>
+        </is>
+      </c>
+      <c r="C67" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pa</t>
+        </is>
+      </c>
+      <c r="D67" s="25">
+        <f>Summary!$D$10</f>
+        <v>0.0</v>
+      </c>
+      <c r="E67" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D10 (blank reads as 0, so P_atm falls back to Pa_per_atm).</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -18643,8 +19276,10 @@
         <f>HYPERLINK("#Geometry!D52","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
-      <c r="F5" s="101" t="s">
-        <v>540</v>
+      <c r="F5" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Magnetic stir bar. Pioreactor max 20 mm; confirm the supplied bar's length.</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -19094,11 +19729,13 @@
         <v>567</v>
       </c>
       <c r="D29" s="22">
-        <f>sigma_0+sigma_k*(T_K-273.15)</f>
+        <f>sigma_0+sigma_k*(T_K-T_zero_C)</f>
         <v>0.071965</v>
       </c>
-      <c r="E29" s="51" t="s">
-        <v>1785</v>
+      <c r="E29" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IAPWS R1-76(2014), evaluated at the reactor temperature (T_C). Feeds the bubble-detachment diameter.</t>
+        </is>
       </c>
       <c r="F29" s="20"/>
     </row>
@@ -19113,7 +19750,7 @@
         <v>570</v>
       </c>
       <c r="D30" s="22">
-        <f>rho_0+rho_k*(T_K-273.15)</f>
+        <f>rho_0+rho_k*(T_K-T_zero_C)</f>
         <v>996.94</v>
       </c>
       <c r="E30" s="51" t="s">
@@ -19153,8 +19790,10 @@
         <f>10^(HB_a+HB_b/T_K-(HB_c/T_K)^2)/10000</f>
         <v>1.997672318404e-09</v>
       </c>
-      <c r="E32" s="37" t="s">
-        <v>1787</v>
+      <c r="E32" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Han &amp; Bartels (1996) evaluated at the reactor temperature. At 25 °C this is 2.00e-9 m²/s.</t>
+        </is>
       </c>
       <c r="F32" s="20"/>
     </row>
@@ -19558,7 +20197,7 @@
         <v>354</v>
       </c>
       <c r="D54" s="48">
-        <f>IF(d_bubble&lt;0.001,0,kLa_sparge*(V_charge/1000000)*O2_ceil_C*3600)</f>
+        <f>IF(d_bubble&lt;d_bubble_min_m,0,kLa_sparge*(V_charge/1000000)*O2_ceil_C*3600)</f>
         <v>0.0003044695410516</v>
       </c>
       <c r="E54" s="75" t="s">
@@ -19746,7 +20385,7 @@
         <v>135</v>
       </c>
       <c r="D64" s="48" t="str">
-        <f>IF(d_bubble&lt;0.001,"Sinter OOR – add fine-bubble model",IF(We_orifice&lt;2,"Static","Dynamic"))</f>
+        <f>IF(d_bubble&lt;d_bubble_min_m,"Sinter OOR – add fine-bubble model",IF(We_orifice&lt;We_static_max,"Static","Dynamic"))</f>
         <v>Static</v>
       </c>
       <c r="E64" s="99" t="s">
@@ -19768,8 +20407,10 @@
         <f>O2_ceil_C*(V_charge/1000000)/O2_excess*60</f>
         <v>22.21910236615</v>
       </c>
-      <c r="E65" s="99" t="s">
-        <v>677</v>
+      <c r="E65" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minutes to reach the O₂ ceiling from ~0 with no removal (steady growth: the O₂ excess after biological uptake), the O₂ timescale.</t>
+        </is>
       </c>
       <c r="F65" s="20"/>
     </row>
@@ -19784,7 +20425,7 @@
         <v>67</v>
       </c>
       <c r="D66" s="48">
-        <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,9999)</f>
+        <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,cleared_min)</f>
         <v>22.588856006099</v>
       </c>
       <c r="E66" s="99" t="s">
@@ -19977,8 +20618,10 @@
         <f>H_O2_T*y_O2_vent*P_atm*1000</f>
         <v>44.468075969604</v>
       </c>
-      <c r="E76" s="69" t="s">
-        <v>1455</v>
+      <c r="E76" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dissolved O₂ in equilibrium with that vent headspace fraction, in µM; the same quantity as DO_hs_floor (D188) ×1000. Compare with the inhibition ceiling (Biology D28). Diagnostic, not a backstop.</t>
+        </is>
       </c>
       <c r="F76" s="20"/>
     </row>
@@ -20050,7 +20693,7 @@
         <v>67</v>
       </c>
       <c r="D80" s="48">
-        <f>IF(O2_net_gen-strip_avg-surf_strip&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_net_gen-strip_avg-surf_strip)*60,9999)</f>
+        <f>IF(O2_net_gen-strip_avg-surf_strip&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_net_gen-strip_avg-surf_strip)*60,cleared_min)</f>
         <v>9999.0</v>
       </c>
       <c r="E80" s="69" t="s">
@@ -20201,8 +20844,10 @@
         <f>MAX(duty_carbon,duty_O2vent)</f>
         <v>0.001485253206</v>
       </c>
-      <c r="E88" s="69" t="s">
-        <v>1456</v>
+      <c r="E88" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Least feasible CO₂ duty (the larger of the two floors). Informative only: D91 takes the interval from the carbon (D112) and DO-dilution (D185) intervals, not from this duty.</t>
+        </is>
       </c>
       <c r="F88" s="20"/>
     </row>
@@ -20220,8 +20865,10 @@
         <f>target_DO_frac*O2_ceil_C*(V_charge/1000000)/O2_src_guard*60</f>
         <v>1.503645716274</v>
       </c>
-      <c r="E89" s="99" t="s">
-        <v>1457</v>
+      <c r="E89" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂-limited fallback interval: zero-surface worst case (no surface credit; sizes on O2_src_guard D132). D91 uses it only when the DO target is unreachable (spg_int_DO, D185, is #N/A).</t>
+        </is>
       </c>
       <c r="F89" s="20"/>
     </row>
@@ -20258,8 +20905,10 @@
         <f>IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max))</f>
         <v>16.46036421628</v>
       </c>
-      <c r="E91" s="80" t="s">
-        <v>1827</v>
+      <c r="E91" s="80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANSWER. The shorter of the two upper bounds on the interval: carbon supply (D112) and headspace-oxygen dilution (spg_int_DO). If the DO target is unreachable at this surface kLa the sheet falls back to the lag-accumulation cap (D89) and D134 says so. kL_surf moves the answer continuously; no branch depends on it.</t>
+        </is>
       </c>
       <c r="F91" s="20"/>
     </row>
@@ -20283,8 +20932,10 @@
       <c r="F92" s="20"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A93" s="17" t="s">
-        <v>748</v>
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  resulting duty</t>
+        </is>
       </c>
       <c r="B93" s="18" t="s">
         <v>749</v>
@@ -20331,7 +20982,7 @@
         <v>135</v>
       </c>
       <c r="D95" s="48" t="str">
-        <f>IF(spg_int*60-spg_dur&gt;=5,"OK","TIGHT")</f>
+        <f>IF(spg_int*60-spg_dur&gt;=od_gap_min_s,"OK","TIGHT")</f>
         <v>OK</v>
       </c>
       <c r="E95" s="99" t="s">
@@ -20605,15 +21256,16 @@
       <c r="F110" s="20"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A111" s="20" t="s">
-        <v>788</v>
+      <c r="A111" s="20" t="str">
+        <f>"Tip-speed shear flag (&lt;"&amp;TEXT(tip_speed_max,"0.0")&amp;" m/s)"</f>
+        <v>Tip-speed shear flag (&lt;1.5 m/s)</v>
       </c>
       <c r="B111" s="20" t="s">
         <v>789</v>
       </c>
       <c r="C111" s="20"/>
       <c r="D111" s="24" t="str">
-        <f>IF(tip_speed&gt;1.5,"TIP SPEED &gt; 1.5 m/s","OK")</f>
+        <f>IF(tip_speed&gt;tip_speed_max,"TIP SPEED &gt; "&amp;TEXT(tip_speed_max,"0.0")&amp;" m/s","OK")</f>
         <v>OK</v>
       </c>
       <c r="E111" s="82" t="s">
@@ -20658,8 +21310,10 @@
       <c r="F113" s="20"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A114" s="103" t="s">
-        <v>796</v>
+      <c r="A114" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ DOSING &amp; SCHEDULE</t>
+        </is>
       </c>
       <c r="B114" s="20"/>
       <c r="C114" s="20"/>
@@ -20704,15 +21358,19 @@
       <c r="B117" s="20" t="s">
         <v>801</v>
       </c>
-      <c r="C117" s="20" t="s">
-        <v>14</v>
+      <c r="C117" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
       </c>
       <c r="D117" s="83">
         <f>IF(ISNUMBER(cal_flow),cal_flow,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*'CO2 flows'!$J$4:$J$201)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*('CO2 flows'!$J$4:$J$201&gt;0)*1)))</f>
         <v>3.33</v>
       </c>
-      <c r="E117" s="20" t="s">
-        <v>1924</v>
+      <c r="E117" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prefers the CO₂-flow calibration recorded on the Calibrations tab (cal_flow); falls back to the per-reactor table on the CO2 flows sheet when no calibration run is included.</t>
+        </is>
       </c>
       <c r="F117" s="20"/>
     </row>
@@ -20934,8 +21592,10 @@
       <c r="F130" s="20"/>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A131" s="20" t="s">
-        <v>832</v>
+      <c r="A131" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical surface kL_surf (DO held at the target DO)</t>
+        </is>
       </c>
       <c r="B131" s="20" t="s">
         <v>833</v>
@@ -21004,8 +21664,10 @@
         <f>IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf"))</f>
         <v>ESTIMATED kLa — DO-limited interval is 16.5 min; confirm by measuring kL_surf</v>
       </c>
-      <c r="E134" s="69" t="s">
-        <v>1826</v>
+      <c r="E134" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whether the dissolved-O₂ target is reachable at all, and whether the surface coefficient behind that verdict has been measured or is still the ~375%-uncertain estimate.</t>
+        </is>
       </c>
       <c r="F134" s="20"/>
     </row>
@@ -21051,7 +21713,7 @@
         <v>577</v>
       </c>
       <c r="D138" s="22">
-        <f>D_CO2_ref*EXP(-Ea_D_CO2/R_gas*(1/T_K-1/298.15))</f>
+        <f>D_CO2_ref*EXP(-Ea_D_CO2/R_gas*(1/T_K-1/T_ref))</f>
         <v>1.92e-09</v>
       </c>
       <c r="E138" s="67" t="s">
@@ -21552,8 +22214,10 @@
       <c r="F164" s="20"/>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A166" s="5" t="s">
-        <v>1757</v>
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TEMPERATURE-DEPENDENT WATER PROPERTIES</t>
+        </is>
       </c>
     </row>
     <row r="167" spans="1:6" ht="24" x14ac:dyDescent="0.2">
@@ -21637,8 +22301,10 @@
       <c r="D171" s="52">
         <v>-4.41</v>
       </c>
-      <c r="E171" s="99" t="s">
-        <v>1773</v>
+      <c r="E171" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Han &amp; Bartels (1996): log₁₀(D[cm²/s]) = a + b/T − (c/T)², evaluated at the reactor temperature.</t>
+        </is>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.2">
@@ -21710,8 +22376,10 @@
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A177" s="5" t="s">
-        <v>1789</v>
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEADSPACE O₂ BALANCE AND THE DO-LIMITED INTERVAL</t>
+        </is>
       </c>
     </row>
     <row r="178" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -21836,8 +22504,10 @@
         <f>IF(ISNUMBER(y_O2_star),O2_excess*(1-y_O2_star)/(y_O2_star*CO2_rate_full),NA())</f>
         <v>0.0007943455761538</v>
       </c>
-      <c r="E184" s="67" t="s">
-        <v>1810</v>
+      <c r="E184" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At steady state everything entering the headspace leaves through the vent, so the vent-gas composition is the flux composition: y = O₂ flux/(O₂ flux + CO₂ flux). Solving for the CO₂ flux that dilutes oxygen to y* gives this duty. Unlike duty_O2vent (D87), it accounts for the surface-transfer excess and the (1−y) term.</t>
+        </is>
       </c>
     </row>
     <row r="185" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -21913,8 +22583,10 @@
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A190" s="5" t="s">
-        <v>1829</v>
+      <c r="A190" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ LIMIT CYCLE – mass-conserving form (supersedes the uncoupled block above)</t>
+        </is>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.2">
@@ -21985,8 +22657,10 @@
         <f>CO2_pulse/(V_L_m3+Vg_CO2)</f>
         <v>5.869170438925</v>
       </c>
-      <c r="E194" s="99" t="s">
-        <v>1927</v>
+      <c r="E194" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The CO₂ actually delivered per pulse (D123, which follows any manual or Summary override), spread over the pooled liquid+headspace capacity: the mass-conservation constraint. It reads the delivered pulse rather than one nominal headspace flush, so an overridden pulse length charges the cycle correctly.</t>
+        </is>
       </c>
     </row>
     <row r="195" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -22164,11 +22838,197 @@
         <v>62</v>
       </c>
       <c r="D206" s="22">
-        <f>pw_A*EXP(pw_B*(T_K-273.15)/((T_K-273.15)+pw_C))</f>
+        <f>pw_A*EXP(pw_B*(T_K-T_zero_C)/((T_K-T_zero_C)+pw_C))</f>
         <v>3161.736035696692</v>
       </c>
-      <c r="E206" s="99" t="s">
-        <v>1922</v>
+      <c r="E206" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3.16 kPa at 25 °C, 4.24 kPa at 30 °C, 3–4% of atmospheric, which is exactly the bias it removes from a faradaic-efficiency measurement made by collecting gas over water.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAMED CONSTANTS, THRESHOLDS AND IMPORTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Reference temperature (25 °C)</t>
+        </is>
+      </c>
+      <c r="B209" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T_ref</t>
+        </is>
+      </c>
+      <c r="C209" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K</t>
+        </is>
+      </c>
+      <c r="D209" s="26">
+        <f>Biology!$D$23</f>
+        <v>298.15</v>
+      </c>
+      <c r="E209" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D23</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Celsius-to-kelvin offset</t>
+        </is>
+      </c>
+      <c r="B210" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T_zero_C</t>
+        </is>
+      </c>
+      <c r="C210" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K</t>
+        </is>
+      </c>
+      <c r="D210" s="26">
+        <f>Biology!$D$66</f>
+        <v>273.15</v>
+      </c>
+      <c r="E210" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D66</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minimum bubble diameter for the bubble model</t>
+        </is>
+      </c>
+      <c r="B211" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d_bubble_min_m</t>
+        </is>
+      </c>
+      <c r="C211" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m</t>
+        </is>
+      </c>
+      <c r="D211" s="36">
+        <v>0.001</v>
+      </c>
+      <c r="E211" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mendelson rise correlation valid ~1–10 mm (E46); sub-mm bubbles are out of range.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quasi-static detachment Weber limit</t>
+        </is>
+      </c>
+      <c r="B212" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We_static_max</t>
+        </is>
+      </c>
+      <c r="C212" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D212" s="36">
+        <v>2</v>
+      </c>
+      <c r="E212" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tate's-law quasi-static detachment holds for We &lt; ~2 (E64).</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cleared-ceiling display value</t>
+        </is>
+      </c>
+      <c r="B213" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cleared_min</t>
+        </is>
+      </c>
+      <c r="C213" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D213" s="36">
+        <v>9999</v>
+      </c>
+      <c r="E213" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined display sentinel: removal exceeds the source, so the ceiling is never reached.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minimum sparge-free gap for an OD read</t>
+        </is>
+      </c>
+      <c r="B214" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">od_gap_min_s</t>
+        </is>
+      </c>
+      <c r="C214" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D214" s="36">
+        <v>5</v>
+      </c>
+      <c r="E214" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: time for one Pioreactor OD read between pulses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stir-bar tip-speed shear limit</t>
+        </is>
+      </c>
+      <c r="B216" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tip_speed_max</t>
+        </is>
+      </c>
+      <c r="C216" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m/s</t>
+        </is>
+      </c>
+      <c r="D216" s="36">
+        <v>1.5</v>
+      </c>
+      <c r="E216" s="82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conservative impeller-tip limit for cell culture (BioProcess International); precautionary for HOB.</t>
+        </is>
       </c>
     </row>
     <row r="230">
@@ -22413,29 +23273,41 @@
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
-      <c r="C3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>12</v>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
       </c>
       <c r="F3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>14</v>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
       </c>
       <c r="I3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="5" t="s">
-        <v>14</v>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="8" t="s">
@@ -22582,8 +23454,10 @@
       <c r="K7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="L7" s="3" t="s">
-        <v>21</v>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2 collected in measuring cylinder over CO2-saturated water</t>
+        </is>
       </c>
       <c r="M7" s="3"/>
       <c r="N7" s="6"/>
@@ -22660,8 +23534,10 @@
       <c r="K9" s="9">
         <v>46190</v>
       </c>
-      <c r="L9" s="3" t="s">
-        <v>23</v>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Collected over saturated NaHCO3 solution</t>
+        </is>
       </c>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
@@ -24770,7 +25646,7 @@
       <c r="G23" s="123"/>
       <c r="H23" s="123"/>
       <c r="I23" s="129" t="str">
-        <f>IFERROR(((G23-'Mass Transfer'!$D$206)*(E23/1000000)/('Mass Transfer'!$D$101*(F23+273.15)))/(D23/(IF(H23="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G23-'Mass Transfer'!$D$206)*(E23/1000000)/('Mass Transfer'!$D$101*(F23+T_zero_C)))/(D23/(IF(H23="H2",z_e_H2,IF(H23="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J23" s="129" t="str">
@@ -24791,7 +25667,7 @@
       <c r="G24" s="123"/>
       <c r="H24" s="123"/>
       <c r="I24" s="129" t="str">
-        <f>IFERROR(((G24-'Mass Transfer'!$D$206)*(E24/1000000)/('Mass Transfer'!$D$101*(F24+273.15)))/(D24/(IF(H24="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G24-'Mass Transfer'!$D$206)*(E24/1000000)/('Mass Transfer'!$D$101*(F24+T_zero_C)))/(D24/(IF(H24="H2",z_e_H2,IF(H24="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J24" s="129" t="str">
@@ -24812,7 +25688,7 @@
       <c r="G25" s="123"/>
       <c r="H25" s="123"/>
       <c r="I25" s="129" t="str">
-        <f>IFERROR(((G25-'Mass Transfer'!$D$206)*(E25/1000000)/('Mass Transfer'!$D$101*(F25+273.15)))/(D25/(IF(H25="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G25-'Mass Transfer'!$D$206)*(E25/1000000)/('Mass Transfer'!$D$101*(F25+T_zero_C)))/(D25/(IF(H25="H2",z_e_H2,IF(H25="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J25" s="129" t="str">
@@ -24833,7 +25709,7 @@
       <c r="G26" s="123"/>
       <c r="H26" s="123"/>
       <c r="I26" s="129" t="str">
-        <f>IFERROR(((G26-'Mass Transfer'!$D$206)*(E26/1000000)/('Mass Transfer'!$D$101*(F26+273.15)))/(D26/(IF(H26="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G26-'Mass Transfer'!$D$206)*(E26/1000000)/('Mass Transfer'!$D$101*(F26+T_zero_C)))/(D26/(IF(H26="H2",z_e_H2,IF(H26="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J26" s="129" t="str">
@@ -24854,7 +25730,7 @@
       <c r="G27" s="123"/>
       <c r="H27" s="123"/>
       <c r="I27" s="129" t="str">
-        <f>IFERROR(((G27-'Mass Transfer'!$D$206)*(E27/1000000)/('Mass Transfer'!$D$101*(F27+273.15)))/(D27/(IF(H27="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G27-'Mass Transfer'!$D$206)*(E27/1000000)/('Mass Transfer'!$D$101*(F27+T_zero_C)))/(D27/(IF(H27="H2",z_e_H2,IF(H27="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J27" s="129" t="str">
@@ -24875,7 +25751,7 @@
       <c r="G28" s="123"/>
       <c r="H28" s="123"/>
       <c r="I28" s="129" t="str">
-        <f>IFERROR(((G28-'Mass Transfer'!$D$206)*(E28/1000000)/('Mass Transfer'!$D$101*(F28+273.15)))/(D28/(IF(H28="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G28-'Mass Transfer'!$D$206)*(E28/1000000)/('Mass Transfer'!$D$101*(F28+T_zero_C)))/(D28/(IF(H28="H2",z_e_H2,IF(H28="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J28" s="129" t="str">
@@ -24896,7 +25772,7 @@
       <c r="G29" s="123"/>
       <c r="H29" s="123"/>
       <c r="I29" s="129" t="str">
-        <f>IFERROR(((G29-'Mass Transfer'!$D$206)*(E29/1000000)/('Mass Transfer'!$D$101*(F29+273.15)))/(D29/(IF(H29="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G29-'Mass Transfer'!$D$206)*(E29/1000000)/('Mass Transfer'!$D$101*(F29+T_zero_C)))/(D29/(IF(H29="H2",z_e_H2,IF(H29="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J29" s="129" t="str">
@@ -24917,7 +25793,7 @@
       <c r="G30" s="123"/>
       <c r="H30" s="123"/>
       <c r="I30" s="129" t="str">
-        <f>IFERROR(((G30-'Mass Transfer'!$D$206)*(E30/1000000)/('Mass Transfer'!$D$101*(F30+273.15)))/(D30/(IF(H30="H2",2,4)*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G30-'Mass Transfer'!$D$206)*(E30/1000000)/('Mass Transfer'!$D$101*(F30+T_zero_C)))/(D30/(IF(H30="H2",z_e_H2,IF(H30="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
         <v/>
       </c>
       <c r="J30" s="129" t="str">
@@ -26051,7 +26927,7 @@
       <c r="C81" s="122"/>
       <c r="D81" s="123"/>
       <c r="E81" s="129" t="str">
-        <f t="shared" ref="E81:E88" si="2">IFERROR(IF((291.2/D81)&gt;160,0,IF((291.2/D81)&gt;100,1,IF((291.2/D81)&gt;40,2,IF((291.2/D81)&gt;16,3,IF((291.2/D81)&gt;10,4,5))))),"")</f>
+        <f>IFERROR(IF((bp_const/D81)&gt;por_break_1,0,IF((bp_const/D81)&gt;por_break_2,1,IF((bp_const/D81)&gt;por_break_3,2,IF((bp_const/D81)&gt;por_break_4,3,IF((bp_const/D81)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F81" s="129" t="str">
@@ -26072,7 +26948,7 @@
       <c r="C82" s="122"/>
       <c r="D82" s="123"/>
       <c r="E82" s="129" t="str">
-        <f t="shared" si="2"/>
+        <f>IFERROR(IF((bp_const/D82)&gt;por_break_1,0,IF((bp_const/D82)&gt;por_break_2,1,IF((bp_const/D82)&gt;por_break_3,2,IF((bp_const/D82)&gt;por_break_4,3,IF((bp_const/D82)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F82" s="130" t="str">
@@ -26093,7 +26969,7 @@
       <c r="C83" s="122"/>
       <c r="D83" s="123"/>
       <c r="E83" s="129" t="str">
-        <f t="shared" si="2"/>
+        <f>IFERROR(IF((bp_const/D83)&gt;por_break_1,0,IF((bp_const/D83)&gt;por_break_2,1,IF((bp_const/D83)&gt;por_break_3,2,IF((bp_const/D83)&gt;por_break_4,3,IF((bp_const/D83)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F83" s="130" t="str">
@@ -26114,7 +26990,7 @@
       <c r="C84" s="122"/>
       <c r="D84" s="123"/>
       <c r="E84" s="129" t="str">
-        <f t="shared" si="2"/>
+        <f>IFERROR(IF((bp_const/D84)&gt;por_break_1,0,IF((bp_const/D84)&gt;por_break_2,1,IF((bp_const/D84)&gt;por_break_3,2,IF((bp_const/D84)&gt;por_break_4,3,IF((bp_const/D84)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F84" s="130" t="str">
@@ -26135,7 +27011,7 @@
       <c r="C85" s="122"/>
       <c r="D85" s="123"/>
       <c r="E85" s="129" t="str">
-        <f t="shared" si="2"/>
+        <f>IFERROR(IF((bp_const/D85)&gt;por_break_1,0,IF((bp_const/D85)&gt;por_break_2,1,IF((bp_const/D85)&gt;por_break_3,2,IF((bp_const/D85)&gt;por_break_4,3,IF((bp_const/D85)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F85" s="130" t="str">
@@ -26156,7 +27032,7 @@
       <c r="C86" s="122"/>
       <c r="D86" s="123"/>
       <c r="E86" s="129" t="str">
-        <f t="shared" si="2"/>
+        <f>IFERROR(IF((bp_const/D86)&gt;por_break_1,0,IF((bp_const/D86)&gt;por_break_2,1,IF((bp_const/D86)&gt;por_break_3,2,IF((bp_const/D86)&gt;por_break_4,3,IF((bp_const/D86)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F86" s="129" t="str">
@@ -26177,7 +27053,7 @@
       <c r="C87" s="122"/>
       <c r="D87" s="123"/>
       <c r="E87" s="129" t="str">
-        <f t="shared" si="2"/>
+        <f>IFERROR(IF((bp_const/D87)&gt;por_break_1,0,IF((bp_const/D87)&gt;por_break_2,1,IF((bp_const/D87)&gt;por_break_3,2,IF((bp_const/D87)&gt;por_break_4,3,IF((bp_const/D87)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F87" s="129" t="str">
@@ -26198,7 +27074,7 @@
       <c r="C88" s="122"/>
       <c r="D88" s="123"/>
       <c r="E88" s="129" t="str">
-        <f t="shared" si="2"/>
+        <f>IFERROR(IF((bp_const/D88)&gt;por_break_1,0,IF((bp_const/D88)&gt;por_break_2,1,IF((bp_const/D88)&gt;por_break_3,2,IF((bp_const/D88)&gt;por_break_4,3,IF((bp_const/D88)&gt;por_break_5,4,5))))),"")</f>
         <v/>
       </c>
       <c r="F88" s="129" t="str">
@@ -27097,7 +27973,11 @@
       <c r="M138" s="97"/>
     </row>
     <row r="139" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A139" s="97"/>
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAMED CONSTANTS AND IMPORTS</t>
+        </is>
+      </c>
       <c r="B139" s="97"/>
       <c r="C139" s="97"/>
       <c r="D139" s="97"/>
@@ -27110,6 +27990,234 @@
       <c r="K139" s="97"/>
       <c r="L139" s="97"/>
       <c r="M139" s="97"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bubble-point constant (water)</t>
+        </is>
+      </c>
+      <c r="B140" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bp_const</t>
+        </is>
+      </c>
+      <c r="C140" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">µm·kPa</t>
+        </is>
+      </c>
+      <c r="D140" s="97">
+        <v>291.2</v>
+      </c>
+      <c r="E140" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bubble-point law d = 4σ/ΔP for water (σ = 72.8 mN/m, θ = 0): d in µm with ΔP in kPa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sinter grade boundary P0/P1</t>
+        </is>
+      </c>
+      <c r="B141" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">por_break_1</t>
+        </is>
+      </c>
+      <c r="C141" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">µm</t>
+        </is>
+      </c>
+      <c r="D141" s="97">
+        <v>160</v>
+      </c>
+      <c r="E141" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 4793 / DURAN pore-size grade boundary between P0 and P1 (Mass Transfer E33:E38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sinter grade boundary P1/P2</t>
+        </is>
+      </c>
+      <c r="B142" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">por_break_2</t>
+        </is>
+      </c>
+      <c r="C142" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">µm</t>
+        </is>
+      </c>
+      <c r="D142" s="97">
+        <v>100</v>
+      </c>
+      <c r="E142" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 4793 / DURAN pore-size grade boundary between P1 and P2 (Mass Transfer E33:E38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sinter grade boundary P2/P3</t>
+        </is>
+      </c>
+      <c r="B143" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">por_break_3</t>
+        </is>
+      </c>
+      <c r="C143" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">µm</t>
+        </is>
+      </c>
+      <c r="D143" s="97">
+        <v>40</v>
+      </c>
+      <c r="E143" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 4793 / DURAN pore-size grade boundary between P2 and P3 (Mass Transfer E33:E38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sinter grade boundary P3/P4</t>
+        </is>
+      </c>
+      <c r="B144" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">por_break_4</t>
+        </is>
+      </c>
+      <c r="C144" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">µm</t>
+        </is>
+      </c>
+      <c r="D144" s="97">
+        <v>16</v>
+      </c>
+      <c r="E144" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 4793 / DURAN pore-size grade boundary between P3 and P4 (Mass Transfer E33:E38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sinter grade boundary P4/P5</t>
+        </is>
+      </c>
+      <c r="B145" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">por_break_5</t>
+        </is>
+      </c>
+      <c r="C145" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">µm</t>
+        </is>
+      </c>
+      <c r="D145" s="97">
+        <v>10</v>
+      </c>
+      <c r="E145" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ISO 4793 / DURAN pore-size grade boundary between P4 and P5 (Mass Transfer E33:E38).</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Electrons per H₂</t>
+        </is>
+      </c>
+      <c r="B146" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z_e_H2</t>
+        </is>
+      </c>
+      <c r="C146" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D146" s="97">
+        <f>Electrochemistry!$D$16</f>
+        <v>2.0</v>
+      </c>
+      <c r="E146" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D16</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Electrons per O₂</t>
+        </is>
+      </c>
+      <c r="B147" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z_e_O2</t>
+        </is>
+      </c>
+      <c r="C147" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D147" s="97">
+        <f>Electrochemistry!$D$17</f>
+        <v>4.0</v>
+      </c>
+      <c r="E147" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D17</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Celsius-to-kelvin offset</t>
+        </is>
+      </c>
+      <c r="B148" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T_zero_C</t>
+        </is>
+      </c>
+      <c r="C148" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">K</t>
+        </is>
+      </c>
+      <c r="D148" s="97">
+        <f>Biology!$D$66</f>
+        <v>273.15</v>
+      </c>
+      <c r="E148" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D66</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Gas model: input/formula font and confidence-fill conventions applied (styles only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -6466,7 +6466,7 @@
     <numFmt numFmtId="170" formatCode="0.00000000"/>
     <numFmt numFmtId="171" formatCode="0.0000000"/>
   </numFmts>
-  <fonts count="41" x14ac:knownFonts="1">
+  <fonts count="47" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6717,8 +6717,52 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="9"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6827,6 +6871,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9999"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -7039,7 +7089,7 @@
     <xf numFmtId="0" fontId="28" fillId="10" borderId="11"/>
     <xf numFmtId="0" fontId="29" fillId="18" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -7221,6 +7271,43 @@
     <xf numFmtId="0" fontId="9" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="168" fontId="26" fillId="20" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="11" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf applyFill="1" numFmtId="0" fontId="30" fillId="21" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf applyFill="1" numFmtId="0" fontId="16" fillId="8" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="42" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="42" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="43" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="43" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf applyFill="1" numFmtId="0" fontId="35" fillId="8" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="43" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="43" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="43" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="43" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf applyFill="1" numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf applyFont="1" numFmtId="0" fontId="45" fillId="0" borderId="11" xfId="0"/>
+    <xf applyFont="1" numFmtId="0" fontId="46" fillId="0" borderId="11" xfId="0"/>
+    <xf applyFill="1" numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -7902,7 +7989,7 @@
         <v>30</v>
       </c>
       <c r="C2" s="19"/>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="131" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="20" t="s">
@@ -7920,7 +8007,7 @@
         <v>34</v>
       </c>
       <c r="C3" s="19"/>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="131" t="s">
         <v>393</v>
       </c>
       <c r="E3" s="20" t="s">
@@ -7940,7 +8027,7 @@
         <v>38</v>
       </c>
       <c r="C4" s="19"/>
-      <c r="D4" s="36" t="s">
+      <c r="D4" s="131" t="s">
         <v>535</v>
       </c>
       <c r="E4" s="20" t="s">
@@ -7958,7 +8045,7 @@
         <v>42</v>
       </c>
       <c r="C5" s="20"/>
-      <c r="D5" s="36" t="inlineStr">
+      <c r="D5" s="131" t="inlineStr">
         <is>
           <t>UdG phosphate</t>
         </is>
@@ -7980,7 +8067,7 @@
       <c r="C6" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="36">
+      <c r="D6" s="131">
         <v>3</v>
       </c>
       <c r="E6" s="20" t="s">
@@ -8000,7 +8087,7 @@
       <c r="C7" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="36">
+      <c r="D7" s="131">
         <v>1000</v>
       </c>
       <c r="E7" s="20" t="s">
@@ -8020,7 +8107,7 @@
       <c r="C8" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="D8" s="36">
+      <c r="D8" s="131">
         <v>25</v>
       </c>
       <c r="E8" s="20" t="s">
@@ -8779,7 +8866,7 @@
       <c r="F51" s="16"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A52" s="87" t="s">
+      <c r="A52" s="132" t="s">
         <v>113</v>
       </c>
       <c r="B52" s="20"/>
@@ -8879,7 +8966,7 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A63" s="86" t="s">
+      <c r="A63" s="133" t="s">
         <v>124</v>
       </c>
       <c r="B63" s="20"/>
@@ -9413,7 +9500,7 @@
           <t xml:space="preserve">s or min</t>
         </is>
       </c>
-      <c r="D93" s="36">
+      <c r="D93" s="131">
         <v>0.5</v>
       </c>
       <c r="E93" s="87" t="inlineStr">
@@ -9645,11 +9732,11 @@
       <c r="C5" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="D5" s="38" t="str">
+      <c r="D5" s="134" t="str">
         <f>Summary!$D$2</f>
         <v>ed04</v>
       </c>
-      <c r="E5" s="23" t="str">
+      <c r="E5" s="135" t="str">
         <f>HYPERLINK("#Summary!D2","→ Summary")</f>
         <v>→ Summary</v>
       </c>
@@ -9668,11 +9755,11 @@
       <c r="C6" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="134">
         <f>Summary!$D$9</f>
         <v>0.0</v>
       </c>
-      <c r="E6" s="23" t="str">
+      <c r="E6" s="135" t="str">
         <f>HYPERLINK("#Summary!D9","→ Summary")</f>
         <v>→ Summary</v>
       </c>
@@ -9702,7 +9789,7 @@
       <c r="C8" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D8" s="105" t="s">
+      <c r="D8" s="136" t="s">
         <v>139</v>
       </c>
       <c r="E8" s="107" t="s">
@@ -9723,7 +9810,7 @@
       <c r="C9" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D9" s="105" t="s">
+      <c r="D9" s="136" t="s">
         <v>143</v>
       </c>
       <c r="E9" s="107" t="s">
@@ -9744,7 +9831,7 @@
       <c r="C10" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D10" s="108">
+      <c r="D10" s="137">
         <v>27.48</v>
       </c>
       <c r="E10" s="109" t="s">
@@ -9765,7 +9852,7 @@
       <c r="C11" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D11" s="108">
+      <c r="D11" s="137">
         <v>27.48</v>
       </c>
       <c r="E11" s="110" t="s">
@@ -9786,7 +9873,7 @@
       <c r="C12" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D12" s="106">
+      <c r="D12" s="138">
         <v>55</v>
       </c>
       <c r="E12" s="111" t="s">
@@ -9807,7 +9894,7 @@
       <c r="C13" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D13" s="106">
+      <c r="D13" s="138">
         <v>95</v>
       </c>
       <c r="E13" s="111" t="s">
@@ -9828,7 +9915,7 @@
       <c r="C14" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="106">
+      <c r="D14" s="138">
         <v>16</v>
       </c>
       <c r="E14" s="109" t="s">
@@ -9849,7 +9936,7 @@
       <c r="C15" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="106">
+      <c r="D15" s="138">
         <v>30</v>
       </c>
       <c r="E15" s="109" t="s">
@@ -9870,7 +9957,7 @@
       <c r="C16" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="106">
+      <c r="D16" s="138">
         <v>20</v>
       </c>
       <c r="E16" s="112" t="s">
@@ -9891,7 +9978,7 @@
       <c r="C17" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="106">
+      <c r="D17" s="138">
         <v>42</v>
       </c>
       <c r="E17" s="112" t="s">
@@ -9912,7 +9999,7 @@
       <c r="C18" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D18" s="40">
+      <c r="D18" s="139">
         <f>VLOOKUP(rx_ver,$A$84:$I$87,7,FALSE)</f>
         <v>27.48</v>
       </c>
@@ -9934,7 +10021,7 @@
       <c r="C19" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D19" s="36">
+      <c r="D19" s="131">
         <v>1.1000000000000001</v>
       </c>
       <c r="E19" s="41" t="s">
@@ -9999,7 +10086,7 @@
       <c r="C22" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D22" s="44">
+      <c r="D22" s="140">
         <f>IF(ISNUMBER(cal_Dint),cal_Dint,VLOOKUP(rx_ver,$A$84:$I$87,4,FALSE))</f>
         <v>55.0</v>
       </c>
@@ -10021,7 +10108,7 @@
       <c r="C23" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D23" s="44">
+      <c r="D23" s="140">
         <f>VLOOKUP(rx_ver,$A$84:$I$87,5,FALSE)</f>
         <v>16.0</v>
       </c>
@@ -10043,7 +10130,7 @@
       <c r="C24" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D24" s="44">
+      <c r="D24" s="140">
         <f>IF(ISNUMBER(cal_Vtot),cal_Vtot,VLOOKUP(rx_ver,$A$84:$I$87,6,FALSE))</f>
         <v>20.0</v>
       </c>
@@ -10087,7 +10174,7 @@
       <c r="C26" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D26" s="36">
+      <c r="D26" s="131">
         <v>6</v>
       </c>
       <c r="E26" s="37" t="s">
@@ -10108,7 +10195,7 @@
       <c r="C27" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D27" s="36">
+      <c r="D27" s="131">
         <v>2</v>
       </c>
       <c r="E27" s="99" t="s">
@@ -10129,7 +10216,7 @@
       <c r="C28" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D28" s="36">
+      <c r="D28" s="131">
         <v>22</v>
       </c>
       <c r="E28" s="37" t="s">
@@ -10172,7 +10259,7 @@
       <c r="C30" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D30" s="36">
+      <c r="D30" s="131">
         <v>3.1749999999999998</v>
       </c>
       <c r="E30" s="99" t="s">
@@ -10193,7 +10280,7 @@
       <c r="C31" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D31" s="36">
+      <c r="D31" s="131">
         <v>1.5874999999999999</v>
       </c>
       <c r="E31" s="99" t="s">
@@ -10236,7 +10323,7 @@
       <c r="C33" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D33" s="131">
         <v>3.1749999999999998</v>
       </c>
       <c r="E33" s="99" t="s">
@@ -10257,7 +10344,7 @@
       <c r="C34" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D34" s="36">
+      <c r="D34" s="131">
         <v>1.5874999999999999</v>
       </c>
       <c r="E34" s="99" t="s">
@@ -10410,7 +10497,7 @@
       <c r="C41" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D41" s="47">
+      <c r="D41" s="49">
         <f>IF(media_volume&gt;0,media_volume,ROUND(V_max-disp_tot,0))</f>
         <v>15.0</v>
       </c>
@@ -10520,7 +10607,7 @@
       <c r="C46" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D46" s="36">
+      <c r="D46" s="131">
         <v>3</v>
       </c>
       <c r="E46" s="37" t="s">
@@ -10541,7 +10628,7 @@
       <c r="C47" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D47" s="36">
+      <c r="D47" s="131">
         <v>5</v>
       </c>
       <c r="E47" s="41" t="s">
@@ -10628,7 +10715,7 @@
         <v>258</v>
       </c>
       <c r="C51" s="20"/>
-      <c r="D51" s="24" t="str">
+      <c r="D51" s="28" t="str">
         <f>VLOOKUP(reactor_sel,$A$59:$B$80,2,FALSE)</f>
         <v>MEP0.3</v>
       </c>
@@ -10646,7 +10733,7 @@
         <v>260</v>
       </c>
       <c r="C52" s="20"/>
-      <c r="D52" s="24">
+      <c r="D52" s="28">
         <f>VLOOKUP(rx_ver,$A$84:$I$87,8,FALSE)</f>
         <v>12.0</v>
       </c>
@@ -10677,7 +10764,7 @@
         <v>263</v>
       </c>
       <c r="C54" s="20"/>
-      <c r="D54" s="24" t="str">
+      <c r="D54" s="28" t="str">
         <f>IF(V_charge&gt;V_max,"MEDIA &gt; MAX WORKING VOLUME","OK")</f>
         <v>OK</v>
       </c>
@@ -10695,7 +10782,7 @@
         <v>265</v>
       </c>
       <c r="C55" s="20"/>
-      <c r="D55" s="24" t="str">
+      <c r="D55" s="28" t="str">
         <f>IF(h_actual&gt;D_int,"LIQUID OVER USABLE DEPTH","OK")</f>
         <v>OK</v>
       </c>
@@ -11275,7 +11362,7 @@
         <v>304</v>
       </c>
       <c r="C90" s="20"/>
-      <c r="D90" s="24" t="str">
+      <c r="D90" s="28" t="str">
         <f>IF(ABS(A_x*D_int/1000-V_vial_total)&lt;=geom_tol_mL,"OK",IF(AND(ISNUMBER(cal_hs),ISNUMBER(cal_hs_fill)),"HEADSPACE MEASURED - bore depth still inconsistent (measure body volume)","VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth"))</f>
         <v>VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth</v>
       </c>
@@ -11306,7 +11393,7 @@
       <c r="C92" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D92" s="36">
+      <c r="D92" s="131">
         <v>14</v>
       </c>
       <c r="E92" s="70" t="s">
@@ -11323,7 +11410,7 @@
       <c r="C93" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D93" s="22">
+      <c r="D93" s="141">
         <f>MAX(0,h_actual-elec_clear)</f>
         <v>9.18130412738</v>
       </c>
@@ -11354,7 +11441,7 @@
           <t xml:space="preserve">mL</t>
         </is>
       </c>
-      <c r="D96" s="36">
+      <c r="D96" s="131">
         <v>3</v>
       </c>
       <c r="E96" s="37" t="inlineStr">
@@ -11459,11 +11546,11 @@
       <c r="C5" s="20" t="s">
         <v>309</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="142">
         <f>Biology!$D$18</f>
         <v>298.15</v>
       </c>
-      <c r="E5" s="23" t="str">
+      <c r="E5" s="135" t="str">
         <f>HYPERLINK("#Biology!D18","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -11482,11 +11569,11 @@
       <c r="C6" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="142">
         <f>Biology!$D$19</f>
         <v>101325.0</v>
       </c>
-      <c r="E6" s="23" t="str">
+      <c r="E6" s="135" t="str">
         <f>HYPERLINK("#Biology!D19","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -11505,11 +11592,11 @@
       <c r="C7" s="20" t="s">
         <v>314</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="141">
         <f>'Mass Transfer'!$D$101</f>
         <v>8.314462618</v>
       </c>
-      <c r="E7" s="23" t="str">
+      <c r="E7" s="135" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D101","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
@@ -11526,11 +11613,11 @@
         <v>34</v>
       </c>
       <c r="C8" s="20"/>
-      <c r="D8" s="38" t="str">
+      <c r="D8" s="134" t="str">
         <f>Summary!$D$3</f>
         <v>Pt/Ti rod</v>
       </c>
-      <c r="E8" s="23" t="str">
+      <c r="E8" s="135" t="str">
         <f>HYPERLINK("#Summary!D3","→ Summary")</f>
         <v>→ Summary</v>
       </c>
@@ -11560,7 +11647,7 @@
       <c r="C10" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="53">
+      <c r="D10" s="143">
         <f>Summary!$D$6</f>
         <v>3.0</v>
       </c>
@@ -11582,7 +11669,7 @@
       <c r="C11" s="19" t="s">
         <v>321</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="141">
         <f>IF(ISNUMBER(cal_gerrit_slope),cal_gerrit_slope,gerrit_slope_default)</f>
         <v>1.03</v>
       </c>
@@ -11604,7 +11691,7 @@
       <c r="C12" s="19" t="s">
         <v>325</v>
       </c>
-      <c r="D12" s="22">
+      <c r="D12" s="141">
         <f>IF(ISNUMBER(cal_gerrit_int),cal_gerrit_int,gerrit_int_default)</f>
         <v>2.6</v>
       </c>
@@ -11626,7 +11713,7 @@
       <c r="C13" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="55">
+      <c r="D13" s="144">
         <v>3</v>
       </c>
       <c r="E13" s="51" t="s">
@@ -11647,7 +11734,7 @@
       <c r="C14" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="55">
+      <c r="D14" s="144">
         <v>25</v>
       </c>
       <c r="E14" s="51" t="s">
@@ -11668,7 +11755,7 @@
       <c r="C15" s="19" t="s">
         <v>335</v>
       </c>
-      <c r="D15" s="56">
+      <c r="D15" s="145">
         <v>96485.332120000006</v>
       </c>
       <c r="E15" s="100" t="s">
@@ -11689,7 +11776,7 @@
       <c r="C16" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D16" s="52">
+      <c r="D16" s="146">
         <v>2</v>
       </c>
       <c r="E16" s="99" t="s">
@@ -11710,7 +11797,7 @@
       <c r="C17" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D17" s="52">
+      <c r="D17" s="146">
         <v>4</v>
       </c>
       <c r="E17" s="99" t="s">
@@ -11731,7 +11818,7 @@
       <c r="C18" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D18" s="108">
+      <c r="D18" s="42">
         <f>IF(ISNUMBER(cal_etaF),cal_etaF,etaF_calc)</f>
         <v>0.977475298652</v>
       </c>
@@ -11909,7 +11996,7 @@
       <c r="C26" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D26" s="108">
+      <c r="D26" s="42">
         <f>IF(ISNUMBER(cal_etaF_OER),cal_etaF_OER,etaF_OER_calc)</f>
         <v>0.975081911036</v>
       </c>
@@ -11933,7 +12020,7 @@
       <c r="C27" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D27" s="40">
+      <c r="D27" s="139">
         <f>VLOOKUP(electrode_sel,$A$35:$I$38,9,FALSE)</f>
         <v>2.0</v>
       </c>
@@ -12010,7 +12097,7 @@
         <v>382</v>
       </c>
       <c r="C31" s="20"/>
-      <c r="D31" s="24" t="str">
+      <c r="D31" s="28" t="str">
         <f>VLOOKUP(electrode_sel,$A$35:$I$38,4,FALSE)</f>
         <v>Tube</v>
       </c>
@@ -12028,11 +12115,11 @@
         <v>384</v>
       </c>
       <c r="C32" s="20"/>
-      <c r="D32" s="24">
+      <c r="D32" s="28">
         <f>IF(ISNUMBER(cal_sinter),cal_sinter,IF(ISNUMBER(VLOOKUP(electrode_sel,$A$35:$I$38,5,FALSE)),VLOOKUP(electrode_sel,$A$35:$I$38,5,FALSE),0))</f>
         <v>0.0</v>
       </c>
-      <c r="E32" s="101" t="s">
+      <c r="E32" s="147" t="s">
         <v>385</v>
       </c>
       <c r="F32" s="20"/>
@@ -12499,7 +12586,7 @@
       <c r="C52" s="19" t="s">
         <v>1282</v>
       </c>
-      <c r="D52" s="52">
+      <c r="D52" s="146">
         <v>80</v>
       </c>
       <c r="E52" s="51" t="s">
@@ -12516,7 +12603,7 @@
       <c r="C53" s="19" t="s">
         <v>1282</v>
       </c>
-      <c r="D53" s="52">
+      <c r="D53" s="146">
         <v>250</v>
       </c>
       <c r="E53" s="51" t="s">
@@ -12533,7 +12620,7 @@
       <c r="C54" s="19" t="s">
         <v>1282</v>
       </c>
-      <c r="D54" s="52">
+      <c r="D54" s="146">
         <v>1</v>
       </c>
       <c r="E54" s="114" t="s">
@@ -12550,7 +12637,7 @@
       <c r="C55" s="19" t="s">
         <v>1282</v>
       </c>
-      <c r="D55" s="52">
+      <c r="D55" s="146">
         <v>2</v>
       </c>
       <c r="E55" s="114" t="s">
@@ -12840,7 +12927,7 @@
       <c r="C73" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="D73" s="52">
+      <c r="D73" s="146">
         <v>10</v>
       </c>
       <c r="E73" s="51" t="s">
@@ -12918,7 +13005,7 @@
       <c r="C79" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D79" s="22">
+      <c r="D79" s="141">
         <f>Biology!$D$60</f>
         <v>0.226086956522</v>
       </c>
@@ -12936,7 +13023,7 @@
       <c r="C80" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D80" s="22">
+      <c r="D80" s="141">
         <f>Biology!$D$27</f>
         <v>0.36477</v>
       </c>
@@ -12954,7 +13041,7 @@
       <c r="C81" s="19" t="s">
         <v>577</v>
       </c>
-      <c r="D81" s="22">
+      <c r="D81" s="141">
         <f>'Mass Transfer'!$D$32</f>
         <v>1.997672318404e-09</v>
       </c>
@@ -12972,7 +13059,7 @@
       <c r="C82" s="19" t="s">
         <v>858</v>
       </c>
-      <c r="D82" s="22">
+      <c r="D82" s="141">
         <f>Biology!$D$6/1000</f>
         <v>0.015</v>
       </c>
@@ -12990,7 +13077,7 @@
       <c r="C83" s="19" t="s">
         <v>1070</v>
       </c>
-      <c r="D83" s="36">
+      <c r="D83" s="131">
         <v>4.0000000000000001E-3</v>
       </c>
       <c r="E83" s="75" t="s">
@@ -13007,7 +13094,7 @@
       <c r="C84" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D84" s="52">
+      <c r="D84" s="146">
         <v>0.64400000000000002</v>
       </c>
       <c r="E84" s="99" t="s">
@@ -13024,7 +13111,7 @@
       <c r="C85" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D85" s="22">
+      <c r="D85" s="141">
         <f>ec_DO_frac*ec_O2_ceil</f>
         <v>0.08246973913</v>
       </c>
@@ -13042,7 +13129,7 @@
       <c r="C86" s="19" t="s">
         <v>1076</v>
       </c>
-      <c r="D86" s="22">
+      <c r="D86" s="141">
         <f>z_e_ORR*F_const*(km_O2/100)*ec_DO_design*(A_cath_wet/10000)</f>
         <v>0.0001281655506682</v>
       </c>
@@ -13060,7 +13147,7 @@
       <c r="C87" s="19" t="s">
         <v>1076</v>
       </c>
-      <c r="D87" s="22">
+      <c r="D87" s="141">
         <f>z_e_ORR*F_const*(km_O2/100)*ec_O2_ceil*(A_cath_wet/10000)</f>
         <v>0.0005668860894942</v>
       </c>
@@ -13078,7 +13165,7 @@
       <c r="C88" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D88" s="22">
+      <c r="D88" s="141">
         <f>MAX(0,1-i_ORR_design/I_app)</f>
         <v>0.977475298652</v>
       </c>
@@ -13098,7 +13185,7 @@
       <c r="C89" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D89" s="22">
+      <c r="D89" s="141">
         <f>MAX(0,1-i_ORR_ceiling/I_app)</f>
         <v>0.90037151327</v>
       </c>
@@ -13121,7 +13208,7 @@
       <c r="C91" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D91" s="36">
+      <c r="D91" s="131">
         <v>0.15</v>
       </c>
       <c r="E91" s="75" t="s">
@@ -13138,7 +13225,7 @@
       <c r="C92" s="19" t="s">
         <v>1258</v>
       </c>
-      <c r="D92" s="52">
+      <c r="D92" s="146">
         <v>34.014699999999998</v>
       </c>
       <c r="E92" s="99" t="s">
@@ -13155,7 +13242,7 @@
       <c r="C93" s="19" t="s">
         <v>1266</v>
       </c>
-      <c r="D93" s="22">
+      <c r="D93" s="141">
         <f>f_HOOH*i_ORR_design/(2*F_const)*M_H2O2*1000*3600/ec_V_L</f>
         <v>0.813296984002</v>
       </c>
@@ -13175,7 +13262,7 @@
       <c r="C94" s="19" t="s">
         <v>639</v>
       </c>
-      <c r="D94" s="36">
+      <c r="D94" s="131">
         <v>4.1000000000000003E-3</v>
       </c>
       <c r="E94" s="75" t="s">
@@ -13192,7 +13279,7 @@
       <c r="C95" s="19" t="s">
         <v>1270</v>
       </c>
-      <c r="D95" s="22">
+      <c r="D95" s="141">
         <f>r_H2O2/(k_cat_cells*3600)</f>
         <v>0.05510142168</v>
       </c>
@@ -13210,7 +13297,7 @@
       <c r="C96" s="19" t="s">
         <v>1270</v>
       </c>
-      <c r="D96" s="22">
+      <c r="D96" s="141">
         <f>r_H2O2</f>
         <v>0.813296984002</v>
       </c>
@@ -13228,7 +13315,7 @@
       <c r="C97" s="19" t="s">
         <v>1270</v>
       </c>
-      <c r="D97" s="52">
+      <c r="D97" s="146">
         <v>0.17</v>
       </c>
       <c r="E97" s="67" t="s">
@@ -13245,7 +13332,7 @@
       <c r="C98" s="19" t="s">
         <v>962</v>
       </c>
-      <c r="D98" s="22">
+      <c r="D98" s="141">
         <f>IF(r_H2O2&gt;0,H2O2_thresh/r_H2O2*60,NA())</f>
         <v>12.541544110741</v>
       </c>
@@ -13263,7 +13350,7 @@
       <c r="C99" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D99" s="22" t="str">
+      <c r="D99" s="141" t="str">
         <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(H2O2_lag_1h&gt;H2O2_thresh,"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases"))</f>
         <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 13 min before biomass can scavenge it</v>
       </c>
@@ -13286,7 +13373,7 @@
       <c r="C101" s="19" t="s">
         <v>1076</v>
       </c>
-      <c r="D101" s="22">
+      <c r="D101" s="141">
         <f>Chemistry!$D$133</f>
         <v>0.0001417839262056</v>
       </c>
@@ -13304,7 +13391,7 @@
       <c r="C102" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D102" s="22">
+      <c r="D102" s="141">
         <f>Chemistry!$D$158</f>
         <v>0.0</v>
       </c>
@@ -13322,7 +13409,7 @@
       <c r="C103" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D103" s="22">
+      <c r="D103" s="141">
         <f>ec_I_Cl/I_app</f>
         <v>0.024918088964</v>
       </c>
@@ -13340,7 +13427,7 @@
       <c r="C104" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D104" s="22">
+      <c r="D104" s="141">
         <f>MAX(0,1-f_Cl_anode-IF(ISNUMBER(ec_corr_I),ec_corr_I,0))</f>
         <v>0.975081911036</v>
       </c>
@@ -13365,7 +13452,7 @@
       <c r="C106" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D106" s="22">
+      <c r="D106" s="141">
         <f>Chemistry!$D$201</f>
         <v>1.229</v>
       </c>
@@ -13383,7 +13470,7 @@
       <c r="C107" s="19" t="s">
         <v>1705</v>
       </c>
-      <c r="D107" s="36">
+      <c r="D107" s="131">
         <v>0.12</v>
       </c>
       <c r="E107" s="75" t="s">
@@ -13400,7 +13487,7 @@
       <c r="C108" s="19" t="s">
         <v>1709</v>
       </c>
-      <c r="D108" s="36">
+      <c r="D108" s="131">
         <v>1E-10</v>
       </c>
       <c r="E108" s="41" t="s">
@@ -13417,7 +13504,7 @@
       <c r="C109" s="19" t="s">
         <v>1705</v>
       </c>
-      <c r="D109" s="36">
+      <c r="D109" s="131">
         <v>0.14000000000000001</v>
       </c>
       <c r="E109" s="67" t="s">
@@ -13434,7 +13521,7 @@
       <c r="C110" s="19" t="s">
         <v>1709</v>
       </c>
-      <c r="D110" s="36">
+      <c r="D110" s="131">
         <v>1.5E-6</v>
       </c>
       <c r="E110" s="67" t="s">
@@ -13451,7 +13538,7 @@
       <c r="C111" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D111" s="22">
+      <c r="D111" s="141">
         <f>b_anode*LOG10(j_anode/1000/j0_anode)</f>
         <v>0.894142423496</v>
       </c>
@@ -13469,7 +13556,7 @@
       <c r="C112" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D112" s="22">
+      <c r="D112" s="141">
         <f>b_cath*LOG10(j_cathode/1000/j0_cath)</f>
         <v>0.458513384477</v>
       </c>
@@ -13487,7 +13574,7 @@
       <c r="C113" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D113" s="36">
+      <c r="D113" s="131">
         <v>-0.15</v>
       </c>
       <c r="E113" s="75" t="s">
@@ -13504,7 +13591,7 @@
       <c r="C114" s="19" t="s">
         <v>1507</v>
       </c>
-      <c r="D114" s="22">
+      <c r="D114" s="141">
         <f>Chemistry!$D$180</f>
         <v>0.706946657056</v>
       </c>
@@ -13522,7 +13609,7 @@
       <c r="C115" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D115" s="22">
+      <c r="D115" s="141">
         <f>Geometry!$D$92</f>
         <v>14.0</v>
       </c>
@@ -13540,7 +13627,7 @@
       <c r="C116" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D116" s="36">
+      <c r="D116" s="131">
         <v>2</v>
       </c>
       <c r="E116" s="75" t="s">
@@ -13557,7 +13644,7 @@
       <c r="C117" s="19" t="s">
         <v>1737</v>
       </c>
-      <c r="D117" s="22">
+      <c r="D117" s="141">
         <f>k_geom*ACOSH(ec_gap/anode_dia)/(PI()*ec_kappa*(L_sub/1000))</f>
         <v>146.239829708796</v>
       </c>
@@ -13575,7 +13662,7 @@
       <c r="C118" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D118" s="22">
+      <c r="D118" s="141">
         <f>I_app*R_cell</f>
         <v>0.832104631043</v>
       </c>
@@ -13593,7 +13680,7 @@
       <c r="C119" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D119" s="22">
+      <c r="D119" s="141">
         <f>ec_E_rev+eta_anode+eta_cath+pcet_credit+V_IR</f>
         <v>3.263760439016</v>
       </c>
@@ -13611,7 +13698,7 @@
       <c r="C120" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D120" s="52">
+      <c r="D120" s="146">
         <v>5</v>
       </c>
       <c r="E120" s="67" t="s">
@@ -13628,7 +13715,7 @@
       <c r="C121" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D121" s="22">
+      <c r="D121" s="141">
         <f>V_rail-V_cell_est</f>
         <v>1.736239560984</v>
       </c>
@@ -13646,7 +13733,7 @@
       <c r="C122" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D122" s="22" t="str">
+      <c r="D122" s="141" t="str">
         <f>IF(V_headroom&lt;0,"OVER RAIL — the drive cannot deliver this current; the linear current law will not hold",IF(V_headroom&lt;V_headroom_min,"watch — within "&amp;TEXT(V_headroom_min,"0")&amp;" V of the rail ("&amp;TEXT(V_cell_est,"0.00")&amp;" V of "&amp;TEXT(V_rail,"0")&amp;" V); expect the current law to bend","OK — "&amp;TEXT(V_cell_est,"0.00")&amp;" V estimated against a "&amp;TEXT(V_rail,"0")&amp;" V rail"))</f>
         <v>OK — 3.26 V estimated against a 5 V rail</v>
       </c>
@@ -13677,7 +13764,7 @@
           <t xml:space="preserve">mA/%</t>
         </is>
       </c>
-      <c r="D125" s="36">
+      <c r="D125" s="131">
         <v>1.03</v>
       </c>
       <c r="E125" s="109" t="inlineStr">
@@ -13702,7 +13789,7 @@
           <t xml:space="preserve">mA</t>
         </is>
       </c>
-      <c r="D126" s="36">
+      <c r="D126" s="131">
         <v>2.6</v>
       </c>
       <c r="E126" s="109" t="inlineStr">
@@ -13727,7 +13814,7 @@
           <t xml:space="preserve">V</t>
         </is>
       </c>
-      <c r="D127" s="36">
+      <c r="D127" s="131">
         <v>1</v>
       </c>
       <c r="E127" s="114" t="inlineStr">
@@ -13917,7 +14004,7 @@
       <c r="C9" s="19" t="s">
         <v>862</v>
       </c>
-      <c r="D9" s="52">
+      <c r="D9" s="148">
         <f>'Mass Transfer'!$D$101</f>
         <v>8.314462618</v>
       </c>
@@ -14106,7 +14193,7 @@
       <c r="C21" s="19" t="s">
         <v>880</v>
       </c>
-      <c r="D21" s="62">
+      <c r="D21" s="149">
         <f>-LOG10(Ka_HOCl)</f>
         <v>7.54</v>
       </c>
@@ -14149,7 +14236,7 @@
       <c r="C25" s="20">
         <v>0</v>
       </c>
-      <c r="D25" s="52">
+      <c r="D25" s="146">
         <v>2.2999999999999998</v>
       </c>
       <c r="E25" s="51" t="s">
@@ -14166,7 +14253,7 @@
       <c r="C26" s="52">
         <v>2.895</v>
       </c>
-      <c r="D26" s="52">
+      <c r="D26" s="146">
         <v>2.9</v>
       </c>
       <c r="E26" s="51" t="s">
@@ -14200,7 +14287,7 @@
       <c r="C28" s="20">
         <v>0</v>
       </c>
-      <c r="D28" s="52">
+      <c r="D28" s="146">
         <v>1.05</v>
       </c>
       <c r="E28" s="51" t="s">
@@ -14251,7 +14338,7 @@
       <c r="C31" s="52">
         <v>0.8</v>
       </c>
-      <c r="D31" s="52">
+      <c r="D31" s="146">
         <v>0.5</v>
       </c>
       <c r="E31" s="51" t="s">
@@ -14268,7 +14355,7 @@
       <c r="C32" s="52">
         <v>0.94299999999999995</v>
       </c>
-      <c r="D32" s="52">
+      <c r="D32" s="146">
         <v>0.47</v>
       </c>
       <c r="E32" s="51" t="s">
@@ -14285,7 +14372,7 @@
       <c r="C33" s="20">
         <v>0</v>
       </c>
-      <c r="D33" s="52">
+      <c r="D33" s="146">
         <v>0.01</v>
       </c>
       <c r="E33" s="51" t="s">
@@ -14302,7 +14389,7 @@
       <c r="C35" s="19" t="s">
         <v>902</v>
       </c>
-      <c r="D35" s="62">
+      <c r="D35" s="149">
         <f>mc_Na2HPO4/MW_Na2HPO4+mc_NaH2PO4_2H2O/MW_NaH2PO4_2H2O</f>
         <v>0.04000719577</v>
       </c>
@@ -14320,7 +14407,7 @@
       <c r="C36" s="19" t="s">
         <v>906</v>
       </c>
-      <c r="D36" s="62">
+      <c r="D36" s="149">
         <f>(2*mc_Na2HPO4/MW_Na2HPO4+mc_NaH2PO4_2H2O/MW_NaH2PO4_2H2O+2*mc_K2SO4/MW_K2SO4+2*mc_MgSO4_7H2O/MW_MgSO4_7H2O+2*mc_CaSO4_2H2O/MW_CaSO4_2H2O)-2*(mc_NH42SO4/MW_NH42SO4+mc_MgSO4_7H2O/MW_MgSO4_7H2O+mc_K2SO4/MW_K2SO4+mc_CaSO4_2H2O/MW_CaSO4_2H2O)</f>
         <v>0.046127523207</v>
       </c>
@@ -14338,7 +14425,7 @@
       <c r="C37" s="19" t="s">
         <v>910</v>
       </c>
-      <c r="D37" s="62">
+      <c r="D37" s="149">
         <f>2*mc_NH42SO4/MW_NH42SO4</f>
         <v>0.014272741032</v>
       </c>
@@ -14356,7 +14443,7 @@
       <c r="C38" s="19" t="s">
         <v>914</v>
       </c>
-      <c r="D38" s="62">
+      <c r="D38" s="149">
         <f>0</f>
         <v>0.0</v>
       </c>
@@ -14374,7 +14461,7 @@
       <c r="C39" s="19" t="s">
         <v>918</v>
       </c>
-      <c r="D39" s="62">
+      <c r="D39" s="149">
         <f>udg_KH2PO4/MW_KH2PO4+udg_Na2HPO4/MW_Na2HPO4</f>
         <v>0.037329366919</v>
       </c>
@@ -14392,7 +14479,7 @@
       <c r="C40" s="19" t="s">
         <v>922</v>
       </c>
-      <c r="D40" s="62">
+      <c r="D40" s="149">
         <f>(udg_NaHCO3/MW_NaHCO3+2*udg_Na2HPO4/MW_Na2HPO4+udg_KH2PO4/MW_KH2PO4+2*udg_MgSO4_7H2O/MW_MgSO4_7H2O+2*udg_CaCl2/MW_CaCl2)-(2*(udg_NH42SO4/MW_NH42SO4+udg_MgSO4_7H2O/MW_MgSO4_7H2O)+2*udg_CaCl2/MW_CaCl2)</f>
         <v>0.063142947676</v>
       </c>
@@ -14410,7 +14497,7 @@
       <c r="C41" s="19" t="s">
         <v>926</v>
       </c>
-      <c r="D41" s="62">
+      <c r="D41" s="149">
         <f>2*udg_NH42SO4/MW_NH42SO4</f>
         <v>0.007113667323</v>
       </c>
@@ -14428,7 +14515,7 @@
       <c r="C42" s="19" t="s">
         <v>930</v>
       </c>
-      <c r="D42" s="62">
+      <c r="D42" s="149">
         <f>2*udg_CaCl2/MW_CaCl2</f>
         <v>0.0001802126509281</v>
       </c>
@@ -14446,7 +14533,7 @@
       <c r="C44" s="19" t="s">
         <v>934</v>
       </c>
-      <c r="D44" s="62">
+      <c r="D44" s="149">
         <f>IF(Summary!$D$5="MC02",SID_mc02,IF(Summary!$D$5="UdG phosphate",SID_udg,NA()))</f>
         <v>0.063142947676</v>
       </c>
@@ -14464,7 +14551,7 @@
       <c r="C45" s="19" t="s">
         <v>938</v>
       </c>
-      <c r="D45" s="62">
+      <c r="D45" s="149">
         <f>IF(Summary!$D$5="MC02",PT_mc02,IF(Summary!$D$5="UdG phosphate",PT_udg,NA()))</f>
         <v>0.037329366919</v>
       </c>
@@ -14482,7 +14569,7 @@
       <c r="C46" s="19" t="s">
         <v>942</v>
       </c>
-      <c r="D46" s="62">
+      <c r="D46" s="149">
         <f>IF(Summary!$D$5="MC02",NT_mc02,IF(Summary!$D$5="UdG phosphate",NT_udg,NA()))</f>
         <v>0.007113667323</v>
       </c>
@@ -14500,7 +14587,7 @@
       <c r="C47" s="19" t="s">
         <v>946</v>
       </c>
-      <c r="D47" s="62">
+      <c r="D47" s="149">
         <f>IF(Summary!$D$5="MC02",Cl_mc02,IF(Summary!$D$5="UdG phosphate",Cl_udg,NA()))</f>
         <v>0.0001802126509281</v>
       </c>
@@ -15215,7 +15302,7 @@
       <c r="C103" s="19" t="s">
         <v>952</v>
       </c>
-      <c r="D103" s="62">
+      <c r="D103" s="149">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
         <v>6.494284837612</v>
       </c>
@@ -15238,7 +15325,7 @@
       <c r="C104" s="19" t="s">
         <v>956</v>
       </c>
-      <c r="D104" s="62">
+      <c r="D104" s="149">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
         <v>0.870210730329</v>
       </c>
@@ -15256,7 +15343,7 @@
       <c r="C105" s="19" t="s">
         <v>1005</v>
       </c>
-      <c r="D105" s="62">
+      <c r="D105" s="149">
         <f>SUMPRODUCT((B50:B99&gt;=0)*(B51:B100&lt;0))</f>
         <v>1.0</v>
       </c>
@@ -15283,7 +15370,7 @@
       <c r="C107" s="19" t="s">
         <v>959</v>
       </c>
-      <c r="D107" s="62">
+      <c r="D107" s="149">
         <f>Iappc/(2*Fcc)*M_HOCl*3600/VLc</f>
         <v>371.244905447914</v>
       </c>
@@ -15306,7 +15393,7 @@
       <c r="C108" s="19" t="s">
         <v>962</v>
       </c>
-      <c r="D108" s="62">
+      <c r="D108" s="149">
         <f>1/(bleach_rate)*60</f>
         <v>0.161618379457</v>
       </c>
@@ -15430,7 +15517,7 @@
       <c r="C125" s="19" t="s">
         <v>985</v>
       </c>
-      <c r="D125" s="62">
+      <c r="D125" s="149">
         <f>pH_Cl*pH_fHOCl*M_HOCl</f>
         <v>8.22693366608</v>
       </c>
@@ -15453,7 +15540,7 @@
       <c r="C128" s="19" t="s">
         <v>1067</v>
       </c>
-      <c r="D128" s="52">
+      <c r="D128" s="146">
         <v>0.5</v>
       </c>
       <c r="E128" s="51" t="s">
@@ -15470,7 +15557,7 @@
       <c r="C129" s="19" t="s">
         <v>1070</v>
       </c>
-      <c r="D129" s="52">
+      <c r="D129" s="146">
         <v>4.0499999999999998E-3</v>
       </c>
       <c r="E129" s="51" t="s">
@@ -15487,7 +15574,7 @@
       <c r="C130" s="19" t="s">
         <v>1073</v>
       </c>
-      <c r="D130" s="22">
+      <c r="D130" s="141">
         <f>Electrochemistry!$D$46</f>
         <v>2.01337839464</v>
       </c>
@@ -15505,7 +15592,7 @@
       <c r="C131" s="19" t="s">
         <v>1076</v>
       </c>
-      <c r="D131" s="62">
+      <c r="D131" s="149">
         <f>Iappc*FE_CER</f>
         <v>0.002845</v>
       </c>
@@ -15523,7 +15610,7 @@
       <c r="C132" s="19" t="s">
         <v>1076</v>
       </c>
-      <c r="D132" s="62">
+      <c r="D132" s="149">
         <f>Fcc*km_Cl*(pH_Cl/1000)*A_anode</f>
         <v>0.0001417839262056</v>
       </c>
@@ -15543,7 +15630,7 @@
       <c r="C133" s="19" t="s">
         <v>1076</v>
       </c>
-      <c r="D133" s="62">
+      <c r="D133" s="149">
         <f>MIN(I_Cl_FE,I_Cl_mt)</f>
         <v>0.0001417839262056</v>
       </c>
@@ -15561,7 +15648,7 @@
       <c r="C134" s="19" t="s">
         <v>1085</v>
       </c>
-      <c r="D134" s="62">
+      <c r="D134" s="149">
         <f>I_Cl/(n_e_Cl*Fcc*VLc)</f>
         <v>4.898289480563e-08</v>
       </c>
@@ -15579,7 +15666,7 @@
       <c r="C135" s="19" t="s">
         <v>1088</v>
       </c>
-      <c r="D135" s="62">
+      <c r="D135" s="149">
         <f>pH_NT*MW_N</f>
         <v>99.641138186772</v>
       </c>
@@ -15597,7 +15684,7 @@
       <c r="C136" s="19" t="s">
         <v>1092</v>
       </c>
-      <c r="D136" s="52">
+      <c r="D136" s="146">
         <v>4200000</v>
       </c>
       <c r="E136" s="51" t="s">
@@ -15614,7 +15701,7 @@
       <c r="C137" s="19" t="s">
         <v>1067</v>
       </c>
-      <c r="D137" s="52">
+      <c r="D137" s="148">
         <f>-LOG10(Ka_NH4)</f>
         <v>9.251811972994</v>
       </c>
@@ -15632,7 +15719,7 @@
       <c r="C138" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D138" s="62">
+      <c r="D138" s="149">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
         <v>1.241103645704e-05</v>
       </c>
@@ -15650,7 +15737,7 @@
       <c r="C139" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D139" s="62">
+      <c r="D139" s="149">
         <f>P_HOCl/(k1_NH2Cl*NH3_free)</f>
         <v>9.396954107506e-10</v>
       </c>
@@ -15668,7 +15755,7 @@
       <c r="C140" s="19" t="s">
         <v>1088</v>
       </c>
-      <c r="D140" s="62">
+      <c r="D140" s="149">
         <f>HOCl_ss*M_HOCl</f>
         <v>4.929642124798e-05</v>
       </c>
@@ -15686,7 +15773,7 @@
       <c r="C141" s="19" t="s">
         <v>1067</v>
       </c>
-      <c r="D141" s="52">
+      <c r="D141" s="146">
         <v>10</v>
       </c>
       <c r="E141" s="51" t="s">
@@ -15703,7 +15790,7 @@
       <c r="C142" s="19" t="s">
         <v>1111</v>
       </c>
-      <c r="D142" s="52">
+      <c r="D142" s="146">
         <v>1</v>
       </c>
       <c r="E142" s="51" t="s">
@@ -15720,7 +15807,7 @@
       <c r="C143" s="19" t="s">
         <v>1088</v>
       </c>
-      <c r="D143" s="62">
+      <c r="D143" s="149">
         <f>MIN(P_HOCl*tau_NH2Cl*3600*M_HOCl,cl_per_N*NH3_N,Cl_pool_mgL)</f>
         <v>9.250713581411</v>
       </c>
@@ -15738,7 +15825,7 @@
       <c r="C144" s="19" t="s">
         <v>1067</v>
       </c>
-      <c r="D144" s="52">
+      <c r="D144" s="146">
         <v>25</v>
       </c>
       <c r="E144" s="51" t="s">
@@ -15755,7 +15842,7 @@
       <c r="C145" s="19" t="s">
         <v>1088</v>
       </c>
-      <c r="D145" s="62">
+      <c r="D145" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_mgL/R_chloramine</f>
         <v>0.370521507469</v>
       </c>
@@ -15773,7 +15860,7 @@
       <c r="C146" s="19" t="s">
         <v>1088</v>
       </c>
-      <c r="D146" s="52">
+      <c r="D146" s="146">
         <v>0.1</v>
       </c>
       <c r="E146" s="51" t="s">
@@ -15790,7 +15877,7 @@
       <c r="C147" s="19" t="s">
         <v>1088</v>
       </c>
-      <c r="D147" s="52">
+      <c r="D147" s="146">
         <v>2</v>
       </c>
       <c r="E147" s="51" t="s">
@@ -15807,7 +15894,7 @@
       <c r="C148" s="19" t="s">
         <v>1215</v>
       </c>
-      <c r="D148" s="62">
+      <c r="D148" s="149">
         <f>2</f>
         <v>2.0</v>
       </c>
@@ -15825,7 +15912,7 @@
       <c r="C149" s="19" t="s">
         <v>1218</v>
       </c>
-      <c r="D149" s="62">
+      <c r="D149" s="149">
         <f>pH_Cl*M_HOCl</f>
         <v>9.453955667688</v>
       </c>
@@ -15843,7 +15930,7 @@
       <c r="C150" s="19" t="s">
         <v>1222</v>
       </c>
-      <c r="D150" s="52">
+      <c r="D150" s="146">
         <v>1.6666666666666666E-2</v>
       </c>
       <c r="E150" s="75" t="s">
@@ -15860,7 +15947,7 @@
       <c r="C151" s="19" t="s">
         <v>1226</v>
       </c>
-      <c r="D151" s="52">
+      <c r="D151" s="146">
         <v>5</v>
       </c>
       <c r="E151" s="75" t="s">
@@ -15877,7 +15964,7 @@
       <c r="C152" s="19" t="s">
         <v>1230</v>
       </c>
-      <c r="D152" s="52">
+      <c r="D152" s="146">
         <v>18</v>
       </c>
       <c r="E152" s="75" t="s">
@@ -15894,7 +15981,7 @@
       <c r="C153" s="19" t="s">
         <v>1234</v>
       </c>
-      <c r="D153" s="52">
+      <c r="D153" s="146">
         <v>70</v>
       </c>
       <c r="E153" s="75" t="s">
@@ -15911,7 +15998,7 @@
       <c r="C154" s="19" t="s">
         <v>1238</v>
       </c>
-      <c r="D154" s="62">
+      <c r="D154" s="149">
         <f>MIN(P_HOCl*tau_NH2Cl_lo*3600*M_HOCl,cl_per_N*NH3_N,Cl_pool_mgL)</f>
         <v>0.15417855969</v>
       </c>
@@ -15929,7 +16016,7 @@
       <c r="C155" s="19" t="s">
         <v>1242</v>
       </c>
-      <c r="D155" s="62">
+      <c r="D155" s="149">
         <f>MIN(P_HOCl*tau_NH2Cl_hi*3600*M_HOCl,cl_per_N*NH3_N,Cl_pool_mgL)</f>
         <v>9.453955667688</v>
       </c>
@@ -15947,7 +16034,7 @@
       <c r="C156" s="19" t="s">
         <v>1246</v>
       </c>
-      <c r="D156" s="62">
+      <c r="D156" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_lo/R_chloramine_hi</f>
         <v>0.002695515065</v>
       </c>
@@ -15965,7 +16052,7 @@
       <c r="C157" s="19" t="s">
         <v>1250</v>
       </c>
-      <c r="D157" s="62">
+      <c r="D157" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_hi/R_chloramine_lo</f>
         <v>0.525712723528</v>
       </c>
@@ -15998,7 +16085,7 @@
       <c r="C159" s="19" t="s">
         <v>1258</v>
       </c>
-      <c r="D159" s="52">
+      <c r="D159" s="146">
         <v>63.55</v>
       </c>
       <c r="E159" s="51" t="s">
@@ -16015,7 +16102,7 @@
       <c r="C160" s="19" t="s">
         <v>1262</v>
       </c>
-      <c r="D160" s="52">
+      <c r="D160" s="146">
         <v>2</v>
       </c>
       <c r="E160" s="51" t="s">
@@ -16032,7 +16119,7 @@
       <c r="C161" s="19" t="s">
         <v>1266</v>
       </c>
-      <c r="D161" s="62" t="e">
+      <c r="D161" s="149" t="e">
         <f>IF(ISNUMBER(corr_I_frac),corr_I_frac*Iappc/(metal_z*Fcc)*metal_MW*1000*3600/VLc,NA())</f>
         <v>#N/A</v>
       </c>
@@ -16050,7 +16137,7 @@
       <c r="C162" s="19" t="s">
         <v>1270</v>
       </c>
-      <c r="D162" s="52">
+      <c r="D162" s="146">
         <v>0.5</v>
       </c>
       <c r="E162" s="51" t="s">
@@ -16090,7 +16177,7 @@
       <c r="C166" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D166" s="52">
+      <c r="D166" s="146">
         <v>50.08</v>
       </c>
       <c r="E166" s="99" t="s">
@@ -16107,7 +16194,7 @@
       <c r="C167" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D167" s="52">
+      <c r="D167" s="146">
         <v>73.48</v>
       </c>
       <c r="E167" s="99" t="s">
@@ -16124,7 +16211,7 @@
       <c r="C168" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D168" s="52">
+      <c r="D168" s="146">
         <v>73.5</v>
       </c>
       <c r="E168" s="99" t="s">
@@ -16141,7 +16228,7 @@
       <c r="C169" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D169" s="52">
+      <c r="D169" s="146">
         <v>106</v>
       </c>
       <c r="E169" s="99" t="s">
@@ -16158,7 +16245,7 @@
       <c r="C170" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D170" s="52">
+      <c r="D170" s="146">
         <v>118.94</v>
       </c>
       <c r="E170" s="99" t="s">
@@ -16175,7 +16262,7 @@
       <c r="C171" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D171" s="52">
+      <c r="D171" s="146">
         <v>36</v>
       </c>
       <c r="E171" s="99" t="s">
@@ -16192,7 +16279,7 @@
       <c r="C172" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D172" s="52">
+      <c r="D172" s="146">
         <v>114</v>
       </c>
       <c r="E172" s="99" t="s">
@@ -16209,7 +16296,7 @@
       <c r="C173" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D173" s="52">
+      <c r="D173" s="146">
         <v>160</v>
       </c>
       <c r="E173" s="99" t="s">
@@ -16226,7 +16313,7 @@
       <c r="C174" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D174" s="52">
+      <c r="D174" s="146">
         <v>44.5</v>
       </c>
       <c r="E174" s="99" t="s">
@@ -16243,7 +16330,7 @@
       <c r="C175" s="19" t="s">
         <v>1485</v>
       </c>
-      <c r="D175" s="52">
+      <c r="D175" s="146">
         <v>76.31</v>
       </c>
       <c r="E175" s="99" t="s">
@@ -16260,7 +16347,7 @@
       <c r="C176" s="19" t="s">
         <v>1507</v>
       </c>
-      <c r="D176" s="22">
+      <c r="D176" s="141">
         <f>(2*mc_Na2HPO4/MW_Na2HPO4*lam_Na+mc_NaH2PO4_2H2O/MW_NaH2PO4_2H2O*lam_Na+2*mc_K2SO4/MW_K2SO4*lam_K+2*mc_NH42SO4/MW_NH42SO4*lam_NH4+mc_MgSO4_7H2O/MW_MgSO4_7H2O*lam_Mg+mc_CaSO4_2H2O/MW_CaSO4_2H2O*lam_Ca+mc_Na2HPO4/MW_Na2HPO4*lam_HPO4+mc_NaH2PO4_2H2O/MW_NaH2PO4_2H2O*lam_H2PO4+(mc_K2SO4/MW_K2SO4+mc_MgSO4_7H2O/MW_MgSO4_7H2O+mc_CaSO4_2H2O/MW_CaSO4_2H2O+mc_NH42SO4/MW_NH42SO4)*lam_SO4)/10</f>
         <v>0.956659526802</v>
       </c>
@@ -16278,7 +16365,7 @@
       <c r="C177" s="19" t="s">
         <v>1507</v>
       </c>
-      <c r="D177" s="22">
+      <c r="D177" s="141">
         <f>((udg_NaHCO3/MW_NaHCO3+2*udg_Na2HPO4/MW_Na2HPO4)*lam_Na+udg_KH2PO4/MW_KH2PO4*lam_K+2*udg_NH42SO4/MW_NH42SO4*lam_NH4+udg_MgSO4_7H2O/MW_MgSO4_7H2O*lam_Mg+udg_CaCl2/MW_CaCl2*lam_Ca+udg_Na2HPO4/MW_Na2HPO4*lam_HPO4+udg_KH2PO4/MW_KH2PO4*lam_H2PO4+(udg_MgSO4_7H2O/MW_MgSO4_7H2O+udg_NH42SO4/MW_NH42SO4)*lam_SO4+udg_NaHCO3/MW_NaHCO3*lam_HCO3+2*udg_CaCl2/MW_CaCl2*lam_Cl)/10</f>
         <v>0.90634186802</v>
       </c>
@@ -16296,7 +16383,7 @@
       <c r="C178" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D178" s="52">
+      <c r="D178" s="146">
         <v>0.78</v>
       </c>
       <c r="E178" s="75" t="s">
@@ -16313,7 +16400,7 @@
       <c r="C179" s="19" t="s">
         <v>1517</v>
       </c>
-      <c r="D179" s="52">
+      <c r="D179" s="146">
         <v>0.02</v>
       </c>
       <c r="E179" s="67" t="s">
@@ -16330,7 +16417,7 @@
       <c r="C180" s="19" t="s">
         <v>1507</v>
       </c>
-      <c r="D180" s="22">
+      <c r="D180" s="141">
         <f>IF(Summary!$D$5="MC02",kappa0_mc02,IF(Summary!$D$5="UdG phosphate",kappa0_udg,NA()))*kappa_fI*(1+kappa_TC*(TKc-T_ref))</f>
         <v>0.706946657056</v>
       </c>
@@ -16353,7 +16440,7 @@
       <c r="C183" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D183" s="22">
+      <c r="D183" s="141">
         <f>0.5*(2*mc_Na2HPO4/MW_Na2HPO4+mc_NaH2PO4_2H2O/MW_NaH2PO4_2H2O+2*mc_K2SO4/MW_K2SO4+2*mc_NH42SO4/MW_NH42SO4+4*mc_MgSO4_7H2O/MW_MgSO4_7H2O+4*mc_CaSO4_2H2O/MW_CaSO4_2H2O+mc_NaH2PO4_2H2O/MW_NaH2PO4_2H2O+4*mc_Na2HPO4/MW_Na2HPO4+4*(mc_K2SO4/MW_K2SO4+mc_MgSO4_7H2O/MW_MgSO4_7H2O+mc_CaSO4_2H2O/MW_CaSO4_2H2O+mc_NH42SO4/MW_NH42SO4))</f>
         <v>0.120365489933</v>
       </c>
@@ -16371,7 +16458,7 @@
       <c r="C184" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D184" s="22">
+      <c r="D184" s="141">
         <f>0.5*((udg_NaHCO3/MW_NaHCO3+2*udg_Na2HPO4/MW_Na2HPO4)+udg_KH2PO4/MW_KH2PO4+2*udg_NH42SO4/MW_NH42SO4+4*udg_MgSO4_7H2O/MW_MgSO4_7H2O+4*udg_CaCl2/MW_CaCl2+udg_KH2PO4/MW_KH2PO4+4*udg_Na2HPO4/MW_Na2HPO4+4*(udg_MgSO4_7H2O/MW_MgSO4_7H2O+udg_NH42SO4/MW_NH42SO4)+udg_NaHCO3/MW_NaHCO3+2*udg_CaCl2/MW_CaCl2)</f>
         <v>0.109739973238</v>
       </c>
@@ -16389,7 +16476,7 @@
       <c r="C185" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D185" s="22">
+      <c r="D185" s="141">
         <f>IF(Summary!$D$5="MC02",I_mc02,IF(Summary!$D$5="UdG phosphate",I_udg,NA()))</f>
         <v>0.109739973238</v>
       </c>
@@ -16407,7 +16494,7 @@
       <c r="C186" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D186" s="22">
+      <c r="D186" s="141">
         <f>DH_const*(eps_water_298*(T_ref/TKc)^eps_T_exp)^-1.5*TKc^-1.5</f>
         <v>0.507905390447</v>
       </c>
@@ -16425,7 +16512,7 @@
       <c r="C187" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D187" s="22">
+      <c r="D187" s="141">
         <f>10^(-A_DH*1*(SQRT(I_ionic)/(1+SQRT(I_ionic))-davies_c*I_ionic))</f>
         <v>0.776846550354</v>
       </c>
@@ -16443,7 +16530,7 @@
       <c r="C188" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D188" s="22">
+      <c r="D188" s="141">
         <f>10^(-A_DH*4*(SQRT(I_ionic)/(1+SQRT(I_ionic))-davies_c*I_ionic))</f>
         <v>0.364200859384</v>
       </c>
@@ -16461,7 +16548,7 @@
       <c r="C189" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D189" s="22">
+      <c r="D189" s="141">
         <f>10^(-A_DH*9*(SQRT(I_ionic)/(1+SQRT(I_ionic))-davies_c*I_ionic))</f>
         <v>0.103042686755</v>
       </c>
@@ -16479,7 +16566,7 @@
       <c r="C190" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D190" s="22">
+      <c r="D190" s="141">
         <f>Ka1c/gamma_1^2</f>
         <v>7.373768993803e-07</v>
       </c>
@@ -16497,7 +16584,7 @@
       <c r="C191" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D191" s="22">
+      <c r="D191" s="141">
         <f>Ka2c/gamma_2</f>
         <v>1.287750942688e-10</v>
       </c>
@@ -16515,7 +16602,7 @@
       <c r="C192" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D192" s="22">
+      <c r="D192" s="141">
         <f>Ka1p/gamma_1^2</f>
         <v>0.011764889855</v>
       </c>
@@ -16533,7 +16620,7 @@
       <c r="C193" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D193" s="22">
+      <c r="D193" s="141">
         <f>Ka2p/gamma_2</f>
         <v>1.732560436751e-07</v>
       </c>
@@ -16551,7 +16638,7 @@
       <c r="C194" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D194" s="22">
+      <c r="D194" s="141">
         <f>Ka3p*gamma_2/(gamma_1*gamma_3)</f>
         <v>1.910899474681e-12</v>
       </c>
@@ -16569,7 +16656,7 @@
       <c r="C195" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D195" s="22">
+      <c r="D195" s="141">
         <f>Kw_w/gamma_1^2</f>
         <v>1.65702674018e-14</v>
       </c>
@@ -16587,7 +16674,7 @@
       <c r="C196" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D196" s="22">
+      <c r="D196" s="141">
         <f>Ka_HOCl/gamma_1^2</f>
         <v>4.778917320203e-08</v>
       </c>
@@ -16605,7 +16692,7 @@
       <c r="C197" s="19" t="s">
         <v>1098</v>
       </c>
-      <c r="D197" s="22">
+      <c r="D197" s="141">
         <f>Ka_NH4</f>
         <v>5.6e-10</v>
       </c>
@@ -16628,7 +16715,7 @@
       <c r="C200" s="19" t="s">
         <v>1567</v>
       </c>
-      <c r="D200" s="22">
+      <c r="D200" s="141">
         <f>R_gas*TKc/Fcc*LN(10)</f>
         <v>0.059159349686</v>
       </c>
@@ -16646,7 +16733,7 @@
       <c r="C201" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D201" s="52">
+      <c r="D201" s="146">
         <v>1.2290000000000001</v>
       </c>
       <c r="E201" s="99" t="s">
@@ -16663,7 +16750,7 @@
       <c r="C202" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D202" s="52">
+      <c r="D202" s="146">
         <v>0</v>
       </c>
       <c r="E202" s="99" t="s">
@@ -16680,7 +16767,7 @@
       <c r="C203" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D203" s="52">
+      <c r="D203" s="146">
         <v>1.3580000000000001</v>
       </c>
       <c r="E203" s="99" t="s">
@@ -16697,7 +16784,7 @@
       <c r="C204" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D204" s="52">
+      <c r="D204" s="146">
         <v>0.69499999999999995</v>
       </c>
       <c r="E204" s="99" t="s">
@@ -16714,7 +16801,7 @@
       <c r="C205" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D205" s="52">
+      <c r="D205" s="146">
         <v>0.34189999999999998</v>
       </c>
       <c r="E205" s="99" t="s">
@@ -16731,7 +16818,7 @@
       <c r="C206" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D206" s="22">
+      <c r="D206" s="141">
         <f>E0_OER-nernst_slope*pH_meas</f>
         <v>0.83831463654</v>
       </c>
@@ -16749,7 +16836,7 @@
       <c r="C207" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D207" s="22">
+      <c r="D207" s="141">
         <f>E0_HER-nernst_slope*pH_meas</f>
         <v>-0.39068536346</v>
       </c>
@@ -16769,7 +16856,7 @@
       <c r="C208" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D208" s="22">
+      <c r="D208" s="141">
         <f>E0_Cl2+nernst_slope*(-LOG10(MAX(pH_Cl,Cl_floor_molL)))</f>
         <v>1.579505308204</v>
       </c>
@@ -16789,7 +16876,7 @@
       <c r="C209" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D209" s="22">
+      <c r="D209" s="141">
         <f>E_HOCl_Cl-E_anode_op</f>
         <v>-0.422483519032</v>
       </c>
@@ -16809,7 +16896,7 @@
       <c r="C210" s="19" t="s">
         <v>1571</v>
       </c>
-      <c r="D210" s="22">
+      <c r="D210" s="141">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
         <v>0.30431463654</v>
       </c>
@@ -16829,7 +16916,7 @@
       <c r="C211" s="19" t="s">
         <v>1595</v>
       </c>
-      <c r="D211" s="22">
+      <c r="D211" s="141">
         <f>E_anode_op-E0_Cu</f>
         <v>1.240557060036</v>
       </c>
@@ -16852,7 +16939,7 @@
       <c r="C214" s="19" t="s">
         <v>577</v>
       </c>
-      <c r="D214" s="52">
+      <c r="D214" s="146">
         <v>7.5899999999999996E-10</v>
       </c>
       <c r="E214" s="99" t="s">
@@ -16869,7 +16956,7 @@
       <c r="C215" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D215" s="36">
+      <c r="D215" s="131">
         <v>40</v>
       </c>
       <c r="E215" s="75" t="s">
@@ -16886,7 +16973,7 @@
       <c r="C216" s="19" t="s">
         <v>1282</v>
       </c>
-      <c r="D216" s="22">
+      <c r="D216" s="141">
         <f>Fcc*(D_HPO4*HPO4_op+D_HCO3*HCO3_op)*1000/(delta_diff/1000000)/10</f>
         <v>8.049160263403</v>
       </c>
@@ -16906,7 +16993,7 @@
       <c r="C217" s="19" t="s">
         <v>1282</v>
       </c>
-      <c r="D217" s="22">
+      <c r="D217" s="141">
         <f>Electrochemistry!$D$48</f>
         <v>2.826095688296</v>
       </c>
@@ -16924,7 +17011,7 @@
       <c r="C218" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D218" s="22">
+      <c r="D218" s="141">
         <f>j_anode_c/j_buffer_lim</f>
         <v>0.35110441286</v>
       </c>
@@ -16942,7 +17029,7 @@
       <c r="C219" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D219" s="22" t="str">
+      <c r="D219" s="141" t="str">
         <f>IF(j_buffer_ratio&gt;1,"BUFFER EXCEEDED — anode surface acidifies (local pH ~1 unit below bulk); the pH solved above is the bulk value only",IF(j_buffer_ratio&gt;buffer_caution_frac,"watch — running at "&amp;TEXT(j_buffer_ratio,"0%")&amp;" of the phosphate buffer limit; expect a 0.4–1.0 unit excursion at each electrode surface","OK — buffer holds the electrode surfaces at the bulk pH"))</f>
         <v>OK — buffer holds the electrode surfaces at the bulk pH</v>
       </c>
@@ -16960,7 +17047,7 @@
       <c r="C220" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D220" s="22">
+      <c r="D220" s="141">
         <f>pH_op-LOG10(gamma_1)</f>
         <v>6.603949596052</v>
       </c>
@@ -16985,7 +17072,7 @@
       <c r="C222" s="19" t="s">
         <v>1885</v>
       </c>
-      <c r="D222" s="52">
+      <c r="D222" s="146">
         <v>52460</v>
       </c>
       <c r="E222" s="99" t="s">
@@ -17002,7 +17089,7 @@
       <c r="C223" s="19" t="s">
         <v>1885</v>
       </c>
-      <c r="D223" s="52">
+      <c r="D223" s="146">
         <v>70906</v>
       </c>
       <c r="E223" s="99" t="s">
@@ -17019,7 +17106,7 @@
       <c r="C224" s="19" t="s">
         <v>1892</v>
       </c>
-      <c r="D224" s="52">
+      <c r="D224" s="146">
         <v>5.0599999999999996</v>
       </c>
       <c r="E224" s="67" t="s">
@@ -17036,7 +17123,7 @@
       <c r="C225" s="19" t="s">
         <v>1885</v>
       </c>
-      <c r="D225" s="52">
+      <c r="D225" s="146">
         <v>14007</v>
       </c>
       <c r="E225" s="99" t="s">
@@ -17053,7 +17140,7 @@
       <c r="C226" s="19" t="s">
         <v>1270</v>
       </c>
-      <c r="D226" s="22">
+      <c r="D226" s="141">
         <f>C_eff*M_Cl2/M_HOCl</f>
         <v>0.500804384457</v>
       </c>
@@ -17084,7 +17171,7 @@
           <t xml:space="preserve">K</t>
         </is>
       </c>
-      <c r="D229" s="22">
+      <c r="D229" s="141">
         <f>Biology!$D$23</f>
         <v>298.15</v>
       </c>
@@ -17110,7 +17197,7 @@
           <t xml:space="preserve">K^1.5</t>
         </is>
       </c>
-      <c r="D230" s="36">
+      <c r="D230" s="131">
         <v>1820000</v>
       </c>
       <c r="E230" s="84" t="inlineStr">
@@ -17135,7 +17222,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D231" s="36">
+      <c r="D231" s="131">
         <v>78.54</v>
       </c>
       <c r="E231" s="84" t="inlineStr">
@@ -17160,7 +17247,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D232" s="36">
+      <c r="D232" s="131">
         <v>1.368</v>
       </c>
       <c r="E232" s="67" t="inlineStr">
@@ -17185,7 +17272,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D233" s="36">
+      <c r="D233" s="131">
         <v>0.3</v>
       </c>
       <c r="E233" s="84" t="inlineStr">
@@ -17210,7 +17297,7 @@
           <t xml:space="preserve">mol/L</t>
         </is>
       </c>
-      <c r="D234" s="36">
+      <c r="D234" s="131">
         <v>1e-12</v>
       </c>
       <c r="E234" s="84" t="inlineStr">
@@ -17235,7 +17322,7 @@
           <t xml:space="preserve">pH</t>
         </is>
       </c>
-      <c r="D235" s="36">
+      <c r="D235" s="131">
         <v>0.1</v>
       </c>
       <c r="E235" s="84" t="inlineStr">
@@ -17260,7 +17347,7 @@
           <t xml:space="preserve">pH</t>
         </is>
       </c>
-      <c r="D236" s="36">
+      <c r="D236" s="131">
         <v>6.5</v>
       </c>
       <c r="E236" s="67" t="inlineStr">
@@ -17285,7 +17372,7 @@
           <t xml:space="preserve">pH</t>
         </is>
       </c>
-      <c r="D237" s="36">
+      <c r="D237" s="131">
         <v>7.5</v>
       </c>
       <c r="E237" s="67" t="inlineStr">
@@ -17310,7 +17397,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D238" s="36">
+      <c r="D238" s="131">
         <v>0.5</v>
       </c>
       <c r="E238" s="75" t="inlineStr">
@@ -17342,7 +17429,7 @@
           <t xml:space="preserve">m²/s</t>
         </is>
       </c>
-      <c r="D251" s="52">
+      <c r="D251" s="146">
         <v>1.185e-09</v>
       </c>
       <c r="E251" s="99" t="inlineStr">
@@ -17367,7 +17454,7 @@
           <t xml:space="preserve">mol/L</t>
         </is>
       </c>
-      <c r="D252" s="22">
+      <c r="D252" s="141">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
         <v>0.01976870305</v>
       </c>
@@ -17393,7 +17480,7 @@
           <t xml:space="preserve">mol/L</t>
         </is>
       </c>
-      <c r="D253" s="22">
+      <c r="D253" s="141">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
         <v>0.013100861499</v>
       </c>
@@ -17419,7 +17506,7 @@
           <t xml:space="preserve">V</t>
         </is>
       </c>
-      <c r="D254" s="22">
+      <c r="D254" s="141">
         <f>Electrochemistry!$D$111</f>
         <v>0.894142423496</v>
       </c>
@@ -17445,7 +17532,7 @@
           <t xml:space="preserve">V</t>
         </is>
       </c>
-      <c r="D255" s="22">
+      <c r="D255" s="141">
         <f>Electrochemistry!$D$113</f>
         <v>-0.15</v>
       </c>
@@ -17471,7 +17558,7 @@
           <t xml:space="preserve">V vs SHE</t>
         </is>
       </c>
-      <c r="D256" s="22">
+      <c r="D256" s="141">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
         <v>1.582457060036</v>
       </c>
@@ -17497,7 +17584,7 @@
           <t xml:space="preserve">V</t>
         </is>
       </c>
-      <c r="D257" s="52">
+      <c r="D257" s="146">
         <v>1.482</v>
       </c>
       <c r="E257" s="99" t="inlineStr">
@@ -17522,7 +17609,7 @@
           <t xml:space="preserve">V vs SHE</t>
         </is>
       </c>
-      <c r="D258" s="22">
+      <c r="D258" s="141">
         <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,1E-12))-pH_meas-LOG10(MAX(pH_Cl,1E-12)))</f>
         <v>1.159973541004</v>
       </c>
@@ -17548,7 +17635,7 @@
           <t xml:space="preserve">mg/L</t>
         </is>
       </c>
-      <c r="D259" s="22">
+      <c r="D259" s="141">
         <f>C_eff_lo*M_Cl2/M_HOCl</f>
         <v>0.003643312833</v>
       </c>
@@ -17574,7 +17661,7 @@
           <t xml:space="preserve">mg/L</t>
         </is>
       </c>
-      <c r="D260" s="22">
+      <c r="D260" s="141">
         <f>C_eff_hi*M_Cl2/M_HOCl</f>
         <v>0.710563979689</v>
       </c>
@@ -17663,11 +17750,11 @@
       <c r="C4" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="D4" s="27">
+      <c r="D4" s="150">
         <f>Electrochemistry!$D$21</f>
         <v>0.000103759833633</v>
       </c>
-      <c r="E4" s="23" t="str">
+      <c r="E4" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D21","→ Electrochemistry")</f>
         <v>→ Electrochemistry</v>
       </c>
@@ -17683,11 +17770,11 @@
       <c r="C5" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="150">
         <f>Electrochemistry!$D$29</f>
         <v>4.936187056172e-05</v>
       </c>
-      <c r="E5" s="23" t="str">
+      <c r="E5" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
         <v>→ Electrochemistry</v>
       </c>
@@ -17703,11 +17790,11 @@
       <c r="C6" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="151">
         <f>Geometry!$D$41</f>
         <v>15.0</v>
       </c>
-      <c r="E6" s="23" t="str">
+      <c r="E6" s="135" t="str">
         <f>HYPERLINK("#Geometry!D41","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
@@ -17721,11 +17808,11 @@
         <v>38</v>
       </c>
       <c r="C7" s="20"/>
-      <c r="D7" s="38" t="str">
+      <c r="D7" s="134" t="str">
         <f>Summary!$D$4</f>
         <v>UdG (mixed)</v>
       </c>
-      <c r="E7" s="23" t="str">
+      <c r="E7" s="135" t="str">
         <f>HYPERLINK("#Summary!D4","→ Summary")</f>
         <v>→ Summary</v>
       </c>
@@ -17767,7 +17854,7 @@
       <c r="C10" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D10" s="105">
+      <c r="D10" s="58">
         <f>IF(ISNUMBER(cal_knall_H2),cal_knall_H2,knall_H2_default)</f>
         <v>6.0</v>
       </c>
@@ -17786,7 +17873,7 @@
       <c r="C11" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D11" s="105">
+      <c r="D11" s="58">
         <f>IF(ISNUMBER(cal_knall_O2),cal_knall_O2,knall_O2_default)</f>
         <v>2.0</v>
       </c>
@@ -17805,7 +17892,7 @@
       <c r="C12" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D12" s="105">
+      <c r="D12" s="58">
         <f>IF(ISNUMBER(cal_knall_CO2),cal_knall_CO2,knall_CO2_default)</f>
         <v>1.0</v>
       </c>
@@ -17900,7 +17987,7 @@
       <c r="C17" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="62">
+      <c r="D17" s="149">
         <f>Summary!$D$8</f>
         <v>25.0</v>
       </c>
@@ -17938,7 +18025,7 @@
       <c r="C19" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D19" s="63">
+      <c r="D19" s="134">
         <f>IF(P_atm_set&gt;0,P_atm_set,Pa_per_atm)</f>
         <v>101325.0</v>
       </c>
@@ -17957,7 +18044,7 @@
       <c r="C20" s="19" t="s">
         <v>436</v>
       </c>
-      <c r="D20" s="52">
+      <c r="D20" s="146">
         <v>101325</v>
       </c>
       <c r="E20" s="99" t="s">
@@ -17975,7 +18062,7 @@
       <c r="C21" s="19" t="s">
         <v>440</v>
       </c>
-      <c r="D21" s="52">
+      <c r="D21" s="146">
         <v>1.2E-5</v>
       </c>
       <c r="E21" s="51" t="s">
@@ -17993,7 +18080,7 @@
       <c r="C22" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="D22" s="52">
+      <c r="D22" s="146">
         <v>1500</v>
       </c>
       <c r="E22" s="51" t="s">
@@ -18011,7 +18098,7 @@
       <c r="C23" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="D23" s="52">
+      <c r="D23" s="146">
         <v>298.14999999999998</v>
       </c>
       <c r="E23" s="99" t="s">
@@ -18048,7 +18135,7 @@
       <c r="C25" s="19" t="s">
         <v>453</v>
       </c>
-      <c r="D25" s="52">
+      <c r="D25" s="146">
         <v>0.3</v>
       </c>
       <c r="E25" s="51" t="s">
@@ -18123,7 +18210,7 @@
       <c r="C29" s="19" t="s">
         <v>440</v>
       </c>
-      <c r="D29" s="66">
+      <c r="D29" s="152">
         <v>3.3E-4</v>
       </c>
       <c r="E29" s="67" t="s">
@@ -18141,7 +18228,7 @@
       <c r="C30" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="D30" s="66">
+      <c r="D30" s="152">
         <v>2400</v>
       </c>
       <c r="E30" s="67" t="s">
@@ -18216,7 +18303,7 @@
       <c r="C34" s="19" t="s">
         <v>463</v>
       </c>
-      <c r="D34" s="36">
+      <c r="D34" s="131">
         <v>50</v>
       </c>
       <c r="E34" s="69" t="s">
@@ -18253,7 +18340,7 @@
       <c r="C36" s="19" t="s">
         <v>487</v>
       </c>
-      <c r="D36" s="66">
+      <c r="D36" s="152">
         <v>4.4499999999999997E-7</v>
       </c>
       <c r="E36" s="67" t="s">
@@ -18290,7 +18377,7 @@
       <c r="C38" s="19" t="s">
         <v>440</v>
       </c>
-      <c r="D38" s="66">
+      <c r="D38" s="152">
         <v>7.7999999999999999E-6</v>
       </c>
       <c r="E38" s="67" t="s">
@@ -18308,7 +18395,7 @@
       <c r="C39" s="19" t="s">
         <v>309</v>
       </c>
-      <c r="D39" s="66">
+      <c r="D39" s="152">
         <v>500</v>
       </c>
       <c r="E39" s="67" t="s">
@@ -18429,7 +18516,7 @@
       <c r="C45" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="D45" s="71" t="e">
+      <c r="D45" s="32" t="e">
         <f>IF(ISNUMBER(cal_DO_min),cal_DO_min,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,2,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,2,FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
@@ -18446,7 +18533,7 @@
       <c r="C46" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="D46" s="24" t="e">
+      <c r="D46" s="28" t="e">
         <f>IF(ISNUMBER(cal_DO_opt),cal_DO_opt,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,3,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,3,FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
@@ -18463,7 +18550,7 @@
       <c r="C47" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="D47" s="24" t="e">
+      <c r="D47" s="28" t="e">
         <f>IF(ISNUMBER(cal_DO_impair),cal_DO_impair,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,4,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,4,FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
@@ -18480,7 +18567,7 @@
       <c r="C48" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="D48" s="24" t="e">
+      <c r="D48" s="28" t="e">
         <f>IF(ISNUMBER(cal_DO_toxic),cal_DO_toxic,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,5,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,5,FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
@@ -18670,7 +18757,7 @@
       <c r="C60" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D60" s="22">
+      <c r="D60" s="141">
         <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_toxic)),DO_opt/DO_toxic,DO_frac_fallback)</f>
         <v>0.226086956522</v>
       </c>
@@ -18688,7 +18775,7 @@
       <c r="C61" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D61" s="52">
+      <c r="D61" s="146">
         <v>0.22608695652173899</v>
       </c>
       <c r="E61" s="68" t="inlineStr">
@@ -18720,7 +18807,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D63" s="36">
+      <c r="D63" s="131">
         <v>6</v>
       </c>
       <c r="E63" s="61" t="inlineStr">
@@ -18745,7 +18832,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D64" s="36">
+      <c r="D64" s="131">
         <v>2</v>
       </c>
       <c r="E64" s="61" t="inlineStr">
@@ -18770,7 +18857,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D65" s="36">
+      <c r="D65" s="131">
         <v>1</v>
       </c>
       <c r="E65" s="61" t="inlineStr">
@@ -18795,7 +18882,7 @@
           <t xml:space="preserve">K</t>
         </is>
       </c>
-      <c r="D66" s="36">
+      <c r="D66" s="131">
         <v>273.15</v>
       </c>
       <c r="E66" s="99" t="inlineStr">
@@ -18820,11 +18907,11 @@
           <t xml:space="preserve">Pa</t>
         </is>
       </c>
-      <c r="D67" s="25">
+      <c r="D67" s="151">
         <f>Summary!$D$10</f>
         <v>0.0</v>
       </c>
-      <c r="E67" s="23" t="inlineStr">
+      <c r="E67" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Summary!D10 (blank reads as 0, so P_atm falls back to Pa_per_atm).</t>
         </is>
@@ -18853,11 +18940,11 @@
           <t xml:space="preserve">mol/h</t>
         </is>
       </c>
-      <c r="D76" s="27">
+      <c r="D76" s="150">
         <f>'Mass Transfer'!$D$100</f>
         <v>0.0003892277799716</v>
       </c>
-      <c r="E76" s="23" t="inlineStr">
+      <c r="E76" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D100 (schedule in use).</t>
         </is>
@@ -18879,11 +18966,11 @@
           <t xml:space="preserve">mol/h</t>
         </is>
       </c>
-      <c r="D77" s="27">
+      <c r="D77" s="150">
         <f>'Mass Transfer'!$D$178</f>
         <v>0.489998045758</v>
       </c>
-      <c r="E77" s="23" t="inlineStr">
+      <c r="E77" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D178.</t>
         </is>
@@ -18905,11 +18992,11 @@
           <t xml:space="preserve">s</t>
         </is>
       </c>
-      <c r="D78" s="27">
+      <c r="D78" s="150">
         <f>'Mass Transfer'!$D$90</f>
         <v>0.784513049825</v>
       </c>
-      <c r="E78" s="23" t="inlineStr">
+      <c r="E78" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D90.</t>
         </is>
@@ -18931,11 +19018,11 @@
           <t xml:space="preserve">J/(mol·K)</t>
         </is>
       </c>
-      <c r="D79" s="27">
+      <c r="D79" s="150">
         <f>'Mass Transfer'!$D$101</f>
         <v>8.314462618</v>
       </c>
-      <c r="E79" s="23" t="inlineStr">
+      <c r="E79" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D101.</t>
         </is>
@@ -18957,7 +19044,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D80" s="52">
+      <c r="D80" s="146">
         <v>0.04</v>
       </c>
       <c r="E80" s="99" t="inlineStr">
@@ -18982,7 +19069,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D81" s="52">
+      <c r="D81" s="146">
         <v>0.052</v>
       </c>
       <c r="E81" s="99" t="inlineStr">
@@ -19007,7 +19094,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D82" s="52">
+      <c r="D82" s="146">
         <v>0.6</v>
       </c>
       <c r="E82" s="99" t="inlineStr">
@@ -19268,7 +19355,7 @@
       <c r="C5" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="D5" s="72">
+      <c r="D5" s="153">
         <f>Geometry!$D$52</f>
         <v>12.0</v>
       </c>
@@ -19292,11 +19379,11 @@
       <c r="C6" s="20" t="s">
         <v>460</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="142">
         <f>Biology!$D$27</f>
         <v>0.36477</v>
       </c>
-      <c r="E6" s="23" t="str">
+      <c r="E6" s="135" t="str">
         <f>HYPERLINK("#Biology!D27","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19312,11 +19399,11 @@
       <c r="C7" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="142">
         <f>Biology!$D$26</f>
         <v>30397.5</v>
       </c>
-      <c r="E7" s="23" t="str">
+      <c r="E7" s="135" t="str">
         <f>HYPERLINK("#Biology!D26","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19332,11 +19419,11 @@
       <c r="C8" s="20" t="s">
         <v>309</v>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="142">
         <f>Biology!$D$18</f>
         <v>298.15</v>
       </c>
-      <c r="E8" s="23" t="str">
+      <c r="E8" s="135" t="str">
         <f>HYPERLINK("#Biology!D18","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19352,11 +19439,11 @@
       <c r="C9" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="26">
+      <c r="D9" s="142">
         <f>Biology!$D$19</f>
         <v>101325.0</v>
       </c>
-      <c r="E9" s="23" t="str">
+      <c r="E9" s="135" t="str">
         <f>HYPERLINK("#Biology!D19","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19372,11 +19459,11 @@
       <c r="C10" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="D10" s="26">
+      <c r="D10" s="142">
         <f>Biology!$D$15</f>
         <v>1.72933056055e-05</v>
       </c>
-      <c r="E10" s="23" t="str">
+      <c r="E10" s="135" t="str">
         <f>HYPERLINK("#Biology!D15","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19392,11 +19479,11 @@
       <c r="C11" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="142">
         <f>Biology!$D$16</f>
         <v>1.477525935072e-05</v>
       </c>
-      <c r="E11" s="23" t="str">
+      <c r="E11" s="135" t="str">
         <f>HYPERLINK("#Biology!D16","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19412,11 +19499,11 @@
       <c r="C12" s="20" t="s">
         <v>440</v>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="142">
         <f>Biology!$D$24</f>
         <v>1.2e-05</v>
       </c>
-      <c r="E12" s="23" t="str">
+      <c r="E12" s="135" t="str">
         <f>HYPERLINK("#Biology!D24","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19432,11 +19519,11 @@
       <c r="C13" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="150">
         <f>Electrochemistry!$D$29</f>
         <v>4.936187056172e-05</v>
       </c>
-      <c r="E13" s="23" t="str">
+      <c r="E13" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
         <v>→ Electrochemistry</v>
       </c>
@@ -19452,11 +19539,11 @@
       <c r="C14" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="D14" s="25">
+      <c r="D14" s="151">
         <f>Geometry!$D$44</f>
         <v>429.547725140567</v>
       </c>
-      <c r="E14" s="23" t="str">
+      <c r="E14" s="135" t="str">
         <f>HYPERLINK("#Geometry!D44","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
@@ -19472,11 +19559,11 @@
       <c r="C15" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="151">
         <f>Geometry!$D$20</f>
         <v>25.28</v>
       </c>
-      <c r="E15" s="23" t="str">
+      <c r="E15" s="135" t="str">
         <f>HYPERLINK("#Geometry!D20","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
@@ -19492,11 +19579,11 @@
       <c r="C16" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="25">
+      <c r="D16" s="151">
         <f>Geometry!$D$41</f>
         <v>15.0</v>
       </c>
-      <c r="E16" s="23" t="str">
+      <c r="E16" s="135" t="str">
         <f>HYPERLINK("#Geometry!D41","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
@@ -19512,11 +19599,11 @@
       <c r="C17" s="20" t="s">
         <v>172</v>
       </c>
-      <c r="D17" s="25">
+      <c r="D17" s="151">
         <f>Geometry!$D$21</f>
         <v>501.93100162698</v>
       </c>
-      <c r="E17" s="23" t="str">
+      <c r="E17" s="135" t="str">
         <f>HYPERLINK("#Geometry!D21","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
@@ -19532,11 +19619,11 @@
       <c r="C18" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="D18" s="25">
+      <c r="D18" s="151">
         <f>Geometry!$D$31</f>
         <v>1.5875</v>
       </c>
-      <c r="E18" s="23" t="str">
+      <c r="E18" s="135" t="str">
         <f>HYPERLINK("#Geometry!D31","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
@@ -19552,11 +19639,11 @@
       <c r="C19" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="151">
         <f>Geometry!$D$49</f>
         <v>2.612428455917</v>
       </c>
-      <c r="E19" s="23" t="str">
+      <c r="E19" s="135" t="str">
         <f>HYPERLINK("#Geometry!D49","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
@@ -19572,11 +19659,11 @@
       <c r="C20" s="20" t="s">
         <v>553</v>
       </c>
-      <c r="D20" s="27">
+      <c r="D20" s="150">
         <f>Electrochemistry!$D$32</f>
         <v>0.0</v>
       </c>
-      <c r="E20" s="23" t="str">
+      <c r="E20" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D32","→ Electrochemistry")</f>
         <v>→ Electrochemistry</v>
       </c>
@@ -19592,11 +19679,11 @@
       <c r="C21" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="D21" s="27" t="str">
+      <c r="D21" s="150" t="str">
         <f>Electrochemistry!$D$31</f>
         <v>Tube</v>
       </c>
-      <c r="E21" s="23" t="str">
+      <c r="E21" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D31","→ Electrochemistry")</f>
         <v>→ Electrochemistry</v>
       </c>
@@ -19610,11 +19697,11 @@
         <v>516</v>
       </c>
       <c r="C22" s="20"/>
-      <c r="D22" s="26" t="e">
+      <c r="D22" s="142" t="e">
         <f>Biology!$D$46</f>
         <v>#N/A</v>
       </c>
-      <c r="E22" s="23" t="str">
+      <c r="E22" s="135" t="str">
         <f>HYPERLINK("#Biology!D46","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19628,11 +19715,11 @@
         <v>518</v>
       </c>
       <c r="C23" s="20"/>
-      <c r="D23" s="26" t="e">
+      <c r="D23" s="142" t="e">
         <f>Biology!$D$47</f>
         <v>#N/A</v>
       </c>
-      <c r="E23" s="23" t="str">
+      <c r="E23" s="135" t="str">
         <f>HYPERLINK("#Biology!D47","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19646,11 +19733,11 @@
         <v>520</v>
       </c>
       <c r="C24" s="20"/>
-      <c r="D24" s="26" t="e">
+      <c r="D24" s="142" t="e">
         <f>Biology!$D$48</f>
         <v>#N/A</v>
       </c>
-      <c r="E24" s="23" t="str">
+      <c r="E24" s="135" t="str">
         <f>HYPERLINK("#Biology!D48","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19664,11 +19751,11 @@
         <v>514</v>
       </c>
       <c r="C25" s="20"/>
-      <c r="D25" s="26" t="e">
+      <c r="D25" s="142" t="e">
         <f>Biology!$D$45</f>
         <v>#N/A</v>
       </c>
-      <c r="E25" s="23" t="str">
+      <c r="E25" s="135" t="str">
         <f>HYPERLINK("#Biology!D45","→ Biology")</f>
         <v>→ Biology</v>
       </c>
@@ -19692,7 +19779,7 @@
       <c r="C27" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D27" s="36" t="s">
+      <c r="D27" s="131" t="s">
         <v>395</v>
       </c>
       <c r="E27" s="37" t="s">
@@ -19710,7 +19797,7 @@
       <c r="C28" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D28" s="36" t="s">
+      <c r="D28" s="131" t="s">
         <v>401</v>
       </c>
       <c r="E28" s="37" t="s">
@@ -19728,7 +19815,7 @@
       <c r="C29" s="19" t="s">
         <v>567</v>
       </c>
-      <c r="D29" s="22">
+      <c r="D29" s="141">
         <f>sigma_0+sigma_k*(T_K-T_zero_C)</f>
         <v>0.071965</v>
       </c>
@@ -19749,7 +19836,7 @@
       <c r="C30" s="19" t="s">
         <v>570</v>
       </c>
-      <c r="D30" s="22">
+      <c r="D30" s="141">
         <f>rho_0+rho_k*(T_K-T_zero_C)</f>
         <v>996.94</v>
       </c>
@@ -19768,7 +19855,7 @@
       <c r="C31" s="19" t="s">
         <v>573</v>
       </c>
-      <c r="D31" s="56">
+      <c r="D31" s="145">
         <v>9.8066499999999994</v>
       </c>
       <c r="E31" s="100" t="s">
@@ -19786,7 +19873,7 @@
       <c r="C32" s="19" t="s">
         <v>577</v>
       </c>
-      <c r="D32" s="22">
+      <c r="D32" s="141">
         <f>10^(HB_a+HB_b/T_K-(HB_c/T_K)^2)/10000</f>
         <v>1.997672318404e-09</v>
       </c>
@@ -19807,7 +19894,7 @@
       <c r="C33" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D33" s="52">
+      <c r="D33" s="146">
         <v>205</v>
       </c>
       <c r="E33" s="51" t="s">
@@ -19825,7 +19912,7 @@
       <c r="C34" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D34" s="52">
+      <c r="D34" s="146">
         <v>130</v>
       </c>
       <c r="E34" s="51" t="s">
@@ -19843,7 +19930,7 @@
       <c r="C35" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D35" s="52">
+      <c r="D35" s="146">
         <v>70</v>
       </c>
       <c r="E35" s="51" t="s">
@@ -19861,7 +19948,7 @@
       <c r="C36" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D36" s="52">
+      <c r="D36" s="146">
         <v>28</v>
       </c>
       <c r="E36" s="51" t="s">
@@ -19879,7 +19966,7 @@
       <c r="C37" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D37" s="52">
+      <c r="D37" s="146">
         <v>13</v>
       </c>
       <c r="E37" s="51" t="s">
@@ -19897,7 +19984,7 @@
       <c r="C38" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D38" s="54">
+      <c r="D38" s="154">
         <v>1.3</v>
       </c>
       <c r="E38" s="51" t="s">
@@ -20008,7 +20095,7 @@
       <c r="C44" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D44" s="50">
+      <c r="D44" s="155">
         <v>2.14</v>
       </c>
       <c r="E44" s="75" t="s">
@@ -20026,7 +20113,7 @@
       <c r="C45" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D45" s="77">
+      <c r="D45" s="156">
         <v>0.505</v>
       </c>
       <c r="E45" s="75" t="s">
@@ -20272,7 +20359,7 @@
       <c r="C58" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="D58" s="36">
+      <c r="D58" s="131">
         <v>0.05</v>
       </c>
       <c r="E58" s="75" t="s">
@@ -20328,7 +20415,7 @@
       <c r="C61" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D61" s="36">
+      <c r="D61" s="131">
         <v>1</v>
       </c>
       <c r="E61" s="70" t="s">
@@ -20443,7 +20530,7 @@
       <c r="C67" s="19" t="s">
         <v>683</v>
       </c>
-      <c r="D67" s="78">
+      <c r="D67" s="157">
         <f>Summary!$D$7</f>
         <v>1000.0</v>
       </c>
@@ -20711,7 +20798,7 @@
       <c r="C81" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D81" s="36" t="s">
+      <c r="D81" s="131" t="s">
         <v>721</v>
       </c>
       <c r="E81" s="68" t="s">
@@ -20729,7 +20816,7 @@
       <c r="C82" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D82" s="36">
+      <c r="D82" s="131">
         <v>1</v>
       </c>
       <c r="E82" s="68" t="s">
@@ -20747,7 +20834,7 @@
       <c r="C83" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="D83" s="36">
+      <c r="D83" s="131">
         <v>1</v>
       </c>
       <c r="E83" s="68" t="s">
@@ -20765,7 +20852,7 @@
       <c r="C84" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D84" s="79">
+      <c r="D84" s="158">
         <f>Biology!$D$60</f>
         <v>0.226086956522</v>
       </c>
@@ -20784,7 +20871,7 @@
       <c r="C85" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="D85" s="36">
+      <c r="D85" s="131">
         <v>2</v>
       </c>
       <c r="E85" s="68" t="s">
@@ -20882,11 +20969,11 @@
       <c r="C90" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="D90" s="119">
+      <c r="D90" s="48">
         <f>MAX(pulse_floor,flush_factor*headspace_V/(Q_CO2/60))</f>
         <v>0.784513049825</v>
       </c>
-      <c r="E90" s="80" t="s">
+      <c r="E90" s="159" t="s">
         <v>742</v>
       </c>
       <c r="F90" s="20"/>
@@ -20901,11 +20988,11 @@
       <c r="C91" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="D91" s="119">
+      <c r="D91" s="48">
         <f>IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max))</f>
         <v>16.46036421628</v>
       </c>
-      <c r="E91" s="80" t="inlineStr">
+      <c r="E91" s="159" t="inlineStr">
         <is>
           <t xml:space="preserve">ANSWER. The shorter of the two upper bounds on the interval: carbon supply (D112) and headspace-oxygen dilution (spg_int_DO). If the DO target is unreachable at this surface kLa the sheet falls back to the lag-accumulation cap (D89) and D134 says so. kL_surf moves the answer continuously; no branch depends on it.</t>
         </is>
@@ -20926,7 +21013,7 @@
         <f>spg_int_opt*60</f>
         <v>987.621852976796</v>
       </c>
-      <c r="E92" s="80" t="s">
+      <c r="E92" s="159" t="s">
         <v>747</v>
       </c>
       <c r="F92" s="20"/>
@@ -21019,7 +21106,7 @@
       <c r="C97" s="19" t="s">
         <v>507</v>
       </c>
-      <c r="D97" s="116">
+      <c r="D97" s="48">
         <f>IF(ISNUMBER(cal_kLa),cal_kLa,0)</f>
         <v>0.0</v>
       </c>
@@ -21057,11 +21144,11 @@
       <c r="C99" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D99" s="24">
+      <c r="D99" s="28">
         <f>min_sparge_cal</f>
         <v>0.25</v>
       </c>
-      <c r="E99" s="20" t="s">
+      <c r="E99" s="160" t="s">
         <v>765</v>
       </c>
       <c r="F99" s="20"/>
@@ -21076,11 +21163,11 @@
       <c r="C100" s="20" t="s">
         <v>354</v>
       </c>
-      <c r="D100" s="24">
+      <c r="D100" s="28">
         <f>CO2_pulse*pulses_h</f>
         <v>0.0003892277799716</v>
       </c>
-      <c r="E100" s="20" t="s">
+      <c r="E100" s="160" t="s">
         <v>765</v>
       </c>
       <c r="F100" s="20"/>
@@ -21095,7 +21182,7 @@
       <c r="C101" s="20" t="s">
         <v>314</v>
       </c>
-      <c r="D101" s="81">
+      <c r="D101" s="161">
         <v>8.3144626180000003</v>
       </c>
       <c r="E101" s="20" t="s">
@@ -21113,11 +21200,11 @@
       <c r="C102" s="20" t="s">
         <v>361</v>
       </c>
-      <c r="D102" s="24">
+      <c r="D102" s="28">
         <f>IF(has_cal&gt;0,flowrate_cal*60,NA())</f>
         <v>199.8</v>
       </c>
-      <c r="E102" s="20" t="s">
+      <c r="E102" s="160" t="s">
         <v>765</v>
       </c>
       <c r="F102" s="20"/>
@@ -21132,7 +21219,7 @@
       <c r="C103" s="20" t="s">
         <v>773</v>
       </c>
-      <c r="D103" s="81">
+      <c r="D103" s="161">
         <v>44.009500000000003</v>
       </c>
       <c r="E103" s="20" t="s">
@@ -21150,11 +21237,11 @@
       <c r="C104" s="20" t="s">
         <v>776</v>
       </c>
-      <c r="D104" s="24">
+      <c r="D104" s="28">
         <f>P_atm*(Q_CO2/1000000/60)/(R_gas*T_K)</f>
         <v>0.000136110568266</v>
       </c>
-      <c r="E104" s="20" t="s">
+      <c r="E104" s="160" t="s">
         <v>765</v>
       </c>
       <c r="F104" s="20"/>
@@ -21169,11 +21256,11 @@
       <c r="C105" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="D105" s="24">
+      <c r="D105" s="28">
         <f>spg_dur/(spg_int*60)</f>
         <v>0.0007943455761538</v>
       </c>
-      <c r="E105" s="20" t="s">
+      <c r="E105" s="160" t="s">
         <v>765</v>
       </c>
       <c r="F105" s="20"/>
@@ -21188,7 +21275,7 @@
       <c r="C106" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="D106" s="81">
+      <c r="D106" s="161">
         <v>1</v>
       </c>
       <c r="E106" s="20" t="s">
@@ -21216,11 +21303,11 @@
       <c r="C108" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="D108" s="24">
+      <c r="D108" s="28">
         <f>(DO_hs_floor+DO_surf_excess)*M_O2</f>
         <v>2.638866712696</v>
       </c>
-      <c r="E108" s="20" t="s">
+      <c r="E108" s="160" t="s">
         <v>1929</v>
       </c>
       <c r="F108" s="20"/>
@@ -21233,7 +21320,7 @@
         <v>785</v>
       </c>
       <c r="C109" s="20"/>
-      <c r="D109" s="24" t="str">
+      <c r="D109" s="28" t="str">
         <f>IF(ISNUMBER(DO_opt),IF(DO_ss&lt;=DO_opt,"at/under optimum",IF(DO_ss&lt;DO_impair,"above optimum, under impairment","OVER IMPAIRMENT - surface strip insufficient")),"organism optimum unknown")</f>
         <v>organism optimum unknown</v>
       </c>
@@ -21248,7 +21335,7 @@
         <v>787</v>
       </c>
       <c r="C110" s="20"/>
-      <c r="D110" s="24" t="str">
+      <c r="D110" s="28" t="str">
         <f>IF(ISNUMBER(DO_min),IF(DO_ss&gt;=DO_min,"above minimum","BELOW MINIMUM"),"minimum DO unknown - measure")</f>
         <v>minimum DO unknown - measure</v>
       </c>
@@ -21264,7 +21351,7 @@
         <v>789</v>
       </c>
       <c r="C111" s="20"/>
-      <c r="D111" s="24" t="str">
+      <c r="D111" s="28" t="str">
         <f>IF(tip_speed&gt;tip_speed_max,"TIP SPEED &gt; "&amp;TEXT(tip_speed_max,"0.0")&amp;" m/s","OK")</f>
         <v>OK</v>
       </c>
@@ -21283,7 +21370,7 @@
       <c r="C112" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D112" s="24">
+      <c r="D112" s="28">
         <f>spg_dur_opt/(60*duty_carbon)</f>
         <v>185.240207036777</v>
       </c>
@@ -21298,7 +21385,7 @@
         <v>794</v>
       </c>
       <c r="C113" s="20"/>
-      <c r="D113" s="24" t="str">
+      <c r="D113" s="28" t="str">
         <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) DO would be "&amp;TEXT(DO_at_carbon*M_O2,"0.0")&amp;" mg/L against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")</f>
         <v>Do NOT relax: at the carbon-limited interval (185 min) DO would be 12.9 mg/L against a 2.6 mg/L target</v>
       </c>
@@ -21329,7 +21416,7 @@
         <v>1</v>
       </c>
       <c r="C115" s="20"/>
-      <c r="D115" s="38" t="str">
+      <c r="D115" s="134" t="str">
         <f>Summary!$D$2</f>
         <v>ed04</v>
       </c>
@@ -21344,7 +21431,7 @@
         <v>799</v>
       </c>
       <c r="C116" s="20"/>
-      <c r="D116" s="83">
+      <c r="D116" s="162">
         <f>SUMPRODUCT(MAX(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$J$4:$J$201&gt;0)*'CO2 flows'!$B$4:$B$201))</f>
         <v>46190.0</v>
       </c>
@@ -21363,11 +21450,11 @@
           <t xml:space="preserve">mL/s</t>
         </is>
       </c>
-      <c r="D117" s="83">
+      <c r="D117" s="162">
         <f>IF(ISNUMBER(cal_flow),cal_flow,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*'CO2 flows'!$J$4:$J$201)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*('CO2 flows'!$J$4:$J$201&gt;0)*1)))</f>
         <v>3.33</v>
       </c>
-      <c r="E117" s="20" t="inlineStr">
+      <c r="E117" s="160" t="inlineStr">
         <is>
           <t xml:space="preserve">Prefers the CO₂-flow calibration recorded on the Calibrations tab (cal_flow); falls back to the per-reactor table on the CO2 flows sheet when no calibration run is included.</t>
         </is>
@@ -21384,7 +21471,7 @@
       <c r="C118" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D118" s="83">
+      <c r="D118" s="162">
         <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*'CO2 flows'!$I$4:$I$201)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*('CO2 flows'!$J$4:$J$201&gt;0)*1))</f>
         <v>0.25</v>
       </c>
@@ -21401,7 +21488,7 @@
       <c r="C119" s="20" t="s">
         <v>806</v>
       </c>
-      <c r="D119" s="83">
+      <c r="D119" s="162">
         <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$J$4:$J$201&gt;0)*1)</f>
         <v>1.0</v>
       </c>
@@ -21416,7 +21503,7 @@
         <v>808</v>
       </c>
       <c r="C120" s="20"/>
-      <c r="D120" s="24" t="str">
+      <c r="D120" s="28" t="str">
         <f>IF(has_cal&gt;0,"calibrated: "&amp;Reactor,"NO CALIBRATION for "&amp;Reactor&amp;" - add a row in CO2 flows with nominal flowrate + minimum sparge")</f>
         <v>calibrated: ed04</v>
       </c>
@@ -21433,7 +21520,7 @@
       <c r="C121" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="D121" s="24">
+      <c r="D121" s="28">
         <f>IF(AND(ISNUMBER(Summary!$G$13),Summary!$G$13&gt;0),Summary!$G$13,IF(sched_mode="Manual",spg_dur_man,spg_dur_opt))</f>
         <v>0.784513049825</v>
       </c>
@@ -21450,7 +21537,7 @@
       <c r="C122" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="D122" s="24">
+      <c r="D122" s="28">
         <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,spg_int_opt))</f>
         <v>16.46036421628</v>
       </c>
@@ -21467,7 +21554,7 @@
       <c r="C123" s="20" t="s">
         <v>815</v>
       </c>
-      <c r="D123" s="24">
+      <c r="D123" s="28">
         <f>nCO2_rate*spg_dur</f>
         <v>0.0001067805170238</v>
       </c>
@@ -21484,7 +21571,7 @@
       <c r="C124" s="20" t="s">
         <v>818</v>
       </c>
-      <c r="D124" s="24">
+      <c r="D124" s="28">
         <f>60/spg_int</f>
         <v>3.645119829163</v>
       </c>
@@ -21501,7 +21588,7 @@
       <c r="C125" s="20" t="s">
         <v>821</v>
       </c>
-      <c r="D125" s="24">
+      <c r="D125" s="28">
         <f>pulses_h*24</f>
         <v>87.482875899902</v>
       </c>
@@ -21518,7 +21605,7 @@
       <c r="C126" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="D126" s="24">
+      <c r="D126" s="28">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
         <v>22.507425060931</v>
       </c>
@@ -21535,7 +21622,7 @@
       <c r="C127" s="20" t="s">
         <v>815</v>
       </c>
-      <c r="D127" s="24">
+      <c r="D127" s="28">
         <f>O2_excess/60*spg_int</f>
         <v>4.05343583838e-06</v>
       </c>
@@ -21552,7 +21639,7 @@
       <c r="C128" s="20" t="s">
         <v>815</v>
       </c>
-      <c r="D128" s="24">
+      <c r="D128" s="28">
         <f>strip_sparge/3600*spg_dur</f>
         <v>6.635009117477e-08</v>
       </c>
@@ -21569,7 +21656,7 @@
       <c r="C129" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="D129" s="24">
+      <c r="D129" s="28">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
         <v>0.016368851962</v>
       </c>
@@ -21584,7 +21671,7 @@
         <v>831</v>
       </c>
       <c r="C130" s="20"/>
-      <c r="D130" s="24" t="str">
+      <c r="D130" s="28" t="str">
         <f>IF(spg_dur&gt;=pulse_floor,"OK","LOW")</f>
         <v>OK</v>
       </c>
@@ -21603,11 +21690,11 @@
       <c r="C131" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="D131" s="24">
+      <c r="D131" s="28">
         <f>kLa_surf_req/a_surf</f>
         <v>0.0001158581442306</v>
       </c>
-      <c r="E131" s="101" t="s">
+      <c r="E131" s="147" t="s">
         <v>1825</v>
       </c>
       <c r="F131" s="20"/>
@@ -21712,7 +21799,7 @@
       <c r="C138" s="19" t="s">
         <v>577</v>
       </c>
-      <c r="D138" s="22">
+      <c r="D138" s="141">
         <f>D_CO2_ref*EXP(-Ea_D_CO2/R_gas*(1/T_K-1/T_ref))</f>
         <v>1.92e-09</v>
       </c>
@@ -21731,7 +21818,7 @@
       <c r="C139" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D139" s="36">
+      <c r="D139" s="131">
         <v>40</v>
       </c>
       <c r="E139" s="67" t="s">
@@ -21787,7 +21874,7 @@
       <c r="C142" s="19" t="s">
         <v>361</v>
       </c>
-      <c r="D142" s="36">
+      <c r="D142" s="131">
         <v>0.5</v>
       </c>
       <c r="E142" s="69" t="s">
@@ -22230,7 +22317,7 @@
       <c r="C167" s="19" t="s">
         <v>567</v>
       </c>
-      <c r="D167" s="52">
+      <c r="D167" s="146">
         <v>7.5889999999999999E-2</v>
       </c>
       <c r="E167" s="99" t="s">
@@ -22247,7 +22334,7 @@
       <c r="C168" s="19" t="s">
         <v>1763</v>
       </c>
-      <c r="D168" s="52">
+      <c r="D168" s="146">
         <v>-1.5699999999999999E-4</v>
       </c>
       <c r="E168" s="99" t="s">
@@ -22264,7 +22351,7 @@
       <c r="C169" s="19" t="s">
         <v>570</v>
       </c>
-      <c r="D169" s="52">
+      <c r="D169" s="146">
         <v>1003.33</v>
       </c>
       <c r="E169" s="99" t="s">
@@ -22281,7 +22368,7 @@
       <c r="C170" s="19" t="s">
         <v>1770</v>
       </c>
-      <c r="D170" s="52">
+      <c r="D170" s="146">
         <v>-0.25559999999999999</v>
       </c>
       <c r="E170" s="99" t="s">
@@ -22298,7 +22385,7 @@
       <c r="C171" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D171" s="52">
+      <c r="D171" s="146">
         <v>-4.41</v>
       </c>
       <c r="E171" s="99" t="inlineStr">
@@ -22317,7 +22404,7 @@
       <c r="C172" s="19" t="s">
         <v>843</v>
       </c>
-      <c r="D172" s="52">
+      <c r="D172" s="146">
         <v>773.8</v>
       </c>
       <c r="E172" s="99" t="s">
@@ -22334,7 +22421,7 @@
       <c r="C173" s="19" t="s">
         <v>843</v>
       </c>
-      <c r="D173" s="52">
+      <c r="D173" s="146">
         <v>506.4</v>
       </c>
       <c r="E173" s="99" t="s">
@@ -22351,7 +22438,7 @@
       <c r="C174" s="19" t="s">
         <v>577</v>
       </c>
-      <c r="D174" s="52">
+      <c r="D174" s="146">
         <v>1.92E-9</v>
       </c>
       <c r="E174" s="67" t="s">
@@ -22368,7 +22455,7 @@
       <c r="C175" s="19" t="s">
         <v>1783</v>
       </c>
-      <c r="D175" s="52">
+      <c r="D175" s="146">
         <v>19000</v>
       </c>
       <c r="E175" s="67" t="s">
@@ -22392,7 +22479,7 @@
       <c r="C178" s="19" t="s">
         <v>991</v>
       </c>
-      <c r="D178" s="22">
+      <c r="D178" s="141">
         <f>nCO2_rate*3600</f>
         <v>0.489998045758</v>
       </c>
@@ -22410,7 +22497,7 @@
       <c r="C179" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D179" s="22">
+      <c r="D179" s="141">
         <f>target_DO_frac*O2_ceil_C</f>
         <v>0.08246973913</v>
       </c>
@@ -22428,7 +22515,7 @@
       <c r="C180" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D180" s="22">
+      <c r="D180" s="141">
         <f>O2_excess/(kLa_surf_used*3600*(V_charge/1000000))</f>
         <v>0.038001663161</v>
       </c>
@@ -22446,7 +22533,7 @@
       <c r="C181" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D181" s="22">
+      <c r="D181" s="141">
         <f>O2_net_gen/(kLa_surf_used*3600*(V_charge/1000000))</f>
         <v>0.126957715838</v>
       </c>
@@ -22464,7 +22551,7 @@
       <c r="C182" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D182" s="22">
+      <c r="D182" s="141">
         <f>DO_target-DO_surf_excess</f>
         <v>0.04446807597</v>
       </c>
@@ -22482,7 +22569,7 @@
       <c r="C183" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D183" s="22">
+      <c r="D183" s="141">
         <f>IF(hs_O2_allow&gt;0,hs_O2_allow/(H_O2_T*P_atm),NA())</f>
         <v>0.036572149</v>
       </c>
@@ -22500,7 +22587,7 @@
       <c r="C184" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D184" s="22">
+      <c r="D184" s="141">
         <f>IF(ISNUMBER(y_O2_star),O2_excess*(1-y_O2_star)/(y_O2_star*CO2_rate_full),NA())</f>
         <v>0.0007943455761538</v>
       </c>
@@ -22520,7 +22607,7 @@
       <c r="C185" s="19" t="s">
         <v>962</v>
       </c>
-      <c r="D185" s="22">
+      <c r="D185" s="141">
         <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_opt/(60*duty_DO),spg_int_carbon),NA())</f>
         <v>16.46036421628</v>
       </c>
@@ -22538,7 +22625,7 @@
       <c r="C186" s="19" t="s">
         <v>639</v>
       </c>
-      <c r="D186" s="22">
+      <c r="D186" s="141">
         <f>O2_excess/(DO_target*3600*(V_charge/1000000))</f>
         <v>0.003317773486</v>
       </c>
@@ -22556,7 +22643,7 @@
       <c r="C187" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D187" s="22">
+      <c r="D187" s="141">
         <f>IF(CO2_supply&gt;0,O2_excess/(O2_excess+CO2_supply),NA())</f>
         <v>0.036572149</v>
       </c>
@@ -22574,7 +22661,7 @@
       <c r="C188" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D188" s="22">
+      <c r="D188" s="141">
         <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_atm,NA())</f>
         <v>0.04446807597</v>
       </c>
@@ -22599,7 +22686,7 @@
       <c r="C191" s="19" t="s">
         <v>440</v>
       </c>
-      <c r="D191" s="22">
+      <c r="D191" s="141">
         <f>Biology!$D$31</f>
         <v>0.00033</v>
       </c>
@@ -22617,7 +22704,7 @@
       <c r="C192" s="19" t="s">
         <v>1163</v>
       </c>
-      <c r="D192" s="22">
+      <c r="D192" s="141">
         <f>headspace_V_m3/(hs_H_CO2*R_gas*T_K)</f>
         <v>3.193459899477e-06</v>
       </c>
@@ -22635,7 +22722,7 @@
       <c r="C193" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D193" s="22">
+      <c r="D193" s="141">
         <f>V_L_m3/(V_L_m3+Vg_CO2)</f>
         <v>0.824472095076</v>
       </c>
@@ -22653,7 +22740,7 @@
       <c r="C194" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D194" s="22">
+      <c r="D194" s="141">
         <f>CO2_pulse/(V_L_m3+Vg_CO2)</f>
         <v>5.869170438925</v>
       </c>
@@ -22673,7 +22760,7 @@
       <c r="C195" s="19" t="s">
         <v>639</v>
       </c>
-      <c r="D195" s="22">
+      <c r="D195" s="141">
         <f>k_vent*Vg_CO2/(V_L_m3+Vg_CO2)</f>
         <v>0.000559912956744</v>
       </c>
@@ -22691,7 +22778,7 @@
       <c r="C196" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D196" s="22">
+      <c r="D196" s="141">
         <f>(kLa_CO2_off*V_L_m3/Vg_CO2)/k_vent</f>
         <v>10.393999248454</v>
       </c>
@@ -22709,7 +22796,7 @@
       <c r="C197" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D197" s="22">
+      <c r="D197" s="141">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
         <v>0.575484483576</v>
       </c>
@@ -22727,7 +22814,7 @@
       <c r="C198" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D198" s="22">
+      <c r="D198" s="141">
         <f>(C_air_CO2*(1-pool_e)+pool_b*pool_e)/(1-pool_a*pool_e)</f>
         <v>6.437740764668</v>
       </c>
@@ -22745,7 +22832,7 @@
       <c r="C199" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D199" s="22">
+      <c r="D199" s="141">
         <f>pool_a*C_cycle_start+pool_b</f>
         <v>11.176908054727</v>
       </c>
@@ -22763,7 +22850,7 @@
       <c r="C200" s="19" t="s">
         <v>1001</v>
       </c>
-      <c r="D200" s="22">
+      <c r="D200" s="141">
         <f>C_air_CO2+(C_cycle_peak-C_air_CO2)*(1-pool_e)/(k_eff_CO2*t_off_CO2)</f>
         <v>8.59021062192</v>
       </c>
@@ -22786,7 +22873,7 @@
       <c r="C203" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D203" s="52">
+      <c r="D203" s="146">
         <v>610.94000000000005</v>
       </c>
       <c r="E203" s="99" t="s">
@@ -22803,7 +22890,7 @@
       <c r="C204" s="19" t="s">
         <v>1274</v>
       </c>
-      <c r="D204" s="52">
+      <c r="D204" s="146">
         <v>17.625</v>
       </c>
       <c r="E204" s="99" t="s">
@@ -22820,7 +22907,7 @@
       <c r="C205" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="D205" s="52">
+      <c r="D205" s="146">
         <v>243.04</v>
       </c>
       <c r="E205" s="99" t="s">
@@ -22837,7 +22924,7 @@
       <c r="C206" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="D206" s="22">
+      <c r="D206" s="141">
         <f>pw_A*EXP(pw_B*(T_K-T_zero_C)/((T_K-T_zero_C)+pw_C))</f>
         <v>3161.736035696692</v>
       </c>
@@ -22870,11 +22957,11 @@
           <t xml:space="preserve">K</t>
         </is>
       </c>
-      <c r="D209" s="26">
+      <c r="D209" s="142">
         <f>Biology!$D$23</f>
         <v>298.15</v>
       </c>
-      <c r="E209" s="23" t="inlineStr">
+      <c r="E209" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Biology!D23</t>
         </is>
@@ -22896,11 +22983,11 @@
           <t xml:space="preserve">K</t>
         </is>
       </c>
-      <c r="D210" s="26">
+      <c r="D210" s="142">
         <f>Biology!$D$66</f>
         <v>273.15</v>
       </c>
-      <c r="E210" s="23" t="inlineStr">
+      <c r="E210" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Biology!D66</t>
         </is>
@@ -22922,7 +23009,7 @@
           <t xml:space="preserve">m</t>
         </is>
       </c>
-      <c r="D211" s="36">
+      <c r="D211" s="131">
         <v>0.001</v>
       </c>
       <c r="E211" s="67" t="inlineStr">
@@ -22947,7 +23034,7 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D212" s="36">
+      <c r="D212" s="131">
         <v>2</v>
       </c>
       <c r="E212" s="67" t="inlineStr">
@@ -22972,7 +23059,7 @@
           <t xml:space="preserve">min</t>
         </is>
       </c>
-      <c r="D213" s="36">
+      <c r="D213" s="131">
         <v>9999</v>
       </c>
       <c r="E213" s="99" t="inlineStr">
@@ -22997,7 +23084,7 @@
           <t xml:space="preserve">s</t>
         </is>
       </c>
-      <c r="D214" s="36">
+      <c r="D214" s="131">
         <v>5</v>
       </c>
       <c r="E214" s="68" t="inlineStr">
@@ -23022,7 +23109,7 @@
           <t xml:space="preserve">m/s</t>
         </is>
       </c>
-      <c r="D216" s="36">
+      <c r="D216" s="131">
         <v>1.5</v>
       </c>
       <c r="E216" s="82" t="inlineStr">
@@ -23054,7 +23141,7 @@
           <t xml:space="preserve">g/mol</t>
         </is>
       </c>
-      <c r="D231" s="52">
+      <c r="D231" s="146">
         <v>31.998</v>
       </c>
       <c r="E231" s="99" t="inlineStr">
@@ -23079,7 +23166,7 @@
           <t xml:space="preserve">mol/m³</t>
         </is>
       </c>
-      <c r="D232" s="22">
+      <c r="D232" s="141">
         <f>H_O2_T*P_atm*O2_excess/(O2_excess+CO2_rate_full*duty_carbon)+DO_surf_excess</f>
         <v>0.401951360368</v>
       </c>
@@ -28007,7 +28094,7 @@
           <t xml:space="preserve">µm·kPa</t>
         </is>
       </c>
-      <c r="D140" s="97">
+      <c r="D140" s="163">
         <v>291.2</v>
       </c>
       <c r="E140" s="97" t="inlineStr">
@@ -28032,7 +28119,7 @@
           <t xml:space="preserve">µm</t>
         </is>
       </c>
-      <c r="D141" s="97">
+      <c r="D141" s="163">
         <v>160</v>
       </c>
       <c r="E141" s="97" t="inlineStr">
@@ -28057,7 +28144,7 @@
           <t xml:space="preserve">µm</t>
         </is>
       </c>
-      <c r="D142" s="97">
+      <c r="D142" s="163">
         <v>100</v>
       </c>
       <c r="E142" s="97" t="inlineStr">
@@ -28082,7 +28169,7 @@
           <t xml:space="preserve">µm</t>
         </is>
       </c>
-      <c r="D143" s="97">
+      <c r="D143" s="163">
         <v>40</v>
       </c>
       <c r="E143" s="97" t="inlineStr">
@@ -28107,7 +28194,7 @@
           <t xml:space="preserve">µm</t>
         </is>
       </c>
-      <c r="D144" s="97">
+      <c r="D144" s="163">
         <v>16</v>
       </c>
       <c r="E144" s="97" t="inlineStr">
@@ -28132,7 +28219,7 @@
           <t xml:space="preserve">µm</t>
         </is>
       </c>
-      <c r="D145" s="97">
+      <c r="D145" s="163">
         <v>10</v>
       </c>
       <c r="E145" s="97" t="inlineStr">
@@ -28157,11 +28244,11 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D146" s="97">
+      <c r="D146" s="164">
         <f>Electrochemistry!$D$16</f>
         <v>2.0</v>
       </c>
-      <c r="E146" s="97" t="inlineStr">
+      <c r="E146" s="165" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Electrochemistry!D16</t>
         </is>
@@ -28183,11 +28270,11 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D147" s="97">
+      <c r="D147" s="164">
         <f>Electrochemistry!$D$17</f>
         <v>4.0</v>
       </c>
-      <c r="E147" s="97" t="inlineStr">
+      <c r="E147" s="165" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Electrochemistry!D17</t>
         </is>
@@ -28209,11 +28296,11 @@
           <t xml:space="preserve">K</t>
         </is>
       </c>
-      <c r="D148" s="97">
+      <c r="D148" s="164">
         <f>Biology!$D$66</f>
         <v>273.15</v>
       </c>
-      <c r="E148" s="97" t="inlineStr">
+      <c r="E148" s="165" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Biology!D66</t>
         </is>

</xml_diff>

<commit_message>
Gas model: Summary result rows carry defined names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -638,6 +638,48 @@
     <definedName name="z_e_H2" localSheetId="7">Calibrations!$D$146</definedName>
     <definedName name="z_e_O2" localSheetId="7">Calibrations!$D$147</definedName>
     <definedName name="T_zero_C" localSheetId="7">Calibrations!$D$148</definedName>
+    <definedName name="res_spg_dur" localSheetId="0">Summary!$D$13</definedName>
+    <definedName name="res_spg_dur_run" localSheetId="0">Summary!$D$14</definedName>
+    <definedName name="res_spg_int" localSheetId="0">Summary!$D$15</definedName>
+    <definedName name="res_spg_int_run" localSheetId="0">Summary!$D$16</definedName>
+    <definedName name="chk_geom" localSheetId="0">Summary!$D$19</definedName>
+    <definedName name="chk_cal" localSheetId="0">Summary!$D$20</definedName>
+    <definedName name="chk_DO_opt" localSheetId="0">Summary!$D$21</definedName>
+    <definedName name="chk_DO_min" localSheetId="0">Summary!$D$22</definedName>
+    <definedName name="chk_relax" localSheetId="0">Summary!$D$23</definedName>
+    <definedName name="chk_H2" localSheetId="0">Summary!$D$24</definedName>
+    <definedName name="chk_bubble" localSheetId="0">Summary!$D$25</definedName>
+    <definedName name="chk_CO2_supply" localSheetId="0">Summary!$D$26</definedName>
+    <definedName name="chk_pulse_floor" localSheetId="0">Summary!$D$27</definedName>
+    <definedName name="chk_od_window" localSheetId="0">Summary!$D$28</definedName>
+    <definedName name="chk_carryover" localSheetId="0">Summary!$D$29</definedName>
+    <definedName name="chk_tip" localSheetId="0">Summary!$D$30</definedName>
+    <definedName name="chk_media_vol" localSheetId="0">Summary!$D$31</definedName>
+    <definedName name="chk_level" localSheetId="0">Summary!$D$32</definedName>
+    <definedName name="chk_led_law" localSheetId="0">Summary!$D$33</definedName>
+    <definedName name="chk_DO_data" localSheetId="0">Summary!$D$34</definedName>
+    <definedName name="res_pH" localSheetId="0">Summary!$D$35</definedName>
+    <definedName name="res_Cl2" localSheetId="0">Summary!$D$36</definedName>
+    <definedName name="res_DO_ss" localSheetId="0">Summary!$D$38</definedName>
+    <definedName name="res_spg_int_carbon" localSheetId="0">Summary!$D$39</definedName>
+    <definedName name="res_tip_speed" localSheetId="0">Summary!$D$40</definedName>
+    <definedName name="res_carbon_margin" localSheetId="0">Summary!$D$41</definedName>
+    <definedName name="res_I_mA" localSheetId="0">Summary!$D$43</definedName>
+    <definedName name="res_j_anode" localSheetId="0">Summary!$D$44</definedName>
+    <definedName name="res_j_status" localSheetId="0">Summary!$D$45</definedName>
+    <definedName name="res_power_max" localSheetId="0">Summary!$D$46</definedName>
+    <definedName name="res_I_max" localSheetId="0">Summary!$D$47</definedName>
+    <definedName name="res_j_anode_max" localSheetId="0">Summary!$D$48</definedName>
+    <definedName name="res_j_status_max" localSheetId="0">Summary!$D$49</definedName>
+    <definedName name="res_etaF" localSheetId="0">Summary!$D$82</definedName>
+    <definedName name="res_V_cell" localSheetId="0">Summary!$D$83</definedName>
+    <definedName name="res_V_flag" localSheetId="0">Summary!$D$84</definedName>
+    <definedName name="res_H2O2_flag" localSheetId="0">Summary!$D$85</definedName>
+    <definedName name="res_buffer_flag" localSheetId="0">Summary!$D$86</definedName>
+    <definedName name="res_E_Cl_margin" localSheetId="0">Summary!$D$87</definedName>
+    <definedName name="res_E_Cu_margin" localSheetId="0">Summary!$D$88</definedName>
+    <definedName name="res_pH_probe" localSheetId="0">Summary!$D$89</definedName>
+    <definedName name="res_kLa_req" localSheetId="0">Summary!$D$90</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8188,7 +8230,11 @@
       <c r="A13" s="28" t="s">
         <v>1058</v>
       </c>
-      <c r="B13" s="20"/>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_dur</t>
+        </is>
+      </c>
       <c r="C13" s="20" t="s">
         <v>13</v>
       </c>
@@ -8209,7 +8255,11 @@
       <c r="A14" s="28" t="s">
         <v>1059</v>
       </c>
-      <c r="B14" s="20"/>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_dur_run</t>
+        </is>
+      </c>
       <c r="C14" s="20" t="s">
         <v>13</v>
       </c>
@@ -8224,7 +8274,11 @@
       <c r="A15" s="89" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="20"/>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_int</t>
+        </is>
+      </c>
       <c r="C15" s="20" t="s">
         <v>67</v>
       </c>
@@ -8247,7 +8301,11 @@
       <c r="A16" s="28" t="s">
         <v>1057</v>
       </c>
-      <c r="B16" s="20"/>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_int_run</t>
+        </is>
+      </c>
       <c r="C16" s="20" t="s">
         <v>67</v>
       </c>
@@ -8286,7 +8344,11 @@
       <c r="A19" s="89" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="20"/>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_geom</t>
+        </is>
+      </c>
       <c r="C19" s="20"/>
       <c r="D19" s="94" t="str">
         <f>Geometry!$D$90</f>
@@ -8306,7 +8368,11 @@
       <c r="A20" s="89" t="s">
         <v>72</v>
       </c>
-      <c r="B20" s="20"/>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_cal</t>
+        </is>
+      </c>
       <c r="C20" s="20"/>
       <c r="D20" s="90" t="str">
         <f>'Mass Transfer'!$D$120</f>
@@ -8324,7 +8390,11 @@
       <c r="A21" s="89" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="20"/>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_DO_opt</t>
+        </is>
+      </c>
       <c r="C21" s="20"/>
       <c r="D21" s="90" t="str">
         <f>'Mass Transfer'!$D$109</f>
@@ -8342,7 +8412,11 @@
       <c r="A22" s="89" t="s">
         <v>76</v>
       </c>
-      <c r="B22" s="20"/>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_DO_min</t>
+        </is>
+      </c>
       <c r="C22" s="20"/>
       <c r="D22" s="90" t="str">
         <f>'Mass Transfer'!$D$110</f>
@@ -8362,7 +8436,11 @@
           <t xml:space="preserve">Can the interval relax to the carbon-limited one?</t>
         </is>
       </c>
-      <c r="B23" s="20"/>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_relax</t>
+        </is>
+      </c>
       <c r="C23" s="20"/>
       <c r="D23" s="90" t="str">
         <f>'Mass Transfer'!$D$113</f>
@@ -8384,7 +8462,11 @@
           <t xml:space="preserve">H₂ headspace flammable?</t>
         </is>
       </c>
-      <c r="B24" s="20"/>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_H2</t>
+        </is>
+      </c>
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
@@ -8404,7 +8486,11 @@
       <c r="A25" s="89" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="20"/>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_bubble</t>
+        </is>
+      </c>
       <c r="C25" s="20"/>
       <c r="D25" s="90" t="str">
         <f>'Mass Transfer'!$D$64</f>
@@ -8422,7 +8508,11 @@
       <c r="A26" s="89" t="s">
         <v>84</v>
       </c>
-      <c r="B26" s="20"/>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_CO2_supply</t>
+        </is>
+      </c>
       <c r="C26" s="20"/>
       <c r="D26" s="90" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)"),"calibrate this reactor first")</f>
@@ -8440,7 +8530,11 @@
       <c r="A27" s="89" t="s">
         <v>86</v>
       </c>
-      <c r="B27" s="20"/>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_pulse_floor</t>
+        </is>
+      </c>
       <c r="C27" s="20"/>
       <c r="D27" s="90" t="str">
         <f>IFERROR('Mass Transfer'!$D$130,"calibrate this reactor first (see CO2 flows)")</f>
@@ -8458,7 +8552,11 @@
       <c r="A28" s="89" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="20"/>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_od_window</t>
+        </is>
+      </c>
       <c r="C28" s="20"/>
       <c r="D28" s="90" t="str">
         <f>IFERROR('Mass Transfer'!$D$95,"calibrate this reactor first (see CO2 flows)")</f>
@@ -8476,7 +8574,11 @@
       <c r="A29" s="89" t="s">
         <v>90</v>
       </c>
-      <c r="B29" s="20"/>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_carryover</t>
+        </is>
+      </c>
       <c r="C29" s="20"/>
       <c r="D29" s="90" t="str">
         <f>'Mass Transfer'!$D$59</f>
@@ -8494,7 +8596,11 @@
       <c r="A30" s="89" t="s">
         <v>92</v>
       </c>
-      <c r="B30" s="20"/>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_tip</t>
+        </is>
+      </c>
       <c r="C30" s="20"/>
       <c r="D30" s="90" t="str">
         <f>'Mass Transfer'!$D$111</f>
@@ -8512,7 +8618,11 @@
       <c r="A31" s="89" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="20"/>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_media_vol</t>
+        </is>
+      </c>
       <c r="C31" s="20"/>
       <c r="D31" s="94" t="str">
         <f>Geometry!$D$54</f>
@@ -8530,7 +8640,11 @@
       <c r="A32" s="89" t="s">
         <v>96</v>
       </c>
-      <c r="B32" s="20"/>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_level</t>
+        </is>
+      </c>
       <c r="C32" s="20"/>
       <c r="D32" s="94" t="str">
         <f>Geometry!$D$55</f>
@@ -8548,7 +8662,11 @@
       <c r="A33" s="89" t="s">
         <v>98</v>
       </c>
-      <c r="B33" s="20"/>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_led_law</t>
+        </is>
+      </c>
       <c r="C33" s="20"/>
       <c r="D33" s="96" t="str">
         <f>Electrochemistry!$D$20</f>
@@ -8562,9 +8680,14 @@
         <v>99</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A34" s="89" t="s">
         <v>986</v>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_DO_data</t>
+        </is>
       </c>
       <c r="C34" s="20"/>
       <c r="D34" s="94" t="str">
@@ -8579,10 +8702,15 @@
         <v>987</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A35" s="89" t="inlineStr">
         <is>
           <t xml:space="preserve">Cycle-average pH (activity scale, as a probe reads)</t>
+        </is>
+      </c>
+      <c r="B35" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_pH</t>
         </is>
       </c>
       <c r="C35" s="20"/>
@@ -8600,9 +8728,14 @@
         </is>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="89" t="s">
         <v>1128</v>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_Cl2</t>
+        </is>
       </c>
       <c r="C36" s="20" t="s">
         <v>102</v>
@@ -8635,7 +8768,11 @@
       <c r="A38" s="89" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="102"/>
+      <c r="B38" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_DO_ss</t>
+        </is>
+      </c>
       <c r="C38" s="20" t="s">
         <v>102</v>
       </c>
@@ -8657,7 +8794,11 @@
           <t xml:space="preserve">Carbon-limited sparge interval</t>
         </is>
       </c>
-      <c r="B39" s="102"/>
+      <c r="B39" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_int_carbon</t>
+        </is>
+      </c>
       <c r="C39" s="20" t="s">
         <v>67</v>
       </c>
@@ -8679,7 +8820,11 @@
       <c r="A40" s="89" t="s">
         <v>106</v>
       </c>
-      <c r="B40" s="20"/>
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_tip_speed</t>
+        </is>
+      </c>
       <c r="C40" s="20" t="s">
         <v>107</v>
       </c>
@@ -8699,7 +8844,11 @@
       <c r="A41" s="89" t="s">
         <v>109</v>
       </c>
-      <c r="B41" s="20"/>
+      <c r="B41" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_carbon_margin</t>
+        </is>
+      </c>
       <c r="C41" s="20" t="s">
         <v>110</v>
       </c>
@@ -8720,9 +8869,14 @@
         <v>1278</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" x14ac:dyDescent="0.2">
       <c r="A43" s="89" t="s">
         <v>1279</v>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_I_mA</t>
+        </is>
       </c>
       <c r="C43" s="20" t="s">
         <v>325</v>
@@ -8739,9 +8893,14 @@
         <v>1280</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" x14ac:dyDescent="0.2">
       <c r="A44" s="89" t="s">
         <v>1281</v>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_j_anode</t>
+        </is>
       </c>
       <c r="C44" s="20" t="s">
         <v>1282</v>
@@ -8758,9 +8917,14 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" x14ac:dyDescent="0.2">
       <c r="A45" s="89" t="s">
         <v>1284</v>
+      </c>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_j_status</t>
+        </is>
       </c>
       <c r="D45" s="90" t="str">
         <f>Electrochemistry!$D$62</f>
@@ -8774,9 +8938,14 @@
         <v>1285</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" x14ac:dyDescent="0.2">
       <c r="A46" s="89" t="s">
         <v>1286</v>
+      </c>
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_power_max</t>
+        </is>
       </c>
       <c r="C46" s="20" t="s">
         <v>45</v>
@@ -8793,9 +8962,14 @@
         <v>1287</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" x14ac:dyDescent="0.2">
       <c r="A47" s="89" t="s">
         <v>1288</v>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_I_max</t>
+        </is>
       </c>
       <c r="C47" s="20" t="s">
         <v>325</v>
@@ -8812,9 +8986,14 @@
         <v>1289</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" x14ac:dyDescent="0.2">
       <c r="A48" s="89" t="s">
         <v>1290</v>
+      </c>
+      <c r="B48" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_j_anode_max</t>
+        </is>
       </c>
       <c r="C48" s="20" t="s">
         <v>1282</v>
@@ -8831,9 +9010,14 @@
         <v>1291</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" x14ac:dyDescent="0.2">
       <c r="A49" s="89" t="s">
         <v>1292</v>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_j_status_max</t>
+        </is>
       </c>
       <c r="D49" s="90" t="str">
         <f>Electrochemistry!$D$76</f>
@@ -9298,9 +9482,14 @@
         </is>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>1652</v>
+      </c>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_etaF</t>
+        </is>
       </c>
       <c r="C82" s="19" t="s">
         <v>1274</v>
@@ -9319,9 +9508,14 @@
         </is>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>1742</v>
+      </c>
+      <c r="B83" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_V_cell</t>
+        </is>
       </c>
       <c r="C83" s="19" t="s">
         <v>1595</v>
@@ -9338,9 +9532,14 @@
         <v>1867</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>1751</v>
+      </c>
+      <c r="B84" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_V_flag</t>
+        </is>
       </c>
       <c r="C84" s="19" t="s">
         <v>1274</v>
@@ -9357,9 +9556,14 @@
         <v>1868</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>1683</v>
+      </c>
+      <c r="B85" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_H2O2_flag</t>
+        </is>
       </c>
       <c r="C85" s="19" t="s">
         <v>1274</v>
@@ -9376,9 +9580,14 @@
         <v>1869</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>1870</v>
+      </c>
+      <c r="B86" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_buffer_flag</t>
+        </is>
       </c>
       <c r="C86" s="19" t="s">
         <v>1274</v>
@@ -9395,10 +9604,15 @@
         <v>1871</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" x14ac:dyDescent="0.2">
       <c r="A87" t="inlineStr">
         <is>
           <t xml:space="preserve">HOCl/Cl⁻ couple minus anode potential</t>
+        </is>
+      </c>
+      <c r="B87" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_E_Cl_margin</t>
         </is>
       </c>
       <c r="C87" s="19" t="s">
@@ -9418,9 +9632,14 @@
         </is>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>1600</v>
+      </c>
+      <c r="B88" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_E_Cu_margin</t>
+        </is>
       </c>
       <c r="C88" s="19" t="s">
         <v>1595</v>
@@ -9439,9 +9658,14 @@
         </is>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>1622</v>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_pH_probe</t>
+        </is>
       </c>
       <c r="C89" s="19" t="s">
         <v>1274</v>
@@ -9458,9 +9682,14 @@
         <v>1874</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>1875</v>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_kLa_req</t>
+        </is>
       </c>
       <c r="C90" s="19" t="s">
         <v>639</v>

</xml_diff>

<commit_message>
Gas model: superseded Geometry and Mass Transfer rows cleared; note fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -50,7 +50,6 @@
     <definedName name="C_eff_lo" localSheetId="3">Chemistry!$D$156</definedName>
     <definedName name="C_H2_sat" localSheetId="4">Biology!$D$41</definedName>
     <definedName name="C_sat_CO2" localSheetId="5">'Mass Transfer'!$D$145</definedName>
-    <definedName name="Ca_CO2" localSheetId="5">'Mass Transfer'!$D$157</definedName>
     <definedName name="cal_Dint">Calibrations!$D$75</definedName>
     <definedName name="cal_DO_impair">Calibrations!$D$105</definedName>
     <definedName name="cal_DO_min">Calibrations!$D$103</definedName>
@@ -76,7 +75,6 @@
     <definedName name="cath_j_max" localSheetId="2">Electrochemistry!$D$53</definedName>
     <definedName name="cathode_dia" localSheetId="2">Electrochemistry!$D$44</definedName>
     <definedName name="cathode_shape" localSheetId="2">Electrochemistry!$D$43</definedName>
-    <definedName name="Cb_CO2" localSheetId="5">'Mass Transfer'!$D$158</definedName>
     <definedName name="Cl_kill" localSheetId="3">Chemistry!$D$147</definedName>
     <definedName name="Cl_mc02" localSheetId="3">Chemistry!$D$38</definedName>
     <definedName name="Cl_onset" localSheetId="3">Chemistry!$D$146</definedName>
@@ -86,18 +84,14 @@
     <definedName name="CO2_carbon_margin" localSheetId="4">Biology!$D$35</definedName>
     <definedName name="CO2_cons" localSheetId="4">Biology!$D$15</definedName>
     <definedName name="CO2_cons" localSheetId="5">'Mass Transfer'!$D$10</definedName>
-    <definedName name="CO2_cyc_avg" localSheetId="5">'Mass Transfer'!$D$161</definedName>
     <definedName name="CO2_cyc_avg_new" localSheetId="5">'Mass Transfer'!$D$200</definedName>
     <definedName name="CO2_diss" localSheetId="4">Biology!$D$33</definedName>
-    <definedName name="CO2_int_off" localSheetId="5">'Mass Transfer'!$D$160</definedName>
-    <definedName name="CO2_int_on" localSheetId="5">'Mass Transfer'!$D$159</definedName>
     <definedName name="CO2_pulse" localSheetId="5">'Mass Transfer'!$D$123</definedName>
     <definedName name="CO2_rate_full" localSheetId="5">'Mass Transfer'!$D$178</definedName>
     <definedName name="CO2_sd_ratio" localSheetId="5">'Mass Transfer'!$D$126</definedName>
     <definedName name="CO2_supply" localSheetId="5">'Mass Transfer'!$D$100</definedName>
     <definedName name="CO2aqc" localSheetId="3">Chemistry!$D$5</definedName>
     <definedName name="CO2aqc_ss" localSheetId="5">'Mass Transfer'!$D$162</definedName>
-    <definedName name="coef_CO2" localSheetId="5">'Mass Transfer'!$D$156</definedName>
     <definedName name="corr_I_frac" localSheetId="3">Chemistry!$D$158</definedName>
     <definedName name="d_bubble" localSheetId="5">'Mass Transfer'!$D$42</definedName>
     <definedName name="d_bubble_mm" localSheetId="5">'Mass Transfer'!$D$43</definedName>
@@ -105,8 +99,6 @@
     <definedName name="D_CO2_ref" localSheetId="5">'Mass Transfer'!$D$174</definedName>
     <definedName name="D_HPO4" localSheetId="3">Chemistry!$D$214</definedName>
     <definedName name="D_int" localSheetId="1">Geometry!$D$22</definedName>
-    <definedName name="D_int_1" localSheetId="1">Geometry!$D$12</definedName>
-    <definedName name="D_int_2" localSheetId="1">Geometry!$D$13</definedName>
     <definedName name="D_O2" localSheetId="5">'Mass Transfer'!$D$32</definedName>
     <definedName name="d_orifice" localSheetId="5">'Mass Transfer'!$D$41</definedName>
     <definedName name="delta_diff" localSheetId="3">Chemistry!$D$215</definedName>
@@ -150,8 +142,6 @@
     <definedName name="E0_HER" localSheetId="3">Chemistry!$D$202</definedName>
     <definedName name="E0_OER" localSheetId="3">Chemistry!$D$201</definedName>
     <definedName name="E0_ORR2" localSheetId="3">Chemistry!$D$204</definedName>
-    <definedName name="e1_CO2" localSheetId="5">'Mass Transfer'!$D$154</definedName>
-    <definedName name="e2_CO2" localSheetId="5">'Mass Transfer'!$D$155</definedName>
     <definedName name="Ea_D_CO2" localSheetId="5">'Mass Transfer'!$D$175</definedName>
     <definedName name="ec_corr_I" localSheetId="2">Electrochemistry!$D$102</definedName>
     <definedName name="ec_D_O2" localSheetId="2">Electrochemistry!$D$81</definedName>
@@ -176,7 +166,6 @@
     <definedName name="electrode_sel" localSheetId="2">Electrochemistry!$D$8</definedName>
     <definedName name="electrode_sel" localSheetId="0">Summary!$D$3</definedName>
     <definedName name="ElectrodeList">Electrochemistry!$A$35:$A$38</definedName>
-    <definedName name="eon_CO2" localSheetId="5">'Mass Transfer'!$D$153</definedName>
     <definedName name="eta_anode" localSheetId="2">Electrochemistry!$D$111</definedName>
     <definedName name="eta_cath" localSheetId="2">Electrochemistry!$D$112</definedName>
     <definedName name="etaF" localSheetId="2">Electrochemistry!$D$18</definedName>
@@ -551,20 +540,12 @@
     <definedName name="V_rail" localSheetId="2">Electrochemistry!$D$120</definedName>
     <definedName name="V_vial_total" localSheetId="1">Geometry!$D$24</definedName>
     <definedName name="vent_floor_chk" localSheetId="5">'Mass Transfer'!$D$163</definedName>
-    <definedName name="ver_name_1" localSheetId="1">Geometry!$D$8</definedName>
-    <definedName name="ver_name_2" localSheetId="1">Geometry!$D$9</definedName>
     <definedName name="Vg_CO2" localSheetId="5">'Mass Transfer'!$D$192</definedName>
     <definedName name="vial_ID" localSheetId="1">Geometry!$D$20</definedName>
     <definedName name="vial_ID" localSheetId="5">'Mass Transfer'!$D$15</definedName>
     <definedName name="vial_OD" localSheetId="1">Geometry!$D$18</definedName>
-    <definedName name="vial_OD_1" localSheetId="1">Geometry!$D$10</definedName>
-    <definedName name="vial_OD_2" localSheetId="1">Geometry!$D$11</definedName>
     <definedName name="vial_wall" localSheetId="1">Geometry!$D$19</definedName>
     <definedName name="VLc" localSheetId="3">Chemistry!$D$8</definedName>
-    <definedName name="Vmax_1" localSheetId="1">Geometry!$D$14</definedName>
-    <definedName name="Vmax_2" localSheetId="1">Geometry!$D$15</definedName>
-    <definedName name="Vtot_1" localSheetId="1">Geometry!$D$16</definedName>
-    <definedName name="Vtot_2" localSheetId="1">Geometry!$D$17</definedName>
     <definedName name="We_orifice" localSheetId="5">'Mass Transfer'!$D$63</definedName>
     <definedName name="xtube_n" localSheetId="1">Geometry!$D$46</definedName>
     <definedName name="xtube_OD" localSheetId="1">Geometry!$D$45</definedName>
@@ -10009,210 +9990,110 @@
       <c r="I7" s="20"/>
     </row>
     <row r="8" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D8" s="136" t="s">
-        <v>139</v>
-      </c>
-      <c r="E8" s="107" t="s">
-        <v>140</v>
-      </c>
+      <c r="A8" s="17"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="136"/>
+      <c r="E8" s="107"/>
       <c r="F8" s="20"/>
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
       <c r="I8" s="20"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D9" s="136" t="s">
-        <v>143</v>
-      </c>
-      <c r="E9" s="107" t="s">
-        <v>140</v>
-      </c>
+      <c r="A9" s="17"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="136"/>
+      <c r="E9" s="107"/>
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
       <c r="H9" s="20"/>
       <c r="I9" s="20"/>
     </row>
     <row r="10" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
-        <v>144</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="D10" s="137">
-        <v>27.48</v>
-      </c>
-      <c r="E10" s="109" t="s">
-        <v>140</v>
-      </c>
+      <c r="A10" s="17"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="137"/>
+      <c r="E10" s="109"/>
       <c r="F10" s="20"/>
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
       <c r="I10" s="20"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="17" t="s">
-        <v>147</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="D11" s="137">
-        <v>27.48</v>
-      </c>
-      <c r="E11" s="110" t="s">
-        <v>140</v>
-      </c>
+      <c r="A11" s="17"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="137"/>
+      <c r="E11" s="110"/>
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
       <c r="H11" s="20"/>
       <c r="I11" s="20"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="D12" s="138">
-        <v>55</v>
-      </c>
-      <c r="E12" s="111" t="s">
-        <v>140</v>
-      </c>
+      <c r="A12" s="17"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="138"/>
+      <c r="E12" s="111"/>
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="B13" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="D13" s="138">
-        <v>95</v>
-      </c>
-      <c r="E13" s="111" t="s">
-        <v>140</v>
-      </c>
+      <c r="A13" s="17"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="138"/>
+      <c r="E13" s="111"/>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
       <c r="H13" s="20"/>
       <c r="I13" s="20"/>
     </row>
     <row r="14" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="17" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>154</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="138">
-        <v>16</v>
-      </c>
-      <c r="E14" s="109" t="s">
-        <v>140</v>
-      </c>
+      <c r="A14" s="17"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="138"/>
+      <c r="E14" s="109"/>
       <c r="F14" s="20"/>
       <c r="G14" s="20"/>
       <c r="H14" s="20"/>
       <c r="I14" s="20"/>
     </row>
     <row r="15" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="17" t="s">
-        <v>155</v>
-      </c>
-      <c r="B15" s="18" t="s">
-        <v>156</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D15" s="138">
-        <v>30</v>
-      </c>
-      <c r="E15" s="109" t="s">
-        <v>140</v>
-      </c>
+      <c r="A15" s="17"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="138"/>
+      <c r="E15" s="109"/>
       <c r="F15" s="20"/>
       <c r="G15" s="20"/>
       <c r="H15" s="20"/>
       <c r="I15" s="20"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>158</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16" s="138">
-        <v>20</v>
-      </c>
-      <c r="E16" s="112" t="s">
-        <v>140</v>
-      </c>
+      <c r="A16" s="17"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="138"/>
+      <c r="E16" s="112"/>
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
       <c r="H16" s="20"/>
       <c r="I16" s="20"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A17" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D17" s="138">
-        <v>42</v>
-      </c>
-      <c r="E17" s="112" t="s">
-        <v>140</v>
-      </c>
+      <c r="A17" s="17"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="138"/>
+      <c r="E17" s="112"/>
       <c r="F17" s="20"/>
       <c r="G17" s="20"/>
       <c r="H17" s="20"/>
@@ -18726,7 +18607,7 @@
       </c>
       <c r="E44" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests the lag-phase headspace mix (rows 84–85) against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin. Replaces a dissolved-H₂ turnover proxy, which said nothing about flammability.</t>
+          <t xml:space="preserve">Tests the lag-phase headspace mix (rows 84–85) against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin.</t>
         </is>
       </c>
       <c r="F44" s="101" t="inlineStr">
@@ -21085,8 +20966,10 @@
         <f>Biology!$D$60</f>
         <v>0.226086956522</v>
       </c>
-      <c r="E84" s="68" t="s">
-        <v>1479</v>
+      <c r="E84" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Imported from Biology D60: one definition of the target DO fraction, from the selected organism's measured band where there is one and from C. necator's 2.6/11.5 otherwise. Sizes the O₂ guards below.</t>
+        </is>
       </c>
       <c r="F84" s="20"/>
     </row>
@@ -21620,7 +21503,7 @@
       </c>
       <c r="E113" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests the carbon-limited interval against the same DO balance the schedule uses (D232). Replaces a test of DO_ss against the impairment level, which was circular (DO_ss sits at the target by construction) and invited an unsafe 185 min interval.</t>
+          <t xml:space="preserve">Tests the carbon-limited interval against the same DO balance the schedule uses (D232). DO_ss cannot test it: it sits at the target by construction.</t>
         </is>
       </c>
       <c r="F113" s="20"/>
@@ -22302,174 +22185,75 @@
       <c r="F152" s="20"/>
     </row>
     <row r="153" spans="1:6" ht="24" x14ac:dyDescent="0.2">
-      <c r="A153" s="17" t="s">
-        <v>1191</v>
-      </c>
-      <c r="B153" s="18" t="s">
-        <v>1192</v>
-      </c>
-      <c r="C153" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D153" s="48">
-        <f>EXP(-kLa_CO2_off*t_on_CO2)</f>
-        <v>0.994477630348</v>
-      </c>
-      <c r="E153" s="67" t="s">
-        <v>1860</v>
-      </c>
+      <c r="A153" s="17"/>
+      <c r="B153" s="18"/>
+      <c r="C153" s="19"/>
+      <c r="D153" s="48"/>
+      <c r="E153" s="67"/>
       <c r="F153" s="20"/>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A154" s="17" t="s">
-        <v>1193</v>
-      </c>
-      <c r="B154" s="18" t="s">
-        <v>1194</v>
-      </c>
-      <c r="C154" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D154" s="48">
-        <f>EXP(-kLa_CO2_off*t_off_CO2)</f>
-        <v>0.0009435803483064</v>
-      </c>
-      <c r="E154" s="67" t="s">
-        <v>1195</v>
-      </c>
+      <c r="A154" s="17"/>
+      <c r="B154" s="18"/>
+      <c r="C154" s="19"/>
+      <c r="D154" s="48"/>
+      <c r="E154" s="67"/>
       <c r="F154" s="20"/>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A155" s="17" t="s">
-        <v>1196</v>
-      </c>
-      <c r="B155" s="18" t="s">
-        <v>1197</v>
-      </c>
-      <c r="C155" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D155" s="48">
-        <f>EXP(-k_vent*t_off_CO2)</f>
-        <v>0.042942523813</v>
-      </c>
-      <c r="E155" s="67" t="s">
-        <v>1198</v>
-      </c>
+      <c r="A155" s="17"/>
+      <c r="B155" s="18"/>
+      <c r="C155" s="19"/>
+      <c r="D155" s="48"/>
+      <c r="E155" s="67"/>
       <c r="F155" s="20"/>
     </row>
     <row r="156" spans="1:6" ht="24" x14ac:dyDescent="0.2">
-      <c r="A156" s="17" t="s">
-        <v>1199</v>
-      </c>
-      <c r="B156" s="18" t="s">
-        <v>1200</v>
-      </c>
-      <c r="C156" s="19" t="s">
-        <v>460</v>
-      </c>
-      <c r="D156" s="48">
-        <f>(C_sat_CO2-C_air_CO2)*kLa_CO2_off/(kLa_CO2_off-k_vent)</f>
-        <v>60.982216114206</v>
-      </c>
-      <c r="E156" s="67" t="s">
-        <v>1861</v>
-      </c>
+      <c r="A156" s="17"/>
+      <c r="B156" s="18"/>
+      <c r="C156" s="19"/>
+      <c r="D156" s="48"/>
+      <c r="E156" s="67"/>
       <c r="F156" s="20"/>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A157" s="17" t="s">
-        <v>1201</v>
-      </c>
-      <c r="B157" s="18" t="s">
-        <v>1202</v>
-      </c>
-      <c r="C157" s="19" t="s">
-        <v>460</v>
-      </c>
-      <c r="D157" s="48">
-        <f>(e1_CO2*C_sat_CO2*(1-eon_CO2)+C_air_CO2*(1-e1_CO2)+coef_CO2*(e2_CO2-e1_CO2))/(1-e1_CO2*eon_CO2)</f>
-        <v>2.576968575334</v>
-      </c>
-      <c r="E157" s="67" t="s">
-        <v>1862</v>
-      </c>
+      <c r="A157" s="17"/>
+      <c r="B157" s="18"/>
+      <c r="C157" s="19"/>
+      <c r="D157" s="48"/>
+      <c r="E157" s="67"/>
       <c r="F157" s="20"/>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A158" s="17" t="s">
-        <v>1203</v>
-      </c>
-      <c r="B158" s="18" t="s">
-        <v>1204</v>
-      </c>
-      <c r="C158" s="19" t="s">
-        <v>460</v>
-      </c>
-      <c r="D158" s="48">
-        <f>C_sat_CO2+(Ca_CO2-C_sat_CO2)*eon_CO2</f>
-        <v>2.747390456932</v>
-      </c>
-      <c r="E158" s="67" t="s">
-        <v>1863</v>
-      </c>
+      <c r="A158" s="17"/>
+      <c r="B158" s="18"/>
+      <c r="C158" s="19"/>
+      <c r="D158" s="48"/>
+      <c r="E158" s="67"/>
       <c r="F158" s="20"/>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A159" s="17" t="s">
-        <v>1205</v>
-      </c>
-      <c r="B159" s="18" t="s">
-        <v>1149</v>
-      </c>
-      <c r="C159" s="19" t="s">
-        <v>1150</v>
-      </c>
-      <c r="D159" s="48">
-        <f>C_sat_CO2*t_on_CO2+(Ca_CO2-C_sat_CO2)/kLa_CO2_off*(1-eon_CO2)</f>
-        <v>2.088576269438</v>
-      </c>
-      <c r="E159" s="67" t="s">
-        <v>1206</v>
-      </c>
+      <c r="A159" s="17"/>
+      <c r="B159" s="18"/>
+      <c r="C159" s="19"/>
+      <c r="D159" s="48"/>
+      <c r="E159" s="67"/>
       <c r="F159" s="20"/>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A160" s="17" t="s">
-        <v>1207</v>
-      </c>
-      <c r="B160" s="18" t="s">
-        <v>1151</v>
-      </c>
-      <c r="C160" s="19" t="s">
-        <v>1150</v>
-      </c>
-      <c r="D160" s="48">
-        <f>C_air_CO2*t_off_CO2+(Cb_CO2-C_air_CO2)/kLa_CO2_off*(1-e1_CO2)+coef_CO2*((1-e2_CO2)/k_vent-(1-e1_CO2)/kLa_CO2_off)</f>
-        <v>10065.36403274</v>
-      </c>
-      <c r="E160" s="67" t="s">
-        <v>1208</v>
-      </c>
+      <c r="A160" s="17"/>
+      <c r="B160" s="18"/>
+      <c r="C160" s="19"/>
+      <c r="D160" s="48"/>
+      <c r="E160" s="67"/>
       <c r="F160" s="20"/>
     </row>
     <row r="161" spans="1:6" ht="36" x14ac:dyDescent="0.2">
-      <c r="A161" s="17" t="s">
-        <v>1152</v>
-      </c>
-      <c r="B161" s="18" t="s">
-        <v>1153</v>
-      </c>
-      <c r="C161" s="19" t="s">
-        <v>460</v>
-      </c>
-      <c r="D161" s="48">
-        <f>(CO2_int_on+CO2_int_off)/(t_on_CO2+t_off_CO2)</f>
-        <v>10.193630870628</v>
-      </c>
-      <c r="E161" s="67" t="s">
-        <v>1864</v>
-      </c>
+      <c r="A161" s="17"/>
+      <c r="B161" s="18"/>
+      <c r="C161" s="19"/>
+      <c r="D161" s="48"/>
+      <c r="E161" s="67"/>
       <c r="F161" s="20"/>
     </row>
     <row r="162" spans="1:6" ht="24" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Gas model: chlorine recycling, ORR electrons, cell-voltage geometry, lag peroxide, trough carbon margin, pulse rounding
Interval 16.46 -> 17.88 min (as run 0.8 s / 18 min); chlorine 0.50 -> 0.34 mg/L as Cl2;
cathodic etaF 0.977 -> 0.958; cell voltage 3.26 -> 2.85 V. Excel-verified; twin 210/210.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -661,6 +661,31 @@
     <definedName name="res_E_Cu_margin" localSheetId="0">Summary!$D$88</definedName>
     <definedName name="res_pH_probe" localSheetId="0">Summary!$D$89</definedName>
     <definedName name="res_kLa_req" localSheetId="0">Summary!$D$90</definedName>
+    <definedName name="k_Cl_turn" localSheetId="3">Chemistry!$D$271</definedName>
+    <definedName name="n_ORR_eff" localSheetId="2">Electrochemistry!$D$141</definedName>
+    <definedName name="I_at_gerrit_max" localSheetId="2">Electrochemistry!$D$142</definedName>
+    <definedName name="V_at_gerrit_max" localSheetId="2">Electrochemistry!$D$143</definedName>
+    <definedName name="V_gerrit_flag" localSheetId="2">Electrochemistry!$D$144</definedName>
+    <definedName name="f_HOR_anode" localSheetId="2">Electrochemistry!$D$145</definedName>
+    <definedName name="ec_C_H2_sat" localSheetId="2">Electrochemistry!$D$146</definedName>
+    <definedName name="i_HOR_lim" localSheetId="2">Electrochemistry!$D$147</definedName>
+    <definedName name="f_HOR_lim" localSheetId="2">Electrochemistry!$D$148</definedName>
+    <definedName name="r_H2_HOR" localSheetId="2">Electrochemistry!$D$149</definedName>
+    <definedName name="H2_HOR_b" localSheetId="4">Biology!$D$96</definedName>
+    <definedName name="ec_DO_lag" localSheetId="2">Electrochemistry!$D$150</definedName>
+    <definedName name="k_H2O2_anode" localSheetId="2">Electrochemistry!$D$151</definedName>
+    <definedName name="r_H2O2_lag" localSheetId="2">Electrochemistry!$D$152</definedName>
+    <definedName name="km_O2_c" localSheetId="3">Chemistry!$D$272</definedName>
+    <definedName name="km_exp_c" localSheetId="3">Chemistry!$D$273</definedName>
+    <definedName name="D_O2_c" localSheetId="3">Chemistry!$D$274</definedName>
+    <definedName name="km_HPO4" localSheetId="3">Chemistry!$D$275</definedName>
+    <definedName name="km_HCO3" localSheetId="3">Chemistry!$D$276</definedName>
+    <definedName name="ca_rho_0" localSheetId="7">Calibrations!$D$155</definedName>
+    <definedName name="ca_rho_k" localSheetId="7">Calibrations!$D$156</definedName>
+    <definedName name="C_cycle_start_b" localSheetId="4">Biology!$D$97</definedName>
+    <definedName name="CO2_margin_trough" localSheetId="4">Biology!$D$98</definedName>
+    <definedName name="pulse_res" localSheetId="5">'Mass Transfer'!$D$241</definedName>
+    <definedName name="spg_dur_run" localSheetId="5">'Mass Transfer'!$D$242</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8233,8 +8258,10 @@
       <c r="G13" s="36"/>
     </row>
     <row r="14" spans="1:7" s="3" customFormat="1" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28" t="s">
-        <v>1059</v>
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ sparge duration (as run)</t>
+        </is>
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
@@ -8245,11 +8272,15 @@
         <v>13</v>
       </c>
       <c r="D14" s="91">
-        <f>IF(AND(ISNUMBER($G$13),$G$13&gt;0),$G$13,IF(NOT(ISNUMBER(D13)),D13,IF(D13&gt;round_split,ROUND(D13,0),ROUND(D13,1-(1+INT(LOG10(ABS(D13))))))))</f>
-        <v>1.0</v>
+        <f>IF(AND(ISNUMBER($G$13),$G$13&gt;0),$G$13,IF(NOT(ISNUMBER(D13)),D13,'Mass Transfer'!$D$242))</f>
+        <v>0.8</v>
       </c>
       <c r="E14" s="20"/>
-      <c r="F14" s="21"/>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse to type in: the optimum rounded to the solenoid command resolution (Mass Transfer D241–D242). An override in G13 wins.</t>
+        </is>
+      </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="89" t="s">
@@ -8265,7 +8296,7 @@
       </c>
       <c r="D15" s="90">
         <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$91)</f>
-        <v>16.46036421628</v>
+        <v>17.879338726534</v>
       </c>
       <c r="E15" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
@@ -8279,8 +8310,10 @@
       <c r="G15" s="36"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="28" t="s">
-        <v>1057</v>
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ sparge interval (as run)</t>
+        </is>
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
@@ -8291,11 +8324,15 @@
         <v>67</v>
       </c>
       <c r="D16" s="91">
-        <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,IF(D15&gt;round_split,ROUND(D15,0),ROUND(D15,1-(1+INT(LOG10(ABS(D15))))))))</f>
-        <v>16.0</v>
+        <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,ROUND(D14/(60*'Mass Transfer'!$D$93),0)))</f>
+        <v>18.0</v>
       </c>
       <c r="E16" s="92"/>
-      <c r="F16" s="21"/>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval to type in: recomputed from the as-run pulse at the optimised duty (Mass Transfer D93) and rounded to whole minutes, so rounding does not shift the CO₂ dose (row 95). An override in G15 wins.</t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="89"/>
@@ -8425,7 +8462,7 @@
       <c r="C23" s="20"/>
       <c r="D23" s="90" t="str">
         <f>'Mass Transfer'!$D$113</f>
-        <v>Do NOT relax: at the carbon-limited interval (185 min) DO would be 12.9 mg/L against a 2.6 mg/L target</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 12.6 mg/L against a 2.6 mg/L target</v>
       </c>
       <c r="E23" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
@@ -8451,7 +8488,7 @@
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 19%, O₂ 9% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 20%, O₂ 9% – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="23" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -8497,7 +8534,7 @@
       <c r="C26" s="20"/>
       <c r="D26" s="90" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)"),"calibrate this reactor first")</f>
-        <v>×22.5 OK</v>
+        <v>×21.1 OK</v>
       </c>
       <c r="E26" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
@@ -8697,7 +8734,7 @@
       <c r="C35" s="20"/>
       <c r="D35" s="121">
         <f>Chemistry!$D$220</f>
-        <v>6.603949596052</v>
+        <v>6.622298153844</v>
       </c>
       <c r="E35" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -8723,7 +8760,7 @@
       </c>
       <c r="D36" s="121">
         <f>Chemistry!$D$226</f>
-        <v>0.500804384457</v>
+        <v>0.33955111704</v>
       </c>
       <c r="E36" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
@@ -8785,7 +8822,7 @@
       </c>
       <c r="D39" s="90">
         <f>'Mass Transfer'!$D$112</f>
-        <v>185.240207036777</v>
+        <v>188.941031253092</v>
       </c>
       <c r="E39" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D112","→ Mass")</f>
@@ -8822,8 +8859,10 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A41" s="89" t="s">
-        <v>109</v>
+      <c r="A41" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carbon margin at the cycle trough</t>
+        </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
@@ -8834,15 +8873,17 @@
         <v>110</v>
       </c>
       <c r="D41" s="95">
-        <f>Biology!$D$35</f>
-        <v>668.745</v>
+        <f>Biology!$D$98</f>
+        <v>117.832076175326</v>
       </c>
       <c r="E41" s="23" t="str">
-        <f>HYPERLINK("#Biology!D35","→ Biology")</f>
+        <f>HYPERLINK("#Biology!D98","→ Biology")</f>
         <v>→ Biology</v>
       </c>
-      <c r="F41" s="21" t="s">
-        <v>111</v>
+      <c r="F41" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dissolved CO₂ at the lowest point of the dosing cycle vs RuBisCO Km (was the in-sparge saturation peak, which a sub-second pulse never reaches); large = ample carbon. Complements the supply:demand ratio (D26).</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
@@ -9432,8 +9473,10 @@
         <v>gerrit-current.md →</v>
       </c>
       <c r="E79" s="20"/>
-      <c r="F79" t="s">
-        <v>1909</v>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The voltage budget is a testable prediction (about 2.8 V of a 5 V rail at 3 %, 3.5 V at 10 %). A multimeter reading across the electrodes discriminates the cell-constant choice (k_geom 1 vs 2: 2.85 vs 3.26 V at 3 %) and, with the 25 % point, bounds the j₀ errors.</t>
+        </is>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
@@ -9477,7 +9520,7 @@
       </c>
       <c r="D82" s="22">
         <f>Electrochemistry!$D$88</f>
-        <v>0.977475298652</v>
+        <v>0.958329302507</v>
       </c>
       <c r="E82" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D88","→ Electrochemistry")</f>
@@ -9503,7 +9546,7 @@
       </c>
       <c r="D83" s="22">
         <f>Electrochemistry!$D$119</f>
-        <v>3.263760439016</v>
+        <v>2.847708123495</v>
       </c>
       <c r="E83" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D119","→ Electrochemistry")</f>
@@ -9527,7 +9570,7 @@
       </c>
       <c r="D84" s="22" t="str">
         <f>Electrochemistry!$D$122</f>
-        <v>OK — 3.26 V estimated against a 5 V rail</v>
+        <v>OK — 2.85 V estimated against a 5 V rail</v>
       </c>
       <c r="E84" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D122","→ Electrochemistry")</f>
@@ -9551,7 +9594,7 @@
       </c>
       <c r="D85" s="22" t="str">
         <f>Electrochemistry!$D$99</f>
-        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 13 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 7 min before biomass can scavenge it</v>
       </c>
       <c r="E85" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D99","→ Electrochemistry")</f>
@@ -9601,7 +9644,7 @@
       </c>
       <c r="D87" s="22">
         <f>Chemistry!$D$209</f>
-        <v>-0.422483519032</v>
+        <v>-0.413578182478</v>
       </c>
       <c r="E87" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D209","→ Chemistry")</f>
@@ -9627,7 +9670,7 @@
       </c>
       <c r="D88" s="22">
         <f>Chemistry!$D$211</f>
-        <v>1.240557060036</v>
+        <v>1.239471571289</v>
       </c>
       <c r="E88" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
@@ -9653,7 +9696,7 @@
       </c>
       <c r="D89" s="22">
         <f>Chemistry!$D$220</f>
-        <v>6.603949596052</v>
+        <v>6.622298153844</v>
       </c>
       <c r="E89" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -9677,7 +9720,7 @@
       </c>
       <c r="D90" s="22">
         <f>'Mass Transfer'!$D$186</f>
-        <v>0.003317773486</v>
+        <v>0.00317292045</v>
       </c>
       <c r="E90" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D186","→ Mass Transfer")</f>
@@ -9715,7 +9758,32 @@
       </c>
       <c r="E93" s="87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Defined display rule for rows 14 and 16: whole units above this value, else two significant figures.</t>
+          <t xml:space="preserve">Former display rule for rows 14 and 16 (whole units above this value, else two significant figures); superseded by the pulse-resolution rounding (Mass Transfer D241) and no longer referenced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As-run duty ÷ optimised duty</t>
+        </is>
+      </c>
+      <c r="C95" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">×</t>
+        </is>
+      </c>
+      <c r="D95" s="95">
+        <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),D14/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (see CO2 flows)")</f>
+        <v>1.012905109625</v>
+      </c>
+      <c r="E95" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
+        <v>→ Mass</v>
+      </c>
+      <c r="F95" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duty of the schedule as typed in (rows 14 and 16) against the optimised duty; 1 = rounding has not moved the CO₂ dose, pH or DO. Should sit within a few per cent.</t>
         </is>
       </c>
     </row>
@@ -11930,7 +11998,7 @@
       </c>
       <c r="D18" s="42">
         <f>IF(ISNUMBER(cal_etaF),cal_etaF,etaF_calc)</f>
-        <v>0.977475298652</v>
+        <v>0.958329302507</v>
       </c>
       <c r="E18" s="67" t="inlineStr">
         <is>
@@ -11998,7 +12066,7 @@
       </c>
       <c r="D21" s="48">
         <f>I_app*etaF/(z_e_H2*F_const)*3600</f>
-        <v>0.000103759833633</v>
+        <v>0.0001017274698715</v>
       </c>
       <c r="E21" s="99" t="s">
         <v>355</v>
@@ -12020,7 +12088,7 @@
       </c>
       <c r="D22" s="48">
         <f>I_app*etaF_OER/(z_e_O2*F_const)*3600</f>
-        <v>5.175288675179e-05</v>
+        <v>5.043034859204e-05</v>
       </c>
       <c r="E22" s="99" t="s">
         <v>358</v>
@@ -12042,7 +12110,7 @@
       </c>
       <c r="D23" s="48">
         <f>rH2_gen/60*R_gas*T_K/P_atm*1000000</f>
-        <v>0.042308770289</v>
+        <v>0.041480060291</v>
       </c>
       <c r="E23" s="99" t="s">
         <v>362</v>
@@ -12064,7 +12132,7 @@
       </c>
       <c r="D24" s="48">
         <f>rO2_gen/60*R_gas*T_K/P_atm*1000000</f>
-        <v>0.021102587781</v>
+        <v>0.020563313948</v>
       </c>
       <c r="E24" s="99" t="s">
         <v>365</v>
@@ -12086,7 +12154,7 @@
       </c>
       <c r="D25" s="48">
         <f>V_H2_gen+V_O2_gen</f>
-        <v>0.063411358069</v>
+        <v>0.062043374238</v>
       </c>
       <c r="E25" s="99" t="s">
         <v>368</v>
@@ -12108,11 +12176,11 @@
       </c>
       <c r="D26" s="42">
         <f>IF(ISNUMBER(cal_etaF_OER),cal_etaF_OER,etaF_OER_calc)</f>
-        <v>0.975081911036</v>
+        <v>0.950163822072</v>
       </c>
       <c r="E26" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anodic O₂ faradaic efficiency: measured if available, otherwise CALCULATED (etaF_OER_calc) as 1 − the chlorine share − the metal-dissolution share. UdG contains chloride, so the chlorine current is modelled explicitly (D101).</t>
+          <t xml:space="preserve">Anodic O₂ faradaic efficiency: measured if available, otherwise CALCULATED (etaF_OER_calc) as 1 − the chlorine share − the metal-dissolution share − the anodic H₂-oxidation share. UdG contains chloride, so the chlorine current is modelled explicitly (D101). The faradaic-efficiency screen measures the sum of cathodic ORR and anodic HOR losses.</t>
         </is>
       </c>
       <c r="F26" s="20"/>
@@ -12121,8 +12189,10 @@
       <c r="I26" s="20"/>
     </row>
     <row r="27" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="17" t="s">
-        <v>371</v>
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrons per O₂ on the peroxide branch (cathode)</t>
+        </is>
       </c>
       <c r="B27" s="18" t="s">
         <v>372</v>
@@ -12134,8 +12204,10 @@
         <f>VLOOKUP(electrode_sel,$A$35:$I$38,9,FALSE)</f>
         <v>2.0</v>
       </c>
-      <c r="E27" s="114" t="s">
-        <v>373</v>
+      <c r="E27" s="114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode lookup: 2 e⁻ per O₂ on the peroxide branch (SS cathode, neutral pH) for every current electrode. The current drawn per O₂ is the weighted n_ORR_eff (D141), not this value.</t>
+        </is>
       </c>
       <c r="F27" s="20"/>
       <c r="G27" s="20"/>
@@ -12153,11 +12225,13 @@
         <v>354</v>
       </c>
       <c r="D28" s="48">
-        <f>I_app*(1-etaF)/(z_e_ORR*F_const)*3600</f>
+        <f>I_app*(1-etaF)/(n_ORR_eff*F_const)*3600</f>
         <v>2.391016190066e-06</v>
       </c>
-      <c r="E28" s="99" t="s">
-        <v>376</v>
+      <c r="E28" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moles of O₂ reduced: the non-H₂ cathodic current (1−etaF) divided by n_ORR_eff·F. Equals the transport-limited O₂ flux when etaF is calculated; stays consistent if a measured etaF is in use. 0 at etaF = 1.</t>
+        </is>
       </c>
       <c r="F28" s="20"/>
       <c r="G28" s="20"/>
@@ -12176,7 +12250,7 @@
       </c>
       <c r="D29" s="48">
         <f>rO2_gen-O2_cathode_ORR</f>
-        <v>4.936187056172e-05</v>
+        <v>4.803933240197e-05</v>
       </c>
       <c r="E29" s="99" t="s">
         <v>379</v>
@@ -12187,8 +12261,10 @@
       <c r="I29" s="20"/>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A30" s="101" t="s">
-        <v>380</v>
+      <c r="A30" s="101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z_e_ORR = 2 is the peroxide branch only; the current per O₂ is n_ORR_eff (D141, 2 and 4 e⁻ weighted by f_HOOH). etaF unmeasured — both live here per electrode.</t>
+        </is>
       </c>
       <c r="B30" s="20"/>
       <c r="C30" s="20"/>
@@ -13240,11 +13316,13 @@
         <v>1076</v>
       </c>
       <c r="D86" s="141">
-        <f>z_e_ORR*F_const*(km_O2/100)*ec_DO_design*(A_cath_wet/10000)</f>
-        <v>0.0001281655506682</v>
-      </c>
-      <c r="E86" s="67" t="s">
-        <v>1648</v>
+        <f>n_ORR_eff*F_const*(km_O2/100)*ec_DO_design*(A_cath_wet/10000)</f>
+        <v>0.0002371062687363</v>
+      </c>
+      <c r="E86" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">i = n_ORR_eff·F·k_m·C·A, the O₂ mass-transport limit at the cathode charged at the effective electron count (D141). Current that does NOT make hydrogen, and it consumes dissolved O₂. Le Bozec 2001 (Corros Sci 43:765) show ORR on 316L in neutral solution running mixed 2e⁻/4e⁻ and limited by the passive film as much as by transport, so this is an upper bound on the loss.</t>
+        </is>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -13258,8 +13336,8 @@
         <v>1076</v>
       </c>
       <c r="D87" s="141">
-        <f>z_e_ORR*F_const*(km_O2/100)*ec_O2_ceil*(A_cath_wet/10000)</f>
-        <v>0.0005668860894942</v>
+        <f>n_ORR_eff*F_const*(km_O2/100)*ec_O2_ceil*(A_cath_wet/10000)</f>
+        <v>0.001048739266</v>
       </c>
       <c r="E87" s="67" t="s">
         <v>1651</v>
@@ -13277,7 +13355,7 @@
       </c>
       <c r="D88" s="141">
         <f>MAX(0,1-i_ORR_design/I_app)</f>
-        <v>0.977475298652</v>
+        <v>0.958329302507</v>
       </c>
       <c r="E88" s="67" t="inlineStr">
         <is>
@@ -13297,7 +13375,7 @@
       </c>
       <c r="D89" s="141">
         <f>MAX(0,1-i_ORR_ceiling/I_app)</f>
-        <v>0.90037151327</v>
+        <v>0.815687299549</v>
       </c>
       <c r="E89" s="67" t="s">
         <v>1657</v>
@@ -13353,12 +13431,12 @@
         <v>1266</v>
       </c>
       <c r="D93" s="141">
-        <f>f_HOOH*i_ORR_design/(2*F_const)*M_H2O2*1000*3600/ec_V_L</f>
+        <f>f_HOOH*I_app*(1-etaF)/(n_ORR_eff*F_const)*M_H2O2*1000*3600/ec_V_L</f>
         <v>0.813296984002</v>
       </c>
       <c r="E93" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 electrons per H₂O₂. This source runs whenever there is current and dissolved O₂.</t>
+          <t xml:space="preserve">Peroxide-branch share of the moles of O₂ reduced (f_HOOH × D28 flux), so it follows a measured etaF too. One H₂O₂ per O₂ on that branch. This source runs whenever there is current and dissolved O₂.</t>
         </is>
       </c>
     </row>
@@ -13408,11 +13486,13 @@
         <v>1270</v>
       </c>
       <c r="D96" s="141">
-        <f>r_H2O2</f>
-        <v>0.813296984002</v>
-      </c>
-      <c r="E96" s="67" t="s">
-        <v>1676</v>
+        <f>r_H2O2_lag/(k_H2O2_anode*3600)*(1-EXP(-k_H2O2_anode*3600))</f>
+        <v>0.740452814989</v>
+      </c>
+      <c r="E96" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No catalase pool at inoculation: peroxide accumulates at the lag-phase rate (D152) against the anodic sink (D151), approaching the plateau r/k. This is the exposed window.</t>
+        </is>
       </c>
     </row>
     <row r="97" spans="1:5" ht="60" x14ac:dyDescent="0.2">
@@ -13443,11 +13523,13 @@
         <v>962</v>
       </c>
       <c r="D98" s="141">
-        <f>IF(r_H2O2&gt;0,H2O2_thresh/r_H2O2*60,NA())</f>
-        <v>12.541544110741</v>
-      </c>
-      <c r="E98" s="67" t="s">
-        <v>1682</v>
+        <f>IF(r_H2O2_lag&gt;0,IF(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag&gt;0,-LN(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag)/k_H2O2_anode/60,NA()),NA())</f>
+        <v>6.785954745632</v>
+      </c>
+      <c r="E98" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time for an un-inoculated or just-inoculated vessel to pass the growth-inhibition threshold, with the anodic sink. #N/A = the plateau r/k never reaches the threshold.</t>
+        </is>
       </c>
     </row>
     <row r="99" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -13462,7 +13544,7 @@
       </c>
       <c r="D99" s="141" t="str">
         <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(H2O2_lag_1h&gt;H2O2_thresh,"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases"))</f>
-        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 13 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 7 min before biomass can scavenge it</v>
       </c>
       <c r="E99" s="67" t="s">
         <v>1685</v>
@@ -13485,7 +13567,7 @@
       </c>
       <c r="D101" s="141">
         <f>Chemistry!$D$133</f>
-        <v>0.0001417839262056</v>
+        <v>0.0002835678524112</v>
       </c>
       <c r="E101" s="67" t="s">
         <v>1689</v>
@@ -13521,10 +13603,12 @@
       </c>
       <c r="D103" s="141">
         <f>ec_I_Cl/I_app</f>
-        <v>0.024918088964</v>
-      </c>
-      <c r="E103" s="67" t="s">
-        <v>1695</v>
+        <v>0.049836177928</v>
+      </c>
+      <c r="E103" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chlorine evolution as a fraction of the applied current, at the chloride mass-transport limit (2 e⁻ per net chloride, Chemistry D132). The anode sits above the HOCl/Cl⁻ couple (Chemistry D209), so chlorine is accessible and transport-limited; the share is small only because UdG chloride is trace.</t>
+        </is>
       </c>
     </row>
     <row r="104" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -13538,12 +13622,12 @@
         <v>1274</v>
       </c>
       <c r="D104" s="141">
-        <f>MAX(0,1-f_Cl_anode-IF(ISNUMBER(ec_corr_I),ec_corr_I,0))</f>
-        <v>0.975081911036</v>
+        <f>MAX(0,1-f_Cl_anode-IF(ISNUMBER(ec_corr_I),ec_corr_I,0)-IF(ISNUMBER(f_HOR_anode),f_HOR_anode,0))</f>
+        <v>0.950163822072</v>
       </c>
       <c r="E104" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 − chlorine share − metal-dissolution share. It remains an UPPER BOUND while the metal-dissolution charge is unmeasured: a corroding anode takes current that this cell still credits to oxygen.</t>
+          <t xml:space="preserve">1 − chlorine share − metal-dissolution share − anodic H₂-oxidation share (f_HOR_anode, D145). It remains an UPPER BOUND while those charges are unmeasured: a corroding anode, or one oxidising crossed-over H₂ (ceiling ~22 %, D148), takes current that this cell still credits to oxygen.</t>
         </is>
       </c>
     </row>
@@ -13738,10 +13822,12 @@
         <v>1274</v>
       </c>
       <c r="D116" s="131">
-        <v>2</v>
-      </c>
-      <c r="E116" s="75" t="s">
-        <v>1734</v>
+        <v>1</v>
+      </c>
+      <c r="E116" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~1.2 by Gerrit’s Law holding linear to 25 % on a 5 V rail (D143–D144). Measure with a conductivity standard.</t>
+        </is>
       </c>
     </row>
     <row r="117" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -13756,7 +13842,7 @@
       </c>
       <c r="D117" s="141">
         <f>k_geom*ACOSH(ec_gap/anode_dia)/(PI()*ec_kappa*(L_sub/1000))</f>
-        <v>146.239829708796</v>
+        <v>73.119914854398</v>
       </c>
       <c r="E117" s="67" t="s">
         <v>1738</v>
@@ -13774,7 +13860,7 @@
       </c>
       <c r="D118" s="141">
         <f>I_app*R_cell</f>
-        <v>0.832104631043</v>
+        <v>0.416052315522</v>
       </c>
       <c r="E118" s="67" t="s">
         <v>1741</v>
@@ -13792,7 +13878,7 @@
       </c>
       <c r="D119" s="141">
         <f>ec_E_rev+eta_anode+eta_cath+pcet_credit+V_IR</f>
-        <v>3.263760439016</v>
+        <v>2.847708123495</v>
       </c>
       <c r="E119" s="67" t="s">
         <v>1744</v>
@@ -13827,7 +13913,7 @@
       </c>
       <c r="D121" s="141">
         <f>V_rail-V_cell_est</f>
-        <v>1.736239560984</v>
+        <v>2.152291876505</v>
       </c>
       <c r="E121" s="67" t="s">
         <v>1750</v>
@@ -13845,10 +13931,12 @@
       </c>
       <c r="D122" s="141" t="str">
         <f>IF(V_headroom&lt;0,"OVER RAIL — the drive cannot deliver this current; the linear current law will not hold",IF(V_headroom&lt;V_headroom_min,"watch — within "&amp;TEXT(V_headroom_min,"0")&amp;" V of the rail ("&amp;TEXT(V_cell_est,"0.00")&amp;" V of "&amp;TEXT(V_rail,"0")&amp;" V); expect the current law to bend","OK — "&amp;TEXT(V_cell_est,"0.00")&amp;" V estimated against a "&amp;TEXT(V_rail,"0")&amp;" V rail"))</f>
-        <v>OK — 3.26 V estimated against a 5 V rail</v>
-      </c>
-      <c r="E122" s="67" t="s">
-        <v>1753</v>
+        <v>OK — 2.85 V estimated against a 5 V rail</v>
+      </c>
+      <c r="E122" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cross-check on Gerrit's Law: the fit is validated linear to gerrit_max (25 %), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (about 4.7 V at 25 % with k_geom = 1).</t>
+        </is>
       </c>
     </row>
     <row r="124">
@@ -13930,6 +14018,322 @@
       <c r="E127" s="114" t="inlineStr">
         <is>
           <t xml:space="preserve">Design assumption: the current law starts to bend within this margin of the drive rail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PHYSICS CORRECTIONS — ORR electron count, voltage cross-check, anodic H₂ oxidation, lag-phase peroxide</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effective electrons per O₂ reduced (cathode)</t>
+        </is>
+      </c>
+      <c r="B141" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n_ORR_eff</t>
+        </is>
+      </c>
+      <c r="C141" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e⁻/O₂</t>
+        </is>
+      </c>
+      <c r="D141" s="141">
+        <f>z_e_ORR*f_HOOH+z_e_O2*(1-f_HOOH)</f>
+        <v>3.7</v>
+      </c>
+      <c r="E141" s="114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Effective electrons per O₂ reduced at the SS cathode: 2 on the peroxide branch (z_e_ORR), 4 to water (z_e_O2, direct or 2+2 in series), weighted by the RRDE escape fraction f_HOOH (Le Bozec 2001). This is the mixed 2e⁻/4e⁻ regime E86 cites.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Current at the top of the validated Gerrit band</t>
+        </is>
+      </c>
+      <c r="B142" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I_at_gerrit_max</t>
+        </is>
+      </c>
+      <c r="C142" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="D142" s="141">
+        <f>(gerrit_slope*gerrit_max+gerrit_int)/1000</f>
+        <v>0.02835</v>
+      </c>
+      <c r="E142" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gerrit's Law at gerrit_max (25 %), where the fit is still validated linear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cell voltage budget at the top of the validated band</t>
+        </is>
+      </c>
+      <c r="B143" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_at_gerrit_max</t>
+        </is>
+      </c>
+      <c r="C143" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="D143" s="141">
+        <f>ec_E_rev+b_anode*LOG10(I_at_gerrit_max/A_anode_wet/j0_anode)+b_cath*LOG10(I_at_gerrit_max/A_cath_wet/j0_cath)+pcet_credit+I_at_gerrit_max*R_cell</f>
+        <v>4.685940001272</v>
+      </c>
+      <c r="E143" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same budget as D119, evaluated at I_at_gerrit_max (j in A/cm²). A current source on the rail cannot deliver that current into a load needing more than V_rail, so this must not exceed V_rail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Voltage budget vs validated Gerrit band</t>
+        </is>
+      </c>
+      <c r="B144" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_gerrit_flag</t>
+        </is>
+      </c>
+      <c r="C144" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D144" s="141" t="str">
+        <f>IF(V_at_gerrit_max&gt;V_rail,"INCONSISTENT — the budget needs "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" %, above the "&amp;TEXT(V_rail,"0")&amp;" V rail, where Gerrit's Law is validated linear: R_cell (k_geom) or j₀ is too high","OK — "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" %, under the "&amp;TEXT(V_rail,"0")&amp;" V rail across the validated band")</f>
+        <v>OK — 4.69 V at 25 %, under the 5 V rail across the validated band</v>
+      </c>
+      <c r="E144" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Live form of the E122 cross-check: the voltage budget and the empirical current law must agree across the band the law is validated on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anodic current oxidising crossed-over H₂</t>
+        </is>
+      </c>
+      <c r="B145" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f_HOR_anode</t>
+        </is>
+      </c>
+      <c r="C145" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D145" s="131"/>
+      <c r="E145" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DATA GAP — fraction of the anodic current oxidising dissolved H₂ on the Pt anode (or recombining H₂ + O₂). Measure: anode-gas O₂ collection per faradaic-efficiency.md, or initial-slope vs plateau rates with a divided cell. Left empty = not modelled (0); transport ceiling D148.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) dissolved-H₂ saturation</t>
+        </is>
+      </c>
+      <c r="B146" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ec_C_H2_sat</t>
+        </is>
+      </c>
+      <c r="C146" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D146" s="141">
+        <f>Biology!$D$41</f>
+        <v>0.790335</v>
+      </c>
+      <c r="E146" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Biology (C_H2_sat, 1 atm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anodic H₂ oxidation — transport-limited ceiling</t>
+        </is>
+      </c>
+      <c r="B147" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">i_HOR_lim</t>
+        </is>
+      </c>
+      <c r="C147" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A</t>
+        </is>
+      </c>
+      <c r="D147" s="141">
+        <f>z_e_H2*F_const*(km_O2/100)*ec_C_H2_sat*(A_anode_wet/10000)</f>
+        <v>0.001228253194</v>
+      </c>
+      <c r="E147" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Informational ceiling: every H₂ molecule reaching the anode at k_m(O₂) and saturated H₂ is oxidised. The actual value depends on HOR activity of hydrous-oxide Pt at ~1.6 V (strongly suppressed; PEM anodes pass crossover H₂ largely unoxidised) — unmeasured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same, as a fraction of the applied current</t>
+        </is>
+      </c>
+      <c r="B148" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f_HOR_lim</t>
+        </is>
+      </c>
+      <c r="C148" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D148" s="141">
+        <f>i_HOR_lim/I_app</f>
+        <v>0.215861721249</v>
+      </c>
+      <c r="E148" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upper bound for f_HOR_anode (D145).</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ oxidised at the anode</t>
+        </is>
+      </c>
+      <c r="B149" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">r_H2_HOR</t>
+        </is>
+      </c>
+      <c r="C149" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D149" s="141">
+        <f>IF(ISNUMBER(f_HOR_anode),f_HOR_anode*I_app/(z_e_H2*F_const)*3600,0)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E149" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crossed-over H₂ consumed by the anode; 0 while f_HOR_anode is a data gap. Subtracted from the H₂ the culture receives (Biology H2_cons).</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) lag-phase dissolved O₂</t>
+        </is>
+      </c>
+      <c r="B150" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ec_DO_lag</t>
+        </is>
+      </c>
+      <c r="C150" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D150" s="141">
+        <f>'Mass Transfer'!$D$135</f>
+        <v>0.169683392542</v>
+      </c>
+      <c r="E150" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Mass Transfer (DO_ss_sawtooth_lag: steady DO with the lag source, no uptake)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anodic peroxide sink (transport-limited)</t>
+        </is>
+      </c>
+      <c r="B151" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_H2O2_anode</t>
+        </is>
+      </c>
+      <c r="C151" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/s</t>
+        </is>
+      </c>
+      <c r="D151" s="141">
+        <f>(km_O2/100)*(A_anode_wet/10000)/(ec_V_L/1000)</f>
+        <v>0.0005369009052374</v>
+      </c>
+      <c r="E151" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂O₂ is oxidised at the anode (E° 0.695 V, ~0.9 V below the anode potential) at the transport limit: k = k_m·A/V. Reuses the ferricyanide-measurable km_O2, so no new unknown; heterogeneous decomposition on Pt would add to it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peroxide production during lag</t>
+        </is>
+      </c>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">r_H2O2_lag</t>
+        </is>
+      </c>
+      <c r="C152" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L/h</t>
+        </is>
+      </c>
+      <c r="D152" s="141">
+        <f>r_H2O2*ec_DO_lag/ec_DO_design</f>
+        <v>1.673377324158</v>
+      </c>
+      <c r="E152" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">r_H2O2 scaled to the lag-phase DO (D150): the cathodic O₂ flux is first order in DO, and before uptake starts DO runs above the design value.</t>
         </is>
       </c>
     </row>
@@ -14042,7 +14446,7 @@
       </c>
       <c r="D5" s="64">
         <f>'Mass Transfer'!$D$162</f>
-        <v>0.008590210622</v>
+        <v>0.008068720944</v>
       </c>
       <c r="E5" s="51" t="inlineStr">
         <is>
@@ -14722,7 +15126,7 @@
       </c>
       <c r="B50" s="64">
         <f t="shared" ref="B50:B81" si="1">pH_SID + pH_NT*(10^-A50)/((10^-A50)+KaN_c) + (10^-A50) - (pH_PT*Ka1p_c*(10^-A50)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A50) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A50)^3 + Ka1p_c*(10^-A50)^2 + Ka1p_c*Ka2p_c*(10^-A50) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A50) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A50)^2 - Kw_c/(10^-A50)</f>
-        <v>0.033213926229</v>
+        <v>0.033217771584</v>
       </c>
       <c r="C50" s="64">
         <f>IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
@@ -14735,7 +15139,7 @@
       </c>
       <c r="B51" s="64">
         <f t="shared" si="1"/>
-        <v>0.033095991179</v>
+        <v>0.033100832196</v>
       </c>
       <c r="C51" s="64">
         <f>IF(AND(B51&gt;=0,B52&lt;0),A51+pH_step*B51/(B51-B52),0)</f>
@@ -14748,7 +15152,7 @@
       </c>
       <c r="B52" s="64">
         <f t="shared" si="1"/>
-        <v>0.032986799309</v>
+        <v>0.032992893794</v>
       </c>
       <c r="C52" s="64">
         <f>IF(AND(B52&gt;=0,B53&lt;0),A52+pH_step*B52/(B52-B53),0)</f>
@@ -14761,7 +15165,7 @@
       </c>
       <c r="B53" s="64">
         <f t="shared" si="1"/>
-        <v>0.032880652062</v>
+        <v>0.032888324572</v>
       </c>
       <c r="C53" s="64">
         <f>IF(AND(B53&gt;=0,B54&lt;0),A53+pH_step*B53/(B53-B54),0)</f>
@@ -14774,7 +15178,7 @@
       </c>
       <c r="B54" s="64">
         <f t="shared" si="1"/>
-        <v>0.032771986272</v>
+        <v>0.032781645403</v>
       </c>
       <c r="C54" s="64">
         <f>IF(AND(B54&gt;=0,B55&lt;0),A54+pH_step*B54/(B54-B55),0)</f>
@@ -14787,7 +15191,7 @@
       </c>
       <c r="B55" s="64">
         <f t="shared" si="1"/>
-        <v>0.032655096798</v>
+        <v>0.032667256944</v>
       </c>
       <c r="C55" s="64">
         <f>IF(AND(B55&gt;=0,B56&lt;0),A55+pH_step*B55/(B55-B56),0)</f>
@@ -14800,7 +15204,7 @@
       </c>
       <c r="B56" s="64">
         <f t="shared" si="1"/>
-        <v>0.032523849984</v>
+        <v>0.032539158733</v>
       </c>
       <c r="C56" s="64">
         <f>IF(AND(B56&gt;=0,B57&lt;0),A56+pH_step*B56/(B56-B57),0)</f>
@@ -14813,7 +15217,7 @@
       </c>
       <c r="B57" s="64">
         <f t="shared" si="1"/>
-        <v>0.032371376227</v>
+        <v>0.032390648851</v>
       </c>
       <c r="C57" s="64">
         <f>IF(AND(B57&gt;=0,B58&lt;0),A57+pH_step*B57/(B57-B58),0)</f>
@@ -14826,7 +15230,7 @@
       </c>
       <c r="B58" s="64">
         <f t="shared" si="1"/>
-        <v>0.032189729231</v>
+        <v>0.032213992108</v>
       </c>
       <c r="C58" s="64">
         <f>IF(AND(B58&gt;=0,B59&lt;0),A58+pH_step*B58/(B58-B59),0)</f>
@@ -14839,7 +15243,7 @@
       </c>
       <c r="B59" s="64">
         <f t="shared" si="1"/>
-        <v>0.031969498815</v>
+        <v>0.032000044096</v>
       </c>
       <c r="C59" s="64">
         <f>IF(AND(B59&gt;=0,B60&lt;0),A59+pH_step*B59/(B59-B60),0)</f>
@@ -14852,7 +15256,7 @@
       </c>
       <c r="B60" s="64">
         <f t="shared" si="1"/>
-        <v>0.031699363744</v>
+        <v>0.031737818179</v>
       </c>
       <c r="C60" s="64">
         <f>IF(AND(B60&gt;=0,B61&lt;0),A60+pH_step*B60/(B60-B61),0)</f>
@@ -14865,7 +15269,7 @@
       </c>
       <c r="B61" s="64">
         <f t="shared" si="1"/>
-        <v>0.031365571066</v>
+        <v>0.031413982653</v>
       </c>
       <c r="C61" s="64">
         <f>IF(AND(B61&gt;=0,B62&lt;0),A61+pH_step*B61/(B61-B62),0)</f>
@@ -14878,7 +15282,7 @@
       </c>
       <c r="B62" s="64">
         <f t="shared" si="1"/>
-        <v>0.030951329376</v>
+        <v>0.031012276465</v>
       </c>
       <c r="C62" s="64">
         <f>IF(AND(B62&gt;=0,B63&lt;0),A62+pH_step*B62/(B62-B63),0)</f>
@@ -14891,7 +15295,7 @@
       </c>
       <c r="B63" s="64">
         <f t="shared" si="1"/>
-        <v>0.030436105853</v>
+        <v>0.030512834504</v>
       </c>
       <c r="C63" s="64">
         <f>IF(AND(B63&gt;=0,B64&lt;0),A63+pH_step*B63/(B63-B64),0)</f>
@@ -14904,7 +15308,7 @@
       </c>
       <c r="B64" s="64">
         <f t="shared" si="1"/>
-        <v>0.029794821411</v>
+        <v>0.029891418344</v>
       </c>
       <c r="C64" s="64">
         <f>IF(AND(B64&gt;=0,B65&lt;0),A64+pH_step*B64/(B64-B65),0)</f>
@@ -14917,7 +15321,7 @@
       </c>
       <c r="B65" s="64">
         <f t="shared" si="1"/>
-        <v>0.028996945562</v>
+        <v>0.029118555933</v>
       </c>
       <c r="C65" s="64">
         <f>IF(AND(B65&gt;=0,B66&lt;0),A65+pH_step*B65/(B65-B66),0)</f>
@@ -14930,7 +15334,7 @@
       </c>
       <c r="B66" s="64">
         <f t="shared" si="1"/>
-        <v>0.028005502639</v>
+        <v>0.028158604254</v>
       </c>
       <c r="C66" s="64">
         <f>IF(AND(B66&gt;=0,B67&lt;0),A66+pH_step*B66/(B66-B67),0)</f>
@@ -14943,7 +15347,7 @@
       </c>
       <c r="B67" s="64">
         <f t="shared" si="1"/>
-        <v>0.026776012764</v>
+        <v>0.026968761394</v>
       </c>
       <c r="C67" s="64">
         <f>IF(AND(B67&gt;=0,B68&lt;0),A67+pH_step*B67/(B67-B68),0)</f>
@@ -14956,7 +15360,7 @@
       </c>
       <c r="B68" s="64">
         <f t="shared" si="1"/>
-        <v>0.025255400836</v>
+        <v>0.025498065093</v>
       </c>
       <c r="C68" s="64">
         <f>IF(AND(B68&gt;=0,B69&lt;0),A68+pH_step*B68/(B68-B69),0)</f>
@@ -14969,7 +15373,7 @@
       </c>
       <c r="B69" s="64">
         <f t="shared" si="1"/>
-        <v>0.02338090709</v>
+        <v>0.023686416142</v>
       </c>
       <c r="C69" s="64">
         <f>IF(AND(B69&gt;=0,B70&lt;0),A69+pH_step*B69/(B69-B70),0)</f>
@@ -14982,7 +15386,7 @@
       </c>
       <c r="B70" s="64">
         <f t="shared" si="1"/>
-        <v>0.021079010121</v>
+        <v>0.021463643599</v>
       </c>
       <c r="C70" s="64">
         <f>IF(AND(B70&gt;=0,B71&lt;0),A70+pH_step*B70/(B70-B71),0)</f>
@@ -14995,7 +15399,7 @@
       </c>
       <c r="B71" s="64">
         <f t="shared" si="1"/>
-        <v>0.01826430841</v>
+        <v>0.018748565553</v>
       </c>
       <c r="C71" s="64">
         <f>IF(AND(B71&gt;=0,B72&lt;0),A71+pH_step*B71/(B71-B72),0)</f>
@@ -15008,7 +15412,7 @@
       </c>
       <c r="B72" s="64">
         <f t="shared" si="1"/>
-        <v>0.014838178095</v>
+        <v>0.015447872883</v>
       </c>
       <c r="C72" s="64">
         <f>IF(AND(B72&gt;=0,B73&lt;0),A72+pH_step*B72/(B72-B73),0)</f>
@@ -15021,7 +15425,7 @@
       </c>
       <c r="B73" s="64">
         <f t="shared" si="1"/>
-        <v>0.010686819787</v>
+        <v>0.011454461141</v>
       </c>
       <c r="C73" s="64">
         <f>IF(AND(B73&gt;=0,B74&lt;0),A73+pH_step*B73/(B73-B74),0)</f>
@@ -15034,11 +15438,11 @@
       </c>
       <c r="B74" s="64">
         <f t="shared" si="1"/>
-        <v>0.005678038225</v>
+        <v>0.006644569952</v>
       </c>
       <c r="C74" s="64">
         <f>IF(AND(B74&gt;=0,B75&lt;0),A74+pH_step*B74/(B74-B75),0)</f>
-        <v>6.494284837612</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -15047,11 +15451,11 @@
       </c>
       <c r="B75" s="64">
         <f t="shared" si="1"/>
-        <v>-0.0003441795237407</v>
+        <v>0.0008728155195231</v>
       </c>
       <c r="C75" s="64">
         <f>IF(AND(B75&gt;=0,B76&lt;0),A75+pH_step*B75/(B75-B76),0)</f>
-        <v>0.0</v>
+        <v>6.512633395404</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -15060,7 +15464,7 @@
       </c>
       <c r="B76" s="64">
         <f t="shared" si="1"/>
-        <v>-0.00756840932</v>
+        <v>-0.006035980506</v>
       </c>
       <c r="C76" s="64">
         <f>IF(AND(B76&gt;=0,B77&lt;0),A76+pH_step*B76/(B76-B77),0)</f>
@@ -15073,7 +15477,7 @@
       </c>
       <c r="B77" s="64">
         <f t="shared" si="1"/>
-        <v>-0.016228970854</v>
+        <v>-0.014299245629</v>
       </c>
       <c r="C77" s="64">
         <f>IF(AND(B77&gt;=0,B78&lt;0),A77+pH_step*B77/(B77-B78),0)</f>
@@ -15086,7 +15490,7 @@
       </c>
       <c r="B78" s="64">
         <f t="shared" si="1"/>
-        <v>-0.02662440719</v>
+        <v>-0.024194216159</v>
       </c>
       <c r="C78" s="64">
         <f>IF(AND(B78&gt;=0,B79&lt;0),A78+pH_step*B78/(B78-B79),0)</f>
@@ -15099,7 +15503,7 @@
       </c>
       <c r="B79" s="64">
         <f t="shared" si="1"/>
-        <v>-0.039141735033</v>
+        <v>-0.036081020585</v>
       </c>
       <c r="C79" s="64">
         <f>IF(AND(B79&gt;=0,B80&lt;0),A79+pH_step*B79/(B79-B80),0)</f>
@@ -15112,7 +15516,7 @@
       </c>
       <c r="B80" s="64">
         <f t="shared" si="1"/>
-        <v>-0.054286645726</v>
+        <v>-0.050431397619</v>
       </c>
       <c r="C80" s="64">
         <f>IF(AND(B80&gt;=0,B81&lt;0),A80+pH_step*B80/(B80-B81),0)</f>
@@ -15125,7 +15529,7 @@
       </c>
       <c r="B81" s="64">
         <f t="shared" si="1"/>
-        <v>-0.072719923595</v>
+        <v>-0.0678632255</v>
       </c>
       <c r="C81" s="64">
         <f>IF(AND(B81&gt;=0,B82&lt;0),A81+pH_step*B81/(B81-B82),0)</f>
@@ -15138,7 +15542,7 @@
       </c>
       <c r="B82" s="64">
         <f t="shared" ref="B82:B113" si="3">pH_SID + pH_NT*(10^-A82)/((10^-A82)+KaN_c) + (10^-A82) - (pH_PT*Ka1p_c*(10^-A82)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A82) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A82)^3 + Ka1p_c*(10^-A82)^2 + Ka1p_c*Ka2p_c*(10^-A82) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A82) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A82)^2 - Kw_c/(10^-A82)</f>
-        <v>-0.095300976728</v>
+        <v>-0.089181639593</v>
       </c>
       <c r="C82" s="64">
         <f>IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
@@ -15151,7 +15555,7 @@
       </c>
       <c r="B83" s="64">
         <f t="shared" si="3"/>
-        <v>-0.123140508482</v>
+        <v>-0.115428610375</v>
       </c>
       <c r="C83" s="64">
         <f>IF(AND(B83&gt;=0,B84&lt;0),A83+pH_step*B83/(B83-B84),0)</f>
@@ -15164,7 +15568,7 @@
       </c>
       <c r="B84" s="64">
         <f t="shared" si="3"/>
-        <v>-0.157665823938</v>
+        <v>-0.147944267405</v>
       </c>
       <c r="C84" s="64">
         <f>IF(AND(B84&gt;=0,B85&lt;0),A84+pH_step*B84/(B84-B85),0)</f>
@@ -15177,7 +15581,7 @@
       </c>
       <c r="B85" s="64">
         <f t="shared" si="3"/>
-        <v>-0.200703923131</v>
+        <v>-0.188444839472</v>
       </c>
       <c r="C85" s="64">
         <f>IF(AND(B85&gt;=0,B86&lt;0),A85+pH_step*B85/(B85-B86),0)</f>
@@ -15190,7 +15594,7 @@
       </c>
       <c r="B86" s="64">
         <f t="shared" si="3"/>
-        <v>-0.2545894166</v>
+        <v>-0.239123861813</v>
       </c>
       <c r="C86" s="64">
         <f>IF(AND(B86&gt;=0,B87&lt;0),A86+pH_step*B86/(B86-B87),0)</f>
@@ -15203,7 +15607,7 @@
       </c>
       <c r="B87" s="64">
         <f t="shared" si="3"/>
-        <v>-0.322306667774</v>
+        <v>-0.302785522984</v>
       </c>
       <c r="C87" s="64">
         <f>IF(AND(B87&gt;=0,B88&lt;0),A87+pH_step*B87/(B87-B88),0)</f>
@@ -15216,7 +15620,7 @@
       </c>
       <c r="B88" s="64">
         <f t="shared" si="3"/>
-        <v>-0.407678885978</v>
+        <v>-0.383022129896</v>
       </c>
       <c r="C88" s="64">
         <f>IF(AND(B88&gt;=0,B89&lt;0),A88+pH_step*B88/(B88-B89),0)</f>
@@ -15229,7 +15633,7 @@
       </c>
       <c r="B89" s="64">
         <f t="shared" si="3"/>
-        <v>-0.515621824235</v>
+        <v>-0.484452287112</v>
       </c>
       <c r="C89" s="64">
         <f>IF(AND(B89&gt;=0,B90&lt;0),A89+pH_step*B89/(B89-B90),0)</f>
@@ -15242,7 +15646,7 @@
       </c>
       <c r="B90" s="64">
         <f t="shared" si="3"/>
-        <v>-0.65248719742</v>
+        <v>-0.613043384086</v>
       </c>
       <c r="C90" s="64">
         <f>IF(AND(B90&gt;=0,B91&lt;0),A90+pH_step*B90/(B90-B91),0)</f>
@@ -15255,7 +15659,7 @@
       </c>
       <c r="B91" s="64">
         <f t="shared" si="3"/>
-        <v>-0.826532271905</v>
+        <v>-0.776552624517</v>
       </c>
       <c r="C91" s="64">
         <f>IF(AND(B91&gt;=0,B92&lt;0),A91+pH_step*B91/(B91-B92),0)</f>
@@ -15268,7 +15672,7 @@
       </c>
       <c r="B92" s="64">
         <f t="shared" si="3"/>
-        <v>-1.048569336646</v>
+        <v>-0.985137039874</v>
       </c>
       <c r="C92" s="64">
         <f>IF(AND(B92&gt;=0,B93&lt;0),A92+pH_step*B92/(B92-B93),0)</f>
@@ -15281,7 +15685,7 @@
       </c>
       <c r="B93" s="64">
         <f t="shared" si="3"/>
-        <v>-1.332875144027</v>
+        <v>-1.252207705306</v>
       </c>
       <c r="C93" s="64">
         <f>IF(AND(B93&gt;=0,B94&lt;0),A93+pH_step*B93/(B93-B94),0)</f>
@@ -15294,7 +15698,7 @@
       </c>
       <c r="B94" s="64">
         <f t="shared" si="3"/>
-        <v>-1.698480927379</v>
+        <v>-1.595641435687</v>
       </c>
       <c r="C94" s="64">
         <f>IF(AND(B94&gt;=0,B95&lt;0),A94+pH_step*B94/(B94-B95),0)</f>
@@ -15307,7 +15711,7 @@
       </c>
       <c r="B95" s="64">
         <f t="shared" si="3"/>
-        <v>-2.171026165161</v>
+        <v>-2.03952200596</v>
       </c>
       <c r="C95" s="64">
         <f>IF(AND(B95&gt;=0,B96&lt;0),A95+pH_step*B95/(B95-B96),0)</f>
@@ -15320,7 +15724,7 @@
       </c>
       <c r="B96" s="64">
         <f t="shared" si="3"/>
-        <v>-2.785456321043</v>
+        <v>-2.616674108835</v>
       </c>
       <c r="C96" s="64">
         <f>IF(AND(B96&gt;=0,B97&lt;0),A96+pH_step*B96/(B96-B97),0)</f>
@@ -15333,7 +15737,7 @@
       </c>
       <c r="B97" s="64">
         <f t="shared" si="3"/>
-        <v>-3.589995975505</v>
+        <v>-3.372395273475</v>
       </c>
       <c r="C97" s="64">
         <f>IF(AND(B97&gt;=0,B98&lt;0),A97+pH_step*B97/(B97-B98),0)</f>
@@ -15346,7 +15750,7 @@
       </c>
       <c r="B98" s="64">
         <f t="shared" si="3"/>
-        <v>-4.652065051273</v>
+        <v>-4.370012913997</v>
       </c>
       <c r="C98" s="64">
         <f>IF(AND(B98&gt;=0,B99&lt;0),A98+pH_step*B98/(B98-B99),0)</f>
@@ -15359,7 +15763,7 @@
       </c>
       <c r="B99" s="64">
         <f t="shared" si="3"/>
-        <v>-6.067176130696</v>
+        <v>-5.699241495811</v>
       </c>
       <c r="C99" s="64">
         <f>IF(AND(B99&gt;=0,B100&lt;0),A99+pH_step*B99/(B99-B100),0)</f>
@@ -15372,7 +15776,7 @@
       </c>
       <c r="B100" s="64">
         <f t="shared" si="3"/>
-        <v>-7.972432454632</v>
+        <v>-7.488861095159</v>
       </c>
       <c r="C100" s="64">
         <f>0</f>
@@ -15414,7 +15818,7 @@
       </c>
       <c r="D103" s="149">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
-        <v>6.494284837612</v>
+        <v>6.512633395404</v>
       </c>
       <c r="E103" s="51" t="s">
         <v>1878</v>
@@ -15437,7 +15841,7 @@
       </c>
       <c r="D104" s="149">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
-        <v>0.870210730329</v>
+        <v>0.865363856191</v>
       </c>
       <c r="E104" s="51" t="s">
         <v>1879</v>
@@ -15526,7 +15930,7 @@
       </c>
       <c r="D109" s="64" t="str">
         <f>IF(C_eff_Cl2&lt;Cl_onset,"negligible free chlorine ("&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ &lt; onset); does NOT account for the Exp-2 death - see metal_flag",IF(C_eff_Cl2&lt;Cl_kill,"sub-lethal "&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ (band "&amp;TEXT(C_eff_lo_Cl2,"0.00")&amp;"-"&amp;TEXT(C_eff_hi_Cl2,"0.00")&amp;"); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag","SEVERE free chlorine: "&amp;TEXT(C_eff_Cl2,"0.0")&amp;" mg/L as Cl₂ - biofilm/electrode damage (Baek 2021)"))</f>
-        <v>sub-lethal 0.50 mg/L as Cl₂ (band 0.00-0.71); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
+        <v>sub-lethal 0.34 mg/L as Cl₂ (band 0.01-0.65); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
       </c>
       <c r="E109" s="51" t="s">
         <v>1127</v>
@@ -15629,7 +16033,7 @@
       </c>
       <c r="D125" s="149">
         <f>pH_Cl*pH_fHOCl*M_HOCl</f>
-        <v>8.22693366608</v>
+        <v>8.181111532849</v>
       </c>
       <c r="E125" s="51" t="s">
         <v>1460</v>
@@ -15721,12 +16125,12 @@
         <v>1076</v>
       </c>
       <c r="D132" s="149">
-        <f>Fcc*km_Cl*(pH_Cl/1000)*A_anode</f>
-        <v>0.0001417839262056</v>
-      </c>
-      <c r="E132" s="51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">i_lim = n·F·k_m·[Cl⁻]·A, n = 1 per ARRIVING chloride; [Cl⁻] in mol/cm³ = pH_Cl/1000. Caps chlorine at the chloride flux; it binds at trace Cl⁻ such as UdG, so production scales with chloride.</t>
+        <f>n_e_Cl*Fcc*km_Cl*(pH_Cl/1000)*A_anode</f>
+        <v>0.0002835678524112</v>
+      </c>
+      <c r="E132" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">i_lim = n_e_Cl·F·k_m·[Cl⁻]·A with n_e_Cl = 2 per NET chloride consumed: Cl₂ hydrolysis (k ≈ 11–22 s⁻¹) is faster than diffusion across the layer (δ²/D ≈ 0.8 s), so the chloride it regenerates is re-oxidised at the surface (the direct route Cl⁻ + H₂O → HOCl + H⁺ + 2e⁻ gives the same). [Cl⁻] in mol/cm³ = pH_Cl/1000. At the anode potential (D256, above the HOCl/Cl⁻ couple) this transport limit is the central estimate, not a cap; the factor 2 rests on where hydrolysis happens.</t>
         </is>
       </c>
     </row>
@@ -15742,7 +16146,7 @@
       </c>
       <c r="D133" s="149">
         <f>MIN(I_Cl_FE,I_Cl_mt)</f>
-        <v>0.0001417839262056</v>
+        <v>0.0002835678524112</v>
       </c>
       <c r="E133" s="51" t="s">
         <v>1082</v>
@@ -15760,10 +16164,12 @@
       </c>
       <c r="D134" s="149">
         <f>I_Cl/(n_e_Cl*Fcc*VLc)</f>
-        <v>4.898289480563e-08</v>
-      </c>
-      <c r="E134" s="51" t="s">
-        <v>1463</v>
+        <v>9.796578961125e-08</v>
+      </c>
+      <c r="E134" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P_HOCl = I_Cl/(n_e_Cl·F·V), n_e_Cl = 2 on every route (D148); at the transport limit this is k_m·[Cl⁻]·A/V, one HOCl per arriving chloride.</t>
+        </is>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
@@ -15831,7 +16237,7 @@
       </c>
       <c r="D138" s="149">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
-        <v>1.241103645704e-05</v>
+        <v>1.294565152087e-05</v>
       </c>
       <c r="E138" s="51" t="s">
         <v>1099</v>
@@ -15849,7 +16255,7 @@
       </c>
       <c r="D139" s="149">
         <f>P_HOCl/(k1_NH2Cl*NH3_free)</f>
-        <v>9.396954107506e-10</v>
+        <v>1.801777837529e-09</v>
       </c>
       <c r="E139" s="51" t="s">
         <v>1102</v>
@@ -15867,7 +16273,7 @@
       </c>
       <c r="D140" s="149">
         <f>HOCl_ss*M_HOCl</f>
-        <v>4.929642124798e-05</v>
+        <v>9.452126535676e-05</v>
       </c>
       <c r="E140" s="51" t="s">
         <v>1105</v>
@@ -15918,11 +16324,13 @@
         <v>1088</v>
       </c>
       <c r="D143" s="149">
-        <f>MIN(P_HOCl*tau_NH2Cl*3600*M_HOCl,cl_per_N*NH3_N,Cl_pool_mgL)</f>
-        <v>9.250713581411</v>
-      </c>
-      <c r="E143" s="51" t="s">
-        <v>1115</v>
+        <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl*3600)/(1+k_Cl_turn*tau_NH2Cl*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
+        <v>6.256815485116</v>
+      </c>
+      <c r="E143" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steady combined chlorine, HOCl basis. Chloride is recycled: the pool bounds free + combined chlorine at any instant, and the steady share held as monochloramine is kτ/(1+kτ) with k = k_Cl_turn (D271) and τ its residence. Reduces to production×τ when kτ ≪ 1 and to the pool when kτ ≫ 1. Second argument: breakpoint ammonium capacity (5.06 mg Cl₂/mg N) converted to the HOCl basis; it does not bind in UdG.</t>
+        </is>
       </c>
     </row>
     <row r="144" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -15954,10 +16362,12 @@
       </c>
       <c r="D145" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_mgL/R_chloramine</f>
-        <v>0.370521507469</v>
-      </c>
-      <c r="E145" s="51" t="s">
-        <v>1464</v>
+        <v>0.251217832058</v>
+      </c>
+      <c r="E145" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OPERATIVE bleaching value (HOCl basis): local-weighted free HOCl + combined chlorine ÷ potency. Combined chlorine is the recycling steady state (D143), so it rises with current and residence until it approaches the chloride pool (D149); Summary reports it as Cl₂ (D226).</t>
+        </is>
       </c>
     </row>
     <row r="146" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -16008,8 +16418,10 @@
         <f>2</f>
         <v>2.0</v>
       </c>
-      <c r="E148" s="51" t="s">
-        <v>1480</v>
+      <c r="E148" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrons per HOCl formed and per net chloride consumed — 2 on every route. 2Cl⁻ → Cl₂ + 2e⁻ then Cl₂ + H₂O → HOCl + H⁺ + Cl⁻ is 2 e⁻ per HOCl and 1 net chloride, because the regenerated chloride is re-oxidised inside the diffusion layer; the direct route Cl⁻ + H₂O → HOCl + H⁺ + 2e⁻ is also 2. Used both in the transport-limited current (D132) and in the production rate (D134).</t>
+        </is>
       </c>
     </row>
     <row r="149" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -16026,8 +16438,10 @@
         <f>pH_Cl*M_HOCl</f>
         <v>9.453955667688</v>
       </c>
-      <c r="E149" s="51" t="s">
-        <v>1219</v>
+      <c r="E149" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total chloride pool as HOCl-equivalent; free + combined chlorine cannot exceed it at any instant, and the steady combined share is kτ/(1+kτ) of it (D143). UdG chloride is CaCl₂-derived (a closed batch also depletes it).</t>
+        </is>
       </c>
     </row>
     <row r="150" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -16109,11 +16523,13 @@
         <v>1238</v>
       </c>
       <c r="D154" s="149">
-        <f>MIN(P_HOCl*tau_NH2Cl_lo*3600*M_HOCl,cl_per_N*NH3_N,Cl_pool_mgL)</f>
-        <v>0.15417855969</v>
-      </c>
-      <c r="E154" s="51" t="s">
-        <v>1239</v>
+        <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl_lo*3600)/(1+k_Cl_turn*tau_NH2Cl_lo*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
+        <v>0.298617202708</v>
+      </c>
+      <c r="E154" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combined chlorine at the low-τ bound, recycling steady state (as D143)</t>
+        </is>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
@@ -16127,11 +16543,13 @@
         <v>1242</v>
       </c>
       <c r="D155" s="149">
-        <f>MIN(P_HOCl*tau_NH2Cl_hi*3600*M_HOCl,cl_per_N*NH3_N,Cl_pool_mgL)</f>
-        <v>9.453955667688</v>
-      </c>
-      <c r="E155" s="51" t="s">
-        <v>1243</v>
+        <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl_hi*3600)/(1+k_Cl_turn*tau_NH2Cl_hi*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
+        <v>8.577373468854</v>
+      </c>
+      <c r="E155" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combined chlorine at the high-τ bound, recycling steady state (as D143)</t>
+        </is>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
@@ -16146,7 +16564,7 @@
       </c>
       <c r="D156" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_lo/R_chloramine_hi</f>
-        <v>0.002695515065</v>
+        <v>0.005211172692</v>
       </c>
       <c r="E156" s="51" t="s">
         <v>1247</v>
@@ -16164,7 +16582,7 @@
       </c>
       <c r="D157" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_hi/R_chloramine_lo</f>
-        <v>0.525712723528</v>
+        <v>0.477465960923</v>
       </c>
       <c r="E157" s="51" t="s">
         <v>1251</v>
@@ -16930,7 +17348,7 @@
       </c>
       <c r="D206" s="141">
         <f>E0_OER-nernst_slope*pH_meas</f>
-        <v>0.83831463654</v>
+        <v>0.837229147794</v>
       </c>
       <c r="E206" s="99" t="s">
         <v>1586</v>
@@ -16948,7 +17366,7 @@
       </c>
       <c r="D207" s="141">
         <f>E0_HER-nernst_slope*pH_meas</f>
-        <v>-0.39068536346</v>
+        <v>-0.391770852206</v>
       </c>
       <c r="E207" s="99" t="s">
         <v>1589</v>
@@ -16988,7 +17406,7 @@
       </c>
       <c r="D209" s="141">
         <f>E_HOCl_Cl-E_anode_op</f>
-        <v>-0.422483519032</v>
+        <v>-0.413578182478</v>
       </c>
       <c r="E209" s="67" t="inlineStr">
         <is>
@@ -17008,7 +17426,7 @@
       </c>
       <c r="D210" s="141">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
-        <v>0.30431463654</v>
+        <v>0.303229147794</v>
       </c>
       <c r="E210" s="67" t="s">
         <v>1599</v>
@@ -17028,7 +17446,7 @@
       </c>
       <c r="D211" s="141">
         <f>E_anode_op-E0_Cu</f>
-        <v>1.240557060036</v>
+        <v>1.239471571289</v>
       </c>
       <c r="E211" s="67" t="s">
         <v>1602</v>
@@ -17057,8 +17475,10 @@
       </c>
     </row>
     <row r="215" spans="1:5" ht="60" x14ac:dyDescent="0.2">
-      <c r="A215" t="s">
-        <v>1607</v>
+      <c r="A215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diffusion layer thickness for O₂ (derived, display only)</t>
+        </is>
       </c>
       <c r="B215" s="18" t="s">
         <v>1608</v>
@@ -17066,11 +17486,14 @@
       <c r="C215" s="19" t="s">
         <v>580</v>
       </c>
-      <c r="D215" s="131">
-        <v>40</v>
-      </c>
-      <c r="E215" s="75" t="s">
-        <v>1609</v>
+      <c r="D215" s="141">
+        <f>D_O2_c/(km_O2_c/100)*1000000</f>
+        <v>49.941807960105</v>
+      </c>
+      <c r="E215" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">δ = D_O₂/k_m(O₂), display only — the buffer limit uses species-specific k_m (D275–D276); δ_i ∝ D_i^0.356 under the same correlation, so a single fixed δ is not used.</t>
+        </is>
       </c>
     </row>
     <row r="216" spans="1:5" ht="60" x14ac:dyDescent="0.2">
@@ -17084,12 +17507,12 @@
         <v>1282</v>
       </c>
       <c r="D216" s="141">
-        <f>Fcc*(D_HPO4*HPO4_op+D_HCO3*HCO3_op)*1000/(delta_diff/1000000)/10</f>
-        <v>8.049160263403</v>
+        <f>Fcc*((km_HPO4/100)*HPO4_op+(km_HCO3/100)*HCO3_op)*1000/10</f>
+        <v>8.126539606735</v>
       </c>
       <c r="E216" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">j_lim = F·Σ(D·C)/δ over the proton acceptors reaching the anode: hydrogen phosphate and bicarbonate (D251–D253). At the CO₂-dosed operating point bicarbonate is the larger term; at air equilibrium it falls to ~0.4 mM and the phosphate term alone applies, so re-read this verdict whenever the schedule changes.</t>
+          <t xml:space="preserve">j_lim = F·Σ k_m,i·C_i over the proton acceptors reaching the anode: hydrogen phosphate and bicarbonate (D252–D253), each with its own k_m scaled from km_O2 (D275–D276), so the verdict hangs on the one ferricyanide-measurable coefficient. At the CO₂-dosed operating point bicarbonate is the larger term; at air equilibrium it falls to ~0.4 mM and the phosphate term alone applies, so re-read this verdict whenever the schedule changes.</t>
         </is>
       </c>
     </row>
@@ -17123,7 +17546,7 @@
       </c>
       <c r="D218" s="141">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>0.35110441286</v>
+        <v>0.347761264334</v>
       </c>
       <c r="E218" s="67" t="s">
         <v>1618</v>
@@ -17159,7 +17582,7 @@
       </c>
       <c r="D220" s="141">
         <f>pH_op-LOG10(gamma_1)</f>
-        <v>6.603949596052</v>
+        <v>6.622298153844</v>
       </c>
       <c r="E220" s="67" t="s">
         <v>1624</v>
@@ -17252,7 +17675,7 @@
       </c>
       <c r="D226" s="141">
         <f>C_eff*M_Cl2/M_HOCl</f>
-        <v>0.500804384457</v>
+        <v>0.33955111704</v>
       </c>
       <c r="E226" s="67" t="s">
         <v>1899</v>
@@ -17566,7 +17989,7 @@
       </c>
       <c r="D252" s="141">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
-        <v>0.01976870305</v>
+        <v>0.01936991072</v>
       </c>
       <c r="E252" s="67" t="inlineStr">
         <is>
@@ -17592,7 +18015,7 @@
       </c>
       <c r="D253" s="141">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
-        <v>0.013100861499</v>
+        <v>0.013462331212</v>
       </c>
       <c r="E253" s="67" t="inlineStr">
         <is>
@@ -17670,7 +18093,7 @@
       </c>
       <c r="D256" s="141">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
-        <v>1.582457060036</v>
+        <v>1.581371571289</v>
       </c>
       <c r="E256" s="67" t="inlineStr">
         <is>
@@ -17721,7 +18144,7 @@
       </c>
       <c r="D258" s="141">
         <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,1E-12))-pH_meas-LOG10(MAX(pH_Cl,1E-12)))</f>
-        <v>1.159973541004</v>
+        <v>1.167793388811</v>
       </c>
       <c r="E258" s="67" t="inlineStr">
         <is>
@@ -17747,7 +18170,7 @@
       </c>
       <c r="D259" s="141">
         <f>C_eff_lo*M_Cl2/M_HOCl</f>
-        <v>0.003643312833</v>
+        <v>0.007043526704</v>
       </c>
       <c r="E259" s="67" t="inlineStr">
         <is>
@@ -17773,11 +18196,174 @@
       </c>
       <c r="D260" s="141">
         <f>C_eff_hi*M_Cl2/M_HOCl</f>
-        <v>0.710563979689</v>
+        <v>0.645352676806</v>
       </c>
       <c r="E260" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">C_eff_hi on the as-Cl₂ basis the thresholds use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CHLORIDE RECYCLING AND SPECIES-SPECIFIC ELECTRODE MASS TRANSFER</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-order anodic chloride turnover</t>
+        </is>
+      </c>
+      <c r="B271" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_Cl_turn</t>
+        </is>
+      </c>
+      <c r="C271" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/s</t>
+        </is>
+      </c>
+      <c r="D271" s="141">
+        <f>IF(pH_Cl&gt;0,P_HOCl/pH_Cl,0)</f>
+        <v>0.0005436121665528</v>
+      </c>
+      <c r="E271" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chlorine production per unit bulk chloride, = km_Cl·A_anode/V at the chloride transport limit (D132–D134). Chloride cycles Cl⁻ → HOCl → NH₂Cl → Cl⁻ (chloramine decay and cathodic reduction both return chloride), so the pool is shared, not consumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) electrode mass-transfer coefficient — O₂</t>
+        </is>
+      </c>
+      <c r="B272" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_O2_c</t>
+        </is>
+      </c>
+      <c r="C272" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm/s</t>
+        </is>
+      </c>
+      <c r="D272" s="141">
+        <f>Electrochemistry!$D$83</f>
+        <v>0.004</v>
+      </c>
+      <c r="E272" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Electrochemistry (km_O2; Eisenberg–Tobias–Wilke, unmeasured swirl)</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) diffusivity exponent for k_m scaling</t>
+        </is>
+      </c>
+      <c r="B273" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_exp_c</t>
+        </is>
+      </c>
+      <c r="C273" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D273" s="141">
+        <f>Electrochemistry!$D$84</f>
+        <v>0.644</v>
+      </c>
+      <c r="E273" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Electrochemistry (km_exp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) O₂ diffusivity at reactor T</t>
+        </is>
+      </c>
+      <c r="B274" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D_O2_c</t>
+        </is>
+      </c>
+      <c r="C274" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m²/s</t>
+        </is>
+      </c>
+      <c r="D274" s="141">
+        <f>Electrochemistry!$D$81</f>
+        <v>1.997672318404e-09</v>
+      </c>
+      <c r="E274" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Electrochemistry (ec_D_O2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode mass-transfer coefficient — HPO₄²⁻</t>
+        </is>
+      </c>
+      <c r="B275" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_HPO4</t>
+        </is>
+      </c>
+      <c r="C275" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm/s</t>
+        </is>
+      </c>
+      <c r="D275" s="141">
+        <f>km_O2_c*(D_HPO4/D_O2_c)^km_exp_c</f>
+        <v>0.002144855688</v>
+      </c>
+      <c r="E275" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_m,i = k_m(O₂)·(D_i/D_O₂)^km_exp, the same Eisenberg scaling as km_Cl (D129).</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode mass-transfer coefficient — HCO₃⁻</t>
+        </is>
+      </c>
+      <c r="B276" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_HCO3</t>
+        </is>
+      </c>
+      <c r="C276" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm/s</t>
+        </is>
+      </c>
+      <c r="D276" s="141">
+        <f>km_O2_c*(D_HCO3/D_O2_c)^km_exp_c</f>
+        <v>0.002857570744</v>
+      </c>
+      <c r="E276" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D275, for bicarbonate.</t>
         </is>
       </c>
     </row>
@@ -17862,7 +18448,7 @@
       </c>
       <c r="D4" s="150">
         <f>Electrochemistry!$D$21</f>
-        <v>0.000103759833633</v>
+        <v>0.0001017274698715</v>
       </c>
       <c r="E4" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D21","→ Electrochemistry")</f>
@@ -17882,7 +18468,7 @@
       </c>
       <c r="D5" s="150">
         <f>Electrochemistry!$D$29</f>
-        <v>4.936187056172e-05</v>
+        <v>4.803933240197e-05</v>
       </c>
       <c r="E5" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -18022,11 +18608,13 @@
         <v>354</v>
       </c>
       <c r="D13" s="48">
-        <f>rH2_gen</f>
-        <v>0.000103759833633</v>
-      </c>
-      <c r="E13" s="37" t="s">
-        <v>418</v>
+        <f>MAX(0,rH2_gen-H2_HOR_b)</f>
+        <v>0.0001017274698715</v>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Evolved H₂ minus any crossed-over H₂ the Pt anode oxidises (D96; 0 until measured), assumed fully consumed — steady growth only; ~0 during lag (see §13).</t>
+        </is>
       </c>
       <c r="F13" s="20"/>
     </row>
@@ -18042,7 +18630,7 @@
       </c>
       <c r="D14" s="48">
         <f>H2_cons*bio_O2/bio_H2</f>
-        <v>3.4586611211e-05</v>
+        <v>3.390915662382e-05</v>
       </c>
       <c r="E14" s="107" t="s">
         <v>421</v>
@@ -18061,7 +18649,7 @@
       </c>
       <c r="D15" s="48">
         <f>H2_cons*bio_CO2/bio_H2</f>
-        <v>1.72933056055e-05</v>
+        <v>1.695457831191e-05</v>
       </c>
       <c r="E15" s="37" t="s">
         <v>424</v>
@@ -18080,7 +18668,7 @@
       </c>
       <c r="D16" s="48">
         <f>MAX(0,O2_net_gen-O2_cons)</f>
-        <v>1.477525935072e-05</v>
+        <v>1.413017577815e-05</v>
       </c>
       <c r="E16" s="115" t="s">
         <v>1926</v>
@@ -18563,7 +19151,7 @@
       </c>
       <c r="D42" s="48">
         <f>C_H2_sat*(V_charge/1000000)/rH2_gen*60</f>
-        <v>6.855268316214</v>
+        <v>6.992226395671</v>
       </c>
       <c r="E42" s="99" t="s">
         <v>504</v>
@@ -18582,7 +19170,7 @@
       </c>
       <c r="D43" s="48">
         <f>rH2_gen/(V_charge/1000000)/C_H2_sat</f>
-        <v>8.75239264641</v>
+        <v>8.580957853016</v>
       </c>
       <c r="E43" s="69" t="s">
         <v>508</v>
@@ -18603,7 +19191,7 @@
       </c>
       <c r="D44" s="48" t="str">
         <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;", O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag basis)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 19%, O₂ 9% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 20%, O₂ 9% – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="70" t="inlineStr">
         <is>
@@ -19052,7 +19640,7 @@
       </c>
       <c r="D76" s="150">
         <f>'Mass Transfer'!$D$100</f>
-        <v>0.0003892277799716</v>
+        <v>0.0003583371353617</v>
       </c>
       <c r="E76" s="135" t="inlineStr">
         <is>
@@ -19231,7 +19819,7 @@
       </c>
       <c r="D83" s="48">
         <f>rH2_gen+O2_net_gen</f>
-        <v>0.0001531217041947</v>
+        <v>0.0001497668022734</v>
       </c>
       <c r="E83" s="69" t="inlineStr">
         <is>
@@ -19257,7 +19845,7 @@
       </c>
       <c r="D84" s="48">
         <f>rH2_gen/(n_flamm_src+CO2_supply_b)</f>
-        <v>0.191315446335</v>
+        <v>0.200209961657</v>
       </c>
       <c r="E84" s="69" t="inlineStr">
         <is>
@@ -19283,7 +19871,7 @@
       </c>
       <c r="D85" s="48">
         <f>O2_net_gen/(n_flamm_src+CO2_supply_b)</f>
-        <v>0.0910148751</v>
+        <v>0.094546270642</v>
       </c>
       <c r="E85" s="69" t="inlineStr">
         <is>
@@ -19309,7 +19897,7 @@
       </c>
       <c r="D86" s="48">
         <f>MAX(0,MIN(rH2_gen/H2_LFL-n_flamm_src,O2_net_gen/(O2_LOC_H2*LOC_margin)-n_flamm_src))/CO2_rate_full_b</f>
-        <v>0.002916316798</v>
+        <v>0.002836654967</v>
       </c>
       <c r="E86" s="69" t="inlineStr">
         <is>
@@ -19335,7 +19923,7 @@
       </c>
       <c r="D87" s="48">
         <f>IF(duty_H2safe&gt;0,spg_dur_b/(60*duty_H2safe),NA())</f>
-        <v>4.483469527972</v>
+        <v>4.609378881561</v>
       </c>
       <c r="E87" s="69" t="inlineStr">
         <is>
@@ -19361,11 +19949,96 @@
       </c>
       <c r="D88" s="48">
         <f>MAX(0,rH2_gen/H2_LFL-n_flamm_src)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
-        <v>0.995282852087</v>
+        <v>0.975933085966</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuous inert headspace sweep that dilutes H₂ below the LFL with no CO₂ at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANODIC H₂ LOSS AND CARBON AT THE CYCLE TROUGH</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) H₂ oxidised at the anode</t>
+        </is>
+      </c>
+      <c r="B96" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_HOR_b</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D96" s="48">
+        <f>Electrochemistry!$D$149</f>
+        <v>0.0</v>
+      </c>
+      <c r="E96" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Electrochemistry (r_H2_HOR; 0 while f_HOR_anode is a data gap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) dissolved CO₂ at the start of a pulse (cycle trough)</t>
+        </is>
+      </c>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C_cycle_start_b</t>
+        </is>
+      </c>
+      <c r="C97" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D97" s="48">
+        <f>'Mass Transfer'!$D$198</f>
+        <v>5.891603808766</v>
+      </c>
+      <c r="E97" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Mass Transfer (C_cycle_start, mass-conserving limit cycle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carbon margin at the cycle trough (dissolved CO₂ : Km)</t>
+        </is>
+      </c>
+      <c r="B98" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_margin_trough</t>
+        </is>
+      </c>
+      <c r="C98" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">×</t>
+        </is>
+      </c>
+      <c r="D98" s="48">
+        <f>C_cycle_start_b*1000/Km_CO2</f>
+        <v>117.832076175326</v>
+      </c>
+      <c r="E98" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lowest dissolved CO₂ of the dosing cycle (mol/m³ = mM, ×1000 → µM) against RuBisCO Km. A sub-second pulse never approaches the full-sparge saturation D33 uses, so this, not D35, is the carbon-availability test; schedule-dependent.</t>
         </is>
       </c>
     </row>
@@ -19571,7 +20244,7 @@
       </c>
       <c r="D10" s="142">
         <f>Biology!$D$15</f>
-        <v>1.72933056055e-05</v>
+        <v>1.695457831191e-05</v>
       </c>
       <c r="E10" s="135" t="str">
         <f>HYPERLINK("#Biology!D15","→ Biology")</f>
@@ -19591,7 +20264,7 @@
       </c>
       <c r="D11" s="142">
         <f>Biology!$D$16</f>
-        <v>1.477525935072e-05</v>
+        <v>1.413017577815e-05</v>
       </c>
       <c r="E11" s="135" t="str">
         <f>HYPERLINK("#Biology!D16","→ Biology")</f>
@@ -19631,7 +20304,7 @@
       </c>
       <c r="D13" s="150">
         <f>Electrochemistry!$D$29</f>
-        <v>4.936187056172e-05</v>
+        <v>4.803933240197e-05</v>
       </c>
       <c r="E13" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -20376,7 +21049,7 @@
       </c>
       <c r="D53" s="64">
         <f>kLa_sparge*duty</f>
-        <v>1.22783627739e-05</v>
+        <v>1.1303903703e-05</v>
       </c>
       <c r="E53" s="117" t="s">
         <v>643</v>
@@ -20414,7 +21087,7 @@
       </c>
       <c r="D55" s="48">
         <f>strip_sparge*duty</f>
-        <v>2.418540330079e-07</v>
+        <v>2.226595475021e-07</v>
       </c>
       <c r="E55" s="75" t="s">
         <v>649</v>
@@ -20433,7 +21106,7 @@
       </c>
       <c r="D56" s="45">
         <f>IF(O2_excess&gt;0,strip_avg/O2_excess,NA())</f>
-        <v>0.016368851962</v>
+        <v>0.015757733732</v>
       </c>
       <c r="E56" s="75" t="s">
         <v>652</v>
@@ -20452,7 +21125,7 @@
       </c>
       <c r="D57" s="48">
         <f>IF(O2_excess&gt;0,O2_excess/3600/((V_charge/1000000)*O2_ceil_C),NA())</f>
-        <v>0.0007501053099273</v>
+        <v>0.0007173559278932</v>
       </c>
       <c r="E57" s="75" t="s">
         <v>655</v>
@@ -20602,7 +21275,7 @@
       </c>
       <c r="D65" s="48">
         <f>O2_ceil_C*(V_charge/1000000)/O2_excess*60</f>
-        <v>22.21910236615</v>
+        <v>23.233468935867</v>
       </c>
       <c r="E65" s="99" t="inlineStr">
         <is>
@@ -20623,7 +21296,7 @@
       </c>
       <c r="D66" s="48">
         <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,cleared_min)</f>
-        <v>22.588856006099</v>
+        <v>23.605437128776</v>
       </c>
       <c r="E66" s="99" t="s">
         <v>680</v>
@@ -20775,7 +21448,7 @@
       </c>
       <c r="D74" s="48">
         <f>IF(O2_excess&gt;0,surf_strip/O2_excess,NA())</f>
-        <v>9.59879041231</v>
+        <v>10.037003079208</v>
       </c>
       <c r="E74" s="69" t="s">
         <v>702</v>
@@ -20794,7 +21467,7 @@
       </c>
       <c r="D75" s="48">
         <f>IF(CO2_supply&gt;0,O2_excess/(O2_excess+CO2_supply),NA())</f>
-        <v>0.036572149</v>
+        <v>0.03793668694</v>
       </c>
       <c r="E75" s="99" t="s">
         <v>705</v>
@@ -20813,7 +21486,7 @@
       </c>
       <c r="D76" s="48">
         <f>H_O2_T*y_O2_vent*P_atm*1000</f>
-        <v>44.468075969604</v>
+        <v>46.12721765053</v>
       </c>
       <c r="E76" s="69" t="inlineStr">
         <is>
@@ -20834,7 +21507,7 @@
       </c>
       <c r="D77" s="48">
         <f>headspace_V/(Q_CO2*duty)</f>
-        <v>16.46036421628</v>
+        <v>17.879338726534</v>
       </c>
       <c r="E77" s="99" t="s">
         <v>710</v>
@@ -20853,7 +21526,7 @@
       </c>
       <c r="D78" s="48">
         <f>IF(O2_excess&gt;0,(strip_avg+surf_strip)/O2_excess,NA())</f>
-        <v>9.615159264271</v>
+        <v>10.052760812941</v>
       </c>
       <c r="E78" s="118" t="s">
         <v>713</v>
@@ -20872,7 +21545,7 @@
       </c>
       <c r="D79" s="48">
         <f>O2_ceil_C*(V_charge/1000000)/O2_net_gen*60</f>
-        <v>6.650740668134</v>
+        <v>6.833837682277</v>
       </c>
       <c r="E79" s="99" t="s">
         <v>716</v>
@@ -21003,7 +21676,7 @@
       </c>
       <c r="D86" s="48">
         <f>carbon_margin_min*CO2_cons/(nCO2_rate*3600)</f>
-        <v>7.058520235019e-05</v>
+        <v>6.920263645416e-05</v>
       </c>
       <c r="E86" s="99" t="s">
         <v>733</v>
@@ -21022,7 +21695,7 @@
       </c>
       <c r="D87" s="48">
         <f>O2_src_guard/(target_DO_frac*(O2_ceil_Pa/P_atm))/(nCO2_rate*3600)</f>
-        <v>0.001485253206</v>
+        <v>0.001445459252</v>
       </c>
       <c r="E87" s="99" t="s">
         <v>1063</v>
@@ -21041,7 +21714,7 @@
       </c>
       <c r="D88" s="48">
         <f>MAX(duty_carbon,duty_O2vent)</f>
-        <v>0.001485253206</v>
+        <v>0.001445459252</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
@@ -21062,7 +21735,7 @@
       </c>
       <c r="D89" s="48">
         <f>target_DO_frac*O2_ceil_C*(V_charge/1000000)/O2_src_guard*60</f>
-        <v>1.503645716274</v>
+        <v>1.54504156295</v>
       </c>
       <c r="E89" s="99" t="inlineStr">
         <is>
@@ -21102,7 +21775,7 @@
       </c>
       <c r="D91" s="48">
         <f>IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max))</f>
-        <v>16.46036421628</v>
+        <v>17.879338726534</v>
       </c>
       <c r="E91" s="159" t="inlineStr">
         <is>
@@ -21123,7 +21796,7 @@
       </c>
       <c r="D92" s="48">
         <f>spg_int_opt*60</f>
-        <v>987.621852976796</v>
+        <v>1072.760323592056</v>
       </c>
       <c r="E92" s="159" t="s">
         <v>747</v>
@@ -21144,7 +21817,7 @@
       </c>
       <c r="D93" s="48">
         <f>spg_dur_opt/(spg_int_opt*60)</f>
-        <v>0.0007943455761538</v>
+        <v>0.000731303192868</v>
       </c>
       <c r="E93" s="99" t="s">
         <v>750</v>
@@ -21277,7 +21950,7 @@
       </c>
       <c r="D100" s="28">
         <f>CO2_pulse*pulses_h</f>
-        <v>0.0003892277799716</v>
+        <v>0.0003583371353617</v>
       </c>
       <c r="E100" s="160" t="s">
         <v>765</v>
@@ -21370,7 +22043,7 @@
       </c>
       <c r="D105" s="28">
         <f>spg_dur/(spg_int*60)</f>
-        <v>0.0007943455761538</v>
+        <v>0.000731303192868</v>
       </c>
       <c r="E105" s="160" t="s">
         <v>765</v>
@@ -21484,7 +22157,7 @@
       </c>
       <c r="D112" s="28">
         <f>spg_dur_opt/(60*duty_carbon)</f>
-        <v>185.240207036777</v>
+        <v>188.941031253092</v>
       </c>
       <c r="E112" s="20"/>
       <c r="F112" s="20"/>
@@ -21499,7 +22172,7 @@
       <c r="C113" s="20"/>
       <c r="D113" s="28" t="str">
         <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) DO would be "&amp;TEXT(DO_at_carbon*M_O2,"0.0")&amp;" mg/L against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")</f>
-        <v>Do NOT relax: at the carbon-limited interval (185 min) DO would be 12.9 mg/L against a 2.6 mg/L target</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 12.6 mg/L against a 2.6 mg/L target</v>
       </c>
       <c r="E113" s="82" t="inlineStr">
         <is>
@@ -21651,7 +22324,7 @@
       </c>
       <c r="D122" s="28">
         <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,spg_int_opt))</f>
-        <v>16.46036421628</v>
+        <v>17.879338726534</v>
       </c>
       <c r="E122" s="20"/>
       <c r="F122" s="20"/>
@@ -21685,7 +22358,7 @@
       </c>
       <c r="D124" s="28">
         <f>60/spg_int</f>
-        <v>3.645119829163</v>
+        <v>3.355828809874</v>
       </c>
       <c r="E124" s="20"/>
       <c r="F124" s="20"/>
@@ -21702,7 +22375,7 @@
       </c>
       <c r="D125" s="28">
         <f>pulses_h*24</f>
-        <v>87.482875899902</v>
+        <v>80.539891436977</v>
       </c>
       <c r="E125" s="20"/>
       <c r="F125" s="20"/>
@@ -21719,7 +22392,7 @@
       </c>
       <c r="D126" s="28">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v>22.507425060931</v>
+        <v>21.135125201548</v>
       </c>
       <c r="E126" s="20"/>
       <c r="F126" s="20"/>
@@ -21736,7 +22409,7 @@
       </c>
       <c r="D127" s="28">
         <f>O2_excess/60*spg_int</f>
-        <v>4.05343583838e-06</v>
+        <v>4.21063665005e-06</v>
       </c>
       <c r="E127" s="20"/>
       <c r="F127" s="20"/>
@@ -21770,7 +22443,7 @@
       </c>
       <c r="D129" s="28">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v>0.016368851962</v>
+        <v>0.015757733732</v>
       </c>
       <c r="E129" s="20"/>
       <c r="F129" s="20"/>
@@ -21804,7 +22477,7 @@
       </c>
       <c r="D131" s="28">
         <f>kLa_surf_req/a_surf</f>
-        <v>0.0001158581442306</v>
+        <v>0.0001107998109846</v>
       </c>
       <c r="E131" s="147" t="s">
         <v>1825</v>
@@ -21823,7 +22496,7 @@
       </c>
       <c r="D132" s="28">
         <f>O2_net_gen</f>
-        <v>4.936187056172e-05</v>
+        <v>4.803933240197e-05</v>
       </c>
       <c r="E132" s="69" t="s">
         <v>992</v>
@@ -21861,7 +22534,7 @@
       </c>
       <c r="D134" s="28" t="str">
         <f>IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf"))</f>
-        <v>ESTIMATED kLa — DO-limited interval is 16.5 min; confirm by measuring kL_surf</v>
+        <v>ESTIMATED kLa — DO-limited interval is 17.9 min; confirm by measuring kL_surf</v>
       </c>
       <c r="E134" s="69" t="inlineStr">
         <is>
@@ -21882,7 +22555,7 @@
       </c>
       <c r="D135" s="28">
         <f>DO_hs_floor+DO_surf_excess_lag</f>
-        <v>0.171425791807</v>
+        <v>0.169683392542</v>
       </c>
       <c r="E135" s="69" t="s">
         <v>1824</v>
@@ -22100,11 +22773,13 @@
         <v>639</v>
       </c>
       <c r="D148" s="48">
-        <f>kLa_surf*sqrtD_CO2</f>
+        <f>kLa_surf_used*sqrtD_CO2</f>
         <v>0.007058740843</v>
       </c>
-      <c r="E148" s="67" t="s">
-        <v>1182</v>
+      <c r="E148" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface kLa for CO₂ between pulses (surface path), scaled from the O₂ value in use (kLa_surf_used) so a measured surface kLa also reaches the CO₂ side.</t>
+        </is>
       </c>
       <c r="F148" s="20"/>
     </row>
@@ -22177,7 +22852,7 @@
       </c>
       <c r="D152" s="48">
         <f>MAX(0,spg_int*60-spg_dur)</f>
-        <v>986.837339926971</v>
+        <v>1071.975810542231</v>
       </c>
       <c r="E152" s="67" t="s">
         <v>1190</v>
@@ -22268,7 +22943,7 @@
       </c>
       <c r="D162" s="48">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,CO2_cyc_avg_new))/1000</f>
-        <v>0.008590210622</v>
+        <v>0.008068720944</v>
       </c>
       <c r="E162" s="67" t="s">
         <v>1859</v>
@@ -22511,11 +23186,13 @@
         <v>1001</v>
       </c>
       <c r="D179" s="141">
-        <f>target_DO_frac*O2_ceil_C</f>
+        <f>IF(ISNUMBER(DO_opt),DO_opt/M_O2,target_DO_frac*O2_ceil_C)</f>
         <v>0.08246973913</v>
       </c>
-      <c r="E179" s="99" t="s">
-        <v>1795</v>
+      <c r="E179" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The dissolved O₂ the schedule aims to hold: the organism optimum DO_opt (mg/L ÷ M_O2 g/mol = mol/m³) when it is known, otherwise the target fraction of the inhibition ceiling. Avoids a Henry-derived ceiling (11.67 mg/L) that differs from the table’s 11.5 pushing the target above the optimum.</t>
+        </is>
       </c>
     </row>
     <row r="180" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -22530,7 +23207,7 @@
       </c>
       <c r="D180" s="141">
         <f>O2_excess/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.038001663161</v>
+        <v>0.03634252148</v>
       </c>
       <c r="E180" s="67" t="s">
         <v>1798</v>
@@ -22548,7 +23225,7 @@
       </c>
       <c r="D181" s="141">
         <f>O2_net_gen/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.126957715838</v>
+        <v>0.123556174892</v>
       </c>
       <c r="E181" s="67" t="s">
         <v>1801</v>
@@ -22566,7 +23243,7 @@
       </c>
       <c r="D182" s="141">
         <f>DO_target-DO_surf_excess</f>
-        <v>0.04446807597</v>
+        <v>0.046127217651</v>
       </c>
       <c r="E182" s="67" t="s">
         <v>1804</v>
@@ -22584,7 +23261,7 @@
       </c>
       <c r="D183" s="141">
         <f>IF(hs_O2_allow&gt;0,hs_O2_allow/(H_O2_T*P_atm),NA())</f>
-        <v>0.036572149</v>
+        <v>0.03793668694</v>
       </c>
       <c r="E183" s="67" t="s">
         <v>1807</v>
@@ -22602,7 +23279,7 @@
       </c>
       <c r="D184" s="141">
         <f>IF(ISNUMBER(y_O2_star),O2_excess*(1-y_O2_star)/(y_O2_star*CO2_rate_full),NA())</f>
-        <v>0.0007943455761538</v>
+        <v>0.000731303192868</v>
       </c>
       <c r="E184" s="67" t="inlineStr">
         <is>
@@ -22622,7 +23299,7 @@
       </c>
       <c r="D185" s="141">
         <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_opt/(60*duty_DO),spg_int_carbon),NA())</f>
-        <v>16.46036421628</v>
+        <v>17.879338726534</v>
       </c>
       <c r="E185" s="67" t="s">
         <v>1813</v>
@@ -22640,7 +23317,7 @@
       </c>
       <c r="D186" s="141">
         <f>O2_excess/(DO_target*3600*(V_charge/1000000))</f>
-        <v>0.003317773486</v>
+        <v>0.00317292045</v>
       </c>
       <c r="E186" s="67" t="s">
         <v>1816</v>
@@ -22658,7 +23335,7 @@
       </c>
       <c r="D187" s="141">
         <f>IF(CO2_supply&gt;0,O2_excess/(O2_excess+CO2_supply),NA())</f>
-        <v>0.036572149</v>
+        <v>0.03793668694</v>
       </c>
       <c r="E187" s="67" t="s">
         <v>1819</v>
@@ -22676,7 +23353,7 @@
       </c>
       <c r="D188" s="141">
         <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_atm,NA())</f>
-        <v>0.04446807597</v>
+        <v>0.046127217651</v>
       </c>
       <c r="E188" s="67" t="s">
         <v>1822</v>
@@ -22811,7 +23488,7 @@
       </c>
       <c r="D197" s="141">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
-        <v>0.575484483576</v>
+        <v>0.548694671753</v>
       </c>
       <c r="E197" s="99" t="s">
         <v>1849</v>
@@ -22829,7 +23506,7 @@
       </c>
       <c r="D198" s="141">
         <f>(C_air_CO2*(1-pool_e)+pool_b*pool_e)/(1-pool_a*pool_e)</f>
-        <v>6.437740764668</v>
+        <v>5.891603808766</v>
       </c>
       <c r="E198" s="99" t="s">
         <v>1852</v>
@@ -22847,7 +23524,7 @@
       </c>
       <c r="D199" s="141">
         <f>pool_a*C_cycle_start+pool_b</f>
-        <v>11.176908054727</v>
+        <v>10.726633374496</v>
       </c>
       <c r="E199" s="99" t="s">
         <v>1855</v>
@@ -22865,7 +23542,7 @@
       </c>
       <c r="D200" s="141">
         <f>C_air_CO2+(C_cycle_peak-C_air_CO2)*(1-pool_e)/(k_eff_CO2*t_off_CO2)</f>
-        <v>8.59021062192</v>
+        <v>8.068720944288</v>
       </c>
       <c r="E200" s="99" t="s">
         <v>1858</v>
@@ -23181,11 +23858,69 @@
       </c>
       <c r="D232" s="141">
         <f>H_O2_T*P_atm*O2_excess/(O2_excess+CO2_rate_full*duty_carbon)+DO_surf_excess</f>
-        <v>0.401951360368</v>
+        <v>0.393984475887</v>
       </c>
       <c r="E232" s="99" t="inlineStr">
         <is>
           <t xml:space="preserve">Same headspace back-pressure + surface-excess balance as D188/D180, evaluated at the carbon-limited duty instead of the DO-limited one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AS-RUN PULSE (solenoid command resolution)</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solenoid pulse command resolution</t>
+        </is>
+      </c>
+      <c r="B241" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pulse_res</t>
+        </is>
+      </c>
+      <c r="C241" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D241" s="146">
+        <v>0.05</v>
+      </c>
+      <c r="E241" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: the dosing command is issued in 0.05 s steps — confirm in the AEP-Plugin dosing code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Optimal pulse rounded to the command resolution</t>
+        </is>
+      </c>
+      <c r="B242" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_dur_run</t>
+        </is>
+      </c>
+      <c r="C242" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D242" s="141">
+        <f>MAX(pulse_floor,MROUND(spg_dur_opt,pulse_res))</f>
+        <v>0.8</v>
+      </c>
+      <c r="E242" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse as it can actually be commanded; never below the solenoid floor. Summary D14 shows it.</t>
         </is>
       </c>
     </row>
@@ -26619,11 +27354,11 @@
       <c r="E66" s="123"/>
       <c r="F66" s="123"/>
       <c r="G66" s="129" t="str">
-        <f>IF(E66="","",IFERROR(E66/(0.99705-0.00028*(F66-25)),""))</f>
+        <f>IF(E66="","",IFERROR(E66/((ca_rho_0+ca_rho_k*F66)/1000),""))</f>
         <v/>
       </c>
       <c r="H66" s="129" t="str">
-        <f>IF(E66="","",IFERROR((E66/(0.99705-0.00028*(F66-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E66="","",IFERROR((E66/((ca_rho_0+ca_rho_k*F66)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I66" s="129" t="str">
@@ -26633,12 +27368,12 @@
       <c r="J66" s="122"/>
       <c r="K66" s="122"/>
       <c r="L66" s="129" t="str">
-        <f>IF(D66="","",IFERROR(D66/(0.99705-0.00028*(F66-25)),""))</f>
+        <f>IF(D66="","",IFERROR(D66/((ca_rho_0+ca_rho_k*F66)/1000),""))</f>
         <v/>
       </c>
       <c r="M66" s="123"/>
       <c r="N66" s="129" t="str">
-        <f>IF(M66="","",IFERROR(M66/(0.99705-0.00028*(F66-25)),""))</f>
+        <f>IF(M66="","",IFERROR(M66/((ca_rho_0+ca_rho_k*F66)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -26650,11 +27385,11 @@
       <c r="E67" s="123"/>
       <c r="F67" s="123"/>
       <c r="G67" s="129" t="str">
-        <f>IF(E67="","",IFERROR(E67/(0.99705-0.00028*(F67-25)),""))</f>
+        <f>IF(E67="","",IFERROR(E67/((ca_rho_0+ca_rho_k*F67)/1000),""))</f>
         <v/>
       </c>
       <c r="H67" s="129" t="str">
-        <f>IF(E67="","",IFERROR((E67/(0.99705-0.00028*(F67-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E67="","",IFERROR((E67/((ca_rho_0+ca_rho_k*F67)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I67" s="129" t="str">
@@ -26664,12 +27399,12 @@
       <c r="J67" s="122"/>
       <c r="K67" s="122"/>
       <c r="L67" s="129" t="str">
-        <f>IF(D67="","",IFERROR(D67/(0.99705-0.00028*(F67-25)),""))</f>
+        <f>IF(D67="","",IFERROR(D67/((ca_rho_0+ca_rho_k*F67)/1000),""))</f>
         <v/>
       </c>
       <c r="M67" s="123"/>
       <c r="N67" s="129" t="str">
-        <f>IF(M67="","",IFERROR(M67/(0.99705-0.00028*(F67-25)),""))</f>
+        <f>IF(M67="","",IFERROR(M67/((ca_rho_0+ca_rho_k*F67)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -26681,11 +27416,11 @@
       <c r="E68" s="123"/>
       <c r="F68" s="123"/>
       <c r="G68" s="129" t="str">
-        <f>IF(E68="","",IFERROR(E68/(0.99705-0.00028*(F68-25)),""))</f>
+        <f>IF(E68="","",IFERROR(E68/((ca_rho_0+ca_rho_k*F68)/1000),""))</f>
         <v/>
       </c>
       <c r="H68" s="129" t="str">
-        <f>IF(E68="","",IFERROR((E68/(0.99705-0.00028*(F68-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E68="","",IFERROR((E68/((ca_rho_0+ca_rho_k*F68)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I68" s="129" t="str">
@@ -26695,12 +27430,12 @@
       <c r="J68" s="122"/>
       <c r="K68" s="122"/>
       <c r="L68" s="129" t="str">
-        <f>IF(D68="","",IFERROR(D68/(0.99705-0.00028*(F68-25)),""))</f>
+        <f>IF(D68="","",IFERROR(D68/((ca_rho_0+ca_rho_k*F68)/1000),""))</f>
         <v/>
       </c>
       <c r="M68" s="123"/>
       <c r="N68" s="129" t="str">
-        <f>IF(M68="","",IFERROR(M68/(0.99705-0.00028*(F68-25)),""))</f>
+        <f>IF(M68="","",IFERROR(M68/((ca_rho_0+ca_rho_k*F68)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -26712,11 +27447,11 @@
       <c r="E69" s="123"/>
       <c r="F69" s="123"/>
       <c r="G69" s="129" t="str">
-        <f>IF(E69="","",IFERROR(E69/(0.99705-0.00028*(F69-25)),""))</f>
+        <f>IF(E69="","",IFERROR(E69/((ca_rho_0+ca_rho_k*F69)/1000),""))</f>
         <v/>
       </c>
       <c r="H69" s="129" t="str">
-        <f>IF(E69="","",IFERROR((E69/(0.99705-0.00028*(F69-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E69="","",IFERROR((E69/((ca_rho_0+ca_rho_k*F69)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I69" s="129" t="str">
@@ -26726,12 +27461,12 @@
       <c r="J69" s="122"/>
       <c r="K69" s="122"/>
       <c r="L69" s="129" t="str">
-        <f>IF(D69="","",IFERROR(D69/(0.99705-0.00028*(F69-25)),""))</f>
+        <f>IF(D69="","",IFERROR(D69/((ca_rho_0+ca_rho_k*F69)/1000),""))</f>
         <v/>
       </c>
       <c r="M69" s="123"/>
       <c r="N69" s="129" t="str">
-        <f>IF(M69="","",IFERROR(M69/(0.99705-0.00028*(F69-25)),""))</f>
+        <f>IF(M69="","",IFERROR(M69/((ca_rho_0+ca_rho_k*F69)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -26743,11 +27478,11 @@
       <c r="E70" s="123"/>
       <c r="F70" s="123"/>
       <c r="G70" s="129" t="str">
-        <f>IF(E70="","",IFERROR(E70/(0.99705-0.00028*(F70-25)),""))</f>
+        <f>IF(E70="","",IFERROR(E70/((ca_rho_0+ca_rho_k*F70)/1000),""))</f>
         <v/>
       </c>
       <c r="H70" s="129" t="str">
-        <f>IF(E70="","",IFERROR((E70/(0.99705-0.00028*(F70-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E70="","",IFERROR((E70/((ca_rho_0+ca_rho_k*F70)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I70" s="129" t="str">
@@ -26757,12 +27492,12 @@
       <c r="J70" s="122"/>
       <c r="K70" s="122"/>
       <c r="L70" s="129" t="str">
-        <f>IF(D70="","",IFERROR(D70/(0.99705-0.00028*(F70-25)),""))</f>
+        <f>IF(D70="","",IFERROR(D70/((ca_rho_0+ca_rho_k*F70)/1000),""))</f>
         <v/>
       </c>
       <c r="M70" s="123"/>
       <c r="N70" s="129" t="str">
-        <f>IF(M70="","",IFERROR(M70/(0.99705-0.00028*(F70-25)),""))</f>
+        <f>IF(M70="","",IFERROR(M70/((ca_rho_0+ca_rho_k*F70)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -26774,11 +27509,11 @@
       <c r="E71" s="123"/>
       <c r="F71" s="123"/>
       <c r="G71" s="129" t="str">
-        <f>IF(E71="","",IFERROR(E71/(0.99705-0.00028*(F71-25)),""))</f>
+        <f>IF(E71="","",IFERROR(E71/((ca_rho_0+ca_rho_k*F71)/1000),""))</f>
         <v/>
       </c>
       <c r="H71" s="129" t="str">
-        <f>IF(E71="","",IFERROR((E71/(0.99705-0.00028*(F71-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E71="","",IFERROR((E71/((ca_rho_0+ca_rho_k*F71)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I71" s="129" t="str">
@@ -26788,12 +27523,12 @@
       <c r="J71" s="122"/>
       <c r="K71" s="122"/>
       <c r="L71" s="129" t="str">
-        <f>IF(D71="","",IFERROR(D71/(0.99705-0.00028*(F71-25)),""))</f>
+        <f>IF(D71="","",IFERROR(D71/((ca_rho_0+ca_rho_k*F71)/1000),""))</f>
         <v/>
       </c>
       <c r="M71" s="123"/>
       <c r="N71" s="129" t="str">
-        <f>IF(M71="","",IFERROR(M71/(0.99705-0.00028*(F71-25)),""))</f>
+        <f>IF(M71="","",IFERROR(M71/((ca_rho_0+ca_rho_k*F71)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -26805,11 +27540,11 @@
       <c r="E72" s="123"/>
       <c r="F72" s="123"/>
       <c r="G72" s="129" t="str">
-        <f>IF(E72="","",IFERROR(E72/(0.99705-0.00028*(F72-25)),""))</f>
+        <f>IF(E72="","",IFERROR(E72/((ca_rho_0+ca_rho_k*F72)/1000),""))</f>
         <v/>
       </c>
       <c r="H72" s="129" t="str">
-        <f>IF(E72="","",IFERROR((E72/(0.99705-0.00028*(F72-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E72="","",IFERROR((E72/((ca_rho_0+ca_rho_k*F72)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I72" s="129" t="str">
@@ -26819,12 +27554,12 @@
       <c r="J72" s="122"/>
       <c r="K72" s="122"/>
       <c r="L72" s="129" t="str">
-        <f>IF(D72="","",IFERROR(D72/(0.99705-0.00028*(F72-25)),""))</f>
+        <f>IF(D72="","",IFERROR(D72/((ca_rho_0+ca_rho_k*F72)/1000),""))</f>
         <v/>
       </c>
       <c r="M72" s="123"/>
       <c r="N72" s="129" t="str">
-        <f>IF(M72="","",IFERROR(M72/(0.99705-0.00028*(F72-25)),""))</f>
+        <f>IF(M72="","",IFERROR(M72/((ca_rho_0+ca_rho_k*F72)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -26836,11 +27571,11 @@
       <c r="E73" s="123"/>
       <c r="F73" s="123"/>
       <c r="G73" s="129" t="str">
-        <f>IF(E73="","",IFERROR(E73/(0.99705-0.00028*(F73-25)),""))</f>
+        <f>IF(E73="","",IFERROR(E73/((ca_rho_0+ca_rho_k*F73)/1000),""))</f>
         <v/>
       </c>
       <c r="H73" s="129" t="str">
-        <f>IF(E73="","",IFERROR((E73/(0.99705-0.00028*(F73-25)))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E73="","",IFERROR((E73/((ca_rho_0+ca_rho_k*F73)/1000))*1000/Geometry!$D$21,""))</f>
         <v/>
       </c>
       <c r="I73" s="129" t="str">
@@ -26850,12 +27585,12 @@
       <c r="J73" s="122"/>
       <c r="K73" s="122"/>
       <c r="L73" s="129" t="str">
-        <f>IF(D73="","",IFERROR(D73/(0.99705-0.00028*(F73-25)),""))</f>
+        <f>IF(D73="","",IFERROR(D73/((ca_rho_0+ca_rho_k*F73)/1000),""))</f>
         <v/>
       </c>
       <c r="M73" s="123"/>
       <c r="N73" s="129" t="str">
-        <f>IF(M73="","",IFERROR(M73/(0.99705-0.00028*(F73-25)),""))</f>
+        <f>IF(M73="","",IFERROR(M73/((ca_rho_0+ca_rho_k*F73)/1000),""))</f>
         <v/>
       </c>
     </row>
@@ -28316,6 +29051,58 @@
       <c r="E148" s="165" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Biology!D66</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Liquid density intercept</t>
+        </is>
+      </c>
+      <c r="B155" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ca_rho_0</t>
+        </is>
+      </c>
+      <c r="C155" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³</t>
+        </is>
+      </c>
+      <c r="D155" s="164">
+        <f>'Mass Transfer'!$D$169</f>
+        <v>1003.33</v>
+      </c>
+      <c r="E155" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D169 (rho_0; density law ρ = ρ₀ + k·T[°C])</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Liquid density slope</t>
+        </is>
+      </c>
+      <c r="B156" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ca_rho_k</t>
+        </is>
+      </c>
+      <c r="C156" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kg/m³/K</t>
+        </is>
+      </c>
+      <c r="D156" s="164">
+        <f>'Mass Transfer'!$D$170</f>
+        <v>-0.2556</v>
+      </c>
+      <c r="E156" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D170 (rho_k)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: schedule-mode and Summary input validation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -9880,7 +9880,7 @@
       <formula>ISNUMBER(SEARCH("OK",D49))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a listed reactor" error="Pick a reactor from the list (Geometry A59:A80)." sqref="D2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>ReactorList</formula1>
     </dataValidation>
@@ -9892,6 +9892,25 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a listed medium" error="Pick a medium from the list (Chemistry A114:A115)." sqref="D5" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>MediaList</formula1>
+    </dataValidation>
+    <dataValidation operator="between" type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Electrolysis power is 0–25 % (Gerrit's Law is validated to 25 %; the plugin clamps at 10 %)." sqref="D6">
+      <formula1>0</formula1>
+      <formula2>25</formula2>
+    </dataValidation>
+    <dataValidation operator="between" type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Stirrer rate 125–2000 rpm." sqref="D7">
+      <formula1>125</formula1>
+      <formula2>2000</formula2>
+    </dataValidation>
+    <dataValidation operator="between" type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Temperature 15–40 °C: the water-property fits are valid in that range." sqref="D8">
+      <formula1>15</formula1>
+      <formula2>40</formula2>
+    </dataValidation>
+    <dataValidation operator="greaterThan" type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Media volume in mL, or leave blank for the recommended working volume." sqref="D9">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation operator="between" type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Ambient pressure in Pa (80000–110000), or leave blank for 101325 Pa." sqref="D10">
+      <formula1>80000</formula1>
+      <formula2>110000</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22306,7 +22325,7 @@
         <v>13</v>
       </c>
       <c r="D121" s="28">
-        <f>IF(AND(ISNUMBER(Summary!$G$13),Summary!$G$13&gt;0),Summary!$G$13,IF(sched_mode="Manual",spg_dur_man,spg_dur_opt))</f>
+        <f>IF(AND(ISNUMBER(Summary!$G$13),Summary!$G$13&gt;0),Summary!$G$13,IF(sched_mode="Manual",spg_dur_man,IF(sched_mode="Optimal",spg_dur_opt,NA())))</f>
         <v>0.784513049825</v>
       </c>
       <c r="E121" s="20"/>
@@ -22323,7 +22342,7 @@
         <v>67</v>
       </c>
       <c r="D122" s="28">
-        <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,spg_int_opt))</f>
+        <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
         <v>17.879338726534</v>
       </c>
       <c r="E122" s="20"/>
@@ -24026,6 +24045,11 @@
       <formula>OR(ISNUMBER(SEARCH("OK",D110)),ISNUMBER(SEARCH("calibrated",D110)),ISNUMBER(SEARCH("under optimum",D110)),ISNUMBER(SEARCH("above min",D110)),ISNUMBER(SEARCH("exact",D110)))</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose Optimal or Manual." sqref="D81">
+      <formula1>"Optimal,Manual"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Gas model: chlorine current acts on the free chloride share; km_Cl derived from km_O2 (interval 17.9 -> 14.3 min)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -686,6 +686,8 @@
     <definedName name="CO2_margin_trough" localSheetId="4">Biology!$D$98</definedName>
     <definedName name="pulse_res" localSheetId="5">'Mass Transfer'!$D$241</definedName>
     <definedName name="spg_dur_run" localSheetId="5">'Mass Transfer'!$D$242</definedName>
+    <definedName name="D_Cl" localSheetId="3">Chemistry!$D$277</definedName>
+    <definedName name="Cl_free_frac" localSheetId="3">Chemistry!$D$278</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8296,7 +8298,7 @@
       </c>
       <c r="D15" s="90">
         <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$91)</f>
-        <v>17.879338726534</v>
+        <v>14.299822696002</v>
       </c>
       <c r="E15" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
@@ -8325,7 +8327,7 @@
       </c>
       <c r="D16" s="91">
         <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,ROUND(D14/(60*'Mass Transfer'!$D$93),0)))</f>
-        <v>18.0</v>
+        <v>15.0</v>
       </c>
       <c r="E16" s="92"/>
       <c r="F16" s="21" t="inlineStr">
@@ -8462,7 +8464,7 @@
       <c r="C23" s="20"/>
       <c r="D23" s="90" t="str">
         <f>'Mass Transfer'!$D$113</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 12.6 mg/L against a 2.6 mg/L target</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 13.7 mg/L against a 2.6 mg/L target</v>
       </c>
       <c r="E23" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
@@ -8488,7 +8490,7 @@
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 20%, O₂ 9% – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 17%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="23" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -8534,7 +8536,7 @@
       <c r="C26" s="20"/>
       <c r="D26" s="90" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)"),"calibrate this reactor first")</f>
-        <v>×21.1 OK</v>
+        <v>×26.4 OK</v>
       </c>
       <c r="E26" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
@@ -8734,7 +8736,7 @@
       <c r="C35" s="20"/>
       <c r="D35" s="121">
         <f>Chemistry!$D$220</f>
-        <v>6.622298153844</v>
+        <v>6.570596176702</v>
       </c>
       <c r="E35" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -8760,7 +8762,7 @@
       </c>
       <c r="D36" s="121">
         <f>Chemistry!$D$226</f>
-        <v>0.33955111704</v>
+        <v>0.338593949713</v>
       </c>
       <c r="E36" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
@@ -8874,7 +8876,7 @@
       </c>
       <c r="D41" s="95">
         <f>Biology!$D$98</f>
-        <v>117.832076175326</v>
+        <v>148.503370342395</v>
       </c>
       <c r="E41" s="23" t="str">
         <f>HYPERLINK("#Biology!D98","→ Biology")</f>
@@ -9644,7 +9646,7 @@
       </c>
       <c r="D87" s="22">
         <f>Chemistry!$D$209</f>
-        <v>-0.413578182478</v>
+        <v>-0.42751475509</v>
       </c>
       <c r="E87" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D209","→ Chemistry")</f>
@@ -9670,7 +9672,7 @@
       </c>
       <c r="D88" s="22">
         <f>Chemistry!$D$211</f>
-        <v>1.239471571289</v>
+        <v>1.242530226635</v>
       </c>
       <c r="E88" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
@@ -9696,7 +9698,7 @@
       </c>
       <c r="D89" s="22">
         <f>Chemistry!$D$220</f>
-        <v>6.622298153844</v>
+        <v>6.570596176702</v>
       </c>
       <c r="E89" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -9720,7 +9722,7 @@
       </c>
       <c r="D90" s="22">
         <f>'Mass Transfer'!$D$186</f>
-        <v>0.00317292045</v>
+        <v>0.003566106821</v>
       </c>
       <c r="E90" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D186","→ Mass Transfer")</f>
@@ -9775,7 +9777,7 @@
       </c>
       <c r="D95" s="95">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),D14/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (see CO2 flows)")</f>
-        <v>1.012905109625</v>
+        <v>0.972140884876</v>
       </c>
       <c r="E95" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
@@ -12107,7 +12109,7 @@
       </c>
       <c r="D22" s="48">
         <f>I_app*etaF_OER/(z_e_O2*F_const)*3600</f>
-        <v>5.043034859204e-05</v>
+        <v>5.218135137208e-05</v>
       </c>
       <c r="E22" s="99" t="s">
         <v>358</v>
@@ -12151,7 +12153,7 @@
       </c>
       <c r="D24" s="48">
         <f>rO2_gen/60*R_gas*T_K/P_atm*1000000</f>
-        <v>0.020563313948</v>
+        <v>0.021277297113</v>
       </c>
       <c r="E24" s="99" t="s">
         <v>365</v>
@@ -12173,7 +12175,7 @@
       </c>
       <c r="D25" s="48">
         <f>V_H2_gen+V_O2_gen</f>
-        <v>0.062043374238</v>
+        <v>0.062757357403</v>
       </c>
       <c r="E25" s="99" t="s">
         <v>368</v>
@@ -12195,7 +12197,7 @@
       </c>
       <c r="D26" s="42">
         <f>IF(ISNUMBER(cal_etaF_OER),cal_etaF_OER,etaF_OER_calc)</f>
-        <v>0.950163822072</v>
+        <v>0.983154660731</v>
       </c>
       <c r="E26" s="67" t="inlineStr">
         <is>
@@ -12269,7 +12271,7 @@
       </c>
       <c r="D29" s="48">
         <f>rO2_gen-O2_cathode_ORR</f>
-        <v>4.803933240197e-05</v>
+        <v>4.979033518202e-05</v>
       </c>
       <c r="E29" s="99" t="s">
         <v>379</v>
@@ -13586,7 +13588,7 @@
       </c>
       <c r="D101" s="141">
         <f>Chemistry!$D$133</f>
-        <v>0.0002835678524112</v>
+        <v>9.584998043788e-05</v>
       </c>
       <c r="E101" s="67" t="s">
         <v>1689</v>
@@ -13622,7 +13624,7 @@
       </c>
       <c r="D103" s="141">
         <f>ec_I_Cl/I_app</f>
-        <v>0.049836177928</v>
+        <v>0.016845339269</v>
       </c>
       <c r="E103" s="67" t="inlineStr">
         <is>
@@ -13642,7 +13644,7 @@
       </c>
       <c r="D104" s="141">
         <f>MAX(0,1-f_Cl_anode-IF(ISNUMBER(ec_corr_I),ec_corr_I,0)-IF(ISNUMBER(f_HOR_anode),f_HOR_anode,0))</f>
-        <v>0.950163822072</v>
+        <v>0.983154660731</v>
       </c>
       <c r="E104" s="67" t="inlineStr">
         <is>
@@ -14465,7 +14467,7 @@
       </c>
       <c r="D5" s="64">
         <f>'Mass Transfer'!$D$162</f>
-        <v>0.008068720944</v>
+        <v>0.00952617025</v>
       </c>
       <c r="E5" s="51" t="inlineStr">
         <is>
@@ -15145,7 +15147,7 @@
       </c>
       <c r="B50" s="64">
         <f t="shared" ref="B50:B81" si="1">pH_SID + pH_NT*(10^-A50)/((10^-A50)+KaN_c) + (10^-A50) - (pH_PT*Ka1p_c*(10^-A50)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A50) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A50)^3 + Ka1p_c*(10^-A50)^2 + Ka1p_c*Ka2p_c*(10^-A50) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A50) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A50)^2 - Kw_c/(10^-A50)</f>
-        <v>0.033217771584</v>
+        <v>0.033207024661</v>
       </c>
       <c r="C50" s="64">
         <f>IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
@@ -15158,7 +15160,7 @@
       </c>
       <c r="B51" s="64">
         <f t="shared" si="1"/>
-        <v>0.033100832196</v>
+        <v>0.033087302614</v>
       </c>
       <c r="C51" s="64">
         <f>IF(AND(B51&gt;=0,B52&lt;0),A51+pH_step*B51/(B51-B52),0)</f>
@@ -15171,7 +15173,7 @@
       </c>
       <c r="B52" s="64">
         <f t="shared" si="1"/>
-        <v>0.032992893794</v>
+        <v>0.032975861045</v>
       </c>
       <c r="C52" s="64">
         <f>IF(AND(B52&gt;=0,B53&lt;0),A52+pH_step*B52/(B52-B53),0)</f>
@@ -15184,7 +15186,7 @@
       </c>
       <c r="B53" s="64">
         <f t="shared" si="1"/>
-        <v>0.032888324572</v>
+        <v>0.032866881589</v>
       </c>
       <c r="C53" s="64">
         <f>IF(AND(B53&gt;=0,B54&lt;0),A53+pH_step*B53/(B53-B54),0)</f>
@@ -15197,7 +15199,7 @@
       </c>
       <c r="B54" s="64">
         <f t="shared" si="1"/>
-        <v>0.032781645403</v>
+        <v>0.03275465025</v>
       </c>
       <c r="C54" s="64">
         <f>IF(AND(B54&gt;=0,B55&lt;0),A54+pH_step*B54/(B54-B55),0)</f>
@@ -15210,7 +15212,7 @@
       </c>
       <c r="B55" s="64">
         <f t="shared" si="1"/>
-        <v>0.032667256944</v>
+        <v>0.032633272003</v>
       </c>
       <c r="C55" s="64">
         <f>IF(AND(B55&gt;=0,B56&lt;0),A55+pH_step*B55/(B55-B56),0)</f>
@@ -15223,7 +15225,7 @@
       </c>
       <c r="B56" s="64">
         <f t="shared" si="1"/>
-        <v>0.032539158733</v>
+        <v>0.032496374136</v>
       </c>
       <c r="C56" s="64">
         <f>IF(AND(B56&gt;=0,B57&lt;0),A56+pH_step*B56/(B56-B57),0)</f>
@@ -15236,7 +15238,7 @@
       </c>
       <c r="B57" s="64">
         <f t="shared" si="1"/>
-        <v>0.032390648851</v>
+        <v>0.032336786093</v>
       </c>
       <c r="C57" s="64">
         <f>IF(AND(B57&gt;=0,B58&lt;0),A57+pH_step*B57/(B57-B58),0)</f>
@@ -15249,7 +15251,7 @@
       </c>
       <c r="B58" s="64">
         <f t="shared" si="1"/>
-        <v>0.032213992108</v>
+        <v>0.032146182686</v>
       </c>
       <c r="C58" s="64">
         <f>IF(AND(B58&gt;=0,B59&lt;0),A58+pH_step*B58/(B58-B59),0)</f>
@@ -15262,7 +15264,7 @@
       </c>
       <c r="B59" s="64">
         <f t="shared" si="1"/>
-        <v>0.032000044096</v>
+        <v>0.031914676733</v>
       </c>
       <c r="C59" s="64">
         <f>IF(AND(B59&gt;=0,B60&lt;0),A59+pH_step*B59/(B59-B60),0)</f>
@@ -15275,7 +15277,7 @@
       </c>
       <c r="B60" s="64">
         <f t="shared" si="1"/>
-        <v>0.031737818179</v>
+        <v>0.031630346466</v>
       </c>
       <c r="C60" s="64">
         <f>IF(AND(B60&gt;=0,B61&lt;0),A60+pH_step*B60/(B60-B61),0)</f>
@@ -15288,7 +15290,7 @@
       </c>
       <c r="B61" s="64">
         <f t="shared" si="1"/>
-        <v>0.031413982653</v>
+        <v>0.031278682881</v>
       </c>
       <c r="C61" s="64">
         <f>IF(AND(B61&gt;=0,B62&lt;0),A61+pH_step*B61/(B61-B62),0)</f>
@@ -15301,7 +15303,7 @@
       </c>
       <c r="B62" s="64">
         <f t="shared" si="1"/>
-        <v>0.031012276465</v>
+        <v>0.030841942713</v>
       </c>
       <c r="C62" s="64">
         <f>IF(AND(B62&gt;=0,B63&lt;0),A62+pH_step*B62/(B62-B63),0)</f>
@@ -15314,7 +15316,7 @@
       </c>
       <c r="B63" s="64">
         <f t="shared" si="1"/>
-        <v>0.030512834504</v>
+        <v>0.030298394749</v>
       </c>
       <c r="C63" s="64">
         <f>IF(AND(B63&gt;=0,B64&lt;0),A63+pH_step*B63/(B63-B64),0)</f>
@@ -15327,7 +15329,7 @@
       </c>
       <c r="B64" s="64">
         <f t="shared" si="1"/>
-        <v>0.029891418344</v>
+        <v>0.029621451096</v>
       </c>
       <c r="C64" s="64">
         <f>IF(AND(B64&gt;=0,B65&lt;0),A64+pH_step*B64/(B64-B65),0)</f>
@@ -15340,7 +15342,7 @@
       </c>
       <c r="B65" s="64">
         <f t="shared" si="1"/>
-        <v>0.029118555933</v>
+        <v>0.028778681611</v>
       </c>
       <c r="C65" s="64">
         <f>IF(AND(B65&gt;=0,B66&lt;0),A65+pH_step*B65/(B65-B66),0)</f>
@@ -15353,7 +15355,7 @@
       </c>
       <c r="B66" s="64">
         <f t="shared" si="1"/>
-        <v>0.028158604254</v>
+        <v>0.02773071881</v>
       </c>
       <c r="C66" s="64">
         <f>IF(AND(B66&gt;=0,B67&lt;0),A66+pH_step*B66/(B66-B67),0)</f>
@@ -15366,7 +15368,7 @@
       </c>
       <c r="B67" s="64">
         <f t="shared" si="1"/>
-        <v>0.026968761394</v>
+        <v>0.026430071236</v>
       </c>
       <c r="C67" s="64">
         <f>IF(AND(B67&gt;=0,B68&lt;0),A67+pH_step*B67/(B67-B68),0)</f>
@@ -15379,7 +15381,7 @@
       </c>
       <c r="B68" s="64">
         <f t="shared" si="1"/>
-        <v>0.025498065093</v>
+        <v>0.024819871701</v>
       </c>
       <c r="C68" s="64">
         <f>IF(AND(B68&gt;=0,B69&lt;0),A68+pH_step*B68/(B68-B69),0)</f>
@@ -15392,7 +15394,7 @@
       </c>
       <c r="B69" s="64">
         <f t="shared" si="1"/>
-        <v>0.023686416142</v>
+        <v>0.022832585328</v>
       </c>
       <c r="C69" s="64">
         <f>IF(AND(B69&gt;=0,B70&lt;0),A69+pH_step*B69/(B69-B70),0)</f>
@@ -15405,7 +15407,7 @@
       </c>
       <c r="B70" s="64">
         <f t="shared" si="1"/>
-        <v>0.021463643599</v>
+        <v>0.020388677363</v>
       </c>
       <c r="C70" s="64">
         <f>IF(AND(B70&gt;=0,B71&lt;0),A70+pH_step*B70/(B70-B71),0)</f>
@@ -15418,7 +15420,7 @@
       </c>
       <c r="B71" s="64">
         <f t="shared" si="1"/>
-        <v>0.018748565553</v>
+        <v>0.017395173018</v>
       </c>
       <c r="C71" s="64">
         <f>IF(AND(B71&gt;=0,B72&lt;0),A71+pH_step*B71/(B71-B72),0)</f>
@@ -15431,7 +15433,7 @@
       </c>
       <c r="B72" s="64">
         <f t="shared" si="1"/>
-        <v>0.015447872883</v>
+        <v>0.013743909634</v>
       </c>
       <c r="C72" s="64">
         <f>IF(AND(B72&gt;=0,B73&lt;0),A72+pH_step*B72/(B72-B73),0)</f>
@@ -15444,7 +15446,7 @@
       </c>
       <c r="B73" s="64">
         <f t="shared" si="1"/>
-        <v>0.011454461141</v>
+        <v>0.009309071874</v>
       </c>
       <c r="C73" s="64">
         <f>IF(AND(B73&gt;=0,B74&lt;0),A73+pH_step*B73/(B73-B74),0)</f>
@@ -15457,11 +15459,11 @@
       </c>
       <c r="B74" s="64">
         <f t="shared" si="1"/>
-        <v>0.006644569952</v>
+        <v>0.003943325701</v>
       </c>
       <c r="C74" s="64">
         <f>IF(AND(B74&gt;=0,B75&lt;0),A74+pH_step*B74/(B74-B75),0)</f>
-        <v>0.0</v>
+        <v>6.460931418262</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -15470,11 +15472,11 @@
       </c>
       <c r="B75" s="64">
         <f t="shared" si="1"/>
-        <v>0.0008728155195231</v>
+        <v>-0.002528418784</v>
       </c>
       <c r="C75" s="64">
         <f>IF(AND(B75&gt;=0,B76&lt;0),A75+pH_step*B75/(B75-B76),0)</f>
-        <v>6.512633395404</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
@@ -15483,7 +15485,7 @@
       </c>
       <c r="B76" s="64">
         <f t="shared" si="1"/>
-        <v>-0.006035980506</v>
+        <v>-0.010318783037</v>
       </c>
       <c r="C76" s="64">
         <f>IF(AND(B76&gt;=0,B77&lt;0),A76+pH_step*B76/(B76-B77),0)</f>
@@ -15496,7 +15498,7 @@
       </c>
       <c r="B77" s="64">
         <f t="shared" si="1"/>
-        <v>-0.014299245629</v>
+        <v>-0.019692404515</v>
       </c>
       <c r="C77" s="64">
         <f>IF(AND(B77&gt;=0,B78&lt;0),A77+pH_step*B77/(B77-B78),0)</f>
@@ -15509,7 +15511,7 @@
       </c>
       <c r="B78" s="64">
         <f t="shared" si="1"/>
-        <v>-0.024194216159</v>
+        <v>-0.03098606724</v>
       </c>
       <c r="C78" s="64">
         <f>IF(AND(B78&gt;=0,B79&lt;0),A78+pH_step*B78/(B78-B79),0)</f>
@@ -15522,7 +15524,7 @@
       </c>
       <c r="B79" s="64">
         <f t="shared" si="1"/>
-        <v>-0.036081020585</v>
+        <v>-0.044635046365</v>
       </c>
       <c r="C79" s="64">
         <f>IF(AND(B79&gt;=0,B80&lt;0),A79+pH_step*B79/(B79-B80),0)</f>
@@ -15535,7 +15537,7 @@
       </c>
       <c r="B80" s="64">
         <f t="shared" si="1"/>
-        <v>-0.050431397619</v>
+        <v>-0.061205970764</v>
       </c>
       <c r="C80" s="64">
         <f>IF(AND(B80&gt;=0,B81&lt;0),A80+pH_step*B80/(B80-B81),0)</f>
@@ -15548,7 +15550,7 @@
       </c>
       <c r="B81" s="64">
         <f t="shared" si="1"/>
-        <v>-0.0678632255</v>
+        <v>-0.08143663178</v>
       </c>
       <c r="C81" s="64">
         <f>IF(AND(B81&gt;=0,B82&lt;0),A81+pH_step*B81/(B81-B82),0)</f>
@@ -15561,7 +15563,7 @@
       </c>
       <c r="B82" s="64">
         <f t="shared" ref="B82:B113" si="3">pH_SID + pH_NT*(10^-A82)/((10^-A82)+KaN_c) + (10^-A82) - (pH_PT*Ka1p_c*(10^-A82)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A82) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A82)^3 + Ka1p_c*(10^-A82)^2 + Ka1p_c*Ka2p_c*(10^-A82) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A82) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A82)^2 - Kw_c/(10^-A82)</f>
-        <v>-0.089181639593</v>
+        <v>-0.10628384514</v>
       </c>
       <c r="C82" s="64">
         <f>IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
@@ -15574,7 +15576,7 @@
       </c>
       <c r="B83" s="64">
         <f t="shared" si="3"/>
-        <v>-0.115428610375</v>
+        <v>-0.136981674648</v>
       </c>
       <c r="C83" s="64">
         <f>IF(AND(B83&gt;=0,B84&lt;0),A83+pH_step*B83/(B83-B84),0)</f>
@@ -15587,7 +15589,7 @@
       </c>
       <c r="B84" s="64">
         <f t="shared" si="3"/>
-        <v>-0.147944267405</v>
+        <v>-0.175113886331</v>
       </c>
       <c r="C84" s="64">
         <f>IF(AND(B84&gt;=0,B85&lt;0),A84+pH_step*B84/(B84-B85),0)</f>
@@ -15600,7 +15602,7 @@
       </c>
       <c r="B85" s="64">
         <f t="shared" si="3"/>
-        <v>-0.188444839472</v>
+        <v>-0.222706290329</v>
       </c>
       <c r="C85" s="64">
         <f>IF(AND(B85&gt;=0,B86&lt;0),A85+pH_step*B85/(B85-B86),0)</f>
@@ -15613,7 +15615,7 @@
       </c>
       <c r="B86" s="64">
         <f t="shared" si="3"/>
-        <v>-0.239123861813</v>
+        <v>-0.282346696413</v>
       </c>
       <c r="C86" s="64">
         <f>IF(AND(B86&gt;=0,B87&lt;0),A86+pH_step*B86/(B86-B87),0)</f>
@@ -15626,7 +15628,7 @@
       </c>
       <c r="B87" s="64">
         <f t="shared" si="3"/>
-        <v>-0.302785522984</v>
+        <v>-0.357342842397</v>
       </c>
       <c r="C87" s="64">
         <f>IF(AND(B87&gt;=0,B88&lt;0),A87+pH_step*B87/(B87-B88),0)</f>
@@ -15639,7 +15641,7 @@
       </c>
       <c r="B88" s="64">
         <f t="shared" si="3"/>
-        <v>-0.383022129896</v>
+        <v>-0.45193235682</v>
       </c>
       <c r="C88" s="64">
         <f>IF(AND(B88&gt;=0,B89&lt;0),A88+pH_step*B88/(B88-B89),0)</f>
@@ -15652,7 +15654,7 @@
       </c>
       <c r="B89" s="64">
         <f t="shared" si="3"/>
-        <v>-0.484452287112</v>
+        <v>-0.571564309028</v>
       </c>
       <c r="C89" s="64">
         <f>IF(AND(B89&gt;=0,B90&lt;0),A89+pH_step*B89/(B89-B90),0)</f>
@@ -15665,7 +15667,7 @@
       </c>
       <c r="B90" s="64">
         <f t="shared" si="3"/>
-        <v>-0.613043384086</v>
+        <v>-0.723280193768</v>
       </c>
       <c r="C90" s="64">
         <f>IF(AND(B90&gt;=0,B91&lt;0),A90+pH_step*B90/(B90-B91),0)</f>
@@ -15678,7 +15680,7 @@
       </c>
       <c r="B91" s="64">
         <f t="shared" si="3"/>
-        <v>-0.776552624517</v>
+        <v>-0.916234780256</v>
       </c>
       <c r="C91" s="64">
         <f>IF(AND(B91&gt;=0,B92&lt;0),A91+pH_step*B91/(B91-B92),0)</f>
@@ -15691,7 +15693,7 @@
       </c>
       <c r="B92" s="64">
         <f t="shared" si="3"/>
-        <v>-0.985137039874</v>
+        <v>-1.162416400965</v>
       </c>
       <c r="C92" s="64">
         <f>IF(AND(B92&gt;=0,B93&lt;0),A92+pH_step*B92/(B92-B93),0)</f>
@@ -15704,7 +15706,7 @@
       </c>
       <c r="B93" s="64">
         <f t="shared" si="3"/>
-        <v>-1.252207705306</v>
+        <v>-1.477655509108</v>
       </c>
       <c r="C93" s="64">
         <f>IF(AND(B93&gt;=0,B94&lt;0),A93+pH_step*B93/(B93-B94),0)</f>
@@ -15717,7 +15719,7 @@
       </c>
       <c r="B94" s="64">
         <f t="shared" si="3"/>
-        <v>-1.595641435687</v>
+        <v>-1.883055266022</v>
       </c>
       <c r="C94" s="64">
         <f>IF(AND(B94&gt;=0,B95&lt;0),A94+pH_step*B94/(B94-B95),0)</f>
@@ -15730,7 +15732,7 @@
       </c>
       <c r="B95" s="64">
         <f t="shared" si="3"/>
-        <v>-2.03952200596</v>
+        <v>-2.407047296867</v>
       </c>
       <c r="C95" s="64">
         <f>IF(AND(B95&gt;=0,B96&lt;0),A95+pH_step*B95/(B95-B96),0)</f>
@@ -15743,7 +15745,7 @@
       </c>
       <c r="B96" s="64">
         <f t="shared" si="3"/>
-        <v>-2.616674108835</v>
+        <v>-3.088383384182</v>
       </c>
       <c r="C96" s="64">
         <f>IF(AND(B96&gt;=0,B97&lt;0),A96+pH_step*B96/(B96-B97),0)</f>
@@ -15756,7 +15758,7 @@
       </c>
       <c r="B97" s="64">
         <f t="shared" si="3"/>
-        <v>-3.372395273475</v>
+        <v>-3.980541523763</v>
       </c>
       <c r="C97" s="64">
         <f>IF(AND(B97&gt;=0,B98&lt;0),A97+pH_step*B97/(B97-B98),0)</f>
@@ -15769,7 +15771,7 @@
       </c>
       <c r="B98" s="64">
         <f t="shared" si="3"/>
-        <v>-4.370012913997</v>
+        <v>-5.158286793953</v>
       </c>
       <c r="C98" s="64">
         <f>IF(AND(B98&gt;=0,B99&lt;0),A98+pH_step*B98/(B98-B99),0)</f>
@@ -15782,7 +15784,7 @@
       </c>
       <c r="B99" s="64">
         <f t="shared" si="3"/>
-        <v>-5.699241495811</v>
+        <v>-6.727538125688</v>
       </c>
       <c r="C99" s="64">
         <f>IF(AND(B99&gt;=0,B100&lt;0),A99+pH_step*B99/(B99-B100),0)</f>
@@ -15795,7 +15797,7 @@
       </c>
       <c r="B100" s="64">
         <f t="shared" si="3"/>
-        <v>-7.488861095159</v>
+        <v>-8.840337015349</v>
       </c>
       <c r="C100" s="64">
         <f>0</f>
@@ -15837,7 +15839,7 @@
       </c>
       <c r="D103" s="149">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
-        <v>6.512633395404</v>
+        <v>6.460931418262</v>
       </c>
       <c r="E103" s="51" t="s">
         <v>1878</v>
@@ -15860,7 +15862,7 @@
       </c>
       <c r="D104" s="149">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
-        <v>0.865363856191</v>
+        <v>0.878640899134</v>
       </c>
       <c r="E104" s="51" t="s">
         <v>1879</v>
@@ -15949,7 +15951,7 @@
       </c>
       <c r="D109" s="64" t="str">
         <f>IF(C_eff_Cl2&lt;Cl_onset,"negligible free chlorine ("&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ &lt; onset); does NOT account for the Exp-2 death - see metal_flag",IF(C_eff_Cl2&lt;Cl_kill,"sub-lethal "&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ (band "&amp;TEXT(C_eff_lo_Cl2,"0.00")&amp;"-"&amp;TEXT(C_eff_hi_Cl2,"0.00")&amp;"); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag","SEVERE free chlorine: "&amp;TEXT(C_eff_Cl2,"0.0")&amp;" mg/L as Cl₂ - biofilm/electrode damage (Baek 2021)"))</f>
-        <v>sub-lethal 0.34 mg/L as Cl₂ (band 0.01-0.65); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
+        <v>sub-lethal 0.34 mg/L as Cl₂ (band 0.01-0.64); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
       </c>
       <c r="E109" s="51" t="s">
         <v>1127</v>
@@ -16052,7 +16054,7 @@
       </c>
       <c r="D125" s="149">
         <f>pH_Cl*pH_fHOCl*M_HOCl</f>
-        <v>8.181111532849</v>
+        <v>8.306632108229</v>
       </c>
       <c r="E125" s="51" t="s">
         <v>1460</v>
@@ -16091,10 +16093,13 @@
         <v>1070</v>
       </c>
       <c r="D129" s="146">
-        <v>4.0499999999999998E-3</v>
-      </c>
-      <c r="E129" s="51" t="s">
-        <v>1756</v>
+        <f>km_O2_c*(D_Cl/D_O2_c)^km_exp_c</f>
+        <v>0.004044131217</v>
+      </c>
+      <c r="E129" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scaled from the electrode O₂ mass-transfer coefficient by (D_Cl/D_O2)^0.644, the same correlation as km_HPO4/km_HCO3 (rows 275–276), so it follows a measured km_O2.</t>
+        </is>
       </c>
     </row>
     <row r="130" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -16144,8 +16149,8 @@
         <v>1076</v>
       </c>
       <c r="D132" s="149">
-        <f>n_e_Cl*Fcc*km_Cl*(pH_Cl/1000)*A_anode</f>
-        <v>0.0002835678524112</v>
+        <f>n_e_Cl*Fcc*km_Cl*(pH_Cl*Cl_free_frac/1000)*A_anode</f>
+        <v>9.584998043788e-05</v>
       </c>
       <c r="E132" s="75" t="inlineStr">
         <is>
@@ -16165,7 +16170,7 @@
       </c>
       <c r="D133" s="149">
         <f>MIN(I_Cl_FE,I_Cl_mt)</f>
-        <v>0.0002835678524112</v>
+        <v>9.584998043788e-05</v>
       </c>
       <c r="E133" s="51" t="s">
         <v>1082</v>
@@ -16183,7 +16188,7 @@
       </c>
       <c r="D134" s="149">
         <f>I_Cl/(n_e_Cl*Fcc*VLc)</f>
-        <v>9.796578961125e-08</v>
+        <v>3.311383479466e-08</v>
       </c>
       <c r="E134" s="51" t="inlineStr">
         <is>
@@ -16256,7 +16261,7 @@
       </c>
       <c r="D138" s="149">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
-        <v>1.294565152087e-05</v>
+        <v>1.149504426795e-05</v>
       </c>
       <c r="E138" s="51" t="s">
         <v>1099</v>
@@ -16274,7 +16279,7 @@
       </c>
       <c r="D139" s="149">
         <f>P_HOCl/(k1_NH2Cl*NH3_free)</f>
-        <v>1.801777837529e-09</v>
+        <v>6.858822111426e-10</v>
       </c>
       <c r="E139" s="51" t="s">
         <v>1102</v>
@@ -16292,7 +16297,7 @@
       </c>
       <c r="D140" s="149">
         <f>HOCl_ss*M_HOCl</f>
-        <v>9.452126535676e-05</v>
+        <v>3.598138079654e-05</v>
       </c>
       <c r="E140" s="51" t="s">
         <v>1105</v>
@@ -16344,7 +16349,7 @@
       </c>
       <c r="D143" s="149">
         <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl*3600)/(1+k_Cl_turn*tau_NH2Cl*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
-        <v>6.256815485116</v>
+        <v>6.25374638398</v>
       </c>
       <c r="E143" s="51" t="inlineStr">
         <is>
@@ -16381,7 +16386,7 @@
       </c>
       <c r="D145" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_mgL/R_chloramine</f>
-        <v>0.251217832058</v>
+        <v>0.250509669167</v>
       </c>
       <c r="E145" s="51" t="inlineStr">
         <is>
@@ -16543,7 +16548,7 @@
       </c>
       <c r="D154" s="149">
         <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl_lo*3600)/(1+k_Cl_turn*tau_NH2Cl_lo*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
-        <v>0.298617202708</v>
+        <v>0.298198130773</v>
       </c>
       <c r="E154" s="51" t="inlineStr">
         <is>
@@ -16563,7 +16568,7 @@
       </c>
       <c r="D155" s="149">
         <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl_hi*3600)/(1+k_Cl_turn*tau_NH2Cl_hi*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
-        <v>8.577373468854</v>
+        <v>8.57621949016</v>
       </c>
       <c r="E155" s="51" t="inlineStr">
         <is>
@@ -16583,7 +16588,7 @@
       </c>
       <c r="D156" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_lo/R_chloramine_hi</f>
-        <v>0.005211172692</v>
+        <v>0.004619787105</v>
       </c>
       <c r="E156" s="51" t="s">
         <v>1247</v>
@@ -16601,7 +16606,7 @@
       </c>
       <c r="D157" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_hi/R_chloramine_lo</f>
-        <v>0.477465960923</v>
+        <v>0.47681645215</v>
       </c>
       <c r="E157" s="51" t="s">
         <v>1251</v>
@@ -17367,7 +17372,7 @@
       </c>
       <c r="D206" s="141">
         <f>E0_OER-nernst_slope*pH_meas</f>
-        <v>0.837229147794</v>
+        <v>0.840287803139</v>
       </c>
       <c r="E206" s="99" t="s">
         <v>1586</v>
@@ -17385,7 +17390,7 @@
       </c>
       <c r="D207" s="141">
         <f>E0_HER-nernst_slope*pH_meas</f>
-        <v>-0.391770852206</v>
+        <v>-0.388712196861</v>
       </c>
       <c r="E207" s="99" t="s">
         <v>1589</v>
@@ -17425,7 +17430,7 @@
       </c>
       <c r="D209" s="141">
         <f>E_HOCl_Cl-E_anode_op</f>
-        <v>-0.413578182478</v>
+        <v>-0.42751475509</v>
       </c>
       <c r="E209" s="67" t="inlineStr">
         <is>
@@ -17445,7 +17450,7 @@
       </c>
       <c r="D210" s="141">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
-        <v>0.303229147794</v>
+        <v>0.306287803139</v>
       </c>
       <c r="E210" s="67" t="s">
         <v>1599</v>
@@ -17465,7 +17470,7 @@
       </c>
       <c r="D211" s="141">
         <f>E_anode_op-E0_Cu</f>
-        <v>1.239471571289</v>
+        <v>1.242530226635</v>
       </c>
       <c r="E211" s="67" t="s">
         <v>1602</v>
@@ -17527,7 +17532,7 @@
       </c>
       <c r="D216" s="141">
         <f>Fcc*((km_HPO4/100)*HPO4_op+(km_HCO3/100)*HCO3_op)*1000/10</f>
-        <v>8.126539606735</v>
+        <v>8.175182209731</v>
       </c>
       <c r="E216" s="67" t="inlineStr">
         <is>
@@ -17565,7 +17570,7 @@
       </c>
       <c r="D218" s="141">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>0.347761264334</v>
+        <v>0.345692073374</v>
       </c>
       <c r="E218" s="67" t="s">
         <v>1618</v>
@@ -17601,7 +17606,7 @@
       </c>
       <c r="D220" s="141">
         <f>pH_op-LOG10(gamma_1)</f>
-        <v>6.622298153844</v>
+        <v>6.570596176702</v>
       </c>
       <c r="E220" s="67" t="s">
         <v>1624</v>
@@ -17694,7 +17699,7 @@
       </c>
       <c r="D226" s="141">
         <f>C_eff*M_Cl2/M_HOCl</f>
-        <v>0.33955111704</v>
+        <v>0.338593949713</v>
       </c>
       <c r="E226" s="67" t="s">
         <v>1899</v>
@@ -18008,7 +18013,7 @@
       </c>
       <c r="D252" s="141">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
-        <v>0.01936991072</v>
+        <v>0.020302021576</v>
       </c>
       <c r="E252" s="67" t="inlineStr">
         <is>
@@ -18034,7 +18039,7 @@
       </c>
       <c r="D253" s="141">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
-        <v>0.013462331212</v>
+        <v>0.012455537296</v>
       </c>
       <c r="E253" s="67" t="inlineStr">
         <is>
@@ -18112,7 +18117,7 @@
       </c>
       <c r="D256" s="141">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
-        <v>1.581371571289</v>
+        <v>1.584430226635</v>
       </c>
       <c r="E256" s="67" t="inlineStr">
         <is>
@@ -18163,7 +18168,7 @@
       </c>
       <c r="D258" s="141">
         <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,1E-12))-pH_meas-LOG10(MAX(pH_Cl,1E-12)))</f>
-        <v>1.167793388811</v>
+        <v>1.156915471544</v>
       </c>
       <c r="E258" s="67" t="inlineStr">
         <is>
@@ -18189,7 +18194,7 @@
       </c>
       <c r="D259" s="141">
         <f>C_eff_lo*M_Cl2/M_HOCl</f>
-        <v>0.007043526704</v>
+        <v>0.00624419795</v>
       </c>
       <c r="E259" s="67" t="inlineStr">
         <is>
@@ -18215,7 +18220,7 @@
       </c>
       <c r="D260" s="141">
         <f>C_eff_hi*M_Cl2/M_HOCl</f>
-        <v>0.645352676806</v>
+        <v>0.644474787575</v>
       </c>
       <c r="E260" s="67" t="inlineStr">
         <is>
@@ -18247,12 +18252,12 @@
         </is>
       </c>
       <c r="D271" s="141">
-        <f>IF(pH_Cl&gt;0,P_HOCl/pH_Cl,0)</f>
-        <v>0.0005436121665528</v>
+        <f>km_Cl*A_anode/1000/VLc</f>
+        <v>0.0005428244278184</v>
       </c>
       <c r="E271" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chlorine production per unit bulk chloride, = km_Cl·A_anode/V at the chloride transport limit (D132–D134). Chloride cycles Cl⁻ → HOCl → NH₂Cl → Cl⁻ (chloramine decay and cathodic reduction both return chloride), so the pool is shared, not consumed.</t>
+          <t xml:space="preserve">First-order anodic chloride turnover at the transport limit, km_Cl·A/V (cm³ → L by /1000). Independent of the chloride level, so the recycling split (D278, D143) is not circular.</t>
         </is>
       </c>
     </row>
@@ -18383,6 +18388,57 @@
       <c r="E276" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">As D275, for bicarbonate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Diffusion coefficient — Cl⁻</t>
+        </is>
+      </c>
+      <c r="B277" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D_Cl</t>
+        </is>
+      </c>
+      <c r="C277" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m²/s</t>
+        </is>
+      </c>
+      <c r="D277" s="146">
+        <v>2.032e-09</v>
+      </c>
+      <c r="E277" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CRC Handbook (Vanýsek), ionic diffusion coefficient at 25 °C, 2.032×10⁻⁵ cm²/s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Free share of the chloride pool</t>
+        </is>
+      </c>
+      <c r="B278" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cl_free_frac</t>
+        </is>
+      </c>
+      <c r="C278" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D278" s="141">
+        <f>1/(1+k_Cl_turn*tau_NH2Cl*3600)</f>
+        <v>0.338504790608</v>
+      </c>
+      <c r="E278" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At steady state the chloride pool splits free : combined = 1 : kτ (row 271 and D143), so only this share is available to the anode.</t>
         </is>
       </c>
     </row>
@@ -18487,7 +18543,7 @@
       </c>
       <c r="D5" s="150">
         <f>Electrochemistry!$D$29</f>
-        <v>4.803933240197e-05</v>
+        <v>4.979033518202e-05</v>
       </c>
       <c r="E5" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -18687,7 +18743,7 @@
       </c>
       <c r="D16" s="48">
         <f>MAX(0,O2_net_gen-O2_cons)</f>
-        <v>1.413017577815e-05</v>
+        <v>1.58811785582e-05</v>
       </c>
       <c r="E16" s="115" t="s">
         <v>1926</v>
@@ -19210,7 +19266,7 @@
       </c>
       <c r="D44" s="48" t="str">
         <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;", O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag basis)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 20%, O₂ 9% – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 17%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="70" t="inlineStr">
         <is>
@@ -19659,7 +19715,7 @@
       </c>
       <c r="D76" s="150">
         <f>'Mass Transfer'!$D$100</f>
-        <v>0.0003583371353617</v>
+        <v>0.0004480356964998</v>
       </c>
       <c r="E76" s="135" t="inlineStr">
         <is>
@@ -19838,7 +19894,7 @@
       </c>
       <c r="D83" s="48">
         <f>rH2_gen+O2_net_gen</f>
-        <v>0.0001497668022734</v>
+        <v>0.0001515178050535</v>
       </c>
       <c r="E83" s="69" t="inlineStr">
         <is>
@@ -19864,7 +19920,7 @@
       </c>
       <c r="D84" s="48">
         <f>rH2_gen/(n_flamm_src+CO2_supply_b)</f>
-        <v>0.200209961657</v>
+        <v>0.169672046961</v>
       </c>
       <c r="E84" s="69" t="inlineStr">
         <is>
@@ -19890,7 +19946,7 @@
       </c>
       <c r="D85" s="48">
         <f>O2_net_gen/(n_flamm_src+CO2_supply_b)</f>
-        <v>0.094546270642</v>
+        <v>0.083045691591</v>
       </c>
       <c r="E85" s="69" t="inlineStr">
         <is>
@@ -19916,7 +19972,7 @@
       </c>
       <c r="D86" s="48">
         <f>MAX(0,MIN(rH2_gen/H2_LFL-n_flamm_src,O2_net_gen/(O2_LOC_H2*LOC_margin)-n_flamm_src))/CO2_rate_full_b</f>
-        <v>0.002836654967</v>
+        <v>0.002947616391</v>
       </c>
       <c r="E86" s="69" t="inlineStr">
         <is>
@@ -19942,7 +19998,7 @@
       </c>
       <c r="D87" s="48">
         <f>IF(duty_H2safe&gt;0,spg_dur_b/(60*duty_H2safe),NA())</f>
-        <v>4.609378881561</v>
+        <v>4.43586130694</v>
       </c>
       <c r="E87" s="69" t="inlineStr">
         <is>
@@ -19968,7 +20024,7 @@
       </c>
       <c r="D88" s="48">
         <f>MAX(0,rH2_gen/H2_LFL-n_flamm_src)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
-        <v>0.975933085966</v>
+        <v>0.975219102801</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
@@ -20027,7 +20083,7 @@
       </c>
       <c r="D97" s="48">
         <f>'Mass Transfer'!$D$198</f>
-        <v>5.891603808766</v>
+        <v>7.42516851712</v>
       </c>
       <c r="E97" s="67" t="inlineStr">
         <is>
@@ -20053,7 +20109,7 @@
       </c>
       <c r="D98" s="48">
         <f>C_cycle_start_b*1000/Km_CO2</f>
-        <v>117.832076175326</v>
+        <v>148.503370342395</v>
       </c>
       <c r="E98" s="69" t="inlineStr">
         <is>
@@ -20283,7 +20339,7 @@
       </c>
       <c r="D11" s="142">
         <f>Biology!$D$16</f>
-        <v>1.413017577815e-05</v>
+        <v>1.58811785582e-05</v>
       </c>
       <c r="E11" s="135" t="str">
         <f>HYPERLINK("#Biology!D16","→ Biology")</f>
@@ -20323,7 +20379,7 @@
       </c>
       <c r="D13" s="150">
         <f>Electrochemistry!$D$29</f>
-        <v>4.803933240197e-05</v>
+        <v>4.979033518202e-05</v>
       </c>
       <c r="E13" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -21068,7 +21124,7 @@
       </c>
       <c r="D53" s="64">
         <f>kLa_sparge*duty</f>
-        <v>1.1303903703e-05</v>
+        <v>1.413348455674e-05</v>
       </c>
       <c r="E53" s="117" t="s">
         <v>643</v>
@@ -21106,7 +21162,7 @@
       </c>
       <c r="D55" s="48">
         <f>strip_sparge*duty</f>
-        <v>2.226595475021e-07</v>
+        <v>2.783954427351e-07</v>
       </c>
       <c r="E55" s="75" t="s">
         <v>649</v>
@@ -21125,7 +21181,7 @@
       </c>
       <c r="D56" s="45">
         <f>IF(O2_excess&gt;0,strip_avg/O2_excess,NA())</f>
-        <v>0.015757733732</v>
+        <v>0.017529898157</v>
       </c>
       <c r="E56" s="75" t="s">
         <v>652</v>
@@ -21144,7 +21200,7 @@
       </c>
       <c r="D57" s="48">
         <f>IF(O2_excess&gt;0,O2_excess/3600/((V_charge/1000000)*O2_ceil_C),NA())</f>
-        <v>0.0007173559278932</v>
+        <v>0.000806250237755</v>
       </c>
       <c r="E57" s="75" t="s">
         <v>655</v>
@@ -21294,7 +21350,7 @@
       </c>
       <c r="D65" s="48">
         <f>O2_ceil_C*(V_charge/1000000)/O2_excess*60</f>
-        <v>23.233468935867</v>
+        <v>20.671828529408</v>
       </c>
       <c r="E65" s="99" t="inlineStr">
         <is>
@@ -21315,7 +21371,7 @@
       </c>
       <c r="D66" s="48">
         <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,cleared_min)</f>
-        <v>23.605437128776</v>
+        <v>21.040669319734</v>
       </c>
       <c r="E66" s="99" t="s">
         <v>680</v>
@@ -21467,7 +21523,7 @@
       </c>
       <c r="D74" s="48">
         <f>IF(O2_excess&gt;0,surf_strip/O2_excess,NA())</f>
-        <v>10.037003079208</v>
+        <v>8.930358491677</v>
       </c>
       <c r="E74" s="69" t="s">
         <v>702</v>
@@ -21486,7 +21542,7 @@
       </c>
       <c r="D75" s="48">
         <f>IF(CO2_supply&gt;0,O2_excess/(O2_excess+CO2_supply),NA())</f>
-        <v>0.03793668694</v>
+        <v>0.034232810687</v>
       </c>
       <c r="E75" s="99" t="s">
         <v>705</v>
@@ -21505,7 +21561,7 @@
       </c>
       <c r="D76" s="48">
         <f>H_O2_T*y_O2_vent*P_atm*1000</f>
-        <v>46.12721765053</v>
+        <v>41.623674513885</v>
       </c>
       <c r="E76" s="69" t="inlineStr">
         <is>
@@ -21526,7 +21582,7 @@
       </c>
       <c r="D77" s="48">
         <f>headspace_V/(Q_CO2*duty)</f>
-        <v>17.879338726534</v>
+        <v>14.299822696002</v>
       </c>
       <c r="E77" s="99" t="s">
         <v>710</v>
@@ -21545,7 +21601,7 @@
       </c>
       <c r="D78" s="48">
         <f>IF(O2_excess&gt;0,(strip_avg+surf_strip)/O2_excess,NA())</f>
-        <v>10.052760812941</v>
+        <v>8.947888389834</v>
       </c>
       <c r="E78" s="118" t="s">
         <v>713</v>
@@ -21564,7 +21620,7 @@
       </c>
       <c r="D79" s="48">
         <f>O2_ceil_C*(V_charge/1000000)/O2_net_gen*60</f>
-        <v>6.833837682277</v>
+        <v>6.593508535339</v>
       </c>
       <c r="E79" s="99" t="s">
         <v>716</v>
@@ -21714,7 +21770,7 @@
       </c>
       <c r="D87" s="48">
         <f>O2_src_guard/(target_DO_frac*(O2_ceil_Pa/P_atm))/(nCO2_rate*3600)</f>
-        <v>0.001445459252</v>
+        <v>0.001498145312</v>
       </c>
       <c r="E87" s="99" t="s">
         <v>1063</v>
@@ -21733,7 +21789,7 @@
       </c>
       <c r="D88" s="48">
         <f>MAX(duty_carbon,duty_O2vent)</f>
-        <v>0.001445459252</v>
+        <v>0.001498145312</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
@@ -21754,7 +21810,7 @@
       </c>
       <c r="D89" s="48">
         <f>target_DO_frac*O2_ceil_C*(V_charge/1000000)/O2_src_guard*60</f>
-        <v>1.54504156295</v>
+        <v>1.490706277555</v>
       </c>
       <c r="E89" s="99" t="inlineStr">
         <is>
@@ -21794,7 +21850,7 @@
       </c>
       <c r="D91" s="48">
         <f>IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max))</f>
-        <v>17.879338726534</v>
+        <v>14.299822696002</v>
       </c>
       <c r="E91" s="159" t="inlineStr">
         <is>
@@ -21815,7 +21871,7 @@
       </c>
       <c r="D92" s="48">
         <f>spg_int_opt*60</f>
-        <v>1072.760323592056</v>
+        <v>857.98936176009</v>
       </c>
       <c r="E92" s="159" t="s">
         <v>747</v>
@@ -21836,7 +21892,7 @@
       </c>
       <c r="D93" s="48">
         <f>spg_dur_opt/(spg_int_opt*60)</f>
-        <v>0.000731303192868</v>
+        <v>0.0009143622109901</v>
       </c>
       <c r="E93" s="99" t="s">
         <v>750</v>
@@ -21969,7 +22025,7 @@
       </c>
       <c r="D100" s="28">
         <f>CO2_pulse*pulses_h</f>
-        <v>0.0003583371353617</v>
+        <v>0.0004480356964998</v>
       </c>
       <c r="E100" s="160" t="s">
         <v>765</v>
@@ -22062,7 +22118,7 @@
       </c>
       <c r="D105" s="28">
         <f>spg_dur/(spg_int*60)</f>
-        <v>0.000731303192868</v>
+        <v>0.0009143622109901</v>
       </c>
       <c r="E105" s="160" t="s">
         <v>765</v>
@@ -22191,7 +22247,7 @@
       <c r="C113" s="20"/>
       <c r="D113" s="28" t="str">
         <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) DO would be "&amp;TEXT(DO_at_carbon*M_O2,"0.0")&amp;" mg/L against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 12.6 mg/L against a 2.6 mg/L target</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 13.7 mg/L against a 2.6 mg/L target</v>
       </c>
       <c r="E113" s="82" t="inlineStr">
         <is>
@@ -22343,7 +22399,7 @@
       </c>
       <c r="D122" s="28">
         <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
-        <v>17.879338726534</v>
+        <v>14.299822696002</v>
       </c>
       <c r="E122" s="20"/>
       <c r="F122" s="20"/>
@@ -22377,7 +22433,7 @@
       </c>
       <c r="D124" s="28">
         <f>60/spg_int</f>
-        <v>3.355828809874</v>
+        <v>4.195856219726</v>
       </c>
       <c r="E124" s="20"/>
       <c r="F124" s="20"/>
@@ -22394,7 +22450,7 @@
       </c>
       <c r="D125" s="28">
         <f>pulses_h*24</f>
-        <v>80.539891436977</v>
+        <v>100.700549273429</v>
       </c>
       <c r="E125" s="20"/>
       <c r="F125" s="20"/>
@@ -22411,7 +22467,7 @@
       </c>
       <c r="D126" s="28">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v>21.135125201548</v>
+        <v>26.425646704826</v>
       </c>
       <c r="E126" s="20"/>
       <c r="F126" s="20"/>
@@ -22428,7 +22484,7 @@
       </c>
       <c r="D127" s="28">
         <f>O2_excess/60*spg_int</f>
-        <v>4.21063665005e-06</v>
+        <v>3.784967293096e-06</v>
       </c>
       <c r="E127" s="20"/>
       <c r="F127" s="20"/>
@@ -22462,7 +22518,7 @@
       </c>
       <c r="D129" s="28">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v>0.015757733732</v>
+        <v>0.017529898157</v>
       </c>
       <c r="E129" s="20"/>
       <c r="F129" s="20"/>
@@ -22496,7 +22552,7 @@
       </c>
       <c r="D131" s="28">
         <f>kLa_surf_req/a_surf</f>
-        <v>0.0001107998109846</v>
+        <v>0.0001245300561075</v>
       </c>
       <c r="E131" s="147" t="s">
         <v>1825</v>
@@ -22515,7 +22571,7 @@
       </c>
       <c r="D132" s="28">
         <f>O2_net_gen</f>
-        <v>4.803933240197e-05</v>
+        <v>4.979033518202e-05</v>
       </c>
       <c r="E132" s="69" t="s">
         <v>992</v>
@@ -22553,7 +22609,7 @@
       </c>
       <c r="D134" s="28" t="str">
         <f>IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf"))</f>
-        <v>ESTIMATED kLa — DO-limited interval is 17.9 min; confirm by measuring kL_surf</v>
+        <v>ESTIMATED kLa — DO-limited interval is 14.3 min; confirm by measuring kL_surf</v>
       </c>
       <c r="E134" s="69" t="inlineStr">
         <is>
@@ -22871,7 +22927,7 @@
       </c>
       <c r="D152" s="48">
         <f>MAX(0,spg_int*60-spg_dur)</f>
-        <v>1071.975810542231</v>
+        <v>857.204848710266</v>
       </c>
       <c r="E152" s="67" t="s">
         <v>1190</v>
@@ -22962,7 +23018,7 @@
       </c>
       <c r="D162" s="48">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,CO2_cyc_avg_new))/1000</f>
-        <v>0.008068720944</v>
+        <v>0.00952617025</v>
       </c>
       <c r="E162" s="67" t="s">
         <v>1859</v>
@@ -23226,7 +23282,7 @@
       </c>
       <c r="D180" s="141">
         <f>O2_excess/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.03634252148</v>
+        <v>0.040846064617</v>
       </c>
       <c r="E180" s="67" t="s">
         <v>1798</v>
@@ -23244,7 +23300,7 @@
       </c>
       <c r="D181" s="141">
         <f>O2_net_gen/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.123556174892</v>
+        <v>0.128059718029</v>
       </c>
       <c r="E181" s="67" t="s">
         <v>1801</v>
@@ -23262,7 +23318,7 @@
       </c>
       <c r="D182" s="141">
         <f>DO_target-DO_surf_excess</f>
-        <v>0.046127217651</v>
+        <v>0.041623674514</v>
       </c>
       <c r="E182" s="67" t="s">
         <v>1804</v>
@@ -23280,7 +23336,7 @@
       </c>
       <c r="D183" s="141">
         <f>IF(hs_O2_allow&gt;0,hs_O2_allow/(H_O2_T*P_atm),NA())</f>
-        <v>0.03793668694</v>
+        <v>0.034232810687</v>
       </c>
       <c r="E183" s="67" t="s">
         <v>1807</v>
@@ -23298,7 +23354,7 @@
       </c>
       <c r="D184" s="141">
         <f>IF(ISNUMBER(y_O2_star),O2_excess*(1-y_O2_star)/(y_O2_star*CO2_rate_full),NA())</f>
-        <v>0.000731303192868</v>
+        <v>0.0009143622109901</v>
       </c>
       <c r="E184" s="67" t="inlineStr">
         <is>
@@ -23318,7 +23374,7 @@
       </c>
       <c r="D185" s="141">
         <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_opt/(60*duty_DO),spg_int_carbon),NA())</f>
-        <v>17.879338726534</v>
+        <v>14.299822696002</v>
       </c>
       <c r="E185" s="67" t="s">
         <v>1813</v>
@@ -23336,7 +23392,7 @@
       </c>
       <c r="D186" s="141">
         <f>O2_excess/(DO_target*3600*(V_charge/1000000))</f>
-        <v>0.00317292045</v>
+        <v>0.003566106821</v>
       </c>
       <c r="E186" s="67" t="s">
         <v>1816</v>
@@ -23354,7 +23410,7 @@
       </c>
       <c r="D187" s="141">
         <f>IF(CO2_supply&gt;0,O2_excess/(O2_excess+CO2_supply),NA())</f>
-        <v>0.03793668694</v>
+        <v>0.034232810687</v>
       </c>
       <c r="E187" s="67" t="s">
         <v>1819</v>
@@ -23372,7 +23428,7 @@
       </c>
       <c r="D188" s="141">
         <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_atm,NA())</f>
-        <v>0.046127217651</v>
+        <v>0.041623674514</v>
       </c>
       <c r="E188" s="67" t="s">
         <v>1822</v>
@@ -23507,7 +23563,7 @@
       </c>
       <c r="D197" s="141">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
-        <v>0.548694671753</v>
+        <v>0.618808080904</v>
       </c>
       <c r="E197" s="99" t="s">
         <v>1849</v>
@@ -23525,7 +23581,7 @@
       </c>
       <c r="D198" s="141">
         <f>(C_air_CO2*(1-pool_e)+pool_b*pool_e)/(1-pool_a*pool_e)</f>
-        <v>5.891603808766</v>
+        <v>7.42516851712</v>
       </c>
       <c r="E198" s="99" t="s">
         <v>1852</v>
@@ -23543,7 +23599,7 @@
       </c>
       <c r="D199" s="141">
         <f>pool_a*C_cycle_start+pool_b</f>
-        <v>10.726633374496</v>
+        <v>11.991014682526</v>
       </c>
       <c r="E199" s="99" t="s">
         <v>1855</v>
@@ -23561,7 +23617,7 @@
       </c>
       <c r="D200" s="141">
         <f>C_air_CO2+(C_cycle_peak-C_air_CO2)*(1-pool_e)/(k_eff_CO2*t_off_CO2)</f>
-        <v>8.068720944288</v>
+        <v>9.526170249632</v>
       </c>
       <c r="E200" s="99" t="s">
         <v>1858</v>
@@ -23877,7 +23933,7 @@
       </c>
       <c r="D232" s="141">
         <f>H_O2_T*P_atm*O2_excess/(O2_excess+CO2_rate_full*duty_carbon)+DO_surf_excess</f>
-        <v>0.393984475887</v>
+        <v>0.428670828967</v>
       </c>
       <c r="E232" s="99" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Gas model: one headspace balance for O2, CO2 pool and flammability; vent and sizing-phase selectors; both-phase DO; sawtooth peak
Default (outflow only, growth): 0.78 s every 12.7 min, pH 6.16 (below band) - CO2 cannot both
dilute O2 and hold pH. Excel-verified in all four selector combinations; twin 289/289.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -688,6 +688,91 @@
     <definedName name="spg_dur_run" localSheetId="5">'Mass Transfer'!$D$242</definedName>
     <definedName name="D_Cl" localSheetId="3">Chemistry!$D$277</definedName>
     <definedName name="Cl_free_frac" localSheetId="3">Chemistry!$D$278</definedName>
+    <definedName name="vent_model" localSheetId="5">'Mass Transfer'!$D$301</definedName>
+    <definedName name="vent_name_1" localSheetId="5">'Mass Transfer'!$D$302</definedName>
+    <definedName name="vent_name_2" localSheetId="5">'Mass Transfer'!$D$303</definedName>
+    <definedName name="O2_sizing_phase" localSheetId="5">'Mass Transfer'!$D$304</definedName>
+    <definedName name="phase_name_1" localSheetId="5">'Mass Transfer'!$D$305</definedName>
+    <definedName name="phase_name_2" localSheetId="5">'Mass Transfer'!$D$306</definedName>
+    <definedName name="y_O2_air" localSheetId="5">'Mass Transfer'!$D$307</definedName>
+    <definedName name="F_vent_ex" localSheetId="5">'Mass Transfer'!$D$308</definedName>
+    <definedName name="O2_src_g" localSheetId="5">'Mass Transfer'!$D$309</definedName>
+    <definedName name="O2_src_l" localSheetId="5">'Mass Transfer'!$D$310</definedName>
+    <definedName name="rH2_gen" localSheetId="5">'Mass Transfer'!$D$311</definedName>
+    <definedName name="H2_cons" localSheetId="5">'Mass Transfer'!$D$312</definedName>
+    <definedName name="H2_src_g" localSheetId="5">'Mass Transfer'!$D$313</definedName>
+    <definedName name="H2_src_l" localSheetId="5">'Mass Transfer'!$D$314</definedName>
+    <definedName name="CO2_fix_g" localSheetId="5">'Mass Transfer'!$D$315</definedName>
+    <definedName name="CO2_fix_l" localSheetId="5">'Mass Transfer'!$D$316</definedName>
+    <definedName name="O2_src_sched" localSheetId="5">'Mass Transfer'!$D$317</definedName>
+    <definedName name="H2_src_sched" localSheetId="5">'Mass Transfer'!$D$318</definedName>
+    <definedName name="CO2_fix_sched" localSheetId="5">'Mass Transfer'!$D$319</definedName>
+    <definedName name="flush_vol_opt" localSheetId="5">'Mass Transfer'!$D$320</definedName>
+    <definedName name="flush_ret_opt" localSheetId="5">'Mass Transfer'!$D$321</definedName>
+    <definedName name="saw_factor" localSheetId="5">'Mass Transfer'!$D$322</definedName>
+    <definedName name="flush_vol" localSheetId="5">'Mass Transfer'!$D$323</definedName>
+    <definedName name="flush_ret" localSheetId="5">'Mass Transfer'!$D$324</definedName>
+    <definedName name="t_gap_h" localSheetId="5">'Mass Transfer'!$D$325</definedName>
+    <definedName name="tau_L_h" localSheetId="5">'Mass Transfer'!$D$326</definedName>
+    <definedName name="S_O2_g" localSheetId="5">'Mass Transfer'!$D$327</definedName>
+    <definedName name="F_hs_net_g" localSheetId="5">'Mass Transfer'!$D$328</definedName>
+    <definedName name="y_O2_mf_g" localSheetId="5">'Mass Transfer'!$D$329</definedName>
+    <definedName name="y_H2_mf_g" localSheetId="5">'Mass Transfer'!$D$330</definedName>
+    <definedName name="F_gap_g" localSheetId="5">'Mass Transfer'!$D$331</definedName>
+    <definedName name="x_hs_g" localSheetId="5">'Mass Transfer'!$D$332</definedName>
+    <definedName name="phi_hs_g" localSheetId="5">'Mass Transfer'!$D$333</definedName>
+    <definedName name="psi_hs_g" localSheetId="5">'Mass Transfer'!$D$334</definedName>
+    <definedName name="dy_O2_g" localSheetId="5">'Mass Transfer'!$D$335</definedName>
+    <definedName name="y_O2_end_g" localSheetId="5">'Mass Transfer'!$D$336</definedName>
+    <definedName name="y_O2_post_g" localSheetId="5">'Mass Transfer'!$D$337</definedName>
+    <definedName name="y_O2_avg_g" localSheetId="5">'Mass Transfer'!$D$338</definedName>
+    <definedName name="DO_surf_excess_g" localSheetId="5">'Mass Transfer'!$D$339</definedName>
+    <definedName name="DO_mf_g" localSheetId="5">'Mass Transfer'!$D$340</definedName>
+    <definedName name="DO_avg_g" localSheetId="5">'Mass Transfer'!$D$341</definedName>
+    <definedName name="DO_peak_g" localSheetId="5">'Mass Transfer'!$D$342</definedName>
+    <definedName name="DO_avg_g_mgL" localSheetId="5">'Mass Transfer'!$D$343</definedName>
+    <definedName name="DO_peak_g_mgL" localSheetId="5">'Mass Transfer'!$D$344</definedName>
+    <definedName name="kLa_surf_req_g" localSheetId="5">'Mass Transfer'!$D$345</definedName>
+    <definedName name="kLa_margin_g" localSheetId="5">'Mass Transfer'!$D$346</definedName>
+    <definedName name="DO_feas_g" localSheetId="5">'Mass Transfer'!$D$347</definedName>
+    <definedName name="DO_peak_chk_g" localSheetId="5">'Mass Transfer'!$D$348</definedName>
+    <definedName name="S_O2_l" localSheetId="5">'Mass Transfer'!$D$349</definedName>
+    <definedName name="F_hs_net_l" localSheetId="5">'Mass Transfer'!$D$350</definedName>
+    <definedName name="y_O2_mf_l" localSheetId="5">'Mass Transfer'!$D$351</definedName>
+    <definedName name="y_H2_mf_l" localSheetId="5">'Mass Transfer'!$D$352</definedName>
+    <definedName name="F_gap_l" localSheetId="5">'Mass Transfer'!$D$353</definedName>
+    <definedName name="x_hs_l" localSheetId="5">'Mass Transfer'!$D$354</definedName>
+    <definedName name="phi_hs_l" localSheetId="5">'Mass Transfer'!$D$355</definedName>
+    <definedName name="psi_hs_l" localSheetId="5">'Mass Transfer'!$D$356</definedName>
+    <definedName name="dy_O2_l" localSheetId="5">'Mass Transfer'!$D$357</definedName>
+    <definedName name="y_O2_end_l" localSheetId="5">'Mass Transfer'!$D$358</definedName>
+    <definedName name="y_O2_post_l" localSheetId="5">'Mass Transfer'!$D$359</definedName>
+    <definedName name="y_O2_avg_l" localSheetId="5">'Mass Transfer'!$D$360</definedName>
+    <definedName name="DO_mf_l" localSheetId="5">'Mass Transfer'!$D$361</definedName>
+    <definedName name="DO_avg_l" localSheetId="5">'Mass Transfer'!$D$362</definedName>
+    <definedName name="DO_peak_l" localSheetId="5">'Mass Transfer'!$D$363</definedName>
+    <definedName name="DO_avg_l_mgL" localSheetId="5">'Mass Transfer'!$D$364</definedName>
+    <definedName name="DO_peak_l_mgL" localSheetId="5">'Mass Transfer'!$D$365</definedName>
+    <definedName name="kLa_surf_req_l" localSheetId="5">'Mass Transfer'!$D$366</definedName>
+    <definedName name="kLa_margin_l" localSheetId="5">'Mass Transfer'!$D$367</definedName>
+    <definedName name="DO_feas_l" localSheetId="5">'Mass Transfer'!$D$368</definedName>
+    <definedName name="DO_peak_chk_l" localSheetId="5">'Mass Transfer'!$D$369</definedName>
+    <definedName name="F_gap_sched" localSheetId="5">'Mass Transfer'!$D$371</definedName>
+    <definedName name="DO_avg_sched" localSheetId="5">'Mass Transfer'!$D$372</definedName>
+    <definedName name="DO_peak_sched" localSheetId="5">'Mass Transfer'!$D$373</definedName>
+    <definedName name="DO_peak_band" localSheetId="5">'Mass Transfer'!$D$374</definedName>
+    <definedName name="pool_D_raw" localSheetId="5">'Mass Transfer'!$D$375</definedName>
+    <definedName name="pool_x" localSheetId="5">'Mass Transfer'!$D$376</definedName>
+    <definedName name="pool_phi" localSheetId="5">'Mass Transfer'!$D$377</definedName>
+    <definedName name="pool_psi" localSheetId="5">'Mass Transfer'!$D$378</definedName>
+    <definedName name="pool_D_gap" localSheetId="5">'Mass Transfer'!$D$379</definedName>
+    <definedName name="pool_ret" localSheetId="5">'Mass Transfer'!$D$380</definedName>
+    <definedName name="y_CO2_mf" localSheetId="5">'Mass Transfer'!$D$381</definedName>
+    <definedName name="C_CO2_mf" localSheetId="5">'Mass Transfer'!$D$382</definedName>
+    <definedName name="F_vent_ex_b" localSheetId="4">Biology!$D$111</definedName>
+    <definedName name="y_O2_air_b" localSheetId="4">Biology!$D$112</definedName>
+    <definedName name="vent_model_sel" localSheetId="0">Summary!$D$111</definedName>
+    <definedName name="O2_phase_sel" localSheetId="0">Summary!$D$112</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8298,7 +8383,7 @@
       </c>
       <c r="D15" s="90">
         <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$91)</f>
-        <v>14.299822696002</v>
+        <v>12.736715659111</v>
       </c>
       <c r="E15" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
@@ -8306,7 +8391,7 @@
       </c>
       <c r="F15" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Time between doses: the shorter of the carbon-limited interval and the headspace-O₂-dilution interval (binding constraint on Mass Transfer D94). Credits surface O₂ stripping via the kL_surf estimate; measuring kL_surf refines it.</t>
+          <t xml:space="preserve">Time between doses: the shorter of the carbon-limited interval and the headspace-O₂-dilution interval (binding constraint on Mass Transfer D94), sized on the phase in D112 under the vent model in D111. Credits surface O₂ stripping via the kL_surf estimate; measuring kL_surf refines it.</t>
         </is>
       </c>
       <c r="G15" s="36"/>
@@ -8327,7 +8412,7 @@
       </c>
       <c r="D16" s="91">
         <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,ROUND(D14/(60*'Mass Transfer'!$D$93),0)))</f>
-        <v>15.0</v>
+        <v>13.0</v>
       </c>
       <c r="E16" s="92"/>
       <c r="F16" s="21" t="inlineStr">
@@ -8407,8 +8492,10 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="89" t="s">
-        <v>74</v>
+      <c r="A21" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak O₂ within the organism band?</t>
+        </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
@@ -8417,15 +8504,17 @@
       </c>
       <c r="C21" s="20"/>
       <c r="D21" s="90" t="str">
-        <f>'Mass Transfer'!$D$109</f>
-        <v>organism optimum unknown</v>
+        <f>'Mass Transfer'!$D$374</f>
+        <v>organism band unknown – peak 3.0 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E21" s="23" t="str">
-        <f>HYPERLINK("#'Mass Transfer'!D109","→ Mass")</f>
-        <v>→ Mass</v>
-      </c>
-      <c r="F21" s="21" t="s">
-        <v>75</v>
+        <f>HYPERLINK("#'Mass Transfer'!D374","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sawtooth PEAK dissolved O₂ (just before a pulse, sizing phase) against the organism optimum / impairment, or against the inhibition ceiling when the band is unmeasured. Not a tautology: the schedule is sized on the cycle mean, not the peak.</t>
+        </is>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -8464,7 +8553,7 @@
       <c r="C23" s="20"/>
       <c r="D23" s="90" t="str">
         <f>'Mass Transfer'!$D$113</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 13.7 mg/L against a 2.6 mg/L target</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 20.1 mg/L against a 2.6 mg/L target</v>
       </c>
       <c r="E23" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
@@ -8490,7 +8579,7 @@
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 17%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 16%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="23" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -8536,7 +8625,7 @@
       <c r="C26" s="20"/>
       <c r="D26" s="90" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)"),"calibrate this reactor first")</f>
-        <v>×26.4 OK</v>
+        <v>×29.7 OK</v>
       </c>
       <c r="E26" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
@@ -8736,7 +8825,7 @@
       <c r="C35" s="20"/>
       <c r="D35" s="121">
         <f>Chemistry!$D$220</f>
-        <v>6.570596176702</v>
+        <v>6.164822774553</v>
       </c>
       <c r="E35" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -8762,7 +8851,7 @@
       </c>
       <c r="D36" s="121">
         <f>Chemistry!$D$226</f>
-        <v>0.338593949713</v>
+        <v>0.339344361561</v>
       </c>
       <c r="E36" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
@@ -8785,8 +8874,10 @@
       <c r="F37" s="21"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A38" s="89" t="s">
-        <v>101</v>
+      <c r="A38" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO (sawtooth, sizing phase)</t>
+        </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
@@ -8798,14 +8889,16 @@
       </c>
       <c r="D38" s="90">
         <f>'Mass Transfer'!$D$108</f>
-        <v>2.638866712696</v>
+        <v>2.634660261764</v>
       </c>
       <c r="E38" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D108","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F38" s="21" t="s">
-        <v>103</v>
+      <c r="F38" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean dissolved O₂ of the sawtooth model at the schedule in use, on the sizing phase; near the target by construction when O₂ dilution binds. Both phases, mean and peak: rows 114–117.</t>
+        </is>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
@@ -8876,7 +8969,7 @@
       </c>
       <c r="D41" s="95">
         <f>Biology!$D$98</f>
-        <v>148.503370342395</v>
+        <v>633.123209647745</v>
       </c>
       <c r="E41" s="23" t="str">
         <f>HYPERLINK("#Biology!D98","→ Biology")</f>
@@ -9596,7 +9689,7 @@
       </c>
       <c r="D85" s="22" t="str">
         <f>Electrochemistry!$D$99</f>
-        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 7 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
       </c>
       <c r="E85" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D99","→ Electrochemistry")</f>
@@ -9646,7 +9739,7 @@
       </c>
       <c r="D87" s="22">
         <f>Chemistry!$D$209</f>
-        <v>-0.42751475509</v>
+        <v>-0.427527364769</v>
       </c>
       <c r="E87" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D209","→ Chemistry")</f>
@@ -9672,7 +9765,7 @@
       </c>
       <c r="D88" s="22">
         <f>Chemistry!$D$211</f>
-        <v>1.242530226635</v>
+        <v>1.266535517225</v>
       </c>
       <c r="E88" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
@@ -9698,7 +9791,7 @@
       </c>
       <c r="D89" s="22">
         <f>Chemistry!$D$220</f>
-        <v>6.570596176702</v>
+        <v>6.164822774553</v>
       </c>
       <c r="E89" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -9728,8 +9821,10 @@
         <f>HYPERLINK("#'Mass Transfer'!D186","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F90" t="s">
-        <v>1876</v>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Below this, no sparge interval holds the target dissolved O₂ on the sizing phase. Both phases and their margins: rows 120–123.</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -9777,7 +9872,7 @@
       </c>
       <c r="D95" s="95">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),D14/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (see CO2 flows)")</f>
-        <v>0.972140884876</v>
+        <v>0.999088398707</v>
       </c>
       <c r="E95" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
@@ -9786,6 +9881,452 @@
       <c r="F95" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">Duty of the schedule as typed in (rows 14 and 16) against the optimised duty; 1 = rounding has not moved the CO₂ dose, pH or DO. Should sit within a few per cent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEADSPACE MODEL — owner decisions (dropdowns) and both-phase dissolved O₂</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vent model</t>
+        </is>
+      </c>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vent_model_sel</t>
+        </is>
+      </c>
+      <c r="C111" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D111" s="131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outflow only</t>
+        </is>
+      </c>
+      <c r="E111" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="F111" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Outflow only" = gas leaves through the vent, none enters between pulses (check valve / sealed cap). "Air exchange" = room air exchanges with the headspace at Q_vent (Mass Transfer D142, unmeasured). Anything else → #N/A throughout. Default pending the vent-hardware answer; it moves the pH and the lag DO materially.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ sizing phase</t>
+        </is>
+      </c>
+      <c r="B112" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_phase_sel</t>
+        </is>
+      </c>
+      <c r="C112" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D112" s="131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Growth</t>
+        </is>
+      </c>
+      <c r="E112" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">select</t>
+        </is>
+      </c>
+      <c r="F112" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Growth" sizes the sparge interval on the O₂ surplus after knallgas uptake; "Lag" on the whole net electrolytic O₂ plus H₂ (no uptake yet). Anything else → #N/A. Both phases are reported below whichever is chosen; "Lag" is currently unreachable at the estimated surface kLa, so the schedule falls back to the O₂ flush interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vent air-exchange flow in use</t>
+        </is>
+      </c>
+      <c r="C113" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D113" s="90">
+        <f>'Mass Transfer'!$D$308</f>
+        <v>0.0</v>
+      </c>
+      <c r="E113" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D308","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F113" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zero for "Outflow only"; Q_vent converted for "Air exchange". The single number that reconciles the O₂, CO₂ and flammability blocks — measure it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — growth phase</t>
+        </is>
+      </c>
+      <c r="C114" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D114" s="90">
+        <f>'Mass Transfer'!$D$343</f>
+        <v>2.634660261764</v>
+      </c>
+      <c r="E114" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D343","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F114" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean dissolved O₂ at the schedule in use with the growth-phase O₂ surplus (sawtooth model).</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — growth phase</t>
+        </is>
+      </c>
+      <c r="C115" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D115" s="90">
+        <f>'Mass Transfer'!$D$344</f>
+        <v>3.024959328002</v>
+      </c>
+      <c r="E115" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D344","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F115" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dissolved O₂ just before a pulse, growth phase. Compare with the organism band and the ceiling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — lag phase</t>
+        </is>
+      </c>
+      <c r="C116" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D116" s="90">
+        <f>'Mass Transfer'!$D$364</f>
+        <v>7.292294135948</v>
+      </c>
+      <c r="E116" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F116" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same schedule, no uptake yet: the whole net electrolytic O₂ crosses the surface. Expect this from inoculation until growth is established, and in every abiotic run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — lag phase</t>
+        </is>
+      </c>
+      <c r="C117" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D117" s="90">
+        <f>'Mass Transfer'!$D$365</f>
+        <v>8.21297180544</v>
+      </c>
+      <c r="E117" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D365","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F117" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag-phase sawtooth peak; the discriminating prediction for an abiotic DO trace (R2 experiment 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO under the inhibition ceiling? — growth</t>
+        </is>
+      </c>
+      <c r="D118" s="90" t="str">
+        <f>'Mass Transfer'!$D$348</f>
+        <v>peak 3.0 mg/L under the 11.7 mg/L ceiling</v>
+      </c>
+      <c r="E118" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D348","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F118" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Red = the growth-phase sawtooth peaks above the 0.30 atm growth-inhibition ceiling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO under the inhibition ceiling? — lag</t>
+        </is>
+      </c>
+      <c r="D119" s="90" t="str">
+        <f>'Mass Transfer'!$D$369</f>
+        <v>peak 8.2 mg/L under the 11.7 mg/L ceiling</v>
+      </c>
+      <c r="E119" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D369","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F119" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Red = the lag-phase peak breaches the ceiling at this schedule; the culture would then be inhibited before it starts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO target reachable? — growth</t>
+        </is>
+      </c>
+      <c r="D120" s="90" t="str">
+        <f>'Mass Transfer'!$D$347</f>
+        <v>reachable – kLa margin 2.02×</v>
+      </c>
+      <c r="E120" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D347","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F120" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface kLa in use ÷ kLa required on the growth source. Below 1× no interval holds the target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO target reachable? — lag</t>
+        </is>
+      </c>
+      <c r="D121" s="90" t="str">
+        <f>'Mass Transfer'!$D$368</f>
+        <v>UNREACHABLE at this surface kLa – margin 0.64× (raise kL_surf, lower the current, or accept a higher DO)</v>
+      </c>
+      <c r="E121" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D368","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F121" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same on the lag source (3.3× larger). Currently 0.65×: the target cannot be held during lag at the estimated kLa, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface kLa required — growth</t>
+        </is>
+      </c>
+      <c r="C122" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/s</t>
+        </is>
+      </c>
+      <c r="D122" s="90">
+        <f>'Mass Transfer'!$D$345</f>
+        <v>0.003566106821</v>
+      </c>
+      <c r="E122" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D345","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F122" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compare with the estimate in use (Mass Transfer D98).</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface kLa required — lag</t>
+        </is>
+      </c>
+      <c r="C123" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/s</t>
+        </is>
+      </c>
+      <c r="D123" s="90">
+        <f>'Mass Transfer'!$D$366</f>
+        <v>0.011180382694</v>
+      </c>
+      <c r="E123" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D366","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F123" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compare with the estimate in use (Mass Transfer D98).</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ fraction (mean-field) — growth</t>
+        </is>
+      </c>
+      <c r="C124" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D124" s="90">
+        <f>'Mass Transfer'!$D$329</f>
+        <v>0.031639138319</v>
+      </c>
+      <c r="E124" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D329","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F124" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flux-mean O₂ in the vent gas at the schedule in use, growth phase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ fraction (mean-field) — lag</t>
+        </is>
+      </c>
+      <c r="C125" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D125" s="90">
+        <f>'Mass Transfer'!$D$351</f>
+        <v>0.076069380811</v>
+      </c>
+      <c r="E125" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D351","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F125" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag phase; with the H₂ fraction below it, the flammability basis of row 24.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace H₂ fraction (mean-field) — lag</t>
+        </is>
+      </c>
+      <c r="C126" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D126" s="90">
+        <f>'Mass Transfer'!$D$352</f>
+        <v>0.155418629263</v>
+      </c>
+      <c r="E126" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D352","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F126" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag-phase H₂ in the headspace (LFL 4 %). Growth is zero only by the 100 % uptake assumption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace CO₂ fraction (mean-field, sizing phase)</t>
+        </is>
+      </c>
+      <c r="C127" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D127" s="90">
+        <f>'Mass Transfer'!$D$381</f>
+        <v>0.968360861681</v>
+      </c>
+      <c r="E127" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D381","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F127" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What the vent model implies for the CO₂ the pH rests on: ~96 % for "Outflow only", lower with air exchange. The pool model (Mass Transfer D200) should agree within the sawtooth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO target and pH band met together at the schedule in use?</t>
+        </is>
+      </c>
+      <c r="D128" s="90" t="str">
+        <f>IF(NOT(ISNUMBER('Mass Transfer'!$D$185)),"DO target unreachable on the sizing phase (rows 120–121) – the schedule is the O₂ flush fallback",IF(Chemistry!$D$220&gt;=Chemistry!$D$236,"yes – the schedule holds the DO target at pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", within the band","NO – holding the DO target drives pH to "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor"))</f>
+        <v>NO – holding the DO target drives pH to 6.16, below the 6.5 band floor</v>
+      </c>
+      <c r="E128" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F128" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The vent model couples the two: CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH. Red means the two targets conflict under the vent model in use — decouple them (inert sweep) or measure the vent before trusting either.</t>
         </is>
       </c>
     </row>
@@ -9882,7 +10423,7 @@
       <formula>ISNUMBER(SEARCH("OK",D49))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="9">
+  <dataValidations count="11">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a listed reactor" error="Pick a reactor from the list (Geometry A59:A80)." sqref="D2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>ReactorList</formula1>
     </dataValidation>
@@ -9913,6 +10454,12 @@
     <dataValidation operator="between" type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Ambient pressure in Pa (80000–110000), or leave blank for 101325 Pa." sqref="D10">
       <formula1>80000</formula1>
       <formula2>110000</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose Outflow only or Air exchange." sqref="D111">
+      <formula1>"Outflow only,Air exchange"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose Growth or Lag." sqref="D112">
+      <formula1>"Growth,Lag"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13508,7 +14055,7 @@
       </c>
       <c r="D96" s="141">
         <f>r_H2O2_lag/(k_H2O2_anode*3600)*(1-EXP(-k_H2O2_anode*3600))</f>
-        <v>0.740452814989</v>
+        <v>0.962431861224</v>
       </c>
       <c r="E96" s="67" t="inlineStr">
         <is>
@@ -13545,7 +14092,7 @@
       </c>
       <c r="D98" s="141">
         <f>IF(r_H2O2_lag&gt;0,IF(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag&gt;0,-LN(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag)/k_H2O2_anode/60,NA()),NA())</f>
-        <v>6.785954745632</v>
+        <v>5.084081971057</v>
       </c>
       <c r="E98" s="67" t="inlineStr">
         <is>
@@ -13565,7 +14112,7 @@
       </c>
       <c r="D99" s="141" t="str">
         <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(H2O2_lag_1h&gt;H2O2_thresh,"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases"))</f>
-        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 7 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
       </c>
       <c r="E99" s="67" t="s">
         <v>1685</v>
@@ -14298,7 +14845,7 @@
       </c>
       <c r="D150" s="141">
         <f>'Mass Transfer'!$D$135</f>
-        <v>0.169683392542</v>
+        <v>0.220552478156</v>
       </c>
       <c r="E150" s="67" t="inlineStr">
         <is>
@@ -14350,7 +14897,7 @@
       </c>
       <c r="D152" s="141">
         <f>r_H2O2*ec_DO_lag/ec_DO_design</f>
-        <v>1.673377324158</v>
+        <v>2.175036167083</v>
       </c>
       <c r="E152" s="67" t="inlineStr">
         <is>
@@ -14467,7 +15014,7 @@
       </c>
       <c r="D5" s="64">
         <f>'Mass Transfer'!$D$162</f>
-        <v>0.00952617025</v>
+        <v>0.031754970696</v>
       </c>
       <c r="E5" s="51" t="inlineStr">
         <is>
@@ -15147,7 +15694,7 @@
       </c>
       <c r="B50" s="64">
         <f t="shared" ref="B50:B81" si="1">pH_SID + pH_NT*(10^-A50)/((10^-A50)+KaN_c) + (10^-A50) - (pH_PT*Ka1p_c*(10^-A50)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A50) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A50)^3 + Ka1p_c*(10^-A50)^2 + Ka1p_c*Ka2p_c*(10^-A50) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A50) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A50)^2 - Kw_c/(10^-A50)</f>
-        <v>0.033207024661</v>
+        <v>0.0330431142</v>
       </c>
       <c r="C50" s="64">
         <f>IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
@@ -15160,7 +15707,7 @@
       </c>
       <c r="B51" s="64">
         <f t="shared" si="1"/>
-        <v>0.033087302614</v>
+        <v>0.032880951431</v>
       </c>
       <c r="C51" s="64">
         <f>IF(AND(B51&gt;=0,B52&lt;0),A51+pH_step*B51/(B51-B52),0)</f>
@@ -15173,7 +15720,7 @@
       </c>
       <c r="B52" s="64">
         <f t="shared" si="1"/>
-        <v>0.032975861045</v>
+        <v>0.032716080079</v>
       </c>
       <c r="C52" s="64">
         <f>IF(AND(B52&gt;=0,B53&lt;0),A52+pH_step*B52/(B52-B53),0)</f>
@@ -15186,7 +15733,7 @@
       </c>
       <c r="B53" s="64">
         <f t="shared" si="1"/>
-        <v>0.032866881589</v>
+        <v>0.032539836383</v>
       </c>
       <c r="C53" s="64">
         <f>IF(AND(B53&gt;=0,B54&lt;0),A53+pH_step*B53/(B53-B54),0)</f>
@@ -15199,7 +15746,7 @@
       </c>
       <c r="B54" s="64">
         <f t="shared" si="1"/>
-        <v>0.03275465025</v>
+        <v>0.032342924182</v>
       </c>
       <c r="C54" s="64">
         <f>IF(AND(B54&gt;=0,B55&lt;0),A54+pH_step*B54/(B54-B55),0)</f>
@@ -15212,7 +15759,7 @@
       </c>
       <c r="B55" s="64">
         <f t="shared" si="1"/>
-        <v>0.032633272003</v>
+        <v>0.032114938725</v>
       </c>
       <c r="C55" s="64">
         <f>IF(AND(B55&gt;=0,B56&lt;0),A55+pH_step*B55/(B55-B56),0)</f>
@@ -15225,7 +15772,7 @@
       </c>
       <c r="B56" s="64">
         <f t="shared" si="1"/>
-        <v>0.032496374136</v>
+        <v>0.031843829825</v>
       </c>
       <c r="C56" s="64">
         <f>IF(AND(B56&gt;=0,B57&lt;0),A56+pH_step*B56/(B56-B57),0)</f>
@@ -15238,7 +15785,7 @@
       </c>
       <c r="B57" s="64">
         <f t="shared" si="1"/>
-        <v>0.032336786093</v>
+        <v>0.031515279296</v>
       </c>
       <c r="C57" s="64">
         <f>IF(AND(B57&gt;=0,B58&lt;0),A57+pH_step*B57/(B57-B58),0)</f>
@@ -15251,7 +15798,7 @@
       </c>
       <c r="B58" s="64">
         <f t="shared" si="1"/>
-        <v>0.032146182686</v>
+        <v>0.031111963448</v>
       </c>
       <c r="C58" s="64">
         <f>IF(AND(B58&gt;=0,B59&lt;0),A58+pH_step*B58/(B58-B59),0)</f>
@@ -15264,7 +15811,7 @@
       </c>
       <c r="B59" s="64">
         <f t="shared" si="1"/>
-        <v>0.031914676733</v>
+        <v>0.030612666373</v>
       </c>
       <c r="C59" s="64">
         <f>IF(AND(B59&gt;=0,B60&lt;0),A59+pH_step*B59/(B59-B60),0)</f>
@@ -15277,7 +15824,7 @@
       </c>
       <c r="B60" s="64">
         <f t="shared" si="1"/>
-        <v>0.031630346466</v>
+        <v>0.029991203856</v>
       </c>
       <c r="C60" s="64">
         <f>IF(AND(B60&gt;=0,B61&lt;0),A60+pH_step*B60/(B60-B61),0)</f>
@@ -15290,7 +15837,7 @@
       </c>
       <c r="B61" s="64">
         <f t="shared" si="1"/>
-        <v>0.031278682881</v>
+        <v>0.029215110835</v>
       </c>
       <c r="C61" s="64">
         <f>IF(AND(B61&gt;=0,B62&lt;0),A61+pH_step*B61/(B61-B62),0)</f>
@@ -15303,7 +15850,7 @@
       </c>
       <c r="B62" s="64">
         <f t="shared" si="1"/>
-        <v>0.030841942713</v>
+        <v>0.028244037616</v>
       </c>
       <c r="C62" s="64">
         <f>IF(AND(B62&gt;=0,B63&lt;0),A62+pH_step*B62/(B62-B63),0)</f>
@@ -15316,7 +15863,7 @@
       </c>
       <c r="B63" s="64">
         <f t="shared" si="1"/>
-        <v>0.030298394749</v>
+        <v>0.027027791439</v>
       </c>
       <c r="C63" s="64">
         <f>IF(AND(B63&gt;=0,B64&lt;0),A63+pH_step*B63/(B63-B64),0)</f>
@@ -15329,7 +15876,7 @@
       </c>
       <c r="B64" s="64">
         <f t="shared" si="1"/>
-        <v>0.029621451096</v>
+        <v>0.025503950695</v>
       </c>
       <c r="C64" s="64">
         <f>IF(AND(B64&gt;=0,B65&lt;0),A64+pH_step*B64/(B64-B65),0)</f>
@@ -15342,7 +15889,7 @@
       </c>
       <c r="B65" s="64">
         <f t="shared" si="1"/>
-        <v>0.028778681611</v>
+        <v>0.023594968898</v>
       </c>
       <c r="C65" s="64">
         <f>IF(AND(B65&gt;=0,B66&lt;0),A65+pH_step*B65/(B65-B66),0)</f>
@@ -15355,7 +15902,7 @@
       </c>
       <c r="B66" s="64">
         <f t="shared" si="1"/>
-        <v>0.02773071881</v>
+        <v>0.021204673541</v>
       </c>
       <c r="C66" s="64">
         <f>IF(AND(B66&gt;=0,B67&lt;0),A66+pH_step*B66/(B66-B67),0)</f>
@@ -15368,7 +15915,7 @@
       </c>
       <c r="B67" s="64">
         <f t="shared" si="1"/>
-        <v>0.026430071236</v>
+        <v>0.018214048916</v>
       </c>
       <c r="C67" s="64">
         <f>IF(AND(B67&gt;=0,B68&lt;0),A67+pH_step*B67/(B67-B68),0)</f>
@@ -15381,7 +15928,7 @@
       </c>
       <c r="B68" s="64">
         <f t="shared" si="1"/>
-        <v>0.024819871701</v>
+        <v>0.014476166764</v>
       </c>
       <c r="C68" s="64">
         <f>IF(AND(B68&gt;=0,B69&lt;0),A68+pH_step*B68/(B68-B69),0)</f>
@@ -15394,7 +15941,7 @@
       </c>
       <c r="B69" s="64">
         <f t="shared" si="1"/>
-        <v>0.022832585328</v>
+        <v>0.009810084505</v>
       </c>
       <c r="C69" s="64">
         <f>IF(AND(B69&gt;=0,B70&lt;0),A69+pH_step*B69/(B69-B70),0)</f>
@@ -15407,11 +15954,11 @@
       </c>
       <c r="B70" s="64">
         <f t="shared" si="1"/>
-        <v>0.020388677363</v>
+        <v>0.003993451907</v>
       </c>
       <c r="C70" s="64">
         <f>IF(AND(B70&gt;=0,B71&lt;0),A70+pH_step*B70/(B70-B71),0)</f>
-        <v>0.0</v>
+        <v>6.055158016113</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -15420,7 +15967,7 @@
       </c>
       <c r="B71" s="64">
         <f t="shared" si="1"/>
-        <v>0.017395173018</v>
+        <v>-0.003246569015</v>
       </c>
       <c r="C71" s="64">
         <f>IF(AND(B71&gt;=0,B72&lt;0),A71+pH_step*B71/(B71-B72),0)</f>
@@ -15433,7 +15980,7 @@
       </c>
       <c r="B72" s="64">
         <f t="shared" si="1"/>
-        <v>0.013743909634</v>
+        <v>-0.012244684888</v>
       </c>
       <c r="C72" s="64">
         <f>IF(AND(B72&gt;=0,B73&lt;0),A72+pH_step*B72/(B72-B73),0)</f>
@@ -15446,7 +15993,7 @@
       </c>
       <c r="B73" s="64">
         <f t="shared" si="1"/>
-        <v>0.009309071874</v>
+        <v>-0.02341208673</v>
       </c>
       <c r="C73" s="64">
         <f>IF(AND(B73&gt;=0,B74&lt;0),A73+pH_step*B73/(B73-B74),0)</f>
@@ -15459,11 +16006,11 @@
       </c>
       <c r="B74" s="64">
         <f t="shared" si="1"/>
-        <v>0.003943325701</v>
+        <v>-0.037255650623</v>
       </c>
       <c r="C74" s="64">
         <f>IF(AND(B74&gt;=0,B75&lt;0),A74+pH_step*B74/(B74-B75),0)</f>
-        <v>6.460931418262</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.2">
@@ -15472,7 +16019,7 @@
       </c>
       <c r="B75" s="64">
         <f t="shared" si="1"/>
-        <v>-0.002528418784</v>
+        <v>-0.054403539464</v>
       </c>
       <c r="C75" s="64">
         <f>IF(AND(B75&gt;=0,B76&lt;0),A75+pH_step*B75/(B75-B76),0)</f>
@@ -15485,7 +16032,7 @@
       </c>
       <c r="B76" s="64">
         <f t="shared" si="1"/>
-        <v>-0.010318783037</v>
+        <v>-0.07563945145</v>
       </c>
       <c r="C76" s="64">
         <f>IF(AND(B76&gt;=0,B77&lt;0),A76+pH_step*B76/(B76-B77),0)</f>
@@ -15498,7 +16045,7 @@
       </c>
       <c r="B77" s="64">
         <f t="shared" si="1"/>
-        <v>-0.019692404515</v>
+        <v>-0.101948063215</v>
       </c>
       <c r="C77" s="64">
         <f>IF(AND(B77&gt;=0,B78&lt;0),A77+pH_step*B77/(B77-B78),0)</f>
@@ -15511,7 +16058,7 @@
       </c>
       <c r="B78" s="64">
         <f t="shared" si="1"/>
-        <v>-0.03098606724</v>
+        <v>-0.134574371683</v>
       </c>
       <c r="C78" s="64">
         <f>IF(AND(B78&gt;=0,B79&lt;0),A78+pH_step*B78/(B78-B79),0)</f>
@@ -15524,7 +16071,7 @@
       </c>
       <c r="B79" s="64">
         <f t="shared" si="1"/>
-        <v>-0.044635046365</v>
+        <v>-0.175099777725</v>
       </c>
       <c r="C79" s="64">
         <f>IF(AND(B79&gt;=0,B80&lt;0),A79+pH_step*B79/(B79-B80),0)</f>
@@ -15537,7 +16084,7 @@
       </c>
       <c r="B80" s="64">
         <f t="shared" si="1"/>
-        <v>-0.061205970764</v>
+        <v>-0.225538160877</v>
       </c>
       <c r="C80" s="64">
         <f>IF(AND(B80&gt;=0,B81&lt;0),A80+pH_step*B80/(B80-B81),0)</f>
@@ -15550,7 +16097,7 @@
       </c>
       <c r="B81" s="64">
         <f t="shared" si="1"/>
-        <v>-0.08143663178</v>
+        <v>-0.28845620939</v>
       </c>
       <c r="C81" s="64">
         <f>IF(AND(B81&gt;=0,B82&lt;0),A81+pH_step*B81/(B81-B82),0)</f>
@@ -15563,7 +16110,7 @@
       </c>
       <c r="B82" s="64">
         <f t="shared" ref="B82:B113" si="3">pH_SID + pH_NT*(10^-A82)/((10^-A82)+KaN_c) + (10^-A82) - (pH_PT*Ka1p_c*(10^-A82)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A82) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A82)^3 + Ka1p_c*(10^-A82)^2 + Ka1p_c*Ka2p_c*(10^-A82) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A82) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A82)^2 - Kw_c/(10^-A82)</f>
-        <v>-0.10628384514</v>
+        <v>-0.367124145321</v>
       </c>
       <c r="C82" s="64">
         <f>IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
@@ -15576,7 +16123,7 @@
       </c>
       <c r="B83" s="64">
         <f t="shared" si="3"/>
-        <v>-0.136981674648</v>
+        <v>-0.465705811375</v>
       </c>
       <c r="C83" s="64">
         <f>IF(AND(B83&gt;=0,B84&lt;0),A83+pH_step*B83/(B83-B84),0)</f>
@@ -15589,7 +16136,7 @@
       </c>
       <c r="B84" s="64">
         <f t="shared" si="3"/>
-        <v>-0.175113886331</v>
+        <v>-0.58950088085</v>
       </c>
       <c r="C84" s="64">
         <f>IF(AND(B84&gt;=0,B85&lt;0),A84+pH_step*B84/(B84-B85),0)</f>
@@ -15602,7 +16149,7 @@
       </c>
       <c r="B85" s="64">
         <f t="shared" si="3"/>
-        <v>-0.222706290329</v>
+        <v>-0.745256852669</v>
       </c>
       <c r="C85" s="64">
         <f>IF(AND(B85&gt;=0,B86&lt;0),A85+pH_step*B85/(B85-B86),0)</f>
@@ -15615,7 +16162,7 @@
       </c>
       <c r="B86" s="64">
         <f t="shared" si="3"/>
-        <v>-0.282346696413</v>
+        <v>-0.941574953283</v>
       </c>
       <c r="C86" s="64">
         <f>IF(AND(B86&gt;=0,B87&lt;0),A86+pH_step*B86/(B86-B87),0)</f>
@@ -15628,7 +16175,7 @@
       </c>
       <c r="B87" s="64">
         <f t="shared" si="3"/>
-        <v>-0.357342842397</v>
+        <v>-1.189442979033</v>
       </c>
       <c r="C87" s="64">
         <f>IF(AND(B87&gt;=0,B88&lt;0),A87+pH_step*B87/(B87-B88),0)</f>
@@ -15641,7 +16188,7 @@
       </c>
       <c r="B88" s="64">
         <f t="shared" si="3"/>
-        <v>-0.45193235682</v>
+        <v>-1.502940908092</v>
       </c>
       <c r="C88" s="64">
         <f>IF(AND(B88&gt;=0,B89&lt;0),A88+pH_step*B88/(B88-B89),0)</f>
@@ -15654,7 +16201,7 @@
       </c>
       <c r="B89" s="64">
         <f t="shared" si="3"/>
-        <v>-0.571564309028</v>
+        <v>-1.900183935458</v>
       </c>
       <c r="C89" s="64">
         <f>IF(AND(B89&gt;=0,B90&lt;0),A89+pH_step*B89/(B89-B90),0)</f>
@@ -15667,7 +16214,7 @@
       </c>
       <c r="B90" s="64">
         <f t="shared" si="3"/>
-        <v>-0.723280193768</v>
+        <v>-2.404595650325</v>
       </c>
       <c r="C90" s="64">
         <f>IF(AND(B90&gt;=0,B91&lt;0),A90+pH_step*B90/(B90-B91),0)</f>
@@ -15680,7 +16227,7 @@
       </c>
       <c r="B91" s="64">
         <f t="shared" si="3"/>
-        <v>-0.916234780256</v>
+        <v>-3.046646283691</v>
       </c>
       <c r="C91" s="64">
         <f>IF(AND(B91&gt;=0,B92&lt;0),A91+pH_step*B91/(B91-B92),0)</f>
@@ -15693,7 +16240,7 @@
       </c>
       <c r="B92" s="64">
         <f t="shared" si="3"/>
-        <v>-1.162416400965</v>
+        <v>-3.86625489911</v>
       </c>
       <c r="C92" s="64">
         <f>IF(AND(B92&gt;=0,B93&lt;0),A92+pH_step*B92/(B92-B93),0)</f>
@@ -15706,7 +16253,7 @@
       </c>
       <c r="B93" s="64">
         <f t="shared" si="3"/>
-        <v>-1.477655509108</v>
+        <v>-4.916151944852</v>
       </c>
       <c r="C93" s="64">
         <f>IF(AND(B93&gt;=0,B94&lt;0),A93+pH_step*B93/(B93-B94),0)</f>
@@ -15719,7 +16266,7 @@
       </c>
       <c r="B94" s="64">
         <f t="shared" si="3"/>
-        <v>-1.883055266022</v>
+        <v>-6.266648339548</v>
       </c>
       <c r="C94" s="64">
         <f>IF(AND(B94&gt;=0,B95&lt;0),A94+pH_step*B94/(B94-B95),0)</f>
@@ -15732,7 +16279,7 @@
       </c>
       <c r="B95" s="64">
         <f t="shared" si="3"/>
-        <v>-2.407047296867</v>
+        <v>-8.012488474449</v>
       </c>
       <c r="C95" s="64">
         <f>IF(AND(B95&gt;=0,B96&lt;0),A95+pH_step*B95/(B95-B96),0)</f>
@@ -15745,7 +16292,7 @@
       </c>
       <c r="B96" s="64">
         <f t="shared" si="3"/>
-        <v>-3.088383384182</v>
+        <v>-10.282823226284</v>
       </c>
       <c r="C96" s="64">
         <f>IF(AND(B96&gt;=0,B97&lt;0),A96+pH_step*B96/(B96-B97),0)</f>
@@ -15758,7 +16305,7 @@
       </c>
       <c r="B97" s="64">
         <f t="shared" si="3"/>
-        <v>-3.980541523763</v>
+        <v>-13.255897853524</v>
       </c>
       <c r="C97" s="64">
         <f>IF(AND(B97&gt;=0,B98&lt;0),A97+pH_step*B97/(B97-B98),0)</f>
@@ -15771,7 +16318,7 @@
       </c>
       <c r="B98" s="64">
         <f t="shared" si="3"/>
-        <v>-5.158286793953</v>
+        <v>-17.180922991367</v>
       </c>
       <c r="C98" s="64">
         <f>IF(AND(B98&gt;=0,B99&lt;0),A98+pH_step*B98/(B98-B99),0)</f>
@@ -15784,7 +16331,7 @@
       </c>
       <c r="B99" s="64">
         <f t="shared" si="3"/>
-        <v>-6.727538125688</v>
+        <v>-22.410965673407</v>
       </c>
       <c r="C99" s="64">
         <f>IF(AND(B99&gt;=0,B100&lt;0),A99+pH_step*B99/(B99-B100),0)</f>
@@ -15797,7 +16344,7 @@
       </c>
       <c r="B100" s="64">
         <f t="shared" si="3"/>
-        <v>-8.840337015349</v>
+        <v>-29.452847122759</v>
       </c>
       <c r="C100" s="64">
         <f>0</f>
@@ -15839,7 +16386,7 @@
       </c>
       <c r="D103" s="149">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
-        <v>6.460931418262</v>
+        <v>6.055158016113</v>
       </c>
       <c r="E103" s="51" t="s">
         <v>1878</v>
@@ -15862,7 +16409,7 @@
       </c>
       <c r="D104" s="149">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
-        <v>0.878640899134</v>
+        <v>0.948531749585</v>
       </c>
       <c r="E104" s="51" t="s">
         <v>1879</v>
@@ -15951,7 +16498,7 @@
       </c>
       <c r="D109" s="64" t="str">
         <f>IF(C_eff_Cl2&lt;Cl_onset,"negligible free chlorine ("&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ &lt; onset); does NOT account for the Exp-2 death - see metal_flag",IF(C_eff_Cl2&lt;Cl_kill,"sub-lethal "&amp;TEXT(C_eff_Cl2,"0.00")&amp;" mg/L as Cl₂ (band "&amp;TEXT(C_eff_lo_Cl2,"0.00")&amp;"-"&amp;TEXT(C_eff_hi_Cl2,"0.00")&amp;"); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag","SEVERE free chlorine: "&amp;TEXT(C_eff_Cl2,"0.0")&amp;" mg/L as Cl₂ - biofilm/electrode damage (Baek 2021)"))</f>
-        <v>sub-lethal 0.34 mg/L as Cl₂ (band 0.01-0.64); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
+        <v>sub-lethal 0.34 mg/L as Cl₂ (band 0.01-0.65); chloride-pool-bounded, cannot reach the kill threshold in this medium; does NOT explain the death - see metal_flag</v>
       </c>
       <c r="E109" s="51" t="s">
         <v>1127</v>
@@ -15972,7 +16519,7 @@
       </c>
       <c r="D110" s="64" t="str">
         <f>IF(pH_meas&lt;pH_band_lo,"pH BELOW HOB optimum (&lt;"&amp;TEXT(pH_band_lo,"0.0")&amp;") — reduce the CO₂ dose or lengthen the interval",IF(pH_meas&gt;pH_band_hi,"pH above optimum (&gt;"&amp;TEXT(pH_band_hi,"0.0")&amp;")","pH in HOB band "&amp;TEXT(pH_band_lo,"0.0")&amp;"–"&amp;TEXT(pH_band_hi,"0.0")))</f>
-        <v>pH in HOB band 6.5–7.5</v>
+        <v>pH BELOW HOB optimum (&lt;6.5) — reduce the CO₂ dose or lengthen the interval</v>
       </c>
       <c r="E110" s="51" t="s">
         <v>1880</v>
@@ -16054,7 +16601,7 @@
       </c>
       <c r="D125" s="149">
         <f>pH_Cl*pH_fHOCl*M_HOCl</f>
-        <v>8.306632108229</v>
+        <v>8.967377109974</v>
       </c>
       <c r="E125" s="51" t="s">
         <v>1460</v>
@@ -16261,7 +16808,7 @@
       </c>
       <c r="D138" s="149">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
-        <v>1.149504426795e-05</v>
+        <v>4.520261308413e-06</v>
       </c>
       <c r="E138" s="51" t="s">
         <v>1099</v>
@@ -16279,7 +16826,7 @@
       </c>
       <c r="D139" s="149">
         <f>P_HOCl/(k1_NH2Cl*NH3_free)</f>
-        <v>6.858822111426e-10</v>
+        <v>1.74420146132e-09</v>
       </c>
       <c r="E139" s="51" t="s">
         <v>1102</v>
@@ -16297,7 +16844,7 @@
       </c>
       <c r="D140" s="149">
         <f>HOCl_ss*M_HOCl</f>
-        <v>3.598138079654e-05</v>
+        <v>9.150080866082e-05</v>
       </c>
       <c r="E140" s="51" t="s">
         <v>1105</v>
@@ -16386,7 +16933,7 @@
       </c>
       <c r="D145" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_mgL/R_chloramine</f>
-        <v>0.250509669167</v>
+        <v>0.251064863446</v>
       </c>
       <c r="E145" s="51" t="inlineStr">
         <is>
@@ -16588,7 +17135,7 @@
       </c>
       <c r="D156" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_lo/R_chloramine_hi</f>
-        <v>0.004619787105</v>
+        <v>0.005174981383</v>
       </c>
       <c r="E156" s="51" t="s">
         <v>1247</v>
@@ -16606,7 +17153,7 @@
       </c>
       <c r="D157" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_hi/R_chloramine_lo</f>
-        <v>0.47681645215</v>
+        <v>0.477371646429</v>
       </c>
       <c r="E157" s="51" t="s">
         <v>1251</v>
@@ -17372,7 +17919,7 @@
       </c>
       <c r="D206" s="141">
         <f>E0_OER-nernst_slope*pH_meas</f>
-        <v>0.840287803139</v>
+        <v>0.86429309373</v>
       </c>
       <c r="E206" s="99" t="s">
         <v>1586</v>
@@ -17390,7 +17937,7 @@
       </c>
       <c r="D207" s="141">
         <f>E0_HER-nernst_slope*pH_meas</f>
-        <v>-0.388712196861</v>
+        <v>-0.36470690627</v>
       </c>
       <c r="E207" s="99" t="s">
         <v>1589</v>
@@ -17430,7 +17977,7 @@
       </c>
       <c r="D209" s="141">
         <f>E_HOCl_Cl-E_anode_op</f>
-        <v>-0.42751475509</v>
+        <v>-0.427527364769</v>
       </c>
       <c r="E209" s="67" t="inlineStr">
         <is>
@@ -17450,7 +17997,7 @@
       </c>
       <c r="D210" s="141">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
-        <v>0.306287803139</v>
+        <v>0.33029309373</v>
       </c>
       <c r="E210" s="67" t="s">
         <v>1599</v>
@@ -17470,7 +18017,7 @@
       </c>
       <c r="D211" s="141">
         <f>E_anode_op-E0_Cu</f>
-        <v>1.242530226635</v>
+        <v>1.266535517225</v>
       </c>
       <c r="E211" s="67" t="s">
         <v>1602</v>
@@ -17532,7 +18079,7 @@
       </c>
       <c r="D216" s="141">
         <f>Fcc*((km_HPO4/100)*HPO4_op+(km_HCO3/100)*HCO3_op)*1000/10</f>
-        <v>8.175182209731</v>
+        <v>8.600113527674</v>
       </c>
       <c r="E216" s="67" t="inlineStr">
         <is>
@@ -17570,7 +18117,7 @@
       </c>
       <c r="D218" s="141">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>0.345692073374</v>
+        <v>0.328611439745</v>
       </c>
       <c r="E218" s="67" t="s">
         <v>1618</v>
@@ -17606,7 +18153,7 @@
       </c>
       <c r="D220" s="141">
         <f>pH_op-LOG10(gamma_1)</f>
-        <v>6.570596176702</v>
+        <v>6.164822774553</v>
       </c>
       <c r="E220" s="67" t="s">
         <v>1624</v>
@@ -17699,7 +18246,7 @@
       </c>
       <c r="D226" s="141">
         <f>C_eff*M_Cl2/M_HOCl</f>
-        <v>0.338593949713</v>
+        <v>0.339344361561</v>
       </c>
       <c r="E226" s="67" t="s">
         <v>1899</v>
@@ -18013,7 +18560,7 @@
       </c>
       <c r="D252" s="141">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
-        <v>0.020302021576</v>
+        <v>0.026586383209</v>
       </c>
       <c r="E252" s="67" t="inlineStr">
         <is>
@@ -18039,7 +18586,7 @@
       </c>
       <c r="D253" s="141">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
-        <v>0.012455537296</v>
+        <v>0.006136275232</v>
       </c>
       <c r="E253" s="67" t="inlineStr">
         <is>
@@ -18117,7 +18664,7 @@
       </c>
       <c r="D256" s="141">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
-        <v>1.584430226635</v>
+        <v>1.608435517225</v>
       </c>
       <c r="E256" s="67" t="inlineStr">
         <is>
@@ -18168,7 +18715,7 @@
       </c>
       <c r="D258" s="141">
         <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,1E-12))-pH_meas-LOG10(MAX(pH_Cl,1E-12)))</f>
-        <v>1.156915471544</v>
+        <v>1.180908152456</v>
       </c>
       <c r="E258" s="67" t="inlineStr">
         <is>
@@ -18194,7 +18741,7 @@
       </c>
       <c r="D259" s="141">
         <f>C_eff_lo*M_Cl2/M_HOCl</f>
-        <v>0.00624419795</v>
+        <v>0.006994609797</v>
       </c>
       <c r="E259" s="67" t="inlineStr">
         <is>
@@ -18220,7 +18767,7 @@
       </c>
       <c r="D260" s="141">
         <f>C_eff_hi*M_Cl2/M_HOCl</f>
-        <v>0.644474787575</v>
+        <v>0.645225199422</v>
       </c>
       <c r="E260" s="67" t="inlineStr">
         <is>
@@ -18745,8 +19292,10 @@
         <f>MAX(0,O2_net_gen-O2_cons)</f>
         <v>1.58811785582e-05</v>
       </c>
-      <c r="E16" s="115" t="s">
-        <v>1926</v>
+      <c r="E16" s="115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Net electrolytic O₂ minus biological uptake, floored at zero. The floor matters: at the knallgas cap (O₂:H₂ = 0.5, i.e. bio_O2 = 3) uptake exactly consumes the electrolytic surplus and everything downstream that divides by this would blow up. A LOWER bound on the surplus: full H₂ uptake maximises respiration, so any H₂ that bubbles off uncaught raises the surplus (half uptake → ×2.2). Sensitive: ±10 % in bio_O2 moves it +29 % / −12 %.</t>
+        </is>
       </c>
       <c r="F16" s="20"/>
     </row>
@@ -19266,7 +19815,7 @@
       </c>
       <c r="D44" s="48" t="str">
         <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;", O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag basis)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 17%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 16%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="70" t="inlineStr">
         <is>
@@ -19715,7 +20264,7 @@
       </c>
       <c r="D76" s="150">
         <f>'Mass Transfer'!$D$100</f>
-        <v>0.0004480356964998</v>
+        <v>0.0005030206524901</v>
       </c>
       <c r="E76" s="135" t="inlineStr">
         <is>
@@ -19919,12 +20468,12 @@
         </is>
       </c>
       <c r="D84" s="48">
-        <f>rH2_gen/(n_flamm_src+CO2_supply_b)</f>
-        <v>0.169672046961</v>
+        <f>rH2_gen/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
+        <v>0.155418629263</v>
       </c>
       <c r="E84" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outflow-only mean-field balance: H₂ over all gas entering the headspace. Air ingress through the vent would lower H₂ and raise O₂.</t>
+          <t xml:space="preserve">Mean-field balance shared with Mass Transfer §300 (= y_H2_mf_l there): H₂ over all gas leaving the headspace — evolved gas, CO₂ pulses and, in the "Air exchange" vent model, the exchanged air. The pulse-to-pulse sawtooth peaks higher (D87 note).</t>
         </is>
       </c>
     </row>
@@ -19945,12 +20494,12 @@
         </is>
       </c>
       <c r="D85" s="48">
-        <f>O2_net_gen/(n_flamm_src+CO2_supply_b)</f>
-        <v>0.083045691591</v>
+        <f>(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
+        <v>0.076069380811</v>
       </c>
       <c r="E85" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">As above, for O₂.</t>
+          <t xml:space="preserve">As above for O₂ (= y_O2_mf_l on Mass Transfer), including the O₂ carried in by exchanged air. Air ingress lowers H₂ but raises O₂ toward 21 %, so it does not make the mixture safe.</t>
         </is>
       </c>
     </row>
@@ -19971,12 +20520,12 @@
         </is>
       </c>
       <c r="D86" s="48">
-        <f>MAX(0,MIN(rH2_gen/H2_LFL-n_flamm_src,O2_net_gen/(O2_LOC_H2*LOC_margin)-n_flamm_src))/CO2_rate_full_b</f>
+        <f>MAX(0,MIN(rH2_gen/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
         <v>0.002947616391</v>
       </c>
       <c r="E86" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Least valve-open fraction that brings H₂ below the LFL or O₂ below the LOC margin, whichever needs less CO₂.</t>
+          <t xml:space="preserve">Least valve-open fraction that brings H₂ below the LFL or O₂ below the LOC margin, whichever needs less CO₂, from the same balance; exchanged air counts as diluent for H₂ and as an O₂ source for the LOC route.</t>
         </is>
       </c>
     </row>
@@ -20023,12 +20572,12 @@
         </is>
       </c>
       <c r="D88" s="48">
-        <f>MAX(0,rH2_gen/H2_LFL-n_flamm_src)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
+        <f>MAX(0,rH2_gen/H2_LFL-n_flamm_src-F_vent_ex_b)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
         <v>0.975219102801</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Continuous inert headspace sweep that dilutes H₂ below the LFL with no CO₂ at all.</t>
+          <t xml:space="preserve">Continuous inert headspace sweep that dilutes H₂ below the LFL with no CO₂ at all, net of any air exchange already diluting it.</t>
         </is>
       </c>
     </row>
@@ -20083,7 +20632,7 @@
       </c>
       <c r="D97" s="48">
         <f>'Mass Transfer'!$D$198</f>
-        <v>7.42516851712</v>
+        <v>31.656160482387</v>
       </c>
       <c r="E97" s="67" t="inlineStr">
         <is>
@@ -20109,11 +20658,70 @@
       </c>
       <c r="D98" s="48">
         <f>C_cycle_start_b*1000/Km_CO2</f>
-        <v>148.503370342395</v>
+        <v>633.123209647745</v>
       </c>
       <c r="E98" s="69" t="inlineStr">
         <is>
           <t xml:space="preserve">Lowest dissolved CO₂ of the dosing cycle (mol/m³ = mM, ×1000 → µM) against RuBisCO Km. A sub-second pulse never approaches the full-sparge saturation D33 uses, so this, not D35, is the carbon-availability test; schedule-dependent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IMPORTS FOR THE SHARED HEADSPACE BALANCE (Mass Transfer §300)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) vent air-exchange flow</t>
+        </is>
+      </c>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_vent_ex_b</t>
+        </is>
+      </c>
+      <c r="C111" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D111" s="150">
+        <f>'Mass Transfer'!$D$308</f>
+        <v>0.0</v>
+      </c>
+      <c r="E111" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D308: zero for "Outflow only", Q_vent as mol/h for "Air exchange".</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) dry-air O₂ mole fraction</t>
+        </is>
+      </c>
+      <c r="B112" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_air_b</t>
+        </is>
+      </c>
+      <c r="C112" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D112" s="150">
+        <f>'Mass Transfer'!$D$307</f>
+        <v>0.2095</v>
+      </c>
+      <c r="E112" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D307.</t>
         </is>
       </c>
     </row>
@@ -21124,7 +21732,7 @@
       </c>
       <c r="D53" s="64">
         <f>kLa_sparge*duty</f>
-        <v>1.413348455674e-05</v>
+        <v>1.586800935557e-05</v>
       </c>
       <c r="E53" s="117" t="s">
         <v>643</v>
@@ -21162,7 +21770,7 @@
       </c>
       <c r="D55" s="48">
         <f>strip_sparge*duty</f>
-        <v>2.783954427351e-07</v>
+        <v>3.125613837221e-07</v>
       </c>
       <c r="E55" s="75" t="s">
         <v>649</v>
@@ -21181,7 +21789,7 @@
       </c>
       <c r="D56" s="45">
         <f>IF(O2_excess&gt;0,strip_avg/O2_excess,NA())</f>
-        <v>0.017529898157</v>
+        <v>0.01968124611</v>
       </c>
       <c r="E56" s="75" t="s">
         <v>652</v>
@@ -21371,7 +21979,7 @@
       </c>
       <c r="D66" s="48">
         <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,cleared_min)</f>
-        <v>21.040669319734</v>
+        <v>21.086843893767</v>
       </c>
       <c r="E66" s="99" t="s">
         <v>680</v>
@@ -21541,11 +22149,13 @@
         <v>135</v>
       </c>
       <c r="D75" s="48">
-        <f>IF(CO2_supply&gt;0,O2_excess/(O2_excess+CO2_supply),NA())</f>
-        <v>0.034232810687</v>
-      </c>
-      <c r="E75" s="99" t="s">
-        <v>705</v>
+        <f>y_O2_actual</f>
+        <v>0.031639138319</v>
+      </c>
+      <c r="E75" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">= y_O2_actual (D187): the mean-field headspace O₂ fraction of the sizing phase at the schedule in use, from the shared vent balance (§300). Kept so D76 (µM form) still reads.</t>
+        </is>
       </c>
       <c r="F75" s="20"/>
     </row>
@@ -21561,7 +22171,7 @@
       </c>
       <c r="D76" s="48">
         <f>H_O2_T*y_O2_vent*P_atm*1000</f>
-        <v>41.623674513885</v>
+        <v>38.470028282145</v>
       </c>
       <c r="E76" s="69" t="inlineStr">
         <is>
@@ -21582,7 +22192,7 @@
       </c>
       <c r="D77" s="48">
         <f>headspace_V/(Q_CO2*duty)</f>
-        <v>14.299822696002</v>
+        <v>12.736715659111</v>
       </c>
       <c r="E77" s="99" t="s">
         <v>710</v>
@@ -21601,7 +22211,7 @@
       </c>
       <c r="D78" s="48">
         <f>IF(O2_excess&gt;0,(strip_avg+surf_strip)/O2_excess,NA())</f>
-        <v>8.947888389834</v>
+        <v>8.950039737787</v>
       </c>
       <c r="E78" s="118" t="s">
         <v>713</v>
@@ -21850,7 +22460,7 @@
       </c>
       <c r="D91" s="48">
         <f>IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max))</f>
-        <v>14.299822696002</v>
+        <v>12.736715659111</v>
       </c>
       <c r="E91" s="159" t="inlineStr">
         <is>
@@ -21871,7 +22481,7 @@
       </c>
       <c r="D92" s="48">
         <f>spg_int_opt*60</f>
-        <v>857.98936176009</v>
+        <v>764.202939546678</v>
       </c>
       <c r="E92" s="159" t="s">
         <v>747</v>
@@ -21892,7 +22502,7 @@
       </c>
       <c r="D93" s="48">
         <f>spg_dur_opt/(spg_int_opt*60)</f>
-        <v>0.0009143622109901</v>
+        <v>0.001026576854</v>
       </c>
       <c r="E93" s="99" t="s">
         <v>750</v>
@@ -22025,7 +22635,7 @@
       </c>
       <c r="D100" s="28">
         <f>CO2_pulse*pulses_h</f>
-        <v>0.0004480356964998</v>
+        <v>0.0005030206524901</v>
       </c>
       <c r="E100" s="160" t="s">
         <v>765</v>
@@ -22118,7 +22728,7 @@
       </c>
       <c r="D105" s="28">
         <f>spg_dur/(spg_int*60)</f>
-        <v>0.0009143622109901</v>
+        <v>0.001026576854</v>
       </c>
       <c r="E105" s="160" t="s">
         <v>765</v>
@@ -22154,8 +22764,10 @@
       <c r="F107" s="20"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A108" s="20" t="s">
-        <v>782</v>
+      <c r="A108" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO at the schedule in use (sawtooth model, sizing phase)</t>
+        </is>
       </c>
       <c r="B108" s="20" t="s">
         <v>783</v>
@@ -22164,11 +22776,13 @@
         <v>102</v>
       </c>
       <c r="D108" s="28">
-        <f>(DO_hs_floor+DO_surf_excess)*M_O2</f>
-        <v>2.638866712696</v>
-      </c>
-      <c r="E108" s="160" t="s">
-        <v>1929</v>
+        <f>DO_avg_sched*M_O2</f>
+        <v>2.634660261764</v>
+      </c>
+      <c r="E108" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean dissolved O₂ of the sawtooth model (§300) on the sizing phase: the surface excess plus equilibrium with the time-mean headspace O₂. Sits near DO_target when the DO constraint binds, because the sizing applies the same sawtooth factor; the peak (D374 / Summary D21) is the non-tautological check.</t>
+        </is>
       </c>
       <c r="F108" s="20"/>
     </row>
@@ -22247,7 +22861,7 @@
       <c r="C113" s="20"/>
       <c r="D113" s="28" t="str">
         <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) DO would be "&amp;TEXT(DO_at_carbon*M_O2,"0.0")&amp;" mg/L against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 13.7 mg/L against a 2.6 mg/L target</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 20.1 mg/L against a 2.6 mg/L target</v>
       </c>
       <c r="E113" s="82" t="inlineStr">
         <is>
@@ -22399,7 +23013,7 @@
       </c>
       <c r="D122" s="28">
         <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
-        <v>14.299822696002</v>
+        <v>12.736715659111</v>
       </c>
       <c r="E122" s="20"/>
       <c r="F122" s="20"/>
@@ -22433,7 +23047,7 @@
       </c>
       <c r="D124" s="28">
         <f>60/spg_int</f>
-        <v>4.195856219726</v>
+        <v>4.710790568452</v>
       </c>
       <c r="E124" s="20"/>
       <c r="F124" s="20"/>
@@ -22450,7 +23064,7 @@
       </c>
       <c r="D125" s="28">
         <f>pulses_h*24</f>
-        <v>100.700549273429</v>
+        <v>113.058973642855</v>
       </c>
       <c r="E125" s="20"/>
       <c r="F125" s="20"/>
@@ -22467,7 +23081,7 @@
       </c>
       <c r="D126" s="28">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v>26.425646704826</v>
+        <v>29.668720934024</v>
       </c>
       <c r="E126" s="20"/>
       <c r="F126" s="20"/>
@@ -22484,7 +23098,7 @@
       </c>
       <c r="D127" s="28">
         <f>O2_excess/60*spg_int</f>
-        <v>3.784967293096e-06</v>
+        <v>3.371234260456e-06</v>
       </c>
       <c r="E127" s="20"/>
       <c r="F127" s="20"/>
@@ -22518,7 +23132,7 @@
       </c>
       <c r="D129" s="28">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v>0.017529898157</v>
+        <v>0.01968124611</v>
       </c>
       <c r="E129" s="20"/>
       <c r="F129" s="20"/>
@@ -22579,8 +23193,10 @@
       <c r="F132" s="20"/>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A133" s="17" t="s">
-        <v>993</v>
+      <c r="A133" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field steady DO (sizing-phase source)</t>
+        </is>
       </c>
       <c r="B133" s="18" t="s">
         <v>994</v>
@@ -22590,10 +23206,12 @@
       </c>
       <c r="D133" s="28">
         <f>DO_hs_floor+DO_surf_excess</f>
-        <v>0.08246973913</v>
-      </c>
-      <c r="E133" s="69" t="s">
-        <v>1823</v>
+        <v>0.079316092899</v>
+      </c>
+      <c r="E133" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flux-mean form of D108 in mol/m³: headspace floor (D188, from the shared vent balance) plus the surface excess on the sizing-phase source. Equals DO_target ÷ saw_factor-adjusted by construction when the DO constraint binds.</t>
+        </is>
       </c>
       <c r="F133" s="20"/>
     </row>
@@ -22609,7 +23227,7 @@
       </c>
       <c r="D134" s="28" t="str">
         <f>IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf"))</f>
-        <v>ESTIMATED kLa — DO-limited interval is 14.3 min; confirm by measuring kL_surf</v>
+        <v>ESTIMATED kLa — DO-limited interval is 12.7 min; confirm by measuring kL_surf</v>
       </c>
       <c r="E134" s="69" t="inlineStr">
         <is>
@@ -22619,8 +23237,10 @@
       <c r="F134" s="20"/>
     </row>
     <row r="135" spans="1:6" ht="24" x14ac:dyDescent="0.2">
-      <c r="A135" s="20" t="s">
-        <v>999</v>
+      <c r="A135" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field steady DO (LAG source)</t>
+        </is>
       </c>
       <c r="B135" s="20" t="s">
         <v>1000</v>
@@ -22629,11 +23249,13 @@
         <v>1001</v>
       </c>
       <c r="D135" s="28">
-        <f>DO_hs_floor+DO_surf_excess_lag</f>
-        <v>0.169683392542</v>
-      </c>
-      <c r="E135" s="69" t="s">
-        <v>1824</v>
+        <f>DO_mf_l</f>
+        <v>0.220552478156</v>
+      </c>
+      <c r="E135" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag-phase companion evaluated on the LAG headspace balance (y_O2_mf_l, with the H₂ as a diluent and the vent model in use) — not the growth headspace fraction, which understated it by ~30 % (R2-B2). The sawtooth mean and peak are in the lag block of §300.</t>
+        </is>
       </c>
       <c r="F135" s="20"/>
     </row>
@@ -22737,14 +23359,18 @@
       <c r="D142" s="131">
         <v>0.5</v>
       </c>
-      <c r="E142" s="69" t="s">
-        <v>1170</v>
+      <c r="E142" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bidirectional air-exchange flow through the vent, used ONLY when vent_model (Summary D111) = "Air exchange", by the O₂ balance, the CO₂ pool and the flammability block alike. KEY UNCERTAIN PARAMETER — measure (pressure-decay or headspace-O₂ tracer, R2 experiment 1); include any per-pulse back-draw in it. Not free membrane diffusion, which would clear in seconds.</t>
+        </is>
       </c>
       <c r="F142" s="20"/>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A143" s="17" t="s">
-        <v>1171</v>
+      <c r="A143" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace turnover between pulses</t>
+        </is>
       </c>
       <c r="B143" s="18" t="s">
         <v>1172</v>
@@ -22753,11 +23379,13 @@
         <v>639</v>
       </c>
       <c r="D143" s="48">
-        <f>(Q_vent/1000000/60)/headspace_V_m3</f>
-        <v>0.003189880019</v>
-      </c>
-      <c r="E143" s="67" t="s">
-        <v>1173</v>
+        <f>F_gap_sched/3600/n_hs_gas</f>
+        <v>0.0</v>
+      </c>
+      <c r="E143" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-order headspace clearance between pulses from the ONE vent balance (§300): exchange flow plus net evolved gas, over the headspace inventory. Zero when nothing leaves between pulses (outflow-only vent, growth phase).</t>
+        </is>
       </c>
       <c r="F143" s="20"/>
     </row>
@@ -22772,11 +23400,13 @@
         <v>67</v>
       </c>
       <c r="D144" s="48">
-        <f>headspace_V_m3/(Q_vent/1000000/60)/60</f>
-        <v>5.224856911834</v>
-      </c>
-      <c r="E144" s="67" t="s">
-        <v>1176</v>
+        <f>IF(k_vent&gt;0,1/k_vent/60,cleared_min)</f>
+        <v>9999.0</v>
+      </c>
+      <c r="E144" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time constant for the headspace to clear between pulses; the 9999 sentinel means nothing leaves between pulses, so only the pulses clear it.</t>
+        </is>
       </c>
       <c r="F144" s="20"/>
     </row>
@@ -22927,7 +23557,7 @@
       </c>
       <c r="D152" s="48">
         <f>MAX(0,spg_int*60-spg_dur)</f>
-        <v>857.204848710266</v>
+        <v>763.418426496853</v>
       </c>
       <c r="E152" s="67" t="s">
         <v>1190</v>
@@ -23018,7 +23648,7 @@
       </c>
       <c r="D162" s="48">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,CO2_cyc_avg_new))/1000</f>
-        <v>0.00952617025</v>
+        <v>0.031754970696</v>
       </c>
       <c r="E162" s="67" t="s">
         <v>1859</v>
@@ -23281,11 +23911,13 @@
         <v>1001</v>
       </c>
       <c r="D180" s="141">
-        <f>O2_excess/(kLa_surf_used*3600*(V_charge/1000000))</f>
+        <f>O2_src_sched/(kLa_surf_used*3600*(V_charge/1000000))</f>
         <v>0.040846064617</v>
       </c>
-      <c r="E180" s="67" t="s">
-        <v>1798</v>
+      <c r="E180" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steady state across the free surface is flux = kLa·V·(C − C*), so the liquid must sit THIS far above the headspace-equilibrium concentration to push the source O₂ out. Evaluated on the sizing-phase source (O2_src_sched, §300); the growth and lag values are DO_surf_excess_g and D181. The smaller the surface kLa, the larger this excess — it decides whether any sparge schedule can hold the target at all.</t>
+        </is>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.2">
@@ -23353,12 +23985,12 @@
         <v>1274</v>
       </c>
       <c r="D184" s="141">
-        <f>IF(ISNUMBER(y_O2_star),O2_excess*(1-y_O2_star)/(y_O2_star*CO2_rate_full),NA())</f>
-        <v>0.0009143622109901</v>
+        <f>IF(ISNUMBER(y_O2_star),MAX(0,((O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_vent_ex-O2_src_sched-H2_src_sched+CO2_fix_sched)/CO2_rate_full),NA())</f>
+        <v>0.001026576854</v>
       </c>
       <c r="E184" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">At steady state everything entering the headspace leaves through the vent, so the vent-gas composition is the flux composition: y = O₂ flux/(O₂ flux + CO₂ flux). Solving for the CO₂ flux that dilutes oxygen to y* gives this duty. Unlike duty_O2vent (D87), it accounts for the surface-transfer excess and the (1−y) term.</t>
+          <t xml:space="preserve">Inverts the shared headspace balance (§300): y = (O₂ + air O₂)/(exchange + CO₂ supply + O₂ + H₂ − fixation). Solving for the CO₂ supply that puts the TIME-mean headspace O₂ at y* (flux mean = y*/saw_factor) gives this duty. Reduces to the old O₂(1−y*)/(y*·CO₂ rate) form with no exchange, no H₂, no fixation and no sawtooth. Zero when O₂ imposes no constraint (D185 then uses the carbon interval).</t>
         </is>
       </c>
     </row>
@@ -23374,7 +24006,7 @@
       </c>
       <c r="D185" s="141">
         <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_opt/(60*duty_DO),spg_int_carbon),NA())</f>
-        <v>14.299822696002</v>
+        <v>12.736715659111</v>
       </c>
       <c r="E185" s="67" t="s">
         <v>1813</v>
@@ -23391,11 +24023,13 @@
         <v>639</v>
       </c>
       <c r="D186" s="141">
-        <f>O2_excess/(DO_target*3600*(V_charge/1000000))</f>
+        <f>O2_src_sched/(DO_target*3600*(V_charge/1000000))</f>
         <v>0.003566106821</v>
       </c>
-      <c r="E186" s="67" t="s">
-        <v>1816</v>
+      <c r="E186" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The surface kLa below which the DO target is unreachable at any sparge interval, on the sizing-phase source. Both phases: kLa_surf_req_g / kLa_surf_req_l and their margins in §300 (Summary rows 120–123). The ratio to kLa_surf_used is the whole safety margin of the DO strategy, and it rests on a coefficient nobody has measured yet.</t>
+        </is>
       </c>
     </row>
     <row r="187" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -23409,11 +24043,13 @@
         <v>1274</v>
       </c>
       <c r="D187" s="141">
-        <f>IF(CO2_supply&gt;0,O2_excess/(O2_excess+CO2_supply),NA())</f>
-        <v>0.034232810687</v>
-      </c>
-      <c r="E187" s="67" t="s">
-        <v>1819</v>
+        <f>IF(O2_sizing_phase=phase_name_1,y_O2_mf_g,IF(O2_sizing_phase=phase_name_2,y_O2_mf_l,NA()))</f>
+        <v>0.031639138319</v>
+      </c>
+      <c r="E187" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flux-mean headspace O₂ fraction at the schedule in use, from the ONE vent balance (§300) on the sizing phase: includes air O₂ ingress in "Air exchange", the H₂ diluent in "Lag", and the fixation sink. The CO₂ pool (§190) and the flammability block (Biology 83–88) now use the same balance.</t>
+        </is>
       </c>
     </row>
     <row r="188" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -23428,10 +24064,12 @@
       </c>
       <c r="D188" s="141">
         <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_atm,NA())</f>
-        <v>0.041623674514</v>
-      </c>
-      <c r="E188" s="67" t="s">
-        <v>1822</v>
+        <v>0.038470028282</v>
+      </c>
+      <c r="E188" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface stripping can only move oxygen into the headspace, so the liquid can never fall below equilibrium with it. Set by the vent balance (CO₂ flush, exchange, evolved gas), not by the surface kLa — which is why the sparge schedule and the vent, not the stirring, govern dissolved oxygen here.</t>
+        </is>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
@@ -23496,8 +24134,10 @@
       </c>
     </row>
     <row r="194" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A194" t="s">
-        <v>1839</v>
+      <c r="A194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ retained in the headspace by a pulse, as pool concentration</t>
+        </is>
       </c>
       <c r="B194" s="18" t="s">
         <v>1840</v>
@@ -23506,12 +24146,12 @@
         <v>1001</v>
       </c>
       <c r="D194" s="141">
-        <f>CO2_pulse/(V_L_m3+Vg_CO2)</f>
-        <v>5.869170438925</v>
+        <f>C_sat_CO2*(1-pool_a)*(1-flush_ret)</f>
+        <v>3.710023297714</v>
       </c>
       <c r="E194" s="99" t="inlineStr">
         <is>
-          <t xml:space="preserve">The CO₂ actually delivered per pulse (D123, which follows any manual or Summary override), spread over the pooled liquid+headspace capacity: the mass-conservation constraint. It reads the delivered pulse rather than one nominal headspace flush, so an overridden pulse length charges the cycle correctly.</t>
+          <t xml:space="preserve">A well-mixed flush leaves the headspace at 1 atm with (1 − flush_ret) of fresh CO₂; the rest of the delivered pulse blows straight through the vent. As pool concentration: C_sat·(headspace share)·(1 − flush_ret). Equals the old CO2_pulse/(V_L+Vg) for a plug-flow one-headspace pulse. Pure-CO₂ saturation is the no-loss limit by construction.</t>
         </is>
       </c>
     </row>
@@ -23527,10 +24167,12 @@
       </c>
       <c r="D195" s="141">
         <f>k_vent*Vg_CO2/(V_L_m3+Vg_CO2)</f>
-        <v>0.000559912956744</v>
-      </c>
-      <c r="E195" s="99" t="s">
-        <v>1843</v>
+        <v>0.0</v>
+      </c>
+      <c r="E195" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only the headspace share of the pool is exposed to what leaves between pulses (k_vent, now from the shared vent balance), so the whole inventory decays at that rate scaled by the share. Zero for an outflow-only vent in growth: then only fixation drains the pool (pool_D_raw).</t>
+        </is>
       </c>
     </row>
     <row r="196" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -23544,11 +24186,13 @@
         <v>110</v>
       </c>
       <c r="D196" s="141">
-        <f>(kLa_CO2_off*V_L_m3/Vg_CO2)/k_vent</f>
-        <v>10.393999248454</v>
-      </c>
-      <c r="E196" s="67" t="s">
-        <v>1846</v>
+        <f>IF(k_vent&gt;0,(kLa_CO2_off*V_L_m3/Vg_CO2)/k_vent,cleared_min)</f>
+        <v>9999.0</v>
+      </c>
+      <c r="E196" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid-uptake rate constant ÷ headspace turnover between pulses. Well above 1 means the two compartments stay in quasi-equilibrium, which the pool model assumes; the 9999 sentinel is the outflow-only growth case (no turnover at all).</t>
+        </is>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
@@ -23563,7 +24207,7 @@
       </c>
       <c r="D197" s="141">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
-        <v>0.618808080904</v>
+        <v>1.0</v>
       </c>
       <c r="E197" s="99" t="s">
         <v>1849</v>
@@ -23580,11 +24224,13 @@
         <v>1001</v>
       </c>
       <c r="D198" s="141">
-        <f>(C_air_CO2*(1-pool_e)+pool_b*pool_e)/(1-pool_a*pool_e)</f>
-        <v>7.42516851712</v>
-      </c>
-      <c r="E198" s="99" t="s">
-        <v>1852</v>
+        <f>(pool_D_gap+pool_b*pool_e)/(1-pool_ret*pool_e)</f>
+        <v>31.656160482387</v>
+      </c>
+      <c r="E198" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed point of the limit cycle: decay over the gap toward the vent/fixation asymptote (pool_D_gap), then a pulse that keeps pool_ret of the pool and adds pool_b, repeated. With an air-exchange vent and no fixation it is the previous (C_air(1−e)+b·e)/(1−a·e).</t>
+        </is>
       </c>
     </row>
     <row r="199" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -23598,11 +24244,13 @@
         <v>1001</v>
       </c>
       <c r="D199" s="141">
-        <f>pool_a*C_cycle_start+pool_b</f>
-        <v>11.991014682526</v>
-      </c>
-      <c r="E199" s="99" t="s">
-        <v>1855</v>
+        <f>pool_ret*C_cycle_start+pool_b</f>
+        <v>31.853780908877</v>
+      </c>
+      <c r="E199" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After the pulse and the fast headspace-to-liquid equilibration (tens of seconds): the retained pool plus the fresh CO₂.</t>
+        </is>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.2">
@@ -23616,11 +24264,13 @@
         <v>1001</v>
       </c>
       <c r="D200" s="141">
-        <f>C_air_CO2+(C_cycle_peak-C_air_CO2)*(1-pool_e)/(k_eff_CO2*t_off_CO2)</f>
-        <v>9.526170249632</v>
-      </c>
-      <c r="E200" s="99" t="s">
-        <v>1858</v>
+        <f>C_cycle_peak*pool_phi+pool_D_raw*pool_psi</f>
+        <v>31.754970695632</v>
+      </c>
+      <c r="E200" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-average of the decay over the gap, written with Φ/Ψ so the no-turnover case (outflow-only vent, growth) is the linear-drain limit rather than 0/0. This is what the pH solve consumes (Chemistry D5 via D162).</t>
+        </is>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.2">
@@ -23932,12 +24582,12 @@
         </is>
       </c>
       <c r="D232" s="141">
-        <f>H_O2_T*P_atm*O2_excess/(O2_excess+CO2_rate_full*duty_carbon)+DO_surf_excess</f>
-        <v>0.428670828967</v>
+        <f>DO_surf_excess+H_O2_T*P_atm*(O2_src_sched+y_O2_air*F_vent_ex)/(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)</f>
+        <v>0.628922200193</v>
       </c>
       <c r="E232" s="99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same headspace back-pressure + surface-excess balance as D188/D180, evaluated at the carbon-limited duty instead of the DO-limited one.</t>
+          <t xml:space="preserve">Same shared headspace balance as D187/D180 (sizing phase, vent model in use) evaluated at the carbon-limited duty instead of the DO-limited one. At that duty the CO₂ leaving is only twice the fixation, so O₂ is a large fraction of the vent gas.</t>
         </is>
       </c>
     </row>
@@ -23996,6 +24646,2121 @@
       <c r="E242" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">Pulse as it can actually be commanded; never below the solenoid floor. Summary D14 shows it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEADSPACE BALANCE — one vent model shared by the O₂ block (§177), the CO₂ pool (§190) and the lag-phase flammability block (Biology rows 83–88)</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Vent model</t>
+        </is>
+      </c>
+      <c r="B301" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vent_model</t>
+        </is>
+      </c>
+      <c r="C301" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D301" s="134" t="str">
+        <f>Summary!$D$111</f>
+        <v>Outflow only</v>
+      </c>
+      <c r="E301" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D111. Owner decision: "Outflow only" or "Air exchange"; anything else returns #N/A by design. Default "Outflow only" until the vent hardware is characterised (R2 experiment 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  valid vent model 1</t>
+        </is>
+      </c>
+      <c r="B302" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vent_name_1</t>
+        </is>
+      </c>
+      <c r="C302" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D302" s="131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outflow only</t>
+        </is>
+      </c>
+      <c r="E302" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas leaves through the vent but none enters between pulses (check valve or sealed cap; the small sub-atmospheric dip after each pulse is tolerated). The headspace is then diluted only by the CO₂ pulses and by what electrolysis evolves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  valid vent model 2</t>
+        </is>
+      </c>
+      <c r="B303" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vent_name_2</t>
+        </is>
+      </c>
+      <c r="C303" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D303" s="131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Air exchange</t>
+        </is>
+      </c>
+      <c r="E303" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Room air exchanges with the headspace at Q_vent (D142) continuously — an open tube, diffusion, or per-pulse back-draw of the same average volume. Q_vent must then be the TOTAL air ingress, including the back-draw that refills whatever the liquid absorbs after each pulse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) O₂ sizing phase</t>
+        </is>
+      </c>
+      <c r="B304" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_sizing_phase</t>
+        </is>
+      </c>
+      <c r="C304" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D304" s="134" t="str">
+        <f>Summary!$D$112</f>
+        <v>Growth</v>
+      </c>
+      <c r="E304" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D112. Owner decision: "Growth" sizes the schedule on the surplus after knallgas uptake; "Lag" on the whole net electrolytic O₂ with the H₂ as a diluent. Anything else returns #N/A by design. Both phases are always reported (rows 327–369).</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  valid sizing phase 1</t>
+        </is>
+      </c>
+      <c r="B305" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phase_name_1</t>
+        </is>
+      </c>
+      <c r="C305" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D305" s="131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Growth</t>
+        </is>
+      </c>
+      <c r="E305" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steady growth: 100 % H₂ uptake (Biology D13), so the O₂ source is O2_excess and no H₂ reaches the headspace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  valid sizing phase 2</t>
+        </is>
+      </c>
+      <c r="B306" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phase_name_2</t>
+        </is>
+      </c>
+      <c r="C306" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D306" s="131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag</t>
+        </is>
+      </c>
+      <c r="E306" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag / establishment: no uptake, so all net electrolytic O₂ and all H₂ reach the headspace and no CO₂ is fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dry-air O₂ mole fraction</t>
+        </is>
+      </c>
+      <c r="B307" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_air</t>
+        </is>
+      </c>
+      <c r="C307" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D307" s="131">
+        <v>0.2095</v>
+      </c>
+      <c r="E307" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard dry air, 20.95 vol % O₂ (CRC Handbook; ISO 2533). Enters the balance only in the "Air exchange" vent model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vent air-exchange flow</t>
+        </is>
+      </c>
+      <c r="B308" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_vent_ex</t>
+        </is>
+      </c>
+      <c r="C308" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D308" s="48">
+        <f>IF(vent_model=vent_name_1,0,IF(vent_model=vent_name_2,P_atm*(Q_vent/1000000/60)/(R_gas*T_K)*3600,NA()))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E308" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Molar air flow exchanged through the vent (ideal gas at P_atm, T_K). Zero in "Outflow only"; Q_vent converted mL/min → mol/h in "Air exchange". Inherits the uncertainty of Q_vent — measure it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ source — growth phase</t>
+        </is>
+      </c>
+      <c r="B309" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_src_g</t>
+        </is>
+      </c>
+      <c r="C309" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D309" s="48">
+        <f>O2_excess</f>
+        <v>1.58811785582e-05</v>
+      </c>
+      <c r="E309" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surplus O₂ after full-H₂-uptake respiration (Biology D16). A LOWER bound on the surplus: any H₂ that bubbles off uncaught raises it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ source — lag phase</t>
+        </is>
+      </c>
+      <c r="B310" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_src_l</t>
+        </is>
+      </c>
+      <c r="C310" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D310" s="48">
+        <f>O2_net_gen</f>
+        <v>4.979033518202e-05</v>
+      </c>
+      <c r="E310" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Net electrolytic O₂ with no biological uptake (Electrochemistry D29).</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) H₂ generation rate</t>
+        </is>
+      </c>
+      <c r="B311" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rH2_gen</t>
+        </is>
+      </c>
+      <c r="C311" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D311" s="142">
+        <f>Electrochemistry!$D$21</f>
+        <v>0.0001017274698715</v>
+      </c>
+      <c r="E311" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D21.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) H₂ consumed</t>
+        </is>
+      </c>
+      <c r="B312" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_cons</t>
+        </is>
+      </c>
+      <c r="C312" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D312" s="142">
+        <f>Biology!$D$13</f>
+        <v>0.0001017274698715</v>
+      </c>
+      <c r="E312" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D13 (100 % uptake in steady growth).</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ to headspace — growth phase</t>
+        </is>
+      </c>
+      <c r="B313" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_src_g</t>
+        </is>
+      </c>
+      <c r="C313" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D313" s="48">
+        <f>MAX(0,rH2_gen-H2_cons)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E313" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residual H₂ reaching the headspace in growth: zero under the 100 % uptake assumption. A real residual (cathode bubbles bypassing the liquid) is a DATA GAP — see the off-gas H₂ experiment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ to headspace — lag phase</t>
+        </is>
+      </c>
+      <c r="B314" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_src_l</t>
+        </is>
+      </c>
+      <c r="C314" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D314" s="48">
+        <f>rH2_gen</f>
+        <v>0.0001017274698715</v>
+      </c>
+      <c r="E314" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All evolved H₂ reaches the headspace before uptake starts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ fixation sink — growth phase</t>
+        </is>
+      </c>
+      <c r="B315" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_fix_g</t>
+        </is>
+      </c>
+      <c r="C315" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D315" s="48">
+        <f>CO2_cons</f>
+        <v>1.695457831191e-05</v>
+      </c>
+      <c r="E315" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carbon fixed by the culture (Biology D15) is drawn from the dissolved pool and hence from the headspace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ fixation sink — lag phase</t>
+        </is>
+      </c>
+      <c r="B316" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_fix_l</t>
+        </is>
+      </c>
+      <c r="C316" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D316" s="131">
+        <v>0</v>
+      </c>
+      <c r="E316" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">By definition of the lag phase: no carbon fixation yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ source — sizing phase</t>
+        </is>
+      </c>
+      <c r="B317" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_src_sched</t>
+        </is>
+      </c>
+      <c r="C317" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D317" s="48">
+        <f>IF(O2_sizing_phase=phase_name_1,O2_src_g,IF(O2_sizing_phase=phase_name_2,O2_src_l,NA()))</f>
+        <v>1.58811785582e-05</v>
+      </c>
+      <c r="E317" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The O₂ source the schedule is sized on, picked by O2_sizing_phase (D304).</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ to headspace — sizing phase</t>
+        </is>
+      </c>
+      <c r="B318" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_src_sched</t>
+        </is>
+      </c>
+      <c r="C318" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D318" s="48">
+        <f>IF(O2_sizing_phase=phase_name_1,H2_src_g,IF(O2_sizing_phase=phase_name_2,H2_src_l,NA()))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E318" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above, for H₂ (a diluent in the balance).</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ fixation sink — sizing phase</t>
+        </is>
+      </c>
+      <c r="B319" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_fix_sched</t>
+        </is>
+      </c>
+      <c r="C319" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D319" s="48">
+        <f>IF(O2_sizing_phase=phase_name_1,CO2_fix_g,IF(O2_sizing_phase=phase_name_2,CO2_fix_l,NA()))</f>
+        <v>1.695457831191e-05</v>
+      </c>
+      <c r="E319" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above, for the fixation sink.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace volumes per pulse (optimal pulse)</t>
+        </is>
+      </c>
+      <c r="B320" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flush_vol_opt</t>
+        </is>
+      </c>
+      <c r="C320" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D320" s="48">
+        <f>nCO2_rate*spg_dur_opt/n_hs_gas</f>
+        <v>1.0</v>
+      </c>
+      <c r="E320" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ delivered by the optimal pulse (D90) in headspace volumes; = flush_factor unless the solenoid floor binds. Used for sizing, so it must not depend on the schedule in use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace retained through the optimal pulse</t>
+        </is>
+      </c>
+      <c r="B321" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flush_ret_opt</t>
+        </is>
+      </c>
+      <c r="C321" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D321" s="48">
+        <f>EXP(-flush_vol_opt)</f>
+        <v>0.367879441171</v>
+      </c>
+      <c r="E321" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: the pulse flushes a WELL-MIXED headspace, so exp(−volumes) of the old gas survives it (plug flow would leave none). The 5 mm-high headspace disk sits between the two; well-mixed is the conservative choice for every dilution verdict here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sawtooth factor (time-mean ÷ flux-mean headspace O₂)</t>
+        </is>
+      </c>
+      <c r="B322" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">saw_factor</t>
+        </is>
+      </c>
+      <c r="C322" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D322" s="48">
+        <f>flush_vol_opt*(1+flush_ret_opt)/(2*(1-flush_ret_opt))</f>
+        <v>1.081976706869</v>
+      </c>
+      <c r="E322" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The headspace O₂ ramps up between pulses and is knocked down by each flush. The gas LEAVING carries the flux-weighted mean; the liquid sees the TIME mean, which is higher by this factor in the slow-vent limit (little gas leaves between pulses): f·(1+e^−f)/(2(1−e^−f)), 1.08 for one well-mixed headspace volume. Applied to the sizing so that the cycle-mean DO, not the flux mean, sits at the target. Conservative (overstates the sawtooth) when the vent turns the headspace over within a gap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace volumes per pulse (schedule in use)</t>
+        </is>
+      </c>
+      <c r="B323" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flush_vol</t>
+        </is>
+      </c>
+      <c r="C323" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D323" s="48">
+        <f>CO2_pulse/n_hs_gas</f>
+        <v>1.0</v>
+      </c>
+      <c r="E323" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ actually delivered per pulse (D123, follows any override) in headspace volumes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace retained through a pulse (schedule in use)</t>
+        </is>
+      </c>
+      <c r="B324" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flush_ret</t>
+        </is>
+      </c>
+      <c r="C324" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D324" s="48">
+        <f>EXP(-flush_vol)</f>
+        <v>0.367879441171</v>
+      </c>
+      <c r="E324" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exp(−volumes), well-mixed flush as above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap between pulses</t>
+        </is>
+      </c>
+      <c r="B325" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">t_gap_h</t>
+        </is>
+      </c>
+      <c r="C325" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="D325" s="48">
+        <f>t_off_CO2/3600</f>
+        <v>0.212060674027</v>
+      </c>
+      <c r="E325" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D152 in hours, to match the mol/h flows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid O₂ response time</t>
+        </is>
+      </c>
+      <c r="B326" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tau_L_h</t>
+        </is>
+      </c>
+      <c r="C326" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="D326" s="48">
+        <f>1/(kLa_surf_used*3600)</f>
+        <v>0.038579691488</v>
+      </c>
+      <c r="E326" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/kLa: how fast the dissolved O₂ follows the headspace (D98).</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ inflow — growth</t>
+        </is>
+      </c>
+      <c r="B327" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S_O2_g</t>
+        </is>
+      </c>
+      <c r="C327" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D327" s="48">
+        <f>O2_src_g+y_O2_air*F_vent_ex</f>
+        <v>1.58811785582e-05</v>
+      </c>
+      <c r="E327" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ entering the headspace: from the liquid (the whole source must leave this way at steady state) plus the O₂ in any exchanged air.</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Net vent outflow, cycle mean — growth</t>
+        </is>
+      </c>
+      <c r="B328" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_hs_net_g</t>
+        </is>
+      </c>
+      <c r="C328" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D328" s="48">
+        <f>CO2_supply+O2_src_g+H2_src_g-CO2_fix_g</f>
+        <v>0.0005019472527364</v>
+      </c>
+      <c r="E328" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Everything entering the headspace over a cycle minus the fixation sink: the gas that must leave through the vent on average.</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field headspace O₂ — growth</t>
+        </is>
+      </c>
+      <c r="B329" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_mf_g</t>
+        </is>
+      </c>
+      <c r="C329" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D329" s="48">
+        <f>IF(F_vent_ex+F_hs_net_g&gt;0,S_O2_g/(F_vent_ex+F_hs_net_g),NA())</f>
+        <v>0.031639138319</v>
+      </c>
+      <c r="E329" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ONE headspace balance, flux-weighted: O₂ in ÷ all gas out (vent outflow plus exchange). Reduces to O₂/(O₂+CO₂) with no exchange, no H₂ and no fixation — the old D187. Biology D85 is the same balance on the lag source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field headspace H₂ — growth</t>
+        </is>
+      </c>
+      <c r="B330" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_H2_mf_g</t>
+        </is>
+      </c>
+      <c r="C330" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D330" s="48">
+        <f>IF(F_vent_ex+F_hs_net_g&gt;0,H2_src_g/(F_vent_ex+F_hs_net_g),NA())</f>
+        <v>0.0</v>
+      </c>
+      <c r="E330" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same balance for H₂ (Biology D84 on the lag source).</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas leaving between pulses — growth</t>
+        </is>
+      </c>
+      <c r="B331" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_gap_g</t>
+        </is>
+      </c>
+      <c r="C331" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D331" s="48">
+        <f>F_vent_ex+MAX(0,O2_src_g+H2_src_g-CO2_fix_g)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E331" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What leaves the headspace during the gap: the exchange flow plus the net evolved gas that must be vented to hold 1 atm. Floored at zero — when fixation outpaces evolution the headspace merely sags, nothing leaves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace turnovers per gap — growth</t>
+        </is>
+      </c>
+      <c r="B332" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x_hs_g</t>
+        </is>
+      </c>
+      <c r="C332" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D332" s="48">
+        <f>F_gap_g*t_gap_h/n_hs_gas</f>
+        <v>0.0</v>
+      </c>
+      <c r="E332" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dimensionless gap length for the headspace ramp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Φ(x) = (1−e^−x)/x — growth</t>
+        </is>
+      </c>
+      <c r="B333" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phi_hs_g</t>
+        </is>
+      </c>
+      <c r="C333" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D333" s="48">
+        <f>IF(x_hs_g&gt;0,(1-EXP(-x_hs_g))/x_hs_g,1)</f>
+        <v>1.0</v>
+      </c>
+      <c r="E333" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exponential-ramp helper; the limit at x → 0 is 1, which keeps the slow-vent case singularity-free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ψ(x) = (x−1+e^−x)/x² — growth</t>
+        </is>
+      </c>
+      <c r="B334" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">psi_hs_g</t>
+        </is>
+      </c>
+      <c r="C334" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D334" s="48">
+        <f>IF(x_hs_g&gt;0,(x_hs_g-1+EXP(-x_hs_g))/x_hs_g^2,1/2)</f>
+        <v>0.5</v>
+      </c>
+      <c r="E334" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean helper for the same ramp; the limit at x → 0 is ½ (mean of a linear ramp).</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ rise per gap, undiluted — growth</t>
+        </is>
+      </c>
+      <c r="B335" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dy_O2_g</t>
+        </is>
+      </c>
+      <c r="C335" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D335" s="48">
+        <f>S_O2_g*t_gap_h/n_hs_gas</f>
+        <v>0.031539212614</v>
+      </c>
+      <c r="E335" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ fraction gained over one gap if nothing left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ just before a pulse — growth</t>
+        </is>
+      </c>
+      <c r="B336" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_end_g</t>
+        </is>
+      </c>
+      <c r="C336" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D336" s="48">
+        <f>dy_O2_g*phi_hs_g/(1-flush_ret*EXP(-x_hs_g))</f>
+        <v>0.049894299708</v>
+      </c>
+      <c r="E336" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Periodic solution of n·dy/dt = S − y·L over the gap with each pulse retaining flush_ret of the headspace: the sawtooth top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ just after a pulse — growth</t>
+        </is>
+      </c>
+      <c r="B337" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_post_g</t>
+        </is>
+      </c>
+      <c r="C337" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D337" s="48">
+        <f>y_O2_end_g*flush_ret</f>
+        <v>0.018355087094</v>
+      </c>
+      <c r="E337" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sawtooth bottom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean headspace O₂ — growth</t>
+        </is>
+      </c>
+      <c r="B338" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_avg_g</t>
+        </is>
+      </c>
+      <c r="C338" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D338" s="48">
+        <f>y_O2_post_g*phi_hs_g+dy_O2_g*psi_hs_g</f>
+        <v>0.034124693401</v>
+      </c>
+      <c r="E338" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact time average of that ramp — what the liquid equilibrates with.</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO excess needed to drive the surface flux — growth</t>
+        </is>
+      </c>
+      <c r="B339" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_surf_excess_g</t>
+        </is>
+      </c>
+      <c r="C339" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D339" s="48">
+        <f>O2_src_g/(kLa_surf_used*3600*V_L_m3)</f>
+        <v>0.040846064617</v>
+      </c>
+      <c r="E339" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flux = kLa·V·(C − C*) on the growth source (companion of D181 for lag).</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field DO — growth</t>
+        </is>
+      </c>
+      <c r="B340" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_mf_g</t>
+        </is>
+      </c>
+      <c r="C340" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D340" s="48">
+        <f>DO_surf_excess_g+H_O2_T*P_atm*y_O2_mf_g</f>
+        <v>0.079316092899</v>
+      </c>
+      <c r="E340" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface excess plus Henry equilibrium with the flux-mean headspace: the quantity the sizing (D184) holds at DO_target ÷ saw_factor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — growth</t>
+        </is>
+      </c>
+      <c r="B341" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_avg_g</t>
+        </is>
+      </c>
+      <c r="C341" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D341" s="48">
+        <f>DO_surf_excess_g+H_O2_T*P_atm*y_O2_avg_g</f>
+        <v>0.082338279323</v>
+      </c>
+      <c r="E341" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface excess plus equilibrium with the TIME-mean headspace: the time-mean of the liquid is exactly this (linear liquid balance).</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — growth</t>
+        </is>
+      </c>
+      <c r="B342" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_g</t>
+        </is>
+      </c>
+      <c r="C342" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D342" s="48">
+        <f>DO_surf_excess_g+H_O2_T*P_atm*MAX(y_O2_avg_g,y_O2_end_g-(S_O2_g-F_gap_g*y_O2_end_g)/n_hs_gas*tau_L_h)</f>
+        <v>0.094535887493</v>
+      </c>
+      <c r="E342" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid DO just before a pulse: the headspace top minus the lag of a first-order liquid (τ = 1/kLa) behind the end-of-gap ramp slope. Quasi-steady approximation, valid while the gap ≫ τ; floored at the cycle mean. Time-stepped check: within 4 % of the limit-cycle ODE in all four vent/phase cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — growth (mg/L)</t>
+        </is>
+      </c>
+      <c r="B343" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_avg_g_mgL</t>
+        </is>
+      </c>
+      <c r="C343" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D343" s="48">
+        <f>DO_avg_g*M_O2</f>
+        <v>2.634660261764</v>
+      </c>
+      <c r="E343" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For the Summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — growth (mg/L)</t>
+        </is>
+      </c>
+      <c r="B344" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_g_mgL</t>
+        </is>
+      </c>
+      <c r="C344" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D344" s="48">
+        <f>DO_peak_g*M_O2</f>
+        <v>3.024959328002</v>
+      </c>
+      <c r="E344" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For the Summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface kLa required at the target DO — growth</t>
+        </is>
+      </c>
+      <c r="B345" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa_surf_req_g</t>
+        </is>
+      </c>
+      <c r="C345" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/s</t>
+        </is>
+      </c>
+      <c r="D345" s="48">
+        <f>O2_src_g/(DO_target*3600*V_L_m3)</f>
+        <v>0.003566106821</v>
+      </c>
+      <c r="E345" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Below this no sparge interval can hold the target on this source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa feasibility margin — growth</t>
+        </is>
+      </c>
+      <c r="B346" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa_margin_g</t>
+        </is>
+      </c>
+      <c r="C346" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">×</t>
+        </is>
+      </c>
+      <c r="D346" s="48">
+        <f>kLa_surf_used/kLa_surf_req_g</f>
+        <v>2.019037572031</v>
+      </c>
+      <c r="E346" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa in use ÷ kLa required. Below 1 the target is unreachable on this phase at any interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO target reachable? — growth</t>
+        </is>
+      </c>
+      <c r="B347" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_feas_g</t>
+        </is>
+      </c>
+      <c r="C347" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D347" s="28" t="str">
+        <f>IF(kLa_margin_g&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)")</f>
+        <v>reachable – kLa margin 2.02×</v>
+      </c>
+      <c r="E347" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feasibility verdict for this phase, independent of which phase the schedule is sized on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO vs inhibition ceiling — growth</t>
+        </is>
+      </c>
+      <c r="B348" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_chk_g</t>
+        </is>
+      </c>
+      <c r="C348" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D348" s="28" t="str">
+        <f>IF(DO_peak_g&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
+        <v>peak 3.0 mg/L under the 11.7 mg/L ceiling</v>
+      </c>
+      <c r="E348" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The sawtooth peak against the growth-inhibition ceiling (Biology D27). Not a tautology: the peak is not what the schedule is sized on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ inflow — lag</t>
+        </is>
+      </c>
+      <c r="B349" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S_O2_l</t>
+        </is>
+      </c>
+      <c r="C349" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D349" s="48">
+        <f>O2_src_l+y_O2_air*F_vent_ex</f>
+        <v>4.979033518202e-05</v>
+      </c>
+      <c r="E349" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ entering the headspace: from the liquid (the whole source must leave this way at steady state) plus the O₂ in any exchanged air.</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Net vent outflow, cycle mean — lag</t>
+        </is>
+      </c>
+      <c r="B350" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_hs_net_l</t>
+        </is>
+      </c>
+      <c r="C350" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D350" s="48">
+        <f>CO2_supply+O2_src_l+H2_src_l-CO2_fix_l</f>
+        <v>0.0006545384575436</v>
+      </c>
+      <c r="E350" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Everything entering the headspace over a cycle minus the fixation sink: the gas that must leave through the vent on average.</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field headspace O₂ — lag</t>
+        </is>
+      </c>
+      <c r="B351" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_mf_l</t>
+        </is>
+      </c>
+      <c r="C351" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D351" s="48">
+        <f>IF(F_vent_ex+F_hs_net_l&gt;0,S_O2_l/(F_vent_ex+F_hs_net_l),NA())</f>
+        <v>0.076069380811</v>
+      </c>
+      <c r="E351" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ONE headspace balance, flux-weighted: O₂ in ÷ all gas out (vent outflow plus exchange). Reduces to O₂/(O₂+CO₂) with no exchange, no H₂ and no fixation — the old D187. Biology D85 is the same balance on the lag source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field headspace H₂ — lag</t>
+        </is>
+      </c>
+      <c r="B352" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_H2_mf_l</t>
+        </is>
+      </c>
+      <c r="C352" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D352" s="48">
+        <f>IF(F_vent_ex+F_hs_net_l&gt;0,H2_src_l/(F_vent_ex+F_hs_net_l),NA())</f>
+        <v>0.155418629263</v>
+      </c>
+      <c r="E352" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same balance for H₂ (Biology D84 on the lag source).</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas leaving between pulses — lag</t>
+        </is>
+      </c>
+      <c r="B353" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_gap_l</t>
+        </is>
+      </c>
+      <c r="C353" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D353" s="48">
+        <f>F_vent_ex+MAX(0,O2_src_l+H2_src_l-CO2_fix_l)</f>
+        <v>0.0001515178050535</v>
+      </c>
+      <c r="E353" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">What leaves the headspace during the gap: the exchange flow plus the net evolved gas that must be vented to hold 1 atm. Floored at zero — when fixation outpaces evolution the headspace merely sags, nothing leaves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace turnovers per gap — lag</t>
+        </is>
+      </c>
+      <c r="B354" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x_hs_l</t>
+        </is>
+      </c>
+      <c r="C354" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D354" s="48">
+        <f>F_gap_l*t_gap_h/n_hs_gas</f>
+        <v>0.300906651909</v>
+      </c>
+      <c r="E354" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dimensionless gap length for the headspace ramp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Φ(x) = (1−e^−x)/x — lag</t>
+        </is>
+      </c>
+      <c r="B355" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phi_hs_l</t>
+        </is>
+      </c>
+      <c r="C355" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D355" s="48">
+        <f>IF(x_hs_l&gt;0,(1-EXP(-x_hs_l))/x_hs_l,1)</f>
+        <v>0.863567280859</v>
+      </c>
+      <c r="E355" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exponential-ramp helper; the limit at x → 0 is 1, which keeps the slow-vent case singularity-free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ψ(x) = (x−1+e^−x)/x² — lag</t>
+        </is>
+      </c>
+      <c r="B356" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">psi_hs_l</t>
+        </is>
+      </c>
+      <c r="C356" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D356" s="48">
+        <f>IF(x_hs_l&gt;0,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2)</f>
+        <v>0.453405460715</v>
+      </c>
+      <c r="E356" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean helper for the same ramp; the limit at x → 0 is ½ (mean of a linear ramp).</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ rise per gap, undiluted — lag</t>
+        </is>
+      </c>
+      <c r="B357" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dy_O2_l</t>
+        </is>
+      </c>
+      <c r="C357" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D357" s="48">
+        <f>S_O2_l*t_gap_h/n_hs_gas</f>
+        <v>0.098881072437</v>
+      </c>
+      <c r="E357" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ fraction gained over one gap if nothing left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ just before a pulse — lag</t>
+        </is>
+      </c>
+      <c r="B358" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_end_l</t>
+        </is>
+      </c>
+      <c r="C358" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D358" s="48">
+        <f>dy_O2_l*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
+        <v>0.117340493152</v>
+      </c>
+      <c r="E358" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Periodic solution of n·dy/dt = S − y·L over the gap with each pulse retaining flush_ret of the headspace: the sawtooth top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ just after a pulse — lag</t>
+        </is>
+      </c>
+      <c r="B359" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_post_l</t>
+        </is>
+      </c>
+      <c r="C359" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D359" s="48">
+        <f>y_O2_end_l*flush_ret</f>
+        <v>0.043167155048</v>
+      </c>
+      <c r="E359" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sawtooth bottom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean headspace O₂ — lag</t>
+        </is>
+      </c>
+      <c r="B360" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_avg_l</t>
+        </is>
+      </c>
+      <c r="C360" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D360" s="48">
+        <f>y_O2_post_l*phi_hs_l+dy_O2_l*psi_hs_l</f>
+        <v>0.082110960911</v>
+      </c>
+      <c r="E360" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact time average of that ramp — what the liquid equilibrates with.</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field DO — lag</t>
+        </is>
+      </c>
+      <c r="B361" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_mf_l</t>
+        </is>
+      </c>
+      <c r="C361" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D361" s="48">
+        <f>DO_surf_excess_lag+H_O2_T*P_atm*y_O2_mf_l</f>
+        <v>0.220552478156</v>
+      </c>
+      <c r="E361" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface excess plus Henry equilibrium with the flux-mean headspace: the quantity the sizing (D184) holds at DO_target ÷ saw_factor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — lag</t>
+        </is>
+      </c>
+      <c r="B362" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_avg_l</t>
+        </is>
+      </c>
+      <c r="C362" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D362" s="48">
+        <f>DO_surf_excess_lag+H_O2_T*P_atm*y_O2_avg_l</f>
+        <v>0.227898435401</v>
+      </c>
+      <c r="E362" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface excess plus equilibrium with the TIME-mean headspace: the time-mean of the liquid is exactly this (linear liquid balance).</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — lag</t>
+        </is>
+      </c>
+      <c r="B363" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_l</t>
+        </is>
+      </c>
+      <c r="C363" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D363" s="48">
+        <f>DO_surf_excess_lag+H_O2_T*P_atm*MAX(y_O2_avg_l,y_O2_end_l-(S_O2_l-F_gap_l*y_O2_end_l)/n_hs_gas*tau_L_h)</f>
+        <v>0.256671410883</v>
+      </c>
+      <c r="E363" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid DO just before a pulse: the headspace top minus the lag of a first-order liquid (τ = 1/kLa) behind the end-of-gap ramp slope. Quasi-steady approximation, valid while the gap ≫ τ; floored at the cycle mean. Time-stepped check: within 4 % of the limit-cycle ODE in all four vent/phase cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — lag (mg/L)</t>
+        </is>
+      </c>
+      <c r="B364" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_avg_l_mgL</t>
+        </is>
+      </c>
+      <c r="C364" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D364" s="48">
+        <f>DO_avg_l*M_O2</f>
+        <v>7.292294135948</v>
+      </c>
+      <c r="E364" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For the Summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — lag (mg/L)</t>
+        </is>
+      </c>
+      <c r="B365" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_l_mgL</t>
+        </is>
+      </c>
+      <c r="C365" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D365" s="48">
+        <f>DO_peak_l*M_O2</f>
+        <v>8.21297180544</v>
+      </c>
+      <c r="E365" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">For the Summary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Surface kLa required at the target DO — lag</t>
+        </is>
+      </c>
+      <c r="B366" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa_surf_req_l</t>
+        </is>
+      </c>
+      <c r="C366" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/s</t>
+        </is>
+      </c>
+      <c r="D366" s="48">
+        <f>O2_src_l/(DO_target*3600*V_L_m3)</f>
+        <v>0.011180382694</v>
+      </c>
+      <c r="E366" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Below this no sparge interval can hold the target on this source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa feasibility margin — lag</t>
+        </is>
+      </c>
+      <c r="B367" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa_margin_l</t>
+        </is>
+      </c>
+      <c r="C367" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">×</t>
+        </is>
+      </c>
+      <c r="D367" s="48">
+        <f>kLa_surf_used/kLa_surf_req_l</f>
+        <v>0.643994383246</v>
+      </c>
+      <c r="E367" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kLa in use ÷ kLa required. Below 1 the target is unreachable on this phase at any interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO target reachable? — lag</t>
+        </is>
+      </c>
+      <c r="B368" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_feas_l</t>
+        </is>
+      </c>
+      <c r="C368" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D368" s="28" t="str">
+        <f>IF(kLa_margin_l&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)")</f>
+        <v>UNREACHABLE at this surface kLa – margin 0.64× (raise kL_surf, lower the current, or accept a higher DO)</v>
+      </c>
+      <c r="E368" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feasibility verdict for this phase, independent of which phase the schedule is sized on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO vs inhibition ceiling — lag</t>
+        </is>
+      </c>
+      <c r="B369" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_chk_l</t>
+        </is>
+      </c>
+      <c r="C369" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D369" s="28" t="str">
+        <f>IF(DO_peak_l&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
+        <v>peak 8.2 mg/L under the 11.7 mg/L ceiling</v>
+      </c>
+      <c r="E369" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The sawtooth peak against the growth-inhibition ceiling (Biology D27). Not a tautology: the peak is not what the schedule is sized on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas leaving between pulses — sizing phase</t>
+        </is>
+      </c>
+      <c r="B371" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_gap_sched</t>
+        </is>
+      </c>
+      <c r="C371" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D371" s="48">
+        <f>IF(O2_sizing_phase=phase_name_1,F_gap_g,IF(O2_sizing_phase=phase_name_2,F_gap_l,NA()))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E371" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeds the headspace turnover k_vent (D143) and hence the CO₂ pool decay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — sizing phase</t>
+        </is>
+      </c>
+      <c r="B372" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_avg_sched</t>
+        </is>
+      </c>
+      <c r="C372" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D372" s="48">
+        <f>IF(O2_sizing_phase=phase_name_1,DO_avg_g,IF(O2_sizing_phase=phase_name_2,DO_avg_l,NA()))</f>
+        <v>0.082338279323</v>
+      </c>
+      <c r="E372" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeds D108 (DO_ss).</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — sizing phase</t>
+        </is>
+      </c>
+      <c r="B373" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_sched</t>
+        </is>
+      </c>
+      <c r="C373" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D373" s="48">
+        <f>IF(O2_sizing_phase=phase_name_1,DO_peak_g,IF(O2_sizing_phase=phase_name_2,DO_peak_l,NA()))</f>
+        <v>0.094535887493</v>
+      </c>
+      <c r="E373" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeds the organism-band check below and Summary D21.</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO vs organism band — sizing phase</t>
+        </is>
+      </c>
+      <c r="B374" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_band</t>
+        </is>
+      </c>
+      <c r="C374" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D374" s="28" t="str">
+        <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_impair)),IF(DO_peak_sched*M_O2&lt;=DO_opt,"peak at/under optimum",IF(DO_peak_sched*M_O2&lt;DO_impair,"peak above optimum, under impairment","PEAK OVER IMPAIRMENT")),IF(DO_peak_sched&lt;=O2_ceil_C,"organism band unknown – peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L is under the inhibition ceiling","organism band unknown – PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER THE INHIBITION CEILING"))</f>
+        <v>organism band unknown – peak 3.0 mg/L is under the inhibition ceiling</v>
+      </c>
+      <c r="E374" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Replaces the tautological D109 as the Summary O₂ check: the sawtooth peak against the organism band, or against the inhibition ceiling when the band is unmeasured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap CO₂ change, slow-vent limit</t>
+        </is>
+      </c>
+      <c r="B375" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool_D_raw</t>
+        </is>
+      </c>
+      <c r="C375" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D375" s="48">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*t_gap_h/(V_L_m3+Vg_CO2)</f>
+        <v>-0.19762042649</v>
+      </c>
+      <c r="E375" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pool concentration change over one gap if the decay were linear: CO₂ carried in by exchanged air (air is 0.04 % CO₂) minus carbon fixed, spread over the liquid plus headspace-equivalent volume. Negative = loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pool turnovers per gap</t>
+        </is>
+      </c>
+      <c r="B376" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool_x</t>
+        </is>
+      </c>
+      <c r="C376" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D376" s="48">
+        <f>k_eff_CO2*t_off_CO2</f>
+        <v>0.0</v>
+      </c>
+      <c r="E376" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_eff·t_gap; pool_e (D197) is exp(−this).</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Φ(x) — pool</t>
+        </is>
+      </c>
+      <c r="B377" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool_phi</t>
+        </is>
+      </c>
+      <c r="C377" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D377" s="48">
+        <f>IF(pool_x&gt;0,(1-EXP(-pool_x))/pool_x,1)</f>
+        <v>1.0</v>
+      </c>
+      <c r="E377" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As phi_hs; limit 1 at x → 0 so an outflow-only growth headspace (nothing vented between pulses) stays singularity-free.</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ψ(x) — pool</t>
+        </is>
+      </c>
+      <c r="B378" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool_psi</t>
+        </is>
+      </c>
+      <c r="C378" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D378" s="48">
+        <f>IF(pool_x&gt;0,(pool_x-1+EXP(-pool_x))/pool_x^2,1/2)</f>
+        <v>0.5</v>
+      </c>
+      <c r="E378" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As psi_hs; limit ½.</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap CO₂ change</t>
+        </is>
+      </c>
+      <c r="B379" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool_D_gap</t>
+        </is>
+      </c>
+      <c r="C379" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D379" s="48">
+        <f>pool_D_raw*pool_phi</f>
+        <v>-0.19762042649</v>
+      </c>
+      <c r="E379" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The asymptote term of the exponential decay, written as D_raw·Φ so it needs no division by k_eff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pool share retained through a pulse</t>
+        </is>
+      </c>
+      <c r="B380" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool_ret</t>
+        </is>
+      </c>
+      <c r="C380" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D380" s="48">
+        <f>pool_a+(1-pool_a)*flush_ret</f>
+        <v>0.889045202649</v>
+      </c>
+      <c r="E380" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The liquid share survives the pulse untouched; of the headspace share, flush_ret survives the well-mixed flush. Replaces the hard-coded full displacement (R2-m3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field headspace CO₂ — sizing phase (cross-check)</t>
+        </is>
+      </c>
+      <c r="B381" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_CO2_mf</t>
+        </is>
+      </c>
+      <c r="C381" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D381" s="48">
+        <f>IF(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_atm*F_vent_ex)/(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
+        <v>0.968360861681</v>
+      </c>
+      <c r="E381" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The same flux balance as y_O2_mf, for CO₂. Diagnostic: the pool model (D198–D200) and this should agree to within the sawtooth; 96 % CO₂ in "Outflow only" at the optimal schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field dissolved CO₂ (cross-check)</t>
+        </is>
+      </c>
+      <c r="B382" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C_CO2_mf</t>
+        </is>
+      </c>
+      <c r="C382" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D382" s="48">
+        <f>y_CO2_mf*C_sat_CO2</f>
+        <v>32.379324222241</v>
+      </c>
+      <c r="E382" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Henry equilibrium with the flux-mean headspace CO₂; compare with CO2_cyc_avg_new (D200).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: open-vent option and default (9.0 min, pH 6.19), selector #N/A guards, peak-vs-impairment DO test; wave-5 review record and backlog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -117,13 +117,11 @@
     <definedName name="DO_ss_sawtooth" localSheetId="5">'Mass Transfer'!$D$133</definedName>
     <definedName name="DO_ss_sawtooth_lag" localSheetId="5">'Mass Transfer'!$D$135</definedName>
     <definedName name="DO_ss_vs_min" localSheetId="5">'Mass Transfer'!$D$110</definedName>
-    <definedName name="DO_ss_vs_opt" localSheetId="5">'Mass Transfer'!$D$109</definedName>
     <definedName name="DO_surf_excess" localSheetId="5">'Mass Transfer'!$D$180</definedName>
     <definedName name="DO_surf_excess_lag" localSheetId="5">'Mass Transfer'!$D$181</definedName>
     <definedName name="DO_target" localSheetId="5">'Mass Transfer'!$D$179</definedName>
     <definedName name="DO_toxic" localSheetId="4">Biology!$D$48</definedName>
     <definedName name="DO_toxic" localSheetId="5">'Mass Transfer'!$D$24</definedName>
-    <definedName name="DO_vent_eq" localSheetId="5">'Mass Transfer'!$D$76</definedName>
     <definedName name="dur_ok" localSheetId="5">'Mass Transfer'!$D$130</definedName>
     <definedName name="duty" localSheetId="5">'Mass Transfer'!$D$105</definedName>
     <definedName name="duty_actual" localSheetId="5">'Mass Transfer'!$D$93</definedName>
@@ -552,7 +550,6 @@
     <definedName name="xtube_pro" localSheetId="1">Geometry!$D$47</definedName>
     <definedName name="y_O2_actual" localSheetId="5">'Mass Transfer'!$D$187</definedName>
     <definedName name="y_O2_star" localSheetId="5">'Mass Transfer'!$D$183</definedName>
-    <definedName name="y_O2_vent" localSheetId="5">'Mass Transfer'!$D$75</definedName>
     <definedName name="z_e_H2" localSheetId="2">Electrochemistry!$D$16</definedName>
     <definedName name="z_e_O2" localSheetId="2">Electrochemistry!$D$17</definedName>
     <definedName name="z_e_ORR" localSheetId="2">Electrochemistry!$D$27</definedName>
@@ -773,6 +770,16 @@
     <definedName name="y_O2_air_b" localSheetId="4">Biology!$D$112</definedName>
     <definedName name="vent_model_sel" localSheetId="0">Summary!$D$111</definedName>
     <definedName name="O2_phase_sel" localSheetId="0">Summary!$D$112</definedName>
+    <definedName name="vent_name_3" localSheetId="5">'Mass Transfer'!$D$384</definedName>
+    <definedName name="Q_backdraw" localSheetId="5">'Mass Transfer'!$D$385</definedName>
+    <definedName name="Q_vent_used" localSheetId="5">'Mass Transfer'!$D$386</definedName>
+    <definedName name="H2_HOR_mt" localSheetId="5">'Mass Transfer'!$D$387</definedName>
+    <definedName name="H2_src_l_b" localSheetId="4">Biology!$D$113</definedName>
+    <definedName name="y_H2_end_l" localSheetId="5">'Mass Transfer'!$D$388</definedName>
+    <definedName name="y_H2_end_b" localSheetId="4">Biology!$D$114</definedName>
+    <definedName name="hs_sag" localSheetId="5">'Mass Transfer'!$D$389</definedName>
+    <definedName name="hs_sag_max" localSheetId="5">'Mass Transfer'!$D$390</definedName>
+    <definedName name="hs_sag_chk" localSheetId="5">'Mass Transfer'!$D$391</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8370,8 +8377,9 @@
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="89" t="s">
-        <v>66</v>
+      <c r="A15" s="89" t="str">
+        <f>"CO₂ sparge interval ("&amp;vent_model_sel&amp;", sized on "&amp;O2_phase_sel&amp;")"</f>
+        <v>CO₂ sparge interval (Open vent, sized on Growth)</v>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
@@ -8383,7 +8391,7 @@
       </c>
       <c r="D15" s="90">
         <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$91)</f>
-        <v>12.736715659111</v>
+        <v>9.026013902172</v>
       </c>
       <c r="E15" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
@@ -8412,7 +8420,7 @@
       </c>
       <c r="D16" s="91">
         <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,ROUND(D14/(60*'Mass Transfer'!$D$93),0)))</f>
-        <v>13.0</v>
+        <v>9.0</v>
       </c>
       <c r="E16" s="92"/>
       <c r="F16" s="21" t="inlineStr">
@@ -8494,7 +8502,7 @@
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peak O₂ within the organism band?</t>
+          <t xml:space="preserve">O₂ within the organism band (mean vs optimum, peak vs impairment)?</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
@@ -8505,7 +8513,7 @@
       <c r="C21" s="20"/>
       <c r="D21" s="90" t="str">
         <f>'Mass Transfer'!$D$374</f>
-        <v>organism band unknown – peak 3.0 mg/L is under the inhibition ceiling</v>
+        <v>organism band unknown – peak 2.9 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E21" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D374","→ Mass Transfer")</f>
@@ -8513,7 +8521,7 @@
       </c>
       <c r="F21" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sawtooth PEAK dissolved O₂ (just before a pulse, sizing phase) against the organism optimum / impairment, or against the inhibition ceiling when the band is unmeasured. Not a tautology: the schedule is sized on the cycle mean, not the peak.</t>
+          <t xml:space="preserve">Rule (owner decision, option a): the cycle-MEAN dissolved O₂ is tested against the organism optimum — the schedule is sized on the mean, and the optimum is a time-averaged quantity — and the sawtooth PEAK (just before a pulse, sizing phase) against the impairment threshold. With the band unmeasured, the peak is tested against the inhibition ceiling. Not a tautology: the peak is not what the schedule is sized on.</t>
         </is>
       </c>
     </row>
@@ -8553,7 +8561,7 @@
       <c r="C23" s="20"/>
       <c r="D23" s="90" t="str">
         <f>'Mass Transfer'!$D$113</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 20.1 mg/L against a 2.6 mg/L target</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) the cycle-mean DO would be ≈16 mg/L, above the 11.7 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E23" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
@@ -8579,7 +8587,7 @@
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 16%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 18% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="23" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -8625,7 +8633,7 @@
       <c r="C26" s="20"/>
       <c r="D26" s="90" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)"),"calibrate this reactor first")</f>
-        <v>×29.7 OK</v>
+        <v>×41.9 OK</v>
       </c>
       <c r="E26" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
@@ -8825,7 +8833,7 @@
       <c r="C35" s="20"/>
       <c r="D35" s="121">
         <f>Chemistry!$D$220</f>
-        <v>6.164822774553</v>
+        <v>6.187122404381</v>
       </c>
       <c r="E35" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -8851,7 +8859,7 @@
       </c>
       <c r="D36" s="121">
         <f>Chemistry!$D$226</f>
-        <v>0.339344361561</v>
+        <v>0.339282500863</v>
       </c>
       <c r="E36" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
@@ -8889,7 +8897,7 @@
       </c>
       <c r="D38" s="90">
         <f>'Mass Transfer'!$D$108</f>
-        <v>2.634660261764</v>
+        <v>2.634776001183</v>
       </c>
       <c r="E38" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D108","→ Mass")</f>
@@ -8969,7 +8977,7 @@
       </c>
       <c r="D41" s="95">
         <f>Biology!$D$98</f>
-        <v>633.123209647745</v>
+        <v>594.524480534657</v>
       </c>
       <c r="E41" s="23" t="str">
         <f>HYPERLINK("#Biology!D98","→ Biology")</f>
@@ -9739,7 +9747,7 @@
       </c>
       <c r="D87" s="22">
         <f>Chemistry!$D$209</f>
-        <v>-0.427527364769</v>
+        <v>-0.427526934687</v>
       </c>
       <c r="E87" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D209","→ Chemistry")</f>
@@ -9765,7 +9773,7 @@
       </c>
       <c r="D88" s="22">
         <f>Chemistry!$D$211</f>
-        <v>1.266535517225</v>
+        <v>1.265216285627</v>
       </c>
       <c r="E88" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
@@ -9791,7 +9799,7 @@
       </c>
       <c r="D89" s="22">
         <f>Chemistry!$D$220</f>
-        <v>6.164822774553</v>
+        <v>6.187122404381</v>
       </c>
       <c r="E89" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -9872,7 +9880,7 @@
       </c>
       <c r="D95" s="95">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),D14/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (see CO2 flows)")</f>
-        <v>0.999088398707</v>
+        <v>1.022688337739</v>
       </c>
       <c r="E95" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
@@ -9909,7 +9917,7 @@
       </c>
       <c r="D111" s="131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Outflow only</t>
+          <t xml:space="preserve">Open vent</t>
         </is>
       </c>
       <c r="E111" s="20" t="inlineStr">
@@ -9919,7 +9927,7 @@
       </c>
       <c r="F111" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Outflow only" = gas leaves through the vent, none enters between pulses (check valve / sealed cap). "Air exchange" = room air exchanges with the headspace at Q_vent (Mass Transfer D142, unmeasured). Anything else → #N/A throughout. Default pending the vent-hardware answer; it moves the pH and the lag DO materially.</t>
+          <t xml:space="preserve">"Outflow only" = check valve or sealed cap that holds a vacuum (no air ever enters). "Open vent" = a plain needle or tube with no forced flow (air is drawn back after each pulse; Q_backdraw, Mass Transfer D385, an estimate). "Air exchange" = measured bidirectional exchange at Q_vent (Mass Transfer D142). Unsure → Open vent. Anything else → #N/A throughout. The choice moves the interval and the lag DO materially; the pH much less.</t>
         </is>
       </c>
     </row>
@@ -9951,32 +9959,32 @@
       </c>
       <c r="F112" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Growth" sizes the sparge interval on the O₂ surplus after knallgas uptake; "Lag" on the whole net electrolytic O₂ plus H₂ (no uptake yet). Anything else → #N/A. Both phases are reported below whichever is chosen; "Lag" is currently unreachable at the estimated surface kLa, so the schedule falls back to the O₂ flush interval.</t>
+          <t xml:space="preserve">"Growth" sizes the sparge interval on the O₂ surplus after knallgas uptake; "Lag" on the whole net electrolytic O₂ plus H₂ (no uptake yet). Anything else → #N/A. Both phases are reported below whichever is chosen. If the chosen phase's DO target is unreachable (rows 120–121), the schedule falls back to the legacy O₂ flush guard (Mass Transfer D89), which is not derived from the headspace balance and does not respond to the vent model.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vent air-exchange flow in use</t>
+          <t xml:space="preserve">Vent air ingress in use</t>
         </is>
       </c>
       <c r="C113" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">mol/h</t>
+          <t xml:space="preserve">mL/min</t>
         </is>
       </c>
       <c r="D113" s="90">
-        <f>'Mass Transfer'!$D$308</f>
-        <v>0.0</v>
+        <f>'Mass Transfer'!$D$386</f>
+        <v>0.015</v>
       </c>
       <c r="E113" s="23" t="str">
-        <f>HYPERLINK("#'Mass Transfer'!D308","→ Mass Transfer")</f>
+        <f>HYPERLINK("#'Mass Transfer'!D386","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
       <c r="F113" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zero for "Outflow only"; Q_vent converted for "Air exchange". The single number that reconciles the O₂, CO₂ and flammability blocks — measure it.</t>
+          <t xml:space="preserve">0 for "Outflow only"; Q_backdraw (Mass Transfer D385, an estimate) for "Open vent"; the measured Q_vent (D142) for "Air exchange". The single number that reconciles the O₂, CO₂ and flammability blocks — measure it.</t>
         </is>
       </c>
     </row>
@@ -9993,7 +10001,7 @@
       </c>
       <c r="D114" s="90">
         <f>'Mass Transfer'!$D$343</f>
-        <v>2.634660261764</v>
+        <v>2.634776001183</v>
       </c>
       <c r="E114" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D343","→ Mass Transfer")</f>
@@ -10018,7 +10026,7 @@
       </c>
       <c r="D115" s="90">
         <f>'Mass Transfer'!$D$344</f>
-        <v>3.024959328002</v>
+        <v>2.934788844069</v>
       </c>
       <c r="E115" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D344","→ Mass Transfer")</f>
@@ -10043,7 +10051,7 @@
       </c>
       <c r="D116" s="90">
         <f>'Mass Transfer'!$D$364</f>
-        <v>7.292294135948</v>
+        <v>6.785801971106</v>
       </c>
       <c r="E116" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
@@ -10068,7 +10076,7 @@
       </c>
       <c r="D117" s="90">
         <f>'Mass Transfer'!$D$365</f>
-        <v>8.21297180544</v>
+        <v>7.403376944733</v>
       </c>
       <c r="E117" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D365","→ Mass Transfer")</f>
@@ -10088,7 +10096,7 @@
       </c>
       <c r="D118" s="90" t="str">
         <f>'Mass Transfer'!$D$348</f>
-        <v>peak 3.0 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 2.9 mg/L under the 11.7 mg/L ceiling</v>
       </c>
       <c r="E118" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D348","→ Mass Transfer")</f>
@@ -10108,7 +10116,7 @@
       </c>
       <c r="D119" s="90" t="str">
         <f>'Mass Transfer'!$D$369</f>
-        <v>peak 8.2 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 7.4 mg/L under the 11.7 mg/L ceiling</v>
       </c>
       <c r="E119" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D369","→ Mass Transfer")</f>
@@ -10154,10 +10162,9 @@
         <f>HYPERLINK("#'Mass Transfer'!D368","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F121" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Same on the lag source (3.3× larger). Currently 0.65×: the target cannot be held during lag at the estimated kLa, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</t>
-        </is>
+      <c r="F121" s="21" t="str">
+        <f>"Same on the lag source. Currently "&amp;TEXT('Mass Transfer'!$D$367,"0.00")&amp;"×: "&amp;IF('Mass Transfer'!$D$367&lt;1,"the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).","the target can be held during lag at the kLa in use.")</f>
+        <v>Same on the lag source. Currently 0.64×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
       </c>
     </row>
     <row r="122">
@@ -10213,7 +10220,7 @@
     <row r="124">
       <c r="A124" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Headspace O₂ fraction (mean-field) — growth</t>
+          <t xml:space="preserve">Headspace O₂ fraction (flux-mean; the headspace swings around it) — growth</t>
         </is>
       </c>
       <c r="C124" s="20" t="inlineStr">
@@ -10248,7 +10255,7 @@
       </c>
       <c r="D125" s="90">
         <f>'Mass Transfer'!$D$351</f>
-        <v>0.076069380811</v>
+        <v>0.064019231488</v>
       </c>
       <c r="E125" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D351","→ Mass Transfer")</f>
@@ -10273,7 +10280,7 @@
       </c>
       <c r="D126" s="90">
         <f>'Mass Transfer'!$D$352</f>
-        <v>0.155418629263</v>
+        <v>0.113266761861</v>
       </c>
       <c r="E126" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D352","→ Mass Transfer")</f>
@@ -10298,7 +10305,7 @@
       </c>
       <c r="D127" s="90">
         <f>'Mass Transfer'!$D$381</f>
-        <v>0.968360861681</v>
+        <v>0.929374836165</v>
       </c>
       <c r="E127" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D381","→ Mass Transfer")</f>
@@ -10306,7 +10313,7 @@
       </c>
       <c r="F127" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">What the vent model implies for the CO₂ the pH rests on: ~96 % for "Outflow only", lower with air exchange. The pool model (Mass Transfer D200) should agree within the sawtooth.</t>
+          <t xml:space="preserve">What the vent model implies for the CO₂ the pH rests on: ~97 % for "Outflow only", lower when air enters ("Open vent", "Air exchange"). The pool model (Mass Transfer D200) should agree within the sawtooth.</t>
         </is>
       </c>
     </row>
@@ -10317,8 +10324,8 @@
         </is>
       </c>
       <c r="D128" s="90" t="str">
-        <f>IF(NOT(ISNUMBER('Mass Transfer'!$D$185)),"DO target unreachable on the sizing phase (rows 120–121) – the schedule is the O₂ flush fallback",IF(Chemistry!$D$220&gt;=Chemistry!$D$236,"yes – the schedule holds the DO target at pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", within the band","NO – holding the DO target drives pH to "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor"))</f>
-        <v>NO – holding the DO target drives pH to 6.16, below the 6.5 band floor</v>
+        <f>IF(ISNA('Mass Transfer'!$D$308+'Mass Transfer'!$D$317),"#N/A – check the selectors in D111/D112",IF(NOT(ISNUMBER('Mass Transfer'!$D$185)),"DO target unreachable on the sizing phase (rows 120–121) – the schedule is the legacy O₂ flush guard (Mass Transfer D89)",IF(Chemistry!$D$220&gt;=Chemistry!$D$236,"yes – the schedule holds the DO target at pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", within the band",IF('Mass Transfer'!$D$185&lt;='Mass Transfer'!$D$112,"NO – holding the DO target drives pH to "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor","NO – the carbon-limited interval (not the DO target) gives pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor"))))</f>
+        <v>NO – holding the DO target drives pH to 6.19, below the 6.5 band floor</v>
       </c>
       <c r="E128" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -10326,7 +10333,52 @@
       </c>
       <c r="F128" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">The vent model couples the two: CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH. Red means the two targets conflict under the vent model in use — decouple them (inert sweep) or measure the vent before trusting either.</t>
+          <t xml:space="preserve">The vent model couples the two: when O₂ dilution binds, CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH (the text says which constraint binds). Red means the two targets conflict under the vent model in use — decouple them (inert sweep) or measure the vent before trusting either. #N/A = a selector in D111/D112 is not a listed value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace sag per cycle if the vent held a vacuum</t>
+        </is>
+      </c>
+      <c r="C129" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D129" s="90">
+        <f>'Mass Transfer'!$D$389</f>
+        <v>0.059351496276</v>
+      </c>
+      <c r="E129" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D389","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F129" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upper bound on the per-cycle pressure deficit (fraction of 1 atm) that the "Outflow only" model implies at the schedule in use; 0.05 = 5 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outflow-only headspace physically plausible?</t>
+        </is>
+      </c>
+      <c r="D130" s="90" t="str">
+        <f>'Mass Transfer'!$D$391</f>
+        <v>n/a – the vent admits air (Open vent / Air exchange), so the headspace refills</v>
+      </c>
+      <c r="E130" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D391","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F130" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"HEADSPACE SAGS" = the check-valve model needs more vacuum than a real cap holds: switch D111 to Open vent or Air exchange. n/a when the vent model already admits air.</t>
         </is>
       </c>
     </row>
@@ -10455,11 +10507,11 @@
       <formula1>80000</formula1>
       <formula2>110000</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose Outflow only or Air exchange." sqref="D111">
-      <formula1>"Outflow only,Air exchange"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose Growth or Lag." sqref="D112">
       <formula1>"Growth,Lag"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose Outflow only, Open vent or Air exchange." sqref="D111">
+      <formula1>"Outflow only,Open vent,Air exchange"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14055,7 +14107,7 @@
       </c>
       <c r="D96" s="141">
         <f>r_H2O2_lag/(k_H2O2_anode*3600)*(1-EXP(-k_H2O2_anode*3600))</f>
-        <v>0.962431861224</v>
+        <v>0.925414707501</v>
       </c>
       <c r="E96" s="67" t="inlineStr">
         <is>
@@ -14092,7 +14144,7 @@
       </c>
       <c r="D98" s="141">
         <f>IF(r_H2O2_lag&gt;0,IF(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag&gt;0,-LN(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag)/k_H2O2_anode/60,NA()),NA())</f>
-        <v>5.084081971057</v>
+        <v>5.305839767983</v>
       </c>
       <c r="E98" s="67" t="inlineStr">
         <is>
@@ -14845,7 +14897,7 @@
       </c>
       <c r="D150" s="141">
         <f>'Mass Transfer'!$D$135</f>
-        <v>0.220552478156</v>
+        <v>0.212069565945</v>
       </c>
       <c r="E150" s="67" t="inlineStr">
         <is>
@@ -14897,7 +14949,7 @@
       </c>
       <c r="D152" s="141">
         <f>r_H2O2*ec_DO_lag/ec_DO_design</f>
-        <v>2.175036167083</v>
+        <v>2.091379701213</v>
       </c>
       <c r="E152" s="67" t="inlineStr">
         <is>
@@ -15014,7 +15066,7 @@
       </c>
       <c r="D5" s="64">
         <f>'Mass Transfer'!$D$162</f>
-        <v>0.031754970696</v>
+        <v>0.029931790408</v>
       </c>
       <c r="E5" s="51" t="inlineStr">
         <is>
@@ -15694,7 +15746,7 @@
       </c>
       <c r="B50" s="64">
         <f t="shared" ref="B50:B81" si="1">pH_SID + pH_NT*(10^-A50)/((10^-A50)+KaN_c) + (10^-A50) - (pH_PT*Ka1p_c*(10^-A50)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A50) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A50)^3 + Ka1p_c*(10^-A50)^2 + Ka1p_c*Ka2p_c*(10^-A50) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A50) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A50)^2 - Kw_c/(10^-A50)</f>
-        <v>0.0330431142</v>
+        <v>0.033056557945</v>
       </c>
       <c r="C50" s="64">
         <f>IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
@@ -15707,7 +15759,7 @@
       </c>
       <c r="B51" s="64">
         <f t="shared" si="1"/>
-        <v>0.032880951431</v>
+        <v>0.032897876114</v>
       </c>
       <c r="C51" s="64">
         <f>IF(AND(B51&gt;=0,B52&lt;0),A51+pH_step*B51/(B51-B52),0)</f>
@@ -15720,7 +15772,7 @@
       </c>
       <c r="B52" s="64">
         <f t="shared" si="1"/>
-        <v>0.032716080079</v>
+        <v>0.03273738701</v>
       </c>
       <c r="C52" s="64">
         <f>IF(AND(B52&gt;=0,B53&lt;0),A52+pH_step*B52/(B52-B53),0)</f>
@@ -15733,7 +15785,7 @@
       </c>
       <c r="B53" s="64">
         <f t="shared" si="1"/>
-        <v>0.032539836383</v>
+        <v>0.032566660249</v>
       </c>
       <c r="C53" s="64">
         <f>IF(AND(B53&gt;=0,B54&lt;0),A53+pH_step*B53/(B53-B54),0)</f>
@@ -15746,7 +15798,7 @@
       </c>
       <c r="B54" s="64">
         <f t="shared" si="1"/>
-        <v>0.032342924182</v>
+        <v>0.032376693474</v>
       </c>
       <c r="C54" s="64">
         <f>IF(AND(B54&gt;=0,B55&lt;0),A54+pH_step*B54/(B54-B55),0)</f>
@@ -15759,7 +15811,7 @@
       </c>
       <c r="B55" s="64">
         <f t="shared" si="1"/>
-        <v>0.032114938725</v>
+        <v>0.032157451816</v>
       </c>
       <c r="C55" s="64">
         <f>IF(AND(B55&gt;=0,B56&lt;0),A55+pH_step*B55/(B55-B56),0)</f>
@@ -15772,7 +15824,7 @@
       </c>
       <c r="B56" s="64">
         <f t="shared" si="1"/>
-        <v>0.031843829825</v>
+        <v>0.031897350748</v>
       </c>
       <c r="C56" s="64">
         <f>IF(AND(B56&gt;=0,B57&lt;0),A56+pH_step*B56/(B56-B57),0)</f>
@@ -15785,7 +15837,7 @@
       </c>
       <c r="B57" s="64">
         <f t="shared" si="1"/>
-        <v>0.031515279296</v>
+        <v>0.031582658325</v>
       </c>
       <c r="C57" s="64">
         <f>IF(AND(B57&gt;=0,B58&lt;0),A57+pH_step*B57/(B57-B58),0)</f>
@@ -15798,7 +15850,7 @@
       </c>
       <c r="B58" s="64">
         <f t="shared" si="1"/>
-        <v>0.031111963448</v>
+        <v>0.031196788903</v>
       </c>
       <c r="C58" s="64">
         <f>IF(AND(B58&gt;=0,B59&lt;0),A58+pH_step*B58/(B58-B59),0)</f>
@@ -15811,7 +15863,7 @@
       </c>
       <c r="B59" s="64">
         <f t="shared" si="1"/>
-        <v>0.030612666373</v>
+        <v>0.030719455744</v>
       </c>
       <c r="C59" s="64">
         <f>IF(AND(B59&gt;=0,B60&lt;0),A59+pH_step*B59/(B59-B60),0)</f>
@@ -15824,7 +15876,7 @@
       </c>
       <c r="B60" s="64">
         <f t="shared" si="1"/>
-        <v>0.029991203856</v>
+        <v>0.030125644421</v>
       </c>
       <c r="C60" s="64">
         <f>IF(AND(B60&gt;=0,B61&lt;0),A60+pH_step*B60/(B60-B61),0)</f>
@@ -15837,7 +15889,7 @@
       </c>
       <c r="B61" s="64">
         <f t="shared" si="1"/>
-        <v>0.029215110835</v>
+        <v>0.029384362607</v>
       </c>
       <c r="C61" s="64">
         <f>IF(AND(B61&gt;=0,B62&lt;0),A61+pH_step*B61/(B61-B62),0)</f>
@@ -15850,7 +15902,7 @@
       </c>
       <c r="B62" s="64">
         <f t="shared" si="1"/>
-        <v>0.028244037616</v>
+        <v>0.028457114762</v>
       </c>
       <c r="C62" s="64">
         <f>IF(AND(B62&gt;=0,B63&lt;0),A62+pH_step*B62/(B62-B63),0)</f>
@@ -15863,7 +15915,7 @@
       </c>
       <c r="B63" s="64">
         <f t="shared" si="1"/>
-        <v>0.027027791439</v>
+        <v>0.027296042508</v>
       </c>
       <c r="C63" s="64">
         <f>IF(AND(B63&gt;=0,B64&lt;0),A63+pH_step*B63/(B63-B64),0)</f>
@@ -15876,7 +15928,7 @@
       </c>
       <c r="B64" s="64">
         <f t="shared" si="1"/>
-        <v>0.025503950695</v>
+        <v>0.025841663275</v>
       </c>
       <c r="C64" s="64">
         <f>IF(AND(B64&gt;=0,B65&lt;0),A64+pH_step*B64/(B64-B65),0)</f>
@@ -15889,7 +15941,7 @@
       </c>
       <c r="B65" s="64">
         <f t="shared" si="1"/>
-        <v>0.023594968898</v>
+        <v>0.024020130969</v>
       </c>
       <c r="C65" s="64">
         <f>IF(AND(B65&gt;=0,B66&lt;0),A65+pH_step*B65/(B65-B66),0)</f>
@@ -15902,7 +15954,7 @@
       </c>
       <c r="B66" s="64">
         <f t="shared" si="1"/>
-        <v>0.021204673541</v>
+        <v>0.021739932163</v>
       </c>
       <c r="C66" s="64">
         <f>IF(AND(B66&gt;=0,B67&lt;0),A66+pH_step*B66/(B66-B67),0)</f>
@@ -15915,7 +15967,7 @@
       </c>
       <c r="B67" s="64">
         <f t="shared" si="1"/>
-        <v>0.018214048916</v>
+        <v>0.018887917484</v>
       </c>
       <c r="C67" s="64">
         <f>IF(AND(B67&gt;=0,B68&lt;0),A67+pH_step*B67/(B67-B68),0)</f>
@@ -15928,7 +15980,7 @@
       </c>
       <c r="B68" s="64">
         <f t="shared" si="1"/>
-        <v>0.014476166764</v>
+        <v>0.015324545379</v>
       </c>
       <c r="C68" s="64">
         <f>IF(AND(B68&gt;=0,B69&lt;0),A68+pH_step*B68/(B68-B69),0)</f>
@@ -15941,7 +15993,7 @@
       </c>
       <c r="B69" s="64">
         <f t="shared" si="1"/>
-        <v>0.009810084505</v>
+        <v>0.010878174835</v>
       </c>
       <c r="C69" s="64">
         <f>IF(AND(B69&gt;=0,B70&lt;0),A69+pH_step*B69/(B69-B70),0)</f>
@@ -15954,11 +16006,11 @@
       </c>
       <c r="B70" s="64">
         <f t="shared" si="1"/>
-        <v>0.003993451907</v>
+        <v>0.005338169177</v>
       </c>
       <c r="C70" s="64">
         <f>IF(AND(B70&gt;=0,B71&lt;0),A70+pH_step*B70/(B70-B71),0)</f>
-        <v>6.055158016113</v>
+        <v>6.077457645941</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -15967,7 +16019,7 @@
       </c>
       <c r="B71" s="64">
         <f t="shared" si="1"/>
-        <v>-0.003246569015</v>
+        <v>-0.001553557408</v>
       </c>
       <c r="C71" s="64">
         <f>IF(AND(B71&gt;=0,B72&lt;0),A71+pH_step*B71/(B71-B72),0)</f>
@@ -15980,7 +16032,7 @@
       </c>
       <c r="B72" s="64">
         <f t="shared" si="1"/>
-        <v>-0.012244684888</v>
+        <v>-0.010113130675</v>
       </c>
       <c r="C72" s="64">
         <f>IF(AND(B72&gt;=0,B73&lt;0),A72+pH_step*B72/(B72-B73),0)</f>
@@ -15993,7 +16045,7 @@
       </c>
       <c r="B73" s="64">
         <f t="shared" si="1"/>
-        <v>-0.02341208673</v>
+        <v>-0.020728335463</v>
       </c>
       <c r="C73" s="64">
         <f>IF(AND(B73&gt;=0,B74&lt;0),A73+pH_step*B73/(B73-B74),0)</f>
@@ -16006,7 +16058,7 @@
       </c>
       <c r="B74" s="64">
         <f t="shared" si="1"/>
-        <v>-0.037255650623</v>
+        <v>-0.033876558634</v>
       </c>
       <c r="C74" s="64">
         <f>IF(AND(B74&gt;=0,B75&lt;0),A74+pH_step*B74/(B74-B75),0)</f>
@@ -16019,7 +16071,7 @@
       </c>
       <c r="B75" s="64">
         <f t="shared" si="1"/>
-        <v>-0.054403539464</v>
+        <v>-0.050148802566</v>
       </c>
       <c r="C75" s="64">
         <f>IF(AND(B75&gt;=0,B76&lt;0),A75+pH_step*B75/(B75-B76),0)</f>
@@ -16032,7 +16084,7 @@
       </c>
       <c r="B76" s="64">
         <f t="shared" si="1"/>
-        <v>-0.07563945145</v>
+        <v>-0.070281926409</v>
       </c>
       <c r="C76" s="64">
         <f>IF(AND(B76&gt;=0,B77&lt;0),A76+pH_step*B76/(B76-B77),0)</f>
@@ -16045,7 +16097,7 @@
       </c>
       <c r="B77" s="64">
         <f t="shared" si="1"/>
-        <v>-0.101948063215</v>
+        <v>-0.095201550021</v>
       </c>
       <c r="C77" s="64">
         <f>IF(AND(B77&gt;=0,B78&lt;0),A77+pH_step*B77/(B77-B78),0)</f>
@@ -16058,7 +16110,7 @@
       </c>
       <c r="B78" s="64">
         <f t="shared" si="1"/>
-        <v>-0.134574371683</v>
+        <v>-0.126078179765</v>
       </c>
       <c r="C78" s="64">
         <f>IF(AND(B78&gt;=0,B79&lt;0),A78+pH_step*B78/(B78-B79),0)</f>
@@ -16071,7 +16123,7 @@
       </c>
       <c r="B79" s="64">
         <f t="shared" si="1"/>
-        <v>-0.175099777725</v>
+        <v>-0.164399212616</v>
       </c>
       <c r="C79" s="64">
         <f>IF(AND(B79&gt;=0,B80&lt;0),A79+pH_step*B79/(B79-B80),0)</f>
@@ -16084,7 +16136,7 @@
       </c>
       <c r="B80" s="64">
         <f t="shared" si="1"/>
-        <v>-0.225538160877</v>
+        <v>-0.2120598263</v>
       </c>
       <c r="C80" s="64">
         <f>IF(AND(B80&gt;=0,B81&lt;0),A80+pH_step*B80/(B80-B81),0)</f>
@@ -16097,7 +16149,7 @@
       </c>
       <c r="B81" s="64">
         <f t="shared" si="1"/>
-        <v>-0.28845620939</v>
+        <v>-0.271476705075</v>
       </c>
       <c r="C81" s="64">
         <f>IF(AND(B81&gt;=0,B82&lt;0),A81+pH_step*B81/(B81-B82),0)</f>
@@ -16110,7 +16162,7 @@
       </c>
       <c r="B82" s="64">
         <f t="shared" ref="B82:B113" si="3">pH_SID + pH_NT*(10^-A82)/((10^-A82)+KaN_c) + (10^-A82) - (pH_PT*Ka1p_c*(10^-A82)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A82) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A82)^3 + Ka1p_c*(10^-A82)^2 + Ka1p_c*Ka2p_c*(10^-A82) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A82) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A82)^2 - Kw_c/(10^-A82)</f>
-        <v>-0.367124145321</v>
+        <v>-0.34573032811</v>
       </c>
       <c r="C82" s="64">
         <f>IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
@@ -16123,7 +16175,7 @@
       </c>
       <c r="B83" s="64">
         <f t="shared" si="3"/>
-        <v>-0.465705811375</v>
+        <v>-0.438744241063</v>
       </c>
       <c r="C83" s="64">
         <f>IF(AND(B83&gt;=0,B84&lt;0),A83+pH_step*B83/(B83-B84),0)</f>
@@ -16136,7 +16188,7 @@
       </c>
       <c r="B84" s="64">
         <f t="shared" si="3"/>
-        <v>-0.58950088085</v>
+        <v>-0.555513342847</v>
       </c>
       <c r="C84" s="64">
         <f>IF(AND(B84&gt;=0,B85&lt;0),A84+pH_step*B84/(B84-B85),0)</f>
@@ -16149,7 +16201,7 @@
       </c>
       <c r="B85" s="64">
         <f t="shared" si="3"/>
-        <v>-0.745256852669</v>
+        <v>-0.702397864982</v>
       </c>
       <c r="C85" s="64">
         <f>IF(AND(B85&gt;=0,B86&lt;0),A85+pH_step*B85/(B85-B86),0)</f>
@@ -16162,7 +16214,7 @@
       </c>
       <c r="B86" s="64">
         <f t="shared" si="3"/>
-        <v>-0.941574953283</v>
+        <v>-0.887505820494</v>
       </c>
       <c r="C86" s="64">
         <f>IF(AND(B86&gt;=0,B87&lt;0),A86+pH_step*B86/(B86-B87),0)</f>
@@ -16175,7 +16227,7 @@
       </c>
       <c r="B87" s="64">
         <f t="shared" si="3"/>
-        <v>-1.189442979033</v>
+        <v>-1.121195096281</v>
       </c>
       <c r="C87" s="64">
         <f>IF(AND(B87&gt;=0,B88&lt;0),A87+pH_step*B87/(B87-B88),0)</f>
@@ -16188,7 +16240,7 @@
       </c>
       <c r="B88" s="64">
         <f t="shared" si="3"/>
-        <v>-1.502940908092</v>
+        <v>-1.416738412478</v>
       </c>
       <c r="C88" s="64">
         <f>IF(AND(B88&gt;=0,B89&lt;0),A88+pH_step*B88/(B88-B89),0)</f>
@@ -16201,7 +16253,7 @@
       </c>
       <c r="B89" s="64">
         <f t="shared" si="3"/>
-        <v>-1.900183935458</v>
+        <v>-1.79121210323</v>
       </c>
       <c r="C89" s="64">
         <f>IF(AND(B89&gt;=0,B90&lt;0),A89+pH_step*B89/(B89-B90),0)</f>
@@ -16214,7 +16266,7 @@
       </c>
       <c r="B90" s="64">
         <f t="shared" si="3"/>
-        <v>-2.404595650325</v>
+        <v>-2.266696117449</v>
       </c>
       <c r="C90" s="64">
         <f>IF(AND(B90&gt;=0,B91&lt;0),A90+pH_step*B90/(B90-B91),0)</f>
@@ -16227,7 +16279,7 @@
       </c>
       <c r="B91" s="64">
         <f t="shared" si="3"/>
-        <v>-3.046646283691</v>
+        <v>-2.871912416818</v>
       </c>
       <c r="C91" s="64">
         <f>IF(AND(B91&gt;=0,B92&lt;0),A91+pH_step*B91/(B91-B92),0)</f>
@@ -16240,7 +16292,7 @@
       </c>
       <c r="B92" s="64">
         <f t="shared" si="3"/>
-        <v>-3.86625489911</v>
+        <v>-3.644489218902</v>
       </c>
       <c r="C92" s="64">
         <f>IF(AND(B92&gt;=0,B93&lt;0),A92+pH_step*B92/(B92-B93),0)</f>
@@ -16253,7 +16305,7 @@
       </c>
       <c r="B93" s="64">
         <f t="shared" si="3"/>
-        <v>-4.916151944852</v>
+        <v>-4.634130477414</v>
       </c>
       <c r="C93" s="64">
         <f>IF(AND(B93&gt;=0,B94&lt;0),A93+pH_step*B93/(B93-B94),0)</f>
@@ -16266,7 +16318,7 @@
       </c>
       <c r="B94" s="64">
         <f t="shared" si="3"/>
-        <v>-6.266648339548</v>
+        <v>-5.907111148118</v>
       </c>
       <c r="C94" s="64">
         <f>IF(AND(B94&gt;=0,B95&lt;0),A94+pH_step*B94/(B94-B95),0)</f>
@@ -16279,7 +16331,7 @@
       </c>
       <c r="B95" s="64">
         <f t="shared" si="3"/>
-        <v>-8.012488474449</v>
+        <v>-7.552736726532</v>
       </c>
       <c r="C95" s="64">
         <f>IF(AND(B95&gt;=0,B96&lt;0),A95+pH_step*B95/(B95-B96),0)</f>
@@ -16292,7 +16344,7 @@
       </c>
       <c r="B96" s="64">
         <f t="shared" si="3"/>
-        <v>-10.282823226284</v>
+        <v>-9.692743661107</v>
       </c>
       <c r="C96" s="64">
         <f>IF(AND(B96&gt;=0,B97&lt;0),A96+pH_step*B96/(B96-B97),0)</f>
@@ -16305,7 +16357,7 @@
       </c>
       <c r="B97" s="64">
         <f t="shared" si="3"/>
-        <v>-13.255897853524</v>
+        <v>-12.495143944944</v>
       </c>
       <c r="C97" s="64">
         <f>IF(AND(B97&gt;=0,B98&lt;0),A97+pH_step*B97/(B97-B98),0)</f>
@@ -16318,7 +16370,7 @@
       </c>
       <c r="B98" s="64">
         <f t="shared" si="3"/>
-        <v>-17.180922991367</v>
+        <v>-16.194840392116</v>
       </c>
       <c r="C98" s="64">
         <f>IF(AND(B98&gt;=0,B99&lt;0),A98+pH_step*B98/(B98-B99),0)</f>
@@ -16331,7 +16383,7 @@
       </c>
       <c r="B99" s="64">
         <f t="shared" si="3"/>
-        <v>-22.410965673407</v>
+        <v>-21.124629237082</v>
       </c>
       <c r="C99" s="64">
         <f>IF(AND(B99&gt;=0,B100&lt;0),A99+pH_step*B99/(B99-B100),0)</f>
@@ -16344,7 +16396,7 @@
       </c>
       <c r="B100" s="64">
         <f t="shared" si="3"/>
-        <v>-29.452847122759</v>
+        <v>-27.762233083538</v>
       </c>
       <c r="C100" s="64">
         <f>0</f>
@@ -16386,7 +16438,7 @@
       </c>
       <c r="D103" s="149">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
-        <v>6.055158016113</v>
+        <v>6.077457645941</v>
       </c>
       <c r="E103" s="51" t="s">
         <v>1878</v>
@@ -16409,7 +16461,7 @@
       </c>
       <c r="D104" s="149">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
-        <v>0.948531749585</v>
+        <v>0.945966521198</v>
       </c>
       <c r="E104" s="51" t="s">
         <v>1879</v>
@@ -16601,7 +16653,7 @@
       </c>
       <c r="D125" s="149">
         <f>pH_Cl*pH_fHOCl*M_HOCl</f>
-        <v>8.967377109974</v>
+        <v>8.943125554526</v>
       </c>
       <c r="E125" s="51" t="s">
         <v>1460</v>
@@ -16808,7 +16860,7 @@
       </c>
       <c r="D138" s="149">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
-        <v>4.520261308413e-06</v>
+        <v>4.758265066161e-06</v>
       </c>
       <c r="E138" s="51" t="s">
         <v>1099</v>
@@ -16826,7 +16878,7 @@
       </c>
       <c r="D139" s="149">
         <f>P_HOCl/(k1_NH2Cl*NH3_free)</f>
-        <v>1.74420146132e-09</v>
+        <v>1.656958212721e-09</v>
       </c>
       <c r="E139" s="51" t="s">
         <v>1102</v>
@@ -16844,7 +16896,7 @@
       </c>
       <c r="D140" s="149">
         <f>HOCl_ss*M_HOCl</f>
-        <v>9.150080866082e-05</v>
+        <v>8.692402783936e-05</v>
       </c>
       <c r="E140" s="51" t="s">
         <v>1105</v>
@@ -16933,7 +16985,7 @@
       </c>
       <c r="D145" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_mgL/R_chloramine</f>
-        <v>0.251064863446</v>
+        <v>0.251019095638</v>
       </c>
       <c r="E145" s="51" t="inlineStr">
         <is>
@@ -17135,7 +17187,7 @@
       </c>
       <c r="D156" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_lo/R_chloramine_hi</f>
-        <v>0.005174981383</v>
+        <v>0.005129213575</v>
       </c>
       <c r="E156" s="51" t="s">
         <v>1247</v>
@@ -17153,7 +17205,7 @@
       </c>
       <c r="D157" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_hi/R_chloramine_lo</f>
-        <v>0.477371646429</v>
+        <v>0.477325878621</v>
       </c>
       <c r="E157" s="51" t="s">
         <v>1251</v>
@@ -17919,7 +17971,7 @@
       </c>
       <c r="D206" s="141">
         <f>E0_OER-nernst_slope*pH_meas</f>
-        <v>0.86429309373</v>
+        <v>0.862973862131</v>
       </c>
       <c r="E206" s="99" t="s">
         <v>1586</v>
@@ -17937,7 +17989,7 @@
       </c>
       <c r="D207" s="141">
         <f>E0_HER-nernst_slope*pH_meas</f>
-        <v>-0.36470690627</v>
+        <v>-0.366026137869</v>
       </c>
       <c r="E207" s="99" t="s">
         <v>1589</v>
@@ -17977,7 +18029,7 @@
       </c>
       <c r="D209" s="141">
         <f>E_HOCl_Cl-E_anode_op</f>
-        <v>-0.427527364769</v>
+        <v>-0.427526934687</v>
       </c>
       <c r="E209" s="67" t="inlineStr">
         <is>
@@ -17997,7 +18049,7 @@
       </c>
       <c r="D210" s="141">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
-        <v>0.33029309373</v>
+        <v>0.328973862131</v>
       </c>
       <c r="E210" s="67" t="s">
         <v>1599</v>
@@ -18017,7 +18069,7 @@
       </c>
       <c r="D211" s="141">
         <f>E_anode_op-E0_Cu</f>
-        <v>1.266535517225</v>
+        <v>1.265216285627</v>
       </c>
       <c r="E211" s="67" t="s">
         <v>1602</v>
@@ -18079,7 +18131,7 @@
       </c>
       <c r="D216" s="141">
         <f>Fcc*((km_HPO4/100)*HPO4_op+(km_HCO3/100)*HCO3_op)*1000/10</f>
-        <v>8.600113527674</v>
+        <v>8.598724981667</v>
       </c>
       <c r="E216" s="67" t="inlineStr">
         <is>
@@ -18117,7 +18169,7 @@
       </c>
       <c r="D218" s="141">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>0.328611439745</v>
+        <v>0.328664504833</v>
       </c>
       <c r="E218" s="67" t="s">
         <v>1618</v>
@@ -18153,7 +18205,7 @@
       </c>
       <c r="D220" s="141">
         <f>pH_op-LOG10(gamma_1)</f>
-        <v>6.164822774553</v>
+        <v>6.187122404381</v>
       </c>
       <c r="E220" s="67" t="s">
         <v>1624</v>
@@ -18246,7 +18298,7 @@
       </c>
       <c r="D226" s="141">
         <f>C_eff*M_Cl2/M_HOCl</f>
-        <v>0.339344361561</v>
+        <v>0.339282500863</v>
       </c>
       <c r="E226" s="67" t="s">
         <v>1899</v>
@@ -18560,7 +18612,7 @@
       </c>
       <c r="D252" s="141">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
-        <v>0.026586383209</v>
+        <v>0.026380308456</v>
       </c>
       <c r="E252" s="67" t="inlineStr">
         <is>
@@ -18586,7 +18638,7 @@
       </c>
       <c r="D253" s="141">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
-        <v>0.006136275232</v>
+        <v>0.006404116991</v>
       </c>
       <c r="E253" s="67" t="inlineStr">
         <is>
@@ -18664,7 +18716,7 @@
       </c>
       <c r="D256" s="141">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
-        <v>1.608435517225</v>
+        <v>1.607116285627</v>
       </c>
       <c r="E256" s="67" t="inlineStr">
         <is>
@@ -18715,7 +18767,7 @@
       </c>
       <c r="D258" s="141">
         <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,1E-12))-pH_meas-LOG10(MAX(pH_Cl,1E-12)))</f>
-        <v>1.180908152456</v>
+        <v>1.179589350939</v>
       </c>
       <c r="E258" s="67" t="inlineStr">
         <is>
@@ -18741,7 +18793,7 @@
       </c>
       <c r="D259" s="141">
         <f>C_eff_lo*M_Cl2/M_HOCl</f>
-        <v>0.006994609797</v>
+        <v>0.0069327491</v>
       </c>
       <c r="E259" s="67" t="inlineStr">
         <is>
@@ -18767,7 +18819,7 @@
       </c>
       <c r="D260" s="141">
         <f>C_eff_hi*M_Cl2/M_HOCl</f>
-        <v>0.645225199422</v>
+        <v>0.645163338724</v>
       </c>
       <c r="E260" s="67" t="inlineStr">
         <is>
@@ -19814,12 +19866,12 @@
         <v>135</v>
       </c>
       <c r="D44" s="48" t="str">
-        <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;", O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag basis)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 16%, O₂ 8% – until uptake starts, sparge every ≤2.2 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag, mean basis; H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse)")</f>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 18% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests the lag-phase headspace mix (rows 84–85) against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin.</t>
+          <t xml:space="preserve">Tests the lag-phase headspace mix (rows 84–85, mean-field) against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin. The text also quotes the H₂ fraction just before each pulse (y_H2_end_b, sawtooth top), which is higher than the mean.</t>
         </is>
       </c>
       <c r="F44" s="101" t="inlineStr">
@@ -20264,7 +20316,7 @@
       </c>
       <c r="D76" s="150">
         <f>'Mass Transfer'!$D$100</f>
-        <v>0.0005030206524901</v>
+        <v>0.0007098184304685</v>
       </c>
       <c r="E76" s="135" t="inlineStr">
         <is>
@@ -20442,12 +20494,12 @@
         </is>
       </c>
       <c r="D83" s="48">
-        <f>rH2_gen+O2_net_gen</f>
+        <f>H2_src_l_b+O2_net_gen</f>
         <v>0.0001515178050535</v>
       </c>
       <c r="E83" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lag phase: no uptake, so all electrolytic H₂ and net O₂ reach the headspace.</t>
+          <t xml:space="preserve">Lag phase: no uptake, so all electrolytic H₂ not oxidised at the anode (H2_src_l_b) and the net O₂ reach the headspace.</t>
         </is>
       </c>
     </row>
@@ -20468,12 +20520,12 @@
         </is>
       </c>
       <c r="D84" s="48">
-        <f>rH2_gen/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.155418629263</v>
+        <f>H2_src_l_b/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
+        <v>0.113266761861</v>
       </c>
       <c r="E84" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mean-field balance shared with Mass Transfer §300 (= y_H2_mf_l there): H₂ over all gas leaving the headspace — evolved gas, CO₂ pulses and, in the "Air exchange" vent model, the exchanged air. The pulse-to-pulse sawtooth peaks higher (D87 note).</t>
+          <t xml:space="preserve">Mean-field balance shared with Mass Transfer §300 (= y_H2_mf_l there): H₂ (net of anodic oxidation) over all gas leaving the headspace — evolved gas, CO₂ pulses and, in the "Open vent" and "Air exchange" vent models, the air drawn in. The pulse-to-pulse sawtooth peaks higher (y_H2_end_b, quoted in D44).</t>
         </is>
       </c>
     </row>
@@ -20495,7 +20547,7 @@
       </c>
       <c r="D85" s="48">
         <f>(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.076069380811</v>
+        <v>0.064019231488</v>
       </c>
       <c r="E85" s="69" t="inlineStr">
         <is>
@@ -20520,8 +20572,8 @@
         </is>
       </c>
       <c r="D86" s="48">
-        <f>MAX(0,MIN(rH2_gen/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
-        <v>0.002947616391</v>
+        <f>MAX(0,MIN(H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
+        <v>0.003376651195</v>
       </c>
       <c r="E86" s="69" t="inlineStr">
         <is>
@@ -20547,7 +20599,7 @@
       </c>
       <c r="D87" s="48">
         <f>IF(duty_H2safe&gt;0,spg_dur_b/(60*duty_H2safe),NA())</f>
-        <v>4.43586130694</v>
+        <v>3.872244049322</v>
       </c>
       <c r="E87" s="69" t="inlineStr">
         <is>
@@ -20572,8 +20624,8 @@
         </is>
       </c>
       <c r="D88" s="48">
-        <f>MAX(0,rH2_gen/H2_LFL-n_flamm_src-F_vent_ex_b)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
-        <v>0.975219102801</v>
+        <f>MAX(0,H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
+        <v>0.960219102801</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
@@ -20632,7 +20684,7 @@
       </c>
       <c r="D97" s="48">
         <f>'Mass Transfer'!$D$198</f>
-        <v>31.656160482387</v>
+        <v>29.726224026733</v>
       </c>
       <c r="E97" s="67" t="inlineStr">
         <is>
@@ -20658,7 +20710,7 @@
       </c>
       <c r="D98" s="48">
         <f>C_cycle_start_b*1000/Km_CO2</f>
-        <v>633.123209647745</v>
+        <v>594.524480534657</v>
       </c>
       <c r="E98" s="69" t="inlineStr">
         <is>
@@ -20691,7 +20743,7 @@
       </c>
       <c r="D111" s="150">
         <f>'Mass Transfer'!$D$308</f>
-        <v>0.0</v>
+        <v>3.67866400719e-05</v>
       </c>
       <c r="E111" s="135" t="inlineStr">
         <is>
@@ -20722,6 +20774,58 @@
       <c r="E112" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D307.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) H₂ to headspace — lag (net of anodic oxidation)</t>
+        </is>
+      </c>
+      <c r="B113" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_src_l_b</t>
+        </is>
+      </c>
+      <c r="C113" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D113" s="150">
+        <f>'Mass Transfer'!$D$314</f>
+        <v>0.0001017274698715</v>
+      </c>
+      <c r="E113" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D314: evolved H₂ less the anodic H₂ oxidation (r_H2_HOR).</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) headspace H₂ just before a pulse (lag)</t>
+        </is>
+      </c>
+      <c r="B114" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_H2_end_b</t>
+        </is>
+      </c>
+      <c r="C114" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D114" s="150">
+        <f>'Mass Transfer'!$D$388</f>
+        <v>0.175164116673</v>
+      </c>
+      <c r="E114" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D388 (sawtooth top).</t>
         </is>
       </c>
     </row>
@@ -21732,7 +21836,7 @@
       </c>
       <c r="D53" s="64">
         <f>kLa_sparge*duty</f>
-        <v>1.586800935557e-05</v>
+        <v>2.239153688755e-05</v>
       </c>
       <c r="E53" s="117" t="s">
         <v>643</v>
@@ -21770,7 +21874,7 @@
       </c>
       <c r="D55" s="48">
         <f>strip_sparge*duty</f>
-        <v>3.125613837221e-07</v>
+        <v>4.410590891654e-07</v>
       </c>
       <c r="E55" s="75" t="s">
         <v>649</v>
@@ -21789,7 +21893,7 @@
       </c>
       <c r="D56" s="45">
         <f>IF(O2_excess&gt;0,strip_avg/O2_excess,NA())</f>
-        <v>0.01968124611</v>
+        <v>0.027772440663</v>
       </c>
       <c r="E56" s="75" t="s">
         <v>652</v>
@@ -21978,11 +22082,13 @@
         <v>67</v>
       </c>
       <c r="D66" s="48">
-        <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,cleared_min)</f>
-        <v>21.086843893767</v>
-      </c>
-      <c r="E66" s="99" t="s">
-        <v>680</v>
+        <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,"never (strip ≥ source)")</f>
+        <v>21.262335479879</v>
+      </c>
+      <c r="E66" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above, crediting time-averaged bubble strip (≈unchanged → bubbles aren't the mechanism). "never" = cleared.</t>
+        </is>
       </c>
       <c r="F66" s="20"/>
     </row>
@@ -22139,45 +22245,19 @@
       <c r="F74" s="20"/>
     </row>
     <row r="75" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="17" t="s">
-        <v>703</v>
-      </c>
-      <c r="B75" s="18" t="s">
-        <v>704</v>
-      </c>
-      <c r="C75" s="19" t="s">
-        <v>135</v>
-      </c>
-      <c r="D75" s="48">
-        <f>y_O2_actual</f>
-        <v>0.031639138319</v>
-      </c>
-      <c r="E75" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">= y_O2_actual (D187): the mean-field headspace O₂ fraction of the sizing phase at the schedule in use, from the shared vent balance (§300). Kept so D76 (µM form) still reads.</t>
-        </is>
-      </c>
+      <c r="A75" s="17"/>
+      <c r="B75" s="18"/>
+      <c r="C75" s="19"/>
+      <c r="D75" s="48"/>
+      <c r="E75" s="99"/>
       <c r="F75" s="20"/>
     </row>
     <row r="76" spans="1:6" ht="36" x14ac:dyDescent="0.2">
-      <c r="A76" s="17" t="s">
-        <v>706</v>
-      </c>
-      <c r="B76" s="18" t="s">
-        <v>707</v>
-      </c>
-      <c r="C76" s="19" t="s">
-        <v>463</v>
-      </c>
-      <c r="D76" s="48">
-        <f>H_O2_T*y_O2_vent*P_atm*1000</f>
-        <v>38.470028282145</v>
-      </c>
-      <c r="E76" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dissolved O₂ in equilibrium with that vent headspace fraction, in µM; the same quantity as DO_hs_floor (D188) ×1000. Compare with the inhibition ceiling (Biology D28). Diagnostic, not a backstop.</t>
-        </is>
-      </c>
+      <c r="A76" s="17"/>
+      <c r="B76" s="18"/>
+      <c r="C76" s="19"/>
+      <c r="D76" s="48"/>
+      <c r="E76" s="69"/>
       <c r="F76" s="20"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
@@ -22192,7 +22272,7 @@
       </c>
       <c r="D77" s="48">
         <f>headspace_V/(Q_CO2*duty)</f>
-        <v>12.736715659111</v>
+        <v>9.026013902172</v>
       </c>
       <c r="E77" s="99" t="s">
         <v>710</v>
@@ -22211,7 +22291,7 @@
       </c>
       <c r="D78" s="48">
         <f>IF(O2_excess&gt;0,(strip_avg+surf_strip)/O2_excess,NA())</f>
-        <v>8.950039737787</v>
+        <v>8.95813093234</v>
       </c>
       <c r="E78" s="118" t="s">
         <v>713</v>
@@ -22247,12 +22327,14 @@
       <c r="C80" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="D80" s="48">
-        <f>IF(O2_net_gen-strip_avg-surf_strip&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_net_gen-strip_avg-surf_strip)*60,cleared_min)</f>
-        <v>9999.0</v>
-      </c>
-      <c r="E80" s="69" t="s">
-        <v>1458</v>
+      <c r="D80" s="48" t="str">
+        <f>IF(O2_net_gen-strip_avg-surf_strip&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_net_gen-strip_avg-surf_strip)*60,"never (removal ≥ source)")</f>
+        <v>never (removal ≥ source)</v>
+      </c>
+      <c r="E80" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Companion to t_O2_ceiling_lag crediting BOTH removal paths at their best-case ceiling driving force. Best-case diagnostic only: surf_strip is the ~375%-uncertain surface proxy, so this cell must never gate a schedule or a guard. "never" = removal exceeds the source at that best case.</t>
+        </is>
       </c>
       <c r="F80" s="20"/>
     </row>
@@ -22409,8 +22491,10 @@
       <c r="F88" s="20"/>
     </row>
     <row r="89" spans="1:6" ht="36" x14ac:dyDescent="0.2">
-      <c r="A89" s="17" t="s">
-        <v>738</v>
+      <c r="A89" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max interval — legacy O₂ flush guard (fallback)</t>
+        </is>
       </c>
       <c r="B89" s="18" t="s">
         <v>739</v>
@@ -22424,7 +22508,7 @@
       </c>
       <c r="E89" s="99" t="inlineStr">
         <is>
-          <t xml:space="preserve">O₂-limited fallback interval: zero-surface worst case (no surface credit; sizes on O2_src_guard D132). D91 uses it only when the DO target is unreachable (spg_int_DO, D185, is #N/A).</t>
+          <t xml:space="preserve">LEGACY O₂ flush guard, kept only as the fallback: fills target_DO_frac of the ceiling in the liquid from the zero-surface worst-case source (O2_src_guard, D132) with no venting. It predates the shared headspace balance (§300), so the vent model does not move it and the DO it gives is neither the target nor a ceiling margin. D91 uses it only when the DO target is unreachable (spg_int_DO, D185, is #N/A). A balance-derived replacement (size on the ceiling with a margin) is an owner decision.</t>
         </is>
       </c>
       <c r="F89" s="20"/>
@@ -22459,12 +22543,12 @@
         <v>67</v>
       </c>
       <c r="D91" s="48">
-        <f>IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max))</f>
-        <v>12.736715659111</v>
+        <f>IF(ISNA(F_vent_ex+O2_src_sched),NA(),IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max)))</f>
+        <v>9.026013902172</v>
       </c>
       <c r="E91" s="159" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANSWER. The shorter of the two upper bounds on the interval: carbon supply (D112) and headspace-oxygen dilution (spg_int_DO). If the DO target is unreachable at this surface kLa the sheet falls back to the lag-accumulation cap (D89) and D134 says so. kL_surf moves the answer continuously; no branch depends on it.</t>
+          <t xml:space="preserve">ANSWER. The shorter of the two upper bounds on the interval: carbon supply (D112) and headspace-oxygen dilution (spg_int_DO). An invalid vent or phase selector (Summary D111/D112) returns #N/A here instead of falling through to the fallback. If the DO target is unreachable at this surface kLa the sheet falls back to the legacy O₂ flush guard (D89) and D134 says so. kL_surf moves the answer continuously; no branch depends on it.</t>
         </is>
       </c>
       <c r="F91" s="20"/>
@@ -22481,7 +22565,7 @@
       </c>
       <c r="D92" s="48">
         <f>spg_int_opt*60</f>
-        <v>764.202939546678</v>
+        <v>541.560834130326</v>
       </c>
       <c r="E92" s="159" t="s">
         <v>747</v>
@@ -22502,7 +22586,7 @@
       </c>
       <c r="D93" s="48">
         <f>spg_dur_opt/(spg_int_opt*60)</f>
-        <v>0.001026576854</v>
+        <v>0.001448614819</v>
       </c>
       <c r="E93" s="99" t="s">
         <v>750</v>
@@ -22520,7 +22604,7 @@
         <v>135</v>
       </c>
       <c r="D94" s="48" t="str">
-        <f>IF(NOT(ISNUMBER(spg_int_DO)),"O2-INFEASIBLE (see D134)",IF(spg_int_DO&lt;=spg_int_carbon,"O2-DILUTION (headspace O2 sets the interval)","CARBON (CO2 supply sets the interval)"))</f>
+        <f>IF(ISNA(F_vent_ex+O2_src_sched),"INVALID SELECTOR (Summary D111/D112)",IF(NOT(ISNUMBER(spg_int_DO)),"O2-INFEASIBLE – the legacy O2 flush guard (D89) sets the interval (see D134)",IF(spg_int_DO&lt;=spg_int_carbon,"O2-DILUTION (headspace O2 sets the interval)","CARBON (CO2 supply sets the interval)")))</f>
         <v>O2-DILUTION (headspace O2 sets the interval)</v>
       </c>
       <c r="E94" s="99" t="s">
@@ -22635,7 +22719,7 @@
       </c>
       <c r="D100" s="28">
         <f>CO2_pulse*pulses_h</f>
-        <v>0.0005030206524901</v>
+        <v>0.0007098184304685</v>
       </c>
       <c r="E100" s="160" t="s">
         <v>765</v>
@@ -22728,7 +22812,7 @@
       </c>
       <c r="D105" s="28">
         <f>spg_dur/(spg_int*60)</f>
-        <v>0.001026576854</v>
+        <v>0.001448614819</v>
       </c>
       <c r="E105" s="160" t="s">
         <v>765</v>
@@ -22777,7 +22861,7 @@
       </c>
       <c r="D108" s="28">
         <f>DO_avg_sched*M_O2</f>
-        <v>2.634660261764</v>
+        <v>2.634776001183</v>
       </c>
       <c r="E108" s="160" t="inlineStr">
         <is>
@@ -22787,17 +22871,10 @@
       <c r="F108" s="20"/>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A109" s="20" t="s">
-        <v>784</v>
-      </c>
-      <c r="B109" s="20" t="s">
-        <v>785</v>
-      </c>
+      <c r="A109" s="20"/>
+      <c r="B109" s="20"/>
       <c r="C109" s="20"/>
-      <c r="D109" s="28" t="str">
-        <f>IF(ISNUMBER(DO_opt),IF(DO_ss&lt;=DO_opt,"at/under optimum",IF(DO_ss&lt;DO_impair,"above optimum, under impairment","OVER IMPAIRMENT - surface strip insufficient")),"organism optimum unknown")</f>
-        <v>organism optimum unknown</v>
-      </c>
+      <c r="D109" s="28"/>
       <c r="E109" s="20"/>
       <c r="F109" s="20"/>
     </row>
@@ -22860,12 +22937,12 @@
       </c>
       <c r="C113" s="20"/>
       <c r="D113" s="28" t="str">
-        <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) DO would be "&amp;TEXT(DO_at_carbon*M_O2,"0.0")&amp;" mg/L against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) DO would be 20.1 mg/L against a 2.6 mg/L target</v>
+        <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) the cycle-mean DO would be ≈"&amp;TEXT(DO_at_carbon*M_O2,"0")&amp;" mg/L, "&amp;IF(DO_at_carbon&gt;O2_ceil_C,"above the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L inhibition ceiling","against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")&amp;" (peaks higher)")</f>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) the cycle-mean DO would be ≈16 mg/L, above the 11.7 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E113" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests the carbon-limited interval against the same DO balance the schedule uses (D232). DO_ss cannot test it: it sits at the target by construction.</t>
+          <t xml:space="preserve">Tests the carbon-limited interval against the same DO balance the schedule uses (D232, cycle mean), and states it against the inhibition ceiling when it exceeds it. DO_ss cannot test it: it sits at the target by construction.</t>
         </is>
       </c>
       <c r="F113" s="20"/>
@@ -23013,7 +23090,7 @@
       </c>
       <c r="D122" s="28">
         <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
-        <v>12.736715659111</v>
+        <v>9.026013902172</v>
       </c>
       <c r="E122" s="20"/>
       <c r="F122" s="20"/>
@@ -23047,7 +23124,7 @@
       </c>
       <c r="D124" s="28">
         <f>60/spg_int</f>
-        <v>4.710790568452</v>
+        <v>6.647452646352</v>
       </c>
       <c r="E124" s="20"/>
       <c r="F124" s="20"/>
@@ -23064,7 +23141,7 @@
       </c>
       <c r="D125" s="28">
         <f>pulses_h*24</f>
-        <v>113.058973642855</v>
+        <v>159.538863512438</v>
       </c>
       <c r="E125" s="20"/>
       <c r="F125" s="20"/>
@@ -23081,7 +23158,7 @@
       </c>
       <c r="D126" s="28">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v>29.668720934024</v>
+        <v>41.865885273592</v>
       </c>
       <c r="E126" s="20"/>
       <c r="F126" s="20"/>
@@ -23098,7 +23175,7 @@
       </c>
       <c r="D127" s="28">
         <f>O2_excess/60*spg_int</f>
-        <v>3.371234260456e-06</v>
+        <v>2.389062307486e-06</v>
       </c>
       <c r="E127" s="20"/>
       <c r="F127" s="20"/>
@@ -23132,7 +23209,7 @@
       </c>
       <c r="D129" s="28">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v>0.01968124611</v>
+        <v>0.027772440663</v>
       </c>
       <c r="E129" s="20"/>
       <c r="F129" s="20"/>
@@ -23195,7 +23272,7 @@
     <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mean-field steady DO (sizing-phase source)</t>
+          <t xml:space="preserve">Cycle-mean DO (sawtooth, sizing phase)</t>
         </is>
       </c>
       <c r="B133" s="18" t="s">
@@ -23205,12 +23282,12 @@
         <v>995</v>
       </c>
       <c r="D133" s="28">
-        <f>DO_hs_floor+DO_surf_excess</f>
-        <v>0.079316092899</v>
+        <f>DO_avg_sched</f>
+        <v>0.082341896405</v>
       </c>
       <c r="E133" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flux-mean form of D108 in mol/m³: headspace floor (D188, from the shared vent balance) plus the surface excess on the sizing-phase source. Equals DO_target ÷ saw_factor-adjusted by construction when the DO constraint binds.</t>
+          <t xml:space="preserve">Cycle-mean dissolved O₂ of the sawtooth model on the sizing phase in mol/m³ (= DO_avg_sched, D372; D108 is the same in mg/L). One DO definition per statistic: mean = DO_avg_*, peak = DO_peak_*; the flux-mean (mean-field) form appears only as the labelled cross-check rows 340/361.</t>
         </is>
       </c>
       <c r="F133" s="20"/>
@@ -23226,8 +23303,8 @@
         <v>998</v>
       </c>
       <c r="D134" s="28" t="str">
-        <f>IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf"))</f>
-        <v>ESTIMATED kLa — DO-limited interval is 12.7 min; confirm by measuring kL_surf</v>
+        <f>IF(ISNA(F_vent_ex+O2_src_sched),"INVALID SELECTOR (Summary D111/D112) – no schedule until both are listed values",IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf")))</f>
+        <v>ESTIMATED kLa — DO-limited interval is 9.0 min; confirm by measuring kL_surf</v>
       </c>
       <c r="E134" s="69" t="inlineStr">
         <is>
@@ -23239,7 +23316,7 @@
     <row r="135" spans="1:6" ht="24" x14ac:dyDescent="0.2">
       <c r="A135" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mean-field steady DO (LAG source)</t>
+          <t xml:space="preserve">Cycle-mean DO (LAG source, sawtooth)</t>
         </is>
       </c>
       <c r="B135" s="20" t="s">
@@ -23249,12 +23326,12 @@
         <v>1001</v>
       </c>
       <c r="D135" s="28">
-        <f>DO_mf_l</f>
-        <v>0.220552478156</v>
+        <f>DO_avg_l</f>
+        <v>0.212069565945</v>
       </c>
       <c r="E135" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lag-phase companion evaluated on the LAG headspace balance (y_O2_mf_l, with the H₂ as a diluent and the vent model in use) — not the growth headspace fraction, which understated it by ~30 % (R2-B2). The sawtooth mean and peak are in the lag block of §300.</t>
+          <t xml:space="preserve">Lag-phase time-mean dissolved O₂ (DO_avg_l, D362) at the schedule in use, on the LAG headspace balance with the H₂ as a diluent and the vent model in use. Feeds the lag-phase peroxide (Electrochemistry D150), which is first order in DO, so it takes the time mean — not the flux-mean D361, which is ~3 % lower.</t>
         </is>
       </c>
       <c r="F135" s="20"/>
@@ -23347,8 +23424,10 @@
       <c r="F141" s="20"/>
     </row>
     <row r="142" spans="1:6" ht="36" x14ac:dyDescent="0.2">
-      <c r="A142" s="17" t="s">
-        <v>1168</v>
+      <c r="A142" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace air exchange ("Air exchange" model)</t>
+        </is>
       </c>
       <c r="B142" s="18" t="s">
         <v>1169</v>
@@ -23361,7 +23440,7 @@
       </c>
       <c r="E142" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bidirectional air-exchange flow through the vent, used ONLY when vent_model (Summary D111) = "Air exchange", by the O₂ balance, the CO₂ pool and the flammability block alike. KEY UNCERTAIN PARAMETER — measure (pressure-decay or headspace-O₂ tracer, R2 experiment 1); include any per-pulse back-draw in it. Not free membrane diffusion, which would clear in seconds.</t>
+          <t xml:space="preserve">Bidirectional air-exchange flow through the vent, used ONLY when vent_model (Summary D111) = "Air exchange" (an "Open vent" uses Q_backdraw, D385), by the O₂ balance, the CO₂ pool and the flammability block alike. KEY UNCERTAIN PARAMETER — measure (pressure-decay or headspace-O₂ tracer, R2 experiment 1); include any per-pulse back-draw in it. Not free membrane diffusion, which would clear in seconds.</t>
         </is>
       </c>
       <c r="F142" s="20"/>
@@ -23380,7 +23459,7 @@
       </c>
       <c r="D143" s="48">
         <f>F_gap_sched/3600/n_hs_gas</f>
-        <v>0.0</v>
+        <v>9.569640057845e-05</v>
       </c>
       <c r="E143" s="67" t="inlineStr">
         <is>
@@ -23400,12 +23479,12 @@
         <v>67</v>
       </c>
       <c r="D144" s="48">
-        <f>IF(k_vent&gt;0,1/k_vent/60,cleared_min)</f>
-        <v>9999.0</v>
+        <f>IF(k_vent&gt;0,1/k_vent/60,"none between pulses")</f>
+        <v>174.161897061142</v>
       </c>
       <c r="E144" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Time constant for the headspace to clear between pulses; the 9999 sentinel means nothing leaves between pulses, so only the pulses clear it.</t>
+          <t xml:space="preserve">Time constant for the headspace to clear between pulses; "none between pulses" when nothing leaves between pulses (outflow-only vent, growth phase), so only the pulses clear it.</t>
         </is>
       </c>
       <c r="F144" s="20"/>
@@ -23557,7 +23636,7 @@
       </c>
       <c r="D152" s="48">
         <f>MAX(0,spg_int*60-spg_dur)</f>
-        <v>763.418426496853</v>
+        <v>540.776321080501</v>
       </c>
       <c r="E152" s="67" t="s">
         <v>1190</v>
@@ -23648,7 +23727,7 @@
       </c>
       <c r="D162" s="48">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,CO2_cyc_avg_new))/1000</f>
-        <v>0.031754970696</v>
+        <v>0.029931790408</v>
       </c>
       <c r="E162" s="67" t="s">
         <v>1859</v>
@@ -23666,11 +23745,13 @@
         <v>135</v>
       </c>
       <c r="D163" s="48" t="str">
-        <f>IF(tau_hs&gt;=tau_surf_floor,"vent is slow path - OK","WARNING: surface clears faster than vent - run2 cannot stay acidic")</f>
-        <v>vent is slow path - OK</v>
-      </c>
-      <c r="E163" s="67" t="s">
-        <v>1211</v>
+        <f>IF(ISTEXT(tau_hs),"no vent turnover between pulses (OK)",IF(tau_hs&gt;=tau_surf_floor,"vent turnover slower than the surface (OK)","WARNING: the vent turns the headspace over faster than the surface relaxes the liquid"))</f>
+        <v>vent turnover slower than the surface (OK)</v>
+      </c>
+      <c r="E163" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirms the headspace turnover between pulses is slower than the liquid's surface relaxation, as the CO₂ pool's quasi-equilibrium assumes; trivially true when nothing leaves between pulses.</t>
+        </is>
       </c>
       <c r="F163" s="20"/>
     </row>
@@ -23986,7 +24067,7 @@
       </c>
       <c r="D184" s="141">
         <f>IF(ISNUMBER(y_O2_star),MAX(0,((O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_vent_ex-O2_src_sched-H2_src_sched+CO2_fix_sched)/CO2_rate_full),NA())</f>
-        <v>0.001026576854</v>
+        <v>0.001448614819</v>
       </c>
       <c r="E184" s="67" t="inlineStr">
         <is>
@@ -24006,7 +24087,7 @@
       </c>
       <c r="D185" s="141">
         <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_opt/(60*duty_DO),spg_int_carbon),NA())</f>
-        <v>12.736715659111</v>
+        <v>9.026013902172</v>
       </c>
       <c r="E185" s="67" t="s">
         <v>1813</v>
@@ -24167,7 +24248,7 @@
       </c>
       <c r="D195" s="141">
         <f>k_vent*Vg_CO2/(V_L_m3+Vg_CO2)</f>
-        <v>0.0</v>
+        <v>1.679738870232e-05</v>
       </c>
       <c r="E195" s="99" t="inlineStr">
         <is>
@@ -24186,12 +24267,12 @@
         <v>110</v>
       </c>
       <c r="D196" s="141">
-        <f>IF(k_vent&gt;0,(kLa_CO2_off*V_L_m3/Vg_CO2)/k_vent,cleared_min)</f>
-        <v>9999.0</v>
+        <f>IF(k_vent&gt;0,(kLa_CO2_off*V_L_m3/Vg_CO2)/k_vent,"no turnover between pulses")</f>
+        <v>346.46664161513</v>
       </c>
       <c r="E196" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Liquid-uptake rate constant ÷ headspace turnover between pulses. Well above 1 means the two compartments stay in quasi-equilibrium, which the pool model assumes; the 9999 sentinel is the outflow-only growth case (no turnover at all).</t>
+          <t xml:space="preserve">Liquid-uptake rate constant ÷ headspace turnover between pulses. Well above 1 means the two compartments stay in quasi-equilibrium, which the pool model assumes; text when nothing leaves between pulses (outflow-only growth case).</t>
         </is>
       </c>
     </row>
@@ -24207,7 +24288,7 @@
       </c>
       <c r="D197" s="141">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
-        <v>1.0</v>
+        <v>0.990957501466</v>
       </c>
       <c r="E197" s="99" t="s">
         <v>1849</v>
@@ -24225,7 +24306,7 @@
       </c>
       <c r="D198" s="141">
         <f>(pool_D_gap+pool_b*pool_e)/(1-pool_ret*pool_e)</f>
-        <v>31.656160482387</v>
+        <v>29.726224026733</v>
       </c>
       <c r="E198" s="99" t="inlineStr">
         <is>
@@ -24245,7 +24326,7 @@
       </c>
       <c r="D199" s="141">
         <f>pool_ret*C_cycle_start+pool_b</f>
-        <v>31.853780908877</v>
+        <v>30.13798016156</v>
       </c>
       <c r="E199" s="99" t="inlineStr">
         <is>
@@ -24265,7 +24346,7 @@
       </c>
       <c r="D200" s="141">
         <f>C_cycle_peak*pool_phi+pool_D_raw*pool_psi</f>
-        <v>31.754970695632</v>
+        <v>29.931790407874</v>
       </c>
       <c r="E200" s="99" t="inlineStr">
         <is>
@@ -24568,7 +24649,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t xml:space="preserve">DO if the interval relaxed to the carbon-limited one</t>
+          <t xml:space="preserve">Cycle-mean DO if the interval relaxed to the carbon-limited one</t>
         </is>
       </c>
       <c r="B232" s="18" t="inlineStr">
@@ -24582,12 +24663,12 @@
         </is>
       </c>
       <c r="D232" s="141">
-        <f>DO_surf_excess+H_O2_T*P_atm*(O2_src_sched+y_O2_air*F_vent_ex)/(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)</f>
-        <v>0.628922200193</v>
+        <f>IF(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,DO_surf_excess+H_O2_T*P_atm*MIN(1,saw_factor*(O2_src_sched+y_O2_air*F_vent_ex)/(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)),DO_surf_excess+H_O2_T*P_atm)</f>
+        <v>0.486561365549</v>
       </c>
       <c r="E232" s="99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same shared headspace balance as D187/D180 (sizing phase, vent model in use) evaluated at the carbon-limited duty instead of the DO-limited one. At that duty the CO₂ leaving is only twice the fixation, so O₂ is a large fraction of the vent gas.</t>
+          <t xml:space="preserve">Same shared headspace balance as D187/D180 (sizing phase, vent model in use) evaluated at the carbon-limited duty instead of the DO-limited one, raised from the flux mean to the cycle (time) mean by saw_factor (D322; the slow-vent limit, so slightly high when air enters) and capped at a pure-O₂ headspace. Guarded: if nothing would leave the headspace, the O₂ fraction tends to 1, which is returned. At that duty the CO₂ leaving is only carbon_margin_min × the fixation, so O₂ is a large fraction of the vent gas and the number is sensitive to carbon_margin_min; the direction (far above the ceiling) is robust, the value is not.</t>
         </is>
       </c>
     </row>
@@ -24674,11 +24755,11 @@
       </c>
       <c r="D301" s="134" t="str">
         <f>Summary!$D$111</f>
-        <v>Outflow only</v>
+        <v>Open vent</v>
       </c>
       <c r="E301" s="135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import from Summary!D111. Owner decision: "Outflow only" or "Air exchange"; anything else returns #N/A by design. Default "Outflow only" until the vent hardware is characterised (R2 experiment 1).</t>
+          <t xml:space="preserve">Import from Summary!D111. Owner decision: "Outflow only", "Open vent" or "Air exchange"; anything else returns #N/A by design. Default "Open vent" until the vent hardware is characterised (R2 experiment 1).</t>
         </is>
       </c>
     </row>
@@ -24705,7 +24786,7 @@
       </c>
       <c r="E302" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas leaves through the vent but none enters between pulses (check valve or sealed cap; the small sub-atmospheric dip after each pulse is tolerated). The headspace is then diluted only by the CO₂ pulses and by what electrolysis evolves.</t>
+          <t xml:space="preserve">Check valve or sealed cap that HOLDS the vacuum left after each pulse: no air ever enters. The headspace is then diluted only by the CO₂ pulses and by what electrolysis evolves, and it sags below 1 atm between pulses (hs_sag, D389) — which a real cap may not hold.</t>
         </is>
       </c>
     </row>
@@ -24732,7 +24813,7 @@
       </c>
       <c r="E303" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Room air exchanges with the headspace at Q_vent (D142) continuously — an open tube, diffusion, or per-pulse back-draw of the same average volume. Q_vent must then be the TOTAL air ingress, including the back-draw that refills whatever the liquid absorbs after each pulse.</t>
+          <t xml:space="preserve">Measured bidirectional exchange with room air at Q_vent (D142) — forced or diffusive flow through an open port. Q_vent must then be the TOTAL air ingress, including any per-pulse back-draw.</t>
         </is>
       </c>
     </row>
@@ -24844,7 +24925,7 @@
     <row r="308">
       <c r="A308" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vent air-exchange flow</t>
+          <t xml:space="preserve">Vent air ingress (molar)</t>
         </is>
       </c>
       <c r="B308" s="18" t="inlineStr">
@@ -24858,12 +24939,12 @@
         </is>
       </c>
       <c r="D308" s="48">
-        <f>IF(vent_model=vent_name_1,0,IF(vent_model=vent_name_2,P_atm*(Q_vent/1000000/60)/(R_gas*T_K)*3600,NA()))</f>
-        <v>0.0</v>
+        <f>P_atm*(Q_vent_used/1000000/60)/(R_gas*T_K)*3600</f>
+        <v>3.67866400719e-05</v>
       </c>
       <c r="E308" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Molar air flow exchanged through the vent (ideal gas at P_atm, T_K). Zero in "Outflow only"; Q_vent converted mL/min → mol/h in "Air exchange". Inherits the uncertainty of Q_vent — measure it.</t>
+          <t xml:space="preserve">Molar air ingress through the vent (ideal gas at P_atm, T_K): Q_vent_used (D386) converted mL/min → mol/h. Zero only for a true check valve ("Outflow only"). Inherits the uncertainty of Q_backdraw / Q_vent — measure it.</t>
         </is>
       </c>
     </row>
@@ -24988,12 +25069,12 @@
         </is>
       </c>
       <c r="D313" s="48">
-        <f>MAX(0,rH2_gen-H2_cons)</f>
+        <f>MAX(0,rH2_gen-H2_HOR_mt-H2_cons)</f>
         <v>0.0</v>
       </c>
       <c r="E313" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Residual H₂ reaching the headspace in growth: zero under the 100 % uptake assumption. A real residual (cathode bubbles bypassing the liquid) is a DATA GAP — see the off-gas H₂ experiment.</t>
+          <t xml:space="preserve">Residual H₂ reaching the headspace in growth: evolved H₂ less what the anode oxidises (H2_HOR_mt) less uptake; zero under the 100 % uptake assumption. A real residual (cathode bubbles bypassing the liquid) is a DATA GAP — see the off-gas H₂ experiment.</t>
         </is>
       </c>
     </row>
@@ -25014,12 +25095,12 @@
         </is>
       </c>
       <c r="D314" s="48">
-        <f>rH2_gen</f>
+        <f>MAX(0,rH2_gen-H2_HOR_mt)</f>
         <v>0.0001017274698715</v>
       </c>
       <c r="E314" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">All evolved H₂ reaches the headspace before uptake starts.</t>
+          <t xml:space="preserve">All evolved H₂ that the anode does not oxidise (H2_HOR_mt) reaches the headspace before uptake starts.</t>
         </is>
       </c>
     </row>
@@ -25300,7 +25381,7 @@
       </c>
       <c r="D325" s="48">
         <f>t_off_CO2/3600</f>
-        <v>0.212060674027</v>
+        <v>0.150215644745</v>
       </c>
       <c r="E325" s="67" t="inlineStr">
         <is>
@@ -25352,7 +25433,7 @@
       </c>
       <c r="D327" s="48">
         <f>O2_src_g+y_O2_air*F_vent_ex</f>
-        <v>1.58811785582e-05</v>
+        <v>2.358797965326e-05</v>
       </c>
       <c r="E327" s="67" t="inlineStr">
         <is>
@@ -25378,7 +25459,7 @@
       </c>
       <c r="D328" s="48">
         <f>CO2_supply+O2_src_g+H2_src_g-CO2_fix_g</f>
-        <v>0.0005019472527364</v>
+        <v>0.0007087450307148</v>
       </c>
       <c r="E328" s="67" t="inlineStr">
         <is>
@@ -25456,7 +25537,7 @@
       </c>
       <c r="D331" s="48">
         <f>F_vent_ex+MAX(0,O2_src_g+H2_src_g-CO2_fix_g)</f>
-        <v>0.0</v>
+        <v>3.67866400719e-05</v>
       </c>
       <c r="E331" s="67" t="inlineStr">
         <is>
@@ -25482,7 +25563,7 @@
       </c>
       <c r="D332" s="48">
         <f>F_gap_g*t_gap_h/n_hs_gas</f>
-        <v>0.0</v>
+        <v>0.051750347445</v>
       </c>
       <c r="E332" s="67" t="inlineStr">
         <is>
@@ -25508,7 +25589,7 @@
       </c>
       <c r="D333" s="48">
         <f>IF(x_hs_g&gt;0,(1-EXP(-x_hs_g))/x_hs_g,1)</f>
-        <v>1.0</v>
+        <v>0.974565460589</v>
       </c>
       <c r="E333" s="67" t="inlineStr">
         <is>
@@ -25534,7 +25615,7 @@
       </c>
       <c r="D334" s="48">
         <f>IF(x_hs_g&gt;0,(x_hs_g-1+EXP(-x_hs_g))/x_hs_g^2,1/2)</f>
-        <v>0.5</v>
+        <v>0.491485384479</v>
       </c>
       <c r="E334" s="67" t="inlineStr">
         <is>
@@ -25560,7 +25641,7 @@
       </c>
       <c r="D335" s="48">
         <f>S_O2_g*t_gap_h/n_hs_gas</f>
-        <v>0.031539212614</v>
+        <v>0.03318286585</v>
       </c>
       <c r="E335" s="67" t="inlineStr">
         <is>
@@ -25586,7 +25667,7 @@
       </c>
       <c r="D336" s="48">
         <f>dy_O2_g*phi_hs_g/(1-flush_ret*EXP(-x_hs_g))</f>
-        <v>0.049894299708</v>
+        <v>0.049700562217</v>
       </c>
       <c r="E336" s="68" t="inlineStr">
         <is>
@@ -25612,7 +25693,7 @@
       </c>
       <c r="D337" s="48">
         <f>y_O2_end_g*flush_ret</f>
-        <v>0.018355087094</v>
+        <v>0.018283815054</v>
       </c>
       <c r="E337" s="68" t="inlineStr">
         <is>
@@ -25638,7 +25719,7 @@
       </c>
       <c r="D338" s="48">
         <f>y_O2_post_g*phi_hs_g+dy_O2_g*psi_hs_g</f>
-        <v>0.034124693401</v>
+        <v>0.03412766822</v>
       </c>
       <c r="E338" s="68" t="inlineStr">
         <is>
@@ -25716,7 +25797,7 @@
       </c>
       <c r="D341" s="48">
         <f>DO_surf_excess_g+H_O2_T*P_atm*y_O2_avg_g</f>
-        <v>0.082338279323</v>
+        <v>0.082341896405</v>
       </c>
       <c r="E341" s="68" t="inlineStr">
         <is>
@@ -25742,7 +25823,7 @@
       </c>
       <c r="D342" s="48">
         <f>DO_surf_excess_g+H_O2_T*P_atm*MAX(y_O2_avg_g,y_O2_end_g-(S_O2_g-F_gap_g*y_O2_end_g)/n_hs_gas*tau_L_h)</f>
-        <v>0.094535887493</v>
+        <v>0.091717883745</v>
       </c>
       <c r="E342" s="68" t="inlineStr">
         <is>
@@ -25768,7 +25849,7 @@
       </c>
       <c r="D343" s="48">
         <f>DO_avg_g*M_O2</f>
-        <v>2.634660261764</v>
+        <v>2.634776001183</v>
       </c>
       <c r="E343" s="68" t="inlineStr">
         <is>
@@ -25794,7 +25875,7 @@
       </c>
       <c r="D344" s="48">
         <f>DO_peak_g*M_O2</f>
-        <v>3.024959328002</v>
+        <v>2.934788844069</v>
       </c>
       <c r="E344" s="68" t="inlineStr">
         <is>
@@ -25898,7 +25979,7 @@
       </c>
       <c r="D348" s="28" t="str">
         <f>IF(DO_peak_g&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
-        <v>peak 3.0 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 2.9 mg/L under the 11.7 mg/L ceiling</v>
       </c>
       <c r="E348" s="67" t="inlineStr">
         <is>
@@ -25924,7 +26005,7 @@
       </c>
       <c r="D349" s="48">
         <f>O2_src_l+y_O2_air*F_vent_ex</f>
-        <v>4.979033518202e-05</v>
+        <v>5.749713627708e-05</v>
       </c>
       <c r="E349" s="67" t="inlineStr">
         <is>
@@ -25950,7 +26031,7 @@
       </c>
       <c r="D350" s="48">
         <f>CO2_supply+O2_src_l+H2_src_l-CO2_fix_l</f>
-        <v>0.0006545384575436</v>
+        <v>0.000861336235522</v>
       </c>
       <c r="E350" s="67" t="inlineStr">
         <is>
@@ -25976,7 +26057,7 @@
       </c>
       <c r="D351" s="48">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,S_O2_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.076069380811</v>
+        <v>0.064019231488</v>
       </c>
       <c r="E351" s="67" t="inlineStr">
         <is>
@@ -26002,7 +26083,7 @@
       </c>
       <c r="D352" s="48">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,H2_src_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.155418629263</v>
+        <v>0.113266761861</v>
       </c>
       <c r="E352" s="67" t="inlineStr">
         <is>
@@ -26028,7 +26109,7 @@
       </c>
       <c r="D353" s="48">
         <f>F_vent_ex+MAX(0,O2_src_l+H2_src_l-CO2_fix_l)</f>
-        <v>0.0001515178050535</v>
+        <v>0.0001883044451254</v>
       </c>
       <c r="E353" s="67" t="inlineStr">
         <is>
@@ -26054,7 +26135,7 @@
       </c>
       <c r="D354" s="48">
         <f>F_gap_l*t_gap_h/n_hs_gas</f>
-        <v>0.300906651909</v>
+        <v>0.264901073915</v>
       </c>
       <c r="E354" s="67" t="inlineStr">
         <is>
@@ -26080,7 +26161,7 @@
       </c>
       <c r="D355" s="48">
         <f>IF(x_hs_l&gt;0,(1-EXP(-x_hs_l))/x_hs_l,1)</f>
-        <v>0.863567280859</v>
+        <v>0.878509649469</v>
       </c>
       <c r="E355" s="67" t="inlineStr">
         <is>
@@ -26106,7 +26187,7 @@
       </c>
       <c r="D356" s="48">
         <f>IF(x_hs_l&gt;0,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2)</f>
-        <v>0.453405460715</v>
+        <v>0.458625360539</v>
       </c>
       <c r="E356" s="67" t="inlineStr">
         <is>
@@ -26132,7 +26213,7 @@
       </c>
       <c r="D357" s="48">
         <f>S_O2_l*t_gap_h/n_hs_gas</f>
-        <v>0.098881072437</v>
+        <v>0.080885255453</v>
       </c>
       <c r="E357" s="67" t="inlineStr">
         <is>
@@ -26158,7 +26239,7 @@
       </c>
       <c r="D358" s="48">
         <f>dy_O2_l*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.117340493152</v>
+        <v>0.09900408513</v>
       </c>
       <c r="E358" s="68" t="inlineStr">
         <is>
@@ -26184,7 +26265,7 @@
       </c>
       <c r="D359" s="48">
         <f>y_O2_end_l*flush_ret</f>
-        <v>0.043167155048</v>
+        <v>0.036421567511</v>
       </c>
       <c r="E359" s="68" t="inlineStr">
         <is>
@@ -26210,7 +26291,7 @@
       </c>
       <c r="D360" s="48">
         <f>y_O2_post_l*phi_hs_l+dy_O2_l*psi_hs_l</f>
-        <v>0.082110960911</v>
+        <v>0.069092727952</v>
       </c>
       <c r="E360" s="68" t="inlineStr">
         <is>
@@ -26236,7 +26317,7 @@
       </c>
       <c r="D361" s="48">
         <f>DO_surf_excess_lag+H_O2_T*P_atm*y_O2_mf_l</f>
-        <v>0.220552478156</v>
+        <v>0.205900701595</v>
       </c>
       <c r="E361" s="67" t="inlineStr">
         <is>
@@ -26262,7 +26343,7 @@
       </c>
       <c r="D362" s="48">
         <f>DO_surf_excess_lag+H_O2_T*P_atm*y_O2_avg_l</f>
-        <v>0.227898435401</v>
+        <v>0.212069565945</v>
       </c>
       <c r="E362" s="68" t="inlineStr">
         <is>
@@ -26288,7 +26369,7 @@
       </c>
       <c r="D363" s="48">
         <f>DO_surf_excess_lag+H_O2_T*P_atm*MAX(y_O2_avg_l,y_O2_end_l-(S_O2_l-F_gap_l*y_O2_end_l)/n_hs_gas*tau_L_h)</f>
-        <v>0.256671410883</v>
+        <v>0.231369990147</v>
       </c>
       <c r="E363" s="68" t="inlineStr">
         <is>
@@ -26314,7 +26395,7 @@
       </c>
       <c r="D364" s="48">
         <f>DO_avg_l*M_O2</f>
-        <v>7.292294135948</v>
+        <v>6.785801971106</v>
       </c>
       <c r="E364" s="68" t="inlineStr">
         <is>
@@ -26340,7 +26421,7 @@
       </c>
       <c r="D365" s="48">
         <f>DO_peak_l*M_O2</f>
-        <v>8.21297180544</v>
+        <v>7.403376944733</v>
       </c>
       <c r="E365" s="68" t="inlineStr">
         <is>
@@ -26444,7 +26525,7 @@
       </c>
       <c r="D369" s="28" t="str">
         <f>IF(DO_peak_l&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
-        <v>peak 8.2 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 7.4 mg/L under the 11.7 mg/L ceiling</v>
       </c>
       <c r="E369" s="67" t="inlineStr">
         <is>
@@ -26470,7 +26551,7 @@
       </c>
       <c r="D371" s="48">
         <f>IF(O2_sizing_phase=phase_name_1,F_gap_g,IF(O2_sizing_phase=phase_name_2,F_gap_l,NA()))</f>
-        <v>0.0</v>
+        <v>3.67866400719e-05</v>
       </c>
       <c r="E371" s="67" t="inlineStr">
         <is>
@@ -26496,7 +26577,7 @@
       </c>
       <c r="D372" s="48">
         <f>IF(O2_sizing_phase=phase_name_1,DO_avg_g,IF(O2_sizing_phase=phase_name_2,DO_avg_l,NA()))</f>
-        <v>0.082338279323</v>
+        <v>0.082341896405</v>
       </c>
       <c r="E372" s="68" t="inlineStr">
         <is>
@@ -26522,7 +26603,7 @@
       </c>
       <c r="D373" s="48">
         <f>IF(O2_sizing_phase=phase_name_1,DO_peak_g,IF(O2_sizing_phase=phase_name_2,DO_peak_l,NA()))</f>
-        <v>0.094535887493</v>
+        <v>0.091717883745</v>
       </c>
       <c r="E373" s="68" t="inlineStr">
         <is>
@@ -26533,7 +26614,7 @@
     <row r="374">
       <c r="A374" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peak DO vs organism band — sizing phase</t>
+          <t xml:space="preserve">DO vs organism band — mean vs optimum, peak vs impairment (sizing phase)</t>
         </is>
       </c>
       <c r="B374" s="18" t="inlineStr">
@@ -26547,12 +26628,12 @@
         </is>
       </c>
       <c r="D374" s="28" t="str">
-        <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_impair)),IF(DO_peak_sched*M_O2&lt;=DO_opt,"peak at/under optimum",IF(DO_peak_sched*M_O2&lt;DO_impair,"peak above optimum, under impairment","PEAK OVER IMPAIRMENT")),IF(DO_peak_sched&lt;=O2_ceil_C,"organism band unknown – peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L is under the inhibition ceiling","organism band unknown – PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER THE INHIBITION CEILING"))</f>
-        <v>organism band unknown – peak 3.0 mg/L is under the inhibition ceiling</v>
+        <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_impair)),IF(DO_peak_sched*M_O2&lt;DO_impair,"peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L under impairment","PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER IMPAIRMENT")&amp;IF(DO_avg_sched*M_O2&lt;=DO_opt,"; mean "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L at/under optimum","; MEAN "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L ABOVE OPTIMUM"),IF(DO_peak_sched&lt;=O2_ceil_C,"organism band unknown – peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L is under the inhibition ceiling","organism band unknown – PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER THE INHIBITION CEILING"))</f>
+        <v>organism band unknown – peak 2.9 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E374" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Replaces the tautological D109 as the Summary O₂ check: the sawtooth peak against the organism band, or against the inhibition ceiling when the band is unmeasured.</t>
+          <t xml:space="preserve">The Summary O₂ check, rule (a): each statistic against what it is for — the cycle MEAN (DO_avg_sched) against the organism optimum (the schedule is sized on the mean; the optimum is a time-averaged quantity) and the sawtooth PEAK (DO_peak_sched) against the impairment threshold (what a transient must stay under). With the band unmeasured, the peak is tested against the inhibition ceiling.</t>
         </is>
       </c>
     </row>
@@ -26574,7 +26655,7 @@
       </c>
       <c r="D375" s="48">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*t_gap_h/(V_L_m3+Vg_CO2)</f>
-        <v>-0.19762042649</v>
+        <v>-0.139866823543</v>
       </c>
       <c r="E375" s="67" t="inlineStr">
         <is>
@@ -26600,7 +26681,7 @@
       </c>
       <c r="D376" s="48">
         <f>k_eff_CO2*t_off_CO2</f>
-        <v>0.0</v>
+        <v>0.009083630066</v>
       </c>
       <c r="E376" s="67" t="inlineStr">
         <is>
@@ -26626,7 +26707,7 @@
       </c>
       <c r="D377" s="48">
         <f>IF(pool_x&gt;0,(1-EXP(-pool_x))/pool_x,1)</f>
-        <v>1.0</v>
+        <v>0.99547190585</v>
       </c>
       <c r="E377" s="67" t="inlineStr">
         <is>
@@ -26652,7 +26733,7 @@
       </c>
       <c r="D378" s="48">
         <f>IF(pool_x&gt;0,(pool_x-1+EXP(-pool_x))/pool_x^2,1/2)</f>
-        <v>0.5</v>
+        <v>0.498489493433</v>
       </c>
       <c r="E378" s="67" t="inlineStr">
         <is>
@@ -26678,7 +26759,7 @@
       </c>
       <c r="D379" s="48">
         <f>pool_D_raw*pool_phi</f>
-        <v>-0.19762042649</v>
+        <v>-0.139233493397</v>
       </c>
       <c r="E379" s="67" t="inlineStr">
         <is>
@@ -26730,7 +26811,7 @@
       </c>
       <c r="D381" s="48">
         <f>IF(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_atm*F_vent_ex)/(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
-        <v>0.968360861681</v>
+        <v>0.929374836165</v>
       </c>
       <c r="E381" s="67" t="inlineStr">
         <is>
@@ -26756,11 +26837,225 @@
       </c>
       <c r="D382" s="48">
         <f>y_CO2_mf*C_sat_CO2</f>
-        <v>32.379324222241</v>
+        <v>31.075738740549</v>
       </c>
       <c r="E382" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">Henry equilibrium with the flux-mean headspace CO₂; compare with CO2_cyc_avg_new (D200).</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEADSPACE BALANCE (cont.) — open vent and air ingress, anodic H₂ oxidation, pre-pulse H₂, vacuum check</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  valid vent model 3</t>
+        </is>
+      </c>
+      <c r="B384" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vent_name_3</t>
+        </is>
+      </c>
+      <c r="C384" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D384" s="131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open vent</t>
+        </is>
+      </c>
+      <c r="E384" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A plain needle or tube with no forced flow: air is drawn back after each pulse to refill what the liquid absorbs (no check valve), at the equivalent continuous ingress Q_backdraw (D385). Unsure which vent you have → this one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open-vent back-draw (equivalent continuous air ingress)</t>
+        </is>
+      </c>
+      <c r="B385" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q_backdraw</t>
+        </is>
+      </c>
+      <c r="C385" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D385" s="131">
+        <v>0.015</v>
+      </c>
+      <c r="E385" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ODE-equivalent pressure back-draw at the default schedule (review R4: limit-cycle ODE, open vent, no exchange, ≈0.16 mL of air per 12.7 min cycle). Schedule-dependent, coarse — measure (pressure-decay or headspace-O₂ tracer). Used only when vent_model = "Open vent".</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Air ingress for the vent model in use</t>
+        </is>
+      </c>
+      <c r="B386" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q_vent_used</t>
+        </is>
+      </c>
+      <c r="C386" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D386" s="48">
+        <f>IF(vent_model=vent_name_1,0,IF(vent_model=vent_name_3,Q_backdraw,IF(vent_model=vent_name_2,Q_vent,NA())))</f>
+        <v>0.015</v>
+      </c>
+      <c r="E386" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0 for "Outflow only" (check valve), Q_backdraw for "Open vent", the measured Q_vent for "Air exchange"; anything else #N/A by design. The vent is a continuum: 0 is a true check valve. Feeds F_vent_ex (D308) and Summary D113.</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) H₂ oxidised at the anode</t>
+        </is>
+      </c>
+      <c r="B387" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_HOR_mt</t>
+        </is>
+      </c>
+      <c r="C387" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D387" s="142">
+        <f>Electrochemistry!$D$149</f>
+        <v>0.0</v>
+      </c>
+      <c r="E387" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D149 (r_H2_HOR; 0 while f_HOR_anode is a data gap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace H₂ just before a pulse — lag</t>
+        </is>
+      </c>
+      <c r="B388" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_H2_end_l</t>
+        </is>
+      </c>
+      <c r="C388" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D388" s="48">
+        <f>H2_src_l*t_gap_h/n_hs_gas*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
+        <v>0.175164116673</v>
+      </c>
+      <c r="E388" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The H₂ analogue of y_O2_end_l (D358): periodic sawtooth top of the lag headspace at the schedule in use (no H₂ in air). The flammability verdict uses the mean-field mix; this is how high the vial gets before each pulse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace pressure sag per cycle if the vent held a vacuum</t>
+        </is>
+      </c>
+      <c r="B389" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hs_sag</t>
+        </is>
+      </c>
+      <c r="C389" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D389" s="48">
+        <f>(pool_a*(C_cycle_peak-C_cycle_start)*(V_L_m3+Vg_CO2)+MAX(0,CO2_fix_sched-O2_src_sched-H2_src_sched)*t_gap_h)/n_hs_gas</f>
+        <v>0.059351496276</v>
+      </c>
+      <c r="E389" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upper bound on the per-gap pressure deficit (fraction of 1 atm) that an outflow-only (check-valve) headspace implies: the CO₂ the liquid absorbs after each pulse plus the fixation that outruns gas evolution, over the headspace inventory. The limit-cycle ODE gives somewhat less (≈0.022 vs ≈0.03 at the outflow-only default).</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Largest sag a sealed cap is taken to hold</t>
+        </is>
+      </c>
+      <c r="B390" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hs_sag_max</t>
+        </is>
+      </c>
+      <c r="C390" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D390" s="131">
+        <v>0.05</v>
+      </c>
+      <c r="E390" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: the per-cycle pressure deficit (≈5 kPa) a check valve or sealed cap is taken to hold without drawing air back. Confirm on the hardware.</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Outflow-only headspace physically plausible?</t>
+        </is>
+      </c>
+      <c r="B391" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hs_sag_chk</t>
+        </is>
+      </c>
+      <c r="C391" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D391" s="28" t="str">
+        <f>IF(F_vent_ex&gt;0,"n/a – the vent admits air (Open vent / Air exchange), so the headspace refills",IF(hs_sag&gt;hs_sag_max,"HEADSPACE SAGS "&amp;TEXT(hs_sag,"0%")&amp;" below 1 atm each cycle – a real cap will draw air back: use Open vent or Air exchange","OK – sag "&amp;TEXT(hs_sag,"0%")&amp;" per cycle, within what a sealed cap holds"))</f>
+        <v>n/a – the vent admits air (Open vent / Air exchange), so the headspace refills</v>
+      </c>
+      <c r="E391" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Flags the vacuum the check-valve model needs. When it fires, "Outflow only" is not a physical description of the vial.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: cross-sheet references via named imports; header-matched table lookups (values identical)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -780,6 +780,21 @@
     <definedName name="hs_sag" localSheetId="5">'Mass Transfer'!$D$389</definedName>
     <definedName name="hs_sag_max" localSheetId="5">'Mass Transfer'!$D$390</definedName>
     <definedName name="hs_sag_chk" localSheetId="5">'Mass Transfer'!$D$391</definedName>
+    <definedName name="Reactor_sel" localSheetId="7">Calibrations!$D$157</definedName>
+    <definedName name="organism_sel" localSheetId="7">Calibrations!$D$158</definedName>
+    <definedName name="rx_ver" localSheetId="7">Calibrations!$D$159</definedName>
+    <definedName name="A_x" localSheetId="7">Calibrations!$D$160</definedName>
+    <definedName name="R_gas" localSheetId="7">Calibrations!$D$161</definedName>
+    <definedName name="F_const" localSheetId="7">Calibrations!$D$162</definedName>
+    <definedName name="p_sat_w" localSheetId="7">Calibrations!$D$163</definedName>
+    <definedName name="V_charge" localSheetId="2">Electrochemistry!$D$153</definedName>
+    <definedName name="organism_sel" localSheetId="2">Electrochemistry!$D$154</definedName>
+    <definedName name="V_charge" localSheetId="3">Chemistry!$D$279</definedName>
+    <definedName name="media_sel" localSheetId="3">Chemistry!$D$280</definedName>
+    <definedName name="override_spg_dur_s" localSheetId="0">Summary!$G$13</definedName>
+    <definedName name="override_spg_int_min" localSheetId="0">Summary!$G$15</definedName>
+    <definedName name="override_spg_dur_s" localSheetId="5">'Mass Transfer'!$D$392</definedName>
+    <definedName name="override_spg_int_min" localSheetId="5">'Mass Transfer'!$D$393</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -10798,7 +10813,7 @@
         <v>146</v>
       </c>
       <c r="D18" s="139">
-        <f>VLOOKUP(rx_ver,$A$84:$I$87,7,FALSE)</f>
+        <f>VLOOKUP(rx_ver,$A$84:$I$87,MATCH("vial OD (mm)",$A$83:$I$83,0),FALSE)</f>
         <v>27.48</v>
       </c>
       <c r="E18" s="99" t="s">
@@ -10885,7 +10900,7 @@
         <v>146</v>
       </c>
       <c r="D22" s="140">
-        <f>IF(ISNUMBER(cal_Dint),cal_Dint,VLOOKUP(rx_ver,$A$84:$I$87,4,FALSE))</f>
+        <f>IF(ISNUMBER(cal_Dint),cal_Dint,VLOOKUP(rx_ver,$A$84:$I$87,MATCH("usable depth (mm)",$A$83:$I$83,0),FALSE))</f>
         <v>55.0</v>
       </c>
       <c r="E22" s="99" t="s">
@@ -10907,7 +10922,7 @@
         <v>57</v>
       </c>
       <c r="D23" s="140">
-        <f>VLOOKUP(rx_ver,$A$84:$I$87,5,FALSE)</f>
+        <f>VLOOKUP(rx_ver,$A$84:$I$87,MATCH("max working (mL)",$A$83:$I$83,0),FALSE)</f>
         <v>16.0</v>
       </c>
       <c r="E23" s="99" t="s">
@@ -10929,7 +10944,7 @@
         <v>57</v>
       </c>
       <c r="D24" s="140">
-        <f>IF(ISNUMBER(cal_Vtot),cal_Vtot,VLOOKUP(rx_ver,$A$84:$I$87,6,FALSE))</f>
+        <f>IF(ISNUMBER(cal_Vtot),cal_Vtot,VLOOKUP(rx_ver,$A$84:$I$87,MATCH("total vial (mL)",$A$83:$I$83,0),FALSE))</f>
         <v>20.0</v>
       </c>
       <c r="E24" s="99" t="s">
@@ -11514,7 +11529,7 @@
       </c>
       <c r="C51" s="20"/>
       <c r="D51" s="28" t="str">
-        <f>VLOOKUP(reactor_sel,$A$59:$B$80,2,FALSE)</f>
+        <f>VLOOKUP(reactor_sel,$A$59:$B$80,MATCH("Type",$A$58:$B$58,0),FALSE)</f>
         <v>MEP0.3</v>
       </c>
       <c r="E51" s="20"/>
@@ -11532,7 +11547,7 @@
       </c>
       <c r="C52" s="20"/>
       <c r="D52" s="28">
-        <f>VLOOKUP(rx_ver,$A$84:$I$87,8,FALSE)</f>
+        <f>VLOOKUP(rx_ver,$A$84:$I$87,MATCH("stir bar L (mm)",$A$83:$I$83,0),FALSE)</f>
         <v>12.0</v>
       </c>
       <c r="E52" s="20"/>
@@ -12821,7 +12836,7 @@
         <v>135</v>
       </c>
       <c r="D27" s="139">
-        <f>VLOOKUP(electrode_sel,$A$35:$I$38,9,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("z_e_ORR",$A$34:$N$34,0),FALSE)</f>
         <v>2.0</v>
       </c>
       <c r="E27" s="114" t="inlineStr">
@@ -12904,7 +12919,7 @@
       </c>
       <c r="C31" s="20"/>
       <c r="D31" s="28" t="str">
-        <f>VLOOKUP(electrode_sel,$A$35:$I$38,4,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("sparger",$A$34:$N$34,0),FALSE)</f>
         <v>Tube</v>
       </c>
       <c r="E31" s="20"/>
@@ -12922,7 +12937,7 @@
       </c>
       <c r="C32" s="20"/>
       <c r="D32" s="28">
-        <f>IF(ISNUMBER(cal_sinter),cal_sinter,IF(ISNUMBER(VLOOKUP(electrode_sel,$A$35:$I$38,5,FALSE)),VLOOKUP(electrode_sel,$A$35:$I$38,5,FALSE),0))</f>
+        <f>IF(ISNUMBER(cal_sinter),cal_sinter,IF(ISNUMBER(VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("sinter porosity",$A$34:$N$34,0),FALSE)),VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("sinter porosity",$A$34:$N$34,0),FALSE),0))</f>
         <v>0.0</v>
       </c>
       <c r="E32" s="147" t="s">
@@ -13193,7 +13208,7 @@
         <v>135</v>
       </c>
       <c r="D41" s="48" t="str">
-        <f>VLOOKUP(electrode_sel,$A$35:$N$38,10,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("anode shape",$A$34:$N$34,0),FALSE)</f>
         <v>rod</v>
       </c>
       <c r="E41" s="99" t="s">
@@ -13211,7 +13226,7 @@
         <v>146</v>
       </c>
       <c r="D42" s="48">
-        <f>VLOOKUP(electrode_sel,$A$35:$N$38,3,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("anode dia (mm)",$A$34:$N$34,0),FALSE)</f>
         <v>6.0</v>
       </c>
       <c r="E42" s="99" t="s">
@@ -13229,7 +13244,7 @@
         <v>135</v>
       </c>
       <c r="D43" s="48" t="str">
-        <f>VLOOKUP(electrode_sel,$A$35:$N$38,13,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("cathode shape",$A$34:$N$34,0),FALSE)</f>
         <v>rod</v>
       </c>
       <c r="E43" s="99" t="s">
@@ -13247,7 +13262,7 @@
         <v>146</v>
       </c>
       <c r="D44" s="48">
-        <f>VLOOKUP(electrode_sel,$A$35:$N$38,7,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("cathode dia (mm)",$A$34:$N$34,0),FALSE)</f>
         <v>6.0</v>
       </c>
       <c r="E44" s="99" t="s">
@@ -13357,7 +13372,7 @@
         <v>1282</v>
       </c>
       <c r="D50" s="48">
-        <f>VLOOKUP(electrode_sel,$A$35:$N$38,11,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("anode j cont (mA/cm²)",$A$34:$N$34,0),FALSE)</f>
         <v>100.0</v>
       </c>
       <c r="E50" s="99" t="s">
@@ -13375,7 +13390,7 @@
         <v>1282</v>
       </c>
       <c r="D51" s="48">
-        <f>VLOOKUP(electrode_sel,$A$35:$N$38,12,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("anode j max (mA/cm²)",$A$34:$N$34,0),FALSE)</f>
         <v>500.0</v>
       </c>
       <c r="E51" s="99" t="s">
@@ -13461,7 +13476,7 @@
         <v>1282</v>
       </c>
       <c r="D56" s="48">
-        <f>IF(ISNUMBER(cal_j_opt),cal_j_opt,IFERROR(VLOOKUP(Summary!$D$4,$A$66:$E$71,2,FALSE),j_opt_default))</f>
+        <f>IF(ISNUMBER(cal_j_opt),cal_j_opt,IFERROR(VLOOKUP(organism_sel,$A$66:$E$71,MATCH("j_opt",$A$65:$E$65,0),FALSE),j_opt_default))</f>
         <v>2.14</v>
       </c>
       <c r="E56" s="99" t="s">
@@ -13479,7 +13494,7 @@
         <v>1282</v>
       </c>
       <c r="D57" s="48">
-        <f>IF(ISNUMBER(cal_j_ceiling),cal_j_ceiling,IFERROR(VLOOKUP(Summary!$D$4,$A$66:$E$71,3,FALSE),j_ceiling_default))</f>
+        <f>IF(ISNUMBER(cal_j_ceiling),cal_j_ceiling,IFERROR(VLOOKUP(organism_sel,$A$66:$E$71,MATCH("j_ceiling",$A$65:$E$65,0),FALSE),j_ceiling_default))</f>
         <v>4.29</v>
       </c>
       <c r="E57" s="99" t="s">
@@ -13497,7 +13512,7 @@
         <v>135</v>
       </c>
       <c r="D58" s="48" t="str">
-        <f>IFERROR(VLOOKUP(Summary!$D$4,$A$66:$E$71,4,FALSE),"unknown")</f>
+        <f>IFERROR(VLOOKUP(organism_sel,$A$66:$E$71,MATCH("confidence",$A$65:$E$65,0),FALSE),"unknown")</f>
         <v>med</v>
       </c>
       <c r="E58" s="99" t="s">
@@ -13587,7 +13602,7 @@
         <v>135</v>
       </c>
       <c r="D63" s="48" t="str">
-        <f>VLOOKUP(electrode_sel,$A$35:$N$38,2,FALSE)</f>
+        <f>VLOOKUP(electrode_sel,$A$35:$N$38,MATCH("anode material",$A$34:$N$34,0),FALSE)</f>
         <v>Pt/Ti</v>
       </c>
       <c r="E63" s="99" t="s">
@@ -13856,8 +13871,10 @@
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>1635</v>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reactor liquid volume (V_charge in litres)</t>
+        </is>
       </c>
       <c r="B82" s="18" t="s">
         <v>1636</v>
@@ -13866,11 +13883,13 @@
         <v>858</v>
       </c>
       <c r="D82" s="141">
-        <f>Biology!$D$6/1000</f>
+        <f>V_charge/1000</f>
         <v>0.015</v>
       </c>
-      <c r="E82" s="67" t="s">
-        <v>859</v>
+      <c r="E82" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_charge (D153, mL) / 1000 → L</t>
+        </is>
       </c>
     </row>
     <row r="83" spans="1:5" ht="60" x14ac:dyDescent="0.2">
@@ -14954,6 +14973,58 @@
       <c r="E152" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">r_H2O2 scaled to the lag-phase DO (D150): the cathodic O₂ flux is first order in DO, and before uptake starts DO runs above the design value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) reactor liquid charge</t>
+        </is>
+      </c>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_charge</t>
+        </is>
+      </c>
+      <c r="C153" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D153" s="141">
+        <f>Biology!$D$6</f>
+        <v>15.0</v>
+      </c>
+      <c r="E153" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Biology (V_charge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) organism selected on Summary</t>
+        </is>
+      </c>
+      <c r="B154" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">organism_sel</t>
+        </is>
+      </c>
+      <c r="C154" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D154" s="141" t="str">
+        <f>Summary!$D$4</f>
+        <v>UdG (mixed)</v>
+      </c>
+      <c r="E154" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Summary (organism_sel)</t>
         </is>
       </c>
     </row>
@@ -15111,8 +15182,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="17" t="s">
-        <v>856</v>
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reactor liquid volume (V_charge in litres)</t>
+        </is>
       </c>
       <c r="B8" s="18" t="s">
         <v>857</v>
@@ -15121,11 +15194,13 @@
         <v>858</v>
       </c>
       <c r="D8" s="64">
-        <f>Biology!$D$6/1000</f>
+        <f>V_charge/1000</f>
         <v>0.015</v>
       </c>
-      <c r="E8" s="51" t="s">
-        <v>859</v>
+      <c r="E8" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_charge (D279, mL) / 1000 → L</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -15668,7 +15743,7 @@
         <v>934</v>
       </c>
       <c r="D44" s="149">
-        <f>IF(Summary!$D$5="MC02",SID_mc02,IF(Summary!$D$5="UdG phosphate",SID_udg,NA()))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),SID_mc02,IF(media_sel=INDEX(MediaList,2),SID_udg,NA()))</f>
         <v>0.063142947676</v>
       </c>
       <c r="E44" s="51" t="s">
@@ -15686,7 +15761,7 @@
         <v>938</v>
       </c>
       <c r="D45" s="149">
-        <f>IF(Summary!$D$5="MC02",PT_mc02,IF(Summary!$D$5="UdG phosphate",PT_udg,NA()))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),PT_mc02,IF(media_sel=INDEX(MediaList,2),PT_udg,NA()))</f>
         <v>0.037329366919</v>
       </c>
       <c r="E45" s="51" t="s">
@@ -15704,7 +15779,7 @@
         <v>942</v>
       </c>
       <c r="D46" s="149">
-        <f>IF(Summary!$D$5="MC02",NT_mc02,IF(Summary!$D$5="UdG phosphate",NT_udg,NA()))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),NT_mc02,IF(media_sel=INDEX(MediaList,2),NT_udg,NA()))</f>
         <v>0.007113667323</v>
       </c>
       <c r="E46" s="51" t="s">
@@ -15722,7 +15797,7 @@
         <v>946</v>
       </c>
       <c r="D47" s="149">
-        <f>IF(Summary!$D$5="MC02",Cl_mc02,IF(Summary!$D$5="UdG phosphate",Cl_udg,NA()))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),Cl_mc02,IF(media_sel=INDEX(MediaList,2),Cl_udg,NA()))</f>
         <v>0.0001802126509281</v>
       </c>
       <c r="E47" s="51" t="s">
@@ -17569,7 +17644,7 @@
         <v>1507</v>
       </c>
       <c r="D180" s="141">
-        <f>IF(Summary!$D$5="MC02",kappa0_mc02,IF(Summary!$D$5="UdG phosphate",kappa0_udg,NA()))*kappa_fI*(1+kappa_TC*(TKc-T_ref))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),kappa0_mc02,IF(media_sel=INDEX(MediaList,2),kappa0_udg,NA()))*kappa_fI*(1+kappa_TC*(TKc-T_ref))</f>
         <v>0.706946657056</v>
       </c>
       <c r="E180" s="67" t="s">
@@ -17628,7 +17703,7 @@
         <v>1098</v>
       </c>
       <c r="D185" s="141">
-        <f>IF(Summary!$D$5="MC02",I_mc02,IF(Summary!$D$5="UdG phosphate",I_udg,NA()))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),I_mc02,IF(media_sel=INDEX(MediaList,2),I_udg,NA()))</f>
         <v>0.109739973238</v>
       </c>
       <c r="E185" s="67" t="s">
@@ -19038,6 +19113,58 @@
       <c r="E278" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">At steady state the chloride pool splits free : combined = 1 : kτ (row 271 and D143), so only this share is available to the anode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) reactor liquid charge</t>
+        </is>
+      </c>
+      <c r="B279" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_charge</t>
+        </is>
+      </c>
+      <c r="C279" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D279" s="141">
+        <f>Biology!$D$6</f>
+        <v>15.0</v>
+      </c>
+      <c r="E279" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Biology (V_charge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) medium selected on Summary</t>
+        </is>
+      </c>
+      <c r="B280" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">media_sel</t>
+        </is>
+      </c>
+      <c r="C280" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D280" s="141" t="str">
+        <f>Summary!$D$5</f>
+        <v>UdG phosphate</v>
+      </c>
+      <c r="E280" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Summary (media_sel)</t>
         </is>
       </c>
     </row>
@@ -19891,7 +20018,7 @@
         <v>102</v>
       </c>
       <c r="D45" s="32" t="e">
-        <f>IF(ISNUMBER(cal_DO_min),cal_DO_min,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,2,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,2,FALSE),NA()))</f>
+        <f>IF(ISNUMBER(cal_DO_min),cal_DO_min,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,MATCH("minimum DO",$A$51:$F$51,0),FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,MATCH("minimum DO",$A$51:$F$51,0),FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
       <c r="E45" s="20"/>
@@ -19908,7 +20035,7 @@
         <v>102</v>
       </c>
       <c r="D46" s="28" t="e">
-        <f>IF(ISNUMBER(cal_DO_opt),cal_DO_opt,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,3,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,3,FALSE),NA()))</f>
+        <f>IF(ISNUMBER(cal_DO_opt),cal_DO_opt,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,MATCH("optimum DO",$A$51:$F$51,0),FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,MATCH("optimum DO",$A$51:$F$51,0),FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
       <c r="E46" s="20"/>
@@ -19925,7 +20052,7 @@
         <v>102</v>
       </c>
       <c r="D47" s="28" t="e">
-        <f>IF(ISNUMBER(cal_DO_impair),cal_DO_impair,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,4,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,4,FALSE),NA()))</f>
+        <f>IF(ISNUMBER(cal_DO_impair),cal_DO_impair,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,MATCH("impairment DO",$A$51:$F$51,0),FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,MATCH("impairment DO",$A$51:$F$51,0),FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
       <c r="E47" s="20"/>
@@ -19942,7 +20069,7 @@
         <v>102</v>
       </c>
       <c r="D48" s="28" t="e">
-        <f>IF(ISNUMBER(cal_DO_toxic),cal_DO_toxic,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,5,FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,5,FALSE),NA()))</f>
+        <f>IF(ISNUMBER(cal_DO_toxic),cal_DO_toxic,IF(ISNUMBER(VLOOKUP(organism_sel,$A$52:$F$57,MATCH("toxic DO",$A$51:$F$51,0),FALSE)),VLOOKUP(organism_sel,$A$52:$F$57,MATCH("toxic DO",$A$51:$F$51,0),FALSE),NA()))</f>
         <v>#N/A</v>
       </c>
       <c r="E48" s="20"/>
@@ -22093,8 +22220,10 @@
       <c r="F66" s="20"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A67" s="17" t="s">
-        <v>681</v>
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Stir-bar speed</t>
+        </is>
       </c>
       <c r="B67" s="18" t="s">
         <v>682</v>
@@ -22106,8 +22235,10 @@
         <f>Summary!$D$7</f>
         <v>1000.0</v>
       </c>
-      <c r="E67" s="68" t="s">
-        <v>684</v>
+      <c r="E67" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Summary (stir_rpm_set). Pioreactor stir setpoint. RPM floor ~125 (stalls below).</t>
+        </is>
       </c>
       <c r="F67" s="20"/>
     </row>
@@ -23072,7 +23203,7 @@
         <v>13</v>
       </c>
       <c r="D121" s="28">
-        <f>IF(AND(ISNUMBER(Summary!$G$13),Summary!$G$13&gt;0),Summary!$G$13,IF(sched_mode="Manual",spg_dur_man,IF(sched_mode="Optimal",spg_dur_opt,NA())))</f>
+        <f>IF(AND(ISNUMBER(override_spg_dur_s),override_spg_dur_s&gt;0),override_spg_dur_s,IF(sched_mode="Manual",spg_dur_man,IF(sched_mode="Optimal",spg_dur_opt,NA())))</f>
         <v>0.784513049825</v>
       </c>
       <c r="E121" s="20"/>
@@ -23089,7 +23220,7 @@
         <v>67</v>
       </c>
       <c r="D122" s="28">
-        <f>IF(AND(ISNUMBER(Summary!$G$15),Summary!$G$15&gt;0),Summary!$G$15,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
+        <f>IF(AND(ISNUMBER(override_spg_int_min),override_spg_int_min&gt;0),override_spg_int_min,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
         <v>9.026013902172</v>
       </c>
       <c r="E122" s="20"/>
@@ -23500,7 +23631,7 @@
         <v>460</v>
       </c>
       <c r="D145" s="48">
-        <f>Biology!$D$31*P_atm</f>
+        <f>hs_H_CO2*P_atm</f>
         <v>33.43725</v>
       </c>
       <c r="E145" s="67" t="s">
@@ -23519,7 +23650,7 @@
         <v>460</v>
       </c>
       <c r="D146" s="48">
-        <f>Biology!$D$31*pCO2_air</f>
+        <f>hs_H_CO2*pCO2_air</f>
         <v>0.0132</v>
       </c>
       <c r="E146" s="67" t="s">
@@ -27056,6 +27187,58 @@
       <c r="E391" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">Flags the vacuum the check-valve model needs. When it fires, "Outflow only" is not a physical description of the vial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) sparge duration override</t>
+        </is>
+      </c>
+      <c r="B392" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">override_spg_dur_s</t>
+        </is>
+      </c>
+      <c r="C392" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D392" s="142">
+        <f>Summary!$G$13</f>
+        <v>0.0</v>
+      </c>
+      <c r="E392" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Summary (override_spg_dur_s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) sparge interval override</t>
+        </is>
+      </c>
+      <c r="B393" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">override_spg_int_min</t>
+        </is>
+      </c>
+      <c r="C393" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D393" s="142">
+        <f>Summary!$G$15</f>
+        <v>0.0</v>
+      </c>
+      <c r="E393" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Summary (override_spg_int_min)</t>
         </is>
       </c>
     </row>
@@ -29546,7 +29729,7 @@
         <v>321</v>
       </c>
       <c r="D16" s="48" t="str">
-        <f>IFERROR((COUNTIFS(C8:C15,Summary!$D$2,G8:G15,"y")*SUMPRODUCT((C8:C15=Summary!$D$2)*(G8:G15="y")*D8:D15*E8:E15)-SUMIFS(D8:D15,C8:C15,Summary!$D$2,G8:G15,"y")*SUMIFS(E8:E15,C8:C15,Summary!$D$2,G8:G15,"y"))/(COUNTIFS(C8:C15,Summary!$D$2,G8:G15,"y")*SUMPRODUCT((C8:C15=Summary!$D$2)*(G8:G15="y")*D8:D15*D8:D15)-SUMIFS(D8:D15,C8:C15,Summary!$D$2,G8:G15,"y")*SUMIFS(D8:D15,C8:C15,Summary!$D$2,G8:G15,"y")),"no included runs — model uses its default")</f>
+        <f>IFERROR((COUNTIFS(C8:C15,Reactor_sel,G8:G15,"y")*SUMPRODUCT((C8:C15=Reactor_sel)*(G8:G15="y")*D8:D15*E8:E15)-SUMIFS(D8:D15,C8:C15,Reactor_sel,G8:G15,"y")*SUMIFS(E8:E15,C8:C15,Reactor_sel,G8:G15,"y"))/(COUNTIFS(C8:C15,Reactor_sel,G8:G15,"y")*SUMPRODUCT((C8:C15=Reactor_sel)*(G8:G15="y")*D8:D15*D8:D15)-SUMIFS(D8:D15,C8:C15,Reactor_sel,G8:G15,"y")*SUMIFS(D8:D15,C8:C15,Reactor_sel,G8:G15,"y")),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
     </row>
@@ -29558,7 +29741,7 @@
         <v>325</v>
       </c>
       <c r="D17" s="48" t="str">
-        <f>IFERROR((SUMIFS(E8:E15,C8:C15,Summary!$D$2,G8:G15,"y")-((COUNTIFS(C8:C15,Summary!$D$2,G8:G15,"y")*SUMPRODUCT((C8:C15=Summary!$D$2)*(G8:G15="y")*D8:D15*E8:E15)-SUMIFS(D8:D15,C8:C15,Summary!$D$2,G8:G15,"y")*SUMIFS(E8:E15,C8:C15,Summary!$D$2,G8:G15,"y"))/(COUNTIFS(C8:C15,Summary!$D$2,G8:G15,"y")*SUMPRODUCT((C8:C15=Summary!$D$2)*(G8:G15="y")*D8:D15*D8:D15)-SUMIFS(D8:D15,C8:C15,Summary!$D$2,G8:G15,"y")*SUMIFS(D8:D15,C8:C15,Summary!$D$2,G8:G15,"y")))*SUMIFS(D8:D15,C8:C15,Summary!$D$2,G8:G15,"y"))/COUNTIFS(C8:C15,Summary!$D$2,G8:G15,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR((SUMIFS(E8:E15,C8:C15,Reactor_sel,G8:G15,"y")-((COUNTIFS(C8:C15,Reactor_sel,G8:G15,"y")*SUMPRODUCT((C8:C15=Reactor_sel)*(G8:G15="y")*D8:D15*E8:E15)-SUMIFS(D8:D15,C8:C15,Reactor_sel,G8:G15,"y")*SUMIFS(E8:E15,C8:C15,Reactor_sel,G8:G15,"y"))/(COUNTIFS(C8:C15,Reactor_sel,G8:G15,"y")*SUMPRODUCT((C8:C15=Reactor_sel)*(G8:G15="y")*D8:D15*D8:D15)-SUMIFS(D8:D15,C8:C15,Reactor_sel,G8:G15,"y")*SUMIFS(D8:D15,C8:C15,Reactor_sel,G8:G15,"y")))*SUMIFS(D8:D15,C8:C15,Reactor_sel,G8:G15,"y"))/COUNTIFS(C8:C15,Reactor_sel,G8:G15,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
     </row>
@@ -29621,7 +29804,7 @@
       <c r="G23" s="123"/>
       <c r="H23" s="123"/>
       <c r="I23" s="129" t="str">
-        <f>IFERROR(((G23-'Mass Transfer'!$D$206)*(E23/1000000)/('Mass Transfer'!$D$101*(F23+T_zero_C)))/(D23/(IF(H23="H2",z_e_H2,IF(H23="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G23-p_sat_w)*(E23/1000000)/(R_gas*(F23+T_zero_C)))/(D23/(IF(H23="H2",z_e_H2,IF(H23="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J23" s="129" t="str">
@@ -29642,7 +29825,7 @@
       <c r="G24" s="123"/>
       <c r="H24" s="123"/>
       <c r="I24" s="129" t="str">
-        <f>IFERROR(((G24-'Mass Transfer'!$D$206)*(E24/1000000)/('Mass Transfer'!$D$101*(F24+T_zero_C)))/(D24/(IF(H24="H2",z_e_H2,IF(H24="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G24-p_sat_w)*(E24/1000000)/(R_gas*(F24+T_zero_C)))/(D24/(IF(H24="H2",z_e_H2,IF(H24="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J24" s="129" t="str">
@@ -29663,7 +29846,7 @@
       <c r="G25" s="123"/>
       <c r="H25" s="123"/>
       <c r="I25" s="129" t="str">
-        <f>IFERROR(((G25-'Mass Transfer'!$D$206)*(E25/1000000)/('Mass Transfer'!$D$101*(F25+T_zero_C)))/(D25/(IF(H25="H2",z_e_H2,IF(H25="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G25-p_sat_w)*(E25/1000000)/(R_gas*(F25+T_zero_C)))/(D25/(IF(H25="H2",z_e_H2,IF(H25="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J25" s="129" t="str">
@@ -29684,7 +29867,7 @@
       <c r="G26" s="123"/>
       <c r="H26" s="123"/>
       <c r="I26" s="129" t="str">
-        <f>IFERROR(((G26-'Mass Transfer'!$D$206)*(E26/1000000)/('Mass Transfer'!$D$101*(F26+T_zero_C)))/(D26/(IF(H26="H2",z_e_H2,IF(H26="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G26-p_sat_w)*(E26/1000000)/(R_gas*(F26+T_zero_C)))/(D26/(IF(H26="H2",z_e_H2,IF(H26="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J26" s="129" t="str">
@@ -29705,7 +29888,7 @@
       <c r="G27" s="123"/>
       <c r="H27" s="123"/>
       <c r="I27" s="129" t="str">
-        <f>IFERROR(((G27-'Mass Transfer'!$D$206)*(E27/1000000)/('Mass Transfer'!$D$101*(F27+T_zero_C)))/(D27/(IF(H27="H2",z_e_H2,IF(H27="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G27-p_sat_w)*(E27/1000000)/(R_gas*(F27+T_zero_C)))/(D27/(IF(H27="H2",z_e_H2,IF(H27="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J27" s="129" t="str">
@@ -29726,7 +29909,7 @@
       <c r="G28" s="123"/>
       <c r="H28" s="123"/>
       <c r="I28" s="129" t="str">
-        <f>IFERROR(((G28-'Mass Transfer'!$D$206)*(E28/1000000)/('Mass Transfer'!$D$101*(F28+T_zero_C)))/(D28/(IF(H28="H2",z_e_H2,IF(H28="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G28-p_sat_w)*(E28/1000000)/(R_gas*(F28+T_zero_C)))/(D28/(IF(H28="H2",z_e_H2,IF(H28="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J28" s="129" t="str">
@@ -29747,7 +29930,7 @@
       <c r="G29" s="123"/>
       <c r="H29" s="123"/>
       <c r="I29" s="129" t="str">
-        <f>IFERROR(((G29-'Mass Transfer'!$D$206)*(E29/1000000)/('Mass Transfer'!$D$101*(F29+T_zero_C)))/(D29/(IF(H29="H2",z_e_H2,IF(H29="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G29-p_sat_w)*(E29/1000000)/(R_gas*(F29+T_zero_C)))/(D29/(IF(H29="H2",z_e_H2,IF(H29="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J29" s="129" t="str">
@@ -29768,7 +29951,7 @@
       <c r="G30" s="123"/>
       <c r="H30" s="123"/>
       <c r="I30" s="129" t="str">
-        <f>IFERROR(((G30-'Mass Transfer'!$D$206)*(E30/1000000)/('Mass Transfer'!$D$101*(F30+T_zero_C)))/(D30/(IF(H30="H2",z_e_H2,IF(H30="O2",z_e_O2,NA()))*Electrochemistry!$D$15)),"")</f>
+        <f>IFERROR(((G30-p_sat_w)*(E30/1000000)/(R_gas*(F30+T_zero_C)))/(D30/(IF(H30="H2",z_e_H2,IF(H30="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J30" s="129" t="str">
@@ -29788,7 +29971,7 @@
         <v>135</v>
       </c>
       <c r="D31" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(I23:I30,C23:C30,Summary!$D$2,K23:K30,"y",H23:H30,"H2"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(I23:I30,C23:C30,Reactor_sel,K23:K30,"y",H23:H30,"H2"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E31" s="97"/>
@@ -29810,7 +29993,7 @@
         <v>135</v>
       </c>
       <c r="D32" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(I23:I30,C23:C30,Summary!$D$2,K23:K30,"y",H23:H30,"O2"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(I23:I30,C23:C30,Reactor_sel,K23:K30,"y",H23:H30,"O2"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E32" s="97"/>
@@ -30070,7 +30253,7 @@
         <v>507</v>
       </c>
       <c r="D46" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(D38:D45,C38:C45,Summary!$D$2,F38:F45,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(D38:D45,C38:C45,Reactor_sel,F38:F45,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E46" s="97"/>
@@ -30358,7 +30541,7 @@
         <v>1421</v>
       </c>
       <c r="D60" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(F52:F59,C52:C59,Summary!$D$2,H52:H59,"y",B52:B59,SUMPRODUCT(MAX((C52:C59=Summary!$D$2)*(H52:H59="y")*B52:B59))),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(F52:F59,C52:C59,Reactor_sel,H52:H59,"y",B52:B59,SUMPRODUCT(MAX((C52:C59=Reactor_sel)*(H52:H59="y")*B52:B59))),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E60" s="97"/>
@@ -30498,7 +30681,7 @@
         <v/>
       </c>
       <c r="H66" s="129" t="str">
-        <f>IF(E66="","",IFERROR((E66/((ca_rho_0+ca_rho_k*F66)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E66="","",IFERROR((E66/((ca_rho_0+ca_rho_k*F66)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I66" s="129" t="str">
@@ -30529,7 +30712,7 @@
         <v/>
       </c>
       <c r="H67" s="129" t="str">
-        <f>IF(E67="","",IFERROR((E67/((ca_rho_0+ca_rho_k*F67)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E67="","",IFERROR((E67/((ca_rho_0+ca_rho_k*F67)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I67" s="129" t="str">
@@ -30560,7 +30743,7 @@
         <v/>
       </c>
       <c r="H68" s="129" t="str">
-        <f>IF(E68="","",IFERROR((E68/((ca_rho_0+ca_rho_k*F68)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E68="","",IFERROR((E68/((ca_rho_0+ca_rho_k*F68)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I68" s="129" t="str">
@@ -30591,7 +30774,7 @@
         <v/>
       </c>
       <c r="H69" s="129" t="str">
-        <f>IF(E69="","",IFERROR((E69/((ca_rho_0+ca_rho_k*F69)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E69="","",IFERROR((E69/((ca_rho_0+ca_rho_k*F69)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I69" s="129" t="str">
@@ -30622,7 +30805,7 @@
         <v/>
       </c>
       <c r="H70" s="129" t="str">
-        <f>IF(E70="","",IFERROR((E70/((ca_rho_0+ca_rho_k*F70)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E70="","",IFERROR((E70/((ca_rho_0+ca_rho_k*F70)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I70" s="129" t="str">
@@ -30653,7 +30836,7 @@
         <v/>
       </c>
       <c r="H71" s="129" t="str">
-        <f>IF(E71="","",IFERROR((E71/((ca_rho_0+ca_rho_k*F71)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E71="","",IFERROR((E71/((ca_rho_0+ca_rho_k*F71)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I71" s="129" t="str">
@@ -30684,7 +30867,7 @@
         <v/>
       </c>
       <c r="H72" s="129" t="str">
-        <f>IF(E72="","",IFERROR((E72/((ca_rho_0+ca_rho_k*F72)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E72="","",IFERROR((E72/((ca_rho_0+ca_rho_k*F72)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I72" s="129" t="str">
@@ -30715,7 +30898,7 @@
         <v/>
       </c>
       <c r="H73" s="129" t="str">
-        <f>IF(E73="","",IFERROR((E73/((ca_rho_0+ca_rho_k*F73)/1000))*1000/Geometry!$D$21,""))</f>
+        <f>IF(E73="","",IFERROR((E73/((ca_rho_0+ca_rho_k*F73)/1000))*1000/A_x,""))</f>
         <v/>
       </c>
       <c r="I73" s="129" t="str">
@@ -30743,7 +30926,7 @@
         <v>57</v>
       </c>
       <c r="D74" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(G66:G73,I66:I73,Geometry!$D$51,J66:J73,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(G66:G73,I66:I73,rx_ver,J66:J73,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E74" s="97"/>
@@ -30765,7 +30948,7 @@
         <v>146</v>
       </c>
       <c r="D75" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(H66:H73,I66:I73,Geometry!$D$51,J66:J73,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(H66:H73,I66:I73,rx_ver,J66:J73,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E75" s="97"/>
@@ -30791,7 +30974,7 @@
         </is>
       </c>
       <c r="D76" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(L66:L73,I66:I73,Geometry!$D$51,J66:J73,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(L66:L73,I66:I73,rx_ver,J66:J73,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E76" s="97"/>
@@ -30817,7 +31000,7 @@
         </is>
       </c>
       <c r="D77" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(N66:N73,I66:I73,Geometry!$D$51,J66:J73,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(N66:N73,I66:I73,rx_ver,J66:J73,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E77" s="97"/>
@@ -31073,7 +31256,7 @@
         <v>553</v>
       </c>
       <c r="D89" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(E81:E88,C81:C88,Summary!$D$2,G81:G88,"y",B81:B88,SUMPRODUCT(MAX((C81:C88=Summary!$D$2)*(G81:G88="y")*B81:B88))),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(E81:E88,C81:C88,Reactor_sel,G81:G88,"y",B81:B88,SUMPRODUCT(MAX((C81:C88=Reactor_sel)*(G81:G88="y")*B81:B88))),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E89" s="97"/>
@@ -31313,7 +31496,7 @@
         <v>102</v>
       </c>
       <c r="D103" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(D95:D102,C95:C102,Summary!$D$4,H95:H102,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(D95:D102,C95:C102,organism_sel,H95:H102,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E103" s="97"/>
@@ -31335,7 +31518,7 @@
         <v>102</v>
       </c>
       <c r="D104" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(E95:E102,C95:C102,Summary!$D$4,H95:H102,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(E95:E102,C95:C102,organism_sel,H95:H102,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E104" s="97"/>
@@ -31357,7 +31540,7 @@
         <v>102</v>
       </c>
       <c r="D105" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(F95:F102,C95:C102,Summary!$D$4,H95:H102,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(F95:F102,C95:C102,organism_sel,H95:H102,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E105" s="97"/>
@@ -31379,7 +31562,7 @@
         <v>102</v>
       </c>
       <c r="D106" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(G95:G102,C95:C102,Summary!$D$4,H95:H102,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(G95:G102,C95:C102,organism_sel,H95:H102,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E106" s="97"/>
@@ -31617,7 +31800,7 @@
         <v>1447</v>
       </c>
       <c r="D120" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(D112:D119,C112:C119,Summary!$D$4,G112:G119,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(D112:D119,C112:C119,organism_sel,G112:G119,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E120" s="97"/>
@@ -31639,7 +31822,7 @@
         <v>1447</v>
       </c>
       <c r="D121" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(E112:E119,C112:C119,Summary!$D$4,G112:G119,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(E112:E119,C112:C119,organism_sel,G112:G119,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E121" s="97"/>
@@ -31661,7 +31844,7 @@
         <v>1447</v>
       </c>
       <c r="D122" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(F112:F119,C112:C119,Summary!$D$4,G112:G119,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(F112:F119,C112:C119,organism_sel,G112:G119,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E122" s="97"/>
@@ -31897,7 +32080,7 @@
         <v>1282</v>
       </c>
       <c r="D136" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(D128:D135,C128:C135,Summary!$D$4,F128:F135,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(D128:D135,C128:C135,organism_sel,F128:F135,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E136" s="97"/>
@@ -31919,7 +32102,7 @@
         <v>1282</v>
       </c>
       <c r="D137" s="124" t="str">
-        <f>IFERROR(AVERAGEIFS(E128:E135,C128:C135,Summary!$D$4,F128:F135,"y"),"no included runs — model uses its default")</f>
+        <f>IFERROR(AVERAGEIFS(E128:E135,C128:C135,organism_sel,F128:F135,"y"),"no included runs — model uses its default")</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E137" s="97"/>
@@ -32243,6 +32426,188 @@
       <c r="E156" s="165" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D170 (rho_k)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Reactor selected on Summary</t>
+        </is>
+      </c>
+      <c r="B157" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reactor_sel</t>
+        </is>
+      </c>
+      <c r="C157" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D157" s="164" t="str">
+        <f>Summary!$D$2</f>
+        <v>ed04</v>
+      </c>
+      <c r="E157" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D2 (Reactor_sel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Organism selected on Summary</t>
+        </is>
+      </c>
+      <c r="B158" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">organism_sel</t>
+        </is>
+      </c>
+      <c r="C158" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D158" s="164" t="str">
+        <f>Summary!$D$4</f>
+        <v>UdG (mixed)</v>
+      </c>
+      <c r="E158" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D4 (organism_sel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Reactor type (resolved from reactor)</t>
+        </is>
+      </c>
+      <c r="B159" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rx_ver</t>
+        </is>
+      </c>
+      <c r="C159" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D159" s="164" t="str">
+        <f>Geometry!$D$51</f>
+        <v>MEP0.3</v>
+      </c>
+      <c r="E159" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Geometry!D51 (rx_ver)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Internal cross-sectional area</t>
+        </is>
+      </c>
+      <c r="B160" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A_x</t>
+        </is>
+      </c>
+      <c r="C160" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mm²</t>
+        </is>
+      </c>
+      <c r="D160" s="164">
+        <f>Geometry!$D$21</f>
+        <v>501.93100162698</v>
+      </c>
+      <c r="E160" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Geometry!D21 (A_x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Molar gas constant</t>
+        </is>
+      </c>
+      <c r="B161" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R_gas</t>
+        </is>
+      </c>
+      <c r="C161" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">J/mol/K</t>
+        </is>
+      </c>
+      <c r="D161" s="164">
+        <f>'Mass Transfer'!$D$101</f>
+        <v>8.314462618</v>
+      </c>
+      <c r="E161" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D101 (R_gas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Faraday constant</t>
+        </is>
+      </c>
+      <c r="B162" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_const</t>
+        </is>
+      </c>
+      <c r="C162" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C/mol</t>
+        </is>
+      </c>
+      <c r="D162" s="164">
+        <f>Electrochemistry!$D$15</f>
+        <v>96485.33212</v>
+      </c>
+      <c r="E162" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D15 (F_const)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Saturated water vapour pressure at reactor T</t>
+        </is>
+      </c>
+      <c r="B163" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p_sat_w</t>
+        </is>
+      </c>
+      <c r="C163" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pa</t>
+        </is>
+      </c>
+      <c r="D163" s="164">
+        <f>'Mass Transfer'!$D$206</f>
+        <v>3161.736035696692</v>
+      </c>
+      <c r="E163" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D206 (p_sat_w)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: pulse-volume intercept, carryover vs measured max flow, CO2 uptake ratio, bicarbonate/dry-gas/salting-out, CF thresholds named (0.67 s every 8.95 min, pH 6.20)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -795,6 +795,47 @@
     <definedName name="override_spg_int_min" localSheetId="0">Summary!$G$15</definedName>
     <definedName name="override_spg_dur_s" localSheetId="5">'Mass Transfer'!$D$392</definedName>
     <definedName name="override_spg_int_min" localSheetId="5">'Mass Transfer'!$D$393</definedName>
+    <definedName name="fit_n" localSheetId="5">'Mass Transfer'!$D$401</definedName>
+    <definedName name="fit_St" localSheetId="5">'Mass Transfer'!$D$402</definedName>
+    <definedName name="fit_SV" localSheetId="5">'Mass Transfer'!$D$403</definedName>
+    <definedName name="fit_Stt" localSheetId="5">'Mass Transfer'!$D$404</definedName>
+    <definedName name="fit_StV" localSheetId="5">'Mass Transfer'!$D$405</definedName>
+    <definedName name="fit_n_min" localSheetId="5">'Mass Transfer'!$D$406</definedName>
+    <definedName name="Q_CO2_fit" localSheetId="5">'Mass Transfer'!$D$407</definedName>
+    <definedName name="pulse_V0" localSheetId="5">'Mass Transfer'!$D$408</definedName>
+    <definedName name="spg_dur_eq_opt" localSheetId="5">'Mass Transfer'!$D$409</definedName>
+    <definedName name="spg_dur_eq" localSheetId="5">'Mass Transfer'!$D$410</definedName>
+    <definedName name="V_pulse" localSheetId="5">'Mass Transfer'!$D$411</definedName>
+    <definedName name="carry_n" localSheetId="5">'Mass Transfer'!$D$412</definedName>
+    <definedName name="Q_carry_max" localSheetId="5">'Mass Transfer'!$D$413</definedName>
+    <definedName name="carry_flag_usg" localSheetId="5">'Mass Transfer'!$D$414</definedName>
+    <definedName name="chk_carry_usg" localSheetId="0">Summary!$D$136</definedName>
+    <definedName name="CO2_uptake_ratio" localSheetId="5">'Mass Transfer'!$D$417</definedName>
+    <definedName name="res_CO2_uptake" localSheetId="0">Summary!$D$135</definedName>
+    <definedName name="pH_ref_DIC" localSheetId="3">Chemistry!$D$291</definedName>
+    <definedName name="h_ref_DIC" localSheetId="3">Chemistry!$D$292</definedName>
+    <definedName name="r_HCO3_ref" localSheetId="3">Chemistry!$D$293</definedName>
+    <definedName name="HCO3_ref" localSheetId="3">Chemistry!$D$294</definedName>
+    <definedName name="beta_nonC" localSheetId="3">Chemistry!$D$295</definedName>
+    <definedName name="DIC_cap" localSheetId="3">Chemistry!$D$296</definedName>
+    <definedName name="DIC_cap_mt" localSheetId="5">'Mass Transfer'!$D$415</definedName>
+    <definedName name="V_L_CO2" localSheetId="5">'Mass Transfer'!$D$416</definedName>
+    <definedName name="P_dry" localSheetId="5">'Mass Transfer'!$D$418</definedName>
+    <definedName name="I_ionic_b" localSheetId="4">Biology!$D$121</definedName>
+    <definedName name="ks_O2" localSheetId="4">Biology!$D$122</definedName>
+    <definedName name="f_salt_O2" localSheetId="4">Biology!$D$123</definedName>
+    <definedName name="ec_jbuf_ratio" localSheetId="2">Electrochemistry!$D$161</definedName>
+    <definedName name="pcet_credit_op" localSheetId="2">Electrochemistry!$D$162</definedName>
+    <definedName name="pcet_credit_gmax" localSheetId="2">Electrochemistry!$D$163</definedName>
+    <definedName name="pH_red_lo" localSheetId="3">Chemistry!$D$299</definedName>
+    <definedName name="pH_red_hi" localSheetId="3">Chemistry!$D$300</definedName>
+    <definedName name="cf_pH_red_lo" localSheetId="0">Summary!$D$138</definedName>
+    <definedName name="cf_pH_lo" localSheetId="0">Summary!$D$139</definedName>
+    <definedName name="cf_pH_hi" localSheetId="0">Summary!$D$140</definedName>
+    <definedName name="cf_pH_red_hi" localSheetId="0">Summary!$D$141</definedName>
+    <definedName name="cf_Cl_onset" localSheetId="0">Summary!$D$142</definedName>
+    <definedName name="cf_Cl_kill" localSheetId="0">Summary!$D$143</definedName>
+    <definedName name="ReactorTypeList">Geometry!$B$59:$B$80</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8355,7 +8396,7 @@
       </c>
       <c r="D13" s="90">
         <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$90)</f>
-        <v>0.784513049825</v>
+        <v>0.674076519917</v>
       </c>
       <c r="E13" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D90","→ Mass")</f>
@@ -8382,7 +8423,7 @@
       </c>
       <c r="D14" s="91">
         <f>IF(AND(ISNUMBER($G$13),$G$13&gt;0),$G$13,IF(NOT(ISNUMBER(D13)),D13,'Mass Transfer'!$D$242))</f>
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="E14" s="20"/>
       <c r="F14" s="21" t="inlineStr">
@@ -8406,7 +8447,7 @@
       </c>
       <c r="D15" s="90">
         <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$91)</f>
-        <v>9.026013902172</v>
+        <v>8.95302011459</v>
       </c>
       <c r="E15" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
@@ -8434,13 +8475,13 @@
         <v>67</v>
       </c>
       <c r="D16" s="91">
-        <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,ROUND(D14/(60*'Mass Transfer'!$D$93),0)))</f>
+        <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,ROUND(('Mass Transfer'!$D$408+'Mass Transfer'!$D$407*D14)/('Mass Transfer'!$D$102/60)/(60*'Mass Transfer'!$D$93),0)))</f>
         <v>9.0</v>
       </c>
       <c r="E16" s="92"/>
       <c r="F16" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interval to type in: recomputed from the as-run pulse at the optimised duty (Mass Transfer D93) and rounded to whole minutes, so rounding does not shift the CO₂ dose (row 95). An override in G15 wins.</t>
+          <t xml:space="preserve">Interval to type in: the as-run pulse converted to delivered CO₂ (V₀ + Q·t, Mass Transfer D407–D408) at the optimised full-flow-equivalent duty (D93), rounded to whole minutes, so rounding does not shift the CO₂ dose (row 95). An override in G15 wins.</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8569,7 @@
       <c r="C21" s="20"/>
       <c r="D21" s="90" t="str">
         <f>'Mass Transfer'!$D$374</f>
-        <v>organism band unknown – peak 2.9 mg/L is under the inhibition ceiling</v>
+        <v>organism band unknown – peak 2.8 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E21" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D374","→ Mass Transfer")</f>
@@ -8576,7 +8617,7 @@
       <c r="C23" s="20"/>
       <c r="D23" s="90" t="str">
         <f>'Mass Transfer'!$D$113</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) the cycle-mean DO would be ≈16 mg/L, above the 11.7 mg/L inhibition ceiling (peaks higher)</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) the cycle-mean DO would be ≈15 mg/L, above the 11.3 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E23" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
@@ -8602,7 +8643,7 @@
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 18% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 17% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="23" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -8647,15 +8688,17 @@
       </c>
       <c r="C26" s="20"/>
       <c r="D26" s="90" t="str">
-        <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)"),"calibrate this reactor first")</f>
-        <v>×41.9 OK</v>
+        <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)")&amp;" delivered; ×"&amp;TEXT('Mass Transfer'!$D$417,"0.0")&amp;" absorbed per pulse (row 135)","calibrate this reactor first")</f>
+        <v>×42.1 OK delivered; ×2.4 absorbed per pulse (row 135)</v>
       </c>
       <c r="E26" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F26" s="21" t="s">
-        <v>85</v>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ratio of CO₂ delivered to carbon demand (should be ≥ 1), with the absorbed ratio beside it (row 135): delivered counts gas the pulse expels unabsorbed, absorbed does not.</t>
+        </is>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -8714,14 +8757,16 @@
       <c r="C29" s="20"/>
       <c r="D29" s="90" t="str">
         <f>'Mass Transfer'!$D$59</f>
-        <v>OK</v>
+        <v>not measured – record the max flow without carryover for ed04 in CO2 flows column M</v>
       </c>
       <c r="E29" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D59","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F29" s="21" t="s">
-        <v>91</v>
+      <c r="F29" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse flow against the measured no-carryover maximum for this reactor (CO2 flows column M). Reads "not measured" (amber) until one is recorded; the superficial-velocity rule of thumb is row 136.</t>
+        </is>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -8848,7 +8893,7 @@
       <c r="C35" s="20"/>
       <c r="D35" s="121">
         <f>Chemistry!$D$220</f>
-        <v>6.187122404381</v>
+        <v>6.199874888233</v>
       </c>
       <c r="E35" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -8856,7 +8901,7 @@
       </c>
       <c r="F35" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">pH at the cycle-average dissolved CO₂ of the schedule in use, on the activity scale a probe reads; the trough just after a pulse is lower. Green 6.5–7.5; red outside 6–8.</t>
+          <t xml:space="preserve">pH at the cycle-average dissolved CO₂ of the schedule in use, on the activity scale a probe reads; the trough just after a pulse is lower. Colour: green inside the HOB band (Chemistry pH_band_lo–pH_band_hi), red outside pH_red_lo–pH_red_hi (Chemistry D299–D300), amber between; thresholds in rows 138–141.</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8919,7 @@
       </c>
       <c r="D36" s="121">
         <f>Chemistry!$D$226</f>
-        <v>0.339282500863</v>
+        <v>0.339248526308</v>
       </c>
       <c r="E36" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
@@ -8882,7 +8927,7 @@
       </c>
       <c r="F36" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Effective biocidal chlorine from the medium’s chloride, as Cl₂ (the basis of the thresholds). Onset 0.1 mg/L, kill 2 mg/L (Chemistry D146/D147); colour: green below 0.1, red above 1. Zero for chloride-free media.</t>
+          <t xml:space="preserve">Effective biocidal chlorine from the medium’s chloride, as Cl₂ (the basis of the thresholds). Colour: green below the onset (Chemistry Cl_onset, 0.1 mg/L), amber up to the kill threshold (Cl_kill, 2 mg/L), red above it; thresholds in rows 142–143. Zero for chloride-free media.</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8957,7 @@
       </c>
       <c r="D38" s="90">
         <f>'Mass Transfer'!$D$108</f>
-        <v>2.634776001183</v>
+        <v>2.543598660379</v>
       </c>
       <c r="E38" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D108","→ Mass")</f>
@@ -8940,7 +8985,7 @@
       </c>
       <c r="D39" s="90">
         <f>'Mass Transfer'!$D$112</f>
-        <v>188.941031253092</v>
+        <v>188.655905904325</v>
       </c>
       <c r="E39" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D112","→ Mass")</f>
@@ -8992,7 +9037,7 @@
       </c>
       <c r="D41" s="95">
         <f>Biology!$D$98</f>
-        <v>594.524480534657</v>
+        <v>575.774841144035</v>
       </c>
       <c r="E41" s="23" t="str">
         <f>HYPERLINK("#Biology!D98","→ Biology")</f>
@@ -9638,7 +9683,7 @@
       </c>
       <c r="D82" s="22">
         <f>Electrochemistry!$D$88</f>
-        <v>0.958329302507</v>
+        <v>0.959777674745</v>
       </c>
       <c r="E82" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D88","→ Electrochemistry")</f>
@@ -9712,7 +9757,7 @@
       </c>
       <c r="D85" s="22" t="str">
         <f>Electrochemistry!$D$99</f>
-        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.053 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
       </c>
       <c r="E85" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D99","→ Electrochemistry")</f>
@@ -9762,7 +9807,7 @@
       </c>
       <c r="D87" s="22">
         <f>Chemistry!$D$209</f>
-        <v>-0.427526934687</v>
+        <v>-0.427526678634</v>
       </c>
       <c r="E87" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D209","→ Chemistry")</f>
@@ -9788,7 +9833,7 @@
       </c>
       <c r="D88" s="22">
         <f>Chemistry!$D$211</f>
-        <v>1.265216285627</v>
+        <v>1.264461856975</v>
       </c>
       <c r="E88" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
@@ -9814,7 +9859,7 @@
       </c>
       <c r="D89" s="22">
         <f>Chemistry!$D$220</f>
-        <v>6.187122404381</v>
+        <v>6.199874888233</v>
       </c>
       <c r="E89" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -9838,7 +9883,7 @@
       </c>
       <c r="D90" s="22">
         <f>'Mass Transfer'!$D$186</f>
-        <v>0.003566106821</v>
+        <v>0.003701930458</v>
       </c>
       <c r="E90" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D186","→ Mass Transfer")</f>
@@ -9894,8 +9939,8 @@
         </is>
       </c>
       <c r="D95" s="95">
-        <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),D14/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (see CO2 flows)")</f>
-        <v>1.022688337739</v>
+        <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),('Mass Transfer'!$D$408+'Mass Transfer'!$D$407*D14)/('Mass Transfer'!$D$102/60)/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (see CO2 flows)")</f>
+        <v>0.964353979896</v>
       </c>
       <c r="E95" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
@@ -10016,7 +10061,7 @@
       </c>
       <c r="D114" s="90">
         <f>'Mass Transfer'!$D$343</f>
-        <v>2.634776001183</v>
+        <v>2.543598660379</v>
       </c>
       <c r="E114" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D343","→ Mass Transfer")</f>
@@ -10041,7 +10086,7 @@
       </c>
       <c r="D115" s="90">
         <f>'Mass Transfer'!$D$344</f>
-        <v>2.934788844069</v>
+        <v>2.82014387887</v>
       </c>
       <c r="E115" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D344","→ Mass Transfer")</f>
@@ -10066,7 +10111,7 @@
       </c>
       <c r="D116" s="90">
         <f>'Mass Transfer'!$D$364</f>
-        <v>6.785801971106</v>
+        <v>6.605507737565</v>
       </c>
       <c r="E116" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
@@ -10091,7 +10136,7 @@
       </c>
       <c r="D117" s="90">
         <f>'Mass Transfer'!$D$365</f>
-        <v>7.403376944733</v>
+        <v>7.175982939307</v>
       </c>
       <c r="E117" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D365","→ Mass Transfer")</f>
@@ -10111,7 +10156,7 @@
       </c>
       <c r="D118" s="90" t="str">
         <f>'Mass Transfer'!$D$348</f>
-        <v>peak 2.9 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 2.8 mg/L under the 11.3 mg/L ceiling</v>
       </c>
       <c r="E118" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D348","→ Mass Transfer")</f>
@@ -10131,7 +10176,7 @@
       </c>
       <c r="D119" s="90" t="str">
         <f>'Mass Transfer'!$D$369</f>
-        <v>peak 7.4 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 7.2 mg/L under the 11.3 mg/L ceiling</v>
       </c>
       <c r="E119" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D369","→ Mass Transfer")</f>
@@ -10151,7 +10196,7 @@
       </c>
       <c r="D120" s="90" t="str">
         <f>'Mass Transfer'!$D$347</f>
-        <v>reachable – kLa margin 2.02×</v>
+        <v>reachable – kLa margin 1.94×</v>
       </c>
       <c r="E120" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D347","→ Mass Transfer")</f>
@@ -10171,7 +10216,7 @@
       </c>
       <c r="D121" s="90" t="str">
         <f>'Mass Transfer'!$D$368</f>
-        <v>UNREACHABLE at this surface kLa – margin 0.64× (raise kL_surf, lower the current, or accept a higher DO)</v>
+        <v>UNREACHABLE at this surface kLa – margin 0.62× (raise kL_surf, lower the current, or accept a higher DO)</v>
       </c>
       <c r="E121" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D368","→ Mass Transfer")</f>
@@ -10179,7 +10224,7 @@
       </c>
       <c r="F121" s="21" t="str">
         <f>"Same on the lag source. Currently "&amp;TEXT('Mass Transfer'!$D$367,"0.00")&amp;"×: "&amp;IF('Mass Transfer'!$D$367&lt;1,"the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).","the target can be held during lag at the kLa in use.")</f>
-        <v>Same on the lag source. Currently 0.64×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
+        <v>Same on the lag source. Currently 0.62×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
       </c>
     </row>
     <row r="122">
@@ -10195,7 +10240,7 @@
       </c>
       <c r="D122" s="90">
         <f>'Mass Transfer'!$D$345</f>
-        <v>0.003566106821</v>
+        <v>0.003701930458</v>
       </c>
       <c r="E122" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D345","→ Mass Transfer")</f>
@@ -10220,7 +10265,7 @@
       </c>
       <c r="D123" s="90">
         <f>'Mass Transfer'!$D$366</f>
-        <v>0.011180382694</v>
+        <v>0.01160231226</v>
       </c>
       <c r="E123" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D366","→ Mass Transfer")</f>
@@ -10245,7 +10290,7 @@
       </c>
       <c r="D124" s="90">
         <f>'Mass Transfer'!$D$329</f>
-        <v>0.031639138319</v>
+        <v>0.031437574558</v>
       </c>
       <c r="E124" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D329","→ Mass Transfer")</f>
@@ -10270,7 +10315,7 @@
       </c>
       <c r="D125" s="90">
         <f>'Mass Transfer'!$D$351</f>
-        <v>0.064019231488</v>
+        <v>0.063684612076</v>
       </c>
       <c r="E125" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D351","→ Mass Transfer")</f>
@@ -10295,7 +10340,7 @@
       </c>
       <c r="D126" s="90">
         <f>'Mass Transfer'!$D$352</f>
-        <v>0.113266761861</v>
+        <v>0.112682153807</v>
       </c>
       <c r="E126" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D352","→ Mass Transfer")</f>
@@ -10320,7 +10365,7 @@
       </c>
       <c r="D127" s="90">
         <f>'Mass Transfer'!$D$381</f>
-        <v>0.929374836165</v>
+        <v>0.929877016008</v>
       </c>
       <c r="E127" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D381","→ Mass Transfer")</f>
@@ -10340,7 +10385,7 @@
       </c>
       <c r="D128" s="90" t="str">
         <f>IF(ISNA('Mass Transfer'!$D$308+'Mass Transfer'!$D$317),"#N/A – check the selectors in D111/D112",IF(NOT(ISNUMBER('Mass Transfer'!$D$185)),"DO target unreachable on the sizing phase (rows 120–121) – the schedule is the legacy O₂ flush guard (Mass Transfer D89)",IF(Chemistry!$D$220&gt;=Chemistry!$D$236,"yes – the schedule holds the DO target at pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", within the band",IF('Mass Transfer'!$D$185&lt;='Mass Transfer'!$D$112,"NO – holding the DO target drives pH to "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor","NO – the carbon-limited interval (not the DO target) gives pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor"))))</f>
-        <v>NO – holding the DO target drives pH to 6.19, below the 6.5 band floor</v>
+        <v>NO – holding the DO target drives pH to 6.20, below the 6.5 band floor</v>
       </c>
       <c r="E128" s="23" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -10365,7 +10410,7 @@
       </c>
       <c r="D129" s="90">
         <f>'Mass Transfer'!$D$389</f>
-        <v>0.059351496276</v>
+        <v>0.059032852289</v>
       </c>
       <c r="E129" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D389","→ Mass Transfer")</f>
@@ -10394,6 +10439,248 @@
       <c r="F130" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">"HEADSPACE SAGS" = the check-valve model needs more vacuum than a real cap holds: switch D111 to Open vent or Air exchange. n/a when the vent model already admits air.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ absorbed per pulse : carbon demand (dissolved, not delivered)</t>
+        </is>
+      </c>
+      <c r="B135" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_CO2_uptake</t>
+        </is>
+      </c>
+      <c r="C135" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">×</t>
+        </is>
+      </c>
+      <c r="D135" s="90">
+        <f>'Mass Transfer'!$D$417</f>
+        <v>2.425083542153</v>
+      </c>
+      <c r="E135" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D417","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F135" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shown beside D26: CO₂ the liquid takes up after each pulse (incl. bicarbonate), per hour, over fixation. Informative, not pass/fail: below 1 the culture also draws on headspace CO₂ between pulses. Carbon sufficiency is row 41.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carryover — superficial-velocity rule of thumb (secondary)</t>
+        </is>
+      </c>
+      <c r="B136" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_carry_usg</t>
+        </is>
+      </c>
+      <c r="D136" s="90" t="str">
+        <f>'Mass Transfer'!$D$414</f>
+        <v>OK – 6.6 mm/s against the 50 mm/s rule of thumb</v>
+      </c>
+      <c r="E136" s="23" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D414","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F136" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Secondary to row 29: gas velocity against the provisional 50 mm/s entrainment rule of thumb. It cannot fail at bench flows; row 29 tests the measured limit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COLOUR THRESHOLDS (the conditional formatting on D35 and D36 reads these cells)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH red below</t>
+        </is>
+      </c>
+      <c r="B138" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cf_pH_red_lo</t>
+        </is>
+      </c>
+      <c r="C138" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D138" s="90">
+        <f>Chemistry!$D$299</f>
+        <v>6.0</v>
+      </c>
+      <c r="E138" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D299","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F138" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same-sheet copy so the conditional-format rule can reference it by a Summary-local name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH amber below (band floor)</t>
+        </is>
+      </c>
+      <c r="B139" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cf_pH_lo</t>
+        </is>
+      </c>
+      <c r="C139" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D139" s="90">
+        <f>Chemistry!$D$236</f>
+        <v>6.5</v>
+      </c>
+      <c r="E139" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D236","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F139" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same-sheet copy so the conditional-format rule can reference it by a Summary-local name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH amber above (band ceiling)</t>
+        </is>
+      </c>
+      <c r="B140" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cf_pH_hi</t>
+        </is>
+      </c>
+      <c r="C140" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D140" s="90">
+        <f>Chemistry!$D$237</f>
+        <v>7.5</v>
+      </c>
+      <c r="E140" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D237","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F140" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same-sheet copy so the conditional-format rule can reference it by a Summary-local name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH red above</t>
+        </is>
+      </c>
+      <c r="B141" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cf_pH_red_hi</t>
+        </is>
+      </c>
+      <c r="C141" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D141" s="90">
+        <f>Chemistry!$D$300</f>
+        <v>8.0</v>
+      </c>
+      <c r="E141" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D300","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F141" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same-sheet copy so the conditional-format rule can reference it by a Summary-local name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chlorine amber above (onset)</t>
+        </is>
+      </c>
+      <c r="B142" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cf_Cl_onset</t>
+        </is>
+      </c>
+      <c r="C142" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D142" s="90">
+        <f>Chemistry!$D$146</f>
+        <v>0.1</v>
+      </c>
+      <c r="E142" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D146","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F142" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same-sheet copy so the conditional-format rule can reference it by a Summary-local name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chlorine red above (kill)</t>
+        </is>
+      </c>
+      <c r="B143" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cf_Cl_kill</t>
+        </is>
+      </c>
+      <c r="C143" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D143" s="90">
+        <f>Chemistry!$D$147</f>
+        <v>2.0</v>
+      </c>
+      <c r="E143" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D147","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F143" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same-sheet copy so the conditional-format rule can reference it by a Summary-local name.</t>
         </is>
       </c>
     </row>
@@ -10435,23 +10722,23 @@
       <formula>AND(ISNUMBER($G$15),$G$15&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D19:D36">
+  <conditionalFormatting sqref="D19:D36 D84:D86 D118:D121 D128:D130">
     <cfRule type="expression" dxfId="36" priority="12" stopIfTrue="1">
-      <formula>OR(ISNUMBER(SEARCH("INCONSISTENT",D19)),ISNUMBER(SEARCH("OVER",D19)),ISNUMBER(SEARCH("BELOW",D19)),ISNUMBER(SEARCH("EXCEED",D19)),ISNUMBER(SEARCH("NO CALIB",D19)),ISNUMBER(SEARCH("calibrate this",D19)),ISNUMBER(SEARCH("RISK",D19)),ISNUMBER(SEARCH("EXPLOSIVE",D19)),ISNUMBER(SEARCH("OOR",D19)),ISNUMBER(SEARCH("insufficient",D19)),ISNUMBER(SEARCH("TIP SPEED",D19)),ISNUMBER(SEARCH("SHORTFALL",D19)),EXACT(D19,"OUT"),EXACT(D19,"LOW"),ISNUMBER(SEARCH("GAP",D19)))</formula>
+      <formula>OR(ISNUMBER(FIND("INCONSISTENT",D19)),ISNUMBER(FIND("OVER",D19)),ISNUMBER(FIND("BELOW",D19)),ISNUMBER(FIND("EXCEED",D19)),ISNUMBER(FIND("NO CALIB",D19)),ISNUMBER(SEARCH("calibrate this",D19)),ISNUMBER(FIND("RISK",D19)),ISNUMBER(FIND("EXPLOSIVE",D19)),ISNUMBER(FIND("FLAMMABLE",D19)),ISNUMBER(FIND("OOR",D19)),ISNUMBER(SEARCH("insufficient",D19)),ISNUMBER(FIND("TIP SPEED",D19)),ISNUMBER(FIND("SHORTFALL",D19)),ISNUMBER(SEARCH("unreachable",D19)),ISNUMBER(FIND("SAGS",D19)),EXACT(LEFT(D19,4),"NO –"),EXACT(D19,"OUT"),EXACT(D19,"LOW"),ISNUMBER(FIND("GAP",D19)))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="35" priority="13" stopIfTrue="1">
-      <formula>OR(ISNUMBER(SEARCH("above optimum",D19)),ISNUMBER(SEARCH("watch",D19)),ISNUMBER(SEARCH("NEAREST",D19)),ISNUMBER(SEARCH("unknown",D19)),ISNUMBER(SEARCH("TIGHT",D19)))</formula>
+      <formula>OR(ISNUMBER(SEARCH("above optimum",D19)),ISNUMBER(SEARCH("watch",D19)),ISNUMBER(SEARCH("NEAREST",D19)),ISNUMBER(SEARCH("unknown",D19)),ISNUMBER(SEARCH("TIGHT",D19)),ISNUMBER(SEARCH("not measured",D19)))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="34" priority="14" stopIfTrue="1">
-      <formula>OR(EXACT(D19,"OK"),ISNUMBER(SEARCH(" OK",D19)),ISNUMBER(SEARCH("calibrated:",D19)),ISNUMBER(SEARCH("optimum",D19)),ISNUMBER(SEARCH("above min",D19)),ISNUMBER(SEARCH("CARBON-limited",D19)),ISNUMBER(SEARCH("Static",D19)),ISNUMBER(SEARCH("Dynamic",D19)),ISNUMBER(SEARCH("present",D19)))</formula>
+      <formula>OR(EXACT(D19,"OK"),EXACT(LEFT(D19,2),"OK"),ISNUMBER(SEARCH(" OK",D19)),ISNUMBER(SEARCH("calibrated:",D19)),ISNUMBER(SEARCH("optimum",D19)),ISNUMBER(SEARCH("above min",D19)),ISNUMBER(SEARCH("CARBON-limited",D19)),ISNUMBER(SEARCH("Static",D19)),ISNUMBER(SEARCH("Dynamic",D19)),ISNUMBER(SEARCH("present",D19)),ISNUMBER(SEARCH("under the",D19)),ISNUMBER(SEARCH("reachable",D19)),EXACT(LEFT(D19,3),"yes"),ISNUMBER(FIND("Below the H₂ LFL",D19)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D35">
     <cfRule type="expression" dxfId="33" priority="22" stopIfTrue="1">
-      <formula>OR(D35&lt;6,D35&gt;8)</formula>
+      <formula>OR(D35&lt;cf_pH_red_lo,D35&gt;cf_pH_red_hi)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="32" priority="23" stopIfTrue="1">
-      <formula>OR(D35&lt;6.5,D35&gt;7.5)</formula>
+      <formula>OR(D35&lt;cf_pH_lo,D35&gt;cf_pH_hi)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="31" priority="24" stopIfTrue="1">
       <formula>ISNUMBER(D35)</formula>
@@ -10459,10 +10746,10 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="D36">
     <cfRule type="expression" dxfId="30" priority="25" stopIfTrue="1">
-      <formula>D36&gt;1</formula>
+      <formula>D36&gt;cf_Cl_kill</formula>
     </cfRule>
     <cfRule type="expression" dxfId="29" priority="26" stopIfTrue="1">
-      <formula>D36&gt;0.1</formula>
+      <formula>D36&gt;cf_Cl_onset</formula>
     </cfRule>
     <cfRule type="expression" dxfId="28" priority="27" stopIfTrue="1">
       <formula>ISNUMBER(D36)</formula>
@@ -12633,7 +12920,7 @@
       </c>
       <c r="D18" s="42">
         <f>IF(ISNUMBER(cal_etaF),cal_etaF,etaF_calc)</f>
-        <v>0.958329302507</v>
+        <v>0.959777674745</v>
       </c>
       <c r="E18" s="67" t="inlineStr">
         <is>
@@ -12701,7 +12988,7 @@
       </c>
       <c r="D21" s="48">
         <f>I_app*etaF/(z_e_H2*F_const)*3600</f>
-        <v>0.0001017274698715</v>
+        <v>0.0001018812158154</v>
       </c>
       <c r="E21" s="99" t="s">
         <v>355</v>
@@ -12745,7 +13032,7 @@
       </c>
       <c r="D23" s="48">
         <f>rH2_gen/60*R_gas*T_K/P_atm*1000000</f>
-        <v>0.041480060291</v>
+        <v>0.041542751234</v>
       </c>
       <c r="E23" s="99" t="s">
         <v>362</v>
@@ -12789,7 +13076,7 @@
       </c>
       <c r="D25" s="48">
         <f>V_H2_gen+V_O2_gen</f>
-        <v>0.062757357403</v>
+        <v>0.062820048346</v>
       </c>
       <c r="E25" s="99" t="s">
         <v>368</v>
@@ -12861,7 +13148,7 @@
       </c>
       <c r="D28" s="48">
         <f>I_app*(1-etaF)/(n_ORR_eff*F_const)*3600</f>
-        <v>2.391016190066e-06</v>
+        <v>2.307910274443e-06</v>
       </c>
       <c r="E28" s="99" t="inlineStr">
         <is>
@@ -12885,7 +13172,7 @@
       </c>
       <c r="D29" s="48">
         <f>rO2_gen-O2_cathode_ORR</f>
-        <v>4.979033518202e-05</v>
+        <v>4.987344109764e-05</v>
       </c>
       <c r="E29" s="99" t="s">
         <v>379</v>
@@ -13846,7 +14133,7 @@
       </c>
       <c r="D80" s="141">
         <f>Biology!$D$27</f>
-        <v>0.36477</v>
+        <v>0.352091480729</v>
       </c>
       <c r="E80" s="67" t="s">
         <v>1631</v>
@@ -13938,7 +14225,7 @@
       </c>
       <c r="D85" s="141">
         <f>ec_DO_frac*ec_O2_ceil</f>
-        <v>0.08246973913</v>
+        <v>0.079603291295</v>
       </c>
       <c r="E85" s="67" t="s">
         <v>1645</v>
@@ -13956,7 +14243,7 @@
       </c>
       <c r="D86" s="141">
         <f>n_ORR_eff*F_const*(km_O2/100)*ec_DO_design*(A_cath_wet/10000)</f>
-        <v>0.0002371062687363</v>
+        <v>0.0002288650307031</v>
       </c>
       <c r="E86" s="67" t="inlineStr">
         <is>
@@ -13976,7 +14263,7 @@
       </c>
       <c r="D87" s="141">
         <f>n_ORR_eff*F_const*(km_O2/100)*ec_O2_ceil*(A_cath_wet/10000)</f>
-        <v>0.001048739266</v>
+        <v>0.001012287636</v>
       </c>
       <c r="E87" s="67" t="s">
         <v>1651</v>
@@ -13994,7 +14281,7 @@
       </c>
       <c r="D88" s="141">
         <f>MAX(0,1-i_ORR_design/I_app)</f>
-        <v>0.958329302507</v>
+        <v>0.959777674745</v>
       </c>
       <c r="E88" s="67" t="inlineStr">
         <is>
@@ -14014,7 +14301,7 @@
       </c>
       <c r="D89" s="141">
         <f>MAX(0,1-i_ORR_ceiling/I_app)</f>
-        <v>0.815687299549</v>
+        <v>0.82209356137</v>
       </c>
       <c r="E89" s="67" t="s">
         <v>1657</v>
@@ -14071,7 +14358,7 @@
       </c>
       <c r="D93" s="141">
         <f>f_HOOH*I_app*(1-etaF)/(n_ORR_eff*F_const)*M_H2O2*1000*3600/ec_V_L</f>
-        <v>0.813296984002</v>
+        <v>0.785028756121</v>
       </c>
       <c r="E93" s="67" t="inlineStr">
         <is>
@@ -14108,7 +14395,7 @@
       </c>
       <c r="D95" s="141">
         <f>r_H2O2/(k_cat_cells*3600)</f>
-        <v>0.05510142168</v>
+        <v>0.053186230089</v>
       </c>
       <c r="E95" s="67" t="s">
         <v>1673</v>
@@ -14126,7 +14413,7 @@
       </c>
       <c r="D96" s="141">
         <f>r_H2O2_lag/(k_H2O2_anode*3600)*(1-EXP(-k_H2O2_anode*3600))</f>
-        <v>0.925414707501</v>
+        <v>0.900827055797</v>
       </c>
       <c r="E96" s="67" t="inlineStr">
         <is>
@@ -14163,7 +14450,7 @@
       </c>
       <c r="D98" s="141">
         <f>IF(r_H2O2_lag&gt;0,IF(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag&gt;0,-LN(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag)/k_H2O2_anode/60,NA()),NA())</f>
-        <v>5.305839767983</v>
+        <v>5.464176174322</v>
       </c>
       <c r="E98" s="67" t="inlineStr">
         <is>
@@ -14183,7 +14470,7 @@
       </c>
       <c r="D99" s="141" t="str">
         <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(H2O2_lag_1h&gt;H2O2_thresh,"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases"))</f>
-        <v>watch — steady growth is clear (0.055 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.053 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
       </c>
       <c r="E99" s="67" t="s">
         <v>1685</v>
@@ -14410,8 +14697,10 @@
       <c r="D113" s="131">
         <v>-0.15</v>
       </c>
-      <c r="E113" s="75" t="s">
-        <v>1725</v>
+      <c r="E113" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Neutral-pH OER in ≥30 mM phosphate proceeds by proton-coupled electron transfer to the buffer base rather than to water, cutting the overpotential by 100–200 mV and the Tafel slope to ~60 mV/dec (Surendranath, Kanan &amp; Nocera 2010; Dau group, Inorganics 2019, 7:20). Established for oxide anodes rather than bare Pt, so this is a stated transfer, not a measurement. The budget applies it through pcet_credit_op (D162): in full while the buffer holds the anode surface, withdrawn past the buffer-limited current (Chemistry j_buffer_ratio &gt; 1).</t>
+        </is>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
@@ -14516,7 +14805,7 @@
         <v>1595</v>
       </c>
       <c r="D119" s="141">
-        <f>ec_E_rev+eta_anode+eta_cath+pcet_credit+V_IR</f>
+        <f>ec_E_rev+eta_anode+eta_cath+pcet_credit_op+V_IR</f>
         <v>2.847708123495</v>
       </c>
       <c r="E119" s="67" t="s">
@@ -14736,8 +15025,8 @@
         </is>
       </c>
       <c r="D143" s="141">
-        <f>ec_E_rev+b_anode*LOG10(I_at_gerrit_max/A_anode_wet/j0_anode)+b_cath*LOG10(I_at_gerrit_max/A_cath_wet/j0_cath)+pcet_credit+I_at_gerrit_max*R_cell</f>
-        <v>4.685940001272</v>
+        <f>ec_E_rev+b_anode*LOG10(I_at_gerrit_max/A_anode_wet/j0_anode)+b_cath*LOG10(I_at_gerrit_max/A_cath_wet/j0_cath)+pcet_credit_gmax+I_at_gerrit_max*R_cell</f>
+        <v>4.835940001272</v>
       </c>
       <c r="E143" s="75" t="inlineStr">
         <is>
@@ -14763,7 +15052,7 @@
       </c>
       <c r="D144" s="141" t="str">
         <f>IF(V_at_gerrit_max&gt;V_rail,"INCONSISTENT — the budget needs "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" %, above the "&amp;TEXT(V_rail,"0")&amp;" V rail, where Gerrit's Law is validated linear: R_cell (k_geom) or j₀ is too high","OK — "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" %, under the "&amp;TEXT(V_rail,"0")&amp;" V rail across the validated band")</f>
-        <v>OK — 4.69 V at 25 %, under the 5 V rail across the validated band</v>
+        <v>OK — 4.84 V at 25 %, under the 5 V rail across the validated band</v>
       </c>
       <c r="E144" s="67" t="inlineStr">
         <is>
@@ -14916,7 +15205,7 @@
       </c>
       <c r="D150" s="141">
         <f>'Mass Transfer'!$D$135</f>
-        <v>0.212069565945</v>
+        <v>0.206435018988</v>
       </c>
       <c r="E150" s="67" t="inlineStr">
         <is>
@@ -14968,7 +15257,7 @@
       </c>
       <c r="D152" s="141">
         <f>r_H2O2*ec_DO_lag/ec_DO_design</f>
-        <v>2.091379701213</v>
+        <v>2.035813137102</v>
       </c>
       <c r="E152" s="67" t="inlineStr">
         <is>
@@ -15025,6 +15314,91 @@
       <c r="E154" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">→ Summary (organism_sel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROTON-COUPLED CREDIT vs THE BUFFER LIMIT (review R1-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) operating : buffer-limited current</t>
+        </is>
+      </c>
+      <c r="B161" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ec_jbuf_ratio</t>
+        </is>
+      </c>
+      <c r="C161" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D161" s="141">
+        <f>Chemistry!$D$218</f>
+        <v>0.328374783131</v>
+      </c>
+      <c r="E161" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Chemistry!D218 (j_buffer_ratio).</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Proton-coupled credit at the operating current</t>
+        </is>
+      </c>
+      <c r="B162" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pcet_credit_op</t>
+        </is>
+      </c>
+      <c r="C162" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="D162" s="141">
+        <f>IF(ec_jbuf_ratio&gt;1,0,pcet_credit)</f>
+        <v>-0.15</v>
+      </c>
+      <c r="E162" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full credit while the buffer holds the anode surface (ratio ≤ 1); none past the buffer-limited current, where no buffer base reaches the surface to accept the proton. No partial scaling in between: how the credit fades with surface depletion on Pt is unmeasured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same, at the top of the validated Gerrit band</t>
+        </is>
+      </c>
+      <c r="B163" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pcet_credit_gmax</t>
+        </is>
+      </c>
+      <c r="C163" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V</t>
+        </is>
+      </c>
+      <c r="D163" s="141">
+        <f>IF(ec_jbuf_ratio*I_at_gerrit_max/I_app&gt;1,0,pcet_credit)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E163" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Buffer ratio scaled to I_at_gerrit_max (j ∝ I at the bulk pH): at 25 % the anode runs ~1.6× past the buffer limit, so the credit is withdrawn for the D143 cross-check.</t>
         </is>
       </c>
     </row>
@@ -15137,7 +15511,7 @@
       </c>
       <c r="D5" s="64">
         <f>'Mass Transfer'!$D$162</f>
-        <v>0.029931790408</v>
+        <v>0.02896589844</v>
       </c>
       <c r="E5" s="51" t="inlineStr">
         <is>
@@ -15821,7 +16195,7 @@
       </c>
       <c r="B50" s="64">
         <f t="shared" ref="B50:B81" si="1">pH_SID + pH_NT*(10^-A50)/((10^-A50)+KaN_c) + (10^-A50) - (pH_PT*Ka1p_c*(10^-A50)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A50) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A50)^3 + Ka1p_c*(10^-A50)^2 + Ka1p_c*Ka2p_c*(10^-A50) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A50) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A50)^2 - Kw_c/(10^-A50)</f>
-        <v>0.033056557945</v>
+        <v>0.033063680227</v>
       </c>
       <c r="C50" s="64">
         <f>IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
@@ -15834,7 +16208,7 @@
       </c>
       <c r="B51" s="64">
         <f t="shared" si="1"/>
-        <v>0.032897876114</v>
+        <v>0.032906842542</v>
       </c>
       <c r="C51" s="64">
         <f>IF(AND(B51&gt;=0,B52&lt;0),A51+pH_step*B51/(B51-B52),0)</f>
@@ -15847,7 +16221,7 @@
       </c>
       <c r="B52" s="64">
         <f t="shared" si="1"/>
-        <v>0.03273738701</v>
+        <v>0.032748675085</v>
       </c>
       <c r="C52" s="64">
         <f>IF(AND(B52&gt;=0,B53&lt;0),A52+pH_step*B52/(B52-B53),0)</f>
@@ -15860,7 +16234,7 @@
       </c>
       <c r="B53" s="64">
         <f t="shared" si="1"/>
-        <v>0.032566660249</v>
+        <v>0.032580871108</v>
       </c>
       <c r="C53" s="64">
         <f>IF(AND(B53&gt;=0,B54&lt;0),A53+pH_step*B53/(B53-B54),0)</f>
@@ -15873,7 +16247,7 @@
       </c>
       <c r="B54" s="64">
         <f t="shared" si="1"/>
-        <v>0.032376693474</v>
+        <v>0.032394583909</v>
       </c>
       <c r="C54" s="64">
         <f>IF(AND(B54&gt;=0,B55&lt;0),A54+pH_step*B54/(B54-B55),0)</f>
@@ -15886,7 +16260,7 @@
       </c>
       <c r="B55" s="64">
         <f t="shared" si="1"/>
-        <v>0.032157451816</v>
+        <v>0.032179974577</v>
       </c>
       <c r="C55" s="64">
         <f>IF(AND(B55&gt;=0,B56&lt;0),A55+pH_step*B55/(B55-B56),0)</f>
@@ -15899,7 +16273,7 @@
       </c>
       <c r="B56" s="64">
         <f t="shared" si="1"/>
-        <v>0.031897350748</v>
+        <v>0.031925705284</v>
       </c>
       <c r="C56" s="64">
         <f>IF(AND(B56&gt;=0,B57&lt;0),A56+pH_step*B56/(B56-B57),0)</f>
@@ -15912,7 +16286,7 @@
       </c>
       <c r="B57" s="64">
         <f t="shared" si="1"/>
-        <v>0.031582658325</v>
+        <v>0.031618354665</v>
       </c>
       <c r="C57" s="64">
         <f>IF(AND(B57&gt;=0,B58&lt;0),A57+pH_step*B57/(B57-B58),0)</f>
@@ -15925,7 +16299,7 @@
       </c>
       <c r="B58" s="64">
         <f t="shared" si="1"/>
-        <v>0.031196788903</v>
+        <v>0.031241728083</v>
       </c>
       <c r="C58" s="64">
         <f>IF(AND(B58&gt;=0,B59&lt;0),A58+pH_step*B58/(B58-B59),0)</f>
@@ -15938,7 +16312,7 @@
       </c>
       <c r="B59" s="64">
         <f t="shared" si="1"/>
-        <v>0.030719455744</v>
+        <v>0.030776031058</v>
       </c>
       <c r="C59" s="64">
         <f>IF(AND(B59&gt;=0,B60&lt;0),A59+pH_step*B59/(B59-B60),0)</f>
@@ -15951,7 +16325,7 @@
       </c>
       <c r="B60" s="64">
         <f t="shared" si="1"/>
-        <v>0.030125644421</v>
+        <v>0.030196868898</v>
       </c>
       <c r="C60" s="64">
         <f>IF(AND(B60&gt;=0,B61&lt;0),A60+pH_step*B60/(B60-B61),0)</f>
@@ -15964,7 +16338,7 @@
       </c>
       <c r="B61" s="64">
         <f t="shared" si="1"/>
-        <v>0.029384362607</v>
+        <v>0.029474029509</v>
       </c>
       <c r="C61" s="64">
         <f>IF(AND(B61&gt;=0,B62&lt;0),A61+pH_step*B61/(B61-B62),0)</f>
@@ -15977,7 +16351,7 @@
       </c>
       <c r="B62" s="64">
         <f t="shared" si="1"/>
-        <v>0.028457114762</v>
+        <v>0.028569999651</v>
       </c>
       <c r="C62" s="64">
         <f>IF(AND(B62&gt;=0,B63&lt;0),A62+pH_step*B62/(B62-B63),0)</f>
@@ -15990,7 +16364,7 @@
       </c>
       <c r="B63" s="64">
         <f t="shared" si="1"/>
-        <v>0.027296042508</v>
+        <v>0.027438157665</v>
       </c>
       <c r="C63" s="64">
         <f>IF(AND(B63&gt;=0,B64&lt;0),A63+pH_step*B63/(B63-B64),0)</f>
@@ -16003,7 +16377,7 @@
       </c>
       <c r="B64" s="64">
         <f t="shared" si="1"/>
-        <v>0.025841663275</v>
+        <v>0.026020578038</v>
       </c>
       <c r="C64" s="64">
         <f>IF(AND(B64&gt;=0,B65&lt;0),A64+pH_step*B64/(B64-B65),0)</f>
@@ -16016,7 +16390,7 @@
       </c>
       <c r="B65" s="64">
         <f t="shared" si="1"/>
-        <v>0.024020130969</v>
+        <v>0.024245375084</v>
       </c>
       <c r="C65" s="64">
         <f>IF(AND(B65&gt;=0,B66&lt;0),A65+pH_step*B65/(B65-B66),0)</f>
@@ -16029,7 +16403,7 @@
       </c>
       <c r="B66" s="64">
         <f t="shared" si="1"/>
-        <v>0.021739932163</v>
+        <v>0.022023503682</v>
       </c>
       <c r="C66" s="64">
         <f>IF(AND(B66&gt;=0,B67&lt;0),A66+pH_step*B66/(B66-B67),0)</f>
@@ -16042,7 +16416,7 @@
       </c>
       <c r="B67" s="64">
         <f t="shared" si="1"/>
-        <v>0.018887917484</v>
+        <v>0.019244922352</v>
       </c>
       <c r="C67" s="64">
         <f>IF(AND(B67&gt;=0,B68&lt;0),A67+pH_step*B67/(B67-B68),0)</f>
@@ -16055,7 +16429,7 @@
       </c>
       <c r="B68" s="64">
         <f t="shared" si="1"/>
-        <v>0.015324545379</v>
+        <v>0.015774002899</v>
       </c>
       <c r="C68" s="64">
         <f>IF(AND(B68&gt;=0,B69&lt;0),A68+pH_step*B68/(B68-B69),0)</f>
@@ -16068,7 +16442,7 @@
       </c>
       <c r="B69" s="64">
         <f t="shared" si="1"/>
-        <v>0.010878174835</v>
+        <v>0.011444032132</v>
       </c>
       <c r="C69" s="64">
         <f>IF(AND(B69&gt;=0,B70&lt;0),A69+pH_step*B69/(B69-B70),0)</f>
@@ -16081,11 +16455,11 @@
       </c>
       <c r="B70" s="64">
         <f t="shared" si="1"/>
-        <v>0.005338169177</v>
+        <v>0.006050579036</v>
       </c>
       <c r="C70" s="64">
         <f>IF(AND(B70&gt;=0,B71&lt;0),A70+pH_step*B70/(B70-B71),0)</f>
-        <v>6.077457645941</v>
+        <v>6.090210129793</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
@@ -16094,7 +16468,7 @@
       </c>
       <c r="B71" s="64">
         <f t="shared" si="1"/>
-        <v>-0.001553557408</v>
+        <v>-0.0006566267399188</v>
       </c>
       <c r="C71" s="64">
         <f>IF(AND(B71&gt;=0,B72&lt;0),A71+pH_step*B71/(B71-B72),0)</f>
@@ -16107,7 +16481,7 @@
       </c>
       <c r="B72" s="64">
         <f t="shared" si="1"/>
-        <v>-0.010113130675</v>
+        <v>-0.008983867099</v>
       </c>
       <c r="C72" s="64">
         <f>IF(AND(B72&gt;=0,B73&lt;0),A72+pH_step*B72/(B72-B73),0)</f>
@@ -16120,7 +16494,7 @@
       </c>
       <c r="B73" s="64">
         <f t="shared" si="1"/>
-        <v>-0.020728335463</v>
+        <v>-0.019306526655</v>
       </c>
       <c r="C73" s="64">
         <f>IF(AND(B73&gt;=0,B74&lt;0),A73+pH_step*B73/(B73-B74),0)</f>
@@ -16133,7 +16507,7 @@
       </c>
       <c r="B74" s="64">
         <f t="shared" si="1"/>
-        <v>-0.033876558634</v>
+        <v>-0.032086369352</v>
       </c>
       <c r="C74" s="64">
         <f>IF(AND(B74&gt;=0,B75&lt;0),A74+pH_step*B74/(B74-B75),0)</f>
@@ -16146,7 +16520,7 @@
       </c>
       <c r="B75" s="64">
         <f t="shared" si="1"/>
-        <v>-0.050148802566</v>
+        <v>-0.047894710516</v>
       </c>
       <c r="C75" s="64">
         <f>IF(AND(B75&gt;=0,B76&lt;0),A75+pH_step*B75/(B75-B76),0)</f>
@@ -16159,7 +16533,7 @@
       </c>
       <c r="B76" s="64">
         <f t="shared" si="1"/>
-        <v>-0.070281926409</v>
+        <v>-0.06744359471</v>
       </c>
       <c r="C76" s="64">
         <f>IF(AND(B76&gt;=0,B77&lt;0),A76+pH_step*B76/(B76-B77),0)</f>
@@ -16172,7 +16546,7 @@
       </c>
       <c r="B77" s="64">
         <f t="shared" si="1"/>
-        <v>-0.095201550021</v>
+        <v>-0.091627354454</v>
       </c>
       <c r="C77" s="64">
         <f>IF(AND(B77&gt;=0,B78&lt;0),A77+pH_step*B77/(B77-B78),0)</f>
@@ -16185,7 +16559,7 @@
       </c>
       <c r="B78" s="64">
         <f t="shared" si="1"/>
-        <v>-0.126078179765</v>
+        <v>-0.121577032191</v>
       </c>
       <c r="C78" s="64">
         <f>IF(AND(B78&gt;=0,B79&lt;0),A78+pH_step*B78/(B78-B79),0)</f>
@@ -16198,7 +16572,7 @@
       </c>
       <c r="B79" s="64">
         <f t="shared" si="1"/>
-        <v>-0.164399212616</v>
+        <v>-0.158730223128</v>
       </c>
       <c r="C79" s="64">
         <f>IF(AND(B79&gt;=0,B80&lt;0),A79+pH_step*B79/(B79-B80),0)</f>
@@ -16211,7 +16585,7 @@
       </c>
       <c r="B80" s="64">
         <f t="shared" si="1"/>
-        <v>-0.2120598263</v>
+        <v>-0.204919218655</v>
       </c>
       <c r="C80" s="64">
         <f>IF(AND(B80&gt;=0,B81&lt;0),A80+pH_step*B80/(B80-B81),0)</f>
@@ -16224,7 +16598,7 @@
       </c>
       <c r="B81" s="64">
         <f t="shared" si="1"/>
-        <v>-0.271476705075</v>
+        <v>-0.262481233295</v>
       </c>
       <c r="C81" s="64">
         <f>IF(AND(B81&gt;=0,B82&lt;0),A81+pH_step*B81/(B81-B82),0)</f>
@@ -16237,7 +16611,7 @@
       </c>
       <c r="B82" s="64">
         <f t="shared" ref="B82:B113" si="3">pH_SID + pH_NT*(10^-A82)/((10^-A82)+KaN_c) + (10^-A82) - (pH_PT*Ka1p_c*(10^-A82)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A82) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A82)^3 + Ka1p_c*(10^-A82)^2 + Ka1p_c*Ka2p_c*(10^-A82) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A82) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A82)^2 - Kw_c/(10^-A82)</f>
-        <v>-0.34573032811</v>
+        <v>-0.33439622345</v>
       </c>
       <c r="C82" s="64">
         <f>IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
@@ -16250,7 +16624,7 @@
       </c>
       <c r="B83" s="64">
         <f t="shared" si="3"/>
-        <v>-0.438744241063</v>
+        <v>-0.424460429215</v>
       </c>
       <c r="C83" s="64">
         <f>IF(AND(B83&gt;=0,B84&lt;0),A83+pH_step*B83/(B83-B84),0)</f>
@@ -16263,7 +16637,7 @@
       </c>
       <c r="B84" s="64">
         <f t="shared" si="3"/>
-        <v>-0.555513342847</v>
+        <v>-0.537507284878</v>
       </c>
       <c r="C84" s="64">
         <f>IF(AND(B84&gt;=0,B85&lt;0),A84+pH_step*B84/(B84-B85),0)</f>
@@ -16276,7 +16650,7 @@
       </c>
       <c r="B85" s="64">
         <f t="shared" si="3"/>
-        <v>-0.702397864982</v>
+        <v>-0.679691853834</v>
       </c>
       <c r="C85" s="64">
         <f>IF(AND(B85&gt;=0,B86&lt;0),A85+pH_step*B85/(B85-B86),0)</f>
@@ -16289,7 +16663,7 @@
       </c>
       <c r="B86" s="64">
         <f t="shared" si="3"/>
-        <v>-0.887505820494</v>
+        <v>-0.858860852469</v>
       </c>
       <c r="C86" s="64">
         <f>IF(AND(B86&gt;=0,B87&lt;0),A86+pH_step*B86/(B86-B87),0)</f>
@@ -16302,7 +16676,7 @@
       </c>
       <c r="B87" s="64">
         <f t="shared" si="3"/>
-        <v>-1.121195096281</v>
+        <v>-1.085038451661</v>
       </c>
       <c r="C87" s="64">
         <f>IF(AND(B87&gt;=0,B88&lt;0),A87+pH_step*B87/(B87-B88),0)</f>
@@ -16315,7 +16689,7 @@
       </c>
       <c r="B88" s="64">
         <f t="shared" si="3"/>
-        <v>-1.416738412478</v>
+        <v>-1.371069699052</v>
       </c>
       <c r="C88" s="64">
         <f>IF(AND(B88&gt;=0,B89&lt;0),A88+pH_step*B88/(B88-B89),0)</f>
@@ -16328,7 +16702,7 @@
       </c>
       <c r="B89" s="64">
         <f t="shared" si="3"/>
-        <v>-1.79121210323</v>
+        <v>-1.733480556804</v>
       </c>
       <c r="C89" s="64">
         <f>IF(AND(B89&gt;=0,B90&lt;0),A89+pH_step*B89/(B89-B90),0)</f>
@@ -16341,7 +16715,7 @@
       </c>
       <c r="B90" s="64">
         <f t="shared" si="3"/>
-        <v>-2.266696117449</v>
+        <v>-2.193639134543</v>
       </c>
       <c r="C90" s="64">
         <f>IF(AND(B90&gt;=0,B91&lt;0),A90+pH_step*B90/(B90-B91),0)</f>
@@ -16354,7 +16728,7 @@
       </c>
       <c r="B91" s="64">
         <f t="shared" si="3"/>
-        <v>-2.871912416818</v>
+        <v>-2.779341188627</v>
       </c>
       <c r="C91" s="64">
         <f>IF(AND(B91&gt;=0,B92&lt;0),A91+pH_step*B91/(B91-B92),0)</f>
@@ -16367,7 +16741,7 @@
       </c>
       <c r="B92" s="64">
         <f t="shared" si="3"/>
-        <v>-3.644489218902</v>
+        <v>-3.527001282793</v>
       </c>
       <c r="C92" s="64">
         <f>IF(AND(B92&gt;=0,B93&lt;0),A92+pH_step*B92/(B92-B93),0)</f>
@@ -16380,7 +16754,7 @@
       </c>
       <c r="B93" s="64">
         <f t="shared" si="3"/>
-        <v>-4.634130477414</v>
+        <v>-4.48471998199</v>
       </c>
       <c r="C93" s="64">
         <f>IF(AND(B93&gt;=0,B94&lt;0),A93+pH_step*B93/(B93-B94),0)</f>
@@ -16393,7 +16767,7 @@
       </c>
       <c r="B94" s="64">
         <f t="shared" si="3"/>
-        <v>-5.907111148118</v>
+        <v>-5.716634052942</v>
       </c>
       <c r="C94" s="64">
         <f>IF(AND(B94&gt;=0,B95&lt;0),A94+pH_step*B94/(B94-B95),0)</f>
@@ -16406,7 +16780,7 @@
       </c>
       <c r="B95" s="64">
         <f t="shared" si="3"/>
-        <v>-7.552736726532</v>
+        <v>-7.309167550567</v>
       </c>
       <c r="C95" s="64">
         <f>IF(AND(B95&gt;=0,B96&lt;0),A95+pH_step*B95/(B95-B96),0)</f>
@@ -16419,7 +16793,7 @@
       </c>
       <c r="B96" s="64">
         <f t="shared" si="3"/>
-        <v>-9.692743661107</v>
+        <v>-9.380128876944</v>
       </c>
       <c r="C96" s="64">
         <f>IF(AND(B96&gt;=0,B97&lt;0),A96+pH_step*B96/(B96-B97),0)</f>
@@ -16432,7 +16806,7 @@
       </c>
       <c r="B97" s="64">
         <f t="shared" si="3"/>
-        <v>-12.495143944944</v>
+        <v>-12.092108603666</v>
       </c>
       <c r="C97" s="64">
         <f>IF(AND(B97&gt;=0,B98&lt;0),A97+pH_step*B97/(B97-B98),0)</f>
@@ -16445,7 +16819,7 @@
       </c>
       <c r="B98" s="64">
         <f t="shared" si="3"/>
-        <v>-16.194840392116</v>
+        <v>-15.67242948836</v>
       </c>
       <c r="C98" s="64">
         <f>IF(AND(B98&gt;=0,B99&lt;0),A98+pH_step*B98/(B98-B99),0)</f>
@@ -16458,7 +16832,7 @@
       </c>
       <c r="B99" s="64">
         <f t="shared" si="3"/>
-        <v>-21.124629237082</v>
+        <v>-20.443148617968</v>
       </c>
       <c r="C99" s="64">
         <f>IF(AND(B99&gt;=0,B100&lt;0),A99+pH_step*B99/(B99-B100),0)</f>
@@ -16471,7 +16845,7 @@
       </c>
       <c r="B100" s="64">
         <f t="shared" si="3"/>
-        <v>-27.762233083538</v>
+        <v>-26.866572609656</v>
       </c>
       <c r="C100" s="64">
         <f>0</f>
@@ -16513,7 +16887,7 @@
       </c>
       <c r="D103" s="149">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
-        <v>6.077457645941</v>
+        <v>6.090210129793</v>
       </c>
       <c r="E103" s="51" t="s">
         <v>1878</v>
@@ -16536,7 +16910,7 @@
       </c>
       <c r="D104" s="149">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
-        <v>0.945966521198</v>
+        <v>0.944445825575</v>
       </c>
       <c r="E104" s="51" t="s">
         <v>1879</v>
@@ -16728,7 +17102,7 @@
       </c>
       <c r="D125" s="149">
         <f>pH_Cl*pH_fHOCl*M_HOCl</f>
-        <v>8.943125554526</v>
+        <v>8.92874896552</v>
       </c>
       <c r="E125" s="51" t="s">
         <v>1460</v>
@@ -16935,7 +17309,7 @@
       </c>
       <c r="D138" s="149">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
-        <v>4.758265066161e-06</v>
+        <v>4.899959143497e-06</v>
       </c>
       <c r="E138" s="51" t="s">
         <v>1099</v>
@@ -16953,7 +17327,7 @@
       </c>
       <c r="D139" s="149">
         <f>P_HOCl/(k1_NH2Cl*NH3_free)</f>
-        <v>1.656958212721e-09</v>
+        <v>1.609043289707e-09</v>
       </c>
       <c r="E139" s="51" t="s">
         <v>1102</v>
@@ -16971,7 +17345,7 @@
       </c>
       <c r="D140" s="149">
         <f>HOCl_ss*M_HOCl</f>
-        <v>8.692402783936e-05</v>
+        <v>8.441041097801e-05</v>
       </c>
       <c r="E140" s="51" t="s">
         <v>1105</v>
@@ -17060,7 +17434,7 @@
       </c>
       <c r="D145" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_mgL/R_chloramine</f>
-        <v>0.251019095638</v>
+        <v>0.250993959469</v>
       </c>
       <c r="E145" s="51" t="inlineStr">
         <is>
@@ -17262,7 +17636,7 @@
       </c>
       <c r="D156" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_lo/R_chloramine_hi</f>
-        <v>0.005129213575</v>
+        <v>0.005104077407</v>
       </c>
       <c r="E156" s="51" t="s">
         <v>1247</v>
@@ -17280,7 +17654,7 @@
       </c>
       <c r="D157" s="149">
         <f>f_local*HOCl_ss_mgL+NH2Cl_hi/R_chloramine_lo</f>
-        <v>0.477325878621</v>
+        <v>0.477300742452</v>
       </c>
       <c r="E157" s="51" t="s">
         <v>1251</v>
@@ -18046,7 +18420,7 @@
       </c>
       <c r="D206" s="141">
         <f>E0_OER-nernst_slope*pH_meas</f>
-        <v>0.862973862131</v>
+        <v>0.862219433479</v>
       </c>
       <c r="E206" s="99" t="s">
         <v>1586</v>
@@ -18064,7 +18438,7 @@
       </c>
       <c r="D207" s="141">
         <f>E0_HER-nernst_slope*pH_meas</f>
-        <v>-0.366026137869</v>
+        <v>-0.366780566521</v>
       </c>
       <c r="E207" s="99" t="s">
         <v>1589</v>
@@ -18104,7 +18478,7 @@
       </c>
       <c r="D209" s="141">
         <f>E_HOCl_Cl-E_anode_op</f>
-        <v>-0.427526934687</v>
+        <v>-0.427526678634</v>
       </c>
       <c r="E209" s="67" t="inlineStr">
         <is>
@@ -18124,7 +18498,7 @@
       </c>
       <c r="D210" s="141">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
-        <v>0.328973862131</v>
+        <v>0.328219433479</v>
       </c>
       <c r="E210" s="67" t="s">
         <v>1599</v>
@@ -18144,7 +18518,7 @@
       </c>
       <c r="D211" s="141">
         <f>E_anode_op-E0_Cu</f>
-        <v>1.265216285627</v>
+        <v>1.264461856975</v>
       </c>
       <c r="E211" s="67" t="s">
         <v>1602</v>
@@ -18206,7 +18580,7 @@
       </c>
       <c r="D216" s="141">
         <f>Fcc*((km_HPO4/100)*HPO4_op+(km_HCO3/100)*HCO3_op)*1000/10</f>
-        <v>8.598724981667</v>
+        <v>8.606311548487</v>
       </c>
       <c r="E216" s="67" t="inlineStr">
         <is>
@@ -18244,7 +18618,7 @@
       </c>
       <c r="D218" s="141">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>0.328664504833</v>
+        <v>0.328374783131</v>
       </c>
       <c r="E218" s="67" t="s">
         <v>1618</v>
@@ -18280,7 +18654,7 @@
       </c>
       <c r="D220" s="141">
         <f>pH_op-LOG10(gamma_1)</f>
-        <v>6.187122404381</v>
+        <v>6.199874888233</v>
       </c>
       <c r="E220" s="67" t="s">
         <v>1624</v>
@@ -18373,7 +18747,7 @@
       </c>
       <c r="D226" s="141">
         <f>C_eff*M_Cl2/M_HOCl</f>
-        <v>0.339282500863</v>
+        <v>0.339248526308</v>
       </c>
       <c r="E226" s="67" t="s">
         <v>1899</v>
@@ -18687,7 +19061,7 @@
       </c>
       <c r="D252" s="141">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
-        <v>0.026380308456</v>
+        <v>0.026289762412</v>
       </c>
       <c r="E252" s="67" t="inlineStr">
         <is>
@@ -18713,7 +19087,7 @@
       </c>
       <c r="D253" s="141">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
-        <v>0.006404116991</v>
+        <v>0.006561410067</v>
       </c>
       <c r="E253" s="67" t="inlineStr">
         <is>
@@ -18750,7 +19124,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t xml:space="preserve">(import) proton-coupled credit</t>
+          <t xml:space="preserve">(import) proton-coupled credit at the operating current</t>
         </is>
       </c>
       <c r="B255" s="18" t="inlineStr">
@@ -18764,12 +19138,12 @@
         </is>
       </c>
       <c r="D255" s="141">
-        <f>Electrochemistry!$D$113</f>
+        <f>Electrochemistry!$D$162</f>
         <v>-0.15</v>
       </c>
       <c r="E255" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import from Electrochemistry!D113.</t>
+          <t xml:space="preserve">Import from Electrochemistry!D162 (pcet_credit_op: withdrawn past the buffer limit).</t>
         </is>
       </c>
     </row>
@@ -18791,7 +19165,7 @@
       </c>
       <c r="D256" s="141">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
-        <v>1.607116285627</v>
+        <v>1.606361856975</v>
       </c>
       <c r="E256" s="67" t="inlineStr">
         <is>
@@ -18842,7 +19216,7 @@
       </c>
       <c r="D258" s="141">
         <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,1E-12))-pH_meas-LOG10(MAX(pH_Cl,1E-12)))</f>
-        <v>1.179589350939</v>
+        <v>1.178835178341</v>
       </c>
       <c r="E258" s="67" t="inlineStr">
         <is>
@@ -18868,7 +19242,7 @@
       </c>
       <c r="D259" s="141">
         <f>C_eff_lo*M_Cl2/M_HOCl</f>
-        <v>0.0069327491</v>
+        <v>0.006898774544</v>
       </c>
       <c r="E259" s="67" t="inlineStr">
         <is>
@@ -18894,7 +19268,7 @@
       </c>
       <c r="D260" s="141">
         <f>C_eff_hi*M_Cl2/M_HOCl</f>
-        <v>0.645163338724</v>
+        <v>0.645129364169</v>
       </c>
       <c r="E260" s="67" t="inlineStr">
         <is>
@@ -19165,6 +19539,225 @@
       <c r="E280" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">→ Summary (media_sel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC STORAGE IN THE CO₂ POOL (review R2-m3) — at a reference pH, so no loop through the pH solve</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reference pH for the DIC capacity (concentration scale)</t>
+        </is>
+      </c>
+      <c r="B291" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH_ref_DIC</t>
+        </is>
+      </c>
+      <c r="C291" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D291" s="131">
+        <v>6.09</v>
+      </c>
+      <c r="E291" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input, not a link: set to the last solved pH_op (D103) and re-enter if it moves by &gt;0.1. Linking D103 would close a loop D103 → CO2aqc → CO₂ pool → D103.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[H⁺] at the reference pH</t>
+        </is>
+      </c>
+      <c r="B292" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h_ref_DIC</t>
+        </is>
+      </c>
+      <c r="C292" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D292" s="141">
+        <f>10^-pH_ref_DIC</f>
+        <v>8.128305161641e-07</v>
+      </c>
+      <c r="E292" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concentration scale, as the charge balance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bicarbonate : CO₂(aq) at the reference pH</t>
+        </is>
+      </c>
+      <c r="B293" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">r_HCO3_ref</t>
+        </is>
+      </c>
+      <c r="C293" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D293" s="141">
+        <f>Ka1c_c/h_ref_DIC</f>
+        <v>0.907171771626</v>
+      </c>
+      <c r="E293" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ka1/[H⁺] on the concentration scale; independent of the CO₂ level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bicarbonate at the reference pH (from the charge balance)</t>
+        </is>
+      </c>
+      <c r="B294" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HCO3_ref</t>
+        </is>
+      </c>
+      <c r="C294" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D294" s="141">
+        <f>(pH_SID+pH_NT*h_ref_DIC/(h_ref_DIC+KaN_c)+h_ref_DIC-(pH_PT*Ka1p_c*h_ref_DIC^2+2*pH_PT*Ka1p_c*Ka2p_c*h_ref_DIC+3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/(h_ref_DIC^3+Ka1p_c*h_ref_DIC^2+Ka1p_c*Ka2p_c*h_ref_DIC+Ka1p_c*Ka2p_c*Ka3p_c)-Kw_c/h_ref_DIC)/(1+2*Ka2c_c/h_ref_DIC)</f>
+        <v>0.026358468464</v>
+      </c>
+      <c r="E294" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The same charge balance as the pH grid (B50), solved for carbonate alkalinity at the reference pH instead of for pH: no CO2aqc term, so no loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non-carbonate buffer capacity at the reference pH</t>
+        </is>
+      </c>
+      <c r="B295" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">beta_nonC</t>
+        </is>
+      </c>
+      <c r="C295" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L/pH</t>
+        </is>
+      </c>
+      <c r="D295" s="141">
+        <f>LN(10)*(pH_PT*Ka1p_c*h_ref_DIC/(Ka1p_c+h_ref_DIC)^2+pH_PT*Ka2p_c*h_ref_DIC/(Ka2p_c+h_ref_DIC)^2+pH_NT*KaN_c*h_ref_DIC/(KaN_c+h_ref_DIC)^2+h_ref_DIC+Kw_c/h_ref_DIC)</f>
+        <v>0.012467843562</v>
+      </c>
+      <c r="E295" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">β = ln10·Σ C·Ka·[H⁺]/(Ka+[H⁺])² over phosphate (pKa1, pKa2), ammonium and water — what takes up the proton when absorbed CO₂ becomes bicarbonate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC capacity factor of the liquid (dDIC/dCO₂(aq))</t>
+        </is>
+      </c>
+      <c r="B296" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC_cap</t>
+        </is>
+      </c>
+      <c r="C296" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D296" s="141">
+        <f>1+r_HCO3_ref*beta_nonC/(beta_nonC+LN(10)*HCO3_ref)</f>
+        <v>1.154598203915</v>
+      </c>
+      <c r="E296" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At constant alkalinity each mol of CO₂ absorbed forms Ka1/[H⁺]·β/(β+ln10·[HCO₃⁻]) mol of bicarbonate as the pH falls. Bounds: 1 (no buffer) and 1+Ka1/[H⁺] (infinite buffer, R2-m3's form, ≈1.9 here). Linearised about the reference pH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DISPLAY THRESHOLDS (read by the Summary colour rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH red band, lower edge</t>
+        </is>
+      </c>
+      <c r="B299" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH_red_lo</t>
+        </is>
+      </c>
+      <c r="C299" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D299" s="131">
+        <v>6</v>
+      </c>
+      <c r="E299" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: below pH 6 HOB growth is taken as severely impaired; the red edge of the Summary D35 colour (was embedded in the rule).</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH red band, upper edge</t>
+        </is>
+      </c>
+      <c r="B300" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH_red_hi</t>
+        </is>
+      </c>
+      <c r="C300" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D300" s="131">
+        <v>8</v>
+      </c>
+      <c r="E300" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption, as above, for the alkaline side.</t>
         </is>
       </c>
     </row>
@@ -19249,7 +19842,7 @@
       </c>
       <c r="D4" s="150">
         <f>Electrochemistry!$D$21</f>
-        <v>0.0001017274698715</v>
+        <v>0.0001018812158154</v>
       </c>
       <c r="E4" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D21","→ Electrochemistry")</f>
@@ -19269,7 +19862,7 @@
       </c>
       <c r="D5" s="150">
         <f>Electrochemistry!$D$29</f>
-        <v>4.979033518202e-05</v>
+        <v>4.987344109764e-05</v>
       </c>
       <c r="E5" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -19410,7 +20003,7 @@
       </c>
       <c r="D13" s="48">
         <f>MAX(0,rH2_gen-H2_HOR_b)</f>
-        <v>0.0001017274698715</v>
+        <v>0.0001018812158154</v>
       </c>
       <c r="E13" s="37" t="inlineStr">
         <is>
@@ -19431,7 +20024,7 @@
       </c>
       <c r="D14" s="48">
         <f>H2_cons*bio_O2/bio_H2</f>
-        <v>3.390915662382e-05</v>
+        <v>3.396040527179e-05</v>
       </c>
       <c r="E14" s="107" t="s">
         <v>421</v>
@@ -19450,7 +20043,7 @@
       </c>
       <c r="D15" s="48">
         <f>H2_cons*bio_CO2/bio_H2</f>
-        <v>1.695457831191e-05</v>
+        <v>1.698020263589e-05</v>
       </c>
       <c r="E15" s="37" t="s">
         <v>424</v>
@@ -19469,7 +20062,7 @@
       </c>
       <c r="D16" s="48">
         <f>MAX(0,O2_net_gen-O2_cons)</f>
-        <v>1.58811785582e-05</v>
+        <v>1.591303582585e-05</v>
       </c>
       <c r="E16" s="115" t="inlineStr">
         <is>
@@ -19618,11 +20211,13 @@
         <v>440</v>
       </c>
       <c r="D24" s="64">
-        <f>H_O2ref*EXP(H_O2T*(1/T_K-1/T_ref))</f>
-        <v>1.2e-05</v>
-      </c>
-      <c r="E24" s="99" t="s">
-        <v>450</v>
+        <f>H_O2ref*EXP(H_O2T*(1/T_K-1/T_ref))*f_salt_O2</f>
+        <v>1.158290914481e-05</v>
+      </c>
+      <c r="E24" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">van 't Hoff correction to reactor T, then salted out for the medium's ionic strength (f_salt_O2, D123). Moves the dissolved-O₂ ceiling (D27) and every Henry O₂ term.</t>
+        </is>
       </c>
       <c r="F24" s="20"/>
     </row>
@@ -19675,7 +20270,7 @@
       </c>
       <c r="D27" s="46">
         <f>H_O2_T*O2_ceil_Pa</f>
-        <v>0.36477</v>
+        <v>0.352091480729</v>
       </c>
       <c r="E27" s="99" t="s">
         <v>461</v>
@@ -19694,7 +20289,7 @@
       </c>
       <c r="D28" s="43">
         <f>O2_ceil_C*1000</f>
-        <v>364.77</v>
+        <v>352.091480729401</v>
       </c>
       <c r="E28" s="65" t="s">
         <v>464</v>
@@ -19954,7 +20549,7 @@
       </c>
       <c r="D42" s="48">
         <f>C_H2_sat*(V_charge/1000000)/rH2_gen*60</f>
-        <v>6.992226395671</v>
+        <v>6.981674632634</v>
       </c>
       <c r="E42" s="99" t="s">
         <v>504</v>
@@ -19973,7 +20568,7 @@
       </c>
       <c r="D43" s="48">
         <f>rH2_gen/(V_charge/1000000)/C_H2_sat</f>
-        <v>8.580957853016</v>
+        <v>8.593926694829</v>
       </c>
       <c r="E43" s="69" t="s">
         <v>508</v>
@@ -19994,7 +20589,7 @@
       </c>
       <c r="D44" s="48" t="str">
         <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag, mean basis; H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 18% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 17% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="70" t="inlineStr">
         <is>
@@ -20443,7 +21038,7 @@
       </c>
       <c r="D76" s="150">
         <f>'Mass Transfer'!$D$100</f>
-        <v>0.0007098184304685</v>
+        <v>0.0007156055654322</v>
       </c>
       <c r="E76" s="135" t="inlineStr">
         <is>
@@ -20480,7 +21075,7 @@
     <row r="78">
       <c r="A78" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">(import) pulse duration</t>
+          <t xml:space="preserve">(import) optimal pulse, full-flow equivalent</t>
         </is>
       </c>
       <c r="B78" s="18" t="inlineStr">
@@ -20494,12 +21089,12 @@
         </is>
       </c>
       <c r="D78" s="150">
-        <f>'Mass Transfer'!$D$90</f>
+        <f>'Mass Transfer'!$D$409</f>
         <v>0.784513049825</v>
       </c>
       <c r="E78" s="135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import from Mass Transfer!D90.</t>
+          <t xml:space="preserve">Import from Mass Transfer!D409 (spg_dur_eq_opt): converts the H₂-safe duty to an interval on the same basis as the schedule.</t>
         </is>
       </c>
     </row>
@@ -20622,7 +21217,7 @@
       </c>
       <c r="D83" s="48">
         <f>H2_src_l_b+O2_net_gen</f>
-        <v>0.0001515178050535</v>
+        <v>0.000151754656913</v>
       </c>
       <c r="E83" s="69" t="inlineStr">
         <is>
@@ -20648,7 +21243,7 @@
       </c>
       <c r="D84" s="48">
         <f>H2_src_l_b/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.113266761861</v>
+        <v>0.112682153807</v>
       </c>
       <c r="E84" s="69" t="inlineStr">
         <is>
@@ -20674,7 +21269,7 @@
       </c>
       <c r="D85" s="48">
         <f>(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.064019231488</v>
+        <v>0.063684612076</v>
       </c>
       <c r="E85" s="69" t="inlineStr">
         <is>
@@ -20700,7 +21295,7 @@
       </c>
       <c r="D86" s="48">
         <f>MAX(0,MIN(H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
-        <v>0.003376651195</v>
+        <v>0.003381603867</v>
       </c>
       <c r="E86" s="69" t="inlineStr">
         <is>
@@ -20726,7 +21321,7 @@
       </c>
       <c r="D87" s="48">
         <f>IF(duty_H2safe&gt;0,spg_dur_b/(60*duty_H2safe),NA())</f>
-        <v>3.872244049322</v>
+        <v>3.866572790086</v>
       </c>
       <c r="E87" s="69" t="inlineStr">
         <is>
@@ -20752,7 +21347,7 @@
       </c>
       <c r="D88" s="48">
         <f>MAX(0,H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
-        <v>0.960219102801</v>
+        <v>0.961689798439</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
@@ -20811,7 +21406,7 @@
       </c>
       <c r="D97" s="48">
         <f>'Mass Transfer'!$D$198</f>
-        <v>29.726224026733</v>
+        <v>28.788742057202</v>
       </c>
       <c r="E97" s="67" t="inlineStr">
         <is>
@@ -20837,7 +21432,7 @@
       </c>
       <c r="D98" s="48">
         <f>C_cycle_start_b*1000/Km_CO2</f>
-        <v>594.524480534657</v>
+        <v>575.774841144035</v>
       </c>
       <c r="E98" s="69" t="inlineStr">
         <is>
@@ -20922,7 +21517,7 @@
       </c>
       <c r="D113" s="150">
         <f>'Mass Transfer'!$D$314</f>
-        <v>0.0001017274698715</v>
+        <v>0.0001018812158154</v>
       </c>
       <c r="E113" s="135" t="inlineStr">
         <is>
@@ -20948,11 +21543,95 @@
       </c>
       <c r="D114" s="150">
         <f>'Mass Transfer'!$D$388</f>
-        <v>0.175164116673</v>
+        <v>0.174311272995</v>
       </c>
       <c r="E114" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D388 (sawtooth top).</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ SALTING-OUT (review R2-m8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) ionic strength of the medium</t>
+        </is>
+      </c>
+      <c r="B121" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I_ionic_b</t>
+        </is>
+      </c>
+      <c r="C121" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D121" s="150">
+        <f>Chemistry!$D$185</f>
+        <v>0.109739973238</v>
+      </c>
+      <c r="E121" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Chemistry!D185 (I_ionic, by media_sel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Setschenow coefficient for O₂ (per unit ionic strength)</t>
+        </is>
+      </c>
+      <c r="B122" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ks_O2</t>
+        </is>
+      </c>
+      <c r="C122" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L/mol</t>
+        </is>
+      </c>
+      <c r="D122" s="131">
+        <v>0.14</v>
+      </c>
+      <c r="E122" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weisenberger &amp; Schumpe (1996) AIChE J 42:298, ion-specific h_i summed over the UdG recipe at 25 °C (Na⁺ 0.1143, K⁺ 0.0922, NH₄⁺ 0.0556, Mg²⁺ 0.1694, SO₄²⁻ 0.1117, H₂PO₄⁻ 0.0906, HPO₄²⁻ 0.1499, HCO₃⁻ 0.0967 L/mol; h_G(O₂) = 0) gives Σh·c = 0.0154 = 0.14 × I. Lumped per unit I, so approximate for other media.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ salting-out factor</t>
+        </is>
+      </c>
+      <c r="B123" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f_salt_O2</t>
+        </is>
+      </c>
+      <c r="C123" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D123" s="150">
+        <f>10^(-ks_O2*I_ionic_b)</f>
+        <v>0.965242428734</v>
+      </c>
+      <c r="E123" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Setschenow: log₁₀(H₀/H) = k_s·I. 0.965 for UdG (−3.5 %).</t>
         </is>
       </c>
     </row>
@@ -21078,7 +21757,7 @@
       </c>
       <c r="D6" s="142">
         <f>Biology!$D$27</f>
-        <v>0.36477</v>
+        <v>0.352091480729</v>
       </c>
       <c r="E6" s="135" t="str">
         <f>HYPERLINK("#Biology!D27","→ Biology")</f>
@@ -21158,7 +21837,7 @@
       </c>
       <c r="D10" s="142">
         <f>Biology!$D$15</f>
-        <v>1.695457831191e-05</v>
+        <v>1.698020263589e-05</v>
       </c>
       <c r="E10" s="135" t="str">
         <f>HYPERLINK("#Biology!D15","→ Biology")</f>
@@ -21178,7 +21857,7 @@
       </c>
       <c r="D11" s="142">
         <f>Biology!$D$16</f>
-        <v>1.58811785582e-05</v>
+        <v>1.591303582585e-05</v>
       </c>
       <c r="E11" s="135" t="str">
         <f>HYPERLINK("#Biology!D16","→ Biology")</f>
@@ -21198,7 +21877,7 @@
       </c>
       <c r="D12" s="142">
         <f>Biology!$D$24</f>
-        <v>1.2e-05</v>
+        <v>1.158290914481e-05</v>
       </c>
       <c r="E12" s="135" t="str">
         <f>HYPERLINK("#Biology!D24","→ Biology")</f>
@@ -21218,7 +21897,7 @@
       </c>
       <c r="D13" s="150">
         <f>Electrochemistry!$D$29</f>
-        <v>4.979033518202e-05</v>
+        <v>4.987344109764e-05</v>
       </c>
       <c r="E13" s="135" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -21963,7 +22642,7 @@
       </c>
       <c r="D53" s="64">
         <f>kLa_sparge*duty</f>
-        <v>2.239153688755e-05</v>
+        <v>1.939632125669e-05</v>
       </c>
       <c r="E53" s="117" t="s">
         <v>643</v>
@@ -21982,7 +22661,7 @@
       </c>
       <c r="D54" s="48">
         <f>IF(d_bubble&lt;d_bubble_min_m,0,kLa_sparge*(V_charge/1000000)*O2_ceil_C*3600)</f>
-        <v>0.0003044695410516</v>
+        <v>0.0002938869192802</v>
       </c>
       <c r="E54" s="75" t="s">
         <v>646</v>
@@ -22001,7 +22680,7 @@
       </c>
       <c r="D55" s="48">
         <f>strip_sparge*duty</f>
-        <v>4.410590891654e-07</v>
+        <v>3.687810914865e-07</v>
       </c>
       <c r="E55" s="75" t="s">
         <v>649</v>
@@ -22020,7 +22699,7 @@
       </c>
       <c r="D56" s="45">
         <f>IF(O2_excess&gt;0,strip_avg/O2_excess,NA())</f>
-        <v>0.027772440663</v>
+        <v>0.023174779189</v>
       </c>
       <c r="E56" s="75" t="s">
         <v>652</v>
@@ -22039,7 +22718,7 @@
       </c>
       <c r="D57" s="48">
         <f>IF(O2_excess&gt;0,O2_excess/3600/((V_charge/1000000)*O2_ceil_C),NA())</f>
-        <v>0.000806250237755</v>
+        <v>0.0008369581905715</v>
       </c>
       <c r="E57" s="75" t="s">
         <v>655</v>
@@ -22075,11 +22754,13 @@
         <v>135</v>
       </c>
       <c r="D59" s="58" t="str">
-        <f>IF(u_sg&gt;u_g_max,"RISK","OK")</f>
-        <v>OK</v>
-      </c>
-      <c r="E59" s="75" t="s">
-        <v>661</v>
+        <f>IF(carry_n=0,"not measured – record the max flow without carryover for "&amp;Reactor&amp;" in CO2 flows column M",IF(Q_CO2/60&gt;Q_carry_max,"RISK – pulse flow "&amp;TEXT(Q_CO2/60,"0.00")&amp;" mL/s exceeds the measured "&amp;TEXT(Q_carry_max,"0.00")&amp;" mL/s no-carryover limit","OK – pulse flow "&amp;TEXT(Q_CO2/60,"0.00")&amp;" mL/s within the measured "&amp;TEXT(Q_carry_max,"0.00")&amp;" mL/s no-carryover limit"))</f>
+        <v>not measured – record the max flow without carryover for ed04 in CO2 flows column M</v>
+      </c>
+      <c r="E59" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse flow (Q_CO2) against the measured per-reactor no-carryover maximum (D413, CO2 flows column M). "not measured" until a value is entered, never a default OK. The superficial-velocity rule is the secondary line D414.</t>
+        </is>
       </c>
       <c r="F59" s="20"/>
     </row>
@@ -22189,7 +22870,7 @@
       </c>
       <c r="D65" s="48">
         <f>O2_ceil_C*(V_charge/1000000)/O2_excess*60</f>
-        <v>20.671828529408</v>
+        <v>19.913380207541</v>
       </c>
       <c r="E65" s="99" t="inlineStr">
         <is>
@@ -22210,7 +22891,7 @@
       </c>
       <c r="D66" s="48">
         <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,"never (strip ≥ source)")</f>
-        <v>21.262335479879</v>
+        <v>20.385817015456</v>
       </c>
       <c r="E66" s="99" t="inlineStr">
         <is>
@@ -22349,7 +23030,7 @@
       </c>
       <c r="D73" s="48">
         <f>kLa_surf_used*(V_charge/1000000)*O2_ceil_C*3600</f>
-        <v>0.0001418246177951</v>
+        <v>0.0001368951385348</v>
       </c>
       <c r="E73" s="69" t="s">
         <v>1002</v>
@@ -22368,7 +23049,7 @@
       </c>
       <c r="D74" s="48">
         <f>IF(O2_excess&gt;0,surf_strip/O2_excess,NA())</f>
-        <v>8.930358491677</v>
+        <v>8.602704099515</v>
       </c>
       <c r="E74" s="69" t="s">
         <v>702</v>
@@ -22402,11 +23083,13 @@
         <v>67</v>
       </c>
       <c r="D77" s="48">
-        <f>headspace_V/(Q_CO2*duty)</f>
-        <v>9.026013902172</v>
-      </c>
-      <c r="E77" s="99" t="s">
-        <v>710</v>
+        <f>headspace_V*spg_int/V_pulse</f>
+        <v>8.95302011459</v>
+      </c>
+      <c r="E77" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean time to deliver one headspace volume of CO₂: the interval × headspace ÷ pulse volume (D411).</t>
+        </is>
       </c>
       <c r="F77" s="20"/>
     </row>
@@ -22422,7 +23105,7 @@
       </c>
       <c r="D78" s="48">
         <f>IF(O2_excess&gt;0,(strip_avg+surf_strip)/O2_excess,NA())</f>
-        <v>8.95813093234</v>
+        <v>8.625878878704</v>
       </c>
       <c r="E78" s="118" t="s">
         <v>713</v>
@@ -22441,7 +23124,7 @@
       </c>
       <c r="D79" s="48">
         <f>O2_ceil_C*(V_charge/1000000)/O2_net_gen*60</f>
-        <v>6.593508535339</v>
+        <v>6.353729072676</v>
       </c>
       <c r="E79" s="99" t="s">
         <v>716</v>
@@ -22574,7 +23257,7 @@
       </c>
       <c r="D86" s="48">
         <f>carbon_margin_min*CO2_cons/(nCO2_rate*3600)</f>
-        <v>6.920263645416e-05</v>
+        <v>6.930722594878e-05</v>
       </c>
       <c r="E86" s="99" t="s">
         <v>733</v>
@@ -22593,7 +23276,7 @@
       </c>
       <c r="D87" s="48">
         <f>O2_src_guard/(target_DO_frac*(O2_ceil_Pa/P_atm))/(nCO2_rate*3600)</f>
-        <v>0.001498145312</v>
+        <v>0.001500645892</v>
       </c>
       <c r="E87" s="99" t="s">
         <v>1063</v>
@@ -22612,7 +23295,7 @@
       </c>
       <c r="D88" s="48">
         <f>MAX(duty_carbon,duty_O2vent)</f>
-        <v>0.001498145312</v>
+        <v>0.001500645892</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
@@ -22635,7 +23318,7 @@
       </c>
       <c r="D89" s="48">
         <f>target_DO_frac*O2_ceil_C*(V_charge/1000000)/O2_src_guard*60</f>
-        <v>1.490706277555</v>
+        <v>1.436495268605</v>
       </c>
       <c r="E89" s="99" t="inlineStr">
         <is>
@@ -22655,11 +23338,13 @@
         <v>13</v>
       </c>
       <c r="D90" s="48">
-        <f>MAX(pulse_floor,flush_factor*headspace_V/(Q_CO2/60))</f>
-        <v>0.784513049825</v>
-      </c>
-      <c r="E90" s="159" t="s">
-        <v>742</v>
+        <f>MAX(pulse_floor,(flush_factor*headspace_V-pulse_V0)/Q_CO2_fit)</f>
+        <v>0.674076519917</v>
+      </c>
+      <c r="E90" s="159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANSWER. Shortest reliable pulse: the time at which V₀ + Q_fit·t delivers flush_factor headspace volumes (R2-M3), never below the solenoid floor (pulse_floor).</t>
+        </is>
       </c>
       <c r="F90" s="20"/>
     </row>
@@ -22675,7 +23360,7 @@
       </c>
       <c r="D91" s="48">
         <f>IF(ISNA(F_vent_ex+O2_src_sched),NA(),IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max)))</f>
-        <v>9.026013902172</v>
+        <v>8.95302011459</v>
       </c>
       <c r="E91" s="159" t="inlineStr">
         <is>
@@ -22696,7 +23381,7 @@
       </c>
       <c r="D92" s="48">
         <f>spg_int_opt*60</f>
-        <v>541.560834130326</v>
+        <v>537.181206875374</v>
       </c>
       <c r="E92" s="159" t="s">
         <v>747</v>
@@ -22706,7 +23391,7 @@
     <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  resulting duty</t>
+          <t xml:space="preserve">  resulting duty (full-flow equivalent)</t>
         </is>
       </c>
       <c r="B93" s="18" t="s">
@@ -22716,11 +23401,13 @@
         <v>135</v>
       </c>
       <c r="D93" s="48">
-        <f>spg_dur_opt/(spg_int_opt*60)</f>
-        <v>0.001448614819</v>
-      </c>
-      <c r="E93" s="99" t="s">
-        <v>750</v>
+        <f>spg_dur_eq_opt/(spg_int_opt*60)</f>
+        <v>0.001460425346</v>
+      </c>
+      <c r="E93" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ actually delivered at the optimum as a fraction of continuous full flow: the full-flow-equivalent pulse (D409) over the interval. With a pulse intercept this exceeds the valve-open fraction (D105).</t>
+        </is>
       </c>
       <c r="F93" s="20"/>
     </row>
@@ -22850,7 +23537,7 @@
       </c>
       <c r="D100" s="28">
         <f>CO2_pulse*pulses_h</f>
-        <v>0.0007098184304685</v>
+        <v>0.0007156055654322</v>
       </c>
       <c r="E100" s="160" t="s">
         <v>765</v>
@@ -22943,7 +23630,7 @@
       </c>
       <c r="D105" s="28">
         <f>spg_dur/(spg_int*60)</f>
-        <v>0.001448614819</v>
+        <v>0.001254840101</v>
       </c>
       <c r="E105" s="160" t="s">
         <v>765</v>
@@ -22992,7 +23679,7 @@
       </c>
       <c r="D108" s="28">
         <f>DO_avg_sched*M_O2</f>
-        <v>2.634776001183</v>
+        <v>2.543598660379</v>
       </c>
       <c r="E108" s="160" t="inlineStr">
         <is>
@@ -23053,8 +23740,8 @@
         <v>67</v>
       </c>
       <c r="D112" s="28">
-        <f>spg_dur_opt/(60*duty_carbon)</f>
-        <v>188.941031253092</v>
+        <f>spg_dur_eq_opt/(60*duty_carbon)</f>
+        <v>188.655905904325</v>
       </c>
       <c r="E112" s="20"/>
       <c r="F112" s="20"/>
@@ -23069,7 +23756,7 @@
       <c r="C113" s="20"/>
       <c r="D113" s="28" t="str">
         <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) the cycle-mean DO would be ≈"&amp;TEXT(DO_at_carbon*M_O2,"0")&amp;" mg/L, "&amp;IF(DO_at_carbon&gt;O2_ceil_C,"above the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L inhibition ceiling","against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")&amp;" (peaks higher)")</f>
-        <v>Do NOT relax: at the carbon-limited interval (189 min) the cycle-mean DO would be ≈16 mg/L, above the 11.7 mg/L inhibition ceiling (peaks higher)</v>
+        <v>Do NOT relax: at the carbon-limited interval (189 min) the cycle-mean DO would be ≈15 mg/L, above the 11.3 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E113" s="82" t="inlineStr">
         <is>
@@ -23204,7 +23891,7 @@
       </c>
       <c r="D121" s="28">
         <f>IF(AND(ISNUMBER(override_spg_dur_s),override_spg_dur_s&gt;0),override_spg_dur_s,IF(sched_mode="Manual",spg_dur_man,IF(sched_mode="Optimal",spg_dur_opt,NA())))</f>
-        <v>0.784513049825</v>
+        <v>0.674076519917</v>
       </c>
       <c r="E121" s="20"/>
       <c r="F121" s="20"/>
@@ -23221,7 +23908,7 @@
       </c>
       <c r="D122" s="28">
         <f>IF(AND(ISNUMBER(override_spg_int_min),override_spg_int_min&gt;0),override_spg_int_min,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
-        <v>9.026013902172</v>
+        <v>8.95302011459</v>
       </c>
       <c r="E122" s="20"/>
       <c r="F122" s="20"/>
@@ -23237,10 +23924,14 @@
         <v>815</v>
       </c>
       <c r="D123" s="28">
-        <f>nCO2_rate*spg_dur</f>
+        <f>P_atm*(V_pulse/1000000)/(R_gas*T_K)</f>
         <v>0.0001067805170238</v>
       </c>
-      <c r="E123" s="20"/>
+      <c r="E123" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ideal-gas moles in the pulse volume V₀ + Q_fit·t (D411), so the fixed solenoid volume is counted (R2-M3).</t>
+        </is>
+      </c>
       <c r="F123" s="20"/>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.2">
@@ -23255,7 +23946,7 @@
       </c>
       <c r="D124" s="28">
         <f>60/spg_int</f>
-        <v>6.647452646352</v>
+        <v>6.701649190112</v>
       </c>
       <c r="E124" s="20"/>
       <c r="F124" s="20"/>
@@ -23272,7 +23963,7 @@
       </c>
       <c r="D125" s="28">
         <f>pulses_h*24</f>
-        <v>159.538863512438</v>
+        <v>160.8395805627</v>
       </c>
       <c r="E125" s="20"/>
       <c r="F125" s="20"/>
@@ -23289,7 +23980,7 @@
       </c>
       <c r="D126" s="28">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v>41.865885273592</v>
+        <v>42.143523300455</v>
       </c>
       <c r="E126" s="20"/>
       <c r="F126" s="20"/>
@@ -23306,7 +23997,7 @@
       </c>
       <c r="D127" s="28">
         <f>O2_excess/60*spg_int</f>
-        <v>2.389062307486e-06</v>
+        <v>2.374495497218e-06</v>
       </c>
       <c r="E127" s="20"/>
       <c r="F127" s="20"/>
@@ -23323,7 +24014,7 @@
       </c>
       <c r="D128" s="28">
         <f>strip_sparge/3600*spg_dur</f>
-        <v>6.635009117477e-08</v>
+        <v>5.502840883265e-08</v>
       </c>
       <c r="E128" s="20"/>
       <c r="F128" s="20"/>
@@ -23340,7 +24031,7 @@
       </c>
       <c r="D129" s="28">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v>0.027772440663</v>
+        <v>0.023174779189</v>
       </c>
       <c r="E129" s="20"/>
       <c r="F129" s="20"/>
@@ -23374,7 +24065,7 @@
       </c>
       <c r="D131" s="28">
         <f>kLa_surf_req/a_surf</f>
-        <v>0.0001245300561075</v>
+        <v>0.0001292730786929</v>
       </c>
       <c r="E131" s="147" t="s">
         <v>1825</v>
@@ -23393,7 +24084,7 @@
       </c>
       <c r="D132" s="28">
         <f>O2_net_gen</f>
-        <v>4.979033518202e-05</v>
+        <v>4.987344109764e-05</v>
       </c>
       <c r="E132" s="69" t="s">
         <v>992</v>
@@ -23414,7 +24105,7 @@
       </c>
       <c r="D133" s="28">
         <f>DO_avg_sched</f>
-        <v>0.082341896405</v>
+        <v>0.079492426413</v>
       </c>
       <c r="E133" s="69" t="inlineStr">
         <is>
@@ -23458,7 +24149,7 @@
       </c>
       <c r="D135" s="28">
         <f>DO_avg_l</f>
-        <v>0.212069565945</v>
+        <v>0.206435018988</v>
       </c>
       <c r="E135" s="69" t="inlineStr">
         <is>
@@ -23631,11 +24322,13 @@
         <v>460</v>
       </c>
       <c r="D145" s="48">
-        <f>hs_H_CO2*P_atm</f>
-        <v>33.43725</v>
-      </c>
-      <c r="E145" s="67" t="s">
-        <v>1177</v>
+        <f>hs_H_CO2*P_dry</f>
+        <v>32.39387710822</v>
+      </c>
+      <c r="E145" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Henry-law dissolved CO₂ under a pure-CO₂ headspace, on the dry-gas basis (P_dry, D418).</t>
+        </is>
       </c>
       <c r="F145" s="20"/>
     </row>
@@ -23748,7 +24441,7 @@
       </c>
       <c r="D151" s="48">
         <f>spg_dur</f>
-        <v>0.784513049825</v>
+        <v>0.674076519917</v>
       </c>
       <c r="E151" s="67" t="s">
         <v>1189</v>
@@ -23767,7 +24460,7 @@
       </c>
       <c r="D152" s="48">
         <f>MAX(0,spg_int*60-spg_dur)</f>
-        <v>540.776321080501</v>
+        <v>536.507130355457</v>
       </c>
       <c r="E152" s="67" t="s">
         <v>1190</v>
@@ -23858,7 +24551,7 @@
       </c>
       <c r="D162" s="48">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,CO2_cyc_avg_new))/1000</f>
-        <v>0.029931790408</v>
+        <v>0.02896589844</v>
       </c>
       <c r="E162" s="67" t="s">
         <v>1859</v>
@@ -24104,7 +24797,7 @@
       </c>
       <c r="D179" s="141">
         <f>IF(ISNUMBER(DO_opt),DO_opt/M_O2,target_DO_frac*O2_ceil_C)</f>
-        <v>0.08246973913</v>
+        <v>0.079603291295</v>
       </c>
       <c r="E179" s="99" t="inlineStr">
         <is>
@@ -24124,7 +24817,7 @@
       </c>
       <c r="D180" s="141">
         <f>O2_src_sched/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.040846064617</v>
+        <v>0.040928000854</v>
       </c>
       <c r="E180" s="67" t="inlineStr">
         <is>
@@ -24144,7 +24837,7 @@
       </c>
       <c r="D181" s="141">
         <f>O2_net_gen/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.128059718029</v>
+        <v>0.128273464734</v>
       </c>
       <c r="E181" s="67" t="s">
         <v>1801</v>
@@ -24162,7 +24855,7 @@
       </c>
       <c r="D182" s="141">
         <f>DO_target-DO_surf_excess</f>
-        <v>0.041623674514</v>
+        <v>0.038675290442</v>
       </c>
       <c r="E182" s="67" t="s">
         <v>1804</v>
@@ -24179,8 +24872,8 @@
         <v>1274</v>
       </c>
       <c r="D183" s="141">
-        <f>IF(hs_O2_allow&gt;0,hs_O2_allow/(H_O2_T*P_atm),NA())</f>
-        <v>0.034232810687</v>
+        <f>IF(hs_O2_allow&gt;0,hs_O2_allow/(H_O2_T*P_dry),NA())</f>
+        <v>0.034014723392</v>
       </c>
       <c r="E183" s="67" t="s">
         <v>1807</v>
@@ -24198,7 +24891,7 @@
       </c>
       <c r="D184" s="141">
         <f>IF(ISNUMBER(y_O2_star),MAX(0,((O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_vent_ex-O2_src_sched-H2_src_sched+CO2_fix_sched)/CO2_rate_full),NA())</f>
-        <v>0.001448614819</v>
+        <v>0.001460425346</v>
       </c>
       <c r="E184" s="67" t="inlineStr">
         <is>
@@ -24217,8 +24910,8 @@
         <v>962</v>
       </c>
       <c r="D185" s="141">
-        <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_opt/(60*duty_DO),spg_int_carbon),NA())</f>
-        <v>9.026013902172</v>
+        <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_eq_opt/(60*duty_DO),spg_int_carbon),NA())</f>
+        <v>8.95302011459</v>
       </c>
       <c r="E185" s="67" t="s">
         <v>1813</v>
@@ -24236,7 +24929,7 @@
       </c>
       <c r="D186" s="141">
         <f>O2_src_sched/(DO_target*3600*(V_charge/1000000))</f>
-        <v>0.003566106821</v>
+        <v>0.003701930458</v>
       </c>
       <c r="E186" s="67" t="inlineStr">
         <is>
@@ -24256,7 +24949,7 @@
       </c>
       <c r="D187" s="141">
         <f>IF(O2_sizing_phase=phase_name_1,y_O2_mf_g,IF(O2_sizing_phase=phase_name_2,y_O2_mf_l,NA()))</f>
-        <v>0.031639138319</v>
+        <v>0.031437574558</v>
       </c>
       <c r="E187" s="67" t="inlineStr">
         <is>
@@ -24275,8 +24968,8 @@
         <v>1001</v>
       </c>
       <c r="D188" s="141">
-        <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_atm,NA())</f>
-        <v>0.038470028282</v>
+        <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_dry,NA())</f>
+        <v>0.03574503055</v>
       </c>
       <c r="E188" s="67" t="inlineStr">
         <is>
@@ -24338,11 +25031,13 @@
         <v>1274</v>
       </c>
       <c r="D193" s="141">
-        <f>V_L_m3/(V_L_m3+Vg_CO2)</f>
-        <v>0.824472095076</v>
-      </c>
-      <c r="E193" s="99" t="s">
-        <v>1838</v>
+        <f>V_L_CO2/(V_L_CO2+Vg_CO2)</f>
+        <v>0.844315888516</v>
+      </c>
+      <c r="E193" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fraction of a pooled CO₂ inventory that ends up in the liquid, counting the bicarbonate the absorbed CO₂ forms (V_L_CO2 = DIC_cap × V_L, D416).</t>
+        </is>
       </c>
     </row>
     <row r="194" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -24359,7 +25054,7 @@
       </c>
       <c r="D194" s="141">
         <f>C_sat_CO2*(1-pool_a)*(1-flush_ret)</f>
-        <v>3.710023297714</v>
+        <v>3.187917972005</v>
       </c>
       <c r="E194" s="99" t="inlineStr">
         <is>
@@ -24378,8 +25073,8 @@
         <v>639</v>
       </c>
       <c r="D195" s="141">
-        <f>k_vent*Vg_CO2/(V_L_m3+Vg_CO2)</f>
-        <v>1.679738870232e-05</v>
+        <f>k_vent*Vg_CO2/(V_L_CO2+Vg_CO2)</f>
+        <v>1.489840909629e-05</v>
       </c>
       <c r="E195" s="99" t="inlineStr">
         <is>
@@ -24419,7 +25114,7 @@
       </c>
       <c r="D197" s="141">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
-        <v>0.990957501466</v>
+        <v>0.992038757191</v>
       </c>
       <c r="E197" s="99" t="s">
         <v>1849</v>
@@ -24437,7 +25132,7 @@
       </c>
       <c r="D198" s="141">
         <f>(pool_D_gap+pool_b*pool_e)/(1-pool_ret*pool_e)</f>
-        <v>29.726224026733</v>
+        <v>28.788742057202</v>
       </c>
       <c r="E198" s="99" t="inlineStr">
         <is>
@@ -24457,7 +25152,7 @@
       </c>
       <c r="D199" s="141">
         <f>pool_ret*C_cycle_start+pool_b</f>
-        <v>30.13798016156</v>
+        <v>29.14352746255</v>
       </c>
       <c r="E199" s="99" t="inlineStr">
         <is>
@@ -24477,7 +25172,7 @@
       </c>
       <c r="D200" s="141">
         <f>C_cycle_peak*pool_phi+pool_D_raw*pool_psi</f>
-        <v>29.931790407874</v>
+        <v>28.965898440445</v>
       </c>
       <c r="E200" s="99" t="inlineStr">
         <is>
@@ -24794,8 +25489,8 @@
         </is>
       </c>
       <c r="D232" s="141">
-        <f>IF(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,DO_surf_excess+H_O2_T*P_atm*MIN(1,saw_factor*(O2_src_sched+y_O2_air*F_vent_ex)/(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)),DO_surf_excess+H_O2_T*P_atm)</f>
-        <v>0.486561365549</v>
+        <f>IF(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,DO_surf_excess+H_O2_T*P_dry*MIN(1,saw_factor*(O2_src_sched+y_O2_air*F_vent_ex)/(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)),DO_surf_excess+H_O2_T*P_dry)</f>
+        <v>0.457945290479</v>
       </c>
       <c r="E232" s="99" t="inlineStr">
         <is>
@@ -24853,7 +25548,7 @@
       </c>
       <c r="D242" s="141">
         <f>MAX(pulse_floor,MROUND(spg_dur_opt,pulse_res))</f>
-        <v>0.8</v>
+        <v>0.65</v>
       </c>
       <c r="E242" s="67" t="inlineStr">
         <is>
@@ -25097,7 +25792,7 @@
       </c>
       <c r="D309" s="48">
         <f>O2_excess</f>
-        <v>1.58811785582e-05</v>
+        <v>1.591303582585e-05</v>
       </c>
       <c r="E309" s="67" t="inlineStr">
         <is>
@@ -25123,7 +25818,7 @@
       </c>
       <c r="D310" s="48">
         <f>O2_net_gen</f>
-        <v>4.979033518202e-05</v>
+        <v>4.987344109764e-05</v>
       </c>
       <c r="E310" s="67" t="inlineStr">
         <is>
@@ -25149,7 +25844,7 @@
       </c>
       <c r="D311" s="142">
         <f>Electrochemistry!$D$21</f>
-        <v>0.0001017274698715</v>
+        <v>0.0001018812158154</v>
       </c>
       <c r="E311" s="135" t="inlineStr">
         <is>
@@ -25175,7 +25870,7 @@
       </c>
       <c r="D312" s="142">
         <f>Biology!$D$13</f>
-        <v>0.0001017274698715</v>
+        <v>0.0001018812158154</v>
       </c>
       <c r="E312" s="135" t="inlineStr">
         <is>
@@ -25227,7 +25922,7 @@
       </c>
       <c r="D314" s="48">
         <f>MAX(0,rH2_gen-H2_HOR_mt)</f>
-        <v>0.0001017274698715</v>
+        <v>0.0001018812158154</v>
       </c>
       <c r="E314" s="67" t="inlineStr">
         <is>
@@ -25253,7 +25948,7 @@
       </c>
       <c r="D315" s="48">
         <f>CO2_cons</f>
-        <v>1.695457831191e-05</v>
+        <v>1.698020263589e-05</v>
       </c>
       <c r="E315" s="67" t="inlineStr">
         <is>
@@ -25304,7 +25999,7 @@
       </c>
       <c r="D317" s="48">
         <f>IF(O2_sizing_phase=phase_name_1,O2_src_g,IF(O2_sizing_phase=phase_name_2,O2_src_l,NA()))</f>
-        <v>1.58811785582e-05</v>
+        <v>1.591303582585e-05</v>
       </c>
       <c r="E317" s="67" t="inlineStr">
         <is>
@@ -25356,7 +26051,7 @@
       </c>
       <c r="D319" s="48">
         <f>IF(O2_sizing_phase=phase_name_1,CO2_fix_g,IF(O2_sizing_phase=phase_name_2,CO2_fix_l,NA()))</f>
-        <v>1.695457831191e-05</v>
+        <v>1.698020263589e-05</v>
       </c>
       <c r="E319" s="67" t="inlineStr">
         <is>
@@ -25381,7 +26076,7 @@
         </is>
       </c>
       <c r="D320" s="48">
-        <f>nCO2_rate*spg_dur_opt/n_hs_gas</f>
+        <f>nCO2_rate*spg_dur_eq_opt/n_hs_gas</f>
         <v>1.0</v>
       </c>
       <c r="E320" s="67" t="inlineStr">
@@ -25512,7 +26207,7 @@
       </c>
       <c r="D325" s="48">
         <f>t_off_CO2/3600</f>
-        <v>0.150215644745</v>
+        <v>0.149029758432</v>
       </c>
       <c r="E325" s="67" t="inlineStr">
         <is>
@@ -25564,7 +26259,7 @@
       </c>
       <c r="D327" s="48">
         <f>O2_src_g+y_O2_air*F_vent_ex</f>
-        <v>2.358797965326e-05</v>
+        <v>2.361983692092e-05</v>
       </c>
       <c r="E327" s="67" t="inlineStr">
         <is>
@@ -25590,7 +26285,7 @@
       </c>
       <c r="D328" s="48">
         <f>CO2_supply+O2_src_g+H2_src_g-CO2_fix_g</f>
-        <v>0.0007087450307148</v>
+        <v>0.0007145383986222</v>
       </c>
       <c r="E328" s="67" t="inlineStr">
         <is>
@@ -25616,7 +26311,7 @@
       </c>
       <c r="D329" s="48">
         <f>IF(F_vent_ex+F_hs_net_g&gt;0,S_O2_g/(F_vent_ex+F_hs_net_g),NA())</f>
-        <v>0.031639138319</v>
+        <v>0.031437574558</v>
       </c>
       <c r="E329" s="67" t="inlineStr">
         <is>
@@ -25694,7 +26389,7 @@
       </c>
       <c r="D332" s="48">
         <f>F_gap_g*t_gap_h/n_hs_gas</f>
-        <v>0.051750347445</v>
+        <v>0.05134180126</v>
       </c>
       <c r="E332" s="67" t="inlineStr">
         <is>
@@ -25720,7 +26415,7 @@
       </c>
       <c r="D333" s="48">
         <f>IF(x_hs_g&gt;0,(1-EXP(-x_hs_g))/x_hs_g,1)</f>
-        <v>0.974565460589</v>
+        <v>0.974762847875</v>
       </c>
       <c r="E333" s="67" t="inlineStr">
         <is>
@@ -25746,7 +26441,7 @@
       </c>
       <c r="D334" s="48">
         <f>IF(x_hs_g&gt;0,(x_hs_g-1+EXP(-x_hs_g))/x_hs_g^2,1/2)</f>
-        <v>0.491485384479</v>
+        <v>0.491551747427</v>
       </c>
       <c r="E334" s="67" t="inlineStr">
         <is>
@@ -25772,7 +26467,7 @@
       </c>
       <c r="D335" s="48">
         <f>S_O2_g*t_gap_h/n_hs_gas</f>
-        <v>0.03318286585</v>
+        <v>0.032965363801</v>
       </c>
       <c r="E335" s="67" t="inlineStr">
         <is>
@@ -25798,7 +26493,7 @@
       </c>
       <c r="D336" s="48">
         <f>dy_O2_g*phi_hs_g/(1-flush_ret*EXP(-x_hs_g))</f>
-        <v>0.049700562217</v>
+        <v>0.049395629179</v>
       </c>
       <c r="E336" s="68" t="inlineStr">
         <is>
@@ -25824,7 +26519,7 @@
       </c>
       <c r="D337" s="48">
         <f>y_O2_end_g*flush_ret</f>
-        <v>0.018283815054</v>
+        <v>0.018171636459</v>
       </c>
       <c r="E337" s="68" t="inlineStr">
         <is>
@@ -25850,7 +26545,7 @@
       </c>
       <c r="D338" s="48">
         <f>y_O2_post_g*phi_hs_g+dy_O2_g*psi_hs_g</f>
-        <v>0.03412766822</v>
+        <v>0.033917218286</v>
       </c>
       <c r="E338" s="68" t="inlineStr">
         <is>
@@ -25876,7 +26571,7 @@
       </c>
       <c r="D339" s="48">
         <f>O2_src_g/(kLa_surf_used*3600*V_L_m3)</f>
-        <v>0.040846064617</v>
+        <v>0.040928000854</v>
       </c>
       <c r="E339" s="67" t="inlineStr">
         <is>
@@ -25901,8 +26596,8 @@
         </is>
       </c>
       <c r="D340" s="48">
-        <f>DO_surf_excess_g+H_O2_T*P_atm*y_O2_mf_g</f>
-        <v>0.079316092899</v>
+        <f>DO_surf_excess_g+H_O2_T*P_dry*y_O2_mf_g</f>
+        <v>0.076673031404</v>
       </c>
       <c r="E340" s="67" t="inlineStr">
         <is>
@@ -25927,8 +26622,8 @@
         </is>
       </c>
       <c r="D341" s="48">
-        <f>DO_surf_excess_g+H_O2_T*P_atm*y_O2_avg_g</f>
-        <v>0.082341896405</v>
+        <f>DO_surf_excess_g+H_O2_T*P_dry*y_O2_avg_g</f>
+        <v>0.079492426413</v>
       </c>
       <c r="E341" s="68" t="inlineStr">
         <is>
@@ -25953,8 +26648,8 @@
         </is>
       </c>
       <c r="D342" s="48">
-        <f>DO_surf_excess_g+H_O2_T*P_atm*MAX(y_O2_avg_g,y_O2_end_g-(S_O2_g-F_gap_g*y_O2_end_g)/n_hs_gas*tau_L_h)</f>
-        <v>0.091717883745</v>
+        <f>DO_surf_excess_g+H_O2_T*P_dry*MAX(y_O2_avg_g,y_O2_end_g-(S_O2_g-F_gap_g*y_O2_end_g)/n_hs_gas*tau_L_h)</f>
+        <v>0.088135004652</v>
       </c>
       <c r="E342" s="68" t="inlineStr">
         <is>
@@ -25980,7 +26675,7 @@
       </c>
       <c r="D343" s="48">
         <f>DO_avg_g*M_O2</f>
-        <v>2.634776001183</v>
+        <v>2.543598660379</v>
       </c>
       <c r="E343" s="68" t="inlineStr">
         <is>
@@ -26006,7 +26701,7 @@
       </c>
       <c r="D344" s="48">
         <f>DO_peak_g*M_O2</f>
-        <v>2.934788844069</v>
+        <v>2.82014387887</v>
       </c>
       <c r="E344" s="68" t="inlineStr">
         <is>
@@ -26032,7 +26727,7 @@
       </c>
       <c r="D345" s="48">
         <f>O2_src_g/(DO_target*3600*V_L_m3)</f>
-        <v>0.003566106821</v>
+        <v>0.003701930458</v>
       </c>
       <c r="E345" s="67" t="inlineStr">
         <is>
@@ -26058,7 +26753,7 @@
       </c>
       <c r="D346" s="48">
         <f>kLa_surf_used/kLa_surf_req_g</f>
-        <v>2.019037572031</v>
+        <v>1.944959187716</v>
       </c>
       <c r="E346" s="67" t="inlineStr">
         <is>
@@ -26084,7 +26779,7 @@
       </c>
       <c r="D347" s="28" t="str">
         <f>IF(kLa_margin_g&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)")</f>
-        <v>reachable – kLa margin 2.02×</v>
+        <v>reachable – kLa margin 1.94×</v>
       </c>
       <c r="E347" s="67" t="inlineStr">
         <is>
@@ -26110,7 +26805,7 @@
       </c>
       <c r="D348" s="28" t="str">
         <f>IF(DO_peak_g&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
-        <v>peak 2.9 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 2.8 mg/L under the 11.3 mg/L ceiling</v>
       </c>
       <c r="E348" s="67" t="inlineStr">
         <is>
@@ -26136,7 +26831,7 @@
       </c>
       <c r="D349" s="48">
         <f>O2_src_l+y_O2_air*F_vent_ex</f>
-        <v>5.749713627708e-05</v>
+        <v>5.75802421927e-05</v>
       </c>
       <c r="E349" s="67" t="inlineStr">
         <is>
@@ -26162,7 +26857,7 @@
       </c>
       <c r="D350" s="48">
         <f>CO2_supply+O2_src_l+H2_src_l-CO2_fix_l</f>
-        <v>0.000861336235522</v>
+        <v>0.0008673602223452</v>
       </c>
       <c r="E350" s="67" t="inlineStr">
         <is>
@@ -26188,7 +26883,7 @@
       </c>
       <c r="D351" s="48">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,S_O2_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.064019231488</v>
+        <v>0.063684612076</v>
       </c>
       <c r="E351" s="67" t="inlineStr">
         <is>
@@ -26214,7 +26909,7 @@
       </c>
       <c r="D352" s="48">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,H2_src_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.113266761861</v>
+        <v>0.112682153807</v>
       </c>
       <c r="E352" s="67" t="inlineStr">
         <is>
@@ -26240,7 +26935,7 @@
       </c>
       <c r="D353" s="48">
         <f>F_vent_ex+MAX(0,O2_src_l+H2_src_l-CO2_fix_l)</f>
-        <v>0.0001883044451254</v>
+        <v>0.0001885412969849</v>
       </c>
       <c r="E353" s="67" t="inlineStr">
         <is>
@@ -26266,7 +26961,7 @@
       </c>
       <c r="D354" s="48">
         <f>F_gap_l*t_gap_h/n_hs_gas</f>
-        <v>0.264901073915</v>
+        <v>0.263140362374</v>
       </c>
       <c r="E354" s="67" t="inlineStr">
         <is>
@@ -26292,7 +26987,7 @@
       </c>
       <c r="D355" s="48">
         <f>IF(x_hs_l&gt;0,(1-EXP(-x_hs_l))/x_hs_l,1)</f>
-        <v>0.878509649469</v>
+        <v>0.879249368918</v>
       </c>
       <c r="E355" s="67" t="inlineStr">
         <is>
@@ -26318,7 +27013,7 @@
       </c>
       <c r="D356" s="48">
         <f>IF(x_hs_l&gt;0,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2)</f>
-        <v>0.458625360539</v>
+        <v>0.458882970262</v>
       </c>
       <c r="E356" s="67" t="inlineStr">
         <is>
@@ -26344,7 +27039,7 @@
       </c>
       <c r="D357" s="48">
         <f>S_O2_l*t_gap_h/n_hs_gas</f>
-        <v>0.080885255453</v>
+        <v>0.08036268997</v>
       </c>
       <c r="E357" s="67" t="inlineStr">
         <is>
@@ -26370,7 +27065,7 @@
       </c>
       <c r="D358" s="48">
         <f>dy_O2_l*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.09900408513</v>
+        <v>0.098515562811</v>
       </c>
       <c r="E358" s="68" t="inlineStr">
         <is>
@@ -26396,7 +27091,7 @@
       </c>
       <c r="D359" s="48">
         <f>y_O2_end_l*flush_ret</f>
-        <v>0.036421567511</v>
+        <v>0.036241850194</v>
       </c>
       <c r="E359" s="68" t="inlineStr">
         <is>
@@ -26422,7 +27117,7 @@
       </c>
       <c r="D360" s="48">
         <f>y_O2_post_l*phi_hs_l+dy_O2_l*psi_hs_l</f>
-        <v>0.069092727952</v>
+        <v>0.068742693783</v>
       </c>
       <c r="E360" s="68" t="inlineStr">
         <is>
@@ -26447,8 +27142,8 @@
         </is>
       </c>
       <c r="D361" s="48">
-        <f>DO_surf_excess_lag+H_O2_T*P_atm*y_O2_mf_l</f>
-        <v>0.205900701595</v>
+        <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_mf_l</f>
+        <v>0.200683898308</v>
       </c>
       <c r="E361" s="67" t="inlineStr">
         <is>
@@ -26473,8 +27168,8 @@
         </is>
       </c>
       <c r="D362" s="48">
-        <f>DO_surf_excess_lag+H_O2_T*P_atm*y_O2_avg_l</f>
-        <v>0.212069565945</v>
+        <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_avg_l</f>
+        <v>0.206435018988</v>
       </c>
       <c r="E362" s="68" t="inlineStr">
         <is>
@@ -26499,8 +27194,8 @@
         </is>
       </c>
       <c r="D363" s="48">
-        <f>DO_surf_excess_lag+H_O2_T*P_atm*MAX(y_O2_avg_l,y_O2_end_l-(S_O2_l-F_gap_l*y_O2_end_l)/n_hs_gas*tau_L_h)</f>
-        <v>0.231369990147</v>
+        <f>DO_surf_excess_lag+H_O2_T*P_dry*MAX(y_O2_avg_l,y_O2_end_l-(S_O2_l-F_gap_l*y_O2_end_l)/n_hs_gas*tau_L_h)</f>
+        <v>0.224263483321</v>
       </c>
       <c r="E363" s="68" t="inlineStr">
         <is>
@@ -26526,7 +27221,7 @@
       </c>
       <c r="D364" s="48">
         <f>DO_avg_l*M_O2</f>
-        <v>6.785801971106</v>
+        <v>6.605507737565</v>
       </c>
       <c r="E364" s="68" t="inlineStr">
         <is>
@@ -26552,7 +27247,7 @@
       </c>
       <c r="D365" s="48">
         <f>DO_peak_l*M_O2</f>
-        <v>7.403376944733</v>
+        <v>7.175982939307</v>
       </c>
       <c r="E365" s="68" t="inlineStr">
         <is>
@@ -26578,7 +27273,7 @@
       </c>
       <c r="D366" s="48">
         <f>O2_src_l/(DO_target*3600*V_L_m3)</f>
-        <v>0.011180382694</v>
+        <v>0.01160231226</v>
       </c>
       <c r="E366" s="67" t="inlineStr">
         <is>
@@ -26604,7 +27299,7 @@
       </c>
       <c r="D367" s="48">
         <f>kLa_surf_used/kLa_surf_req_l</f>
-        <v>0.643994383246</v>
+        <v>0.620574890218</v>
       </c>
       <c r="E367" s="67" t="inlineStr">
         <is>
@@ -26630,7 +27325,7 @@
       </c>
       <c r="D368" s="28" t="str">
         <f>IF(kLa_margin_l&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)")</f>
-        <v>UNREACHABLE at this surface kLa – margin 0.64× (raise kL_surf, lower the current, or accept a higher DO)</v>
+        <v>UNREACHABLE at this surface kLa – margin 0.62× (raise kL_surf, lower the current, or accept a higher DO)</v>
       </c>
       <c r="E368" s="67" t="inlineStr">
         <is>
@@ -26656,7 +27351,7 @@
       </c>
       <c r="D369" s="28" t="str">
         <f>IF(DO_peak_l&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
-        <v>peak 7.4 mg/L under the 11.7 mg/L ceiling</v>
+        <v>peak 7.2 mg/L under the 11.3 mg/L ceiling</v>
       </c>
       <c r="E369" s="67" t="inlineStr">
         <is>
@@ -26708,7 +27403,7 @@
       </c>
       <c r="D372" s="48">
         <f>IF(O2_sizing_phase=phase_name_1,DO_avg_g,IF(O2_sizing_phase=phase_name_2,DO_avg_l,NA()))</f>
-        <v>0.082341896405</v>
+        <v>0.079492426413</v>
       </c>
       <c r="E372" s="68" t="inlineStr">
         <is>
@@ -26734,7 +27429,7 @@
       </c>
       <c r="D373" s="48">
         <f>IF(O2_sizing_phase=phase_name_1,DO_peak_g,IF(O2_sizing_phase=phase_name_2,DO_peak_l,NA()))</f>
-        <v>0.091717883745</v>
+        <v>0.088135004652</v>
       </c>
       <c r="E373" s="68" t="inlineStr">
         <is>
@@ -26760,7 +27455,7 @@
       </c>
       <c r="D374" s="28" t="str">
         <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_impair)),IF(DO_peak_sched*M_O2&lt;DO_impair,"peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L under impairment","PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER IMPAIRMENT")&amp;IF(DO_avg_sched*M_O2&lt;=DO_opt,"; mean "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L at/under optimum","; MEAN "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L ABOVE OPTIMUM"),IF(DO_peak_sched&lt;=O2_ceil_C,"organism band unknown – peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L is under the inhibition ceiling","organism band unknown – PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER THE INHIBITION CEILING"))</f>
-        <v>organism band unknown – peak 2.9 mg/L is under the inhibition ceiling</v>
+        <v>organism band unknown – peak 2.8 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E374" s="67" t="inlineStr">
         <is>
@@ -26785,8 +27480,8 @@
         </is>
       </c>
       <c r="D375" s="48">
-        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*t_gap_h/(V_L_m3+Vg_CO2)</f>
-        <v>-0.139866823543</v>
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*t_gap_h/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.123258003994</v>
       </c>
       <c r="E375" s="67" t="inlineStr">
         <is>
@@ -26812,7 +27507,7 @@
       </c>
       <c r="D376" s="48">
         <f>k_eff_CO2*t_off_CO2</f>
-        <v>0.009083630066</v>
+        <v>0.007993102711</v>
       </c>
       <c r="E376" s="67" t="inlineStr">
         <is>
@@ -26838,7 +27533,7 @@
       </c>
       <c r="D377" s="48">
         <f>IF(pool_x&gt;0,(1-EXP(-pool_x))/pool_x,1)</f>
-        <v>0.99547190585</v>
+        <v>0.996014075682</v>
       </c>
       <c r="E377" s="67" t="inlineStr">
         <is>
@@ -26864,7 +27559,7 @@
       </c>
       <c r="D378" s="48">
         <f>IF(pool_x&gt;0,(pool_x-1+EXP(-pool_x))/pool_x^2,1/2)</f>
-        <v>0.498489493433</v>
+        <v>0.498670474036</v>
       </c>
       <c r="E378" s="67" t="inlineStr">
         <is>
@@ -26890,7 +27585,7 @@
       </c>
       <c r="D379" s="48">
         <f>pool_D_raw*pool_phi</f>
-        <v>-0.139233493397</v>
+        <v>-0.122766706919</v>
       </c>
       <c r="E379" s="67" t="inlineStr">
         <is>
@@ -26916,7 +27611,7 @@
       </c>
       <c r="D380" s="48">
         <f>pool_a+(1-pool_a)*flush_ret</f>
-        <v>0.889045202649</v>
+        <v>0.901588872448</v>
       </c>
       <c r="E380" s="68" t="inlineStr">
         <is>
@@ -26942,7 +27637,7 @@
       </c>
       <c r="D381" s="48">
         <f>IF(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_atm*F_vent_ex)/(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
-        <v>0.929374836165</v>
+        <v>0.929877016008</v>
       </c>
       <c r="E381" s="67" t="inlineStr">
         <is>
@@ -26968,7 +27663,7 @@
       </c>
       <c r="D382" s="48">
         <f>y_CO2_mf*C_sat_CO2</f>
-        <v>31.075738740549</v>
+        <v>30.122321782312</v>
       </c>
       <c r="E382" s="67" t="inlineStr">
         <is>
@@ -27105,7 +27800,7 @@
       </c>
       <c r="D388" s="48">
         <f>H2_src_l*t_gap_h/n_hs_gas*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.175164116673</v>
+        <v>0.174311272995</v>
       </c>
       <c r="E388" s="68" t="inlineStr">
         <is>
@@ -27130,8 +27825,8 @@
         </is>
       </c>
       <c r="D389" s="48">
-        <f>(pool_a*(C_cycle_peak-C_cycle_start)*(V_L_m3+Vg_CO2)+MAX(0,CO2_fix_sched-O2_src_sched-H2_src_sched)*t_gap_h)/n_hs_gas</f>
-        <v>0.059351496276</v>
+        <f>(pool_a*(C_cycle_peak-C_cycle_start)*(V_L_CO2+Vg_CO2)+MAX(0,CO2_fix_sched-O2_src_sched-H2_src_sched)*t_gap_h)/n_hs_gas</f>
+        <v>0.059032852289</v>
       </c>
       <c r="E389" s="68" t="inlineStr">
         <is>
@@ -27239,6 +27934,480 @@
       <c r="E393" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">→ Summary (override_spg_int_min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PULSE-VOLUME FIT, CARRYOVER LIMIT, CO₂ UPTAKE, DIC STORAGE AND DRY-GAS BASIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Points in the pulse-volume fit (this reactor)</t>
+        </is>
+      </c>
+      <c r="B401" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fit_n</t>
+        </is>
+      </c>
+      <c r="C401" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="D401" s="28">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$F$4:$F$201&gt;0)*('CO2 flows'!$N$4:$N$201&lt;&gt;1)*1)</f>
+        <v>34.0</v>
+      </c>
+      <c r="E401" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2 flows rows with a pulse time (F &gt; 0) for the selected reactor, less those flagged 1 in column N (the red outliers). SUMPRODUCT normal equations: no dynamic arrays, no CSE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Σ t (pulse time)</t>
+        </is>
+      </c>
+      <c r="B402" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fit_St</t>
+        </is>
+      </c>
+      <c r="C402" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D402" s="28">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$F$4:$F$201&gt;0)*('CO2 flows'!$N$4:$N$201&lt;&gt;1)*'CO2 flows'!$F$4:$F$201)</f>
+        <v>49.85</v>
+      </c>
+      <c r="E402" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Normal-equation sum over the selected rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Σ V (pulse volume)</t>
+        </is>
+      </c>
+      <c r="B403" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fit_SV</t>
+        </is>
+      </c>
+      <c r="C403" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D403" s="28">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$F$4:$F$201&gt;0)*('CO2 flows'!$N$4:$N$201&lt;&gt;1)*'CO2 flows'!$E$4:$E$201)</f>
+        <v>178.2</v>
+      </c>
+      <c r="E403" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Σ t²</t>
+        </is>
+      </c>
+      <c r="B404" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fit_Stt</t>
+        </is>
+      </c>
+      <c r="C404" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s²</t>
+        </is>
+      </c>
+      <c r="D404" s="28">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$F$4:$F$201&gt;0)*('CO2 flows'!$N$4:$N$201&lt;&gt;1)*'CO2 flows'!$F$4:$F$201^2)</f>
+        <v>304.7325</v>
+      </c>
+      <c r="E404" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Σ t·V</t>
+        </is>
+      </c>
+      <c r="B405" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fit_StV</t>
+        </is>
+      </c>
+      <c r="C405" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL·s</t>
+        </is>
+      </c>
+      <c r="D405" s="28">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$F$4:$F$201&gt;0)*('CO2 flows'!$N$4:$N$201&lt;&gt;1)*'CO2 flows'!$F$4:$F$201*'CO2 flows'!$E$4:$E$201)</f>
+        <v>1030.03</v>
+      </c>
+      <c r="E405" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minimum points for a pulse-volume fit</t>
+        </is>
+      </c>
+      <c r="B406" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fit_n_min</t>
+        </is>
+      </c>
+      <c r="C406" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="D406" s="131">
+        <v>3</v>
+      </c>
+      <c r="E406" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: fewer points (or all at one pulse length) and the fit falls back to the nominal flow with no intercept.</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fitted steady CO₂ flow (slope)</t>
+        </is>
+      </c>
+      <c r="B407" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q_CO2_fit</t>
+        </is>
+      </c>
+      <c r="C407" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
+      </c>
+      <c r="D407" s="28">
+        <f>IF(AND(fit_n&gt;=fit_n_min,fit_n*fit_Stt-fit_St^2&gt;0),(fit_n*fit_StV-fit_St*fit_SV)/(fit_n*fit_Stt-fit_St^2),Q_CO2/60)</f>
+        <v>3.318707459132</v>
+      </c>
+      <c r="E407" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Least-squares slope of pulse volume on pulse time (R2-M3). ed04: 3.319 mL/s over 34 runs, vs the 3.33 nominal. Falls back to Q_CO2/60 when there is no usable fit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed volume per pulse (solenoid opening + line decompression)</t>
+        </is>
+      </c>
+      <c r="B408" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pulse_V0</t>
+        </is>
+      </c>
+      <c r="C408" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D408" s="28">
+        <f>IF(AND(fit_n&gt;=fit_n_min,fit_n*fit_Stt-fit_St^2&gt;0),(fit_SV-Q_CO2_fit*fit_St)/fit_n,0)</f>
+        <v>0.375365681243</v>
+      </c>
+      <c r="E408" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Least-squares intercept (R2-M3): ed04 0.375 mL (0.327 if the 15 s run is dropped, 0.131 on ≤2 s runs only). Weak: captured at the inlet tube over CO₂-saturated water / NaHCO₃ (CO2 flows L7–L9), ±0.2 mL. Re-measure at the operating pulse length downstream of a sealed cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Optimal pulse as full-flow equivalent time</t>
+        </is>
+      </c>
+      <c r="B409" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_dur_eq_opt</t>
+        </is>
+      </c>
+      <c r="C409" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D409" s="28">
+        <f>(pulse_V0+Q_CO2_fit*spg_dur_opt)/(Q_CO2/60)</f>
+        <v>0.784513049825</v>
+      </c>
+      <c r="E409" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The time the steady flow Q_CO2 would take to deliver what the optimal pulse actually delivers (V₀ + Q_fit·t). Every duty-based interval (carbon, O₂ dilution, H₂ safety) converts duty to interval through this, so the intercept moves the pulse, not the dose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse in use as full-flow equivalent time</t>
+        </is>
+      </c>
+      <c r="B410" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_dur_eq</t>
+        </is>
+      </c>
+      <c r="C410" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D410" s="28">
+        <f>(pulse_V0+Q_CO2_fit*spg_dur)/(Q_CO2/60)</f>
+        <v>0.784513049825</v>
+      </c>
+      <c r="E410" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above for the schedule in use (follows any override).</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ volume per pulse (schedule in use)</t>
+        </is>
+      </c>
+      <c r="B411" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_pulse</t>
+        </is>
+      </c>
+      <c r="C411" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL</t>
+        </is>
+      </c>
+      <c r="D411" s="28">
+        <f>pulse_V0+Q_CO2_fit*spg_dur</f>
+        <v>2.612428455917</v>
+      </c>
+      <c r="E411" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V = V₀ + Q_fit·t at the pulse in use; CO2_pulse (D123) converts it to moles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measured no-carryover limits for this reactor</t>
+        </is>
+      </c>
+      <c r="B412" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">carry_n</t>
+        </is>
+      </c>
+      <c r="C412" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">count</t>
+        </is>
+      </c>
+      <c r="D412" s="28">
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$M$4:$M$201&gt;0)*1)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E412" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rows of CO2 flows column M with a value for the selected reactor (review R3 M-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max flow without carryover (lowest measured)</t>
+        </is>
+      </c>
+      <c r="B413" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q_carry_max</t>
+        </is>
+      </c>
+      <c r="C413" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
+      </c>
+      <c r="D413" s="28" t="str">
+        <f>IF(carry_n&gt;0,SUMPRODUCT(MIN(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$M$4:$M$201&gt;0)*'CO2 flows'!$M$4:$M$201+(1-('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$M$4:$M$201&gt;0))*MAX('CO2 flows'!$M$4:$M$201))),"not measured")</f>
+        <v>not measured</v>
+      </c>
+      <c r="E413" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DATA GAP until measured (CO2 flows column M). The lowest entry for the reactor is used (conservative). Key L3 says the nominal flow was set as the largest without bubbles reaching the neck; if that run is taken as the measurement, enter J4 in M4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carryover — superficial-velocity rule of thumb (secondary)</t>
+        </is>
+      </c>
+      <c r="B414" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">carry_flag_usg</t>
+        </is>
+      </c>
+      <c r="C414" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D414" s="28" t="str">
+        <f>IF(u_sg&gt;u_g_max,"RISK – "&amp;TEXT(u_sg*1000,"0.0")&amp;" mm/s superficial gas velocity over the "&amp;TEXT(u_g_max*1000,"0")&amp;" mm/s rule of thumb","OK – "&amp;TEXT(u_sg*1000,"0.0")&amp;" mm/s against the "&amp;TEXT(u_g_max*1000,"0")&amp;" mm/s rule of thumb")</f>
+        <v>OK – 6.6 mm/s against the 50 mm/s rule of thumb</v>
+      </c>
+      <c r="E414" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The former carry_flag test, kept as a secondary line: u_sg vs u_g_max (D58, provisional). It cannot bind below ~25 mL/s, which is why the primary check (D59) now uses the measured limit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) DIC capacity factor of the liquid</t>
+        </is>
+      </c>
+      <c r="B415" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC_cap_mt</t>
+        </is>
+      </c>
+      <c r="C415" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D415" s="28">
+        <f>Chemistry!$D$296</f>
+        <v>1.154598203915</v>
+      </c>
+      <c r="E415" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Chemistry!D296 (DIC_cap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid CO₂ capacity as CO₂(aq)-equivalent volume</t>
+        </is>
+      </c>
+      <c r="B416" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V_L_CO2</t>
+        </is>
+      </c>
+      <c r="C416" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m³</t>
+        </is>
+      </c>
+      <c r="D416" s="28">
+        <f>V_L_m3*DIC_cap_mt</f>
+        <v>1.731897305873e-05</v>
+      </c>
+      <c r="E416" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The liquid holds CO₂(aq) plus the bicarbonate it forms, so for the pool it counts as DIC_cap × its volume (R2-m3). Used in D193, D195, D375, D389 and D417.</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ absorbed after each pulse, per hour : carbon demand</t>
+        </is>
+      </c>
+      <c r="B417" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_uptake_ratio</t>
+        </is>
+      </c>
+      <c r="C417" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">×</t>
+        </is>
+      </c>
+      <c r="D417" s="28">
+        <f>IF(CO2_cons&gt;0,(C_cycle_peak-C_cycle_start)*V_L_CO2*pulses_h/CO2_cons,NA())</f>
+        <v>2.425083542153</v>
+      </c>
+      <c r="E417" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review R3 M-18: the CO₂ the liquid actually takes up when each pulse equilibrates (rise of the pool from trough to peak × the liquid capacity incl. bicarbonate, V_L_CO2) × pulses per hour, over fixation. Unlike D126 it ignores gas expelled unabsorbed. Not a sufficiency test: below 1 the culture also draws on headspace CO₂ between pulses (Outflow only, growth: 0.84×); carbon sufficiency is the trough margin (Biology D98).</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dry-gas pressure in the headspace</t>
+        </is>
+      </c>
+      <c r="B418" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P_dry</t>
+        </is>
+      </c>
+      <c r="C418" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pa</t>
+        </is>
+      </c>
+      <c r="D418" s="28">
+        <f>P_atm-p_sat_w</f>
+        <v>98163.2639643</v>
+      </c>
+      <c r="E418" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The headspace over the culture is saturated with water vapour, so the gases the Henry terms see share P_atm − p_sat_w (R2-m8, −3.1 % at 25 °C).</t>
         </is>
       </c>
     </row>
@@ -27422,8 +28591,16 @@
       <c r="L2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="3"/>
-      <c r="N2" s="6"/>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">max flow without carryover</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">excluded from pulse fit</t>
+        </is>
+      </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3"/>
@@ -27471,8 +28648,16 @@
       <c r="L3" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="M3" s="3"/>
-      <c r="N3" s="6"/>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/s</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 = yes</t>
+        </is>
+      </c>
       <c r="O3" s="6"/>
       <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
@@ -27723,7 +28908,11 @@
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Column M: highest steady flow at which no liquid is carried into the vial neck or vent for this reactor (measured; blank = not measured, and Mass Transfer carry_flag then reads "not measured"). If the lowest entry for the reactor is below the pulse flow, carry_flag reads RISK.</t>
+        </is>
+      </c>
       <c r="M10" s="3"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
@@ -27761,7 +28950,11 @@
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Column N: 1 = point excluded from the pulse-volume fit V = V₀ + Q·t on Mass Transfer (rows 401–408); 1 is set on the two red outliers (G36, G46). Blank = used.</t>
+        </is>
+      </c>
       <c r="M11" s="3"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
@@ -28626,7 +29819,9 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
-      <c r="N36" s="3"/>
+      <c r="N36" s="3">
+        <v>1</v>
+      </c>
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
@@ -28974,7 +30169,9 @@
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
-      <c r="N46" s="3"/>
+      <c r="N46" s="3">
+        <v>1</v>
+      </c>
       <c r="O46" s="3"/>
       <c r="P46" s="3"/>
       <c r="Q46" s="3"/>
@@ -29624,7 +30821,7 @@
       <c r="D8" s="123"/>
       <c r="E8" s="123"/>
       <c r="F8" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C8,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C8,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G8" s="122"/>
@@ -29637,7 +30834,7 @@
       <c r="D9" s="123"/>
       <c r="E9" s="123"/>
       <c r="F9" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C9,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C9,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G9" s="122"/>
@@ -29650,7 +30847,7 @@
       <c r="D10" s="123"/>
       <c r="E10" s="123"/>
       <c r="F10" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C10,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C10,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G10" s="122"/>
@@ -29663,7 +30860,7 @@
       <c r="D11" s="123"/>
       <c r="E11" s="123"/>
       <c r="F11" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C11,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C11,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G11" s="122"/>
@@ -29676,7 +30873,7 @@
       <c r="D12" s="123"/>
       <c r="E12" s="123"/>
       <c r="F12" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C12,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C12,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G12" s="122"/>
@@ -29689,7 +30886,7 @@
       <c r="D13" s="123"/>
       <c r="E13" s="123"/>
       <c r="F13" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C13,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C13,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G13" s="122"/>
@@ -29702,7 +30899,7 @@
       <c r="D14" s="123"/>
       <c r="E14" s="123"/>
       <c r="F14" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C14,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C14,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G14" s="122"/>
@@ -29715,7 +30912,7 @@
       <c r="D15" s="123"/>
       <c r="E15" s="123"/>
       <c r="F15" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C15,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C15,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G15" s="122"/>
@@ -29808,7 +31005,7 @@
         <v/>
       </c>
       <c r="J23" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C23,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C23,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K23" s="122"/>
@@ -29829,7 +31026,7 @@
         <v/>
       </c>
       <c r="J24" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C24,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C24,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K24" s="122"/>
@@ -29850,7 +31047,7 @@
         <v/>
       </c>
       <c r="J25" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C25,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C25,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K25" s="122"/>
@@ -29871,7 +31068,7 @@
         <v/>
       </c>
       <c r="J26" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C26,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C26,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K26" s="122"/>
@@ -29892,7 +31089,7 @@
         <v/>
       </c>
       <c r="J27" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C27,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C27,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K27" s="122"/>
@@ -29913,7 +31110,7 @@
         <v/>
       </c>
       <c r="J28" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C28,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C28,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K28" s="122"/>
@@ -29934,7 +31131,7 @@
         <v/>
       </c>
       <c r="J29" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C29,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C29,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K29" s="122"/>
@@ -29955,7 +31152,7 @@
         <v/>
       </c>
       <c r="J30" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C30,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C30,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="K30" s="122"/>
@@ -30106,7 +31303,7 @@
       <c r="C38" s="122"/>
       <c r="D38" s="123"/>
       <c r="E38" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C38,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C38,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F38" s="122"/>
@@ -30124,7 +31321,7 @@
       <c r="C39" s="122"/>
       <c r="D39" s="123"/>
       <c r="E39" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C39,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C39,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F39" s="122"/>
@@ -30142,7 +31339,7 @@
       <c r="C40" s="122"/>
       <c r="D40" s="123"/>
       <c r="E40" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C40,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C40,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F40" s="122"/>
@@ -30160,7 +31357,7 @@
       <c r="C41" s="122"/>
       <c r="D41" s="123"/>
       <c r="E41" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C41,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C41,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F41" s="122"/>
@@ -30178,7 +31375,7 @@
       <c r="C42" s="122"/>
       <c r="D42" s="123"/>
       <c r="E42" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C42,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C42,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F42" s="122"/>
@@ -30196,7 +31393,7 @@
       <c r="C43" s="122"/>
       <c r="D43" s="123"/>
       <c r="E43" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C43,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C43,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F43" s="122"/>
@@ -30214,7 +31411,7 @@
       <c r="C44" s="122"/>
       <c r="D44" s="123"/>
       <c r="E44" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C44,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C44,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F44" s="122"/>
@@ -30232,7 +31429,7 @@
       <c r="C45" s="122"/>
       <c r="D45" s="123"/>
       <c r="E45" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C45,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C45,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="F45" s="122"/>
@@ -30375,7 +31572,7 @@
         <v/>
       </c>
       <c r="G52" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C52,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C52,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H52" s="122"/>
@@ -30396,7 +31593,7 @@
         <v/>
       </c>
       <c r="G53" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C53,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C53,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H53" s="122"/>
@@ -30417,7 +31614,7 @@
         <v/>
       </c>
       <c r="G54" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C54,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C54,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H54" s="122"/>
@@ -30438,7 +31635,7 @@
         <v/>
       </c>
       <c r="G55" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C55,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C55,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H55" s="122"/>
@@ -30459,7 +31656,7 @@
         <v/>
       </c>
       <c r="G56" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C56,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C56,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H56" s="122"/>
@@ -30480,7 +31677,7 @@
         <v/>
       </c>
       <c r="G57" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C57,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C57,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H57" s="122"/>
@@ -30501,7 +31698,7 @@
         <v/>
       </c>
       <c r="G58" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C58,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C58,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H58" s="122"/>
@@ -30522,7 +31719,7 @@
         <v/>
       </c>
       <c r="G59" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C59,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C59,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="H59" s="122"/>
@@ -30685,7 +31882,7 @@
         <v/>
       </c>
       <c r="I66" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C66,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C66,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J66" s="122"/>
@@ -30716,7 +31913,7 @@
         <v/>
       </c>
       <c r="I67" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C67,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C67,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J67" s="122"/>
@@ -30747,7 +31944,7 @@
         <v/>
       </c>
       <c r="I68" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C68,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C68,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J68" s="122"/>
@@ -30778,7 +31975,7 @@
         <v/>
       </c>
       <c r="I69" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C69,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C69,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J69" s="122"/>
@@ -30809,7 +32006,7 @@
         <v/>
       </c>
       <c r="I70" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C70,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C70,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J70" s="122"/>
@@ -30840,7 +32037,7 @@
         <v/>
       </c>
       <c r="I71" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C71,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C71,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J71" s="122"/>
@@ -30871,7 +32068,7 @@
         <v/>
       </c>
       <c r="I72" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C72,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C72,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J72" s="122"/>
@@ -30902,7 +32099,7 @@
         <v/>
       </c>
       <c r="I73" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C73,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C73,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="J73" s="122"/>
@@ -31089,7 +32286,7 @@
         <v/>
       </c>
       <c r="F81" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C81,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C81,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G81" s="122"/>
@@ -31110,7 +32307,7 @@
         <v/>
       </c>
       <c r="F82" s="130" t="str">
-        <f>IFERROR(VLOOKUP(C82,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C82,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G82" s="122"/>
@@ -31131,7 +32328,7 @@
         <v/>
       </c>
       <c r="F83" s="130" t="str">
-        <f>IFERROR(VLOOKUP(C83,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C83,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G83" s="122"/>
@@ -31152,7 +32349,7 @@
         <v/>
       </c>
       <c r="F84" s="130" t="str">
-        <f>IFERROR(VLOOKUP(C84,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C84,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G84" s="122"/>
@@ -31173,7 +32370,7 @@
         <v/>
       </c>
       <c r="F85" s="130" t="str">
-        <f>IFERROR(VLOOKUP(C85,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C85,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G85" s="122"/>
@@ -31194,7 +32391,7 @@
         <v/>
       </c>
       <c r="F86" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C86,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C86,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G86" s="122"/>
@@ -31215,7 +32412,7 @@
         <v/>
       </c>
       <c r="F87" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C87,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C87,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G87" s="122"/>
@@ -31236,7 +32433,7 @@
         <v/>
       </c>
       <c r="F88" s="129" t="str">
-        <f>IFERROR(VLOOKUP(C88,Geometry!$A$59:$B$80,2,FALSE),"")</f>
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C88,ReactorList,0)),"")</f>
         <v/>
       </c>
       <c r="G88" s="122"/>

</xml_diff>

<commit_message>
Gas model: final-gate fixes - Calibrations-tab flow calibrates a reactor, min-pulse route, D128 both band edges, exact flammability remedy, stale notes, units; protocol update
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -144,7 +144,6 @@
     <definedName name="ec_corr_I" localSheetId="2">Electrochemistry!$D$102</definedName>
     <definedName name="ec_D_O2" localSheetId="2">Electrochemistry!$D$81</definedName>
     <definedName name="ec_DO_design" localSheetId="2">Electrochemistry!$D$85</definedName>
-    <definedName name="ec_DO_frac" localSheetId="2">Electrochemistry!$D$79</definedName>
     <definedName name="ec_E_rev" localSheetId="2">Electrochemistry!$D$106</definedName>
     <definedName name="ec_gap" localSheetId="2">Electrochemistry!$D$115</definedName>
     <definedName name="ec_I_Cl" localSheetId="2">Electrochemistry!$D$101</definedName>
@@ -606,7 +605,6 @@
     <definedName name="od_gap_min_s" localSheetId="5">'Mass Transfer'!$D$214</definedName>
     <definedName name="tip_speed_max" localSheetId="5">'Mass Transfer'!$D$216</definedName>
     <definedName name="geom_tol_mL" localSheetId="1">Geometry!$D$96</definedName>
-    <definedName name="round_split" localSheetId="0">Summary!$D$93</definedName>
     <definedName name="bp_const" localSheetId="7">Calibrations!$D$140</definedName>
     <definedName name="por_break_1" localSheetId="7">Calibrations!$D$141</definedName>
     <definedName name="por_break_2" localSheetId="7">Calibrations!$D$142</definedName>
@@ -786,7 +784,6 @@
     <definedName name="A_x" localSheetId="7">Calibrations!$D$160</definedName>
     <definedName name="R_gas" localSheetId="7">Calibrations!$D$161</definedName>
     <definedName name="F_const" localSheetId="7">Calibrations!$D$162</definedName>
-    <definedName name="p_sat_w" localSheetId="7">Calibrations!$D$163</definedName>
     <definedName name="V_charge" localSheetId="2">Electrochemistry!$D$153</definedName>
     <definedName name="organism_sel" localSheetId="2">Electrochemistry!$D$154</definedName>
     <definedName name="V_charge" localSheetId="3">Chemistry!$D$279</definedName>
@@ -836,6 +833,28 @@
     <definedName name="cf_Cl_onset" localSheetId="0">Summary!$D$142</definedName>
     <definedName name="cf_Cl_kill" localSheetId="0">Summary!$D$143</definedName>
     <definedName name="ReactorTypeList">Geometry!$B$59:$B$80</definedName>
+    <definedName name="cal_pulse_floor">Calibrations!$D$61</definedName>
+    <definedName name="pulse_floor_default" localSheetId="5">'Mass Transfer'!$D$396</definedName>
+    <definedName name="DO_lag_ref" localSheetId="2">Electrochemistry!$D$129</definedName>
+    <definedName name="DO_lag_tol" localSheetId="2">Electrochemistry!$D$130</definedName>
+    <definedName name="O2_ORR_lag" localSheetId="2">Electrochemistry!$D$131</definedName>
+    <definedName name="O2_net_lag" localSheetId="2">Electrochemistry!$D$132</definedName>
+    <definedName name="rH2_lag" localSheetId="2">Electrochemistry!$D$133</definedName>
+    <definedName name="DO_lag_ref_chk" localSheetId="2">Electrochemistry!$D$134</definedName>
+    <definedName name="O2_net_lag_mt" localSheetId="5">'Mass Transfer'!$D$394</definedName>
+    <definedName name="rH2_lag_mt" localSheetId="5">'Mass Transfer'!$D$395</definedName>
+    <definedName name="O2_src_l_b" localSheetId="4">Biology!$D$115</definedName>
+    <definedName name="F_gap_l_b" localSheetId="4">Biology!$D$116</definedName>
+    <definedName name="n_hs_gas_b" localSheetId="4">Biology!$D$117</definedName>
+    <definedName name="flush_ret_opt_b" localSheetId="4">Biology!$D$118</definedName>
+    <definedName name="y_O2_end_b" localSheetId="4">Biology!$D$119</definedName>
+    <definedName name="spg_dur_opt_b" localSheetId="4">Biology!$D$89</definedName>
+    <definedName name="t_gap_H2_LFL" localSheetId="4">Biology!$D$90</definedName>
+    <definedName name="t_gap_O2_LOC" localSheetId="4">Biology!$D$91</definedName>
+    <definedName name="spg_int_H2safe_saw" localSheetId="4">Biology!$D$92</definedName>
+    <definedName name="pw_A" localSheetId="7">Calibrations!$D$149</definedName>
+    <definedName name="pw_B" localSheetId="7">Calibrations!$D$150</definedName>
+    <definedName name="pw_C" localSheetId="7">Calibrations!$D$151</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -8395,7 +8414,7 @@
         <v>13</v>
       </c>
       <c r="D13" s="90">
-        <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$90)</f>
+        <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)",'Mass Transfer'!$D$90)</f>
         <v>0.674076519917</v>
       </c>
       <c r="E13" s="23" t="str">
@@ -8446,7 +8465,7 @@
         <v>67</v>
       </c>
       <c r="D15" s="90">
-        <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (see CO2 flows)",'Mass Transfer'!$D$91)</f>
+        <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)",'Mass Transfer'!$D$91)</f>
         <v>8.95302011459</v>
       </c>
       <c r="E15" s="23" t="str">
@@ -8479,10 +8498,9 @@
         <v>9.0</v>
       </c>
       <c r="E16" s="92"/>
-      <c r="F16" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Interval to type in: the as-run pulse converted to delivered CO₂ (V₀ + Q·t, Mass Transfer D407–D408) at the optimised full-flow-equivalent duty (D93), rounded to whole minutes, so rounding does not shift the CO₂ dose (row 95). An override in G15 wins.</t>
-        </is>
+      <c r="F16" s="21" t="str">
+        <f>"Interval to type in: the as-run pulse converted to delivered CO₂ (V₀ + Q·t, Mass Transfer D407–D408) at the optimised full-flow-equivalent duty (D93), rounded to whole minutes; "&amp;IF(ISNUMBER(D95),"rounding moves the CO₂ dose by "&amp;TEXT(D95-1,"+0.0%;-0.0%")&amp;" (row 95)","row 95 shows how far rounding moves the CO₂ dose")&amp;". An override in G15 wins."</f>
+        <v>Interval to type in: the as-run pulse converted to delivered CO₂ (V₀ + Q·t, Mass Transfer D407–D408) at the optimised full-flow-equivalent duty (D93), rounded to whole minutes; rounding moves the CO₂ dose by -3.6% (row 95). An override in G15 wins.</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -8545,14 +8563,16 @@
       <c r="C20" s="20"/>
       <c r="D20" s="90" t="str">
         <f>'Mass Transfer'!$D$120</f>
-        <v>calibrated: ed04</v>
+        <v>calibrated: ed04 (flow from CO2 flows)</v>
       </c>
       <c r="E20" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D120","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F20" s="21" t="s">
-        <v>73</v>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Red = no CO₂-flow calibration for this reactor (neither an included run in the Calibrations tab CO₂ flow section nor a CO2 flows row); results read 'calibrate first' (flow-calibration.md). Green names the source in use.</t>
+        </is>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -8643,7 +8663,7 @@
       <c r="C24" s="20"/>
       <c r="D24" s="95" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 17% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 17% before each pulse; O₂ 6% mean, 9% before each pulse – until uptake starts, sparge every ≤2.5 min or sweep ≥0.9 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="23" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -8651,7 +8671,7 @@
       </c>
       <c r="F24" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lag-phase headspace (electrolysis on, no H₂ uptake) against the H₂ flammability limit and the O₂ limiting concentration; the text names the remedy.</t>
+          <t xml:space="preserve">Lag-phase headspace (electrolysis on, no H₂ uptake) at its worst point, just before each pulse, against the H₂ flammability limit and the O₂ limiting concentration; the text names the remedy (Biology D92).</t>
         </is>
       </c>
     </row>
@@ -8712,15 +8732,17 @@
       </c>
       <c r="C27" s="20"/>
       <c r="D27" s="90" t="str">
-        <f>IFERROR('Mass Transfer'!$D$130,"calibrate this reactor first (see CO2 flows)")</f>
+        <f>IFERROR('Mass Transfer'!$D$130,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)")</f>
         <v>OK</v>
       </c>
       <c r="E27" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D130","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F27" s="21" t="s">
-        <v>87</v>
+      <c r="F27" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The optimal pulse must exceed the shortest reliable sparge (Calibrations tab CO₂-flow Min pulse, else CO2 flows column I, else the default on Mass Transfer D396).</t>
+        </is>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -8734,7 +8756,7 @@
       </c>
       <c r="C28" s="20"/>
       <c r="D28" s="90" t="str">
-        <f>IFERROR('Mass Transfer'!$D$95,"calibrate this reactor first (see CO2 flows)")</f>
+        <f>IFERROR('Mass Transfer'!$D$95,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)")</f>
         <v>OK</v>
       </c>
       <c r="E28" s="23" t="str">
@@ -9406,8 +9428,10 @@
         <v>vial-geometry.md →</v>
       </c>
       <c r="E67" s="103"/>
-      <c r="F67" s="21" t="s">
-        <v>1019</v>
+      <c r="F67" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sets the headspace volume: the pulse moves slightly more than 1:1 with it (one headspace volume per pulse, less the fixed V₀; Mass Transfer D90) and the interval through the flush; also the liquid charge. Water-fill.</t>
+        </is>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
@@ -9446,8 +9470,9 @@
         <v>knallgas-stoichiometry.md →</v>
       </c>
       <c r="E69" s="103"/>
-      <c r="F69" s="21" t="s">
-        <v>1026</v>
+      <c r="F69" s="21" t="str">
+        <f>IFERROR("Sets the O₂ surplus and the carbon demand: each 1 % on the O₂:H₂ uptake ratio moves the surplus "&amp;TEXT(Biology!$D$14/Biology!$D$16,"0.0")&amp;" % (Biology E16); needs a growing culture.","Sets the O₂ surplus and the carbon demand; needs a growing culture.")</f>
+        <v>Sets the O₂ surplus and the carbon demand: each 1 % on the O₂:H₂ uptake ratio moves the surplus 2.1 % (Biology E16); needs a growing culture.</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
@@ -9503,8 +9528,9 @@
         <v>flow-calibration.md →</v>
       </c>
       <c r="E72" s="103"/>
-      <c r="F72" s="21" t="s">
-        <v>1037</v>
+      <c r="F72" s="21" t="str">
+        <f>"Sets the solenoid floor (pulse_floor, now "&amp;TEXT('Mass Transfer'!$D$99,"0.00")&amp;" s), which binds only when it exceeds the optimal pulse ("&amp;IF(ISNUMBER(D13),TEXT(D13,"0.00")&amp;" s","not yet computed")&amp;"): "&amp;IF(AND(ISNUMBER(D13),'Mass Transfer'!$D$99&gt;=D13),"it does now, so the pulse IS the floor","it does not now, so it matters only for a smaller headspace or a faster flow")&amp;". Trivial to characterise on the bench (flow-calibration.md)."</f>
+        <v>Sets the solenoid floor (pulse_floor, now 0.25 s), which binds only when it exceeds the optimal pulse (0.67 s): it does not now, so it matters only for a smaller headspace or a faster flow. Trivial to characterise on the bench (flow-calibration.md).</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
@@ -9579,8 +9605,10 @@
         <v>README.md →</v>
       </c>
       <c r="E76" s="103"/>
-      <c r="F76" s="21" t="s">
-        <v>1053</v>
+      <c r="F76" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enters every Henry solubility and gas-volume conversion through P_atm (blank = 101 325 Pa), including the O₂ ceiling the DO target is a fraction of; small near sea level, larger at altitude.</t>
+        </is>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
@@ -9757,7 +9785,7 @@
       </c>
       <c r="D85" s="22" t="str">
         <f>Electrochemistry!$D$99</f>
-        <v>watch — steady growth is clear (0.053 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.053 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min before biomass can scavenge it</v>
       </c>
       <c r="E85" s="23" t="str">
         <f>HYPERLINK("#Electrochemistry!D99","→ Electrochemistry")</f>
@@ -9878,12 +9906,14 @@
           <t xml:space="preserve">res_kLa_req</t>
         </is>
       </c>
-      <c r="C90" s="19" t="s">
-        <v>639</v>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/h</t>
+        </is>
       </c>
       <c r="D90" s="22">
-        <f>'Mass Transfer'!$D$186</f>
-        <v>0.003701930458</v>
+        <f>'Mass Transfer'!$D$186*3600</f>
+        <v>13.32694964987</v>
       </c>
       <c r="E90" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D186","→ Mass Transfer")</f>
@@ -9891,41 +9921,24 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Below this, no sparge interval holds the target dissolved O₂ on the sizing phase. Both phases and their margins: rows 120–123.</t>
+          <t xml:space="preserve">Below this, no sparge interval holds the target dissolved O₂ on the sizing phase. Per hour, the unit you measure in and the Calibrations tab takes (D46). Both phases and their margins: rows 120–123.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">DISPLAY SETTINGS</t>
+          <t xml:space="preserve">AS-RUN SCHEDULE CHECK</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rounding split</t>
-        </is>
-      </c>
-      <c r="B93" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">round_split</t>
-        </is>
-      </c>
-      <c r="C93" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">s or min</t>
-        </is>
-      </c>
-      <c r="D93" s="131">
-        <v>0.5</v>
-      </c>
-      <c r="E93" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Former display rule for rows 14 and 16 (whole units above this value, else two significant figures); superseded by the pulse-resolution rounding (Mass Transfer D241) and no longer referenced.</t>
-        </is>
-      </c>
+      <c r="A93" s="20"/>
+      <c r="B93" s="18"/>
+      <c r="C93" s="20"/>
+      <c r="D93" s="131"/>
+      <c r="E93" s="87"/>
+      <c r="F93"/>
     </row>
     <row r="95">
       <c r="A95" s="89" t="inlineStr">
@@ -9939,7 +9952,7 @@
         </is>
       </c>
       <c r="D95" s="95">
-        <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),('Mass Transfer'!$D$408+'Mass Transfer'!$D$407*D14)/('Mass Transfer'!$D$102/60)/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (see CO2 flows)")</f>
+        <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),('Mass Transfer'!$D$408+'Mass Transfer'!$D$407*D14)/('Mass Transfer'!$D$102/60)/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)")</f>
         <v>0.964353979896</v>
       </c>
       <c r="E95" s="23" t="str">
@@ -10111,7 +10124,7 @@
       </c>
       <c r="D116" s="90">
         <f>'Mass Transfer'!$D$364</f>
-        <v>6.605507737565</v>
+        <v>6.213538763708</v>
       </c>
       <c r="E116" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
@@ -10136,7 +10149,7 @@
       </c>
       <c r="D117" s="90">
         <f>'Mass Transfer'!$D$365</f>
-        <v>7.175982939307</v>
+        <v>6.756400324589</v>
       </c>
       <c r="E117" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D365","→ Mass Transfer")</f>
@@ -10176,7 +10189,7 @@
       </c>
       <c r="D119" s="90" t="str">
         <f>'Mass Transfer'!$D$369</f>
-        <v>peak 7.2 mg/L under the 11.3 mg/L ceiling</v>
+        <v>peak 6.8 mg/L under the 11.3 mg/L ceiling</v>
       </c>
       <c r="E119" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D369","→ Mass Transfer")</f>
@@ -10216,7 +10229,7 @@
       </c>
       <c r="D121" s="90" t="str">
         <f>'Mass Transfer'!$D$368</f>
-        <v>UNREACHABLE at this surface kLa – margin 0.62× (raise kL_surf, lower the current, or accept a higher DO)</v>
+        <v>UNREACHABLE at this surface kLa – margin 0.66× (raise kL_surf, lower the current, or accept a higher DO)</v>
       </c>
       <c r="E121" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D368","→ Mass Transfer")</f>
@@ -10224,7 +10237,7 @@
       </c>
       <c r="F121" s="21" t="str">
         <f>"Same on the lag source. Currently "&amp;TEXT('Mass Transfer'!$D$367,"0.00")&amp;"×: "&amp;IF('Mass Transfer'!$D$367&lt;1,"the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).","the target can be held during lag at the kLa in use.")</f>
-        <v>Same on the lag source. Currently 0.62×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
+        <v>Same on the lag source. Currently 0.66×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
       </c>
     </row>
     <row r="122">
@@ -10235,12 +10248,12 @@
       </c>
       <c r="C122" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1/s</t>
+          <t xml:space="preserve">1/h</t>
         </is>
       </c>
       <c r="D122" s="90">
-        <f>'Mass Transfer'!$D$345</f>
-        <v>0.003701930458</v>
+        <f>'Mass Transfer'!$D$345*3600</f>
+        <v>13.32694964987</v>
       </c>
       <c r="E122" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D345","→ Mass Transfer")</f>
@@ -10248,7 +10261,7 @@
       </c>
       <c r="F122" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compare with the estimate in use (Mass Transfer D98).</t>
+          <t xml:space="preserve">Per hour: compare with your measured kLa (Calibrations D46, 1/h); the estimate in use is Mass Transfer D98 (1/s × 3600).</t>
         </is>
       </c>
     </row>
@@ -10260,12 +10273,12 @@
       </c>
       <c r="C123" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">1/s</t>
+          <t xml:space="preserve">1/h</t>
         </is>
       </c>
       <c r="D123" s="90">
-        <f>'Mass Transfer'!$D$366</f>
-        <v>0.01160231226</v>
+        <f>'Mass Transfer'!$D$366*3600</f>
+        <v>38.99066377049</v>
       </c>
       <c r="E123" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D366","→ Mass Transfer")</f>
@@ -10273,7 +10286,7 @@
       </c>
       <c r="F123" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compare with the estimate in use (Mass Transfer D98).</t>
+          <t xml:space="preserve">Per hour: compare with your measured kLa (Calibrations D46, 1/h); the estimate in use is Mass Transfer D98 (1/s × 3600).</t>
         </is>
       </c>
     </row>
@@ -10315,7 +10328,7 @@
       </c>
       <c r="D125" s="90">
         <f>'Mass Transfer'!$D$351</f>
-        <v>0.063684612076</v>
+        <v>0.060650407932</v>
       </c>
       <c r="E125" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D351","→ Mass Transfer")</f>
@@ -10340,7 +10353,7 @@
       </c>
       <c r="D126" s="90">
         <f>'Mass Transfer'!$D$352</f>
-        <v>0.112682153807</v>
+        <v>0.107014631173</v>
       </c>
       <c r="E126" s="23" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D352","→ Mass Transfer")</f>
@@ -10384,7 +10397,7 @@
         </is>
       </c>
       <c r="D128" s="90" t="str">
-        <f>IF(ISNA('Mass Transfer'!$D$308+'Mass Transfer'!$D$317),"#N/A – check the selectors in D111/D112",IF(NOT(ISNUMBER('Mass Transfer'!$D$185)),"DO target unreachable on the sizing phase (rows 120–121) – the schedule is the legacy O₂ flush guard (Mass Transfer D89)",IF(Chemistry!$D$220&gt;=Chemistry!$D$236,"yes – the schedule holds the DO target at pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", within the band",IF('Mass Transfer'!$D$185&lt;='Mass Transfer'!$D$112,"NO – holding the DO target drives pH to "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor","NO – the carbon-limited interval (not the DO target) gives pH "&amp;TEXT(Chemistry!$D$220,"0.00")&amp;", below the "&amp;TEXT(Chemistry!$D$236,"0.0")&amp;" band floor"))))</f>
+        <f>IF(ISNA('Mass Transfer'!$D$308+'Mass Transfer'!$D$317),"#N/A – check the selectors in D111/D112",IF(NOT(ISNUMBER('Mass Transfer'!$D$185)),"DO target unreachable on the sizing phase (rows 120–121) – the schedule is the legacy O₂ flush guard (Mass Transfer D89)",IF(OR(AND(ISNUMBER(override_spg_dur_s),override_spg_dur_s&gt;0),AND(ISNUMBER(override_spg_int_min),override_spg_int_min&gt;0)),"watch – override in use (G13/G15), not the optimised schedule: pH "&amp;TEXT(res_pH,"0.00")&amp;", cycle-mean DO "&amp;TEXT(res_DO_ss,"0.0")&amp;" mg/L against the "&amp;TEXT('Mass Transfer'!$D$179*'Mass Transfer'!$D$231,"0.0")&amp;" mg/L target; neither target is claimed",IF(AND(res_pH&gt;=cf_pH_lo,res_pH&lt;=cf_pH_hi),"yes – the schedule holds the DO target at pH "&amp;TEXT(res_pH,"0.00")&amp;", within the "&amp;TEXT(cf_pH_lo,"0.0")&amp;"–"&amp;TEXT(cf_pH_hi,"0.0")&amp;" band",IF(res_pH&gt;cf_pH_hi,"NO – pH "&amp;TEXT(res_pH,"0.00")&amp;" above the "&amp;TEXT(cf_pH_hi,"0.0")&amp;" band ceiling",IF('Mass Transfer'!$D$185&lt;='Mass Transfer'!$D$112,"NO – holding the DO target drives pH to "&amp;TEXT(res_pH,"0.00")&amp;", below the "&amp;TEXT(cf_pH_lo,"0.0")&amp;" band floor","NO – the carbon-limited interval (not the DO target) gives pH "&amp;TEXT(res_pH,"0.00")&amp;", below the "&amp;TEXT(cf_pH_lo,"0.0")&amp;" band floor"))))))</f>
         <v>NO – holding the DO target drives pH to 6.20, below the 6.5 band floor</v>
       </c>
       <c r="E128" s="23" t="str">
@@ -10393,7 +10406,7 @@
       </c>
       <c r="F128" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">The vent model couples the two: when O₂ dilution binds, CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH (the text says which constraint binds). Red means the two targets conflict under the vent model in use — decouple them (inert sweep) or measure the vent before trusting either. #N/A = a selector in D111/D112 is not a listed value.</t>
+          <t xml:space="preserve">The vent model couples the two: when O₂ dilution binds, CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH (the text says which constraint binds). Tests both band edges (rows 139–140). Red means the two targets conflict under the vent model in use — decouple them (inert sweep) or measure the vent before trusting either. Amber "watch" = an override in G13/G15 is in use: the DO and pH shown are those of the typed schedule, and no claim is made that it holds the DO target. #N/A = a selector in D111/D112 is not a listed value.</t>
         </is>
       </c>
     </row>
@@ -13174,8 +13187,10 @@
         <f>rO2_gen-O2_cathode_ORR</f>
         <v>4.987344109764e-05</v>
       </c>
-      <c r="E29" s="99" t="s">
-        <v>379</v>
+      <c r="E29" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anodic O₂ minus cathodic consumption at the design DO (D85) — the O₂ the dissolved pool receives in growth. The lag phase uses O2_net_lag (D132), the loss at the lag DO.</t>
+        </is>
       </c>
       <c r="F29" s="20"/>
       <c r="G29" s="20"/>
@@ -14104,22 +14119,11 @@
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
-        <v>1626</v>
-      </c>
-      <c r="B79" s="18" t="s">
-        <v>1627</v>
-      </c>
-      <c r="C79" s="19" t="s">
-        <v>1274</v>
-      </c>
-      <c r="D79" s="141">
-        <f>Biology!$D$60</f>
-        <v>0.226086956522</v>
-      </c>
-      <c r="E79" s="67" t="s">
-        <v>1628</v>
-      </c>
+      <c r="A79"/>
+      <c r="B79" s="18"/>
+      <c r="C79" s="19"/>
+      <c r="D79" s="141"/>
+      <c r="E79" s="67"/>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
@@ -14214,8 +14218,10 @@
       </c>
     </row>
     <row r="85" spans="1:5" ht="36" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>1643</v>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Design DO for the cathodic O₂ flux (= the DO target)</t>
+        </is>
       </c>
       <c r="B85" s="18" t="s">
         <v>1644</v>
@@ -14224,11 +14230,13 @@
         <v>1001</v>
       </c>
       <c r="D85" s="141">
-        <f>ec_DO_frac*ec_O2_ceil</f>
+        <f>'Mass Transfer'!$D$179</f>
         <v>0.079603291295</v>
       </c>
-      <c r="E85" s="67" t="s">
-        <v>1645</v>
+      <c r="E85" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">→ Mass Transfer (DO_target, D179): the dissolved O₂ the schedule is designed to hold — the organism optimum once one is entered, otherwise the target fraction of the inhibition ceiling. The growth-phase cathodic O₂ reduction is evaluated here rather than at the modelled steady DO, which would make the sheet circular (DO depends on the net O₂, which depends on this loss). The lag phase uses DO_lag_ref (D129).</t>
+        </is>
       </c>
     </row>
     <row r="86" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -14413,7 +14421,7 @@
       </c>
       <c r="D96" s="141">
         <f>r_H2O2_lag/(k_H2O2_anode*3600)*(1-EXP(-k_H2O2_anode*3600))</f>
-        <v>0.900827055797</v>
+        <v>0.847372231321</v>
       </c>
       <c r="E96" s="67" t="inlineStr">
         <is>
@@ -14450,7 +14458,7 @@
       </c>
       <c r="D98" s="141">
         <f>IF(r_H2O2_lag&gt;0,IF(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag&gt;0,-LN(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag)/k_H2O2_anode/60,NA()),NA())</f>
-        <v>5.464176174322</v>
+        <v>5.843378301553</v>
       </c>
       <c r="E98" s="67" t="inlineStr">
         <is>
@@ -14470,7 +14478,7 @@
       </c>
       <c r="D99" s="141" t="str">
         <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(H2O2_lag_1h&gt;H2O2_thresh,"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases"))</f>
-        <v>watch — steady growth is clear (0.053 mg/L) but LAG PHASE is not: peroxide passes the threshold in 5 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.053 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min before biomass can scavenge it</v>
       </c>
       <c r="E99" s="67" t="s">
         <v>1685</v>
@@ -14752,10 +14760,9 @@
       <c r="D116" s="131">
         <v>1</v>
       </c>
-      <c r="E116" s="75" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~1.2 by Gerrit’s Law holding linear to 25 % on a 5 V rail (D143–D144). Measure with a conductivity standard.</t>
-        </is>
+      <c r="E116" s="75" t="str">
+        <f>("Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for "&amp;"rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~")&amp;TEXT(k_geom*(1+(V_rail-V_at_gerrit_max)/(I_at_gerrit_max*R_cell)),"0.00")&amp;" by Gerrit’s Law holding linear to "&amp;TEXT(gerrit_max,"0")&amp;" % on a "&amp;TEXT(V_rail,"0")&amp;" V rail (D143–D144); that leaves only "&amp;TEXT(V_rail-V_at_gerrit_max,"0.00")&amp;" V of headroom at "&amp;TEXT(gerrit_max,"0")&amp;" %, against the ±0.12 V j₀ uncertainty (E108), so the bound is soft. Measure with a conductivity standard."</f>
+        <v>Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~1.08 by Gerrit’s Law holding linear to 25 % on a 5 V rail (D143–D144); that leaves only 0.16 V of headroom at 25 %, against the ±0.12 V j₀ uncertainty (E108), so the bound is soft. Measure with a conductivity standard.</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -14861,10 +14868,9 @@
         <f>IF(V_headroom&lt;0,"OVER RAIL — the drive cannot deliver this current; the linear current law will not hold",IF(V_headroom&lt;V_headroom_min,"watch — within "&amp;TEXT(V_headroom_min,"0")&amp;" V of the rail ("&amp;TEXT(V_cell_est,"0.00")&amp;" V of "&amp;TEXT(V_rail,"0")&amp;" V); expect the current law to bend","OK — "&amp;TEXT(V_cell_est,"0.00")&amp;" V estimated against a "&amp;TEXT(V_rail,"0")&amp;" V rail"))</f>
         <v>OK — 2.85 V estimated against a 5 V rail</v>
       </c>
-      <c r="E122" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cross-check on Gerrit's Law: the fit is validated linear to gerrit_max (25 %), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (about 4.7 V at 25 % with k_geom = 1).</t>
-        </is>
+      <c r="E122" s="67" t="str">
+        <f>"Cross-check on Gerrit's Law: the fit is validated linear to gerrit_max ("&amp;TEXT(gerrit_max,"0")&amp;" %), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (currently "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" % with k_geom = "&amp;TEXT(k_geom,"0.0#")&amp;")."</f>
+        <v>Cross-check on Gerrit's Law: the fit is validated linear to gerrit_max (25 %), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (currently 4.84 V at 25 % with k_geom = 1.0).</v>
       </c>
     </row>
     <row r="124">
@@ -14946,6 +14952,167 @@
       <c r="E127" s="114" t="inlineStr">
         <is>
           <t xml:space="preserve">Design assumption: the current law starts to bend within this margin of the drive rail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LAG-PHASE CATHODIC O₂ LOSS AT THE LAG DO (review R5-m2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reference lag-phase DO for the cathodic loss</t>
+        </is>
+      </c>
+      <c r="B129" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_lag_ref</t>
+        </is>
+      </c>
+      <c r="C129" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D129" s="131">
+        <v>0.194</v>
+      </c>
+      <c r="E129" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Input, not a link: set to the last lag-phase cycle-mean DO (D150 = Mass Transfer D135) and re-enter it when D134 says so. Linking it would close a loop (lag DO → lag O₂ source → lag DO, and through the schedule when it is sized on Lag). Same pattern as Chemistry pH_ref_DIC. 0.194 is the self-consistent value at the defaults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tolerance before DO_lag_ref must be re-entered</t>
+        </is>
+      </c>
+      <c r="B130" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_lag_tol</t>
+        </is>
+      </c>
+      <c r="C130" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D130" s="131">
+        <v>0.05</v>
+      </c>
+      <c r="E130" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: re-enter DO_lag_ref when the lag DO has moved by more than 5 %. Only the cathodic share of the lag O₂ budget (~1/8 here) carries the error, so 5 % on DO is &lt;1 % on the source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ reduced at the cathode during lag</t>
+        </is>
+      </c>
+      <c r="B131" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_ORR_lag</t>
+        </is>
+      </c>
+      <c r="C131" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D131" s="141">
+        <f>MIN(I_app/(n_ORR_eff*F_const)*3600,O2_cathode_ORR*DO_lag_ref/ec_DO_design)</f>
+        <v>5.624573883267e-06</v>
+      </c>
+      <c r="E131" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The design-DO loss (D28) scaled to DO_lag_ref: the cathodic O₂ reduction is first order in DO, as for the lag peroxide (D152). Capped at the whole current. Follows a measured etaF too, because D28 does.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Net O₂ to the liquid during lag</t>
+        </is>
+      </c>
+      <c r="B132" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_net_lag</t>
+        </is>
+      </c>
+      <c r="C132" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D132" s="141">
+        <f>rO2_gen-O2_ORR_lag</f>
+        <v>4.655677748882e-05</v>
+      </c>
+      <c r="E132" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anodic O₂ less the cathodic loss at the lag DO: the lag-phase O₂ source (Mass Transfer O2_src_l, D310; Biology flammability). Below O2_net_gen (D29) because the lag DO runs above the design DO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ evolved during lag</t>
+        </is>
+      </c>
+      <c r="B133" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rH2_lag</t>
+        </is>
+      </c>
+      <c r="C133" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D133" s="141">
+        <f>MAX(0,I_app-O2_ORR_lag/3600*n_ORR_eff*F_const)/(z_e_H2*F_const)*3600</f>
+        <v>9.574538813904e-05</v>
+      </c>
+      <c r="E133" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The cathodic current not spent reducing O₂ at the lag DO, as H₂ (Mass Transfer H2_src_l, D314). Below rH2_gen (D21) for the same reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_lag_ref still matches the lag DO?</t>
+        </is>
+      </c>
+      <c r="B134" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_lag_ref_chk</t>
+        </is>
+      </c>
+      <c r="C134" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D134" s="141" t="str">
+        <f>IFERROR(IF(ABS(DO_lag_ref/ec_DO_lag-1)&gt;DO_lag_tol,"RE-ENTER DO_lag_ref (D129): the lag DO is now "&amp;TEXT(ec_DO_lag,"0.000")&amp;" mol/m³ ("&amp;TEXT(DO_lag_ref/ec_DO_lag-1,"+0%;-0%")&amp;" off)","OK – DO_lag_ref within "&amp;TEXT(DO_lag_tol,"0%")&amp;" of the lag DO ("&amp;TEXT(ec_DO_lag,"0.000")&amp;" mol/m³)"),"lag DO not available")</f>
+        <v>OK – DO_lag_ref within 5% of the lag DO (0.194 mol/m³)</v>
+      </c>
+      <c r="E134" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Display only (nothing reads it), so it closes no loop: compares the typed reference with the lag DO it produces.</t>
         </is>
       </c>
     </row>
@@ -15205,7 +15372,7 @@
       </c>
       <c r="D150" s="141">
         <f>'Mass Transfer'!$D$135</f>
-        <v>0.206435018988</v>
+        <v>0.194185222942</v>
       </c>
       <c r="E150" s="67" t="inlineStr">
         <is>
@@ -15257,11 +15424,11 @@
       </c>
       <c r="D152" s="141">
         <f>r_H2O2*ec_DO_lag/ec_DO_design</f>
-        <v>2.035813137102</v>
+        <v>1.915008557345</v>
       </c>
       <c r="E152" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">r_H2O2 scaled to the lag-phase DO (D150): the cathodic O₂ flux is first order in DO, and before uptake starts DO runs above the design value.</t>
+          <t xml:space="preserve">r_H2O2 scaled to the lag-phase DO (D150): the cathodic O₂ flux is first order in DO, and before uptake starts DO runs above the design value. The lag O₂ and H₂ sources use the same scaling (rows 129–133).</t>
         </is>
       </c>
     </row>
@@ -16912,8 +17079,10 @@
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
         <v>0.944445825575</v>
       </c>
-      <c r="E104" s="51" t="s">
-        <v>1879</v>
+      <c r="E104" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concentration-scale constant (KaHOCl_c) with the concentration-scale root pH_op, the consistent pair (R1-10); pH_meas (D220) is only for comparison with a probe.</t>
+        </is>
       </c>
     </row>
     <row r="105" spans="1:7" ht="36" x14ac:dyDescent="0.2">
@@ -16957,10 +17126,9 @@
         <f>Iappc/(2*Fcc)*M_HOCl*3600/VLc</f>
         <v>371.244905447914</v>
       </c>
-      <c r="E107" s="51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Naïve FE=1 upper bound (all anode current → Cl₂). Superseded by the mass-transport-limited chlorine current I_Cl (D133) and the production rate P_HOCl (D134). Kept only to show the overstatement (~40× at the current operating point).</t>
-        </is>
+      <c r="E107" s="51" t="str">
+        <f>"Naïve FE=1 upper bound (all anode current → Cl₂). Superseded by the mass-transport-limited chlorine current I_Cl (D133) and the production rate P_HOCl (D134). Kept only to show the overstatement ("&amp;TEXT(bleach_rate/(P_HOCl*M_HOCl*3600),"0")&amp;"× at the current operating point)."</f>
+        <v>Naïve FE=1 upper bound (all anode current → Cl₂). Superseded by the mass-transport-limited chlorine current I_Cl (D133) and the production rate P_HOCl (D134). Kept only to show the overstatement (59× at the current operating point).</v>
       </c>
       <c r="G107" s="69" t="s">
         <v>1009</v>
@@ -19909,21 +20077,11 @@
       <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:6" s="15" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="20" t="s">
-        <v>406</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>38</v>
-      </c>
+      <c r="A8" s="20"/>
+      <c r="B8" s="18"/>
       <c r="C8" s="20"/>
-      <c r="D8" s="38" t="str">
-        <f>Summary!$D$4</f>
-        <v>UdG (mixed)</v>
-      </c>
-      <c r="E8" s="23" t="str">
-        <f>HYPERLINK("#Summary!D4","→ Summary")</f>
-        <v>→ Summary</v>
-      </c>
+      <c r="D8" s="38"/>
+      <c r="E8" s="23"/>
       <c r="F8" s="20"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -20064,10 +20222,9 @@
         <f>MAX(0,O2_net_gen-O2_cons)</f>
         <v>1.591303582585e-05</v>
       </c>
-      <c r="E16" s="115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Net electrolytic O₂ minus biological uptake, floored at zero. The floor matters: at the knallgas cap (O₂:H₂ = 0.5, i.e. bio_O2 = 3) uptake exactly consumes the electrolytic surplus and everything downstream that divides by this would blow up. A LOWER bound on the surplus: full H₂ uptake maximises respiration, so any H₂ that bubbles off uncaught raises the surplus (half uptake → ×2.2). Sensitive: ±10 % in bio_O2 moves it +29 % / −12 %.</t>
-        </is>
+      <c r="E16" s="115" t="str">
+        <f>IFERROR(("Net electrolytic O₂ minus biological uptake, floored at zero. The floor matters: at the knallgas cap (O₂:H₂ = 0.5, i.e. bio_O2 = 3) uptake exactly consumes the electrolytic surplus and everything "&amp;"downstream that divides by this would blow up. A LOWER bound on the surplus: full H₂ uptake maximises respiration, so any H₂ that bubbles off uncaught raises the surplus (half uptake → ×")&amp;TEXT((O2_net_gen-O2_cons/2)/O2_excess,"0.0")&amp;"). Sensitive: each 1 % on bio_O2 moves it "&amp;TEXT(O2_cons/O2_excess,"0.0")&amp;" % the other way (linear, so symmetric).","Net electrolytic O₂ minus biological uptake, floored at zero: uptake consumes the whole surplus at these ratios.")</f>
+        <v>Net electrolytic O₂ minus biological uptake, floored at zero. The floor matters: at the knallgas cap (O₂:H₂ = 0.5, i.e. bio_O2 = 3) uptake exactly consumes the electrolytic surplus and everything downstream that divides by this would blow up. A LOWER bound on the surplus: full H₂ uptake maximises respiration, so any H₂ that bubbles off uncaught raises the surplus (half uptake → ×2.1). Sensitive: each 1 % on bio_O2 moves it 2.1 % the other way (linear, so symmetric).</v>
       </c>
       <c r="F16" s="20"/>
     </row>
@@ -20352,8 +20509,10 @@
       <c r="F31" s="20"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="17" t="s">
-        <v>473</v>
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) CO₂ partial pressure at sparge (dry-gas basis)</t>
+        </is>
       </c>
       <c r="B32" s="18" t="s">
         <v>474</v>
@@ -20362,11 +20521,13 @@
         <v>62</v>
       </c>
       <c r="D32" s="48">
-        <f>P_atm</f>
-        <v>101325.0</v>
-      </c>
-      <c r="E32" s="68" t="s">
-        <v>475</v>
+        <f>'Mass Transfer'!$D$418</f>
+        <v>98163.2639643</v>
+      </c>
+      <c r="E32" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D418 (P_dry): a pure-CO₂ pulse in a water-saturated headspace carries p_CO₂ = P_atm − p_sat_w, the basis of Mass Transfer D145.</t>
+        </is>
       </c>
       <c r="F32" s="20"/>
     </row>
@@ -20382,10 +20543,12 @@
       </c>
       <c r="D33" s="48">
         <f>H_CO2_T*p_CO2_sparge</f>
-        <v>33.43725</v>
-      </c>
-      <c r="E33" s="99" t="s">
-        <v>478</v>
+        <v>32.39387710822</v>
+      </c>
+      <c r="E33" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Equilibrium dissolved CO₂ under a pure-CO₂ headspace on the dry-gas basis (= Mass Transfer C_sat_CO2, D145; mol/m³ = mM). Legacy upper bound: a sub-second pulse never reaches it.</t>
+        </is>
       </c>
       <c r="F33" s="20"/>
     </row>
@@ -20419,10 +20582,12 @@
       </c>
       <c r="D35" s="48">
         <f>CO2_diss*1000/Km_CO2</f>
-        <v>668.745</v>
-      </c>
-      <c r="E35" s="99" t="s">
-        <v>484</v>
+        <v>647.877542164402</v>
+      </c>
+      <c r="E35" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dissolved CO₂ at full dry-basis saturation : RuBisCO Km. Legacy upper bound, superseded by the cycle-trough margin D98 (Summary D41).</t>
+        </is>
       </c>
       <c r="F35" s="20"/>
     </row>
@@ -20456,7 +20621,7 @@
       </c>
       <c r="D37" s="48">
         <f>-LOG10(SQRT(Ka1_carb*(CO2_diss/1000)))</f>
-        <v>3.913704718364</v>
+        <v>3.920588529366</v>
       </c>
       <c r="E37" s="69" t="s">
         <v>491</v>
@@ -20588,12 +20753,12 @@
         <v>135</v>
       </c>
       <c r="D44" s="48" t="str">
-        <f>IF(AND(y_H2_hs_lag&gt;=H2_LFL,y_O2_hs_lag&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe/2,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin (lag, mean basis; H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 17% before each pulse; O₂ 6% – until uptake starts, sparge every ≤1.9 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <f>IF(AND(y_H2_end_b&gt;=H2_LFL,y_O2_end_b&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe_saw,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin at every point of the cycle (lag): H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;", O₂ "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse ("&amp;TEXT(y_H2_hs_lag,"0%")&amp;" / "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean)")</f>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 11% mean, 17% before each pulse; O₂ 6% mean, 9% before each pulse – until uptake starts, sparge every ≤2.5 min or sweep ≥0.9 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tests the lag-phase headspace mix (rows 84–85, mean-field) against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin. The text also quotes the H₂ fraction just before each pulse (y_H2_end_b, sawtooth top), which is higher than the mean.</t>
+          <t xml:space="preserve">Tests the lag-phase headspace at its worst point, just before each pulse (sawtooth tops y_H2_end_b / y_O2_end_b, rows 114 and 119), against the H₂ lower flammability limit and the limiting O₂ concentration with a design margin; quotes mean and pre-pulse for both gases. The remedy interval (D92) is solved on the same pre-pulse basis, so at that interval the verdict clears.</t>
         </is>
       </c>
       <c r="F44" s="101" t="inlineStr">
@@ -21216,12 +21381,12 @@
         </is>
       </c>
       <c r="D83" s="48">
-        <f>H2_src_l_b+O2_net_gen</f>
-        <v>0.000151754656913</v>
+        <f>H2_src_l_b+O2_src_l_b</f>
+        <v>0.0001423021656279</v>
       </c>
       <c r="E83" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lag phase: no uptake, so all electrolytic H₂ not oxidised at the anode (H2_src_l_b) and the net O₂ reach the headspace.</t>
+          <t xml:space="preserve">Lag phase: no uptake, so all electrolytic H₂ not oxidised at the anode (H2_src_l_b) and the net O₂ (O2_src_l_b, cathodic loss at the lag DO) reach the headspace.</t>
         </is>
       </c>
     </row>
@@ -21243,7 +21408,7 @@
       </c>
       <c r="D84" s="48">
         <f>H2_src_l_b/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.112682153807</v>
+        <v>0.107014631173</v>
       </c>
       <c r="E84" s="69" t="inlineStr">
         <is>
@@ -21268,8 +21433,8 @@
         </is>
       </c>
       <c r="D85" s="48">
-        <f>(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.063684612076</v>
+        <f>(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
+        <v>0.060650407932</v>
       </c>
       <c r="E85" s="69" t="inlineStr">
         <is>
@@ -21294,8 +21459,8 @@
         </is>
       </c>
       <c r="D86" s="48">
-        <f>MAX(0,MIN(H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_net_gen+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
-        <v>0.003381603867</v>
+        <f>MAX(0,MIN(H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
+        <v>0.003183948324</v>
       </c>
       <c r="E86" s="69" t="inlineStr">
         <is>
@@ -21321,11 +21486,11 @@
       </c>
       <c r="D87" s="48">
         <f>IF(duty_H2safe&gt;0,spg_dur_b/(60*duty_H2safe),NA())</f>
-        <v>3.866572790086</v>
+        <v>4.106604808281</v>
       </c>
       <c r="E87" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mean-field; the pulse-to-pulse sawtooth peaks need roughly half this interval.</t>
+          <t xml:space="preserve">Mean-field (flux-mean) interval, kept for comparison only: the verdict and remedy (D44) use the pre-pulse sawtooth tops (D92), which need a shorter interval.</t>
         </is>
       </c>
     </row>
@@ -21347,11 +21512,115 @@
       </c>
       <c r="D88" s="48">
         <f>MAX(0,H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
-        <v>0.961689798439</v>
+        <v>0.902995989895</v>
       </c>
       <c r="E88" s="69" t="inlineStr">
         <is>
           <t xml:space="preserve">Continuous inert headspace sweep that dilutes H₂ below the LFL with no CO₂ at all, net of any air exchange already diluting it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) optimal pulse duration</t>
+        </is>
+      </c>
+      <c r="B89" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_dur_opt_b</t>
+        </is>
+      </c>
+      <c r="C89" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D89" s="150">
+        <f>'Mass Transfer'!$D$90</f>
+        <v>0.674076519917</v>
+      </c>
+      <c r="E89" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D90 (spg_dur_opt): the valve-open time added to the gap to give an interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longest gap keeping the lag pre-pulse H₂ below the LFL</t>
+        </is>
+      </c>
+      <c r="B90" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">t_gap_H2_LFL</t>
+        </is>
+      </c>
+      <c r="C90" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D90" s="48">
+        <f>IF(H2_src_l_b&gt;H2_LFL*F_gap_l_b,n_hs_gas_b/F_gap_l_b*LN((1-H2_LFL*F_gap_l_b/(H2_src_l_b)*flush_ret_opt_b)/(1-H2_LFL*F_gap_l_b/(H2_src_l_b)))*60,"none needed")</f>
+        <v>1.783559274358</v>
+      </c>
+      <c r="E90" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact on the Mass Transfer sawtooth (D388 form): the pre-pulse top y_end = (S/F)(1−e^−x)/(1−r·e^−x), x = F·t/n, r = flush_ret_opt, solved for y_end = LFL: x = ln((1−k·r)/(1−k)), k = LFL·F/S. Not circular: S, F, n and r do not depend on the interval. "none needed" = H₂ never reaches the LFL even with no pulses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longest gap keeping the lag pre-pulse O₂ under the LOC margin</t>
+        </is>
+      </c>
+      <c r="B91" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">t_gap_O2_LOC</t>
+        </is>
+      </c>
+      <c r="C91" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D91" s="48">
+        <f>IF(O2_src_l_b+y_O2_air_b*F_vent_ex_b&gt;O2_LOC_H2*LOC_margin*F_gap_l_b,n_hs_gas_b/F_gap_l_b*LN((1-O2_LOC_H2*LOC_margin*F_gap_l_b/(O2_src_l_b+y_O2_air_b*F_vent_ex_b)*flush_ret_opt_b)/(1-O2_LOC_H2*LOC_margin*F_gap_l_b/(O2_src_l_b+y_O2_air_b*F_vent_ex_b)))*60,"none needed")</f>
+        <v>2.506010430502</v>
+      </c>
+      <c r="E91" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As above for O₂ (source incl. the O₂ in admitted air, Mass Transfer S_O2_l), against LOC × margin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval that keeps the lag headspace non-flammable at every point of the cycle</t>
+        </is>
+      </c>
+      <c r="B92" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_H2safe_saw</t>
+        </is>
+      </c>
+      <c r="C92" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D92" s="48">
+        <f>IF(OR(ISTEXT(t_gap_H2_LFL),ISTEXT(t_gap_O2_LOC)),"any interval",MAX(t_gap_H2_LFL,t_gap_O2_LOC)+spg_dur_opt_b/60)</f>
+        <v>2.517245039167</v>
+      </c>
+      <c r="E92" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Either route suffices (H₂ below the LFL or O₂ under the LOC margin, as D86 encodes), so the longer of the two gaps, plus the pulse. Quoted as the remedy in D44 (replaces the "mean-field ÷ 2" heuristic).</t>
         </is>
       </c>
     </row>
@@ -21517,7 +21786,7 @@
       </c>
       <c r="D113" s="150">
         <f>'Mass Transfer'!$D$314</f>
-        <v>0.0001018812158154</v>
+        <v>9.574538813904e-05</v>
       </c>
       <c r="E113" s="135" t="inlineStr">
         <is>
@@ -21543,11 +21812,141 @@
       </c>
       <c r="D114" s="150">
         <f>'Mass Transfer'!$D$388</f>
-        <v>0.174311272995</v>
+        <v>0.165718619171</v>
       </c>
       <c r="E114" s="135" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Mass Transfer!D388 (sawtooth top).</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) O₂ to the headspace — lag (cathodic loss at the lag DO)</t>
+        </is>
+      </c>
+      <c r="B115" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_src_l_b</t>
+        </is>
+      </c>
+      <c r="C115" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D115" s="150">
+        <f>'Mass Transfer'!$D$310</f>
+        <v>4.655677748882e-05</v>
+      </c>
+      <c r="E115" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D310 (O2_src_l = Electrochemistry O2_net_lag).</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) gas leaving the headspace between pulses — lag</t>
+        </is>
+      </c>
+      <c r="B116" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_gap_l_b</t>
+        </is>
+      </c>
+      <c r="C116" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D116" s="150">
+        <f>'Mass Transfer'!$D$353</f>
+        <v>0.0001790888056997</v>
+      </c>
+      <c r="E116" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D353 (F_gap_l).</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) headspace gas inventory</t>
+        </is>
+      </c>
+      <c r="B117" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n_hs_gas_b</t>
+        </is>
+      </c>
+      <c r="C117" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol</t>
+        </is>
+      </c>
+      <c r="D117" s="150">
+        <f>'Mass Transfer'!$D$150</f>
+        <v>0.0001067805170238</v>
+      </c>
+      <c r="E117" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D150 (n_hs_gas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) headspace retained through the optimal pulse</t>
+        </is>
+      </c>
+      <c r="B118" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flush_ret_opt_b</t>
+        </is>
+      </c>
+      <c r="C118" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D118" s="150">
+        <f>'Mass Transfer'!$D$321</f>
+        <v>0.367879441171</v>
+      </c>
+      <c r="E118" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D321 (flush_ret_opt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) headspace O₂ just before a pulse (lag)</t>
+        </is>
+      </c>
+      <c r="B119" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_end_b</t>
+        </is>
+      </c>
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D119" s="150">
+        <f>'Mass Transfer'!$D$358</f>
+        <v>0.093920819467</v>
+      </c>
+      <c r="E119" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D358 (y_O2_end_l, sawtooth top).</t>
         </is>
       </c>
     </row>
@@ -23520,8 +23919,10 @@
         <f>min_sparge_cal</f>
         <v>0.25</v>
       </c>
-      <c r="E99" s="160" t="s">
-        <v>765</v>
+      <c r="E99" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solenoid floor in use = min_sparge_cal (D118): Calibrations tab Min pulse, else CO2 flows column I, else pulse_floor_default (D396).</t>
+        </is>
       </c>
       <c r="F99" s="20"/>
     </row>
@@ -23825,7 +24226,7 @@
       </c>
       <c r="E117" s="160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prefers the CO₂-flow calibration recorded on the Calibrations tab (cal_flow); falls back to the per-reactor table on the CO2 flows sheet when no calibration run is included.</t>
+          <t xml:space="preserve">Prefers the CO₂-flow calibration recorded on the Calibrations tab (cal_flow); falls back to the per-reactor table on the CO2 flows sheet when no calibration run is included. Either route switches the reactor on (has_cal, D119).</t>
         </is>
       </c>
       <c r="F117" s="20"/>
@@ -23841,10 +24242,14 @@
         <v>13</v>
       </c>
       <c r="D118" s="162">
-        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*'CO2 flows'!$I$4:$I$201)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*('CO2 flows'!$J$4:$J$201&gt;0)*1))</f>
+        <f>IF(ISNUMBER(cal_pulse_floor),cal_pulse_floor,IF(SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$J$4:$J$201&gt;0)*1)&gt;0,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*'CO2 flows'!$I$4:$I$201)/MAX(1,SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$B$4:$B$201=latest_date)*('CO2 flows'!$J$4:$J$201&gt;0)*1)),pulse_floor_default))</f>
         <v>0.25</v>
       </c>
-      <c r="E118" s="20"/>
+      <c r="E118" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solenoid floor for the selected reactor, same precedence as the flow (D117): the latest included Min pulse on the Calibrations tab (cal_pulse_floor, CO₂-flow column J); otherwise the CO2 flows column I average on the latest date; otherwise pulse_floor_default (D396).</t>
+        </is>
+      </c>
       <c r="F118" s="20"/>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.2">
@@ -23858,10 +24263,14 @@
         <v>806</v>
       </c>
       <c r="D119" s="162">
-        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$J$4:$J$201&gt;0)*1)</f>
+        <f>SUMPRODUCT(('CO2 flows'!$A$4:$A$201=Reactor)*('CO2 flows'!$J$4:$J$201&gt;0)*1)+IF(ISNUMBER(cal_flow),1,0)</f>
         <v>1.0</v>
       </c>
-      <c r="E119" s="20"/>
+      <c r="E119" s="160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calibration count for the selected reactor: CO2 flows rows with a nominal flowrate (column J), plus 1 when the CO₂-flow section of the Calibrations tab has an included run (cal_flow). 0 = uncalibrated: Q_CO2 and every schedule result read "calibrate this reactor first".</t>
+        </is>
+      </c>
       <c r="F119" s="20"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.2">
@@ -23873,8 +24282,8 @@
       </c>
       <c r="C120" s="20"/>
       <c r="D120" s="28" t="str">
-        <f>IF(has_cal&gt;0,"calibrated: "&amp;Reactor,"NO CALIBRATION for "&amp;Reactor&amp;" - add a row in CO2 flows with nominal flowrate + minimum sparge")</f>
-        <v>calibrated: ed04</v>
+        <f>IF(has_cal&gt;0,"calibrated: "&amp;Reactor&amp;IF(ISNUMBER(cal_flow)," (flow from the Calibrations tab)"," (flow from CO2 flows)"),"NO CALIBRATION for "&amp;Reactor&amp;" – record a CO₂ flow in the Calibrations tab (CO₂ flow section, Include = y) or add a row in CO2 flows with nominal flowrate + minimum sparge")</f>
+        <v>calibrated: ed04 (flow from CO2 flows)</v>
       </c>
       <c r="E120" s="20"/>
       <c r="F120" s="20"/>
@@ -24149,7 +24558,7 @@
       </c>
       <c r="D135" s="28">
         <f>DO_avg_l</f>
-        <v>0.206435018988</v>
+        <v>0.194185222942</v>
       </c>
       <c r="E135" s="69" t="inlineStr">
         <is>
@@ -24836,11 +25245,13 @@
         <v>1001</v>
       </c>
       <c r="D181" s="141">
-        <f>O2_net_gen/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.128273464734</v>
-      </c>
-      <c r="E181" s="67" t="s">
-        <v>1801</v>
+        <f>O2_src_l/(kLa_surf_used*3600*(V_charge/1000000))</f>
+        <v>0.119743074148</v>
+      </c>
+      <c r="E181" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Before the culture consumes oxygen, the whole net electrolytic O₂ (lag source O2_src_l, D310) has to cross the surface.</t>
+        </is>
       </c>
     </row>
     <row r="182" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -25817,12 +26228,12 @@
         </is>
       </c>
       <c r="D310" s="48">
-        <f>O2_net_gen</f>
-        <v>4.987344109764e-05</v>
+        <f>O2_net_lag_mt</f>
+        <v>4.655677748882e-05</v>
       </c>
       <c r="E310" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Net electrolytic O₂ with no biological uptake (Electrochemistry D29).</t>
+          <t xml:space="preserve">Net electrolytic O₂ with no biological uptake, with the cathodic loss at the lag DO (Electrochemistry D132, via DO_lag_ref) rather than at the design DO (D29): at the higher lag DO the cathode reduces ~2.4× more O₂, so this is ~7 % below O2_net_gen.</t>
         </is>
       </c>
     </row>
@@ -25921,12 +26332,12 @@
         </is>
       </c>
       <c r="D314" s="48">
-        <f>MAX(0,rH2_gen-H2_HOR_mt)</f>
-        <v>0.0001018812158154</v>
+        <f>MAX(0,rH2_lag_mt-H2_HOR_mt)</f>
+        <v>9.574538813904e-05</v>
       </c>
       <c r="E314" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">All evolved H₂ that the anode does not oxidise (H2_HOR_mt) reaches the headspace before uptake starts.</t>
+          <t xml:space="preserve">All H₂ evolved during lag (Electrochemistry D133, at the lag DO) that the anode does not oxidise (H2_HOR_mt) reaches the headspace before uptake starts.</t>
         </is>
       </c>
     </row>
@@ -26831,7 +27242,7 @@
       </c>
       <c r="D349" s="48">
         <f>O2_src_l+y_O2_air*F_vent_ex</f>
-        <v>5.75802421927e-05</v>
+        <v>5.426357858388e-05</v>
       </c>
       <c r="E349" s="67" t="inlineStr">
         <is>
@@ -26857,7 +27268,7 @@
       </c>
       <c r="D350" s="48">
         <f>CO2_supply+O2_src_l+H2_src_l-CO2_fix_l</f>
-        <v>0.0008673602223452</v>
+        <v>0.0008579077310601</v>
       </c>
       <c r="E350" s="67" t="inlineStr">
         <is>
@@ -26883,7 +27294,7 @@
       </c>
       <c r="D351" s="48">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,S_O2_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.063684612076</v>
+        <v>0.060650407932</v>
       </c>
       <c r="E351" s="67" t="inlineStr">
         <is>
@@ -26909,7 +27320,7 @@
       </c>
       <c r="D352" s="48">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,H2_src_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.112682153807</v>
+        <v>0.107014631173</v>
       </c>
       <c r="E352" s="67" t="inlineStr">
         <is>
@@ -26935,7 +27346,7 @@
       </c>
       <c r="D353" s="48">
         <f>F_vent_ex+MAX(0,O2_src_l+H2_src_l-CO2_fix_l)</f>
-        <v>0.0001885412969849</v>
+        <v>0.0001790888056997</v>
       </c>
       <c r="E353" s="67" t="inlineStr">
         <is>
@@ -26961,7 +27372,7 @@
       </c>
       <c r="D354" s="48">
         <f>F_gap_l*t_gap_h/n_hs_gas</f>
-        <v>0.263140362374</v>
+        <v>0.249947857486</v>
       </c>
       <c r="E354" s="67" t="inlineStr">
         <is>
@@ -26987,7 +27398,7 @@
       </c>
       <c r="D355" s="48">
         <f>IF(x_hs_l&gt;0,(1-EXP(-x_hs_l))/x_hs_l,1)</f>
-        <v>0.879249368918</v>
+        <v>0.8848189757</v>
       </c>
       <c r="E355" s="67" t="inlineStr">
         <is>
@@ -27013,7 +27424,7 @@
       </c>
       <c r="D356" s="48">
         <f>IF(x_hs_l&gt;0,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2)</f>
-        <v>0.458882970262</v>
+        <v>0.460820210498</v>
       </c>
       <c r="E356" s="67" t="inlineStr">
         <is>
@@ -27039,7 +27450,7 @@
       </c>
       <c r="D357" s="48">
         <f>S_O2_l*t_gap_h/n_hs_gas</f>
-        <v>0.08036268997</v>
+        <v>0.075733740887</v>
       </c>
       <c r="E357" s="67" t="inlineStr">
         <is>
@@ -27065,7 +27476,7 @@
       </c>
       <c r="D358" s="48">
         <f>dy_O2_l*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.098515562811</v>
+        <v>0.093920819467</v>
       </c>
       <c r="E358" s="68" t="inlineStr">
         <is>
@@ -27091,7 +27502,7 @@
       </c>
       <c r="D359" s="48">
         <f>y_O2_end_l*flush_ret</f>
-        <v>0.036241850194</v>
+        <v>0.03455153858</v>
       </c>
       <c r="E359" s="68" t="inlineStr">
         <is>
@@ -27117,7 +27528,7 @@
       </c>
       <c r="D360" s="48">
         <f>y_O2_post_l*phi_hs_l+dy_O2_l*psi_hs_l</f>
-        <v>0.068742693783</v>
+        <v>0.065471495392</v>
       </c>
       <c r="E360" s="68" t="inlineStr">
         <is>
@@ -27143,7 +27554,7 @@
       </c>
       <c r="D361" s="48">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_mf_l</f>
-        <v>0.200683898308</v>
+        <v>0.188703568554</v>
       </c>
       <c r="E361" s="67" t="inlineStr">
         <is>
@@ -27169,7 +27580,7 @@
       </c>
       <c r="D362" s="48">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_avg_l</f>
-        <v>0.206435018988</v>
+        <v>0.194185222942</v>
       </c>
       <c r="E362" s="68" t="inlineStr">
         <is>
@@ -27195,7 +27606,7 @@
       </c>
       <c r="D363" s="48">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*MAX(y_O2_avg_l,y_O2_end_l-(S_O2_l-F_gap_l*y_O2_end_l)/n_hs_gas*tau_L_h)</f>
-        <v>0.224263483321</v>
+        <v>0.211150707063</v>
       </c>
       <c r="E363" s="68" t="inlineStr">
         <is>
@@ -27221,7 +27632,7 @@
       </c>
       <c r="D364" s="48">
         <f>DO_avg_l*M_O2</f>
-        <v>6.605507737565</v>
+        <v>6.213538763708</v>
       </c>
       <c r="E364" s="68" t="inlineStr">
         <is>
@@ -27247,7 +27658,7 @@
       </c>
       <c r="D365" s="48">
         <f>DO_peak_l*M_O2</f>
-        <v>7.175982939307</v>
+        <v>6.756400324589</v>
       </c>
       <c r="E365" s="68" t="inlineStr">
         <is>
@@ -27273,7 +27684,7 @@
       </c>
       <c r="D366" s="48">
         <f>O2_src_l/(DO_target*3600*V_L_m3)</f>
-        <v>0.01160231226</v>
+        <v>0.010830739936</v>
       </c>
       <c r="E366" s="67" t="inlineStr">
         <is>
@@ -27299,7 +27710,7 @@
       </c>
       <c r="D367" s="48">
         <f>kLa_surf_used/kLa_surf_req_l</f>
-        <v>0.620574890218</v>
+        <v>0.664784095965</v>
       </c>
       <c r="E367" s="67" t="inlineStr">
         <is>
@@ -27325,7 +27736,7 @@
       </c>
       <c r="D368" s="28" t="str">
         <f>IF(kLa_margin_l&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)")</f>
-        <v>UNREACHABLE at this surface kLa – margin 0.62× (raise kL_surf, lower the current, or accept a higher DO)</v>
+        <v>UNREACHABLE at this surface kLa – margin 0.66× (raise kL_surf, lower the current, or accept a higher DO)</v>
       </c>
       <c r="E368" s="67" t="inlineStr">
         <is>
@@ -27351,7 +27762,7 @@
       </c>
       <c r="D369" s="28" t="str">
         <f>IF(DO_peak_l&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
-        <v>peak 7.2 mg/L under the 11.3 mg/L ceiling</v>
+        <v>peak 6.8 mg/L under the 11.3 mg/L ceiling</v>
       </c>
       <c r="E369" s="67" t="inlineStr">
         <is>
@@ -27800,7 +28211,7 @@
       </c>
       <c r="D388" s="48">
         <f>H2_src_l*t_gap_h/n_hs_gas*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.174311272995</v>
+        <v>0.165718619171</v>
       </c>
       <c r="E388" s="68" t="inlineStr">
         <is>
@@ -27937,6 +28348,83 @@
         </is>
       </c>
     </row>
+    <row r="394">
+      <c r="A394" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Net O₂ to the liquid — lag (cathodic loss at the lag DO)</t>
+        </is>
+      </c>
+      <c r="B394" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_net_lag_mt</t>
+        </is>
+      </c>
+      <c r="C394" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D394" s="142">
+        <f>Electrochemistry!$D$132</f>
+        <v>4.655677748882e-05</v>
+      </c>
+      <c r="E394" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D132 (O2_net_lag).</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) H₂ evolved — lag</t>
+        </is>
+      </c>
+      <c r="B395" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rH2_lag_mt</t>
+        </is>
+      </c>
+      <c r="C395" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D395" s="142">
+        <f>Electrochemistry!$D$133</f>
+        <v>9.574538813904e-05</v>
+      </c>
+      <c r="E395" s="135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D133 (rH2_lag).</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solenoid floor when no minimum pulse is recorded</t>
+        </is>
+      </c>
+      <c r="B396" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pulse_floor_default</t>
+        </is>
+      </c>
+      <c r="C396" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D396" s="131">
+        <v>0.25</v>
+      </c>
+      <c r="E396" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weak estimate: the shortest pulse logged for ed04 (CO2 flows I4, 0.25 s), used only for a reactor calibrated on the Calibrations tab with no Min pulse entry and no CO2 flows row. Confirm per reactor (flow-calibration.md, minimum-pulse step).</t>
+        </is>
+      </c>
+    </row>
     <row r="400">
       <c r="A400" s="5" t="inlineStr">
         <is>
@@ -28116,12 +28604,12 @@
         </is>
       </c>
       <c r="D407" s="28">
-        <f>IF(AND(fit_n&gt;=fit_n_min,fit_n*fit_Stt-fit_St^2&gt;0),(fit_n*fit_StV-fit_St*fit_SV)/(fit_n*fit_Stt-fit_St^2),Q_CO2/60)</f>
+        <f>IF(ISNUMBER(cal_flow),cal_flow,IF(AND(fit_n&gt;=fit_n_min,fit_n*fit_Stt-fit_St^2&gt;0),(fit_n*fit_StV-fit_St*fit_SV)/(fit_n*fit_Stt-fit_St^2),Q_CO2/60))</f>
         <v>3.318707459132</v>
       </c>
       <c r="E407" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Least-squares slope of pulse volume on pulse time (R2-M3). ed04: 3.319 mL/s over 34 runs, vs the 3.33 nominal. Falls back to Q_CO2/60 when there is no usable fit.</t>
+          <t xml:space="preserve">One rule: the source that sets Q_CO2 also sets the pulse model. A Calibrations-tab flow (cal_flow) is a steady open-valve flow, so it is the slope here; otherwise the least-squares slope of pulse volume on pulse time over the CO2 flows rows (R2-M3; ed04: 3.319 mL/s over 34 runs, vs the 3.33 nominal); Q_CO2/60 when there is no usable fit.</t>
         </is>
       </c>
     </row>
@@ -28142,12 +28630,12 @@
         </is>
       </c>
       <c r="D408" s="28">
-        <f>IF(AND(fit_n&gt;=fit_n_min,fit_n*fit_Stt-fit_St^2&gt;0),(fit_SV-Q_CO2_fit*fit_St)/fit_n,0)</f>
+        <f>IF(ISNUMBER(cal_flow),0,IF(AND(fit_n&gt;=fit_n_min,fit_n*fit_Stt-fit_St^2&gt;0),(fit_SV-Q_CO2_fit*fit_St)/fit_n,0))</f>
         <v>0.375365681243</v>
       </c>
       <c r="E408" s="69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Least-squares intercept (R2-M3): ed04 0.375 mL (0.327 if the 15 s run is dropped, 0.131 on ≤2 s runs only). Weak: captured at the inlet tube over CO₂-saturated water / NaHCO₃ (CO2 flows L7–L9), ±0.2 mL. Re-measure at the operating pulse length downstream of a sealed cap.</t>
+          <t xml:space="preserve">Least-squares intercept (R2-M3): ed04 0.375 mL (0.327 if the 15 s run is dropped, 0.131 on ≤2 s runs only). Weak: captured at the inlet tube over CO₂-saturated water / NaHCO₃ (CO2 flows L7–L9), ±0.2 mL. 0 while a Calibrations-tab flow is in use (steady flow, intercept unknown) until the per-pulse volume is re-measured downstream of a sealed cap.</t>
         </is>
       </c>
     </row>
@@ -31001,7 +31489,7 @@
       <c r="G23" s="123"/>
       <c r="H23" s="123"/>
       <c r="I23" s="129" t="str">
-        <f>IFERROR(((G23-p_sat_w)*(E23/1000000)/(R_gas*(F23+T_zero_C)))/(D23/(IF(H23="H2",z_e_H2,IF(H23="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G23-pw_A*EXP(pw_B*F23/(F23+pw_C)))*(E23/1000000)/(R_gas*(F23+T_zero_C)))/(D23/(IF(H23="H2",z_e_H2,IF(H23="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J23" s="129" t="str">
@@ -31022,7 +31510,7 @@
       <c r="G24" s="123"/>
       <c r="H24" s="123"/>
       <c r="I24" s="129" t="str">
-        <f>IFERROR(((G24-p_sat_w)*(E24/1000000)/(R_gas*(F24+T_zero_C)))/(D24/(IF(H24="H2",z_e_H2,IF(H24="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G24-pw_A*EXP(pw_B*F24/(F24+pw_C)))*(E24/1000000)/(R_gas*(F24+T_zero_C)))/(D24/(IF(H24="H2",z_e_H2,IF(H24="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J24" s="129" t="str">
@@ -31043,7 +31531,7 @@
       <c r="G25" s="123"/>
       <c r="H25" s="123"/>
       <c r="I25" s="129" t="str">
-        <f>IFERROR(((G25-p_sat_w)*(E25/1000000)/(R_gas*(F25+T_zero_C)))/(D25/(IF(H25="H2",z_e_H2,IF(H25="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G25-pw_A*EXP(pw_B*F25/(F25+pw_C)))*(E25/1000000)/(R_gas*(F25+T_zero_C)))/(D25/(IF(H25="H2",z_e_H2,IF(H25="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J25" s="129" t="str">
@@ -31064,7 +31552,7 @@
       <c r="G26" s="123"/>
       <c r="H26" s="123"/>
       <c r="I26" s="129" t="str">
-        <f>IFERROR(((G26-p_sat_w)*(E26/1000000)/(R_gas*(F26+T_zero_C)))/(D26/(IF(H26="H2",z_e_H2,IF(H26="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G26-pw_A*EXP(pw_B*F26/(F26+pw_C)))*(E26/1000000)/(R_gas*(F26+T_zero_C)))/(D26/(IF(H26="H2",z_e_H2,IF(H26="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J26" s="129" t="str">
@@ -31085,7 +31573,7 @@
       <c r="G27" s="123"/>
       <c r="H27" s="123"/>
       <c r="I27" s="129" t="str">
-        <f>IFERROR(((G27-p_sat_w)*(E27/1000000)/(R_gas*(F27+T_zero_C)))/(D27/(IF(H27="H2",z_e_H2,IF(H27="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G27-pw_A*EXP(pw_B*F27/(F27+pw_C)))*(E27/1000000)/(R_gas*(F27+T_zero_C)))/(D27/(IF(H27="H2",z_e_H2,IF(H27="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J27" s="129" t="str">
@@ -31106,7 +31594,7 @@
       <c r="G28" s="123"/>
       <c r="H28" s="123"/>
       <c r="I28" s="129" t="str">
-        <f>IFERROR(((G28-p_sat_w)*(E28/1000000)/(R_gas*(F28+T_zero_C)))/(D28/(IF(H28="H2",z_e_H2,IF(H28="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G28-pw_A*EXP(pw_B*F28/(F28+pw_C)))*(E28/1000000)/(R_gas*(F28+T_zero_C)))/(D28/(IF(H28="H2",z_e_H2,IF(H28="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J28" s="129" t="str">
@@ -31127,7 +31615,7 @@
       <c r="G29" s="123"/>
       <c r="H29" s="123"/>
       <c r="I29" s="129" t="str">
-        <f>IFERROR(((G29-p_sat_w)*(E29/1000000)/(R_gas*(F29+T_zero_C)))/(D29/(IF(H29="H2",z_e_H2,IF(H29="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G29-pw_A*EXP(pw_B*F29/(F29+pw_C)))*(E29/1000000)/(R_gas*(F29+T_zero_C)))/(D29/(IF(H29="H2",z_e_H2,IF(H29="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J29" s="129" t="str">
@@ -31148,7 +31636,7 @@
       <c r="G30" s="123"/>
       <c r="H30" s="123"/>
       <c r="I30" s="129" t="str">
-        <f>IFERROR(((G30-p_sat_w)*(E30/1000000)/(R_gas*(F30+T_zero_C)))/(D30/(IF(H30="H2",z_e_H2,IF(H30="O2",z_e_O2,NA()))*F_const)),"")</f>
+        <f>IFERROR(((G30-pw_A*EXP(pw_B*F30/(F30+pw_C)))*(E30/1000000)/(R_gas*(F30+T_zero_C)))/(D30/(IF(H30="H2",z_e_H2,IF(H30="O2",z_e_O2,NA()))*F_const)),"")</f>
         <v/>
       </c>
       <c r="J30" s="129" t="str">
@@ -31512,8 +32000,10 @@
       <c r="M49" s="97"/>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A50" s="97" t="s">
-        <v>1416</v>
+      <c r="A50" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use: the most recent included measurement for the active reactor (a flow rate is a valve/hardware setting, so the latest reading replaces older ones). An included flow here calibrates the reactor on its own (no CO2 flows row needed). Min pulse (column J, optional): the shortest commanded pulse that still delivers a repeatable volume; the latest included entry sets the solenoid floor (row 61).</t>
+        </is>
       </c>
       <c r="B50" s="97"/>
       <c r="C50" s="97"/>
@@ -31556,7 +32046,11 @@
       <c r="I51" s="128" t="s">
         <v>1403</v>
       </c>
-      <c r="J51" s="97"/>
+      <c r="J51" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Min pulse (s)</t>
+        </is>
+      </c>
       <c r="K51" s="97"/>
       <c r="L51" s="97"/>
       <c r="M51" s="97"/>
@@ -31577,7 +32071,7 @@
       </c>
       <c r="H52" s="122"/>
       <c r="I52" s="122"/>
-      <c r="J52" s="97"/>
+      <c r="J52" s="123"/>
       <c r="K52" s="97"/>
       <c r="L52" s="97"/>
       <c r="M52" s="97"/>
@@ -31598,7 +32092,7 @@
       </c>
       <c r="H53" s="122"/>
       <c r="I53" s="122"/>
-      <c r="J53" s="97"/>
+      <c r="J53" s="123"/>
       <c r="K53" s="97"/>
       <c r="L53" s="97"/>
       <c r="M53" s="97"/>
@@ -31619,7 +32113,7 @@
       </c>
       <c r="H54" s="122"/>
       <c r="I54" s="122"/>
-      <c r="J54" s="97"/>
+      <c r="J54" s="123"/>
       <c r="K54" s="97"/>
       <c r="L54" s="97"/>
       <c r="M54" s="97"/>
@@ -31640,7 +32134,7 @@
       </c>
       <c r="H55" s="122"/>
       <c r="I55" s="122"/>
-      <c r="J55" s="97"/>
+      <c r="J55" s="123"/>
       <c r="K55" s="97"/>
       <c r="L55" s="97"/>
       <c r="M55" s="97"/>
@@ -31661,7 +32155,7 @@
       </c>
       <c r="H56" s="122"/>
       <c r="I56" s="122"/>
-      <c r="J56" s="97"/>
+      <c r="J56" s="123"/>
       <c r="K56" s="97"/>
       <c r="L56" s="97"/>
       <c r="M56" s="97"/>
@@ -31682,7 +32176,7 @@
       </c>
       <c r="H57" s="122"/>
       <c r="I57" s="122"/>
-      <c r="J57" s="97"/>
+      <c r="J57" s="123"/>
       <c r="K57" s="97"/>
       <c r="L57" s="97"/>
       <c r="M57" s="97"/>
@@ -31703,7 +32197,7 @@
       </c>
       <c r="H58" s="122"/>
       <c r="I58" s="122"/>
-      <c r="J58" s="97"/>
+      <c r="J58" s="123"/>
       <c r="K58" s="97"/>
       <c r="L58" s="97"/>
       <c r="M58" s="97"/>
@@ -31724,7 +32218,7 @@
       </c>
       <c r="H59" s="122"/>
       <c r="I59" s="122"/>
-      <c r="J59" s="97"/>
+      <c r="J59" s="123"/>
       <c r="K59" s="97"/>
       <c r="L59" s="97"/>
       <c r="M59" s="97"/>
@@ -31752,10 +32246,21 @@
       <c r="M60" s="97"/>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A61" s="97"/>
+      <c r="A61" s="125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - minimum reliable pulse</t>
+        </is>
+      </c>
       <c r="B61" s="97"/>
-      <c r="C61" s="97"/>
-      <c r="D61" s="97"/>
+      <c r="C61" s="126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D61" s="124" t="str">
+        <f>IFERROR(AVERAGEIFS(J52:J59,C52:C59,Reactor_sel,H52:H59,"y",J52:J59,"&gt;0",B52:B59,SUMPRODUCT(MAX((C52:C59=Reactor_sel)*(H52:H59="y")*(J52:J59&gt;0)*B52:B59))),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
       <c r="E61" s="97"/>
       <c r="F61" s="97"/>
       <c r="G61" s="97"/>
@@ -33574,6 +34079,84 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Magnus coefficient A</t>
+        </is>
+      </c>
+      <c r="B149" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pw_A</t>
+        </is>
+      </c>
+      <c r="C149" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pa</t>
+        </is>
+      </c>
+      <c r="D149" s="164">
+        <f>'Mass Transfer'!$D$203</f>
+        <v>610.94</v>
+      </c>
+      <c r="E149" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D203 (pw_A; Magnus–Tetens, T in °C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Magnus coefficient B</t>
+        </is>
+      </c>
+      <c r="B150" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pw_B</t>
+        </is>
+      </c>
+      <c r="C150" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D150" s="164">
+        <f>'Mass Transfer'!$D$204</f>
+        <v>17.625</v>
+      </c>
+      <c r="E150" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D204 (pw_B; Magnus–Tetens, T in °C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Magnus coefficient C</t>
+        </is>
+      </c>
+      <c r="B151" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pw_C</t>
+        </is>
+      </c>
+      <c r="C151" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">°C</t>
+        </is>
+      </c>
+      <c r="D151" s="164">
+        <f>'Mass Transfer'!$D$205</f>
+        <v>243.04</v>
+      </c>
+      <c r="E151" s="165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D205 (pw_C; Magnus–Tetens, T in °C)</t>
+        </is>
+      </c>
+    </row>
     <row r="155">
       <c r="A155" s="17" t="inlineStr">
         <is>
@@ -33783,30 +34366,11 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(import) Saturated water vapour pressure at reactor T</t>
-        </is>
-      </c>
-      <c r="B163" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p_sat_w</t>
-        </is>
-      </c>
-      <c r="C163" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pa</t>
-        </is>
-      </c>
-      <c r="D163" s="164">
-        <f>'Mass Transfer'!$D$206</f>
-        <v>3161.736035696692</v>
-      </c>
-      <c r="E163" s="165" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Import from Mass Transfer!D206 (p_sat_w)</t>
-        </is>
-      </c>
+      <c r="A163" s="17"/>
+      <c r="B163" s="97"/>
+      <c r="C163" s="19"/>
+      <c r="D163" s="164"/>
+      <c r="E163" s="165"/>
     </row>
   </sheetData>
   <dataValidations count="4">

</xml_diff>

<commit_message>
Gas model: alkalinity needed for a target pH (2.6 g/L NaHCO3 for pH 6.5, first order)
Chemistry rows 302-308 evaluate the charge-balance residual at the target
probe pH; Summary D131-D132 report NaHCO3 (g/L) and extra alkalinity (mM).
Excel-recalculated; twin 366/366; sensitivity 49/49.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BZjvK3H9KbkmZeLMwx9pSC
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -855,6 +855,12 @@
     <definedName name="z_e_O2" localSheetId="7">Calibrations!$D$147</definedName>
     <definedName name="z_e_O2" localSheetId="2">Electrochemistry!$D$17</definedName>
     <definedName name="z_e_ORR" localSheetId="2">Electrochemistry!$D$27</definedName>
+    <definedName name="alk_pH_target" localSheetId="3">Chemistry!$D$303</definedName>
+    <definedName name="alk_pH_target_c" localSheetId="3">Chemistry!$D$304</definedName>
+    <definedName name="alk_resid_t" localSheetId="3">Chemistry!$D$305</definedName>
+    <definedName name="alk_needed" localSheetId="3">Chemistry!$D$306</definedName>
+    <definedName name="M_NaHCO3" localSheetId="3">Chemistry!$D$307</definedName>
+    <definedName name="alk_NaHCO3_gL" localSheetId="3">Chemistry!$D$308</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
@@ -12430,6 +12436,56 @@
         <v>1832</v>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NaHCO₃ to lift pH to the target (first-order)</t>
+        </is>
+      </c>
+      <c r="C131" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g/L</t>
+        </is>
+      </c>
+      <c r="D131" s="68">
+        <f>Chemistry!$D$308</f>
+        <v>2.584020698787</v>
+      </c>
+      <c r="E131" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F131" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alkalinity the medium would need for a probe pH of Chemistry D303 (the 6.5 band floor by default) at today’s dissolved CO₂. A media-design lever for row 128; not fed back into the model yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same, as extra alkalinity</t>
+        </is>
+      </c>
+      <c r="C132" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mM</t>
+        </is>
+      </c>
+      <c r="D132" s="68">
+        <f>Chemistry!$D$306*1000</f>
+        <v>30.759587877041</v>
+      </c>
+      <c r="E132" s="23" t="str">
+        <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
+        <v>→ Chemistry</v>
+      </c>
+      <c r="F132" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Any strong base counts (NaHCO₃, KHCO₃, NaOH). Using nitrate or urea instead of NH₄⁺ also avoids the acid released as the culture takes up ammonium.</t>
+        </is>
+      </c>
+    </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="67" t="s">
         <v>1833</v>
@@ -12823,7 +12879,7 @@
     <row r="154">
       <c r="A154" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Model: alkalinity for target pH</t>
+          <t xml:space="preserve">Model: couple alkalinity into pH</t>
         </is>
       </c>
       <c r="B154" s="20" t="inlineStr">
@@ -12838,7 +12894,7 @@
       </c>
       <c r="F154" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Under a CO₂ headspace pH is set by alkalinity. Rough estimate: about +26 mM (≈2.2 g/L NaHCO₃) reaches the 6.5 band floor, about +140 mM pH 7.0. Nitrate or urea instead of NH₄⁺ avoids acidification during growth.</t>
+          <t xml:space="preserve">Rows 131–132 now give the NaHCO₃ for a target pH at first order (about 2 g/L for the 6.5 floor). Still to do: an added-alkalinity input that feeds the charge balance, ionic strength and CO₂ storage, so the schedule and pH respond to it.</t>
         </is>
       </c>
     </row>
@@ -21553,6 +21609,168 @@
         <v>2099</v>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALKALINITY NEEDED FOR A TARGET pH (first-order: dissolved CO₂ and activity coefficients held at the schedule in use)</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Target pH a probe should read</t>
+        </is>
+      </c>
+      <c r="B303" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alk_pH_target</t>
+        </is>
+      </c>
+      <c r="C303" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D303" s="116">
+        <f>pH_band_lo</f>
+        <v>6.5</v>
+      </c>
+      <c r="E303" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defaults to the HOB band floor (D236). Type a number (e.g. 7.0) to size for another target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Target pH on the concentration scale</t>
+        </is>
+      </c>
+      <c r="B304" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alk_pH_target_c</t>
+        </is>
+      </c>
+      <c r="C304" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D304" s="116">
+        <f>alk_pH_target+LOG10(gamma_1)</f>
+        <v>6.39033524156</v>
+      </c>
+      <c r="E304" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Probe (activity) pH to the concentration scale the charge balance solves on: the inverse of D220.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charge-balance residual at the target pH</t>
+        </is>
+      </c>
+      <c r="B305" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alk_resid_t</t>
+        </is>
+      </c>
+      <c r="C305" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D305" s="116">
+        <f>pH_SID + pH_NT*(10^-alk_pH_target_c)/((10^-alk_pH_target_c)+KaN_c) + (10^-alk_pH_target_c) - (pH_PT*Ka1p_c*(10^-alk_pH_target_c)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-alk_pH_target_c) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-alk_pH_target_c)^3 + Ka1p_c*(10^-alk_pH_target_c)^2 + Ka1p_c*Ka2p_c*(10^-alk_pH_target_c) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-alk_pH_target_c) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-alk_pH_target_c)^2 - Kw_c/(10^-alk_pH_target_c)</f>
+        <v>-0.030759587877</v>
+      </c>
+      <c r="E305" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Same residual as the pH grid (B50), at the target. Negative = the medium lacks that much strong cation (alkalinity) to sit at the target pH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extra alkalinity needed for the target pH</t>
+        </is>
+      </c>
+      <c r="B306" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alk_needed</t>
+        </is>
+      </c>
+      <c r="C306" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D306" s="116">
+        <f>MAX(0,-alk_resid_t)</f>
+        <v>0.030759587877</v>
+      </c>
+      <c r="E306" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Strong base (Na⁺ or K⁺ added as bicarbonate or hydroxide) that zeroes the residual at the target, holding dissolved CO₂ (D5) and γ fixed. 0 = the target is already met.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Molar mass of NaHCO₃</t>
+        </is>
+      </c>
+      <c r="B307" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M_NaHCO3</t>
+        </is>
+      </c>
+      <c r="C307" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g/mol</t>
+        </is>
+      </c>
+      <c r="D307" s="135">
+        <v>84.007</v>
+      </c>
+      <c r="E307" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IUPAC standard atomic weights (Na 22.990, H 1.008, C 12.011, O 15.999).</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NaHCO₃ to add for the target pH</t>
+        </is>
+      </c>
+      <c r="B308" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alk_NaHCO3_gL</t>
+        </is>
+      </c>
+      <c r="C308" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g/L</t>
+        </is>
+      </c>
+      <c r="D308" s="116">
+        <f>alk_needed*M_NaHCO3</f>
+        <v>2.584020698787</v>
+      </c>
+      <c r="E308" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-order: added Na⁺ raises ionic strength a little and the extra bicarbonate enlarges the CO₂ storage (D296), neither fed back here. Full coupling is on the Summary TODO.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="D109:D110 D163">
     <cfRule type="expression" dxfId="11" priority="101" stopIfTrue="1">

</xml_diff>

<commit_message>
Gas model: reconcile commanded schedule and gas/charge balances
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -862,6 +862,13 @@
     <definedName name="z_e_O2" localSheetId="7">Calibrations!$D$147</definedName>
     <definedName name="z_e_O2" localSheetId="2">Electrochemistry!$D$17</definedName>
     <definedName name="z_e_ORR" localSheetId="2">Electrochemistry!$D$27</definedName>
+    <definedName name="interval_res" localSheetId="5">'Mass Transfer'!$D$419</definedName>
+    <definedName name="spg_int_run" localSheetId="5">'Mass Transfer'!$D$420</definedName>
+    <definedName name="DIC_ref_tol" localSheetId="3">Chemistry!$D$309</definedName>
+    <definedName name="DIC_ref_check" localSheetId="3">Chemistry!$D$310</definedName>
+    <definedName name="Cl_bound" localSheetId="3">Chemistry!$D$311</definedName>
+    <definedName name="Cl_model_check" localSheetId="3">Chemistry!$D$312</definedName>
+    <definedName name="remedy_res" localSheetId="4">Biology!$D$120</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -11186,13 +11193,15 @@
       <c r="C14" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="66">
-        <f>IF(AND(ISNUMBER($G$13),$G$13&gt;0),$G$13,IF(NOT(ISNUMBER(D13)),D13,'Mass Transfer'!$D$242))</f>
+      <c r="D14" s="111">
+        <f>IF(NOT(ISNUMBER(res_spg_dur)),res_spg_dur,'Mass Transfer'!spg_dur)</f>
         <v>0.65</v>
       </c>
       <c r="E14" s="21"/>
-      <c r="F14" s="22" t="s">
-        <v>1712</v>
+      <c r="F14" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse actually evaluated by every operating check below. Summary override wins, then Manual mode, otherwise the optimum rounded to the pulse resolution.</t>
+        </is>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -11208,7 +11217,7 @@
       </c>
       <c r="D15" s="65">
         <f>IF('Mass Transfer'!$D$119=0,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)",'Mass Transfer'!$D$91)</f>
-        <v>7.450071557247</v>
+        <v>7.398866407059</v>
       </c>
       <c r="E15" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
@@ -11229,14 +11238,15 @@
       <c r="C16" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="66">
-        <f>IF(AND(ISNUMBER($G$15),$G$15&gt;0),$G$15,IF(NOT(ISNUMBER(D15)),D15,ROUND(('Mass Transfer'!$D$408+'Mass Transfer'!$D$407*D14)/('Mass Transfer'!$D$102/60)/(60*'Mass Transfer'!$D$93),0)))</f>
-        <v>7.0</v>
+      <c r="D16" s="111">
+        <f>IF(NOT(ISNUMBER(res_spg_int)),res_spg_int,'Mass Transfer'!spg_int)</f>
+        <v>7.17</v>
       </c>
       <c r="E16" s="67"/>
-      <c r="F16" s="22" t="str">
-        <f>"Interval to type in: the as-run pulse converted to delivered CO₂ (V₀ + Q·t, Mass Transfer D407–D408) at the optimised full-flow-equivalent duty (D93), rounded to whole minutes; "&amp;IF(ISNUMBER(D95),"rounding moves the CO₂ dose by "&amp;TEXT(D95-1,"+0.0%;-0.0%")&amp;" (row 95)","row 95 shows how far rounding moves the CO₂ dose")&amp;". An override in G15 wins."</f>
-        <v>Interval to type in: the as-run pulse converted to delivered CO₂ (V₀ + Q·t, Mass Transfer D407–D408) at the optimised full-flow-equivalent duty (D93), rounded to whole minutes; rounding moves the CO₂ dose by +3.2% (row 95). An override in G15 wins.</v>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval actually evaluated below, in decimal minutes. Default converts the commanded pulse to the ideal delivery duty and rounds down to 0.01 min; overrides and Manual mode are evaluated directly.</t>
+        </is>
       </c>
     </row>
     <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -11313,7 +11323,7 @@
       <c r="C21" s="21"/>
       <c r="D21" s="65" t="str">
         <f>'Mass Transfer'!$D$374</f>
-        <v>organism band unknown – peak 2.5 mg/L is under the inhibition ceiling</v>
+        <v>organism band unknown – peak 2.4 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E21" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D374","→ Mass Transfer")</f>
@@ -11353,7 +11363,7 @@
       <c r="C23" s="21"/>
       <c r="D23" s="65" t="str">
         <f>'Mass Transfer'!$D$113</f>
-        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈13 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
+        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈14 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E23" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
@@ -11373,7 +11383,7 @@
       <c r="C24" s="21"/>
       <c r="D24" s="70" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.4 min or sweep ≥0.9 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="24" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -11413,7 +11423,7 @@
       <c r="C26" s="21"/>
       <c r="D26" s="65" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!$D$126,"0.0")&amp;IF('Mass Transfer'!$D$126&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)")&amp;" delivered; ×"&amp;TEXT('Mass Transfer'!$D$417,"0.0")&amp;" absorbed per pulse (row 135)","calibrate this reactor first")</f>
-        <v>×49.6 OK delivered; ×2.4 absorbed per pulse (row 135)</v>
+        <v>×50.0 OK delivered; ×2.5 absorbed per pulse (row 135)</v>
       </c>
       <c r="E26" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
@@ -11593,7 +11603,7 @@
       <c r="C35" s="21"/>
       <c r="D35" s="92">
         <f>Chemistry!$D$220</f>
-        <v>6.487893381735</v>
+        <v>6.487611781829</v>
       </c>
       <c r="E35" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -11621,8 +11631,9 @@
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F36" s="22" t="s">
-        <v>1748</v>
+      <c r="F36" s="111" t="str">
+        <f>IF(Chemistry!Cl_model_check&lt;&gt;"OK",Chemistry!Cl_model_check,"Effective chlorine on the as-Cl2 basis; zero for chloride-free medium. Lifetime and potency require measurement.")</f>
+        <v>Effective chlorine on the as-Cl2 basis; zero for chloride-free medium. Lifetime and potency require measurement.</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -11647,7 +11658,7 @@
       </c>
       <c r="D38" s="65">
         <f>'Mass Transfer'!$D$108</f>
-        <v>2.27518163832</v>
+        <v>2.270165488391</v>
       </c>
       <c r="E38" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D108","→ Mass")</f>
@@ -11713,7 +11724,7 @@
       </c>
       <c r="D41" s="70">
         <f>Biology!$D$98</f>
-        <v>507.959765236247</v>
+        <v>508.83519620388</v>
       </c>
       <c r="E41" s="24" t="str">
         <f>HYPERLINK("#Biology!D98","→ Biology")</f>
@@ -12399,7 +12410,7 @@
       </c>
       <c r="D85" s="23" t="str">
         <f>Electrochemistry!$D$99</f>
-        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 7 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min before biomass can scavenge it</v>
       </c>
       <c r="E85" s="24" t="str">
         <f>HYPERLINK("#Electrochemistry!D99","→ Electrochemistry")</f>
@@ -12441,9 +12452,9 @@
       <c r="C87" s="20" t="s">
         <v>1445</v>
       </c>
-      <c r="D87" s="23">
+      <c r="D87" s="23" t="e">
         <f>Chemistry!$D$209</f>
-        <v>-0.30390069301</v>
+        <v>#N/A</v>
       </c>
       <c r="E87" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D209","→ Chemistry")</f>
@@ -12465,7 +12476,7 @@
       </c>
       <c r="D88" s="23">
         <f>Chemistry!$D$211</f>
-        <v>1.248872573638</v>
+        <v>1.248889512283</v>
       </c>
       <c r="E88" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
@@ -12487,7 +12498,7 @@
       </c>
       <c r="D89" s="23">
         <f>Chemistry!$D$220</f>
-        <v>6.487893381735</v>
+        <v>6.487611781829</v>
       </c>
       <c r="E89" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -12541,7 +12552,7 @@
       </c>
       <c r="D95" s="70">
         <f>IF(AND(ISNUMBER(D14),ISNUMBER(D16),ISNUMBER('Mass Transfer'!$D$93)),('Mass Transfer'!$D$408+'Mass Transfer'!$D$407*D14)/('Mass Transfer'!$D$102/60)/(60*D16)/'Mass Transfer'!$D$93,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)")</f>
-        <v>1.031743711429</v>
+        <v>1.000358015991</v>
       </c>
       <c r="E95" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
@@ -12624,7 +12635,7 @@
       </c>
       <c r="D114" s="65">
         <f>'Mass Transfer'!$D$343</f>
-        <v>2.27518163832</v>
+        <v>2.270165488391</v>
       </c>
       <c r="E114" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D343","→ Mass Transfer")</f>
@@ -12643,7 +12654,7 @@
       </c>
       <c r="D115" s="65">
         <f>'Mass Transfer'!$D$344</f>
-        <v>2.461241182614</v>
+        <v>2.447092253397</v>
       </c>
       <c r="E115" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D344","→ Mass Transfer")</f>
@@ -12662,7 +12673,7 @@
       </c>
       <c r="D116" s="65">
         <f>'Mass Transfer'!$D$364</f>
-        <v>5.543911888859</v>
+        <v>5.594849867262</v>
       </c>
       <c r="E116" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
@@ -12681,7 +12692,7 @@
       </c>
       <c r="D117" s="65">
         <f>'Mass Transfer'!$D$365</f>
-        <v>5.915267968126</v>
+        <v>5.953949768528</v>
       </c>
       <c r="E117" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D365","→ Mass Transfer")</f>
@@ -12697,7 +12708,7 @@
       </c>
       <c r="D118" s="65" t="str">
         <f>'Mass Transfer'!$D$348</f>
-        <v>peak 2.5 mg/L under the 10.1 mg/L ceiling</v>
+        <v>peak 2.4 mg/L under the 10.1 mg/L ceiling</v>
       </c>
       <c r="E118" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D348","→ Mass Transfer")</f>
@@ -12713,7 +12724,7 @@
       </c>
       <c r="D119" s="65" t="str">
         <f>'Mass Transfer'!$D$369</f>
-        <v>peak 5.9 mg/L under the 10.1 mg/L ceiling</v>
+        <v>peak 6.0 mg/L under the 10.1 mg/L ceiling</v>
       </c>
       <c r="E119" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D369","→ Mass Transfer")</f>
@@ -12745,7 +12756,7 @@
       </c>
       <c r="D121" s="65" t="str">
         <f>'Mass Transfer'!$D$368</f>
-        <v>UNREACHABLE at this surface kLa – margin 0.62× (raise kL_surf, lower the current, or accept a higher DO)</v>
+        <v>UNREACHABLE at this surface kLa – margin 0.61× (raise kL_surf, lower the current, or accept a higher DO)</v>
       </c>
       <c r="E121" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D368","→ Mass Transfer")</f>
@@ -12753,7 +12764,7 @@
       </c>
       <c r="F121" s="22" t="str">
         <f>"Same on the lag source. Currently "&amp;TEXT('Mass Transfer'!$D$367,"0.00")&amp;"×: "&amp;IF('Mass Transfer'!$D$367&lt;1,"the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).","the target can be held during lag at the kLa in use.")</f>
-        <v>Same on the lag source. Currently 0.62×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
+        <v>Same on the lag source. Currently 0.61×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.2">
@@ -12784,7 +12795,7 @@
       </c>
       <c r="D123" s="65">
         <f>'Mass Transfer'!$D$366*3600</f>
-        <v>44.455069334556</v>
+        <v>44.975226114474</v>
       </c>
       <c r="E123" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D366","→ Mass Transfer")</f>
@@ -12803,7 +12814,7 @@
       </c>
       <c r="D124" s="65">
         <f>'Mass Transfer'!$D$329</f>
-        <v>0.027761802038</v>
+        <v>0.027569266375</v>
       </c>
       <c r="E124" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D329","→ Mass Transfer")</f>
@@ -12822,7 +12833,7 @@
       </c>
       <c r="D125" s="65">
         <f>'Mass Transfer'!$D$351</f>
-        <v>0.053679883871</v>
+        <v>0.053815126441</v>
       </c>
       <c r="E125" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D351","→ Mass Transfer")</f>
@@ -12841,7 +12852,7 @@
       </c>
       <c r="D126" s="65">
         <f>'Mass Transfer'!$D$352</f>
-        <v>0.093395436531</v>
+        <v>0.093689942909</v>
       </c>
       <c r="E126" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D352","→ Mass Transfer")</f>
@@ -12860,7 +12871,7 @@
       </c>
       <c r="D127" s="65">
         <f>'Mass Transfer'!$D$381</f>
-        <v>0.939820877487</v>
+        <v>0.940238937993</v>
       </c>
       <c r="E127" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D381","→ Mass Transfer")</f>
@@ -12874,9 +12885,9 @@
       <c r="A128" s="64" t="s">
         <v>1827</v>
       </c>
-      <c r="D128" s="65" t="str">
-        <f>IF(ISNA('Mass Transfer'!$D$308+'Mass Transfer'!$D$317),"#N/A – check the selectors in D111/D112",IF(NOT(ISNUMBER('Mass Transfer'!$D$185)),"DO target unreachable on the sizing phase (rows 120–121) – the schedule is the legacy O₂ flush guard (Mass Transfer D89)",IF(OR(AND(ISNUMBER(override_spg_dur_s),override_spg_dur_s&gt;0),AND(ISNUMBER(override_spg_int_min),override_spg_int_min&gt;0)),"watch – override in use (G13/G15), not the optimised schedule: pH "&amp;TEXT(res_pH,"0.00")&amp;", cycle-mean DO "&amp;TEXT(res_DO_ss,"0.0")&amp;" mg/L against the "&amp;TEXT('Mass Transfer'!$D$179*'Mass Transfer'!$D$231,"0.0")&amp;" mg/L target; neither target is claimed",IF(AND(res_pH&gt;=cf_pH_lo,res_pH&lt;=cf_pH_hi),"yes – the schedule holds the DO target at pH "&amp;TEXT(res_pH,"0.00")&amp;", within the "&amp;TEXT(cf_pH_lo,"0.0")&amp;"–"&amp;TEXT(cf_pH_hi,"0.0")&amp;" band",IF(res_pH&gt;cf_pH_hi,"NO – pH "&amp;TEXT(res_pH,"0.00")&amp;" above the "&amp;TEXT(cf_pH_hi,"0.0")&amp;" band ceiling",IF('Mass Transfer'!$D$185&lt;='Mass Transfer'!$D$112,"NO – holding the DO target drives pH to "&amp;TEXT(res_pH,"0.00")&amp;", below the "&amp;TEXT(cf_pH_lo,"0.0")&amp;" band floor","NO – the carbon-limited interval (not the DO target) gives pH "&amp;TEXT(res_pH,"0.00")&amp;", below the "&amp;TEXT(cf_pH_lo,"0.0")&amp;" band floor"))))))</f>
-        <v>NO – holding the DO target drives pH to 6.49, below the 6.5 band floor</v>
+      <c r="D128" s="111" t="str">
+        <f>IF(ISNA('Mass Transfer'!F_vent_ex+'Mass Transfer'!O2_src_sched),"#N/A – check the selectors in D111/D112",IF(NOT(ISNUMBER('Mass Transfer'!spg_int_DO)),"DO target unreachable on the sizing phase; schedule is a legacy fallback",IF(OR(Chemistry!DIC_ref_check&lt;&gt;"OK",ABS(Electrochemistry!DO_lag_ref/Electrochemistry!ec_DO_lag-1)&gt;Electrochemistry!DO_lag_tol),"watch – refresh the DIC or lag-DO reference before claiming either target",IF(AND(res_pH&gt;=cf_pH_lo,res_pH&lt;=cf_pH_hi,res_DO_ss&lt;='Mass Transfer'!DO_target*'Mass Transfer'!M_O2),"yes – both targets met by the evaluated schedule","NO – evaluated schedule misses the pH band or mean DO target"))))</f>
+        <v>NO – evaluated schedule misses the pH band or mean DO target</v>
       </c>
       <c r="E128" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -12895,7 +12906,7 @@
       </c>
       <c r="D129" s="65">
         <f>'Mass Transfer'!$D$389</f>
-        <v>0.047702404255</v>
+        <v>0.050856361228</v>
       </c>
       <c r="E129" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D389","→ Mass Transfer")</f>
@@ -12911,7 +12922,7 @@
       </c>
       <c r="D130" s="65" t="str">
         <f>'Mass Transfer'!$D$391</f>
-        <v>n/a – the vent admits air (Open vent / Air exchange), so the headspace refills</v>
+        <v>UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow</v>
       </c>
       <c r="E130" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D391","→ Mass Transfer")</f>
@@ -12930,7 +12941,7 @@
       </c>
       <c r="D131" s="65">
         <f>Chemistry!$D$308</f>
-        <v>0.120777240215</v>
+        <v>0.124226377682</v>
       </c>
       <c r="E131" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
@@ -12949,7 +12960,7 @@
       </c>
       <c r="D132" s="65">
         <f>Chemistry!$D$306*1000</f>
-        <v>1.437704479563</v>
+        <v>1.47876221841</v>
       </c>
       <c r="E132" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
@@ -12971,7 +12982,7 @@
       </c>
       <c r="D135" s="65">
         <f>'Mass Transfer'!$D$417</f>
-        <v>2.356485959356</v>
+        <v>2.501832900863</v>
       </c>
       <c r="E135" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D417","→ Mass Transfer")</f>
@@ -17060,7 +17071,7 @@
       </c>
       <c r="D96" s="111">
         <f>r_H2O2_lag/(k_H2O2_anode*3600)*(1-EXP(-k_H2O2_anode*3600))</f>
-        <v>0.833154224922</v>
+        <v>0.840809324217</v>
       </c>
       <c r="E96" s="51" t="s">
         <v>1877</v>
@@ -17095,7 +17106,7 @@
       </c>
       <c r="D98" s="111">
         <f>IF(r_H2O2_lag&gt;0,IF(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag&gt;0,-LN(1-H2O2_thresh*k_H2O2_anode*3600/r_H2O2_lag)/k_H2O2_anode/60,NA()),NA())</f>
-        <v>6.52524470598</v>
+        <v>6.460189095256</v>
       </c>
       <c r="E98" s="51" t="s">
         <v>1878</v>
@@ -17113,7 +17124,7 @@
       </c>
       <c r="D99" s="111" t="str">
         <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(H2O2_lag_1h&gt;H2O2_thresh,"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases"))</f>
-        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 7 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min before biomass can scavenge it</v>
       </c>
       <c r="E99" s="51" t="s">
         <v>1519</v>
@@ -17574,7 +17585,7 @@
         <v>406</v>
       </c>
       <c r="D129" s="130">
-        <v>0.19400000000000001</v>
+        <v>0.174849986629</v>
       </c>
       <c r="E129" s="57" t="s">
         <v>1894</v>
@@ -17608,8 +17619,8 @@
         <v>307</v>
       </c>
       <c r="D131" s="111">
-        <f>MIN(I_app/(n_ORR_eff*F_const)*3600,O2_cathode_ORR*DO_lag_ref/ec_DO_design)</f>
-        <v>5.624573883267e-06</v>
+        <f>MIN(I_app/(n_ORR_eff*F_const)*3600,IF(ISNUMBER(cal_etaF),(O2_cathode_ORR*DO_lag_ref/ec_DO_design),(i_ORR_design/(n_ORR_eff*F_const)*3600*DO_lag_ref/ec_DO_design)))</f>
+        <v>5.0693642695e-06</v>
       </c>
       <c r="E131" s="57" t="s">
         <v>1900</v>
@@ -17627,7 +17638,7 @@
       </c>
       <c r="D132" s="111">
         <f>rO2_gen-O2_ORR_lag</f>
-        <v>4.745085102827e-05</v>
+        <v>4.800606064204e-05</v>
       </c>
       <c r="E132" s="57" t="s">
         <v>1903</v>
@@ -17645,7 +17656,7 @@
       </c>
       <c r="D133" s="111">
         <f>MAX(0,I_app-O2_ORR_lag/3600*n_ORR_eff*F_const)/(z_e_H2*F_const)*3600</f>
-        <v>9.574538813904e-05</v>
+        <v>9.67725259245e-05</v>
       </c>
       <c r="E133" s="57" t="s">
         <v>1906</v>
@@ -17663,7 +17674,7 @@
       </c>
       <c r="D134" s="111" t="str">
         <f>IFERROR(IF(ABS(DO_lag_ref/ec_DO_lag-1)&gt;DO_lag_tol,"RE-ENTER DO_lag_ref (D129): the lag DO is now "&amp;TEXT(ec_DO_lag,"0.000")&amp;" mol/m³ ("&amp;TEXT(DO_lag_ref/ec_DO_lag-1,"+0%;-0%")&amp;" off)","OK – DO_lag_ref within "&amp;TEXT(DO_lag_tol,"0%")&amp;" of the lag DO ("&amp;TEXT(ec_DO_lag,"0.000")&amp;" mol/m³)"),"lag DO not available")</f>
-        <v>RE-ENTER DO_lag_ref (D129): the lag DO is now 0.173 mol/m³ (+12% off)</v>
+        <v>OK – DO_lag_ref within 5% of the lag DO (0.175 mol/m³)</v>
       </c>
       <c r="E134" s="57" t="s">
         <v>1909</v>
@@ -17845,7 +17856,7 @@
       </c>
       <c r="D150" s="111">
         <f>'Mass Transfer'!$D$135</f>
-        <v>0.173258075157</v>
+        <v>0.174849986476</v>
       </c>
       <c r="E150" s="51" t="s">
         <v>1941</v>
@@ -17880,11 +17891,13 @@
         <v>870</v>
       </c>
       <c r="D152" s="111">
-        <f>r_H2O2*ec_DO_lag/ec_DO_design</f>
-        <v>1.708629995252</v>
-      </c>
-      <c r="E152" s="51" t="s">
-        <v>1947</v>
+        <f>f_HOOH*O2_ORR_lag*M_H2O2*1000/ec_V_L</f>
+        <v>1.724329048178</v>
+      </c>
+      <c r="E152" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peroxide is f_HOOH times the same capped lag ORR oxygen flux used by the H2/O2 budgets (D131). No separate uncapped scaling by the solved lag DO.</t>
+        </is>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
@@ -17940,7 +17953,7 @@
       </c>
       <c r="D161" s="111">
         <f>Chemistry!$D$218</f>
-        <v>0.199715551957</v>
+        <v>0.199711947856</v>
       </c>
       <c r="E161" s="140" t="s">
         <v>1955</v>
@@ -18089,7 +18102,7 @@
       </c>
       <c r="D5" s="49">
         <f>'Mass Transfer'!$D$162</f>
-        <v>0.025542123443</v>
+        <v>0.025562568426</v>
       </c>
       <c r="E5" s="138" t="s">
         <v>1963</v>
@@ -18765,7 +18778,7 @@
       </c>
       <c r="B50" s="49">
         <f t="shared" ref="B50:B81" si="1">pH_SID + pH_NT*(10^-A50)/((10^-A50)+KaN_c) + (10^-A50) - (pH_PT*Ka1p_c*(10^-A50)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A50) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A50)^3 + Ka1p_c*(10^-A50)^2 + Ka1p_c*Ka2p_c*(10^-A50) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A50) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A50)^2 - Kw_c/(10^-A50)</f>
-        <v>0.069961208004</v>
+        <v>0.069961033937</v>
       </c>
       <c r="C50" s="49">
         <f t="shared" ref="C50:C81" si="2">IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
@@ -18778,7 +18791,7 @@
       </c>
       <c r="B51" s="49">
         <f t="shared" si="1"/>
-        <v>0.06975156695</v>
+        <v>0.069751347811</v>
       </c>
       <c r="C51" s="49">
         <f t="shared" si="2"/>
@@ -18791,7 +18804,7 @@
       </c>
       <c r="B52" s="49">
         <f t="shared" si="1"/>
-        <v>0.069543628739</v>
+        <v>0.06954335286</v>
       </c>
       <c r="C52" s="49">
         <f t="shared" si="2"/>
@@ -18804,7 +18817,7 @@
       </c>
       <c r="B53" s="49">
         <f t="shared" si="1"/>
-        <v>0.069326510002</v>
+        <v>0.06932616269</v>
       </c>
       <c r="C53" s="49">
         <f t="shared" si="2"/>
@@ -18817,7 +18830,7 @@
       </c>
       <c r="B54" s="49">
         <f t="shared" si="1"/>
-        <v>0.069088805882</v>
+        <v>0.069088368641</v>
       </c>
       <c r="C54" s="49">
         <f t="shared" si="2"/>
@@ -18830,7 +18843,7 @@
       </c>
       <c r="B55" s="49">
         <f t="shared" si="1"/>
-        <v>0.068818015909</v>
+        <v>0.068817465454</v>
       </c>
       <c r="C55" s="49">
         <f t="shared" si="2"/>
@@ -18843,7 +18856,7 @@
       </c>
       <c r="B56" s="49">
         <f t="shared" si="1"/>
-        <v>0.068499911658</v>
+        <v>0.068499218674</v>
       </c>
       <c r="C56" s="49">
         <f t="shared" si="2"/>
@@ -18856,7 +18869,7 @@
       </c>
       <c r="B57" s="49">
         <f t="shared" si="1"/>
-        <v>0.068117819329</v>
+        <v>0.068116946912</v>
       </c>
       <c r="C57" s="49">
         <f t="shared" si="2"/>
@@ -18869,7 +18882,7 @@
       </c>
       <c r="B58" s="49">
         <f t="shared" si="1"/>
-        <v>0.067651787194</v>
+        <v>0.067650688881</v>
       </c>
       <c r="C58" s="49">
         <f t="shared" si="2"/>
@@ -18882,7 +18895,7 @@
       </c>
       <c r="B59" s="49">
         <f t="shared" si="1"/>
-        <v>0.067077604497</v>
+        <v>0.067076221795</v>
       </c>
       <c r="C59" s="49">
         <f t="shared" si="2"/>
@@ -18895,7 +18908,7 @@
       </c>
       <c r="B60" s="49">
         <f t="shared" si="1"/>
-        <v>0.06636563522</v>
+        <v>0.066363894488</v>
       </c>
       <c r="C60" s="49">
         <f t="shared" si="2"/>
@@ -18908,7 +18921,7 @@
       </c>
       <c r="B61" s="49">
         <f t="shared" si="1"/>
-        <v>0.065479427437</v>
+        <v>0.065477235967</v>
       </c>
       <c r="C61" s="49">
         <f t="shared" si="2"/>
@@ -18921,7 +18934,7 @@
       </c>
       <c r="B62" s="49">
         <f t="shared" si="1"/>
-        <v>0.06437405756</v>
+        <v>0.064371298632</v>
       </c>
       <c r="C62" s="49">
         <f t="shared" si="2"/>
@@ -18934,7 +18947,7 @@
       </c>
       <c r="B63" s="49">
         <f t="shared" si="1"/>
-        <v>0.062994169269</v>
+        <v>0.062990695937</v>
       </c>
       <c r="C63" s="49">
         <f t="shared" si="2"/>
@@ -18947,7 +18960,7 @@
       </c>
       <c r="B64" s="49">
         <f t="shared" si="1"/>
-        <v>0.06127167011</v>
+        <v>0.061267297369</v>
       </c>
       <c r="C64" s="49">
         <f t="shared" si="2"/>
@@ -18960,7 +18973,7 @@
       </c>
       <c r="B65" s="49">
         <f t="shared" si="1"/>
-        <v>0.059123054466</v>
+        <v>0.059117549391</v>
       </c>
       <c r="C65" s="49">
         <f t="shared" si="2"/>
@@ -18973,7 +18986,7 @@
       </c>
       <c r="B66" s="49">
         <f t="shared" si="1"/>
-        <v>0.056446328096</v>
+        <v>0.056439397427</v>
       </c>
       <c r="C66" s="49">
         <f t="shared" si="2"/>
@@ -18986,7 +18999,7 @@
       </c>
       <c r="B67" s="49">
         <f t="shared" si="1"/>
-        <v>0.053117511059</v>
+        <v>0.053108785561</v>
       </c>
       <c r="C67" s="49">
         <f t="shared" si="2"/>
@@ -18999,7 +19012,7 @@
       </c>
       <c r="B68" s="49">
         <f t="shared" si="1"/>
-        <v>0.048986680763</v>
+        <v>0.048975695534</v>
       </c>
       <c r="C68" s="49">
         <f t="shared" si="2"/>
@@ -19012,7 +19025,7 @@
       </c>
       <c r="B69" s="49">
         <f t="shared" si="1"/>
-        <v>0.043873464183</v>
+        <v>0.043859633841</v>
       </c>
       <c r="C69" s="49">
         <f t="shared" si="2"/>
@@ -19025,7 +19038,7 @@
       </c>
       <c r="B70" s="49">
         <f t="shared" si="1"/>
-        <v>0.037561767097</v>
+        <v>0.037544354526</v>
       </c>
       <c r="C70" s="49">
         <f t="shared" si="2"/>
@@ -19038,7 +19051,7 @@
       </c>
       <c r="B71" s="49">
         <f t="shared" si="1"/>
-        <v>0.029793302153</v>
+        <v>0.02977137912</v>
       </c>
       <c r="C71" s="49">
         <f t="shared" si="2"/>
@@ -19051,7 +19064,7 @@
       </c>
       <c r="B72" s="49">
         <f t="shared" si="1"/>
-        <v>0.020259119105</v>
+        <v>0.020231516623</v>
       </c>
       <c r="C72" s="49">
         <f t="shared" si="2"/>
@@ -19064,11 +19077,11 @@
       </c>
       <c r="B73" s="49">
         <f t="shared" si="1"/>
-        <v>0.008587856904</v>
+        <v>0.008553102653</v>
       </c>
       <c r="C73" s="49">
         <f t="shared" si="2"/>
-        <v>6.360227804438</v>
+        <v>6.359946204531</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -19077,7 +19090,7 @@
       </c>
       <c r="B74" s="49">
         <f t="shared" si="1"/>
-        <v>-0.005671100374</v>
+        <v>-0.005714860965</v>
       </c>
       <c r="C74" s="49">
         <f t="shared" si="2"/>
@@ -19090,7 +19103,7 @@
       </c>
       <c r="B75" s="49">
         <f t="shared" si="1"/>
-        <v>-0.023071830034</v>
+        <v>-0.023126933372</v>
       </c>
       <c r="C75" s="49">
         <f t="shared" si="2"/>
@@ -19103,7 +19116,7 @@
       </c>
       <c r="B76" s="49">
         <f t="shared" si="1"/>
-        <v>-0.044305894942</v>
+        <v>-0.044375284982</v>
       </c>
       <c r="C76" s="49">
         <f t="shared" si="2"/>
@@ -19116,7 +19129,7 @@
       </c>
       <c r="B77" s="49">
         <f t="shared" si="1"/>
-        <v>-0.070248485151</v>
+        <v>-0.070335872221</v>
       </c>
       <c r="C77" s="49">
         <f t="shared" si="2"/>
@@ -19129,7 +19142,7 @@
       </c>
       <c r="B78" s="49">
         <f t="shared" si="1"/>
-        <v>-0.102018603865</v>
+        <v>-0.102128665511</v>
       </c>
       <c r="C78" s="49">
         <f t="shared" si="2"/>
@@ -19142,7 +19155,7 @@
       </c>
       <c r="B79" s="49">
         <f t="shared" si="1"/>
-        <v>-0.141055008418</v>
+        <v>-0.141193643645</v>
       </c>
       <c r="C79" s="49">
         <f t="shared" si="2"/>
@@ -19155,7 +19168,7 @@
       </c>
       <c r="B80" s="49">
         <f t="shared" si="1"/>
-        <v>-0.189210043149</v>
+        <v>-0.189384694734</v>
       </c>
       <c r="C80" s="49">
         <f t="shared" si="2"/>
@@ -19168,7 +19181,7 @@
       </c>
       <c r="B81" s="49">
         <f t="shared" si="1"/>
-        <v>-0.248864922646</v>
+        <v>-0.249084986427</v>
       </c>
       <c r="C81" s="49">
         <f t="shared" si="2"/>
@@ -19181,7 +19194,7 @@
       </c>
       <c r="B82" s="49">
         <f t="shared" ref="B82:B100" si="3">pH_SID + pH_NT*(10^-A82)/((10^-A82)+KaN_c) + (10^-A82) - (pH_PT*Ka1p_c*(10^-A82)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A82) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A82)^3 + Ka1p_c*(10^-A82)^2 + Ka1p_c*Ka2p_c*(10^-A82) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A82) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A82)^2 - Kw_c/(10^-A82)</f>
-        <v>-0.323072497969</v>
+        <v>-0.32334984372</v>
       </c>
       <c r="C82" s="49">
         <f t="shared" ref="C82:C99" si="4">IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
@@ -19194,7 +19207,7 @@
       </c>
       <c r="B83" s="49">
         <f t="shared" si="3"/>
-        <v>-0.415736899954</v>
+        <v>-0.416086535989</v>
       </c>
       <c r="C83" s="49">
         <f t="shared" si="4"/>
@@ -19207,7 +19220,7 @@
       </c>
       <c r="B84" s="49">
         <f t="shared" si="3"/>
-        <v>-0.531843581218</v>
+        <v>-0.532284505155</v>
       </c>
       <c r="C84" s="49">
         <f t="shared" si="4"/>
@@ -19220,7 +19233,7 @@
       </c>
       <c r="B85" s="49">
         <f t="shared" si="3"/>
-        <v>-0.677758370306</v>
+        <v>-0.678314662396</v>
       </c>
       <c r="C85" s="49">
         <f t="shared" si="4"/>
@@ -19233,7 +19246,7 @@
       </c>
       <c r="B86" s="49">
         <f t="shared" si="3"/>
-        <v>-0.861620869308</v>
+        <v>-0.862323104188</v>
       </c>
       <c r="C86" s="49">
         <f t="shared" si="4"/>
@@ -19246,7 +19259,7 @@
       </c>
       <c r="B87" s="49">
         <f t="shared" si="3"/>
-        <v>-1.0938670348</v>
+        <v>-1.094754114774</v>
       </c>
       <c r="C87" s="49">
         <f t="shared" si="4"/>
@@ -19259,7 +19272,7 @@
       </c>
       <c r="B88" s="49">
         <f t="shared" si="3"/>
-        <v>-1.387929812121</v>
+        <v>-1.389051363861</v>
       </c>
       <c r="C88" s="49">
         <f t="shared" si="4"/>
@@ -19272,7 +19285,7 @@
       </c>
       <c r="B89" s="49">
         <f t="shared" si="3"/>
-        <v>-1.761187762627</v>
+        <v>-1.762607295089</v>
       </c>
       <c r="C89" s="49">
         <f t="shared" si="4"/>
@@ -19285,7 +19298,7 @@
       </c>
       <c r="B90" s="49">
         <f t="shared" si="3"/>
-        <v>-2.23626349732</v>
+        <v>-2.238062600223</v>
       </c>
       <c r="C90" s="49">
         <f t="shared" si="4"/>
@@ -19298,7 +19311,7 @@
       </c>
       <c r="B91" s="49">
         <f t="shared" si="3"/>
-        <v>-2.842822195742</v>
+        <v>-2.845106178424</v>
       </c>
       <c r="C91" s="49">
         <f t="shared" si="4"/>
@@ -19311,7 +19324,7 @@
       </c>
       <c r="B92" s="49">
         <f t="shared" si="3"/>
-        <v>-3.620094577901</v>
+        <v>-3.623000128118</v>
       </c>
       <c r="C92" s="49">
         <f t="shared" si="4"/>
@@ -19324,7 +19337,7 @@
       </c>
       <c r="B93" s="49">
         <f t="shared" si="3"/>
-        <v>-4.620462586028</v>
+        <v>-4.624168299219</v>
       </c>
       <c r="C93" s="49">
         <f t="shared" si="4"/>
@@ -19337,7 +19350,7 @@
       </c>
       <c r="B94" s="49">
         <f t="shared" si="3"/>
-        <v>-5.914622025451</v>
+        <v>-5.919363066712</v>
       </c>
       <c r="C94" s="49">
         <f t="shared" si="4"/>
@@ -19350,7 +19363,7 @@
       </c>
       <c r="B95" s="49">
         <f t="shared" si="3"/>
-        <v>-7.599109637773</v>
+        <v>-7.605198429237</v>
       </c>
       <c r="C95" s="49">
         <f t="shared" si="4"/>
@@ -19363,7 +19376,7 @@
       </c>
       <c r="B96" s="49">
         <f t="shared" si="3"/>
-        <v>-9.807407915847</v>
+        <v>-9.815263713325</v>
       </c>
       <c r="C96" s="49">
         <f t="shared" si="4"/>
@@ -19376,7 +19389,7 @@
       </c>
       <c r="B97" s="49">
         <f t="shared" si="3"/>
-        <v>-12.72650680719</v>
+        <v>-12.73669853406</v>
       </c>
       <c r="C97" s="49">
         <f t="shared" si="4"/>
@@ -19389,7 +19402,7 @@
       </c>
       <c r="B98" s="49">
         <f t="shared" si="3"/>
-        <v>-16.621845301131</v>
+        <v>-16.635154346949</v>
       </c>
       <c r="C98" s="49">
         <f t="shared" si="4"/>
@@ -19402,7 +19415,7 @@
       </c>
       <c r="B99" s="49">
         <f t="shared" si="3"/>
-        <v>-21.875195872484</v>
+        <v>-21.892709216041</v>
       </c>
       <c r="C99" s="49">
         <f t="shared" si="4"/>
@@ -19415,7 +19428,7 @@
       </c>
       <c r="B100" s="49">
         <f t="shared" si="3"/>
-        <v>-29.042635799684</v>
+        <v>-29.065885534343</v>
       </c>
       <c r="C100" s="49">
         <f>0</f>
@@ -19455,7 +19468,7 @@
       </c>
       <c r="D103" s="119">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
-        <v>6.360227804438</v>
+        <v>6.359946204531</v>
       </c>
       <c r="E103" s="138" t="s">
         <v>1670</v>
@@ -19476,7 +19489,7 @@
       </c>
       <c r="D104" s="119">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
-        <v>0.884605723802</v>
+        <v>0.884671895747</v>
       </c>
       <c r="E104" s="138" t="s">
         <v>1968</v>
@@ -19523,9 +19536,9 @@
         <f>Iappc/(2*Fcc)*M_HOCl*3600/VLc</f>
         <v>371.244905447914</v>
       </c>
-      <c r="E107" s="138" t="e">
-        <f>"Naïve FE=1 upper bound (all anode current → Cl₂). Superseded by the mass-transport-limited chlorine current I_Cl (D133) and the production rate P_HOCl (D134). Kept only to show the overstatement ("&amp;TEXT(bleach_rate/(P_HOCl*M_HOCl*3600),"0")&amp;"× at the current operating point)."</f>
-        <v>#DIV/0!</v>
+      <c r="E107" s="111" t="str">
+        <f>IF(P_HOCl&gt;0,"Naive FE=1 ceiling; overstates operative production by "&amp;TEXT(bleach_rate/(P_HOCl*M_HOCl*3600),"0")&amp;" times","No chlorine production at the selected chloride inventory")</f>
+        <v>No chlorine production at the selected chloride inventory</v>
       </c>
       <c r="G107" s="53" t="s">
         <v>917</v>
@@ -19886,7 +19899,7 @@
       </c>
       <c r="D138" s="119">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
-        <v>2.588026171876e-05</v>
+        <v>2.586351659465e-05</v>
       </c>
       <c r="E138" s="138" t="s">
         <v>1001</v>
@@ -19972,12 +19985,14 @@
       <c r="C143" s="20" t="s">
         <v>990</v>
       </c>
-      <c r="D143" s="119">
-        <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl*3600)/(1+k_Cl_turn*tau_NH2Cl*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
+      <c r="D143" s="111">
+        <f>Cl_bound*M_HOCl</f>
         <v>0.0</v>
       </c>
-      <c r="E143" s="138" t="s">
-        <v>1972</v>
+      <c r="E143" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steady combined chlorine from D311, on HOCl-equivalent mass basis; both the chloride transport/recycling limit and the actual current limit apply.</t>
+        </is>
       </c>
     </row>
     <row r="144" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -20163,8 +20178,8 @@
       <c r="C154" s="20" t="s">
         <v>1106</v>
       </c>
-      <c r="D154" s="119">
-        <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl_lo*3600)/(1+k_Cl_turn*tau_NH2Cl_lo*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
+      <c r="D154" s="111">
+        <f>MIN(pH_Cl*k_Cl_turn*tau_NH2Cl_lo*3600/(1+k_Cl_turn*tau_NH2Cl_lo*3600),I_Cl_FE/(n_e_Cl*Fcc*VLc)*tau_NH2Cl_lo*3600,pH_NT)*M_HOCl</f>
         <v>0.0</v>
       </c>
       <c r="E154" s="138" t="s">
@@ -20181,8 +20196,8 @@
       <c r="C155" s="20" t="s">
         <v>1109</v>
       </c>
-      <c r="D155" s="119">
-        <f>MIN(Cl_pool_mgL*(k_Cl_turn*tau_NH2Cl_hi*3600)/(1+k_Cl_turn*tau_NH2Cl_hi*3600),cl_per_N*NH3_N*M_HOCl/M_Cl2)</f>
+      <c r="D155" s="111">
+        <f>MIN(pH_Cl*k_Cl_turn*tau_NH2Cl_hi*3600/(1+k_Cl_turn*tau_NH2Cl_hi*3600),I_Cl_FE/(n_e_Cl*Fcc*VLc)*tau_NH2Cl_hi*3600,pH_NT)*M_HOCl</f>
         <v>0.0</v>
       </c>
       <c r="E155" s="138" t="s">
@@ -20551,8 +20566,10 @@
       <c r="D178" s="116">
         <v>0.78</v>
       </c>
-      <c r="E178" s="57" t="s">
-        <v>1366</v>
+      <c r="E178" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estimate anchored near I=0.1 M, not calibrated for AMYBO03 at about 0.2 M. Retained 0.78 pending conductivity measurement; sweep 0.66–0.90 is illustrative, not a validated uncertainty bound.</t>
+        </is>
       </c>
     </row>
     <row r="179" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -20985,7 +21002,7 @@
       </c>
       <c r="D206" s="111">
         <f>E0_OER-nernst_slope*pH_meas</f>
-        <v>0.838743761258</v>
+        <v>0.838760699902</v>
       </c>
       <c r="E206" s="74" t="s">
         <v>1438</v>
@@ -21003,7 +21020,7 @@
       </c>
       <c r="D207" s="111">
         <f>E0_HER-nernst_slope*pH_meas</f>
-        <v>-0.390256238742</v>
+        <v>-0.390239300098</v>
       </c>
       <c r="E207" s="74" t="s">
         <v>1441</v>
@@ -21019,9 +21036,9 @@
       <c r="C208" s="20" t="s">
         <v>1423</v>
       </c>
-      <c r="D208" s="111">
-        <f>E0_Cl2+nernst_slope*(-LOG10(MAX(pH_Cl,Cl_floor_molL)))</f>
-        <v>2.079817482095</v>
+      <c r="D208" s="111" t="e">
+        <f>IF(pH_Cl&gt;0,E0_Cl2+nernst_slope*(-LOG10(MAX(gamma_1*pH_Cl*Cl_free_frac,Cl_floor_molL))),NA())</f>
+        <v>#N/A</v>
       </c>
       <c r="E208" s="51" t="s">
         <v>1443</v>
@@ -21037,12 +21054,14 @@
       <c r="C209" s="20" t="s">
         <v>1445</v>
       </c>
-      <c r="D209" s="111">
+      <c r="D209" s="111" t="e">
         <f>E_HOCl_Cl-E_anode_op</f>
-        <v>-0.30390069301</v>
-      </c>
-      <c r="E209" s="51" t="s">
-        <v>1980</v>
+        <v>#N/A</v>
+      </c>
+      <c r="E209" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not applicable (#N/A) without chloride. Otherwise HOCl/Cl- couple minus operating anode potential; chloride uses free-ion activity, not total analytical concentration.</t>
+        </is>
       </c>
     </row>
     <row r="210" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -21057,7 +21076,7 @@
       </c>
       <c r="D210" s="111">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
-        <v>0.304743761258</v>
+        <v>0.304760699902</v>
       </c>
       <c r="E210" s="51" t="s">
         <v>1448</v>
@@ -21075,7 +21094,7 @@
       </c>
       <c r="D211" s="111">
         <f>E_anode_op-E0_Cu</f>
-        <v>1.248872573638</v>
+        <v>1.248889512283</v>
       </c>
       <c r="E211" s="51" t="s">
         <v>1451</v>
@@ -21133,7 +21152,7 @@
       </c>
       <c r="D216" s="111">
         <f>Fcc*((km_HPO4/100)*HPO4_op+(km_HCO3/100)*HCO3_op)*1000/10</f>
-        <v>16.462465768267</v>
+        <v>16.462762858095</v>
       </c>
       <c r="E216" s="51" t="s">
         <v>1984</v>
@@ -21169,7 +21188,7 @@
       </c>
       <c r="D218" s="111">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>0.199715551957</v>
+        <v>0.199711947856</v>
       </c>
       <c r="E218" s="51" t="s">
         <v>1464</v>
@@ -21205,7 +21224,7 @@
       </c>
       <c r="D220" s="111">
         <f>pH_op-LOG10(gamma_1)</f>
-        <v>6.487893381735</v>
+        <v>6.487611781829</v>
       </c>
       <c r="E220" s="51" t="s">
         <v>1470</v>
@@ -21512,7 +21531,7 @@
       </c>
       <c r="D252" s="111">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
-        <v>0.049844265613</v>
+        <v>0.049851828253</v>
       </c>
       <c r="E252" s="51" t="s">
         <v>2022</v>
@@ -21530,7 +21549,7 @@
       </c>
       <c r="D253" s="111">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
-        <v>0.019464016532</v>
+        <v>0.019455490571</v>
       </c>
       <c r="E253" s="51" t="s">
         <v>2025</v>
@@ -21584,7 +21603,7 @@
       </c>
       <c r="D256" s="111">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
-        <v>1.590772573638</v>
+        <v>1.590789512283</v>
       </c>
       <c r="E256" s="51" t="s">
         <v>2034</v>
@@ -21617,9 +21636,9 @@
       <c r="C258" s="20" t="s">
         <v>1423</v>
       </c>
-      <c r="D258" s="111">
-        <f>E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,0.000000000001))-pH_meas-LOG10(MAX(pH_Cl,0.000000000001)))</f>
-        <v>1.286871880629</v>
+      <c r="D258" s="111" t="e">
+        <f>IF(pH_Cl&gt;0,E0_HOCl+nernst_slope/2*(LOG10(MAX(HOCl_ss*f_local,Cl_floor_molL))-pH_meas-LOG10(MAX(gamma_1*pH_Cl*Cl_free_frac,Cl_floor_molL))),NA())</f>
+        <v>#N/A</v>
       </c>
       <c r="E258" s="51" t="s">
         <v>2040</v>
@@ -21802,8 +21821,8 @@
         <v>111</v>
       </c>
       <c r="D278" s="111">
-        <f>1/(1+k_Cl_turn*tau_NH2Cl*3600)</f>
-        <v>0.391224738169</v>
+        <f>IF(pH_Cl&gt;0,MAX(0,1-Cl_bound/pH_Cl),1)</f>
+        <v>1.0</v>
       </c>
       <c r="E278" s="51" t="s">
         <v>2070</v>
@@ -21861,7 +21880,7 @@
         <v>1842</v>
       </c>
       <c r="D291" s="130">
-        <v>6.09</v>
+        <v>6.35994620453</v>
       </c>
       <c r="E291" s="34" t="s">
         <v>2076</v>
@@ -21879,7 +21898,7 @@
       </c>
       <c r="D292" s="111">
         <f>10^-pH_ref_DIC</f>
-        <v>8.128305161641e-07</v>
+        <v>4.365699062148e-07</v>
       </c>
       <c r="E292" s="60" t="s">
         <v>2079</v>
@@ -21897,7 +21916,7 @@
       </c>
       <c r="D293" s="111">
         <f>Ka1c_c/h_ref_DIC</f>
-        <v>1.047442997582</v>
+        <v>1.950188550006</v>
       </c>
       <c r="E293" s="60" t="s">
         <v>2082</v>
@@ -21915,7 +21934,7 @@
       </c>
       <c r="D294" s="111">
         <f>(pH_SID+pH_NT*h_ref_DIC/(h_ref_DIC+KaN_c)+h_ref_DIC-(pH_PT*Ka1p_c*h_ref_DIC^2+2*pH_PT*Ka1p_c*Ka2p_c*h_ref_DIC+3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/(h_ref_DIC^3+Ka1p_c*h_ref_DIC^2+Ka1p_c*Ka2p_c*h_ref_DIC+Ka1p_c*Ka2p_c*Ka3p_c)-Kw_c/h_ref_DIC)/(1+2*Ka2c_c/h_ref_DIC)</f>
-        <v>0.057385332923</v>
+        <v>0.050195278773</v>
       </c>
       <c r="E294" s="60" t="s">
         <v>2085</v>
@@ -21933,7 +21952,7 @@
       </c>
       <c r="D295" s="111">
         <f>LN(10)*(pH_PT*Ka1p_c*h_ref_DIC/(Ka1p_c+h_ref_DIC)^2+pH_PT*Ka2p_c*h_ref_DIC/(Ka2p_c+h_ref_DIC)^2+pH_NT*KaN_c*h_ref_DIC/(KaN_c+h_ref_DIC)^2+h_ref_DIC+Kw_c/h_ref_DIC)</f>
-        <v>0.022552516262</v>
+        <v>0.030338975539</v>
       </c>
       <c r="E295" s="60" t="s">
         <v>2089</v>
@@ -21951,7 +21970,7 @@
       </c>
       <c r="D296" s="111">
         <f>1+r_HCO3_ref*beta_nonC/(beta_nonC+LN(10)*HCO3_ref)</f>
-        <v>1.152711317868</v>
+        <v>1.405479604448</v>
       </c>
       <c r="E296" s="51" t="s">
         <v>2092</v>
@@ -22049,7 +22068,7 @@
       </c>
       <c r="D305" s="111">
         <f>pH_SID + pH_NT*(10^-alk_pH_target_c)/((10^-alk_pH_target_c)+KaN_c) + (10^-alk_pH_target_c) - (pH_PT*Ka1p_c*(10^-alk_pH_target_c)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-alk_pH_target_c) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-alk_pH_target_c)^3 + Ka1p_c*(10^-alk_pH_target_c)^2 + Ka1p_c*Ka2p_c*(10^-alk_pH_target_c) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-alk_pH_target_c) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-alk_pH_target_c)^2 - Kw_c/(10^-alk_pH_target_c)</f>
-        <v>-0.00143770448</v>
+        <v>-0.001478762218</v>
       </c>
       <c r="E305" s="60" t="s">
         <v>2734</v>
@@ -22067,7 +22086,7 @@
       </c>
       <c r="D306" s="111">
         <f>MAX(0,-alk_resid_t)</f>
-        <v>0.00143770448</v>
+        <v>0.001478762218</v>
       </c>
       <c r="E306" s="60" t="s">
         <v>2737</v>
@@ -22102,10 +22121,113 @@
       </c>
       <c r="D308" s="111">
         <f>alk_needed*M_NaHCO3</f>
-        <v>0.120777240215</v>
+        <v>0.124226377682</v>
       </c>
       <c r="E308" s="60" t="s">
         <v>2743</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC reference tolerance</t>
+        </is>
+      </c>
+      <c r="B309" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC_ref_tol</t>
+        </is>
+      </c>
+      <c r="C309" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D309" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="E309" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Validity criterion from the DIC linearisation: refresh the reference if solved concentration-scale pH moves by more than this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC reference validity</t>
+        </is>
+      </c>
+      <c r="B310" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DIC_ref_check</t>
+        </is>
+      </c>
+      <c r="C310" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D310" s="111" t="str">
+        <f>IF(ABS(pH_ref_DIC-pH_op)&lt;=DIC_ref_tol,"OK","REFRESH DIC reference pH")</f>
+        <v>OK</v>
+      </c>
+      <c r="E310" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the linearisation at the actual schedule. D291 must be iterated after input changes; no circular reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steady combined chlorine inventory</t>
+        </is>
+      </c>
+      <c r="B311" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cl_bound</t>
+        </is>
+      </c>
+      <c r="C311" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D311" s="111">
+        <f>MIN(pH_Cl*k_Cl_turn*tau_NH2Cl*3600/(1+k_Cl_turn*tau_NH2Cl*3600),I_Cl_FE/(n_e_Cl*Fcc*VLc)*tau_NH2Cl*3600,pH_NT)</f>
+        <v>0.0</v>
+      </c>
+      <c r="E311" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steady B=min(C*k*tau/(1+k*tau), pmax*tau, nitrogen). Free chloride=C-B; zero current gives zero combined chlorine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chloramine approximation check</t>
+        </is>
+      </c>
+      <c r="B312" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cl_model_check</t>
+        </is>
+      </c>
+      <c r="C312" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D312" s="111" t="str">
+        <f>IF(AND(pH_Cl&gt;0,Cl_bound&gt;=pH_NT,P_HOCl&gt;pH_NT/(tau_NH2Cl*3600)),"UNSUPPORTED – nitrogen capacity exhausted","OK")</f>
+        <v>OK</v>
+      </c>
+      <c r="E312" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The simple chloramine steady state does not resolve breakpoint chemistry after ammonium is exhausted.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -22917,12 +23039,14 @@
       <c r="C44" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D44" s="41" t="str">
-        <f>IF(AND(y_H2_end_b&gt;=H2_LFL,y_O2_end_b&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse – until uptake starts, sparge every ≤"&amp;TEXT(spg_int_H2safe_saw,"0.0")&amp;" min or sweep ≥"&amp;TEXT(N2_sweep_H2safe,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin at every point of the cycle (lag): H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;", O₂ "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse ("&amp;TEXT(y_H2_hs_lag,"0%")&amp;" / "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.4 min or sweep ≥0.9 mL/min N₂; vent to a hood; no ignition sources</v>
-      </c>
-      <c r="E44" s="54" t="s">
-        <v>2107</v>
+      <c r="D44" s="111" t="str">
+        <f>IF(AND(y_H2_end_b&gt;=H2_LFL,y_O2_end_b&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse – until uptake starts, "&amp;IF(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res)*60&gt;spg_dur_opt_b,"sparge every ≤"&amp;TEXT(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res),"0.0")&amp;" min or ","interval remedy unavailable; ")&amp;"sweep ≥"&amp;TEXT(FLOOR(N2_sweep_H2safe,remedy_res)+remedy_res,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin at every point of the cycle (lag): H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;", O₂ "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse ("&amp;TEXT(y_H2_hs_lag,"0%")&amp;" / "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean)")</f>
+        <v>FLAMMABLE HEADSPACE (lag): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+      </c>
+      <c r="E44" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pre-pulse lag hazard check. Remedy assumes the actual commanded pulse; displayed upper interval is rounded strictly down and minimum sweep strictly up. Bench safety verification remains required.</t>
+        </is>
       </c>
       <c r="F44" s="75" t="s">
         <v>2108</v>
@@ -23310,7 +23434,7 @@
       </c>
       <c r="D76" s="120">
         <f>'Mass Transfer'!$D$100</f>
-        <v>0.0008457851714831</v>
+        <v>0.0008519434760509</v>
       </c>
       <c r="E76" s="140" t="s">
         <v>2129</v>
@@ -23433,7 +23557,7 @@
       </c>
       <c r="D83" s="41">
         <f>H2_src_l_b+O2_src_l_b</f>
-        <v>0.0001431962391673</v>
+        <v>0.0001447785865665</v>
       </c>
       <c r="E83" s="53" t="s">
         <v>2151</v>
@@ -23451,7 +23575,7 @@
       </c>
       <c r="D84" s="41">
         <f>H2_src_l_b/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.093395436531</v>
+        <v>0.093689942909</v>
       </c>
       <c r="E84" s="53" t="s">
         <v>2154</v>
@@ -23469,7 +23593,7 @@
       </c>
       <c r="D85" s="41">
         <f>(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
-        <v>0.053679883871</v>
+        <v>0.053815126441</v>
       </c>
       <c r="E85" s="53" t="s">
         <v>2157</v>
@@ -23487,7 +23611,7 @@
       </c>
       <c r="D86" s="41">
         <f>MAX(0,MIN(H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
-        <v>0.003287756237</v>
+        <v>0.003321398663</v>
       </c>
       <c r="E86" s="53" t="s">
         <v>2160</v>
@@ -23505,7 +23629,7 @@
       </c>
       <c r="D87" s="41">
         <f>IF(duty_H2safe&gt;0,spg_dur_b/(60*duty_H2safe),NA())</f>
-        <v>3.976942496757</v>
+        <v>3.936660071253</v>
       </c>
       <c r="E87" s="53" t="s">
         <v>2163</v>
@@ -23523,7 +23647,7 @@
       </c>
       <c r="D88" s="41">
         <f>MAX(0,H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b)/3600*R_gas_b*T_K/P_atm*1000000*60</f>
-        <v>0.918020179803</v>
+        <v>0.928010297432</v>
       </c>
       <c r="E88" s="53" t="s">
         <v>2166</v>
@@ -23539,12 +23663,14 @@
       <c r="C89" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D89" s="120">
-        <f>'Mass Transfer'!$D$90</f>
-        <v>0.674076519917</v>
-      </c>
-      <c r="E89" s="140" t="s">
-        <v>2169</v>
+      <c r="D89" s="111">
+        <f>'Mass Transfer'!spg_dur</f>
+        <v>0.65</v>
+      </c>
+      <c r="E89" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actual commanded pulse (Mass Transfer spg_dur), also the pulse required for the interval remedy.</t>
+        </is>
       </c>
     </row>
     <row r="90" spans="1:5" ht="48" x14ac:dyDescent="0.2">
@@ -23559,7 +23685,7 @@
       </c>
       <c r="D90" s="41">
         <f>IF(H2_src_l_b&gt;H2_LFL*F_gap_l_b,n_hs_gas_b/F_gap_l_b*LN((1-H2_LFL*F_gap_l_b/(H2_src_l_b)*flush_ret_opt_b)/(1-H2_LFL*F_gap_l_b/(H2_src_l_b)))*60,"none needed")</f>
-        <v>1.754295192528</v>
+        <v>1.673926467146</v>
       </c>
       <c r="E90" s="53" t="s">
         <v>2172</v>
@@ -23577,7 +23703,7 @@
       </c>
       <c r="D91" s="41">
         <f>IF(O2_src_l_b+y_O2_air_b*F_vent_ex_b&gt;O2_LOC_H2*LOC_margin*F_gap_l_b,n_hs_gas_b/F_gap_l_b*LN((1-O2_LOC_H2*LOC_margin*F_gap_l_b/(O2_src_l_b+y_O2_air_b*F_vent_ex_b)*flush_ret_opt_b)/(1-O2_LOC_H2*LOC_margin*F_gap_l_b/(O2_src_l_b+y_O2_air_b*F_vent_ex_b)))*60,"none needed")</f>
-        <v>2.428028403314</v>
+        <v>2.318132447064</v>
       </c>
       <c r="E91" s="53" t="s">
         <v>2175</v>
@@ -23595,7 +23721,7 @@
       </c>
       <c r="D92" s="41">
         <f>IF(OR(ISTEXT(t_gap_H2_LFL),ISTEXT(t_gap_O2_LOC)),"any interval",MAX(t_gap_H2_LFL,t_gap_O2_LOC)+spg_dur_opt_b/60)</f>
-        <v>2.439263011979</v>
+        <v>2.328965780397</v>
       </c>
       <c r="E92" s="53" t="s">
         <v>2178</v>
@@ -23636,7 +23762,7 @@
       </c>
       <c r="D97" s="41">
         <f>'Mass Transfer'!$D$198</f>
-        <v>25.397988261812</v>
+        <v>25.441759810194</v>
       </c>
       <c r="E97" s="51" t="s">
         <v>2185</v>
@@ -23654,7 +23780,7 @@
       </c>
       <c r="D98" s="41">
         <f>C_cycle_start_b*1000/Km_CO2</f>
-        <v>507.959765236247</v>
+        <v>508.83519620388</v>
       </c>
       <c r="E98" s="53" t="s">
         <v>2188</v>
@@ -23713,7 +23839,7 @@
       </c>
       <c r="D113" s="120">
         <f>'Mass Transfer'!$D$314</f>
-        <v>9.574538813904e-05</v>
+        <v>9.67725259245e-05</v>
       </c>
       <c r="E113" s="140" t="s">
         <v>2198</v>
@@ -23731,7 +23857,7 @@
       </c>
       <c r="D114" s="120">
         <f>'Mass Transfer'!$D$388</f>
-        <v>0.145040740595</v>
+        <v>0.146149332991</v>
       </c>
       <c r="E114" s="140" t="s">
         <v>2201</v>
@@ -23749,7 +23875,7 @@
       </c>
       <c r="D115" s="120">
         <f>'Mass Transfer'!$D$310</f>
-        <v>4.745085102827e-05</v>
+        <v>4.800606064204e-05</v>
       </c>
       <c r="E115" s="140" t="s">
         <v>2204</v>
@@ -23767,7 +23893,7 @@
       </c>
       <c r="D116" s="120">
         <f>'Mass Transfer'!$D$353</f>
-        <v>0.0001793761393403</v>
+        <v>0.0001809584867395</v>
       </c>
       <c r="E116" s="140" t="s">
         <v>2207</v>
@@ -23785,7 +23911,7 @@
       </c>
       <c r="D117" s="120">
         <f>'Mass Transfer'!$D$150</f>
-        <v>0.0001050193341601</v>
+        <v>0.0001006282146096</v>
       </c>
       <c r="E117" s="140" t="s">
         <v>2210</v>
@@ -23801,12 +23927,14 @@
       <c r="C118" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="D118" s="120">
-        <f>'Mass Transfer'!$D$321</f>
-        <v>0.367879441171</v>
-      </c>
-      <c r="E118" s="140" t="s">
-        <v>2213</v>
+      <c r="D118" s="111">
+        <f>'Mass Transfer'!flush_ret</f>
+        <v>0.363594260592</v>
+      </c>
+      <c r="E118" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retention of the actual commanded pulse, not the ideal design pulse.</t>
+        </is>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
@@ -23821,15 +23949,35 @@
       </c>
       <c r="D119" s="120">
         <f>'Mass Transfer'!$D$358</f>
-        <v>0.08336349613</v>
+        <v>0.083947589143</v>
       </c>
       <c r="E119" s="140" t="s">
         <v>2216</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A120" s="6" t="s">
-        <v>2217</v>
+    <row r="120" x14ac:dyDescent="0.2">
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remedy display resolution</t>
+        </is>
+      </c>
+      <c r="B120" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">remedy_res</t>
+        </is>
+      </c>
+      <c r="C120" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D120" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="E120" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Display increment: min for interval, mL/min for sweep. Bounds are rounded strictly in the protective direction.</t>
+        </is>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
@@ -24886,7 +25034,7 @@
       </c>
       <c r="D53" s="49">
         <f>kLa_sparge*duty</f>
-        <v>6.303155783939e-05</v>
+        <v>6.315438152323e-05</v>
       </c>
       <c r="E53" s="89" t="s">
         <v>581</v>
@@ -24924,7 +25072,7 @@
       </c>
       <c r="D55" s="41">
         <f>strip_sparge*duty</f>
-        <v>1.071291719445e-06</v>
+        <v>1.073379245122e-06</v>
       </c>
       <c r="E55" s="57" t="s">
         <v>587</v>
@@ -24943,7 +25091,7 @@
       </c>
       <c r="D56" s="39">
         <f>IF(O2_excess&gt;0,strip_avg/O2_excess,NA())</f>
-        <v>0.063386460696</v>
+        <v>0.063509975945</v>
       </c>
       <c r="E56" s="57" t="s">
         <v>590</v>
@@ -25110,8 +25258,8 @@
       <c r="C65" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D65" s="41">
-        <f>O2_ceil_C*(V_charge/1000000)/O2_excess*60</f>
+      <c r="D65" s="111">
+        <f>IF(O2_excess&gt;0,O2_ceil_C*(V_charge/1000000)/O2_excess*60,"never (source &lt;= 0)")</f>
         <v>16.760509303688</v>
       </c>
       <c r="E65" s="74" t="s">
@@ -25131,7 +25279,7 @@
       </c>
       <c r="D66" s="41">
         <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_C*(V_charge/1000000)/(O2_excess-strip_avg)*60,"never (strip ≥ source)")</f>
-        <v>17.894797160561</v>
+        <v>17.897157335559</v>
       </c>
       <c r="E66" s="74" t="s">
         <v>2233</v>
@@ -25318,7 +25466,7 @@
       </c>
       <c r="D77" s="41">
         <f>headspace_V*spg_int/V_pulse</f>
-        <v>7.450071557247</v>
+        <v>7.396218442584</v>
       </c>
       <c r="E77" s="74" t="s">
         <v>2236</v>
@@ -25337,7 +25485,7 @@
       </c>
       <c r="D78" s="41">
         <f>IF(O2_excess&gt;0,(strip_avg+surf_strip)/O2_excess,NA())</f>
-        <v>7.746944444342</v>
+        <v>7.747067959591</v>
       </c>
       <c r="E78" s="90" t="s">
         <v>640</v>
@@ -25580,7 +25728,7 @@
       </c>
       <c r="D91" s="41">
         <f>IF(ISNA(F_vent_ex+O2_src_sched),NA(),IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max)))</f>
-        <v>7.450071557247</v>
+        <v>7.398866407059</v>
       </c>
       <c r="E91" s="129" t="s">
         <v>2243</v>
@@ -25599,7 +25747,7 @@
       </c>
       <c r="D92" s="41">
         <f>spg_int_opt*60</f>
-        <v>447.004293434794</v>
+        <v>443.931984423528</v>
       </c>
       <c r="E92" s="129" t="s">
         <v>672</v>
@@ -25618,7 +25766,7 @@
       </c>
       <c r="D93" s="41">
         <f>spg_dur_eq_opt/(spg_int_opt*60)</f>
-        <v>0.001755045894</v>
+        <v>0.001767191996</v>
       </c>
       <c r="E93" s="74" t="s">
         <v>2245</v>
@@ -25751,7 +25899,7 @@
       </c>
       <c r="D100" s="25">
         <f>CO2_pulse*pulses_h</f>
-        <v>0.0008457851714831</v>
+        <v>0.0008519434760509</v>
       </c>
       <c r="E100" s="102" t="s">
         <v>688</v>
@@ -25827,8 +25975,10 @@
         <f>P_atm*(Q_CO2/1000000/60)/(R_gas*T_K)</f>
         <v>0.00013386563064</v>
       </c>
-      <c r="E104" s="102" t="s">
-        <v>688</v>
+      <c r="E104" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dry CO2-equivalent flow at P_atm and T_K. Calibration collection humidity/temperature remain unrecorded; verify before using absolute molar delivery. This convention is distinct from saturated headspace inventory.</t>
+        </is>
       </c>
       <c r="F104" s="21"/>
     </row>
@@ -25844,7 +25994,7 @@
       </c>
       <c r="D105" s="25">
         <f>spg_dur/(spg_int*60)</f>
-        <v>0.001507986679</v>
+        <v>0.001510925151</v>
       </c>
       <c r="E105" s="102" t="s">
         <v>688</v>
@@ -25891,7 +26041,7 @@
       </c>
       <c r="D108" s="25">
         <f>DO_avg_sched*M_O2</f>
-        <v>2.27518163832</v>
+        <v>2.270165488391</v>
       </c>
       <c r="E108" s="102" t="s">
         <v>2248</v>
@@ -25966,7 +26116,7 @@
       <c r="C113" s="21"/>
       <c r="D113" s="25" t="str">
         <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) the cycle-mean DO would be ≈"&amp;TEXT(DO_at_carbon*M_O2,"0")&amp;" mg/L, "&amp;IF(DO_at_carbon&gt;O2_ceil_C,"above the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L inhibition ceiling","against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")&amp;" (peaks higher)")</f>
-        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈13 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
+        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈14 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E113" s="59" t="s">
         <v>2249</v>
@@ -26095,9 +26245,9 @@
       <c r="C121" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D121" s="25">
-        <f>IF(AND(ISNUMBER(override_spg_dur_s),override_spg_dur_s&gt;0),override_spg_dur_s,IF(sched_mode="Manual",spg_dur_man,IF(sched_mode="Optimal",spg_dur_opt,NA())))</f>
-        <v>0.674076519917</v>
+      <c r="D121" s="111">
+        <f>IF(AND(ISNUMBER(override_spg_dur_s),override_spg_dur_s&gt;0),override_spg_dur_s,IF(sched_mode="Manual",spg_dur_man,IF(sched_mode="Optimal",spg_dur_run,NA())))</f>
+        <v>0.65</v>
       </c>
       <c r="E121" s="21"/>
       <c r="F121" s="21"/>
@@ -26112,9 +26262,9 @@
       <c r="C122" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D122" s="25">
-        <f>IF(AND(ISNUMBER(override_spg_int_min),override_spg_int_min&gt;0),override_spg_int_min,IF(sched_mode="Manual",spg_int_man,IF(sched_mode="Optimal",spg_int_opt,NA())))</f>
-        <v>7.450071557247</v>
+      <c r="D122" s="111">
+        <f>IF(AND(ISNUMBER(override_spg_int_min),override_spg_int_min&gt;0),IF(override_spg_int_min*60&gt;spg_dur,override_spg_int_min,NA()),IF(sched_mode="Manual",IF(spg_int_man*60&gt;spg_dur,spg_int_man,NA()),IF(sched_mode="Optimal",spg_int_run,NA())))</f>
+        <v>7.17</v>
       </c>
       <c r="E122" s="21"/>
       <c r="F122" s="21"/>
@@ -26131,7 +26281,7 @@
       </c>
       <c r="D123" s="25">
         <f>P_atm*(V_pulse/1000000)/(R_gas*T_K)</f>
-        <v>0.0001050193341601</v>
+        <v>0.0001018072453881</v>
       </c>
       <c r="E123" s="21" t="s">
         <v>2254</v>
@@ -26150,7 +26300,7 @@
       </c>
       <c r="D124" s="25">
         <f>60/spg_int</f>
-        <v>8.05361392021</v>
+        <v>8.36820083682</v>
       </c>
       <c r="E124" s="21"/>
       <c r="F124" s="21"/>
@@ -26167,7 +26317,7 @@
       </c>
       <c r="D125" s="25">
         <f>pulses_h*24</f>
-        <v>193.286734085035</v>
+        <v>200.836820083682</v>
       </c>
       <c r="E125" s="21"/>
       <c r="F125" s="21"/>
@@ -26184,7 +26334,7 @@
       </c>
       <c r="D126" s="25">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v>49.589627400178</v>
+        <v>49.950697845996</v>
       </c>
       <c r="E126" s="21"/>
       <c r="F126" s="21"/>
@@ -26201,7 +26351,7 @@
       </c>
       <c r="D127" s="25">
         <f>O2_excess/60*spg_int</f>
-        <v>2.098555401519e-06</v>
+        <v>2.019664121784e-06</v>
       </c>
       <c r="E127" s="21"/>
       <c r="F127" s="21"/>
@@ -26218,7 +26368,7 @@
       </c>
       <c r="D128" s="25">
         <f>strip_sparge/3600*spg_dur</f>
-        <v>1.330199994759e-07</v>
+        <v>1.282688197921e-07</v>
       </c>
       <c r="E128" s="21"/>
       <c r="F128" s="21"/>
@@ -26235,7 +26385,7 @@
       </c>
       <c r="D129" s="25">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v>0.063386460696</v>
+        <v>0.063509975945</v>
       </c>
       <c r="E129" s="21"/>
       <c r="F129" s="21"/>
@@ -26305,7 +26455,7 @@
       </c>
       <c r="D133" s="25">
         <f>DO_avg_sched</f>
-        <v>0.071103870189</v>
+        <v>0.070947105706</v>
       </c>
       <c r="E133" s="53" t="s">
         <v>2256</v>
@@ -26324,7 +26474,7 @@
       </c>
       <c r="D134" s="25" t="str">
         <f>IF(ISNA(F_vent_ex+O2_src_sched),"INVALID SELECTOR (Summary D111/D112) – no schedule until both are listed values",IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf")))</f>
-        <v>ESTIMATED kLa — DO-limited interval is 7.5 min; confirm by measuring kL_surf</v>
+        <v>ESTIMATED kLa — DO-limited interval is 7.4 min; confirm by measuring kL_surf</v>
       </c>
       <c r="E134" s="53" t="s">
         <v>2257</v>
@@ -26343,7 +26493,7 @@
       </c>
       <c r="D135" s="25">
         <f>DO_avg_l</f>
-        <v>0.173258075157</v>
+        <v>0.174849986476</v>
       </c>
       <c r="E135" s="53" t="s">
         <v>2259</v>
@@ -26467,7 +26617,7 @@
       </c>
       <c r="D143" s="41">
         <f>F_gap_sched/3600/n_hs_gas</f>
-        <v>9.569640057845e-05</v>
+        <v>9.987231025874e-05</v>
       </c>
       <c r="E143" s="51" t="s">
         <v>2263</v>
@@ -26486,7 +26636,7 @@
       </c>
       <c r="D144" s="41">
         <f>IF(k_vent&gt;0,1/k_vent/60,"none between pulses")</f>
-        <v>174.161897061142</v>
+        <v>166.87975499403</v>
       </c>
       <c r="E144" s="51" t="s">
         <v>2264</v>
@@ -26598,12 +26748,14 @@
       <c r="C150" s="20" t="s">
         <v>732</v>
       </c>
-      <c r="D150" s="41">
-        <f>P_atm*headspace_V_m3/(R_gas*T_K)</f>
-        <v>0.0001050193341601</v>
-      </c>
-      <c r="E150" s="51" t="s">
-        <v>1076</v>
+      <c r="D150" s="111">
+        <f>P_dry*headspace_V_m3/(R_gas*T_K)</f>
+        <v>0.0001006282146096</v>
+      </c>
+      <c r="E150" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dry-gas species inventory above saturated culture: (P_atm - p_sat_w)*V_hs/(R*T). Flush ratios and all species balances use this same inventory.</t>
+        </is>
       </c>
       <c r="F150" s="21"/>
     </row>
@@ -26619,7 +26771,7 @@
       </c>
       <c r="D151" s="41">
         <f>spg_dur</f>
-        <v>0.674076519917</v>
+        <v>0.65</v>
       </c>
       <c r="E151" s="51" t="s">
         <v>1077</v>
@@ -26638,7 +26790,7 @@
       </c>
       <c r="D152" s="41">
         <f>MAX(0,spg_int*60-spg_dur)</f>
-        <v>446.330216914877</v>
+        <v>429.55</v>
       </c>
       <c r="E152" s="51" t="s">
         <v>1078</v>
@@ -26729,7 +26881,7 @@
       </c>
       <c r="D162" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,CO2_cyc_avg_new))/1000</f>
-        <v>0.025542123443</v>
+        <v>0.025562568426</v>
       </c>
       <c r="E162" s="51" t="s">
         <v>1661</v>
@@ -27003,7 +27155,7 @@
       </c>
       <c r="D181" s="111">
         <f>O2_src_l/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.115007545523</v>
+        <v>0.116353217804</v>
       </c>
       <c r="E181" s="51" t="s">
         <v>2273</v>
@@ -27057,7 +27209,7 @@
       </c>
       <c r="D184" s="111">
         <f>IF(ISNUMBER(y_O2_star),MAX(0,((O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_vent_ex-O2_src_sched-H2_src_sched+CO2_fix_sched)/CO2_rate_full),NA())</f>
-        <v>0.001755045894</v>
+        <v>0.001767191996</v>
       </c>
       <c r="E184" s="51" t="s">
         <v>2274</v>
@@ -27075,7 +27227,7 @@
       </c>
       <c r="D185" s="111">
         <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_eq_opt/(60*duty_DO),spg_int_carbon),NA())</f>
-        <v>7.450071557247</v>
+        <v>7.398866407059</v>
       </c>
       <c r="E185" s="51" t="s">
         <v>1630</v>
@@ -27111,7 +27263,7 @@
       </c>
       <c r="D187" s="111">
         <f>IF(O2_sizing_phase=phase_name_1,y_O2_mf_g,IF(O2_sizing_phase=phase_name_2,y_O2_mf_l,NA()))</f>
-        <v>0.027761802038</v>
+        <v>0.027569266375</v>
       </c>
       <c r="E187" s="51" t="s">
         <v>2276</v>
@@ -27129,7 +27281,7 @@
       </c>
       <c r="D188" s="111">
         <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_dry,NA())</f>
-        <v>0.027908265922</v>
+        <v>0.027714714491</v>
       </c>
       <c r="E188" s="51" t="s">
         <v>2277</v>
@@ -27188,7 +27340,7 @@
       </c>
       <c r="D193" s="111">
         <f>V_L_CO2/(V_L_CO2+Vg_CO2)</f>
-        <v>0.828200405029</v>
+        <v>0.854605382181</v>
       </c>
       <c r="E193" s="74" t="s">
         <v>2279</v>
@@ -27206,7 +27358,7 @@
       </c>
       <c r="D194" s="111">
         <f>C_sat_CO2*(1-pool_a)*(1-flush_ret)</f>
-        <v>3.046795495863</v>
+        <v>2.595993924837</v>
       </c>
       <c r="E194" s="74" t="s">
         <v>2281</v>
@@ -27224,7 +27376,7 @@
       </c>
       <c r="D195" s="111">
         <f>k_vent*Vg_CO2/(V_L_CO2+Vg_CO2)</f>
-        <v>1.644060285952e-05</v>
+        <v>1.452089638081e-05</v>
       </c>
       <c r="E195" s="74" t="s">
         <v>2282</v>
@@ -27242,7 +27394,7 @@
       </c>
       <c r="D196" s="111">
         <f>IF(k_vent&gt;0,(kLa_CO2_off*V_L_m3/Vg_CO2)/k_vent,"no turnover between pulses")</f>
-        <v>328.605591411156</v>
+        <v>314.865774372625</v>
       </c>
       <c r="E196" s="51" t="s">
         <v>2283</v>
@@ -27260,7 +27412,7 @@
       </c>
       <c r="D197" s="111">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
-        <v>0.992688919094</v>
+        <v>0.993781961475</v>
       </c>
       <c r="E197" s="74" t="s">
         <v>1654</v>
@@ -27278,7 +27430,7 @@
       </c>
       <c r="D198" s="111">
         <f>(pool_D_gap+pool_b*pool_e)/(1-pool_ret*pool_e)</f>
-        <v>25.397988261812</v>
+        <v>25.441759810194</v>
       </c>
       <c r="E198" s="74" t="s">
         <v>2284</v>
@@ -27296,7 +27448,7 @@
       </c>
       <c r="D199" s="111">
         <f>pool_ret*C_cycle_start+pool_b</f>
-        <v>25.686611606656</v>
+        <v>25.683628481892</v>
       </c>
       <c r="E199" s="74" t="s">
         <v>2285</v>
@@ -27314,7 +27466,7 @@
       </c>
       <c r="D200" s="111">
         <f>C_cycle_peak*pool_phi+pool_D_raw*pool_psi</f>
-        <v>25.542123442712</v>
+        <v>25.562568425791</v>
       </c>
       <c r="E200" s="74" t="s">
         <v>2286</v>
@@ -27554,7 +27706,7 @@
       </c>
       <c r="D232" s="111">
         <f>IF(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,DO_surf_excess+H_O2_T*P_dry*MIN(1,saw_factor*(O2_src_sched+y_O2_air*F_vent_ex)/(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)),DO_surf_excess+H_O2_T*P_dry)</f>
-        <v>0.42061159324</v>
+        <v>0.423131676776</v>
       </c>
       <c r="E232" s="74" t="s">
         <v>2311</v>
@@ -27740,8 +27892,10 @@
         <f>P_atm*(Q_vent_used/1000000/60)/(R_gas*T_K)*3600</f>
         <v>3.617990017297e-05</v>
       </c>
-      <c r="E308" s="53" t="s">
-        <v>2346</v>
+      <c r="E308" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dry-air-equivalent ingress at P_atm and T_K, converted mL/min to mol/h. Flow reference conditions and the actual ingress are unmeasured; not a claim that pressure closure has been measured.</t>
+        </is>
       </c>
     </row>
     <row r="309" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -27774,7 +27928,7 @@
       </c>
       <c r="D310" s="41">
         <f>O2_net_lag_mt</f>
-        <v>4.745085102827e-05</v>
+        <v>4.800606064204e-05</v>
       </c>
       <c r="E310" s="51" t="s">
         <v>2352</v>
@@ -27846,7 +28000,7 @@
       </c>
       <c r="D314" s="41">
         <f>MAX(0,rH2_lag_mt-H2_HOR_mt)</f>
-        <v>9.574538813904e-05</v>
+        <v>9.67725259245e-05</v>
       </c>
       <c r="E314" s="51" t="s">
         <v>2361</v>
@@ -27953,7 +28107,7 @@
       </c>
       <c r="D320" s="41">
         <f>nCO2_rate*spg_dur_eq_opt/n_hs_gas</f>
-        <v>1.0</v>
+        <v>1.043637061112</v>
       </c>
       <c r="E320" s="51" t="s">
         <v>2379</v>
@@ -27971,7 +28125,7 @@
       </c>
       <c r="D321" s="41">
         <f>EXP(-flush_vol_opt)</f>
-        <v>0.367879441171</v>
+        <v>0.352171480635</v>
       </c>
       <c r="E321" s="52" t="s">
         <v>2382</v>
@@ -27989,7 +28143,7 @@
       </c>
       <c r="D322" s="41">
         <f>flush_vol_opt*(1+flush_ret_opt)/(2*(1-flush_ret_opt))</f>
-        <v>1.081976706869</v>
+        <v>1.089158803594</v>
       </c>
       <c r="E322" s="52" t="s">
         <v>2385</v>
@@ -28007,7 +28161,7 @@
       </c>
       <c r="D323" s="41">
         <f>CO2_pulse/n_hs_gas</f>
-        <v>1.0</v>
+        <v>1.011716701753</v>
       </c>
       <c r="E323" s="51" t="s">
         <v>2388</v>
@@ -28025,7 +28179,7 @@
       </c>
       <c r="D324" s="41">
         <f>EXP(-flush_vol)</f>
-        <v>0.367879441171</v>
+        <v>0.363594260592</v>
       </c>
       <c r="E324" s="52" t="s">
         <v>2391</v>
@@ -28043,7 +28197,7 @@
       </c>
       <c r="D325" s="41">
         <f>t_off_CO2/3600</f>
-        <v>0.12398061581</v>
+        <v>0.119319444444</v>
       </c>
       <c r="E325" s="51" t="s">
         <v>2394</v>
@@ -28097,7 +28251,7 @@
       </c>
       <c r="D328" s="41">
         <f>CO2_supply+O2_src_g+H2_src_g-CO2_fix_g</f>
-        <v>0.0008456304393138</v>
+        <v>0.0008517887438816</v>
       </c>
       <c r="E328" s="51" t="s">
         <v>2403</v>
@@ -28115,7 +28269,7 @@
       </c>
       <c r="D329" s="41">
         <f>IF(F_vent_ex+F_hs_net_g&gt;0,S_O2_g/(F_vent_ex+F_hs_net_g),NA())</f>
-        <v>0.027761802038</v>
+        <v>0.027569266375</v>
       </c>
       <c r="E329" s="51" t="s">
         <v>2406</v>
@@ -28169,7 +28323,7 @@
       </c>
       <c r="D332" s="41">
         <f>F_gap_g*t_gap_h/n_hs_gas</f>
-        <v>0.042712195228</v>
+        <v>0.042900150872</v>
       </c>
       <c r="E332" s="51" t="s">
         <v>2415</v>
@@ -28187,7 +28341,7 @@
       </c>
       <c r="D333" s="41">
         <f>IF(x_hs_g&gt;0,(1-EXP(-x_hs_g))/x_hs_g,1)</f>
-        <v>0.978944738478</v>
+        <v>0.97885339998</v>
       </c>
       <c r="E333" s="51" t="s">
         <v>2418</v>
@@ -28205,7 +28359,7 @@
       </c>
       <c r="D334" s="41">
         <f>IF(x_hs_g&gt;0,(x_hs_g-1+EXP(-x_hs_g))/x_hs_g^2,1/2)</f>
-        <v>0.492956669864</v>
+        <v>0.492926005866</v>
       </c>
       <c r="E334" s="51" t="s">
         <v>2421</v>
@@ -28223,7 +28377,7 @@
       </c>
       <c r="D335" s="41">
         <f>S_O2_g*t_gap_h/n_hs_gas</f>
-        <v>0.028900633895</v>
+        <v>0.02902781156</v>
       </c>
       <c r="E335" s="51" t="s">
         <v>2424</v>
@@ -28241,7 +28395,7 @@
       </c>
       <c r="D336" s="41">
         <f>dy_O2_g*phi_hs_g/(1-flush_ret*EXP(-x_hs_g))</f>
-        <v>0.043694219894</v>
+        <v>0.043601503232</v>
       </c>
       <c r="E336" s="52" t="s">
         <v>2427</v>
@@ -28259,7 +28413,7 @@
       </c>
       <c r="D337" s="41">
         <f>y_O2_end_g*flush_ret</f>
-        <v>0.016074205197</v>
+        <v>0.015853256328</v>
       </c>
       <c r="E337" s="52" t="s">
         <v>2430</v>
@@ -28277,7 +28431,7 @@
       </c>
       <c r="D338" s="41">
         <f>y_O2_post_g*phi_hs_g+dy_O2_g*psi_hs_g</f>
-        <v>0.029982518845</v>
+        <v>0.029826577069</v>
       </c>
       <c r="E338" s="52" t="s">
         <v>2433</v>
@@ -28313,7 +28467,7 @@
       </c>
       <c r="D340" s="41">
         <f>DO_surf_excess_g+H_O2_T*P_dry*y_O2_mf_g</f>
-        <v>0.068871437472</v>
+        <v>0.068677886041</v>
       </c>
       <c r="E340" s="51" t="s">
         <v>2439</v>
@@ -28331,7 +28485,7 @@
       </c>
       <c r="D341" s="41">
         <f>DO_surf_excess_g+H_O2_T*P_dry*y_O2_avg_g</f>
-        <v>0.071103870189</v>
+        <v>0.070947105706</v>
       </c>
       <c r="E341" s="52" t="s">
         <v>2442</v>
@@ -28349,7 +28503,7 @@
       </c>
       <c r="D342" s="41">
         <f>DO_surf_excess_g+H_O2_T*P_dry*MAX(y_O2_avg_g,y_O2_end_g-(S_O2_g-F_gap_g*y_O2_end_g)/n_hs_gas*tau_L_h)</f>
-        <v>0.076918594369</v>
+        <v>0.076476412694</v>
       </c>
       <c r="E342" s="52" t="s">
         <v>2445</v>
@@ -28367,7 +28521,7 @@
       </c>
       <c r="D343" s="41">
         <f>DO_avg_g*M_O2</f>
-        <v>2.27518163832</v>
+        <v>2.270165488391</v>
       </c>
       <c r="E343" s="52" t="s">
         <v>2448</v>
@@ -28385,7 +28539,7 @@
       </c>
       <c r="D344" s="41">
         <f>DO_peak_g*M_O2</f>
-        <v>2.461241182614</v>
+        <v>2.447092253397</v>
       </c>
       <c r="E344" s="52" t="s">
         <v>2448</v>
@@ -28419,8 +28573,8 @@
       <c r="C346" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D346" s="41">
-        <f>kLa_surf_used/kLa_surf_req_g</f>
+      <c r="D346" s="111">
+        <f>IF(kLa_surf_req_g&gt;0,kLa_surf_used/kLa_surf_req_g,"no positive source")</f>
         <v>1.737152239781</v>
       </c>
       <c r="E346" s="51" t="s">
@@ -28437,8 +28591,8 @@
       <c r="C347" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D347" s="25" t="str">
-        <f>IF(kLa_margin_g&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)")</f>
+      <c r="D347" s="111" t="str">
+        <f>IF(kLa_surf_req_g&lt;=0,"No positive biological O2 surplus; check air ingress and operating DO",IF(kLa_margin_g&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)"))</f>
         <v>reachable – kLa margin 1.74×</v>
       </c>
       <c r="E347" s="51" t="s">
@@ -28457,7 +28611,7 @@
       </c>
       <c r="D348" s="25" t="str">
         <f>IF(DO_peak_g&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
-        <v>peak 2.5 mg/L under the 10.1 mg/L ceiling</v>
+        <v>peak 2.4 mg/L under the 10.1 mg/L ceiling</v>
       </c>
       <c r="E348" s="51" t="s">
         <v>2461</v>
@@ -28475,7 +28629,7 @@
       </c>
       <c r="D349" s="41">
         <f>O2_src_l+y_O2_air*F_vent_ex</f>
-        <v>5.503054011451e-05</v>
+        <v>5.558574972828e-05</v>
       </c>
       <c r="E349" s="51" t="s">
         <v>2400</v>
@@ -28493,7 +28647,7 @@
       </c>
       <c r="D350" s="41">
         <f>CO2_supply+O2_src_l+H2_src_l-CO2_fix_l</f>
-        <v>0.0009889814106504</v>
+        <v>0.0009967220626175</v>
       </c>
       <c r="E350" s="51" t="s">
         <v>2403</v>
@@ -28511,7 +28665,7 @@
       </c>
       <c r="D351" s="41">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,S_O2_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.053679883871</v>
+        <v>0.053815126441</v>
       </c>
       <c r="E351" s="51" t="s">
         <v>2406</v>
@@ -28529,7 +28683,7 @@
       </c>
       <c r="D352" s="41">
         <f>IF(F_vent_ex+F_hs_net_l&gt;0,H2_src_l/(F_vent_ex+F_hs_net_l),NA())</f>
-        <v>0.093395436531</v>
+        <v>0.093689942909</v>
       </c>
       <c r="E352" s="51" t="s">
         <v>2409</v>
@@ -28547,7 +28701,7 @@
       </c>
       <c r="D353" s="41">
         <f>F_vent_ex+MAX(0,O2_src_l+H2_src_l-CO2_fix_l)</f>
-        <v>0.0001793761393403</v>
+        <v>0.0001809584867395</v>
       </c>
       <c r="E353" s="51" t="s">
         <v>2412</v>
@@ -28565,7 +28719,7 @@
       </c>
       <c r="D354" s="41">
         <f>F_gap_l*t_gap_h/n_hs_gas</f>
-        <v>0.2117625711</v>
+        <v>0.214570696589</v>
       </c>
       <c r="E354" s="51" t="s">
         <v>2415</v>
@@ -28583,7 +28737,7 @@
       </c>
       <c r="D355" s="41">
         <f>IF(x_hs_l&gt;0,(1-EXP(-x_hs_l))/x_hs_l,1)</f>
-        <v>0.901213122982</v>
+        <v>0.899993510611</v>
       </c>
       <c r="E355" s="51" t="s">
         <v>2418</v>
@@ -28601,7 +28755,7 @@
       </c>
       <c r="D356" s="41">
         <f>IF(x_hs_l&gt;0,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2)</f>
-        <v>0.466498288648</v>
+        <v>0.466077106423</v>
       </c>
       <c r="E356" s="51" t="s">
         <v>2421</v>
@@ -28619,7 +28773,7 @@
       </c>
       <c r="D357" s="41">
         <f>S_O2_l*t_gap_h/n_hs_gas</f>
-        <v>0.064966325547</v>
+        <v>0.065910548074</v>
       </c>
       <c r="E357" s="51" t="s">
         <v>2424</v>
@@ -28637,7 +28791,7 @@
       </c>
       <c r="D358" s="41">
         <f>dy_O2_l*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.08336349613</v>
+        <v>0.083947589143</v>
       </c>
       <c r="E358" s="52" t="s">
         <v>2427</v>
@@ -28655,7 +28809,7 @@
       </c>
       <c r="D359" s="41">
         <f>y_O2_end_l*flush_ret</f>
-        <v>0.03066771637</v>
+        <v>0.030522861603</v>
       </c>
       <c r="E359" s="52" t="s">
         <v>2430</v>
@@ -28673,7 +28827,7 @@
       </c>
       <c r="D360" s="41">
         <f>y_O2_post_l*phi_hs_l+dy_O2_l*psi_hs_l</f>
-        <v>0.057944828132</v>
+        <v>0.058189774897</v>
       </c>
       <c r="E360" s="52" t="s">
         <v>2433</v>
@@ -28691,7 +28845,7 @@
       </c>
       <c r="D361" s="41">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_mf_l</f>
-        <v>0.168970630184</v>
+        <v>0.170452258538</v>
       </c>
       <c r="E361" s="51" t="s">
         <v>2439</v>
@@ -28709,7 +28863,7 @@
       </c>
       <c r="D362" s="41">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_avg_l</f>
-        <v>0.173258075157</v>
+        <v>0.174849986476</v>
       </c>
       <c r="E362" s="52" t="s">
         <v>2442</v>
@@ -28727,7 +28881,7 @@
       </c>
       <c r="D363" s="41">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*MAX(y_O2_avg_l,y_O2_end_l-(S_O2_l-F_gap_l*y_O2_end_l)/n_hs_gas*tau_L_h)</f>
-        <v>0.184863677984</v>
+        <v>0.186072559802</v>
       </c>
       <c r="E363" s="52" t="s">
         <v>2445</v>
@@ -28745,7 +28899,7 @@
       </c>
       <c r="D364" s="41">
         <f>DO_avg_l*M_O2</f>
-        <v>5.543911888859</v>
+        <v>5.594849867262</v>
       </c>
       <c r="E364" s="52" t="s">
         <v>2448</v>
@@ -28763,7 +28917,7 @@
       </c>
       <c r="D365" s="41">
         <f>DO_peak_l*M_O2</f>
-        <v>5.915267968126</v>
+        <v>5.953949768528</v>
       </c>
       <c r="E365" s="52" t="s">
         <v>2448</v>
@@ -28781,7 +28935,7 @@
       </c>
       <c r="D366" s="41">
         <f>O2_src_l/(DO_target*3600*V_L_m3)</f>
-        <v>0.012348630371</v>
+        <v>0.012493118365</v>
       </c>
       <c r="E366" s="51" t="s">
         <v>2453</v>
@@ -28799,7 +28953,7 @@
       </c>
       <c r="D367" s="41">
         <f>kLa_surf_used/kLa_surf_req_l</f>
-        <v>0.618735621934</v>
+        <v>0.611579692847</v>
       </c>
       <c r="E367" s="51" t="s">
         <v>2456</v>
@@ -28817,7 +28971,7 @@
       </c>
       <c r="D368" s="25" t="str">
         <f>IF(kLa_margin_l&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_l,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)")</f>
-        <v>UNREACHABLE at this surface kLa – margin 0.62× (raise kL_surf, lower the current, or accept a higher DO)</v>
+        <v>UNREACHABLE at this surface kLa – margin 0.61× (raise kL_surf, lower the current, or accept a higher DO)</v>
       </c>
       <c r="E368" s="51" t="s">
         <v>2458</v>
@@ -28835,7 +28989,7 @@
       </c>
       <c r="D369" s="25" t="str">
         <f>IF(DO_peak_l&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
-        <v>peak 5.9 mg/L under the 10.1 mg/L ceiling</v>
+        <v>peak 6.0 mg/L under the 10.1 mg/L ceiling</v>
       </c>
       <c r="E369" s="51" t="s">
         <v>2461</v>
@@ -28871,7 +29025,7 @@
       </c>
       <c r="D372" s="41">
         <f>IF(O2_sizing_phase=phase_name_1,DO_avg_g,IF(O2_sizing_phase=phase_name_2,DO_avg_l,NA()))</f>
-        <v>0.071103870189</v>
+        <v>0.070947105706</v>
       </c>
       <c r="E372" s="52" t="s">
         <v>2508</v>
@@ -28889,7 +29043,7 @@
       </c>
       <c r="D373" s="41">
         <f>IF(O2_sizing_phase=phase_name_1,DO_peak_g,IF(O2_sizing_phase=phase_name_2,DO_peak_l,NA()))</f>
-        <v>0.076918594369</v>
+        <v>0.076476412694</v>
       </c>
       <c r="E373" s="52" t="s">
         <v>2511</v>
@@ -28907,7 +29061,7 @@
       </c>
       <c r="D374" s="25" t="str">
         <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_impair)),IF(DO_peak_sched*M_O2&lt;DO_impair,"peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L under impairment","PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER IMPAIRMENT")&amp;IF(DO_avg_sched*M_O2&lt;=DO_opt,"; mean "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L at/under optimum","; MEAN "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L ABOVE OPTIMUM"),IF(DO_peak_sched&lt;=O2_ceil_C,"organism band unknown – peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L is under the inhibition ceiling","organism band unknown – PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER THE INHIBITION CEILING"))</f>
-        <v>organism band unknown – peak 2.5 mg/L is under the inhibition ceiling</v>
+        <v>organism band unknown – peak 2.4 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E374" s="51" t="s">
         <v>2514</v>
@@ -28925,7 +29079,7 @@
       </c>
       <c r="D375" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*t_gap_h/(V_L_CO2+Vg_CO2)</f>
-        <v>-0.101196830707</v>
+        <v>-0.082423402676</v>
       </c>
       <c r="E375" s="51" t="s">
         <v>2517</v>
@@ -28943,7 +29097,7 @@
       </c>
       <c r="D376" s="41">
         <f>k_eff_CO2*t_off_CO2</f>
-        <v>0.007337937841</v>
+        <v>0.00623745104</v>
       </c>
       <c r="E376" s="51" t="s">
         <v>2520</v>
@@ -28961,7 +29115,7 @@
       </c>
       <c r="D377" s="41">
         <f>IF(pool_x&gt;0,(1-EXP(-pool_x))/pool_x,1)</f>
-        <v>0.996339988863</v>
+        <v>0.99688774868</v>
       </c>
       <c r="E377" s="51" t="s">
         <v>2523</v>
@@ -28979,7 +29133,7 @@
       </c>
       <c r="D378" s="41">
         <f>IF(pool_x&gt;0,(pool_x-1+EXP(-pool_x))/pool_x^2,1/2)</f>
-        <v>0.498779250627</v>
+        <v>0.498962043881</v>
       </c>
       <c r="E378" s="51" t="s">
         <v>2526</v>
@@ -28997,7 +29151,7 @@
       </c>
       <c r="D379" s="41">
         <f>pool_D_raw*pool_phi</f>
-        <v>-0.10082644918</v>
+        <v>-0.082166880332</v>
       </c>
       <c r="E379" s="51" t="s">
         <v>2529</v>
@@ -29015,7 +29169,7 @@
       </c>
       <c r="D380" s="41">
         <f>pool_a+(1-pool_a)*flush_ret</f>
-        <v>0.891401944021</v>
+        <v>0.907470030741</v>
       </c>
       <c r="E380" s="52" t="s">
         <v>2532</v>
@@ -29031,9 +29185,9 @@
       <c r="C381" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D381" s="41">
-        <f>IF(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_atm*F_vent_ex)/(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
-        <v>0.939820877487</v>
+      <c r="D381" s="111">
+        <f>IF(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_dry*F_vent_ex)/(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
+        <v>0.940238937993</v>
       </c>
       <c r="E381" s="51" t="s">
         <v>2535</v>
@@ -29051,7 +29205,7 @@
       </c>
       <c r="D382" s="41">
         <f>y_CO2_mf*C_sat_CO2</f>
-        <v>26.367341391371</v>
+        <v>26.379070375426</v>
       </c>
       <c r="E382" s="51" t="s">
         <v>2538</v>
@@ -29144,7 +29298,7 @@
       </c>
       <c r="D388" s="41">
         <f>H2_src_l*t_gap_h/n_hs_gas*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.145040740595</v>
+        <v>0.146149332991</v>
       </c>
       <c r="E388" s="52" t="s">
         <v>2553</v>
@@ -29162,7 +29316,7 @@
       </c>
       <c r="D389" s="41">
         <f>(pool_a*(C_cycle_peak-C_cycle_start)*(V_L_CO2+Vg_CO2)+MAX(0,CO2_fix_sched-O2_src_sched-H2_src_sched)*t_gap_h)/n_hs_gas</f>
-        <v>0.047702404255</v>
+        <v>0.050856361228</v>
       </c>
       <c r="E389" s="52" t="s">
         <v>2556</v>
@@ -29195,9 +29349,9 @@
       <c r="C391" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D391" s="25" t="str">
-        <f>IF(F_vent_ex&gt;0,"n/a – the vent admits air (Open vent / Air exchange), so the headspace refills",IF(hs_sag&gt;hs_sag_max,"HEADSPACE SAGS "&amp;TEXT(hs_sag,"0%")&amp;" below 1 atm each cycle – a real cap will draw air back: use Open vent or Air exchange","OK – sag "&amp;TEXT(hs_sag,"0%")&amp;" per cycle, within what a sealed cap holds"))</f>
-        <v>n/a – the vent admits air (Open vent / Air exchange), so the headspace refills</v>
+      <c r="D391" s="111" t="str">
+        <f>IF(F_vent_ex&gt;0,"UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow",IF(hs_sag&gt;hs_sag_max,"HEADSPACE SAGS "&amp;TEXT(hs_sag,"0%")&amp;" below 1 atm each cycle – a real cap will draw air back: use Open vent or Air exchange","OK – sag "&amp;TEXT(hs_sag,"0%")&amp;" per cycle, within the assumed sag tolerance; cap performance unverified"))</f>
+        <v>UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow</v>
       </c>
       <c r="E391" s="51" t="s">
         <v>2561</v>
@@ -29251,7 +29405,7 @@
       </c>
       <c r="D394" s="112">
         <f>Electrochemistry!$D$132</f>
-        <v>4.745085102827e-05</v>
+        <v>4.800606064204e-05</v>
       </c>
       <c r="E394" s="140" t="s">
         <v>2570</v>
@@ -29269,7 +29423,7 @@
       </c>
       <c r="D395" s="112">
         <f>Electrochemistry!$D$133</f>
-        <v>9.574538813904e-05</v>
+        <v>9.67725259245e-05</v>
       </c>
       <c r="E395" s="140" t="s">
         <v>2573</v>
@@ -29470,7 +29624,7 @@
       </c>
       <c r="D410" s="25">
         <f>(pulse_V0+Q_CO2_fit*spg_dur)/(Q_CO2/60)</f>
-        <v>0.784513049825</v>
+        <v>0.760518177081</v>
       </c>
       <c r="E410" s="102" t="s">
         <v>2606</v>
@@ -29488,7 +29642,7 @@
       </c>
       <c r="D411" s="25">
         <f>pulse_V0+Q_CO2_fit*spg_dur</f>
-        <v>2.612428455917</v>
+        <v>2.532525529679</v>
       </c>
       <c r="E411" s="102" t="s">
         <v>2609</v>
@@ -29560,7 +29714,7 @@
       </c>
       <c r="D415" s="25">
         <f>Chemistry!$D$296</f>
-        <v>1.152711317868</v>
+        <v>1.405479604448</v>
       </c>
       <c r="E415" s="140" t="s">
         <v>2620</v>
@@ -29578,7 +29732,7 @@
       </c>
       <c r="D416" s="25">
         <f>V_L_m3*DIC_cap_mt</f>
-        <v>1.729066976802e-05</v>
+        <v>2.108219406672e-05</v>
       </c>
       <c r="E416" s="102" t="s">
         <v>2623</v>
@@ -29596,7 +29750,7 @@
       </c>
       <c r="D417" s="25">
         <f>IF(CO2_cons&gt;0,(C_cycle_peak-C_cycle_start)*V_L_CO2*pulses_h/CO2_cons,NA())</f>
-        <v>2.356485959356</v>
+        <v>2.501832900863</v>
       </c>
       <c r="E417" s="102" t="s">
         <v>2626</v>
@@ -29618,6 +29772,57 @@
       </c>
       <c r="E418" s="102" t="s">
         <v>2629</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval command resolution</t>
+        </is>
+      </c>
+      <c r="B419" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">interval_res</t>
+        </is>
+      </c>
+      <c r="C419" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D419" s="116">
+        <v>0.01</v>
+      </c>
+      <c r="E419" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reporting resolution; plugin accepts decimal minutes (UI min 0.01). Round down so an upper interval bound is not exceeded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rounded executable interval</t>
+        </is>
+      </c>
+      <c r="B420" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_run</t>
+        </is>
+      </c>
+      <c r="C420" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D420" s="111">
+        <f>IF(FLOOR((pulse_V0+Q_CO2_fit*spg_dur)/(Q_CO2/60)/(60*duty_actual),interval_res)*60&gt;spg_dur,FLOOR((pulse_V0+Q_CO2_fit*spg_dur)/(Q_CO2/60)/(60*duty_actual),interval_res),NA())</f>
+        <v>7.17</v>
+      </c>
+      <c r="E420" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ideal duty converted to the pulse actually commanded, rounded down. Reject a non-positive gap. Re-evaluate DO and pH at this schedule.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gas model: correct protocol inference and require validated measurements
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -11573,14 +11573,16 @@
       <c r="C24" s="21"/>
       <c r="D24" s="70" t="str">
         <f>Biology!$D$44</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>POTENTIAL FLAMMABILITY (lag screen): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E24" s="24" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
         <v>→ Biology</v>
       </c>
-      <c r="F24" s="22" t="s">
-        <v>1730</v>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nominal lag-phase hazard screen, not safety certification. Predictions depend on unmeasured vent/transfer behaviour; validate mixture-specific limits, sampling and gas clearance before operation.</t>
+        </is>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -23234,12 +23236,12 @@
         <v>111</v>
       </c>
       <c r="D44" s="111" t="str">
-        <f>IF(AND(y_H2_end_b&gt;=H2_LFL,y_O2_end_b&gt;=O2_LOC_H2*LOC_margin),"FLAMMABLE HEADSPACE (lag): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse – until uptake starts, "&amp;IF(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res)*60&gt;spg_dur_opt_b,"sparge every ≤"&amp;TEXT(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res),"0.0")&amp;" min or ","interval remedy unavailable; ")&amp;"sweep ≥"&amp;TEXT(FLOOR(N2_sweep_H2safe,remedy_res)+remedy_res,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below the H₂ LFL or under the O₂ LOC margin at every point of the cycle (lag): H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;", O₂ "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse ("&amp;TEXT(y_H2_hs_lag,"0%")&amp;" / "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean)")</f>
-        <v>FLAMMABLE HEADSPACE (lag): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <f>IF(AND(y_H2_end_b&gt;=H2_LFL,y_O2_end_b&gt;=O2_LOC_H2*LOC_margin),"POTENTIAL FLAMMABILITY (lag screen): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse – until uptake starts, "&amp;IF(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res)*60&gt;spg_dur_opt_b,"sparge every ≤"&amp;TEXT(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res),"0.0")&amp;" min or ","interval remedy unavailable; ")&amp;"sweep ≥"&amp;TEXT(FLOOR(N2_sweep_H2safe,remedy_res)+remedy_res,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below nominal H₂/O₂ screening thresholds (lag; not safety certification): H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;", O₂ "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse ("&amp;TEXT(y_H2_hs_lag,"0%")&amp;" / "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean)")</f>
+        <v>POTENTIAL FLAMMABILITY (lag screen): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-pulse lag hazard check. Remedy assumes the actual commanded pulse; displayed upper interval is rounded strictly down and minimum sweep strictly up. Bench safety verification remains required.</t>
+          <t xml:space="preserve">Conservative screen using nominal air LFL and diluted-mixture LOC with an assumed margin, not a validated H2/O2/CO2/N2 flammability envelope. Below threshold is not safety certification. Validate mixture limits and the actual vent/sweep before unattended use.</t>
         </is>
       </c>
       <c r="F44" s="75" t="s">
@@ -23904,8 +23906,10 @@
       </c>
     </row>
     <row r="92" spans="1:5" ht="24" x14ac:dyDescent="0.2">
-      <c r="A92" s="18" t="s">
-        <v>2176</v>
+      <c r="A92" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval clearing the nominal lag hazard screen</t>
+        </is>
       </c>
       <c r="B92" s="19" t="s">
         <v>2177</v>

</xml_diff>

<commit_message>
Gas model: measured electrode k_m and monochloramine lifetime as Calibrations inputs
Two Calibrations sections feed Electrochemistry D83 km_O2 and Chemistry D142
tau_NH2Cl, with the old values kept as named defaults (D165, D314). k_m is keyed
on reactor, electrode, Summary rpm and temperature (±1 °C); tau inverts the
model's own steady state with tau-independent readings (k_Cl_turn, Cl pool, new
P_Cl_max). Inert at baseline. Twin, sensitivity, tests, protocols updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -975,6 +975,20 @@
     <definedName name="Cl_AMYBO03" localSheetId="8">AMYBO03!$D$57</definedName>
     <definedName name="kappa0_AMYBO03" localSheetId="8">AMYBO03!$D$58</definedName>
     <definedName name="I_AMYBO03" localSheetId="8">AMYBO03!$D$59</definedName>
+    <definedName name="cal_km_O2">Calibrations!$D$176</definedName>
+    <definedName name="cal_tau_NH2Cl">Calibrations!$D$189</definedName>
+    <definedName name="n_e_fcn" localSheetId="7">Calibrations!$D$192</definedName>
+    <definedName name="km_T_tol" localSheetId="7">Calibrations!$D$193</definedName>
+    <definedName name="stir_rpm_set" localSheetId="7">Calibrations!$D$194</definedName>
+    <definedName name="temp_C" localSheetId="7">Calibrations!$D$195</definedName>
+    <definedName name="media_sel" localSheetId="7">Calibrations!$D$196</definedName>
+    <definedName name="electrode_sel" localSheetId="7">Calibrations!$D$197</definedName>
+    <definedName name="D_O2" localSheetId="7">Calibrations!$D$198</definedName>
+    <definedName name="km_exp" localSheetId="7">Calibrations!$D$199</definedName>
+    <definedName name="M_Cl2" localSheetId="7">Calibrations!$D$200</definedName>
+    <definedName name="km_O2_default" localSheetId="2">Electrochemistry!$D$165</definedName>
+    <definedName name="tau_NH2Cl_default" localSheetId="3">Chemistry!$D$314</definedName>
+    <definedName name="P_Cl_max" localSheetId="3">Chemistry!$D$315</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -12459,8 +12473,10 @@
         <v>electrode-mass-transfer.md →</v>
       </c>
       <c r="E77" s="21"/>
-      <c r="F77" t="s">
-        <v>1691</v>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One ferricyanide limiting-current run in the same vial at the same rpm and temperature replaces the assumed swirl velocity behind k_m — which sets the cathodic O₂ loss, the peroxide source, the chlorine cap and the electrode-surface pH verdict. Enter it in the electrode mass-transfer section of the Calibrations tab.</t>
+        </is>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
@@ -13450,8 +13466,10 @@
         <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/chlorine-species.md","chlorine-species.md →")</f>
         <v>chlorine-species.md →</v>
       </c>
-      <c r="F151" s="22" t="s">
-        <v>2708</v>
+      <c r="F151" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Settles the monochloramine lifetime (Chemistry D142, entered in the Calibrations monochloramine section), which moves the UdG interval by about ±32 %. Also confirm the CaCl₂ hydrate state (−24 % on every chlorine figure).</t>
+        </is>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.2">
@@ -13533,21 +13551,29 @@
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A157" s="21" t="s">
-        <v>2719</v>
-      </c>
-      <c r="B157" s="21" t="s">
-        <v>941</v>
-      </c>
-      <c r="C157" s="21" t="s">
-        <v>926</v>
+      <c r="A157" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measure: no-carryover maximum flow</t>
+        </is>
+      </c>
+      <c r="B157" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOW</t>
+        </is>
+      </c>
+      <c r="C157" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">low</t>
+        </is>
       </c>
       <c r="D157" s="33" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/electrode-mass-transfer.md","electrode-mass-transfer.md →")</f>
-        <v>electrode-mass-transfer.md →</v>
-      </c>
-      <c r="F157" s="22" t="s">
-        <v>2720</v>
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/flow-calibration.md","flow-calibration.md →")</f>
+        <v>flow-calibration.md →</v>
+      </c>
+      <c r="F157" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record the highest flow without liquid carryover for each reactor in CO2 flows column M; D29 reads "not measured" until then.</t>
+        </is>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.2">
@@ -15457,7 +15483,7 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="A1:N163"/>
+  <dimension ref="A1:N165"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -17049,11 +17075,14 @@
       <c r="C83" s="20" t="s">
         <v>972</v>
       </c>
-      <c r="D83" s="130">
-        <v>4.0000000000000001E-3</v>
-      </c>
-      <c r="E83" s="57" t="s">
-        <v>1480</v>
+      <c r="D83" s="111">
+        <f>IF(ISNUMBER(cal_km_O2),cal_km_O2,km_O2_default)</f>
+        <v>0.004</v>
+      </c>
+      <c r="E83" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The measured value from the Calibrations tab (electrode mass-transfer section: ferricyanide limiting current scaled to O₂) when a run for this reactor at the Summary rpm and temperature is included; otherwise the swirl-velocity estimate km_O2_default (D165).</t>
+        </is>
       </c>
     </row>
     <row r="84" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -18189,6 +18218,31 @@
       </c>
       <c r="E163" s="57" t="s">
         <v>1961</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode mass-transfer coefficient — O₂ (estimate)</t>
+        </is>
+      </c>
+      <c r="B165" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_O2_default</t>
+        </is>
+      </c>
+      <c r="C165" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm/s</t>
+        </is>
+      </c>
+      <c r="D165" s="130">
+        <v>0.004</v>
+      </c>
+      <c r="E165" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eisenberg, Tobias &amp; Wilke 1954 (JES 101:306): Sh = 0.0791·Re^0.7·Sc^0.356 for a cylinder in axial swirl. At an assumed 20 cm/s swirl past a 6 mm rod this gives 3.7e-3 cm/s; bracket 2–6e-3 for 10–40 cm/s. The swirl velocity past a STATIONARY rod is the weak link — Sh goes as u^0.7, so a 4× velocity error is a 2.6× error here. Replaced by a ferricyanide run entered on the Calibrations tab.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -18231,7 +18285,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFC00"/>
   </sheetPr>
-  <dimension ref="A1:G308"/>
+  <dimension ref="A1:G315"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.33203125" customWidth="1"/>
@@ -20164,11 +20218,14 @@
       <c r="C142" s="20" t="s">
         <v>1013</v>
       </c>
-      <c r="D142" s="116">
-        <v>1</v>
-      </c>
-      <c r="E142" s="138" t="s">
-        <v>1014</v>
+      <c r="D142" s="111">
+        <f>IF(ISNUMBER(cal_tau_NH2Cl),cal_tau_NH2Cl,tau_NH2Cl_default)</f>
+        <v>1.0</v>
+      </c>
+      <c r="E142" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The measured lifetime from the Calibrations tab (monochloramine section: DPD combined chlorine at plateau ÷ production rate) when one is included for this reactor and medium; otherwise tau_NH2Cl_default (D314). SENSITIVITY parameter: the fixed τ band (D150–D155, 1 min to 5 h) is shown beside it.</t>
+        </is>
       </c>
     </row>
     <row r="143" spans="1:5" ht="84" x14ac:dyDescent="0.2">
@@ -22423,6 +22480,57 @@
       <c r="E312" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">The simple chloramine steady state does not resolve breakpoint chemistry after ammonium is exhausted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monochloramine effective residence (default)</t>
+        </is>
+      </c>
+      <c r="B314" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tau_NH2Cl_default</t>
+        </is>
+      </c>
+      <c r="C314" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="D314" s="116">
+        <v>1</v>
+      </c>
+      <c r="E314" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time combined chlorine persists before consumption (growth N-uptake, cathodic reduction, dilution). Lit: minutes–hours; system-specific value unknown, so 1 h is a weak central estimate until a DPD run is entered on the Calibrations tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Efficiency-limited chlorine production (independent of τ)</t>
+        </is>
+      </c>
+      <c r="B315" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P_Cl_max</t>
+        </is>
+      </c>
+      <c r="C315" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L/s</t>
+        </is>
+      </c>
+      <c r="D315" s="111">
+        <f>I_Cl_FE/(n_e_Cl*Fcc*VLc)</f>
+        <v>9.828782391025813e-07</v>
+      </c>
+      <c r="E315" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The production ceiling P in the chloramine steady state (the second term of D311): the CER-efficiency-limited current as mol/L/s. Read with D271 and D47 to turn a DPD plateau into a lifetime (Calibrations rows 181–188).</t>
         </is>
       </c>
     </row>
@@ -24262,7 +24370,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:F418"/>
+  <dimension ref="A1:F420"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -32340,7 +32448,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:N163"/>
+  <dimension ref="A1:O200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16" width="12" customWidth="1"/>
@@ -35284,8 +35392,812 @@
       <c r="D163" s="133"/>
       <c r="E163" s="134"/>
     </row>
+    <row r="165">
+      <c r="A165" s="98" t="str">
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/electrode-mass-transfer.md","ELECTRODE MASS TRANSFER  (ferricyanide limiting current)")</f>
+        <v>ELECTRODE MASS TRANSFER  (ferricyanide limiting current)</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use: average O₂-scaled k_m of the included runs for the active reactor and electrode, at the Summary stirrer rate and within the temperature tolerance (D193) of the Summary temperature; other runs are kept but not used. One k_m serves both electrodes in the model. Feeds Electrochemistry km_O2 (D83).</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Researcher</t>
+        </is>
+      </c>
+      <c r="B167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="C167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reactor</t>
+        </is>
+      </c>
+      <c r="D167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode (Summary D3 list)</t>
+        </is>
+      </c>
+      <c r="E167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stir rate (rpm)</t>
+        </is>
+      </c>
+      <c r="F167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temp (°C)</t>
+        </is>
+      </c>
+      <c r="G167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limiting current (mA)</t>
+        </is>
+      </c>
+      <c r="H167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode area (cm²)</t>
+        </is>
+      </c>
+      <c r="I167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ferricyanide (mM)</t>
+        </is>
+      </c>
+      <c r="J167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D ferricyanide (m²/s)</t>
+        </is>
+      </c>
+      <c r="K167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_m ferricyanide (computed, cm/s)</t>
+        </is>
+      </c>
+      <c r="L167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_m O₂ (computed, cm/s)</t>
+        </is>
+      </c>
+      <c r="M167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type (auto)</t>
+        </is>
+      </c>
+      <c r="N167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Include?</t>
+        </is>
+      </c>
+      <c r="O167" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="93"/>
+      <c r="B168" s="94"/>
+      <c r="C168" s="93"/>
+      <c r="D168" s="93"/>
+      <c r="E168" s="94"/>
+      <c r="F168" s="94"/>
+      <c r="G168" s="94"/>
+      <c r="H168" s="94"/>
+      <c r="I168" s="94"/>
+      <c r="J168" s="94"/>
+      <c r="K168" s="100" t="str">
+        <f>IF(OR(G168="",H168="",I168=""),"",IFERROR((G168/1000)/(n_e_fcn*F_const*(H168/10000)*I168)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L168" s="100" t="str">
+        <f>IF(OR(K168="",J168=""),"",IFERROR(K168*(D_O2/J168)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M168" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C168,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N168" s="93"/>
+      <c r="O168" s="93"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="93"/>
+      <c r="B169" s="94"/>
+      <c r="C169" s="93"/>
+      <c r="D169" s="93"/>
+      <c r="E169" s="94"/>
+      <c r="F169" s="94"/>
+      <c r="G169" s="94"/>
+      <c r="H169" s="94"/>
+      <c r="I169" s="94"/>
+      <c r="J169" s="94"/>
+      <c r="K169" s="100" t="str">
+        <f>IF(OR(G169="",H169="",I169=""),"",IFERROR((G169/1000)/(n_e_fcn*F_const*(H169/10000)*I169)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L169" s="100" t="str">
+        <f>IF(OR(K169="",J169=""),"",IFERROR(K169*(D_O2/J169)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M169" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C169,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N169" s="93"/>
+      <c r="O169" s="93"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="93"/>
+      <c r="B170" s="94"/>
+      <c r="C170" s="93"/>
+      <c r="D170" s="93"/>
+      <c r="E170" s="94"/>
+      <c r="F170" s="94"/>
+      <c r="G170" s="94"/>
+      <c r="H170" s="94"/>
+      <c r="I170" s="94"/>
+      <c r="J170" s="94"/>
+      <c r="K170" s="100" t="str">
+        <f>IF(OR(G170="",H170="",I170=""),"",IFERROR((G170/1000)/(n_e_fcn*F_const*(H170/10000)*I170)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L170" s="100" t="str">
+        <f>IF(OR(K170="",J170=""),"",IFERROR(K170*(D_O2/J170)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M170" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C170,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N170" s="93"/>
+      <c r="O170" s="93"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="93"/>
+      <c r="B171" s="94"/>
+      <c r="C171" s="93"/>
+      <c r="D171" s="93"/>
+      <c r="E171" s="94"/>
+      <c r="F171" s="94"/>
+      <c r="G171" s="94"/>
+      <c r="H171" s="94"/>
+      <c r="I171" s="94"/>
+      <c r="J171" s="94"/>
+      <c r="K171" s="100" t="str">
+        <f>IF(OR(G171="",H171="",I171=""),"",IFERROR((G171/1000)/(n_e_fcn*F_const*(H171/10000)*I171)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L171" s="100" t="str">
+        <f>IF(OR(K171="",J171=""),"",IFERROR(K171*(D_O2/J171)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M171" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C171,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N171" s="93"/>
+      <c r="O171" s="93"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="93"/>
+      <c r="B172" s="94"/>
+      <c r="C172" s="93"/>
+      <c r="D172" s="93"/>
+      <c r="E172" s="94"/>
+      <c r="F172" s="94"/>
+      <c r="G172" s="94"/>
+      <c r="H172" s="94"/>
+      <c r="I172" s="94"/>
+      <c r="J172" s="94"/>
+      <c r="K172" s="100" t="str">
+        <f>IF(OR(G172="",H172="",I172=""),"",IFERROR((G172/1000)/(n_e_fcn*F_const*(H172/10000)*I172)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L172" s="100" t="str">
+        <f>IF(OR(K172="",J172=""),"",IFERROR(K172*(D_O2/J172)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M172" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C172,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N172" s="93"/>
+      <c r="O172" s="93"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="93"/>
+      <c r="B173" s="94"/>
+      <c r="C173" s="93"/>
+      <c r="D173" s="93"/>
+      <c r="E173" s="94"/>
+      <c r="F173" s="94"/>
+      <c r="G173" s="94"/>
+      <c r="H173" s="94"/>
+      <c r="I173" s="94"/>
+      <c r="J173" s="94"/>
+      <c r="K173" s="100" t="str">
+        <f>IF(OR(G173="",H173="",I173=""),"",IFERROR((G173/1000)/(n_e_fcn*F_const*(H173/10000)*I173)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L173" s="100" t="str">
+        <f>IF(OR(K173="",J173=""),"",IFERROR(K173*(D_O2/J173)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M173" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C173,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N173" s="93"/>
+      <c r="O173" s="93"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="93"/>
+      <c r="B174" s="94"/>
+      <c r="C174" s="93"/>
+      <c r="D174" s="93"/>
+      <c r="E174" s="94"/>
+      <c r="F174" s="94"/>
+      <c r="G174" s="94"/>
+      <c r="H174" s="94"/>
+      <c r="I174" s="94"/>
+      <c r="J174" s="94"/>
+      <c r="K174" s="100" t="str">
+        <f>IF(OR(G174="",H174="",I174=""),"",IFERROR((G174/1000)/(n_e_fcn*F_const*(H174/10000)*I174)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L174" s="100" t="str">
+        <f>IF(OR(K174="",J174=""),"",IFERROR(K174*(D_O2/J174)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M174" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C174,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N174" s="93"/>
+      <c r="O174" s="93"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="93"/>
+      <c r="B175" s="94"/>
+      <c r="C175" s="93"/>
+      <c r="D175" s="93"/>
+      <c r="E175" s="94"/>
+      <c r="F175" s="94"/>
+      <c r="G175" s="94"/>
+      <c r="H175" s="94"/>
+      <c r="I175" s="94"/>
+      <c r="J175" s="94"/>
+      <c r="K175" s="100" t="str">
+        <f>IF(OR(G175="",H175="",I175=""),"",IFERROR((G175/1000)/(n_e_fcn*F_const*(H175/10000)*I175)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L175" s="100" t="str">
+        <f>IF(OR(K175="",J175=""),"",IFERROR(K175*(D_O2/J175)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M175" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C175,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N175" s="93"/>
+      <c r="O175" s="93"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - k_m O₂</t>
+        </is>
+      </c>
+      <c r="C176" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm/s</t>
+        </is>
+      </c>
+      <c r="D176" s="95" t="str">
+        <f>IFERROR(AVERAGEIFS(L168:L175,C168:C175,Reactor_sel,D168:D175,electrode_sel,N168:N175,"y",E168:E175,stir_rpm_set,F168:F175,"&gt;="&amp;(temp_C-km_T_tol),F168:F175,"&lt;="&amp;(temp_C+km_T_tol)),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="98" t="str">
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/chlorine-species.md","MONOCHLORAMINE LIFETIME  (DPD combined chlorine at plateau)")</f>
+        <v>MONOCHLORAMINE LIFETIME  (DPD combined chlorine at plateau)</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use: average of the included runs for the active reactor and medium. Inverts the model’s own steady state B = min(C·kτ/(1+kτ), P·τ): τ = max(B/(k(C−B)), B/P), with k, C and P read from Chemistry D271, D47 and D315 at the run settings (none depends on τ). Feeds Chemistry tau_NH2Cl (D142).</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Researcher</t>
+        </is>
+      </c>
+      <c r="B180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="C180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reactor</t>
+        </is>
+      </c>
+      <c r="D180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combined chlorine plateau (mg/L as Cl₂)</t>
+        </is>
+      </c>
+      <c r="F180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chloride turnover k (1/s, Chemistry D271)</t>
+        </is>
+      </c>
+      <c r="G180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chloride pool C (mol/L, Chemistry D47)</t>
+        </is>
+      </c>
+      <c r="H180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max production P (mol/L/s, Chemistry D315)</t>
+        </is>
+      </c>
+      <c r="I180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lifetime (computed, h)</t>
+        </is>
+      </c>
+      <c r="J180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type (auto)</t>
+        </is>
+      </c>
+      <c r="K180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Include?</t>
+        </is>
+      </c>
+      <c r="L180" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="93"/>
+      <c r="B181" s="94"/>
+      <c r="C181" s="93"/>
+      <c r="D181" s="93"/>
+      <c r="E181" s="94"/>
+      <c r="F181" s="94"/>
+      <c r="G181" s="94"/>
+      <c r="H181" s="94"/>
+      <c r="I181" s="100" t="str">
+        <f>IF(OR(E181="",F181="",G181="",H181=""),"",IF(E181/M_Cl2&gt;=G181,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E181/M_Cl2/(F181*(G181-E181/M_Cl2)),E181/M_Cl2/H181)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J181" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C181,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K181" s="93"/>
+      <c r="L181" s="93"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="93"/>
+      <c r="B182" s="94"/>
+      <c r="C182" s="93"/>
+      <c r="D182" s="93"/>
+      <c r="E182" s="94"/>
+      <c r="F182" s="94"/>
+      <c r="G182" s="94"/>
+      <c r="H182" s="94"/>
+      <c r="I182" s="100" t="str">
+        <f>IF(OR(E182="",F182="",G182="",H182=""),"",IF(E182/M_Cl2&gt;=G182,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E182/M_Cl2/(F182*(G182-E182/M_Cl2)),E182/M_Cl2/H182)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J182" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C182,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K182" s="93"/>
+      <c r="L182" s="93"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="93"/>
+      <c r="B183" s="94"/>
+      <c r="C183" s="93"/>
+      <c r="D183" s="93"/>
+      <c r="E183" s="94"/>
+      <c r="F183" s="94"/>
+      <c r="G183" s="94"/>
+      <c r="H183" s="94"/>
+      <c r="I183" s="100" t="str">
+        <f>IF(OR(E183="",F183="",G183="",H183=""),"",IF(E183/M_Cl2&gt;=G183,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E183/M_Cl2/(F183*(G183-E183/M_Cl2)),E183/M_Cl2/H183)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J183" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C183,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K183" s="93"/>
+      <c r="L183" s="93"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="93"/>
+      <c r="B184" s="94"/>
+      <c r="C184" s="93"/>
+      <c r="D184" s="93"/>
+      <c r="E184" s="94"/>
+      <c r="F184" s="94"/>
+      <c r="G184" s="94"/>
+      <c r="H184" s="94"/>
+      <c r="I184" s="100" t="str">
+        <f>IF(OR(E184="",F184="",G184="",H184=""),"",IF(E184/M_Cl2&gt;=G184,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E184/M_Cl2/(F184*(G184-E184/M_Cl2)),E184/M_Cl2/H184)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J184" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C184,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K184" s="93"/>
+      <c r="L184" s="93"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="93"/>
+      <c r="B185" s="94"/>
+      <c r="C185" s="93"/>
+      <c r="D185" s="93"/>
+      <c r="E185" s="94"/>
+      <c r="F185" s="94"/>
+      <c r="G185" s="94"/>
+      <c r="H185" s="94"/>
+      <c r="I185" s="100" t="str">
+        <f>IF(OR(E185="",F185="",G185="",H185=""),"",IF(E185/M_Cl2&gt;=G185,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E185/M_Cl2/(F185*(G185-E185/M_Cl2)),E185/M_Cl2/H185)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J185" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C185,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K185" s="93"/>
+      <c r="L185" s="93"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="93"/>
+      <c r="B186" s="94"/>
+      <c r="C186" s="93"/>
+      <c r="D186" s="93"/>
+      <c r="E186" s="94"/>
+      <c r="F186" s="94"/>
+      <c r="G186" s="94"/>
+      <c r="H186" s="94"/>
+      <c r="I186" s="100" t="str">
+        <f>IF(OR(E186="",F186="",G186="",H186=""),"",IF(E186/M_Cl2&gt;=G186,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E186/M_Cl2/(F186*(G186-E186/M_Cl2)),E186/M_Cl2/H186)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J186" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C186,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K186" s="93"/>
+      <c r="L186" s="93"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="93"/>
+      <c r="B187" s="94"/>
+      <c r="C187" s="93"/>
+      <c r="D187" s="93"/>
+      <c r="E187" s="94"/>
+      <c r="F187" s="94"/>
+      <c r="G187" s="94"/>
+      <c r="H187" s="94"/>
+      <c r="I187" s="100" t="str">
+        <f>IF(OR(E187="",F187="",G187="",H187=""),"",IF(E187/M_Cl2&gt;=G187,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E187/M_Cl2/(F187*(G187-E187/M_Cl2)),E187/M_Cl2/H187)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J187" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C187,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K187" s="93"/>
+      <c r="L187" s="93"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="93"/>
+      <c r="B188" s="94"/>
+      <c r="C188" s="93"/>
+      <c r="D188" s="93"/>
+      <c r="E188" s="94"/>
+      <c r="F188" s="94"/>
+      <c r="G188" s="94"/>
+      <c r="H188" s="94"/>
+      <c r="I188" s="100" t="str">
+        <f>IF(OR(E188="",F188="",G188="",H188=""),"",IF(E188/M_Cl2&gt;=G188,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E188/M_Cl2/(F188*(G188-E188/M_Cl2)),E188/M_Cl2/H188)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J188" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C188,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K188" s="93"/>
+      <c r="L188" s="93"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - monochloramine lifetime</t>
+        </is>
+      </c>
+      <c r="C189" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="D189" s="95" t="str">
+        <f>IFERROR(AVERAGEIFS(I181:I188,C181:C188,Reactor_sel,D181:D188,media_sel,K181:K188,"y"),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAMED CONSTANTS AND IMPORTS (electrode mass transfer, monochloramine lifetime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrons per ferricyanide reduced</t>
+        </is>
+      </c>
+      <c r="B192" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n_e_fcn</t>
+        </is>
+      </c>
+      <c r="C192" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D192" s="132">
+        <v>1</v>
+      </c>
+      <c r="E192" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fe(CN)₆³⁻ + e⁻ → Fe(CN)₆⁴⁻: a one-electron couple (protocols/electrode-mass-transfer.md).</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature tolerance for a k_m run</t>
+        </is>
+      </c>
+      <c r="B193" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_T_tol</t>
+        </is>
+      </c>
+      <c r="C193" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">°C</t>
+        </is>
+      </c>
+      <c r="D193" s="132">
+        <v>1</v>
+      </c>
+      <c r="E193" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: diffusivity and viscosity move ~2 %/K, so a run within ±1 °C of the Summary temperature is used as measured; others need a separate temperature correction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Stirrer rate on Summary</t>
+        </is>
+      </c>
+      <c r="B194" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stir_rpm_set</t>
+        </is>
+      </c>
+      <c r="C194" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rpm</t>
+        </is>
+      </c>
+      <c r="D194" s="133">
+        <f>Summary!$D$7</f>
+        <v>1000.0</v>
+      </c>
+      <c r="E194" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D7 (stir_rpm_set)</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Temperature setpoint on Summary</t>
+        </is>
+      </c>
+      <c r="B195" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">temp_C</t>
+        </is>
+      </c>
+      <c r="C195" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">°C</t>
+        </is>
+      </c>
+      <c r="D195" s="133">
+        <f>Summary!$D$8</f>
+        <v>30.0</v>
+      </c>
+      <c r="E195" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D8 (temp_C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Medium selected on Summary</t>
+        </is>
+      </c>
+      <c r="B196" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">media_sel</t>
+        </is>
+      </c>
+      <c r="C196" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D196" s="133" t="str">
+        <f>Summary!$D$5</f>
+        <v>AMYBO03</v>
+      </c>
+      <c r="E196" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D5 (media_sel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Electrode selected on Summary</t>
+        </is>
+      </c>
+      <c r="B197" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">electrode_sel</t>
+        </is>
+      </c>
+      <c r="C197" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D197" s="133" t="str">
+        <f>Summary!$D$3</f>
+        <v>MMO tube</v>
+      </c>
+      <c r="E197" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D3 (electrode_sel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) O₂ diffusivity at reactor T</t>
+        </is>
+      </c>
+      <c r="B198" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D_O2</t>
+        </is>
+      </c>
+      <c r="C198" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m²/s</t>
+        </is>
+      </c>
+      <c r="D198" s="133">
+        <f>'Mass Transfer'!$D$32</f>
+        <v>2.249544435762e-09</v>
+      </c>
+      <c r="E198" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D32 (D_O2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Diffusivity exponent for k_m scaling</t>
+        </is>
+      </c>
+      <c r="B199" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_exp</t>
+        </is>
+      </c>
+      <c r="C199" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D199" s="133">
+        <f>Electrochemistry!$D$84</f>
+        <v>0.644</v>
+      </c>
+      <c r="E199" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D84 (km_exp): the same Eisenberg scaling the model uses for every species.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Cl₂ molar mass</t>
+        </is>
+      </c>
+      <c r="B200" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M_Cl2</t>
+        </is>
+      </c>
+      <c r="C200" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/mol</t>
+        </is>
+      </c>
+      <c r="D200" s="133">
+        <f>Chemistry!$D$223</f>
+        <v>70906.0</v>
+      </c>
+      <c r="E200" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Chemistry!D223 (M_Cl2): DPD results are mg/L as Cl₂.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C8:C15 C81:C88 C66:C73 C52:C59 C38:C45 C23:C30" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>ReactorList</formula1>
     </dataValidation>
@@ -35298,6 +36210,18 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C95:C102 C128:C135 C112:C119" xr:uid="{00000000-0002-0000-0700-00000D000000}">
       <formula1>OrganismList</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose a reactor from the list." sqref="C168:C175 C181:C188">
+      <formula1>ReactorList</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="y or n." sqref="N168:N175 K181:K188">
+      <formula1>"y,n"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose an electrode from the list." sqref="D168:D175">
+      <formula1>ElectrodeList</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose a medium from the list." sqref="D181:D188">
+      <formula1>MediaList</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -35306,7 +36230,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A2:I62"/>
+  <dimension ref="A1:I135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43" customWidth="1"/>

</xml_diff>

<commit_message>
Gas model: added NaHCO3 is an input coupled into pH, ionic strength, conductivity and CO2 storage
Summary D133 (blank = none) -> Chemistry D317/D318 -> SID (D44), I (D185),
kappa (D180), DIC_cap via SID. Row 131 now reports what is still needed.
D6 validation narrowed to the model's 3-10 % domain. Inert at baseline.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -989,6 +989,9 @@
     <definedName name="km_O2_default" localSheetId="2">Electrochemistry!$D$165</definedName>
     <definedName name="tau_NH2Cl_default" localSheetId="3">Chemistry!$D$314</definedName>
     <definedName name="P_Cl_max" localSheetId="3">Chemistry!$D$315</definedName>
+    <definedName name="NaHCO3_add_gL" localSheetId="0">Summary!$D$133</definedName>
+    <definedName name="NaHCO3_add_gL" localSheetId="3">Chemistry!$D$317</definedName>
+    <definedName name="alk_add_M" localSheetId="3">Chemistry!$D$318</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -11253,8 +11256,10 @@
       <c r="E6" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="22" t="s">
-        <v>1143</v>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LED channel D %, the AEP-Plugin 'electrolysis_power' setting (runtime-clamped 0–10 %); drives the electrolysis current via Gerrit's Law. The model needs 3–10 % (fit range ∩ plugin clamp), which the D6 validation enforces.</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -13141,8 +13146,10 @@
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A131" s="64" t="s">
-        <v>2691</v>
+      <c r="A131" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NaHCO₃ still needed to lift pH to the target (first-order)</t>
+        </is>
       </c>
       <c r="C131" s="21" t="s">
         <v>2692</v>
@@ -13155,8 +13162,10 @@
         <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F131" s="22" t="s">
-        <v>2693</v>
+      <c r="F131" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alkalinity still needed, on top of the recipe and any NaHCO₃ in D133, for a probe pH of Chemistry D303 (the 6.5 band floor by default) at today’s dissolved CO₂. Enter it in D133 to see the coupled result; re-read, as CO₂ storage moves with it.</t>
+        </is>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.2">
@@ -13178,6 +13187,34 @@
         <v>2696</v>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Added NaHCO₃ (on top of the recipe)</t>
+        </is>
+      </c>
+      <c r="B133" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NaHCO3_add_gL</t>
+        </is>
+      </c>
+      <c r="C133" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g/L</t>
+        </is>
+      </c>
+      <c r="D133" s="135"/>
+      <c r="E133" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">input/blank</t>
+        </is>
+      </c>
+      <c r="F133" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NaHCO₃ added to the medium; blank = none. It feeds the charge balance, ionic strength, conductivity and CO₂ storage (Chemistry D44, D185, D180, D296), so pH, DO and the schedule respond. Row 131 then shows what is still needed. After a large addition (pH up by more than 0.1) re-enter the DIC reference pH, Chemistry D291 (D310 says when).</t>
+        </is>
+      </c>
+    </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="64" t="s">
         <v>1833</v>
@@ -13505,18 +13542,24 @@
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A154" s="21" t="s">
-        <v>2713</v>
-      </c>
-      <c r="B154" s="21" t="s">
-        <v>922</v>
-      </c>
-      <c r="C154" s="21" t="s">
-        <v>923</v>
+      <c r="A154" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model: nitrate or urea instead of NH₄⁺</t>
+        </is>
+      </c>
+      <c r="B154" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MED</t>
+        </is>
+      </c>
+      <c r="C154" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">med</t>
+        </is>
       </c>
       <c r="F154" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rows 131–132 give the NaHCO₃ for a target pH at first order (AMYBO03 already carries 40 mM; about 0.1 g/L more reaches the 6.5 floor). Still to do: an added-alkalinity input that feeds the charge balance, ionic strength and CO₂ storage.</t>
+          <t xml:space="preserve">Ammonium uptake releases acid as the culture grows; the model holds NH₄⁺ at its recipe value. Needs the owner’s choice of nitrogen source and an uptake rate before it can enter the charge balance.</t>
         </is>
       </c>
     </row>
@@ -13707,7 +13750,7 @@
       <formula>ISNUMBER(SEARCH("OK",D49))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="11">
+  <dataValidations count="12">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a listed reactor" error="Pick a reactor from the list (Geometry A59:A80)." sqref="D2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>ReactorList</formula1>
     </dataValidation>
@@ -13719,10 +13762,6 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a listed medium" error="Pick a medium from the list (Chemistry A114:A116)." sqref="D5" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>MediaList</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Electrolysis power is 0–25 % (Gerrit's Law is validated to 25 %; the plugin clamps at 10 %)." sqref="D6" xr:uid="{00000000-0002-0000-0000-000004000000}">
-      <formula1>0</formula1>
-      <formula2>25</formula2>
     </dataValidation>
     <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Stirrer rate 125–2000 rpm." sqref="D7" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>125</formula1>
@@ -13744,6 +13783,14 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose Outflow only, Open vent or Air exchange." sqref="D111" xr:uid="{00000000-0002-0000-0000-00000A000000}">
       <formula1>"Outflow only,Open vent,Air exchange"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Added NaHCO₃ in g/L (0–10), or leave blank for none." sqref="D133">
+      <formula1>0</formula1>
+      <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Electrolysis power 3–10 %: Gerrit's Law fit range intersected with the AEP-Plugin clamp; outside it the model returns no schedule." sqref="D6">
+      <formula1>3</formula1>
+      <formula2>10</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18285,7 +18332,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFC00"/>
   </sheetPr>
-  <dimension ref="A1:G315"/>
+  <dimension ref="A1:G318"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.33203125" customWidth="1"/>
@@ -18950,11 +18997,13 @@
         <v>847</v>
       </c>
       <c r="D44" s="119">
-        <f>IF(media_sel=INDEX(MediaList,1),SID_mc02,IF(media_sel=INDEX(MediaList,2),SID_udg,IF(media_sel=INDEX(MediaList,3),AMYBO03!SID_AMYBO03,NA())))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),SID_mc02,IF(media_sel=INDEX(MediaList,2),SID_udg,IF(media_sel=INDEX(MediaList,3),AMYBO03!SID_AMYBO03,NA())))+alk_add_M</f>
         <v>0.115446909129</v>
       </c>
-      <c r="E44" s="138" t="s">
-        <v>848</v>
+      <c r="E44" s="138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">by media_sel, plus any NaHCO₃ added on Summary D133 (alk_add_M, D318)</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -20853,11 +20902,13 @@
         <v>1359</v>
       </c>
       <c r="D180" s="111">
-        <f>IF(media_sel=INDEX(MediaList,1),kappa0_mc02,IF(media_sel=INDEX(MediaList,2),kappa0_udg,IF(media_sel=INDEX(MediaList,3),AMYBO03!kappa0_AMYBO03,NA())))*kappa_fI*(1+kappa_TC*(TKc-T_ref))</f>
+        <f>(IF(media_sel=INDEX(MediaList,1),kappa0_mc02,IF(media_sel=INDEX(MediaList,2),kappa0_udg,IF(media_sel=INDEX(MediaList,3),AMYBO03!kappa0_AMYBO03,NA())))+alk_add_M*(lam_Na+lam_HCO3)/10)*kappa_fI*(1+kappa_TC*(TKc-T_ref))</f>
         <v>1.401288519775</v>
       </c>
-      <c r="E180" s="51" t="s">
-        <v>1373</v>
+      <c r="E180" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(Kohlrausch sum of the recipe + the added NaHCO₃, D318) × finite-strength factor × temperature correction. Feeds the ohmic term of the cell-voltage budget (Electrochemistry).</t>
+        </is>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.2">
@@ -20912,11 +20963,13 @@
         <v>1000</v>
       </c>
       <c r="D185" s="111">
-        <f>IF(media_sel=INDEX(MediaList,1),I_mc02,IF(media_sel=INDEX(MediaList,2),I_udg,IF(media_sel=INDEX(MediaList,3),AMYBO03!I_AMYBO03,NA())))</f>
+        <f>IF(media_sel=INDEX(MediaList,1),I_mc02,IF(media_sel=INDEX(MediaList,2),I_udg,IF(media_sel=INDEX(MediaList,3),AMYBO03!I_AMYBO03,NA())))+alk_add_M</f>
         <v>0.200184197377</v>
       </c>
-      <c r="E185" s="51" t="s">
-        <v>860</v>
+      <c r="E185" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">by media_sel, plus the added NaHCO₃ (D318: Na⁺ and HCO₃⁻, each z = 1)</t>
+        </is>
       </c>
     </row>
     <row r="186" spans="1:5" ht="36" x14ac:dyDescent="0.2">
@@ -22328,8 +22381,10 @@
       </c>
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A306" t="s">
-        <v>2735</v>
+      <c r="A306" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extra alkalinity still needed for the target pH</t>
+        </is>
       </c>
       <c r="B306" s="19" t="s">
         <v>2736</v>
@@ -22376,8 +22431,10 @@
         <f>alk_needed*M_NaHCO3</f>
         <v>0.124226377682</v>
       </c>
-      <c r="E308" s="60" t="s">
-        <v>2743</v>
+      <c r="E308" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">First-order, on top of any NaHCO₃ already entered (Summary D133, which is fully coupled through D44, D185, D180 and D296). Holds dissolved CO₂ and γ at the current schedule, so after entering it re-read: the coupled pH can differ slightly because CO₂ storage and ionic strength move with it.</t>
+        </is>
       </c>
     </row>
     <row r="309">
@@ -22531,6 +22588,65 @@
       <c r="E315" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">The production ceiling P in the chloramine steady state (the second term of D311): the CER-efficiency-limited current as mol/L/s. Read with D271 and D47 to turn a DPD plateau into a lifetime (Calibrations rows 181–188).</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ADDED ALKALINITY (Summary D133) — feeds the charge balance, ionic strength, conductivity and CO₂ storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) NaHCO₃ added on Summary</t>
+        </is>
+      </c>
+      <c r="B317" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NaHCO3_add_gL</t>
+        </is>
+      </c>
+      <c r="C317" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g/L</t>
+        </is>
+      </c>
+      <c r="D317" s="111">
+        <f>Summary!$D$133</f>
+        <v>0.0</v>
+      </c>
+      <c r="E317" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D133 (NaHCO3_add_gL); blank reads as 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Added alkalinity (strong cation, as NaHCO₃)</t>
+        </is>
+      </c>
+      <c r="B318" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">alk_add_M</t>
+        </is>
+      </c>
+      <c r="C318" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D318" s="111">
+        <f>NaHCO3_add_gL/M_NaHCO3</f>
+        <v>0.0</v>
+      </c>
+      <c r="E318" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">One Na⁺ per NaHCO₃ raises the strong-ion difference by this amount. Its bicarbonate equilibrates with the dosed CO₂ like the recipe’s own NaHCO₃, so only the Na⁺ enters the balance; it adds this amount to the ionic strength (Na⁺ + HCO₃⁻, z = 1). CO₂ storage uses the typed reference pH D291: re-enter it when D310 asks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: N2 headspace sweep as an inert inflow in the shared balance
Summary D98 input (blank = none) -> MT F_N2/F_dil; every gas-leaving term counts
air + N2, only air carries O2/CO2. Summary D99/D100: sweep for the DO target at
the carbon-limited duty and for lag H2 below the LFL. Inert at baseline.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -992,6 +992,12 @@
     <definedName name="NaHCO3_add_gL" localSheetId="0">Summary!$D$133</definedName>
     <definedName name="NaHCO3_add_gL" localSheetId="3">Chemistry!$D$317</definedName>
     <definedName name="alk_add_M" localSheetId="3">Chemistry!$D$318</definedName>
+    <definedName name="N2_sweep_set" localSheetId="0">Summary!$D$98</definedName>
+    <definedName name="N2_sweep_set" localSheetId="5">'Mass Transfer'!$D$423</definedName>
+    <definedName name="F_N2" localSheetId="5">'Mass Transfer'!$D$424</definedName>
+    <definedName name="F_dil" localSheetId="5">'Mass Transfer'!$D$425</definedName>
+    <definedName name="N2_for_DO" localSheetId="5">'Mass Transfer'!$D$426</definedName>
+    <definedName name="F_dil_b" localSheetId="4">Biology!$D$120</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -12775,6 +12781,91 @@
         <v>1789</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ HEADSPACE SWEEP — owner decision T7 (blank = none); timed N₂ pulses of the same mean flow give the same mean-field balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ sweep flow</t>
+        </is>
+      </c>
+      <c r="B98" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N2_sweep_set</t>
+        </is>
+      </c>
+      <c r="C98" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D98" s="135"/>
+      <c r="E98" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">input/blank</t>
+        </is>
+      </c>
+      <c r="F98" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Continuous inert N₂ into the headspace. It dilutes O₂ and H₂ without adding CO₂, so CO₂ is left for carbon and pH; it also strips CO₂ between pulses. Enters the shared vent balance as an inflow with no O₂ or CO₂ (Mass Transfer D424–D425).</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ sweep that holds the DO target at the carbon-limited interval</t>
+        </is>
+      </c>
+      <c r="C99" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D99" s="65">
+        <f>'Mass Transfer'!$D$426</f>
+        <v>0.3389425610299732</v>
+      </c>
+      <c r="E99" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D426","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F99" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sizing phase (D112). Enter it in D98 and re-read pH (D35) and row 128: CO₂ then only supplies carbon. #N/A = the DO target is unreachable at this surface kLa, which no sweep fixes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ sweep that keeps lag-phase H₂ below the LFL</t>
+        </is>
+      </c>
+      <c r="C100" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D100" s="65">
+        <f>Biology!$D$88</f>
+        <v>0.928010297432</v>
+      </c>
+      <c r="E100" s="24" t="str">
+        <f>HYPERLINK("#Biology!D88","→ Biology")</f>
+        <v>→ Biology</v>
+      </c>
+      <c r="F100" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mean-field, with no CO₂ at all; the pre-pulse sawtooth peaks higher, so treat it as a lower bound and check rows 24–26 with the sweep entered. A screen, not a mixture safety certification.</t>
+        </is>
+      </c>
+    </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="77" t="s">
         <v>1790</v>
@@ -13528,8 +13619,10 @@
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A153" s="21" t="s">
-        <v>2711</v>
+      <c r="A153" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Decide: N₂ sweep hardware and flow (T7)</t>
+        </is>
       </c>
       <c r="B153" s="21" t="s">
         <v>922</v>
@@ -13537,8 +13630,10 @@
       <c r="C153" s="21" t="s">
         <v>932</v>
       </c>
-      <c r="F153" s="22" t="s">
-        <v>2712</v>
+      <c r="F153" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The model now takes an N₂ sweep (D98) as an inert inflow in the shared headspace balance; rows 99–100 give the flow for the DO target at the carbon-limited interval and for lag H₂ below the LFL. Needs the owner’s choice of hardware (own line or shared), flow control and objective.</t>
+        </is>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.2">
@@ -13750,7 +13845,7 @@
       <formula>ISNUMBER(SEARCH("OK",D49))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
+  <dataValidations count="13">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a listed reactor" error="Pick a reactor from the list (Geometry A59:A80)." sqref="D2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>ReactorList</formula1>
     </dataValidation>
@@ -13791,6 +13886,10 @@
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Electrolysis power 3–10 %: Gerrit's Law fit range intersected with the AEP-Plugin clamp; outside it the model returns no schedule." sqref="D6">
       <formula1>3</formula1>
       <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="N₂ sweep in mL/min (0–20), or leave blank for none." sqref="D98">
+      <formula1>0</formula1>
+      <formula2>20</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23994,7 +24093,7 @@
         <v>111</v>
       </c>
       <c r="D84" s="41">
-        <f>H2_src_l_b/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
+        <f>H2_src_l_b/(n_flamm_src+CO2_supply_b+F_dil_b)</f>
         <v>0.093689942909</v>
       </c>
       <c r="E84" s="53" t="s">
@@ -24012,7 +24111,7 @@
         <v>111</v>
       </c>
       <c r="D85" s="41">
-        <f>(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_vent_ex_b)</f>
+        <f>(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_dil_b)</f>
         <v>0.053815126441</v>
       </c>
       <c r="E85" s="53" t="s">
@@ -24030,7 +24129,7 @@
         <v>111</v>
       </c>
       <c r="D86" s="41">
-        <f>MAX(0,MIN(H2_src_l_b/H2_LFL-n_flamm_src-F_vent_ex_b,(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_vent_ex_b))/CO2_rate_full_b</f>
+        <f>MAX(0,MIN(H2_src_l_b/H2_LFL-n_flamm_src-F_dil_b,(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(O2_LOC_H2*LOC_margin)-n_flamm_src-F_dil_b))/CO2_rate_full_b</f>
         <v>0.003321398663</v>
       </c>
       <c r="E86" s="53" t="s">
@@ -24378,27 +24477,28 @@
       </c>
     </row>
     <row r="120" x14ac:dyDescent="0.2">
-      <c r="A120" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Remedy display resolution</t>
+      <c r="A120" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) non-pulse inflow to the headspace (air + N₂)</t>
         </is>
       </c>
       <c r="B120" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">remedy_res</t>
-        </is>
-      </c>
-      <c r="C120" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D120" s="116">
-        <v>0.1</v>
-      </c>
-      <c r="E120" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Display increment: min for interval, mL/min for sweep. Bounds are rounded strictly in the protective direction.</t>
+          <t xml:space="preserve">F_dil_b</t>
+        </is>
+      </c>
+      <c r="C120" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D120" s="120">
+        <f>'Mass Transfer'!$D$425</f>
+        <v>3.617990017297e-05</v>
+      </c>
+      <c r="E120" s="140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D425 (F_dil): air ingress plus any N₂ sweep (Summary D98).</t>
         </is>
       </c>
     </row>
@@ -24486,7 +24586,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:F420"/>
+  <dimension ref="A1:F426"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -27630,7 +27730,7 @@
         <v>1140</v>
       </c>
       <c r="D184" s="111">
-        <f>IF(ISNUMBER(y_O2_star),MAX(0,((O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_vent_ex-O2_src_sched-H2_src_sched+CO2_fix_sched)/CO2_rate_full),NA())</f>
+        <f>IF(ISNUMBER(y_O2_star),MAX(0,((O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_dil-O2_src_sched-H2_src_sched+CO2_fix_sched)/CO2_rate_full),NA())</f>
         <v>0.001767191996</v>
       </c>
       <c r="E184" s="51" t="s">
@@ -28127,7 +28227,7 @@
         <v>406</v>
       </c>
       <c r="D232" s="111">
-        <f>IF(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,DO_surf_excess+H_O2_T*P_dry*MIN(1,saw_factor*(O2_src_sched+y_O2_air*F_vent_ex)/(F_vent_ex+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)),DO_surf_excess+H_O2_T*P_dry)</f>
+        <f>IF(F_dil+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,DO_surf_excess+H_O2_T*P_dry*MIN(1,saw_factor*(O2_src_sched+y_O2_air*F_vent_ex)/(F_dil+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)),DO_surf_excess+H_O2_T*P_dry)</f>
         <v>0.423131676776</v>
       </c>
       <c r="E232" s="74" t="s">
@@ -28690,7 +28790,7 @@
         <v>111</v>
       </c>
       <c r="D329" s="41">
-        <f>IF(F_vent_ex+F_hs_net_g&gt;0,S_O2_g/(F_vent_ex+F_hs_net_g),NA())</f>
+        <f>IF(F_dil+F_hs_net_g&gt;0,S_O2_g/(F_dil+F_hs_net_g),NA())</f>
         <v>0.027569266375</v>
       </c>
       <c r="E329" s="51" t="s">
@@ -28708,7 +28808,7 @@
         <v>111</v>
       </c>
       <c r="D330" s="41">
-        <f>IF(F_vent_ex+F_hs_net_g&gt;0,H2_src_g/(F_vent_ex+F_hs_net_g),NA())</f>
+        <f>IF(F_dil+F_hs_net_g&gt;0,H2_src_g/(F_dil+F_hs_net_g),NA())</f>
         <v>0.0</v>
       </c>
       <c r="E330" s="51" t="s">
@@ -28726,7 +28826,7 @@
         <v>307</v>
       </c>
       <c r="D331" s="41">
-        <f>F_vent_ex+MAX(0,O2_src_g+H2_src_g-CO2_fix_g)</f>
+        <f>F_dil+MAX(0,O2_src_g+H2_src_g-CO2_fix_g)</f>
         <v>3.617990017297e-05</v>
       </c>
       <c r="E331" s="51" t="s">
@@ -29086,7 +29186,7 @@
         <v>111</v>
       </c>
       <c r="D351" s="41">
-        <f>IF(F_vent_ex+F_hs_net_l&gt;0,S_O2_l/(F_vent_ex+F_hs_net_l),NA())</f>
+        <f>IF(F_dil+F_hs_net_l&gt;0,S_O2_l/(F_dil+F_hs_net_l),NA())</f>
         <v>0.053815126441</v>
       </c>
       <c r="E351" s="51" t="s">
@@ -29104,7 +29204,7 @@
         <v>111</v>
       </c>
       <c r="D352" s="41">
-        <f>IF(F_vent_ex+F_hs_net_l&gt;0,H2_src_l/(F_vent_ex+F_hs_net_l),NA())</f>
+        <f>IF(F_dil+F_hs_net_l&gt;0,H2_src_l/(F_dil+F_hs_net_l),NA())</f>
         <v>0.093689942909</v>
       </c>
       <c r="E352" s="51" t="s">
@@ -29122,7 +29222,7 @@
         <v>307</v>
       </c>
       <c r="D353" s="41">
-        <f>F_vent_ex+MAX(0,O2_src_l+H2_src_l-CO2_fix_l)</f>
+        <f>F_dil+MAX(0,O2_src_l+H2_src_l-CO2_fix_l)</f>
         <v>0.0001809584867395</v>
       </c>
       <c r="E353" s="51" t="s">
@@ -29608,7 +29708,7 @@
         <v>111</v>
       </c>
       <c r="D381" s="111">
-        <f>IF(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_dry*F_vent_ex)/(F_vent_ex+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
+        <f>IF(F_dil+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_dry*F_vent_ex)/(F_dil+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
         <v>0.940238937993</v>
       </c>
       <c r="E381" s="51" t="s">
@@ -29772,7 +29872,7 @@
         <v>111</v>
       </c>
       <c r="D391" s="111" t="str">
-        <f>IF(F_vent_ex&gt;0,"UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow",IF(hs_sag&gt;hs_sag_max,"HEADSPACE SAGS "&amp;TEXT(hs_sag,"0%")&amp;" below 1 atm each cycle – a real cap will draw air back: use Open vent or Air exchange","OK – sag "&amp;TEXT(hs_sag,"0%")&amp;" per cycle, within the assumed sag tolerance; cap performance unverified"))</f>
+        <f>IF(AND(F_N2&gt;0,F_N2*t_gap_h&gt;=hs_sag*n_hs_gas),"OK – the N₂ sweep supplies the per-cycle make-up gas; vent outflow unverified",IF(F_vent_ex&gt;0,"UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow",IF(hs_sag&gt;hs_sag_max,"HEADSPACE SAGS "&amp;TEXT(hs_sag,"0%")&amp;" below 1 atm each cycle – a real cap will draw air back: use Open vent or Air exchange","OK – sag "&amp;TEXT(hs_sag,"0%")&amp;" per cycle, within the assumed sag tolerance; cap performance unverified")))</f>
         <v>UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow</v>
       </c>
       <c r="E391" s="51" t="s">
@@ -30244,6 +30344,117 @@
       <c r="E420" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">Ideal duty converted to the pulse actually commanded, rounded down. Reject a non-positive gap. Re-evaluate DO and pH at this schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ HEADSPACE SWEEP (Summary D98) — an inert inflow in the shared balance (§300)</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) N₂ sweep flow</t>
+        </is>
+      </c>
+      <c r="B423" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N2_sweep_set</t>
+        </is>
+      </c>
+      <c r="C423" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D423" s="41">
+        <f>Summary!$D$98</f>
+        <v>0.0</v>
+      </c>
+      <c r="E423" s="140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D98 (N2_sweep_set); blank reads as 0. Owner decision T7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ sweep (molar)</t>
+        </is>
+      </c>
+      <c r="B424" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_N2</t>
+        </is>
+      </c>
+      <c r="C424" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D424" s="41">
+        <f>P_atm*(N2_sweep_set/1000000/60)/(R_gas*T_K)*3600</f>
+        <v>0.0</v>
+      </c>
+      <c r="E424" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dry N₂ at P_atm and T_K, mL/min to mol/h, the same reference as F_vent_ex (D308); the flow-meter reference conditions are unmeasured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non-pulse inflow to the headspace (air + N₂)</t>
+        </is>
+      </c>
+      <c r="B425" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_dil</t>
+        </is>
+      </c>
+      <c r="C425" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D425" s="41">
+        <f>F_vent_ex+F_N2</f>
+        <v>3.617990017297e-05</v>
+      </c>
+      <c r="E425" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Every "gas leaving" term of the shared balance (D184, D232, D329–D331, D351–D353, D381; Biology D84–D86) counts this; only the air part (F_vent_ex) carries O₂ and CO₂.</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N₂ sweep that holds the DO target at the carbon-limited duty</t>
+        </is>
+      </c>
+      <c r="B426" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N2_for_DO</t>
+        </is>
+      </c>
+      <c r="C426" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mL/min</t>
+        </is>
+      </c>
+      <c r="D426" s="41">
+        <f>IF(ISNUMBER(y_O2_star),MAX(0,(O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_vent_ex-O2_src_sched-H2_src_sched+CO2_fix_sched-CO2_rate_full*duty_carbon)/3600*R_gas*T_K/P_atm*1000000*60,NA())</f>
+        <v>0.3389425610299732</v>
+      </c>
+      <c r="E426" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The duty_DO inversion (D184) solved for the inert inflow instead of the CO₂ supply, with CO₂ at the carbon-limited duty (D86): total N₂ needed, net of air ingress. #N/A when the target is unreachable at this surface kLa.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: pH-ceiling interval for the joint CO2/N2 schedule; restore remedy_res
The interval is the shortest of the carbon, DO and pH-ceiling bounds. Chemistry
D320-D324 give the CO2 that holds pH at the band ceiling; a 100-row interval grid
(MT 439-539) finds the longest interval keeping the cycle-mean CO2 above it, on
the pulse in use and restated on D91's basis. Unreachable ceiling -> #N/A, not
the carbon interval. Inert without a sweep.

Fixes 21019da, which wrote F_dil_b over Biology D120 remedy_res: restored, moved
to D125, twin reads remedy_res, test forbids two names on one cell.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -997,7 +997,22 @@
     <definedName name="F_N2" localSheetId="5">'Mass Transfer'!$D$424</definedName>
     <definedName name="F_dil" localSheetId="5">'Mass Transfer'!$D$425</definedName>
     <definedName name="N2_for_DO" localSheetId="5">'Mass Transfer'!$D$426</definedName>
-    <definedName name="F_dil_b" localSheetId="4">Biology!$D$120</definedName>
+    <definedName name="F_dil_b" localSheetId="4">Biology!$D$125</definedName>
+    <definedName name="pH_hi_c" localSheetId="3">Chemistry!$D$321</definedName>
+    <definedName name="h_hi" localSheetId="3">Chemistry!$D$322</definedName>
+    <definedName name="resid_noC_hi" localSheetId="3">Chemistry!$D$323</definedName>
+    <definedName name="CO2_pH_hi" localSheetId="3">Chemistry!$D$324</definedName>
+    <definedName name="CO2_pH_hi_mt" localSheetId="5">'Mass Transfer'!$D$429</definedName>
+    <definedName name="grid_t_min" localSheetId="5">'Mass Transfer'!$D$430</definedName>
+    <definedName name="grid_ratio" localSheetId="5">'Mass Transfer'!$D$431</definedName>
+    <definedName name="spg_int_pH" localSheetId="5">'Mass Transfer'!$D$432</definedName>
+    <definedName name="spg_int_pH_opt" localSheetId="5">'Mass Transfer'!$D$433</definedName>
+    <definedName name="ph_unreach" localSheetId="5">'Mass Transfer'!$D$434</definedName>
+    <definedName name="pool_start_chk" localSheetId="5">'Mass Transfer'!$D$435</definedName>
+    <definedName name="pHg_t" localSheetId="5">'Mass Transfer'!$A$440:$A$539</definedName>
+    <definedName name="pHg_start" localSheetId="5">'Mass Transfer'!$H$440:$H$539</definedName>
+    <definedName name="pHg_C" localSheetId="5">'Mass Transfer'!$I$440:$I$539</definedName>
+    <definedName name="pHg_x" localSheetId="5">'Mass Transfer'!$J$440:$J$539</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -12804,7 +12819,7 @@
           <t xml:space="preserve">mL/min</t>
         </is>
       </c>
-      <c r="D98" s="135"/>
+      <c r="D98" s="130"/>
       <c r="E98" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">input/blank</t>
@@ -12837,7 +12852,7 @@
       </c>
       <c r="F99" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sizing phase (D112). Enter it in D98 and re-read pH (D35) and row 128: CO₂ then only supplies carbon. #N/A = the DO target is unreachable at this surface kLa, which no sweep fixes.</t>
+          <t xml:space="preserve">Sizing phase (D112): the sweep that removes the DO bound on the CO₂ schedule. With it entered, the pH ceiling (row 101) usually sets the interval, so CO₂ still supplies more than carbon needs. #N/A = the DO target is unreachable at this surface kLa, which no sweep fixes.</t>
         </is>
       </c>
     </row>
@@ -12863,6 +12878,31 @@
       <c r="F100" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Mean-field, with no CO₂ at all; the pre-pulse sawtooth peaks higher, so treat it as a lower bound and check rows 24–26 with the sweep entered. A screen, not a mixture safety certification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH-ceiling interval (longest keeping pH at or under the band ceiling)</t>
+        </is>
+      </c>
+      <c r="C101" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D101" s="65">
+        <f>'Mass Transfer'!$D$432</f>
+        <v>212.46010616654434</v>
+      </c>
+      <c r="E101" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D432","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F101" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caps the interval (D16) with the carbon and DO bounds, for the pulse in use. Far above them, or "no pH bound", without a sweep; with an N₂ sweep it stops pH overshooting the band once CO₂ no longer has to dilute O₂. Mass Transfer D435 warns if the capped interval lets the carbon pool run dry.</t>
         </is>
       </c>
     </row>
@@ -18431,7 +18471,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFC00"/>
   </sheetPr>
-  <dimension ref="A1:G318"/>
+  <dimension ref="A1:G324"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="39.33203125" customWidth="1"/>
@@ -22746,6 +22786,117 @@
       <c r="E318" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">One Na⁺ per NaHCO₃ raises the strong-ion difference by this amount. Its bicarbonate equilibrates with the dosed CO₂ like the recipe’s own NaHCO₃, so only the Na⁺ enters the balance; it adds this amount to the ionic strength (Na⁺ + HCO₃⁻, z = 1). CO₂ storage uses the typed reference pH D291: re-enter it when D310 asks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ THAT HOLDS pH AT THE BAND CEILING (for the pH-ceiling interval, Mass Transfer D432)</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Band ceiling on the concentration scale</t>
+        </is>
+      </c>
+      <c r="B321" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH_hi_c</t>
+        </is>
+      </c>
+      <c r="C321" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH</t>
+        </is>
+      </c>
+      <c r="D321" s="111">
+        <f>pH_band_hi+LOG10(gamma_1)</f>
+        <v>7.372334422702037</v>
+      </c>
+      <c r="E321" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Probe (activity) pH ceiling D237 to the concentration scale the charge balance solves on, as D304.</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[H⁺] at the ceiling</t>
+        </is>
+      </c>
+      <c r="B322" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h_hi</t>
+        </is>
+      </c>
+      <c r="C322" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D322" s="111">
+        <f>10^-pH_hi_c</f>
+        <v>4.242927171446188e-08</v>
+      </c>
+      <c r="E322" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Concentration scale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charge balance at the ceiling without the carbonate terms</t>
+        </is>
+      </c>
+      <c r="B323" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">resid_noC_hi</t>
+        </is>
+      </c>
+      <c r="C323" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D323" s="111">
+        <f>pH_SID+pH_NT*h_hi/(h_hi+KaN_c)+h_hi-(pH_PT*Ka1p_c*h_hi^2+2*pH_PT*Ka1p_c*Ka2p_c*h_hi+3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/(h_hi^3+Ka1p_c*h_hi^2+Ka1p_c*Ka2p_c*h_hi+Ka1p_c*Ka2p_c*Ka3p_c)-Kw_c/h_hi</f>
+        <v>0.019548509304140926</v>
+      </c>
+      <c r="E323" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The B50 residual with dissolved CO₂ set to zero: the charge the carbonate species must carry for pH to sit exactly at the ceiling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dissolved CO₂ that holds pH at the band ceiling</t>
+        </is>
+      </c>
+      <c r="B324" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_pH_hi</t>
+        </is>
+      </c>
+      <c r="C324" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/L</t>
+        </is>
+      </c>
+      <c r="D324" s="111">
+        <f>MAX(0,resid_noC_hi)/(Ka1c_c/h_hi+2*Ka1c_c*Ka2c_c/h_hi^2)</f>
+        <v>0.0009665547632061539</v>
+      </c>
+      <c r="E324" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The residual is linear in dissolved CO₂, so this inverts it exactly (γ and the DIC reference held at the schedule in use). Less dissolved CO₂ than this and pH rises above the band. 0 = the ceiling is out of reach even without CO₂ (no pH bound).</t>
         </is>
       </c>
     </row>
@@ -22771,7 +22922,7 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -24477,28 +24628,27 @@
       </c>
     </row>
     <row r="120" x14ac:dyDescent="0.2">
-      <c r="A120" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(import) non-pulse inflow to the headspace (air + N₂)</t>
+      <c r="A120" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Remedy display resolution</t>
         </is>
       </c>
       <c r="B120" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">F_dil_b</t>
-        </is>
-      </c>
-      <c r="C120" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mol/h</t>
-        </is>
-      </c>
-      <c r="D120" s="120">
-        <f>'Mass Transfer'!$D$425</f>
-        <v>3.617990017297e-05</v>
-      </c>
-      <c r="E120" s="140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Import from Mass Transfer!D425 (F_dil): air ingress plus any N₂ sweep (Summary D98).</t>
+          <t xml:space="preserve">remedy_res</t>
+        </is>
+      </c>
+      <c r="C120" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D120" s="116">
+        <v>0.1</v>
+      </c>
+      <c r="E120" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Display increment: min for interval, mL/min for sweep. Bounds are rounded strictly in the protective direction.</t>
         </is>
       </c>
     </row>
@@ -24553,6 +24703,32 @@
       </c>
       <c r="E123" s="50" t="s">
         <v>2227</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) non-pulse inflow to the headspace (air + N₂)</t>
+        </is>
+      </c>
+      <c r="B125" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_dil_b</t>
+        </is>
+      </c>
+      <c r="C125" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D125" s="120">
+        <f>'Mass Transfer'!$D$425</f>
+        <v>3.617990017297e-05</v>
+      </c>
+      <c r="E125" s="140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Mass Transfer!D425 (F_dil): air ingress plus any N₂ sweep (Summary D98).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -24586,7 +24762,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:F426"/>
+  <dimension ref="A1:J539"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -26249,11 +26425,13 @@
         <v>61</v>
       </c>
       <c r="D91" s="41">
-        <f>IF(ISNA(F_vent_ex+O2_src_sched),NA(),IF(ISNUMBER(spg_int_DO),MIN(spg_int_carbon,spg_int_DO),MIN(spg_int_carbon,spg_int_max)))</f>
+        <f>IF(ISNA(F_vent_ex+O2_src_sched),NA(),IF(ph_unreach,NA(),MIN(spg_int_carbon,IF(ISNUMBER(spg_int_DO),spg_int_DO,spg_int_max),IF(ISNUMBER(spg_int_pH_opt),spg_int_pH_opt,spg_int_carbon))))</f>
         <v>7.398866407059</v>
       </c>
-      <c r="E91" s="129" t="s">
-        <v>2243</v>
+      <c r="E91" s="129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANSWER. The shortest of the upper bounds on the interval: carbon supply (D112), headspace-oxygen dilution (spg_int_DO) and the pH ceiling (D433, which binds only when an N₂ sweep dilutes the headspace). #N/A for an invalid vent or phase selector (Summary D111/D112) or when no interval keeps pH under the band ceiling (D434). If the DO target is unreachable at this surface kLa the sheet falls back to the legacy O₂ flush guard (D89) and D134 says so.</t>
+        </is>
       </c>
       <c r="F91" s="21"/>
     </row>
@@ -26306,7 +26484,7 @@
         <v>111</v>
       </c>
       <c r="D94" s="41" t="str">
-        <f>IF(ISNA(F_vent_ex+O2_src_sched),"INVALID SELECTOR (Summary D111/D112)",IF(NOT(ISNUMBER(spg_int_DO)),"O2-INFEASIBLE – the legacy O2 flush guard (D89) sets the interval (see D134)",IF(spg_int_DO&lt;=spg_int_carbon,"O2-DILUTION (headspace O2 sets the interval)","CARBON (CO2 supply sets the interval)")))</f>
+        <f>IF(ISNA(F_vent_ex+O2_src_sched),"INVALID SELECTOR (Summary D111/D112)",IF(ph_unreach,"pH CEILING UNREACHABLE – reduce the N₂ sweep or the added alkalinity",IF(AND(ISNUMBER(spg_int_pH_opt),spg_int_pH_opt&lt;MIN(spg_int_carbon,IF(ISNUMBER(spg_int_DO),spg_int_DO,spg_int_max))),"pH CEILING (keeping pH at or under the band ceiling sets the interval)",IF(NOT(ISNUMBER(spg_int_DO)),"O2-INFEASIBLE – the legacy O2 flush guard (D89) sets the interval (see D134)",IF(spg_int_DO&lt;spg_int_carbon,"O2-DILUTION (headspace O2 sets the interval)","CARBON (CO2 supply sets the interval)")))))</f>
         <v>O2-DILUTION (headspace O2 sets the interval)</v>
       </c>
       <c r="E94" s="74" t="s">
@@ -26637,7 +26815,7 @@
       </c>
       <c r="C113" s="21"/>
       <c r="D113" s="25" t="str">
-        <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(spg_int_carbon,"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) the cycle-mean DO would be ≈"&amp;TEXT(DO_at_carbon*M_O2,"0")&amp;" mg/L, "&amp;IF(DO_at_carbon&gt;O2_ceil_C,"above the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L inhibition ceiling","against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")&amp;" (peaks higher)")</f>
+        <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(MIN(spg_int_carbon,IF(ISNUMBER(spg_int_pH_opt),spg_int_pH_opt,spg_int_carbon)),"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) the cycle-mean DO would be ≈"&amp;TEXT(DO_at_carbon*M_O2,"0")&amp;" mg/L, "&amp;IF(DO_at_carbon&gt;O2_ceil_C,"above the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L inhibition ceiling","against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")&amp;" (peaks higher)")</f>
         <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈14 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E113" s="59" t="s">
@@ -29872,7 +30050,7 @@
         <v>111</v>
       </c>
       <c r="D391" s="111" t="str">
-        <f>IF(AND(F_N2&gt;0,F_N2*t_gap_h&gt;=hs_sag*n_hs_gas),"OK – the N₂ sweep supplies the per-cycle make-up gas; vent outflow unverified",IF(F_vent_ex&gt;0,"UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow",IF(hs_sag&gt;hs_sag_max,"HEADSPACE SAGS "&amp;TEXT(hs_sag,"0%")&amp;" below 1 atm each cycle – a real cap will draw air back: use Open vent or Air exchange","OK – sag "&amp;TEXT(hs_sag,"0%")&amp;" per cycle, within the assumed sag tolerance; cap performance unverified")))</f>
+        <f>IF(AND(F_N2&gt;0,F_N2*t_gap_h&gt;=hs_sag*n_hs_gas),"OK – the N₂ sweep supplies the per-cycle make-up gas; vent outflow unverified",IF(F_vent_ex&gt;0,"UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow",IF(hs_sag-F_N2*t_gap_h/n_hs_gas&gt;hs_sag_max,"HEADSPACE SAGS "&amp;TEXT(hs_sag-F_N2*t_gap_h/n_hs_gas,"0%")&amp;" below 1 atm each cycle – a real cap will draw air back: use Open vent or Air exchange","OK – sag "&amp;TEXT(MAX(0,hs_sag-F_N2*t_gap_h/n_hs_gas),"0%")&amp;" per cycle, within the assumed sag tolerance; cap performance unverified")))</f>
         <v>UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow</v>
       </c>
       <c r="E391" s="51" t="s">
@@ -30456,6 +30634,4445 @@
         <is>
           <t xml:space="preserve">The duty_DO inversion (D184) solved for the inert inflow instead of the CO₂ supply, with CO₂ at the carbon-limited duty (D86): total N₂ needed, net of air ingress. #N/A when the target is unreachable at this surface kLa.</t>
         </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH-CEILING INTERVAL — the longest interval whose cycle-mean dissolved CO₂ still holds pH at the band ceiling (binds with an N₂ sweep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Dissolved CO₂ that holds pH at the band ceiling</t>
+        </is>
+      </c>
+      <c r="B429" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO2_pH_hi_mt</t>
+        </is>
+      </c>
+      <c r="C429" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D429" s="41">
+        <f>Chemistry!$D$324*1000</f>
+        <v>0.9665547632061539</v>
+      </c>
+      <c r="E429" s="140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Chemistry!D324 (CO2_pH_hi, mol/L → mol/m³).</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shortest trial interval in the grid</t>
+        </is>
+      </c>
+      <c r="B430" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid_t_min</t>
+        </is>
+      </c>
+      <c r="C430" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D430" s="106">
+        <v>0.25</v>
+      </c>
+      <c r="E430" s="102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined: first row of the interval grid (rows 440–539).</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Grid step ratio</t>
+        </is>
+      </c>
+      <c r="B431" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid_ratio</t>
+        </is>
+      </c>
+      <c r="C431" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D431" s="106">
+        <v>1.09</v>
+      </c>
+      <c r="E431" s="102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Defined: each grid row is 9 % longer than the last, 0.25 to ~1260 min in 100 rows; the crossing is interpolated in ln(interval).</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH-ceiling interval (pulse in use)</t>
+        </is>
+      </c>
+      <c r="B432" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_pH</t>
+        </is>
+      </c>
+      <c r="C432" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D432" s="41">
+        <f>IF(CO2_pH_hi_mt&lt;=0,"no pH bound",IF(INDEX(pHg_C,1)&lt;CO2_pH_hi_mt,"pH above the band ceiling at any interval – reduce the N₂ sweep or the added alkalinity",IF(MAX(pHg_x)&gt;0,MAX(pHg_x),"no pH bound")))</f>
+        <v>212.46010616654434</v>
+      </c>
+      <c r="E432" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longest interval, for the pulse in use, keeping the cycle-mean dissolved CO₂ (the limit cycle of D198–D200 with the bounds of D162) at or above D429, so pH stays at or under the band ceiling. "no pH bound" = the ceiling is not reached on the grid (0.25–1268 min). CO₂ storage uses the typed DIC reference pH (Chemistry D291): re-enter it when D310 asks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH-ceiling interval on the optimal-pulse basis</t>
+        </is>
+      </c>
+      <c r="B433" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_pH_opt</t>
+        </is>
+      </c>
+      <c r="C433" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D433" s="41">
+        <f>IF(ISNUMBER(spg_int_pH),spg_int_pH*spg_dur_eq_opt/spg_dur_eq,"no pH bound")</f>
+        <v>219.16336897384215</v>
+      </c>
+      <c r="E433" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D432 restated on the full-flow-equivalent basis of D91 (D112, D185), so the executable interval D420 comes back to D432 for whatever pulse is in use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pH ceiling unreachable?</t>
+        </is>
+      </c>
+      <c r="B434" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ph_unreach</t>
+        </is>
+      </c>
+      <c r="C434" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D434" s="41" t="b">
+        <f>AND(CO2_pH_hi_mt&gt;0,INDEX(pHg_C,1)&lt;CO2_pH_hi_mt)</f>
+        <v>0</v>
+      </c>
+      <c r="E434" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TRUE = even the shortest interval leaves pH above the band ceiling; D91 then returns #N/A rather than a schedule that overshoots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carbon pool at the pulse start (schedule in use)</t>
+        </is>
+      </c>
+      <c r="B435" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pool_start_chk</t>
+        </is>
+      </c>
+      <c r="C435" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D435" s="41" t="str">
+        <f>IF(C_cycle_start&lt;C_air_CO2,"WATCH – the carbon pool empties within the cycle (pulse-start CO₂ below air equilibrium): fixation outruns supply at this interval","OK")</f>
+        <v>OK</v>
+      </c>
+      <c r="E435" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The limit cycle drains the pool linearly by fixation between pulses; below air equilibrium it has run dry for part of the cycle. Can fire when a long, pH-capped interval comes close to the carbon bound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval (min)</t>
+        </is>
+      </c>
+      <c r="B439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap (s)</t>
+        </is>
+      </c>
+      <c r="C439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pool turnovers x</t>
+        </is>
+      </c>
+      <c r="D439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e^−x</t>
+        </is>
+      </c>
+      <c r="E439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Φ(x)</t>
+        </is>
+      </c>
+      <c r="F439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ψ(x)</t>
+        </is>
+      </c>
+      <c r="G439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap CO₂ change (mol/m³)</t>
+        </is>
+      </c>
+      <c r="H439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CO₂ at pulse start (mol/m³)</t>
+        </is>
+      </c>
+      <c r="I439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean CO₂ (mol/m³)</t>
+        </is>
+      </c>
+      <c r="J439" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crossing (min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="41">
+        <f>grid_t_min</f>
+        <v>0.25</v>
+      </c>
+      <c r="B440" s="41">
+        <f>MAX(0,A440*60-spg_dur)</f>
+        <v>14.35</v>
+      </c>
+      <c r="C440" s="41">
+        <f>k_eff_CO2*B440</f>
+        <v>0.00020837486306468875</v>
+      </c>
+      <c r="D440" s="41">
+        <f>EXP(-C440)</f>
+        <v>0.9997916468454692</v>
+      </c>
+      <c r="E440" s="41">
+        <f>IF(C440&gt;0,(1-D440)/C440,1)</f>
+        <v>0.9998958198050262</v>
+      </c>
+      <c r="F440" s="41">
+        <f>IF(C440&gt;0,(C440-1+D440)/C440^2,1/2)</f>
+        <v>0.4999652713887201</v>
+      </c>
+      <c r="G440" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B440/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0027535230552878757</v>
+      </c>
+      <c r="H440" s="41">
+        <f>(G440*E440+pool_b*D440)/(1-pool_ret*D440)</f>
+        <v>27.9629697112026</v>
+      </c>
+      <c r="I440" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H440+pool_b)*E440+G440*F440))</f>
+        <v>27.96726016073522</v>
+      </c>
+      <c r="J440" s="41">
+        <f>IF(AND(I440&gt;=CO2_pH_hi_mt,I441&lt;CO2_pH_hi_mt),EXP(LN(A440)+(LN(A441)-LN(A440))*(I440-CO2_pH_hi_mt)/(I440-I441)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="41">
+        <f>A440*grid_ratio</f>
+        <v>0.2725</v>
+      </c>
+      <c r="B441" s="41">
+        <f>MAX(0,A441*60-spg_dur)</f>
+        <v>15.700000000000001</v>
+      </c>
+      <c r="C441" s="41">
+        <f>k_eff_CO2*B441</f>
+        <v>0.0002279780731787884</v>
+      </c>
+      <c r="D441" s="41">
+        <f>EXP(-C441)</f>
+        <v>0.9997720479118474</v>
+      </c>
+      <c r="E441" s="41">
+        <f>IF(C441&gt;0,(1-D441)/C441,1)</f>
+        <v>0.9998860196254907</v>
+      </c>
+      <c r="F441" s="41">
+        <f>IF(C441&gt;0,(C441-1+D441)/C441^2,1/2)</f>
+        <v>0.4999620041893962</v>
+      </c>
+      <c r="G441" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B441/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0030125652939386517</v>
+      </c>
+      <c r="H441" s="41">
+        <f>(G441*E441+pool_b*D441)/(1-pool_ret*D441)</f>
+        <v>27.954265528553602</v>
+      </c>
+      <c r="I441" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H441+pool_b)*E441+G441*F441))</f>
+        <v>27.958958647644337</v>
+      </c>
+      <c r="J441" s="41">
+        <f>IF(AND(I441&gt;=CO2_pH_hi_mt,I442&lt;CO2_pH_hi_mt),EXP(LN(A441)+(LN(A442)-LN(A441))*(I441-CO2_pH_hi_mt)/(I441-I442)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="41">
+        <f>A441*grid_ratio</f>
+        <v>0.29702500000000004</v>
+      </c>
+      <c r="B442" s="41">
+        <f>MAX(0,A442*60-spg_dur)</f>
+        <v>17.171500000000005</v>
+      </c>
+      <c r="C442" s="41">
+        <f>k_eff_CO2*B442</f>
+        <v>0.0002493455722031571</v>
+      </c>
+      <c r="D442" s="41">
+        <f>EXP(-C442)</f>
+        <v>0.9997506855118204</v>
+      </c>
+      <c r="E442" s="41">
+        <f>IF(C442&gt;0,(1-D442)/C442,1)</f>
+        <v>0.9998753375753593</v>
+      </c>
+      <c r="F442" s="41">
+        <f>IF(C442&gt;0,(C442-1+D442)/C442^2,1/2)</f>
+        <v>0.4999584449450705</v>
+      </c>
+      <c r="G442" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B442/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0032949213340679982</v>
+      </c>
+      <c r="H442" s="41">
+        <f>(G442*E442+pool_b*D442)/(1-pool_ret*D442)</f>
+        <v>27.94478196579263</v>
+      </c>
+      <c r="I442" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H442+pool_b)*E442+G442*F442))</f>
+        <v>27.94991380680691</v>
+      </c>
+      <c r="J442" s="41">
+        <f>IF(AND(I442&gt;=CO2_pH_hi_mt,I443&lt;CO2_pH_hi_mt),EXP(LN(A442)+(LN(A443)-LN(A442))*(I442-CO2_pH_hi_mt)/(I442-I443)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="41">
+        <f>A442*grid_ratio</f>
+        <v>0.32375725000000005</v>
+      </c>
+      <c r="B443" s="41">
+        <f>MAX(0,A443*60-spg_dur)</f>
+        <v>18.775435000000005</v>
+      </c>
+      <c r="C443" s="41">
+        <f>k_eff_CO2*B443</f>
+        <v>0.00027263614613971885</v>
+      </c>
+      <c r="D443" s="41">
+        <f>EXP(-C443)</f>
+        <v>0.9997274010157171</v>
+      </c>
+      <c r="E443" s="41">
+        <f>IF(C443&gt;0,(1-D443)/C443,1)</f>
+        <v>0.9998636943143643</v>
+      </c>
+      <c r="F443" s="41">
+        <f>IF(C443&gt;0,(C443-1+D443)/C443^2,1/2)</f>
+        <v>0.4999545640297274</v>
+      </c>
+      <c r="G443" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B443/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0036026894178089845</v>
+      </c>
+      <c r="H443" s="41">
+        <f>(G443*E443+pool_b*D443)/(1-pool_ret*D443)</f>
+        <v>27.934449627284874</v>
+      </c>
+      <c r="I443" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H443+pool_b)*E443+G443*F443))</f>
+        <v>27.940059452136566</v>
+      </c>
+      <c r="J443" s="41">
+        <f>IF(AND(I443&gt;=CO2_pH_hi_mt,I444&lt;CO2_pH_hi_mt),EXP(LN(A443)+(LN(A444)-LN(A443))*(I443-CO2_pH_hi_mt)/(I443-I444)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="41">
+        <f>A443*grid_ratio</f>
+        <v>0.3528954025000001</v>
+      </c>
+      <c r="B444" s="41">
+        <f>MAX(0,A444*60-spg_dur)</f>
+        <v>20.52372415000001</v>
+      </c>
+      <c r="C444" s="41">
+        <f>k_eff_CO2*B444</f>
+        <v>0.00029802287173057125</v>
+      </c>
+      <c r="D444" s="41">
+        <f>EXP(-C444)</f>
+        <v>0.9997020215326742</v>
+      </c>
+      <c r="E444" s="41">
+        <f>IF(C444&gt;0,(1-D444)/C444,1)</f>
+        <v>0.999851003365976</v>
+      </c>
+      <c r="F444" s="41">
+        <f>IF(C444&gt;0,(C444-1+D444)/C444^2,1/2)</f>
+        <v>0.49995033273911005</v>
+      </c>
+      <c r="G444" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B444/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.003938156629086661</v>
+      </c>
+      <c r="H444" s="41">
+        <f>(G444*E444+pool_b*D444)/(1-pool_ret*D444)</f>
+        <v>27.923193011674726</v>
+      </c>
+      <c r="I444" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H444+pool_b)*E444+G444*F444))</f>
+        <v>27.929323574076747</v>
+      </c>
+      <c r="J444" s="41">
+        <f>IF(AND(I444&gt;=CO2_pH_hi_mt,I445&lt;CO2_pH_hi_mt),EXP(LN(A444)+(LN(A445)-LN(A444))*(I444-CO2_pH_hi_mt)/(I444-I445)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="41">
+        <f>A444*grid_ratio</f>
+        <v>0.3846559887250001</v>
+      </c>
+      <c r="B445" s="41">
+        <f>MAX(0,A445*60-spg_dur)</f>
+        <v>22.42935932350001</v>
+      </c>
+      <c r="C445" s="41">
+        <f>k_eff_CO2*B445</f>
+        <v>0.0003256944026246003</v>
+      </c>
+      <c r="D445" s="41">
+        <f>EXP(-C445)</f>
+        <v>0.9996743586300397</v>
+      </c>
+      <c r="E445" s="41">
+        <f>IF(C445&gt;0,(1-D445)/C445,1)</f>
+        <v>0.999837170476678</v>
+      </c>
+      <c r="F445" s="41">
+        <f>IF(C445&gt;0,(C445-1+D445)/C445^2,1/2)</f>
+        <v>0.499945722560935</v>
+      </c>
+      <c r="G445" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B445/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.004303815889379327</v>
+      </c>
+      <c r="H445" s="41">
+        <f>(G445*E445+pool_b*D445)/(1-pool_ret*D445)</f>
+        <v>27.910929988413315</v>
+      </c>
+      <c r="I445" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H445+pool_b)*E445+G445*F445))</f>
+        <v>27.917627840320293</v>
+      </c>
+      <c r="J445" s="41">
+        <f>IF(AND(I445&gt;=CO2_pH_hi_mt,I446&lt;CO2_pH_hi_mt),EXP(LN(A445)+(LN(A446)-LN(A445))*(I445-CO2_pH_hi_mt)/(I445-I446)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="41">
+        <f>A445*grid_ratio</f>
+        <v>0.41927502771025016</v>
+      </c>
+      <c r="B446" s="41">
+        <f>MAX(0,A446*60-spg_dur)</f>
+        <v>24.506501662615012</v>
+      </c>
+      <c r="C446" s="41">
+        <f>k_eff_CO2*B446</f>
+        <v>0.000355856371299092</v>
+      </c>
+      <c r="D446" s="41">
+        <f>EXP(-C446)</f>
+        <v>0.9996442069380695</v>
+      </c>
+      <c r="E446" s="41">
+        <f>IF(C446&gt;0,(1-D446)/C446,1)</f>
+        <v>0.9998220929179743</v>
+      </c>
+      <c r="F446" s="41">
+        <f>IF(C446&gt;0,(C446-1+D446)/C446^2,1/2)</f>
+        <v>0.49994069621839937</v>
+      </c>
+      <c r="G446" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B446/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.004702384483098334</v>
+      </c>
+      <c r="H446" s="41">
+        <f>(G446*E446+pool_b*D446)/(1-pool_ret*D446)</f>
+        <v>27.89757123199304</v>
+      </c>
+      <c r="I446" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H446+pool_b)*E446+G446*F446))</f>
+        <v>27.90488705623134</v>
+      </c>
+      <c r="J446" s="41">
+        <f>IF(AND(I446&gt;=CO2_pH_hi_mt,I447&lt;CO2_pH_hi_mt),EXP(LN(A446)+(LN(A447)-LN(A446))*(I446-CO2_pH_hi_mt)/(I446-I447)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="41">
+        <f>A446*grid_ratio</f>
+        <v>0.4570097802041727</v>
+      </c>
+      <c r="B447" s="41">
+        <f>MAX(0,A447*60-spg_dur)</f>
+        <v>26.770586812250365</v>
+      </c>
+      <c r="C447" s="41">
+        <f>k_eff_CO2*B447</f>
+        <v>0.00038873291715428793</v>
+      </c>
+      <c r="D447" s="41">
+        <f>EXP(-C447)</f>
+        <v>0.9996113426296966</v>
+      </c>
+      <c r="E447" s="41">
+        <f>IF(C447&gt;0,(1-D447)/C447,1)</f>
+        <v>0.9998056587245481</v>
+      </c>
+      <c r="F447" s="41">
+        <f>IF(C447&gt;0,(C447-1+D447)/C447^2,1/2)</f>
+        <v>0.4999352171205103</v>
+      </c>
+      <c r="G447" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B447/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.005136824250252052</v>
+      </c>
+      <c r="H447" s="41">
+        <f>(G447*E447+pool_b*D447)/(1-pool_ret*D447)</f>
+        <v>27.883019610966254</v>
+      </c>
+      <c r="I447" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H447+pool_b)*E447+G447*F447))</f>
+        <v>27.891008582028626</v>
+      </c>
+      <c r="J447" s="41">
+        <f>IF(AND(I447&gt;=CO2_pH_hi_mt,I448&lt;CO2_pH_hi_mt),EXP(LN(A447)+(LN(A448)-LN(A447))*(I447-CO2_pH_hi_mt)/(I447-I448)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="41">
+        <f>A447*grid_ratio</f>
+        <v>0.49814066042254834</v>
+      </c>
+      <c r="B448" s="41">
+        <f>MAX(0,A448*60-spg_dur)</f>
+        <v>29.238439625352903</v>
+      </c>
+      <c r="C448" s="41">
+        <f>k_eff_CO2*B448</f>
+        <v>0.0004245683521364516</v>
+      </c>
+      <c r="D448" s="41">
+        <f>EXP(-C448)</f>
+        <v>0.9995755217642524</v>
+      </c>
+      <c r="E448" s="41">
+        <f>IF(C448&gt;0,(1-D448)/C448,1)</f>
+        <v>0.9997877458638906</v>
+      </c>
+      <c r="F448" s="41">
+        <f>IF(C448&gt;0,(C448-1+D448)/C448^2,1/2)</f>
+        <v>0.4999292458471452</v>
+      </c>
+      <c r="G448" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B448/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.005610363596449605</v>
+      </c>
+      <c r="H448" s="41">
+        <f>(G448*E448+pool_b*D448)/(1-pool_ret*D448)</f>
+        <v>27.867169528721917</v>
+      </c>
+      <c r="I448" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H448+pool_b)*E448+G448*F448))</f>
+        <v>27.875891703990053</v>
+      </c>
+      <c r="J448" s="41">
+        <f>IF(AND(I448&gt;=CO2_pH_hi_mt,I449&lt;CO2_pH_hi_mt),EXP(LN(A448)+(LN(A449)-LN(A448))*(I448-CO2_pH_hi_mt)/(I448-I449)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="41">
+        <f>A448*grid_ratio</f>
+        <v>0.5429733198605777</v>
+      </c>
+      <c r="B449" s="41">
+        <f>MAX(0,A449*60-spg_dur)</f>
+        <v>31.928399191634668</v>
+      </c>
+      <c r="C449" s="41">
+        <f>k_eff_CO2*B449</f>
+        <v>0.00046362897626700994</v>
+      </c>
+      <c r="D449" s="41">
+        <f>EXP(-C449)</f>
+        <v>0.9995364784830391</v>
+      </c>
+      <c r="E449" s="41">
+        <f>IF(C449&gt;0,(1-D449)/C449,1)</f>
+        <v>0.9997682213330703</v>
+      </c>
+      <c r="F449" s="41">
+        <f>IF(C449&gt;0,(C449-1+D449)/C449^2,1/2)</f>
+        <v>0.49992273758602135</v>
+      </c>
+      <c r="G449" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B449/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0061265214838049364</v>
+      </c>
+      <c r="H449" s="41">
+        <f>(G449*E449+pool_b*D449)/(1-pool_ret*D449)</f>
+        <v>27.849906212907875</v>
+      </c>
+      <c r="I449" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H449+pool_b)*E449+G449*F449))</f>
+        <v>27.859426956711125</v>
+      </c>
+      <c r="J449" s="41">
+        <f>IF(AND(I449&gt;=CO2_pH_hi_mt,I450&lt;CO2_pH_hi_mt),EXP(LN(A449)+(LN(A450)-LN(A449))*(I449-CO2_pH_hi_mt)/(I449-I450)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="41">
+        <f>A449*grid_ratio</f>
+        <v>0.5918409186480298</v>
+      </c>
+      <c r="B450" s="41">
+        <f>MAX(0,A450*60-spg_dur)</f>
+        <v>34.86045511888179</v>
+      </c>
+      <c r="C450" s="41">
+        <f>k_eff_CO2*B450</f>
+        <v>0.0005062050565693185</v>
+      </c>
+      <c r="D450" s="41">
+        <f>EXP(-C450)</f>
+        <v>0.9994939230435944</v>
+      </c>
+      <c r="E450" s="41">
+        <f>IF(C450&gt;0,(1-D450)/C450,1)</f>
+        <v>0.999746940173615</v>
+      </c>
+      <c r="F450" s="41">
+        <f>IF(C450&gt;0,(C450-1+D450)/C450^2,1/2)</f>
+        <v>0.49991564295533436</v>
+      </c>
+      <c r="G450" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B450/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0066891335810222476</v>
+      </c>
+      <c r="H450" s="41">
+        <f>(G450*E450+pool_b*D450)/(1-pool_ret*D450)</f>
+        <v>27.831104950329255</v>
+      </c>
+      <c r="I450" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H450+pool_b)*E450+G450*F450))</f>
+        <v>27.841495393307913</v>
+      </c>
+      <c r="J450" s="41">
+        <f>IF(AND(I450&gt;=CO2_pH_hi_mt,I451&lt;CO2_pH_hi_mt),EXP(LN(A450)+(LN(A451)-LN(A450))*(I450-CO2_pH_hi_mt)/(I450-I451)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="41">
+        <f>A450*grid_ratio</f>
+        <v>0.6451066013263524</v>
+      </c>
+      <c r="B451" s="41">
+        <f>MAX(0,A451*60-spg_dur)</f>
+        <v>38.05639607958115</v>
+      </c>
+      <c r="C451" s="41">
+        <f>k_eff_CO2*B451</f>
+        <v>0.0005526129840988348</v>
+      </c>
+      <c r="D451" s="41">
+        <f>EXP(-C451)</f>
+        <v>0.9994475396783339</v>
+      </c>
+      <c r="E451" s="41">
+        <f>IF(C451&gt;0,(1-D451)/C451,1)</f>
+        <v>0.9997237443977746</v>
+      </c>
+      <c r="F451" s="41">
+        <f>IF(C451&gt;0,(C451-1+D451)/C451^2,1/2)</f>
+        <v>0.49990791047292515</v>
+      </c>
+      <c r="G451" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B451/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.007302380766989116</v>
+      </c>
+      <c r="H451" s="41">
+        <f>(G451*E451+pool_b*D451)/(1-pool_ret*D451)</f>
+        <v>27.810630264123937</v>
+      </c>
+      <c r="I451" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H451+pool_b)*E451+G451*F451))</f>
+        <v>27.821967800525204</v>
+      </c>
+      <c r="J451" s="41">
+        <f>IF(AND(I451&gt;=CO2_pH_hi_mt,I452&lt;CO2_pH_hi_mt),EXP(LN(A451)+(LN(A452)-LN(A451))*(I451-CO2_pH_hi_mt)/(I451-I452)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="41">
+        <f>A451*grid_ratio</f>
+        <v>0.7031661954457242</v>
+      </c>
+      <c r="B452" s="41">
+        <f>MAX(0,A452*60-spg_dur)</f>
+        <v>41.53997172674345</v>
+      </c>
+      <c r="C452" s="41">
+        <f>k_eff_CO2*B452</f>
+        <v>0.0006031976251060076</v>
+      </c>
+      <c r="D452" s="41">
+        <f>EXP(-C452)</f>
+        <v>0.9993969842620083</v>
+      </c>
+      <c r="E452" s="41">
+        <f>IF(C452&gt;0,(1-D452)/C452,1)</f>
+        <v>0.9996984618195938</v>
+      </c>
+      <c r="F452" s="41">
+        <f>IF(C452&gt;0,(C452-1+D452)/C452^2,1/2)</f>
+        <v>0.49989948200713774</v>
+      </c>
+      <c r="G452" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B452/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.007970820199693003</v>
+      </c>
+      <c r="H452" s="41">
+        <f>(G452*E452+pool_b*D452)/(1-pool_ret*D452)</f>
+        <v>27.7883350300331</v>
+      </c>
+      <c r="I452" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H452+pool_b)*E452+G452*F452))</f>
+        <v>27.800703855808</v>
+      </c>
+      <c r="J452" s="41">
+        <f>IF(AND(I452&gt;=CO2_pH_hi_mt,I453&lt;CO2_pH_hi_mt),EXP(LN(A452)+(LN(A453)-LN(A452))*(I452-CO2_pH_hi_mt)/(I452-I453)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="41">
+        <f>A452*grid_ratio</f>
+        <v>0.7664511530358394</v>
+      </c>
+      <c r="B453" s="41">
+        <f>MAX(0,A453*60-spg_dur)</f>
+        <v>45.337069182150366</v>
+      </c>
+      <c r="C453" s="41">
+        <f>k_eff_CO2*B453</f>
+        <v>0.000658334883803826</v>
+      </c>
+      <c r="D453" s="41">
+        <f>EXP(-C453)</f>
+        <v>0.9993418817710593</v>
+      </c>
+      <c r="E453" s="41">
+        <f>IF(C453&gt;0,(1-D453)/C453,1)</f>
+        <v>0.9996709047804224</v>
+      </c>
+      <c r="F453" s="41">
+        <f>IF(C453&gt;0,(C453-1+D453)/C453^2,1/2)</f>
+        <v>0.4998902955081181</v>
+      </c>
+      <c r="G453" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B453/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.008699419181340241</v>
+      </c>
+      <c r="H453" s="41">
+        <f>(G453*E453+pool_b*D453)/(1-pool_ret*D453)</f>
+        <v>27.76405952865314</v>
+      </c>
+      <c r="I453" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H453+pool_b)*E453+G453*F453))</f>
+        <v>27.777551223220293</v>
+      </c>
+      <c r="J453" s="41">
+        <f>IF(AND(I453&gt;=CO2_pH_hi_mt,I454&lt;CO2_pH_hi_mt),EXP(LN(A453)+(LN(A454)-LN(A453))*(I453-CO2_pH_hi_mt)/(I453-I454)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="41">
+        <f>A453*grid_ratio</f>
+        <v>0.8354317568090651</v>
+      </c>
+      <c r="B454" s="41">
+        <f>MAX(0,A454*60-spg_dur)</f>
+        <v>49.47590540854391</v>
+      </c>
+      <c r="C454" s="41">
+        <f>k_eff_CO2*B454</f>
+        <v>0.0007184344957844481</v>
+      </c>
+      <c r="D454" s="41">
+        <f>EXP(-C454)</f>
+        <v>0.9992818235164859</v>
+      </c>
+      <c r="E454" s="41">
+        <f>IF(C454&gt;0,(1-D454)/C454,1)</f>
+        <v>0.9996408687614117</v>
+      </c>
+      <c r="F454" s="41">
+        <f>IF(C454&gt;0,(C454-1+D454)/C454^2,1/2)</f>
+        <v>0.49988028235124377</v>
+      </c>
+      <c r="G454" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B454/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.009493592071335733</v>
+      </c>
+      <c r="H454" s="41">
+        <f>(G454*E454+pool_b*D454)/(1-pool_ret*D454)</f>
+        <v>27.737630430688444</v>
+      </c>
+      <c r="I454" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H454+pool_b)*E454+G454*F454))</f>
+        <v>27.75234458550076</v>
+      </c>
+      <c r="J454" s="41">
+        <f>IF(AND(I454&gt;=CO2_pH_hi_mt,I455&lt;CO2_pH_hi_mt),EXP(LN(A454)+(LN(A455)-LN(A454))*(I454-CO2_pH_hi_mt)/(I454-I455)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="41">
+        <f>A454*grid_ratio</f>
+        <v>0.9106206149218811</v>
+      </c>
+      <c r="B455" s="41">
+        <f>MAX(0,A455*60-spg_dur)</f>
+        <v>53.98723689531287</v>
+      </c>
+      <c r="C455" s="41">
+        <f>k_eff_CO2*B455</f>
+        <v>0.0007839430728433263</v>
+      </c>
+      <c r="D455" s="41">
+        <f>EXP(-C455)</f>
+        <v>0.9992163641302456</v>
+      </c>
+      <c r="E455" s="41">
+        <f>IF(C455&gt;0,(1-D455)/C455,1)</f>
+        <v>0.9996081308712536</v>
+      </c>
+      <c r="F455" s="41">
+        <f>IF(C455&gt;0,(C455-1+D455)/C455^2,1/2)</f>
+        <v>0.49986936852119324</v>
+      </c>
+      <c r="G455" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B455/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.010359240521430816</v>
+      </c>
+      <c r="H455" s="41">
+        <f>(G455*E455+pool_b*D455)/(1-pool_ret*D455)</f>
+        <v>27.708859712442802</v>
+      </c>
+      <c r="I455" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H455+pool_b)*E455+G455*F455))</f>
+        <v>27.72490460950332</v>
+      </c>
+      <c r="J455" s="41">
+        <f>IF(AND(I455&gt;=CO2_pH_hi_mt,I456&lt;CO2_pH_hi_mt),EXP(LN(A455)+(LN(A456)-LN(A455))*(I455-CO2_pH_hi_mt)/(I455-I456)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="41">
+        <f>A455*grid_ratio</f>
+        <v>0.9925764702648504</v>
+      </c>
+      <c r="B456" s="41">
+        <f>MAX(0,A456*60-spg_dur)</f>
+        <v>58.904588215891025</v>
+      </c>
+      <c r="C456" s="41">
+        <f>k_eff_CO2*B456</f>
+        <v>0.0008553474218375032</v>
+      </c>
+      <c r="D456" s="41">
+        <f>EXP(-C456)</f>
+        <v>0.9991450182834927</v>
+      </c>
+      <c r="E456" s="41">
+        <f>IF(C456&gt;0,(1-D456)/C456,1)</f>
+        <v>0.9995724481996014</v>
+      </c>
+      <c r="F456" s="41">
+        <f>IF(C456&gt;0,(C456-1+D456)/C456^2,1/2)</f>
+        <v>0.49985747245218703</v>
+      </c>
+      <c r="G456" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B456/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.011302797332034455</v>
+      </c>
+      <c r="H456" s="41">
+        <f>(G456*E456+pool_b*D456)/(1-pool_ret*D456)</f>
+        <v>27.677543499100235</v>
+      </c>
+      <c r="I456" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H456+pool_b)*E456+G456*F456))</f>
+        <v>27.695036842779814</v>
+      </c>
+      <c r="J456" s="41">
+        <f>IF(AND(I456&gt;=CO2_pH_hi_mt,I457&lt;CO2_pH_hi_mt),EXP(LN(A456)+(LN(A457)-LN(A456))*(I456-CO2_pH_hi_mt)/(I456-I457)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="41">
+        <f>A456*grid_ratio</f>
+        <v>1.081908352588687</v>
+      </c>
+      <c r="B457" s="41">
+        <f>MAX(0,A457*60-spg_dur)</f>
+        <v>64.26450115532121</v>
+      </c>
+      <c r="C457" s="41">
+        <f>k_eff_CO2*B457</f>
+        <v>0.0009331781622411561</v>
+      </c>
+      <c r="D457" s="41">
+        <f>EXP(-C457)</f>
+        <v>0.9990672571130931</v>
+      </c>
+      <c r="E457" s="41">
+        <f>IF(C457&gt;0,(1-D457)/C457,1)</f>
+        <v>0.9995335560219417</v>
+      </c>
+      <c r="F457" s="41">
+        <f>IF(C457&gt;0,(C457-1+D457)/C457^2,1/2)</f>
+        <v>0.4998445065677697</v>
+      </c>
+      <c r="G457" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B457/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.012331274255592424</v>
+      </c>
+      <c r="H457" s="41">
+        <f>(G457*E457+pool_b*D457)/(1-pool_ret*D457)</f>
+        <v>27.643460833784374</v>
+      </c>
+      <c r="I457" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H457+pool_b)*E457+G457*F457))</f>
+        <v>27.66253053925143</v>
+      </c>
+      <c r="J457" s="41">
+        <f>IF(AND(I457&gt;=CO2_pH_hi_mt,I458&lt;CO2_pH_hi_mt),EXP(LN(A457)+(LN(A458)-LN(A457))*(I457-CO2_pH_hi_mt)/(I457-I458)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="41">
+        <f>A457*grid_ratio</f>
+        <v>1.179280104321669</v>
+      </c>
+      <c r="B458" s="41">
+        <f>MAX(0,A458*60-spg_dur)</f>
+        <v>70.10680625930013</v>
+      </c>
+      <c r="C458" s="41">
+        <f>k_eff_CO2*B458</f>
+        <v>0.0010180136692811378</v>
+      </c>
+      <c r="D458" s="41">
+        <f>EXP(-C458)</f>
+        <v>0.9989825043308423</v>
+      </c>
+      <c r="E458" s="41">
+        <f>IF(C458&gt;0,(1-D458)/C458,1)</f>
+        <v>0.9994911658466723</v>
+      </c>
+      <c r="F458" s="41">
+        <f>IF(C458&gt;0,(C458-1+D458)/C458^2,1/2)</f>
+        <v>0.499830374246769</v>
+      </c>
+      <c r="G458" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B458/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.013452314102270612</v>
+      </c>
+      <c r="H458" s="41">
+        <f>(G458*E458+pool_b*D458)/(1-pool_ret*D458)</f>
+        <v>27.606372370963225</v>
+      </c>
+      <c r="I458" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H458+pool_b)*E458+G458*F458))</f>
+        <v>27.62715741278323</v>
+      </c>
+      <c r="J458" s="41">
+        <f>IF(AND(I458&gt;=CO2_pH_hi_mt,I459&lt;CO2_pH_hi_mt),EXP(LN(A458)+(LN(A459)-LN(A458))*(I458-CO2_pH_hi_mt)/(I458-I459)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="41">
+        <f>A458*grid_ratio</f>
+        <v>1.2854153137106192</v>
+      </c>
+      <c r="B459" s="41">
+        <f>MAX(0,A459*60-spg_dur)</f>
+        <v>76.47491882263715</v>
+      </c>
+      <c r="C459" s="41">
+        <f>k_eff_CO2*B459</f>
+        <v>0.001110484371954718</v>
+      </c>
+      <c r="D459" s="41">
+        <f>EXP(-C459)</f>
+        <v>0.9988901319876418</v>
+      </c>
+      <c r="E459" s="41">
+        <f>IF(C459&gt;0,(1-D459)/C459,1)</f>
+        <v>0.9994449632862517</v>
+      </c>
+      <c r="F459" s="41">
+        <f>IF(C459&gt;0,(C459-1+D459)/C459^2,1/2)</f>
+        <v>0.4998149706203079</v>
+      </c>
+      <c r="G459" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B459/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.014674247535149832</v>
+      </c>
+      <c r="H459" s="41">
+        <f>(G459*E459+pool_b*D459)/(1-pool_ret*D459)</f>
+        <v>27.56601899352119</v>
+      </c>
+      <c r="I459" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H459+pool_b)*E459+G459*F459))</f>
+        <v>27.588670317805498</v>
+      </c>
+      <c r="J459" s="41">
+        <f>IF(AND(I459&gt;=CO2_pH_hi_mt,I460&lt;CO2_pH_hi_mt),EXP(LN(A459)+(LN(A460)-LN(A459))*(I459-CO2_pH_hi_mt)/(I459-I460)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="41">
+        <f>A459*grid_ratio</f>
+        <v>1.401102691944575</v>
+      </c>
+      <c r="B460" s="41">
+        <f>MAX(0,A460*60-spg_dur)</f>
+        <v>83.41616151667449</v>
+      </c>
+      <c r="C460" s="41">
+        <f>k_eff_CO2*B460</f>
+        <v>0.0012112774378689203</v>
+      </c>
+      <c r="D460" s="41">
+        <f>EXP(-C460)</f>
+        <v>0.9987894558625402</v>
+      </c>
+      <c r="E460" s="41">
+        <f>IF(C460&gt;0,(1-D460)/C460,1)</f>
+        <v>0.9993946057392028</v>
+      </c>
+      <c r="F460" s="41">
+        <f>IF(C460&gt;0,(C460-1+D460)/C460^2,1/2)</f>
+        <v>0.4997981815846509</v>
+      </c>
+      <c r="G460" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B460/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.016006154976988186</v>
+      </c>
+      <c r="H460" s="41">
+        <f>(G460*E460+pool_b*D460)/(1-pool_ret*D460)</f>
+        <v>27.522120353775826</v>
+      </c>
+      <c r="I460" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H460+pool_b)*E460+G460*F460))</f>
+        <v>27.54680185735383</v>
+      </c>
+      <c r="J460" s="41">
+        <f>IF(AND(I460&gt;=CO2_pH_hi_mt,I461&lt;CO2_pH_hi_mt),EXP(LN(A460)+(LN(A461)-LN(A460))*(I460-CO2_pH_hi_mt)/(I460-I461)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="41">
+        <f>A460*grid_ratio</f>
+        <v>1.5272019342195868</v>
+      </c>
+      <c r="B461" s="41">
+        <f>MAX(0,A461*60-spg_dur)</f>
+        <v>90.9821160531752</v>
+      </c>
+      <c r="C461" s="41">
+        <f>k_eff_CO2*B461</f>
+        <v>0.0013211418797154009</v>
+      </c>
+      <c r="D461" s="41">
+        <f>EXP(-C461)</f>
+        <v>0.998679730444021</v>
+      </c>
+      <c r="E461" s="41">
+        <f>IF(C461&gt;0,(1-D461)/C461,1)</f>
+        <v>0.9993397198667121</v>
+      </c>
+      <c r="F461" s="41">
+        <f>IF(C461&gt;0,(C461-1+D461)/C461^2,1/2)</f>
+        <v>0.4997798824284758</v>
+      </c>
+      <c r="G461" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B461/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.01745793408859199</v>
+      </c>
+      <c r="H461" s="41">
+        <f>(G461*E461+pool_b*D461)/(1-pool_ret*D461)</f>
+        <v>27.474373339913324</v>
+      </c>
+      <c r="I461" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H461+pool_b)*E461+G461*F461))</f>
+        <v>27.501262919921896</v>
+      </c>
+      <c r="J461" s="41">
+        <f>IF(AND(I461&gt;=CO2_pH_hi_mt,I462&lt;CO2_pH_hi_mt),EXP(LN(A461)+(LN(A462)-LN(A461))*(I461-CO2_pH_hi_mt)/(I461-I462)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="41">
+        <f>A461*grid_ratio</f>
+        <v>1.66465010829935</v>
+      </c>
+      <c r="B462" s="41">
+        <f>MAX(0,A462*60-spg_dur)</f>
+        <v>99.229006497961</v>
+      </c>
+      <c r="C462" s="41">
+        <f>k_eff_CO2*B462</f>
+        <v>0.001440894121328065</v>
+      </c>
+      <c r="D462" s="41">
+        <f>EXP(-C462)</f>
+        <v>0.9985601434681943</v>
+      </c>
+      <c r="E462" s="41">
+        <f>IF(C462&gt;0,(1-D462)/C462,1)</f>
+        <v>0.999279898844034</v>
+      </c>
+      <c r="F462" s="41">
+        <f>IF(C462&gt;0,(C462-1+D462)/C462^2,1/2)</f>
+        <v>0.4997599374725605</v>
+      </c>
+      <c r="G462" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B462/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.019040373320240143</v>
+      </c>
+      <c r="H462" s="41">
+        <f>(G462*E462+pool_b*D462)/(1-pool_ret*D462)</f>
+        <v>27.4224504707964</v>
+      </c>
+      <c r="I462" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H462+pool_b)*E462+G462*F462))</f>
+        <v>27.451741147859565</v>
+      </c>
+      <c r="J462" s="41">
+        <f>IF(AND(I462&gt;=CO2_pH_hi_mt,I463&lt;CO2_pH_hi_mt),EXP(LN(A462)+(LN(A463)-LN(A462))*(I462-CO2_pH_hi_mt)/(I462-I463)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="41">
+        <f>A462*grid_ratio</f>
+        <v>1.8144686180462914</v>
+      </c>
+      <c r="B463" s="41">
+        <f>MAX(0,A463*60-spg_dur)</f>
+        <v>108.21811708277748</v>
+      </c>
+      <c r="C463" s="41">
+        <f>k_eff_CO2*B463</f>
+        <v>0.0015714240646858685</v>
+      </c>
+      <c r="D463" s="41">
+        <f>EXP(-C463)</f>
+        <v>0.9984298099756248</v>
+      </c>
+      <c r="E463" s="41">
+        <f>IF(C463&gt;0,(1-D463)/C463,1)</f>
+        <v>0.9992146993682958</v>
+      </c>
+      <c r="F463" s="41">
+        <f>IF(C463&gt;0,(C463-1+D463)/C463^2,1/2)</f>
+        <v>0.49973819886005444</v>
+      </c>
+      <c r="G463" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B463/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.02076523208273662</v>
+      </c>
+      <c r="H463" s="41">
+        <f>(G463*E463+pool_b*D463)/(1-pool_ret*D463)</f>
+        <v>27.36599822389911</v>
+      </c>
+      <c r="I463" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H463+pool_b)*E463+G463*F463))</f>
+        <v>27.39789934189507</v>
+      </c>
+      <c r="J463" s="41">
+        <f>IF(AND(I463&gt;=CO2_pH_hi_mt,I464&lt;CO2_pH_hi_mt),EXP(LN(A463)+(LN(A464)-LN(A463))*(I463-CO2_pH_hi_mt)/(I463-I464)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="41">
+        <f>A463*grid_ratio</f>
+        <v>1.9777707936704578</v>
+      </c>
+      <c r="B464" s="41">
+        <f>MAX(0,A464*60-spg_dur)</f>
+        <v>118.01624762022746</v>
+      </c>
+      <c r="C464" s="41">
+        <f>k_eff_CO2*B464</f>
+        <v>0.0017137017029458742</v>
+      </c>
+      <c r="D464" s="41">
+        <f>EXP(-C464)</f>
+        <v>0.9982877658453844</v>
+      </c>
+      <c r="E464" s="41">
+        <f>IF(C464&gt;0,(1-D464)/C464,1)</f>
+        <v>0.9991436384011764</v>
+      </c>
+      <c r="F464" s="41">
+        <f>IF(C464&gt;0,(C464-1+D464)/C464^2,1/2)</f>
+        <v>0.49971450534391765</v>
+      </c>
+      <c r="G464" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B464/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.02264532813385779</v>
+      </c>
+      <c r="H464" s="41">
+        <f>(G464*E464+pool_b*D464)/(1-pool_ret*D464)</f>
+        <v>27.30463530330444</v>
+      </c>
+      <c r="I464" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H464+pool_b)*E464+G464*F464))</f>
+        <v>27.339373808358975</v>
+      </c>
+      <c r="J464" s="41">
+        <f>IF(AND(I464&gt;=CO2_pH_hi_mt,I465&lt;CO2_pH_hi_mt),EXP(LN(A464)+(LN(A465)-LN(A464))*(I464-CO2_pH_hi_mt)/(I464-I465)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="41">
+        <f>A464*grid_ratio</f>
+        <v>2.155770165100799</v>
+      </c>
+      <c r="B465" s="41">
+        <f>MAX(0,A465*60-spg_dur)</f>
+        <v>128.69620990604795</v>
+      </c>
+      <c r="C465" s="41">
+        <f>k_eff_CO2*B465</f>
+        <v>0.001868784328649281</v>
+      </c>
+      <c r="D465" s="41">
+        <f>EXP(-C465)</f>
+        <v>0.9981329607615492</v>
+      </c>
+      <c r="E465" s="41">
+        <f>IF(C465&gt;0,(1-D465)/C465,1)</f>
+        <v>0.9990661896229789</v>
+      </c>
+      <c r="F465" s="41">
+        <f>IF(C465&gt;0,(C465-1+D465)/C465^2,1/2)</f>
+        <v>0.49968868139501266</v>
+      </c>
+      <c r="G465" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B465/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.024694632829579857</v>
+      </c>
+      <c r="H465" s="41">
+        <f>(G465*E465+pool_b*D465)/(1-pool_ret*D465)</f>
+        <v>27.237950857306664</v>
+      </c>
+      <c r="I465" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H465+pool_b)*E465+G465*F465))</f>
+        <v>27.27577265816822</v>
+      </c>
+      <c r="J465" s="41">
+        <f>IF(AND(I465&gt;=CO2_pH_hi_mt,I466&lt;CO2_pH_hi_mt),EXP(LN(A465)+(LN(A466)-LN(A465))*(I465-CO2_pH_hi_mt)/(I465-I466)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="41">
+        <f>A465*grid_ratio</f>
+        <v>2.3497894799598713</v>
+      </c>
+      <c r="B466" s="41">
+        <f>MAX(0,A466*60-spg_dur)</f>
+        <v>140.33736879759226</v>
+      </c>
+      <c r="C466" s="41">
+        <f>k_eff_CO2*B466</f>
+        <v>0.0020378243906659936</v>
+      </c>
+      <c r="D466" s="41">
+        <f>EXP(-C466)</f>
+        <v>0.997964250563754</v>
+      </c>
+      <c r="E466" s="41">
+        <f>IF(C466&gt;0,(1-D466)/C466,1)</f>
+        <v>0.9989817795735794</v>
+      </c>
+      <c r="F466" s="41">
+        <f>IF(C466&gt;0,(C466-1+D466)/C466^2,1/2)</f>
+        <v>0.4996605355681513</v>
+      </c>
+      <c r="G466" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B466/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.026928374947916906</v>
+      </c>
+      <c r="H466" s="41">
+        <f>(G466*E466+pool_b*D466)/(1-pool_ret*D466)</f>
+        <v>27.165502658257026</v>
+      </c>
+      <c r="I466" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H466+pool_b)*E466+G466*F466))</f>
+        <v>27.206674069633827</v>
+      </c>
+      <c r="J466" s="41">
+        <f>IF(AND(I466&gt;=CO2_pH_hi_mt,I467&lt;CO2_pH_hi_mt),EXP(LN(A466)+(LN(A467)-LN(A466))*(I466-CO2_pH_hi_mt)/(I466-I467)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="41">
+        <f>A466*grid_ratio</f>
+        <v>2.56127053315626</v>
+      </c>
+      <c r="B467" s="41">
+        <f>MAX(0,A467*60-spg_dur)</f>
+        <v>153.0262319893756</v>
+      </c>
+      <c r="C467" s="41">
+        <f>k_eff_CO2*B467</f>
+        <v>0.0022220780582642113</v>
+      </c>
+      <c r="D467" s="41">
+        <f>EXP(-C467)</f>
+        <v>0.9977803889295661</v>
+      </c>
+      <c r="E467" s="41">
+        <f>IF(C467&gt;0,(1-D467)/C467,1)</f>
+        <v>0.9988897834524106</v>
+      </c>
+      <c r="F467" s="41">
+        <f>IF(C467&gt;0,(C467-1+D467)/C467^2,1/2)</f>
+        <v>0.49962985929974874</v>
+      </c>
+      <c r="G467" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B467/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0293631538569043</v>
+      </c>
+      <c r="H467" s="41">
+        <f>(G467*E467+pool_b*D467)/(1-pool_ret*D467)</f>
+        <v>27.086815260934205</v>
+      </c>
+      <c r="I467" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H467+pool_b)*E467+G467*F467))</f>
+        <v>27.131624530544354</v>
+      </c>
+      <c r="J467" s="41">
+        <f>IF(AND(I467&gt;=CO2_pH_hi_mt,I468&lt;CO2_pH_hi_mt),EXP(LN(A467)+(LN(A468)-LN(A467))*(I467-CO2_pH_hi_mt)/(I467-I468)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="41">
+        <f>A467*grid_ratio</f>
+        <v>2.7917848811403236</v>
+      </c>
+      <c r="B468" s="41">
+        <f>MAX(0,A468*60-spg_dur)</f>
+        <v>166.85709286841941</v>
+      </c>
+      <c r="C468" s="41">
+        <f>k_eff_CO2*B468</f>
+        <v>0.002422914555946268</v>
+      </c>
+      <c r="D468" s="41">
+        <f>EXP(-C468)</f>
+        <v>0.9975800183323357</v>
+      </c>
+      <c r="E468" s="41">
+        <f>IF(C468&gt;0,(1-D468)/C468,1)</f>
+        <v>0.9987895205488191</v>
+      </c>
+      <c r="F468" s="41">
+        <f>IF(C468&gt;0,(C468-1+D468)/C468^2,1/2)</f>
+        <v>0.4995964253857359</v>
+      </c>
+      <c r="G468" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B468/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.03201706286770056</v>
+      </c>
+      <c r="H468" s="41">
+        <f>(G468*E468+pool_b*D468)/(1-pool_ret*D468)</f>
+        <v>27.00137815997113</v>
+      </c>
+      <c r="I468" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H468+pool_b)*E468+G468*F468))</f>
+        <v>27.050137079105117</v>
+      </c>
+      <c r="J468" s="41">
+        <f>IF(AND(I468&gt;=CO2_pH_hi_mt,I469&lt;CO2_pH_hi_mt),EXP(LN(A468)+(LN(A469)-LN(A468))*(I468-CO2_pH_hi_mt)/(I468-I469)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="41">
+        <f>A468*grid_ratio</f>
+        <v>3.043045520442953</v>
+      </c>
+      <c r="B469" s="41">
+        <f>MAX(0,A469*60-spg_dur)</f>
+        <v>181.93273122657718</v>
+      </c>
+      <c r="C469" s="41">
+        <f>k_eff_CO2*B469</f>
+        <v>0.00264182633841971</v>
+      </c>
+      <c r="D469" s="41">
+        <f>EXP(-C469)</f>
+        <v>0.9973616602138171</v>
+      </c>
+      <c r="E469" s="41">
+        <f>IF(C469&gt;0,(1-D469)/C469,1)</f>
+        <v>0.998680249270696</v>
+      </c>
+      <c r="F469" s="41">
+        <f>IF(C469&gt;0,(C469-1+D469)/C469^2,1/2)</f>
+        <v>0.49955998625092557</v>
+      </c>
+      <c r="G469" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B469/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.034909823689468475</v>
+      </c>
+      <c r="H469" s="41">
+        <f>(G469*E469+pool_b*D469)/(1-pool_ret*D469)</f>
+        <v>26.908643971793175</v>
+      </c>
+      <c r="I469" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H469+pool_b)*E469+G469*F469))</f>
+        <v>26.961689567958537</v>
+      </c>
+      <c r="J469" s="41">
+        <f>IF(AND(I469&gt;=CO2_pH_hi_mt,I470&lt;CO2_pH_hi_mt),EXP(LN(A469)+(LN(A470)-LN(A469))*(I469-CO2_pH_hi_mt)/(I469-I470)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="41">
+        <f>A469*grid_ratio</f>
+        <v>3.316919617282819</v>
+      </c>
+      <c r="B470" s="41">
+        <f>MAX(0,A470*60-spg_dur)</f>
+        <v>198.36517703696913</v>
+      </c>
+      <c r="C470" s="41">
+        <f>k_eff_CO2*B470</f>
+        <v>0.002880440181315762</v>
+      </c>
+      <c r="D470" s="41">
+        <f>EXP(-C470)</f>
+        <v>0.9971237043062322</v>
+      </c>
+      <c r="E470" s="41">
+        <f>IF(C470&gt;0,(1-D470)/C470,1)</f>
+        <v>0.9985611617367195</v>
+      </c>
+      <c r="F470" s="41">
+        <f>IF(C470&gt;0,(C470-1+D470)/C470^2,1/2)</f>
+        <v>0.49952027214472794</v>
+      </c>
+      <c r="G470" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B470/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.03806293298519551</v>
+      </c>
+      <c r="H470" s="41">
+        <f>(G470*E470+pool_b*D470)/(1-pool_ret*D470)</f>
+        <v>26.80802667217039</v>
+      </c>
+      <c r="I470" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H470+pool_b)*E470+G470*F470))</f>
+        <v>26.865722980888727</v>
+      </c>
+      <c r="J470" s="41">
+        <f>IF(AND(I470&gt;=CO2_pH_hi_mt,I471&lt;CO2_pH_hi_mt),EXP(LN(A470)+(LN(A471)-LN(A470))*(I470-CO2_pH_hi_mt)/(I470-I471)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="41">
+        <f>A470*grid_ratio</f>
+        <v>3.615442382838273</v>
+      </c>
+      <c r="B471" s="41">
+        <f>MAX(0,A471*60-spg_dur)</f>
+        <v>216.27654297029636</v>
+      </c>
+      <c r="C471" s="41">
+        <f>k_eff_CO2*B471</f>
+        <v>0.0031405292700724583</v>
+      </c>
+      <c r="D471" s="41">
+        <f>EXP(-C471)</f>
+        <v>0.9968643970335593</v>
+      </c>
+      <c r="E471" s="41">
+        <f>IF(C471&gt;0,(1-D471)/C471,1)</f>
+        <v>0.9984313778958411</v>
+      </c>
+      <c r="F471" s="41">
+        <f>IF(C471&gt;0,(C471-1+D471)/C471^2,1/2)</f>
+        <v>0.4994769891527052</v>
+      </c>
+      <c r="G471" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B471/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.04149982211753798</v>
+      </c>
+      <c r="H471" s="41">
+        <f>(G471*E471+pool_b*D471)/(1-pool_ret*D471)</f>
+        <v>26.698899926909363</v>
+      </c>
+      <c r="I471" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H471+pool_b)*E471+G471*F471))</f>
+        <v>26.76163983796764</v>
+      </c>
+      <c r="J471" s="41">
+        <f>IF(AND(I471&gt;=CO2_pH_hi_mt,I472&lt;CO2_pH_hi_mt),EXP(LN(A471)+(LN(A472)-LN(A471))*(I471-CO2_pH_hi_mt)/(I471-I472)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="41">
+        <f>A471*grid_ratio</f>
+        <v>3.9408321972937177</v>
+      </c>
+      <c r="B472" s="41">
+        <f>MAX(0,A472*60-spg_dur)</f>
+        <v>235.79993183762306</v>
+      </c>
+      <c r="C472" s="41">
+        <f>k_eff_CO2*B472</f>
+        <v>0.0034240263768172577</v>
+      </c>
+      <c r="D472" s="41">
+        <f>EXP(-C472)</f>
+        <v>0.9965818289166978</v>
+      </c>
+      <c r="E472" s="41">
+        <f>IF(C472&gt;0,(1-D472)/C472,1)</f>
+        <v>0.9982899391328648</v>
+      </c>
+      <c r="F472" s="41">
+        <f>IF(C472&gt;0,(C472-1+D472)/C472^2,1/2)</f>
+        <v>0.4994298171055251</v>
+      </c>
+      <c r="G472" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B472/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.04524603127179127</v>
+      </c>
+      <c r="H472" s="41">
+        <f>(G472*E472+pool_b*D472)/(1-pool_ret*D472)</f>
+        <v>26.5805955604465</v>
+      </c>
+      <c r="I472" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H472+pool_b)*E472+G472*F472))</f>
+        <v>26.64880273173718</v>
+      </c>
+      <c r="J472" s="41">
+        <f>IF(AND(I472&gt;=CO2_pH_hi_mt,I473&lt;CO2_pH_hi_mt),EXP(LN(A472)+(LN(A473)-LN(A472))*(I472-CO2_pH_hi_mt)/(I472-I473)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="41">
+        <f>A472*grid_ratio</f>
+        <v>4.295507095050152</v>
+      </c>
+      <c r="B473" s="41">
+        <f>MAX(0,A473*60-spg_dur)</f>
+        <v>257.08042570300915</v>
+      </c>
+      <c r="C473" s="41">
+        <f>k_eff_CO2*B473</f>
+        <v>0.003733038223169089</v>
+      </c>
+      <c r="D473" s="41">
+        <f>EXP(-C473)</f>
+        <v>0.9962739209017657</v>
+      </c>
+      <c r="E473" s="41">
+        <f>IF(C473&gt;0,(1-D473)/C473,1)</f>
+        <v>0.9981358013181879</v>
+      </c>
+      <c r="F473" s="41">
+        <f>IF(C473&gt;0,(C473-1+D473)/C473^2,1/2)</f>
+        <v>0.49937840717365445</v>
+      </c>
+      <c r="G473" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B473/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.04932939924992736</v>
+      </c>
+      <c r="H473" s="41">
+        <f>(G473*E473+pool_b*D473)/(1-pool_ret*D473)</f>
+        <v>26.45240221516257</v>
+      </c>
+      <c r="I473" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H473+pool_b)*E473+G473*F473))</f>
+        <v>26.52653304477366</v>
+      </c>
+      <c r="J473" s="41">
+        <f>IF(AND(I473&gt;=CO2_pH_hi_mt,I474&lt;CO2_pH_hi_mt),EXP(LN(A473)+(LN(A474)-LN(A473))*(I473-CO2_pH_hi_mt)/(I473-I474)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="41">
+        <f>A473*grid_ratio</f>
+        <v>4.682102733604666</v>
+      </c>
+      <c r="B474" s="41">
+        <f>MAX(0,A474*60-spg_dur)</f>
+        <v>280.27616401628</v>
+      </c>
+      <c r="C474" s="41">
+        <f>k_eff_CO2*B474</f>
+        <v>0.004069861135692585</v>
+      </c>
+      <c r="D474" s="41">
+        <f>EXP(-C474)</f>
+        <v>0.9959384095251879</v>
+      </c>
+      <c r="E474" s="41">
+        <f>IF(C474&gt;0,(1-D474)/C474,1)</f>
+        <v>0.9979678272538801</v>
+      </c>
+      <c r="F474" s="41">
+        <f>IF(C474&gt;0,(C474-1+D474)/C474^2,1/2)</f>
+        <v>0.49932237940732177</v>
+      </c>
+      <c r="G474" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B474/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.05378027034609569</v>
+      </c>
+      <c r="H474" s="41">
+        <f>(G474*E474+pool_b*D474)/(1-pool_ret*D474)</f>
+        <v>26.313564263114948</v>
+      </c>
+      <c r="I474" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H474+pool_b)*E474+G474*F474))</f>
+        <v>26.39410990734904</v>
+      </c>
+      <c r="J474" s="41">
+        <f>IF(AND(I474&gt;=CO2_pH_hi_mt,I475&lt;CO2_pH_hi_mt),EXP(LN(A474)+(LN(A475)-LN(A474))*(I474-CO2_pH_hi_mt)/(I474-I475)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="41">
+        <f>A474*grid_ratio</f>
+        <v>5.103491979629087</v>
+      </c>
+      <c r="B475" s="41">
+        <f>MAX(0,A475*60-spg_dur)</f>
+        <v>305.55951877774527</v>
+      </c>
+      <c r="C475" s="41">
+        <f>k_eff_CO2*B475</f>
+        <v>0.004436998110343196</v>
+      </c>
+      <c r="D475" s="41">
+        <f>EXP(-C475)</f>
+        <v>0.9955728308234121</v>
+      </c>
+      <c r="E475" s="41">
+        <f>IF(C475&gt;0,(1-D475)/C475,1)</f>
+        <v>0.9977847784671434</v>
+      </c>
+      <c r="F475" s="41">
+        <f>IF(C475&gt;0,(C475-1+D475)/C475^2,1/2)</f>
+        <v>0.4992613198734643</v>
+      </c>
+      <c r="G475" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B475/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.05863171984091919</v>
+      </c>
+      <c r="H475" s="41">
+        <f>(G475*E475+pool_b*D475)/(1-pool_ret*D475)</f>
+        <v>26.16328104151489</v>
+      </c>
+      <c r="I475" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H475+pool_b)*E475+G475*F475))</f>
+        <v>26.25076946316899</v>
+      </c>
+      <c r="J475" s="41">
+        <f>IF(AND(I475&gt;=CO2_pH_hi_mt,I476&lt;CO2_pH_hi_mt),EXP(LN(A475)+(LN(A476)-LN(A475))*(I475-CO2_pH_hi_mt)/(I475-I476)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="41">
+        <f>A475*grid_ratio</f>
+        <v>5.562806257795705</v>
+      </c>
+      <c r="B476" s="41">
+        <f>MAX(0,A476*60-spg_dur)</f>
+        <v>333.11837546774234</v>
+      </c>
+      <c r="C476" s="41">
+        <f>k_eff_CO2*B476</f>
+        <v>0.0048371774127123615</v>
+      </c>
+      <c r="D476" s="41">
+        <f>EXP(-C476)</f>
+        <v>0.9951745028891287</v>
+      </c>
+      <c r="E476" s="41">
+        <f>IF(C476&gt;0,(1-D476)/C476,1)</f>
+        <v>0.9975853062965313</v>
+      </c>
+      <c r="F476" s="41">
+        <f>IF(C476&gt;0,(C476-1+D476)/C476^2,1/2)</f>
+        <v>0.49919477774965354</v>
+      </c>
+      <c r="G476" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B476/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.06391979979027676</v>
+      </c>
+      <c r="H476" s="41">
+        <f>(G476*E476+pool_b*D476)/(1-pool_ret*D476)</f>
+        <v>26.00070649357209</v>
+      </c>
+      <c r="I476" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H476+pool_b)*E476+G476*F476))</f>
+        <v>26.095704520890113</v>
+      </c>
+      <c r="J476" s="41">
+        <f>IF(AND(I476&gt;=CO2_pH_hi_mt,I477&lt;CO2_pH_hi_mt),EXP(LN(A476)+(LN(A477)-LN(A476))*(I476-CO2_pH_hi_mt)/(I476-I477)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="41">
+        <f>A476*grid_ratio</f>
+        <v>6.063458820997319</v>
+      </c>
+      <c r="B477" s="41">
+        <f>MAX(0,A477*60-spg_dur)</f>
+        <v>363.1575292598392</v>
+      </c>
+      <c r="C477" s="41">
+        <f>k_eff_CO2*B477</f>
+        <v>0.005273372852294751</v>
+      </c>
+      <c r="D477" s="41">
+        <f>EXP(-C477)</f>
+        <v>0.9947405069697814</v>
+      </c>
+      <c r="E477" s="41">
+        <f>IF(C477&gt;0,(1-D477)/C477,1)</f>
+        <v>0.9973679422136522</v>
+      </c>
+      <c r="F477" s="41">
+        <f>IF(C477&gt;0,(C477-1+D477)/C477^2,1/2)</f>
+        <v>0.49912226199016396</v>
+      </c>
+      <c r="G477" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B477/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.06968380693507656</v>
+      </c>
+      <c r="H477" s="41">
+        <f>(G477*E477+pool_b*D477)/(1-pool_ret*D477)</f>
+        <v>25.824949307106877</v>
+      </c>
+      <c r="I477" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H477+pool_b)*E477+G477*F477))</f>
+        <v>25.928064679456654</v>
+      </c>
+      <c r="J477" s="41">
+        <f>IF(AND(I477&gt;=CO2_pH_hi_mt,I478&lt;CO2_pH_hi_mt),EXP(LN(A477)+(LN(A478)-LN(A477))*(I477-CO2_pH_hi_mt)/(I477-I478)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="41">
+        <f>A477*grid_ratio</f>
+        <v>6.609170114887078</v>
+      </c>
+      <c r="B478" s="41">
+        <f>MAX(0,A478*60-spg_dur)</f>
+        <v>395.9002068932247</v>
+      </c>
+      <c r="C478" s="41">
+        <f>k_eff_CO2*B478</f>
+        <v>0.005748825881439558</v>
+      </c>
+      <c r="D478" s="41">
+        <f>EXP(-C478)</f>
+        <v>0.9942676669980354</v>
+      </c>
+      <c r="E478" s="41">
+        <f>IF(C478&gt;0,(1-D478)/C478,1)</f>
+        <v>0.997131087318512</v>
+      </c>
+      <c r="F478" s="41">
+        <f>IF(C478&gt;0,(C478-1+D478)/C478^2,1/2)</f>
+        <v>0.49904323781111204</v>
+      </c>
+      <c r="G478" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B478/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.0759665747229083</v>
+      </c>
+      <c r="H478" s="41">
+        <f>(G478*E478+pool_b*D478)/(1-pool_ret*D478)</f>
+        <v>25.635073654350986</v>
+      </c>
+      <c r="I478" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H478+pool_b)*E478+G478*F478))</f>
+        <v>25.746957025750188</v>
+      </c>
+      <c r="J478" s="41">
+        <f>IF(AND(I478&gt;=CO2_pH_hi_mt,I479&lt;CO2_pH_hi_mt),EXP(LN(A478)+(LN(A479)-LN(A478))*(I478-CO2_pH_hi_mt)/(I478-I479)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="41">
+        <f>A478*grid_ratio</f>
+        <v>7.203995425226916</v>
+      </c>
+      <c r="B479" s="41">
+        <f>MAX(0,A479*60-spg_dur)</f>
+        <v>431.58972551361495</v>
+      </c>
+      <c r="C479" s="41">
+        <f>k_eff_CO2*B479</f>
+        <v>0.006267069683207395</v>
+      </c>
+      <c r="D479" s="41">
+        <f>EXP(-C479)</f>
+        <v>0.9937525274377871</v>
+      </c>
+      <c r="E479" s="41">
+        <f>IF(C479&gt;0,(1-D479)/C479,1)</f>
+        <v>0.9968730009422128</v>
+      </c>
+      <c r="F479" s="41">
+        <f>IF(C479&gt;0,(C479-1+D479)/C479^2,1/2)</f>
+        <v>0.498957122843962</v>
+      </c>
+      <c r="G479" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B479/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.08281479161164493</v>
+      </c>
+      <c r="H479" s="41">
+        <f>(G479*E479+pool_b*D479)/(1-pool_ret*D479)</f>
+        <v>25.43010064726742</v>
+      </c>
+      <c r="I479" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H479+pool_b)*E479+G479*F479))</f>
+        <v>25.551447513453944</v>
+      </c>
+      <c r="J479" s="41">
+        <f>IF(AND(I479&gt;=CO2_pH_hi_mt,I480&lt;CO2_pH_hi_mt),EXP(LN(A479)+(LN(A480)-LN(A479))*(I479-CO2_pH_hi_mt)/(I479-I480)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="41">
+        <f>A479*grid_ratio</f>
+        <v>7.8523550134973386</v>
+      </c>
+      <c r="B480" s="41">
+        <f>MAX(0,A480*60-spg_dur)</f>
+        <v>470.4913008098403</v>
+      </c>
+      <c r="C480" s="41">
+        <f>k_eff_CO2*B480</f>
+        <v>0.006831955427134338</v>
+      </c>
+      <c r="D480" s="41">
+        <f>EXP(-C480)</f>
+        <v>0.9931913293233763</v>
+      </c>
+      <c r="E480" s="41">
+        <f>IF(C480&gt;0,(1-D480)/C480,1)</f>
+        <v>0.9965917882868293</v>
+      </c>
+      <c r="F480" s="41">
+        <f>IF(C480&gt;0,(C480-1+D480)/C480^2,1/2)</f>
+        <v>0.4988632829238114</v>
+      </c>
+      <c r="G480" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B480/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.09027934802036784</v>
+      </c>
+      <c r="H480" s="41">
+        <f>(G480*E480+pool_b*D480)/(1-pool_ret*D480)</f>
+        <v>25.20901063305166</v>
+      </c>
+      <c r="I480" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H480+pool_b)*E480+G480*F480))</f>
+        <v>25.34056314188324</v>
+      </c>
+      <c r="J480" s="41">
+        <f>IF(AND(I480&gt;=CO2_pH_hi_mt,I481&lt;CO2_pH_hi_mt),EXP(LN(A480)+(LN(A481)-LN(A480))*(I480-CO2_pH_hi_mt)/(I480-I481)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="41">
+        <f>A480*grid_ratio</f>
+        <v>8.5590669647121</v>
+      </c>
+      <c r="B481" s="41">
+        <f>MAX(0,A481*60-spg_dur)</f>
+        <v>512.8940178827261</v>
+      </c>
+      <c r="C481" s="41">
+        <f>k_eff_CO2*B481</f>
+        <v>0.007447680888014709</v>
+      </c>
+      <c r="D481" s="41">
+        <f>EXP(-C481)</f>
+        <v>0.992579984364029</v>
+      </c>
+      <c r="E481" s="41">
+        <f>IF(C481&gt;0,(1-D481)/C481,1)</f>
+        <v>0.9962853870272175</v>
+      </c>
+      <c r="F481" s="41">
+        <f>IF(C481&gt;0,(C481-1+D481)/C481^2,1/2)</f>
+        <v>0.49876102757881635</v>
+      </c>
+      <c r="G481" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B481/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.09841571450587584</v>
+      </c>
+      <c r="H481" s="41">
+        <f>(G481*E481+pool_b*D481)/(1-pool_ret*D481)</f>
+        <v>24.970746463634658</v>
+      </c>
+      <c r="I481" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H481+pool_b)*E481+G481*F481))</f>
+        <v>25.11329506223249</v>
+      </c>
+      <c r="J481" s="41">
+        <f>IF(AND(I481&gt;=CO2_pH_hi_mt,I482&lt;CO2_pH_hi_mt),EXP(LN(A481)+(LN(A482)-LN(A481))*(I481-CO2_pH_hi_mt)/(I481-I482)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="41">
+        <f>A481*grid_ratio</f>
+        <v>9.329382991536189</v>
+      </c>
+      <c r="B482" s="41">
+        <f>MAX(0,A482*60-spg_dur)</f>
+        <v>559.1129794921713</v>
+      </c>
+      <c r="C482" s="41">
+        <f>k_eff_CO2*B482</f>
+        <v>0.00811882164037431</v>
+      </c>
+      <c r="D482" s="41">
+        <f>EXP(-C482)</f>
+        <v>0.9919140469804008</v>
+      </c>
+      <c r="E482" s="41">
+        <f>IF(C482&gt;0,(1-D482)/C482,1)</f>
+        <v>0.9959515527953453</v>
+      </c>
+      <c r="F482" s="41">
+        <f>IF(C482&gt;0,(C482-1+D482)/C482^2,1/2)</f>
+        <v>0.4986496050767622</v>
+      </c>
+      <c r="G482" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B482/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.10728435397507952</v>
+      </c>
+      <c r="H482" s="41">
+        <f>(G482*E482+pool_b*D482)/(1-pool_ret*D482)</f>
+        <v>24.714217880236223</v>
+      </c>
+      <c r="I482" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H482+pool_b)*E482+G482*F482))</f>
+        <v>24.868602745599283</v>
+      </c>
+      <c r="J482" s="41">
+        <f>IF(AND(I482&gt;=CO2_pH_hi_mt,I483&lt;CO2_pH_hi_mt),EXP(LN(A482)+(LN(A483)-LN(A482))*(I482-CO2_pH_hi_mt)/(I482-I483)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="41">
+        <f>A482*grid_ratio</f>
+        <v>10.169027460774448</v>
+      </c>
+      <c r="B483" s="41">
+        <f>MAX(0,A483*60-spg_dur)</f>
+        <v>609.4916476464668</v>
+      </c>
+      <c r="C483" s="41">
+        <f>k_eff_CO2*B483</f>
+        <v>0.008850365060446275</v>
+      </c>
+      <c r="D483" s="41">
+        <f>EXP(-C483)</f>
+        <v>0.9911886841356119</v>
+      </c>
+      <c r="E483" s="41">
+        <f>IF(C483&gt;0,(1-D483)/C483,1)</f>
+        <v>0.9955878434627866</v>
+      </c>
+      <c r="F483" s="41">
+        <f>IF(C483&gt;0,(C483-1+D483)/C483^2,1/2)</f>
+        <v>0.49852819709402535</v>
+      </c>
+      <c r="G483" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B483/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.11695117099651156</v>
+      </c>
+      <c r="H483" s="41">
+        <f>(G483*E483+pool_b*D483)/(1-pool_ret*D483)</f>
+        <v>24.438307158409216</v>
+      </c>
+      <c r="I483" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H483+pool_b)*E483+G483*F483))</f>
+        <v>24.60541935129978</v>
+      </c>
+      <c r="J483" s="41">
+        <f>IF(AND(I483&gt;=CO2_pH_hi_mt,I484&lt;CO2_pH_hi_mt),EXP(LN(A483)+(LN(A484)-LN(A483))*(I483-CO2_pH_hi_mt)/(I483-I484)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="41">
+        <f>A483*grid_ratio</f>
+        <v>11.084239932244149</v>
+      </c>
+      <c r="B484" s="41">
+        <f>MAX(0,A484*60-spg_dur)</f>
+        <v>664.404395934649</v>
+      </c>
+      <c r="C484" s="41">
+        <f>k_eff_CO2*B484</f>
+        <v>0.00964774738832472</v>
+      </c>
+      <c r="D484" s="41">
+        <f>EXP(-C484)</f>
+        <v>0.9903986428196412</v>
+      </c>
+      <c r="E484" s="41">
+        <f>IF(C484&gt;0,(1-D484)/C484,1)</f>
+        <v>0.9951916021327379</v>
+      </c>
+      <c r="F484" s="41">
+        <f>IF(C484&gt;0,(C484-1+D484)/C484^2,1/2)</f>
+        <v>0.498395912924052</v>
+      </c>
+      <c r="G484" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B484/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.1274880015498725</v>
+      </c>
+      <c r="H484" s="41">
+        <f>(G484*E484+pool_b*D484)/(1-pool_ret*D484)</f>
+        <v>24.14187615949378</v>
+      </c>
+      <c r="I484" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H484+pool_b)*E484+G484*F484))</f>
+        <v>24.322658434457665</v>
+      </c>
+      <c r="J484" s="41">
+        <f>IF(AND(I484&gt;=CO2_pH_hi_mt,I485&lt;CO2_pH_hi_mt),EXP(LN(A484)+(LN(A485)-LN(A484))*(I484-CO2_pH_hi_mt)/(I484-I485)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="41">
+        <f>A484*grid_ratio</f>
+        <v>12.081821526146124</v>
+      </c>
+      <c r="B485" s="41">
+        <f>MAX(0,A485*60-spg_dur)</f>
+        <v>724.2592915687675</v>
+      </c>
+      <c r="C485" s="41">
+        <f>k_eff_CO2*B485</f>
+        <v>0.010516894125712224</v>
+      </c>
+      <c r="D485" s="41">
+        <f>EXP(-C485)</f>
+        <v>0.9895382150436837</v>
+      </c>
+      <c r="E485" s="41">
+        <f>IF(C485&gt;0,(1-D485)/C485,1)</f>
+        <v>0.9947599387483461</v>
+      </c>
+      <c r="F485" s="41">
+        <f>IF(C485&gt;0,(C485-1+D485)/C485^2,1/2)</f>
+        <v>0.4982517831801733</v>
+      </c>
+      <c r="G485" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B485/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.13897314685303588</v>
+      </c>
+      <c r="H485" s="41">
+        <f>(G485*E485+pool_b*D485)/(1-pool_ret*D485)</f>
+        <v>23.823774929736796</v>
+      </c>
+      <c r="I485" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H485+pool_b)*E485+G485*F485))</f>
+        <v>24.019222127391632</v>
+      </c>
+      <c r="J485" s="41">
+        <f>IF(AND(I485&gt;=CO2_pH_hi_mt,I486&lt;CO2_pH_hi_mt),EXP(LN(A485)+(LN(A486)-LN(A485))*(I485-CO2_pH_hi_mt)/(I485-I486)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="41">
+        <f>A485*grid_ratio</f>
+        <v>13.169185463499275</v>
+      </c>
+      <c r="B486" s="41">
+        <f>MAX(0,A486*60-spg_dur)</f>
+        <v>789.5011278099565</v>
+      </c>
+      <c r="C486" s="41">
+        <f>k_eff_CO2*B486</f>
+        <v>0.0114642640694646</v>
+      </c>
+      <c r="D486" s="41">
+        <f>EXP(-C486)</f>
+        <v>0.9886012002004883</v>
+      </c>
+      <c r="E486" s="41">
+        <f>IF(C486&gt;0,(1-D486)/C486,1)</f>
+        <v>0.9942897102198459</v>
+      </c>
+      <c r="F486" s="41">
+        <f>IF(C486&gt;0,(C486-1+D486)/C486^2,1/2)</f>
+        <v>0.4980947530124414</v>
+      </c>
+      <c r="G486" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B486/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.151491955233484</v>
+      </c>
+      <c r="H486" s="41">
+        <f>(G486*E486+pool_b*D486)/(1-pool_ret*D486)</f>
+        <v>23.4828519771669</v>
+      </c>
+      <c r="I486" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H486+pool_b)*E486+G486*F486))</f>
+        <v>23.69401091866648</v>
+      </c>
+      <c r="J486" s="41">
+        <f>IF(AND(I486&gt;=CO2_pH_hi_mt,I487&lt;CO2_pH_hi_mt),EXP(LN(A486)+(LN(A487)-LN(A486))*(I486-CO2_pH_hi_mt)/(I486-I487)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="41">
+        <f>A486*grid_ratio</f>
+        <v>14.354412155214211</v>
+      </c>
+      <c r="B487" s="41">
+        <f>MAX(0,A487*60-spg_dur)</f>
+        <v>860.6147293128527</v>
+      </c>
+      <c r="C487" s="41">
+        <f>k_eff_CO2*B487</f>
+        <v>0.012496897308154693</v>
+      </c>
+      <c r="D487" s="41">
+        <f>EXP(-C487)</f>
+        <v>0.9875808646482231</v>
+      </c>
+      <c r="E487" s="41">
+        <f>IF(C487&gt;0,(1-D487)/C487,1)</f>
+        <v>0.9937774989695166</v>
+      </c>
+      <c r="F487" s="41">
+        <f>IF(C487&gt;0,(C487-1+D487)/C487^2,1/2)</f>
+        <v>0.49792367473692745</v>
+      </c>
+      <c r="G487" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B487/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.16513745636817243</v>
+      </c>
+      <c r="H487" s="41">
+        <f>(G487*E487+pool_b*D487)/(1-pool_ret*D487)</f>
+        <v>23.117966337201608</v>
+      </c>
+      <c r="I487" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H487+pool_b)*E487+G487*F487))</f>
+        <v>23.34593513547111</v>
+      </c>
+      <c r="J487" s="41">
+        <f>IF(AND(I487&gt;=CO2_pH_hi_mt,I488&lt;CO2_pH_hi_mt),EXP(LN(A487)+(LN(A488)-LN(A487))*(I487-CO2_pH_hi_mt)/(I487-I488)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="41">
+        <f>A487*grid_ratio</f>
+        <v>15.64630924918349</v>
+      </c>
+      <c r="B488" s="41">
+        <f>MAX(0,A488*60-spg_dur)</f>
+        <v>938.1285549510094</v>
+      </c>
+      <c r="C488" s="41">
+        <f>k_eff_CO2*B488</f>
+        <v>0.013622467538326893</v>
+      </c>
+      <c r="D488" s="41">
+        <f>EXP(-C488)</f>
+        <v>0.9864698983796578</v>
+      </c>
+      <c r="E488" s="41">
+        <f>IF(C488&gt;0,(1-D488)/C488,1)</f>
+        <v>0.9932195897898206</v>
+      </c>
+      <c r="F488" s="41">
+        <f>IF(C488&gt;0,(C488-1+D488)/C488^2,1/2)</f>
+        <v>0.4977372998760988</v>
+      </c>
+      <c r="G488" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B488/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.1800110526049828</v>
+      </c>
+      <c r="H488" s="41">
+        <f>(G488*E488+pool_b*D488)/(1-pool_ret*D488)</f>
+        <v>22.728001509447175</v>
+      </c>
+      <c r="I488" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H488+pool_b)*E488+G488*F488))</f>
+        <v>22.973928207779746</v>
+      </c>
+      <c r="J488" s="41">
+        <f>IF(AND(I488&gt;=CO2_pH_hi_mt,I489&lt;CO2_pH_hi_mt),EXP(LN(A488)+(LN(A489)-LN(A488))*(I488-CO2_pH_hi_mt)/(I488-I489)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="41">
+        <f>A488*grid_ratio</f>
+        <v>17.054477081610006</v>
+      </c>
+      <c r="B489" s="41">
+        <f>MAX(0,A489*60-spg_dur)</f>
+        <v>1022.6186248966004</v>
+      </c>
+      <c r="C489" s="41">
+        <f>k_eff_CO2*B489</f>
+        <v>0.014849339089214594</v>
+      </c>
+      <c r="D489" s="41">
+        <f>EXP(-C489)</f>
+        <v>0.9852603686460555</v>
+      </c>
+      <c r="E489" s="41">
+        <f>IF(C489&gt;0,(1-D489)/C489,1)</f>
+        <v>0.9926119449080558</v>
+      </c>
+      <c r="F489" s="41">
+        <f>IF(C489&gt;0,(C489-1+D489)/C489^2,1/2)</f>
+        <v>0.49753427055285904</v>
+      </c>
+      <c r="G489" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B489/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.19622327250310617</v>
+      </c>
+      <c r="H489" s="41">
+        <f>(G489*E489+pool_b*D489)/(1-pool_ret*D489)</f>
+        <v>22.31188130885804</v>
+      </c>
+      <c r="I489" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H489+pool_b)*E489+G489*F489))</f>
+        <v>22.57696175531391</v>
+      </c>
+      <c r="J489" s="41">
+        <f>IF(AND(I489&gt;=CO2_pH_hi_mt,I490&lt;CO2_pH_hi_mt),EXP(LN(A489)+(LN(A490)-LN(A489))*(I489-CO2_pH_hi_mt)/(I489-I490)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="41">
+        <f>A489*grid_ratio</f>
+        <v>18.58938001895491</v>
+      </c>
+      <c r="B490" s="41">
+        <f>MAX(0,A490*60-spg_dur)</f>
+        <v>1114.7128011372945</v>
+      </c>
+      <c r="C490" s="41">
+        <f>k_eff_CO2*B490</f>
+        <v>0.016186629079682185</v>
+      </c>
+      <c r="D490" s="41">
+        <f>EXP(-C490)</f>
+        <v>0.9839436704169676</v>
+      </c>
+      <c r="E490" s="41">
+        <f>IF(C490&gt;0,(1-D490)/C490,1)</f>
+        <v>0.9919501771487826</v>
+      </c>
+      <c r="F490" s="41">
+        <f>IF(C490&gt;0,(C490-1+D490)/C490^2,1/2)</f>
+        <v>0.4973131101966102</v>
+      </c>
+      <c r="G490" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B490/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.21389459219206058</v>
+      </c>
+      <c r="H490" s="41">
+        <f>(G490*E490+pool_b*D490)/(1-pool_ret*D490)</f>
+        <v>21.86858762321278</v>
+      </c>
+      <c r="I490" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H490+pool_b)*E490+G490*F490))</f>
+        <v>22.154062489492794</v>
+      </c>
+      <c r="J490" s="41">
+        <f>IF(AND(I490&gt;=CO2_pH_hi_mt,I491&lt;CO2_pH_hi_mt),EXP(LN(A490)+(LN(A491)-LN(A490))*(I490-CO2_pH_hi_mt)/(I490-I491)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="41">
+        <f>A490*grid_ratio</f>
+        <v>20.26242422066085</v>
+      </c>
+      <c r="B491" s="41">
+        <f>MAX(0,A491*60-spg_dur)</f>
+        <v>1215.0954532396509</v>
+      </c>
+      <c r="C491" s="41">
+        <f>k_eff_CO2*B491</f>
+        <v>0.01764427516929186</v>
+      </c>
+      <c r="D491" s="41">
+        <f>EXP(-C491)</f>
+        <v>0.9825104735740383</v>
+      </c>
+      <c r="E491" s="41">
+        <f>IF(C491&gt;0,(1-D491)/C491,1)</f>
+        <v>0.9912295210857119</v>
+      </c>
+      <c r="F491" s="41">
+        <f>IF(C491&gt;0,(C491-1+D491)/C491^2,1/2)</f>
+        <v>0.4970722135162926</v>
+      </c>
+      <c r="G491" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B491/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.23315633065302088</v>
+      </c>
+      <c r="H491" s="41">
+        <f>(G491*E491+pool_b*D491)/(1-pool_ret*D491)</f>
+        <v>21.397180004974093</v>
+      </c>
+      <c r="I491" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H491+pool_b)*E491+G491*F491))</f>
+        <v>21.70433086167661</v>
+      </c>
+      <c r="J491" s="41">
+        <f>IF(AND(I491&gt;=CO2_pH_hi_mt,I492&lt;CO2_pH_hi_mt),EXP(LN(A491)+(LN(A492)-LN(A491))*(I491-CO2_pH_hi_mt)/(I491-I492)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="41">
+        <f>A491*grid_ratio</f>
+        <v>22.08604240052033</v>
+      </c>
+      <c r="B492" s="41">
+        <f>MAX(0,A492*60-spg_dur)</f>
+        <v>1324.5125440312197</v>
+      </c>
+      <c r="C492" s="41">
+        <f>k_eff_CO2*B492</f>
+        <v>0.019233109406966407</v>
+      </c>
+      <c r="D492" s="41">
+        <f>EXP(-C492)</f>
+        <v>0.9809506667601157</v>
+      </c>
+      <c r="E492" s="41">
+        <f>IF(C492&gt;0,(1-D492)/C492,1)</f>
+        <v>0.9904448020757629</v>
+      </c>
+      <c r="F492" s="41">
+        <f>IF(C492&gt;0,(C492-1+D492)/C492^2,1/2)</f>
+        <v>0.49680983568769094</v>
+      </c>
+      <c r="G492" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B492/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.25415162557546767</v>
+      </c>
+      <c r="H492" s="41">
+        <f>(G492*E492+pool_b*D492)/(1-pool_ret*D492)</f>
+        <v>20.896816948876385</v>
+      </c>
+      <c r="I492" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H492+pool_b)*E492+G492*F492))</f>
+        <v>21.226961315867836</v>
+      </c>
+      <c r="J492" s="41">
+        <f>IF(AND(I492&gt;=CO2_pH_hi_mt,I493&lt;CO2_pH_hi_mt),EXP(LN(A492)+(LN(A493)-LN(A492))*(I492-CO2_pH_hi_mt)/(I492-I493)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="41">
+        <f>A492*grid_ratio</f>
+        <v>24.07378621656716</v>
+      </c>
+      <c r="B493" s="41">
+        <f>MAX(0,A493*60-spg_dur)</f>
+        <v>1443.7771729940296</v>
+      </c>
+      <c r="C493" s="41">
+        <f>k_eff_CO2*B493</f>
+        <v>0.02096493872603166</v>
+      </c>
+      <c r="D493" s="41">
+        <f>EXP(-C493)</f>
+        <v>0.9792532978357319</v>
+      </c>
+      <c r="E493" s="41">
+        <f>IF(C493&gt;0,(1-D493)/C493,1)</f>
+        <v>0.9895904030717448</v>
+      </c>
+      <c r="F493" s="41">
+        <f>IF(C493&gt;0,(C493-1+D493)/C493^2,1/2)</f>
+        <v>0.49652408071816123</v>
+      </c>
+      <c r="G493" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B493/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.27703649704093464</v>
+      </c>
+      <c r="H493" s="41">
+        <f>(G493*E493+pool_b*D493)/(1-pool_ret*D493)</f>
+        <v>20.36677861766155</v>
+      </c>
+      <c r="I493" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H493+pool_b)*E493+G493*F493))</f>
+        <v>20.72126391927885</v>
+      </c>
+      <c r="J493" s="41">
+        <f>IF(AND(I493&gt;=CO2_pH_hi_mt,I494&lt;CO2_pH_hi_mt),EXP(LN(A493)+(LN(A494)-LN(A493))*(I493-CO2_pH_hi_mt)/(I493-I494)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="41">
+        <f>A493*grid_ratio</f>
+        <v>26.240426976058206</v>
+      </c>
+      <c r="B494" s="41">
+        <f>MAX(0,A494*60-spg_dur)</f>
+        <v>1573.7756185634923</v>
+      </c>
+      <c r="C494" s="41">
+        <f>k_eff_CO2*B494</f>
+        <v>0.022852632683812792</v>
+      </c>
+      <c r="D494" s="41">
+        <f>EXP(-C494)</f>
+        <v>0.9774065109349087</v>
+      </c>
+      <c r="E494" s="41">
+        <f>IF(C494&gt;0,(1-D494)/C494,1)</f>
+        <v>0.9886602291164001</v>
+      </c>
+      <c r="F494" s="41">
+        <f>IF(C494&gt;0,(C494-1+D494)/C494^2,1/2)</f>
+        <v>0.49621288892597354</v>
+      </c>
+      <c r="G494" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B494/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.30198100693829366</v>
+      </c>
+      <c r="H494" s="41">
+        <f>(G494*E494+pool_b*D494)/(1-pool_ret*D494)</f>
+        <v>19.806490678935862</v>
+      </c>
+      <c r="I494" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H494+pool_b)*E494+G494*F494))</f>
+        <v>20.186687049394266</v>
+      </c>
+      <c r="J494" s="41">
+        <f>IF(AND(I494&gt;=CO2_pH_hi_mt,I495&lt;CO2_pH_hi_mt),EXP(LN(A494)+(LN(A495)-LN(A494))*(I494-CO2_pH_hi_mt)/(I494-I495)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="41">
+        <f>A494*grid_ratio</f>
+        <v>28.60206540390345</v>
+      </c>
+      <c r="B495" s="41">
+        <f>MAX(0,A495*60-spg_dur)</f>
+        <v>1715.4739242342068</v>
+      </c>
+      <c r="C495" s="41">
+        <f>k_eff_CO2*B495</f>
+        <v>0.02491021909779422</v>
+      </c>
+      <c r="D495" s="41">
+        <f>EXP(-C495)</f>
+        <v>0.975397480163079</v>
+      </c>
+      <c r="E495" s="41">
+        <f>IF(C495&gt;0,(1-D495)/C495,1)</f>
+        <v>0.9876476694297521</v>
+      </c>
+      <c r="F495" s="41">
+        <f>IF(C495&gt;0,(C495-1+D495)/C495^2,1/2)</f>
+        <v>0.49587402349832826</v>
+      </c>
+      <c r="G495" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B495/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.32917052272641495</v>
+      </c>
+      <c r="H495" s="41">
+        <f>(G495*E495+pool_b*D495)/(1-pool_ret*D495)</f>
+        <v>19.21554880905163</v>
+      </c>
+      <c r="I495" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H495+pool_b)*E495+G495*F495))</f>
+        <v>19.62284071409303</v>
+      </c>
+      <c r="J495" s="41">
+        <f>IF(AND(I495&gt;=CO2_pH_hi_mt,I496&lt;CO2_pH_hi_mt),EXP(LN(A495)+(LN(A496)-LN(A495))*(I495-CO2_pH_hi_mt)/(I495-I496)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="41">
+        <f>A495*grid_ratio</f>
+        <v>31.17625129025476</v>
+      </c>
+      <c r="B496" s="41">
+        <f>MAX(0,A496*60-spg_dur)</f>
+        <v>1869.9250774152856</v>
+      </c>
+      <c r="C496" s="41">
+        <f>k_eff_CO2*B496</f>
+        <v>0.027152988289033984</v>
+      </c>
+      <c r="D496" s="41">
+        <f>EXP(-C496)</f>
+        <v>0.9732123400437658</v>
+      </c>
+      <c r="E496" s="41">
+        <f>IF(C496&gt;0,(1-D496)/C496,1)</f>
+        <v>0.9865455570152732</v>
+      </c>
+      <c r="F496" s="41">
+        <f>IF(C496&gt;0,(C496-1+D496)/C496^2,1/2)</f>
+        <v>0.4955050560737503</v>
+      </c>
+      <c r="G496" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B496/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.3588070949354672</v>
+      </c>
+      <c r="H496" s="41">
+        <f>(G496*E496+pool_b*D496)/(1-pool_ret*D496)</f>
+        <v>18.593743309502308</v>
+      </c>
+      <c r="I496" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H496+pool_b)*E496+G496*F496))</f>
+        <v>19.02951997616225</v>
+      </c>
+      <c r="J496" s="41">
+        <f>IF(AND(I496&gt;=CO2_pH_hi_mt,I497&lt;CO2_pH_hi_mt),EXP(LN(A496)+(LN(A497)-LN(A496))*(I496-CO2_pH_hi_mt)/(I496-I497)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="41">
+        <f>A496*grid_ratio</f>
+        <v>33.98211390637769</v>
+      </c>
+      <c r="B497" s="41">
+        <f>MAX(0,A497*60-spg_dur)</f>
+        <v>2038.2768343826615</v>
+      </c>
+      <c r="C497" s="41">
+        <f>k_eff_CO2*B497</f>
+        <v>0.029597606707485322</v>
+      </c>
+      <c r="D497" s="41">
+        <f>EXP(-C497)</f>
+        <v>0.9708361128999443</v>
+      </c>
+      <c r="E497" s="41">
+        <f>IF(C497&gt;0,(1-D497)/C497,1)</f>
+        <v>0.9853461257284716</v>
+      </c>
+      <c r="F497" s="41">
+        <f>IF(C497&gt;0,(C497-1+D497)/C497^2,1/2)</f>
+        <v>0.49510335130655203</v>
+      </c>
+      <c r="G497" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B497/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.39111095864333423</v>
+      </c>
+      <c r="H497" s="41">
+        <f>(G497*E497+pool_b*D497)/(1-pool_ret*D497)</f>
+        <v>17.941083173279143</v>
+      </c>
+      <c r="I497" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H497+pool_b)*E497+G497*F497))</f>
+        <v>18.40672785054989</v>
+      </c>
+      <c r="J497" s="41">
+        <f>IF(AND(I497&gt;=CO2_pH_hi_mt,I498&lt;CO2_pH_hi_mt),EXP(LN(A497)+(LN(A498)-LN(A497))*(I497-CO2_pH_hi_mt)/(I497-I498)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="41">
+        <f>A497*grid_ratio</f>
+        <v>37.04050415795169</v>
+      </c>
+      <c r="B498" s="41">
+        <f>MAX(0,A498*60-spg_dur)</f>
+        <v>2221.7802494771013</v>
+      </c>
+      <c r="C498" s="41">
+        <f>k_eff_CO2*B498</f>
+        <v>0.03226224078359728</v>
+      </c>
+      <c r="D498" s="41">
+        <f>EXP(-C498)</f>
+        <v>0.9682526334534927</v>
+      </c>
+      <c r="E498" s="41">
+        <f>IF(C498&gt;0,(1-D498)/C498,1)</f>
+        <v>0.9840409647754004</v>
+      </c>
+      <c r="F498" s="41">
+        <f>IF(C498&gt;0,(C498-1+D498)/C498^2,1/2)</f>
+        <v>0.4946660503728531</v>
+      </c>
+      <c r="G498" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B498/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.42632217008490914</v>
+      </c>
+      <c r="H498" s="41">
+        <f>(G498*E498+pool_b*D498)/(1-pool_ret*D498)</f>
+        <v>17.25781884005553</v>
+      </c>
+      <c r="I498" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H498+pool_b)*E498+G498*F498))</f>
+        <v>17.754696948734153</v>
+      </c>
+      <c r="J498" s="41">
+        <f>IF(AND(I498&gt;=CO2_pH_hi_mt,I499&lt;CO2_pH_hi_mt),EXP(LN(A498)+(LN(A499)-LN(A498))*(I498-CO2_pH_hi_mt)/(I498-I499)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="41">
+        <f>A498*grid_ratio</f>
+        <v>40.374149532167344</v>
+      </c>
+      <c r="B499" s="41">
+        <f>MAX(0,A499*60-spg_dur)</f>
+        <v>2421.7989719300404</v>
+      </c>
+      <c r="C499" s="41">
+        <f>k_eff_CO2*B499</f>
+        <v>0.035166691926559315</v>
+      </c>
+      <c r="D499" s="41">
+        <f>EXP(-C499)</f>
+        <v>0.9654444710449408</v>
+      </c>
+      <c r="E499" s="41">
+        <f>IF(C499&gt;0,(1-D499)/C499,1)</f>
+        <v>0.9826209706395915</v>
+      </c>
+      <c r="F499" s="41">
+        <f>IF(C499&gt;0,(C499-1+D499)/C499^2,1/2)</f>
+        <v>0.4941900533806751</v>
+      </c>
+      <c r="G499" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B499/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.4647023905562259</v>
+      </c>
+      <c r="H499" s="41">
+        <f>(G499*E499+pool_b*D499)/(1-pool_ret*D499)</f>
+        <v>16.54446279814715</v>
+      </c>
+      <c r="I499" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H499+pool_b)*E499+G499*F499))</f>
+        <v>17.073909067454217</v>
+      </c>
+      <c r="J499" s="41">
+        <f>IF(AND(I499&gt;=CO2_pH_hi_mt,I500&lt;CO2_pH_hi_mt),EXP(LN(A499)+(LN(A500)-LN(A499))*(I499-CO2_pH_hi_mt)/(I499-I500)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="41">
+        <f>A499*grid_ratio</f>
+        <v>44.00782299006241</v>
+      </c>
+      <c r="B500" s="41">
+        <f>MAX(0,A500*60-spg_dur)</f>
+        <v>2639.8193794037443</v>
+      </c>
+      <c r="C500" s="41">
+        <f>k_eff_CO2*B500</f>
+        <v>0.038332543672387934</v>
+      </c>
+      <c r="D500" s="41">
+        <f>EXP(-C500)</f>
+        <v>0.962392850019427</v>
+      </c>
+      <c r="E500" s="41">
+        <f>IF(C500&gt;0,(1-D500)/C500,1)</f>
+        <v>0.9810762964750123</v>
+      </c>
+      <c r="F500" s="41">
+        <f>IF(C500&gt;0,(C500-1+D500)/C500^2,1/2)</f>
+        <v>0.4936720006561611</v>
+      </c>
+      <c r="G500" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B500/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.5065368308699612</v>
+      </c>
+      <c r="H500" s="41">
+        <f>(G500*E500+pool_b*D500)/(1-pool_ret*D500)</f>
+        <v>15.80180713684607</v>
+      </c>
+      <c r="I500" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H500+pool_b)*E500+G500*F500))</f>
+        <v>16.365111867225448</v>
+      </c>
+      <c r="J500" s="41">
+        <f>IF(AND(I500&gt;=CO2_pH_hi_mt,I501&lt;CO2_pH_hi_mt),EXP(LN(A500)+(LN(A501)-LN(A500))*(I500-CO2_pH_hi_mt)/(I500-I501)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="41">
+        <f>A500*grid_ratio</f>
+        <v>47.968527059168025</v>
+      </c>
+      <c r="B501" s="41">
+        <f>MAX(0,A501*60-spg_dur)</f>
+        <v>2877.461623550081</v>
+      </c>
+      <c r="C501" s="41">
+        <f>k_eff_CO2*B501</f>
+        <v>0.04178332207534113</v>
+      </c>
+      <c r="D501" s="41">
+        <f>EXP(-C501)</f>
+        <v>0.9590775689973264</v>
+      </c>
+      <c r="E501" s="41">
+        <f>IF(C501&gt;0,(1-D501)/C501,1)</f>
+        <v>0.9793962990516825</v>
+      </c>
+      <c r="F501" s="41">
+        <f>IF(C501&gt;0,(C501-1+D501)/C501^2,1/2)</f>
+        <v>0.4931082528853263</v>
+      </c>
+      <c r="G501" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B501/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.5521363708119325</v>
+      </c>
+      <c r="H501" s="41">
+        <f>(G501*E501+pool_b*D501)/(1-pool_ret*D501)</f>
+        <v>15.03093713389027</v>
+      </c>
+      <c r="I501" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H501+pool_b)*E501+G501*F501))</f>
+        <v>15.629331768087608</v>
+      </c>
+      <c r="J501" s="41">
+        <f>IF(AND(I501&gt;=CO2_pH_hi_mt,I502&lt;CO2_pH_hi_mt),EXP(LN(A501)+(LN(A502)-LN(A501))*(I501-CO2_pH_hi_mt)/(I501-I502)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="41">
+        <f>A501*grid_ratio</f>
+        <v>52.28569449449315</v>
+      </c>
+      <c r="B502" s="41">
+        <f>MAX(0,A502*60-spg_dur)</f>
+        <v>3136.491669669589</v>
+      </c>
+      <c r="C502" s="41">
+        <f>k_eff_CO2*B502</f>
+        <v>0.045544670534560114</v>
+      </c>
+      <c r="D502" s="41">
+        <f>EXP(-C502)</f>
+        <v>0.9554769199538596</v>
+      </c>
+      <c r="E502" s="41">
+        <f>IF(C502&gt;0,(1-D502)/C502,1)</f>
+        <v>0.977569483401037</v>
+      </c>
+      <c r="F502" s="41">
+        <f>IF(C502&gt;0,(C502-1+D502)/C502^2,1/2)</f>
+        <v>0.49249487010653925</v>
+      </c>
+      <c r="G502" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B502/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.6018398693486814</v>
+      </c>
+      <c r="H502" s="41">
+        <f>(G502*E502+pool_b*D502)/(1-pool_ret*D502)</f>
+        <v>14.233239987677994</v>
+      </c>
+      <c r="I502" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H502+pool_b)*E502+G502*F502))</f>
+        <v>14.867882213683291</v>
+      </c>
+      <c r="J502" s="41">
+        <f>IF(AND(I502&gt;=CO2_pH_hi_mt,I503&lt;CO2_pH_hi_mt),EXP(LN(A502)+(LN(A503)-LN(A502))*(I502-CO2_pH_hi_mt)/(I502-I503)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="41">
+        <f>A502*grid_ratio</f>
+        <v>56.99140699899754</v>
+      </c>
+      <c r="B503" s="41">
+        <f>MAX(0,A503*60-spg_dur)</f>
+        <v>3418.8344199398525</v>
+      </c>
+      <c r="C503" s="41">
+        <f>k_eff_CO2*B503</f>
+        <v>0.049644540355108804</v>
+      </c>
+      <c r="D503" s="41">
+        <f>EXP(-C503)</f>
+        <v>0.9515676082759386</v>
+      </c>
+      <c r="E503" s="41">
+        <f>IF(C503&gt;0,(1-D503)/C503,1)</f>
+        <v>0.9755834453823757</v>
+      </c>
+      <c r="F503" s="41">
+        <f>IF(C503&gt;0,(C503-1+D503)/C503^2,1/2)</f>
+        <v>0.4918275895591262</v>
+      </c>
+      <c r="G503" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B503/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.6560166827537377</v>
+      </c>
+      <c r="H503" s="41">
+        <f>(G503*E503+pool_b*D503)/(1-pool_ret*D503)</f>
+        <v>13.410407878796054</v>
+      </c>
+      <c r="I503" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H503+pool_b)*E503+G503*F503))</f>
+        <v>14.082366526176253</v>
+      </c>
+      <c r="J503" s="41">
+        <f>IF(AND(I503&gt;=CO2_pH_hi_mt,I504&lt;CO2_pH_hi_mt),EXP(LN(A503)+(LN(A504)-LN(A503))*(I503-CO2_pH_hi_mt)/(I503-I504)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="41">
+        <f>A503*grid_ratio</f>
+        <v>62.12063362890732</v>
+      </c>
+      <c r="B504" s="41">
+        <f>MAX(0,A504*60-spg_dur)</f>
+        <v>3726.5880177344393</v>
+      </c>
+      <c r="C504" s="41">
+        <f>k_eff_CO2*B504</f>
+        <v>0.05411339845950688</v>
+      </c>
+      <c r="D504" s="41">
+        <f>EXP(-C504)</f>
+        <v>0.9473246752518178</v>
+      </c>
+      <c r="E504" s="41">
+        <f>IF(C504&gt;0,(1-D504)/C504,1)</f>
+        <v>0.9734248124814996</v>
+      </c>
+      <c r="F504" s="41">
+        <f>IF(C504&gt;0,(C504-1+D504)/C504^2,1/2)</f>
+        <v>0.49110180241936374</v>
+      </c>
+      <c r="G504" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B504/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.715069409365249</v>
+      </c>
+      <c r="H504" s="41">
+        <f>(G504*E504+pool_b*D504)/(1-pool_ret*D504)</f>
+        <v>12.56443467418827</v>
+      </c>
+      <c r="I504" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H504+pool_b)*E504+G504*F504))</f>
+        <v>13.274674697186969</v>
+      </c>
+      <c r="J504" s="41">
+        <f>IF(AND(I504&gt;=CO2_pH_hi_mt,I505&lt;CO2_pH_hi_mt),EXP(LN(A504)+(LN(A505)-LN(A504))*(I504-CO2_pH_hi_mt)/(I504-I505)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="41">
+        <f>A504*grid_ratio</f>
+        <v>67.71149065550898</v>
+      </c>
+      <c r="B505" s="41">
+        <f>MAX(0,A505*60-spg_dur)</f>
+        <v>4062.0394393305387</v>
+      </c>
+      <c r="C505" s="41">
+        <f>k_eff_CO2*B505</f>
+        <v>0.05898445379330077</v>
+      </c>
+      <c r="D505" s="41">
+        <f>EXP(-C505)</f>
+        <v>0.9427214247853093</v>
+      </c>
+      <c r="E505" s="41">
+        <f>IF(C505&gt;0,(1-D505)/C505,1)</f>
+        <v>0.9710791832609322</v>
+      </c>
+      <c r="F505" s="41">
+        <f>IF(C505&gt;0,(C505-1+D505)/C505^2,1/2)</f>
+        <v>0.4903125294745401</v>
+      </c>
+      <c r="G505" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B505/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.7794368813717961</v>
+      </c>
+      <c r="H505" s="41">
+        <f>(G505*E505+pool_b*D505)/(1-pool_ret*D505)</f>
+        <v>11.697605769853773</v>
+      </c>
+      <c r="I505" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H505+pool_b)*E505+G505*F505))</f>
+        <v>12.446973633876029</v>
+      </c>
+      <c r="J505" s="41">
+        <f>IF(AND(I505&gt;=CO2_pH_hi_mt,I506&lt;CO2_pH_hi_mt),EXP(LN(A505)+(LN(A506)-LN(A505))*(I505-CO2_pH_hi_mt)/(I505-I506)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="41">
+        <f>A505*grid_ratio</f>
+        <v>73.8055248145048</v>
+      </c>
+      <c r="B506" s="41">
+        <f>MAX(0,A506*60-spg_dur)</f>
+        <v>4427.681488870288</v>
+      </c>
+      <c r="C506" s="41">
+        <f>k_eff_CO2*B506</f>
+        <v>0.06429390410713613</v>
+      </c>
+      <c r="D506" s="41">
+        <f>EXP(-C506)</f>
+        <v>0.9377293565171443</v>
+      </c>
+      <c r="E506" s="41">
+        <f>IF(C506&gt;0,(1-D506)/C506,1)</f>
+        <v>0.9685310660104112</v>
+      </c>
+      <c r="F506" s="41">
+        <f>IF(C506&gt;0,(C506-1+D506)/C506^2,1/2)</f>
+        <v>0.4894543958187682</v>
+      </c>
+      <c r="G506" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B506/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.8495974258589328</v>
+      </c>
+      <c r="H506" s="41">
+        <f>(G506*E506+pool_b*D506)/(1-pool_ret*D506)</f>
+        <v>10.81248079996858</v>
+      </c>
+      <c r="I506" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H506+pool_b)*E506+G506*F506))</f>
+        <v>11.601690600368505</v>
+      </c>
+      <c r="J506" s="41">
+        <f>IF(AND(I506&gt;=CO2_pH_hi_mt,I507&lt;CO2_pH_hi_mt),EXP(LN(A506)+(LN(A507)-LN(A506))*(I506-CO2_pH_hi_mt)/(I506-I507)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="41">
+        <f>A506*grid_ratio</f>
+        <v>80.44802204781024</v>
+      </c>
+      <c r="B507" s="41">
+        <f>MAX(0,A507*60-spg_dur)</f>
+        <v>4826.231322868614</v>
+      </c>
+      <c r="C507" s="41">
+        <f>k_eff_CO2*B507</f>
+        <v>0.07008120494921667</v>
+      </c>
+      <c r="D507" s="41">
+        <f>EXP(-C507)</f>
+        <v>0.9323181079872856</v>
+      </c>
+      <c r="E507" s="41">
+        <f>IF(C507&gt;0,(1-D507)/C507,1)</f>
+        <v>0.9657638172996462</v>
+      </c>
+      <c r="F507" s="41">
+        <f>IF(C507&gt;0,(C507-1+D507)/C507^2,1/2)</f>
+        <v>0.4885216046893365</v>
+      </c>
+      <c r="G507" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B507/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-0.9260724193499118</v>
+      </c>
+      <c r="H507" s="41">
+        <f>(G507*E507+pool_b*D507)/(1-pool_ret*D507)</f>
+        <v>9.911869212691476</v>
+      </c>
+      <c r="I507" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H507+pool_b)*E507+G507*F507))</f>
+        <v>10.741489854242179</v>
+      </c>
+      <c r="J507" s="41">
+        <f>IF(AND(I507&gt;=CO2_pH_hi_mt,I508&lt;CO2_pH_hi_mt),EXP(LN(A507)+(LN(A508)-LN(A507))*(I507-CO2_pH_hi_mt)/(I507-I508)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="41">
+        <f>A507*grid_ratio</f>
+        <v>87.68834403211316</v>
+      </c>
+      <c r="B508" s="41">
+        <f>MAX(0,A508*60-spg_dur)</f>
+        <v>5260.65064192679</v>
+      </c>
+      <c r="C508" s="41">
+        <f>k_eff_CO2*B508</f>
+        <v>0.07638936286708445</v>
+      </c>
+      <c r="D508" s="41">
+        <f>EXP(-C508)</f>
+        <v>0.9264554089890823</v>
+      </c>
+      <c r="E508" s="41">
+        <f>IF(C508&gt;0,(1-D508)/C508,1)</f>
+        <v>0.962759581316098</v>
+      </c>
+      <c r="F508" s="41">
+        <f>IF(C508&gt;0,(C508-1+D508)/C508^2,1/2)</f>
+        <v>0.48750791060659926</v>
+      </c>
+      <c r="G508" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B508/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.0094301622550788</v>
+      </c>
+      <c r="H508" s="41">
+        <f>(G508*E508+pool_b*D508)/(1-pool_ret*D508)</f>
+        <v>8.998799012005922</v>
+      </c>
+      <c r="I508" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H508+pool_b)*E508+G508*F508))</f>
+        <v>9.869242762800441</v>
+      </c>
+      <c r="J508" s="41">
+        <f>IF(AND(I508&gt;=CO2_pH_hi_mt,I509&lt;CO2_pH_hi_mt),EXP(LN(A508)+(LN(A509)-LN(A508))*(I508-CO2_pH_hi_mt)/(I508-I509)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="41">
+        <f>A508*grid_ratio</f>
+        <v>95.58029499500336</v>
+      </c>
+      <c r="B509" s="41">
+        <f>MAX(0,A509*60-spg_dur)</f>
+        <v>5734.167699700201</v>
+      </c>
+      <c r="C509" s="41">
+        <f>k_eff_CO2*B509</f>
+        <v>0.08326525499756034</v>
+      </c>
+      <c r="D509" s="41">
+        <f>EXP(-C509)</f>
+        <v>0.9201070518540033</v>
+      </c>
+      <c r="E509" s="41">
+        <f>IF(C509&gt;0,(1-D509)/C509,1)</f>
+        <v>0.9594992310818904</v>
+      </c>
+      <c r="F509" s="41">
+        <f>IF(C509&gt;0,(C509-1+D509)/C509^2,1/2)</f>
+        <v>0.4864065920328481</v>
+      </c>
+      <c r="G509" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B509/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.1002901020217108</v>
+      </c>
+      <c r="H509" s="41">
+        <f>(G509*E509+pool_b*D509)/(1-pool_ret*D509)</f>
+        <v>8.076479273282729</v>
+      </c>
+      <c r="I509" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H509+pool_b)*E509+G509*F509))</f>
+        <v>8.987991977656108</v>
+      </c>
+      <c r="J509" s="41">
+        <f>IF(AND(I509&gt;=CO2_pH_hi_mt,I510&lt;CO2_pH_hi_mt),EXP(LN(A509)+(LN(A510)-LN(A509))*(I509-CO2_pH_hi_mt)/(I509-I510)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="41">
+        <f>A509*grid_ratio</f>
+        <v>104.18252154455367</v>
+      </c>
+      <c r="B510" s="41">
+        <f>MAX(0,A510*60-spg_dur)</f>
+        <v>6250.30129267322</v>
+      </c>
+      <c r="C510" s="41">
+        <f>k_eff_CO2*B510</f>
+        <v>0.09075997741977904</v>
+      </c>
+      <c r="D510" s="41">
+        <f>EXP(-C510)</f>
+        <v>0.9132368820679858</v>
+      </c>
+      <c r="E510" s="41">
+        <f>IF(C510&gt;0,(1-D510)/C510,1)</f>
+        <v>0.9559623128895377</v>
+      </c>
+      <c r="F510" s="41">
+        <f>IF(C510&gt;0,(C510-1+D510)/C510^2,1/2)</f>
+        <v>0.48521042382790686</v>
+      </c>
+      <c r="G510" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B510/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.1993274363673396</v>
+      </c>
+      <c r="H510" s="41">
+        <f>(G510*E510+pool_b*D510)/(1-pool_ret*D510)</f>
+        <v>7.148257337755102</v>
+      </c>
+      <c r="I510" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H510+pool_b)*E510+G510*F510))</f>
+        <v>8.1009105296435</v>
+      </c>
+      <c r="J510" s="41">
+        <f>IF(AND(I510&gt;=CO2_pH_hi_mt,I511&lt;CO2_pH_hi_mt),EXP(LN(A510)+(LN(A511)-LN(A510))*(I510-CO2_pH_hi_mt)/(I510-I511)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="41">
+        <f>A510*grid_ratio</f>
+        <v>113.55894848356351</v>
+      </c>
+      <c r="B511" s="41">
+        <f>MAX(0,A511*60-spg_dur)</f>
+        <v>6812.886909013811</v>
+      </c>
+      <c r="C511" s="41">
+        <f>k_eff_CO2*B511</f>
+        <v>0.09892922485999746</v>
+      </c>
+      <c r="D511" s="41">
+        <f>EXP(-C511)</f>
+        <v>0.9058068143590559</v>
+      </c>
+      <c r="E511" s="41">
+        <f>IF(C511&gt;0,(1-D511)/C511,1)</f>
+        <v>0.9521269955793583</v>
+      </c>
+      <c r="F511" s="41">
+        <f>IF(C511&gt;0,(C511-1+D511)/C511^2,1/2)</f>
+        <v>0.4839116498526134</v>
+      </c>
+      <c r="G511" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B511/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.3072781308040753</v>
+      </c>
+      <c r="H511" s="41">
+        <f>(G511*E511+pool_b*D511)/(1-pool_ret*D511)</f>
+        <v>6.2175718568540965</v>
+      </c>
+      <c r="I511" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H511+pool_b)*E511+G511*F511))</f>
+        <v>7.2112569593139115</v>
+      </c>
+      <c r="J511" s="41">
+        <f>IF(AND(I511&gt;=CO2_pH_hi_mt,I512&lt;CO2_pH_hi_mt),EXP(LN(A511)+(LN(A512)-LN(A511))*(I511-CO2_pH_hi_mt)/(I511-I512)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="41">
+        <f>A511*grid_ratio</f>
+        <v>123.77925384708423</v>
+      </c>
+      <c r="B512" s="41">
+        <f>MAX(0,A512*60-spg_dur)</f>
+        <v>7426.105230825055</v>
+      </c>
+      <c r="C512" s="41">
+        <f>k_eff_CO2*B512</f>
+        <v>0.10783370456983551</v>
+      </c>
+      <c r="D512" s="41">
+        <f>EXP(-C512)</f>
+        <v>0.8977768802099719</v>
+      </c>
+      <c r="E512" s="41">
+        <f>IF(C512&gt;0,(1-D512)/C512,1)</f>
+        <v>0.947970026605421</v>
+      </c>
+      <c r="F512" s="41">
+        <f>IF(C512&gt;0,(C512-1+D512)/C512^2,1/2)</f>
+        <v>0.482501956156793</v>
+      </c>
+      <c r="G512" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B512/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.424944387740117</v>
+      </c>
+      <c r="H512" s="41">
+        <f>(G512*E512+pool_b*D512)/(1-pool_ret*D512)</f>
+        <v>5.287903071576869</v>
+      </c>
+      <c r="I512" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H512+pool_b)*E512+G512*F512))</f>
+        <v>6.32232780240464</v>
+      </c>
+      <c r="J512" s="41">
+        <f>IF(AND(I512&gt;=CO2_pH_hi_mt,I513&lt;CO2_pH_hi_mt),EXP(LN(A512)+(LN(A513)-LN(A512))*(I512-CO2_pH_hi_mt)/(I512-I513)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="41">
+        <f>A512*grid_ratio</f>
+        <v>134.91938669332183</v>
+      </c>
+      <c r="B513" s="41">
+        <f>MAX(0,A513*60-spg_dur)</f>
+        <v>8094.5132015993095</v>
+      </c>
+      <c r="C513" s="41">
+        <f>k_eff_CO2*B513</f>
+        <v>0.11753958745355898</v>
+      </c>
+      <c r="D513" s="41">
+        <f>EXP(-C513)</f>
+        <v>0.8891053136344383</v>
+      </c>
+      <c r="E513" s="41">
+        <f>IF(C513&gt;0,(1-D513)/C513,1)</f>
+        <v>0.9434666972042692</v>
+      </c>
+      <c r="F513" s="41">
+        <f>IF(C513&gt;0,(C513-1+D513)/C513^2,1/2)</f>
+        <v>0.4809724452884225</v>
+      </c>
+      <c r="G513" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B513/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.5532006078004024</v>
+      </c>
+      <c r="H513" s="41">
+        <f>(G513*E513+pool_b*D513)/(1-pool_ret*D513)</f>
+        <v>4.362721858149232</v>
+      </c>
+      <c r="I513" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H513+pool_b)*E513+G513*F513))</f>
+        <v>5.437408888882788</v>
+      </c>
+      <c r="J513" s="41">
+        <f>IF(AND(I513&gt;=CO2_pH_hi_mt,I514&lt;CO2_pH_hi_mt),EXP(LN(A513)+(LN(A514)-LN(A513))*(I513-CO2_pH_hi_mt)/(I513-I514)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="41">
+        <f>A513*grid_ratio</f>
+        <v>147.0621314957208</v>
+      </c>
+      <c r="B514" s="41">
+        <f>MAX(0,A514*60-spg_dur)</f>
+        <v>8823.077889743248</v>
+      </c>
+      <c r="C514" s="41">
+        <f>k_eff_CO2*B514</f>
+        <v>0.1281189997968176</v>
+      </c>
+      <c r="D514" s="41">
+        <f>EXP(-C514)</f>
+        <v>0.8797486830008298</v>
+      </c>
+      <c r="E514" s="41">
+        <f>IF(C514&gt;0,(1-D514)/C514,1)</f>
+        <v>0.9385908193934965</v>
+      </c>
+      <c r="F514" s="41">
+        <f>IF(C514&gt;0,(C514-1+D514)/C514^2,1/2)</f>
+        <v>0.47931361237514947</v>
+      </c>
+      <c r="G514" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B514/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.6929998876661139</v>
+      </c>
+      <c r="H514" s="41">
+        <f>(G514*E514+pool_b*D514)/(1-pool_ret*D514)</f>
+        <v>3.4454391375650975</v>
+      </c>
+      <c r="I514" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H514+pool_b)*E514+G514*F514))</f>
+        <v>4.5597269773730735</v>
+      </c>
+      <c r="J514" s="41">
+        <f>IF(AND(I514&gt;=CO2_pH_hi_mt,I515&lt;CO2_pH_hi_mt),EXP(LN(A514)+(LN(A515)-LN(A514))*(I514-CO2_pH_hi_mt)/(I514-I515)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="41">
+        <f>A514*grid_ratio</f>
+        <v>160.29772333033569</v>
+      </c>
+      <c r="B515" s="41">
+        <f>MAX(0,A515*60-spg_dur)</f>
+        <v>9617.21339982014</v>
+      </c>
+      <c r="C515" s="41">
+        <f>k_eff_CO2*B515</f>
+        <v>0.13965055925096945</v>
+      </c>
+      <c r="D515" s="41">
+        <f>EXP(-C515)</f>
+        <v>0.8696620776761042</v>
+      </c>
+      <c r="E515" s="41">
+        <f>IF(C515&gt;0,(1-D515)/C515,1)</f>
+        <v>0.9333147179859292</v>
+      </c>
+      <c r="F515" s="41">
+        <f>IF(C515&gt;0,(C515-1+D515)/C515^2,1/2)</f>
+        <v>0.4775153237605673</v>
+      </c>
+      <c r="G515" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B515/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-1.8453811027197387</v>
+      </c>
+      <c r="H515" s="41">
+        <f>(G515*E515+pool_b*D515)/(1-pool_ret*D515)</f>
+        <v>2.5393572277784644</v>
+      </c>
+      <c r="I515" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H515+pool_b)*E515+G515*F515))</f>
+        <v>3.6924032288782063</v>
+      </c>
+      <c r="J515" s="41">
+        <f>IF(AND(I515&gt;=CO2_pH_hi_mt,I516&lt;CO2_pH_hi_mt),EXP(LN(A515)+(LN(A516)-LN(A515))*(I515-CO2_pH_hi_mt)/(I515-I516)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="41">
+        <f>A515*grid_ratio</f>
+        <v>174.7245184300659</v>
+      </c>
+      <c r="B516" s="41">
+        <f>MAX(0,A516*60-spg_dur)</f>
+        <v>10482.821105803954</v>
+      </c>
+      <c r="C516" s="41">
+        <f>k_eff_CO2*B516</f>
+        <v>0.15221995905599497</v>
+      </c>
+      <c r="D516" s="41">
+        <f>EXP(-C516)</f>
+        <v>0.8587993592680371</v>
+      </c>
+      <c r="E516" s="41">
+        <f>IF(C516&gt;0,(1-D516)/C516,1)</f>
+        <v>0.9276092413086346</v>
+      </c>
+      <c r="F516" s="41">
+        <f>IF(C516&gt;0,(C516-1+D516)/C516^2,1/2)</f>
+        <v>0.4755667991260979</v>
+      </c>
+      <c r="G516" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B516/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-2.0114766271281908</v>
+      </c>
+      <c r="H516" s="41">
+        <f>(G516*E516+pool_b*D516)/(1-pool_ret*D516)</f>
+        <v>1.647624614901869</v>
+      </c>
+      <c r="I516" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H516+pool_b)*E516+G516*F516))</f>
+        <v>2.838409926141868</v>
+      </c>
+      <c r="J516" s="41">
+        <f>IF(AND(I516&gt;=CO2_pH_hi_mt,I517&lt;CO2_pH_hi_mt),EXP(LN(A516)+(LN(A517)-LN(A516))*(I516-CO2_pH_hi_mt)/(I516-I517)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="41">
+        <f>A516*grid_ratio</f>
+        <v>190.44972508877186</v>
+      </c>
+      <c r="B517" s="41">
+        <f>MAX(0,A517*60-spg_dur)</f>
+        <v>11426.333505326313</v>
+      </c>
+      <c r="C517" s="41">
+        <f>k_eff_CO2*B517</f>
+        <v>0.16592060484347285</v>
+      </c>
+      <c r="D517" s="41">
+        <f>EXP(-C517)</f>
+        <v>0.847113488227536</v>
+      </c>
+      <c r="E517" s="41">
+        <f>IF(C517&gt;0,(1-D517)/C517,1)</f>
+        <v>0.9214437948601683</v>
+      </c>
+      <c r="F517" s="41">
+        <f>IF(C517&gt;0,(C517-1+D517)/C517^2,1/2)</f>
+        <v>0.47345659819610925</v>
+      </c>
+      <c r="G517" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B517/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-2.192520748733403</v>
+      </c>
+      <c r="H517" s="41">
+        <f>(G517*E517+pool_b*D517)/(1-pool_ret*D517)</f>
+        <v>0.7731954419499237</v>
+      </c>
+      <c r="I517" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H517+pool_b)*E517+G517*F517))</f>
+        <v>2.000531675629027</v>
+      </c>
+      <c r="J517" s="41">
+        <f>IF(AND(I517&gt;=CO2_pH_hi_mt,I518&lt;CO2_pH_hi_mt),EXP(LN(A517)+(LN(A518)-LN(A517))*(I517-CO2_pH_hi_mt)/(I517-I518)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="41">
+        <f>A517*grid_ratio</f>
+        <v>207.59020034676132</v>
+      </c>
+      <c r="B518" s="41">
+        <f>MAX(0,A518*60-spg_dur)</f>
+        <v>12454.76202080568</v>
+      </c>
+      <c r="C518" s="41">
+        <f>k_eff_CO2*B518</f>
+        <v>0.18085430875182368</v>
+      </c>
+      <c r="D518" s="41">
+        <f>EXP(-C518)</f>
+        <v>0.8345569374809878</v>
+      </c>
+      <c r="E518" s="41">
+        <f>IF(C518&gt;0,(1-D518)/C518,1)</f>
+        <v>0.9147864027173415</v>
+      </c>
+      <c r="F518" s="41">
+        <f>IF(C518&gt;0,(C518-1+D518)/C518^2,1/2)</f>
+        <v>0.4711726133082772</v>
+      </c>
+      <c r="G518" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B518/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-2.389858841283084</v>
+      </c>
+      <c r="H518" s="41">
+        <f>(G518*E518+pool_b*D518)/(1-pool_ret*D518)</f>
+        <v>-0.08120522555268145</v>
+      </c>
+      <c r="I518" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H518+pool_b)*E518+G518*F518))</f>
+        <v>1.181332101252369</v>
+      </c>
+      <c r="J518" s="41">
+        <f>IF(AND(I518&gt;=CO2_pH_hi_mt,I519&lt;CO2_pH_hi_mt),EXP(LN(A518)+(LN(A519)-LN(A518))*(I518-CO2_pH_hi_mt)/(I518-I519)),0)</f>
+        <v>212.46010616654434</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="41">
+        <f>A518*grid_ratio</f>
+        <v>226.27331837796987</v>
+      </c>
+      <c r="B519" s="41">
+        <f>MAX(0,A519*60-spg_dur)</f>
+        <v>13575.749102678192</v>
+      </c>
+      <c r="C519" s="41">
+        <f>k_eff_CO2*B519</f>
+        <v>0.19713204601192608</v>
+      </c>
+      <c r="D519" s="41">
+        <f>EXP(-C519)</f>
+        <v>0.8210822055233841</v>
+      </c>
+      <c r="E519" s="41">
+        <f>IF(C519&gt;0,(1-D519)/C519,1)</f>
+        <v>0.9076038021022304</v>
+      </c>
+      <c r="F519" s="41">
+        <f>IF(C519&gt;0,(C519-1+D519)/C519^2,1/2)</f>
+        <v>0.4687020693336694</v>
+      </c>
+      <c r="G519" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B519/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-2.6049573621622364</v>
+      </c>
+      <c r="H519" s="41">
+        <f>(G519*E519+pool_b*D519)/(1-pool_ret*D519)</f>
+        <v>-0.9131095801769972</v>
+      </c>
+      <c r="I519" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H519+pool_b)*E519+G519*F519))</f>
+        <v>0.38312677003649</v>
+      </c>
+      <c r="J519" s="41">
+        <f>IF(AND(I519&gt;=CO2_pH_hi_mt,I520&lt;CO2_pH_hi_mt),EXP(LN(A519)+(LN(A520)-LN(A519))*(I519-CO2_pH_hi_mt)/(I519-I520)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="41">
+        <f>A519*grid_ratio</f>
+        <v>246.63791703198717</v>
+      </c>
+      <c r="B520" s="41">
+        <f>MAX(0,A520*60-spg_dur)</f>
+        <v>14797.625021919232</v>
+      </c>
+      <c r="C520" s="41">
+        <f>k_eff_CO2*B520</f>
+        <v>0.21487477962543775</v>
+      </c>
+      <c r="D520" s="41">
+        <f>EXP(-C520)</f>
+        <v>0.806642441922172</v>
+      </c>
+      <c r="E520" s="41">
+        <f>IF(C520&gt;0,(1-D520)/C520,1)</f>
+        <v>0.8998615771235793</v>
+      </c>
+      <c r="F520" s="41">
+        <f>IF(C520&gt;0,(C520-1+D520)/C520^2,1/2)</f>
+        <v>0.466031532648823</v>
+      </c>
+      <c r="G520" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B520/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-2.839414749920513</v>
+      </c>
+      <c r="H520" s="41">
+        <f>(G520*E520+pool_b*D520)/(1-pool_ret*D520)</f>
+        <v>-1.7203282275491723</v>
+      </c>
+      <c r="I520" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H520+pool_b)*E520+G520*F520))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J520" s="41">
+        <f>IF(AND(I520&gt;=CO2_pH_hi_mt,I521&lt;CO2_pH_hi_mt),EXP(LN(A520)+(LN(A521)-LN(A520))*(I520-CO2_pH_hi_mt)/(I520-I521)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="41">
+        <f>A520*grid_ratio</f>
+        <v>268.835329564866</v>
+      </c>
+      <c r="B521" s="41">
+        <f>MAX(0,A521*60-spg_dur)</f>
+        <v>16129.469773891962</v>
+      </c>
+      <c r="C521" s="41">
+        <f>k_eff_CO2*B521</f>
+        <v>0.23421435926416542</v>
+      </c>
+      <c r="D521" s="41">
+        <f>EXP(-C521)</f>
+        <v>0.7911921983392366</v>
+      </c>
+      <c r="E521" s="41">
+        <f>IF(C521&gt;0,(1-D521)/C521,1)</f>
+        <v>0.8915243382889838</v>
+      </c>
+      <c r="F521" s="41">
+        <f>IF(C521&gt;0,(C521-1+D521)/C521^2,1/2)</f>
+        <v>0.4631469310925933</v>
+      </c>
+      <c r="G521" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B521/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-3.094973302577034</v>
+      </c>
+      <c r="H521" s="41">
+        <f>(G521*E521+pool_b*D521)/(1-pool_ret*D521)</f>
+        <v>-2.500964150769591</v>
+      </c>
+      <c r="I521" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H521+pool_b)*E521+G521*F521))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J521" s="41">
+        <f>IF(AND(I521&gt;=CO2_pH_hi_mt,I522&lt;CO2_pH_hi_mt),EXP(LN(A521)+(LN(A522)-LN(A521))*(I521-CO2_pH_hi_mt)/(I521-I522)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="41">
+        <f>A521*grid_ratio</f>
+        <v>293.030509225704</v>
+      </c>
+      <c r="B522" s="41">
+        <f>MAX(0,A522*60-spg_dur)</f>
+        <v>17581.18055354224</v>
+      </c>
+      <c r="C522" s="41">
+        <f>k_eff_CO2*B522</f>
+        <v>0.2552945010703786</v>
+      </c>
+      <c r="D522" s="41">
+        <f>EXP(-C522)</f>
+        <v>0.7746883178242738</v>
+      </c>
+      <c r="E522" s="41">
+        <f>IF(C522&gt;0,(1-D522)/C522,1)</f>
+        <v>0.8825559549111209</v>
+      </c>
+      <c r="F522" s="41">
+        <f>IF(C522&gt;0,(C522-1+D522)/C522^2,1/2)</f>
+        <v>0.46003358707872355</v>
+      </c>
+      <c r="G522" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B522/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-3.3735321249726424</v>
+      </c>
+      <c r="H522" s="41">
+        <f>(G522*E522+pool_b*D522)/(1-pool_ret*D522)</f>
+        <v>-3.2534196091813303</v>
+      </c>
+      <c r="I522" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H522+pool_b)*E522+G522*F522))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J522" s="41">
+        <f>IF(AND(I522&gt;=CO2_pH_hi_mt,I523&lt;CO2_pH_hi_mt),EXP(LN(A522)+(LN(A523)-LN(A522))*(I522-CO2_pH_hi_mt)/(I522-I523)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="41">
+        <f>A522*grid_ratio</f>
+        <v>319.4032550560174</v>
+      </c>
+      <c r="B523" s="41">
+        <f>MAX(0,A523*60-spg_dur)</f>
+        <v>19163.54530336104</v>
+      </c>
+      <c r="C523" s="41">
+        <f>k_eff_CO2*B523</f>
+        <v>0.2782718556391509</v>
+      </c>
+      <c r="D523" s="41">
+        <f>EXP(-C523)</f>
+        <v>0.7570909740845558</v>
+      </c>
+      <c r="E523" s="41">
+        <f>IF(C523&gt;0,(1-D523)/C523,1)</f>
+        <v>0.8729198479577341</v>
+      </c>
+      <c r="F523" s="41">
+        <f>IF(C523&gt;0,(C523-1+D523)/C523^2,1/2)</f>
+        <v>0.4566762662734281</v>
+      </c>
+      <c r="G523" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B523/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-3.677161241383854</v>
+      </c>
+      <c r="H523" s="41">
+        <f>(G523*E523+pool_b*D523)/(1-pool_ret*D523)</f>
+        <v>-3.976396353096525</v>
+      </c>
+      <c r="I523" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H523+pool_b)*E523+G523*F523))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J523" s="41">
+        <f>IF(AND(I523&gt;=CO2_pH_hi_mt,I524&lt;CO2_pH_hi_mt),EXP(LN(A523)+(LN(A524)-LN(A523))*(I523-CO2_pH_hi_mt)/(I523-I524)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="41">
+        <f>A523*grid_ratio</f>
+        <v>348.149548011059</v>
+      </c>
+      <c r="B524" s="41">
+        <f>MAX(0,A524*60-spg_dur)</f>
+        <v>20888.322880663538</v>
+      </c>
+      <c r="C524" s="41">
+        <f>k_eff_CO2*B524</f>
+        <v>0.30331717211911285</v>
+      </c>
+      <c r="D524" s="41">
+        <f>EXP(-C524)</f>
+        <v>0.738364870476837</v>
+      </c>
+      <c r="E524" s="41">
+        <f>IF(C524&gt;0,(1-D524)/C524,1)</f>
+        <v>0.8625793511632066</v>
+      </c>
+      <c r="F524" s="41">
+        <f>IF(C524&gt;0,(C524-1+D524)/C524^2,1/2)</f>
+        <v>0.4530592444757068</v>
+      </c>
+      <c r="G524" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B524/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-4.008116978272077</v>
+      </c>
+      <c r="H524" s="41">
+        <f>(G524*E524+pool_b*D524)/(1-pool_ret*D524)</f>
+        <v>-4.668889748104208</v>
+      </c>
+      <c r="I524" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H524+pool_b)*E524+G524*F524))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J524" s="41">
+        <f>IF(AND(I524&gt;=CO2_pH_hi_mt,I525&lt;CO2_pH_hi_mt),EXP(LN(A524)+(LN(A525)-LN(A524))*(I524-CO2_pH_hi_mt)/(I524-I525)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="41">
+        <f>A524*grid_ratio</f>
+        <v>379.48300733205434</v>
+      </c>
+      <c r="B525" s="41">
+        <f>MAX(0,A525*60-spg_dur)</f>
+        <v>22768.33043992326</v>
+      </c>
+      <c r="C525" s="41">
+        <f>k_eff_CO2*B525</f>
+        <v>0.33061656708227133</v>
+      </c>
+      <c r="D525" s="41">
+        <f>EXP(-C525)</f>
+        <v>0.7184806053463619</v>
+      </c>
+      <c r="E525" s="41">
+        <f>IF(C525&gt;0,(1-D525)/C525,1)</f>
+        <v>0.8514981482569933</v>
+      </c>
+      <c r="F525" s="41">
+        <f>IF(C525&gt;0,(C525-1+D525)/C525^2,1/2)</f>
+        <v>0.4491663955425842</v>
+      </c>
+      <c r="G525" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B525/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-4.368858731480239</v>
+      </c>
+      <c r="H525" s="41">
+        <f>(G525*E525+pool_b*D525)/(1-pool_ret*D525)</f>
+        <v>-5.330177562957667</v>
+      </c>
+      <c r="I525" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H525+pool_b)*E525+G525*F525))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J525" s="41">
+        <f>IF(AND(I525&gt;=CO2_pH_hi_mt,I526&lt;CO2_pH_hi_mt),EXP(LN(A525)+(LN(A526)-LN(A525))*(I525-CO2_pH_hi_mt)/(I525-I526)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="41">
+        <f>A525*grid_ratio</f>
+        <v>413.6364779919392</v>
+      </c>
+      <c r="B526" s="41">
+        <f>MAX(0,A526*60-spg_dur)</f>
+        <v>24817.53867951635</v>
+      </c>
+      <c r="C526" s="41">
+        <f>k_eff_CO2*B526</f>
+        <v>0.360372907592114</v>
+      </c>
+      <c r="D526" s="41">
+        <f>EXP(-C526)</f>
+        <v>0.6974162057756318</v>
+      </c>
+      <c r="E526" s="41">
+        <f>IF(C526&gt;0,(1-D526)/C526,1)</f>
+        <v>0.8396407938824467</v>
+      </c>
+      <c r="F526" s="41">
+        <f>IF(C526&gt;0,(C526-1+D526)/C526^2,1/2)</f>
+        <v>0.44498130336438907</v>
+      </c>
+      <c r="G526" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B526/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-4.762067242477135</v>
+      </c>
+      <c r="H526" s="41">
+        <f>(G526*E526+pool_b*D526)/(1-pool_ret*D526)</f>
+        <v>-5.959804281471193</v>
+      </c>
+      <c r="I526" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H526+pool_b)*E526+G526*F526))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J526" s="41">
+        <f>IF(AND(I526&gt;=CO2_pH_hi_mt,I527&lt;CO2_pH_hi_mt),EXP(LN(A526)+(LN(A527)-LN(A526))*(I526-CO2_pH_hi_mt)/(I526-I527)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="41">
+        <f>A526*grid_ratio</f>
+        <v>450.8637610112138</v>
+      </c>
+      <c r="B527" s="41">
+        <f>MAX(0,A527*60-spg_dur)</f>
+        <v>27051.175660672827</v>
+      </c>
+      <c r="C527" s="41">
+        <f>k_eff_CO2*B527</f>
+        <v>0.3928073187478426</v>
+      </c>
+      <c r="D527" s="41">
+        <f>EXP(-C527)</f>
+        <v>0.6751588255018458</v>
+      </c>
+      <c r="E527" s="41">
+        <f>IF(C527&gt;0,(1-D527)/C527,1)</f>
+        <v>0.8269733250736137</v>
+      </c>
+      <c r="F527" s="41">
+        <f>IF(C527&gt;0,(C527-1+D527)/C527^2,1/2)</f>
+        <v>0.44048740099330613</v>
+      </c>
+      <c r="G527" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B527/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-5.190664519463754</v>
+      </c>
+      <c r="H527" s="41">
+        <f>(G527*E527+pool_b*D527)/(1-pool_ret*D527)</f>
+        <v>-6.557561853164483</v>
+      </c>
+      <c r="I527" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H527+pool_b)*E527+G527*F527))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J527" s="41">
+        <f>IF(AND(I527&gt;=CO2_pH_hi_mt,I528&lt;CO2_pH_hi_mt),EXP(LN(A527)+(LN(A528)-LN(A527))*(I527-CO2_pH_hi_mt)/(I527-I528)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="41">
+        <f>A527*grid_ratio</f>
+        <v>491.4414995022231</v>
+      </c>
+      <c r="B528" s="41">
+        <f>MAX(0,A528*60-spg_dur)</f>
+        <v>29485.839970133384</v>
+      </c>
+      <c r="C528" s="41">
+        <f>k_eff_CO2*B528</f>
+        <v>0.4281608269075868</v>
+      </c>
+      <c r="D528" s="41">
+        <f>EXP(-C528)</f>
+        <v>0.6517065944137552</v>
+      </c>
+      <c r="E528" s="41">
+        <f>IF(C528&gt;0,(1-D528)/C528,1)</f>
+        <v>0.8134639689058233</v>
+      </c>
+      <c r="F528" s="41">
+        <f>IF(C528&gt;0,(C528-1+D528)/C528^2,1/2)</f>
+        <v>0.4356681400338337</v>
+      </c>
+      <c r="G528" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B528/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-5.657835551379167</v>
+      </c>
+      <c r="H528" s="41">
+        <f>(G528*E528+pool_b*D528)/(1-pool_ret*D528)</f>
+        <v>-7.123467804701378</v>
+      </c>
+      <c r="I528" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H528+pool_b)*E528+G528*F528))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J528" s="41">
+        <f>IF(AND(I528&gt;=CO2_pH_hi_mt,I529&lt;CO2_pH_hi_mt),EXP(LN(A528)+(LN(A529)-LN(A528))*(I528-CO2_pH_hi_mt)/(I528-I529)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="41">
+        <f>A528*grid_ratio</f>
+        <v>535.6712344574232</v>
+      </c>
+      <c r="B529" s="41">
+        <f>MAX(0,A529*60-spg_dur)</f>
+        <v>32139.62406744539</v>
+      </c>
+      <c r="C529" s="41">
+        <f>k_eff_CO2*B529</f>
+        <v>0.4666961508017079</v>
+      </c>
+      <c r="D529" s="41">
+        <f>EXP(-C529)</f>
+        <v>0.6270705963663491</v>
+      </c>
+      <c r="E529" s="41">
+        <f>IF(C529&gt;0,(1-D529)/C529,1)</f>
+        <v>0.799083950002628</v>
+      </c>
+      <c r="F529" s="41">
+        <f>IF(C529&gt;0,(C529-1+D529)/C529^2,1/2)</f>
+        <v>0.4305071932824622</v>
+      </c>
+      <c r="G529" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B529/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-6.167051976166967</v>
+      </c>
+      <c r="H529" s="41">
+        <f>(G529*E529+pool_b*D529)/(1-pool_ret*D529)</f>
+        <v>-7.657741601928435</v>
+      </c>
+      <c r="I529" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H529+pool_b)*E529+G529*F529))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J529" s="41">
+        <f>IF(AND(I529&gt;=CO2_pH_hi_mt,I530&lt;CO2_pH_hi_mt),EXP(LN(A529)+(LN(A530)-LN(A529))*(I529-CO2_pH_hi_mt)/(I529-I530)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="41">
+        <f>A529*grid_ratio</f>
+        <v>583.8816455585913</v>
+      </c>
+      <c r="B530" s="41">
+        <f>MAX(0,A530*60-spg_dur)</f>
+        <v>35032.24873351548</v>
+      </c>
+      <c r="C530" s="41">
+        <f>k_eff_CO2*B530</f>
+        <v>0.5086996538462999</v>
+      </c>
+      <c r="D530" s="41">
+        <f>EXP(-C530)</f>
+        <v>0.6012769388376401</v>
+      </c>
+      <c r="E530" s="41">
+        <f>IF(C530&gt;0,(1-D530)/C530,1)</f>
+        <v>0.7838083988215792</v>
+      </c>
+      <c r="F530" s="41">
+        <f>IF(C530&gt;0,(C530-1+D530)/C530^2,1/2)</f>
+        <v>0.42498869331596134</v>
+      </c>
+      <c r="G530" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B530/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-6.72209787918567</v>
+      </c>
+      <c r="H530" s="41">
+        <f>(G530*E530+pool_b*D530)/(1-pool_ret*D530)</f>
+        <v>-8.160780089307275</v>
+      </c>
+      <c r="I530" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H530+pool_b)*E530+G530*F530))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J530" s="41">
+        <f>IF(AND(I530&gt;=CO2_pH_hi_mt,I531&lt;CO2_pH_hi_mt),EXP(LN(A530)+(LN(A531)-LN(A530))*(I530-CO2_pH_hi_mt)/(I530-I531)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="41">
+        <f>A530*grid_ratio</f>
+        <v>636.4309936588646</v>
+      </c>
+      <c r="B531" s="41">
+        <f>MAX(0,A531*60-spg_dur)</f>
+        <v>38185.20961953187</v>
+      </c>
+      <c r="C531" s="41">
+        <f>k_eff_CO2*B531</f>
+        <v>0.5544834721649052</v>
+      </c>
+      <c r="D531" s="41">
+        <f>EXP(-C531)</f>
+        <v>0.574368862093415</v>
+      </c>
+      <c r="E531" s="41">
+        <f>IF(C531&gt;0,(1-D531)/C531,1)</f>
+        <v>0.7676173579074705</v>
+      </c>
+      <c r="F531" s="41">
+        <f>IF(C531&gt;0,(C531-1+D531)/C531^2,1/2)</f>
+        <v>0.4190975092282248</v>
+      </c>
+      <c r="G531" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B531/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-7.327097913476055</v>
+      </c>
+      <c r="H531" s="41">
+        <f>(G531*E531+pool_b*D531)/(1-pool_ret*D531)</f>
+        <v>-8.633132748945192</v>
+      </c>
+      <c r="I531" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H531+pool_b)*E531+G531*F531))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J531" s="41">
+        <f>IF(AND(I531&gt;=CO2_pH_hi_mt,I532&lt;CO2_pH_hi_mt),EXP(LN(A531)+(LN(A532)-LN(A531))*(I531-CO2_pH_hi_mt)/(I531-I532)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="41">
+        <f>A531*grid_ratio</f>
+        <v>693.7097830881625</v>
+      </c>
+      <c r="B532" s="41">
+        <f>MAX(0,A532*60-spg_dur)</f>
+        <v>41621.93698528974</v>
+      </c>
+      <c r="C532" s="41">
+        <f>k_eff_CO2*B532</f>
+        <v>0.604387834132185</v>
+      </c>
+      <c r="D532" s="41">
+        <f>EXP(-C532)</f>
+        <v>0.5464088171057572</v>
+      </c>
+      <c r="E532" s="41">
+        <f>IF(C532&gt;0,(1-D532)/C532,1)</f>
+        <v>0.750496878458077</v>
+      </c>
+      <c r="F532" s="41">
+        <f>IF(C532&gt;0,(C532-1+D532)/C532^2,1/2)</f>
+        <v>0.4128195629552571</v>
+      </c>
+      <c r="G532" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B532/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-7.986547950852575</v>
+      </c>
+      <c r="H532" s="41">
+        <f>(G532*E532+pool_b*D532)/(1-pool_ret*D532)</f>
+        <v>-9.075477424111533</v>
+      </c>
+      <c r="I532" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H532+pool_b)*E532+G532*F532))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J532" s="41">
+        <f>IF(AND(I532&gt;=CO2_pH_hi_mt,I533&lt;CO2_pH_hi_mt),EXP(LN(A532)+(LN(A533)-LN(A532))*(I532-CO2_pH_hi_mt)/(I532-I533)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="41">
+        <f>A532*grid_ratio</f>
+        <v>756.1436635660972</v>
+      </c>
+      <c r="B533" s="41">
+        <f>MAX(0,A533*60-spg_dur)</f>
+        <v>45367.96981396583</v>
+      </c>
+      <c r="C533" s="41">
+        <f>k_eff_CO2*B533</f>
+        <v>0.65878358867652</v>
+      </c>
+      <c r="D533" s="41">
+        <f>EXP(-C533)</f>
+        <v>0.5174804208438425</v>
+      </c>
+      <c r="E533" s="41">
+        <f>IF(C533&gt;0,(1-D533)/C533,1)</f>
+        <v>0.7324401934867981</v>
+      </c>
+      <c r="F533" s="41">
+        <f>IF(C533&gt;0,(C533-1+D533)/C533^2,1/2)</f>
+        <v>0.40614218555553727</v>
+      </c>
+      <c r="G533" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B533/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-8.705348491592982</v>
+      </c>
+      <c r="H533" s="41">
+        <f>(G533*E533+pool_b*D533)/(1-pool_ret*D533)</f>
+        <v>-9.48859705002255</v>
+      </c>
+      <c r="I533" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H533+pool_b)*E533+G533*F533))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J533" s="41">
+        <f>IF(AND(I533&gt;=CO2_pH_hi_mt,I534&lt;CO2_pH_hi_mt),EXP(LN(A533)+(LN(A534)-LN(A533))*(I533-CO2_pH_hi_mt)/(I533-I534)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="41">
+        <f>A533*grid_ratio</f>
+        <v>824.196593287046</v>
+      </c>
+      <c r="B534" s="41">
+        <f>MAX(0,A534*60-spg_dur)</f>
+        <v>49451.145597222756</v>
+      </c>
+      <c r="C534" s="41">
+        <f>k_eff_CO2*B534</f>
+        <v>0.7180749611298451</v>
+      </c>
+      <c r="D534" s="41">
+        <f>EXP(-C534)</f>
+        <v>0.4876901754489236</v>
+      </c>
+      <c r="E534" s="41">
+        <f>IF(C534&gt;0,(1-D534)/C534,1)</f>
+        <v>0.7134489465347595</v>
+      </c>
+      <c r="F534" s="41">
+        <f>IF(C534&gt;0,(C534-1+D534)/C534^2,1/2)</f>
+        <v>0.39905451237900114</v>
+      </c>
+      <c r="G534" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B534/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-9.488841081000027</v>
+      </c>
+      <c r="H534" s="41">
+        <f>(G534*E534+pool_b*D534)/(1-pool_ret*D534)</f>
+        <v>-9.873357834443105</v>
+      </c>
+      <c r="I534" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H534+pool_b)*E534+G534*F534))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J534" s="41">
+        <f>IF(AND(I534&gt;=CO2_pH_hi_mt,I535&lt;CO2_pH_hi_mt),EXP(LN(A534)+(LN(A535)-LN(A534))*(I534-CO2_pH_hi_mt)/(I534-I535)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="41">
+        <f>A534*grid_ratio</f>
+        <v>898.3742866828801</v>
+      </c>
+      <c r="B535" s="41">
+        <f>MAX(0,A535*60-spg_dur)</f>
+        <v>53901.807200972806</v>
+      </c>
+      <c r="C535" s="41">
+        <f>k_eff_CO2*B535</f>
+        <v>0.7827025571039695</v>
+      </c>
+      <c r="D535" s="41">
+        <f>EXP(-C535)</f>
+        <v>0.4571688154321369</v>
+      </c>
+      <c r="E535" s="41">
+        <f>IF(C535&gt;0,(1-D535)/C535,1)</f>
+        <v>0.6935344463117126</v>
+      </c>
+      <c r="F535" s="41">
+        <f>IF(C535&gt;0,(C535-1+D535)/C535^2,1/2)</f>
+        <v>0.3915479142194476</v>
+      </c>
+      <c r="G535" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B535/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-10.342848003453703</v>
+      </c>
+      <c r="H535" s="41">
+        <f>(G535*E535+pool_b*D535)/(1-pool_ret*D535)</f>
+        <v>-10.230689237457902</v>
+      </c>
+      <c r="I535" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H535+pool_b)*E535+G535*F535))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J535" s="41">
+        <f>IF(AND(I535&gt;=CO2_pH_hi_mt,I536&lt;CO2_pH_hi_mt),EXP(LN(A535)+(LN(A536)-LN(A535))*(I535-CO2_pH_hi_mt)/(I535-I536)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="41">
+        <f>A535*grid_ratio</f>
+        <v>979.2279724843394</v>
+      </c>
+      <c r="B536" s="41">
+        <f>MAX(0,A536*60-spg_dur)</f>
+        <v>58753.02834906036</v>
+      </c>
+      <c r="C536" s="41">
+        <f>k_eff_CO2*B536</f>
+        <v>0.8531466367157651</v>
+      </c>
+      <c r="D536" s="41">
+        <f>EXP(-C536)</f>
+        <v>0.4260721261998889</v>
+      </c>
+      <c r="E536" s="41">
+        <f>IF(C536&gt;0,(1-D536)/C536,1)</f>
+        <v>0.672718907982194</v>
+      </c>
+      <c r="F536" s="41">
+        <f>IF(C536&gt;0,(C536-1+D536)/C536^2,1/2)</f>
+        <v>0.3836164592732763</v>
+      </c>
+      <c r="G536" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B536/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-11.273715548928212</v>
+      </c>
+      <c r="H536" s="41">
+        <f>(G536*E536+pool_b*D536)/(1-pool_ret*D536)</f>
+        <v>-10.561566017211053</v>
+      </c>
+      <c r="I536" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H536+pool_b)*E536+G536*F536))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J536" s="41">
+        <f>IF(AND(I536&gt;=CO2_pH_hi_mt,I537&lt;CO2_pH_hi_mt),EXP(LN(A536)+(LN(A537)-LN(A536))*(I536-CO2_pH_hi_mt)/(I536-I537)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="41">
+        <f>A536*grid_ratio</f>
+        <v>1067.35849000793</v>
+      </c>
+      <c r="B537" s="41">
+        <f>MAX(0,A537*60-spg_dur)</f>
+        <v>64040.8594004758</v>
+      </c>
+      <c r="C537" s="41">
+        <f>k_eff_CO2*B537</f>
+        <v>0.9299306834926223</v>
+      </c>
+      <c r="D537" s="41">
+        <f>EXP(-C537)</f>
+        <v>0.39458106040467045</v>
+      </c>
+      <c r="E537" s="41">
+        <f>IF(C537&gt;0,(1-D537)/C537,1)</f>
+        <v>0.6510366313771953</v>
+      </c>
+      <c r="F537" s="41">
+        <f>IF(C537&gt;0,(C537-1+D537)/C537^2,1/2)</f>
+        <v>0.3752573980161321</v>
+      </c>
+      <c r="G537" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B537/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-12.28836117349543</v>
+      </c>
+      <c r="H537" s="41">
+        <f>(G537*E537+pool_b*D537)/(1-pool_ret*D537)</f>
+        <v>-10.86699253853565</v>
+      </c>
+      <c r="I537" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H537+pool_b)*E537+G537*F537))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J537" s="41">
+        <f>IF(AND(I537&gt;=CO2_pH_hi_mt,I538&lt;CO2_pH_hi_mt),EXP(LN(A537)+(LN(A538)-LN(A537))*(I537-CO2_pH_hi_mt)/(I537-I538)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="41">
+        <f>A537*grid_ratio</f>
+        <v>1163.420754108644</v>
+      </c>
+      <c r="B538" s="41">
+        <f>MAX(0,A538*60-spg_dur)</f>
+        <v>69804.59524651864</v>
+      </c>
+      <c r="C538" s="41">
+        <f>k_eff_CO2*B538</f>
+        <v>1.0136252944793969</v>
+      </c>
+      <c r="D538" s="41">
+        <f>EXP(-C538)</f>
+        <v>0.36290096904725416</v>
+      </c>
+      <c r="E538" s="41">
+        <f>IF(C538&gt;0,(1-D538)/C538,1)</f>
+        <v>0.62853505572783</v>
+      </c>
+      <c r="F538" s="41">
+        <f>IF(C538&gt;0,(C538-1+D538)/C538^2,1/2)</f>
+        <v>0.3664716599865005</v>
+      </c>
+      <c r="G538" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B538/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-13.394324904273695</v>
+      </c>
+      <c r="H538" s="41">
+        <f>(G538*E538+pool_b*D538)/(1-pool_ret*D538)</f>
+        <v>-11.1479894846928</v>
+      </c>
+      <c r="I538" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H538+pool_b)*E538+G538*F538))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J538" s="41">
+        <f>IF(AND(I538&gt;=CO2_pH_hi_mt,I539&lt;CO2_pH_hi_mt),EXP(LN(A538)+(LN(A539)-LN(A538))*(I538-CO2_pH_hi_mt)/(I538-I539)),0)</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="41">
+        <f>A538*grid_ratio</f>
+        <v>1268.128621978422</v>
+      </c>
+      <c r="B539" s="41">
+        <f>MAX(0,A539*60-spg_dur)</f>
+        <v>76087.06731870532</v>
+      </c>
+      <c r="C539" s="41">
+        <f>k_eff_CO2*B539</f>
+        <v>1.1048524204549808</v>
+      </c>
+      <c r="D539" s="41">
+        <f>EXP(-C539)</f>
+        <v>0.3312597658003056</v>
+      </c>
+      <c r="E539" s="41">
+        <f>IF(C539&gt;0,(1-D539)/C539,1)</f>
+        <v>0.6052756203623155</v>
+      </c>
+      <c r="F539" s="41">
+        <f>IF(C539&gt;0,(C539-1+D539)/C539^2,1/2)</f>
+        <v>0.35726434800689133</v>
+      </c>
+      <c r="G539" s="41">
+        <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B539/3600)/(V_L_CO2+Vg_CO2)</f>
+        <v>-14.599825370822003</v>
+      </c>
+      <c r="H539" s="41">
+        <f>(G539*E539+pool_b*D539)/(1-pool_ret*D539)</f>
+        <v>-11.405583067879368</v>
+      </c>
+      <c r="I539" s="41">
+        <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H539+pool_b)*E539+G539*F539))</f>
+        <v>0.01155883664100928</v>
+      </c>
+      <c r="J539" s="41">
+        <f>0</f>
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gas model: session record in the review, backlog tidy, start-up TODO row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -13715,8 +13715,10 @@
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A156" s="21" t="s">
-        <v>2717</v>
+      <c r="A156" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model: start-up current ramp</t>
+        </is>
       </c>
       <c r="B156" s="21" t="s">
         <v>931</v>
@@ -13724,8 +13726,10 @@
       <c r="C156" s="21" t="s">
         <v>923</v>
       </c>
-      <c r="F156" s="22" t="s">
-        <v>2718</v>
+      <c r="F156" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag flammability now has a modelled remedy (N₂ sweep, row 100). Lag DO stays unreachable at the estimated surface kLa at any interval or sweep, so the remaining lever is less current until uptake starts; that needs the low-power current curve below 3 % first.</t>
+        </is>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Gas model: owner answers in (resolution input, start-up schedule, vent/N2/media notes); experiments and model-improvement lists
Summary D15 solenoid resolution input (T8). Start-up (lag) schedule beside the
growth one (T4: both), MT D541-D558, Summary rows 31/33. Binding constraint,
DO-limited interval and pool check rows. Improvements table -> Experiments to
improve accuracy (all measurements); TODO block -> Potential model improvements
(spreadsheet changes only); TODO.md rewritten to match. Excel-verified.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -96,12 +96,12 @@
     <definedName name="cath_j_max" localSheetId="2">Electrochemistry!$D$53</definedName>
     <definedName name="cathode_dia" localSheetId="2">Electrochemistry!$D$44</definedName>
     <definedName name="cathode_shape" localSheetId="2">Electrochemistry!$D$43</definedName>
-    <definedName name="cf_Cl_kill" localSheetId="0">Summary!$D$161</definedName>
-    <definedName name="cf_Cl_onset" localSheetId="0">Summary!$D$160</definedName>
-    <definedName name="cf_pH_hi" localSheetId="0">Summary!$D$158</definedName>
-    <definedName name="cf_pH_lo" localSheetId="0">Summary!$D$157</definedName>
-    <definedName name="cf_pH_red_hi" localSheetId="0">Summary!$D$159</definedName>
-    <definedName name="cf_pH_red_lo" localSheetId="0">Summary!$D$156</definedName>
+    <definedName name="cf_Cl_kill" localSheetId="0">Summary!$D$164</definedName>
+    <definedName name="cf_Cl_onset" localSheetId="0">Summary!$D$163</definedName>
+    <definedName name="cf_pH_hi" localSheetId="0">Summary!$D$161</definedName>
+    <definedName name="cf_pH_lo" localSheetId="0">Summary!$D$160</definedName>
+    <definedName name="cf_pH_red_hi" localSheetId="0">Summary!$D$162</definedName>
+    <definedName name="cf_pH_red_lo" localSheetId="0">Summary!$D$159</definedName>
     <definedName name="chk_bubble" localSheetId="0">Summary!$D$41</definedName>
     <definedName name="chk_cal" localSheetId="0">Summary!$D$36</definedName>
     <definedName name="chk_carry_usg" localSheetId="0">Summary!$D$51</definedName>
@@ -1013,6 +1013,29 @@
     <definedName name="pHg_start" localSheetId="5">'Mass Transfer'!$H$440:$H$539</definedName>
     <definedName name="pHg_C" localSheetId="5">'Mass Transfer'!$I$440:$I$539</definedName>
     <definedName name="pHg_x" localSheetId="5">'Mass Transfer'!$J$440:$J$539</definedName>
+    <definedName name="pulse_res_set" localSheetId="0">Summary!$D$15</definedName>
+    <definedName name="res_binding" localSheetId="0">Summary!$D$22</definedName>
+    <definedName name="res_spg_int_DO" localSheetId="0">Summary!$D$29</definedName>
+    <definedName name="res_spg_int_su" localSheetId="0">Summary!$D$31</definedName>
+    <definedName name="res_su_state" localSheetId="0">Summary!$D$33</definedName>
+    <definedName name="chk_pool" localSheetId="0">Summary!$D$55</definedName>
+    <definedName name="y_O2_star_l" localSheetId="5">'Mass Transfer'!$D$542</definedName>
+    <definedName name="duty_DO_l" localSheetId="5">'Mass Transfer'!$D$543</definedName>
+    <definedName name="spg_int_DO_l" localSheetId="5">'Mass Transfer'!$D$544</definedName>
+    <definedName name="spg_int_H2safe_mt" localSheetId="5">'Mass Transfer'!$D$545</definedName>
+    <definedName name="spg_int_su_opt" localSheetId="5">'Mass Transfer'!$D$546</definedName>
+    <definedName name="spg_int_su_run" localSheetId="5">'Mass Transfer'!$D$547</definedName>
+    <definedName name="su_binding" localSheetId="5">'Mass Transfer'!$D$548</definedName>
+    <definedName name="t_gap_su_h" localSheetId="5">'Mass Transfer'!$D$549</definedName>
+    <definedName name="x_su" localSheetId="5">'Mass Transfer'!$D$550</definedName>
+    <definedName name="phi_su" localSheetId="5">'Mass Transfer'!$D$551</definedName>
+    <definedName name="psi_su" localSheetId="5">'Mass Transfer'!$D$552</definedName>
+    <definedName name="dy_O2_su" localSheetId="5">'Mass Transfer'!$D$553</definedName>
+    <definedName name="y_O2_end_su" localSheetId="5">'Mass Transfer'!$D$554</definedName>
+    <definedName name="y_O2_avg_su" localSheetId="5">'Mass Transfer'!$D$555</definedName>
+    <definedName name="DO_avg_su_mgL" localSheetId="5">'Mass Transfer'!$D$556</definedName>
+    <definedName name="DO_peak_su_mgL" localSheetId="5">'Mass Transfer'!$D$557</definedName>
+    <definedName name="y_H2_end_su" localSheetId="5">'Mass Transfer'!$D$558</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -11158,7 +11181,7 @@
   <sheetPr>
     <tabColor theme="1"/>
   </sheetPr>
-  <dimension ref="A1:G159"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -11360,8 +11383,10 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="18" t="s">
-        <v>1791</v>
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vent model</t>
+        </is>
       </c>
       <c r="B11" s="19" t="s">
         <v>1792</v>
@@ -11375,8 +11400,10 @@
       <c r="E11" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="22" t="s">
-        <v>1794</v>
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Outflow only" = check valve or sealed cap that holds a vacuum (no air ever enters). "Open vent" = a plain needle or tube with no forced flow (air drawn back after each pulse; Q_backdraw, Mass Transfer D385, an estimate). "Air exchange" = measured bidirectional exchange at Q_vent (Mass Transfer D142). The MEP0.3 and AEP0.1.1 caps vent through 2 × 1/16" ID tubes to 0.2 µm PTFE filters, AEP0.2 through needles to the same filters, with no check valve: Open vent (owner, T5). Anything else → #N/A throughout.</t>
+        </is>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -11397,7 +11424,7 @@
       </c>
       <c r="F12" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Growth" sizes the sparge interval on the O₂ surplus after knallgas uptake; "Lag" on the whole net electrolytic O₂ plus H₂ (no uptake yet). Anything else → #N/A. Both phases are reported below whichever is chosen. If the chosen phase's DO target is unreachable (rows 65–66), the schedule falls back to the legacy O₂ flush guard (Mass Transfer D89), which is not derived from the headspace balance and does not respond to the vent model.</t>
+          <t xml:space="preserve">"Growth" sizes the headline schedule (rows 18–21) on the O₂ surplus after knallgas uptake; "Lag" on the whole net electrolytic O₂ plus H₂ (no uptake yet). Anything else → #N/A. Both phases are shown either way, and the start-up schedule (rows 31 and 33) is always the lag one. If the chosen phase’s DO target is unreachable (rows 65–66), the schedule falls back to the legacy O₂ flush guard (Mass Transfer D89).</t>
         </is>
       </c>
     </row>
@@ -11432,7 +11459,7 @@
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">N₂ sweep flow</t>
+          <t xml:space="preserve">N₂ dose (mean flow of timed pulses)</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
@@ -11453,7 +11480,37 @@
       </c>
       <c r="F14" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Continuous inert N₂ into the headspace. It dilutes O₂ and H₂ without adding CO₂, so CO₂ is left for carbon and pH; it also strips CO₂ between pulses. Enters the shared vent balance as an inflow with no O₂ or CO₂ (Mass Transfer D424–D425).</t>
+          <t xml:space="preserve">Blank = none, the owner’s preference: fix the medium first (rows 80–81). If N₂ must be used it is pulsed apart from the CO₂ pulses (owner, T7); the balance takes its mean flow as an inert inflow with no O₂ or CO₂ (Mass Transfer D424–D425), exact for the mean-field fractions; the sawtooth of a separate N₂ flush is a model improvement (row 135).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solenoid command resolution</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pulse_res_set</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D15" s="130">
+        <v>0.05</v>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">input</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smallest step the AEP-Plugin solenoid timer is commanded in; the pulse is rounded to it (row 19). Same solenoid as ed04, whose logged pulses (0.2, 0.25, 0.4, 0.6 s) are all 0.05 s multiples (owner, T8).</t>
         </is>
       </c>
     </row>
@@ -11571,6 +11628,31 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Binding constraint on the interval</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_binding</t>
+        </is>
+      </c>
+      <c r="D22" s="65" t="str">
+        <f>'Mass Transfer'!$D$94</f>
+        <v>O2-DILUTION (headspace O2 sets the interval)</v>
+      </c>
+      <c r="E22" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D94","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which upper bound sets row 20: carbon supply, headspace-O₂ dilution or the pH ceiling (rows 28–30); an invalid selector or an unreachable target is named here instead.</t>
+        </is>
+      </c>
+    </row>
     <row r="23" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A23" s="64" t="s">
         <v>1744</v>
@@ -11589,7 +11671,7 @@
       </c>
       <c r="F23" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">pH at the cycle-average dissolved CO₂ of the schedule in use, on the activity scale a probe reads; the trough just after a pulse is lower. Colour: green inside the HOB band (Chemistry pH_band_lo–pH_band_hi), red outside pH_red_lo–pH_red_hi (Chemistry D299–D300), amber between; thresholds in rows 156–159.</t>
+          <t xml:space="preserve">pH at the cycle-average dissolved CO₂ of the schedule in use, on the activity scale a probe reads; the trough just after a pulse is lower. Colour: green inside the HOB band (Chemistry pH_band_lo–pH_band_hi), red outside pH_red_lo–pH_red_hi (Chemistry D299–D300), amber between; thresholds in rows 159–162.</t>
         </is>
       </c>
     </row>
@@ -11641,8 +11723,10 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="77" t="s">
-        <v>1787</v>
+      <c r="A27" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SCHEDULE BOUNDS AND THE START-UP (LAG-PHASE) SCHEDULE</t>
+        </is>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -11667,6 +11751,36 @@
         <v>1754</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO-limited sparge interval</t>
+        </is>
+      </c>
+      <c r="B29" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_int_DO</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D29" s="65">
+        <f>'Mass Transfer'!$D$185</f>
+        <v>7.398866407059</v>
+      </c>
+      <c r="E29" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D185","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longest interval that still dilutes headspace O₂ enough to hold the DO target on the sizing phase (row 12). #N/A = the target is unreachable at this surface kLa.</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
       <c r="A30" s="64" t="inlineStr">
         <is>
@@ -11688,7 +11802,37 @@
       </c>
       <c r="F30" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caps the interval (D21) with the carbon and DO bounds, for the pulse in use. Far above them, or "no pH bound", without a sweep; with an N₂ sweep it stops pH overshooting the band once CO₂ no longer has to dilute O₂. Mass Transfer D435 warns if the capped interval lets the carbon pool run dry.</t>
+          <t xml:space="preserve">Longest interval keeping pH at or under the band ceiling, for the pulse in use. Far above the other bounds, or "no pH bound", unless N₂ dilutes the headspace; then it stops pH overshooting the band once CO₂ no longer has to dilute O₂. Row 55 warns if a long interval lets the carbon pool run dry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-up (lag-phase) interval, same pulse</t>
+        </is>
+      </c>
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_int_su</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D31" s="65">
+        <f>'Mass Transfer'!$D$547</f>
+        <v>1.21</v>
+      </c>
+      <c r="E31" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D547","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner asked for both schedules (T4). Until uptake starts: the shorter of the lag-phase O₂ bound (the legacy guard when the lag DO target is unreachable) and the interval clearing the H₂ flammability screen (Biology D92). Select Lag in row 12 to evaluate every output at it.</t>
         </is>
       </c>
     </row>
@@ -11710,6 +11854,31 @@
       <c r="F32" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Duty of the schedule as typed in (rows 19 and 21) against the optimised duty; 1 = rounding has not moved the CO₂ dose, pH or DO. Should sit within a few per cent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-up schedule: lag-phase DO and H₂</t>
+        </is>
+      </c>
+      <c r="B33" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_su_state</t>
+        </is>
+      </c>
+      <c r="D33" s="65" t="str">
+        <f>IF(ISNUMBER('Mass Transfer'!$D$547),"DO "&amp;TEXT('Mass Transfer'!$D$556,"0.0")&amp;" mg/L mean, "&amp;TEXT('Mass Transfer'!$D$557,"0.0")&amp;" peak; H₂ "&amp;TEXT('Mass Transfer'!$D$558,"0%")&amp;" before each pulse; set by "&amp;'Mass Transfer'!$D$548,"no executable start-up schedule")</f>
+        <v>DO 4.1 mg/L mean, 4.1 peak; H₂ 3% before each pulse; set by the legacy O₂ flush guard (lag DO target unreachable)</v>
+      </c>
+      <c r="E33" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D556","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The lag sawtooth evaluated at the start-up interval (rows 61–62 show the lag phase at the headline schedule instead).</t>
         </is>
       </c>
     </row>
@@ -12090,7 +12259,7 @@
       </c>
       <c r="F52" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">The vent model couples the two: when O₂ dilution binds, CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH (the text says which constraint binds). Tests both band edges (rows 157–158). Red means the two targets conflict under the vent model in use — decouple them (inert sweep) or measure the vent before trusting either. Amber "watch" = an override in G18/G20 is in use: the DO and pH shown are those of the typed schedule, and no claim is made that it holds the DO target. #N/A = a selector in D11/D12 is not a listed value.</t>
+          <t xml:space="preserve">The vent model couples the two: when O₂ dilution binds, CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH (the text says which constraint binds). Tests both band edges (rows 160–161). Red means the two targets conflict under the vent model in use — decouple them (inert sweep) or measure the vent before trusting either. Amber "watch" = an override in G18/G20 is in use: the DO and pH shown are those of the typed schedule, and no claim is made that it holds the DO target. #N/A = a selector in D11/D12 is not a listed value.</t>
         </is>
       </c>
     </row>
@@ -12131,9 +12300,36 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carbon pool stays above air equilibrium through the cycle?</t>
+        </is>
+      </c>
+      <c r="B55" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_pool</t>
+        </is>
+      </c>
+      <c r="D55" s="65" t="str">
+        <f>'Mass Transfer'!$D$435</f>
+        <v>OK</v>
+      </c>
+      <c r="E55" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D435","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
+      <c r="F55" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse-start dissolved CO₂ against air equilibrium at the schedule in use; WATCH = fixation empties the pool within the cycle (only reachable with a long, N₂-relaxed interval).</t>
+        </is>
+      </c>
+    </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A57" s="77" t="s">
-        <v>1790</v>
+      <c r="A57" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DISSOLVED O₂ AND HEADSPACE BY PHASE (both shown; row 12 picks which sizes the headline schedule)</t>
+        </is>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -12497,7 +12693,7 @@
     <row r="79">
       <c r="A79" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">N₂ HEADSPACE SWEEP — owner decision T7 (blank = none); timed N₂ pulses of the same mean flow give the same mean-field balance</t>
+          <t xml:space="preserve">MEDIA DESIGN — fix the medium first (owner, T7); N₂ only if it must, pulsed apart from CO₂</t>
         </is>
       </c>
     </row>
@@ -12546,7 +12742,7 @@
     <row r="82">
       <c r="A82" s="64" t="inlineStr">
         <is>
-          <t xml:space="preserve">N₂ sweep that holds the DO target at the carbon-limited interval</t>
+          <t xml:space="preserve">N₂ (mean of timed pulses) that holds the DO target at the carbon-limited interval</t>
         </is>
       </c>
       <c r="C82" s="21" t="inlineStr">
@@ -12564,14 +12760,14 @@
       </c>
       <c r="F82" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sizing phase (D12): the sweep that removes the DO bound on the CO₂ schedule. With it entered, the pH ceiling (row 30) usually sets the interval, so CO₂ still supplies more than carbon needs. #N/A = the DO target is unreachable at this surface kLa, which no sweep fixes.</t>
+          <t xml:space="preserve">Sizing phase (row 12): the N₂ that removes the DO bound on the CO₂ schedule. With it in row 14 the pH ceiling (row 30) then usually sets the interval. #N/A = the DO target is unreachable at this surface kLa, which no N₂ fixes.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="64" t="inlineStr">
         <is>
-          <t xml:space="preserve">N₂ sweep that keeps lag-phase H₂ below the LFL</t>
+          <t xml:space="preserve">N₂ (mean of timed pulses) that keeps lag-phase H₂ below the LFL</t>
         </is>
       </c>
       <c r="C83" s="21" t="inlineStr">
@@ -12589,7 +12785,7 @@
       </c>
       <c r="F83" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mean-field, with no CO₂ at all; the pre-pulse sawtooth peaks higher, so treat it as a lower bound and check rows 40–42 with the sweep entered. A screen, not a mixture safety certification.</t>
+          <t xml:space="preserve">Mean-field, with no CO₂ at all; the pre-pulse sawtooth peaks higher, so treat it as a lower bound and re-read row 40 with it entered. A screen, not a mixture safety certification.</t>
         </is>
       </c>
     </row>
@@ -12952,8 +13148,10 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A105" s="32" t="s">
-        <v>101</v>
+      <c r="A105" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXPERIMENTS TO IMPROVE ACCURACY (bench measurements; each replaces an estimate or a data gap)</t>
+        </is>
       </c>
       <c r="B105" s="32" t="s">
         <v>102</v>
@@ -13080,8 +13278,10 @@
         <v>vial-geometry.md →</v>
       </c>
       <c r="E111" s="77"/>
-      <c r="F111" s="22" t="s">
-        <v>939</v>
+      <c r="F111" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calipers on the vial body; drives the headspace and displacement budget alongside the total volume (row 107).</t>
+        </is>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.2">
@@ -13119,8 +13319,10 @@
         <v>dissolved-oxygen.md →</v>
       </c>
       <c r="E113" s="77"/>
-      <c r="F113" s="22" t="s">
-        <v>946</v>
+      <c r="F113" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lower DO guardrail for the organism; a data gap for every organism today (row 38).</t>
+        </is>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
@@ -13138,8 +13340,10 @@
         <v>flow-calibration.md →</v>
       </c>
       <c r="E114" s="77"/>
-      <c r="F114" s="22" t="s">
-        <v>950</v>
+      <c r="F114" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each reactor needs its own CO₂ flow calibration; only ed04 has one (row 128 for the reactor actually in use).</t>
+        </is>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.2">
@@ -13157,8 +13361,10 @@
         <v>sinter-porosity.md →</v>
       </c>
       <c r="E115" s="77"/>
-      <c r="F115" s="22" t="s">
-        <v>954</v>
+      <c r="F115" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sets bubble size, and only matters when the sparger is a sintered frit; grade 0 (Gerrit’s disc) is assumed today.</t>
+        </is>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.2">
@@ -13235,8 +13441,9 @@
         <v>gerrit-current.md →</v>
       </c>
       <c r="E119" s="21"/>
-      <c r="F119" t="s">
-        <v>1770</v>
+      <c r="F119" t="str">
+        <f>"The cell-voltage budget is a testable prediction: about "&amp;TEXT(Electrochemistry!$D$119,"0.00")&amp;" V of the "&amp;TEXT(Electrochemistry!$D$120,"0")&amp;" V rail at the current settings (row 96). A multimeter reading across the electrodes tests the cell-constant choice and, with a high-power point, bounds the j₀ errors."</f>
+        <v>The cell-voltage budget is a testable prediction: about 2.65 V of the 5 V rail at the current settings (row 96). A multimeter reading across the electrodes tests the cell-constant choice and, with a high-power point, bounds the j₀ errors.</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.2">
@@ -13260,8 +13467,10 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A121" s="21" t="s">
-        <v>2699</v>
+      <c r="A121" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Characterise the headspace vent</t>
+        </is>
       </c>
       <c r="B121" s="21" t="s">
         <v>922</v>
@@ -13275,13 +13484,15 @@
       </c>
       <c r="F121" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Decides the vent model (D11), the single biggest input: across plausible vents the interval runs from about 0.9 to 12.7 min. Fix the cap leak noted on CO2 flows L8 first.</t>
+          <t xml:space="preserve">The vent is confirmed open (row 11; owner, T5), so the measurement is now its back-draw flow (Q_backdraw, Mass Transfer D385), the single biggest input after the vent type: the interval moves several-fold across plausible ingress. Pressure-decay test or a headspace O₂ tracer.</t>
         </is>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A122" s="21" t="s">
-        <v>2701</v>
+      <c r="A122" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abiotic DO trace under the schedule</t>
+        </is>
       </c>
       <c r="B122" s="21" t="s">
         <v>922</v>
@@ -13300,8 +13511,10 @@
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A123" s="21" t="s">
-        <v>2703</v>
+      <c r="A123" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace H₂/O₂ during lag (safety)</t>
+        </is>
       </c>
       <c r="B123" s="21" t="s">
         <v>922</v>
@@ -13320,8 +13533,10 @@
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A124" s="21" t="s">
-        <v>2705</v>
+      <c r="A124" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Off-gas H₂ at steady growth</t>
+        </is>
       </c>
       <c r="B124" s="21" t="s">
         <v>922</v>
@@ -13333,13 +13548,17 @@
         <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/knallgas-stoichiometry.md","knallgas-stoichiometry.md →")</f>
         <v>knallgas-stoichiometry.md →</v>
       </c>
-      <c r="F124" s="22" t="s">
-        <v>2706</v>
+      <c r="F124" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ fraction in the vent gas × vent flow, against the H₂ the current makes, gives the H₂ uptake fraction behind the growth O₂ surplus (up to ±200 % on the schedule). Row 109 measures the same ratio in sealed bottles.</t>
+        </is>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A125" s="21" t="s">
-        <v>2707</v>
+      <c r="A125" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Free and combined chlorine (DPD)</t>
+        </is>
       </c>
       <c r="B125" s="21" t="s">
         <v>931</v>
@@ -13358,8 +13577,10 @@
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A126" s="21" t="s">
-        <v>2709</v>
+      <c r="A126" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sparger-attached flow check</t>
+        </is>
       </c>
       <c r="B126" s="21" t="s">
         <v>941</v>
@@ -13378,7 +13599,7 @@
     <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Measure: no-carryover maximum flow</t>
+          <t xml:space="preserve">No-carryover maximum flow</t>
         </is>
       </c>
       <c r="B127" s="21" t="inlineStr">
@@ -13404,7 +13625,7 @@
     <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Measure: CO₂ flow of the reactor in use</t>
+          <t xml:space="preserve">CO₂ flow of the reactor in use</t>
         </is>
       </c>
       <c r="B128" s="21" t="inlineStr">
@@ -13425,159 +13646,260 @@
         </is>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A130" s="77" t="s">
-        <v>2697</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A131" s="32" t="s">
-        <v>2698</v>
-      </c>
-      <c r="B131" s="32" t="s">
+    <row r="129">
+      <c r="A129" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AMYBO03 conductivity at the operating temperature</t>
+        </is>
+      </c>
+      <c r="B129" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MED</t>
+        </is>
+      </c>
+      <c r="C129" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">low</t>
+        </is>
+      </c>
+      <c r="D129" s="33" t="str">
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/README.md","README.md →")</f>
+        <v>README.md →</v>
+      </c>
+      <c r="F129" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The ohmic term uses a Kohlrausch sum × a finite-strength factor (0.78) anchored near I ≈ 0.1 M; AMYBO03 is about 0.2 M. A conductivity-meter reading at 30 °C replaces both (Chemistry D178–D180).</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low-power current curve below 3 %</t>
+        </is>
+      </c>
+      <c r="B130" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MED</t>
+        </is>
+      </c>
+      <c r="C130" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">low</t>
+        </is>
+      </c>
+      <c r="D130" s="33" t="str">
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/gerrit-current.md","gerrit-current.md →")</f>
+        <v>gerrit-current.md →</v>
+      </c>
+      <c r="F130" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gerrit’s Law is fitted and validated for 3–10 %; below that the model refuses to run. Needed before a start-up current ramp can be modelled (row 138).</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrochemist review of the calculated electrochemistry</t>
+        </is>
+      </c>
+      <c r="B131" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HIGH</t>
+        </is>
+      </c>
+      <c r="C131" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">low</t>
+        </is>
+      </c>
+      <c r="D131" s="33" t="str">
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/README.md","README.md →")</f>
+        <v>README.md →</v>
+      </c>
+      <c r="F131" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Weakest inputs: the anodic exchange-current density (four decades in the literature) and the electrode mass-transfer coefficient. Rows 94–103 are the numbers to hand over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A133" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POTENTIAL MODEL IMPROVEMENTS (changes to the spreadsheet itself; each waits on the decision or data in column D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A134" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Improvement</t>
+        </is>
+      </c>
+      <c r="B134" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="C131" s="32" t="s">
+      <c r="C134" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="D131" s="32" t="s">
-        <v>104</v>
-      </c>
-      <c r="F131" s="32" t="s">
+      <c r="D134" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Waits on</t>
+        </is>
+      </c>
+      <c r="F134" s="32" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A132" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Decide: N₂ sweep hardware and flow (T7)</t>
-        </is>
-      </c>
-      <c r="B132" s="21" t="s">
-        <v>922</v>
-      </c>
-      <c r="C132" s="21" t="s">
-        <v>932</v>
-      </c>
-      <c r="F132" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The model now takes an N₂ sweep (D14) as an inert inflow in the shared headspace balance; rows 82–83 give the flow for the DO target at the carbon-limited interval and for lag H₂ below the LFL. Needs the owner’s choice of hardware (own line or shared), flow control and objective.</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A133" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Model: nitrate or urea instead of NH₄⁺</t>
-        </is>
-      </c>
-      <c r="B133" s="21" t="inlineStr">
+    <row r="135" x14ac:dyDescent="0.2">
+      <c r="A135" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Separate N₂ flush in the sawtooth</t>
+        </is>
+      </c>
+      <c r="B135" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOW</t>
+        </is>
+      </c>
+      <c r="C135" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">med</t>
+        </is>
+      </c>
+      <c r="D135" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner: only if N₂ is used at all (T7 prefers fixing the medium)</t>
+        </is>
+      </c>
+      <c r="F135" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Row 14 enters N₂ by its mean flow, exact for the mean-field fractions. Pulsing N₂ midway between CO₂ pulses adds a second flush per cycle, which would lower the pre-pulse O₂ and H₂ peaks a little further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" x14ac:dyDescent="0.2">
+      <c r="A136" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitrate or urea instead of NH₄⁺</t>
+        </is>
+      </c>
+      <c r="B136" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">MED</t>
         </is>
       </c>
-      <c r="C133" s="21" t="inlineStr">
+      <c r="C136" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">med</t>
         </is>
       </c>
-      <c r="F133" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ammonium uptake releases acid as the culture grows; the model holds NH₄⁺ at its recipe value. Needs the owner’s choice of nitrogen source and an uptake rate before it can enter the charge balance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A134" s="21" t="s">
-        <v>2715</v>
-      </c>
-      <c r="B134" s="21" t="s">
-        <v>931</v>
-      </c>
-      <c r="C134" s="21" t="s">
-        <v>926</v>
-      </c>
-      <c r="F134" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pulse length (D18) is a rule of thumb: about one headspace volume per pulse. A twin trial (UdG, 25 °C) at the 0.25 s default floor gave 0.25 s every 4.4 min: same pH and growth DO on about 7 % less CO₂, but higher lag-phase DO. Wait for the measured floor (flow-calibration step 9).</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A135" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Model: start-up current ramp</t>
-        </is>
-      </c>
-      <c r="B135" s="21" t="s">
-        <v>931</v>
-      </c>
-      <c r="C135" s="21" t="s">
-        <v>923</v>
-      </c>
-      <c r="F135" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lag flammability now has a modelled remedy (N₂ sweep, row 83). Lag DO stays unreachable at the estimated surface kLa at any interval or sweep, so the remaining lever is less current until uptake starts; that needs the low-power current curve below 3 % first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A136" s="21" t="s">
-        <v>2723</v>
-      </c>
-      <c r="B136" s="21" t="s">
-        <v>941</v>
-      </c>
-      <c r="C136" s="21" t="s">
-        <v>926</v>
-      </c>
-      <c r="F136" s="22" t="s">
-        <v>2724</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A141" s="17" t="s">
+      <c r="D136" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner: nitrogen source; a measured uptake rate</t>
+        </is>
+      </c>
+      <c r="F136" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ammonium uptake releases acid as the culture grows, which the model does not see: it holds NH₄⁺ at its recipe value. Part of fixing the medium (T7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" x14ac:dyDescent="0.2">
+      <c r="A137" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse length from the shortest reliable pulse</t>
+        </is>
+      </c>
+      <c r="B137" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MED</t>
+        </is>
+      </c>
+      <c r="C137" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">low</t>
+        </is>
+      </c>
+      <c r="D137" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measured solenoid floor (flow-calibration step 9)</t>
+        </is>
+      </c>
+      <c r="F137" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pulse length (row 18) is a rule of thumb: about one headspace volume per pulse. A twin trial at a 0.25 s floor held pH and growth DO on about 7 % less CO₂ but raised lag-phase DO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" x14ac:dyDescent="0.2">
+      <c r="A138" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-up current ramp</t>
+        </is>
+      </c>
+      <c r="B138" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MED</t>
+        </is>
+      </c>
+      <c r="C138" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">med</t>
+        </is>
+      </c>
+      <c r="D138" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Measured low-power current curve below 3 %</t>
+        </is>
+      </c>
+      <c r="F138" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag DO stays unreachable at the estimated surface kLa at any interval (row 66), so the remaining lever is less current until uptake starts; the current fit is not valid below 3 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" x14ac:dyDescent="0.2">
+      <c r="A139" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carbon bound on the pool trough</t>
+        </is>
+      </c>
+      <c r="B139" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOW</t>
+        </is>
+      </c>
+      <c r="C139" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">low</t>
+        </is>
+      </c>
+      <c r="D139" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Owner: trough margin over RuBisCO Km</t>
+        </is>
+      </c>
+      <c r="F139" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The carbon interval (row 28) is sized on mean supply; row 55 warns when a long interval lets the pool run dry within the cycle. A bound on the trough (Biology D98) would close it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A144" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="B141" s="17"/>
-      <c r="C141" s="17"/>
-      <c r="D141" s="17"/>
-      <c r="E141" s="17"/>
-      <c r="F141" s="17"/>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A142" s="102" t="s">
+      <c r="B144" s="17"/>
+      <c r="C144" s="17"/>
+      <c r="D144" s="17"/>
+      <c r="E144" s="17"/>
+      <c r="F144" s="17"/>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A145" s="102" t="s">
         <v>89</v>
-      </c>
-      <c r="B142" s="21"/>
-      <c r="C142" s="21"/>
-      <c r="D142" s="25"/>
-      <c r="E142" s="21"/>
-      <c r="F142" s="21"/>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A143" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="B143" s="21"/>
-      <c r="C143" s="21"/>
-      <c r="D143" s="25"/>
-      <c r="E143" s="21"/>
-      <c r="F143" s="21"/>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A144" s="73" t="s">
-        <v>91</v>
-      </c>
-      <c r="B144" s="21"/>
-      <c r="C144" s="21"/>
-      <c r="D144" s="25"/>
-      <c r="E144" s="21"/>
-      <c r="F144" s="21"/>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A145" s="27" t="s">
-        <v>92</v>
       </c>
       <c r="B145" s="21"/>
       <c r="C145" s="21"/>
@@ -13586,68 +13908,78 @@
       <c r="F145" s="21"/>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A146" s="28" t="s">
-        <v>93</v>
+      <c r="A146" s="26" t="s">
+        <v>90</v>
       </c>
       <c r="B146" s="21"/>
       <c r="C146" s="21"/>
       <c r="D146" s="25"/>
-      <c r="E146" s="67"/>
+      <c r="E146" s="21"/>
       <c r="F146" s="21"/>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A147" s="29" t="s">
-        <v>94</v>
+      <c r="A147" s="73" t="s">
+        <v>91</v>
       </c>
       <c r="B147" s="21"/>
       <c r="C147" s="21"/>
       <c r="D147" s="25"/>
-      <c r="E147" s="67"/>
+      <c r="E147" s="21"/>
       <c r="F147" s="21"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A148" s="63" t="s">
-        <v>95</v>
+      <c r="A148" s="27" t="s">
+        <v>92</v>
       </c>
       <c r="B148" s="21"/>
       <c r="C148" s="21"/>
       <c r="D148" s="25"/>
-      <c r="E148" s="67"/>
+      <c r="E148" s="21"/>
       <c r="F148" s="21"/>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A149" s="30" t="s">
-        <v>96</v>
+      <c r="A149" s="28" t="s">
+        <v>93</v>
       </c>
       <c r="B149" s="21"/>
       <c r="C149" s="21"/>
-      <c r="D149" s="21"/>
-      <c r="E149" s="21"/>
+      <c r="D149" s="25"/>
+      <c r="E149" s="67"/>
       <c r="F149" s="21"/>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A150" s="31" t="s">
-        <v>97</v>
+      <c r="A150" s="29" t="s">
+        <v>94</v>
       </c>
       <c r="B150" s="21"/>
       <c r="C150" s="21"/>
-      <c r="D150" s="21"/>
-      <c r="E150" s="21"/>
+      <c r="D150" s="25"/>
+      <c r="E150" s="67"/>
       <c r="F150" s="21"/>
     </row>
-    <row r="151" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="60" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="61" t="s">
-        <v>99</v>
-      </c>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A151" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="B151" s="21"/>
+      <c r="C151" s="21"/>
+      <c r="D151" s="25"/>
+      <c r="E151" s="67"/>
+      <c r="F151" s="21"/>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A152" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="B152" s="21"/>
+      <c r="C152" s="21"/>
+      <c r="D152" s="21"/>
+      <c r="E152" s="21"/>
+      <c r="F152" s="21"/>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A153" s="103" t="s">
-        <v>100</v>
+      <c r="A153" s="31" t="s">
+        <v>97</v>
       </c>
       <c r="B153" s="21"/>
       <c r="C153" s="21"/>
@@ -13655,147 +13987,167 @@
       <c r="E153" s="21"/>
       <c r="F153" s="21"/>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A155" s="77" t="inlineStr">
+    <row r="154" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A154" s="60" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" s="21" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A155" s="61" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A156" s="103" t="s">
+        <v>100</v>
+      </c>
+      <c r="B156" s="21"/>
+      <c r="C156" s="21"/>
+      <c r="D156" s="21"/>
+      <c r="E156" s="21"/>
+      <c r="F156" s="21"/>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A158" s="77" t="inlineStr">
         <is>
           <t xml:space="preserve">COLOUR THRESHOLDS (the conditional formatting on D23 and D25 reads these cells)</t>
         </is>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A156" s="64" t="s">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A159" s="64" t="s">
         <v>1840</v>
       </c>
-      <c r="B156" s="19" t="s">
+      <c r="B159" s="19" t="s">
         <v>1841</v>
       </c>
-      <c r="C156" s="21" t="s">
+      <c r="C159" s="21" t="s">
         <v>1842</v>
       </c>
-      <c r="D156" s="65">
+      <c r="D159" s="65">
         <f>Chemistry!$D$299</f>
         <v>6.0</v>
       </c>
-      <c r="E156" s="24" t="str">
+      <c r="E159" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D299","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F156" s="22" t="s">
+      <c r="F159" s="22" t="s">
         <v>1843</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A157" s="64" t="s">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A160" s="64" t="s">
         <v>1844</v>
       </c>
-      <c r="B157" s="19" t="s">
+      <c r="B160" s="19" t="s">
         <v>1845</v>
       </c>
-      <c r="C157" s="21" t="s">
+      <c r="C160" s="21" t="s">
         <v>1842</v>
       </c>
-      <c r="D157" s="65">
+      <c r="D160" s="65">
         <f>Chemistry!$D$236</f>
         <v>6.5</v>
       </c>
-      <c r="E157" s="24" t="str">
+      <c r="E160" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D236","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F157" s="22" t="s">
+      <c r="F160" s="22" t="s">
         <v>1843</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A158" s="64" t="s">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A161" s="64" t="s">
         <v>1846</v>
       </c>
-      <c r="B158" s="19" t="s">
+      <c r="B161" s="19" t="s">
         <v>1847</v>
       </c>
-      <c r="C158" s="21" t="s">
+      <c r="C161" s="21" t="s">
         <v>1842</v>
       </c>
-      <c r="D158" s="65">
+      <c r="D161" s="65">
         <f>Chemistry!$D$237</f>
         <v>7.5</v>
       </c>
-      <c r="E158" s="24" t="str">
+      <c r="E161" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D237","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F158" s="22" t="s">
+      <c r="F161" s="22" t="s">
         <v>1843</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A159" s="64" t="s">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A162" s="64" t="s">
         <v>1848</v>
       </c>
-      <c r="B159" s="19" t="s">
+      <c r="B162" s="19" t="s">
         <v>1849</v>
       </c>
-      <c r="C159" s="21" t="s">
+      <c r="C162" s="21" t="s">
         <v>1842</v>
       </c>
-      <c r="D159" s="65">
+      <c r="D162" s="65">
         <f>Chemistry!$D$300</f>
         <v>8.0</v>
       </c>
-      <c r="E159" s="24" t="str">
+      <c r="E162" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D300","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F159" s="22" t="s">
+      <c r="F162" s="22" t="s">
         <v>1843</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A160" s="64" t="s">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A163" s="64" t="s">
         <v>1850</v>
       </c>
-      <c r="B160" s="19" t="s">
+      <c r="B163" s="19" t="s">
         <v>1851</v>
       </c>
-      <c r="C160" s="21" t="s">
+      <c r="C163" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="D160" s="65">
+      <c r="D163" s="65">
         <f>Chemistry!$D$146</f>
         <v>0.1</v>
       </c>
-      <c r="E160" s="24" t="str">
+      <c r="E163" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D146","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F160" s="22" t="s">
+      <c r="F163" s="22" t="s">
         <v>1843</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A161" s="64" t="s">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A164" s="64" t="s">
         <v>1852</v>
       </c>
-      <c r="B161" s="19" t="s">
+      <c r="B164" s="19" t="s">
         <v>1853</v>
       </c>
-      <c r="C161" s="21" t="s">
+      <c r="C164" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="D161" s="65">
+      <c r="D164" s="65">
         <f>Chemistry!$D$147</f>
         <v>2.0</v>
       </c>
-      <c r="E161" s="24" t="str">
+      <c r="E164" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D147","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F161" s="22" t="s">
+      <c r="F164" s="22" t="s">
         <v>1843</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B105:B128 B132:B136">
+  <conditionalFormatting sqref="B105:B131 B135:B139">
     <cfRule type="expression" dxfId="45" priority="16" stopIfTrue="1">
       <formula>EXACT(B105,"HIGH")</formula>
     </cfRule>
@@ -13806,7 +14158,7 @@
       <formula>EXACT(B105,"LOW")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C105:C128 C132:C136">
+  <conditionalFormatting sqref="C105:C131 C135:C139">
     <cfRule type="expression" dxfId="42" priority="19" stopIfTrue="1">
       <formula>EXACT(C105,"low")</formula>
     </cfRule>
@@ -13832,7 +14184,7 @@
       <formula>AND(ISNUMBER($G$20),$G$20&gt;0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D23 D25 D35:D50 D52:D54 D63:D66 D97:D99">
+  <conditionalFormatting sqref="D23 D25 D35:D50 D52:D55 D63:D66 D97:D99">
     <cfRule type="expression" dxfId="36" priority="12" stopIfTrue="1">
       <formula>OR(ISNUMBER(FIND("INCONSISTENT",D23)),ISNUMBER(FIND("OVER",D23)),ISNUMBER(FIND("BELOW",D23)),ISNUMBER(FIND("EXCEED",D23)),ISNUMBER(FIND("NO CALIB",D23)),ISNUMBER(SEARCH("calibrate this",D23)),ISNUMBER(FIND("RISK",D23)),ISNUMBER(FIND("EXPLOSIVE",D23)),ISNUMBER(FIND("FLAMMABLE",D23)),ISNUMBER(FIND("OOR",D23)),ISNUMBER(SEARCH("insufficient",D23)),ISNUMBER(FIND("TIP SPEED",D23)),ISNUMBER(FIND("SHORTFALL",D23)),ISNUMBER(SEARCH("unreachable",D23)),ISNUMBER(FIND("SAGS",D23)),EXACT(LEFT(D23,4),"NO –"),EXACT(D23,"OUT"),EXACT(D23,"LOW"),ISNUMBER(FIND("GAP",D23)))</formula>
     </cfRule>
@@ -13887,7 +14239,7 @@
       <formula>ISNUMBER(SEARCH("OK",D92))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="13">
+  <dataValidations count="14">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not a listed reactor" error="Pick a reactor from the list (Geometry A59:A80)." sqref="D2" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>ReactorList</formula1>
     </dataValidation>
@@ -13932,6 +14284,10 @@
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="N₂ sweep in mL/min (0–20), or leave blank for none." sqref="D14">
       <formula1>0</formula1>
       <formula2>20</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Command resolution in seconds (0.001–1)." sqref="D15">
+      <formula1>0.001</formula1>
+      <formula2>1</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24768,7 +25124,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:J539"/>
+  <dimension ref="A1:J558"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -28430,8 +28786,10 @@
       </c>
     </row>
     <row r="241" spans="1:5" ht="24" x14ac:dyDescent="0.2">
-      <c r="A241" t="s">
-        <v>2313</v>
+      <c r="A241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Solenoid pulse command resolution</t>
+        </is>
       </c>
       <c r="B241" s="19" t="s">
         <v>2314</v>
@@ -28439,11 +28797,14 @@
       <c r="C241" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="D241" s="116">
+      <c r="D241" s="111">
+        <f>Summary!$D$15</f>
         <v>0.05</v>
       </c>
-      <c r="E241" s="52" t="s">
-        <v>2315</v>
+      <c r="E241" s="140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D15 (pulse_res_set): an input on the Summary (owner, T8); same solenoid as ed04.</t>
+        </is>
       </c>
     </row>
     <row r="242" spans="1:5" x14ac:dyDescent="0.2">
@@ -35091,6 +35452,455 @@
       <c r="J539" s="41">
         <f>0</f>
         <v>0.0</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">START-UP (LAG-PHASE) SCHEDULE — shown beside the growth one (owner, T4: both)</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ fraction allowed — lag</t>
+        </is>
+      </c>
+      <c r="B542" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_star_l</t>
+        </is>
+      </c>
+      <c r="C542" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D542" s="41" t="e">
+        <f>IF(DO_target-DO_surf_excess_lag&gt;0,(DO_target-DO_surf_excess_lag)/(H_O2_T*P_dry),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E542" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D183 on the lag source (D181). #N/A = the surface cannot carry the lag O₂ flux at the target DO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Duty needed to hold it — lag</t>
+        </is>
+      </c>
+      <c r="B543" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">duty_DO_l</t>
+        </is>
+      </c>
+      <c r="C543" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D543" s="41" t="e">
+        <f>IF(ISNUMBER(y_O2_star_l),MAX(0,((O2_src_l+y_O2_air*F_vent_ex)*saw_factor/y_O2_star_l-F_dil-O2_src_l-H2_src_l+CO2_fix_l)/CO2_rate_full),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E543" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D184 on the lag sources (D310, D314, D316).</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO-limited interval — lag</t>
+        </is>
+      </c>
+      <c r="B544" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_DO_l</t>
+        </is>
+      </c>
+      <c r="C544" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D544" s="41" t="str">
+        <f>IF(ISNUMBER(duty_DO_l),IF(duty_DO_l&gt;0,spg_dur_eq_opt/(60*duty_DO_l),spg_int_carbon),"lag DO target unreachable at this surface kLa")</f>
+        <v>lag DO target unreachable at this surface kLa</v>
+      </c>
+      <c r="E544" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D185 on the lag source; text when the lag target is unreachable (then the legacy guard D89 applies).</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Interval clearing the lag H₂ flammability screen</t>
+        </is>
+      </c>
+      <c r="B545" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_H2safe_mt</t>
+        </is>
+      </c>
+      <c r="C545" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D545" s="41">
+        <f>Biology!$D$92</f>
+        <v>2.328965780397</v>
+      </c>
+      <c r="E545" s="140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D92 (on the pulse in use; "any interval" when nothing is needed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-up interval (optimal-pulse basis)</t>
+        </is>
+      </c>
+      <c r="B546" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_su_opt</t>
+        </is>
+      </c>
+      <c r="C546" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D546" s="41">
+        <f>MIN(IF(ISNUMBER(spg_int_DO_l),spg_int_DO_l,spg_int_max),IF(ISNUMBER(spg_int_H2safe_mt),spg_int_H2safe_mt*spg_dur_eq_opt/spg_dur_eq,IF(ISNUMBER(spg_int_DO_l),spg_int_DO_l,spg_int_max)))</f>
+        <v>1.255448232589</v>
+      </c>
+      <c r="E546" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The shorter of the lag O₂ bound (or the legacy guard D89) and the H₂-screen interval restated on the basis of D91.</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-up interval (as run)</t>
+        </is>
+      </c>
+      <c r="B547" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_su_run</t>
+        </is>
+      </c>
+      <c r="C547" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D547" s="41">
+        <f>IF(FLOOR(spg_int_su_opt*spg_dur_eq/spg_dur_eq_opt,interval_res)*60&gt;spg_dur,FLOOR(spg_int_su_opt*spg_dur_eq/spg_dur_eq_opt,interval_res),NA())</f>
+        <v>1.21</v>
+      </c>
+      <c r="E547" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rounded down to the command resolution for the pulse in use, as D420; #N/A if no gap is left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-up binding constraint</t>
+        </is>
+      </c>
+      <c r="B548" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">su_binding</t>
+        </is>
+      </c>
+      <c r="C548" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D548" s="41" t="str">
+        <f>IF(AND(ISNUMBER(spg_int_H2safe_mt),spg_int_H2safe_mt*spg_dur_eq_opt/spg_dur_eq&lt;IF(ISNUMBER(spg_int_DO_l),spg_int_DO_l,spg_int_max)),"the H₂ flammability screen (Biology D92)",IF(ISNUMBER(spg_int_DO_l),"lag O₂ dilution","the legacy O₂ flush guard (lag DO target unreachable)"))</f>
+        <v>the legacy O₂ flush guard (lag DO target unreachable)</v>
+      </c>
+      <c r="E548" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which bound sets the start-up interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gap between pulses — start-up</t>
+        </is>
+      </c>
+      <c r="B549" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">t_gap_su_h</t>
+        </is>
+      </c>
+      <c r="C549" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="D549" s="41">
+        <f>MAX(0,spg_int_su_run*60-spg_dur)/3600</f>
+        <v>0.019986111111</v>
+      </c>
+      <c r="E549" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D325 at the start-up interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace turnovers per gap — start-up</t>
+        </is>
+      </c>
+      <c r="B550" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x_su</t>
+        </is>
+      </c>
+      <c r="C550" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D550" s="41">
+        <f>F_gap_l*t_gap_su_h/n_hs_gas</f>
+        <v>0.035940779</v>
+      </c>
+      <c r="E550" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D354.</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Φ(x) — start-up</t>
+        </is>
+      </c>
+      <c r="B551" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">phi_su</t>
+        </is>
+      </c>
+      <c r="C551" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D551" s="41">
+        <f>IF(x_su&gt;0,(1-EXP(-x_su))/x_su,1)</f>
+        <v>0.982242979832</v>
+      </c>
+      <c r="E551" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D355.</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ψ(x) — start-up</t>
+        </is>
+      </c>
+      <c r="B552" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">psi_su</t>
+        </is>
+      </c>
+      <c r="C552" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D552" s="41">
+        <f>IF(x_su&gt;0,(x_su-1+EXP(-x_su))/x_su^2,1/2)</f>
+        <v>0.494063308071</v>
+      </c>
+      <c r="E552" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D356.</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ rise per gap, undiluted — start-up</t>
+        </is>
+      </c>
+      <c r="B553" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dy_O2_su</t>
+        </is>
+      </c>
+      <c r="C553" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D553" s="41">
+        <f>S_O2_l*t_gap_su_h/n_hs_gas</f>
+        <v>0.011040074343</v>
+      </c>
+      <c r="E553" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D357.</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ just before a pulse — start-up</t>
+        </is>
+      </c>
+      <c r="B554" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_end_su</t>
+        </is>
+      </c>
+      <c r="C554" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D554" s="41">
+        <f>dy_O2_su*phi_su/(1-flush_ret*EXP(-x_su))</f>
+        <v>0.016702620853</v>
+      </c>
+      <c r="E554" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D358.</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Time-mean headspace O₂ — start-up</t>
+        </is>
+      </c>
+      <c r="B555" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_O2_avg_su</t>
+        </is>
+      </c>
+      <c r="C555" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D555" s="41">
+        <f>y_O2_end_su*flush_ret*phi_su+dy_O2_su*psi_su</f>
+        <v>0.011419634754</v>
+      </c>
+      <c r="E555" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D360.</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO — start-up (mg/L)</t>
+        </is>
+      </c>
+      <c r="B556" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_avg_su_mgL</t>
+        </is>
+      </c>
+      <c r="C556" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D556" s="41">
+        <f>(DO_surf_excess_lag+H_O2_T*P_dry*y_O2_avg_su)*M_O2</f>
+        <v>4.090403518227</v>
+      </c>
+      <c r="E556" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D364 at the start-up interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peak DO — start-up (mg/L)</t>
+        </is>
+      </c>
+      <c r="B557" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_peak_su_mgL</t>
+        </is>
+      </c>
+      <c r="C557" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mg/L</t>
+        </is>
+      </c>
+      <c r="D557" s="41">
+        <f>(DO_surf_excess_lag+H_O2_T*P_dry*MAX(y_O2_avg_su,y_O2_end_su-(S_O2_l-F_gap_l*y_O2_end_su)/n_hs_gas*tau_L_h))*M_O2</f>
+        <v>4.090403518227</v>
+      </c>
+      <c r="E557" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D365 at the start-up interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace H₂ just before a pulse — start-up</t>
+        </is>
+      </c>
+      <c r="B558" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">y_H2_end_su</t>
+        </is>
+      </c>
+      <c r="C558" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D558" s="41">
+        <f>H2_src_l*t_gap_su_h/n_hs_gas*phi_su/(1-flush_ret*EXP(-x_su))</f>
+        <v>0.029078582503</v>
+      </c>
+      <c r="E558" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D388 at the start-up interval.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gas model: Calibrations sections in logical order (pure move, Excel-verified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -25,7 +25,7 @@
     <definedName name="A_DH" localSheetId="3">Chemistry!$D$186</definedName>
     <definedName name="a_int" localSheetId="5">'Mass Transfer'!$D$49</definedName>
     <definedName name="a_surf" localSheetId="5">'Mass Transfer'!$D$71</definedName>
-    <definedName name="A_x" localSheetId="7">Calibrations!$D$160</definedName>
+    <definedName name="A_x" localSheetId="7">Calibrations!$D$186</definedName>
     <definedName name="A_x" localSheetId="1">Geometry!$D$21</definedName>
     <definedName name="A_x" localSheetId="5">'Mass Transfer'!$D$17</definedName>
     <definedName name="alk_NaHCO3_gL" localSheetId="3">Chemistry!$D$308</definedName>
@@ -47,7 +47,7 @@
     <definedName name="bleach_flag" localSheetId="3">Chemistry!$D$109</definedName>
     <definedName name="bleach_rate" localSheetId="3">Chemistry!$D$107</definedName>
     <definedName name="bleach_t1ppm" localSheetId="3">Chemistry!$D$108</definedName>
-    <definedName name="bp_const" localSheetId="7">Calibrations!$D$140</definedName>
+    <definedName name="bp_const" localSheetId="7">Calibrations!$D$166</definedName>
     <definedName name="bubble_regime" localSheetId="5">'Mass Transfer'!$D$64</definedName>
     <definedName name="buffer_caution_frac" localSheetId="3">Chemistry!$D$238</definedName>
     <definedName name="buffer_flag" localSheetId="3">Chemistry!$D$219</definedName>
@@ -64,8 +64,8 @@
     <definedName name="C_eff_lo_Cl2" localSheetId="3">Chemistry!$D$259</definedName>
     <definedName name="C_H2_sat" localSheetId="4">Biology!$D$41</definedName>
     <definedName name="C_sat_CO2" localSheetId="5">'Mass Transfer'!$D$145</definedName>
-    <definedName name="ca_rho_0" localSheetId="7">Calibrations!$D$155</definedName>
-    <definedName name="ca_rho_k" localSheetId="7">Calibrations!$D$156</definedName>
+    <definedName name="ca_rho_0" localSheetId="7">Calibrations!$D$181</definedName>
+    <definedName name="ca_rho_k" localSheetId="7">Calibrations!$D$182</definedName>
     <definedName name="cal_Dint">Calibrations!$D$75</definedName>
     <definedName name="cal_DO_impair">Calibrations!$D$105</definedName>
     <definedName name="cal_DO_min">Calibrations!$D$103</definedName>
@@ -267,7 +267,7 @@
     <definedName name="etaF_OER" localSheetId="2">Electrochemistry!$D$26</definedName>
     <definedName name="etaF_OER_calc" localSheetId="2">Electrochemistry!$D$104</definedName>
     <definedName name="f_Cl_anode" localSheetId="2">Electrochemistry!$D$103</definedName>
-    <definedName name="F_const" localSheetId="7">Calibrations!$D$162</definedName>
+    <definedName name="F_const" localSheetId="7">Calibrations!$D$188</definedName>
     <definedName name="F_const" localSheetId="2">Electrochemistry!$D$15</definedName>
     <definedName name="F_gap_g" localSheetId="5">'Mass Transfer'!$D$331</definedName>
     <definedName name="F_gap_l" localSheetId="5">'Mass Transfer'!$D$353</definedName>
@@ -548,7 +548,7 @@
     <definedName name="od_ok" localSheetId="5">'Mass Transfer'!$D$95</definedName>
     <definedName name="opt_binding" localSheetId="5">'Mass Transfer'!$D$94</definedName>
     <definedName name="organism_sel" localSheetId="4">Biology!$D$7</definedName>
-    <definedName name="organism_sel" localSheetId="7">Calibrations!$D$158</definedName>
+    <definedName name="organism_sel" localSheetId="7">Calibrations!$D$184</definedName>
     <definedName name="organism_sel" localSheetId="2">Electrochemistry!$D$154</definedName>
     <definedName name="organism_sel" localSheetId="0">Summary!$D$4</definedName>
     <definedName name="OrganismList">Biology!$A$52:$A$57</definedName>
@@ -602,11 +602,11 @@
     <definedName name="pool_psi" localSheetId="5">'Mass Transfer'!$D$378</definedName>
     <definedName name="pool_ret" localSheetId="5">'Mass Transfer'!$D$380</definedName>
     <definedName name="pool_x" localSheetId="5">'Mass Transfer'!$D$376</definedName>
-    <definedName name="por_break_1" localSheetId="7">Calibrations!$D$141</definedName>
-    <definedName name="por_break_2" localSheetId="7">Calibrations!$D$142</definedName>
-    <definedName name="por_break_3" localSheetId="7">Calibrations!$D$143</definedName>
-    <definedName name="por_break_4" localSheetId="7">Calibrations!$D$144</definedName>
-    <definedName name="por_break_5" localSheetId="7">Calibrations!$D$145</definedName>
+    <definedName name="por_break_1" localSheetId="7">Calibrations!$D$167</definedName>
+    <definedName name="por_break_2" localSheetId="7">Calibrations!$D$168</definedName>
+    <definedName name="por_break_3" localSheetId="7">Calibrations!$D$169</definedName>
+    <definedName name="por_break_4" localSheetId="7">Calibrations!$D$170</definedName>
+    <definedName name="por_break_5" localSheetId="7">Calibrations!$D$171</definedName>
     <definedName name="por_grade" localSheetId="5">'Mass Transfer'!$D$20</definedName>
     <definedName name="por_grade_e" localSheetId="2">Electrochemistry!$D$32</definedName>
     <definedName name="por_pore" localSheetId="5">'Mass Transfer'!$D$39</definedName>
@@ -627,11 +627,11 @@
     <definedName name="pulse_V0" localSheetId="5">'Mass Transfer'!$D$408</definedName>
     <definedName name="pulses_d" localSheetId="5">'Mass Transfer'!$D$125</definedName>
     <definedName name="pulses_h" localSheetId="5">'Mass Transfer'!$D$124</definedName>
-    <definedName name="pw_A" localSheetId="7">Calibrations!$D$149</definedName>
+    <definedName name="pw_A" localSheetId="7">Calibrations!$D$175</definedName>
     <definedName name="pw_A" localSheetId="5">'Mass Transfer'!$D$203</definedName>
-    <definedName name="pw_B" localSheetId="7">Calibrations!$D$150</definedName>
+    <definedName name="pw_B" localSheetId="7">Calibrations!$D$176</definedName>
     <definedName name="pw_B" localSheetId="5">'Mass Transfer'!$D$204</definedName>
-    <definedName name="pw_C" localSheetId="7">Calibrations!$D$151</definedName>
+    <definedName name="pw_C" localSheetId="7">Calibrations!$D$177</definedName>
     <definedName name="pw_C" localSheetId="5">'Mass Transfer'!$D$205</definedName>
     <definedName name="Q_backdraw" localSheetId="5">'Mass Transfer'!$D$385</definedName>
     <definedName name="Q_carry_max" localSheetId="5">'Mass Transfer'!$D$413</definedName>
@@ -643,7 +643,7 @@
     <definedName name="R_chloramine" localSheetId="3">Chemistry!$D$144</definedName>
     <definedName name="R_chloramine_hi" localSheetId="3">Chemistry!$D$153</definedName>
     <definedName name="R_chloramine_lo" localSheetId="3">Chemistry!$D$152</definedName>
-    <definedName name="R_gas" localSheetId="7">Calibrations!$D$161</definedName>
+    <definedName name="R_gas" localSheetId="7">Calibrations!$D$187</definedName>
     <definedName name="R_gas" localSheetId="3">Chemistry!$D$9</definedName>
     <definedName name="R_gas" localSheetId="2">Electrochemistry!$D$7</definedName>
     <definedName name="R_gas" localSheetId="5">'Mass Transfer'!$D$101</definedName>
@@ -653,7 +653,7 @@
     <definedName name="r_H2O2_lag" localSheetId="2">Electrochemistry!$D$152</definedName>
     <definedName name="r_HCO3_ref" localSheetId="3">Chemistry!$D$293</definedName>
     <definedName name="Reactor" localSheetId="5">'Mass Transfer'!$D$115</definedName>
-    <definedName name="Reactor_sel" localSheetId="7">Calibrations!$D$157</definedName>
+    <definedName name="Reactor_sel" localSheetId="7">Calibrations!$D$183</definedName>
     <definedName name="reactor_sel" localSheetId="1">Geometry!$D$5</definedName>
     <definedName name="Reactor_sel" localSheetId="0">Summary!$D$2</definedName>
     <definedName name="ReactorList">Geometry!$A$59:$A$80</definedName>
@@ -697,7 +697,7 @@
     <definedName name="rO2_gen" localSheetId="2">Electrochemistry!$D$22</definedName>
     <definedName name="rod_d" localSheetId="1">Geometry!$D$26</definedName>
     <definedName name="rod_n" localSheetId="1">Geometry!$D$27</definedName>
-    <definedName name="rx_ver" localSheetId="7">Calibrations!$D$159</definedName>
+    <definedName name="rx_ver" localSheetId="7">Calibrations!$D$185</definedName>
     <definedName name="rx_ver" localSheetId="1">Geometry!$D$51</definedName>
     <definedName name="S_O2_g" localSheetId="5">'Mass Transfer'!$D$327</definedName>
     <definedName name="S_O2_l" localSheetId="5">'Mass Transfer'!$D$349</definedName>
@@ -771,7 +771,7 @@
     <definedName name="T_ref" localSheetId="3">Chemistry!$D$229</definedName>
     <definedName name="T_ref" localSheetId="5">'Mass Transfer'!$D$209</definedName>
     <definedName name="T_zero_C" localSheetId="4">Biology!$D$66</definedName>
-    <definedName name="T_zero_C" localSheetId="7">Calibrations!$D$148</definedName>
+    <definedName name="T_zero_C" localSheetId="7">Calibrations!$D$174</definedName>
     <definedName name="T_zero_C" localSheetId="5">'Mass Transfer'!$D$210</definedName>
     <definedName name="target_DO_frac" localSheetId="5">'Mass Transfer'!$D$84</definedName>
     <definedName name="tau_hs" localSheetId="5">'Mass Transfer'!$D$144</definedName>
@@ -857,9 +857,9 @@
     <definedName name="y_O2_post_g" localSheetId="5">'Mass Transfer'!$D$337</definedName>
     <definedName name="y_O2_post_l" localSheetId="5">'Mass Transfer'!$D$359</definedName>
     <definedName name="y_O2_star" localSheetId="5">'Mass Transfer'!$D$183</definedName>
-    <definedName name="z_e_H2" localSheetId="7">Calibrations!$D$146</definedName>
+    <definedName name="z_e_H2" localSheetId="7">Calibrations!$D$172</definedName>
     <definedName name="z_e_H2" localSheetId="2">Electrochemistry!$D$16</definedName>
-    <definedName name="z_e_O2" localSheetId="7">Calibrations!$D$147</definedName>
+    <definedName name="z_e_O2" localSheetId="7">Calibrations!$D$173</definedName>
     <definedName name="z_e_O2" localSheetId="2">Electrochemistry!$D$17</definedName>
     <definedName name="z_e_ORR" localSheetId="2">Electrochemistry!$D$27</definedName>
     <definedName name="interval_res" localSheetId="5">'Mass Transfer'!$D$419</definedName>
@@ -975,17 +975,17 @@
     <definedName name="Cl_AMYBO03" localSheetId="8">AMYBO03!$D$57</definedName>
     <definedName name="kappa0_AMYBO03" localSheetId="8">AMYBO03!$D$58</definedName>
     <definedName name="I_AMYBO03" localSheetId="8">AMYBO03!$D$59</definedName>
-    <definedName name="cal_km_O2">Calibrations!$D$176</definedName>
-    <definedName name="cal_tau_NH2Cl">Calibrations!$D$189</definedName>
-    <definedName name="n_e_fcn" localSheetId="7">Calibrations!$D$192</definedName>
-    <definedName name="km_T_tol" localSheetId="7">Calibrations!$D$193</definedName>
-    <definedName name="stir_rpm_set" localSheetId="7">Calibrations!$D$194</definedName>
-    <definedName name="temp_C" localSheetId="7">Calibrations!$D$195</definedName>
-    <definedName name="media_sel" localSheetId="7">Calibrations!$D$196</definedName>
-    <definedName name="electrode_sel" localSheetId="7">Calibrations!$D$197</definedName>
-    <definedName name="D_O2" localSheetId="7">Calibrations!$D$198</definedName>
-    <definedName name="km_exp" localSheetId="7">Calibrations!$D$199</definedName>
-    <definedName name="M_Cl2" localSheetId="7">Calibrations!$D$200</definedName>
+    <definedName name="cal_km_O2">Calibrations!$D$150</definedName>
+    <definedName name="cal_tau_NH2Cl">Calibrations!$D$163</definedName>
+    <definedName name="n_e_fcn" localSheetId="7">Calibrations!$D$190</definedName>
+    <definedName name="km_T_tol" localSheetId="7">Calibrations!$D$191</definedName>
+    <definedName name="stir_rpm_set" localSheetId="7">Calibrations!$D$192</definedName>
+    <definedName name="temp_C" localSheetId="7">Calibrations!$D$193</definedName>
+    <definedName name="media_sel" localSheetId="7">Calibrations!$D$194</definedName>
+    <definedName name="electrode_sel" localSheetId="7">Calibrations!$D$195</definedName>
+    <definedName name="D_O2" localSheetId="7">Calibrations!$D$196</definedName>
+    <definedName name="km_exp" localSheetId="7">Calibrations!$D$197</definedName>
+    <definedName name="M_Cl2" localSheetId="7">Calibrations!$D$198</definedName>
     <definedName name="km_O2_default" localSheetId="2">Electrochemistry!$D$165</definedName>
     <definedName name="tau_NH2Cl_default" localSheetId="3">Chemistry!$D$314</definedName>
     <definedName name="P_Cl_max" localSheetId="3">Chemistry!$D$315</definedName>
@@ -23086,7 +23086,7 @@
       </c>
       <c r="E315" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">The production ceiling P in the chloramine steady state (the second term of D311): the CER-efficiency-limited current as mol/L/s. Read with D271 and D47 to turn a DPD plateau into a lifetime (Calibrations rows 181–188).</t>
+          <t xml:space="preserve">The production ceiling P in the chloramine steady state (the second term of D311): the CER-efficiency-limited current as mol/L/s. Read with D271 and D47 to turn a DPD plateau into a lifetime (Calibrations rows 155–162).</t>
         </is>
       </c>
     </row>
@@ -38220,7 +38220,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:O200"/>
+  <dimension ref="A1:O198"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16" width="12" customWidth="1"/>
@@ -40786,990 +40786,1041 @@
       <c r="L138" s="72"/>
       <c r="M138" s="72"/>
     </row>
-    <row r="139" spans="1:13" ht="16" x14ac:dyDescent="0.2">
-      <c r="A139" s="5" t="s">
+    <row r="139">
+      <c r="A139" s="98" t="str">
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/electrode-mass-transfer.md","ELECTRODE MASS TRANSFER  (ferricyanide limiting current)")</f>
+        <v>ELECTRODE MASS TRANSFER  (ferricyanide limiting current)</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use: average O₂-scaled k_m of the included runs for the active reactor and electrode, at the Summary stirrer rate and within the temperature tolerance (D191) of the Summary temperature; other runs are kept but not used. One k_m serves both electrodes in the model. Feeds Electrochemistry km_O2 (D83).</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Researcher</t>
+        </is>
+      </c>
+      <c r="B141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="C141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reactor</t>
+        </is>
+      </c>
+      <c r="D141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode (Summary D3 list)</t>
+        </is>
+      </c>
+      <c r="E141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stir rate (rpm)</t>
+        </is>
+      </c>
+      <c r="F141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temp (°C)</t>
+        </is>
+      </c>
+      <c r="G141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Limiting current (mA)</t>
+        </is>
+      </c>
+      <c r="H141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrode area (cm²)</t>
+        </is>
+      </c>
+      <c r="I141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ferricyanide (mM)</t>
+        </is>
+      </c>
+      <c r="J141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D ferricyanide (m²/s)</t>
+        </is>
+      </c>
+      <c r="K141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_m ferricyanide (computed, cm/s)</t>
+        </is>
+      </c>
+      <c r="L141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">k_m O₂ (computed, cm/s)</t>
+        </is>
+      </c>
+      <c r="M141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type (auto)</t>
+        </is>
+      </c>
+      <c r="N141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Include?</t>
+        </is>
+      </c>
+      <c r="O141" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="93"/>
+      <c r="B142" s="94"/>
+      <c r="C142" s="93"/>
+      <c r="D142" s="93"/>
+      <c r="E142" s="94"/>
+      <c r="F142" s="94"/>
+      <c r="G142" s="94"/>
+      <c r="H142" s="94"/>
+      <c r="I142" s="94"/>
+      <c r="J142" s="94"/>
+      <c r="K142" s="100" t="str">
+        <f>IF(OR(G142="",H142="",I142=""),"",IFERROR((G142/1000)/(n_e_fcn*F_const*(H142/10000)*I142)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L142" s="100" t="str">
+        <f>IF(OR(K142="",J142=""),"",IFERROR(K142*(D_O2/J142)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M142" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C142,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N142" s="93"/>
+      <c r="O142" s="93"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="93"/>
+      <c r="B143" s="94"/>
+      <c r="C143" s="93"/>
+      <c r="D143" s="93"/>
+      <c r="E143" s="94"/>
+      <c r="F143" s="94"/>
+      <c r="G143" s="94"/>
+      <c r="H143" s="94"/>
+      <c r="I143" s="94"/>
+      <c r="J143" s="94"/>
+      <c r="K143" s="100" t="str">
+        <f>IF(OR(G143="",H143="",I143=""),"",IFERROR((G143/1000)/(n_e_fcn*F_const*(H143/10000)*I143)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L143" s="100" t="str">
+        <f>IF(OR(K143="",J143=""),"",IFERROR(K143*(D_O2/J143)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M143" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C143,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N143" s="93"/>
+      <c r="O143" s="93"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="93"/>
+      <c r="B144" s="94"/>
+      <c r="C144" s="93"/>
+      <c r="D144" s="93"/>
+      <c r="E144" s="94"/>
+      <c r="F144" s="94"/>
+      <c r="G144" s="94"/>
+      <c r="H144" s="94"/>
+      <c r="I144" s="94"/>
+      <c r="J144" s="94"/>
+      <c r="K144" s="100" t="str">
+        <f>IF(OR(G144="",H144="",I144=""),"",IFERROR((G144/1000)/(n_e_fcn*F_const*(H144/10000)*I144)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L144" s="100" t="str">
+        <f>IF(OR(K144="",J144=""),"",IFERROR(K144*(D_O2/J144)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M144" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C144,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N144" s="93"/>
+      <c r="O144" s="93"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="93"/>
+      <c r="B145" s="94"/>
+      <c r="C145" s="93"/>
+      <c r="D145" s="93"/>
+      <c r="E145" s="94"/>
+      <c r="F145" s="94"/>
+      <c r="G145" s="94"/>
+      <c r="H145" s="94"/>
+      <c r="I145" s="94"/>
+      <c r="J145" s="94"/>
+      <c r="K145" s="100" t="str">
+        <f>IF(OR(G145="",H145="",I145=""),"",IFERROR((G145/1000)/(n_e_fcn*F_const*(H145/10000)*I145)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L145" s="100" t="str">
+        <f>IF(OR(K145="",J145=""),"",IFERROR(K145*(D_O2/J145)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M145" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C145,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N145" s="93"/>
+      <c r="O145" s="93"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="93"/>
+      <c r="B146" s="94"/>
+      <c r="C146" s="93"/>
+      <c r="D146" s="93"/>
+      <c r="E146" s="94"/>
+      <c r="F146" s="94"/>
+      <c r="G146" s="94"/>
+      <c r="H146" s="94"/>
+      <c r="I146" s="94"/>
+      <c r="J146" s="94"/>
+      <c r="K146" s="100" t="str">
+        <f>IF(OR(G146="",H146="",I146=""),"",IFERROR((G146/1000)/(n_e_fcn*F_const*(H146/10000)*I146)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L146" s="100" t="str">
+        <f>IF(OR(K146="",J146=""),"",IFERROR(K146*(D_O2/J146)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M146" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C146,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N146" s="93"/>
+      <c r="O146" s="93"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="93"/>
+      <c r="B147" s="94"/>
+      <c r="C147" s="93"/>
+      <c r="D147" s="93"/>
+      <c r="E147" s="94"/>
+      <c r="F147" s="94"/>
+      <c r="G147" s="94"/>
+      <c r="H147" s="94"/>
+      <c r="I147" s="94"/>
+      <c r="J147" s="94"/>
+      <c r="K147" s="100" t="str">
+        <f>IF(OR(G147="",H147="",I147=""),"",IFERROR((G147/1000)/(n_e_fcn*F_const*(H147/10000)*I147)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L147" s="100" t="str">
+        <f>IF(OR(K147="",J147=""),"",IFERROR(K147*(D_O2/J147)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M147" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C147,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N147" s="93"/>
+      <c r="O147" s="93"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="93"/>
+      <c r="B148" s="94"/>
+      <c r="C148" s="93"/>
+      <c r="D148" s="93"/>
+      <c r="E148" s="94"/>
+      <c r="F148" s="94"/>
+      <c r="G148" s="94"/>
+      <c r="H148" s="94"/>
+      <c r="I148" s="94"/>
+      <c r="J148" s="94"/>
+      <c r="K148" s="100" t="str">
+        <f>IF(OR(G148="",H148="",I148=""),"",IFERROR((G148/1000)/(n_e_fcn*F_const*(H148/10000)*I148)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L148" s="100" t="str">
+        <f>IF(OR(K148="",J148=""),"",IFERROR(K148*(D_O2/J148)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M148" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C148,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N148" s="93"/>
+      <c r="O148" s="93"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="93"/>
+      <c r="B149" s="94"/>
+      <c r="C149" s="93"/>
+      <c r="D149" s="93"/>
+      <c r="E149" s="94"/>
+      <c r="F149" s="94"/>
+      <c r="G149" s="94"/>
+      <c r="H149" s="94"/>
+      <c r="I149" s="94"/>
+      <c r="J149" s="94"/>
+      <c r="K149" s="100" t="str">
+        <f>IF(OR(G149="",H149="",I149=""),"",IFERROR((G149/1000)/(n_e_fcn*F_const*(H149/10000)*I149)*100,""))</f>
+        <v/>
+      </c>
+      <c r="L149" s="100" t="str">
+        <f>IF(OR(K149="",J149=""),"",IFERROR(K149*(D_O2/J149)^km_exp,""))</f>
+        <v/>
+      </c>
+      <c r="M149" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C149,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N149" s="93"/>
+      <c r="O149" s="93"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - k_m O₂</t>
+        </is>
+      </c>
+      <c r="C150" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cm/s</t>
+        </is>
+      </c>
+      <c r="D150" s="95" t="str">
+        <f>IFERROR(AVERAGEIFS(L142:L149,C142:C149,Reactor_sel,D142:D149,electrode_sel,N142:N149,"y",E142:E149,stir_rpm_set,F142:F149,"&gt;="&amp;(temp_C-km_T_tol),F142:F149,"&lt;="&amp;(temp_C+km_T_tol)),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="98" t="str">
+        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/chlorine-species.md","MONOCHLORAMINE LIFETIME  (DPD combined chlorine at plateau)")</f>
+        <v>MONOCHLORAMINE LIFETIME  (DPD combined chlorine at plateau)</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use: average of the included runs for the active reactor and medium. Inverts the model’s own steady state B = min(C·kτ/(1+kτ), P·τ): τ = max(B/(k(C−B)), B/P), with k, C and P read from Chemistry D271, D47 and D315 at the run settings (none depends on τ). Feeds Chemistry tau_NH2Cl (D142).</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Researcher</t>
+        </is>
+      </c>
+      <c r="B154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Date</t>
+        </is>
+      </c>
+      <c r="C154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reactor</t>
+        </is>
+      </c>
+      <c r="D154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Combined chlorine plateau (mg/L as Cl₂)</t>
+        </is>
+      </c>
+      <c r="F154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chloride turnover k (1/s, Chemistry D271)</t>
+        </is>
+      </c>
+      <c r="G154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chloride pool C (mol/L, Chemistry D47)</t>
+        </is>
+      </c>
+      <c r="H154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max production P (mol/L/s, Chemistry D315)</t>
+        </is>
+      </c>
+      <c r="I154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lifetime (computed, h)</t>
+        </is>
+      </c>
+      <c r="J154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type (auto)</t>
+        </is>
+      </c>
+      <c r="K154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Include?</t>
+        </is>
+      </c>
+      <c r="L154" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="93"/>
+      <c r="B155" s="94"/>
+      <c r="C155" s="93"/>
+      <c r="D155" s="93"/>
+      <c r="E155" s="94"/>
+      <c r="F155" s="94"/>
+      <c r="G155" s="94"/>
+      <c r="H155" s="94"/>
+      <c r="I155" s="100" t="str">
+        <f>IF(OR(E155="",F155="",G155="",H155=""),"",IF(E155/M_Cl2&gt;=G155,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E155/M_Cl2/(F155*(G155-E155/M_Cl2)),E155/M_Cl2/H155)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J155" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C155,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K155" s="93"/>
+      <c r="L155" s="93"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="93"/>
+      <c r="B156" s="94"/>
+      <c r="C156" s="93"/>
+      <c r="D156" s="93"/>
+      <c r="E156" s="94"/>
+      <c r="F156" s="94"/>
+      <c r="G156" s="94"/>
+      <c r="H156" s="94"/>
+      <c r="I156" s="100" t="str">
+        <f>IF(OR(E156="",F156="",G156="",H156=""),"",IF(E156/M_Cl2&gt;=G156,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E156/M_Cl2/(F156*(G156-E156/M_Cl2)),E156/M_Cl2/H156)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J156" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C156,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K156" s="93"/>
+      <c r="L156" s="93"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="93"/>
+      <c r="B157" s="94"/>
+      <c r="C157" s="93"/>
+      <c r="D157" s="93"/>
+      <c r="E157" s="94"/>
+      <c r="F157" s="94"/>
+      <c r="G157" s="94"/>
+      <c r="H157" s="94"/>
+      <c r="I157" s="100" t="str">
+        <f>IF(OR(E157="",F157="",G157="",H157=""),"",IF(E157/M_Cl2&gt;=G157,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E157/M_Cl2/(F157*(G157-E157/M_Cl2)),E157/M_Cl2/H157)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J157" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C157,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K157" s="93"/>
+      <c r="L157" s="93"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="93"/>
+      <c r="B158" s="94"/>
+      <c r="C158" s="93"/>
+      <c r="D158" s="93"/>
+      <c r="E158" s="94"/>
+      <c r="F158" s="94"/>
+      <c r="G158" s="94"/>
+      <c r="H158" s="94"/>
+      <c r="I158" s="100" t="str">
+        <f>IF(OR(E158="",F158="",G158="",H158=""),"",IF(E158/M_Cl2&gt;=G158,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E158/M_Cl2/(F158*(G158-E158/M_Cl2)),E158/M_Cl2/H158)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J158" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C158,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K158" s="93"/>
+      <c r="L158" s="93"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="93"/>
+      <c r="B159" s="94"/>
+      <c r="C159" s="93"/>
+      <c r="D159" s="93"/>
+      <c r="E159" s="94"/>
+      <c r="F159" s="94"/>
+      <c r="G159" s="94"/>
+      <c r="H159" s="94"/>
+      <c r="I159" s="100" t="str">
+        <f>IF(OR(E159="",F159="",G159="",H159=""),"",IF(E159/M_Cl2&gt;=G159,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E159/M_Cl2/(F159*(G159-E159/M_Cl2)),E159/M_Cl2/H159)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J159" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C159,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K159" s="93"/>
+      <c r="L159" s="93"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="93"/>
+      <c r="B160" s="94"/>
+      <c r="C160" s="93"/>
+      <c r="D160" s="93"/>
+      <c r="E160" s="94"/>
+      <c r="F160" s="94"/>
+      <c r="G160" s="94"/>
+      <c r="H160" s="94"/>
+      <c r="I160" s="100" t="str">
+        <f>IF(OR(E160="",F160="",G160="",H160=""),"",IF(E160/M_Cl2&gt;=G160,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E160/M_Cl2/(F160*(G160-E160/M_Cl2)),E160/M_Cl2/H160)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J160" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C160,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K160" s="93"/>
+      <c r="L160" s="93"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="93"/>
+      <c r="B161" s="94"/>
+      <c r="C161" s="93"/>
+      <c r="D161" s="93"/>
+      <c r="E161" s="94"/>
+      <c r="F161" s="94"/>
+      <c r="G161" s="94"/>
+      <c r="H161" s="94"/>
+      <c r="I161" s="100" t="str">
+        <f>IF(OR(E161="",F161="",G161="",H161=""),"",IF(E161/M_Cl2&gt;=G161,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E161/M_Cl2/(F161*(G161-E161/M_Cl2)),E161/M_Cl2/H161)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J161" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C161,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K161" s="93"/>
+      <c r="L161" s="93"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="93"/>
+      <c r="B162" s="94"/>
+      <c r="C162" s="93"/>
+      <c r="D162" s="93"/>
+      <c r="E162" s="94"/>
+      <c r="F162" s="94"/>
+      <c r="G162" s="94"/>
+      <c r="H162" s="94"/>
+      <c r="I162" s="100" t="str">
+        <f>IF(OR(E162="",F162="",G162="",H162=""),"",IF(E162/M_Cl2&gt;=G162,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E162/M_Cl2/(F162*(G162-E162/M_Cl2)),E162/M_Cl2/H162)/3600,"")))</f>
+        <v/>
+      </c>
+      <c r="J162" s="100" t="str">
+        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C162,ReactorList,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K162" s="93"/>
+      <c r="L162" s="93"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - monochloramine lifetime</t>
+        </is>
+      </c>
+      <c r="C163" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">h</t>
+        </is>
+      </c>
+      <c r="D163" s="95" t="str">
+        <f>IFERROR(AVERAGEIFS(I155:I162,C155:C162,Reactor_sel,D155:D162,media_sel,K155:K162,"y"),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A164" s="18"/>
+      <c r="B164" s="72"/>
+      <c r="C164" s="20"/>
+      <c r="D164" s="133"/>
+      <c r="E164" s="134"/>
+    </row>
+    <row r="165" spans="1:13" ht="16" x14ac:dyDescent="0.2">
+      <c r="A165" s="5" t="s">
         <v>2645</v>
       </c>
-      <c r="B139" s="72"/>
-      <c r="C139" s="72"/>
-      <c r="D139" s="72"/>
-      <c r="E139" s="72"/>
-      <c r="F139" s="72"/>
-      <c r="G139" s="72"/>
-      <c r="H139" s="72"/>
-      <c r="I139" s="72"/>
-      <c r="J139" s="72"/>
-      <c r="K139" s="72"/>
-      <c r="L139" s="72"/>
-      <c r="M139" s="72"/>
-    </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A140" s="18" t="s">
+      <c r="B165" s="72"/>
+      <c r="C165" s="72"/>
+      <c r="D165" s="72"/>
+      <c r="E165" s="72"/>
+      <c r="F165" s="72"/>
+      <c r="G165" s="72"/>
+      <c r="H165" s="72"/>
+      <c r="I165" s="72"/>
+      <c r="J165" s="72"/>
+      <c r="K165" s="72"/>
+      <c r="L165" s="72"/>
+      <c r="M165" s="72"/>
+    </row>
+    <row r="166" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A166" s="18" t="s">
         <v>2646</v>
       </c>
-      <c r="B140" s="72" t="s">
+      <c r="B166" s="72" t="s">
         <v>2647</v>
       </c>
-      <c r="C140" s="20" t="s">
+      <c r="C166" s="20" t="s">
         <v>2648</v>
       </c>
-      <c r="D140" s="132">
+      <c r="D166" s="132">
         <v>291.2</v>
       </c>
-      <c r="E140" s="72" t="s">
+      <c r="E166" s="72" t="s">
         <v>2649</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A141" s="18" t="s">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A167" s="18" t="s">
         <v>2650</v>
       </c>
-      <c r="B141" s="72" t="s">
+      <c r="B167" s="72" t="s">
         <v>2651</v>
       </c>
-      <c r="C141" s="20" t="s">
+      <c r="C167" s="20" t="s">
         <v>518</v>
       </c>
-      <c r="D141" s="132">
+      <c r="D167" s="132">
         <v>160</v>
       </c>
-      <c r="E141" s="72" t="s">
+      <c r="E167" s="72" t="s">
         <v>2652</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A142" s="18" t="s">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A168" s="18" t="s">
         <v>2653</v>
       </c>
-      <c r="B142" s="72" t="s">
+      <c r="B168" s="72" t="s">
         <v>2654</v>
       </c>
-      <c r="C142" s="20" t="s">
+      <c r="C168" s="20" t="s">
         <v>518</v>
       </c>
-      <c r="D142" s="132">
+      <c r="D168" s="132">
         <v>100</v>
       </c>
-      <c r="E142" s="72" t="s">
+      <c r="E168" s="72" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A143" s="18" t="s">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A169" s="18" t="s">
         <v>2656</v>
       </c>
-      <c r="B143" s="72" t="s">
+      <c r="B169" s="72" t="s">
         <v>2657</v>
       </c>
-      <c r="C143" s="20" t="s">
+      <c r="C169" s="20" t="s">
         <v>518</v>
       </c>
-      <c r="D143" s="132">
+      <c r="D169" s="132">
         <v>40</v>
       </c>
-      <c r="E143" s="72" t="s">
+      <c r="E169" s="72" t="s">
         <v>2658</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A144" s="18" t="s">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A170" s="18" t="s">
         <v>2659</v>
       </c>
-      <c r="B144" s="72" t="s">
+      <c r="B170" s="72" t="s">
         <v>2660</v>
       </c>
-      <c r="C144" s="20" t="s">
+      <c r="C170" s="20" t="s">
         <v>518</v>
       </c>
-      <c r="D144" s="132">
+      <c r="D170" s="132">
         <v>16</v>
       </c>
-      <c r="E144" s="72" t="s">
+      <c r="E170" s="72" t="s">
         <v>2661</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A145" s="18" t="s">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A171" s="18" t="s">
         <v>2662</v>
       </c>
-      <c r="B145" s="72" t="s">
+      <c r="B171" s="72" t="s">
         <v>2663</v>
       </c>
-      <c r="C145" s="20" t="s">
+      <c r="C171" s="20" t="s">
         <v>518</v>
       </c>
-      <c r="D145" s="132">
+      <c r="D171" s="132">
         <v>10</v>
       </c>
-      <c r="E145" s="72" t="s">
+      <c r="E171" s="72" t="s">
         <v>2664</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A146" s="18" t="s">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A172" s="18" t="s">
         <v>2665</v>
       </c>
-      <c r="B146" s="72" t="s">
+      <c r="B172" s="72" t="s">
         <v>291</v>
       </c>
-      <c r="C146" s="20" t="s">
+      <c r="C172" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D146" s="133">
+      <c r="D172" s="133">
         <f>Electrochemistry!$D$16</f>
         <v>2.0</v>
       </c>
-      <c r="E146" s="134" t="s">
+      <c r="E172" s="134" t="s">
         <v>2666</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A147" s="18" t="s">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A173" s="18" t="s">
         <v>2667</v>
       </c>
-      <c r="B147" s="72" t="s">
+      <c r="B173" s="72" t="s">
         <v>294</v>
       </c>
-      <c r="C147" s="20" t="s">
+      <c r="C173" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D147" s="133">
+      <c r="D173" s="133">
         <f>Electrochemistry!$D$17</f>
         <v>4.0</v>
       </c>
-      <c r="E147" s="134" t="s">
+      <c r="E173" s="134" t="s">
         <v>2668</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A148" s="18" t="s">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A174" s="18" t="s">
         <v>2288</v>
       </c>
-      <c r="B148" s="72" t="s">
+      <c r="B174" s="72" t="s">
         <v>2122</v>
       </c>
-      <c r="C148" s="20" t="s">
+      <c r="C174" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="D148" s="133">
+      <c r="D174" s="133">
         <f>Biology!$D$66</f>
         <v>273.15</v>
       </c>
-      <c r="E148" s="134" t="s">
+      <c r="E174" s="134" t="s">
         <v>2289</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A149" s="18" t="s">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A175" s="18" t="s">
         <v>2669</v>
       </c>
-      <c r="B149" s="72" t="s">
+      <c r="B175" s="72" t="s">
         <v>1698</v>
       </c>
-      <c r="C149" s="20" t="s">
+      <c r="C175" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D149" s="133">
+      <c r="D175" s="133">
         <f>'Mass Transfer'!$D$203</f>
         <v>610.94</v>
       </c>
-      <c r="E149" s="134" t="s">
+      <c r="E175" s="134" t="s">
         <v>2670</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A150" s="18" t="s">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A176" s="18" t="s">
         <v>2671</v>
       </c>
-      <c r="B150" s="72" t="s">
+      <c r="B176" s="72" t="s">
         <v>1701</v>
       </c>
-      <c r="C150" s="20" t="s">
+      <c r="C176" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D150" s="133">
+      <c r="D176" s="133">
         <f>'Mass Transfer'!$D$204</f>
         <v>17.625</v>
       </c>
-      <c r="E150" s="134" t="s">
+      <c r="E176" s="134" t="s">
         <v>2672</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A151" s="18" t="s">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A177" s="18" t="s">
         <v>2673</v>
       </c>
-      <c r="B151" s="72" t="s">
+      <c r="B177" s="72" t="s">
         <v>1703</v>
       </c>
-      <c r="C151" s="20" t="s">
+      <c r="C177" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="D151" s="133">
+      <c r="D177" s="133">
         <f>'Mass Transfer'!$D$205</f>
         <v>243.04</v>
       </c>
-      <c r="E151" s="134" t="s">
+      <c r="E177" s="134" t="s">
         <v>2674</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A155" s="18" t="s">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A181" s="18" t="s">
         <v>2675</v>
       </c>
-      <c r="B155" s="72" t="s">
+      <c r="B181" s="72" t="s">
         <v>2676</v>
       </c>
-      <c r="C155" s="20" t="s">
+      <c r="C181" s="20" t="s">
         <v>508</v>
       </c>
-      <c r="D155" s="133">
+      <c r="D181" s="133">
         <f>'Mass Transfer'!$D$169</f>
         <v>1003.33</v>
       </c>
-      <c r="E155" s="134" t="s">
+      <c r="E181" s="134" t="s">
         <v>2677</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A156" s="18" t="s">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A182" s="18" t="s">
         <v>2678</v>
       </c>
-      <c r="B156" s="72" t="s">
+      <c r="B182" s="72" t="s">
         <v>2679</v>
       </c>
-      <c r="C156" s="20" t="s">
+      <c r="C182" s="20" t="s">
         <v>1595</v>
       </c>
-      <c r="D156" s="133">
+      <c r="D182" s="133">
         <f>'Mass Transfer'!$D$170</f>
         <v>-0.2556</v>
       </c>
-      <c r="E156" s="134" t="s">
+      <c r="E182" s="134" t="s">
         <v>2680</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A157" s="18" t="s">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A183" s="18" t="s">
         <v>2681</v>
       </c>
-      <c r="B157" s="72" t="s">
+      <c r="B183" s="72" t="s">
         <v>26</v>
       </c>
-      <c r="C157" s="20" t="s">
+      <c r="C183" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D157" s="133" t="str">
+      <c r="D183" s="133" t="str">
         <f>Summary!$D$2</f>
         <v>ed04</v>
       </c>
-      <c r="E157" s="134" t="s">
+      <c r="E183" s="134" t="s">
         <v>2682</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A158" s="18" t="s">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A184" s="18" t="s">
         <v>2683</v>
       </c>
-      <c r="B158" s="72" t="s">
+      <c r="B184" s="72" t="s">
         <v>33</v>
       </c>
-      <c r="C158" s="20" t="s">
+      <c r="C184" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D158" s="133" t="str">
+      <c r="D184" s="133" t="str">
         <f>Summary!$D$4</f>
         <v>Xanthobacter tagetidis</v>
       </c>
-      <c r="E158" s="134" t="s">
+      <c r="E184" s="134" t="s">
         <v>2684</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A159" s="18" t="s">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A185" s="18" t="s">
         <v>2685</v>
       </c>
-      <c r="B159" s="72" t="s">
+      <c r="B185" s="72" t="s">
         <v>212</v>
       </c>
-      <c r="C159" s="20" t="s">
+      <c r="C185" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="D159" s="133" t="str">
+      <c r="D185" s="133" t="str">
         <f>Geometry!$D$51</f>
         <v>MEP0.3</v>
       </c>
-      <c r="E159" s="134" t="s">
+      <c r="E185" s="134" t="s">
         <v>2686</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A160" s="18" t="s">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A186" s="18" t="s">
         <v>486</v>
       </c>
-      <c r="B160" s="72" t="s">
+      <c r="B186" s="72" t="s">
         <v>126</v>
       </c>
-      <c r="C160" s="20" t="s">
+      <c r="C186" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="D160" s="133">
+      <c r="D186" s="133">
         <f>Geometry!$D$21</f>
         <v>501.93100162698</v>
       </c>
-      <c r="E160" s="134" t="s">
+      <c r="E186" s="134" t="s">
         <v>2687</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A161" s="18" t="s">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A187" s="18" t="s">
         <v>2688</v>
       </c>
-      <c r="B161" s="72" t="s">
+      <c r="B187" s="72" t="s">
         <v>266</v>
       </c>
-      <c r="C161" s="20" t="s">
+      <c r="C187" s="20" t="s">
         <v>267</v>
       </c>
-      <c r="D161" s="133">
+      <c r="D187" s="133">
         <f>'Mass Transfer'!$D$101</f>
         <v>8.314462618</v>
       </c>
-      <c r="E161" s="134" t="s">
+      <c r="E187" s="134" t="s">
         <v>2689</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A162" s="18" t="s">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A188" s="18" t="s">
         <v>767</v>
       </c>
-      <c r="B162" s="72" t="s">
+      <c r="B188" s="72" t="s">
         <v>287</v>
       </c>
-      <c r="C162" s="20" t="s">
+      <c r="C188" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="D162" s="133">
+      <c r="D188" s="133">
         <f>Electrochemistry!$D$15</f>
         <v>96485.33212</v>
       </c>
-      <c r="E162" s="134" t="s">
+      <c r="E188" s="134" t="s">
         <v>2690</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A163" s="18"/>
-      <c r="B163" s="72"/>
-      <c r="C163" s="20"/>
-      <c r="D163" s="133"/>
-      <c r="E163" s="134"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="98" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/electrode-mass-transfer.md","ELECTRODE MASS TRANSFER  (ferricyanide limiting current)")</f>
-        <v>ELECTRODE MASS TRANSFER  (ferricyanide limiting current)</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value in use: average O₂-scaled k_m of the included runs for the active reactor and electrode, at the Summary stirrer rate and within the temperature tolerance (D193) of the Summary temperature; other runs are kept but not used. One k_m serves both electrodes in the model. Feeds Electrochemistry km_O2 (D83).</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Researcher</t>
-        </is>
-      </c>
-      <c r="B167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date</t>
-        </is>
-      </c>
-      <c r="C167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reactor</t>
-        </is>
-      </c>
-      <c r="D167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Electrode (Summary D3 list)</t>
-        </is>
-      </c>
-      <c r="E167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stir rate (rpm)</t>
-        </is>
-      </c>
-      <c r="F167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Temp (°C)</t>
-        </is>
-      </c>
-      <c r="G167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Limiting current (mA)</t>
-        </is>
-      </c>
-      <c r="H167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Electrode area (cm²)</t>
-        </is>
-      </c>
-      <c r="I167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ferricyanide (mM)</t>
-        </is>
-      </c>
-      <c r="J167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">D ferricyanide (m²/s)</t>
-        </is>
-      </c>
-      <c r="K167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">k_m ferricyanide (computed, cm/s)</t>
-        </is>
-      </c>
-      <c r="L167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">k_m O₂ (computed, cm/s)</t>
-        </is>
-      </c>
-      <c r="M167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Type (auto)</t>
-        </is>
-      </c>
-      <c r="N167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Include?</t>
-        </is>
-      </c>
-      <c r="O167" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="93"/>
-      <c r="B168" s="94"/>
-      <c r="C168" s="93"/>
-      <c r="D168" s="93"/>
-      <c r="E168" s="94"/>
-      <c r="F168" s="94"/>
-      <c r="G168" s="94"/>
-      <c r="H168" s="94"/>
-      <c r="I168" s="94"/>
-      <c r="J168" s="94"/>
-      <c r="K168" s="100" t="str">
-        <f>IF(OR(G168="",H168="",I168=""),"",IFERROR((G168/1000)/(n_e_fcn*F_const*(H168/10000)*I168)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L168" s="100" t="str">
-        <f>IF(OR(K168="",J168=""),"",IFERROR(K168*(D_O2/J168)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M168" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C168,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N168" s="93"/>
-      <c r="O168" s="93"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="93"/>
-      <c r="B169" s="94"/>
-      <c r="C169" s="93"/>
-      <c r="D169" s="93"/>
-      <c r="E169" s="94"/>
-      <c r="F169" s="94"/>
-      <c r="G169" s="94"/>
-      <c r="H169" s="94"/>
-      <c r="I169" s="94"/>
-      <c r="J169" s="94"/>
-      <c r="K169" s="100" t="str">
-        <f>IF(OR(G169="",H169="",I169=""),"",IFERROR((G169/1000)/(n_e_fcn*F_const*(H169/10000)*I169)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L169" s="100" t="str">
-        <f>IF(OR(K169="",J169=""),"",IFERROR(K169*(D_O2/J169)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M169" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C169,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N169" s="93"/>
-      <c r="O169" s="93"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="93"/>
-      <c r="B170" s="94"/>
-      <c r="C170" s="93"/>
-      <c r="D170" s="93"/>
-      <c r="E170" s="94"/>
-      <c r="F170" s="94"/>
-      <c r="G170" s="94"/>
-      <c r="H170" s="94"/>
-      <c r="I170" s="94"/>
-      <c r="J170" s="94"/>
-      <c r="K170" s="100" t="str">
-        <f>IF(OR(G170="",H170="",I170=""),"",IFERROR((G170/1000)/(n_e_fcn*F_const*(H170/10000)*I170)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L170" s="100" t="str">
-        <f>IF(OR(K170="",J170=""),"",IFERROR(K170*(D_O2/J170)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M170" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C170,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N170" s="93"/>
-      <c r="O170" s="93"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="93"/>
-      <c r="B171" s="94"/>
-      <c r="C171" s="93"/>
-      <c r="D171" s="93"/>
-      <c r="E171" s="94"/>
-      <c r="F171" s="94"/>
-      <c r="G171" s="94"/>
-      <c r="H171" s="94"/>
-      <c r="I171" s="94"/>
-      <c r="J171" s="94"/>
-      <c r="K171" s="100" t="str">
-        <f>IF(OR(G171="",H171="",I171=""),"",IFERROR((G171/1000)/(n_e_fcn*F_const*(H171/10000)*I171)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L171" s="100" t="str">
-        <f>IF(OR(K171="",J171=""),"",IFERROR(K171*(D_O2/J171)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M171" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C171,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N171" s="93"/>
-      <c r="O171" s="93"/>
-    </row>
-    <row r="172">
-      <c r="A172" s="93"/>
-      <c r="B172" s="94"/>
-      <c r="C172" s="93"/>
-      <c r="D172" s="93"/>
-      <c r="E172" s="94"/>
-      <c r="F172" s="94"/>
-      <c r="G172" s="94"/>
-      <c r="H172" s="94"/>
-      <c r="I172" s="94"/>
-      <c r="J172" s="94"/>
-      <c r="K172" s="100" t="str">
-        <f>IF(OR(G172="",H172="",I172=""),"",IFERROR((G172/1000)/(n_e_fcn*F_const*(H172/10000)*I172)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L172" s="100" t="str">
-        <f>IF(OR(K172="",J172=""),"",IFERROR(K172*(D_O2/J172)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M172" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C172,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N172" s="93"/>
-      <c r="O172" s="93"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="93"/>
-      <c r="B173" s="94"/>
-      <c r="C173" s="93"/>
-      <c r="D173" s="93"/>
-      <c r="E173" s="94"/>
-      <c r="F173" s="94"/>
-      <c r="G173" s="94"/>
-      <c r="H173" s="94"/>
-      <c r="I173" s="94"/>
-      <c r="J173" s="94"/>
-      <c r="K173" s="100" t="str">
-        <f>IF(OR(G173="",H173="",I173=""),"",IFERROR((G173/1000)/(n_e_fcn*F_const*(H173/10000)*I173)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L173" s="100" t="str">
-        <f>IF(OR(K173="",J173=""),"",IFERROR(K173*(D_O2/J173)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M173" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C173,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N173" s="93"/>
-      <c r="O173" s="93"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="93"/>
-      <c r="B174" s="94"/>
-      <c r="C174" s="93"/>
-      <c r="D174" s="93"/>
-      <c r="E174" s="94"/>
-      <c r="F174" s="94"/>
-      <c r="G174" s="94"/>
-      <c r="H174" s="94"/>
-      <c r="I174" s="94"/>
-      <c r="J174" s="94"/>
-      <c r="K174" s="100" t="str">
-        <f>IF(OR(G174="",H174="",I174=""),"",IFERROR((G174/1000)/(n_e_fcn*F_const*(H174/10000)*I174)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L174" s="100" t="str">
-        <f>IF(OR(K174="",J174=""),"",IFERROR(K174*(D_O2/J174)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M174" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C174,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N174" s="93"/>
-      <c r="O174" s="93"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="93"/>
-      <c r="B175" s="94"/>
-      <c r="C175" s="93"/>
-      <c r="D175" s="93"/>
-      <c r="E175" s="94"/>
-      <c r="F175" s="94"/>
-      <c r="G175" s="94"/>
-      <c r="H175" s="94"/>
-      <c r="I175" s="94"/>
-      <c r="J175" s="94"/>
-      <c r="K175" s="100" t="str">
-        <f>IF(OR(G175="",H175="",I175=""),"",IFERROR((G175/1000)/(n_e_fcn*F_const*(H175/10000)*I175)*100,""))</f>
-        <v/>
-      </c>
-      <c r="L175" s="100" t="str">
-        <f>IF(OR(K175="",J175=""),"",IFERROR(K175*(D_O2/J175)^km_exp,""))</f>
-        <v/>
-      </c>
-      <c r="M175" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C175,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="N175" s="93"/>
-      <c r="O175" s="93"/>
-    </row>
-    <row r="176">
-      <c r="A176" s="96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value in use - k_m O₂</t>
-        </is>
-      </c>
-      <c r="C176" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cm/s</t>
-        </is>
-      </c>
-      <c r="D176" s="95" t="str">
-        <f>IFERROR(AVERAGEIFS(L168:L175,C168:C175,Reactor_sel,D168:D175,electrode_sel,N168:N175,"y",E168:E175,stir_rpm_set,F168:F175,"&gt;="&amp;(temp_C-km_T_tol),F168:F175,"&lt;="&amp;(temp_C+km_T_tol)),"no included runs — model uses its default")</f>
-        <v>no included runs — model uses its default</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="98" t="str">
-        <f>HYPERLINK("https://github.com/amy-bo/electroPioreactor/blob/AEP02/Media/protocols/chlorine-species.md","MONOCHLORAMINE LIFETIME  (DPD combined chlorine at plateau)")</f>
-        <v>MONOCHLORAMINE LIFETIME  (DPD combined chlorine at plateau)</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value in use: average of the included runs for the active reactor and medium. Inverts the model’s own steady state B = min(C·kτ/(1+kτ), P·τ): τ = max(B/(k(C−B)), B/P), with k, C and P read from Chemistry D271, D47 and D315 at the run settings (none depends on τ). Feeds Chemistry tau_NH2Cl (D142).</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Researcher</t>
-        </is>
-      </c>
-      <c r="B180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Date</t>
-        </is>
-      </c>
-      <c r="C180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reactor</t>
-        </is>
-      </c>
-      <c r="D180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Medium</t>
-        </is>
-      </c>
-      <c r="E180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Combined chlorine plateau (mg/L as Cl₂)</t>
-        </is>
-      </c>
-      <c r="F180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chloride turnover k (1/s, Chemistry D271)</t>
-        </is>
-      </c>
-      <c r="G180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Chloride pool C (mol/L, Chemistry D47)</t>
-        </is>
-      </c>
-      <c r="H180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Max production P (mol/L/s, Chemistry D315)</t>
-        </is>
-      </c>
-      <c r="I180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lifetime (computed, h)</t>
-        </is>
-      </c>
-      <c r="J180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Type (auto)</t>
-        </is>
-      </c>
-      <c r="K180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Include?</t>
-        </is>
-      </c>
-      <c r="L180" s="99" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="93"/>
-      <c r="B181" s="94"/>
-      <c r="C181" s="93"/>
-      <c r="D181" s="93"/>
-      <c r="E181" s="94"/>
-      <c r="F181" s="94"/>
-      <c r="G181" s="94"/>
-      <c r="H181" s="94"/>
-      <c r="I181" s="100" t="str">
-        <f>IF(OR(E181="",F181="",G181="",H181=""),"",IF(E181/M_Cl2&gt;=G181,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E181/M_Cl2/(F181*(G181-E181/M_Cl2)),E181/M_Cl2/H181)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J181" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C181,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K181" s="93"/>
-      <c r="L181" s="93"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="93"/>
-      <c r="B182" s="94"/>
-      <c r="C182" s="93"/>
-      <c r="D182" s="93"/>
-      <c r="E182" s="94"/>
-      <c r="F182" s="94"/>
-      <c r="G182" s="94"/>
-      <c r="H182" s="94"/>
-      <c r="I182" s="100" t="str">
-        <f>IF(OR(E182="",F182="",G182="",H182=""),"",IF(E182/M_Cl2&gt;=G182,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E182/M_Cl2/(F182*(G182-E182/M_Cl2)),E182/M_Cl2/H182)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J182" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C182,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K182" s="93"/>
-      <c r="L182" s="93"/>
-    </row>
-    <row r="183">
-      <c r="A183" s="93"/>
-      <c r="B183" s="94"/>
-      <c r="C183" s="93"/>
-      <c r="D183" s="93"/>
-      <c r="E183" s="94"/>
-      <c r="F183" s="94"/>
-      <c r="G183" s="94"/>
-      <c r="H183" s="94"/>
-      <c r="I183" s="100" t="str">
-        <f>IF(OR(E183="",F183="",G183="",H183=""),"",IF(E183/M_Cl2&gt;=G183,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E183/M_Cl2/(F183*(G183-E183/M_Cl2)),E183/M_Cl2/H183)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J183" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C183,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K183" s="93"/>
-      <c r="L183" s="93"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="93"/>
-      <c r="B184" s="94"/>
-      <c r="C184" s="93"/>
-      <c r="D184" s="93"/>
-      <c r="E184" s="94"/>
-      <c r="F184" s="94"/>
-      <c r="G184" s="94"/>
-      <c r="H184" s="94"/>
-      <c r="I184" s="100" t="str">
-        <f>IF(OR(E184="",F184="",G184="",H184=""),"",IF(E184/M_Cl2&gt;=G184,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E184/M_Cl2/(F184*(G184-E184/M_Cl2)),E184/M_Cl2/H184)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J184" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C184,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K184" s="93"/>
-      <c r="L184" s="93"/>
-    </row>
-    <row r="185">
-      <c r="A185" s="93"/>
-      <c r="B185" s="94"/>
-      <c r="C185" s="93"/>
-      <c r="D185" s="93"/>
-      <c r="E185" s="94"/>
-      <c r="F185" s="94"/>
-      <c r="G185" s="94"/>
-      <c r="H185" s="94"/>
-      <c r="I185" s="100" t="str">
-        <f>IF(OR(E185="",F185="",G185="",H185=""),"",IF(E185/M_Cl2&gt;=G185,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E185/M_Cl2/(F185*(G185-E185/M_Cl2)),E185/M_Cl2/H185)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J185" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C185,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K185" s="93"/>
-      <c r="L185" s="93"/>
-    </row>
-    <row r="186">
-      <c r="A186" s="93"/>
-      <c r="B186" s="94"/>
-      <c r="C186" s="93"/>
-      <c r="D186" s="93"/>
-      <c r="E186" s="94"/>
-      <c r="F186" s="94"/>
-      <c r="G186" s="94"/>
-      <c r="H186" s="94"/>
-      <c r="I186" s="100" t="str">
-        <f>IF(OR(E186="",F186="",G186="",H186=""),"",IF(E186/M_Cl2&gt;=G186,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E186/M_Cl2/(F186*(G186-E186/M_Cl2)),E186/M_Cl2/H186)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J186" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C186,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K186" s="93"/>
-      <c r="L186" s="93"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="93"/>
-      <c r="B187" s="94"/>
-      <c r="C187" s="93"/>
-      <c r="D187" s="93"/>
-      <c r="E187" s="94"/>
-      <c r="F187" s="94"/>
-      <c r="G187" s="94"/>
-      <c r="H187" s="94"/>
-      <c r="I187" s="100" t="str">
-        <f>IF(OR(E187="",F187="",G187="",H187=""),"",IF(E187/M_Cl2&gt;=G187,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E187/M_Cl2/(F187*(G187-E187/M_Cl2)),E187/M_Cl2/H187)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J187" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C187,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K187" s="93"/>
-      <c r="L187" s="93"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="93"/>
-      <c r="B188" s="94"/>
-      <c r="C188" s="93"/>
-      <c r="D188" s="93"/>
-      <c r="E188" s="94"/>
-      <c r="F188" s="94"/>
-      <c r="G188" s="94"/>
-      <c r="H188" s="94"/>
-      <c r="I188" s="100" t="str">
-        <f>IF(OR(E188="",F188="",G188="",H188=""),"",IF(E188/M_Cl2&gt;=G188,"not invertible: plateau at or above the chloride pool",IFERROR(MAX(E188/M_Cl2/(F188*(G188-E188/M_Cl2)),E188/M_Cl2/H188)/3600,"")))</f>
-        <v/>
-      </c>
-      <c r="J188" s="100" t="str">
-        <f>IFERROR(INDEX(ReactorTypeList,MATCH(C188,ReactorList,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K188" s="93"/>
-      <c r="L188" s="93"/>
-    </row>
     <row r="189">
-      <c r="A189" s="96" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value in use - monochloramine lifetime</t>
-        </is>
-      </c>
-      <c r="C189" s="97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">h</t>
-        </is>
-      </c>
-      <c r="D189" s="95" t="str">
-        <f>IFERROR(AVERAGEIFS(I181:I188,C181:C188,Reactor_sel,D181:D188,media_sel,K181:K188,"y"),"no included runs — model uses its default")</f>
-        <v>no included runs — model uses its default</v>
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NAMED CONSTANTS AND IMPORTS (electrode mass transfer, monochloramine lifetime)</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Electrons per ferricyanide reduced</t>
+        </is>
+      </c>
+      <c r="B190" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">n_e_fcn</t>
+        </is>
+      </c>
+      <c r="C190" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D190" s="132">
+        <v>1</v>
+      </c>
+      <c r="E190" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fe(CN)₆³⁻ + e⁻ → Fe(CN)₆⁴⁻: a one-electron couple (protocols/electrode-mass-transfer.md).</t>
+        </is>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NAMED CONSTANTS AND IMPORTS (electrode mass transfer, monochloramine lifetime)</t>
+      <c r="A191" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Temperature tolerance for a k_m run</t>
+        </is>
+      </c>
+      <c r="B191" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km_T_tol</t>
+        </is>
+      </c>
+      <c r="C191" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">°C</t>
+        </is>
+      </c>
+      <c r="D191" s="132">
+        <v>1</v>
+      </c>
+      <c r="E191" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Design assumption: diffusivity and viscosity move ~2 %/K, so a run within ±1 °C of the Summary temperature is used as measured; others need a separate temperature correction.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Electrons per ferricyanide reduced</t>
+          <t xml:space="preserve">(import) Stirrer rate on Summary</t>
         </is>
       </c>
       <c r="B192" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">n_e_fcn</t>
+          <t xml:space="preserve">stir_rpm_set</t>
         </is>
       </c>
       <c r="C192" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D192" s="132">
-        <v>1</v>
+          <t xml:space="preserve">rpm</t>
+        </is>
+      </c>
+      <c r="D192" s="133">
+        <f>Summary!$D$7</f>
+        <v>1000.0</v>
       </c>
       <c r="E192" s="134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fe(CN)₆³⁻ + e⁻ → Fe(CN)₆⁴⁻: a one-electron couple (protocols/electrode-mass-transfer.md).</t>
+          <t xml:space="preserve">Import from Summary!D7 (stir_rpm_set)</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Temperature tolerance for a k_m run</t>
+          <t xml:space="preserve">(import) Temperature setpoint on Summary</t>
         </is>
       </c>
       <c r="B193" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">km_T_tol</t>
+          <t xml:space="preserve">temp_C</t>
         </is>
       </c>
       <c r="C193" s="20" t="inlineStr">
@@ -41777,102 +41828,103 @@
           <t xml:space="preserve">°C</t>
         </is>
       </c>
-      <c r="D193" s="132">
-        <v>1</v>
-      </c>
-      <c r="E193" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Design assumption: diffusivity and viscosity move ~2 %/K, so a run within ±1 °C of the Summary temperature is used as measured; others need a separate temperature correction.</t>
+      <c r="D193" s="133">
+        <f>Summary!$D$8</f>
+        <v>30.0</v>
+      </c>
+      <c r="E193" s="134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Summary!D8 (temp_C)</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">(import) Stirrer rate on Summary</t>
+          <t xml:space="preserve">(import) Medium selected on Summary</t>
         </is>
       </c>
       <c r="B194" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">stir_rpm_set</t>
+          <t xml:space="preserve">media_sel</t>
         </is>
       </c>
       <c r="C194" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">rpm</t>
-        </is>
-      </c>
-      <c r="D194" s="133">
-        <f>Summary!$D$7</f>
-        <v>1000.0</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D194" s="133" t="str">
+        <f>Summary!$D$5</f>
+        <v>AMYBO03</v>
       </c>
       <c r="E194" s="134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import from Summary!D7 (stir_rpm_set)</t>
+          <t xml:space="preserve">Import from Summary!D5 (media_sel)</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">(import) Temperature setpoint on Summary</t>
+          <t xml:space="preserve">(import) Electrode selected on Summary</t>
         </is>
       </c>
       <c r="B195" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">temp_C</t>
+          <t xml:space="preserve">electrode_sel</t>
         </is>
       </c>
       <c r="C195" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">°C</t>
-        </is>
-      </c>
-      <c r="D195" s="133">
-        <f>Summary!$D$8</f>
-        <v>30.0</v>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D195" s="133" t="str">
+        <f>Summary!$D$3</f>
+        <v>MMO tube</v>
       </c>
       <c r="E195" s="134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import from Summary!D8 (temp_C)</t>
+          <t xml:space="preserve">Import from Summary!D3 (electrode_sel)</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">(import) Medium selected on Summary</t>
+          <t xml:space="preserve">(import) O₂ diffusivity at reactor T</t>
         </is>
       </c>
       <c r="B196" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">media_sel</t>
+          <t xml:space="preserve">D_O2</t>
         </is>
       </c>
       <c r="C196" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D196" s="133" t="str">
-        <f>Summary!$D$5</f>
-        <v>AMYBO03</v>
+          <t xml:space="preserve">m²/s</t>
+        </is>
+      </c>
+      <c r="D196" s="133">
+        <f>'Mass Transfer'!$D$32</f>
+        <v>2.249544435762e-09</v>
       </c>
       <c r="E196" s="134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import from Summary!D5 (media_sel)</t>
+          <t xml:space="preserve">Import from Mass Transfer!D32 (D_O2)</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">(import) Electrode selected on Summary</t>
+          <t xml:space="preserve">(import) Diffusivity exponent for k_m scaling</t>
         </is>
       </c>
       <c r="B197" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">electrode_sel</t>
+          <t xml:space="preserve">km_exp</t>
         </is>
       </c>
       <c r="C197" s="20" t="inlineStr">
@@ -41880,89 +41932,37 @@
           <t xml:space="preserve">-</t>
         </is>
       </c>
-      <c r="D197" s="133" t="str">
-        <f>Summary!$D$3</f>
-        <v>MMO tube</v>
+      <c r="D197" s="133">
+        <f>Electrochemistry!$D$84</f>
+        <v>0.644</v>
       </c>
       <c r="E197" s="134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Import from Summary!D3 (electrode_sel)</t>
+          <t xml:space="preserve">Import from Electrochemistry!D84 (km_exp): the same Eisenberg scaling the model uses for every species.</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">(import) O₂ diffusivity at reactor T</t>
+          <t xml:space="preserve">(import) Cl₂ molar mass</t>
         </is>
       </c>
       <c r="B198" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">D_O2</t>
+          <t xml:space="preserve">M_Cl2</t>
         </is>
       </c>
       <c r="C198" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">m²/s</t>
+          <t xml:space="preserve">mg/mol</t>
         </is>
       </c>
       <c r="D198" s="133">
-        <f>'Mass Transfer'!$D$32</f>
-        <v>2.249544435762e-09</v>
-      </c>
-      <c r="E198" s="134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Import from Mass Transfer!D32 (D_O2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(import) Diffusivity exponent for k_m scaling</t>
-        </is>
-      </c>
-      <c r="B199" s="72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km_exp</t>
-        </is>
-      </c>
-      <c r="C199" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D199" s="133">
-        <f>Electrochemistry!$D$84</f>
-        <v>0.644</v>
-      </c>
-      <c r="E199" s="134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Import from Electrochemistry!D84 (km_exp): the same Eisenberg scaling the model uses for every species.</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(import) Cl₂ molar mass</t>
-        </is>
-      </c>
-      <c r="B200" s="72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">M_Cl2</t>
-        </is>
-      </c>
-      <c r="C200" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mg/mol</t>
-        </is>
-      </c>
-      <c r="D200" s="133">
         <f>Chemistry!$D$223</f>
         <v>70906.0</v>
       </c>
-      <c r="E200" s="134" t="inlineStr">
+      <c r="E198" s="134" t="inlineStr">
         <is>
           <t xml:space="preserve">Import from Chemistry!D223 (M_Cl2): DPD results are mg/L as Cl₂.</t>
         </is>
@@ -41970,28 +41970,28 @@
     </row>
   </sheetData>
   <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C8:C15 C81:C88 C66:C73 C52:C59 C38:C45 C23:C30" xr:uid="{00000000-0002-0000-0700-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C8:C15 C23:C30 C38:C45 C52:C59 C66:C73 C81:C88" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>ReactorList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G8:G15 F128:F135 G112:G119 H95:H102 G81:G88 J66:J73 H52:H59 F38:F45 K23:K30" xr:uid="{00000000-0002-0000-0700-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F38:F45 F128:F135 G8:G15 G81:G88 G112:G119 H52:H59 H95:H102 J66:J73 K23:K30" xr:uid="{00000000-0002-0000-0700-000001000000}">
       <formula1>"y,n"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H23:H30" xr:uid="{00000000-0002-0000-0700-000004000000}">
       <formula1>"H2,O2"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C95:C102 C128:C135 C112:C119" xr:uid="{00000000-0002-0000-0700-00000D000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C95:C102 C112:C119 C128:C135" xr:uid="{00000000-0002-0000-0700-00000D000000}">
       <formula1>OrganismList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose a reactor from the list." sqref="C168:C175 C181:C188">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose a reactor from the list." sqref="C142:C149 C155:C162">
       <formula1>ReactorList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="y or n." sqref="N168:N175 K181:K188">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="y or n." sqref="K155:K162 N142:N149">
       <formula1>"y,n"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose an electrode from the list." sqref="D168:D175">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose an electrode from the list." sqref="D142:D149">
       <formula1>ElectrodeList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose a medium from the list." sqref="D181:D188">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid value" error="Choose a medium from the list." sqref="D155:D162">
       <formula1>MediaList</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Gas model: fourth Codex review fixes (peroxide on the lag plateau, N2 entry, physical depth, voltage check band)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -1066,6 +1066,7 @@
     <definedName name="por_p0_hi" localSheetId="7">Calibrations!$D$200</definedName>
     <definedName name="por_p5_hi" localSheetId="7">Calibrations!$D$201</definedName>
     <definedName name="por_p5_lo" localSheetId="7">Calibrations!$D$202</definedName>
+    <definedName name="gerrit_check_pct" localSheetId="2">Electrochemistry!$D$166</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -10333,7 +10334,7 @@
     <xf numFmtId="0" fontId="26" fillId="17" borderId="11"/>
     <xf numFmtId="44" fontId="49" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="180">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="45" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -10568,6 +10569,21 @@
     <xf numFmtId="0" fontId="56" fillId="0" borderId="1" xfId="0" applyBorder="1" applyFont="1"/>
     <xf numFmtId="0" fontId="57" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="56" fillId="19" borderId="11" xfId="0" applyFill="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -11913,7 +11929,7 @@
           <t xml:space="preserve">res_su_state</t>
         </is>
       </c>
-      <c r="D33" s="170" t="str">
+      <c r="D33" s="175" t="str">
         <f>IF(ISNUMBER('Mass Transfer'!spg_int_su_run),"DO "&amp;TEXT('Mass Transfer'!DO_avg_su_mgL,"0.0")&amp;" mg/L mean, "&amp;TEXT('Mass Transfer'!DO_peak_su_mgL,"0.0")&amp;" peak; H₂ "&amp;TEXT('Mass Transfer'!y_H2_end_su,"0%")&amp;" before each pulse; set by "&amp;'Mass Transfer'!su_binding,"no executable start-up schedule")</f>
         <v>DO 4.1 mg/L mean, 4.1 peak; H₂ 3% before each pulse; set by the legacy O₂ flush guard (lag DO target unreachable)</v>
       </c>
@@ -11951,7 +11967,7 @@
         <v>1717</v>
       </c>
       <c r="C35" s="21"/>
-      <c r="D35" s="171" t="str">
+      <c r="D35" s="176" t="str">
         <f>Geometry!geom_check</f>
         <v>VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth</v>
       </c>
@@ -11991,7 +12007,7 @@
         <v>1722</v>
       </c>
       <c r="C37" s="21"/>
-      <c r="D37" s="170" t="str">
+      <c r="D37" s="175" t="str">
         <f>'Mass Transfer'!DO_peak_band</f>
         <v>organism band unknown – peak 2.5 mg/L is under the inhibition ceiling</v>
       </c>
@@ -12031,7 +12047,7 @@
         <v>1726</v>
       </c>
       <c r="C39" s="21"/>
-      <c r="D39" s="170" t="str">
+      <c r="D39" s="175" t="str">
         <f>'Mass Transfer'!sched_regime</f>
         <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈13 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
       </c>
@@ -12051,7 +12067,7 @@
         <v>1729</v>
       </c>
       <c r="C40" s="21"/>
-      <c r="D40" s="172" t="str">
+      <c r="D40" s="177" t="str">
         <f>Biology!H2_safety</f>
         <v>POTENTIAL FLAMMABILITY (lag screen): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
@@ -12093,7 +12109,7 @@
         <v>1732</v>
       </c>
       <c r="C42" s="21"/>
-      <c r="D42" s="170" t="str">
+      <c r="D42" s="175" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!CO2_sd_ratio,"0.0")&amp;IF('Mass Transfer'!CO2_sd_ratio&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)")&amp;" delivered; ×"&amp;TEXT('Mass Transfer'!CO2_uptake_ratio,"0.0")&amp;" absorbed per pulse (row 77)","calibrate this reactor first")</f>
         <v>×49.7 OK delivered; ×2.5 absorbed per pulse (row 77)</v>
       </c>
@@ -12155,7 +12171,7 @@
         <v>1737</v>
       </c>
       <c r="C45" s="21"/>
-      <c r="D45" s="170" t="str">
+      <c r="D45" s="175" t="str">
         <f>'Mass Transfer'!carry_flag</f>
         <v>not measured – record the max flow without carryover for ed04 in CO2 flows column M</v>
       </c>
@@ -12257,7 +12273,7 @@
         <v>1743</v>
       </c>
       <c r="C50" s="21"/>
-      <c r="D50" s="171" t="str">
+      <c r="D50" s="176" t="str">
         <f>IF(AND(ISNUMBER(Biology!DO_min),ISNUMBER(Biology!DO_opt),ISNUMBER(Biology!DO_impair),ISNUMBER(Biology!DO_toxic)),"inputs present","DATA GAP - organism DO thresholds unmeasured; results unreliable")</f>
         <v>DATA GAP - organism DO thresholds unmeasured; results unreliable</v>
       </c>
@@ -12276,7 +12292,7 @@
       <c r="B51" s="19" t="s">
         <v>1837</v>
       </c>
-      <c r="D51" s="170" t="str">
+      <c r="D51" s="175" t="str">
         <f>'Mass Transfer'!carry_flag_usg</f>
         <v>OK – 6.6 mm/s against the 50 mm/s rule of thumb</v>
       </c>
@@ -12294,7 +12310,7 @@
       <c r="A52" s="64" t="s">
         <v>1827</v>
       </c>
-      <c r="D52" s="173" t="str">
+      <c r="D52" s="178" t="str">
         <f>IF(ISNA('Mass Transfer'!F_vent_ex+'Mass Transfer'!O2_src_sched),"#N/A – check the selectors in D2–D5, D11 and D12",IF(NOT(ISNUMBER('Mass Transfer'!spg_int_DO)),"DO target unreachable on the sizing phase; schedule is a legacy fallback",IF(OR(Chemistry!DIC_ref_check&lt;&gt;"OK",ABS(Electrochemistry!DO_lag_ref/Electrochemistry!ec_DO_lag-1)&gt;Electrochemistry!DO_lag_tol),"watch – refresh the DIC or lag-DO reference before claiming either target",IF(AND(res_pH&gt;=cf_pH_lo,res_pH&lt;=cf_pH_hi,res_DO_ss&lt;='Mass Transfer'!DO_target*'Mass Transfer'!M_O2),"yes – both targets met by the evaluated schedule","NO – evaluated schedule misses the pH band or mean DO target"))))</f>
         <v>NO – evaluated schedule misses the pH band or mean DO target</v>
       </c>
@@ -12331,7 +12347,7 @@
       <c r="A54" s="64" t="s">
         <v>1831</v>
       </c>
-      <c r="D54" s="170" t="str">
+      <c r="D54" s="175" t="str">
         <f>'Mass Transfer'!hs_sag_chk</f>
         <v>UNVERIFIED pressure closure: air ingress is assumed; measure vent make-up flow</v>
       </c>
@@ -12526,7 +12542,7 @@
       <c r="A66" s="64" t="s">
         <v>1815</v>
       </c>
-      <c r="D66" s="170" t="str">
+      <c r="D66" s="175" t="str">
         <f>'Mass Transfer'!DO_feas_l</f>
         <v>UNREACHABLE at this surface kLa – margin 0.61× (raise kL_surf, lower the current, or accept a higher DO)</v>
       </c>
@@ -13068,9 +13084,9 @@
       <c r="C98" s="20" t="s">
         <v>1140</v>
       </c>
-      <c r="D98" s="174" t="str">
+      <c r="D98" s="179" t="str">
         <f>Electrochemistry!H2O2_flag</f>
-        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min (0.84 mg/L after 1 h) before biomass can scavenge it</v>
       </c>
       <c r="E98" s="24" t="str">
         <f>HYPERLINK("#Electrochemistry!D99","→ Electrochemistry")</f>
@@ -13090,7 +13106,7 @@
       <c r="C99" s="20" t="s">
         <v>1140</v>
       </c>
-      <c r="D99" s="174" t="str">
+      <c r="D99" s="179" t="str">
         <f>Chemistry!buffer_flag</f>
         <v>OK — buffer holds the electrode surfaces at the bulk pH</v>
       </c>
@@ -13345,7 +13361,7 @@
       </c>
       <c r="E112" s="77"/>
       <c r="F112" s="154" t="str">
-        <f>"Sets the solenoid floor (pulse_floor, now "&amp;TEXT('Mass Transfer'!pulse_floor,"0.00")&amp;" s), which binds only when it exceeds the optimal pulse ("&amp;IF(ISNUMBER(D18),TEXT(D18,"0.00")&amp;" s","not yet computed")&amp;"): "&amp;IF(AND(ISNUMBER(D18),'Mass Transfer'!pulse_floor&gt;=D18),"it does now, so the pulse IS the floor","it does not now, so it matters only for a smaller headspace or a faster flow")&amp;". Trivial to characterise on the bench (flow-calibration.md)."</f>
+        <f>"Sets the solenoid floor (pulse_floor, now "&amp;TEXT('Mass Transfer'!pulse_floor,"0.00")&amp;" s), which binds only when it exceeds the optimal pulse ("&amp;IF(ISNUMBER(res_spg_dur),TEXT(res_spg_dur,"0.00")&amp;" s","not yet computed")&amp;"): "&amp;IF(AND(ISNUMBER(res_spg_dur),'Mass Transfer'!pulse_floor&gt;=res_spg_dur),"it does now, so the pulse IS the floor","it does not now, so it matters only for a smaller headspace or a faster flow")&amp;". Trivial to characterise on the bench (flow-calibration.md)."</f>
         <v>Sets the solenoid floor (pulse_floor, now 0.25 s), which binds only when it exceeds the optimal pulse (0.67 s): it does not now, so it matters only for a smaller headspace or a faster flow. Trivial to characterise on the bench (flow-calibration.md).</v>
       </c>
     </row>
@@ -13822,7 +13838,7 @@
       </c>
       <c r="F135" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Row 14 enters N₂ by its mean flow, exact for the mean-field fractions. Pulsing N₂ midway between CO₂ pulses adds a second flush per cycle, which would lower the pre-pulse O₂ and H₂ peaks a little further.</t>
+          <t xml:space="preserve">Row 14 enters N₂ by its mean flow. That is exact for the mean-field fractions but not for the sawtooth: a separate N₂ flush lets H₂ and O₂ build for longer between flushes, so the pre-pulse peaks can be substantially higher than the continuous surrogate shows. Model the flush before relying on pulsed N₂.</t>
         </is>
       </c>
     </row>
@@ -14706,11 +14722,13 @@
         <v>115</v>
       </c>
       <c r="D22" s="110">
-        <f>IF(ISNUMBER(cal_Dint),cal_Dint,VLOOKUP(rx_ver,tbl_rxtype,MATCH("usable depth (mm)",tbl_rxtype_hdr,0),FALSE))</f>
+        <f>VLOOKUP(rx_ver,tbl_rxtype,MATCH("usable depth (mm)",tbl_rxtype_hdr,0),FALSE)</f>
         <v>55.0</v>
       </c>
-      <c r="E22" s="74" t="s">
-        <v>131</v>
+      <c r="E22" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Physical cap-to-base depth from the reactor-type table, selected by rx_ver. The Calibrations volume-equivalent depth (D75) is not a physical length and does not replace it.</t>
+        </is>
       </c>
       <c r="F22" s="21"/>
       <c r="G22" s="21"/>
@@ -15393,7 +15411,11 @@
         <f>IF(V_charge&gt;V_max,"MEDIA &gt; MAX WORKING VOLUME","OK")</f>
         <v>OK</v>
       </c>
-      <c r="E54" s="21"/>
+      <c r="E54" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Charge against the reactor-type maximum working volume (Geometry D23).</t>
+        </is>
+      </c>
       <c r="F54" s="21"/>
       <c r="G54" s="21"/>
       <c r="H54" s="21"/>
@@ -15411,7 +15433,11 @@
         <f>IF(h_actual&gt;D_int,"LIQUID OVER USABLE DEPTH","OK")</f>
         <v>OK</v>
       </c>
-      <c r="E55" s="21"/>
+      <c r="E55" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Achieved liquid level against the usable depth (D22).</t>
+        </is>
+      </c>
       <c r="F55" s="21"/>
       <c r="G55" s="21"/>
       <c r="H55" s="21"/>
@@ -16084,7 +16110,7 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="A1:N165"/>
+  <dimension ref="A1:N166"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -16716,7 +16742,11 @@
         <f>VLOOKUP(electrode_sel,tbl_electrode,MATCH("sparger",tbl_electrode_hdr,0),FALSE)</f>
         <v>Sintered</v>
       </c>
-      <c r="E31" s="21"/>
+      <c r="E31" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sparger type of the selected electrode assembly, looked up in the electrode table (tbl_electrode).</t>
+        </is>
+      </c>
       <c r="F31" s="21"/>
       <c r="G31" s="21"/>
       <c r="H31" s="21"/>
@@ -17949,11 +17979,13 @@
         <v>1140</v>
       </c>
       <c r="D99" s="111" t="str">
-        <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(H2O2_lag_1h&gt;H2O2_thresh,"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases"))</f>
-        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min before biomass can scavenge it</v>
-      </c>
-      <c r="E99" s="51" t="s">
-        <v>1519</v>
+        <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(ISNUMBER(t_H2O2_thresh),"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min ("&amp;TEXT(H2O2_lag_1h,"0.00")&amp;" mg/L after 1 h) before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases, including the lag plateau"))</f>
+        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min (0.84 mg/L after 1 h) before biomass can scavenge it</v>
+      </c>
+      <c r="E99" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Steady growth against the threshold first; then lag, judged on whether the lag plateau ever reaches the threshold (D98 is finite), not on the 1-hour level alone, which is quoted beside the crossing time.</t>
+        </is>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -18227,8 +18259,8 @@
         <v>1</v>
       </c>
       <c r="E116" s="157" t="str">
-        <f>("Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for "&amp;"rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~")&amp;TEXT(k_geom*(1+(V_rail-V_at_gerrit_max)/(I_at_gerrit_max*R_cell)),"0.00")&amp;" by Gerrit’s Law holding linear to "&amp;TEXT(gerrit_max,"0")&amp;" % on a "&amp;TEXT(V_rail,"0")&amp;" V rail (D143–D144); that leaves only "&amp;TEXT(V_rail-V_at_gerrit_max,"0.00")&amp;" V of headroom at "&amp;TEXT(gerrit_max,"0")&amp;" %, against the ±0.12 V j₀ uncertainty (E108), so the bound is soft. Measure with a conductivity standard."</f>
-        <v>Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~2.27 by Gerrit’s Law holding linear to 25 % on a 5 V rail (D143–D144); that leaves only 1.33 V of headroom at 25 %, against the ±0.12 V j₀ uncertainty (E108), so the bound is soft. Measure with a conductivity standard.</v>
+        <f>("Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for "&amp;"rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~")&amp;TEXT(k_geom*(1+(V_rail-V_at_gerrit_max)/(I_at_gerrit_max*R_cell)),"0.00")&amp;" by the current law holding linear to "&amp;TEXT(gerrit_check_pct,"0")&amp;" % on a "&amp;TEXT(V_rail,"0")&amp;" V rail (D143–D144); that leaves "&amp;TEXT(V_rail-V_at_gerrit_max,"0.00")&amp;" V of headroom there, against the ±0.12 V j₀ uncertainty (E108)."</f>
+        <v>Parallel-cylinder (2D) formula taken at face value. Lateral confinement by the 25 mm wall raises the resistance and current spreading through the ~22 mm of liquid below the rod tips lowers it; for rods with L/d ≈ 1.5 the two roughly cancel. Bounded above at ~2.27 by the current law holding linear to 25 % on a 5 V rail (D143–D144); that leaves 1.33 V of headroom there, against the ±0.12 V j₀ uncertainty (E108).</v>
       </c>
     </row>
     <row r="117" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -18335,8 +18367,8 @@
         <v>OK — 2.65 V estimated against a 5 V rail</v>
       </c>
       <c r="E122" s="158" t="str">
-        <f>"Cross-check on Gerrit's Law: the fit is validated linear to gerrit_max ("&amp;TEXT(gerrit_max,"0")&amp;" %), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (currently "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" % with k_geom = "&amp;TEXT(k_geom,"0.0#")&amp;")."</f>
-        <v>Cross-check on Gerrit's Law: the fit is validated linear to gerrit_max (25 %), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (currently 3.67 V at 25 % with k_geom = 1.0).</v>
+        <f>"Cross-check on the current law: it is validated linear to "&amp;TEXT(gerrit_check_pct,"0")&amp;" % (D166), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (currently "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V with k_geom = "&amp;TEXT(k_geom,"0.0#")&amp;")."</f>
+        <v>Cross-check on the current law: it is validated linear to 25 % (D166), so the budget evaluated there (V_at_gerrit_max, D143) must stay at or below V_rail; D144 tests it live (currently 3.67 V with k_geom = 1.0).</v>
       </c>
     </row>
     <row r="124" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -18532,8 +18564,10 @@
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
-        <v>1915</v>
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Current at the top of the validated band (D166)</t>
+        </is>
       </c>
       <c r="B142" s="19" t="s">
         <v>1916</v>
@@ -18542,7 +18576,7 @@
         <v>300</v>
       </c>
       <c r="D142" s="111">
-        <f>(gerrit_slope*gerrit_max+gerrit_int)/1000</f>
+        <f>(gerrit_slope*gerrit_check_pct+gerrit_int)/1000</f>
         <v>0.02835</v>
       </c>
       <c r="E142" s="51" t="s">
@@ -18578,7 +18612,7 @@
         <v>111</v>
       </c>
       <c r="D144" s="111" t="str">
-        <f>IF(V_at_gerrit_max&gt;V_rail,"INCONSISTENT — the budget needs "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" %, above the "&amp;TEXT(V_rail,"0")&amp;" V rail, where Gerrit's Law is validated linear: R_cell (k_geom) or j₀ is too high","OK — "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_max,"0")&amp;" %, under the "&amp;TEXT(V_rail,"0")&amp;" V rail across the validated band")</f>
+        <f>IF(V_at_gerrit_max&gt;V_rail,"INCONSISTENT — the budget needs "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_check_pct,"0")&amp;" %, above the "&amp;TEXT(V_rail,"0")&amp;" V rail, where the current law in use is validated linear: R_cell (k_geom) or j₀ is too high","OK — "&amp;TEXT(V_at_gerrit_max,"0.00")&amp;" V at "&amp;TEXT(gerrit_check_pct,"0")&amp;" %, under the "&amp;TEXT(V_rail,"0")&amp;" V rail across the validated band")</f>
         <v>OK — 3.67 V at 25 %, under the 5 V rail across the validated band</v>
       </c>
       <c r="E144" s="51" t="s">
@@ -18847,6 +18881,32 @@
       <c r="E165" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">Eisenberg, Tobias &amp; Wilke 1954 (JES 101:306): Sh = 0.0791·Re^0.7·Sc^0.356 for a cylinder in axial swirl. At an assumed 20 cm/s swirl past a 6 mm rod this gives 3.7e-3 cm/s; bracket 2–6e-3 for 10–40 cm/s. The swirl velocity past a STATIONARY rod is the weak link — Sh goes as u^0.7, so a 4× velocity error is a 2.6× error here. Replaced by a ferricyanide run entered on the Calibrations tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Power at which the voltage cross-check is made</t>
+        </is>
+      </c>
+      <c r="B166" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gerrit_check_pct</t>
+        </is>
+      </c>
+      <c r="C166" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">%</t>
+        </is>
+      </c>
+      <c r="D166" s="111">
+        <f>IF(ISNUMBER(cal_gerrit_slope),power_max,gerrit_max)</f>
+        <v>25.0</v>
+      </c>
+      <c r="E166" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The top of the band the current law in use is validated on: 25 % (gerrit_max) for Gerrit’s default fit, the 10 % plugin clamp (power_max) for a Calibrations fit, whose accepted points span 3–10 % only.</t>
         </is>
       </c>
     </row>
@@ -25995,7 +26055,11 @@
         <f>d_bubble*1000</f>
         <v>2.077511783382</v>
       </c>
-      <c r="E43" s="57"/>
+      <c r="E43" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Display of the Tate’s-law bubble diameter in mm for the sparger in use.</t>
+        </is>
+      </c>
       <c r="F43" s="21"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
@@ -27223,7 +27287,11 @@
         <f>IF(ISNUMBER(DO_min),IF(DO_ss&gt;=DO_min,"above minimum","BELOW MINIMUM"),"minimum DO unknown - measure")</f>
         <v>minimum DO unknown - measure</v>
       </c>
-      <c r="E110" s="21"/>
+      <c r="E110" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cycle-mean DO against the organism minimum (Biology D45); "unknown" while the minimum is a data gap.</t>
+        </is>
+      </c>
       <c r="F110" s="21"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
@@ -27304,7 +27372,11 @@
         <f>Summary!Reactor_sel</f>
         <v>ed04</v>
       </c>
-      <c r="E115" s="21"/>
+      <c r="E115" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Summary reactor, imported as the key for the CO2 flows rows.</t>
+        </is>
+      </c>
       <c r="F115" s="21"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.2">
@@ -27319,7 +27391,11 @@
         <f>SUMPRODUCT(MAX((co2f_reactor=Reactor)*(co2f_nominal&gt;0)*co2f_date))</f>
         <v>46190.0</v>
       </c>
-      <c r="E116" s="21"/>
+      <c r="E116" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Most recent date in CO2 flows for the selected reactor; only rows of that date set the flow (D117).</t>
+        </is>
+      </c>
       <c r="F116" s="21"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
@@ -27391,7 +27467,11 @@
         <f>IF(has_cal&gt;0,"calibrated: "&amp;Reactor&amp;IF(ISNUMBER(cal_flow)," (flow from the Calibrations tab)"," (flow from CO2 flows)"),"NO CALIBRATION for "&amp;Reactor&amp;" – record a CO₂ flow in the Calibrations tab (CO₂ flow section, Include = y) or add a row in CO2 flows with nominal flowrate + minimum sparge")</f>
         <v>calibrated: ed04 (flow from CO2 flows)</v>
       </c>
-      <c r="E120" s="21"/>
+      <c r="E120" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Text verdict from has_cal (D119) and the flow source in use.</t>
+        </is>
+      </c>
       <c r="F120" s="21"/>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
@@ -39040,7 +39120,7 @@
         </is>
       </c>
       <c r="D548" s="41" t="str">
-        <f>IF(ph_unreach_l,"pH ceiling unreachable in lag",IF(D546=IF(ISNUMBER(spg_int_H2safe_opt),spg_int_H2safe_opt,spg_int_carbon),"the H₂ flammability screen (Biology D92)",IF(D546=IF(ISNUMBER(spg_int_pH_l),spg_int_pH_l*spg_dur_eq_opt/spg_dur_eq,spg_int_carbon),"the pH ceiling (lag)",IF(D546=spg_int_carbon,"carbon supply",IF(ISNUMBER(spg_int_DO_l),"lag O₂ dilution","the legacy O₂ flush guard (lag DO target unreachable)")))))</f>
+        <f>IF(ph_unreach_l,"pH ceiling unreachable in lag",IF(spg_int_su_opt=IF(ISNUMBER(spg_int_H2safe_opt),spg_int_H2safe_opt,spg_int_carbon),"the H₂ flammability screen (Biology D92)",IF(spg_int_su_opt=IF(ISNUMBER(spg_int_pH_l),spg_int_pH_l*spg_dur_eq_opt/spg_dur_eq,spg_int_carbon),"the pH ceiling (lag)",IF(spg_int_su_opt=spg_int_carbon,"carbon supply",IF(ISNUMBER(spg_int_DO_l),"lag O₂ dilution","the legacy O₂ flush guard (lag DO target unreachable)")))))</f>
         <v>the legacy O₂ flush guard (lag DO target unreachable)</v>
       </c>
       <c r="E548" s="51" t="inlineStr">
@@ -42811,8 +42891,10 @@
       <c r="M63" s="72"/>
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A64" s="72" t="s">
-        <v>1287</v>
+      <c r="A64" s="72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use: average across included vials of the active reactor type (all vials of a type are nominally identical). Headspace and total volume feed the model; the volume-equivalent depth (D75) is reported for the geometry check only, because a tapered vial’s equivalent depth is not its physical depth.</t>
+        </is>
       </c>
       <c r="B64" s="72"/>
       <c r="C64" s="72"/>
@@ -43142,8 +43224,10 @@
       <c r="M74" s="72"/>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A75" s="96" t="s">
-        <v>1293</v>
+      <c r="A75" s="96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - volume-equivalent depth (body volume ÷ A_x; not the physical depth)</t>
+        </is>
       </c>
       <c r="B75" s="72"/>
       <c r="C75" s="97" t="s">

</xml_diff>

<commit_message>
Gas model: fifth Codex review fixes (organism toxic DO, sinter grading, abiotic diagnostics, depth wording)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -1067,6 +1067,8 @@
     <definedName name="por_p5_hi" localSheetId="7">Calibrations!$D$201</definedName>
     <definedName name="por_p5_lo" localSheetId="7">Calibrations!$D$202</definedName>
     <definedName name="gerrit_check_pct" localSheetId="2">Electrochemistry!$D$166</definedName>
+    <definedName name="O2_ceil_org" localSheetId="5">'Mass Transfer'!$D$565</definedName>
+    <definedName name="cal_bp" localSheetId="7">Calibrations!$D$90</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -11969,7 +11971,7 @@
       <c r="C35" s="21"/>
       <c r="D35" s="176" t="str">
         <f>Geometry!geom_check</f>
-        <v>VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth</v>
+        <v>VIAL GEOMETRY INCONSISTENT - measure the true headspace (protocols/vial-geometry.md)</v>
       </c>
       <c r="E35" s="24" t="str">
         <f>HYPERLINK("#Geometry!D90","→ Geometry")</f>
@@ -13445,8 +13447,10 @@
         <v>README.md →</v>
       </c>
       <c r="E116" s="77"/>
-      <c r="F116" s="22" t="s">
-        <v>1769</v>
+      <c r="F116" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enters every Henry solubility and gas-volume conversion through P_atm (blank = 101 325 Pa): small near sea level, larger at altitude. It does not move the O₂ inhibition criterion, a fixed 0.30 atm partial pressure (Biology D26).</t>
+        </is>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
@@ -16014,16 +16018,18 @@
       </c>
       <c r="C90" s="21"/>
       <c r="D90" s="25" t="str">
-        <f>IF(ABS(A_x*D_int/1000-V_vial_total)&lt;=geom_tol_mL,"OK",IF(AND(ISNUMBER(cal_hs),ISNUMBER(cal_hs_fill)),"HEADSPACE MEASURED - bore depth still inconsistent (measure body volume)","VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth"))</f>
-        <v>VIAL GEOMETRY INCONSISTENT - measure true fill volume &amp; bore depth</v>
+        <f>IF(ABS(A_x*D_int/1000-V_vial_total)&lt;=geom_tol_mL,"OK",IF(AND(ISNUMBER(cal_hs),ISNUMBER(cal_hs_fill)),"OK – headspace measured (the tapered vial differs from the cylinder, which no longer sets the headspace)","VIAL GEOMETRY INCONSISTENT - measure the true headspace (protocols/vial-geometry.md)"))</f>
+        <v>VIAL GEOMETRY INCONSISTENT - measure the true headspace (protocols/vial-geometry.md)</v>
       </c>
       <c r="E90" s="74" t="inlineStr">
         <is>
           <t xml:space="preserve">Compares the cylinder A_x × D_int with the total vial volume within geom_tol_mL; flags the vial-geometry experiment (Summary row 107) until the true headspace is measured.</t>
         </is>
       </c>
-      <c r="F90" s="75" t="s">
-        <v>1855</v>
+      <c r="F90" s="75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fires INCONSISTENT while the headspace comes from the cylinder approximation: the bare cylinder (A_x × usable depth, ~28 mL) overstates the tapered 20 mL vial. Measuring the true headspace (Calibrations rows 63–77) makes it OK, because the measured headspace then replaces the approximation; the cylinder itself still differs from the vial.</t>
+        </is>
       </c>
       <c r="G90" s="21"/>
       <c r="H90" s="21"/>
@@ -25269,7 +25275,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:S564"/>
+  <dimension ref="A1:S565"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -26904,7 +26910,7 @@
         <v>61</v>
       </c>
       <c r="D89" s="41">
-        <f>target_DO_frac*O2_ceil_C*(V_charge/1000000)/O2_src_guard*60</f>
+        <f>target_DO_frac*O2_ceil_org*(V_charge/1000000)/O2_src_guard*60</f>
         <v>1.255448232589</v>
       </c>
       <c r="E89" s="74" t="s">
@@ -28395,7 +28401,7 @@
         <v>909</v>
       </c>
       <c r="D179" s="111">
-        <f>IF(ISNUMBER(DO_opt),DO_opt/M_O2,target_DO_frac*O2_ceil_C)</f>
+        <f>IF(ISNUMBER(DO_opt),MIN(DO_opt/M_O2,O2_ceil_org),target_DO_frac*O2_ceil_org)</f>
         <v>0.071159265207</v>
       </c>
       <c r="E179" s="74" t="s">
@@ -29902,11 +29908,13 @@
         <v>111</v>
       </c>
       <c r="D348" s="25" t="str">
-        <f>IF(DO_peak_g&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
+        <f>IF(DO_peak_g&lt;=O2_ceil_org,"peak "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_org*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_g_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_org*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
         <v>peak 2.5 mg/L under the 10.1 mg/L ceiling</v>
       </c>
-      <c r="E348" s="51" t="s">
-        <v>2461</v>
+      <c r="E348" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The sawtooth peak against the growth-inhibition ceiling (D565: the organism’s toxic DO when known, else the generic Biology D27 ceiling). Not a tautology: the peak is not what the schedule is sized on.</t>
+        </is>
       </c>
     </row>
     <row r="349" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -30280,11 +30288,13 @@
         <v>111</v>
       </c>
       <c r="D369" s="25" t="str">
-        <f>IF(DO_peak_l&lt;=O2_ceil_C,"peak "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_C*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
+        <f>IF(DO_peak_l&lt;=O2_ceil_org,"peak "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L under the "&amp;TEXT(O2_ceil_org*M_O2,"0.0")&amp;" mg/L ceiling","PEAK "&amp;TEXT(DO_peak_l_mgL,"0.0")&amp;" mg/L OVER THE "&amp;TEXT(O2_ceil_org*M_O2,"0.0")&amp;" mg/L INHIBITION CEILING")</f>
         <v>peak 6.0 mg/L under the 10.1 mg/L ceiling</v>
       </c>
-      <c r="E369" s="51" t="s">
-        <v>2461</v>
+      <c r="E369" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The sawtooth peak against the growth-inhibition ceiling (D565: the organism’s toxic DO when known, else the generic Biology D27 ceiling). Not a tautology: the peak is not what the schedule is sized on.</t>
+        </is>
       </c>
     </row>
     <row r="371" spans="1:5" x14ac:dyDescent="0.2">
@@ -30354,7 +30364,7 @@
         <v>111</v>
       </c>
       <c r="D374" s="25" t="str">
-        <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_impair)),IF(DO_peak_sched*M_O2&lt;DO_impair,"peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L under impairment","PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER IMPAIRMENT")&amp;IF(DO_avg_sched*M_O2&lt;=DO_opt,"; mean "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L at/under optimum","; MEAN "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L ABOVE OPTIMUM"),IF(DO_peak_sched&lt;=O2_ceil_C,"organism band unknown – peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L is under the inhibition ceiling","organism band unknown – PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER THE INHIBITION CEILING"))</f>
+        <f>IF(AND(ISNUMBER(DO_opt),ISNUMBER(DO_impair)),IF(DO_peak_sched*M_O2&lt;DO_impair,"peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L under impairment","PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER IMPAIRMENT")&amp;IF(DO_avg_sched*M_O2&lt;=DO_opt,"; mean "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L at/under optimum","; MEAN "&amp;TEXT(DO_avg_sched*M_O2,"0.0")&amp;" mg/L ABOVE OPTIMUM"),IF(DO_peak_sched&lt;=O2_ceil_org,"organism band unknown – peak "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L is under the inhibition ceiling","organism band unknown – PEAK "&amp;TEXT(DO_peak_sched*M_O2,"0.0")&amp;" mg/L OVER THE INHIBITION CEILING"))</f>
         <v>organism band unknown – peak 2.5 mg/L is under the inhibition ceiling</v>
       </c>
       <c r="E374" s="51" t="s">
@@ -39516,6 +39526,32 @@
       <c r="E564" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Exact time average of the lag H₂ sawtooth at the schedule in use (as D360 for O₂): the figure a time-weighted headspace measurement compares with. The mean-field fraction (D352) is the flux-weighted one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inhibition ceiling for this organism</t>
+        </is>
+      </c>
+      <c r="B565" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_ceil_org</t>
+        </is>
+      </c>
+      <c r="C565" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D565" s="41">
+        <f>IF(ISNUMBER(DO_toxic),MIN(O2_ceil_C,DO_toxic/M_O2),O2_ceil_C)</f>
+        <v>0.314742903798</v>
+      </c>
+      <c r="E565" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The organism’s own toxic DO (Biology D48, measured or tabled) when it has one, never above the generic 0.30 atm Henry ceiling (D6); otherwise that generic ceiling. Used by the DO target, the legacy guard and the peak checks.</t>
         </is>
       </c>
     </row>
@@ -42931,8 +42967,10 @@
       <c r="G65" s="99" t="s">
         <v>1290</v>
       </c>
-      <c r="H65" s="99" t="s">
-        <v>1291</v>
+      <c r="H65" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Volume-equivalent depth (computed)</t>
+        </is>
       </c>
       <c r="I65" s="99" t="s">
         <v>1267</v>
@@ -43312,7 +43350,7 @@
     <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" s="72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value in use: the most recent included measurement for the active reactor (the fitted frit is hardware, so the latest reading replaces older ones). A pore size outside the listed DURAN classes is reported in column E and not used.</t>
+          <t xml:space="preserve">Value in use: the bubble points of the most recent included runs for the active reactor are averaged first (D90) and then graded once (D89), so conflicting runs never average into a fractional grade; a pore size outside the listed DURAN classes is reported and the model keeps its default.</t>
         </is>
       </c>
       <c r="B79" s="72"/>
@@ -43536,7 +43574,7 @@
         <v>491</v>
       </c>
       <c r="D89" s="95" t="str">
-        <f>IFERROR(AVERAGEIFS(E81:E88,C81:C88,Reactor_sel,G81:G88,"y",B81:B88,SUMPRODUCT(MAX((C81:C88=Reactor_sel)*(G81:G88="y")*B81:B88))),"no included runs — model uses its default")</f>
+        <f>IF(NOT(ISNUMBER(cal_bp)),"no included runs — model uses its default",IF((bp_const/cal_bp)&gt;por_p0_hi,"above P0 – not a listed grade; model uses its default",IF((bp_const/cal_bp)&gt;por_break_1,0,IF((bp_const/cal_bp)&gt;por_break_2,1,IF((bp_const/cal_bp)&gt;por_break_3,2,IF((bp_const/cal_bp)&gt;por_break_4,3,IF((bp_const/cal_bp)&gt;=por_break_5,4,IF(AND((bp_const/cal_bp)&gt;=por_p5_lo,(bp_const/cal_bp)&lt;=por_p5_hi),5,"between or below the listed grades; model uses its default"))))))))</f>
         <v>no included runs — model uses its default</v>
       </c>
       <c r="E89" s="72"/>
@@ -43550,10 +43588,21 @@
       <c r="M89" s="72"/>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A90" s="72"/>
+      <c r="A90" s="96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value in use - bubble point (mean of the latest included runs)</t>
+        </is>
+      </c>
       <c r="B90" s="72"/>
-      <c r="C90" s="72"/>
-      <c r="D90" s="72"/>
+      <c r="C90" s="97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kPa</t>
+        </is>
+      </c>
+      <c r="D90" s="95" t="str">
+        <f>IFERROR(AVERAGEIFS(D81:D88,C81:C88,Reactor_sel,G81:G88,"y",B81:B88,SUMPRODUCT(MAX((C81:C88=Reactor_sel)*(G81:G88="y")*B81:B88))),"no included runs — model uses its default")</f>
+        <v>no included runs — model uses its default</v>
+      </c>
       <c r="E90" s="72"/>
       <c r="F90" s="72"/>
       <c r="G90" s="72"/>

</xml_diff>

<commit_message>
Gas model: seventh Codex review fixes (catalase O2 return, two-sink peroxide, exact periodic DO peaks, organism-ceiling diagnostics)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -1074,6 +1074,10 @@
     <definedName name="f_H2O2_anode" localSheetId="2">Electrochemistry!$D$170</definedName>
     <definedName name="O2_H2O2_ret_g" localSheetId="2">Electrochemistry!$D$171</definedName>
     <definedName name="O2_H2O2_lag_adj" localSheetId="2">Electrochemistry!$D$172</definedName>
+    <definedName name="O2_cat_ret_g" localSheetId="2">Electrochemistry!$D$173</definedName>
+    <definedName name="z_peak_g" localSheetId="5">'Mass Transfer'!$D$566</definedName>
+    <definedName name="z_peak_l" localSheetId="5">'Mass Transfer'!$D$567</definedName>
+    <definedName name="z_peak_su" localSheetId="5">'Mass Transfer'!$D$568</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -11662,7 +11666,7 @@
       </c>
       <c r="D20" s="65">
         <f>IF('Mass Transfer'!has_cal=0,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)",'Mass Transfer'!spg_int_opt)</f>
-        <v>7.421902768325</v>
+        <v>7.293500622657</v>
       </c>
       <c r="E20" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
@@ -11687,7 +11691,7 @@
       </c>
       <c r="D21" s="111">
         <f>IF(NOT(ISNUMBER(res_spg_int)),res_spg_int,'Mass Transfer'!spg_int)</f>
-        <v>7.19</v>
+        <v>7.07</v>
       </c>
       <c r="E21" s="67"/>
       <c r="F21" s="22" t="inlineStr">
@@ -11731,7 +11735,7 @@
       <c r="C23" s="21"/>
       <c r="D23" s="92">
         <f>Chemistry!pH_meas</f>
-        <v>6.48770186848</v>
+        <v>6.487161438894</v>
       </c>
       <c r="E23" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -11755,7 +11759,7 @@
       </c>
       <c r="D24" s="65">
         <f>'Mass Transfer'!DO_ss</f>
-        <v>2.274565106296</v>
+        <v>2.275287892306</v>
       </c>
       <c r="E24" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D108","→ Mass")</f>
@@ -11837,7 +11841,7 @@
       </c>
       <c r="D29" s="65">
         <f>'Mass Transfer'!spg_int_DO</f>
-        <v>7.421902768325</v>
+        <v>7.293500622657</v>
       </c>
       <c r="E29" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D185","→ Mass Transfer")</f>
@@ -11913,7 +11917,7 @@
       </c>
       <c r="D32" s="70">
         <f>IF(AND(ISNUMBER(res_spg_dur_run),ISNUMBER(res_spg_int_run),ISNUMBER('Mass Transfer'!duty_actual)),('Mass Transfer'!pulse_V0+'Mass Transfer'!Q_CO2_fit*res_spg_dur_run)/('Mass Transfer'!Q_CO2/60)/(60*res_spg_int_run)/'Mass Transfer'!duty_actual,"calibrate this reactor first (CO₂ flow section of the Calibrations tab, or a CO2 flows row)")</f>
-        <v>1.00068132864</v>
+        <v>1.000059954094</v>
       </c>
       <c r="E32" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
@@ -12058,7 +12062,7 @@
       <c r="C39" s="21"/>
       <c r="D39" s="175" t="str">
         <f>'Mass Transfer'!sched_regime</f>
-        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈13 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
+        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈14 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E39" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
@@ -12078,7 +12082,7 @@
       <c r="C40" s="21"/>
       <c r="D40" s="177" t="str">
         <f>Biology!H2_safety</f>
-        <v>POTENTIAL FLAMMABILITY (lag screen): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>POTENTIAL FLAMMABILITY (lag screen): H₂ 9% mean, 14% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E40" s="24" t="str">
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
@@ -12120,7 +12124,7 @@
       <c r="C42" s="21"/>
       <c r="D42" s="175" t="str">
         <f>IFERROR("×"&amp;TEXT('Mass Transfer'!CO2_sd_ratio,"0.0")&amp;IF('Mass Transfer'!CO2_sd_ratio&gt;=1," OK"," SHORTFALL (CO2 &lt; demand)")&amp;" delivered; ×"&amp;TEXT('Mass Transfer'!CO2_uptake_ratio,"0.0")&amp;" absorbed per pulse (row 77)","calibrate this reactor first")</f>
-        <v>×49.8 OK delivered; ×2.5 absorbed per pulse (row 77)</v>
+        <v>×50.7 OK delivered; ×2.5 absorbed per pulse (row 77)</v>
       </c>
       <c r="E42" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
@@ -12342,7 +12346,7 @@
       </c>
       <c r="D53" s="65">
         <f>'Mass Transfer'!hs_sag</f>
-        <v>0.05097124556</v>
+        <v>0.05000728325</v>
       </c>
       <c r="E53" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D389","→ Mass Transfer")</f>
@@ -12432,7 +12436,7 @@
       </c>
       <c r="D59" s="65">
         <f>'Mass Transfer'!DO_avg_g_mgL</f>
-        <v>2.274565106296</v>
+        <v>2.275287892306</v>
       </c>
       <c r="E59" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D343","→ Mass Transfer")</f>
@@ -12451,7 +12455,7 @@
       </c>
       <c r="D60" s="65">
         <f>'Mass Transfer'!DO_peak_g_mgL</f>
-        <v>2.452828748339</v>
+        <v>2.480371102791</v>
       </c>
       <c r="E60" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D344","→ Mass Transfer")</f>
@@ -12470,7 +12474,7 @@
       </c>
       <c r="D61" s="65">
         <f>'Mass Transfer'!DO_avg_l_mgL</f>
-        <v>5.640773717562</v>
+        <v>5.614717330178</v>
       </c>
       <c r="E61" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
@@ -12489,7 +12493,7 @@
       </c>
       <c r="D62" s="65">
         <f>'Mass Transfer'!DO_peak_l_mgL</f>
-        <v>6.004422813773</v>
+        <v>6.006789460768</v>
       </c>
       <c r="E62" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D365","→ Mass Transfer")</f>
@@ -12541,7 +12545,7 @@
       </c>
       <c r="D65" s="65" t="str">
         <f>'Mass Transfer'!DO_feas_g</f>
-        <v>reachable – kLa margin 1.74×</v>
+        <v>reachable – kLa margin 1.72×</v>
       </c>
       <c r="E65" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D347","→ Mass Transfer")</f>
@@ -12577,7 +12581,7 @@
       </c>
       <c r="D67" s="65">
         <f>'Mass Transfer'!kLa_surf_req_g*3600</f>
-        <v>15.848589519808</v>
+        <v>15.978886341621</v>
       </c>
       <c r="E67" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D345","→ Mass Transfer")</f>
@@ -12615,7 +12619,7 @@
       </c>
       <c r="D69" s="65">
         <f>'Mass Transfer'!y_O2_mf_g</f>
-        <v>0.02766022792</v>
+        <v>0.027367364576</v>
       </c>
       <c r="E69" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D329","→ Mass Transfer")</f>
@@ -12634,7 +12638,7 @@
       </c>
       <c r="D70" s="65">
         <f>'Mass Transfer'!y_O2_mf_l</f>
-        <v>0.054287788176</v>
+        <v>0.053538910882</v>
       </c>
       <c r="E70" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D351","→ Mass Transfer")</f>
@@ -12655,7 +12659,7 @@
       </c>
       <c r="D71" s="65">
         <f>'Mass Transfer'!y_H2_mf_l</f>
-        <v>0.093870758852</v>
+        <v>0.09257585106</v>
       </c>
       <c r="E71" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D352","→ Mass Transfer")</f>
@@ -12674,7 +12678,7 @@
       </c>
       <c r="D72" s="65">
         <f>'Mass Transfer'!y_CO2_mf</f>
-        <v>0.940062404006</v>
+        <v>0.940877306879</v>
       </c>
       <c r="E72" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D381","→ Mass Transfer")</f>
@@ -12728,7 +12732,7 @@
       </c>
       <c r="D76" s="70">
         <f>Biology!CO2_margin_trough</f>
-        <v>508.697994922664</v>
+        <v>509.521897908088</v>
       </c>
       <c r="E76" s="24" t="str">
         <f>HYPERLINK("#Biology!D98","→ Biology")</f>
@@ -12752,7 +12756,7 @@
       </c>
       <c r="D77" s="65">
         <f>'Mass Transfer'!CO2_uptake_ratio</f>
-        <v>2.501421260187</v>
+        <v>2.503892293977</v>
       </c>
       <c r="E77" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D417","→ Mass Transfer")</f>
@@ -12782,7 +12786,7 @@
       </c>
       <c r="D80" s="65">
         <f>Chemistry!alk_NaHCO3_gL</f>
-        <v>0.123122489916</v>
+        <v>0.129751405739</v>
       </c>
       <c r="E80" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
@@ -12803,7 +12807,7 @@
       </c>
       <c r="D81" s="65">
         <f>Chemistry!alk_needed*1000</f>
-        <v>1.465621792425</v>
+        <v>1.544530881222</v>
       </c>
       <c r="E81" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
@@ -12826,7 +12830,7 @@
       </c>
       <c r="D82" s="65">
         <f>'Mass Transfer'!N2_for_DO</f>
-        <v>0.337846643585</v>
+        <v>0.344043413938</v>
       </c>
       <c r="E82" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D426","→ Mass Transfer")</f>
@@ -13099,7 +13103,7 @@
       </c>
       <c r="D98" s="179" t="str">
         <f>Electrochemistry!H2O2_flag</f>
-        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min (0.84 mg/L after 1 h) before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.043 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min (0.84 mg/L after 1 h) before biomass can scavenge it</v>
       </c>
       <c r="E98" s="24" t="str">
         <f>HYPERLINK("#Electrochemistry!D99","→ Electrochemistry")</f>
@@ -13165,7 +13169,7 @@
       </c>
       <c r="D101" s="23">
         <f>Chemistry!E_Cu_margin</f>
-        <v>1.24888409344</v>
+        <v>1.248916601067</v>
       </c>
       <c r="E101" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D211","→ Chemistry")</f>
@@ -13187,7 +13191,7 @@
       </c>
       <c r="D102" s="23">
         <f>Chemistry!pH_meas</f>
-        <v>6.48770186848</v>
+        <v>6.487161438894</v>
       </c>
       <c r="E102" s="24" t="str">
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
@@ -13209,7 +13213,7 @@
       </c>
       <c r="D103" s="23">
         <f>'Mass Transfer'!kLa_surf_req*3600</f>
-        <v>15.848589519808</v>
+        <v>15.978886341621</v>
       </c>
       <c r="E103" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D186","→ Mass Transfer")</f>
@@ -13333,8 +13337,10 @@
         <v>faradaic-efficiency.md →</v>
       </c>
       <c r="E110" s="77"/>
-      <c r="F110" s="22" t="s">
-        <v>1689</v>
+      <c r="F110" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Calculated today as 1 − the chlorine, peroxide-oxidation, anodic H₂-oxidation and metal-dissolution shares (Electrochemistry D104), with the last two unmeasured; any anodic metal dissolution comes straight off it, and the corrosion suspicion on Chemistry D163 needs exactly this number. Needs an accepted per-electrode measurement, not a mixed-gas screen.</t>
+        </is>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
@@ -16127,7 +16133,7 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="A1:N172"/>
+  <dimension ref="A1:N173"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -16660,8 +16666,10 @@
         <f>IF(ISNUMBER(cal_etaF_OER),cal_etaF_OER,etaF_OER_calc)</f>
         <v>0.999705046585</v>
       </c>
-      <c r="E26" s="51" t="s">
-        <v>1862</v>
+      <c r="E26" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anodic O₂ faradaic efficiency: an accepted per-electrode measurement from the Calibrations tab if there is one, otherwise CALCULATED (D104) as 1 − the chlorine, metal-dissolution, anodic H₂-oxidation and peroxide-oxidation shares. A mixed-gas screen of the undivided cell cannot separate those contributions (protocols/faradaic-efficiency.md).</t>
+        </is>
       </c>
       <c r="F26" s="21"/>
       <c r="G26" s="21"/>
@@ -16723,12 +16731,12 @@
         <v>307</v>
       </c>
       <c r="D29" s="41">
-        <f>rO2_gen-O2_cathode_ORR+O2_H2O2_ret_g</f>
-        <v>5.102798409848e-05</v>
+        <f>rO2_gen-O2_cathode_ORR+O2_H2O2_ret_g+O2_cat_ret_g</f>
+        <v>5.116706148996e-05</v>
       </c>
       <c r="E29" s="74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anodic O₂ minus cathodic consumption at the design DO (D85), plus the O₂ returned by peroxide oxidation at the anode (D171) — the O₂ the dissolved pool receives in growth. The lag phase uses O2_net_lag (D132).</t>
+          <t xml:space="preserve">Anodic O₂ minus cathodic consumption at the design DO (D85), plus the O₂ that peroxide oxidation at the anode (D171) and catalase (D173) give back — the O₂ the dissolved pool receives in growth. The lag phase uses O2_net_lag (D132).</t>
         </is>
       </c>
       <c r="F29" s="21"/>
@@ -17927,11 +17935,13 @@
         <v>1136</v>
       </c>
       <c r="D95" s="111">
-        <f>r_H2O2/(k_cat_cells*3600)</f>
-        <v>0.047544429265</v>
-      </c>
-      <c r="E95" s="51" t="s">
-        <v>1509</v>
+        <f>r_H2O2/((k_cat_cells+k_H2O2_anode)*3600)</f>
+        <v>0.042734198267</v>
+      </c>
+      <c r="E95" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Production ÷ (catalase clearance + anodic oxidation, D94 + D151): both sinks act on the bulk peroxide. The bulk Fenton route is not modelled: the medium’s Fe(II) is a one-shot capacity oxidised away in minutes.</t>
+        </is>
       </c>
     </row>
     <row r="96" spans="1:5" ht="24" x14ac:dyDescent="0.2">
@@ -17999,7 +18009,7 @@
       </c>
       <c r="D99" s="111" t="str">
         <f>IF(H2O2_ss&gt;H2O2_thresh,"PEROXIDE ABOVE THE GROWTH-INHIBITION THRESHOLD even with a full catalase pool ("&amp;TEXT(H2O2_ss,"0.00")&amp;" mg/L)",IF(ISNUMBER(t_H2O2_thresh),"watch — steady growth is clear ("&amp;TEXT(H2O2_ss,"0.000")&amp;" mg/L) but LAG PHASE is not: peroxide passes the threshold in "&amp;TEXT(t_H2O2_thresh,"0")&amp;" min ("&amp;TEXT(H2O2_lag_1h,"0.00")&amp;" mg/L after 1 h) before biomass can scavenge it","OK — peroxide stays below the growth-inhibition threshold in both phases, including the lag plateau"))</f>
-        <v>watch — steady growth is clear (0.048 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min (0.84 mg/L after 1 h) before biomass can scavenge it</v>
+        <v>watch — steady growth is clear (0.043 mg/L) but LAG PHASE is not: peroxide passes the threshold in 6 min (0.84 mg/L after 1 h) before biomass can scavenge it</v>
       </c>
       <c r="E99" s="51" t="inlineStr">
         <is>
@@ -18557,7 +18567,7 @@
       </c>
       <c r="D134" s="111" t="str">
         <f>IFERROR(IF(ABS(DO_lag_ref/ec_DO_lag-1)&gt;DO_lag_tol,"RE-ENTER DO_lag_ref (D129): the lag DO is now "&amp;TEXT(ec_DO_lag,"0.000")&amp;" mol/m³ ("&amp;TEXT(DO_lag_ref/ec_DO_lag-1,"+0%;-0%")&amp;" off)","OK – DO_lag_ref within "&amp;TEXT(DO_lag_tol,"0%")&amp;" of the lag DO ("&amp;TEXT(ec_DO_lag,"0.000")&amp;" mol/m³)"),"lag DO not available")</f>
-        <v>OK – DO_lag_ref within 5% of the lag DO (0.176 mol/m³)</v>
+        <v>OK – DO_lag_ref within 5% of the lag DO (0.175 mol/m³)</v>
       </c>
       <c r="E134" s="57" t="s">
         <v>1909</v>
@@ -18741,7 +18751,7 @@
       </c>
       <c r="D150" s="111">
         <f>'Mass Transfer'!DO_ss_sawtooth_lag</f>
-        <v>0.176285196499</v>
+        <v>0.175470883498</v>
       </c>
       <c r="E150" s="51" t="s">
         <v>1941</v>
@@ -18838,7 +18848,7 @@
       </c>
       <c r="D161" s="111">
         <f>Chemistry!j_buffer_ratio</f>
-        <v>0.19971310793</v>
+        <v>0.19970604856</v>
       </c>
       <c r="E161" s="140" t="s">
         <v>1955</v>
@@ -19067,6 +19077,32 @@
       <c r="E172" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Added to the lag O₂ source (D132): the lag peroxide turnover returns one O₂ and diverts half an O₂ of OER per H₂O₂, while D22 already carries the growth diversion; net (r_l + r_g)/2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ returned by catalase — growth</t>
+        </is>
+      </c>
+      <c r="B173" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_cat_ret_g</t>
+        </is>
+      </c>
+      <c r="C173" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D173" s="111">
+        <f>f_HOOH*O2_cathode_ORR*k_cat_cells/(k_H2O2_anode+k_cat_cells)/2</f>
+        <v>1.390773914844e-07</v>
+      </c>
+      <c r="E173" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Catalase disproportionates the rest of the growth peroxide, 2 H₂O₂ → O₂ + 2 H₂O: half an O₂ back per H₂O₂. A biological return, so it applies whether or not etaF_OER is measured.</t>
         </is>
       </c>
     </row>
@@ -19177,7 +19213,7 @@
       </c>
       <c r="D5" s="49">
         <f>'Mass Transfer'!CO2aqc_ss</f>
-        <v>0.02555602506</v>
+        <v>0.025595318383</v>
       </c>
       <c r="E5" s="138" t="s">
         <v>1963</v>
@@ -19859,7 +19895,7 @@
       </c>
       <c r="B50" s="49">
         <f t="shared" ref="B50:B81" si="1">pH_SID + pH_NT*(10^-A50)/((10^-A50)+KaN_c) + (10^-A50) - (pH_PT*Ka1p_c*(10^-A50)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A50) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A50)^3 + Ka1p_c*(10^-A50)^2 + Ka1p_c*Ka2p_c*(10^-A50) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A50) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A50)^2 - Kw_c/(10^-A50)</f>
-        <v>0.069961089647</v>
+        <v>0.069960755105</v>
       </c>
       <c r="C50" s="49">
         <f t="shared" ref="C50:C81" si="2">IF(AND(B50&gt;=0,B51&lt;0),A50+pH_step*B50/(B50-B51),0)</f>
@@ -19872,7 +19908,7 @@
       </c>
       <c r="B51" s="49">
         <f t="shared" si="1"/>
-        <v>0.069751417946</v>
+        <v>0.069750996782</v>
       </c>
       <c r="C51" s="49">
         <f t="shared" si="2"/>
@@ -19885,7 +19921,7 @@
       </c>
       <c r="B52" s="49">
         <f t="shared" si="1"/>
-        <v>0.069543441154</v>
+        <v>0.06954291094</v>
       </c>
       <c r="C52" s="49">
         <f t="shared" si="2"/>
@@ -19898,7 +19934,7 @@
       </c>
       <c r="B53" s="49">
         <f t="shared" si="1"/>
-        <v>0.069326273846</v>
+        <v>0.069325606345</v>
       </c>
       <c r="C53" s="49">
         <f t="shared" si="2"/>
@@ -19911,7 +19947,7 @@
       </c>
       <c r="B54" s="49">
         <f t="shared" si="1"/>
-        <v>0.069088508579</v>
+        <v>0.069087668243</v>
       </c>
       <c r="C54" s="49">
         <f t="shared" si="2"/>
@@ -19924,7 +19960,7 @@
       </c>
       <c r="B55" s="49">
         <f t="shared" si="1"/>
-        <v>0.068817641626</v>
+        <v>0.068816583704</v>
       </c>
       <c r="C55" s="49">
         <f t="shared" si="2"/>
@@ -19937,7 +19973,7 @@
       </c>
       <c r="B56" s="49">
         <f t="shared" si="1"/>
-        <v>0.068499440462</v>
+        <v>0.068498108613</v>
       </c>
       <c r="C56" s="49">
         <f t="shared" si="2"/>
@@ -19950,7 +19986,7 @@
       </c>
       <c r="B57" s="49">
         <f t="shared" si="1"/>
-        <v>0.068117226127</v>
+        <v>0.068115549423</v>
       </c>
       <c r="C57" s="49">
         <f t="shared" si="2"/>
@@ -19963,7 +19999,7 @@
       </c>
       <c r="B58" s="49">
         <f t="shared" si="1"/>
-        <v>0.067651040393</v>
+        <v>0.067648929538</v>
       </c>
       <c r="C58" s="49">
         <f t="shared" si="2"/>
@@ -19976,7 +20012,7 @@
       </c>
       <c r="B59" s="49">
         <f t="shared" si="1"/>
-        <v>0.067076664325</v>
+        <v>0.067074006902</v>
       </c>
       <c r="C59" s="49">
         <f t="shared" si="2"/>
@@ -19989,7 +20025,7 @@
       </c>
       <c r="B60" s="49">
         <f t="shared" si="1"/>
-        <v>0.066364451605</v>
+        <v>0.066361106084</v>
       </c>
       <c r="C60" s="49">
         <f t="shared" si="2"/>
@@ -20002,7 +20038,7 @@
       </c>
       <c r="B61" s="49">
         <f t="shared" si="1"/>
-        <v>0.065477937341</v>
+        <v>0.065473725543</v>
       </c>
       <c r="C61" s="49">
         <f t="shared" si="2"/>
@@ -20015,7 +20051,7 @@
       </c>
       <c r="B62" s="49">
         <f t="shared" si="1"/>
-        <v>0.06437218162</v>
+        <v>0.064366879223</v>
       </c>
       <c r="C62" s="49">
         <f t="shared" si="2"/>
@@ -20028,7 +20064,7 @@
       </c>
       <c r="B63" s="49">
         <f t="shared" si="1"/>
-        <v>0.062991807568</v>
+        <v>0.062985132154</v>
       </c>
       <c r="C63" s="49">
         <f t="shared" si="2"/>
@@ -20041,7 +20077,7 @@
       </c>
       <c r="B64" s="49">
         <f t="shared" si="1"/>
-        <v>0.061268696854</v>
+        <v>0.061260292859</v>
       </c>
       <c r="C64" s="49">
         <f t="shared" si="2"/>
@@ -20054,7 +20090,7 @@
       </c>
       <c r="B65" s="49">
         <f t="shared" si="1"/>
-        <v>0.059119311276</v>
+        <v>0.059108731043</v>
       </c>
       <c r="C65" s="49">
         <f t="shared" si="2"/>
@@ -20067,7 +20103,7 @@
       </c>
       <c r="B66" s="49">
         <f t="shared" si="1"/>
-        <v>0.05644161557</v>
+        <v>0.056428295479</v>
       </c>
       <c r="C66" s="49">
         <f t="shared" si="2"/>
@@ -20080,7 +20116,7 @@
       </c>
       <c r="B67" s="49">
         <f t="shared" si="1"/>
-        <v>0.053111578135</v>
+        <v>0.053094808554</v>
       </c>
       <c r="C67" s="49">
         <f t="shared" si="2"/>
@@ -20093,7 +20129,7 @@
       </c>
       <c r="B68" s="49">
         <f t="shared" si="1"/>
-        <v>0.048979211329</v>
+        <v>0.048958098758</v>
       </c>
       <c r="C68" s="49">
         <f t="shared" si="2"/>
@@ -20106,7 +20142,7 @@
       </c>
       <c r="B69" s="49">
         <f t="shared" si="1"/>
-        <v>0.043864060207</v>
+        <v>0.043837479598</v>
       </c>
       <c r="C69" s="49">
         <f t="shared" si="2"/>
@@ -20119,7 +20155,7 @@
       </c>
       <c r="B70" s="49">
         <f t="shared" si="1"/>
-        <v>0.037549927376</v>
+        <v>0.037516462061</v>
       </c>
       <c r="C70" s="49">
         <f t="shared" si="2"/>
@@ -20132,7 +20168,7 @@
       </c>
       <c r="B71" s="49">
         <f t="shared" si="1"/>
-        <v>0.029778395532</v>
+        <v>0.029736261536</v>
       </c>
       <c r="C71" s="49">
         <f t="shared" si="2"/>
@@ -20145,7 +20181,7 @@
       </c>
       <c r="B72" s="49">
         <f t="shared" si="1"/>
-        <v>0.020240350728</v>
+        <v>0.020187301369</v>
       </c>
       <c r="C72" s="49">
         <f t="shared" si="2"/>
@@ -20158,11 +20194,11 @@
       </c>
       <c r="B73" s="49">
         <f t="shared" si="1"/>
-        <v>0.008564225664</v>
+        <v>0.008497431283</v>
       </c>
       <c r="C73" s="49">
         <f t="shared" si="2"/>
-        <v>6.360036291182</v>
+        <v>6.359495861596</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.2">
@@ -20171,7 +20207,7 @@
       </c>
       <c r="B74" s="49">
         <f t="shared" si="1"/>
-        <v>-0.005700855498</v>
+        <v>-0.005784959215</v>
       </c>
       <c r="C74" s="49">
         <f t="shared" si="2"/>
@@ -20184,7 +20220,7 @@
       </c>
       <c r="B75" s="49">
         <f t="shared" si="1"/>
-        <v>-0.023109297687</v>
+        <v>-0.023215201089</v>
       </c>
       <c r="C75" s="49">
         <f t="shared" si="2"/>
@@ -20197,7 +20233,7 @@
       </c>
       <c r="B76" s="49">
         <f t="shared" si="1"/>
-        <v>-0.044353076874</v>
+        <v>-0.044486437963</v>
       </c>
       <c r="C76" s="49">
         <f t="shared" si="2"/>
@@ -20210,7 +20246,7 @@
       </c>
       <c r="B77" s="49">
         <f t="shared" si="1"/>
-        <v>-0.070307904209</v>
+        <v>-0.070475853889</v>
       </c>
       <c r="C77" s="49">
         <f t="shared" si="2"/>
@@ -20223,7 +20259,7 @@
       </c>
       <c r="B78" s="49">
         <f t="shared" si="1"/>
-        <v>-0.102093440558</v>
+        <v>-0.102304968626</v>
       </c>
       <c r="C78" s="49">
         <f t="shared" si="2"/>
@@ -20236,7 +20272,7 @@
       </c>
       <c r="B79" s="49">
         <f t="shared" si="1"/>
-        <v>-0.141149273789</v>
+        <v>-0.141415717577</v>
       </c>
       <c r="C79" s="49">
         <f t="shared" si="2"/>
@@ -20249,7 +20285,7 @@
       </c>
       <c r="B80" s="49">
         <f t="shared" si="1"/>
-        <v>-0.189328797934</v>
+        <v>-0.189664461753</v>
       </c>
       <c r="C80" s="49">
         <f t="shared" si="2"/>
@@ -20262,7 +20298,7 @@
       </c>
       <c r="B81" s="49">
         <f t="shared" si="1"/>
-        <v>-0.249014555568</v>
+        <v>-0.249437497331</v>
       </c>
       <c r="C81" s="49">
         <f t="shared" si="2"/>
@@ -20275,7 +20311,7 @@
       </c>
       <c r="B82" s="49">
         <f t="shared" ref="B82:B100" si="3">pH_SID + pH_NT*(10^-A82)/((10^-A82)+KaN_c) + (10^-A82) - (pH_PT*Ka1p_c*(10^-A82)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-A82) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-A82)^3 + Ka1p_c*(10^-A82)^2 + Ka1p_c*Ka2p_c*(10^-A82) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-A82) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-A82)^2 - Kw_c/(10^-A82)</f>
-        <v>-0.32326107991</v>
+        <v>-0.323794112198</v>
       </c>
       <c r="C82" s="49">
         <f t="shared" ref="C82:C99" si="4">IF(AND(B82&gt;=0,B83&lt;0),A82+pH_step*B82/(B82-B83),0)</f>
@@ -20288,7 +20324,7 @@
       </c>
       <c r="B83" s="49">
         <f t="shared" si="3"/>
-        <v>-0.415974635856</v>
+        <v>-0.416646603229</v>
       </c>
       <c r="C83" s="49">
         <f t="shared" si="4"/>
@@ -20301,7 +20337,7 @@
       </c>
       <c r="B84" s="49">
         <f t="shared" si="3"/>
-        <v>-0.532143388559</v>
+        <v>-0.532990802641</v>
       </c>
       <c r="C84" s="49">
         <f t="shared" si="4"/>
@@ -20314,7 +20350,7 @@
       </c>
       <c r="B85" s="49">
         <f t="shared" si="3"/>
-        <v>-0.678136622512</v>
+        <v>-0.679205763268</v>
       </c>
       <c r="C85" s="49">
         <f t="shared" si="4"/>
@@ -20327,7 +20363,7 @@
       </c>
       <c r="B86" s="49">
         <f t="shared" si="3"/>
-        <v>-0.862098355682</v>
+        <v>-0.86344798467</v>
       </c>
       <c r="C86" s="49">
         <f t="shared" si="4"/>
@@ -20340,7 +20376,7 @@
       </c>
       <c r="B87" s="49">
         <f t="shared" si="3"/>
-        <v>-1.094470207061</v>
+        <v>-1.096175090827</v>
       </c>
       <c r="C87" s="49">
         <f t="shared" si="4"/>
@@ -20353,7 +20389,7 @@
       </c>
       <c r="B88" s="49">
         <f t="shared" si="3"/>
-        <v>-1.388692414049</v>
+        <v>-1.390847930362</v>
       </c>
       <c r="C88" s="49">
         <f t="shared" si="4"/>
@@ -20366,7 +20402,7 @@
       </c>
       <c r="B89" s="49">
         <f t="shared" si="3"/>
-        <v>-1.762152977297</v>
+        <v>-1.764881184359</v>
       </c>
       <c r="C89" s="49">
         <f t="shared" si="4"/>
@@ -20379,7 +20415,7 @@
       </c>
       <c r="B90" s="49">
         <f t="shared" si="3"/>
-        <v>-2.237486801867</v>
+        <v>-2.240944507399</v>
       </c>
       <c r="C90" s="49">
         <f t="shared" si="4"/>
@@ -20392,7 +20428,7 @@
       </c>
       <c r="B91" s="49">
         <f t="shared" si="3"/>
-        <v>-2.844375195515</v>
+        <v>-2.848764794096</v>
       </c>
       <c r="C91" s="49">
         <f t="shared" si="4"/>
@@ -20405,7 +20441,7 @@
       </c>
       <c r="B92" s="49">
         <f t="shared" si="3"/>
-        <v>-3.622070214084</v>
+        <v>-3.62765440665</v>
       </c>
       <c r="C92" s="49">
         <f t="shared" si="4"/>
@@ -20418,7 +20454,7 @@
       </c>
       <c r="B93" s="49">
         <f t="shared" si="3"/>
-        <v>-4.622982295039</v>
+        <v>-4.630104325121</v>
       </c>
       <c r="C93" s="49">
         <f t="shared" si="4"/>
@@ -20431,7 +20467,7 @@
       </c>
       <c r="B94" s="49">
         <f t="shared" si="3"/>
-        <v>-5.917845708389</v>
+        <v>-5.926957541051</v>
       </c>
       <c r="C94" s="49">
         <f t="shared" si="4"/>
@@ -20444,7 +20480,7 @@
       </c>
       <c r="B95" s="49">
         <f t="shared" si="3"/>
-        <v>-7.603249726853</v>
+        <v>-7.614951807867</v>
       </c>
       <c r="C95" s="49">
         <f t="shared" si="4"/>
@@ -20457,7 +20493,7 @@
       </c>
       <c r="B96" s="49">
         <f t="shared" si="3"/>
-        <v>-9.812749485113</v>
+        <v>-9.827847584477</v>
       </c>
       <c r="C96" s="49">
         <f t="shared" si="4"/>
@@ -20470,7 +20506,7 @@
       </c>
       <c r="B97" s="49">
         <f t="shared" si="3"/>
-        <v>-12.733436697525</v>
+        <v>-12.753024232131</v>
       </c>
       <c r="C97" s="49">
         <f t="shared" si="4"/>
@@ -20483,7 +20519,7 @@
       </c>
       <c r="B98" s="49">
         <f t="shared" si="3"/>
-        <v>-16.63089482033</v>
+        <v>-16.656473546967</v>
       </c>
       <c r="C98" s="49">
         <f t="shared" si="4"/>
@@ -20496,7 +20532,7 @@
       </c>
       <c r="B99" s="49">
         <f t="shared" si="3"/>
-        <v>-21.887104114512</v>
+        <v>-21.920763103551</v>
       </c>
       <c r="C99" s="49">
         <f t="shared" si="4"/>
@@ -20509,7 +20545,7 @@
       </c>
       <c r="B100" s="49">
         <f t="shared" si="3"/>
-        <v>-29.05844451528</v>
+        <v>-29.103128305187</v>
       </c>
       <c r="C100" s="49">
         <f>0</f>
@@ -20549,7 +20585,7 @@
       </c>
       <c r="D103" s="119">
         <f>IF(n_cross=1,SUM(C50:C100),NA())</f>
-        <v>6.360036291182</v>
+        <v>6.359495861596</v>
       </c>
       <c r="E103" s="138" t="s">
         <v>1670</v>
@@ -20570,7 +20606,7 @@
       </c>
       <c r="D104" s="119">
         <f>1/(1+KaHOCl_c/10^-pH_op)</f>
-        <v>0.884650730265</v>
+        <v>0.884777651302</v>
       </c>
       <c r="E104" s="138" t="s">
         <v>1968</v>
@@ -20980,7 +21016,7 @@
       </c>
       <c r="D138" s="119">
         <f>pH_NT/(1+10^(pKa_NH4-pH_op))</f>
-        <v>2.586887235199e-05</v>
+        <v>2.583675976917e-05</v>
       </c>
       <c r="E138" s="138" t="s">
         <v>1001</v>
@@ -22090,7 +22126,7 @@
       </c>
       <c r="D206" s="111">
         <f>E0_OER-nernst_slope*pH_meas</f>
-        <v>0.838755281059</v>
+        <v>0.838787788686</v>
       </c>
       <c r="E206" s="74" t="s">
         <v>1438</v>
@@ -22108,7 +22144,7 @@
       </c>
       <c r="D207" s="111">
         <f>E0_HER-nernst_slope*pH_meas</f>
-        <v>-0.390244718941</v>
+        <v>-0.390212211314</v>
       </c>
       <c r="E207" s="74" t="s">
         <v>1441</v>
@@ -22164,7 +22200,7 @@
       </c>
       <c r="D210" s="111">
         <f>E0_ORR2-nernst_slope*pH_meas</f>
-        <v>0.304755281059</v>
+        <v>0.304787788686</v>
       </c>
       <c r="E210" s="51" t="s">
         <v>1448</v>
@@ -22182,7 +22218,7 @@
       </c>
       <c r="D211" s="111">
         <f>E_anode_op-E0_Cu</f>
-        <v>1.24888409344</v>
+        <v>1.248916601067</v>
       </c>
       <c r="E211" s="51" t="s">
         <v>1451</v>
@@ -22240,7 +22276,7 @@
       </c>
       <c r="D216" s="111">
         <f>Fcc*((km_HPO4/100)*HPO4_op+(km_HCO3/100)*HCO3_op)*1000/10</f>
-        <v>16.462667230811</v>
+        <v>16.463249166465</v>
       </c>
       <c r="E216" s="51" t="s">
         <v>1984</v>
@@ -22276,7 +22312,7 @@
       </c>
       <c r="D218" s="111">
         <f>j_anode_c/j_buffer_lim</f>
-        <v>0.19971310793</v>
+        <v>0.19970604856</v>
       </c>
       <c r="E218" s="51" t="s">
         <v>1464</v>
@@ -22312,7 +22348,7 @@
       </c>
       <c r="D220" s="111">
         <f>pH_op-LOG10(gamma_1)</f>
-        <v>6.48770186848</v>
+        <v>6.487161438894</v>
       </c>
       <c r="E220" s="51" t="s">
         <v>1470</v>
@@ -22619,7 +22655,7 @@
       </c>
       <c r="D252" s="111">
         <f>Ka1c_c*CO2aqc/10^-pH_op</f>
-        <v>0.049849406755</v>
+        <v>0.049863963444</v>
       </c>
       <c r="E252" s="51" t="s">
         <v>2022</v>
@@ -22637,7 +22673,7 @@
       </c>
       <c r="D253" s="111">
         <f>pH_PT/(1+10^(-LOG10(Ka2p_c)-pH_op))</f>
-        <v>0.0194582179</v>
+        <v>0.01944185964</v>
       </c>
       <c r="E253" s="51" t="s">
         <v>2025</v>
@@ -22691,7 +22727,7 @@
       </c>
       <c r="D256" s="111">
         <f>E_OER+eta_anode_c+pcet_credit_c</f>
-        <v>1.59078409344</v>
+        <v>1.590816601067</v>
       </c>
       <c r="E256" s="51" t="s">
         <v>2034</v>
@@ -23158,7 +23194,7 @@
       </c>
       <c r="D305" s="111">
         <f>pH_SID + pH_NT*(10^-alk_pH_target_c)/((10^-alk_pH_target_c)+KaN_c) + (10^-alk_pH_target_c) - (pH_PT*Ka1p_c*(10^-alk_pH_target_c)^2 + 2*pH_PT*Ka1p_c*Ka2p_c*(10^-alk_pH_target_c) + 3*pH_PT*Ka1p_c*Ka2p_c*Ka3p_c)/((10^-alk_pH_target_c)^3 + Ka1p_c*(10^-alk_pH_target_c)^2 + Ka1p_c*Ka2p_c*(10^-alk_pH_target_c) + Ka1p_c*Ka2p_c*Ka3p_c) - Ka1c_c*CO2aqc/(10^-alk_pH_target_c) - 2*Ka1c_c*Ka2c_c*CO2aqc/(10^-alk_pH_target_c)^2 - Kw_c/(10^-alk_pH_target_c)</f>
-        <v>-0.001465621792</v>
+        <v>-0.001544530881</v>
       </c>
       <c r="E305" s="60" t="s">
         <v>2734</v>
@@ -23178,7 +23214,7 @@
       </c>
       <c r="D306" s="111">
         <f>MAX(0,-alk_resid_t)</f>
-        <v>0.001465621792</v>
+        <v>0.001544530881</v>
       </c>
       <c r="E306" s="60" t="s">
         <v>2737</v>
@@ -23213,7 +23249,7 @@
       </c>
       <c r="D308" s="111">
         <f>alk_needed*M_NaHCO3</f>
-        <v>0.123122489916</v>
+        <v>0.129751405739</v>
       </c>
       <c r="E308" s="60" t="inlineStr">
         <is>
@@ -23646,7 +23682,7 @@
       </c>
       <c r="D5" s="120">
         <f>Electrochemistry!O2_net_gen</f>
-        <v>5.102798409848e-05</v>
+        <v>5.116706148996e-05</v>
       </c>
       <c r="E5" s="105" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -23834,7 +23870,7 @@
       </c>
       <c r="D16" s="41">
         <f>MAX(0,O2_net_gen-O2_cons)</f>
-        <v>1.691660977184e-05</v>
+        <v>1.705568716332e-05</v>
       </c>
       <c r="E16" s="161" t="str">
         <f>IFERROR(("Net electrolytic O₂ minus biological uptake, floored at zero. The floor matters: at the knallgas cap (O₂:H₂ = 0.5, i.e. bio_O2 = 3) uptake exactly consumes the electrolytic surplus and everything "&amp;"downstream that divides by this would blow up. A LOWER bound on the surplus: full H₂ uptake maximises respiration, so any H₂ that bubbles off uncaught raises the surplus (half uptake → ×")&amp;TEXT((O2_net_gen-O2_cons/2)/O2_excess,"0.0")&amp;"). Sensitive: each 1 % on bio_O2 moves it "&amp;TEXT(O2_cons/O2_excess,"0.0")&amp;" % the other way (linear, so symmetric).","Net electrolytic O₂ minus biological uptake, floored at zero: uptake consumes the whole surplus at these ratios.")</f>
@@ -24358,7 +24394,7 @@
       </c>
       <c r="D44" s="111" t="str">
         <f>IF(AND(y_H2_end_b&gt;=H2_LFL,y_O2_end_b&gt;=O2_LOC_H2*LOC_margin),"POTENTIAL FLAMMABILITY (lag screen): H₂ "&amp;TEXT(y_H2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_H2_end_b,"0%")&amp;" before each pulse; O₂ "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean, "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse – until uptake starts, "&amp;IF(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res)*60&gt;spg_dur_opt_b,"sparge every ≤"&amp;TEXT(MAX(0,CEILING(spg_int_H2safe_saw,remedy_res)-remedy_res),"0.0")&amp;" min or ","interval remedy unavailable; ")&amp;"sweep ≥"&amp;TEXT(FLOOR(N2_sweep_H2safe,remedy_res)+remedy_res,"0.0")&amp;" mL/min N₂; vent to a hood; no ignition sources","Below nominal H₂/O₂ screening thresholds (lag; not safety certification): H₂ "&amp;TEXT(y_H2_end_b,"0%")&amp;", O₂ "&amp;TEXT(y_O2_end_b,"0%")&amp;" before each pulse ("&amp;TEXT(y_H2_hs_lag,"0%")&amp;" / "&amp;TEXT(y_O2_hs_lag,"0%")&amp;" mean)")</f>
-        <v>POTENTIAL FLAMMABILITY (lag screen): H₂ 9% mean, 15% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
+        <v>POTENTIAL FLAMMABILITY (lag screen): H₂ 9% mean, 14% before each pulse; O₂ 5% mean, 8% before each pulse – until uptake starts, sparge every ≤2.3 min or sweep ≥1.0 mL/min N₂; vent to a hood; no ignition sources</v>
       </c>
       <c r="E44" s="57" t="inlineStr">
         <is>
@@ -24771,7 +24807,7 @@
       </c>
       <c r="D76" s="120">
         <f>'Mass Transfer'!CO2_supply</f>
-        <v>0.0008495736750049</v>
+        <v>0.0008639935959385</v>
       </c>
       <c r="E76" s="140" t="s">
         <v>2129</v>
@@ -24912,7 +24948,7 @@
       </c>
       <c r="D84" s="41">
         <f>H2_src_l_b/(n_flamm_src+CO2_supply_b+F_dil_b)</f>
-        <v>0.093870758852</v>
+        <v>0.09257585106</v>
       </c>
       <c r="E84" s="53" t="s">
         <v>2154</v>
@@ -24930,7 +24966,7 @@
       </c>
       <c r="D85" s="41">
         <f>(O2_src_l_b+y_O2_air_b*F_vent_ex_b)/(n_flamm_src+CO2_supply_b+F_dil_b)</f>
-        <v>0.054287788176</v>
+        <v>0.053538910882</v>
       </c>
       <c r="E85" s="53" t="s">
         <v>2157</v>
@@ -25101,7 +25137,7 @@
       </c>
       <c r="D97" s="41">
         <f>'Mass Transfer'!C_cycle_start</f>
-        <v>25.434899746133</v>
+        <v>25.476094895404</v>
       </c>
       <c r="E97" s="51" t="s">
         <v>2185</v>
@@ -25119,7 +25155,7 @@
       </c>
       <c r="D98" s="41">
         <f>C_cycle_start_b*1000/Km_CO2</f>
-        <v>508.697994922664</v>
+        <v>509.521897908088</v>
       </c>
       <c r="E98" s="53" t="s">
         <v>2188</v>
@@ -25196,7 +25232,7 @@
       </c>
       <c r="D114" s="120">
         <f>'Mass Transfer'!y_H2_end_l</f>
-        <v>0.146419454972</v>
+        <v>0.14443867964</v>
       </c>
       <c r="E114" s="140" t="s">
         <v>2201</v>
@@ -25288,7 +25324,7 @@
       </c>
       <c r="D119" s="120">
         <f>'Mass Transfer'!y_O2_end_l</f>
-        <v>0.084678002539</v>
+        <v>0.083532471034</v>
       </c>
       <c r="E119" s="140" t="s">
         <v>2216</v>
@@ -25429,7 +25465,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:S565"/>
+  <dimension ref="A1:S568"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -25618,7 +25654,7 @@
       </c>
       <c r="D11" s="112">
         <f>Biology!O2_excess</f>
-        <v>1.691660977184e-05</v>
+        <v>1.705568716332e-05</v>
       </c>
       <c r="E11" s="105" t="str">
         <f>HYPERLINK("#Biology!D16","→ Biology")</f>
@@ -25658,7 +25694,7 @@
       </c>
       <c r="D13" s="120">
         <f>Electrochemistry!O2_net_gen</f>
-        <v>5.102798409848e-05</v>
+        <v>5.116706148996e-05</v>
       </c>
       <c r="E13" s="105" t="str">
         <f>HYPERLINK("#Electrochemistry!D29","→ Electrochemistry")</f>
@@ -26403,7 +26439,7 @@
       </c>
       <c r="D53" s="49">
         <f>kLa_sparge*duty</f>
-        <v>6.297870869563e-05</v>
+        <v>6.404765424633e-05</v>
       </c>
       <c r="E53" s="89" t="s">
         <v>581</v>
@@ -26443,7 +26479,7 @@
       </c>
       <c r="D55" s="41">
         <f>strip_sparge*duty</f>
-        <v>1.070393489225e-06</v>
+        <v>1.088561412663e-06</v>
       </c>
       <c r="E55" s="57" t="s">
         <v>587</v>
@@ -26462,7 +26498,7 @@
       </c>
       <c r="D56" s="39">
         <f>IF(O2_excess&gt;0,strip_avg/O2_excess,NA())</f>
-        <v>0.063274704782</v>
+        <v>0.063823955156</v>
       </c>
       <c r="E56" s="57" t="s">
         <v>590</v>
@@ -26481,7 +26517,7 @@
       </c>
       <c r="D57" s="41">
         <f>IF(O2_excess&gt;0,O2_excess/3600/((V_charge/1000000)*O2_ceil_C),NA())</f>
-        <v>0.0009953220471377</v>
+        <v>0.001003504939</v>
       </c>
       <c r="E57" s="57" t="inlineStr">
         <is>
@@ -26633,7 +26669,7 @@
       </c>
       <c r="D65" s="111">
         <f>IF(O2_excess&gt;0,O2_ceil_org*(V_charge/1000000)/O2_excess*60,"never (source &lt;= 0)")</f>
-        <v>16.744998982586</v>
+        <v>16.608455039407</v>
       </c>
       <c r="E65" s="74" t="s">
         <v>2232</v>
@@ -26651,11 +26687,13 @@
         <v>61</v>
       </c>
       <c r="D66" s="41">
-        <f>IF(O2_excess-strip_avg&gt;0,O2_ceil_org*(V_charge/1000000)/(O2_excess-strip_avg)*60,"never (strip ≥ source)")</f>
-        <v>17.876104198392</v>
-      </c>
-      <c r="E66" s="74" t="s">
-        <v>2233</v>
+        <f>IF(O2_excess-strip_avg*O2_ceil_org/O2_ceil_C&gt;0,O2_ceil_org*(V_charge/1000000)/(O2_excess-strip_avg*O2_ceil_org/O2_ceil_C)*60,"never (strip ≥ source)")</f>
+        <v>17.740739181348</v>
+      </c>
+      <c r="E66" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D65, crediting the time-averaged bubble strip at the organism ceiling’s driving force (D55 × D565/D6); "never" = strip ≥ source.</t>
+        </is>
       </c>
       <c r="F66" s="21"/>
     </row>
@@ -26806,7 +26844,7 @@
       </c>
       <c r="D74" s="41">
         <f>IF(O2_excess&gt;0,surf_strip/O2_excess,NA())</f>
-        <v>7.676447552252</v>
+        <v>7.613851405219</v>
       </c>
       <c r="E74" s="53" t="s">
         <v>635</v>
@@ -26841,7 +26879,7 @@
       </c>
       <c r="D77" s="41">
         <f>headspace_V*spg_int/V_pulse</f>
-        <v>7.416849456371</v>
+        <v>7.29306337365</v>
       </c>
       <c r="E77" s="74" t="s">
         <v>2236</v>
@@ -26860,7 +26898,7 @@
       </c>
       <c r="D78" s="41">
         <f>IF(O2_excess&gt;0,(strip_avg+surf_strip)/O2_excess,NA())</f>
-        <v>7.739722257034</v>
+        <v>7.677675360374</v>
       </c>
       <c r="E78" s="90" t="s">
         <v>640</v>
@@ -26878,11 +26916,13 @@
         <v>61</v>
       </c>
       <c r="D79" s="41">
-        <f>O2_ceil_org*(V_charge/1000000)/O2_net_gen*60</f>
-        <v>5.551240528561</v>
-      </c>
-      <c r="E79" s="74" t="s">
-        <v>643</v>
+        <f>O2_ceil_org*(V_charge/1000000)/O2_net_lag_mt*60</f>
+        <v>5.854318892931</v>
+      </c>
+      <c r="E79" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lag/establishment: no biological O₂ uptake yet, so the whole lag O₂ source (D394) accumulates up to the organism ceiling (D565). Worst case.</t>
+        </is>
       </c>
       <c r="F79" s="21"/>
     </row>
@@ -26897,11 +26937,13 @@
         <v>61</v>
       </c>
       <c r="D80" s="41" t="str">
-        <f>IF(O2_net_gen-strip_avg-surf_strip&gt;0,O2_ceil_org*(V_charge/1000000)/(O2_net_gen-strip_avg-surf_strip)*60,"never (removal ≥ source)")</f>
+        <f>IF(O2_net_lag_mt-(strip_avg+surf_strip)*O2_ceil_org/O2_ceil_C&gt;0,O2_ceil_org*(V_charge/1000000)/(O2_net_lag_mt-(strip_avg+surf_strip)*O2_ceil_org/O2_ceil_C)*60,"never (removal ≥ source)")</f>
         <v>never (removal ≥ source)</v>
       </c>
-      <c r="E80" s="53" t="s">
-        <v>2237</v>
+      <c r="E80" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Companion to D79 crediting both removal paths at the organism ceiling’s driving force (D55 and D73 scaled by D565/D6), on the lag source.</t>
+        </is>
       </c>
       <c r="F80" s="21"/>
     </row>
@@ -27033,7 +27075,7 @@
       </c>
       <c r="D87" s="41">
         <f>O2_src_guard/(target_DO_frac*(O2_ceil_Pa/P_atm))/(nCO2_rate*3600)</f>
-        <v>0.001561133561</v>
+        <v>0.001565388449</v>
       </c>
       <c r="E87" s="74" t="s">
         <v>965</v>
@@ -27052,7 +27094,7 @@
       </c>
       <c r="D88" s="41">
         <f>MAX(duty_carbon,duty_O2vent)</f>
-        <v>0.001561133561</v>
+        <v>0.001565388449</v>
       </c>
       <c r="E88" s="53" t="s">
         <v>2239</v>
@@ -27071,7 +27113,7 @@
       </c>
       <c r="D89" s="41">
         <f>target_DO_frac*O2_ceil_org*(V_charge/1000000)/O2_src_guard*60</f>
-        <v>1.255063076022</v>
+        <v>1.251651684129</v>
       </c>
       <c r="E89" s="74" t="s">
         <v>2241</v>
@@ -27109,7 +27151,7 @@
       </c>
       <c r="D91" s="41">
         <f>IF(ISNA(F_vent_ex+O2_src_sched),NA(),IF(ph_unreach,NA(),MIN(spg_int_carbon,IF(ISNUMBER(spg_int_DO),spg_int_DO,spg_int_max),IF(ISNUMBER(spg_int_pH_opt),spg_int_pH_opt,spg_int_carbon),IF(O2_sizing_phase=phase_name_2,IF(ISNUMBER(spg_int_H2safe_opt),spg_int_H2safe_opt,spg_int_carbon),spg_int_carbon))))</f>
-        <v>7.421902768325</v>
+        <v>7.293500622657</v>
       </c>
       <c r="E91" s="129" t="inlineStr">
         <is>
@@ -27130,7 +27172,7 @@
       </c>
       <c r="D92" s="41">
         <f>spg_int_opt*60</f>
-        <v>445.314166099472</v>
+        <v>437.610037359391</v>
       </c>
       <c r="E92" s="129" t="s">
         <v>672</v>
@@ -27149,7 +27191,7 @@
       </c>
       <c r="D93" s="41">
         <f>spg_dur_eq_opt/(spg_int_opt*60)</f>
-        <v>0.001761706924</v>
+        <v>0.001792721791</v>
       </c>
       <c r="E93" s="74" t="s">
         <v>2245</v>
@@ -27282,7 +27324,7 @@
       </c>
       <c r="D100" s="25">
         <f>CO2_pulse*pulses_h</f>
-        <v>0.0008495736750049</v>
+        <v>0.0008639935959385</v>
       </c>
       <c r="E100" s="102" t="s">
         <v>688</v>
@@ -27377,7 +27419,7 @@
       </c>
       <c r="D105" s="25">
         <f>spg_dur/(spg_int*60)</f>
-        <v>0.001506722299</v>
+        <v>0.001532296087</v>
       </c>
       <c r="E105" s="102" t="s">
         <v>688</v>
@@ -27424,7 +27466,7 @@
       </c>
       <c r="D108" s="25">
         <f>DO_avg_sched*M_O2</f>
-        <v>2.274565106296</v>
+        <v>2.275287892306</v>
       </c>
       <c r="E108" s="102" t="inlineStr">
         <is>
@@ -27509,7 +27551,7 @@
       <c r="C113" s="21"/>
       <c r="D113" s="25" t="str">
         <f>IF(DO_at_carbon&lt;=DO_target,"Carbon supply alone holds the DO target – the interval may relax to "&amp;TEXT(MIN(spg_int_carbon,IF(ISNUMBER(spg_int_pH_opt),spg_int_pH_opt,spg_int_carbon)),"0")&amp;" min","Do NOT relax: at the carbon-limited interval ("&amp;TEXT(spg_int_carbon,"0")&amp;" min) the cycle-mean DO would be ≈"&amp;TEXT(DO_at_carbon*M_O2,"0")&amp;" mg/L, "&amp;IF(DO_at_carbon&gt;O2_ceil_org,"above the "&amp;TEXT(O2_ceil_org*M_O2,"0.0")&amp;" mg/L inhibition ceiling","against a "&amp;TEXT(DO_target*M_O2,"0.0")&amp;" mg/L target")&amp;" (peaks higher)")</f>
-        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈13 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
+        <v>Do NOT relax: at the carbon-limited interval (185 min) the cycle-mean DO would be ≈14 mg/L, above the 10.1 mg/L inhibition ceiling (peaks higher)</v>
       </c>
       <c r="E113" s="59" t="s">
         <v>2249</v>
@@ -27673,7 +27715,7 @@
       </c>
       <c r="D122" s="111">
         <f>IF(AND(ISNUMBER(override_spg_int_min),override_spg_int_min&gt;0),IF(override_spg_int_min*60&gt;spg_dur,override_spg_int_min,NA()),IF(sched_mode="Manual",IF(spg_int_man*60&gt;spg_dur,spg_int_man,NA()),IF(sched_mode="Optimal",spg_int_run,NA())))</f>
-        <v>7.19</v>
+        <v>7.07</v>
       </c>
       <c r="E122" s="51" t="inlineStr">
         <is>
@@ -27713,7 +27755,7 @@
       </c>
       <c r="D124" s="25">
         <f>60/spg_int</f>
-        <v>8.344923504868</v>
+        <v>8.486562942008</v>
       </c>
       <c r="E124" s="51" t="inlineStr">
         <is>
@@ -27734,7 +27776,7 @@
       </c>
       <c r="D125" s="25">
         <f>pulses_h*24</f>
-        <v>200.278164116829</v>
+        <v>203.677510608204</v>
       </c>
       <c r="E125" s="51" t="inlineStr">
         <is>
@@ -27755,7 +27797,7 @@
       </c>
       <c r="D126" s="25">
         <f>IF(CO2_cons&gt;0,CO2_supply/CO2_cons,NA())</f>
-        <v>49.811752928483</v>
+        <v>50.657214081442</v>
       </c>
       <c r="E126" s="51" t="inlineStr">
         <is>
@@ -27776,7 +27818,7 @@
       </c>
       <c r="D127" s="25">
         <f>O2_excess/60*spg_int</f>
-        <v>2.027173737658e-06</v>
+        <v>2.009728470745e-06</v>
       </c>
       <c r="E127" s="51" t="inlineStr">
         <is>
@@ -27818,7 +27860,7 @@
       </c>
       <c r="D129" s="25">
         <f>IF(O2_accum&gt;0,O2_strip_pulse/O2_accum,NA())</f>
-        <v>0.063274704782</v>
+        <v>0.063823955156</v>
       </c>
       <c r="E129" s="51" t="inlineStr">
         <is>
@@ -27858,7 +27900,7 @@
       </c>
       <c r="D131" s="25">
         <f>kLa_surf_req/a_surf</f>
-        <v>0.0001537333008672</v>
+        <v>0.0001549971963378</v>
       </c>
       <c r="E131" s="117" t="s">
         <v>1637</v>
@@ -27877,7 +27919,7 @@
       </c>
       <c r="D132" s="25">
         <f>O2_net_gen</f>
-        <v>5.102798409848e-05</v>
+        <v>5.116706148996e-05</v>
       </c>
       <c r="E132" s="53" t="s">
         <v>902</v>
@@ -27896,7 +27938,7 @@
       </c>
       <c r="D133" s="25">
         <f>DO_avg_sched</f>
-        <v>0.071084602359</v>
+        <v>0.071107190834</v>
       </c>
       <c r="E133" s="53" t="s">
         <v>2256</v>
@@ -27915,7 +27957,7 @@
       </c>
       <c r="D134" s="25" t="str">
         <f>IF(ISNA(F_vent_ex+O2_src_sched),"INVALID SELECTOR (check Summary D2–D5, D11, D12) – no schedule until both are listed values",IF(NOT(ISNUMBER(spg_int_DO)),"DO TARGET UNREACHABLE — the surface cannot carry the O2 flux at this kLa; no interval fixes it (raise kL_surf, lower the current, or accept a higher DO)",IF(kLa_meas&gt;0,"MEASURED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min","ESTIMATED kLa — DO-limited interval is "&amp;TEXT(spg_int_DO,"0.0")&amp;" min; confirm by measuring kL_surf")))</f>
-        <v>ESTIMATED kLa — DO-limited interval is 7.4 min; confirm by measuring kL_surf</v>
+        <v>ESTIMATED kLa — DO-limited interval is 7.3 min; confirm by measuring kL_surf</v>
       </c>
       <c r="E134" s="53" t="s">
         <v>2257</v>
@@ -27934,7 +27976,7 @@
       </c>
       <c r="D135" s="25">
         <f>DO_avg_l</f>
-        <v>0.176285196499</v>
+        <v>0.175470883498</v>
       </c>
       <c r="E135" s="53" t="s">
         <v>2259</v>
@@ -28233,7 +28275,7 @@
       </c>
       <c r="D152" s="41">
         <f>MAX(0,spg_int*60-spg_dur)</f>
-        <v>430.75</v>
+        <v>423.55</v>
       </c>
       <c r="E152" s="51" t="s">
         <v>1078</v>
@@ -28324,7 +28366,7 @@
       </c>
       <c r="D162" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,CO2_cyc_avg_new))/1000</f>
-        <v>0.02555602506</v>
+        <v>0.025595318383</v>
       </c>
       <c r="E162" s="51" t="s">
         <v>1661</v>
@@ -28580,7 +28622,7 @@
       </c>
       <c r="D180" s="111">
         <f>O2_src_sched/(kLa_surf_used*3600*(V_charge/1000000))</f>
-        <v>0.041001114338</v>
+        <v>0.041338198902</v>
       </c>
       <c r="E180" s="51" t="s">
         <v>2272</v>
@@ -28616,7 +28658,7 @@
       </c>
       <c r="D182" s="111">
         <f>DO_target-DO_surf_excess</f>
-        <v>0.030158150869</v>
+        <v>0.029821066305</v>
       </c>
       <c r="E182" s="51" t="s">
         <v>1622</v>
@@ -28634,7 +28676,7 @@
       </c>
       <c r="D183" s="111">
         <f>IF(hs_O2_allow&gt;0,hs_O2_allow/(H_O2_T*P_dry),NA())</f>
-        <v>0.029999879484</v>
+        <v>0.029664563955</v>
       </c>
       <c r="E183" s="51" t="s">
         <v>1625</v>
@@ -28652,7 +28694,7 @@
       </c>
       <c r="D184" s="111">
         <f>IF(ISNUMBER(y_O2_star),MAX(0,((O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_dil-O2_src_sched-H2_src_sched+CO2_fix_sched)/CO2_rate_full),NA())</f>
-        <v>0.001761706924</v>
+        <v>0.001792721791</v>
       </c>
       <c r="E184" s="51" t="s">
         <v>2274</v>
@@ -28670,7 +28712,7 @@
       </c>
       <c r="D185" s="111">
         <f>IF(ISNUMBER(duty_DO),IF(duty_DO&gt;0,spg_dur_eq_opt/(60*duty_DO),spg_int_carbon),NA())</f>
-        <v>7.421902768325</v>
+        <v>7.293500622657</v>
       </c>
       <c r="E185" s="51" t="s">
         <v>1630</v>
@@ -28688,7 +28730,7 @@
       </c>
       <c r="D186" s="111">
         <f>O2_src_sched/(DO_target*3600*(V_charge/1000000))</f>
-        <v>0.004402385978</v>
+        <v>0.004438579539</v>
       </c>
       <c r="E186" s="51" t="inlineStr">
         <is>
@@ -28708,7 +28750,7 @@
       </c>
       <c r="D187" s="111">
         <f>IF(O2_sizing_phase=phase_name_1,y_O2_mf_g,IF(O2_sizing_phase=phase_name_2,y_O2_mf_l,NA()))</f>
-        <v>0.02766022792</v>
+        <v>0.027367364576</v>
       </c>
       <c r="E187" s="51" t="s">
         <v>2276</v>
@@ -28726,7 +28768,7 @@
       </c>
       <c r="D188" s="111">
         <f>IF(ISNUMBER(y_O2_actual),H_O2_T*y_O2_actual*P_dry,NA())</f>
-        <v>0.027806155925</v>
+        <v>0.027511747512</v>
       </c>
       <c r="E188" s="51" t="s">
         <v>2277</v>
@@ -28857,7 +28899,7 @@
       </c>
       <c r="D197" s="111">
         <f>EXP(-k_eff_CO2*t_off_CO2)</f>
-        <v>0.9937646449</v>
+        <v>0.993868548876</v>
       </c>
       <c r="E197" s="74" t="s">
         <v>1654</v>
@@ -28875,7 +28917,7 @@
       </c>
       <c r="D198" s="111">
         <f>(pool_D_gap+pool_b*pool_e)/(1-pool_ret*pool_e)</f>
-        <v>25.434899746133</v>
+        <v>25.476094895404</v>
       </c>
       <c r="E198" s="74" t="s">
         <v>2284</v>
@@ -28893,7 +28935,7 @@
       </c>
       <c r="D199" s="111">
         <f>pool_ret*C_cycle_start+pool_b</f>
-        <v>25.677403179348</v>
+        <v>25.714786542723</v>
       </c>
       <c r="E199" s="74" t="s">
         <v>2285</v>
@@ -28911,7 +28953,7 @@
       </c>
       <c r="D200" s="111">
         <f>C_cycle_peak*pool_phi+pool_D_raw*pool_psi</f>
-        <v>25.556025060412</v>
+        <v>25.595318383194</v>
       </c>
       <c r="E200" s="74" t="s">
         <v>2286</v>
@@ -29151,7 +29193,7 @@
       </c>
       <c r="D232" s="111">
         <f>IF(F_dil+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,DO_surf_excess+H_O2_T*P_dry*MIN(1,saw_factor*(O2_src_sched+y_O2_air*F_vent_ex)/(F_dil+CO2_rate_full*duty_carbon+O2_src_sched+H2_src_sched-CO2_fix_sched)),DO_surf_excess+H_O2_T*P_dry)</f>
-        <v>0.421474597871</v>
+        <v>0.423214741433</v>
       </c>
       <c r="E232" s="74" t="s">
         <v>2311</v>
@@ -29362,7 +29404,7 @@
       </c>
       <c r="D309" s="41">
         <f>O2_excess</f>
-        <v>1.691660977184e-05</v>
+        <v>1.705568716332e-05</v>
       </c>
       <c r="E309" s="51" t="s">
         <v>2349</v>
@@ -29505,7 +29547,7 @@
       </c>
       <c r="D317" s="41">
         <f>IF(O2_sizing_phase=phase_name_1,O2_src_g,IF(O2_sizing_phase=phase_name_2,O2_src_l,NA()))</f>
-        <v>1.691660977184e-05</v>
+        <v>1.705568716332e-05</v>
       </c>
       <c r="E317" s="51" t="s">
         <v>2370</v>
@@ -29655,7 +29697,7 @@
       </c>
       <c r="D325" s="41">
         <f>t_off_CO2/3600</f>
-        <v>0.119652777778</v>
+        <v>0.117652777778</v>
       </c>
       <c r="E325" s="51" t="s">
         <v>2394</v>
@@ -29691,7 +29733,7 @@
       </c>
       <c r="D327" s="41">
         <f>O2_src_g+y_O2_air*F_vent_ex</f>
-        <v>2.449629885807e-05</v>
+        <v>2.463537624956e-05</v>
       </c>
       <c r="E327" s="51" t="s">
         <v>2400</v>
@@ -29709,7 +29751,7 @@
       </c>
       <c r="D328" s="41">
         <f>CO2_supply+O2_src_g+H2_src_g-CO2_fix_g</f>
-        <v>0.0008494345976134</v>
+        <v>0.0008639935959385</v>
       </c>
       <c r="E328" s="51" t="s">
         <v>2403</v>
@@ -29727,7 +29769,7 @@
       </c>
       <c r="D329" s="41">
         <f>IF(F_dil+F_hs_net_g&gt;0,S_O2_g/(F_dil+F_hs_net_g),NA())</f>
-        <v>0.02766022792</v>
+        <v>0.027367364576</v>
       </c>
       <c r="E329" s="51" t="s">
         <v>2406</v>
@@ -29781,7 +29823,7 @@
       </c>
       <c r="D332" s="41">
         <f>F_gap_g*t_gap_h/n_hs_gas</f>
-        <v>0.043019997644</v>
+        <v>0.04230091701</v>
       </c>
       <c r="E332" s="51" t="s">
         <v>2415</v>
@@ -29799,7 +29841,7 @@
       </c>
       <c r="D333" s="41">
         <f>IF(x_hs_g&gt;0,(1-EXP(-x_hs_g))/x_hs_g,1)</f>
-        <v>0.978795165468</v>
+        <v>0.979144642091</v>
       </c>
       <c r="E333" s="51" t="s">
         <v>2418</v>
@@ -29817,7 +29859,7 @@
       </c>
       <c r="D334" s="41">
         <f>IF(x_hs_g&gt;0,(x_hs_g-1+EXP(-x_hs_g))/x_hs_g^2,1/2)</f>
-        <v>0.492906454979</v>
+        <v>0.493023777802</v>
       </c>
       <c r="E334" s="51" t="s">
         <v>2421</v>
@@ -29835,7 +29877,7 @@
       </c>
       <c r="D335" s="41">
         <f>S_O2_g*t_gap_h/n_hs_gas</f>
-        <v>0.029127518709</v>
+        <v>0.028803258198</v>
       </c>
       <c r="E335" s="51" t="s">
         <v>2424</v>
@@ -29853,7 +29895,7 @@
       </c>
       <c r="D336" s="41">
         <f>dy_O2_g*phi_hs_g/(1-flush_ret*EXP(-x_hs_g))</f>
-        <v>0.043745864279</v>
+        <v>0.043290953345</v>
       </c>
       <c r="E336" s="52" t="s">
         <v>2427</v>
@@ -29871,7 +29913,7 @@
       </c>
       <c r="D337" s="41">
         <f>y_O2_end_g*flush_ret</f>
-        <v>0.015905745177</v>
+        <v>0.015740342172</v>
       </c>
       <c r="E337" s="52" t="s">
         <v>2430</v>
@@ -29889,7 +29931,7 @@
       </c>
       <c r="D338" s="41">
         <f>y_O2_post_g*phi_hs_g+dy_O2_g*psi_hs_g</f>
-        <v>0.029925608471</v>
+        <v>0.029612762872</v>
       </c>
       <c r="E338" s="52" t="s">
         <v>2433</v>
@@ -29907,7 +29949,7 @@
       </c>
       <c r="D339" s="41">
         <f>O2_src_g/(kLa_surf_used*3600*V_L_m3)</f>
-        <v>0.041001114338</v>
+        <v>0.041338198902</v>
       </c>
       <c r="E339" s="51" t="s">
         <v>2436</v>
@@ -29925,7 +29967,7 @@
       </c>
       <c r="D340" s="41">
         <f>DO_surf_excess_g+H_O2_T*P_dry*y_O2_mf_g</f>
-        <v>0.068807270263</v>
+        <v>0.068849946414</v>
       </c>
       <c r="E340" s="51" t="s">
         <v>2439</v>
@@ -29943,7 +29985,7 @@
       </c>
       <c r="D341" s="41">
         <f>DO_surf_excess_g+H_O2_T*P_dry*y_O2_avg_g</f>
-        <v>0.071084602359</v>
+        <v>0.071107190834</v>
       </c>
       <c r="E341" s="52" t="s">
         <v>2442</v>
@@ -29960,11 +30002,13 @@
         <v>406</v>
       </c>
       <c r="D342" s="41">
-        <f>DO_surf_excess_g+H_O2_T*P_dry*MAX(y_O2_avg_g,y_O2_end_g-(S_O2_g-F_gap_g*y_O2_end_g)/n_hs_gas*tau_L_h)</f>
-        <v>0.076655689366</v>
-      </c>
-      <c r="E342" s="52" t="s">
-        <v>2445</v>
+        <f>DO_surf_excess_g+H_O2_T*P_dry*z_peak_g</f>
+        <v>0.07751644174</v>
+      </c>
+      <c r="E342" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid DO just before a pulse: the surface excess plus equilibrium with the liquid’s own peak (D566, exact for a first-order liquid following the headspace sawtooth).</t>
+        </is>
       </c>
     </row>
     <row r="343" spans="1:5" x14ac:dyDescent="0.2">
@@ -29979,7 +30023,7 @@
       </c>
       <c r="D343" s="41">
         <f>DO_avg_g*M_O2</f>
-        <v>2.274565106296</v>
+        <v>2.275287892306</v>
       </c>
       <c r="E343" s="52" t="s">
         <v>2448</v>
@@ -29997,7 +30041,7 @@
       </c>
       <c r="D344" s="41">
         <f>DO_peak_g*M_O2</f>
-        <v>2.452828748339</v>
+        <v>2.480371102791</v>
       </c>
       <c r="E344" s="52" t="s">
         <v>2448</v>
@@ -30015,7 +30059,7 @@
       </c>
       <c r="D345" s="41">
         <f>O2_src_g/(DO_target*3600*V_L_m3)</f>
-        <v>0.004402385978</v>
+        <v>0.004438579539</v>
       </c>
       <c r="E345" s="51" t="s">
         <v>2453</v>
@@ -30033,7 +30077,7 @@
       </c>
       <c r="D346" s="111">
         <f>IF(kLa_surf_req_g&gt;0,kLa_surf_used/kLa_surf_req_g,"no positive source")</f>
-        <v>1.735544663987</v>
+        <v>1.721392491615</v>
       </c>
       <c r="E346" s="51" t="s">
         <v>2456</v>
@@ -30051,7 +30095,7 @@
       </c>
       <c r="D347" s="111" t="str">
         <f>IF(kLa_surf_req_g&lt;=0,"No positive biological O2 surplus; check air ingress and operating DO",IF(kLa_margin_g&gt;=1,"reachable – kLa margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"×","UNREACHABLE at this surface kLa – margin "&amp;TEXT(kLa_margin_g,"0.00")&amp;"× (raise kL_surf, lower the current, or accept a higher DO)"))</f>
-        <v>reachable – kLa margin 1.74×</v>
+        <v>reachable – kLa margin 1.72×</v>
       </c>
       <c r="E347" s="51" t="s">
         <v>2458</v>
@@ -30107,7 +30151,7 @@
       </c>
       <c r="D350" s="41">
         <f>CO2_supply+O2_src_l+H2_src_l-CO2_fix_l</f>
-        <v>0.0009947324638916</v>
+        <v>0.001009152385</v>
       </c>
       <c r="E350" s="51" t="s">
         <v>2403</v>
@@ -30125,7 +30169,7 @@
       </c>
       <c r="D351" s="41">
         <f>IF(F_dil+F_hs_net_l&gt;0,S_O2_l/(F_dil+F_hs_net_l),NA())</f>
-        <v>0.054287788176</v>
+        <v>0.053538910882</v>
       </c>
       <c r="E351" s="51" t="s">
         <v>2406</v>
@@ -30143,7 +30187,7 @@
       </c>
       <c r="D352" s="41">
         <f>IF(F_dil+F_hs_net_l&gt;0,H2_src_l/(F_dil+F_hs_net_l),NA())</f>
-        <v>0.093870758852</v>
+        <v>0.09257585106</v>
       </c>
       <c r="E352" s="51" t="s">
         <v>2409</v>
@@ -30179,7 +30223,7 @@
       </c>
       <c r="D354" s="41">
         <f>F_gap_l*t_gap_h/n_hs_gas</f>
-        <v>0.215622208431</v>
+        <v>0.212018076334</v>
       </c>
       <c r="E354" s="51" t="s">
         <v>2415</v>
@@ -30197,7 +30241,7 @@
       </c>
       <c r="D355" s="41">
         <f>IF(x_hs_l&gt;0,(1-EXP(-x_hs_l))/x_hs_l,1)</f>
-        <v>0.899537399356</v>
+        <v>0.901102060357</v>
       </c>
       <c r="E355" s="51" t="s">
         <v>2418</v>
@@ -30215,7 +30259,7 @@
       </c>
       <c r="D356" s="41">
         <f>IF(x_hs_l&gt;0,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2)</f>
-        <v>0.465919542215</v>
+        <v>0.466459942253</v>
       </c>
       <c r="E356" s="51" t="s">
         <v>2421</v>
@@ -30233,7 +30277,7 @@
       </c>
       <c r="D357" s="41">
         <f>S_O2_l*t_gap_h/n_hs_gas</f>
-        <v>0.066546759769</v>
+        <v>0.065434428555</v>
       </c>
       <c r="E357" s="51" t="s">
         <v>2424</v>
@@ -30251,7 +30295,7 @@
       </c>
       <c r="D358" s="41">
         <f>dy_O2_l*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.084678002539</v>
+        <v>0.083532471034</v>
       </c>
       <c r="E358" s="52" t="s">
         <v>2427</v>
@@ -30269,7 +30313,7 @@
       </c>
       <c r="D359" s="41">
         <f>y_O2_end_l*flush_ret</f>
-        <v>0.030788435722</v>
+        <v>0.030371927041</v>
       </c>
       <c r="E359" s="52" t="s">
         <v>2430</v>
@@ -30287,7 +30331,7 @@
       </c>
       <c r="D360" s="41">
         <f>y_O2_post_l*phi_hs_l+dy_O2_l*psi_hs_l</f>
-        <v>0.058700785247</v>
+        <v>0.057890745799</v>
       </c>
       <c r="E360" s="52" t="s">
         <v>2433</v>
@@ -30305,7 +30349,7 @@
       </c>
       <c r="D361" s="41">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_mf_l</f>
-        <v>0.171848917629</v>
+        <v>0.171096089458</v>
       </c>
       <c r="E361" s="51" t="s">
         <v>2439</v>
@@ -30323,7 +30367,7 @@
       </c>
       <c r="D362" s="41">
         <f>DO_surf_excess_lag+H_O2_T*P_dry*y_O2_avg_l</f>
-        <v>0.176285196499</v>
+        <v>0.175470883498</v>
       </c>
       <c r="E362" s="52" t="s">
         <v>2442</v>
@@ -30340,11 +30384,13 @@
         <v>406</v>
       </c>
       <c r="D363" s="41">
-        <f>DO_surf_excess_lag+H_O2_T*P_dry*MAX(y_O2_avg_l,y_O2_end_l-(S_O2_l-F_gap_l*y_O2_end_l)/n_hs_gas*tau_L_h)</f>
-        <v>0.187649941052</v>
-      </c>
-      <c r="E363" s="52" t="s">
-        <v>2445</v>
+        <f>DO_surf_excess_lag+H_O2_T*P_dry*z_peak_l</f>
+        <v>0.187723903393</v>
+      </c>
+      <c r="E363" s="52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D342 on the lag phase (D567).</t>
+        </is>
       </c>
     </row>
     <row r="364" spans="1:5" x14ac:dyDescent="0.2">
@@ -30359,7 +30405,7 @@
       </c>
       <c r="D364" s="41">
         <f>DO_avg_l*M_O2</f>
-        <v>5.640773717562</v>
+        <v>5.614717330178</v>
       </c>
       <c r="E364" s="52" t="s">
         <v>2448</v>
@@ -30377,7 +30423,7 @@
       </c>
       <c r="D365" s="41">
         <f>DO_peak_l*M_O2</f>
-        <v>6.004422813773</v>
+        <v>6.006789460768</v>
       </c>
       <c r="E365" s="52" t="s">
         <v>2448</v>
@@ -30487,7 +30533,7 @@
       </c>
       <c r="D372" s="41">
         <f>IF(O2_sizing_phase=phase_name_1,DO_avg_g,IF(O2_sizing_phase=phase_name_2,DO_avg_l,NA()))</f>
-        <v>0.071084602359</v>
+        <v>0.071107190834</v>
       </c>
       <c r="E372" s="52" t="s">
         <v>2508</v>
@@ -30505,7 +30551,7 @@
       </c>
       <c r="D373" s="41">
         <f>IF(O2_sizing_phase=phase_name_1,DO_peak_g,IF(O2_sizing_phase=phase_name_2,DO_peak_l,NA()))</f>
-        <v>0.076655689366</v>
+        <v>0.07751644174</v>
       </c>
       <c r="E373" s="52" t="inlineStr">
         <is>
@@ -30543,7 +30589,7 @@
       </c>
       <c r="D375" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*t_gap_h/(V_L_CO2+Vg_CO2)</f>
-        <v>-0.082653662444</v>
+        <v>-0.081272103837</v>
       </c>
       <c r="E375" s="51" t="s">
         <v>2517</v>
@@ -30561,7 +30607,7 @@
       </c>
       <c r="D376" s="41">
         <f>k_eff_CO2*t_off_CO2</f>
-        <v>0.006254876116</v>
+        <v>0.006150325662</v>
       </c>
       <c r="E376" s="51" t="s">
         <v>2520</v>
@@ -30579,7 +30625,7 @@
       </c>
       <c r="D377" s="41">
         <f>IF(pool_x&gt;0,(1-EXP(-pool_x))/pool_x,1)</f>
-        <v>0.996879072338</v>
+        <v>0.996931131905</v>
       </c>
       <c r="E377" s="51" t="s">
         <v>2523</v>
@@ -30597,7 +30643,7 @@
       </c>
       <c r="D378" s="41">
         <f>IF(pool_x&gt;0,(pool_x-1+EXP(-pool_x))/pool_x^2,1/2)</f>
-        <v>0.498959148754</v>
+        <v>0.498976519889</v>
       </c>
       <c r="E378" s="51" t="s">
         <v>2526</v>
@@ -30615,7 +30661,7 @@
       </c>
       <c r="D379" s="41">
         <f>pool_D_raw*pool_phi</f>
-        <v>-0.082395706342</v>
+        <v>-0.081022690471</v>
       </c>
       <c r="E379" s="51" t="s">
         <v>2529</v>
@@ -30651,7 +30697,7 @@
       </c>
       <c r="D381" s="111">
         <f>IF(F_dil+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched&gt;0,(CO2_supply-CO2_fix_sched+pCO2_air/P_dry*F_vent_ex)/(F_dil+CO2_supply+O2_src_sched+H2_src_sched-CO2_fix_sched),NA())</f>
-        <v>0.940062404006</v>
+        <v>0.940877306879</v>
       </c>
       <c r="E381" s="51" t="s">
         <v>2535</v>
@@ -30669,7 +30715,7 @@
       </c>
       <c r="D382" s="41">
         <f>y_CO2_mf*C_sat_CO2</f>
-        <v>26.374117589172</v>
+        <v>26.396980267336</v>
       </c>
       <c r="E382" s="51" t="s">
         <v>2538</v>
@@ -30764,7 +30810,7 @@
       </c>
       <c r="D388" s="41">
         <f>H2_src_l*t_gap_h/n_hs_gas*phi_hs_l/(1-flush_ret*EXP(-x_hs_l))</f>
-        <v>0.146419454972</v>
+        <v>0.14443867964</v>
       </c>
       <c r="E388" s="52" t="inlineStr">
         <is>
@@ -30784,7 +30830,7 @@
       </c>
       <c r="D389" s="41">
         <f>(pool_a*(C_cycle_peak-C_cycle_start)*(V_L_CO2+Vg_CO2)+MAX(0,CO2_fix_sched-O2_src_sched-H2_src_sched)*t_gap_h)/n_hs_gas</f>
-        <v>0.05097124556</v>
+        <v>0.05000728325</v>
       </c>
       <c r="E389" s="52" t="s">
         <v>2556</v>
@@ -31218,7 +31264,7 @@
       </c>
       <c r="D417" s="25">
         <f>IF(CO2_cons&gt;0,(C_cycle_peak-C_cycle_start)*V_L_CO2*pulses_h/CO2_cons,NA())</f>
-        <v>2.501421260187</v>
+        <v>2.503892293977</v>
       </c>
       <c r="E417" s="102" t="s">
         <v>2626</v>
@@ -31285,7 +31331,7 @@
       </c>
       <c r="D420" s="111">
         <f>IF(FLOOR((pulse_V0+Q_CO2_fit*spg_dur)/(Q_CO2/60)/(60*duty_actual),interval_res)*60&gt;spg_dur,FLOOR((pulse_V0+Q_CO2_fit*spg_dur)/(Q_CO2/60)/(60*duty_actual),interval_res),NA())</f>
-        <v>7.19</v>
+        <v>7.07</v>
       </c>
       <c r="E420" s="57" t="inlineStr">
         <is>
@@ -31396,7 +31442,7 @@
       </c>
       <c r="D426" s="41">
         <f>IF(ISNUMBER(y_O2_star),MAX(0,(O2_src_sched+y_O2_air*F_vent_ex)*saw_factor/y_O2_star-F_vent_ex-O2_src_sched-H2_src_sched+CO2_fix_sched-CO2_rate_full*duty_carbon)/3600*R_gas*T_K/P_atm*1000000*60,NA())</f>
-        <v>0.337846643585</v>
+        <v>0.344043413938</v>
       </c>
       <c r="E426" s="51" t="inlineStr">
         <is>
@@ -39239,7 +39285,7 @@
       </c>
       <c r="D546" s="41">
         <f>IF(ph_unreach_l,NA(),MIN(spg_int_carbon,IF(ISNUMBER(spg_int_DO_l),spg_int_DO_l,spg_int_max),IF(ISNUMBER(spg_int_H2safe_opt),spg_int_H2safe_opt,spg_int_carbon),IF(ISNUMBER(spg_int_pH_l),spg_int_pH_l*spg_dur_eq_opt/spg_dur_eq,spg_int_carbon)))</f>
-        <v>1.255063076022</v>
+        <v>1.251651684129</v>
       </c>
       <c r="E546" s="51" t="inlineStr">
         <is>
@@ -39524,12 +39570,12 @@
         </is>
       </c>
       <c r="D557" s="41">
-        <f>(DO_surf_excess_lag+H_O2_T*P_dry*MAX(y_O2_avg_su,y_O2_end_su-(S_O2_l-F_gap_l*y_O2_end_su)/n_hs_gas*tau_L_h))*M_O2</f>
-        <v>4.122375525019</v>
+        <f>(DO_surf_excess_lag+H_O2_T*P_dry*z_peak_su)*M_O2</f>
+        <v>4.13806097293</v>
       </c>
       <c r="E557" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">As D365 at the start-up interval.</t>
+          <t xml:space="preserve">As D365 at the start-up interval (D568).</t>
         </is>
       </c>
     </row>
@@ -39681,7 +39727,7 @@
       </c>
       <c r="D564" s="41">
         <f>y_H2_end_l*flush_ret*phi_hs_l+H2_src_l*t_gap_h/n_hs_gas*psi_hs_l</f>
-        <v>0.10150141388</v>
+        <v>0.100100748644</v>
       </c>
       <c r="E564" s="51" t="inlineStr">
         <is>
@@ -39712,6 +39758,84 @@
       <c r="E565" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">The organism’s own toxic DO (Biology D48, measured or tabled) when it has one, never above the generic 0.30 atm Henry ceiling (D6); otherwise that generic ceiling. Used by the DO target, the legacy guard and the peak checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid-equilibrium O₂ fraction at its peak — growth</t>
+        </is>
+      </c>
+      <c r="B566" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z_peak_g</t>
+        </is>
+      </c>
+      <c r="C566" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D566" s="41">
+        <f>IF(F_gap_g&gt;0,S_O2_g/F_gap_g+(y_O2_post_g-S_O2_g/F_gap_g)*IF(ABS((1/tau_L_h)-(F_gap_g/n_hs_gas))&gt;1E-9*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_g/n_hs_gas))*(EXP(-(F_gap_g/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_g-S_O2_g/n_hs_gas/(1/tau_L_h)+S_O2_g/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
+        <v>0.035988377729</v>
+      </c>
+      <c r="E566" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exact periodic solution of the first-order liquid (rate 1/τ, D326) driven by the exponential headspace ramp of the gap (from y_O2_post to S/F at rate F/n), maximal just before a pulse. Replaces the quasi-steady lag correction, which over-trusted gaps comparable to τ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid-equilibrium O₂ fraction at its peak — lag</t>
+        </is>
+      </c>
+      <c r="B567" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z_peak_l</t>
+        </is>
+      </c>
+      <c r="C567" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D567" s="41">
+        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_post_l-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;1E-9*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_l-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
+        <v>0.070079461273</v>
+      </c>
+      <c r="E567" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D566 on the lag phase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Liquid-equilibrium O₂ fraction at its peak — start-up</t>
+        </is>
+      </c>
+      <c r="B568" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z_peak_su</t>
+        </is>
+      </c>
+      <c r="C568" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D568" s="41">
+        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_end_su*flush_ret-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;1E-9*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_su_h)-EXP(-(1/tau_L_h)*t_gap_su_h)),(1/tau_L_h)*t_gap_su_h*EXP(-(1/tau_L_h)*t_gap_su_h))/(1-EXP(-(1/tau_L_h)*t_gap_su_h)),y_O2_end_su*flush_ret-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_su_h/(1-EXP(-(1/tau_L_h)*t_gap_su_h)))</f>
+        <v>0.011984539296</v>
+      </c>
+      <c r="E568" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D567 at the start-up interval.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: eighth Codex review fixes (first-order time-to-ceiling, zero-back-pressure D80 relabelled, calibrated etaF_OER in the twin, named rate tolerance)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -1078,6 +1078,7 @@
     <definedName name="z_peak_g" localSheetId="5">'Mass Transfer'!$D$566</definedName>
     <definedName name="z_peak_l" localSheetId="5">'Mass Transfer'!$D$567</definedName>
     <definedName name="z_peak_su" localSheetId="5">'Mass Transfer'!$D$568</definedName>
+    <definedName name="rate_tol_rel" localSheetId="5">'Mass Transfer'!$D$569</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -25465,7 +25466,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:S568"/>
+  <dimension ref="A1:S569"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -26687,12 +26688,12 @@
         <v>61</v>
       </c>
       <c r="D66" s="41">
-        <f>IF(O2_excess-strip_avg*O2_ceil_org/O2_ceil_C&gt;0,O2_ceil_org*(V_charge/1000000)/(O2_excess-strip_avg*O2_ceil_org/O2_ceil_C)*60,"never (strip ≥ source)")</f>
-        <v>17.740739181348</v>
+        <f>IF(O2_excess-strip_avg*O2_ceil_org/O2_ceil_C&gt;0,IF(strip_avg&gt;0,-LN(1-strip_avg*O2_ceil_org/O2_ceil_C/O2_excess)*60*(V_charge/1000000)*O2_ceil_C/strip_avg,t_O2_ceiling),"never (strip ≥ source)")</f>
+        <v>17.162152896755</v>
       </c>
       <c r="E66" s="74" t="inlineStr">
         <is>
-          <t xml:space="preserve">As D65, crediting the time-averaged bubble strip at the organism ceiling’s driving force (D55 × D565/D6); "never" = strip ≥ source.</t>
+          <t xml:space="preserve">As D65, with the bubble strip growing in proportion to DO as it rises (first order: rate D55 × DO/D6, so t = −ln(1 − strip at the organism ceiling ÷ source)/k). "never" = the strip at the organism ceiling (D565) matches the source. Bubbles meet fresh CO₂, so no back-pressure term is needed.</t>
         </is>
       </c>
       <c r="F66" s="21"/>
@@ -26927,8 +26928,10 @@
       <c r="F79" s="21"/>
     </row>
     <row r="80" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="18" t="s">
-        <v>644</v>
+      <c r="A80" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ time-to-ceiling, zero headspace O₂ (hypothetical)</t>
+        </is>
       </c>
       <c r="B80" s="19" t="s">
         <v>645</v>
@@ -26937,12 +26940,12 @@
         <v>61</v>
       </c>
       <c r="D80" s="41" t="str">
-        <f>IF(O2_net_lag_mt-(strip_avg+surf_strip)*O2_ceil_org/O2_ceil_C&gt;0,O2_ceil_org*(V_charge/1000000)/(O2_net_lag_mt-(strip_avg+surf_strip)*O2_ceil_org/O2_ceil_C)*60,"never (removal ≥ source)")</f>
-        <v>never (removal ≥ source)</v>
+        <f>IF(O2_net_lag_mt-(strip_avg+surf_strip)*O2_ceil_org/O2_ceil_C&gt;0,IF(strip_avg+surf_strip&gt;0,-LN(1-(strip_avg+surf_strip)*O2_ceil_org/O2_ceil_C/O2_net_lag_mt)*60*(V_charge/1000000)*O2_ceil_C/(strip_avg+surf_strip),t_O2_ceiling_lag),"not reached if the headspace held no O₂ — not a pass; see D363")</f>
+        <v>not reached if the headspace held no O₂ — not a pass; see D363</v>
       </c>
       <c r="E80" s="53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Companion to D79 crediting both removal paths at the organism ceiling’s driving force (D55 and D73 scaled by D565/D6), on the lag source.</t>
+          <t xml:space="preserve">CAPACITY DIAGNOSTIC ONLY: the lag rise (D79) with both removal paths acting first order against an O₂-free headspace (zero back-pressure). The real headspace holds O₂ and pushes back, so the lag ceiling verdict is the lag peak (D363, Summary row 62); a non-crossing here is never a pass.</t>
         </is>
       </c>
       <c r="F80" s="21"/>
@@ -39778,7 +39781,7 @@
         </is>
       </c>
       <c r="D566" s="41">
-        <f>IF(F_gap_g&gt;0,S_O2_g/F_gap_g+(y_O2_post_g-S_O2_g/F_gap_g)*IF(ABS((1/tau_L_h)-(F_gap_g/n_hs_gas))&gt;1E-9*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_g/n_hs_gas))*(EXP(-(F_gap_g/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_g-S_O2_g/n_hs_gas/(1/tau_L_h)+S_O2_g/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
+        <f>IF(F_gap_g&gt;0,S_O2_g/F_gap_g+(y_O2_post_g-S_O2_g/F_gap_g)*IF(ABS((1/tau_L_h)-(F_gap_g/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_g/n_hs_gas))*(EXP(-(F_gap_g/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_g-S_O2_g/n_hs_gas/(1/tau_L_h)+S_O2_g/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
         <v>0.035988377729</v>
       </c>
       <c r="E566" s="51" t="inlineStr">
@@ -39804,7 +39807,7 @@
         </is>
       </c>
       <c r="D567" s="41">
-        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_post_l-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;1E-9*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_l-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
+        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_post_l-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_l-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
         <v>0.070079461273</v>
       </c>
       <c r="E567" s="51" t="inlineStr">
@@ -39830,12 +39833,37 @@
         </is>
       </c>
       <c r="D568" s="41">
-        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_end_su*flush_ret-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;1E-9*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_su_h)-EXP(-(1/tau_L_h)*t_gap_su_h)),(1/tau_L_h)*t_gap_su_h*EXP(-(1/tau_L_h)*t_gap_su_h))/(1-EXP(-(1/tau_L_h)*t_gap_su_h)),y_O2_end_su*flush_ret-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_su_h/(1-EXP(-(1/tau_L_h)*t_gap_su_h)))</f>
+        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_end_su*flush_ret-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_su_h)-EXP(-(1/tau_L_h)*t_gap_su_h)),(1/tau_L_h)*t_gap_su_h*EXP(-(1/tau_L_h)*t_gap_su_h))/(1-EXP(-(1/tau_L_h)*t_gap_su_h)),y_O2_end_su*flush_ret-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_su_h/(1-EXP(-(1/tau_L_h)*t_gap_su_h)))</f>
         <v>0.011984539296</v>
       </c>
       <c r="E568" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">As D567 at the start-up interval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rate-coincidence tolerance (numerical)</t>
+        </is>
+      </c>
+      <c r="B569" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rate_tol_rel</t>
+        </is>
+      </c>
+      <c r="C569" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D569" s="106">
+        <v>1e-09</v>
+      </c>
+      <c r="E569" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Numerical, not a datum: relative gap below which the liquid (1/τ) and headspace (F/n) rates are treated as equal in D566–D568, where the general formula has a removable 0/0 and the coincident-rate limit is used instead.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: ninth Codex review fixes (conservative start-up sources and hazard screen, z_e_ORR not swept, organism ceiling in the twin's relax note, Summary names)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -1079,6 +1079,27 @@
     <definedName name="z_peak_l" localSheetId="5">'Mass Transfer'!$D$567</definedName>
     <definedName name="z_peak_su" localSheetId="5">'Mass Transfer'!$D$568</definedName>
     <definedName name="rate_tol_rel" localSheetId="5">'Mass Transfer'!$D$569</definedName>
+    <definedName name="O2_net_su_max" localSheetId="2">Electrochemistry!$D$174</definedName>
+    <definedName name="rH2_su_max" localSheetId="2">Electrochemistry!$D$175</definedName>
+    <definedName name="O2_net_su_mt" localSheetId="5">'Mass Transfer'!$D$570</definedName>
+    <definedName name="rH2_su_mt" localSheetId="5">'Mass Transfer'!$D$571</definedName>
+    <definedName name="O2_src_su" localSheetId="5">'Mass Transfer'!$D$572</definedName>
+    <definedName name="H2_src_su" localSheetId="5">'Mass Transfer'!$D$573</definedName>
+    <definedName name="S_O2_su" localSheetId="5">'Mass Transfer'!$D$574</definedName>
+    <definedName name="F_gap_su" localSheetId="5">'Mass Transfer'!$D$575</definedName>
+    <definedName name="DO_surf_excess_su" localSheetId="5">'Mass Transfer'!$D$576</definedName>
+    <definedName name="H2_LFL_mt" localSheetId="5">'Mass Transfer'!$D$577</definedName>
+    <definedName name="O2_LOC_lim_mt" localSheetId="5">'Mass Transfer'!$D$578</definedName>
+    <definedName name="t_gap_H2_su" localSheetId="5">'Mass Transfer'!$D$579</definedName>
+    <definedName name="t_gap_O2_su" localSheetId="5">'Mass Transfer'!$D$580</definedName>
+    <definedName name="spg_int_H2safe_su" localSheetId="5">'Mass Transfer'!$D$581</definedName>
+    <definedName name="spg_int_H2safe_su_opt" localSheetId="5">'Mass Transfer'!$D$582</definedName>
+    <definedName name="spg_int_max_su" localSheetId="5">'Mass Transfer'!$D$583</definedName>
+    <definedName name="res_spg_int_pH" localSheetId="0">Summary!$D$30</definedName>
+    <definedName name="res_duty_ratio" localSheetId="0">Summary!$D$32</definedName>
+    <definedName name="chk_DO_pH" localSheetId="0">Summary!$D$52</definedName>
+    <definedName name="chk_hs_sag" localSheetId="0">Summary!$D$53</definedName>
+    <definedName name="chk_hs_sag_ok" localSheetId="0">Summary!$D$54</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -11647,7 +11668,10 @@
         <f>IF(NOT(ISNUMBER(res_spg_dur)),res_spg_dur,'Mass Transfer'!spg_dur)</f>
         <v>0.65</v>
       </c>
-      <c r="E19" s="21"/>
+      <c r="E19" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D121","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
       <c r="F19" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">Pulse actually evaluated by every operating check below. Summary override wins, then Manual mode, otherwise the optimum rounded to the pulse resolution.</t>
@@ -11694,7 +11718,10 @@
         <f>IF(NOT(ISNUMBER(res_spg_int)),res_spg_int,'Mass Transfer'!spg_int)</f>
         <v>7.07</v>
       </c>
-      <c r="E21" s="67"/>
+      <c r="E21" s="24" t="str">
+        <f>HYPERLINK("#'Mass Transfer'!D122","→ Mass Transfer")</f>
+        <v>→ Mass Transfer</v>
+      </c>
       <c r="F21" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Interval actually evaluated below, in decimal minutes. Default converts the commanded pulse to the ideal delivery duty and rounds down to 0.01 min; overrides and Manual mode are evaluated directly.</t>
@@ -11860,6 +11887,11 @@
           <t xml:space="preserve">pH-ceiling interval (longest keeping pH at or under the band ceiling)</t>
         </is>
       </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_spg_int_pH</t>
+        </is>
+      </c>
       <c r="C30" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">min</t>
@@ -11897,7 +11929,7 @@
       </c>
       <c r="D31" s="65">
         <f>'Mass Transfer'!spg_int_su_run</f>
-        <v>1.21</v>
+        <v>1.16</v>
       </c>
       <c r="E31" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D547","→ Mass Transfer")</f>
@@ -11905,13 +11937,18 @@
       </c>
       <c r="F31" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Owner asked for both schedules (T4). Until uptake starts: the shortest of the lag O₂ bound (the legacy guard when the lag DO target is unreachable), the interval clearing the H₂ flammability screen (Biology D92), the lag pH ceiling and the carbon bound. Select Lag in row 12 to evaluate every output at exactly this schedule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+          <t xml:space="preserve">Owner asked for both schedules (T4). Until uptake starts: the shortest of the lag O₂ bound (the legacy guard when the lag DO target is unreachable), the interval clearing the start-up hazard screen (Mass Transfer D581), the lag pH ceiling and the carbon bound. Sized on Growth it assumes no cathodic O₂ loss, an upper bound on the lag O₂ and H₂ sources, because the start-up DO differs from the lag reference (Electrochemistry D129); select Lag in row 12 to size and evaluate every output on the lag phase itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" x14ac:dyDescent="0.2">
       <c r="A32" s="64" t="s">
         <v>1788</v>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">res_duty_ratio</t>
+        </is>
       </c>
       <c r="C32" s="21" t="s">
         <v>87</v>
@@ -11943,7 +11980,7 @@
       </c>
       <c r="D33" s="175" t="str">
         <f>IF(ISNUMBER('Mass Transfer'!spg_int_su_run),"DO "&amp;TEXT('Mass Transfer'!DO_avg_su_mgL,"0.0")&amp;" mg/L mean, "&amp;TEXT('Mass Transfer'!DO_peak_su_mgL,"0.0")&amp;" peak; H₂ "&amp;TEXT('Mass Transfer'!y_H2_end_su,"0%")&amp;" before each pulse; set by "&amp;'Mass Transfer'!su_binding,"no executable start-up schedule")</f>
-        <v>DO 4.1 mg/L mean, 4.1 peak; H₂ 3% before each pulse; set by the legacy O₂ flush guard (lag DO target unreachable)</v>
+        <v>DO 4.5 mg/L mean, 4.5 peak; H₂ 3% before each pulse; set by the legacy O₂ flush guard (lag DO target unreachable)</v>
       </c>
       <c r="E33" s="24" t="str">
         <f>HYPERLINK("#'Mass Transfer'!D556","→ Mass Transfer")</f>
@@ -11951,7 +11988,7 @@
       </c>
       <c r="F33" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">The lag sawtooth evaluated at the start-up interval (rows 61–62 show the lag phase at the headline schedule instead).</t>
+          <t xml:space="preserve">The lag sawtooth at the start-up interval, on start-up sources that assume no cathodic O₂ loss (Mass Transfer D572) unless the schedule is sized on Lag; rows 61–62 show the lag phase at the headline schedule instead.</t>
         </is>
       </c>
     </row>
@@ -12320,9 +12357,14 @@
         </is>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="52" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A52" s="64" t="s">
         <v>1827</v>
+      </c>
+      <c r="B52" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_DO_pH</t>
+        </is>
       </c>
       <c r="D52" s="178" t="str">
         <f>IF(ISNA('Mass Transfer'!F_vent_ex+'Mass Transfer'!O2_src_sched),"#N/A – check the selectors in D2–D5, D11 and D12",IF(NOT(ISNUMBER('Mass Transfer'!spg_int_DO)),"DO target unreachable on the sizing phase; schedule is a legacy fallback",IF(OR(Chemistry!DIC_ref_check&lt;&gt;"OK",ABS(Electrochemistry!DO_lag_ref/Electrochemistry!ec_DO_lag-1)&gt;Electrochemistry!DO_lag_tol),"watch – refresh the DIC or lag-DO reference before claiming either target",IF(AND(res_pH&gt;=cf_pH_lo,res_pH&lt;=cf_pH_hi,res_DO_ss&lt;='Mass Transfer'!DO_target*'Mass Transfer'!M_O2),"yes – both targets met by the evaluated schedule","NO – evaluated schedule misses the pH band or mean DO target"))))</f>
@@ -12338,9 +12380,14 @@
         </is>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" x14ac:dyDescent="0.2">
       <c r="A53" s="64" t="s">
         <v>1829</v>
+      </c>
+      <c r="B53" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_hs_sag</t>
+        </is>
       </c>
       <c r="C53" s="21" t="s">
         <v>111</v>
@@ -12357,9 +12404,14 @@
         <v>1830</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="54" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A54" s="64" t="s">
         <v>1831</v>
+      </c>
+      <c r="B54" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chk_hs_sag_ok</t>
+        </is>
       </c>
       <c r="D54" s="175" t="str">
         <f>'Mass Transfer'!hs_sag_chk</f>
@@ -16134,7 +16186,7 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="A1:N173"/>
+  <dimension ref="A1:N175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -19104,6 +19156,58 @@
       <c r="E173" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Catalase disproportionates the rest of the growth peroxide, 2 H₂O₂ → O₂ + 2 H₂O: half an O₂ back per H₂O₂. A biological return, so it applies whether or not etaF_OER is measured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upper bound on the lag O₂ source (no cathodic O₂ loss)</t>
+        </is>
+      </c>
+      <c r="B174" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_net_su_max</t>
+        </is>
+      </c>
+      <c r="C174" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D174" s="111">
+        <f>rO2_gen+IF(ISNUMBER(cal_etaF_OER),0,r_H2O2_an_g/2)</f>
+        <v>5.307542491154e-05</v>
+      </c>
+      <c r="E174" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_net_lag (D132) at zero cathodic O₂ reduction: no ORR, so no peroxide and the anode’s peroxide diversion (D170) returns to OER. D132 falls as the cathodic loss rises, so this is its ceiling at any lag DO. Sizes the start-up schedule, whose DO differs from DO_lag_ref (D129).</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Upper bound on the lag H₂ evolution (no cathodic O₂ loss)</t>
+        </is>
+      </c>
+      <c r="B175" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rH2_su_max</t>
+        </is>
+      </c>
+      <c r="C175" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D175" s="111">
+        <f>I_app/(z_e_H2*F_const)*3600</f>
+        <v>0.0001061508498231</v>
+      </c>
+      <c r="E175" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All cathodic current to H₂: the ceiling of rH2_lag (D133) at any lag DO.</t>
         </is>
       </c>
     </row>
@@ -25466,7 +25570,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:S569"/>
+  <dimension ref="A1:S583"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -39183,12 +39287,12 @@
         </is>
       </c>
       <c r="D542" s="41" t="e">
-        <f>IF(DO_target-DO_surf_excess_lag&gt;0,(DO_target-DO_surf_excess_lag)/(H_O2_T*P_dry),NA())</f>
+        <f>IF(DO_target-DO_surf_excess_su&gt;0,(DO_target-DO_surf_excess_su)/(H_O2_T*P_dry),NA())</f>
         <v>#N/A</v>
       </c>
       <c r="E542" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">As D183 on the lag source (D181). #N/A = the surface cannot carry the lag O₂ flux at the target DO.</t>
+          <t xml:space="preserve">As D183 on the start-up source (D576). #N/A = the surface cannot carry the lag O₂ flux at the target DO at any interval.</t>
         </is>
       </c>
     </row>
@@ -39209,12 +39313,12 @@
         </is>
       </c>
       <c r="D543" s="41" t="e">
-        <f>IF(ISNUMBER(y_O2_star_l),MAX(0,((O2_src_l+y_O2_air*F_vent_ex)*saw_factor/y_O2_star_l-F_dil-O2_src_l-H2_src_l+CO2_fix_l)/CO2_rate_full),NA())</f>
+        <f>IF(ISNUMBER(y_O2_star_l),MAX(0,((O2_src_su+y_O2_air*F_vent_ex)*saw_factor/y_O2_star_l-F_dil-O2_src_su-H2_src_su+CO2_fix_l)/CO2_rate_full),NA())</f>
         <v>#N/A</v>
       </c>
       <c r="E543" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">As D184 on the lag sources (D310, D314, D316).</t>
+          <t xml:space="preserve">As D184 on the start-up sources (D572, D573).</t>
         </is>
       </c>
     </row>
@@ -39287,12 +39391,12 @@
         </is>
       </c>
       <c r="D546" s="41">
-        <f>IF(ph_unreach_l,NA(),MIN(spg_int_carbon,IF(ISNUMBER(spg_int_DO_l),spg_int_DO_l,spg_int_max),IF(ISNUMBER(spg_int_H2safe_opt),spg_int_H2safe_opt,spg_int_carbon),IF(ISNUMBER(spg_int_pH_l),spg_int_pH_l*spg_dur_eq_opt/spg_dur_eq,spg_int_carbon)))</f>
-        <v>1.251651684129</v>
+        <f>IF(ph_unreach_l,NA(),MIN(spg_int_carbon,IF(ISNUMBER(spg_int_DO_l),spg_int_DO_l,spg_int_max_su),IF(ISNUMBER(spg_int_H2safe_su_opt),spg_int_H2safe_su_opt,spg_int_carbon),IF(ISNUMBER(spg_int_pH_l),spg_int_pH_l*spg_dur_eq_opt/spg_dur_eq,spg_int_carbon)))</f>
+        <v>1.20664768662</v>
       </c>
       <c r="E546" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">The shortest of the carbon bound, the lag O₂ bound (or the legacy guard D89 when the lag DO target is unreachable), the H₂-screen interval (D563) and the lag pH ceiling (D561), on the basis of D91. #N/A when no interval holds the lag pH under the ceiling. Equals D91 when Summary D12 is Lag.</t>
+          <t xml:space="preserve">The shortest of the carbon bound, the lag O₂ bound (or the start-up legacy guard D583 when the lag DO target is unreachable), the start-up hazard-screen interval (D582) and the lag pH ceiling (D561), on the basis of D91, all on the start-up sources (D572–D576). #N/A when no interval holds the lag pH under the ceiling. Equals D91 when Summary D12 is Lag. The lag pH grid (D561) keeps the headline lag gas flow; it binds only at intervals hundreds of times longer.</t>
         </is>
       </c>
     </row>
@@ -39314,7 +39418,7 @@
       </c>
       <c r="D547" s="41">
         <f>IF(FLOOR(spg_int_su_opt*spg_dur_eq/spg_dur_eq_opt,interval_res)*60&gt;spg_dur,FLOOR(spg_int_su_opt*spg_dur_eq/spg_dur_eq_opt,interval_res),NA())</f>
-        <v>1.21</v>
+        <v>1.16</v>
       </c>
       <c r="E547" s="51" t="inlineStr">
         <is>
@@ -39339,7 +39443,7 @@
         </is>
       </c>
       <c r="D548" s="41" t="str">
-        <f>IF(ph_unreach_l,"pH ceiling unreachable in lag",IF(spg_int_su_opt=IF(ISNUMBER(spg_int_H2safe_opt),spg_int_H2safe_opt,spg_int_carbon),"the H₂ flammability screen (Biology D92)",IF(spg_int_su_opt=IF(ISNUMBER(spg_int_pH_l),spg_int_pH_l*spg_dur_eq_opt/spg_dur_eq,spg_int_carbon),"the pH ceiling (lag)",IF(spg_int_su_opt=spg_int_carbon,"carbon supply",IF(ISNUMBER(spg_int_DO_l),"lag O₂ dilution","the legacy O₂ flush guard (lag DO target unreachable)")))))</f>
+        <f>IF(ph_unreach_l,"pH ceiling unreachable in lag",IF(spg_int_su_opt=IF(ISNUMBER(spg_int_H2safe_su_opt),spg_int_H2safe_su_opt,spg_int_carbon),"the start-up hazard screen (D581)",IF(spg_int_su_opt=IF(ISNUMBER(spg_int_pH_l),spg_int_pH_l*spg_dur_eq_opt/spg_dur_eq,spg_int_carbon),"the pH ceiling (lag)",IF(spg_int_su_opt=spg_int_carbon,"carbon supply",IF(ISNUMBER(spg_int_DO_l),"lag O₂ dilution","the legacy O₂ flush guard (lag DO target unreachable)")))))</f>
         <v>the legacy O₂ flush guard (lag DO target unreachable)</v>
       </c>
       <c r="E548" s="51" t="inlineStr">
@@ -39366,7 +39470,7 @@
       </c>
       <c r="D549" s="41">
         <f>MAX(0,spg_int_su_run*60-spg_dur)/3600</f>
-        <v>0.019986111111</v>
+        <v>0.019152777778</v>
       </c>
       <c r="E549" s="51" t="inlineStr">
         <is>
@@ -39391,8 +39495,8 @@
         </is>
       </c>
       <c r="D550" s="41">
-        <f>F_gap_l*t_gap_su_h/n_hs_gas</f>
-        <v>0.036016292273</v>
+        <f>F_gap_su*t_gap_su_h/n_hs_gas</f>
+        <v>0.037192064462</v>
       </c>
       <c r="E550" s="51" t="inlineStr">
         <is>
@@ -39418,7 +39522,7 @@
       </c>
       <c r="D551" s="41">
         <f>IF(x_su&gt;0,(1-EXP(-x_su))/x_su,1)</f>
-        <v>0.982206116713</v>
+        <v>0.981632381646</v>
       </c>
       <c r="E551" s="51" t="inlineStr">
         <is>
@@ -39444,7 +39548,7 @@
       </c>
       <c r="D552" s="41">
         <f>IF(x_su&gt;0,(x_su-1+EXP(-x_su))/x_su^2,1/2)</f>
-        <v>0.494050946506</v>
+        <v>0.49385853192</v>
       </c>
       <c r="E552" s="51" t="inlineStr">
         <is>
@@ -39469,8 +39573,8 @@
         </is>
       </c>
       <c r="D553" s="41">
-        <f>S_O2_l*t_gap_su_h/n_hs_gas</f>
-        <v>0.011115587615</v>
+        <f>S_O2_su*t_gap_su_h/n_hs_gas</f>
+        <v>0.011544614242</v>
       </c>
       <c r="E553" s="51" t="inlineStr">
         <is>
@@ -39496,7 +39600,7 @@
       </c>
       <c r="D554" s="41">
         <f>dy_O2_su*phi_su/(1-flush_ret*EXP(-x_su))</f>
-        <v>0.016815548393</v>
+        <v>0.017443301407</v>
       </c>
       <c r="E554" s="51" t="inlineStr">
         <is>
@@ -39522,7 +39626,7 @@
       </c>
       <c r="D555" s="41">
         <f>y_O2_end_su*flush_ret*phi_su+dy_O2_su*psi_su</f>
-        <v>0.011496911008</v>
+        <v>0.011927197861</v>
       </c>
       <c r="E555" s="51" t="inlineStr">
         <is>
@@ -39547,8 +39651,8 @@
         </is>
       </c>
       <c r="D556" s="41">
-        <f>(DO_surf_excess_lag+H_O2_T*P_dry*y_O2_avg_su)*M_O2</f>
-        <v>4.122375525019</v>
+        <f>(DO_surf_excess_su+H_O2_T*P_dry*y_O2_avg_su)*M_O2</f>
+        <v>4.499880552063</v>
       </c>
       <c r="E556" s="51" t="inlineStr">
         <is>
@@ -39573,8 +39677,8 @@
         </is>
       </c>
       <c r="D557" s="41">
-        <f>(DO_surf_excess_lag+H_O2_T*P_dry*z_peak_su)*M_O2</f>
-        <v>4.13806097293</v>
+        <f>(DO_surf_excess_su+H_O2_T*P_dry*z_peak_su)*M_O2</f>
+        <v>4.515479521662</v>
       </c>
       <c r="E557" s="51" t="inlineStr">
         <is>
@@ -39599,8 +39703,8 @@
         </is>
       </c>
       <c r="D558" s="41">
-        <f>H2_src_l*t_gap_su_h/n_hs_gas*phi_su/(1-flush_ret*EXP(-x_su))</f>
-        <v>0.029076305025</v>
+        <f>H2_src_su*t_gap_su_h/n_hs_gas*phi_su/(1-flush_ret*EXP(-x_su))</f>
+        <v>0.030527042916</v>
       </c>
       <c r="E558" s="51" t="inlineStr">
         <is>
@@ -39833,8 +39937,8 @@
         </is>
       </c>
       <c r="D568" s="41">
-        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_end_su*flush_ret-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_su_h)-EXP(-(1/tau_L_h)*t_gap_su_h)),(1/tau_L_h)*t_gap_su_h*EXP(-(1/tau_L_h)*t_gap_su_h))/(1-EXP(-(1/tau_L_h)*t_gap_su_h)),y_O2_end_su*flush_ret-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_su_h/(1-EXP(-(1/tau_L_h)*t_gap_su_h)))</f>
-        <v>0.011984539296</v>
+        <f>IF(F_gap_su&gt;0,S_O2_su/F_gap_su+(y_O2_end_su*flush_ret-S_O2_su/F_gap_su)*IF(ABS((1/tau_L_h)-(F_gap_su/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_su/n_hs_gas))*(EXP(-(F_gap_su/n_hs_gas)*t_gap_su_h)-EXP(-(1/tau_L_h)*t_gap_su_h)),(1/tau_L_h)*t_gap_su_h*EXP(-(1/tau_L_h)*t_gap_su_h))/(1-EXP(-(1/tau_L_h)*t_gap_su_h)),y_O2_end_su*flush_ret-S_O2_su/n_hs_gas/(1/tau_L_h)+S_O2_su/n_hs_gas*t_gap_su_h/(1-EXP(-(1/tau_L_h)*t_gap_su_h)))</f>
+        <v>0.012412137716</v>
       </c>
       <c r="E568" s="51" t="inlineStr">
         <is>
@@ -39864,6 +39968,370 @@
       <c r="E569" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Numerical, not a datum: relative gap below which the liquid (1/τ) and headspace (F/n) rates are treated as equal in D566–D568, where the general formula has a removable 0/0 and the coincident-rate limit is used instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Upper bound on the lag O₂ source</t>
+        </is>
+      </c>
+      <c r="B570" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_net_su_mt</t>
+        </is>
+      </c>
+      <c r="C570" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D570" s="41">
+        <f>Electrochemistry!O2_net_su_max</f>
+        <v>5.307542491154e-05</v>
+      </c>
+      <c r="E570" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D174.</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) Upper bound on the lag H₂ evolution</t>
+        </is>
+      </c>
+      <c r="B571" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rH2_su_mt</t>
+        </is>
+      </c>
+      <c r="C571" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D571" s="41">
+        <f>Electrochemistry!rH2_su_max</f>
+        <v>0.0001061508498231</v>
+      </c>
+      <c r="E571" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Electrochemistry!D175.</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O₂ source — start-up</t>
+        </is>
+      </c>
+      <c r="B572" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_src_su</t>
+        </is>
+      </c>
+      <c r="C572" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D572" s="41">
+        <f>IF(O2_sizing_phase=phase_name_2,O2_src_l,O2_net_su_mt)</f>
+        <v>5.307542491154e-05</v>
+      </c>
+      <c r="E572" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sized on Lag, the start-up schedule is the headline one and D129 is checked against it, so the lag source (D310) is consistent. Sized on Growth, the start-up runs at a different DO from DO_lag_ref, so the bound D570 (no cathodic loss) is used: conservative for the DO and the hazard screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H₂ to headspace — start-up</t>
+        </is>
+      </c>
+      <c r="B573" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_src_su</t>
+        </is>
+      </c>
+      <c r="C573" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D573" s="41">
+        <f>IF(O2_sizing_phase=phase_name_2,H2_src_l,MAX(0,rH2_su_mt-H2_HOR_mt))</f>
+        <v>0.0001061508498231</v>
+      </c>
+      <c r="E573" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D572 for H₂ (D314, or the bound D571 net of anodic oxidation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Headspace O₂ inflow — start-up</t>
+        </is>
+      </c>
+      <c r="B574" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S_O2_su</t>
+        </is>
+      </c>
+      <c r="C574" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D574" s="41">
+        <f>O2_src_su+y_O2_air*F_vent_ex</f>
+        <v>6.065511399778e-05</v>
+      </c>
+      <c r="E574" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D349 on the start-up source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas leaving between pulses — start-up</t>
+        </is>
+      </c>
+      <c r="B575" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F_gap_su</t>
+        </is>
+      </c>
+      <c r="C575" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/h</t>
+        </is>
+      </c>
+      <c r="D575" s="41">
+        <f>F_dil+MAX(0,O2_src_su+H2_src_su-CO2_fix_l)</f>
+        <v>0.0001954061749076</v>
+      </c>
+      <c r="E575" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D353 on the start-up sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO excess to drive the surface flux — start-up</t>
+        </is>
+      </c>
+      <c r="B576" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DO_surf_excess_su</t>
+        </is>
+      </c>
+      <c r="C576" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mol/m³</t>
+        </is>
+      </c>
+      <c r="D576" s="41">
+        <f>O2_src_su/(kLa_surf_used*3600*(V_charge/1000000))</f>
+        <v>0.128639934046</v>
+      </c>
+      <c r="E576" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D181 on the start-up source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) H₂ lower flammability limit</t>
+        </is>
+      </c>
+      <c r="B577" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H2_LFL_mt</t>
+        </is>
+      </c>
+      <c r="C577" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D577" s="41">
+        <f>Biology!H2_LFL</f>
+        <v>0.04</v>
+      </c>
+      <c r="E577" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D80.</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(import) O₂ limit for the hazard screen (LOC × margin)</t>
+        </is>
+      </c>
+      <c r="B578" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O2_LOC_lim_mt</t>
+        </is>
+      </c>
+      <c r="C578" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D578" s="41">
+        <f>Biology!O2_LOC_H2*Biology!LOC_margin</f>
+        <v>0.0312</v>
+      </c>
+      <c r="E578" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import from Biology!D81 × D82.</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longest gap keeping start-up pre-pulse H₂ below the LFL</t>
+        </is>
+      </c>
+      <c r="B579" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">t_gap_H2_su</t>
+        </is>
+      </c>
+      <c r="C579" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D579" s="41">
+        <f>IF(H2_src_su&gt;H2_LFL_mt*F_gap_su,n_hs_gas/F_gap_su*LN((1-H2_LFL_mt*F_gap_su/H2_src_su*flush_ret)/(1-H2_LFL_mt*F_gap_su/H2_src_su))*60,"none needed")</f>
+        <v>1.524751128368</v>
+      </c>
+      <c r="E579" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As Biology D90 on the start-up sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Longest gap keeping start-up pre-pulse O₂ under the LOC margin</t>
+        </is>
+      </c>
+      <c r="B580" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">t_gap_O2_su</t>
+        </is>
+      </c>
+      <c r="C580" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D580" s="41">
+        <f>IF(S_O2_su&gt;O2_LOC_lim_mt*F_gap_su,n_hs_gas/F_gap_su*LN((1-O2_LOC_lim_mt*F_gap_su/S_O2_su*flush_ret)/(1-O2_LOC_lim_mt*F_gap_su/S_O2_su))*60,"none needed")</f>
+        <v>2.122727097897</v>
+      </c>
+      <c r="E580" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As Biology D91 on the start-up sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interval clearing the start-up hazard screen</t>
+        </is>
+      </c>
+      <c r="B581" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_H2safe_su</t>
+        </is>
+      </c>
+      <c r="C581" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D581" s="41">
+        <f>IF(OR(ISTEXT(t_gap_H2_su),ISTEXT(t_gap_O2_su)),"any interval",MAX(t_gap_H2_su,t_gap_O2_su)+spg_dur/60)</f>
+        <v>2.13356043123</v>
+      </c>
+      <c r="E581" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As Biology D92 (either route suffices) on the start-up sources, pulse in use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Start-up hazard-screen interval on the optimal-pulse basis</t>
+        </is>
+      </c>
+      <c r="B582" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_H2safe_su_opt</t>
+        </is>
+      </c>
+      <c r="C582" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D582" s="41">
+        <f>IF(ISNUMBER(spg_int_H2safe_su),spg_int_H2safe_su*spg_dur_eq_opt/spg_dur_eq,"any interval")</f>
+        <v>2.200875733589</v>
+      </c>
+      <c r="E582" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D563 for D581.</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Legacy O₂ flush guard — start-up</t>
+        </is>
+      </c>
+      <c r="B583" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">spg_int_max_su</t>
+        </is>
+      </c>
+      <c r="C583" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">min</t>
+        </is>
+      </c>
+      <c r="D583" s="41">
+        <f>IF(O2_sizing_phase=phase_name_2,spg_int_max,target_DO_frac*O2_ceil_org*(V_charge/1000000)/MAX(O2_src_guard,O2_src_su)*60)</f>
+        <v>1.20664768662</v>
+      </c>
+      <c r="E583" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">As D89 on the larger of its guard source and the start-up source (D572).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: tenth Codex review fixes (start-up pH grid on the start-up gas flow, monochloramine ratio label)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -22499,8 +22499,10 @@
       </c>
     </row>
     <row r="224" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A224" t="s">
-        <v>1679</v>
+      <c r="A224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Monochloramine-formation chlorine per N</t>
+        </is>
       </c>
       <c r="B224" s="19" t="s">
         <v>1680</v>
@@ -22511,8 +22513,10 @@
       <c r="D224" s="116">
         <v>5.0599999999999996</v>
       </c>
-      <c r="E224" s="51" t="s">
-        <v>1682</v>
+      <c r="E224" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1:1 NH₂Cl formation, 70.906/14.007 = 5.06 mg Cl₂ per mg ammonium-N: the stoichiometric cap on chlorine bound as monochloramine. Not breakpoint demand, which (oxidation to N₂) needs about 7.6. On a Cl₂ basis; multiply by M_HOCl/M_Cl2 for the HOCl-equivalent basis.</t>
+        </is>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.2">
@@ -31906,19 +31910,19 @@
       </c>
       <c r="L440" s="41">
         <f>k_eff_CO2_l*B440</f>
-        <v>4.002941317124e-05</v>
+        <v>4.313472514964e-05</v>
       </c>
       <c r="M440" s="41">
         <f>EXP(-L440)</f>
-        <v>0.999959971388</v>
+        <v>0.999956866205</v>
       </c>
       <c r="N440" s="41">
         <f>IF(L440&gt;0,(1-M440)/L440,1)</f>
-        <v>0.999979985559</v>
+        <v>0.999978432948</v>
       </c>
       <c r="O440" s="41">
         <f>IF(L440&gt;0,(L440-1+M440)/L440^2,1/2)</f>
-        <v>0.499993382275</v>
+        <v>0.499992792176</v>
       </c>
       <c r="P440" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B440/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -31926,11 +31930,11 @@
       </c>
       <c r="Q440" s="41">
         <f>(P440*N440+pool_b*M440)/(1-pool_ret*M440)</f>
-        <v>28.043578177755</v>
+        <v>28.042637432812</v>
       </c>
       <c r="R440" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q440+pool_b)*N440+P440*O440))</f>
-        <v>28.044139423039</v>
+        <v>28.043242201082</v>
       </c>
       <c r="S440" s="41">
         <f>IF(AND(R440&gt;=CO2_pH_hi_mt,R441&lt;CO2_pH_hi_mt),EXP(LN(A440)+(LN(A441)-LN(A440))*(R440-CO2_pH_hi_mt)/(R440-R441)),0)</f>
@@ -31980,19 +31984,19 @@
       </c>
       <c r="L441" s="41">
         <f>k_eff_CO2_l*B441</f>
-        <v>5.051547692092e-05</v>
+        <v>5.44342532194e-05</v>
       </c>
       <c r="M441" s="41">
         <f>EXP(-L441)</f>
-        <v>0.999949485799</v>
+        <v>0.999945567228</v>
       </c>
       <c r="N441" s="41">
         <f>IF(L441&gt;0,(1-M441)/L441,1)</f>
-        <v>0.999974742688</v>
+        <v>0.999972783368</v>
       </c>
       <c r="O441" s="41">
         <f>IF(L441&gt;0,(L441-1+M441)/L441^2,1/2)</f>
-        <v>0.49999156326</v>
+        <v>0.499990907593</v>
       </c>
       <c r="P441" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B441/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32000,11 +32004,11 @@
       </c>
       <c r="Q441" s="41">
         <f>(P441*N441+pool_b*M441)/(1-pool_ret*M441)</f>
-        <v>28.040401958976</v>
+        <v>28.039215043872</v>
       </c>
       <c r="R441" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q441+pool_b)*N441+P441*O441))</f>
-        <v>28.041110149814</v>
+        <v>28.039978146359</v>
       </c>
       <c r="S441" s="41">
         <f>IF(AND(R441&gt;=CO2_pH_hi_mt,R442&lt;CO2_pH_hi_mt),EXP(LN(A441)+(LN(A442)-LN(A441))*(R441-CO2_pH_hi_mt)/(R441-R442)),0)</f>
@@ -32054,19 +32058,19 @@
       </c>
       <c r="L442" s="41">
         <f>k_eff_CO2_l*B442</f>
-        <v>6.226054495309e-05</v>
+        <v>6.709045378032e-05</v>
       </c>
       <c r="M442" s="41">
         <f>EXP(-L442)</f>
-        <v>0.999937741393</v>
+        <v>0.999932911797</v>
       </c>
       <c r="N442" s="41">
         <f>IF(L442&gt;0,(1-M442)/L442,1)</f>
-        <v>0.999968870373</v>
+        <v>0.999966455524</v>
       </c>
       <c r="O442" s="41">
         <f>IF(L442&gt;0,(L442-1+M442)/L442^2,1/2)</f>
-        <v>0.499989630114</v>
+        <v>0.499988805959</v>
       </c>
       <c r="P442" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B442/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32074,11 +32078,11 @@
       </c>
       <c r="Q442" s="41">
         <f>(P442*N442+pool_b*M442)/(1-pool_ret*M442)</f>
-        <v>28.036845203663</v>
+        <v>28.035382693285</v>
       </c>
       <c r="R442" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q442+pool_b)*N442+P442*O442))</f>
-        <v>28.03771794459</v>
+        <v>28.036323095804</v>
       </c>
       <c r="S442" s="41">
         <f>IF(AND(R442&gt;=CO2_pH_hi_mt,R443&lt;CO2_pH_hi_mt),EXP(LN(A442)+(LN(A443)-LN(A442))*(R442-CO2_pH_hi_mt)/(R442-R443)),0)</f>
@@ -32128,19 +32132,19 @@
       </c>
       <c r="L443" s="41">
         <f>k_eff_CO2_l*B443</f>
-        <v>7.54157790212e-05</v>
+        <v>8.126621507314e-05</v>
       </c>
       <c r="M443" s="41">
         <f>EXP(-L443)</f>
-        <v>0.999924587065</v>
+        <v>0.999918737087</v>
       </c>
       <c r="N443" s="41">
         <f>IF(L443&gt;0,(1-M443)/L443,1)</f>
-        <v>0.999962293059</v>
+        <v>0.999959367993</v>
       </c>
       <c r="O443" s="41">
         <f>IF(L443&gt;0,(L443-1+M443)/L443^2,1/2)</f>
-        <v>0.499987413568</v>
+        <v>0.499986444451</v>
       </c>
       <c r="P443" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B443/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32148,11 +32152,11 @@
       </c>
       <c r="Q443" s="41">
         <f>(P443*N443+pool_b*M443)/(1-pool_ret*M443)</f>
-        <v>28.032862429876</v>
+        <v>28.031091399497</v>
       </c>
       <c r="R443" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q443+pool_b)*N443+P443*O443))</f>
-        <v>28.033919429582</v>
+        <v>28.03223033375</v>
       </c>
       <c r="S443" s="41">
         <f>IF(AND(R443&gt;=CO2_pH_hi_mt,R444&lt;CO2_pH_hi_mt),EXP(LN(A443)+(LN(A444)-LN(A443))*(R443-CO2_pH_hi_mt)/(R443-R444)),0)</f>
@@ -32202,19 +32206,19 @@
       </c>
       <c r="L444" s="41">
         <f>k_eff_CO2_l*B444</f>
-        <v>9.015049004312e-05</v>
+        <v>9.714398243813e-05</v>
       </c>
       <c r="M444" s="41">
         <f>EXP(-L444)</f>
-        <v>0.999909853573</v>
+        <v>0.999902860736</v>
       </c>
       <c r="N444" s="41">
         <f>IF(L444&gt;0,(1-M444)/L444,1)</f>
-        <v>0.999954926109</v>
+        <v>0.999951429582</v>
       </c>
       <c r="O444" s="41">
         <f>IF(L444&gt;0,(L444-1+M444)/L444^2,1/2)</f>
-        <v>0.499984981139</v>
+        <v>0.499983806296</v>
       </c>
       <c r="P444" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B444/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32222,11 +32226,11 @@
       </c>
       <c r="Q444" s="41">
         <f>(P444*N444+pool_b*M444)/(1-pool_ret*M444)</f>
-        <v>28.028402747444</v>
+        <v>28.026286360987</v>
       </c>
       <c r="R444" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q444+pool_b)*N444+P444*O444))</f>
-        <v>28.029666068564</v>
+        <v>28.02764759365</v>
       </c>
       <c r="S444" s="41">
         <f>IF(AND(R444&gt;=CO2_pH_hi_mt,R445&lt;CO2_pH_hi_mt),EXP(LN(A444)+(LN(A445)-LN(A444))*(R444-CO2_pH_hi_mt)/(R444-R445)),0)</f>
@@ -32276,19 +32280,19 @@
       </c>
       <c r="L445" s="41">
         <f>k_eff_CO2_l*B445</f>
-        <v>0.000106654317172</v>
+        <v>0.000114928106429</v>
       </c>
       <c r="M445" s="41">
         <f>EXP(-L445)</f>
-        <v>0.99989335137</v>
+        <v>0.999885078498</v>
       </c>
       <c r="N445" s="41">
         <f>IF(L445&gt;0,(1-M445)/L445,1)</f>
-        <v>0.999946674737</v>
+        <v>0.999942538148</v>
       </c>
       <c r="O445" s="41">
         <f>IF(L445&gt;0,(L445-1+M445)/L445^2,1/2)</f>
-        <v>0.499982222515</v>
+        <v>0.499980844274</v>
       </c>
       <c r="P445" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B445/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32296,11 +32300,11 @@
       </c>
       <c r="Q445" s="41">
         <f>(P445*N445+pool_b*M445)/(1-pool_ret*M445)</f>
-        <v>28.023409221948</v>
+        <v>28.020906272939</v>
       </c>
       <c r="R445" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q445+pool_b)*N445+P445*O445))</f>
-        <v>28.024903560881</v>
+        <v>28.02251640649</v>
       </c>
       <c r="S445" s="41">
         <f>IF(AND(R445&gt;=CO2_pH_hi_mt,R446&lt;CO2_pH_hi_mt),EXP(LN(A445)+(LN(A446)-LN(A445))*(R445-CO2_pH_hi_mt)/(R445-R446)),0)</f>
@@ -32350,19 +32354,19 @@
       </c>
       <c r="L446" s="41">
         <f>k_eff_CO2_l*B446</f>
-        <v>0.000125139668496</v>
+        <v>0.0001348474728521</v>
       </c>
       <c r="M446" s="41">
         <f>EXP(-L446)</f>
-        <v>0.999874868161</v>
+        <v>0.999865161619</v>
       </c>
       <c r="N446" s="41">
         <f>IF(L446&gt;0,(1-M446)/L446,1)</f>
-        <v>0.999937432776</v>
+        <v>0.999932579294</v>
       </c>
       <c r="O446" s="41">
         <f>IF(L446&gt;0,(L446-1+M446)/L446^2,1/2)</f>
-        <v>0.499979144048</v>
+        <v>0.499977530016</v>
       </c>
       <c r="P446" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B446/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32370,11 +32374,11 @@
       </c>
       <c r="Q446" s="41">
         <f>(P446*N446+pool_b*M446)/(1-pool_ret*M446)</f>
-        <v>28.017818165691</v>
+        <v>28.014882565771</v>
       </c>
       <c r="R446" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q446+pool_b)*N446+P446*O446))</f>
-        <v>28.019571164762</v>
+        <v>28.016771374425</v>
       </c>
       <c r="S446" s="41">
         <f>IF(AND(R446&gt;=CO2_pH_hi_mt,R447&lt;CO2_pH_hi_mt),EXP(LN(A446)+(LN(A447)-LN(A446))*(R446-CO2_pH_hi_mt)/(R446-R447)),0)</f>
@@ -32424,19 +32428,19 @@
       </c>
       <c r="L447" s="41">
         <f>k_eff_CO2_l*B447</f>
-        <v>0.0001458444547802</v>
+        <v>0.0001571584485796</v>
       </c>
       <c r="M447" s="41">
         <f>EXP(-L447)</f>
-        <v>0.99985416618</v>
+        <v>0.9998428539</v>
       </c>
       <c r="N447" s="41">
         <f>IF(L447&gt;0,(1-M447)/L447,1)</f>
-        <v>0.999927081317</v>
+        <v>0.999921424892</v>
       </c>
       <c r="O447" s="41">
         <f>IF(L447&gt;0,(L447-1+M447)/L447^2,1/2)</f>
-        <v>0.499975694232</v>
+        <v>0.499973806355</v>
       </c>
       <c r="P447" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B447/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32444,11 +32448,11 @@
       </c>
       <c r="Q447" s="41">
         <f>(P447*N447+pool_b*M447)/(1-pool_ret*M447)</f>
-        <v>28.011558347763</v>
+        <v>28.00813855713</v>
       </c>
       <c r="R447" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q447+pool_b)*N447+P447*O447))</f>
-        <v>28.013600944114</v>
+        <v>28.010339362057</v>
       </c>
       <c r="S447" s="41">
         <f>IF(AND(R447&gt;=CO2_pH_hi_mt,R448&lt;CO2_pH_hi_mt),EXP(LN(A447)+(LN(A448)-LN(A447))*(R447-CO2_pH_hi_mt)/(R447-R448)),0)</f>
@@ -32498,19 +32502,19 @@
       </c>
       <c r="L448" s="41">
         <f>k_eff_CO2_l*B448</f>
-        <v>0.0001690351514328</v>
+        <v>0.000182148181051</v>
       </c>
       <c r="M448" s="41">
         <f>EXP(-L448)</f>
-        <v>0.999830979134</v>
+        <v>0.999817868407</v>
       </c>
       <c r="N448" s="41">
         <f>IF(L448&gt;0,(1-M448)/L448,1)</f>
-        <v>0.999915487186</v>
+        <v>0.999908931439</v>
       </c>
       <c r="O448" s="41">
         <f>IF(L448&gt;0,(L448-1+M448)/L448^2,1/2)</f>
-        <v>0.499971831004</v>
+        <v>0.499969643795</v>
       </c>
       <c r="P448" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B448/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32518,11 +32522,11 @@
       </c>
       <c r="Q448" s="41">
         <f>(P448*N448+pool_b*M448)/(1-pool_ret*M448)</f>
-        <v>28.00455011452</v>
+        <v>28.00058850816</v>
       </c>
       <c r="R448" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q448+pool_b)*N448+P448*O448))</f>
-        <v>28.006916929646</v>
+        <v>28.003138596202</v>
       </c>
       <c r="S448" s="41">
         <f>IF(AND(R448&gt;=CO2_pH_hi_mt,R449&lt;CO2_pH_hi_mt),EXP(LN(A448)+(LN(A449)-LN(A448))*(R448-CO2_pH_hi_mt)/(R448-R449)),0)</f>
@@ -32572,19 +32576,19 @@
       </c>
       <c r="L449" s="41">
         <f>k_eff_CO2_l*B449</f>
-        <v>0.000195010228106</v>
+        <v>0.0002101382939275</v>
       </c>
       <c r="M449" s="41">
         <f>EXP(-L449)</f>
-        <v>0.999805008785</v>
+        <v>0.999789883784</v>
       </c>
       <c r="N449" s="41">
         <f>IF(L449&gt;0,(1-M449)/L449,1)</f>
-        <v>0.999902501224</v>
+        <v>0.999894938212</v>
       </c>
       <c r="O449" s="41">
         <f>IF(L449&gt;0,(L449-1+M449)/L449^2,1/2)</f>
-        <v>0.49996750114</v>
+        <v>0.499964978951</v>
       </c>
       <c r="P449" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B449/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32592,11 +32596,11 @@
       </c>
       <c r="Q449" s="41">
         <f>(P449*N449+pool_b*M449)/(1-pool_ret*M449)</f>
-        <v>27.996704411059</v>
+        <v>27.992136574119</v>
       </c>
       <c r="R449" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q449+pool_b)*N449+P449*O449))</f>
-        <v>27.999434185494</v>
+        <v>27.995077665173</v>
       </c>
       <c r="S449" s="41">
         <f>IF(AND(R449&gt;=CO2_pH_hi_mt,R450&lt;CO2_pH_hi_mt),EXP(LN(A449)+(LN(A450)-LN(A449))*(R449-CO2_pH_hi_mt)/(R449-R450)),0)</f>
@@ -32646,19 +32650,19 @@
       </c>
       <c r="L450" s="41">
         <f>k_eff_CO2_l*B450</f>
-        <v>0.0002241039900696</v>
+        <v>0.0002414890264625</v>
       </c>
       <c r="M450" s="41">
         <f>EXP(-L450)</f>
-        <v>0.999775921119</v>
+        <v>0.99975854013</v>
       </c>
       <c r="N450" s="41">
         <f>IF(L450&gt;0,(1-M450)/L450,1)</f>
-        <v>0.999887956375</v>
+        <v>0.999879265205</v>
       </c>
       <c r="O450" s="41">
         <f>IF(L450&gt;0,(L450-1+M450)/L450^2,1/2)</f>
-        <v>0.499962651212</v>
+        <v>0.499959754505</v>
       </c>
       <c r="P450" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B450/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32666,11 +32670,11 @@
       </c>
       <c r="Q450" s="41">
         <f>(P450*N450+pool_b*M450)/(1-pool_ret*M450)</f>
-        <v>27.987921693449</v>
+        <v>27.982675638531</v>
       </c>
       <c r="R450" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q450+pool_b)*N450+P450*O450))</f>
-        <v>27.991057771765</v>
+        <v>27.986054406636</v>
       </c>
       <c r="S450" s="41">
         <f>IF(AND(R450&gt;=CO2_pH_hi_mt,R451&lt;CO2_pH_hi_mt),EXP(LN(A450)+(LN(A451)-LN(A450))*(R450-CO2_pH_hi_mt)/(R450-R451)),0)</f>
@@ -32720,19 +32724,19 @@
       </c>
       <c r="L451" s="41">
         <f>k_eff_CO2_l*B451</f>
-        <v>0.0002566908807971</v>
+        <v>0.0002766038698654</v>
       </c>
       <c r="M451" s="41">
         <f>EXP(-L451)</f>
-        <v>0.999743342061</v>
+        <v>0.999723434381</v>
       </c>
       <c r="N451" s="41">
         <f>IF(L451&gt;0,(1-M451)/L451,1)</f>
-        <v>0.999871665541</v>
+        <v>0.999861710816</v>
       </c>
       <c r="O451" s="41">
         <f>IF(L451&gt;0,(L451-1+M451)/L451^2,1/2)</f>
-        <v>0.499957221456</v>
+        <v>0.499953903111</v>
       </c>
       <c r="P451" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B451/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32740,11 +32744,11 @@
       </c>
       <c r="Q451" s="41">
         <f>(P451*N451+pool_b*M451)/(1-pool_ret*M451)</f>
-        <v>27.978090720656</v>
+        <v>27.972086019301</v>
       </c>
       <c r="R451" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q451+pool_b)*N451+P451*O451))</f>
-        <v>27.981681592283</v>
+        <v>27.97595467362</v>
       </c>
       <c r="S451" s="41">
         <f>IF(AND(R451&gt;=CO2_pH_hi_mt,R452&lt;CO2_pH_hi_mt),EXP(LN(A451)+(LN(A452)-LN(A451))*(R451-CO2_pH_hi_mt)/(R451-R452)),0)</f>
@@ -32794,19 +32798,19 @@
       </c>
       <c r="L452" s="41">
         <f>k_eff_CO2_l*B452</f>
-        <v>0.000293190301141</v>
+        <v>0.0003159347603263</v>
       </c>
       <c r="M452" s="41">
         <f>EXP(-L452)</f>
-        <v>0.999706852675</v>
+        <v>0.999684115142</v>
       </c>
       <c r="N452" s="41">
         <f>IF(L452&gt;0,(1-M452)/L452,1)</f>
-        <v>0.999853419175</v>
+        <v>0.999842049254</v>
       </c>
       <c r="O452" s="41">
         <f>IF(L452&gt;0,(L452-1+M452)/L452^2,1/2)</f>
-        <v>0.499951139352</v>
+        <v>0.499947348393</v>
       </c>
       <c r="P452" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B452/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32814,11 +32818,11 @@
       </c>
       <c r="Q452" s="41">
         <f>(P452*N452+pool_b*M452)/(1-pool_ret*M452)</f>
-        <v>27.967087214288</v>
+        <v>27.960234034374</v>
       </c>
       <c r="R452" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q452+pool_b)*N452+P452*O452))</f>
-        <v>27.971187116248</v>
+        <v>27.964650966364</v>
       </c>
       <c r="S452" s="41">
         <f>IF(AND(R452&gt;=CO2_pH_hi_mt,R453&lt;CO2_pH_hi_mt),EXP(LN(A452)+(LN(A453)-LN(A452))*(R452-CO2_pH_hi_mt)/(R452-R453)),0)</f>
@@ -32868,19 +32872,19 @@
       </c>
       <c r="L453" s="41">
         <f>k_eff_CO2_l*B453</f>
-        <v>0.0003340720071182</v>
+        <v>0.0003599878955405</v>
       </c>
       <c r="M453" s="41">
         <f>EXP(-L453)</f>
-        <v>0.999665983789</v>
+        <v>0.999640076892</v>
       </c>
       <c r="N453" s="41">
         <f>IF(L453&gt;0,(1-M453)/L453,1)</f>
-        <v>0.999832982596</v>
+        <v>0.999820027649</v>
       </c>
       <c r="O453" s="41">
         <f>IF(L453&gt;0,(L453-1+M453)/L453^2,1/2)</f>
-        <v>0.499944325832</v>
+        <v>0.499940007475</v>
       </c>
       <c r="P453" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B453/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32888,11 +32892,11 @@
       </c>
       <c r="Q453" s="41">
         <f>(P453*N453+pool_b*M453)/(1-pool_ret*M453)</f>
-        <v>27.954772373494</v>
+        <v>27.946970413781</v>
       </c>
       <c r="R453" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q453+pool_b)*N453+P453*O453))</f>
-        <v>27.959441961717</v>
+        <v>27.952000917724</v>
       </c>
       <c r="S453" s="41">
         <f>IF(AND(R453&gt;=CO2_pH_hi_mt,R454&lt;CO2_pH_hi_mt),EXP(LN(A453)+(LN(A454)-LN(A453))*(R453-CO2_pH_hi_mt)/(R453-R454)),0)</f>
@@ -32942,19 +32946,19 @@
       </c>
       <c r="L454" s="41">
         <f>k_eff_CO2_l*B454</f>
-        <v>0.0003798621557799</v>
+        <v>0.0004093302495898</v>
       </c>
       <c r="M454" s="41">
         <f>EXP(-L454)</f>
-        <v>0.999620209983</v>
+        <v>0.999590753515</v>
       </c>
       <c r="N454" s="41">
         <f>IF(L454&gt;0,(1-M454)/L454,1)</f>
-        <v>0.999810092969</v>
+        <v>0.999795362798</v>
       </c>
       <c r="O454" s="41">
         <f>IF(L454&gt;0,(L454-1+M454)/L454^2,1/2)</f>
-        <v>0.499936695642</v>
+        <v>0.499931785168</v>
       </c>
       <c r="P454" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B454/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32962,11 +32966,11 @@
       </c>
       <c r="Q454" s="41">
         <f>(P454*N454+pool_b*M454)/(1-pool_ret*M454)</f>
-        <v>27.940991231607</v>
+        <v>27.932128544224</v>
       </c>
       <c r="R454" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q454+pool_b)*N454+P454*O454))</f>
-        <v>27.946298328144</v>
+        <v>27.937845618818</v>
       </c>
       <c r="S454" s="41">
         <f>IF(AND(R454&gt;=CO2_pH_hi_mt,R455&lt;CO2_pH_hi_mt),EXP(LN(A454)+(LN(A455)-LN(A454))*(R454-CO2_pH_hi_mt)/(R454-R455)),0)</f>
@@ -33016,19 +33020,19 @@
       </c>
       <c r="L455" s="41">
         <f>k_eff_CO2_l*B455</f>
-        <v>0.0004311500769744</v>
+        <v>0.000464596870031</v>
       </c>
       <c r="M455" s="41">
         <f>EXP(-L455)</f>
-        <v>0.999568942855</v>
+        <v>0.999535511038</v>
       </c>
       <c r="N455" s="41">
         <f>IF(L455&gt;0,(1-M455)/L455,1)</f>
-        <v>0.99978445594</v>
+        <v>0.999767737536</v>
       </c>
       <c r="O455" s="41">
         <f>IF(L455&gt;0,(L455-1+M455)/L455^2,1/2)</f>
-        <v>0.499928149466</v>
+        <v>0.499922576184</v>
       </c>
       <c r="P455" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B455/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33036,11 +33040,11 @@
       </c>
       <c r="Q455" s="41">
         <f>(P455*N455+pool_b*M455)/(1-pool_ret*M455)</f>
-        <v>27.925570840489</v>
+        <v>27.915522531825</v>
       </c>
       <c r="R455" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q455+pool_b)*N455+P455*O455))</f>
-        <v>27.931591264548</v>
+        <v>27.92200777117</v>
       </c>
       <c r="S455" s="41">
         <f>IF(AND(R455&gt;=CO2_pH_hi_mt,R456&lt;CO2_pH_hi_mt),EXP(LN(A455)+(LN(A456)-LN(A455))*(R455-CO2_pH_hi_mt)/(R455-R456)),0)</f>
@@ -33090,19 +33094,19 @@
       </c>
       <c r="L456" s="41">
         <f>k_eff_CO2_l*B456</f>
-        <v>0.0004885958581595</v>
+        <v>0.0005264990511054</v>
       </c>
       <c r="M456" s="41">
         <f>EXP(-L456)</f>
-        <v>0.999511523485</v>
+        <v>0.999473639525</v>
       </c>
       <c r="N456" s="41">
         <f>IF(L456&gt;0,(1-M456)/L456,1)</f>
-        <v>0.999755741854</v>
+        <v>0.999736796669</v>
       </c>
       <c r="O456" s="41">
         <f>IF(L456&gt;0,(L456-1+M456)/L456^2,1/2)</f>
-        <v>0.49991857741</v>
+        <v>0.499912261586</v>
       </c>
       <c r="P456" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B456/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33110,11 +33114,11 @@
       </c>
       <c r="Q456" s="41">
         <f>(P456*N456+pool_b*M456)/(1-pool_ret*M456)</f>
-        <v>27.908318268052</v>
+        <v>27.896945068309</v>
       </c>
       <c r="R456" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q456+pool_b)*N456+P456*O456))</f>
-        <v>27.915136759468</v>
+        <v>27.904289651388</v>
       </c>
       <c r="S456" s="41">
         <f>IF(AND(R456&gt;=CO2_pH_hi_mt,R457&lt;CO2_pH_hi_mt),EXP(LN(A456)+(LN(A457)-LN(A456))*(R456-CO2_pH_hi_mt)/(R456-R457)),0)</f>
@@ -33164,19 +33168,19 @@
       </c>
       <c r="L457" s="41">
         <f>k_eff_CO2_l*B457</f>
-        <v>0.0005529388398813</v>
+        <v>0.0005958334882605</v>
       </c>
       <c r="M457" s="41">
         <f>EXP(-L457)</f>
-        <v>0.999447214003</v>
+        <v>0.999404343985</v>
       </c>
       <c r="N457" s="41">
         <f>IF(L457&gt;0,(1-M457)/L457,1)</f>
-        <v>0.99972358153</v>
+        <v>0.999702142417</v>
       </c>
       <c r="O457" s="41">
         <f>IF(L457&gt;0,(L457-1+M457)/L457^2,1/2)</f>
-        <v>0.499907856005</v>
+        <v>0.499900709165</v>
       </c>
       <c r="P457" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B457/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33184,11 +33188,11 @@
       </c>
       <c r="Q457" s="41">
         <f>(P457*N457+pool_b*M457)/(1-pool_ret*M457)</f>
-        <v>27.889018394176</v>
+        <v>27.876165085827</v>
       </c>
       <c r="R457" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q457+pool_b)*N457+P457*O457))</f>
-        <v>27.896729638547</v>
+        <v>27.884470874124</v>
       </c>
       <c r="S457" s="41">
         <f>IF(AND(R457&gt;=CO2_pH_hi_mt,R458&lt;CO2_pH_hi_mt),EXP(LN(A457)+(LN(A458)-LN(A457))*(R457-CO2_pH_hi_mt)/(R457-R458)),0)</f>
@@ -33238,19 +33242,19 @@
       </c>
       <c r="L458" s="41">
         <f>k_eff_CO2_l*B458</f>
-        <v>0.0006250071312588</v>
+        <v>0.0006734925318062</v>
       </c>
       <c r="M458" s="41">
         <f>EXP(-L458)</f>
-        <v>0.999375188145</v>
+        <v>0.999326734213</v>
       </c>
       <c r="N458" s="41">
         <f>IF(L458&gt;0,(1-M458)/L458,1)</f>
-        <v>0.99968756153</v>
+        <v>0.99966332932</v>
       </c>
       <c r="O458" s="41">
         <f>IF(L458&gt;0,(L458-1+M458)/L458^2,1/2)</f>
-        <v>0.499895848439</v>
+        <v>0.49988777017</v>
       </c>
       <c r="P458" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B458/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33258,11 +33262,11 @@
       </c>
       <c r="Q458" s="41">
         <f>(P458*N458+pool_b*M458)/(1-pool_ret*M458)</f>
-        <v>27.867431490296</v>
+        <v>27.85292518598</v>
       </c>
       <c r="R458" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q458+pool_b)*N458+P458*O458))</f>
-        <v>27.876141255774</v>
+        <v>27.862305939684</v>
       </c>
       <c r="S458" s="41">
         <f>IF(AND(R458&gt;=CO2_pH_hi_mt,R459&lt;CO2_pH_hi_mt),EXP(LN(A458)+(LN(A459)-LN(A458))*(R458-CO2_pH_hi_mt)/(R458-R459)),0)</f>
@@ -33312,19 +33316,19 @@
       </c>
       <c r="L459" s="41">
         <f>k_eff_CO2_l*B459</f>
-        <v>0.0007057282679405</v>
+        <v>0.0007604756716698</v>
       </c>
       <c r="M459" s="41">
         <f>EXP(-L459)</f>
-        <v>0.9992945207</v>
+        <v>0.999239813417</v>
       </c>
       <c r="N459" s="41">
         <f>IF(L459&gt;0,(1-M459)/L459,1)</f>
-        <v>0.99964721886</v>
+        <v>0.999619858533</v>
       </c>
       <c r="O459" s="41">
         <f>IF(L459&gt;0,(L459-1+M459)/L459^2,1/2)</f>
-        <v>0.499882399229</v>
+        <v>0.499873278291</v>
       </c>
       <c r="P459" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B459/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33332,11 +33336,11 @@
       </c>
       <c r="Q459" s="41">
         <f>(P459*N459+pool_b*M459)/(1-pool_ret*M459)</f>
-        <v>27.843290568422</v>
+        <v>27.826938829406</v>
       </c>
       <c r="R459" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q459+pool_b)*N459+P459*O459))</f>
-        <v>27.853116964726</v>
+        <v>27.837521553104</v>
       </c>
       <c r="S459" s="41">
         <f>IF(AND(R459&gt;=CO2_pH_hi_mt,R460&lt;CO2_pH_hi_mt),EXP(LN(A459)+(LN(A460)-LN(A459))*(R459-CO2_pH_hi_mt)/(R459-R460)),0)</f>
@@ -33386,19 +33390,19 @@
       </c>
       <c r="L460" s="41">
         <f>k_eff_CO2_l*B460</f>
-        <v>0.0007961411497035</v>
+        <v>0.0008579024010638</v>
       </c>
       <c r="M460" s="41">
         <f>EXP(-L460)</f>
-        <v>0.999204175687</v>
+        <v>0.999142465492</v>
       </c>
       <c r="N460" s="41">
         <f>IF(L460&gt;0,(1-M460)/L460,1)</f>
-        <v>0.999602035044</v>
+        <v>0.999571171439</v>
       </c>
       <c r="O460" s="41">
         <f>IF(L460&gt;0,(L460-1+M460)/L460^2,1/2)</f>
-        <v>0.499867336248</v>
+        <v>0.499857046929</v>
       </c>
       <c r="P460" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B460/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33406,11 +33410,11 @@
       </c>
       <c r="Q460" s="41">
         <f>(P460*N460+pool_b*M460)/(1-pool_ret*M460)</f>
-        <v>27.816298486416</v>
+        <v>27.797887273865</v>
       </c>
       <c r="R460" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q460+pool_b)*N460+P460*O460))</f>
-        <v>27.827373357184</v>
+        <v>27.809813703293</v>
       </c>
       <c r="S460" s="41">
         <f>IF(AND(R460&gt;=CO2_pH_hi_mt,R461&lt;CO2_pH_hi_mt),EXP(LN(A460)+(LN(A461)-LN(A460))*(R460-CO2_pH_hi_mt)/(R460-R461)),0)</f>
@@ -33460,19 +33464,19 @@
       </c>
       <c r="L461" s="41">
         <f>k_eff_CO2_l*B461</f>
-        <v>0.0008974094113353</v>
+        <v>0.0009670266246237</v>
       </c>
       <c r="M461" s="41">
         <f>EXP(-L461)</f>
-        <v>0.99910299314</v>
+        <v>0.999033440795</v>
       </c>
       <c r="N461" s="41">
         <f>IF(L461&gt;0,(1-M461)/L461,1)</f>
-        <v>0.999551429488</v>
+        <v>0.999516642507</v>
       </c>
       <c r="O461" s="41">
         <f>IF(L461&gt;0,(L461-1+M461)/L461^2,1/2)</f>
-        <v>0.499850465346</v>
+        <v>0.499838867847</v>
       </c>
       <c r="P461" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B461/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33480,11 +33484,11 @@
       </c>
       <c r="Q461" s="41">
         <f>(P461*N461+pool_b*M461)/(1-pool_ret*M461)</f>
-        <v>27.786124798155</v>
+        <v>27.765416251135</v>
       </c>
       <c r="R461" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q461+pool_b)*N461+P461*O461))</f>
-        <v>27.798595258404</v>
+        <v>27.778844492866</v>
       </c>
       <c r="S461" s="41">
         <f>IF(AND(R461&gt;=CO2_pH_hi_mt,R462&lt;CO2_pH_hi_mt),EXP(LN(A461)+(LN(A462)-LN(A461))*(R461-CO2_pH_hi_mt)/(R461-R462)),0)</f>
@@ -33534,19 +33538,19 @@
       </c>
       <c r="L462" s="41">
         <f>k_eff_CO2_l*B462</f>
-        <v>0.001010836399</v>
+        <v>0.001089252796</v>
       </c>
       <c r="M462" s="41">
         <f>EXP(-L462)</f>
-        <v>0.998989674324</v>
+        <v>0.998911340224</v>
       </c>
       <c r="N462" s="41">
         <f>IF(L462&gt;0,(1-M462)/L462,1)</f>
-        <v>0.999494752056</v>
+        <v>0.999455571293</v>
       </c>
       <c r="O462" s="41">
         <f>IF(L462&gt;0,(L462-1+M462)/L462^2,1/2)</f>
-        <v>0.499831569912</v>
+        <v>0.499818507329</v>
       </c>
       <c r="P462" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B462/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33554,11 +33558,11 @@
       </c>
       <c r="Q462" s="41">
         <f>(P462*N462+pool_b*M462)/(1-pool_ret*M462)</f>
-        <v>27.752402339962</v>
+        <v>27.729132376595</v>
       </c>
       <c r="R462" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q462+pool_b)*N462+P462*O462))</f>
-        <v>27.766432470593</v>
+        <v>27.744238712882</v>
       </c>
       <c r="S462" s="41">
         <f>IF(AND(R462&gt;=CO2_pH_hi_mt,R463&lt;CO2_pH_hi_mt),EXP(LN(A462)+(LN(A463)-LN(A462))*(R462-CO2_pH_hi_mt)/(R462-R463)),0)</f>
@@ -33608,19 +33612,19 @@
       </c>
       <c r="L463" s="41">
         <f>k_eff_CO2_l*B463</f>
-        <v>0.001137881944</v>
+        <v>0.001226153996</v>
       </c>
       <c r="M463" s="41">
         <f>EXP(-L463)</f>
-        <v>0.998862765198</v>
+        <v>0.998774597424</v>
       </c>
       <c r="N463" s="41">
         <f>IF(L463&gt;0,(1-M463)/L463,1)</f>
-        <v>0.999431274762</v>
+        <v>0.999387173501</v>
       </c>
       <c r="O463" s="41">
         <f>IF(L463&gt;0,(L463-1+M463)/L463^2,1/2)</f>
-        <v>0.499810406935</v>
+        <v>0.499795703592</v>
       </c>
       <c r="P463" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B463/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33628,11 +33632,11 @@
       </c>
       <c r="Q463" s="41">
         <f>(P463*N463+pool_b*M463)/(1-pool_ret*M463)</f>
-        <v>27.714723548707</v>
+        <v>27.688599290311</v>
       </c>
       <c r="R463" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q463+pool_b)*N463+P463*O463))</f>
-        <v>27.730496260315</v>
+        <v>27.705580161244</v>
       </c>
       <c r="S463" s="41">
         <f>IF(AND(R463&gt;=CO2_pH_hi_mt,R464&lt;CO2_pH_hi_mt),EXP(LN(A463)+(LN(A464)-LN(A463))*(R463-CO2_pH_hi_mt)/(R463-R464)),0)</f>
@@ -33682,19 +33686,19 @@
       </c>
       <c r="L464" s="41">
         <f>k_eff_CO2_l*B464</f>
-        <v>0.001280181152</v>
+        <v>0.001379492173</v>
       </c>
       <c r="M464" s="41">
         <f>EXP(-L464)</f>
-        <v>0.99872063793</v>
+        <v>0.998621458889</v>
       </c>
       <c r="N464" s="41">
         <f>IF(L464&gt;0,(1-M464)/L464,1)</f>
-        <v>0.99936018248</v>
+        <v>0.999310570971</v>
       </c>
       <c r="O464" s="41">
         <f>IF(L464&gt;0,(L464-1+M464)/L464^2,1/2)</f>
-        <v>0.499786704736</v>
+        <v>0.499770163909</v>
       </c>
       <c r="P464" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B464/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33702,11 +33706,11 @@
       </c>
       <c r="Q464" s="41">
         <f>(P464*N464+pool_b*M464)/(1-pool_ret*M464)</f>
-        <v>27.672636512444</v>
+        <v>27.643333535176</v>
       </c>
       <c r="R464" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q464+pool_b)*N464+P464*O464))</f>
-        <v>27.690355590542</v>
+        <v>27.662407710022</v>
       </c>
       <c r="S464" s="41">
         <f>IF(AND(R464&gt;=CO2_pH_hi_mt,R465&lt;CO2_pH_hi_mt),EXP(LN(A464)+(LN(A465)-LN(A464))*(R464-CO2_pH_hi_mt)/(R464-R465)),0)</f>
@@ -33756,19 +33760,19 @@
       </c>
       <c r="L465" s="41">
         <f>k_eff_CO2_l*B465</f>
-        <v>0.001439565448</v>
+        <v>0.001551240826</v>
       </c>
       <c r="M465" s="41">
         <f>EXP(-L465)</f>
-        <v>0.998561470229</v>
+        <v>0.998449961727</v>
       </c>
       <c r="N465" s="41">
         <f>IF(L465&gt;0,(1-M465)/L465,1)</f>
-        <v>0.999280562543</v>
+        <v>0.99922478049</v>
       </c>
       <c r="O465" s="41">
         <f>IF(L465&gt;0,(L465-1+M465)/L465^2,1/2)</f>
-        <v>0.499760158713</v>
+        <v>0.499741560087</v>
       </c>
       <c r="P465" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B465/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33776,11 +33780,11 @@
       </c>
       <c r="Q465" s="41">
         <f>(P465*N465+pool_b*M465)/(1-pool_ret*M465)</f>
-        <v>27.625640761928</v>
+        <v>27.592800186564</v>
       </c>
       <c r="R465" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q465+pool_b)*N465+P465*O465))</f>
-        <v>27.645533105246</v>
+        <v>27.614211135441</v>
       </c>
       <c r="S465" s="41">
         <f>IF(AND(R465&gt;=CO2_pH_hi_mt,R466&lt;CO2_pH_hi_mt),EXP(LN(A465)+(LN(A466)-LN(A465))*(R465-CO2_pH_hi_mt)/(R465-R466)),0)</f>
@@ -33830,19 +33834,19 @@
       </c>
       <c r="L466" s="41">
         <f>k_eff_CO2_l*B466</f>
-        <v>0.001618086144</v>
+        <v>0.001743610399</v>
       </c>
       <c r="M466" s="41">
         <f>EXP(-L466)</f>
-        <v>0.998383222252</v>
+        <v>0.998257908807</v>
       </c>
       <c r="N466" s="41">
         <f>IF(L466&gt;0,(1-M466)/L466,1)</f>
-        <v>0.999191393119</v>
+        <v>0.999128701276</v>
       </c>
       <c r="O466" s="41">
         <f>IF(L466&gt;0,(L466-1+M466)/L466^2,1/2)</f>
-        <v>0.499730428046</v>
+        <v>0.499709524892</v>
       </c>
       <c r="P466" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B466/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33850,11 +33854,11 @@
       </c>
       <c r="Q466" s="41">
         <f>(P466*N466+pool_b*M466)/(1-pool_ret*M466)</f>
-        <v>27.573182821062</v>
+        <v>27.536408259493</v>
       </c>
       <c r="R466" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q466+pool_b)*N466+P466*O466))</f>
-        <v>27.595500883692</v>
+        <v>27.560426735191</v>
       </c>
       <c r="S466" s="41">
         <f>IF(AND(R466&gt;=CO2_pH_hi_mt,R467&lt;CO2_pH_hi_mt),EXP(LN(A466)+(LN(A467)-LN(A466))*(R466-CO2_pH_hi_mt)/(R466-R467)),0)</f>
@@ -33904,19 +33908,19 @@
       </c>
       <c r="L467" s="41">
         <f>k_eff_CO2_l*B467</f>
-        <v>0.001818040842</v>
+        <v>0.001959076734</v>
       </c>
       <c r="M467" s="41">
         <f>EXP(-L467)</f>
-        <v>0.998183610793</v>
+        <v>0.998042841004</v>
       </c>
       <c r="N467" s="41">
         <f>IF(L467&gt;0,(1-M467)/L467,1)</f>
-        <v>0.999091530207</v>
+        <v>0.999021100983</v>
       </c>
       <c r="O467" s="41">
         <f>IF(L467&gt;0,(L467-1+M467)/L467^2,1/2)</f>
-        <v>0.499697130864</v>
+        <v>0.499673647064</v>
       </c>
       <c r="P467" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B467/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33924,11 +33928,11 @@
       </c>
       <c r="Q467" s="41">
         <f>(P467*N467+pool_b*M467)/(1-pool_ret*M467)</f>
-        <v>27.514651546922</v>
+        <v>27.473505934052</v>
       </c>
       <c r="R467" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q467+pool_b)*N467+P467*O467))</f>
-        <v>27.539675993557</v>
+        <v>27.500432771881</v>
       </c>
       <c r="S467" s="41">
         <f>IF(AND(R467&gt;=CO2_pH_hi_mt,R468&lt;CO2_pH_hi_mt),EXP(LN(A467)+(LN(A468)-LN(A467))*(R467-CO2_pH_hi_mt)/(R467-R468)),0)</f>
@@ -33978,19 +33982,19 @@
       </c>
       <c r="L468" s="41">
         <f>k_eff_CO2_l*B468</f>
-        <v>0.002042003007</v>
+        <v>0.002200412933</v>
       </c>
       <c r="M468" s="41">
         <f>EXP(-L468)</f>
-        <v>0.997960080463</v>
+        <v>0.997802006201</v>
       </c>
       <c r="N468" s="41">
         <f>IF(L468&gt;0,(1-M468)/L468,1)</f>
-        <v>0.998979693105</v>
+        <v>0.998900600059</v>
       </c>
       <c r="O468" s="41">
         <f>IF(L468&gt;0,(L468-1+M468)/L468^2,1/2)</f>
-        <v>0.499659839837</v>
+        <v>0.499633466174</v>
       </c>
       <c r="P468" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B468/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33998,11 +34002,11 @@
       </c>
       <c r="Q468" s="41">
         <f>(P468*N468+pool_b*M468)/(1-pool_ret*M468)</f>
-        <v>27.44937330595</v>
+        <v>27.403375658336</v>
       </c>
       <c r="R468" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q468+pool_b)*N468+P468*O468))</f>
-        <v>27.477415887188</v>
+        <v>27.433544798968</v>
       </c>
       <c r="S468" s="41">
         <f>IF(AND(R468&gt;=CO2_pH_hi_mt,R469&lt;CO2_pH_hi_mt),EXP(LN(A468)+(LN(A469)-LN(A468))*(R468-CO2_pH_hi_mt)/(R468-R469)),0)</f>
@@ -34052,19 +34056,19 @@
       </c>
       <c r="L469" s="41">
         <f>k_eff_CO2_l*B469</f>
-        <v>0.002292855083</v>
+        <v>0.002470725048</v>
       </c>
       <c r="M469" s="41">
         <f>EXP(-L469)</f>
-        <v>0.997709771502</v>
+        <v>0.997532324681</v>
       </c>
       <c r="N469" s="41">
         <f>IF(L469&gt;0,(1-M469)/L469,1)</f>
-        <v>0.998854448154</v>
+        <v>0.998765654261</v>
       </c>
       <c r="O469" s="41">
         <f>IF(L469&gt;0,(L469-1+M469)/L469^2,1/2)</f>
-        <v>0.49961807643</v>
+        <v>0.499588466728</v>
       </c>
       <c r="P469" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B469/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34072,11 +34076,11 @@
       </c>
       <c r="Q469" s="41">
         <f>(P469*N469+pool_b*M469)/(1-pool_ret*M469)</f>
-        <v>27.376607052844</v>
+        <v>27.325229211051</v>
       </c>
       <c r="R469" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q469+pool_b)*N469+P469*O469))</f>
-        <v>27.408013704348</v>
+        <v>27.359010947392</v>
       </c>
       <c r="S469" s="41">
         <f>IF(AND(R469&gt;=CO2_pH_hi_mt,R470&lt;CO2_pH_hi_mt),EXP(LN(A469)+(LN(A470)-LN(A469))*(R469-CO2_pH_hi_mt)/(R469-R470)),0)</f>
@@ -34126,19 +34130,19 @@
       </c>
       <c r="L470" s="41">
         <f>k_eff_CO2_l*B470</f>
-        <v>0.002573825594</v>
+        <v>0.00277349206</v>
       </c>
       <c r="M470" s="41">
         <f>EXP(-L470)</f>
-        <v>0.997429483855</v>
+        <v>0.997230350516</v>
       </c>
       <c r="N470" s="41">
         <f>IF(L470&gt;0,(1-M470)/L470,1)</f>
-        <v>0.998714190589</v>
+        <v>0.998614535125</v>
       </c>
       <c r="O470" s="41">
         <f>IF(L470&gt;0,(L470-1+M470)/L470^2,1/2)</f>
-        <v>0.499571304938</v>
+        <v>0.499538071645</v>
       </c>
       <c r="P470" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B470/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34146,11 +34150,11 @@
       </c>
       <c r="Q470" s="41">
         <f>(P470*N470+pool_b*M470)/(1-pool_ret*M470)</f>
-        <v>27.29553940323</v>
+        <v>27.238202833924</v>
       </c>
       <c r="R470" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q470+pool_b)*N470+P470*O470))</f>
-        <v>27.330693568117</v>
+        <v>27.276007277759</v>
       </c>
       <c r="S470" s="41">
         <f>IF(AND(R470&gt;=CO2_pH_hi_mt,R471&lt;CO2_pH_hi_mt),EXP(LN(A470)+(LN(A471)-LN(A470))*(R470-CO2_pH_hi_mt)/(R470-R471)),0)</f>
@@ -34200,19 +34204,19 @@
       </c>
       <c r="L471" s="41">
         <f>k_eff_CO2_l*B471</f>
-        <v>0.002888530698</v>
+        <v>0.003112610649</v>
       </c>
       <c r="M471" s="41">
         <f>EXP(-L471)</f>
-        <v>0.997115637093</v>
+        <v>0.996892228501</v>
       </c>
       <c r="N471" s="41">
         <f>IF(L471&gt;0,(1-M471)/L471,1)</f>
-        <v>0.998557124249</v>
+        <v>0.998445308144</v>
       </c>
       <c r="O471" s="41">
         <f>IF(L471&gt;0,(L471-1+M471)/L471^2,1/2)</f>
-        <v>0.499518925659</v>
+        <v>0.499481634989</v>
       </c>
       <c r="P471" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B471/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34220,11 +34224,11 @@
       </c>
       <c r="Q471" s="41">
         <f>(P471*N471+pool_b*M471)/(1-pool_ret*M471)</f>
-        <v>27.205279821034</v>
+        <v>27.14135257765</v>
       </c>
       <c r="R471" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q471+pool_b)*N471+P471*O471))</f>
-        <v>27.244605989097</v>
+        <v>27.183633334932</v>
       </c>
       <c r="S471" s="41">
         <f>IF(AND(R471&gt;=CO2_pH_hi_mt,R472&lt;CO2_pH_hi_mt),EXP(LN(A471)+(LN(A472)-LN(A471))*(R471-CO2_pH_hi_mt)/(R471-R472)),0)</f>
@@ -34274,19 +34278,19 @@
       </c>
       <c r="L472" s="41">
         <f>k_eff_CO2_l*B472</f>
-        <v>0.00324102072</v>
+        <v>0.003492445352</v>
       </c>
       <c r="M472" s="41">
         <f>EXP(-L472)</f>
-        <v>0.996764225718</v>
+        <v>0.996513646142</v>
       </c>
       <c r="N472" s="41">
         <f>IF(L472&gt;0,(1-M472)/L472,1)</f>
-        <v>0.998381238925</v>
+        <v>0.998255808413</v>
       </c>
       <c r="O472" s="41">
         <f>IF(L472&gt;0,(L472-1+M472)/L472^2,1/2)</f>
-        <v>0.499460267282</v>
+        <v>0.499418433639</v>
       </c>
       <c r="P472" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B472/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34294,11 +34298,11 @@
       </c>
       <c r="Q472" s="41">
         <f>(P472*N472+pool_b*M472)/(1-pool_ret*M472)</f>
-        <v>27.104856077123</v>
+        <v>27.033650044934</v>
       </c>
       <c r="R472" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q472+pool_b)*N472+P472*O472))</f>
-        <v>27.14882352701</v>
+        <v>27.080908079842</v>
       </c>
       <c r="S472" s="41">
         <f>IF(AND(R472&gt;=CO2_pH_hi_mt,R473&lt;CO2_pH_hi_mt),EXP(LN(A472)+(LN(A473)-LN(A472))*(R472-CO2_pH_hi_mt)/(R472-R473)),0)</f>
@@ -34348,19 +34352,19 @@
       </c>
       <c r="L473" s="41">
         <f>k_eff_CO2_l*B473</f>
-        <v>0.003635832291</v>
+        <v>0.003917884728</v>
       </c>
       <c r="M473" s="41">
         <f>EXP(-L473)</f>
-        <v>0.996370769344</v>
+        <v>0.996089780169</v>
       </c>
       <c r="N473" s="41">
         <f>IF(L473&gt;0,(1-M473)/L473,1)</f>
-        <v>0.998184285066</v>
+        <v>0.998043613435</v>
       </c>
       <c r="O473" s="41">
         <f>IF(L473&gt;0,(L473-1+M473)/L473^2,1/2)</f>
-        <v>0.499394578354</v>
+        <v>0.499347658287</v>
       </c>
       <c r="P473" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B473/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34368,11 +34372,11 @@
       </c>
       <c r="Q473" s="41">
         <f>(P473*N473+pool_b*M473)/(1-pool_ret*M473)</f>
-        <v>26.993210177833</v>
+        <v>26.913978760523</v>
       </c>
       <c r="R473" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q473+pool_b)*N473+P473*O473))</f>
-        <v>27.042336898806</v>
+        <v>26.966766417424</v>
       </c>
       <c r="S473" s="41">
         <f>IF(AND(R473&gt;=CO2_pH_hi_mt,R474&lt;CO2_pH_hi_mt),EXP(LN(A473)+(LN(A474)-LN(A473))*(R473-CO2_pH_hi_mt)/(R473-R474)),0)</f>
@@ -34422,19 +34426,19 @@
       </c>
       <c r="L474" s="41">
         <f>k_eff_CO2_l*B474</f>
-        <v>0.004078046726</v>
+        <v>0.004394404282</v>
       </c>
       <c r="M474" s="41">
         <f>EXP(-L474)</f>
-        <v>0.995930257215</v>
+        <v>0.995615236984</v>
       </c>
       <c r="N474" s="41">
         <f>IF(L474&gt;0,(1-M474)/L474,1)</f>
-        <v>0.997963745558</v>
+        <v>0.997806012791</v>
       </c>
       <c r="O474" s="41">
         <f>IF(L474&gt;0,(L474-1+M474)/L474^2,1/2)</f>
-        <v>0.499321017917</v>
+        <v>0.499268403197</v>
       </c>
       <c r="P474" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B474/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34442,11 +34446,11 @@
       </c>
       <c r="Q474" s="41">
         <f>(P474*N474+pool_b*M474)/(1-pool_ret*M474)</f>
-        <v>26.86919501051</v>
+        <v>26.781131450937</v>
       </c>
       <c r="R474" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q474+pool_b)*N474+P474*O474))</f>
-        <v>26.924051768671</v>
+        <v>26.840056589983</v>
       </c>
       <c r="S474" s="41">
         <f>IF(AND(R474&gt;=CO2_pH_hi_mt,R475&lt;CO2_pH_hi_mt),EXP(LN(A474)+(LN(A475)-LN(A474))*(R474-CO2_pH_hi_mt)/(R474-R475)),0)</f>
@@ -34496,19 +34500,19 @@
       </c>
       <c r="L475" s="41">
         <f>k_eff_CO2_l*B475</f>
-        <v>0.004573355427</v>
+        <v>0.004928136931</v>
       </c>
       <c r="M475" s="41">
         <f>EXP(-L475)</f>
-        <v>0.995437086438</v>
+        <v>0.995083986413</v>
       </c>
       <c r="N475" s="41">
         <f>IF(L475&gt;0,(1-M475)/L475,1)</f>
-        <v>0.997716804234</v>
+        <v>0.997539974308</v>
       </c>
       <c r="O475" s="41">
         <f>IF(L475&gt;0,(L475-1+M475)/L475^2,1/2)</f>
-        <v>0.499238644784</v>
+        <v>0.499179654787</v>
       </c>
       <c r="P475" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B475/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34516,11 +34520,11 @@
       </c>
       <c r="Q475" s="41">
         <f>(P475*N475+pool_b*M475)/(1-pool_ret*M475)</f>
-        <v>26.731572008256</v>
+        <v>26.633808575601</v>
       </c>
       <c r="R475" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q475+pool_b)*N475+P475*O475))</f>
-        <v>26.792786507734</v>
+        <v>26.69953876139</v>
       </c>
       <c r="S475" s="41">
         <f>IF(AND(R475&gt;=CO2_pH_hi_mt,R476&lt;CO2_pH_hi_mt),EXP(LN(A475)+(LN(A476)-LN(A475))*(R475-CO2_pH_hi_mt)/(R475-R476)),0)</f>
@@ -34570,19 +34574,19 @@
       </c>
       <c r="L476" s="41">
         <f>k_eff_CO2_l*B476</f>
-        <v>0.005128133134</v>
+        <v>0.005525951937</v>
       </c>
       <c r="M476" s="41">
         <f>EXP(-L476)</f>
-        <v>0.994884993293</v>
+        <v>0.99448928805</v>
       </c>
       <c r="N476" s="41">
         <f>IF(L476&gt;0,(1-M476)/L476,1)</f>
-        <v>0.997440310778</v>
+        <v>0.997242106366</v>
       </c>
       <c r="O476" s="41">
         <f>IF(L476&gt;0,(L476-1+M476)/L476^2,1/2)</f>
-        <v>0.49914640576</v>
+        <v>0.499080278945</v>
       </c>
       <c r="P476" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B476/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34590,11 +34594,11 @@
       </c>
       <c r="Q476" s="41">
         <f>(P476*N476+pool_b*M476)/(1-pool_ret*M476)</f>
-        <v>26.579010196783</v>
+        <v>26.470618514811</v>
       </c>
       <c r="R476" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q476+pool_b)*N476+P476*O476))</f>
-        <v>26.647271269118</v>
+        <v>26.543885178325</v>
       </c>
       <c r="S476" s="41">
         <f>IF(AND(R476&gt;=CO2_pH_hi_mt,R477&lt;CO2_pH_hi_mt),EXP(LN(A476)+(LN(A477)-LN(A476))*(R476-CO2_pH_hi_mt)/(R476-R477)),0)</f>
@@ -34644,19 +34648,19 @@
       </c>
       <c r="L477" s="41">
         <f>k_eff_CO2_l*B477</f>
-        <v>0.005749519963</v>
+        <v>0.00619554332</v>
       </c>
       <c r="M477" s="41">
         <f>EXP(-L477)</f>
-        <v>0.994266976895</v>
+        <v>0.993823609484</v>
       </c>
       <c r="N477" s="41">
         <f>IF(L477&gt;0,(1-M477)/L477,1)</f>
-        <v>0.997130741605</v>
+        <v>0.996908615903</v>
       </c>
       <c r="O477" s="41">
         <f>IF(L477&gt;0,(L477-1+M477)/L477^2,1/2)</f>
-        <v>0.499043122467</v>
+        <v>0.49896900683</v>
       </c>
       <c r="P477" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B477/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34664,11 +34668,11 @@
       </c>
       <c r="Q477" s="41">
         <f>(P477*N477+pool_b*M477)/(1-pool_ret*M477)</f>
-        <v>26.410087051369</v>
+        <v>26.290079886628</v>
       </c>
       <c r="R477" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q477+pool_b)*N477+P477*O477))</f>
-        <v>26.486148786007</v>
+        <v>26.371682358195</v>
       </c>
       <c r="S477" s="41">
         <f>IF(AND(R477&gt;=CO2_pH_hi_mt,R478&lt;CO2_pH_hi_mt),EXP(LN(A477)+(LN(A478)-LN(A477))*(R477-CO2_pH_hi_mt)/(R477-R478)),0)</f>
@@ -34718,19 +34722,19 @@
       </c>
       <c r="L478" s="41">
         <f>k_eff_CO2_l*B478</f>
-        <v>0.006445513309</v>
+        <v>0.006945528875</v>
       </c>
       <c r="M478" s="41">
         <f>EXP(-L478)</f>
-        <v>0.993575214455</v>
+        <v>0.993078535565</v>
       </c>
       <c r="N478" s="41">
         <f>IF(L478&gt;0,(1-M478)/L478,1)</f>
-        <v>0.99678415631</v>
+        <v>0.996535261683</v>
       </c>
       <c r="O478" s="41">
         <f>IF(L478&gt;0,(L478-1+M478)/L478^2,1/2)</f>
-        <v>0.498927476579</v>
+        <v>0.498844419081</v>
       </c>
       <c r="P478" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B478/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34738,11 +34742,11 @@
       </c>
       <c r="Q478" s="41">
         <f>(P478*N478+pool_b*M478)/(1-pool_ret*M478)</f>
-        <v>26.223291658673</v>
+        <v>26.090626530646</v>
       </c>
       <c r="R478" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q478+pool_b)*N478+P478*O478))</f>
-        <v>26.307977363987</v>
+        <v>26.181435816152</v>
       </c>
       <c r="S478" s="41">
         <f>IF(AND(R478&gt;=CO2_pH_hi_mt,R479&lt;CO2_pH_hi_mt),EXP(LN(A478)+(LN(A479)-LN(A478))*(R478-CO2_pH_hi_mt)/(R478-R479)),0)</f>
@@ -34792,19 +34796,19 @@
       </c>
       <c r="L479" s="41">
         <f>k_eff_CO2_l*B479</f>
-        <v>0.007225070765</v>
+        <v>0.00778556109</v>
       </c>
       <c r="M479" s="41">
         <f>EXP(-L479)</f>
-        <v>0.992800967312</v>
+        <v>0.99224466789</v>
       </c>
       <c r="N479" s="41">
         <f>IF(L479&gt;0,(1-M479)/L479,1)</f>
-        <v>0.9963961492</v>
+        <v>0.996117302316</v>
       </c>
       <c r="O479" s="41">
         <f>IF(L479&gt;0,(L479-1+M479)/L479^2,1/2)</f>
-        <v>0.498797993467</v>
+        <v>0.49870492818</v>
       </c>
       <c r="P479" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B479/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34812,11 +34816,11 @@
       </c>
       <c r="Q479" s="41">
         <f>(P479*N479+pool_b*M479)/(1-pool_ret*M479)</f>
-        <v>26.01703074287</v>
+        <v>25.870615756925</v>
       </c>
       <c r="R479" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q479+pool_b)*N479+P479*O479))</f>
-        <v>26.111236600528</v>
+        <v>25.971577901083</v>
       </c>
       <c r="S479" s="41">
         <f>IF(AND(R479&gt;=CO2_pH_hi_mt,R480&lt;CO2_pH_hi_mt),EXP(LN(A479)+(LN(A480)-LN(A479))*(R479-CO2_pH_hi_mt)/(R479-R480)),0)</f>
@@ -34866,19 +34870,19 @@
       </c>
       <c r="L480" s="41">
         <f>k_eff_CO2_l*B480</f>
-        <v>0.008098225419</v>
+        <v>0.008726451376</v>
       </c>
       <c r="M480" s="41">
         <f>EXP(-L480)</f>
-        <v>0.991934476872</v>
+        <v>0.991311513587</v>
       </c>
       <c r="N480" s="41">
         <f>IF(L480&gt;0,(1-M480)/L480,1)</f>
-        <v>0.995961795406</v>
+        <v>0.995649438497</v>
       </c>
       <c r="O480" s="41">
         <f>IF(L480&gt;0,(L480-1+M480)/L480^2,1/2)</f>
-        <v>0.498653023896</v>
+        <v>0.498548758864</v>
       </c>
       <c r="P480" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B480/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34886,11 +34890,11 @@
       </c>
       <c r="Q480" s="41">
         <f>(P480*N480+pool_b*M480)/(1-pool_ret*M480)</f>
-        <v>25.789638172436</v>
+        <v>25.628340506171</v>
       </c>
       <c r="R480" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q480+pool_b)*N480+P480*O480))</f>
-        <v>25.894336418705</v>
+        <v>25.740479355939</v>
       </c>
       <c r="S480" s="41">
         <f>IF(AND(R480&gt;=CO2_pH_hi_mt,R481&lt;CO2_pH_hi_mt),EXP(LN(A480)+(LN(A481)-LN(A480))*(R480-CO2_pH_hi_mt)/(R480-R481)),0)</f>
@@ -34940,19 +34944,19 @@
       </c>
       <c r="L481" s="41">
         <f>k_eff_CO2_l*B481</f>
-        <v>0.009076214974</v>
+        <v>0.00978030921</v>
       </c>
       <c r="M481" s="41">
         <f>EXP(-L481)</f>
-        <v>0.990964849535</v>
+        <v>0.990267362473</v>
       </c>
       <c r="N481" s="41">
         <f>IF(L481&gt;0,(1-M481)/L481,1)</f>
-        <v>0.995475591029</v>
+        <v>0.995125748899</v>
       </c>
       <c r="O481" s="41">
         <f>IF(L481&gt;0,(L481-1+M481)/L481^2,1/2)</f>
-        <v>0.498490723686</v>
+        <v>0.498373926284</v>
       </c>
       <c r="P481" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B481/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34960,11 +34964,11 @@
       </c>
       <c r="Q481" s="41">
         <f>(P481*N481+pool_b*M481)/(1-pool_ret*M481)</f>
-        <v>25.539388605515</v>
+        <v>25.362046093481</v>
       </c>
       <c r="R481" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q481+pool_b)*N481+P481*O481))</f>
-        <v>25.655630041786</v>
+        <v>25.486465242778</v>
       </c>
       <c r="S481" s="41">
         <f>IF(AND(R481&gt;=CO2_pH_hi_mt,R482&lt;CO2_pH_hi_mt),EXP(LN(A481)+(LN(A482)-LN(A481))*(R481-CO2_pH_hi_mt)/(R481-R482)),0)</f>
@@ -35014,19 +35018,19 @@
       </c>
       <c r="L482" s="41">
         <f>k_eff_CO2_l*B482</f>
-        <v>0.010171626381</v>
+        <v>0.010960697985</v>
       </c>
       <c r="M482" s="41">
         <f>EXP(-L482)</f>
-        <v>0.989879929659</v>
+        <v>0.989099151601</v>
       </c>
       <c r="N482" s="41">
         <f>IF(L482&gt;0,(1-M482)/L482,1)</f>
-        <v>0.994931386713</v>
+        <v>0.994539619078</v>
       </c>
       <c r="O482" s="41">
         <f>IF(L482&gt;0,(L482-1+M482)/L482^2,1/2)</f>
-        <v>0.498309031098</v>
+        <v>0.498178211754</v>
       </c>
       <c r="P482" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B482/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35034,11 +35038,11 @@
       </c>
       <c r="Q482" s="41">
         <f>(P482*N482+pool_b*M482)/(1-pool_ret*M482)</f>
-        <v>25.264515948267</v>
+        <v>25.069952201467</v>
       </c>
       <c r="R482" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q482+pool_b)*N482+P482*O482))</f>
-        <v>25.393431551026</v>
+        <v>25.207835866611</v>
       </c>
       <c r="S482" s="41">
         <f>IF(AND(R482&gt;=CO2_pH_hi_mt,R483&lt;CO2_pH_hi_mt),EXP(LN(A482)+(LN(A483)-LN(A482))*(R482-CO2_pH_hi_mt)/(R482-R483)),0)</f>
@@ -35088,19 +35092,19 @@
       </c>
       <c r="L483" s="41">
         <f>k_eff_CO2_l*B483</f>
-        <v>0.011398557841</v>
+        <v>0.01228280958</v>
       </c>
       <c r="M483" s="41">
         <f>EXP(-L483)</f>
-        <v>0.988666159591</v>
+        <v>0.987792316226</v>
       </c>
       <c r="N483" s="41">
         <f>IF(L483&gt;0,(1-M483)/L483,1)</f>
-        <v>0.994322314032</v>
+        <v>0.993883662756</v>
       </c>
       <c r="O483" s="41">
         <f>IF(L483&gt;0,(L483-1+M483)/L483^2,1/2)</f>
-        <v>0.498105641672</v>
+        <v>0.497959135801</v>
       </c>
       <c r="P483" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B483/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35108,11 +35112,11 @@
       </c>
       <c r="Q483" s="41">
         <f>(P483*N483+pool_b*M483)/(1-pool_ret*M483)</f>
-        <v>24.963237279945</v>
+        <v>24.750280735971</v>
       </c>
       <c r="R483" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q483+pool_b)*N483+P483*O483))</f>
-        <v>25.106038649249</v>
+        <v>24.902893282001</v>
       </c>
       <c r="S483" s="41">
         <f>IF(AND(R483&gt;=CO2_pH_hi_mt,R484&lt;CO2_pH_hi_mt),EXP(LN(A483)+(LN(A484)-LN(A483))*(R483-CO2_pH_hi_mt)/(R483-R484)),0)</f>
@@ -35162,19 +35166,19 @@
       </c>
       <c r="L484" s="41">
         <f>k_eff_CO2_l*B484</f>
-        <v>0.012772800246</v>
+        <v>0.013763659878</v>
       </c>
       <c r="M484" s="41">
         <f>EXP(-L484)</f>
-        <v>0.987308425771</v>
+        <v>0.986330626219</v>
       </c>
       <c r="N484" s="41">
         <f>IF(L484&gt;0,(1-M484)/L484,1)</f>
-        <v>0.99364070401</v>
+        <v>0.993149634775</v>
       </c>
       <c r="O484" s="41">
         <f>IF(L484&gt;0,(L484-1+M484)/L484^2,1/2)</f>
-        <v>0.497877980315</v>
+        <v>0.497713928273</v>
       </c>
       <c r="P484" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B484/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35182,11 +35186,11 @@
       </c>
       <c r="Q484" s="41">
         <f>(P484*N484+pool_b*M484)/(1-pool_ret*M484)</f>
-        <v>24.633782826816</v>
+        <v>24.401290044107</v>
       </c>
       <c r="R484" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q484+pool_b)*N484+P484*O484))</f>
-        <v>24.791761184514</v>
+        <v>24.569973858127</v>
       </c>
       <c r="S484" s="41">
         <f>IF(AND(R484&gt;=CO2_pH_hi_mt,R485&lt;CO2_pH_hi_mt),EXP(LN(A484)+(LN(A485)-LN(A484))*(R484-CO2_pH_hi_mt)/(R484-R485)),0)</f>
@@ -35236,19 +35240,19 @@
       </c>
       <c r="L485" s="41">
         <f>k_eff_CO2_l*B485</f>
-        <v>0.014312040415</v>
+        <v>0.015422307767</v>
       </c>
       <c r="M485" s="41">
         <f>EXP(-L485)</f>
-        <v>0.985789889978</v>
+        <v>0.984696007012</v>
       </c>
       <c r="N485" s="41">
         <f>IF(L485&gt;0,(1-M485)/L485,1)</f>
-        <v>0.992877997075</v>
+        <v>0.99232833501</v>
       </c>
       <c r="O485" s="41">
         <f>IF(L485&gt;0,(L485-1+M485)/L485^2,1/2)</f>
-        <v>0.49762317033</v>
+        <v>0.497439495198</v>
       </c>
       <c r="P485" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B485/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35256,11 +35260,11 @@
       </c>
       <c r="Q485" s="41">
         <f>(P485*N485+pool_b*M485)/(1-pool_ret*M485)</f>
-        <v>24.274432429382</v>
+        <v>24.021315804917</v>
       </c>
       <c r="R485" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q485+pool_b)*N485+P485*O485))</f>
-        <v>24.448955856879</v>
+        <v>24.207487197477</v>
       </c>
       <c r="S485" s="41">
         <f>IF(AND(R485&gt;=CO2_pH_hi_mt,R486&lt;CO2_pH_hi_mt),EXP(LN(A485)+(LN(A486)-LN(A485))*(R485-CO2_pH_hi_mt)/(R485-R486)),0)</f>
@@ -35310,19 +35314,19 @@
       </c>
       <c r="L486" s="41">
         <f>k_eff_CO2_l*B486</f>
-        <v>0.016036088727</v>
+        <v>0.017280100429</v>
       </c>
       <c r="M486" s="41">
         <f>EXP(-L486)</f>
-        <v>0.984091804794</v>
+        <v>0.98286834423</v>
       </c>
       <c r="N486" s="41">
         <f>IF(L486&gt;0,(1-M486)/L486,1)</f>
-        <v>0.992024643719</v>
+        <v>0.99140950251</v>
       </c>
       <c r="O486" s="41">
         <f>IF(L486&gt;0,(L486-1+M486)/L486^2,1/2)</f>
-        <v>0.497337999112</v>
+        <v>0.497132382131</v>
       </c>
       <c r="P486" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B486/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35330,11 +35334,11 @@
       </c>
       <c r="Q486" s="41">
         <f>(P486*N486+pool_b*M486)/(1-pool_ret*M486)</f>
-        <v>23.88355872872</v>
+        <v>23.608818623814</v>
       </c>
       <c r="R486" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q486+pool_b)*N486+P486*O486))</f>
-        <v>24.076067322903</v>
+        <v>23.813961437228</v>
       </c>
       <c r="S486" s="41">
         <f>IF(AND(R486&gt;=CO2_pH_hi_mt,R487&lt;CO2_pH_hi_mt),EXP(LN(A486)+(LN(A487)-LN(A486))*(R486-CO2_pH_hi_mt)/(R486-R487)),0)</f>
@@ -35384,19 +35388,19 @@
       </c>
       <c r="L487" s="41">
         <f>k_eff_CO2_l*B487</f>
-        <v>0.017967134084</v>
+        <v>0.019360948088</v>
       </c>
       <c r="M487" s="41">
         <f>EXP(-L487)</f>
-        <v>0.982193312511</v>
+        <v>0.980825271336</v>
       </c>
       <c r="N487" s="41">
         <f>IF(L487&gt;0,(1-M487)/L487,1)</f>
-        <v>0.991069995137</v>
+        <v>0.990381699117</v>
       </c>
       <c r="O487" s="41">
         <f>IF(L487&gt;0,(L487-1+M487)/L487^2,1/2)</f>
-        <v>0.497018880209</v>
+        <v>0.496788733631</v>
       </c>
       <c r="P487" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B487/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35404,11 +35408,11 @@
       </c>
       <c r="Q487" s="41">
         <f>(P487*N487+pool_b*M487)/(1-pool_ret*M487)</f>
-        <v>23.459676985679</v>
+        <v>23.162437983688</v>
       </c>
       <c r="R487" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q487+pool_b)*N487+P487*O487))</f>
-        <v>23.671675615005</v>
+        <v>23.388094601807</v>
       </c>
       <c r="S487" s="41">
         <f>IF(AND(R487&gt;=CO2_pH_hi_mt,R488&lt;CO2_pH_hi_mt),EXP(LN(A487)+(LN(A488)-LN(A487))*(R487-CO2_pH_hi_mt)/(R487-R488)),0)</f>
@@ -35458,19 +35462,19 @@
       </c>
       <c r="L488" s="41">
         <f>k_eff_CO2_l*B488</f>
-        <v>0.020130029487</v>
+        <v>0.021691631738</v>
       </c>
       <c r="M488" s="41">
         <f>EXP(-L488)</f>
-        <v>0.980071226862</v>
+        <v>0.978541939808</v>
       </c>
       <c r="N488" s="41">
         <f>IF(L488&gt;0,(1-M488)/L488,1)</f>
-        <v>0.990002183091</v>
+        <v>0.989232181847</v>
       </c>
       <c r="O488" s="41">
         <f>IF(L488&gt;0,(L488-1+M488)/L488^2,1/2)</f>
-        <v>0.496661811424</v>
+        <v>0.496404248583</v>
       </c>
       <c r="P488" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B488/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35478,11 +35482,11 @@
       </c>
       <c r="Q488" s="41">
         <f>(P488*N488+pool_b*M488)/(1-pool_ret*M488)</f>
-        <v>23.001501033564</v>
+        <v>22.681051725819</v>
       </c>
       <c r="R488" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q488+pool_b)*N488+P488*O488))</f>
-        <v>23.234549399074</v>
+        <v>22.928811217877</v>
       </c>
       <c r="S488" s="41">
         <f>IF(AND(R488&gt;=CO2_pH_hi_mt,R489&lt;CO2_pH_hi_mt),EXP(LN(A488)+(LN(A489)-LN(A488))*(R488-CO2_pH_hi_mt)/(R488-R489)),0)</f>
@@ -35532,19 +35536,19 @@
       </c>
       <c r="L489" s="41">
         <f>k_eff_CO2_l*B489</f>
-        <v>0.022552611904</v>
+        <v>0.024302147816</v>
       </c>
       <c r="M489" s="41">
         <f>EXP(-L489)</f>
-        <v>0.977699797192</v>
+        <v>0.975990771723</v>
       </c>
       <c r="N489" s="41">
         <f>IF(L489&gt;0,(1-M489)/L489,1)</f>
-        <v>0.9888079883</v>
+        <v>0.987946763355</v>
       </c>
       <c r="O489" s="41">
         <f>IF(L489&gt;0,(L489-1+M489)/L489^2,1/2)</f>
-        <v>0.496262328631</v>
+        <v>0.495974131007</v>
       </c>
       <c r="P489" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B489/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35552,11 +35556,11 @@
       </c>
       <c r="Q489" s="41">
         <f>(P489*N489+pool_b*M489)/(1-pool_ret*M489)</f>
-        <v>22.508004352097</v>
+        <v>22.163839661732</v>
       </c>
       <c r="R489" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q489+pool_b)*N489+P489*O489))</f>
-        <v>22.763704104872</v>
+        <v>22.435322857749</v>
       </c>
       <c r="S489" s="41">
         <f>IF(AND(R489&gt;=CO2_pH_hi_mt,R490&lt;CO2_pH_hi_mt),EXP(LN(A489)+(LN(A490)-LN(A489))*(R489-CO2_pH_hi_mt)/(R489-R490)),0)</f>
@@ -35606,19 +35610,19 @@
       </c>
       <c r="L490" s="41">
         <f>k_eff_CO2_l*B490</f>
-        <v>0.025266060532</v>
+        <v>0.027226094272</v>
       </c>
       <c r="M490" s="41">
         <f>EXP(-L490)</f>
-        <v>0.975050455071</v>
+        <v>0.973141194999</v>
       </c>
       <c r="N490" s="41">
         <f>IF(L490&gt;0,(1-M490)/L490,1)</f>
-        <v>0.987472696702</v>
+        <v>0.986509659889</v>
       </c>
       <c r="O490" s="41">
         <f>IF(L490&gt;0,(L490-1+M490)/L490^2,1/2)</f>
-        <v>0.495815454974</v>
+        <v>0.495493036043</v>
       </c>
       <c r="P490" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B490/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35626,11 +35630,11 @@
       </c>
       <c r="Q490" s="41">
         <f>(P490*N490+pool_b*M490)/(1-pool_ret*M490)</f>
-        <v>21.978484651667</v>
+        <v>21.610349276976</v>
       </c>
       <c r="R490" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q490+pool_b)*N490+P490*O490))</f>
-        <v>22.258463393091</v>
+        <v>21.907190667109</v>
       </c>
       <c r="S490" s="41">
         <f>IF(AND(R490&gt;=CO2_pH_hi_mt,R491&lt;CO2_pH_hi_mt),EXP(LN(A490)+(LN(A491)-LN(A490))*(R490-CO2_pH_hi_mt)/(R490-R491)),0)</f>
@@ -35680,19 +35684,19 @@
       </c>
       <c r="L491" s="41">
         <f>k_eff_CO2_l*B491</f>
-        <v>0.028305298086</v>
+        <v>0.030501102977</v>
       </c>
       <c r="M491" s="41">
         <f>EXP(-L491)</f>
-        <v>0.972091543806</v>
+        <v>0.969959362224</v>
       </c>
       <c r="N491" s="41">
         <f>IF(L491&gt;0,(1-M491)/L491,1)</f>
-        <v>0.985979943018</v>
+        <v>0.984903326247</v>
       </c>
       <c r="O491" s="41">
         <f>IF(L491&gt;0,(L491-1+M491)/L491^2,1/2)</f>
-        <v>0.495315645137</v>
+        <v>0.49495501079</v>
       </c>
       <c r="P491" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B491/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35700,11 +35704,11 @@
       </c>
       <c r="Q491" s="41">
         <f>(P491*N491+pool_b*M491)/(1-pool_ret*M491)</f>
-        <v>21.412629702263</v>
+        <v>21.020560821936</v>
       </c>
       <c r="R491" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q491+pool_b)*N491+P491*O491))</f>
-        <v>21.718521798935</v>
+        <v>21.344387298227</v>
       </c>
       <c r="S491" s="41">
         <f>IF(AND(R491&gt;=CO2_pH_hi_mt,R492&lt;CO2_pH_hi_mt),EXP(LN(A491)+(LN(A492)-LN(A491))*(R491-CO2_pH_hi_mt)/(R491-R492)),0)</f>
@@ -35754,19 +35758,19 @@
       </c>
       <c r="L492" s="41">
         <f>k_eff_CO2_l*B492</f>
-        <v>0.031709440259</v>
+        <v>0.034169324051</v>
       </c>
       <c r="M492" s="41">
         <f>EXP(-L492)</f>
-        <v>0.968788031988</v>
+        <v>0.96640785469</v>
       </c>
       <c r="N492" s="41">
         <f>IF(L492&gt;0,(1-M492)/L492,1)</f>
-        <v>0.984311541206</v>
+        <v>0.983108277465</v>
       </c>
       <c r="O492" s="41">
         <f>IF(L492&gt;0,(L492-1+M492)/L492^2,1/2)</f>
-        <v>0.494756724351</v>
+        <v>0.494353429704</v>
       </c>
       <c r="P492" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B492/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35774,11 +35778,11 @@
       </c>
       <c r="Q492" s="41">
         <f>(P492*N492+pool_b*M492)/(1-pool_ret*M492)</f>
-        <v>20.810581479984</v>
+        <v>20.394948454887</v>
       </c>
       <c r="R492" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q492+pool_b)*N492+P492*O492))</f>
-        <v>21.14400576162</v>
+        <v>20.747355069429</v>
       </c>
       <c r="S492" s="41">
         <f>IF(AND(R492&gt;=CO2_pH_hi_mt,R493&lt;CO2_pH_hi_mt),EXP(LN(A492)+(LN(A493)-LN(A492))*(R492-CO2_pH_hi_mt)/(R492-R493)),0)</f>
@@ -35828,19 +35832,19 @@
       </c>
       <c r="L493" s="41">
         <f>k_eff_CO2_l*B493</f>
-        <v>0.035522299151</v>
+        <v>0.038277968353</v>
       </c>
       <c r="M493" s="41">
         <f>EXP(-L493)</f>
-        <v>0.965101213052</v>
+        <v>0.96244537435</v>
       </c>
       <c r="N493" s="41">
         <f>IF(L493&gt;0,(1-M493)/L493,1)</f>
-        <v>0.982447301603</v>
+        <v>0.981102897202</v>
       </c>
       <c r="O493" s="41">
         <f>IF(L493&gt;0,(L493-1+M493)/L493^2,1/2)</f>
-        <v>0.494131821887</v>
+        <v>0.493680924318</v>
       </c>
       <c r="P493" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B493/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35848,11 +35852,11 @@
       </c>
       <c r="Q493" s="41">
         <f>(P493*N493+pool_b*M493)/(1-pool_ret*M493)</f>
-        <v>20.172995103818</v>
+        <v>19.734533587947</v>
       </c>
       <c r="R493" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q493+pool_b)*N493+P493*O493))</f>
-        <v>20.535529677052</v>
+        <v>20.117056681115</v>
       </c>
       <c r="S493" s="41">
         <f>IF(AND(R493&gt;=CO2_pH_hi_mt,R494&lt;CO2_pH_hi_mt),EXP(LN(A493)+(LN(A494)-LN(A493))*(R493-CO2_pH_hi_mt)/(R493-R494)),0)</f>
@@ -35902,19 +35906,19 @@
       </c>
       <c r="L494" s="41">
         <f>k_eff_CO2_l*B494</f>
-        <v>0.039792947142</v>
+        <v>0.04287991509</v>
       </c>
       <c r="M494" s="41">
         <f>EXP(-L494)</f>
-        <v>0.960988393948</v>
+        <v>0.958026427677</v>
       </c>
       <c r="N494" s="41">
         <f>IF(L494&gt;0,(1-M494)/L494,1)</f>
-        <v>0.980364834823</v>
+        <v>0.978863233167</v>
       </c>
       <c r="O494" s="41">
         <f>IF(L494&gt;0,(L494-1+M494)/L494^2,1/2)</f>
-        <v>0.493433298789</v>
+        <v>0.492929307092</v>
       </c>
       <c r="P494" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B494/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35922,11 +35926,11 @@
       </c>
       <c r="Q494" s="41">
         <f>(P494*N494+pool_b*M494)/(1-pool_ret*M494)</f>
-        <v>19.501088580583</v>
+        <v>19.040926278224</v>
       </c>
       <c r="R494" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q494+pool_b)*N494+P494*O494))</f>
-        <v>19.89424317738</v>
+        <v>19.455014524589</v>
       </c>
       <c r="S494" s="41">
         <f>IF(AND(R494&gt;=CO2_pH_hi_mt,R495&lt;CO2_pH_hi_mt),EXP(LN(A494)+(LN(A495)-LN(A494))*(R494-CO2_pH_hi_mt)/(R494-R495)),0)</f>
@@ -35976,19 +35980,19 @@
       </c>
       <c r="L495" s="41">
         <f>k_eff_CO2_l*B495</f>
-        <v>0.044576348463</v>
+        <v>0.048034392383</v>
       </c>
       <c r="M495" s="41">
         <f>EXP(-L495)</f>
-        <v>0.956402577439</v>
+        <v>0.953101007099</v>
       </c>
       <c r="N495" s="41">
         <f>IF(L495&gt;0,(1-M495)/L495,1)</f>
-        <v>0.978039342924</v>
+        <v>0.976362780382</v>
       </c>
       <c r="O495" s="41">
         <f>IF(L495&gt;0,(L495-1+M495)/L495^2,1/2)</f>
-        <v>0.492652669695</v>
+        <v>0.492089489316</v>
       </c>
       <c r="P495" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B495/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -35996,11 +36000,11 @@
       </c>
       <c r="Q495" s="41">
         <f>(P495*N495+pool_b*M495)/(1-pool_ret*M495)</f>
-        <v>18.796679159107</v>
+        <v>18.316350495978</v>
       </c>
       <c r="R495" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q495+pool_b)*N495+P495*O495))</f>
-        <v>19.221865634381</v>
+        <v>18.763334609817</v>
       </c>
       <c r="S495" s="41">
         <f>IF(AND(R495&gt;=CO2_pH_hi_mt,R496&lt;CO2_pH_hi_mt),EXP(LN(A495)+(LN(A496)-LN(A495))*(R495-CO2_pH_hi_mt)/(R495-R496)),0)</f>
@@ -36050,19 +36054,19 @@
       </c>
       <c r="L496" s="41">
         <f>k_eff_CO2_l*B496</f>
-        <v>0.049934066601</v>
+        <v>0.053807739554</v>
       </c>
       <c r="M496" s="41">
         <f>EXP(-L496)</f>
-        <v>0.951292144358</v>
+        <v>0.947614277732</v>
       </c>
       <c r="N496" s="41">
         <f>IF(L496&gt;0,(1-M496)/L496,1)</f>
-        <v>0.975443398825</v>
+        <v>0.973572253759</v>
       </c>
       <c r="O496" s="41">
         <f>IF(L496&gt;0,(L496-1+M496)/L496^2,1/2)</f>
-        <v>0.491780518714</v>
+        <v>0.491151393095</v>
       </c>
       <c r="P496" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B496/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36070,11 +36074,11 @@
       </c>
       <c r="Q496" s="41">
         <f>(P496*N496+pool_b*M496)/(1-pool_ret*M496)</f>
-        <v>18.062202204727</v>
+        <v>17.563649466671</v>
       </c>
       <c r="R496" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q496+pool_b)*N496+P496*O496))</f>
-        <v>18.520703988247</v>
+        <v>18.044711485962</v>
       </c>
       <c r="S496" s="41">
         <f>IF(AND(R496&gt;=CO2_pH_hi_mt,R497&lt;CO2_pH_hi_mt),EXP(LN(A496)+(LN(A497)-LN(A496))*(R496-CO2_pH_hi_mt)/(R496-R497)),0)</f>
@@ -36124,19 +36128,19 @@
       </c>
       <c r="L497" s="41">
         <f>k_eff_CO2_l*B497</f>
-        <v>0.055935056632</v>
+        <v>0.060274260922</v>
       </c>
       <c r="M497" s="41">
         <f>EXP(-L497)</f>
-        <v>0.945600544381</v>
+        <v>0.941506279791</v>
       </c>
       <c r="N497" s="41">
         <f>IF(L497&gt;0,(1-M497)/L497,1)</f>
-        <v>0.972546715693</v>
+        <v>0.970459352204</v>
       </c>
       <c r="O497" s="41">
         <f>IF(L497&gt;0,(L497-1+M497)/L497^2,1/2)</f>
-        <v>0.490806409442</v>
+        <v>0.490103857663</v>
       </c>
       <c r="P497" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B497/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36144,11 +36148,11 @@
       </c>
       <c r="Q497" s="41">
         <f>(P497*N497+pool_b*M497)/(1-pool_ret*M497)</f>
-        <v>17.300709010795</v>
+        <v>16.786268070515</v>
       </c>
       <c r="R497" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q497+pool_b)*N497+P497*O497))</f>
-        <v>17.79365048506</v>
+        <v>17.302411278107</v>
       </c>
       <c r="S497" s="41">
         <f>IF(AND(R497&gt;=CO2_pH_hi_mt,R498&lt;CO2_pH_hi_mt),EXP(LN(A497)+(LN(A498)-LN(A497))*(R497-CO2_pH_hi_mt)/(R497-R498)),0)</f>
@@ -36198,19 +36202,19 @@
       </c>
       <c r="L498" s="41">
         <f>k_eff_CO2_l*B498</f>
-        <v>0.062656552691</v>
+        <v>0.067517182118</v>
       </c>
       <c r="M498" s="41">
         <f>EXP(-L498)</f>
-        <v>0.939266006682</v>
+        <v>0.934711660152</v>
       </c>
       <c r="N498" s="41">
         <f>IF(L498&gt;0,(1-M498)/L498,1)</f>
-        <v>0.969315908867</v>
+        <v>0.966988517588</v>
       </c>
       <c r="O498" s="41">
         <f>IF(L498&gt;0,(L498-1+M498)/L498^2,1/2)</f>
-        <v>0.489718789419</v>
+        <v>0.488934540463</v>
       </c>
       <c r="P498" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B498/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36218,11 +36222,11 @@
       </c>
       <c r="Q498" s="41">
         <f>(P498*N498+pool_b*M498)/(1-pool_ret*M498)</f>
-        <v>16.515840896598</v>
+        <v>15.988210489308</v>
       </c>
       <c r="R498" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q498+pool_b)*N498+P498*O498))</f>
-        <v>17.044157794881</v>
+        <v>16.540231112838</v>
       </c>
       <c r="S498" s="41">
         <f>IF(AND(R498&gt;=CO2_pH_hi_mt,R499&lt;CO2_pH_hi_mt),EXP(LN(A498)+(LN(A499)-LN(A498))*(R498-CO2_pH_hi_mt)/(R498-R499)),0)</f>
@@ -36272,19 +36276,19 @@
       </c>
       <c r="L499" s="41">
         <f>k_eff_CO2_l*B499</f>
-        <v>0.070185061994</v>
+        <v>0.07562972122</v>
       </c>
       <c r="M499" s="41">
         <f>EXP(-L499)</f>
-        <v>0.932221285212</v>
+        <v>0.927159450478</v>
       </c>
       <c r="N499" s="41">
         <f>IF(L499&gt;0,(1-M499)/L499,1)</f>
-        <v>0.96571425404</v>
+        <v>0.963120693126</v>
       </c>
       <c r="O499" s="41">
         <f>IF(L499&gt;0,(L499-1+M499)/L499^2,1/2)</f>
-        <v>0.488504889593</v>
+        <v>0.487629813772</v>
       </c>
       <c r="P499" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B499/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36292,11 +36296,11 @@
       </c>
       <c r="Q499" s="41">
         <f>(P499*N499+pool_b*M499)/(1-pool_ret*M499)</f>
-        <v>15.711778279102</v>
+        <v>15.173972853626</v>
       </c>
       <c r="R499" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q499+pool_b)*N499+P499*O499))</f>
-        <v>16.276190257301</v>
+        <v>15.762434694971</v>
       </c>
       <c r="S499" s="41">
         <f>IF(AND(R499&gt;=CO2_pH_hi_mt,R500&lt;CO2_pH_hi_mt),EXP(LN(A499)+(LN(A500)-LN(A499))*(R499-CO2_pH_hi_mt)/(R499-R500)),0)</f>
@@ -36346,19 +36350,19 @@
       </c>
       <c r="L500" s="41">
         <f>k_eff_CO2_l*B500</f>
-        <v>0.078617478205</v>
+        <v>0.08471628849</v>
       </c>
       <c r="M500" s="41">
         <f>EXP(-L500)</f>
-        <v>0.924393457469</v>
+        <v>0.918772913878</v>
       </c>
       <c r="N500" s="41">
         <f>IF(L500&gt;0,(1-M500)/L500,1)</f>
-        <v>0.961701446776</v>
+        <v>0.958813087414</v>
       </c>
       <c r="O500" s="41">
         <f>IF(L500&gt;0,(L500-1+M500)/L500^2,1/2)</f>
-        <v>0.487150619664</v>
+        <v>0.48617465803</v>
       </c>
       <c r="P500" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B500/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36366,11 +36370,11 @@
       </c>
       <c r="Q500" s="41">
         <f>(P500*N500+pool_b*M500)/(1-pool_ret*M500)</f>
-        <v>14.8931650652</v>
+        <v>14.348452438396</v>
       </c>
       <c r="R500" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q500+pool_b)*N500+P500*O500))</f>
-        <v>15.494151582372</v>
+        <v>14.973665508069</v>
       </c>
       <c r="S500" s="41">
         <f>IF(AND(R500&gt;=CO2_pH_hi_mt,R501&lt;CO2_pH_hi_mt),EXP(LN(A500)+(LN(A501)-LN(A500))*(R500-CO2_pH_hi_mt)/(R500-R501)),0)</f>
@@ -36420,19 +36424,19 @@
       </c>
       <c r="L501" s="41">
         <f>k_eff_CO2_l*B501</f>
-        <v>0.088062328477</v>
+        <v>0.094893830161</v>
       </c>
       <c r="M501" s="41">
         <f>EXP(-L501)</f>
-        <v>0.915703800521</v>
+        <v>0.909469487572</v>
       </c>
       <c r="N501" s="41">
         <f>IF(L501&gt;0,(1-M501)/L501,1)</f>
-        <v>0.957233370233</v>
+        <v>0.954018952283</v>
       </c>
       <c r="O501" s="41">
         <f>IF(L501&gt;0,(L501-1+M501)/L501^2,1/2)</f>
-        <v>0.485640460637</v>
+        <v>0.484552553513</v>
       </c>
       <c r="P501" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B501/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36440,11 +36444,11 @@
       </c>
       <c r="Q501" s="41">
         <f>(P501*N501+pool_b*M501)/(1-pool_ret*M501)</f>
-        <v>14.065010546225</v>
+        <v>13.516836802482</v>
       </c>
       <c r="R501" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q501+pool_b)*N501+P501*O501))</f>
-        <v>14.702791083418</v>
+        <v>14.178840871942</v>
       </c>
       <c r="S501" s="41">
         <f>IF(AND(R501&gt;=CO2_pH_hi_mt,R502&lt;CO2_pH_hi_mt),EXP(LN(A501)+(LN(A502)-LN(A501))*(R501-CO2_pH_hi_mt)/(R501-R502)),0)</f>
@@ -36494,19 +36498,19 @@
       </c>
       <c r="L502" s="41">
         <f>k_eff_CO2_l*B502</f>
-        <v>0.098641170229</v>
+        <v>0.106293333557</v>
       </c>
       <c r="M502" s="41">
         <f>EXP(-L502)</f>
-        <v>0.90606777379</v>
+        <v>0.899160855337</v>
       </c>
       <c r="N502" s="41">
         <f>IF(L502&gt;0,(1-M502)/L502,1)</f>
-        <v>0.952261880021</v>
+        <v>0.948687385082</v>
       </c>
       <c r="O502" s="41">
         <f>IF(L502&gt;0,(L502-1+M502)/L502^2,1/2)</f>
-        <v>0.483957356422</v>
+        <v>0.482745372649</v>
       </c>
       <c r="P502" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B502/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36514,11 +36518,11 @@
       </c>
       <c r="Q502" s="41">
         <f>(P502*N502+pool_b*M502)/(1-pool_ret*M502)</f>
-        <v>13.232572794503</v>
+        <v>12.68447795744</v>
       </c>
       <c r="R502" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q502+pool_b)*N502+P502*O502))</f>
-        <v>13.907092250637</v>
+        <v>13.383031700278</v>
       </c>
       <c r="S502" s="41">
         <f>IF(AND(R502&gt;=CO2_pH_hi_mt,R503&lt;CO2_pH_hi_mt),EXP(LN(A502)+(LN(A503)-LN(A502))*(R502-CO2_pH_hi_mt)/(R502-R503)),0)</f>
@@ -36568,19 +36572,19 @@
       </c>
       <c r="L503" s="41">
         <f>k_eff_CO2_l*B503</f>
-        <v>0.110490155611</v>
+        <v>0.119061512934</v>
       </c>
       <c r="M503" s="41">
         <f>EXP(-L503)</f>
-        <v>0.895395144764</v>
+        <v>0.887753190779</v>
       </c>
       <c r="N503" s="41">
         <f>IF(L503&gt;0,(1-M503)/L503,1)</f>
-        <v>0.946734617734</v>
+        <v>0.942763168845</v>
       </c>
       <c r="O503" s="41">
         <f>IF(L503&gt;0,(L503-1+M503)/L503^2,1/2)</f>
-        <v>0.482082607008</v>
+        <v>0.480733275977</v>
       </c>
       <c r="P503" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B503/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36588,11 +36592,11 @@
       </c>
       <c r="Q503" s="41">
         <f>(P503*N503+pool_b*M503)/(1-pool_ret*M503)</f>
-        <v>12.401229148279</v>
+        <v>11.856757971806</v>
       </c>
       <c r="R503" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q503+pool_b)*N503+P503*O503))</f>
-        <v>13.11214898619</v>
+        <v>12.591334060517</v>
       </c>
       <c r="S503" s="41">
         <f>IF(AND(R503&gt;=CO2_pH_hi_mt,R504&lt;CO2_pH_hi_mt),EXP(LN(A503)+(LN(A504)-LN(A503))*(R503-CO2_pH_hi_mt)/(R503-R504)),0)</f>
@@ -36642,19 +36646,19 @@
       </c>
       <c r="L504" s="41">
         <f>k_eff_CO2_l*B504</f>
-        <v>0.123761783815</v>
+        <v>0.133362697726</v>
       </c>
       <c r="M504" s="41">
         <f>EXP(-L504)</f>
-        <v>0.883590301324</v>
+        <v>0.875147620487</v>
       </c>
       <c r="N504" s="41">
         <f>IF(L504&gt;0,(1-M504)/L504,1)</f>
-        <v>0.94059486771</v>
+        <v>0.936186667199</v>
       </c>
       <c r="O504" s="41">
         <f>IF(L504&gt;0,(L504-1+M504)/L504^2,1/2)</f>
-        <v>0.47999576653</v>
+        <v>0.478494615731</v>
       </c>
       <c r="P504" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B504/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36662,11 +36666,11 @@
       </c>
       <c r="Q504" s="41">
         <f>(P504*N504+pool_b*M504)/(1-pool_ret*M504)</f>
-        <v>11.576340524337</v>
+        <v>11.03895319595</v>
       </c>
       <c r="R504" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q504+pool_b)*N504+P504*O504))</f>
-        <v>12.323035920163</v>
+        <v>11.80873938012</v>
       </c>
       <c r="S504" s="41">
         <f>IF(AND(R504&gt;=CO2_pH_hi_mt,R505&lt;CO2_pH_hi_mt),EXP(LN(A504)+(LN(A505)-LN(A504))*(R504-CO2_pH_hi_mt)/(R504-R505)),0)</f>
@@ -36716,19 +36720,19 @@
       </c>
       <c r="L505" s="41">
         <f>k_eff_CO2_l*B505</f>
-        <v>0.138626863781</v>
+        <v>0.149380947504</v>
       </c>
       <c r="M505" s="41">
         <f>EXP(-L505)</f>
-        <v>0.870552802643</v>
+        <v>0.861240964803</v>
       </c>
       <c r="N505" s="41">
         <f>IF(L505&gt;0,(1-M505)/L505,1)</f>
-        <v>0.93378147515</v>
+        <v>0.928893794794</v>
       </c>
       <c r="O505" s="41">
         <f>IF(L505&gt;0,(L505-1+M505)/L505^2,1/2)</f>
-        <v>0.477674550547</v>
+        <v>0.476005852111</v>
       </c>
       <c r="P505" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B505/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36736,11 +36740,11 @@
       </c>
       <c r="Q505" s="41">
         <f>(P505*N505+pool_b*M505)/(1-pool_ret*M505)</f>
-        <v>10.763116863008</v>
+        <v>10.236104422493</v>
       </c>
       <c r="R505" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q505+pool_b)*N505+P505*O505))</f>
-        <v>11.544679765623</v>
+        <v>11.040010267306</v>
       </c>
       <c r="S505" s="41">
         <f>IF(AND(R505&gt;=CO2_pH_hi_mt,R506&lt;CO2_pH_hi_mt),EXP(LN(A505)+(LN(A506)-LN(A505))*(R505-CO2_pH_hi_mt)/(R505-R506)),0)</f>
@@ -36790,19 +36794,19 @@
       </c>
       <c r="L506" s="41">
         <f>k_eff_CO2_l*B506</f>
-        <v>0.155276712539</v>
+        <v>0.167322420862</v>
       </c>
       <c r="M506" s="41">
         <f>EXP(-L506)</f>
-        <v>0.85617822945</v>
+        <v>0.845926822908</v>
       </c>
       <c r="N506" s="41">
         <f>IF(L506&gt;0,(1-M506)/L506,1)</f>
-        <v>0.92622884783</v>
+        <v>0.920816088474</v>
       </c>
       <c r="O506" s="41">
         <f>IF(L506&gt;0,(L506-1+M506)/L506^2,1/2)</f>
-        <v>0.475094758021</v>
+        <v>0.473241488604</v>
       </c>
       <c r="P506" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B506/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36810,11 +36814,11 @@
       </c>
       <c r="Q506" s="41">
         <f>(P506*N506+pool_b*M506)/(1-pool_ret*M506)</f>
-        <v>9.966490910413</v>
+        <v>9.452899760523</v>
       </c>
       <c r="R506" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q506+pool_b)*N506+P506*O506))</f>
-        <v>10.781738575932</v>
+        <v>10.289568403111</v>
       </c>
       <c r="S506" s="41">
         <f>IF(AND(R506&gt;=CO2_pH_hi_mt,R507&lt;CO2_pH_hi_mt),EXP(LN(A506)+(LN(A507)-LN(A506))*(R506-CO2_pH_hi_mt)/(R506-R507)),0)</f>
@@ -36864,19 +36868,19 @@
       </c>
       <c r="L507" s="41">
         <f>k_eff_CO2_l*B507</f>
-        <v>0.17392561751</v>
+        <v>0.18741802873</v>
       </c>
       <c r="M507" s="41">
         <f>EXP(-L507)</f>
-        <v>0.840359403359</v>
+        <v>0.829097077536</v>
       </c>
       <c r="N507" s="41">
         <f>IF(L507&gt;0,(1-M507)/L507,1)</f>
-        <v>0.917867068272</v>
+        <v>0.911880909338</v>
       </c>
       <c r="O507" s="41">
         <f>IF(L507&gt;0,(L507-1+M507)/L507^2,1/2)</f>
-        <v>0.472230214868</v>
+        <v>0.470174034267</v>
       </c>
       <c r="P507" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B507/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36884,11 +36888,11 @@
       </c>
       <c r="Q507" s="41">
         <f>(P507*N507+pool_b*M507)/(1-pool_ret*M507)</f>
-        <v>9.191006791321</v>
+        <v>8.693575871972</v>
       </c>
       <c r="R507" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q507+pool_b)*N507+P507*O507))</f>
-        <v>10.038495051729</v>
+        <v>9.561399885387</v>
       </c>
       <c r="S507" s="41">
         <f>IF(AND(R507&gt;=CO2_pH_hi_mt,R508&lt;CO2_pH_hi_mt),EXP(LN(A507)+(LN(A508)-LN(A507))*(R507-CO2_pH_hi_mt)/(R507-R508)),0)</f>
@@ -36938,19 +36942,19 @@
       </c>
       <c r="L508" s="41">
         <f>k_eff_CO2_l*B508</f>
-        <v>0.194813594432</v>
+        <v>0.209926406247</v>
       </c>
       <c r="M508" s="41">
         <f>EXP(-L508)</f>
-        <v>0.822988053314</v>
+        <v>0.810643902102</v>
       </c>
       <c r="N508" s="41">
         <f>IF(L508&gt;0,(1-M508)/L508,1)</f>
-        <v>0.908622148274</v>
+        <v>0.902011811106</v>
       </c>
       <c r="O508" s="41">
         <f>IF(L508&gt;0,(L508-1+M508)/L508^2,1/2)</f>
-        <v>0.469052747538</v>
+        <v>0.466774002592</v>
       </c>
       <c r="P508" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B508/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -36958,11 +36962,11 @@
       </c>
       <c r="Q508" s="41">
         <f>(P508*N508+pool_b*M508)/(1-pool_ret*M508)</f>
-        <v>8.440728525394</v>
+        <v>7.961841646484</v>
       </c>
       <c r="R508" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q508+pool_b)*N508+P508*O508))</f>
-        <v>9.318768806194</v>
+        <v>8.858981908195</v>
       </c>
       <c r="S508" s="41">
         <f>IF(AND(R508&gt;=CO2_pH_hi_mt,R509&lt;CO2_pH_hi_mt),EXP(LN(A508)+(LN(A509)-LN(A508))*(R508-CO2_pH_hi_mt)/(R508-R509)),0)</f>
@@ -37012,19 +37016,19 @@
       </c>
       <c r="L509" s="41">
         <f>k_eff_CO2_l*B509</f>
-        <v>0.21820947642</v>
+        <v>0.235137241462</v>
       </c>
       <c r="M509" s="41">
         <f>EXP(-L509)</f>
-        <v>0.803957013989</v>
+        <v>0.790462357975</v>
       </c>
       <c r="N509" s="41">
         <f>IF(L509&gt;0,(1-M509)/L509,1)</f>
-        <v>0.898416463057</v>
+        <v>0.891129115587</v>
       </c>
       <c r="O509" s="41">
         <f>IF(L509&gt;0,(L509-1+M509)/L509^2,1/2)</f>
-        <v>0.465532196904</v>
+        <v>0.463009958509</v>
       </c>
       <c r="P509" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B509/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37032,11 +37036,11 @@
       </c>
       <c r="Q509" s="41">
         <f>(P509*N509+pool_b*M509)/(1-pool_ret*M509)</f>
-        <v>7.71917196138</v>
+        <v>7.260826577456</v>
       </c>
       <c r="R509" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q509+pool_b)*N509+P509*O509))</f>
-        <v>8.625850898996</v>
+        <v>8.185232933183</v>
       </c>
       <c r="S509" s="41">
         <f>IF(AND(R509&gt;=CO2_pH_hi_mt,R510&lt;CO2_pH_hi_mt),EXP(LN(A509)+(LN(A510)-LN(A509))*(R509-CO2_pH_hi_mt)/(R509-R510)),0)</f>
@@ -37086,19 +37090,19 @@
       </c>
       <c r="L510" s="41">
         <f>k_eff_CO2_l*B510</f>
-        <v>0.244414373908</v>
+        <v>0.263375003677</v>
       </c>
       <c r="M510" s="41">
         <f>EXP(-L510)</f>
-        <v>0.783163044685</v>
+        <v>0.768453670319</v>
       </c>
       <c r="N510" s="41">
         <f>IF(L510&gt;0,(1-M510)/L510,1)</f>
-        <v>0.887169407623</v>
+        <v>0.879150741141</v>
       </c>
       <c r="O510" s="41">
         <f>IF(L510&gt;0,(L510-1+M510)/L510^2,1/2)</f>
-        <v>0.461636484681</v>
+        <v>0.458848627137</v>
       </c>
       <c r="P510" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B510/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37106,11 +37110,11 @@
       </c>
       <c r="Q510" s="41">
         <f>(P510*N510+pool_b*M510)/(1-pool_ret*M510)</f>
-        <v>7.029261757103</v>
+        <v>6.593054260885</v>
       </c>
       <c r="R510" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q510+pool_b)*N510+P510*O510))</f>
-        <v>7.962462191252</v>
+        <v>7.542486757387</v>
       </c>
       <c r="S510" s="41">
         <f>IF(AND(R510&gt;=CO2_pH_hi_mt,R511&lt;CO2_pH_hi_mt),EXP(LN(A510)+(LN(A511)-LN(A510))*(R510-CO2_pH_hi_mt)/(R510-R511)),0)</f>
@@ -37160,19 +37164,19 @@
       </c>
       <c r="L511" s="41">
         <f>k_eff_CO2_l*B511</f>
-        <v>0.273765550015</v>
+        <v>0.295003119452</v>
       </c>
       <c r="M511" s="41">
         <f>EXP(-L511)</f>
-        <v>0.760510356003</v>
+        <v>0.744529264939</v>
       </c>
       <c r="N511" s="41">
         <f>IF(L511&gt;0,(1-M511)/L511,1)</f>
-        <v>0.874798322814</v>
+        <v>0.865993334361</v>
       </c>
       <c r="O511" s="41">
         <f>IF(L511&gt;0,(L511-1+M511)/L511^2,1/2)</f>
-        <v>0.457331746742</v>
+        <v>0.454255080042</v>
       </c>
       <c r="P511" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B511/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37180,11 +37184,11 @@
       </c>
       <c r="Q511" s="41">
         <f>(P511*N511+pool_b*M511)/(1-pool_ret*M511)</f>
-        <v>6.373313229214</v>
+        <v>5.960439764593</v>
       </c>
       <c r="R511" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q511+pool_b)*N511+P511*O511))</f>
-        <v>7.330735357357</v>
+        <v>6.932489289983</v>
       </c>
       <c r="S511" s="41">
         <f>IF(AND(R511&gt;=CO2_pH_hi_mt,R512&lt;CO2_pH_hi_mt),EXP(LN(A511)+(LN(A512)-LN(A511))*(R511-CO2_pH_hi_mt)/(R511-R512)),0)</f>
@@ -37234,19 +37238,19 @@
       </c>
       <c r="L512" s="41">
         <f>k_eff_CO2_l*B512</f>
-        <v>0.306640761193</v>
+        <v>0.330428649982</v>
       </c>
       <c r="M512" s="41">
         <f>EXP(-L512)</f>
-        <v>0.735914922626</v>
+        <v>0.718615632825</v>
       </c>
       <c r="N512" s="41">
         <f>IF(L512&gt;0,(1-M512)/L512,1)</f>
-        <v>0.861219742433</v>
+        <v>0.851573757876</v>
       </c>
       <c r="O512" s="41">
         <f>IF(L512&gt;0,(L512-1+M512)/L512^2,1/2)</f>
-        <v>0.45258254978</v>
+        <v>0.449193016804</v>
       </c>
       <c r="P512" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B512/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37254,11 +37258,11 @@
       </c>
       <c r="Q512" s="41">
         <f>(P512*N512+pool_b*M512)/(1-pool_ret*M512)</f>
-        <v>5.753037315975</v>
+        <v>5.364308255521</v>
       </c>
       <c r="R512" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q512+pool_b)*N512+P512*O512))</f>
-        <v>6.732218887171</v>
+        <v>6.356415559637</v>
       </c>
       <c r="S512" s="41">
         <f>IF(AND(R512&gt;=CO2_pH_hi_mt,R513&lt;CO2_pH_hi_mt),EXP(LN(A512)+(LN(A513)-LN(A512))*(R512-CO2_pH_hi_mt)/(R512-R513)),0)</f>
@@ -37308,19 +37312,19 @@
       </c>
       <c r="L513" s="41">
         <f>k_eff_CO2_l*B513</f>
-        <v>0.343463119045</v>
+        <v>0.370107530072</v>
       </c>
       <c r="M513" s="41">
         <f>EXP(-L513)</f>
-        <v>0.709309640679</v>
+        <v>0.690660059918</v>
       </c>
       <c r="N513" s="41">
         <f>IF(L513&gt;0,(1-M513)/L513,1)</f>
-        <v>0.846351014715</v>
+        <v>0.835810987205</v>
       </c>
       <c r="O513" s="41">
         <f>IF(L513&gt;0,(L513-1+M513)/L513^2,1/2)</f>
-        <v>0.447352209786</v>
+        <v>0.443625161483</v>
       </c>
       <c r="P513" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B513/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37328,11 +37332,11 @@
       </c>
       <c r="Q513" s="41">
         <f>(P513*N513+pool_b*M513)/(1-pool_ret*M513)</f>
-        <v>5.169565666682</v>
+        <v>4.805431313684</v>
       </c>
       <c r="R513" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q513+pool_b)*N513+P513*O513))</f>
-        <v>6.167900245878</v>
+        <v>5.814903567289</v>
       </c>
       <c r="S513" s="41">
         <f>IF(AND(R513&gt;=CO2_pH_hi_mt,R514&lt;CO2_pH_hi_mt),EXP(LN(A513)+(LN(A514)-LN(A513))*(R513-CO2_pH_hi_mt)/(R513-R514)),0)</f>
@@ -37382,19 +37386,19 @@
       </c>
       <c r="L514" s="41">
         <f>k_eff_CO2_l*B514</f>
-        <v>0.38470653587</v>
+        <v>0.414550436127</v>
       </c>
       <c r="M514" s="41">
         <f>EXP(-L514)</f>
-        <v>0.680650353362</v>
+        <v>0.660637212579</v>
       </c>
       <c r="N514" s="41">
         <f>IF(L514&gt;0,(1-M514)/L514,1)</f>
-        <v>0.830112350225</v>
+        <v>0.818628465553</v>
       </c>
       <c r="O514" s="41">
         <f>IF(L514&gt;0,(L514-1+M514)/L514^2,1/2)</f>
-        <v>0.441603232424</v>
+        <v>0.437513794802</v>
       </c>
       <c r="P514" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B514/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37402,11 +37406,11 @@
       </c>
       <c r="Q514" s="41">
         <f>(P514*N514+pool_b*M514)/(1-pool_ret*M514)</f>
-        <v>4.623492057054</v>
+        <v>4.284076826418</v>
       </c>
       <c r="R514" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q514+pool_b)*N514+P514*O514))</f>
-        <v>5.638244590982</v>
+        <v>5.308101099597</v>
       </c>
       <c r="S514" s="41">
         <f>IF(AND(R514&gt;=CO2_pH_hi_mt,R515&lt;CO2_pH_hi_mt),EXP(LN(A514)+(LN(A515)-LN(A514))*(R514-CO2_pH_hi_mt)/(R514-R515)),0)</f>
@@ -37456,19 +37460,19 @@
       </c>
       <c r="L515" s="41">
         <f>k_eff_CO2_l*B515</f>
-        <v>0.430901824022</v>
+        <v>0.464329358668</v>
       </c>
       <c r="M515" s="41">
         <f>EXP(-L515)</f>
-        <v>0.649922714441</v>
+        <v>0.62855649984</v>
       </c>
       <c r="N515" s="41">
         <f>IF(L515&gt;0,(1-M515)/L515,1)</f>
-        <v>0.81242934247</v>
+        <v>0.79995695561</v>
       </c>
       <c r="O515" s="41">
         <f>IF(L515&gt;0,(L515-1+M515)/L515^2,1/2)</f>
-        <v>0.43529789635</v>
+        <v>0.430821443133</v>
       </c>
       <c r="P515" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B515/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37476,11 +37480,11 @@
       </c>
       <c r="Q515" s="41">
         <f>(P515*N515+pool_b*M515)/(1-pool_ret*M515)</f>
-        <v>4.114925934965</v>
+        <v>3.800068215518</v>
       </c>
       <c r="R515" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q515+pool_b)*N515+P515*O515))</f>
-        <v>5.143245080885</v>
+        <v>4.835721497962</v>
       </c>
       <c r="S515" s="41">
         <f>IF(AND(R515&gt;=CO2_pH_hi_mt,R516&lt;CO2_pH_hi_mt),EXP(LN(A515)+(LN(A516)-LN(A515))*(R515-CO2_pH_hi_mt)/(R515-R516)),0)</f>
@@ -37530,19 +37534,19 @@
       </c>
       <c r="L516" s="41">
         <f>k_eff_CO2_l*B516</f>
-        <v>0.482643527587</v>
+        <v>0.52008496399</v>
       </c>
       <c r="M516" s="41">
         <f>EXP(-L516)</f>
-        <v>0.617149781038</v>
+        <v>0.594470037278</v>
       </c>
       <c r="N516" s="41">
         <f>IF(L516&gt;0,(1-M516)/L516,1)</f>
-        <v>0.793235995261</v>
+        <v>0.779737909765</v>
       </c>
       <c r="O516" s="41">
         <f>IF(L516&gt;0,(L516-1+M516)/L516^2,1/2)</f>
-        <v>0.428399000341</v>
+        <v>0.423511744206</v>
       </c>
       <c r="P516" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B516/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37550,11 +37554,11 @@
       </c>
       <c r="Q516" s="41">
         <f>(P516*N516+pool_b*M516)/(1-pool_ret*M516)</f>
-        <v>3.643553879668</v>
+        <v>3.352848933715</v>
       </c>
       <c r="R516" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q516+pool_b)*N516+P516*O516))</f>
-        <v>4.68248080506</v>
+        <v>4.397104572644</v>
       </c>
       <c r="S516" s="41">
         <f>IF(AND(R516&gt;=CO2_pH_hi_mt,R517&lt;CO2_pH_hi_mt),EXP(LN(A516)+(LN(A517)-LN(A516))*(R516-CO2_pH_hi_mt)/(R516-R517)),0)</f>
@@ -37604,19 +37608,19 @@
       </c>
       <c r="L517" s="41">
         <f>k_eff_CO2_l*B517</f>
-        <v>0.540597574309</v>
+        <v>0.582534839684</v>
       </c>
       <c r="M517" s="41">
         <f>EXP(-L517)</f>
-        <v>0.582400121018</v>
+        <v>0.558480911237</v>
       </c>
       <c r="N517" s="41">
         <f>IF(L517&gt;0,(1-M517)/L517,1)</f>
-        <v>0.772478270027</v>
+        <v>0.75792735247</v>
       </c>
       <c r="O517" s="41">
         <f>IF(L517&gt;0,(L517-1+M517)/L517^2,1/2)</f>
-        <v>0.420870793333</v>
+        <v>0.415550506235</v>
       </c>
       <c r="P517" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B517/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37624,11 +37628,11 @@
       </c>
       <c r="Q517" s="41">
         <f>(P517*N517+pool_b*M517)/(1-pool_ret*M517)</f>
-        <v>3.208705032252</v>
+        <v>2.941548585849</v>
       </c>
       <c r="R517" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q517+pool_b)*N517+P517*O517))</f>
-        <v>4.25517864898</v>
+        <v>3.991279276827</v>
       </c>
       <c r="S517" s="41">
         <f>IF(AND(R517&gt;=CO2_pH_hi_mt,R518&lt;CO2_pH_hi_mt),EXP(LN(A517)+(LN(A518)-LN(A517))*(R517-CO2_pH_hi_mt)/(R517-R518)),0)</f>
@@ -37678,19 +37682,19 @@
       </c>
       <c r="L518" s="41">
         <f>k_eff_CO2_l*B518</f>
-        <v>0.605509846228</v>
+        <v>0.652482730154</v>
       </c>
       <c r="M518" s="41">
         <f>EXP(-L518)</f>
-        <v>0.545796083615</v>
+        <v>0.52075128557</v>
       </c>
       <c r="N518" s="41">
         <f>IF(L518&gt;0,(1-M518)/L518,1)</f>
-        <v>0.750118134683</v>
+        <v>0.73450022856</v>
       </c>
       <c r="O518" s="41">
         <f>IF(L518&gt;0,(L518-1+M518)/L518^2,1/2)</f>
-        <v>0.412680102353</v>
+        <v>0.406906971127</v>
       </c>
       <c r="P518" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B518/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37698,11 +37702,11 @@
       </c>
       <c r="Q518" s="41">
         <f>(P518*N518+pool_b*M518)/(1-pool_ret*M518)</f>
-        <v>2.809417032271</v>
+        <v>2.565047589469</v>
       </c>
       <c r="R518" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q518+pool_b)*N518+P518*O518))</f>
-        <v>3.860275890547</v>
+        <v>3.617025323192</v>
       </c>
       <c r="S518" s="41">
         <f>IF(AND(R518&gt;=CO2_pH_hi_mt,R519&lt;CO2_pH_hi_mt),EXP(LN(A518)+(LN(A519)-LN(A518))*(R518-CO2_pH_hi_mt)/(R518-R519)),0)</f>
@@ -37752,19 +37756,19 @@
       </c>
       <c r="L519" s="41">
         <f>k_eff_CO2_l*B519</f>
-        <v>0.678215779361</v>
+        <v>0.730828880997</v>
       </c>
       <c r="M519" s="41">
         <f>EXP(-L519)</f>
-        <v>0.507521715732</v>
+        <v>0.481509710387</v>
       </c>
       <c r="N519" s="41">
         <f>IF(L519&gt;0,(1-M519)/L519,1)</f>
-        <v>0.726138051125</v>
+        <v>0.709455117464</v>
       </c>
       <c r="O519" s="41">
         <f>IF(L519&gt;0,(L519-1+M519)/L519^2,1/2)</f>
-        <v>0.403797666184</v>
+        <v>0.3975552829</v>
       </c>
       <c r="P519" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B519/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37772,11 +37776,11 @@
       </c>
       <c r="Q519" s="41">
         <f>(P519*N519+pool_b*M519)/(1-pool_ret*M519)</f>
-        <v>2.444499582179</v>
+        <v>2.222037902772</v>
       </c>
       <c r="R519" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q519+pool_b)*N519+P519*O519))</f>
-        <v>3.49648092187</v>
+        <v>3.272931554843</v>
       </c>
       <c r="S519" s="41">
         <f>IF(AND(R519&gt;=CO2_pH_hi_mt,R520&lt;CO2_pH_hi_mt),EXP(LN(A519)+(LN(A520)-LN(A519))*(R519-CO2_pH_hi_mt)/(R519-R520)),0)</f>
@@ -37826,19 +37830,19 @@
       </c>
       <c r="L520" s="41">
         <f>k_eff_CO2_l*B520</f>
-        <v>0.759651115954</v>
+        <v>0.81858162537</v>
       </c>
       <c r="M520" s="41">
         <f>EXP(-L520)</f>
-        <v>0.46782961683</v>
+        <v>0.441056794828</v>
       </c>
       <c r="N520" s="41">
         <f>IF(L520&gt;0,(1-M520)/L520,1)</f>
-        <v>0.700545779494</v>
+        <v>0.682819144541</v>
       </c>
       <c r="O520" s="41">
         <f>IF(L520&gt;0,(L520-1+M520)/L520^2,1/2)</f>
-        <v>0.394199671688</v>
+        <v>0.387476148534</v>
       </c>
       <c r="P520" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B520/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37846,11 +37850,11 @@
       </c>
       <c r="Q520" s="41">
         <f>(P520*N520+pool_b*M520)/(1-pool_ret*M520)</f>
-        <v>2.112593375686</v>
+        <v>1.911077944383</v>
       </c>
       <c r="R520" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q520+pool_b)*N520+P520*O520))</f>
-        <v>3.162330124552</v>
+        <v>2.957449507497</v>
       </c>
       <c r="S520" s="41">
         <f>IF(AND(R520&gt;=CO2_pH_hi_mt,R521&lt;CO2_pH_hi_mt),EXP(LN(A520)+(LN(A521)-LN(A520))*(R520-CO2_pH_hi_mt)/(R520-R521)),0)</f>
@@ -37900,19 +37904,19 @@
       </c>
       <c r="L521" s="41">
         <f>k_eff_CO2_l*B521</f>
-        <v>0.850863947703</v>
+        <v>0.916870361474</v>
       </c>
       <c r="M521" s="41">
         <f>EXP(-L521)</f>
-        <v>0.427045827266</v>
+        <v>0.399768215341</v>
       </c>
       <c r="N521" s="41">
         <f>IF(L521&gt;0,(1-M521)/L521,1)</f>
-        <v>0.673379303801</v>
+        <v>0.654652838482</v>
       </c>
       <c r="O521" s="41">
         <f>IF(L521&gt;0,(L521-1+M521)/L521^2,1/2)</f>
-        <v>0.383869474175</v>
+        <v>0.376658659751</v>
       </c>
       <c r="P521" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B521/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37920,11 +37924,11 @@
       </c>
       <c r="Q521" s="41">
         <f>(P521*N521+pool_b*M521)/(1-pool_ret*M521)</f>
-        <v>1.812222704435</v>
+        <v>1.630640359152</v>
       </c>
       <c r="R521" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q521+pool_b)*N521+P521*O521))</f>
-        <v>2.856239538437</v>
+        <v>2.668941173049</v>
       </c>
       <c r="S521" s="41">
         <f>IF(AND(R521&gt;=CO2_pH_hi_mt,R522&lt;CO2_pH_hi_mt),EXP(LN(A521)+(LN(A522)-LN(A521))*(R521-CO2_pH_hi_mt)/(R521-R522)),0)</f>
@@ -37974,19 +37978,19 @@
       </c>
       <c r="L522" s="41">
         <f>k_eff_CO2_l*B522</f>
-        <v>0.953028204938</v>
+        <v>1.026960088173</v>
       </c>
       <c r="M522" s="41">
         <f>EXP(-L522)</f>
-        <v>0.385571663802</v>
+        <v>0.358093881486</v>
       </c>
       <c r="N522" s="41">
         <f>IF(L522&gt;0,(1-M522)/L522,1)</f>
-        <v>0.644711597217</v>
+        <v>0.625054591612</v>
       </c>
       <c r="O522" s="41">
         <f>IF(L522&gt;0,(L522-1+M522)/L522^2,1/2)</f>
-        <v>0.372799462746</v>
+        <v>0.365102220336</v>
       </c>
       <c r="P522" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B522/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -37994,11 +37998,11 @@
       </c>
       <c r="Q522" s="41">
         <f>(P522*N522+pool_b*M522)/(1-pool_ret*M522)</f>
-        <v>1.541840556721</v>
+        <v>1.37915171855</v>
       </c>
       <c r="R522" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q522+pool_b)*N522+P522*O522))</f>
-        <v>2.576550511661</v>
+        <v>2.405720466362</v>
       </c>
       <c r="S522" s="41">
         <f>IF(AND(R522&gt;=CO2_pH_hi_mt,R523&lt;CO2_pH_hi_mt),EXP(LN(A522)+(LN(A523)-LN(A522))*(R522-CO2_pH_hi_mt)/(R522-R523)),0)</f>
@@ -38048,19 +38052,19 @@
       </c>
       <c r="L523" s="41">
         <f>k_eff_CO2_l*B523</f>
-        <v>1.067458765376</v>
+        <v>1.150267685817</v>
       </c>
       <c r="M523" s="41">
         <f>EXP(-L523)</f>
-        <v>0.343881291031</v>
+        <v>0.31655202155</v>
       </c>
       <c r="N523" s="41">
         <f>IF(L523&gt;0,(1-M523)/L523,1)</f>
-        <v>0.614654851551</v>
+        <v>0.594164286172</v>
       </c>
       <c r="O523" s="41">
         <f>IF(L523&gt;0,(L523-1+M523)/L523^2,1/2)</f>
-        <v>0.360993005958</v>
+        <v>0.352818495062</v>
       </c>
       <c r="P523" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B523/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38068,11 +38072,11 @@
       </c>
       <c r="Q523" s="41">
         <f>(P523*N523+pool_b*M523)/(1-pool_ret*M523)</f>
-        <v>1.299865421143</v>
+        <v>1.155023576163</v>
       </c>
       <c r="R523" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q523+pool_b)*N523+P523*O523))</f>
-        <v>2.321568979937</v>
+        <v>2.166088293399</v>
       </c>
       <c r="S523" s="41">
         <f>IF(AND(R523&gt;=CO2_pH_hi_mt,R524&lt;CO2_pH_hi_mt),EXP(LN(A523)+(LN(A524)-LN(A523))*(R523-CO2_pH_hi_mt)/(R523-R524)),0)</f>
@@ -38122,19 +38126,19 @@
       </c>
       <c r="L524" s="41">
         <f>k_eff_CO2_l*B524</f>
-        <v>1.19562837691</v>
+        <v>1.288380151827</v>
       </c>
       <c r="M524" s="41">
         <f>EXP(-L524)</f>
-        <v>0.302513801757</v>
+        <v>0.275717041303</v>
       </c>
       <c r="N524" s="41">
         <f>IF(L524&gt;0,(1-M524)/L524,1)</f>
-        <v>0.583363703734</v>
+        <v>0.562165567104</v>
       </c>
       <c r="O524" s="41">
         <f>IF(L524&gt;0,(L524-1+M524)/L524^2,1/2)</f>
-        <v>0.348466383295</v>
+        <v>0.339833264487</v>
       </c>
       <c r="P524" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B524/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38142,11 +38146,11 @@
       </c>
       <c r="Q524" s="41">
         <f>(P524*N524+pool_b*M524)/(1-pool_ret*M524)</f>
-        <v>1.084709307322</v>
+        <v>0.956674542781</v>
       </c>
       <c r="R524" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q524+pool_b)*N524+P524*O524))</f>
-        <v>2.089598385765</v>
+        <v>1.948361417733</v>
       </c>
       <c r="S524" s="41">
         <f>IF(AND(R524&gt;=CO2_pH_hi_mt,R525&lt;CO2_pH_hi_mt),EXP(LN(A524)+(LN(A525)-LN(A524))*(R524-CO2_pH_hi_mt)/(R524-R525)),0)</f>
@@ -38196,19 +38200,19 @@
       </c>
       <c r="L525" s="41">
         <f>k_eff_CO2_l*B525</f>
-        <v>1.339186612206</v>
+        <v>1.443075025719</v>
       </c>
       <c r="M525" s="41">
         <f>EXP(-L525)</f>
-        <v>0.262058737293</v>
+        <v>0.236200318752</v>
       </c>
       <c r="N525" s="41">
         <f>IF(L525&gt;0,(1-M525)/L525,1)</f>
-        <v>0.55103691747</v>
+        <v>0.529286189308</v>
       </c>
       <c r="O525" s="41">
         <f>IF(L525&gt;0,(L525-1+M525)/L525^2,1/2)</f>
-        <v>0.335250575564</v>
+        <v>0.326188037561</v>
       </c>
       <c r="P525" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B525/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38216,11 +38220,11 @@
       </c>
       <c r="Q525" s="41">
         <f>(P525*N525+pool_b*M525)/(1-pool_ret*M525)</f>
-        <v>0.894796717084</v>
+        <v>0.782543238562</v>
       </c>
       <c r="R525" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q525+pool_b)*N525+P525*O525))</f>
-        <v>1.878966515222</v>
+        <v>1.750895530624</v>
       </c>
       <c r="S525" s="41">
         <f>IF(AND(R525&gt;=CO2_pH_hi_mt,R526&lt;CO2_pH_hi_mt),EXP(LN(A525)+(LN(A526)-LN(A525))*(R525-CO2_pH_hi_mt)/(R525-R526)),0)</f>
@@ -38270,19 +38274,19 @@
       </c>
       <c r="L526" s="41">
         <f>k_eff_CO2_l*B526</f>
-        <v>1.499981099098</v>
+        <v>1.616343266449</v>
       </c>
       <c r="M526" s="41">
         <f>EXP(-L526)</f>
-        <v>0.22313437755</v>
+        <v>0.198623686632</v>
       </c>
       <c r="N526" s="41">
         <f>IF(L526&gt;0,(1-M526)/L526,1)</f>
-        <v>0.517916941032</v>
+        <v>0.495795868367</v>
       </c>
       <c r="O526" s="41">
         <f>IF(L526&gt;0,(L526-1+M526)/L526^2,1/2)</f>
-        <v>0.321392755721</v>
+        <v>0.311941245464</v>
       </c>
       <c r="P526" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B526/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38290,11 +38294,11 @@
       </c>
       <c r="Q526" s="41">
         <f>(P526*N526+pool_b*M526)/(1-pool_ret*M526)</f>
-        <v>0.728574487869</v>
+        <v>0.631092183044</v>
       </c>
       <c r="R526" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q526+pool_b)*N526+P526*O526))</f>
-        <v>1.688046709667</v>
+        <v>1.572103058991</v>
       </c>
       <c r="S526" s="41">
         <f>IF(AND(R526&gt;=CO2_pH_hi_mt,R527&lt;CO2_pH_hi_mt),EXP(LN(A526)+(LN(A527)-LN(A526))*(R526-CO2_pH_hi_mt)/(R526-R527)),0)</f>
@@ -38344,19 +38348,19 @@
       </c>
       <c r="L527" s="41">
         <f>k_eff_CO2_l*B527</f>
-        <v>1.680081299976</v>
+        <v>1.810414876518</v>
       </c>
       <c r="M527" s="41">
         <f>EXP(-L527)</f>
-        <v>0.186358824456</v>
+        <v>0.163586254627</v>
       </c>
       <c r="N527" s="41">
         <f>IF(L527&gt;0,(1-M527)/L527,1)</f>
-        <v>0.484286787524</v>
+        <v>0.462001144722</v>
       </c>
       <c r="O527" s="41">
         <f>IF(L527&gt;0,(L527-1+M527)/L527^2,1/2)</f>
-        <v>0.306957295747</v>
+        <v>0.297168821498</v>
       </c>
       <c r="P527" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B527/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38364,11 +38368,11 @@
       </c>
       <c r="Q527" s="41">
         <f>(P527*N527+pool_b*M527)/(1-pool_ret*M527)</f>
-        <v>0.584512655602</v>
+        <v>0.500802984417</v>
       </c>
       <c r="R527" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q527+pool_b)*N527+P527*O527))</f>
-        <v>1.515274015154</v>
+        <v>1.410466310027</v>
       </c>
       <c r="S527" s="41">
         <f>IF(AND(R527&gt;=CO2_pH_hi_mt,R528&lt;CO2_pH_hi_mt),EXP(LN(A527)+(LN(A528)-LN(A527))*(R527-CO2_pH_hi_mt)/(R527-R528)),0)</f>
@@ -38418,19 +38422,19 @@
       </c>
       <c r="L528" s="41">
         <f>k_eff_CO2_l*B528</f>
-        <v>1.881805146255</v>
+        <v>2.027787602622</v>
       </c>
       <c r="M528" s="41">
         <f>EXP(-L528)</f>
-        <v>0.152314906761</v>
+        <v>0.131626409172</v>
       </c>
       <c r="N528" s="41">
         <f>IF(L528&gt;0,(1-M528)/L528,1)</f>
-        <v>0.450463797979</v>
+        <v>0.42823695623</v>
       </c>
       <c r="O528" s="41">
         <f>IF(L528&gt;0,(L528-1+M528)/L528^2,1/2)</f>
-        <v>0.292026091604</v>
+        <v>0.281963970502</v>
       </c>
       <c r="P528" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B528/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38438,11 +38442,11 @@
       </c>
       <c r="Q528" s="41">
         <f>(P528*N528+pool_b*M528)/(1-pool_ret*M528)</f>
-        <v>0.461096842072</v>
+        <v>0.390163695327</v>
       </c>
       <c r="R528" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q528+pool_b)*N528+P528*O528))</f>
-        <v>1.359156878109</v>
+        <v>1.264546566102</v>
       </c>
       <c r="S528" s="41">
         <f>IF(AND(R528&gt;=CO2_pH_hi_mt,R529&lt;CO2_pH_hi_mt),EXP(LN(A528)+(LN(A529)-LN(A528))*(R528-CO2_pH_hi_mt)/(R528-R529)),0)</f>
@@ -38492,19 +38496,19 @@
       </c>
       <c r="L529" s="41">
         <f>k_eff_CO2_l*B529</f>
-        <v>2.107748870689</v>
+        <v>2.271259082233</v>
       </c>
       <c r="M529" s="41">
         <f>EXP(-L529)</f>
-        <v>0.121511196196</v>
+        <v>0.103182183408</v>
       </c>
       <c r="N529" s="41">
         <f>IF(L529&gt;0,(1-M529)/L529,1)</f>
-        <v>0.41679007211</v>
+        <v>0.394854917084</v>
       </c>
       <c r="O529" s="41">
         <f>IF(L529&gt;0,(L529-1+M529)/L529^2,1/2)</f>
-        <v>0.276698014645</v>
+        <v>0.266435955127</v>
       </c>
       <c r="P529" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B529/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38512,11 +38516,11 @@
       </c>
       <c r="Q529" s="41">
         <f>(P529*N529+pool_b*M529)/(1-pool_ret*M529)</f>
-        <v>0.356813273892</v>
+        <v>0.297650023818</v>
       </c>
       <c r="R529" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q529+pool_b)*N529+P529*O529))</f>
-        <v>1.218284997392</v>
+        <v>1.132989724189</v>
       </c>
       <c r="S529" s="41">
         <f>IF(AND(R529&gt;=CO2_pH_hi_mt,R530&lt;CO2_pH_hi_mt),EXP(LN(A529)+(LN(A530)-LN(A529))*(R529-CO2_pH_hi_mt)/(R529-R530)),0)</f>
@@ -38566,19 +38570,19 @@
       </c>
       <c r="L530" s="41">
         <f>k_eff_CO2_l*B530</f>
-        <v>2.360820421489</v>
+        <v>2.543962849842</v>
       </c>
       <c r="M530" s="41">
         <f>EXP(-L530)</f>
-        <v>0.094342790584</v>
+        <v>0.07855448254</v>
       </c>
       <c r="N530" s="41">
         <f>IF(L530&gt;0,(1-M530)/L530,1)</f>
-        <v>0.383619694735</v>
+        <v>0.362208716027</v>
       </c>
       <c r="O530" s="41">
         <f>IF(L530&gt;0,(L530-1+M530)/L530^2,1/2)</f>
-        <v>0.261087332037</v>
+        <v>0.250707782157</v>
       </c>
       <c r="P530" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B530/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38586,15 +38590,15 @@
       </c>
       <c r="Q530" s="41">
         <f>(P530*N530+pool_b*M530)/(1-pool_ret*M530)</f>
-        <v>0.270128488436</v>
+        <v>0.221703291573</v>
       </c>
       <c r="R530" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q530+pool_b)*N530+P530*O530))</f>
-        <v>1.091333915162</v>
+        <v>1.014529035169</v>
       </c>
       <c r="S530" s="41">
         <f>IF(AND(R530&gt;=CO2_pH_hi_mt,R531&lt;CO2_pH_hi_mt),EXP(LN(A530)+(LN(A531)-LN(A530))*(R530-CO2_pH_hi_mt)/(R530-R531)),0)</f>
-        <v>0.0</v>
+        <v>568.953730792824</v>
       </c>
     </row>
     <row r="531">
@@ -38640,19 +38644,19 @@
       </c>
       <c r="L531" s="41">
         <f>k_eff_CO2_l*B531</f>
-        <v>2.644276888292</v>
+        <v>2.849408666275</v>
       </c>
       <c r="M531" s="41">
         <f>EXP(-L531)</f>
-        <v>0.071056717111</v>
+        <v>0.057878536288</v>
       </c>
       <c r="N531" s="41">
         <f>IF(L531&gt;0,(1-M531)/L531,1)</f>
-        <v>0.351303332492</v>
+        <v>0.330637537136</v>
       </c>
       <c r="O531" s="41">
         <f>IF(L531&gt;0,(L531-1+M531)/L531^2,1/2)</f>
-        <v>0.245321006427</v>
+        <v>0.234912763054</v>
       </c>
       <c r="P531" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B531/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38660,15 +38664,15 @@
       </c>
       <c r="Q531" s="41">
         <f>(P531*N531+pool_b*M531)/(1-pool_ret*M531)</f>
-        <v>0.199467112259</v>
+        <v>0.160709559305</v>
       </c>
       <c r="R531" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q531+pool_b)*N531+P531*O531))</f>
-        <v>0.977066886729</v>
+        <v>0.907985454209</v>
       </c>
       <c r="S531" s="41">
         <f>IF(AND(R531&gt;=CO2_pH_hi_mt,R532&lt;CO2_pH_hi_mt),EXP(LN(A531)+(LN(A532)-LN(A531))*(R531-CO2_pH_hi_mt)/(R531-R532)),0)</f>
-        <v>612.612318746651</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="532">
@@ -38714,19 +38718,19 @@
       </c>
       <c r="L532" s="41">
         <f>k_eff_CO2_l*B532</f>
-        <v>2.96176642166</v>
+        <v>3.191527690132</v>
       </c>
       <c r="M532" s="41">
         <f>EXP(-L532)</f>
-        <v>0.051727463911</v>
+        <v>0.041109021098</v>
       </c>
       <c r="N532" s="41">
         <f>IF(L532&gt;0,(1-M532)/L532,1)</f>
-        <v>0.320171276558</v>
+        <v>0.300448898459</v>
       </c>
       <c r="O532" s="41">
         <f>IF(L532&gt;0,(L532-1+M532)/L532^2,1/2)</f>
-        <v>0.229534887853</v>
+        <v>0.219190046104</v>
       </c>
       <c r="P532" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B532/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38734,11 +38738,11 @@
       </c>
       <c r="Q532" s="41">
         <f>(P532*N532+pool_b*M532)/(1-pool_ret*M532)</f>
-        <v>0.143192683639</v>
+        <v>0.112985896799</v>
       </c>
       <c r="R532" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q532+pool_b)*N532+P532*O532))</f>
-        <v>0.874334526665</v>
+        <v>0.812266076665</v>
       </c>
       <c r="S532" s="41">
         <f>IF(AND(R532&gt;=CO2_pH_hi_mt,R533&lt;CO2_pH_hi_mt),EXP(LN(A532)+(LN(A533)-LN(A532))*(R532-CO2_pH_hi_mt)/(R532-R533)),0)</f>
@@ -38788,19 +38792,19 @@
       </c>
       <c r="L533" s="41">
         <f>k_eff_CO2_l*B533</f>
-        <v>3.317375185628</v>
+        <v>3.574723072711</v>
       </c>
       <c r="M533" s="41">
         <f>EXP(-L533)</f>
-        <v>0.036247850876</v>
+        <v>0.028023185084</v>
       </c>
       <c r="N533" s="41">
         <f>IF(L533&gt;0,(1-M533)/L533,1)</f>
-        <v>0.290516476189</v>
+        <v>0.271902688724</v>
       </c>
       <c r="O533" s="41">
         <f>IF(L533&gt;0,(L533-1+M533)/L533^2,1/2)</f>
-        <v>0.213868942797</v>
+        <v>0.203679361021</v>
       </c>
       <c r="P533" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B533/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38808,11 +38812,11 @@
       </c>
       <c r="Q533" s="41">
         <f>(P533*N533+pool_b*M533)/(1-pool_ret*M533)</f>
-        <v>0.099597933753</v>
+        <v>0.076780739194</v>
       </c>
       <c r="R533" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q533+pool_b)*N533+P533*O533))</f>
-        <v>0.782072696564</v>
+        <v>0.726361113416</v>
       </c>
       <c r="S533" s="41">
         <f>IF(AND(R533&gt;=CO2_pH_hi_mt,R534&lt;CO2_pH_hi_mt),EXP(LN(A533)+(LN(A534)-LN(A533))*(R533-CO2_pH_hi_mt)/(R533-R534)),0)</f>
@@ -38862,19 +38866,19 @@
       </c>
       <c r="L534" s="41">
         <f>k_eff_CO2_l*B534</f>
-        <v>3.71567994758</v>
+        <v>4.003926627584</v>
       </c>
       <c r="M534" s="41">
         <f>EXP(-L534)</f>
-        <v>0.024338886321</v>
+        <v>0.01824386121</v>
       </c>
       <c r="N534" s="41">
         <f>IF(L534&gt;0,(1-M534)/L534,1)</f>
-        <v>0.262579427573</v>
+        <v>0.245198334062</v>
       </c>
       <c r="O534" s="41">
         <f>IF(L534&gt;0,(L534-1+M534)/L534^2,1/2)</f>
-        <v>0.198461811251</v>
+        <v>0.188515359082</v>
       </c>
       <c r="P534" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B534/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38882,11 +38886,11 @@
       </c>
       <c r="Q534" s="41">
         <f>(P534*N534+pool_b*M534)/(1-pool_ret*M534)</f>
-        <v>0.066911501477</v>
+        <v>0.050294720584</v>
       </c>
       <c r="R534" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q534+pool_b)*N534+P534*O534))</f>
-        <v>0.699299085505</v>
+        <v>0.649339855951</v>
       </c>
       <c r="S534" s="41">
         <f>IF(AND(R534&gt;=CO2_pH_hi_mt,R535&lt;CO2_pH_hi_mt),EXP(LN(A534)+(LN(A535)-LN(A534))*(R534-CO2_pH_hi_mt)/(R534-R535)),0)</f>
@@ -38936,19 +38940,19 @@
       </c>
       <c r="L535" s="41">
         <f>k_eff_CO2_l*B535</f>
-        <v>4.161806982313</v>
+        <v>4.48466230419</v>
       </c>
       <c r="M535" s="41">
         <f>EXP(-L535)</f>
-        <v>0.015579380804</v>
+        <v>0.011280696321</v>
       </c>
       <c r="N535" s="41">
         <f>IF(L535&gt;0,(1-M535)/L535,1)</f>
-        <v>0.236536827243</v>
+        <v>0.220466834873</v>
       </c>
       <c r="O535" s="41">
         <f>IF(L535&gt;0,(L535-1+M535)/L535^2,1/2)</f>
-        <v>0.18344511795</v>
+        <v>0.173822043278</v>
       </c>
       <c r="P535" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B535/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -38956,11 +38960,11 @@
       </c>
       <c r="Q535" s="41">
         <f>(P535*N535+pool_b*M535)/(1-pool_ret*M535)</f>
-        <v>0.04332676369</v>
+        <v>0.031725391294</v>
       </c>
       <c r="R535" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q535+pool_b)*N535+P535*O535))</f>
-        <v>0.625108934548</v>
+        <v>0.580346083295</v>
       </c>
       <c r="S535" s="41">
         <f>IF(AND(R535&gt;=CO2_pH_hi_mt,R536&lt;CO2_pH_hi_mt),EXP(LN(A535)+(LN(A536)-LN(A535))*(R535-CO2_pH_hi_mt)/(R535-R536)),0)</f>
@@ -39010,19 +39014,19 @@
       </c>
       <c r="L536" s="41">
         <f>k_eff_CO2_l*B536</f>
-        <v>4.661498048379</v>
+        <v>5.023117282341</v>
       </c>
       <c r="M536" s="41">
         <f>EXP(-L536)</f>
-        <v>0.0094522918</v>
+        <v>0.006583970591</v>
       </c>
       <c r="N536" s="41">
         <f>IF(L536&gt;0,(1-M536)/L536,1)</f>
-        <v>0.21249557501</v>
+        <v>0.197768830304</v>
       </c>
       <c r="O536" s="41">
         <f>IF(L536&gt;0,(L536-1+M536)/L536^2,1/2)</f>
-        <v>0.168938057426</v>
+        <v>0.159707831732</v>
       </c>
       <c r="P536" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B536/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -39030,11 +39034,11 @@
       </c>
       <c r="Q536" s="41">
         <f>(P536*N536+pool_b*M536)/(1-pool_ret*M536)</f>
-        <v>0.027054526763</v>
+        <v>0.019333515078</v>
       </c>
       <c r="R536" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q536+pool_b)*N536+P536*O536))</f>
-        <v>0.558670355068</v>
+        <v>0.518593345206</v>
       </c>
       <c r="S536" s="41">
         <f>IF(AND(R536&gt;=CO2_pH_hi_mt,R537&lt;CO2_pH_hi_mt),EXP(LN(A536)+(LN(A537)-LN(A536))*(R536-CO2_pH_hi_mt)/(R536-R537)),0)</f>
@@ -39084,19 +39088,19 @@
       </c>
       <c r="L537" s="41">
         <f>k_eff_CO2_l*B537</f>
-        <v>5.221184285857</v>
+        <v>5.626221602666</v>
       </c>
       <c r="M537" s="41">
         <f>EXP(-L537)</f>
-        <v>0.005400929094</v>
+        <v>0.003602160039</v>
       </c>
       <c r="N537" s="41">
         <f>IF(L537&gt;0,(1-M537)/L537,1)</f>
-        <v>0.19049300244</v>
+        <v>0.177098932521</v>
       </c>
       <c r="O537" s="41">
         <f>IF(L537&gt;0,(L537-1+M537)/L537^2,1/2)</f>
-        <v>0.155042793596</v>
+        <v>0.146261758884</v>
       </c>
       <c r="P537" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B537/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -39104,11 +39108,11 @@
       </c>
       <c r="Q537" s="41">
         <f>(P537*N537+pool_b*M537)/(1-pool_ret*M537)</f>
-        <v>0.016394846184</v>
+        <v>0.011521282843</v>
       </c>
       <c r="R537" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q537+pool_b)*N537+P537*O537))</f>
-        <v>0.499219659328</v>
+        <v>0.463360488663</v>
       </c>
       <c r="S537" s="41">
         <f>IF(AND(R537&gt;=CO2_pH_hi_mt,R538&lt;CO2_pH_hi_mt),EXP(LN(A537)+(LN(A538)-LN(A537))*(R537-CO2_pH_hi_mt)/(R537-R538)),0)</f>
@@ -39158,19 +39162,19 @@
       </c>
       <c r="L538" s="41">
         <f>k_eff_CO2_l*B538</f>
-        <v>5.848068986615</v>
+        <v>6.301737357844</v>
       </c>
       <c r="M538" s="41">
         <f>EXP(-L538)</f>
-        <v>0.002885465655</v>
+        <v>0.001833117228</v>
       </c>
       <c r="N538" s="41">
         <f>IF(L538&gt;0,(1-M538)/L538,1)</f>
-        <v>0.17050320997</v>
+        <v>0.158395506841</v>
       </c>
       <c r="O538" s="41">
         <f>IF(L538&gt;0,(L538-1+M538)/L538^2,1/2)</f>
-        <v>0.141841143107</v>
+        <v>0.133551185232</v>
       </c>
       <c r="P538" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B538/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -39178,11 +39182,11 @@
       </c>
       <c r="Q538" s="41">
         <f>(P538*N538+pool_b*M538)/(1-pool_ret*M538)</f>
-        <v>0.009815867939</v>
+        <v>0.006906471999</v>
       </c>
       <c r="R538" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q538+pool_b)*N538+P538*O538))</f>
-        <v>0.446057031952</v>
+        <v>0.413987659751</v>
       </c>
       <c r="S538" s="41">
         <f>IF(AND(R538&gt;=CO2_pH_hi_mt,R539&lt;CO2_pH_hi_mt),EXP(LN(A538)+(LN(A539)-LN(A538))*(R538-CO2_pH_hi_mt)/(R538-R539)),0)</f>
@@ -39232,19 +39236,19 @@
       </c>
       <c r="L539" s="41">
         <f>k_eff_CO2_l*B539</f>
-        <v>6.550220302351</v>
+        <v>7.058358592538</v>
       </c>
       <c r="M539" s="41">
         <f>EXP(-L539)</f>
-        <v>0.001429800575</v>
+        <v>0.0008601888562468</v>
       </c>
       <c r="N539" s="41">
         <f>IF(L539&gt;0,(1-M539)/L539,1)</f>
-        <v>0.152448338122</v>
+        <v>0.141554130191</v>
       </c>
       <c r="O539" s="41">
         <f>IF(L539&gt;0,(L539-1+M539)/L539^2,1/2)</f>
-        <v>0.129392848295</v>
+        <v>0.121621175597</v>
       </c>
       <c r="P539" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B539/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -39252,11 +39256,11 @@
       </c>
       <c r="Q539" s="41">
         <f>(P539*N539+pool_b*M539)/(1-pool_ret*M539)</f>
-        <v>0.006022438775</v>
+        <v>0.004374764077</v>
       </c>
       <c r="R539" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q539+pool_b)*N539+P539*O539))</f>
-        <v>0.398542714502</v>
+        <v>0.369872825948</v>
       </c>
       <c r="S539" s="41">
         <f>0</f>
@@ -39715,7 +39719,7 @@
     <row r="560">
       <c r="A560" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pool decay rate through the vent — lag</t>
+          <t xml:space="preserve">Pool decay rate through the vent — start-up</t>
         </is>
       </c>
       <c r="B560" s="19" t="inlineStr">
@@ -39729,12 +39733,12 @@
         </is>
       </c>
       <c r="D560" s="41">
-        <f>F_gap_l/3600/n_hs_gas*Vg_CO2/(V_L_CO2+Vg_CO2)</f>
-        <v>7.278075122043e-05</v>
+        <f>F_gap_su/3600/n_hs_gas*Vg_CO2/(V_L_CO2+Vg_CO2)</f>
+        <v>7.842677299934e-05</v>
       </c>
       <c r="E560" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">As D195 on the lag gas flow (F_gap_l, D353), for the lag columns L–S of the interval grid.</t>
+          <t xml:space="preserve">As D195 on the start-up gas flow (F_gap_su, D575), for the start-up columns L–S of the interval grid, so the start-up pH bound (D561) uses the same sources as the start-up balance. Equals the lag flow (D353) when sized on Lag.</t>
         </is>
       </c>
     </row>
@@ -39756,7 +39760,7 @@
       </c>
       <c r="D561" s="41">
         <f>IF(CO2_pH_hi_mt&lt;=0,"no pH bound",IF(INDEX(pHg_C_l,1)&lt;CO2_pH_hi_mt,"pH above the band ceiling at any interval in lag",IF(MAX(pHg_x_l)&gt;0,MAX(pHg_x_l),"no pH bound")))</f>
-        <v>612.612318746651</v>
+        <v>568.953730792824</v>
       </c>
       <c r="E561" s="51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Gas model: eleventh Codex review fixes (free-chlorine assay includes hypochlorite, start-up pH note, lifetime leverage restated)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -13709,7 +13709,7 @@
       </c>
       <c r="F125" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Settles the monochloramine lifetime (Chemistry D142, entered in the Calibrations monochloramine section), which moves the UdG interval by about ±32 %. Also confirm the CaCl₂ hydrate state (−24 % on every chlorine figure).</t>
+          <t xml:space="preserve">Settles the monochloramine lifetime (Chemistry D142, entered in the Calibrations monochloramine section): over 1 min to 5 h it moves the UdG interval from 9.4 to 7.6 min against 8.1 min at the 1 h default (about +15 %/−7 %). Also confirm the CaCl₂ hydrate state (−24 % on every chlorine figure).</t>
         </is>
       </c>
     </row>
@@ -39400,7 +39400,7 @@
       </c>
       <c r="E546" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">The shortest of the carbon bound, the lag O₂ bound (or the start-up legacy guard D583 when the lag DO target is unreachable), the start-up hazard-screen interval (D582) and the lag pH ceiling (D561), on the basis of D91, all on the start-up sources (D572–D576). #N/A when no interval holds the lag pH under the ceiling. Equals D91 when Summary D12 is Lag. The lag pH grid (D561) keeps the headline lag gas flow; it binds only at intervals hundreds of times longer.</t>
+          <t xml:space="preserve">The shortest of the carbon bound, the lag O₂ bound (or the start-up legacy guard D583 when the lag DO target is unreachable), the start-up hazard-screen interval (D582) and the start-up pH ceiling (D561, on the start-up gas flow D560), on the basis of D91, all on the start-up sources (D572–D576). #N/A when no interval holds the pH under the ceiling. Equals D91 when Summary D12 is Lag. The pH ceiling can bind, e.g. with N₂ and added alkalinity.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: twelfth Codex review fixes (series-stable exponential helpers and DO peak at near-zero vent flow, wrapped Summary notes, sensitivity printout cells)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -1100,6 +1100,7 @@
     <definedName name="chk_DO_pH" localSheetId="0">Summary!$D$52</definedName>
     <definedName name="chk_hs_sag" localSheetId="0">Summary!$D$53</definedName>
     <definedName name="chk_hs_sag_ok" localSheetId="0">Summary!$D$54</definedName>
+    <definedName name="x_series" localSheetId="5">'Mass Transfer'!$D$584</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1" fullCalcOnLoad="1"/>
   <extLst>
@@ -10367,7 +10368,7 @@
     <xf numFmtId="0" fontId="26" fillId="17" borderId="11"/>
     <xf numFmtId="44" fontId="49" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="180">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="45" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -10630,6 +10631,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -11799,7 +11809,7 @@
         </is>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" thickBot="1" x14ac:dyDescent="0.25" ht="32" customHeight="1">
       <c r="A25" s="64" t="s">
         <v>1029</v>
       </c>
@@ -11817,7 +11827,7 @@
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F25" s="111" t="str">
+      <c r="F25" s="180" t="str">
         <f>IF(Chemistry!Cl_model_check&lt;&gt;"OK",Chemistry!Cl_model_check,"Effective chlorine on the as-Cl2 basis; zero for chloride-free medium. Lifetime and potency require measurement.")</f>
         <v>Effective chlorine on the as-Cl2 basis; zero for chloride-free medium. Lifetime and potency require measurement.</v>
       </c>
@@ -12030,7 +12040,7 @@
         </is>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A36" s="64" t="s">
         <v>64</v>
       </c>
@@ -12046,11 +12056,11 @@
         <f>HYPERLINK("#'Mass Transfer'!D120","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F36" s="22" t="s">
+      <c r="F36" s="181" t="s">
         <v>1720</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2" ht="62" customHeight="1">
       <c r="A37" s="64" t="s">
         <v>1721</v>
       </c>
@@ -12066,7 +12076,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D374","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F37" s="22" t="s">
+      <c r="F37" s="181" t="s">
         <v>1723</v>
       </c>
     </row>
@@ -12106,7 +12116,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F39" s="22" t="s">
+      <c r="F39" s="181" t="s">
         <v>1727</v>
       </c>
     </row>
@@ -12132,7 +12142,7 @@
         </is>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A41" s="64" t="s">
         <v>67</v>
       </c>
@@ -12148,7 +12158,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D64","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F41" s="22" t="s">
+      <c r="F41" s="181" t="s">
         <v>68</v>
       </c>
     </row>
@@ -12174,7 +12184,7 @@
         </is>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A43" s="64" t="s">
         <v>70</v>
       </c>
@@ -12190,7 +12200,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D130","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F43" s="22" t="s">
+      <c r="F43" s="181" t="s">
         <v>1735</v>
       </c>
     </row>
@@ -12332,7 +12342,7 @@
         <f>HYPERLINK("#Biology!D45","→ Biology")</f>
         <v>→ Biology</v>
       </c>
-      <c r="F50" s="22" t="s">
+      <c r="F50" s="181" t="s">
         <v>898</v>
       </c>
     </row>
@@ -12380,7 +12390,7 @@
         </is>
       </c>
     </row>
-    <row r="53" x14ac:dyDescent="0.2">
+    <row r="53" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A53" s="64" t="s">
         <v>1829</v>
       </c>
@@ -12400,7 +12410,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D389","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F53" s="22" t="s">
+      <c r="F53" s="181" t="s">
         <v>1830</v>
       </c>
     </row>
@@ -12518,7 +12528,7 @@
         <v>1804</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A61" s="64" t="s">
         <v>1805</v>
       </c>
@@ -12533,7 +12543,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F61" s="22" t="s">
+      <c r="F61" s="181" t="s">
         <v>1806</v>
       </c>
     </row>
@@ -12620,12 +12630,12 @@
         <f>HYPERLINK("#'Mass Transfer'!D368","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F66" s="154" t="str">
+      <c r="F66" s="182" t="str">
         <f>"Same on the lag source. Currently "&amp;TEXT('Mass Transfer'!kLa_margin_l,"0.00")&amp;"×: "&amp;IF('Mass Transfer'!kLa_margin_l&lt;1,"the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).","the target can be held during lag at the kLa in use.")</f>
         <v>Same on the lag source. Currently 0.61×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A67" s="64" t="s">
         <v>1816</v>
       </c>
@@ -12640,11 +12650,11 @@
         <f>HYPERLINK("#'Mass Transfer'!D345","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F67" s="22" t="s">
+      <c r="F67" s="181" t="s">
         <v>1817</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A68" s="64" t="s">
         <v>1818</v>
       </c>
@@ -12659,7 +12669,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D366","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F68" s="22" t="s">
+      <c r="F68" s="181" t="s">
         <v>1817</v>
       </c>
     </row>
@@ -12722,7 +12732,7 @@
         <v>1824</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A72" s="64" t="s">
         <v>1825</v>
       </c>
@@ -12737,7 +12747,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D381","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F72" s="22" t="s">
+      <c r="F72" s="181" t="s">
         <v>1826</v>
       </c>
     </row>
@@ -12851,7 +12861,7 @@
         </is>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A81" s="64" t="s">
         <v>2694</v>
       </c>
@@ -12866,7 +12876,7 @@
         <f>HYPERLINK("#Chemistry!D306","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F81" s="22" t="s">
+      <c r="F81" s="181" t="s">
         <v>2696</v>
       </c>
     </row>
@@ -12969,7 +12979,7 @@
         <v>1149</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A88" s="64" t="s">
         <v>1150</v>
       </c>
@@ -12984,7 +12994,7 @@
         <f>HYPERLINK("#Electrochemistry!D62","→ Electrochemistry")</f>
         <v>→ Electrochemistry</v>
       </c>
-      <c r="F88" s="22" t="s">
+      <c r="F88" s="181" t="s">
         <v>1151</v>
       </c>
     </row>
@@ -13298,7 +13308,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A106" s="21" t="s">
         <v>921</v>
       </c>
@@ -13313,11 +13323,11 @@
         <v>surface-kla.md →</v>
       </c>
       <c r="E106" s="77"/>
-      <c r="F106" s="22" t="s">
+      <c r="F106" s="181" t="s">
         <v>1766</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A107" s="21" t="s">
         <v>924</v>
       </c>
@@ -13332,11 +13342,11 @@
         <v>vial-geometry.md →</v>
       </c>
       <c r="E107" s="77"/>
-      <c r="F107" s="22" t="s">
+      <c r="F107" s="181" t="s">
         <v>1767</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A108" s="21" t="s">
         <v>927</v>
       </c>
@@ -13351,11 +13361,11 @@
         <v>faradaic-efficiency.md →</v>
       </c>
       <c r="E108" s="77"/>
-      <c r="F108" s="22" t="s">
+      <c r="F108" s="181" t="s">
         <v>1768</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A109" s="21" t="s">
         <v>930</v>
       </c>
@@ -13370,7 +13380,7 @@
         <v>knallgas-stoichiometry.md →</v>
       </c>
       <c r="E109" s="77"/>
-      <c r="F109" s="154" t="str">
+      <c r="F109" s="182" t="str">
         <f>IFERROR("Sets the O₂ surplus and the carbon demand: each 1 % on the O₂:H₂ uptake ratio moves the surplus "&amp;TEXT(Biology!O2_cons/Biology!O2_excess,"0.0")&amp;" % (Biology E16); needs a growing culture.","Sets the O₂ surplus and the carbon demand; needs a growing culture.")</f>
         <v>Sets the O₂ surplus and the carbon demand: each 1 % on the O₂:H₂ uptake ratio moves the surplus 2.0 % (Biology E16); needs a growing culture.</v>
       </c>
@@ -13417,7 +13427,7 @@
         </is>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A112" s="21" t="s">
         <v>940</v>
       </c>
@@ -13432,7 +13442,7 @@
         <v>flow-calibration.md →</v>
       </c>
       <c r="E112" s="77"/>
-      <c r="F112" s="154" t="str">
+      <c r="F112" s="182" t="str">
         <f>"Sets the solenoid floor (pulse_floor, now "&amp;TEXT('Mass Transfer'!pulse_floor,"0.00")&amp;" s), which binds only when it exceeds the optimal pulse ("&amp;IF(ISNUMBER(res_spg_dur),TEXT(res_spg_dur,"0.00")&amp;" s","not yet computed")&amp;"): "&amp;IF(AND(ISNUMBER(res_spg_dur),'Mass Transfer'!pulse_floor&gt;=res_spg_dur),"it does now, so the pulse IS the floor","it does not now, so it matters only for a smaller headspace or a faster flow")&amp;". Trivial to characterise on the bench (flow-calibration.md)."</f>
         <v>Sets the solenoid floor (pulse_floor, now 0.25 s), which binds only when it exceeds the optimal pulse (0.67 s): it does not now, so it matters only for a smaller headspace or a faster flow. Trivial to characterise on the bench (flow-calibration.md).</v>
       </c>
@@ -25574,7 +25584,7 @@
   <sheetPr>
     <tabColor theme="6"/>
   </sheetPr>
-  <dimension ref="A1:S583"/>
+  <dimension ref="A1:S584"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -29951,7 +29961,7 @@
         <v>111</v>
       </c>
       <c r="D333" s="41">
-        <f>IF(x_hs_g&gt;0,(1-EXP(-x_hs_g))/x_hs_g,1)</f>
+        <f>IF(x_hs_g&gt;x_series,(1-EXP(-x_hs_g))/x_hs_g,1-x_hs_g/2+x_hs_g^2/6-x_hs_g^3/24)</f>
         <v>0.979144642091</v>
       </c>
       <c r="E333" s="51" t="s">
@@ -29969,7 +29979,7 @@
         <v>111</v>
       </c>
       <c r="D334" s="41">
-        <f>IF(x_hs_g&gt;0,(x_hs_g-1+EXP(-x_hs_g))/x_hs_g^2,1/2)</f>
+        <f>IF(x_hs_g&gt;x_series,(x_hs_g-1+EXP(-x_hs_g))/x_hs_g^2,1/2-x_hs_g/6+x_hs_g^2/24-x_hs_g^3/120)</f>
         <v>0.493023777802</v>
       </c>
       <c r="E334" s="51" t="s">
@@ -30351,7 +30361,7 @@
         <v>111</v>
       </c>
       <c r="D355" s="41">
-        <f>IF(x_hs_l&gt;0,(1-EXP(-x_hs_l))/x_hs_l,1)</f>
+        <f>IF(x_hs_l&gt;x_series,(1-EXP(-x_hs_l))/x_hs_l,1-x_hs_l/2+x_hs_l^2/6-x_hs_l^3/24)</f>
         <v>0.901102060357</v>
       </c>
       <c r="E355" s="51" t="s">
@@ -30369,7 +30379,7 @@
         <v>111</v>
       </c>
       <c r="D356" s="41">
-        <f>IF(x_hs_l&gt;0,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2)</f>
+        <f>IF(x_hs_l&gt;x_series,(x_hs_l-1+EXP(-x_hs_l))/x_hs_l^2,1/2-x_hs_l/6+x_hs_l^2/24-x_hs_l^3/120)</f>
         <v>0.466459942253</v>
       </c>
       <c r="E356" s="51" t="s">
@@ -30735,7 +30745,7 @@
         <v>111</v>
       </c>
       <c r="D377" s="41">
-        <f>IF(pool_x&gt;0,(1-EXP(-pool_x))/pool_x,1)</f>
+        <f>IF(pool_x&gt;x_series,(1-EXP(-pool_x))/pool_x,1-pool_x/2+pool_x^2/6-pool_x^3/24)</f>
         <v>0.996931131905</v>
       </c>
       <c r="E377" s="51" t="s">
@@ -30753,7 +30763,7 @@
         <v>111</v>
       </c>
       <c r="D378" s="41">
-        <f>IF(pool_x&gt;0,(pool_x-1+EXP(-pool_x))/pool_x^2,1/2)</f>
+        <f>IF(pool_x&gt;x_series,(pool_x-1+EXP(-pool_x))/pool_x^2,1/2-pool_x/6+pool_x^2/24-pool_x^3/120)</f>
         <v>0.498976519889</v>
       </c>
       <c r="E378" s="51" t="s">
@@ -31885,12 +31895,12 @@
         <v>0.999992013539</v>
       </c>
       <c r="E440" s="41">
-        <f>IF(C440&gt;0,(1-D440)/C440,1)</f>
-        <v>0.99999600677</v>
+        <f>IF(C440&gt;x_series,(1-EXP(-C440))/C440,1-C440/2+C440^2/6-C440^3/24)</f>
+        <v>0.999996006764</v>
       </c>
       <c r="F440" s="41">
-        <f>IF(C440&gt;0,(C440-1+D440)/C440^2,1/2)</f>
-        <v>0.499998404672</v>
+        <f>IF(C440&gt;x_series,(C440-1+EXP(-C440))/C440^2,1/2-C440/6+C440^2/24-C440^3/120)</f>
+        <v>0.49999866892</v>
       </c>
       <c r="G440" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B440/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -31902,7 +31912,7 @@
       </c>
       <c r="I440" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H440+pool_b)*E440+G440*F440))</f>
-        <v>28.052312327445</v>
+        <v>28.052312327239</v>
       </c>
       <c r="J440" s="41">
         <f>IF(AND(I440&gt;=CO2_pH_hi_mt,I441&lt;CO2_pH_hi_mt),EXP(LN(A440)+(LN(A441)-LN(A440))*(I440-CO2_pH_hi_mt)/(I440-I441)),0)</f>
@@ -31917,12 +31927,12 @@
         <v>0.999956866205</v>
       </c>
       <c r="N440" s="41">
-        <f>IF(L440&gt;0,(1-M440)/L440,1)</f>
+        <f>IF(L440&gt;x_series,(1-EXP(-L440))/L440,1-L440/2+L440^2/6-L440^3/24)</f>
         <v>0.999978432948</v>
       </c>
       <c r="O440" s="41">
-        <f>IF(L440&gt;0,(L440-1+M440)/L440^2,1/2)</f>
-        <v>0.499992792176</v>
+        <f>IF(L440&gt;x_series,(L440-1+EXP(-L440))/L440^2,1/2-L440/6+L440^2/24-L440^3/120)</f>
+        <v>0.499992810957</v>
       </c>
       <c r="P440" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B440/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -31934,7 +31944,7 @@
       </c>
       <c r="R440" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q440+pool_b)*N440+P440*O440))</f>
-        <v>28.043242201082</v>
+        <v>28.043242201079</v>
       </c>
       <c r="S440" s="41">
         <f>IF(AND(R440&gt;=CO2_pH_hi_mt,R441&lt;CO2_pH_hi_mt),EXP(LN(A440)+(LN(A441)-LN(A440))*(R440-CO2_pH_hi_mt)/(R440-R441)),0)</f>
@@ -31959,12 +31969,12 @@
         <v>0.999989921424</v>
       </c>
       <c r="E441" s="41">
-        <f>IF(C441&gt;0,(1-D441)/C441,1)</f>
-        <v>0.999994960707</v>
+        <f>IF(C441&gt;x_series,(1-EXP(-C441))/C441,1-C441/2+C441^2/6-C441^3/24)</f>
+        <v>0.999994960704</v>
       </c>
       <c r="F441" s="41">
-        <f>IF(C441&gt;0,(C441-1+D441)/C441^2,1/2)</f>
-        <v>0.49999798057</v>
+        <f>IF(C441&gt;x_series,(C441-1+EXP(-C441))/C441^2,1/2-C441/6+C441^2/24-C441^3/120)</f>
+        <v>0.499998320233</v>
       </c>
       <c r="G441" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B441/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -31976,7 +31986,7 @@
       </c>
       <c r="I441" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H441+pool_b)*E441+G441*F441))</f>
-        <v>28.051422535946</v>
+        <v>28.051422535813</v>
       </c>
       <c r="J441" s="41">
         <f>IF(AND(I441&gt;=CO2_pH_hi_mt,I442&lt;CO2_pH_hi_mt),EXP(LN(A441)+(LN(A442)-LN(A441))*(I441-CO2_pH_hi_mt)/(I441-I442)),0)</f>
@@ -31991,12 +32001,12 @@
         <v>0.999945567228</v>
       </c>
       <c r="N441" s="41">
-        <f>IF(L441&gt;0,(1-M441)/L441,1)</f>
-        <v>0.999972783368</v>
+        <f>IF(L441&gt;x_series,(1-EXP(-L441))/L441,1-L441/2+L441^2/6-L441^3/24)</f>
+        <v>0.999972783367</v>
       </c>
       <c r="O441" s="41">
-        <f>IF(L441&gt;0,(L441-1+M441)/L441^2,1/2)</f>
-        <v>0.499990907593</v>
+        <f>IF(L441&gt;x_series,(L441-1+EXP(-L441))/L441^2,1/2-L441/6+L441^2/24-L441^3/120)</f>
+        <v>0.499990927748</v>
       </c>
       <c r="P441" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B441/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32008,7 +32018,7 @@
       </c>
       <c r="R441" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q441+pool_b)*N441+P441*O441))</f>
-        <v>28.039978146359</v>
+        <v>28.039978146336</v>
       </c>
       <c r="S441" s="41">
         <f>IF(AND(R441&gt;=CO2_pH_hi_mt,R442&lt;CO2_pH_hi_mt),EXP(LN(A441)+(LN(A442)-LN(A441))*(R441-CO2_pH_hi_mt)/(R441-R442)),0)</f>
@@ -32033,12 +32043,12 @@
         <v>0.999987578126</v>
       </c>
       <c r="E442" s="41">
-        <f>IF(C442&gt;0,(1-D442)/C442,1)</f>
-        <v>0.999993789053</v>
+        <f>IF(C442&gt;x_series,(1-EXP(-C442))/C442,1-C442/2+C442^2/6-C442^3/24)</f>
+        <v>0.99999378905</v>
       </c>
       <c r="F442" s="41">
-        <f>IF(C442&gt;0,(C442-1+D442)/C442^2,1/2)</f>
-        <v>0.499997600822</v>
+        <f>IF(C442&gt;x_series,(C442-1+EXP(-C442))/C442^2,1/2-C442/6+C442^2/24-C442^3/120)</f>
+        <v>0.499997929681</v>
       </c>
       <c r="G442" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B442/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32050,7 +32060,7 @@
       </c>
       <c r="I442" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H442+pool_b)*E442+G442*F442))</f>
-        <v>28.050425957643</v>
+        <v>28.050425957523</v>
       </c>
       <c r="J442" s="41">
         <f>IF(AND(I442&gt;=CO2_pH_hi_mt,I443&lt;CO2_pH_hi_mt),EXP(LN(A442)+(LN(A443)-LN(A442))*(I442-CO2_pH_hi_mt)/(I442-I443)),0)</f>
@@ -32065,12 +32075,12 @@
         <v>0.999932911797</v>
       </c>
       <c r="N442" s="41">
-        <f>IF(L442&gt;0,(1-M442)/L442,1)</f>
-        <v>0.999966455524</v>
+        <f>IF(L442&gt;x_series,(1-EXP(-L442))/L442,1-L442/2+L442^2/6-L442^3/24)</f>
+        <v>0.999966455523</v>
       </c>
       <c r="O442" s="41">
-        <f>IF(L442&gt;0,(L442-1+M442)/L442^2,1/2)</f>
-        <v>0.499988805959</v>
+        <f>IF(L442&gt;x_series,(L442-1+EXP(-L442))/L442^2,1/2-L442/6+L442^2/24-L442^3/120)</f>
+        <v>0.499988818445</v>
       </c>
       <c r="P442" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B442/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32082,7 +32092,7 @@
       </c>
       <c r="R442" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q442+pool_b)*N442+P442*O442))</f>
-        <v>28.036323095804</v>
+        <v>28.036323095797</v>
       </c>
       <c r="S442" s="41">
         <f>IF(AND(R442&gt;=CO2_pH_hi_mt,R443&lt;CO2_pH_hi_mt),EXP(LN(A442)+(LN(A443)-LN(A442))*(R442-CO2_pH_hi_mt)/(R442-R443)),0)</f>
@@ -32107,12 +32117,12 @@
         <v>0.999984953488</v>
       </c>
       <c r="E443" s="41">
-        <f>IF(C443&gt;0,(1-D443)/C443,1)</f>
+        <f>IF(C443&gt;x_series,(1-EXP(-C443))/C443,1-C443/2+C443^2/6-C443^3/24)</f>
         <v>0.999992476725</v>
       </c>
       <c r="F443" s="41">
-        <f>IF(C443&gt;0,(C443-1+D443)/C443^2,1/2)</f>
-        <v>0.499997452808</v>
+        <f>IF(C443&gt;x_series,(C443-1+EXP(-C443))/C443^2,1/2-C443/6+C443^2/24-C443^3/120)</f>
+        <v>0.499997492239</v>
       </c>
       <c r="G443" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B443/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32124,7 +32134,7 @@
       </c>
       <c r="I443" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H443+pool_b)*E443+G443*F443))</f>
-        <v>28.049309782645</v>
+        <v>28.049309782637</v>
       </c>
       <c r="J443" s="41">
         <f>IF(AND(I443&gt;=CO2_pH_hi_mt,I444&lt;CO2_pH_hi_mt),EXP(LN(A443)+(LN(A444)-LN(A443))*(I443-CO2_pH_hi_mt)/(I443-I444)),0)</f>
@@ -32139,12 +32149,12 @@
         <v>0.999918737087</v>
       </c>
       <c r="N443" s="41">
-        <f>IF(L443&gt;0,(1-M443)/L443,1)</f>
+        <f>IF(L443&gt;x_series,(1-EXP(-L443))/L443,1-L443/2+L443^2/6-L443^3/24)</f>
         <v>0.999959367993</v>
       </c>
       <c r="O443" s="41">
-        <f>IF(L443&gt;0,(L443-1+M443)/L443^2,1/2)</f>
-        <v>0.499986444451</v>
+        <f>IF(L443&gt;x_series,(L443-1+EXP(-L443))/L443^2,1/2-L443/6+L443^2/24-L443^3/120)</f>
+        <v>0.499986455906</v>
       </c>
       <c r="P443" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B443/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32156,7 +32166,7 @@
       </c>
       <c r="R443" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q443+pool_b)*N443+P443*O443))</f>
-        <v>28.03223033375</v>
+        <v>28.03223033374</v>
       </c>
       <c r="S443" s="41">
         <f>IF(AND(R443&gt;=CO2_pH_hi_mt,R444&lt;CO2_pH_hi_mt),EXP(LN(A443)+(LN(A444)-LN(A443))*(R443-CO2_pH_hi_mt)/(R443-R444)),0)</f>
@@ -32181,12 +32191,12 @@
         <v>0.999982013731</v>
       </c>
       <c r="E444" s="41">
-        <f>IF(C444&gt;0,(1-D444)/C444,1)</f>
-        <v>0.999991006836</v>
+        <f>IF(C444&gt;x_series,(1-EXP(-C444))/C444,1-C444/2+C444^2/6-C444^3/24)</f>
+        <v>0.999991006839</v>
       </c>
       <c r="F444" s="41">
-        <f>IF(C444&gt;0,(C444-1+D444)/C444^2,1/2)</f>
-        <v>0.49999722252</v>
+        <f>IF(C444&gt;x_series,(C444-1+EXP(-C444))/C444^2,1/2-C444/6+C444^2/24-C444^3/120)</f>
+        <v>0.499997002275</v>
       </c>
       <c r="G444" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B444/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32198,7 +32208,7 @@
       </c>
       <c r="I444" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H444+pool_b)*E444+G444*F444))</f>
-        <v>28.048059666259</v>
+        <v>28.048059666376</v>
       </c>
       <c r="J444" s="41">
         <f>IF(AND(I444&gt;=CO2_pH_hi_mt,I445&lt;CO2_pH_hi_mt),EXP(LN(A444)+(LN(A445)-LN(A444))*(I444-CO2_pH_hi_mt)/(I444-I445)),0)</f>
@@ -32213,12 +32223,12 @@
         <v>0.999902860736</v>
       </c>
       <c r="N444" s="41">
-        <f>IF(L444&gt;0,(1-M444)/L444,1)</f>
+        <f>IF(L444&gt;x_series,(1-EXP(-L444))/L444,1-L444/2+L444^2/6-L444^3/24)</f>
         <v>0.999951429582</v>
       </c>
       <c r="O444" s="41">
-        <f>IF(L444&gt;0,(L444-1+M444)/L444^2,1/2)</f>
-        <v>0.499983806296</v>
+        <f>IF(L444&gt;x_series,(L444-1+EXP(-L444))/L444^2,1/2-L444/6+L444^2/24-L444^3/120)</f>
+        <v>0.499983809729</v>
       </c>
       <c r="P444" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B444/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32230,7 +32240,7 @@
       </c>
       <c r="R444" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q444+pool_b)*N444+P444*O444))</f>
-        <v>28.02764759365</v>
+        <v>28.027647593649</v>
       </c>
       <c r="S444" s="41">
         <f>IF(AND(R444&gt;=CO2_pH_hi_mt,R445&lt;CO2_pH_hi_mt),EXP(LN(A444)+(LN(A445)-LN(A444))*(R444-CO2_pH_hi_mt)/(R444-R445)),0)</f>
@@ -32255,12 +32265,12 @@
         <v>0.999978721025</v>
       </c>
       <c r="E445" s="41">
-        <f>IF(C445&gt;0,(1-D445)/C445,1)</f>
+        <f>IF(C445&gt;x_series,(1-EXP(-C445))/C445,1-C445/2+C445^2/6-C445^3/24)</f>
         <v>0.999989360475</v>
       </c>
       <c r="F445" s="41">
-        <f>IF(C445&gt;0,(C445-1+D445)/C445^2,1/2)</f>
-        <v>0.499996359475</v>
+        <f>IF(C445&gt;x_series,(C445-1+EXP(-C445))/C445^2,1/2-C445/6+C445^2/24-C445^3/120)</f>
+        <v>0.499996453485</v>
       </c>
       <c r="G445" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B445/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32272,7 +32282,7 @@
       </c>
       <c r="I445" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H445+pool_b)*E445+G445*F445))</f>
-        <v>28.046659545402</v>
+        <v>28.046659545359</v>
       </c>
       <c r="J445" s="41">
         <f>IF(AND(I445&gt;=CO2_pH_hi_mt,I446&lt;CO2_pH_hi_mt),EXP(LN(A445)+(LN(A446)-LN(A445))*(I445-CO2_pH_hi_mt)/(I445-I446)),0)</f>
@@ -32287,12 +32297,12 @@
         <v>0.999885078498</v>
       </c>
       <c r="N445" s="41">
-        <f>IF(L445&gt;0,(1-M445)/L445,1)</f>
+        <f>IF(L445&gt;x_series,(1-EXP(-L445))/L445,1-L445/2+L445^2/6-L445^3/24)</f>
         <v>0.999942538148</v>
       </c>
       <c r="O445" s="41">
-        <f>IF(L445&gt;0,(L445-1+M445)/L445^2,1/2)</f>
-        <v>0.499980844274</v>
+        <f>IF(L445&gt;x_series,(L445-1+EXP(-L445))/L445^2,1/2-L445/6+L445^2/24-L445^3/120)</f>
+        <v>0.499980845866</v>
       </c>
       <c r="P445" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B445/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32304,7 +32314,7 @@
       </c>
       <c r="R445" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q445+pool_b)*N445+P445*O445))</f>
-        <v>28.02251640649</v>
+        <v>28.022516406489</v>
       </c>
       <c r="S445" s="41">
         <f>IF(AND(R445&gt;=CO2_pH_hi_mt,R446&lt;CO2_pH_hi_mt),EXP(LN(A445)+(LN(A446)-LN(A445))*(R445-CO2_pH_hi_mt)/(R445-R446)),0)</f>
@@ -32329,12 +32339,12 @@
         <v>0.999975032994</v>
       </c>
       <c r="E446" s="41">
-        <f>IF(C446&gt;0,(1-D446)/C446,1)</f>
-        <v>0.999987516443</v>
+        <f>IF(C446&gt;x_series,(1-EXP(-C446))/C446,1-C446/2+C446^2/6-C446^3/24)</f>
+        <v>0.999987516445</v>
       </c>
       <c r="F446" s="41">
-        <f>IF(C446&gt;0,(C446-1+D446)/C446^2,1/2)</f>
-        <v>0.499995860338</v>
+        <f>IF(C446&gt;x_series,(C446-1+EXP(-C446))/C446^2,1/2-C446/6+C446^2/24-C446^3/120)</f>
+        <v>0.499995838806</v>
       </c>
       <c r="G446" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B446/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32346,7 +32356,7 @@
       </c>
       <c r="I446" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H446+pool_b)*E446+G446*F446))</f>
-        <v>28.045091432132</v>
+        <v>28.045091432197</v>
       </c>
       <c r="J446" s="41">
         <f>IF(AND(I446&gt;=CO2_pH_hi_mt,I447&lt;CO2_pH_hi_mt),EXP(LN(A446)+(LN(A447)-LN(A446))*(I446-CO2_pH_hi_mt)/(I446-I447)),0)</f>
@@ -32361,12 +32371,12 @@
         <v>0.999865161619</v>
       </c>
       <c r="N446" s="41">
-        <f>IF(L446&gt;0,(1-M446)/L446,1)</f>
+        <f>IF(L446&gt;x_series,(1-EXP(-L446))/L446,1-L446/2+L446^2/6-L446^3/24)</f>
         <v>0.999932579294</v>
       </c>
       <c r="O446" s="41">
-        <f>IF(L446&gt;0,(L446-1+M446)/L446^2,1/2)</f>
-        <v>0.499977530016</v>
+        <f>IF(L446&gt;x_series,(L446-1+EXP(-L446))/L446^2,1/2-L446/6+L446^2/24-L446^3/120)</f>
+        <v>0.499977526179</v>
       </c>
       <c r="P446" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B446/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32378,7 +32388,7 @@
       </c>
       <c r="R446" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q446+pool_b)*N446+P446*O446))</f>
-        <v>28.016771374425</v>
+        <v>28.016771374432</v>
       </c>
       <c r="S446" s="41">
         <f>IF(AND(R446&gt;=CO2_pH_hi_mt,R447&lt;CO2_pH_hi_mt),EXP(LN(A446)+(LN(A447)-LN(A446))*(R446-CO2_pH_hi_mt)/(R446-R447)),0)</f>
@@ -32403,12 +32413,12 @@
         <v>0.999970902177</v>
       </c>
       <c r="E447" s="41">
-        <f>IF(C447&gt;0,(1-D447)/C447,1)</f>
-        <v>0.999985451017</v>
+        <f>IF(C447&gt;x_series,(1-EXP(-C447))/C447,1-C447/2+C447^2/6-C447^3/24)</f>
+        <v>0.999985451018</v>
       </c>
       <c r="F447" s="41">
-        <f>IF(C447&gt;0,(C447-1+D447)/C447^2,1/2)</f>
-        <v>0.499995211509</v>
+        <f>IF(C447&gt;x_series,(C447-1+EXP(-C447))/C447^2,1/2-C447/6+C447^2/24-C447^3/120)</f>
+        <v>0.499995150328</v>
       </c>
       <c r="G447" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B447/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32420,7 +32430,7 @@
       </c>
       <c r="I447" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H447+pool_b)*E447+G447*F447))</f>
-        <v>28.043335185624</v>
+        <v>28.04333518567</v>
       </c>
       <c r="J447" s="41">
         <f>IF(AND(I447&gt;=CO2_pH_hi_mt,I448&lt;CO2_pH_hi_mt),EXP(LN(A447)+(LN(A448)-LN(A447))*(I447-CO2_pH_hi_mt)/(I447-I448)),0)</f>
@@ -32435,12 +32445,12 @@
         <v>0.9998428539</v>
       </c>
       <c r="N447" s="41">
-        <f>IF(L447&gt;0,(1-M447)/L447,1)</f>
+        <f>IF(L447&gt;x_series,(1-EXP(-L447))/L447,1-L447/2+L447^2/6-L447^3/24)</f>
         <v>0.999921424892</v>
       </c>
       <c r="O447" s="41">
-        <f>IF(L447&gt;0,(L447-1+M447)/L447^2,1/2)</f>
-        <v>0.499973806355</v>
+        <f>IF(L447&gt;x_series,(L447-1+EXP(-L447))/L447^2,1/2-L447/6+L447^2/24-L447^3/120)</f>
+        <v>0.499973807954</v>
       </c>
       <c r="P447" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B447/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32452,7 +32462,7 @@
       </c>
       <c r="R447" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q447+pool_b)*N447+P447*O447))</f>
-        <v>28.010339362057</v>
+        <v>28.010339362051</v>
       </c>
       <c r="S447" s="41">
         <f>IF(AND(R447&gt;=CO2_pH_hi_mt,R448&lt;CO2_pH_hi_mt),EXP(LN(A447)+(LN(A448)-LN(A447))*(R447-CO2_pH_hi_mt)/(R447-R448)),0)</f>
@@ -32477,12 +32487,12 @@
         <v>0.999966275416</v>
       </c>
       <c r="E448" s="41">
-        <f>IF(C448&gt;0,(1-D448)/C448,1)</f>
+        <f>IF(C448&gt;x_series,(1-EXP(-C448))/C448,1-C448/2+C448^2/6-C448^3/24)</f>
         <v>0.999983137613</v>
       </c>
       <c r="F448" s="41">
-        <f>IF(C448&gt;0,(C448-1+D448)/C448^2,1/2)</f>
-        <v>0.499994367627</v>
+        <f>IF(C448&gt;x_series,(C448-1+EXP(-C448))/C448^2,1/2-C448/6+C448^2/24-C448^3/120)</f>
+        <v>0.499994379189</v>
       </c>
       <c r="G448" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B448/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32494,7 +32504,7 @@
       </c>
       <c r="I448" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H448+pool_b)*E448+G448*F448))</f>
-        <v>28.041368253601</v>
+        <v>28.041368253604</v>
       </c>
       <c r="J448" s="41">
         <f>IF(AND(I448&gt;=CO2_pH_hi_mt,I449&lt;CO2_pH_hi_mt),EXP(LN(A448)+(LN(A449)-LN(A448))*(I448-CO2_pH_hi_mt)/(I448-I449)),0)</f>
@@ -32509,12 +32519,12 @@
         <v>0.999817868407</v>
       </c>
       <c r="N448" s="41">
-        <f>IF(L448&gt;0,(1-M448)/L448,1)</f>
+        <f>IF(L448&gt;x_series,(1-EXP(-L448))/L448,1-L448/2+L448^2/6-L448^3/24)</f>
         <v>0.999908931439</v>
       </c>
       <c r="O448" s="41">
-        <f>IF(L448&gt;0,(L448-1+M448)/L448^2,1/2)</f>
-        <v>0.499969643795</v>
+        <f>IF(L448&gt;x_series,(L448-1+EXP(-L448))/L448^2,1/2-L448/6+L448^2/24-L448^3/120)</f>
+        <v>0.499969643352</v>
       </c>
       <c r="P448" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B448/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32526,7 +32536,7 @@
       </c>
       <c r="R448" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q448+pool_b)*N448+P448*O448))</f>
-        <v>28.003138596202</v>
+        <v>28.00313859621</v>
       </c>
       <c r="S448" s="41">
         <f>IF(AND(R448&gt;=CO2_pH_hi_mt,R449&lt;CO2_pH_hi_mt),EXP(LN(A448)+(LN(A449)-LN(A448))*(R448-CO2_pH_hi_mt)/(R448-R449)),0)</f>
@@ -32551,12 +32561,12 @@
         <v>0.999961093171</v>
       </c>
       <c r="E449" s="41">
-        <f>IF(C449&gt;0,(1-D449)/C449,1)</f>
-        <v>0.999980546458</v>
+        <f>IF(C449&gt;x_series,(1-EXP(-C449))/C449,1-C449/2+C449^2/6-C449^3/24)</f>
+        <v>0.999980546459</v>
       </c>
       <c r="F449" s="41">
-        <f>IF(C449&gt;0,(C449-1+D449)/C449^2,1/2)</f>
-        <v>0.499993536553</v>
+        <f>IF(C449&gt;x_series,(C449-1+EXP(-C449))/C449^2,1/2-C449/6+C449^2/24-C449^3/120)</f>
+        <v>0.499993515465</v>
       </c>
       <c r="G449" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B449/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32568,7 +32578,7 @@
       </c>
       <c r="I449" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H449+pool_b)*E449+G449*F449))</f>
-        <v>28.039165385215</v>
+        <v>28.039165385257</v>
       </c>
       <c r="J449" s="41">
         <f>IF(AND(I449&gt;=CO2_pH_hi_mt,I450&lt;CO2_pH_hi_mt),EXP(LN(A449)+(LN(A450)-LN(A449))*(I449-CO2_pH_hi_mt)/(I449-I450)),0)</f>
@@ -32583,12 +32593,12 @@
         <v>0.999789883784</v>
       </c>
       <c r="N449" s="41">
-        <f>IF(L449&gt;0,(1-M449)/L449,1)</f>
+        <f>IF(L449&gt;x_series,(1-EXP(-L449))/L449,1-L449/2+L449^2/6-L449^3/24)</f>
         <v>0.999894938212</v>
       </c>
       <c r="O449" s="41">
-        <f>IF(L449&gt;0,(L449-1+M449)/L449^2,1/2)</f>
-        <v>0.499964978951</v>
+        <f>IF(L449&gt;x_series,(L449-1+EXP(-L449))/L449^2,1/2-L449/6+L449^2/24-L449^3/120)</f>
+        <v>0.499964978791</v>
       </c>
       <c r="P449" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B449/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32600,7 +32610,7 @@
       </c>
       <c r="R449" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q449+pool_b)*N449+P449*O449))</f>
-        <v>27.995077665173</v>
+        <v>27.995077665176</v>
       </c>
       <c r="S449" s="41">
         <f>IF(AND(R449&gt;=CO2_pH_hi_mt,R450&lt;CO2_pH_hi_mt),EXP(LN(A449)+(LN(A450)-LN(A449))*(R449-CO2_pH_hi_mt)/(R449-R450)),0)</f>
@@ -32625,12 +32635,12 @@
         <v>0.999955288754</v>
       </c>
       <c r="E450" s="41">
-        <f>IF(C450&gt;0,(1-D450)/C450,1)</f>
+        <f>IF(C450&gt;x_series,(1-EXP(-C450))/C450,1-C450/2+C450^2/6-C450^3/24)</f>
         <v>0.99997764421</v>
       </c>
       <c r="F450" s="41">
-        <f>IF(C450&gt;0,(C450-1+D450)/C450^2,1/2)</f>
-        <v>0.499992537834</v>
+        <f>IF(C450&gt;x_series,(C450-1+EXP(-C450))/C450^2,1/2-C450/6+C450^2/24-C450^3/120)</f>
+        <v>0.499992548042</v>
       </c>
       <c r="G450" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B450/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32642,7 +32652,7 @@
       </c>
       <c r="I450" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H450+pool_b)*E450+G450*F450))</f>
-        <v>28.036698309626</v>
+        <v>28.036698309637</v>
       </c>
       <c r="J450" s="41">
         <f>IF(AND(I450&gt;=CO2_pH_hi_mt,I451&lt;CO2_pH_hi_mt),EXP(LN(A450)+(LN(A451)-LN(A450))*(I450-CO2_pH_hi_mt)/(I450-I451)),0)</f>
@@ -32657,12 +32667,12 @@
         <v>0.99975854013</v>
       </c>
       <c r="N450" s="41">
-        <f>IF(L450&gt;0,(1-M450)/L450,1)</f>
-        <v>0.999879265205</v>
+        <f>IF(L450&gt;x_series,(1-EXP(-L450))/L450,1-L450/2+L450^2/6-L450^3/24)</f>
+        <v>0.999879265206</v>
       </c>
       <c r="O450" s="41">
-        <f>IF(L450&gt;0,(L450-1+M450)/L450^2,1/2)</f>
-        <v>0.499959754505</v>
+        <f>IF(L450&gt;x_series,(L450-1+EXP(-L450))/L450^2,1/2-L450/6+L450^2/24-L450^3/120)</f>
+        <v>0.499959754259</v>
       </c>
       <c r="P450" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B450/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32674,7 +32684,7 @@
       </c>
       <c r="R450" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q450+pool_b)*N450+P450*O450))</f>
-        <v>27.986054406636</v>
+        <v>27.986054406642</v>
       </c>
       <c r="S450" s="41">
         <f>IF(AND(R450&gt;=CO2_pH_hi_mt,R451&lt;CO2_pH_hi_mt),EXP(LN(A450)+(LN(A451)-LN(A450))*(R450-CO2_pH_hi_mt)/(R450-R451)),0)</f>
@@ -32699,12 +32709,12 @@
         <v>0.999948787472</v>
       </c>
       <c r="E451" s="41">
-        <f>IF(C451&gt;0,(1-D451)/C451,1)</f>
+        <f>IF(C451&gt;x_series,(1-EXP(-C451))/C451,1-C451/2+C451^2/6-C451^3/24)</f>
         <v>0.999974393518</v>
       </c>
       <c r="F451" s="41">
-        <f>IF(C451&gt;0,(C451-1+D451)/C451^2,1/2)</f>
-        <v>0.499991482431</v>
+        <f>IF(C451&gt;x_series,(C451-1+EXP(-C451))/C451^2,1/2-C451/6+C451^2/24-C451^3/120)</f>
+        <v>0.499991464469</v>
       </c>
       <c r="G451" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B451/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32716,7 +32726,7 @@
       </c>
       <c r="I451" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H451+pool_b)*E451+G451*F451))</f>
-        <v>28.033935375784</v>
+        <v>28.033935375798</v>
       </c>
       <c r="J451" s="41">
         <f>IF(AND(I451&gt;=CO2_pH_hi_mt,I452&lt;CO2_pH_hi_mt),EXP(LN(A451)+(LN(A452)-LN(A451))*(I451-CO2_pH_hi_mt)/(I451-I452)),0)</f>
@@ -32731,12 +32741,12 @@
         <v>0.999723434381</v>
       </c>
       <c r="N451" s="41">
-        <f>IF(L451&gt;0,(1-M451)/L451,1)</f>
+        <f>IF(L451&gt;x_series,(1-EXP(-L451))/L451,1-L451/2+L451^2/6-L451^3/24)</f>
         <v>0.999861710816</v>
       </c>
       <c r="O451" s="41">
-        <f>IF(L451&gt;0,(L451-1+M451)/L451^2,1/2)</f>
-        <v>0.499953903111</v>
+        <f>IF(L451&gt;x_series,(L451-1+EXP(-L451))/L451^2,1/2-L451/6+L451^2/24-L451^3/120)</f>
+        <v>0.499953902543</v>
       </c>
       <c r="P451" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B451/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32748,7 +32758,7 @@
       </c>
       <c r="R451" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q451+pool_b)*N451+P451*O451))</f>
-        <v>27.97595467362</v>
+        <v>27.975954673622</v>
       </c>
       <c r="S451" s="41">
         <f>IF(AND(R451&gt;=CO2_pH_hi_mt,R452&lt;CO2_pH_hi_mt),EXP(LN(A451)+(LN(A452)-LN(A451))*(R451-CO2_pH_hi_mt)/(R451-R452)),0)</f>
@@ -32773,12 +32783,12 @@
         <v>0.999941505667</v>
       </c>
       <c r="E452" s="41">
-        <f>IF(C452&gt;0,(1-D452)/C452,1)</f>
+        <f>IF(C452&gt;x_series,(1-EXP(-C452))/C452,1-C452/2+C452^2/6-C452^3/24)</f>
         <v>0.999970752549</v>
       </c>
       <c r="F452" s="41">
-        <f>IF(C452&gt;0,(C452-1+D452)/C452^2,1/2)</f>
-        <v>0.49999026357</v>
+        <f>IF(C452&gt;x_series,(C452-1+EXP(-C452))/C452^2,1/2-C452/6+C452^2/24-C452^3/120)</f>
+        <v>0.499990250802</v>
       </c>
       <c r="G452" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B452/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32790,7 +32800,7 @@
       </c>
       <c r="I452" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H452+pool_b)*E452+G452*F452))</f>
-        <v>28.030841150665</v>
+        <v>28.030841150676</v>
       </c>
       <c r="J452" s="41">
         <f>IF(AND(I452&gt;=CO2_pH_hi_mt,I453&lt;CO2_pH_hi_mt),EXP(LN(A452)+(LN(A453)-LN(A452))*(I452-CO2_pH_hi_mt)/(I452-I453)),0)</f>
@@ -32805,12 +32815,12 @@
         <v>0.999684115142</v>
       </c>
       <c r="N452" s="41">
-        <f>IF(L452&gt;0,(1-M452)/L452,1)</f>
+        <f>IF(L452&gt;x_series,(1-EXP(-L452))/L452,1-L452/2+L452^2/6-L452^3/24)</f>
         <v>0.999842049254</v>
       </c>
       <c r="O452" s="41">
-        <f>IF(L452&gt;0,(L452-1+M452)/L452^2,1/2)</f>
-        <v>0.499947348393</v>
+        <f>IF(L452&gt;x_series,(L452-1+EXP(-L452))/L452^2,1/2-L452/6+L452^2/24-L452^3/120)</f>
+        <v>0.499947348365</v>
       </c>
       <c r="P452" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B452/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32822,7 +32832,7 @@
       </c>
       <c r="R452" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q452+pool_b)*N452+P452*O452))</f>
-        <v>27.964650966364</v>
+        <v>27.964650966362</v>
       </c>
       <c r="S452" s="41">
         <f>IF(AND(R452&gt;=CO2_pH_hi_mt,R453&lt;CO2_pH_hi_mt),EXP(LN(A452)+(LN(A453)-LN(A452))*(R452-CO2_pH_hi_mt)/(R452-R453)),0)</f>
@@ -32847,12 +32857,12 @@
         <v>0.999933349639</v>
       </c>
       <c r="E453" s="41">
-        <f>IF(C453&gt;0,(1-D453)/C453,1)</f>
+        <f>IF(C453&gt;x_series,(1-EXP(-C453))/C453,1-C453/2+C453^2/6-C453^3/24)</f>
         <v>0.999966674449</v>
       </c>
       <c r="F453" s="41">
-        <f>IF(C453&gt;0,(C453-1+D453)/C453^2,1/2)</f>
-        <v>0.499988885123</v>
+        <f>IF(C453&gt;x_series,(C453-1+EXP(-C453))/C453^2,1/2-C453/6+C453^2/24-C453^3/120)</f>
+        <v>0.499988891421</v>
       </c>
       <c r="G453" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B453/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32864,7 +32874,7 @@
       </c>
       <c r="I453" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H453+pool_b)*E453+G453*F453))</f>
-        <v>28.027375969582</v>
+        <v>28.027375969577</v>
       </c>
       <c r="J453" s="41">
         <f>IF(AND(I453&gt;=CO2_pH_hi_mt,I454&lt;CO2_pH_hi_mt),EXP(LN(A453)+(LN(A454)-LN(A453))*(I453-CO2_pH_hi_mt)/(I453-I454)),0)</f>
@@ -32879,12 +32889,12 @@
         <v>0.999640076892</v>
       </c>
       <c r="N453" s="41">
-        <f>IF(L453&gt;0,(1-M453)/L453,1)</f>
+        <f>IF(L453&gt;x_series,(1-EXP(-L453))/L453,1-L453/2+L453^2/6-L453^3/24)</f>
         <v>0.999820027649</v>
       </c>
       <c r="O453" s="41">
-        <f>IF(L453&gt;0,(L453-1+M453)/L453^2,1/2)</f>
-        <v>0.499940007475</v>
+        <f>IF(L453&gt;x_series,(L453-1+EXP(-L453))/L453^2,1/2-L453/6+L453^2/24-L453^3/120)</f>
+        <v>0.499940007417</v>
       </c>
       <c r="P453" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B453/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32896,7 +32906,7 @@
       </c>
       <c r="R453" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q453+pool_b)*N453+P453*O453))</f>
-        <v>27.952000917724</v>
+        <v>27.952000917722</v>
       </c>
       <c r="S453" s="41">
         <f>IF(AND(R453&gt;=CO2_pH_hi_mt,R454&lt;CO2_pH_hi_mt),EXP(LN(A453)+(LN(A454)-LN(A453))*(R453-CO2_pH_hi_mt)/(R453-R454)),0)</f>
@@ -32921,12 +32931,12 @@
         <v>0.99992421444</v>
       </c>
       <c r="E454" s="41">
-        <f>IF(C454&gt;0,(1-D454)/C454,1)</f>
-        <v>0.999962106742</v>
+        <f>IF(C454&gt;x_series,(1-EXP(-C454))/C454,1-C454/2+C454^2/6-C454^3/24)</f>
+        <v>0.999962106741</v>
       </c>
       <c r="F454" s="41">
-        <f>IF(C454&gt;0,(C454-1+D454)/C454^2,1/2)</f>
-        <v>0.499987365675</v>
+        <f>IF(C454&gt;x_series,(C454-1+EXP(-C454))/C454^2,1/2-C454/6+C454^2/24-C454^3/120)</f>
+        <v>0.499987368834</v>
       </c>
       <c r="G454" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B454/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32938,7 +32948,7 @@
       </c>
       <c r="I454" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H454+pool_b)*E454+G454*F454))</f>
-        <v>28.023495433872</v>
+        <v>28.023495433848</v>
       </c>
       <c r="J454" s="41">
         <f>IF(AND(I454&gt;=CO2_pH_hi_mt,I455&lt;CO2_pH_hi_mt),EXP(LN(A454)+(LN(A455)-LN(A454))*(I454-CO2_pH_hi_mt)/(I454-I455)),0)</f>
@@ -32953,12 +32963,12 @@
         <v>0.999590753515</v>
       </c>
       <c r="N454" s="41">
-        <f>IF(L454&gt;0,(1-M454)/L454,1)</f>
+        <f>IF(L454&gt;x_series,(1-EXP(-L454))/L454,1-L454/2+L454^2/6-L454^3/24)</f>
         <v>0.999795362798</v>
       </c>
       <c r="O454" s="41">
-        <f>IF(L454&gt;0,(L454-1+M454)/L454^2,1/2)</f>
-        <v>0.499931785168</v>
+        <f>IF(L454&gt;x_series,(L454-1+EXP(-L454))/L454^2,1/2-L454/6+L454^2/24-L454^3/120)</f>
+        <v>0.499931785272</v>
       </c>
       <c r="P454" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B454/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -32970,7 +32980,7 @@
       </c>
       <c r="R454" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q454+pool_b)*N454+P454*O454))</f>
-        <v>27.937845618818</v>
+        <v>27.937845618816</v>
       </c>
       <c r="S454" s="41">
         <f>IF(AND(R454&gt;=CO2_pH_hi_mt,R455&lt;CO2_pH_hi_mt),EXP(LN(A454)+(LN(A455)-LN(A454))*(R454-CO2_pH_hi_mt)/(R454-R455)),0)</f>
@@ -32995,12 +33005,12 @@
         <v>0.999913982527</v>
       </c>
       <c r="E455" s="41">
-        <f>IF(C455&gt;0,(1-D455)/C455,1)</f>
+        <f>IF(C455&gt;x_series,(1-EXP(-C455))/C455,1-C455/2+C455^2/6-C455^3/24)</f>
         <v>0.999956990647</v>
       </c>
       <c r="F455" s="41">
-        <f>IF(C455&gt;0,(C455-1+D455)/C455^2,1/2)</f>
-        <v>0.499985658233</v>
+        <f>IF(C455&gt;x_series,(C455-1+EXP(-C455))/C455^2,1/2-C455/6+C455^2/24-C455^3/120)</f>
+        <v>0.499985663446</v>
       </c>
       <c r="G455" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B455/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33012,7 +33022,7 @@
       </c>
       <c r="I455" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H455+pool_b)*E455+G455*F455))</f>
-        <v>28.019149849715</v>
+        <v>28.019149849703</v>
       </c>
       <c r="J455" s="41">
         <f>IF(AND(I455&gt;=CO2_pH_hi_mt,I456&lt;CO2_pH_hi_mt),EXP(LN(A455)+(LN(A456)-LN(A455))*(I455-CO2_pH_hi_mt)/(I455-I456)),0)</f>
@@ -33027,12 +33037,12 @@
         <v>0.999535511038</v>
       </c>
       <c r="N455" s="41">
-        <f>IF(L455&gt;0,(1-M455)/L455,1)</f>
+        <f>IF(L455&gt;x_series,(1-EXP(-L455))/L455,1-L455/2+L455^2/6-L455^3/24)</f>
         <v>0.999767737536</v>
       </c>
       <c r="O455" s="41">
-        <f>IF(L455&gt;0,(L455-1+M455)/L455^2,1/2)</f>
-        <v>0.499922576184</v>
+        <f>IF(L455&gt;x_series,(L455-1+EXP(-L455))/L455^2,1/2-L455/6+L455^2/24-L455^3/120)</f>
+        <v>0.499922576181</v>
       </c>
       <c r="P455" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B455/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33044,7 +33054,7 @@
       </c>
       <c r="R455" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q455+pool_b)*N455+P455*O455))</f>
-        <v>27.92200777117</v>
+        <v>27.922007771172</v>
       </c>
       <c r="S455" s="41">
         <f>IF(AND(R455&gt;=CO2_pH_hi_mt,R456&lt;CO2_pH_hi_mt),EXP(LN(A455)+(LN(A456)-LN(A455))*(R455-CO2_pH_hi_mt)/(R455-R456)),0)</f>
@@ -33069,12 +33079,12 @@
         <v>0.999902522248</v>
       </c>
       <c r="E456" s="41">
-        <f>IF(C456&gt;0,(1-D456)/C456,1)</f>
-        <v>0.999951260333</v>
+        <f>IF(C456&gt;x_series,(1-EXP(-C456))/C456,1-C456/2+C456^2/6-C456^3/24)</f>
+        <v>0.999951260332</v>
       </c>
       <c r="F456" s="41">
-        <f>IF(C456&gt;0,(C456-1+D456)/C456^2,1/2)</f>
-        <v>0.499983751306</v>
+        <f>IF(C456&gt;x_series,(C456-1+EXP(-C456))/C456^2,1/2-C456/6+C456^2/24-C456^3/120)</f>
+        <v>0.499983753312</v>
       </c>
       <c r="G456" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B456/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33086,7 +33096,7 @@
       </c>
       <c r="I456" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H456+pool_b)*E456+G456*F456))</f>
-        <v>28.0142836015</v>
+        <v>28.014283601482</v>
       </c>
       <c r="J456" s="41">
         <f>IF(AND(I456&gt;=CO2_pH_hi_mt,I457&lt;CO2_pH_hi_mt),EXP(LN(A456)+(LN(A457)-LN(A456))*(I456-CO2_pH_hi_mt)/(I456-I457)),0)</f>
@@ -33101,12 +33111,12 @@
         <v>0.999473639525</v>
       </c>
       <c r="N456" s="41">
-        <f>IF(L456&gt;0,(1-M456)/L456,1)</f>
+        <f>IF(L456&gt;x_series,(1-EXP(-L456))/L456,1-L456/2+L456^2/6-L456^3/24)</f>
         <v>0.999736796669</v>
       </c>
       <c r="O456" s="41">
-        <f>IF(L456&gt;0,(L456-1+M456)/L456^2,1/2)</f>
-        <v>0.499912261586</v>
+        <f>IF(L456&gt;x_series,(L456-1+EXP(-L456))/L456^2,1/2-L456/6+L456^2/24-L456^3/120)</f>
+        <v>0.499912261707</v>
       </c>
       <c r="P456" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B456/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33118,7 +33128,7 @@
       </c>
       <c r="R456" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q456+pool_b)*N456+P456*O456))</f>
-        <v>27.904289651388</v>
+        <v>27.904289651386</v>
       </c>
       <c r="S456" s="41">
         <f>IF(AND(R456&gt;=CO2_pH_hi_mt,R457&lt;CO2_pH_hi_mt),EXP(LN(A456)+(LN(A457)-LN(A456))*(R456-CO2_pH_hi_mt)/(R456-R457)),0)</f>
@@ -33143,12 +33153,12 @@
         <v>0.999889686152</v>
       </c>
       <c r="E457" s="41">
-        <f>IF(C457&gt;0,(1-D457)/C457,1)</f>
+        <f>IF(C457&gt;x_series,(1-EXP(-C457))/C457,1-C457/2+C457^2/6-C457^3/24)</f>
         <v>0.999944842062</v>
       </c>
       <c r="F457" s="41">
-        <f>IF(C457&gt;0,(C457-1+D457)/C457^2,1/2)</f>
-        <v>0.499981614053</v>
+        <f>IF(C457&gt;x_series,(C457-1+EXP(-C457))/C457^2,1/2-C457/6+C457^2/24-C457^3/120)</f>
+        <v>0.499981613852</v>
       </c>
       <c r="G457" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B457/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33160,7 +33170,7 @@
       </c>
       <c r="I457" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H457+pool_b)*E457+G457*F457))</f>
-        <v>28.008834451968</v>
+        <v>28.008834451959</v>
       </c>
       <c r="J457" s="41">
         <f>IF(AND(I457&gt;=CO2_pH_hi_mt,I458&lt;CO2_pH_hi_mt),EXP(LN(A457)+(LN(A458)-LN(A457))*(I457-CO2_pH_hi_mt)/(I457-I458)),0)</f>
@@ -33175,12 +33185,12 @@
         <v>0.999404343985</v>
       </c>
       <c r="N457" s="41">
-        <f>IF(L457&gt;0,(1-M457)/L457,1)</f>
+        <f>IF(L457&gt;x_series,(1-EXP(-L457))/L457,1-L457/2+L457^2/6-L457^3/24)</f>
         <v>0.999702142417</v>
       </c>
       <c r="O457" s="41">
-        <f>IF(L457&gt;0,(L457-1+M457)/L457^2,1/2)</f>
-        <v>0.499900709165</v>
+        <f>IF(L457&gt;x_series,(L457-1+EXP(-L457))/L457^2,1/2-L457/6+L457^2/24-L457^3/120)</f>
+        <v>0.499900709209</v>
       </c>
       <c r="P457" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B457/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33192,7 +33202,7 @@
       </c>
       <c r="R457" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q457+pool_b)*N457+P457*O457))</f>
-        <v>27.884470874124</v>
+        <v>27.884470874123</v>
       </c>
       <c r="S457" s="41">
         <f>IF(AND(R457&gt;=CO2_pH_hi_mt,R458&lt;CO2_pH_hi_mt),EXP(LN(A457)+(LN(A458)-LN(A457))*(R457-CO2_pH_hi_mt)/(R457-R458)),0)</f>
@@ -33217,12 +33227,12 @@
         <v>0.999875309092</v>
       </c>
       <c r="E458" s="41">
-        <f>IF(C458&gt;0,(1-D458)/C458,1)</f>
-        <v>0.999937653251</v>
+        <f>IF(C458&gt;x_series,(1-EXP(-C458))/C458,1-C458/2+C458^2/6-C458^3/24)</f>
+        <v>0.99993765325</v>
       </c>
       <c r="F458" s="41">
-        <f>IF(C458&gt;0,(C458-1+D458)/C458^2,1/2)</f>
-        <v>0.499979210658</v>
+        <f>IF(C458&gt;x_series,(C458-1+EXP(-C458))/C458^2,1/2-C458/6+C458^2/24-C458^3/120)</f>
+        <v>0.499979217534</v>
       </c>
       <c r="G458" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B458/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33234,7 +33244,7 @@
       </c>
       <c r="I458" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H458+pool_b)*E458+G458*F458))</f>
-        <v>28.002732761522</v>
+        <v>28.002732761498</v>
       </c>
       <c r="J458" s="41">
         <f>IF(AND(I458&gt;=CO2_pH_hi_mt,I459&lt;CO2_pH_hi_mt),EXP(LN(A458)+(LN(A459)-LN(A458))*(I458-CO2_pH_hi_mt)/(I458-I459)),0)</f>
@@ -33249,12 +33259,12 @@
         <v>0.999326734213</v>
       </c>
       <c r="N458" s="41">
-        <f>IF(L458&gt;0,(1-M458)/L458,1)</f>
+        <f>IF(L458&gt;x_series,(1-EXP(-L458))/L458,1-L458/2+L458^2/6-L458^3/24)</f>
         <v>0.99966332932</v>
       </c>
       <c r="O458" s="41">
-        <f>IF(L458&gt;0,(L458-1+M458)/L458^2,1/2)</f>
-        <v>0.49988777017</v>
+        <f>IF(L458&gt;x_series,(L458-1+EXP(-L458))/L458^2,1/2-L458/6+L458^2/24-L458^3/120)</f>
+        <v>0.499887770142</v>
       </c>
       <c r="P458" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B458/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33266,7 +33276,7 @@
       </c>
       <c r="R458" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q458+pool_b)*N458+P458*O458))</f>
-        <v>27.862305939684</v>
+        <v>27.862305939683</v>
       </c>
       <c r="S458" s="41">
         <f>IF(AND(R458&gt;=CO2_pH_hi_mt,R459&lt;CO2_pH_hi_mt),EXP(LN(A458)+(LN(A459)-LN(A458))*(R458-CO2_pH_hi_mt)/(R458-R459)),0)</f>
@@ -33291,12 +33301,12 @@
         <v>0.999859206103</v>
       </c>
       <c r="E459" s="41">
-        <f>IF(C459&gt;0,(1-D459)/C459,1)</f>
+        <f>IF(C459&gt;x_series,(1-EXP(-C459))/C459,1-C459/2+C459^2/6-C459^3/24)</f>
         <v>0.999929601399</v>
       </c>
       <c r="F459" s="41">
-        <f>IF(C459&gt;0,(C459-1+D459)/C459^2,1/2)</f>
-        <v>0.499976536247</v>
+        <f>IF(C459&gt;x_series,(C459-1+EXP(-C459))/C459^2,1/2-C459/6+C459^2/24-C459^3/120)</f>
+        <v>0.499976533524</v>
       </c>
       <c r="G459" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B459/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33308,7 +33318,7 @@
       </c>
       <c r="I459" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H459+pool_b)*E459+G459*F459))</f>
-        <v>27.995900617042</v>
+        <v>27.995900617048</v>
       </c>
       <c r="J459" s="41">
         <f>IF(AND(I459&gt;=CO2_pH_hi_mt,I460&lt;CO2_pH_hi_mt),EXP(LN(A459)+(LN(A460)-LN(A459))*(I459-CO2_pH_hi_mt)/(I459-I460)),0)</f>
@@ -33323,12 +33333,12 @@
         <v>0.999239813417</v>
       </c>
       <c r="N459" s="41">
-        <f>IF(L459&gt;0,(1-M459)/L459,1)</f>
+        <f>IF(L459&gt;x_series,(1-EXP(-L459))/L459,1-L459/2+L459^2/6-L459^3/24)</f>
         <v>0.999619858533</v>
       </c>
       <c r="O459" s="41">
-        <f>IF(L459&gt;0,(L459-1+M459)/L459^2,1/2)</f>
-        <v>0.499873278291</v>
+        <f>IF(L459&gt;x_series,(L459-1+EXP(-L459))/L459^2,1/2-L459/6+L459^2/24-L459^3/120)</f>
+        <v>0.499873278148</v>
       </c>
       <c r="P459" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B459/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33340,7 +33350,7 @@
       </c>
       <c r="R459" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*Q459+pool_b)*N459+P459*O459))</f>
-        <v>27.837521553104</v>
+        <v>27.837521553105</v>
       </c>
       <c r="S459" s="41">
         <f>IF(AND(R459&gt;=CO2_pH_hi_mt,R460&lt;CO2_pH_hi_mt),EXP(LN(A459)+(LN(A460)-LN(A459))*(R459-CO2_pH_hi_mt)/(R459-R460)),0)</f>
@@ -33365,12 +33375,12 @@
         <v>0.999841170023</v>
       </c>
       <c r="E460" s="41">
-        <f>IF(C460&gt;0,(1-D460)/C460,1)</f>
+        <f>IF(C460&gt;x_series,(1-EXP(-C460))/C460,1-C460/2+C460^2/6-C460^3/24)</f>
         <v>0.999920582909</v>
       </c>
       <c r="F460" s="41">
-        <f>IF(C460&gt;0,(C460-1+D460)/C460^2,1/2)</f>
-        <v>0.499973527706</v>
+        <f>IF(C460&gt;x_series,(C460-1+EXP(-C460))/C460^2,1/2-C460/6+C460^2/24-C460^3/120)</f>
+        <v>0.499973527286</v>
       </c>
       <c r="G460" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B460/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33382,7 +33392,7 @@
       </c>
       <c r="I460" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H460+pool_b)*E460+G460*F460))</f>
-        <v>27.988250861036</v>
+        <v>27.988250861037</v>
       </c>
       <c r="J460" s="41">
         <f>IF(AND(I460&gt;=CO2_pH_hi_mt,I461&lt;CO2_pH_hi_mt),EXP(LN(A460)+(LN(A461)-LN(A460))*(I460-CO2_pH_hi_mt)/(I460-I461)),0)</f>
@@ -33397,12 +33407,12 @@
         <v>0.999142465492</v>
       </c>
       <c r="N460" s="41">
-        <f>IF(L460&gt;0,(1-M460)/L460,1)</f>
+        <f>IF(L460&gt;x_series,(1-EXP(-L460))/L460,1-L460/2+L460^2/6-L460^3/24)</f>
         <v>0.999571171439</v>
       </c>
       <c r="O460" s="41">
-        <f>IF(L460&gt;0,(L460-1+M460)/L460^2,1/2)</f>
-        <v>0.499857046929</v>
+        <f>IF(L460&gt;x_series,(L460-1+EXP(-L460))/L460^2,1/2-L460/6+L460^2/24-L460^3/120)</f>
+        <v>0.499857046928</v>
       </c>
       <c r="P460" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B460/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33439,12 +33449,12 @@
         <v>0.999820968837</v>
       </c>
       <c r="E461" s="41">
-        <f>IF(C461&gt;0,(1-D461)/C461,1)</f>
+        <f>IF(C461&gt;x_series,(1-EXP(-C461))/C461,1-C461/2+C461^2/6-C461^3/24)</f>
         <v>0.999910481747</v>
       </c>
       <c r="F461" s="41">
-        <f>IF(C461&gt;0,(C461-1+D461)/C461^2,1/2)</f>
-        <v>0.499970159888</v>
+        <f>IF(C461&gt;x_series,(C461-1+EXP(-C461))/C461^2,1/2-C461/6+C461^2/24-C461^3/120)</f>
+        <v>0.499970160137</v>
       </c>
       <c r="G461" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B461/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33456,7 +33466,7 @@
       </c>
       <c r="I461" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H461+pool_b)*E461+G461*F461))</f>
-        <v>27.9796860093</v>
+        <v>27.979686009305</v>
       </c>
       <c r="J461" s="41">
         <f>IF(AND(I461&gt;=CO2_pH_hi_mt,I462&lt;CO2_pH_hi_mt),EXP(LN(A461)+(LN(A462)-LN(A461))*(I461-CO2_pH_hi_mt)/(I461-I462)),0)</f>
@@ -33471,12 +33481,12 @@
         <v>0.999033440795</v>
       </c>
       <c r="N461" s="41">
-        <f>IF(L461&gt;0,(1-M461)/L461,1)</f>
+        <f>IF(L461&gt;x_series,(1-EXP(-L461))/L461,1-L461/2+L461^2/6-L461^3/24)</f>
         <v>0.999516642507</v>
       </c>
       <c r="O461" s="41">
-        <f>IF(L461&gt;0,(L461-1+M461)/L461^2,1/2)</f>
-        <v>0.499838867847</v>
+        <f>IF(L461&gt;x_series,(L461-1+EXP(-L461))/L461^2,1/2-L461/6+L461^2/24-L461^3/120)</f>
+        <v>0.499838867853</v>
       </c>
       <c r="P461" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_l)*(B461/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33513,12 +33523,12 @@
         <v>0.999798342689</v>
       </c>
       <c r="E462" s="41">
-        <f>IF(C462&gt;0,(1-D462)/C462,1)</f>
+        <f>IF(C462&gt;x_series,(1-EXP(-C462))/C462,1-C462/2+C462^2/6-C462^3/24)</f>
         <v>0.999899167955</v>
       </c>
       <c r="F462" s="41">
-        <f>IF(C462&gt;0,(C462-1+D462)/C462^2,1/2)</f>
-        <v>0.4999663895</v>
+        <f>IF(C462&gt;x_series,(C462-1+EXP(-C462))/C462^2,1/2-C462/6+C462^2/24-C462^3/120)</f>
+        <v>0.499966388754</v>
       </c>
       <c r="G462" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B462/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33530,7 +33540,7 @@
       </c>
       <c r="I462" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H462+pool_b)*E462+G462*F462))</f>
-        <v>27.970097046132</v>
+        <v>27.970097046135</v>
       </c>
       <c r="J462" s="41">
         <f>IF(AND(I462&gt;=CO2_pH_hi_mt,I463&lt;CO2_pH_hi_mt),EXP(LN(A462)+(LN(A463)-LN(A462))*(I462-CO2_pH_hi_mt)/(I462-I463)),0)</f>
@@ -33545,11 +33555,11 @@
         <v>0.998911340224</v>
       </c>
       <c r="N462" s="41">
-        <f>IF(L462&gt;0,(1-M462)/L462,1)</f>
+        <f>IF(L462&gt;x_series,(1-EXP(-L462))/L462,1-L462/2+L462^2/6-L462^3/24)</f>
         <v>0.999455571293</v>
       </c>
       <c r="O462" s="41">
-        <f>IF(L462&gt;0,(L462-1+M462)/L462^2,1/2)</f>
+        <f>IF(L462&gt;x_series,(L462-1+EXP(-L462))/L462^2,1/2-L462/6+L462^2/24-L462^3/120)</f>
         <v>0.499818507329</v>
       </c>
       <c r="P462" s="41">
@@ -33587,12 +33597,12 @@
         <v>0.999773000552</v>
       </c>
       <c r="E463" s="41">
-        <f>IF(C463&gt;0,(1-D463)/C463,1)</f>
+        <f>IF(C463&gt;x_series,(1-EXP(-C463))/C463,1-C463/2+C463^2/6-C463^3/24)</f>
         <v>0.999886495981</v>
       </c>
       <c r="F463" s="41">
-        <f>IF(C463&gt;0,(C463-1+D463)/C463^2,1/2)</f>
-        <v>0.499962164475</v>
+        <f>IF(C463&gt;x_series,(C463-1+EXP(-C463))/C463^2,1/2-C463/6+C463^2/24-C463^3/120)</f>
+        <v>0.499962164611</v>
       </c>
       <c r="G463" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B463/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33604,7 +33614,7 @@
       </c>
       <c r="I463" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H463+pool_b)*E463+G463*F463))</f>
-        <v>27.959362083412</v>
+        <v>27.959362083411</v>
       </c>
       <c r="J463" s="41">
         <f>IF(AND(I463&gt;=CO2_pH_hi_mt,I464&lt;CO2_pH_hi_mt),EXP(LN(A463)+(LN(A464)-LN(A463))*(I463-CO2_pH_hi_mt)/(I463-I464)),0)</f>
@@ -33619,11 +33629,11 @@
         <v>0.998774597424</v>
       </c>
       <c r="N463" s="41">
-        <f>IF(L463&gt;0,(1-M463)/L463,1)</f>
+        <f>IF(L463&gt;x_series,(1-EXP(-L463))/L463,1-L463/2+L463^2/6-L463^3/24)</f>
         <v>0.999387173501</v>
       </c>
       <c r="O463" s="41">
-        <f>IF(L463&gt;0,(L463-1+M463)/L463^2,1/2)</f>
+        <f>IF(L463&gt;x_series,(L463-1+EXP(-L463))/L463^2,1/2-L463/6+L463^2/24-L463^3/120)</f>
         <v>0.499795703592</v>
       </c>
       <c r="P463" s="41">
@@ -33661,12 +33671,12 @@
         <v>0.999744616485</v>
       </c>
       <c r="E464" s="41">
-        <f>IF(C464&gt;0,(1-D464)/C464,1)</f>
+        <f>IF(C464&gt;x_series,(1-EXP(-C464))/C464,1-C464/2+C464^2/6-C464^3/24)</f>
         <v>0.999872302807</v>
       </c>
       <c r="F464" s="41">
-        <f>IF(C464&gt;0,(C464-1+D464)/C464^2,1/2)</f>
-        <v>0.499957433352</v>
+        <f>IF(C464&gt;x_series,(C464-1+EXP(-C464))/C464^2,1/2-C464/6+C464^2/24-C464^3/120)</f>
+        <v>0.499957433363</v>
       </c>
       <c r="G464" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B464/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33678,7 +33688,7 @@
       </c>
       <c r="I464" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H464+pool_b)*E464+G464*F464))</f>
-        <v>27.947344869786</v>
+        <v>27.947344869785</v>
       </c>
       <c r="J464" s="41">
         <f>IF(AND(I464&gt;=CO2_pH_hi_mt,I465&lt;CO2_pH_hi_mt),EXP(LN(A464)+(LN(A465)-LN(A464))*(I464-CO2_pH_hi_mt)/(I464-I465)),0)</f>
@@ -33693,11 +33703,11 @@
         <v>0.998621458889</v>
       </c>
       <c r="N464" s="41">
-        <f>IF(L464&gt;0,(1-M464)/L464,1)</f>
+        <f>IF(L464&gt;x_series,(1-EXP(-L464))/L464,1-L464/2+L464^2/6-L464^3/24)</f>
         <v>0.999310570971</v>
       </c>
       <c r="O464" s="41">
-        <f>IF(L464&gt;0,(L464-1+M464)/L464^2,1/2)</f>
+        <f>IF(L464&gt;x_series,(L464-1+EXP(-L464))/L464^2,1/2-L464/6+L464^2/24-L464^3/120)</f>
         <v>0.499770163909</v>
       </c>
       <c r="P464" s="41">
@@ -33735,12 +33745,12 @@
         <v>0.999712825456</v>
       </c>
       <c r="E465" s="41">
-        <f>IF(C465&gt;0,(1-D465)/C465,1)</f>
-        <v>0.999856405854</v>
+        <f>IF(C465&gt;x_series,(1-EXP(-C465))/C465,1-C465/2+C465^2/6-C465^3/24)</f>
+        <v>0.999856405855</v>
       </c>
       <c r="F465" s="41">
-        <f>IF(C465&gt;0,(C465-1+D465)/C465^2,1/2)</f>
-        <v>0.499952134143</v>
+        <f>IF(C465&gt;x_series,(C465-1+EXP(-C465))/C465^2,1/2-C465/6+C465^2/24-C465^3/120)</f>
+        <v>0.499952134139</v>
       </c>
       <c r="G465" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B465/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33752,7 +33762,7 @@
       </c>
       <c r="I465" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H465+pool_b)*E465+G465*F465))</f>
-        <v>27.933893134584</v>
+        <v>27.933893134587</v>
       </c>
       <c r="J465" s="41">
         <f>IF(AND(I465&gt;=CO2_pH_hi_mt,I466&lt;CO2_pH_hi_mt),EXP(LN(A465)+(LN(A466)-LN(A465))*(I465-CO2_pH_hi_mt)/(I465-I466)),0)</f>
@@ -33767,11 +33777,11 @@
         <v>0.998449961727</v>
       </c>
       <c r="N465" s="41">
-        <f>IF(L465&gt;0,(1-M465)/L465,1)</f>
+        <f>IF(L465&gt;x_series,(1-EXP(-L465))/L465,1-L465/2+L465^2/6-L465^3/24)</f>
         <v>0.99922478049</v>
       </c>
       <c r="O465" s="41">
-        <f>IF(L465&gt;0,(L465-1+M465)/L465^2,1/2)</f>
+        <f>IF(L465&gt;x_series,(L465-1+EXP(-L465))/L465^2,1/2-L465/6+L465^2/24-L465^3/120)</f>
         <v>0.499741560087</v>
       </c>
       <c r="P465" s="41">
@@ -33809,12 +33819,12 @@
         <v>0.999677218652</v>
       </c>
       <c r="E466" s="41">
-        <f>IF(C466&gt;0,(1-D466)/C466,1)</f>
+        <f>IF(C466&gt;x_series,(1-EXP(-C466))/C466,1-C466/2+C466^2/6-C466^3/24)</f>
         <v>0.999838600642</v>
       </c>
       <c r="F466" s="41">
-        <f>IF(C466&gt;0,(C466-1+D466)/C466^2,1/2)</f>
-        <v>0.499946198387</v>
+        <f>IF(C466&gt;x_series,(C466-1+EXP(-C466))/C466^2,1/2-C466/6+C466^2/24-C466^3/120)</f>
+        <v>0.499946198767</v>
       </c>
       <c r="G466" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B466/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33826,7 +33836,7 @@
       </c>
       <c r="I466" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H466+pool_b)*E466+G466*F466))</f>
-        <v>27.918836750082</v>
+        <v>27.918836750081</v>
       </c>
       <c r="J466" s="41">
         <f>IF(AND(I466&gt;=CO2_pH_hi_mt,I467&lt;CO2_pH_hi_mt),EXP(LN(A466)+(LN(A467)-LN(A466))*(I466-CO2_pH_hi_mt)/(I466-I467)),0)</f>
@@ -33841,11 +33851,11 @@
         <v>0.998257908807</v>
       </c>
       <c r="N466" s="41">
-        <f>IF(L466&gt;0,(1-M466)/L466,1)</f>
+        <f>IF(L466&gt;x_series,(1-EXP(-L466))/L466,1-L466/2+L466^2/6-L466^3/24)</f>
         <v>0.999128701276</v>
       </c>
       <c r="O466" s="41">
-        <f>IF(L466&gt;0,(L466-1+M466)/L466^2,1/2)</f>
+        <f>IF(L466&gt;x_series,(L466-1+EXP(-L466))/L466^2,1/2-L466/6+L466^2/24-L466^3/120)</f>
         <v>0.499709524892</v>
       </c>
       <c r="P466" s="41">
@@ -33883,12 +33893,12 @@
         <v>0.99963733824</v>
       </c>
       <c r="E467" s="41">
-        <f>IF(C467&gt;0,(1-D467)/C467,1)</f>
+        <f>IF(C467&gt;x_series,(1-EXP(-C467))/C467,1-C467/2+C467^2/6-C467^3/24)</f>
         <v>0.999818658158</v>
       </c>
       <c r="F467" s="41">
-        <f>IF(C467&gt;0,(C467-1+D467)/C467^2,1/2)</f>
-        <v>0.499939551164</v>
+        <f>IF(C467&gt;x_series,(C467-1+EXP(-C467))/C467^2,1/2-C467/6+C467^2/24-C467^3/120)</f>
+        <v>0.499939550892</v>
       </c>
       <c r="G467" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B467/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33900,7 +33910,7 @@
       </c>
       <c r="I467" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H467+pool_b)*E467+G467*F467))</f>
-        <v>27.901985694515</v>
+        <v>27.901985694517</v>
       </c>
       <c r="J467" s="41">
         <f>IF(AND(I467&gt;=CO2_pH_hi_mt,I468&lt;CO2_pH_hi_mt),EXP(LN(A467)+(LN(A468)-LN(A467))*(I467-CO2_pH_hi_mt)/(I467-I468)),0)</f>
@@ -33915,11 +33925,11 @@
         <v>0.998042841004</v>
       </c>
       <c r="N467" s="41">
-        <f>IF(L467&gt;0,(1-M467)/L467,1)</f>
+        <f>IF(L467&gt;x_series,(1-EXP(-L467))/L467,1-L467/2+L467^2/6-L467^3/24)</f>
         <v>0.999021100983</v>
       </c>
       <c r="O467" s="41">
-        <f>IF(L467&gt;0,(L467-1+M467)/L467^2,1/2)</f>
+        <f>IF(L467&gt;x_series,(L467-1+EXP(-L467))/L467^2,1/2-L467/6+L467^2/24-L467^3/120)</f>
         <v>0.499673647064</v>
       </c>
       <c r="P467" s="41">
@@ -33957,12 +33967,12 @@
         <v>0.999592671494</v>
       </c>
       <c r="E468" s="41">
-        <f>IF(C468&gt;0,(1-D468)/C468,1)</f>
+        <f>IF(C468&gt;x_series,(1-EXP(-C468))/C468,1-C468/2+C468^2/6-C468^3/24)</f>
         <v>0.999796321918</v>
       </c>
       <c r="F468" s="41">
-        <f>IF(C468&gt;0,(C468-1+D468)/C468^2,1/2)</f>
-        <v>0.499932105242</v>
+        <f>IF(C468&gt;x_series,(C468-1+EXP(-C468))/C468^2,1/2-C468/6+C468^2/24-C468^3/120)</f>
+        <v>0.499932105001</v>
       </c>
       <c r="G468" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B468/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -33974,7 +33984,7 @@
       </c>
       <c r="I468" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H468+pool_b)*E468+G468*F468))</f>
-        <v>27.883127797389</v>
+        <v>27.883127797394</v>
       </c>
       <c r="J468" s="41">
         <f>IF(AND(I468&gt;=CO2_pH_hi_mt,I469&lt;CO2_pH_hi_mt),EXP(LN(A468)+(LN(A469)-LN(A468))*(I468-CO2_pH_hi_mt)/(I468-I469)),0)</f>
@@ -33989,11 +33999,11 @@
         <v>0.997802006201</v>
       </c>
       <c r="N468" s="41">
-        <f>IF(L468&gt;0,(1-M468)/L468,1)</f>
+        <f>IF(L468&gt;x_series,(1-EXP(-L468))/L468,1-L468/2+L468^2/6-L468^3/24)</f>
         <v>0.998900600059</v>
       </c>
       <c r="O468" s="41">
-        <f>IF(L468&gt;0,(L468-1+M468)/L468^2,1/2)</f>
+        <f>IF(L468&gt;x_series,(L468-1+EXP(-L468))/L468^2,1/2-L468/6+L468^2/24-L468^3/120)</f>
         <v>0.499633466174</v>
       </c>
       <c r="P468" s="41">
@@ -34031,12 +34041,12 @@
         <v>0.999542644226</v>
       </c>
       <c r="E469" s="41">
-        <f>IF(C469&gt;0,(1-D469)/C469,1)</f>
+        <f>IF(C469&gt;x_series,(1-EXP(-C469))/C469,1-C469/2+C469^2/6-C469^3/24)</f>
         <v>0.999771304678</v>
       </c>
       <c r="F469" s="41">
-        <f>IF(C469&gt;0,(C469-1+D469)/C469^2,1/2)</f>
-        <v>0.499923765043</v>
+        <f>IF(C469&gt;x_series,(C469-1+EXP(-C469))/C469^2,1/2-C469/6+C469^2/24-C469^3/120)</f>
+        <v>0.49992376532</v>
       </c>
       <c r="G469" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B469/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34048,7 +34058,7 @@
       </c>
       <c r="I469" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H469+pool_b)*E469+G469*F469))</f>
-        <v>27.862026247405</v>
+        <v>27.862026247401</v>
       </c>
       <c r="J469" s="41">
         <f>IF(AND(I469&gt;=CO2_pH_hi_mt,I470&lt;CO2_pH_hi_mt),EXP(LN(A469)+(LN(A470)-LN(A469))*(I469-CO2_pH_hi_mt)/(I469-I470)),0)</f>
@@ -34063,11 +34073,11 @@
         <v>0.997532324681</v>
       </c>
       <c r="N469" s="41">
-        <f>IF(L469&gt;0,(1-M469)/L469,1)</f>
+        <f>IF(L469&gt;x_series,(1-EXP(-L469))/L469,1-L469/2+L469^2/6-L469^3/24)</f>
         <v>0.998765654261</v>
       </c>
       <c r="O469" s="41">
-        <f>IF(L469&gt;0,(L469-1+M469)/L469^2,1/2)</f>
+        <f>IF(L469&gt;x_series,(L469-1+EXP(-L469))/L469^2,1/2-L469/6+L469^2/24-L469^3/120)</f>
         <v>0.499588466728</v>
       </c>
       <c r="P469" s="41">
@@ -34105,12 +34115,12 @@
         <v>0.99948661343</v>
       </c>
       <c r="E470" s="41">
-        <f>IF(C470&gt;0,(1-D470)/C470,1)</f>
+        <f>IF(C470&gt;x_series,(1-EXP(-C470))/C470,1-C470/2+C470^2/6-C470^3/24)</f>
         <v>0.999743284746</v>
       </c>
       <c r="F470" s="41">
-        <f>IF(C470&gt;0,(C470-1+D470)/C470^2,1/2)</f>
-        <v>0.499914424862</v>
+        <f>IF(C470&gt;x_series,(C470-1+EXP(-C470))/C470^2,1/2-C470/6+C470^2/24-C470^3/120)</f>
+        <v>0.499914424587</v>
       </c>
       <c r="G470" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B470/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34122,7 +34132,7 @@
       </c>
       <c r="I470" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H470+pool_b)*E470+G470*F470))</f>
-        <v>27.838416842784</v>
+        <v>27.838416842789</v>
       </c>
       <c r="J470" s="41">
         <f>IF(AND(I470&gt;=CO2_pH_hi_mt,I471&lt;CO2_pH_hi_mt),EXP(LN(A470)+(LN(A471)-LN(A470))*(I470-CO2_pH_hi_mt)/(I470-I471)),0)</f>
@@ -34137,11 +34147,11 @@
         <v>0.997230350516</v>
       </c>
       <c r="N470" s="41">
-        <f>IF(L470&gt;0,(1-M470)/L470,1)</f>
+        <f>IF(L470&gt;x_series,(1-EXP(-L470))/L470,1-L470/2+L470^2/6-L470^3/24)</f>
         <v>0.998614535125</v>
       </c>
       <c r="O470" s="41">
-        <f>IF(L470&gt;0,(L470-1+M470)/L470^2,1/2)</f>
+        <f>IF(L470&gt;x_series,(L470-1+EXP(-L470))/L470^2,1/2-L470/6+L470^2/24-L470^3/120)</f>
         <v>0.499538071645</v>
       </c>
       <c r="P470" s="41">
@@ -34179,12 +34189,12 @@
         <v>0.999423859053</v>
       </c>
       <c r="E471" s="41">
-        <f>IF(C471&gt;0,(1-D471)/C471,1)</f>
+        <f>IF(C471&gt;x_series,(1-EXP(-C471))/C471,1-C471/2+C471^2/6-C471^3/24)</f>
         <v>0.999711901857</v>
       </c>
       <c r="F471" s="41">
-        <f>IF(C471&gt;0,(C471-1+D471)/C471^2,1/2)</f>
-        <v>0.499903962847</v>
+        <f>IF(C471&gt;x_series,(C471-1+EXP(-C471))/C471^2,1/2-C471/6+C471^2/24-C471^3/120)</f>
+        <v>0.499903962674</v>
       </c>
       <c r="G471" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B471/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34196,7 +34206,7 @@
       </c>
       <c r="I471" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H471+pool_b)*E471+G471*F471))</f>
-        <v>27.812004963448</v>
+        <v>27.812004963451</v>
       </c>
       <c r="J471" s="41">
         <f>IF(AND(I471&gt;=CO2_pH_hi_mt,I472&lt;CO2_pH_hi_mt),EXP(LN(A471)+(LN(A472)-LN(A471))*(I471-CO2_pH_hi_mt)/(I471-I472)),0)</f>
@@ -34211,11 +34221,11 @@
         <v>0.996892228501</v>
       </c>
       <c r="N471" s="41">
-        <f>IF(L471&gt;0,(1-M471)/L471,1)</f>
+        <f>IF(L471&gt;x_series,(1-EXP(-L471))/L471,1-L471/2+L471^2/6-L471^3/24)</f>
         <v>0.998445308144</v>
       </c>
       <c r="O471" s="41">
-        <f>IF(L471&gt;0,(L471-1+M471)/L471^2,1/2)</f>
+        <f>IF(L471&gt;x_series,(L471-1+EXP(-L471))/L471^2,1/2-L471/6+L471^2/24-L471^3/120)</f>
         <v>0.499481634989</v>
       </c>
       <c r="P471" s="41">
@@ -34253,12 +34263,12 @@
         <v>0.999353574779</v>
       </c>
       <c r="E472" s="41">
-        <f>IF(C472&gt;0,(1-D472)/C472,1)</f>
+        <f>IF(C472&gt;x_series,(1-EXP(-C472))/C472,1-C472/2+C472^2/6-C472^3/24)</f>
         <v>0.999676752556</v>
       </c>
       <c r="F472" s="41">
-        <f>IF(C472&gt;0,(C472-1+D472)/C472^2,1/2)</f>
-        <v>0.499892245265</v>
+        <f>IF(C472&gt;x_series,(C472-1+EXP(-C472))/C472^2,1/2-C472/6+C472^2/24-C472^3/120)</f>
+        <v>0.499892245046</v>
       </c>
       <c r="G472" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B472/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34270,7 +34280,7 @@
       </c>
       <c r="I472" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H472+pool_b)*E472+G472*F472))</f>
-        <v>27.782462244001</v>
+        <v>27.782462244005</v>
       </c>
       <c r="J472" s="41">
         <f>IF(AND(I472&gt;=CO2_pH_hi_mt,I473&lt;CO2_pH_hi_mt),EXP(LN(A472)+(LN(A473)-LN(A472))*(I472-CO2_pH_hi_mt)/(I472-I473)),0)</f>
@@ -34285,11 +34295,11 @@
         <v>0.996513646142</v>
       </c>
       <c r="N472" s="41">
-        <f>IF(L472&gt;0,(1-M472)/L472,1)</f>
+        <f>IF(L472&gt;x_series,(1-EXP(-L472))/L472,1-L472/2+L472^2/6-L472^3/24)</f>
         <v>0.998255808413</v>
       </c>
       <c r="O472" s="41">
-        <f>IF(L472&gt;0,(L472-1+M472)/L472^2,1/2)</f>
+        <f>IF(L472&gt;x_series,(L472-1+EXP(-L472))/L472^2,1/2-L472/6+L472^2/24-L472^3/120)</f>
         <v>0.499418433639</v>
       </c>
       <c r="P472" s="41">
@@ -34327,12 +34337,12 @@
         <v>0.999274857725</v>
       </c>
       <c r="E473" s="41">
-        <f>IF(C473&gt;0,(1-D473)/C473,1)</f>
+        <f>IF(C473&gt;x_series,(1-EXP(-C473))/C473,1-C473/2+C473^2/6-C473^3/24)</f>
         <v>0.999637385027</v>
       </c>
       <c r="F473" s="41">
-        <f>IF(C473&gt;0,(C473-1+D473)/C473^2,1/2)</f>
-        <v>0.499879120998</v>
+        <f>IF(C473&gt;x_series,(C473-1+EXP(-C473))/C473^2,1/2-C473/6+C473^2/24-C473^3/120)</f>
+        <v>0.499879121036</v>
       </c>
       <c r="G473" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B473/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34344,7 +34354,7 @@
       </c>
       <c r="I473" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H473+pool_b)*E473+G473*F473))</f>
-        <v>27.74942292765</v>
+        <v>27.749422927649</v>
       </c>
       <c r="J473" s="41">
         <f>IF(AND(I473&gt;=CO2_pH_hi_mt,I474&lt;CO2_pH_hi_mt),EXP(LN(A473)+(LN(A474)-LN(A473))*(I473-CO2_pH_hi_mt)/(I473-I474)),0)</f>
@@ -34359,11 +34369,11 @@
         <v>0.996089780169</v>
       </c>
       <c r="N473" s="41">
-        <f>IF(L473&gt;0,(1-M473)/L473,1)</f>
+        <f>IF(L473&gt;x_series,(1-EXP(-L473))/L473,1-L473/2+L473^2/6-L473^3/24)</f>
         <v>0.998043613435</v>
       </c>
       <c r="O473" s="41">
-        <f>IF(L473&gt;0,(L473-1+M473)/L473^2,1/2)</f>
+        <f>IF(L473&gt;x_series,(L473-1+EXP(-L473))/L473^2,1/2-L473/6+L473^2/24-L473^3/120)</f>
         <v>0.499347658287</v>
       </c>
       <c r="P473" s="41">
@@ -34401,12 +34411,12 @@
         <v>0.999186696908</v>
       </c>
       <c r="E474" s="41">
-        <f>IF(C474&gt;0,(1-D474)/C474,1)</f>
+        <f>IF(C474&gt;x_series,(1-EXP(-C474))/C474,1-C474/2+C474^2/6-C474^3/24)</f>
         <v>0.99959329331</v>
       </c>
       <c r="F474" s="41">
-        <f>IF(C474&gt;0,(C474-1+D474)/C474^2,1/2)</f>
-        <v>0.499864421983</v>
+        <f>IF(C474&gt;x_series,(C474-1+EXP(-C474))/C474^2,1/2-C474/6+C474^2/24-C474^3/120)</f>
+        <v>0.499864421912</v>
       </c>
       <c r="G474" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B474/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34418,7 +34428,7 @@
       </c>
       <c r="I474" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H474+pool_b)*E474+G474*F474))</f>
-        <v>27.712479881891</v>
+        <v>27.712479881893</v>
       </c>
       <c r="J474" s="41">
         <f>IF(AND(I474&gt;=CO2_pH_hi_mt,I475&lt;CO2_pH_hi_mt),EXP(LN(A474)+(LN(A475)-LN(A474))*(I474-CO2_pH_hi_mt)/(I474-I475)),0)</f>
@@ -34433,11 +34443,11 @@
         <v>0.995615236984</v>
       </c>
       <c r="N474" s="41">
-        <f>IF(L474&gt;0,(1-M474)/L474,1)</f>
+        <f>IF(L474&gt;x_series,(1-EXP(-L474))/L474,1-L474/2+L474^2/6-L474^3/24)</f>
         <v>0.997806012791</v>
       </c>
       <c r="O474" s="41">
-        <f>IF(L474&gt;0,(L474-1+M474)/L474^2,1/2)</f>
+        <f>IF(L474&gt;x_series,(L474-1+EXP(-L474))/L474^2,1/2-L474/6+L474^2/24-L474^3/120)</f>
         <v>0.499268403197</v>
       </c>
       <c r="P474" s="41">
@@ -34475,12 +34485,12 @@
         <v>0.999087960338</v>
       </c>
       <c r="E475" s="41">
-        <f>IF(C475&gt;0,(1-D475)/C475,1)</f>
+        <f>IF(C475&gt;x_series,(1-EXP(-C475))/C475,1-C475/2+C475^2/6-C475^3/24)</f>
         <v>0.999543910819</v>
       </c>
       <c r="F475" s="41">
-        <f>IF(C475&gt;0,(C475-1+D475)/C475^2,1/2)</f>
-        <v>0.499847958677</v>
+        <f>IF(C475&gt;x_series,(C475-1+EXP(-C475))/C475^2,1/2-C475/6+C475^2/24-C475^3/120)</f>
+        <v>0.499847958714</v>
       </c>
       <c r="G475" s="41">
         <f>(C_air_CO2/C_sat_CO2*F_vent_ex-CO2_fix_sched)*(B475/3600)/(V_L_CO2+Vg_CO2)</f>
@@ -34492,7 +34502,7 @@
       </c>
       <c r="I475" s="41">
         <f>MIN(C_sat_CO2,MAX(C_air_CO2,(pool_ret*H475+pool_b)*E475+G475*F475))</f>
-        <v>27.671180259514</v>
+        <v>27.671180259512</v>
       </c>
       <c r="J475" s="41">
         <f>IF(AND(I475&gt;=CO2_pH_hi_mt,I476&lt;CO2_pH_hi_mt),EXP(LN(A475)+(LN(A476)-LN(A475))*(I475-CO2_pH_hi_mt)/(I475-I476)),0)</f>
@@ -34507,11 +34517,11 @@
         <v>0.995083986413</v>
       </c>
       <c r="N475" s="41">
-        <f>IF(L475&gt;0,(1-M475)/L475,1)</f>
+        <f>IF(L475&gt;x_series,(1-EXP(-L475))/L475,1-L475/2+L475^2/6-L475^3/24)</f>
         <v>0.997539974308</v>
       </c>
       <c r="O475" s="41">
-        <f>IF(L475&gt;0,(L475-1+M475)/L475^2,1/2)</f>
+        <f>IF(L475&gt;x_series,(L475-1+EXP(-L475))/L475^2,1/2-L475/6+L475^2/24-L475^3/120)</f>
         <v>0.499179654787</v>
       </c>
       <c r="P475" s="41">
@@ -34549,11 +34559,11 @@
         <v>0.998977380593</v>
       </c>
       <c r="E476" s="41">
-        <f>IF(C476&gt;0,(1-D476)/C476,1)</f>
+        <f>IF(C476&gt;x_series,(1-EXP(-C476))/C476,1-C476/2+C476^2/6-C476^3/24)</f>
         <v>0.999488603106</v>
       </c>
       <c r="F476" s="41">
-        <f>IF(C476&gt;0,(C476-1+D476)/C476^2,1/2)</f>
+        <f>IF(C476&gt;x_series,(C476-1+EXP(-C476))/C476^2,1/2-C476/6+C476^2/24-C476^3/120)</f>
         <v>0.499829519888</v>
       </c>
       <c r="G476" s="41">
@@ -34581,11 +34591,11 @@
         <v>0.99448928805</v>
       </c>
       <c r="N476" s="41">
-        <f>IF(L476&gt;0,(1-M476)/L476,1)</f>
+        <f>IF(L476&gt;x_series,(1-EXP(-L476))/L476,1-L476/2+L476^2/6-L476^3/24)</f>
         <v>0.997242106366</v>
       </c>
       <c r="O476" s="41">
-        <f>IF(L476&gt;0,(L476-1+M476)/L476^2,1/2)</f>
+        <f>IF(L476&gt;x_series,(L476-1+EXP(-L476))/L476^2,1/2-L476/6+L476^2/24-L476^3/120)</f>
         <v>0.499080278945</v>
       </c>
       <c r="P476" s="41">
@@ -34623,11 +34633,11 @@
         <v>0.998853538675</v>
       </c>
       <c r="E477" s="41">
-        <f>IF(C477&gt;0,(1-D477)/C477,1)</f>
+        <f>IF(C477&gt;x_series,(1-EXP(-C477))/C477,1-C477/2+C477^2/6-C477^3/24)</f>
         <v>0.999426659743</v>
       </c>
       <c r="F477" s="41">
-        <f>IF(C477&gt;0,(C477-1+D477)/C477^2,1/2)</f>
+        <f>IF(C477&gt;x_series,(C477-1+EXP(-C477))/C477^2,1/2-C477/6+C477^2/24-C477^3/120)</f>
         <v>0.499808868312</v>
       </c>
       <c r="G477" s="41">
@@ -34655,11 +34665,11 @@
         <v>0.993823609484</v>
       </c>
       <c r="N477" s="41">
-        <f>IF(L477&gt;0,(1-M477)/L477,1)</f>
+        <f>IF(L477&gt;x_series,(1-EXP(-L477))/L477,1-L477/2+L477^2/6-L477^3/24)</f>
         <v>0.996908615903</v>
       </c>
       <c r="O477" s="41">
-        <f>IF(L477&gt;0,(L477-1+M477)/L477^2,1/2)</f>
+        <f>IF(L477&gt;x_series,(L477-1+EXP(-L477))/L477^2,1/2-L477/6+L477^2/24-L477^3/120)</f>
         <v>0.49896900683</v>
       </c>
       <c r="P477" s="41">
@@ -34697,11 +34707,11 @@
         <v>0.998714845963</v>
       </c>
       <c r="E478" s="41">
-        <f>IF(C478&gt;0,(1-D478)/C478,1)</f>
+        <f>IF(C478&gt;x_series,(1-EXP(-C478))/C478,1-C478/2+C478^2/6-C478^3/24)</f>
         <v>0.999357285258</v>
       </c>
       <c r="F478" s="41">
-        <f>IF(C478&gt;0,(C478-1+D478)/C478^2,1/2)</f>
+        <f>IF(C478&gt;x_series,(C478-1+EXP(-C478))/C478^2,1/2-C478/6+C478^2/24-C478^3/120)</f>
         <v>0.499785738754</v>
       </c>
       <c r="G478" s="41">
@@ -34729,11 +34739,11 @@
         <v>0.993078535565</v>
       </c>
       <c r="N478" s="41">
-        <f>IF(L478&gt;0,(1-M478)/L478,1)</f>
+        <f>IF(L478&gt;x_series,(1-EXP(-L478))/L478,1-L478/2+L478^2/6-L478^3/24)</f>
         <v>0.996535261683</v>
       </c>
       <c r="O478" s="41">
-        <f>IF(L478&gt;0,(L478-1+M478)/L478^2,1/2)</f>
+        <f>IF(L478&gt;x_series,(L478-1+EXP(-L478))/L478^2,1/2-L478/6+L478^2/24-L478^3/120)</f>
         <v>0.498844419081</v>
       </c>
       <c r="P478" s="41">
@@ -34771,11 +34781,11 @@
         <v>0.998559524042</v>
       </c>
       <c r="E479" s="41">
-        <f>IF(C479&gt;0,(1-D479)/C479,1)</f>
+        <f>IF(C479&gt;x_series,(1-EXP(-C479))/C479,1-C479/2+C479^2/6-C479^3/24)</f>
         <v>0.999279588982</v>
       </c>
       <c r="F479" s="41">
-        <f>IF(C479&gt;0,(C479-1+D479)/C479^2,1/2)</f>
+        <f>IF(C479&gt;x_series,(C479-1+EXP(-C479))/C479^2,1/2-C479/6+C479^2/24-C479^3/120)</f>
         <v>0.499759834171</v>
       </c>
       <c r="G479" s="41">
@@ -34803,11 +34813,11 @@
         <v>0.99224466789</v>
       </c>
       <c r="N479" s="41">
-        <f>IF(L479&gt;0,(1-M479)/L479,1)</f>
+        <f>IF(L479&gt;x_series,(1-EXP(-L479))/L479,1-L479/2+L479^2/6-L479^3/24)</f>
         <v>0.996117302316</v>
       </c>
       <c r="O479" s="41">
-        <f>IF(L479&gt;0,(L479-1+M479)/L479^2,1/2)</f>
+        <f>IF(L479&gt;x_series,(L479-1+EXP(-L479))/L479^2,1/2-L479/6+L479^2/24-L479^3/120)</f>
         <v>0.49870492818</v>
       </c>
       <c r="P479" s="41">
@@ -34845,11 +34855,11 @@
         <v>0.998385582147</v>
       </c>
       <c r="E480" s="41">
-        <f>IF(C480&gt;0,(1-D480)/C480,1)</f>
+        <f>IF(C480&gt;x_series,(1-EXP(-C480))/C480,1-C480/2+C480^2/6-C480^3/24)</f>
         <v>0.999192573703</v>
       </c>
       <c r="F480" s="41">
-        <f>IF(C480&gt;0,(C480-1+D480)/C480^2,1/2)</f>
+        <f>IF(C480&gt;x_series,(C480-1+EXP(-C480))/C480^2,1/2-C480/6+C480^2/24-C480^3/120)</f>
         <v>0.499730821667</v>
       </c>
       <c r="G480" s="41">
@@ -34877,11 +34887,11 @@
         <v>0.991311513587</v>
       </c>
       <c r="N480" s="41">
-        <f>IF(L480&gt;0,(1-M480)/L480,1)</f>
+        <f>IF(L480&gt;x_series,(1-EXP(-L480))/L480,1-L480/2+L480^2/6-L480^3/24)</f>
         <v>0.995649438497</v>
       </c>
       <c r="O480" s="41">
-        <f>IF(L480&gt;0,(L480-1+M480)/L480^2,1/2)</f>
+        <f>IF(L480&gt;x_series,(L480-1+EXP(-L480))/L480^2,1/2-L480/6+L480^2/24-L480^3/120)</f>
         <v>0.498548758864</v>
       </c>
       <c r="P480" s="41">
@@ -34919,11 +34929,11 @@
         <v>0.998190791976</v>
       </c>
       <c r="E481" s="41">
-        <f>IF(C481&gt;0,(1-D481)/C481,1)</f>
+        <f>IF(C481&gt;x_series,(1-EXP(-C481))/C481,1-C481/2+C481^2/6-C481^3/24)</f>
         <v>0.999095122972</v>
       </c>
       <c r="F481" s="41">
-        <f>IF(C481&gt;0,(C481-1+D481)/C481^2,1/2)</f>
+        <f>IF(C481&gt;x_series,(C481-1+EXP(-C481))/C481^2,1/2-C481/6+C481^2/24-C481^3/120)</f>
         <v>0.499698328794</v>
       </c>
       <c r="G481" s="41">
@@ -34951,11 +34961,11 @@
         <v>0.990267362473</v>
       </c>
       <c r="N481" s="41">
-        <f>IF(L481&gt;0,(1-M481)/L481,1)</f>
+        <f>IF(L481&gt;x_series,(1-EXP(-L481))/L481,1-L481/2+L481^2/6-L481^3/24)</f>
         <v>0.995125748899</v>
       </c>
       <c r="O481" s="41">
-        <f>IF(L481&gt;0,(L481-1+M481)/L481^2,1/2)</f>
+        <f>IF(L481&gt;x_series,(L481-1+EXP(-L481))/L481^2,1/2-L481/6+L481^2/24-L481^3/120)</f>
         <v>0.498373926284</v>
       </c>
       <c r="P481" s="41">
@@ -34993,11 +35003,11 @@
         <v>0.997972659538</v>
       </c>
       <c r="E482" s="41">
-        <f>IF(C482&gt;0,(1-D482)/C482,1)</f>
+        <f>IF(C482&gt;x_series,(1-EXP(-C482))/C482,1-C482/2+C482^2/6-C482^3/24)</f>
         <v>0.998985986912</v>
       </c>
       <c r="F482" s="41">
-        <f>IF(C482&gt;0,(C482-1+D482)/C482^2,1/2)</f>
+        <f>IF(C482&gt;x_series,(C482-1+EXP(-C482))/C482^2,1/2-C482/6+C482^2/24-C482^3/120)</f>
         <v>0.49966193848</v>
       </c>
       <c r="G482" s="41">
@@ -35025,11 +35035,11 @@
         <v>0.989099151601</v>
       </c>
       <c r="N482" s="41">
-        <f>IF(L482&gt;0,(1-M482)/L482,1)</f>
+        <f>IF(L482&gt;x_series,(1-EXP(-L482))/L482,1-L482/2+L482^2/6-L482^3/24)</f>
         <v>0.994539619078</v>
       </c>
       <c r="O482" s="41">
-        <f>IF(L482&gt;0,(L482-1+M482)/L482^2,1/2)</f>
+        <f>IF(L482&gt;x_series,(L482-1+EXP(-L482))/L482^2,1/2-L482/6+L482^2/24-L482^3/120)</f>
         <v>0.498178211754</v>
       </c>
       <c r="P482" s="41">
@@ -35067,11 +35077,11 @@
         <v>0.997728393727</v>
       </c>
       <c r="E483" s="41">
-        <f>IF(C483&gt;0,(1-D483)/C483,1)</f>
+        <f>IF(C483&gt;x_series,(1-EXP(-C483))/C483,1-C483/2+C483^2/6-C483^3/24)</f>
         <v>0.998863766358</v>
       </c>
       <c r="F483" s="41">
-        <f>IF(C483&gt;0,(C483-1+D483)/C483^2,1/2)</f>
+        <f>IF(C483&gt;x_series,(C483-1+EXP(-C483))/C483^2,1/2-C483/6+C483^2/24-C483^3/120)</f>
         <v>0.49962118368</v>
       </c>
       <c r="G483" s="41">
@@ -35099,11 +35109,11 @@
         <v>0.987792316226</v>
       </c>
       <c r="N483" s="41">
-        <f>IF(L483&gt;0,(1-M483)/L483,1)</f>
+        <f>IF(L483&gt;x_series,(1-EXP(-L483))/L483,1-L483/2+L483^2/6-L483^3/24)</f>
         <v>0.993883662756</v>
       </c>
       <c r="O483" s="41">
-        <f>IF(L483&gt;0,(L483-1+M483)/L483^2,1/2)</f>
+        <f>IF(L483&gt;x_series,(L483-1+EXP(-L483))/L483^2,1/2-L483/6+L483^2/24-L483^3/120)</f>
         <v>0.497959135801</v>
       </c>
       <c r="P483" s="41">
@@ -35141,11 +35151,11 @@
         <v>0.997454871243</v>
       </c>
       <c r="E484" s="41">
-        <f>IF(C484&gt;0,(1-D484)/C484,1)</f>
+        <f>IF(C484&gt;x_series,(1-EXP(-C484))/C484,1-C484/2+C484^2/6-C484^3/24)</f>
         <v>0.998726895127</v>
       </c>
       <c r="F484" s="41">
-        <f>IF(C484&gt;0,(C484-1+D484)/C484^2,1/2)</f>
+        <f>IF(C484&gt;x_series,(C484-1+EXP(-C484))/C484^2,1/2-C484/6+C484^2/24-C484^3/120)</f>
         <v>0.499575541605</v>
       </c>
       <c r="G484" s="41">
@@ -35173,11 +35183,11 @@
         <v>0.986330626219</v>
       </c>
       <c r="N484" s="41">
-        <f>IF(L484&gt;0,(1-M484)/L484,1)</f>
+        <f>IF(L484&gt;x_series,(1-EXP(-L484))/L484,1-L484/2+L484^2/6-L484^3/24)</f>
         <v>0.993149634775</v>
       </c>
       <c r="O484" s="41">
-        <f>IF(L484&gt;0,(L484-1+M484)/L484^2,1/2)</f>
+        <f>IF(L484&gt;x_series,(L484-1+EXP(-L484))/L484^2,1/2-L484/6+L484^2/24-L484^3/120)</f>
         <v>0.497713928273</v>
       </c>
       <c r="P484" s="41">
@@ -35215,11 +35225,11 @@
         <v>0.997148597439</v>
       </c>
       <c r="E485" s="41">
-        <f>IF(C485&gt;0,(1-D485)/C485,1)</f>
+        <f>IF(C485&gt;x_series,(1-EXP(-C485))/C485,1-C485/2+C485^2/6-C485^3/24)</f>
         <v>0.998573620211</v>
       </c>
       <c r="F485" s="41">
-        <f>IF(C485&gt;0,(C485-1+D485)/C485^2,1/2)</f>
+        <f>IF(C485&gt;x_series,(C485-1+EXP(-C485))/C485^2,1/2-C485/6+C485^2/24-C485^3/120)</f>
         <v>0.499524426947</v>
       </c>
       <c r="G485" s="41">
@@ -35247,11 +35257,11 @@
         <v>0.984696007012</v>
       </c>
       <c r="N485" s="41">
-        <f>IF(L485&gt;0,(1-M485)/L485,1)</f>
+        <f>IF(L485&gt;x_series,(1-EXP(-L485))/L485,1-L485/2+L485^2/6-L485^3/24)</f>
         <v>0.99232833501</v>
       </c>
       <c r="O485" s="41">
-        <f>IF(L485&gt;0,(L485-1+M485)/L485^2,1/2)</f>
+        <f>IF(L485&gt;x_series,(L485-1+EXP(-L485))/L485^2,1/2-L485/6+L485^2/24-L485^3/120)</f>
         <v>0.497439495198</v>
       </c>
       <c r="P485" s="41">
@@ -35289,11 +35299,11 @@
         <v>0.996805662673</v>
       </c>
       <c r="E486" s="41">
-        <f>IF(C486&gt;0,(1-D486)/C486,1)</f>
+        <f>IF(C486&gt;x_series,(1-EXP(-C486))/C486,1-C486/2+C486^2/6-C486^3/24)</f>
         <v>0.99840197966</v>
       </c>
       <c r="F486" s="41">
-        <f>IF(C486&gt;0,(C486-1+D486)/C486^2,1/2)</f>
+        <f>IF(C486&gt;x_series,(C486-1+EXP(-C486))/C486^2,1/2-C486/6+C486^2/24-C486^3/120)</f>
         <v>0.499467184561</v>
       </c>
       <c r="G486" s="41">
@@ -35321,11 +35331,11 @@
         <v>0.98286834423</v>
       </c>
       <c r="N486" s="41">
-        <f>IF(L486&gt;0,(1-M486)/L486,1)</f>
+        <f>IF(L486&gt;x_series,(1-EXP(-L486))/L486,1-L486/2+L486^2/6-L486^3/24)</f>
         <v>0.99140950251</v>
       </c>
       <c r="O486" s="41">
-        <f>IF(L486&gt;0,(L486-1+M486)/L486^2,1/2)</f>
+        <f>IF(L486&gt;x_series,(L486-1+EXP(-L486))/L486^2,1/2-L486/6+L486^2/24-L486^3/120)</f>
         <v>0.497132382131</v>
       </c>
       <c r="P486" s="41">
@@ -35363,11 +35373,11 @@
         <v>0.996421693635</v>
       </c>
       <c r="E487" s="41">
-        <f>IF(C487&gt;0,(1-D487)/C487,1)</f>
+        <f>IF(C487&gt;x_series,(1-EXP(-C487))/C487,1-C487/2+C487^2/6-C487^3/24)</f>
         <v>0.998209777881</v>
       </c>
       <c r="F487" s="41">
-        <f>IF(C487&gt;0,(C487-1+D487)/C487^2,1/2)</f>
+        <f>IF(C487&gt;x_series,(C487-1+EXP(-C487))/C487^2,1/2-C487/6+C487^2/24-C487^3/120)</f>
         <v>0.499403081071</v>
       </c>
       <c r="G487" s="41">
@@ -35395,11 +35405,11 @@
         <v>0.980825271336</v>
       </c>
       <c r="N487" s="41">
-        <f>IF(L487&gt;0,(1-M487)/L487,1)</f>
+        <f>IF(L487&gt;x_series,(1-EXP(-L487))/L487,1-L487/2+L487^2/6-L487^3/24)</f>
         <v>0.990381699117</v>
       </c>
       <c r="O487" s="41">
-        <f>IF(L487&gt;0,(L487-1+M487)/L487^2,1/2)</f>
+        <f>IF(L487&gt;x_series,(L487-1+EXP(-L487))/L487^2,1/2-L487/6+L487^2/24-L487^3/120)</f>
         <v>0.496788733631</v>
       </c>
       <c r="P487" s="41">
@@ -35437,11 +35447,11 @@
         <v>0.995991799142</v>
       </c>
       <c r="E488" s="41">
-        <f>IF(C488&gt;0,(1-D488)/C488,1)</f>
+        <f>IF(C488&gt;x_series,(1-EXP(-C488))/C488,1-C488/2+C488^2/6-C488^3/24)</f>
         <v>0.997994558075</v>
       </c>
       <c r="F488" s="41">
-        <f>IF(C488&gt;0,(C488-1+D488)/C488^2,1/2)</f>
+        <f>IF(C488&gt;x_series,(C488-1+EXP(-C488))/C488^2,1/2-C488/6+C488^2/24-C488^3/120)</f>
         <v>0.499331295688</v>
       </c>
       <c r="G488" s="41">
@@ -35469,11 +35479,11 @@
         <v>0.978541939808</v>
       </c>
       <c r="N488" s="41">
-        <f>IF(L488&gt;0,(1-M488)/L488,1)</f>
+        <f>IF(L488&gt;x_series,(1-EXP(-L488))/L488,1-L488/2+L488^2/6-L488^3/24)</f>
         <v>0.989232181847</v>
       </c>
       <c r="O488" s="41">
-        <f>IF(L488&gt;0,(L488-1+M488)/L488^2,1/2)</f>
+        <f>IF(L488&gt;x_series,(L488-1+EXP(-L488))/L488^2,1/2-L488/6+L488^2/24-L488^3/120)</f>
         <v>0.496404248583</v>
       </c>
       <c r="P488" s="41">
@@ -35511,11 +35521,11 @@
         <v>0.995510509779</v>
       </c>
       <c r="E489" s="41">
-        <f>IF(C489&gt;0,(1-D489)/C489,1)</f>
+        <f>IF(C489&gt;x_series,(1-EXP(-C489))/C489,1-C489/2+C489^2/6-C489^3/24)</f>
         <v>0.997753571482</v>
       </c>
       <c r="F489" s="41">
-        <f>IF(C489&gt;0,(C489-1+D489)/C489^2,1/2)</f>
+        <f>IF(C489&gt;x_series,(C489-1+EXP(-C489))/C489^2,1/2-C489/6+C489^2/24-C489^3/120)</f>
         <v>0.499250909798</v>
       </c>
       <c r="G489" s="41">
@@ -35543,11 +35553,11 @@
         <v>0.975990771723</v>
       </c>
       <c r="N489" s="41">
-        <f>IF(L489&gt;0,(1-M489)/L489,1)</f>
+        <f>IF(L489&gt;x_series,(1-EXP(-L489))/L489,1-L489/2+L489^2/6-L489^3/24)</f>
         <v>0.987946763355</v>
       </c>
       <c r="O489" s="41">
-        <f>IF(L489&gt;0,(L489-1+M489)/L489^2,1/2)</f>
+        <f>IF(L489&gt;x_series,(L489-1+EXP(-L489))/L489^2,1/2-L489/6+L489^2/24-L489^3/120)</f>
         <v>0.495974131007</v>
       </c>
       <c r="P489" s="41">
@@ -35585,11 +35595,11 @@
         <v>0.994971710765</v>
       </c>
       <c r="E490" s="41">
-        <f>IF(C490&gt;0,(1-D490)/C490,1)</f>
+        <f>IF(C490&gt;x_series,(1-EXP(-C490))/C490,1-C490/2+C490^2/6-C490^3/24)</f>
         <v>0.997483743094</v>
       </c>
       <c r="F490" s="41">
-        <f>IF(C490&gt;0,(C490-1+D490)/C490^2,1/2)</f>
+        <f>IF(C490&gt;x_series,(C490-1+EXP(-C490))/C490^2,1/2-C490/6+C490^2/24-C490^3/120)</f>
         <v>0.499160895473</v>
       </c>
       <c r="G490" s="41">
@@ -35617,11 +35627,11 @@
         <v>0.973141194999</v>
       </c>
       <c r="N490" s="41">
-        <f>IF(L490&gt;0,(1-M490)/L490,1)</f>
+        <f>IF(L490&gt;x_series,(1-EXP(-L490))/L490,1-L490/2+L490^2/6-L490^3/24)</f>
         <v>0.986509659889</v>
       </c>
       <c r="O490" s="41">
-        <f>IF(L490&gt;0,(L490-1+M490)/L490^2,1/2)</f>
+        <f>IF(L490&gt;x_series,(L490-1+EXP(-L490))/L490^2,1/2-L490/6+L490^2/24-L490^3/120)</f>
         <v>0.495493036043</v>
       </c>
       <c r="P490" s="41">
@@ -35659,11 +35669,11 @@
         <v>0.994368567328</v>
       </c>
       <c r="E491" s="41">
-        <f>IF(C491&gt;0,(1-D491)/C491,1)</f>
+        <f>IF(C491&gt;x_series,(1-EXP(-C491))/C491,1-C491/2+C491^2/6-C491^3/24)</f>
         <v>0.997181633443</v>
       </c>
       <c r="F491" s="41">
-        <f>IF(C491&gt;0,(C491-1+D491)/C491^2,1/2)</f>
+        <f>IF(C491&gt;x_series,(C491-1+EXP(-C491))/C491^2,1/2-C491/6+C491^2/24-C491^3/120)</f>
         <v>0.49906010253</v>
       </c>
       <c r="G491" s="41">
@@ -35691,11 +35701,11 @@
         <v>0.969959362224</v>
       </c>
       <c r="N491" s="41">
-        <f>IF(L491&gt;0,(1-M491)/L491,1)</f>
+        <f>IF(L491&gt;x_series,(1-EXP(-L491))/L491,1-L491/2+L491^2/6-L491^3/24)</f>
         <v>0.984903326247</v>
       </c>
       <c r="O491" s="41">
-        <f>IF(L491&gt;0,(L491-1+M491)/L491^2,1/2)</f>
+        <f>IF(L491&gt;x_series,(L491-1+EXP(-L491))/L491^2,1/2-L491/6+L491^2/24-L491^3/120)</f>
         <v>0.49495501079</v>
       </c>
       <c r="P491" s="41">
@@ -35733,11 +35743,11 @@
         <v>0.993693441852</v>
       </c>
       <c r="E492" s="41">
-        <f>IF(C492&gt;0,(1-D492)/C492,1)</f>
+        <f>IF(C492&gt;x_series,(1-EXP(-C492))/C492,1-C492/2+C492^2/6-C492^3/24)</f>
         <v>0.996843396043</v>
       </c>
       <c r="F492" s="41">
-        <f>IF(C492&gt;0,(C492-1+D492)/C492^2,1/2)</f>
+        <f>IF(C492&gt;x_series,(C492-1+EXP(-C492))/C492^2,1/2-C492/6+C492^2/24-C492^3/120)</f>
         <v>0.498947244183</v>
       </c>
       <c r="G492" s="41">
@@ -35765,11 +35775,11 @@
         <v>0.96640785469</v>
       </c>
       <c r="N492" s="41">
-        <f>IF(L492&gt;0,(1-M492)/L492,1)</f>
+        <f>IF(L492&gt;x_series,(1-EXP(-L492))/L492,1-L492/2+L492^2/6-L492^3/24)</f>
         <v>0.983108277465</v>
       </c>
       <c r="O492" s="41">
-        <f>IF(L492&gt;0,(L492-1+M492)/L492^2,1/2)</f>
+        <f>IF(L492&gt;x_series,(L492-1+EXP(-L492))/L492^2,1/2-L492/6+L492^2/24-L492^3/120)</f>
         <v>0.494353429704</v>
       </c>
       <c r="P492" s="41">
@@ -35807,11 +35817,11 @@
         <v>0.992937801973</v>
       </c>
       <c r="E493" s="41">
-        <f>IF(C493&gt;0,(1-D493)/C493,1)</f>
+        <f>IF(C493&gt;x_series,(1-EXP(-C493))/C493,1-C493/2+C493^2/6-C493^3/24)</f>
         <v>0.996464730024</v>
       </c>
       <c r="F493" s="41">
-        <f>IF(C493&gt;0,(C493-1+D493)/C493^2,1/2)</f>
+        <f>IF(C493&gt;x_series,(C493-1+EXP(-C493))/C493^2,1/2-C493/6+C493^2/24-C493^3/120)</f>
         <v>0.498820881022</v>
       </c>
       <c r="G493" s="41">
@@ -35839,11 +35849,11 @@
         <v>0.96244537435</v>
       </c>
       <c r="N493" s="41">
-        <f>IF(L493&gt;0,(1-M493)/L493,1)</f>
+        <f>IF(L493&gt;x_series,(1-EXP(-L493))/L493,1-L493/2+L493^2/6-L493^3/24)</f>
         <v>0.981102897202</v>
       </c>
       <c r="O493" s="41">
-        <f>IF(L493&gt;0,(L493-1+M493)/L493^2,1/2)</f>
+        <f>IF(L493&gt;x_series,(L493-1+EXP(-L493))/L493^2,1/2-L493/6+L493^2/24-L493^3/120)</f>
         <v>0.493680924318</v>
       </c>
       <c r="P493" s="41">
@@ -35881,11 +35891,11 @@
         <v>0.992092118771</v>
       </c>
       <c r="E494" s="41">
-        <f>IF(C494&gt;0,(1-D494)/C494,1)</f>
+        <f>IF(C494&gt;x_series,(1-EXP(-C494))/C494,1-C494/2+C494^2/6-C494^3/24)</f>
         <v>0.996040827462</v>
       </c>
       <c r="F494" s="41">
-        <f>IF(C494&gt;0,(C494-1+D494)/C494^2,1/2)</f>
+        <f>IF(C494&gt;x_series,(C494-1+EXP(-C494))/C494^2,1/2-C494/6+C494^2/24-C494^3/120)</f>
         <v>0.498679403141</v>
       </c>
       <c r="G494" s="41">
@@ -35913,11 +35923,11 @@
         <v>0.958026427677</v>
       </c>
       <c r="N494" s="41">
-        <f>IF(L494&gt;0,(1-M494)/L494,1)</f>
+        <f>IF(L494&gt;x_series,(1-EXP(-L494))/L494,1-L494/2+L494^2/6-L494^3/24)</f>
         <v>0.978863233167</v>
       </c>
       <c r="O494" s="41">
-        <f>IF(L494&gt;0,(L494-1+M494)/L494^2,1/2)</f>
+        <f>IF(L494&gt;x_series,(L494-1+EXP(-L494))/L494^2,1/2-L494/6+L494^2/24-L494^3/120)</f>
         <v>0.492929307092</v>
       </c>
       <c r="P494" s="41">
@@ -35955,11 +35965,11 @@
         <v>0.991145754163</v>
       </c>
       <c r="E495" s="41">
-        <f>IF(C495&gt;0,(1-D495)/C495,1)</f>
+        <f>IF(C495&gt;x_series,(1-EXP(-C495))/C495,1-C495/2+C495^2/6-C495^3/24)</f>
         <v>0.995566314856</v>
       </c>
       <c r="F495" s="41">
-        <f>IF(C495&gt;0,(C495-1+D495)/C495^2,1/2)</f>
+        <f>IF(C495&gt;x_series,(C495-1+EXP(-C495))/C495^2,1/2-C495/6+C495^2/24-C495^3/120)</f>
         <v>0.498521010276</v>
       </c>
       <c r="G495" s="41">
@@ -35987,11 +35997,11 @@
         <v>0.953101007099</v>
       </c>
       <c r="N495" s="41">
-        <f>IF(L495&gt;0,(1-M495)/L495,1)</f>
+        <f>IF(L495&gt;x_series,(1-EXP(-L495))/L495,1-L495/2+L495^2/6-L495^3/24)</f>
         <v>0.976362780382</v>
       </c>
       <c r="O495" s="41">
-        <f>IF(L495&gt;0,(L495-1+M495)/L495^2,1/2)</f>
+        <f>IF(L495&gt;x_series,(L495-1+EXP(-L495))/L495^2,1/2-L495/6+L495^2/24-L495^3/120)</f>
         <v>0.492089489316</v>
       </c>
       <c r="P495" s="41">
@@ -36029,11 +36039,11 @@
         <v>0.990086836528</v>
       </c>
       <c r="E496" s="41">
-        <f>IF(C496&gt;0,(1-D496)/C496,1)</f>
+        <f>IF(C496&gt;x_series,(1-EXP(-C496))/C496,1-C496/2+C496^2/6-C496^3/24)</f>
         <v>0.995035188183</v>
       </c>
       <c r="F496" s="41">
-        <f>IF(C496&gt;0,(C496-1+D496)/C496^2,1/2)</f>
+        <f>IF(C496&gt;x_series,(C496-1+EXP(-C496))/C496^2,1/2-C496/6+C496^2/24-C496^3/120)</f>
         <v>0.498343689681</v>
       </c>
       <c r="G496" s="41">
@@ -36061,11 +36071,11 @@
         <v>0.947614277732</v>
       </c>
       <c r="N496" s="41">
-        <f>IF(L496&gt;0,(1-M496)/L496,1)</f>
+        <f>IF(L496&gt;x_series,(1-EXP(-L496))/L496,1-L496/2+L496^2/6-L496^3/24)</f>
         <v>0.973572253759</v>
       </c>
       <c r="O496" s="41">
-        <f>IF(L496&gt;0,(L496-1+M496)/L496^2,1/2)</f>
+        <f>IF(L496&gt;x_series,(L496-1+EXP(-L496))/L496^2,1/2-L496/6+L496^2/24-L496^3/120)</f>
         <v>0.491151393095</v>
       </c>
       <c r="P496" s="41">
@@ -36103,11 +36113,11 @@
         <v>0.988902123616</v>
       </c>
       <c r="E497" s="41">
-        <f>IF(C497&gt;0,(1-D497)/C497,1)</f>
+        <f>IF(C497&gt;x_series,(1-EXP(-C497))/C497,1-C497/2+C497^2/6-C497^3/24)</f>
         <v>0.994440740881</v>
       </c>
       <c r="F497" s="41">
-        <f>IF(C497&gt;0,(C497-1+D497)/C497^2,1/2)</f>
+        <f>IF(C497&gt;x_series,(C497-1+EXP(-C497))/C497^2,1/2-C497/6+C497^2/24-C497^3/120)</f>
         <v>0.498145191553</v>
       </c>
       <c r="G497" s="41">
@@ -36135,11 +36145,11 @@
         <v>0.941506279791</v>
       </c>
       <c r="N497" s="41">
-        <f>IF(L497&gt;0,(1-M497)/L497,1)</f>
+        <f>IF(L497&gt;x_series,(1-EXP(-L497))/L497,1-L497/2+L497^2/6-L497^3/24)</f>
         <v>0.970459352204</v>
       </c>
       <c r="O497" s="41">
-        <f>IF(L497&gt;0,(L497-1+M497)/L497^2,1/2)</f>
+        <f>IF(L497&gt;x_series,(L497-1+EXP(-L497))/L497^2,1/2-L497/6+L497^2/24-L497^3/120)</f>
         <v>0.490103857663</v>
       </c>
       <c r="P497" s="41">
@@ -36177,11 +36187,11 @@
         <v>0.987576851749</v>
       </c>
       <c r="E498" s="41">
-        <f>IF(C498&gt;0,(1-D498)/C498,1)</f>
+        <f>IF(C498&gt;x_series,(1-EXP(-C498))/C498,1-C498/2+C498^2/6-C498^3/24)</f>
         <v>0.993775484134</v>
       </c>
       <c r="F498" s="41">
-        <f>IF(C498&gt;0,(C498-1+D498)/C498^2,1/2)</f>
+        <f>IF(C498&gt;x_series,(C498-1+EXP(-C498))/C498^2,1/2-C498/6+C498^2/24-C498^3/120)</f>
         <v>0.497923001725</v>
       </c>
       <c r="G498" s="41">
@@ -36209,11 +36219,11 @@
         <v>0.934711660152</v>
       </c>
       <c r="N498" s="41">
-        <f>IF(L498&gt;0,(1-M498)/L498,1)</f>
+        <f>IF(L498&gt;x_series,(1-EXP(-L498))/L498,1-L498/2+L498^2/6-L498^3/24)</f>
         <v>0.966988517588</v>
       </c>
       <c r="O498" s="41">
-        <f>IF(L498&gt;0,(L498-1+M498)/L498^2,1/2)</f>
+        <f>IF(L498&gt;x_series,(L498-1+EXP(-L498))/L498^2,1/2-L498/6+L498^2/24-L498^3/120)</f>
         <v>0.488934540463</v>
       </c>
       <c r="P498" s="41">
@@ -36251,11 +36261,11 @@
         <v>0.986094570348</v>
       </c>
       <c r="E499" s="41">
-        <f>IF(C499&gt;0,(1-D499)/C499,1)</f>
+        <f>IF(C499&gt;x_series,(1-EXP(-C499))/C499,1-C499/2+C499^2/6-C499^3/24)</f>
         <v>0.993031058731</v>
       </c>
       <c r="F499" s="41">
-        <f>IF(C499&gt;0,(C499-1+D499)/C499^2,1/2)</f>
+        <f>IF(C499&gt;x_series,(C499-1+EXP(-C499))/C499^2,1/2-C499/6+C499^2/24-C499^3/120)</f>
         <v>0.497674311383</v>
       </c>
       <c r="G499" s="41">
@@ -36283,11 +36293,11 @@
         <v>0.927159450478</v>
       </c>
       <c r="N499" s="41">
-        <f>IF(L499&gt;0,(1-M499)/L499,1)</f>
+        <f>IF(L499&gt;x_series,(1-EXP(-L499))/L499,1-L499/2+L499^2/6-L499^3/24)</f>
         <v>0.963120693126</v>
       </c>
       <c r="O499" s="41">
-        <f>IF(L499&gt;0,(L499-1+M499)/L499^2,1/2)</f>
+        <f>IF(L499&gt;x_series,(L499-1+EXP(-L499))/L499^2,1/2-L499/6+L499^2/24-L499^3/120)</f>
         <v>0.487629813772</v>
       </c>
       <c r="P499" s="41">
@@ -36325,11 +36335,11 @@
         <v>0.984436960885</v>
       </c>
       <c r="E500" s="41">
-        <f>IF(C500&gt;0,(1-D500)/C500,1)</f>
+        <f>IF(C500&gt;x_series,(1-EXP(-C500))/C500,1-C500/2+C500^2/6-C500^3/24)</f>
         <v>0.992198137799</v>
       </c>
       <c r="F500" s="41">
-        <f>IF(C500&gt;0,(C500-1+D500)/C500^2,1/2)</f>
+        <f>IF(C500&gt;x_series,(C500-1+EXP(-C500))/C500^2,1/2-C500/6+C500^2/24-C500^3/120)</f>
         <v>0.497395983508</v>
       </c>
       <c r="G500" s="41">
@@ -36357,11 +36367,11 @@
         <v>0.918772913878</v>
       </c>
       <c r="N500" s="41">
-        <f>IF(L500&gt;0,(1-M500)/L500,1)</f>
+        <f>IF(L500&gt;x_series,(1-EXP(-L500))/L500,1-L500/2+L500^2/6-L500^3/24)</f>
         <v>0.958813087414</v>
       </c>
       <c r="O500" s="41">
-        <f>IF(L500&gt;0,(L500-1+M500)/L500^2,1/2)</f>
+        <f>IF(L500&gt;x_series,(L500-1+EXP(-L500))/L500^2,1/2-L500/6+L500^2/24-L500^3/120)</f>
         <v>0.48617465803</v>
       </c>
       <c r="P500" s="41">
@@ -36399,11 +36409,11 @@
         <v>0.982583639427</v>
       </c>
       <c r="E501" s="41">
-        <f>IF(C501&gt;0,(1-D501)/C501,1)</f>
+        <f>IF(C501&gt;x_series,(1-EXP(-C501))/C501,1-C501/2+C501^2/6-C501^3/24)</f>
         <v>0.991266319666</v>
       </c>
       <c r="F501" s="41">
-        <f>IF(C501&gt;0,(C501-1+D501)/C501^2,1/2)</f>
+        <f>IF(C501&gt;x_series,(C501-1+EXP(-C501))/C501^2,1/2-C501/6+C501^2/24-C501^3/120)</f>
         <v>0.497084515747</v>
       </c>
       <c r="G501" s="41">
@@ -36431,11 +36441,11 @@
         <v>0.909469487572</v>
       </c>
       <c r="N501" s="41">
-        <f>IF(L501&gt;0,(1-M501)/L501,1)</f>
+        <f>IF(L501&gt;x_series,(1-EXP(-L501))/L501,1-L501/2+L501^2/6-L501^3/24)</f>
         <v>0.954018952283</v>
       </c>
       <c r="O501" s="41">
-        <f>IF(L501&gt;0,(L501-1+M501)/L501^2,1/2)</f>
+        <f>IF(L501&gt;x_series,(L501-1+EXP(-L501))/L501^2,1/2-L501/6+L501^2/24-L501^3/120)</f>
         <v>0.484552553513</v>
       </c>
       <c r="P501" s="41">
@@ -36473,11 +36483,11 @@
         <v>0.980511942119</v>
       </c>
       <c r="E502" s="41">
-        <f>IF(C502&gt;0,(1-D502)/C502,1)</f>
+        <f>IF(C502&gt;x_series,(1-EXP(-C502))/C502,1-C502/2+C502^2/6-C502^3/24)</f>
         <v>0.990224010114</v>
       </c>
       <c r="F502" s="41">
-        <f>IF(C502&gt;0,(C502-1+D502)/C502^2,1/2)</f>
+        <f>IF(C502&gt;x_series,(C502-1+EXP(-C502))/C502^2,1/2-C502/6+C502^2/24-C502^3/120)</f>
         <v>0.496735999397</v>
       </c>
       <c r="G502" s="41">
@@ -36505,11 +36515,11 @@
         <v>0.899160855337</v>
       </c>
       <c r="N502" s="41">
-        <f>IF(L502&gt;0,(1-M502)/L502,1)</f>
+        <f>IF(L502&gt;x_series,(1-EXP(-L502))/L502,1-L502/2+L502^2/6-L502^3/24)</f>
         <v>0.948687385082</v>
       </c>
       <c r="O502" s="41">
-        <f>IF(L502&gt;0,(L502-1+M502)/L502^2,1/2)</f>
+        <f>IF(L502&gt;x_series,(L502-1+EXP(-L502))/L502^2,1/2-L502/6+L502^2/24-L502^3/120)</f>
         <v>0.482745372649</v>
       </c>
       <c r="P502" s="41">
@@ -36547,11 +36557,11 @@
         <v>0.978196693168</v>
       </c>
       <c r="E503" s="41">
-        <f>IF(C503&gt;0,(1-D503)/C503,1)</f>
+        <f>IF(C503&gt;x_series,(1-EXP(-C503))/C503,1-C503/2+C503^2/6-C503^3/24)</f>
         <v>0.989058293304</v>
       </c>
       <c r="F503" s="41">
-        <f>IF(C503&gt;0,(C503-1+D503)/C503^2,1/2)</f>
+        <f>IF(C503&gt;x_series,(C503-1+EXP(-C503))/C503^2,1/2-C503/6+C503^2/24-C503^3/120)</f>
         <v>0.496346074172</v>
       </c>
       <c r="G503" s="41">
@@ -36579,11 +36589,11 @@
         <v>0.887753190779</v>
       </c>
       <c r="N503" s="41">
-        <f>IF(L503&gt;0,(1-M503)/L503,1)</f>
+        <f>IF(L503&gt;x_series,(1-EXP(-L503))/L503,1-L503/2+L503^2/6-L503^3/24)</f>
         <v>0.942763168845</v>
       </c>
       <c r="O503" s="41">
-        <f>IF(L503&gt;0,(L503-1+M503)/L503^2,1/2)</f>
+        <f>IF(L503&gt;x_series,(L503-1+EXP(-L503))/L503^2,1/2-L503/6+L503^2/24-L503^3/120)</f>
         <v>0.480733275977</v>
       </c>
       <c r="P503" s="41">
@@ -36621,11 +36631,11 @@
         <v>0.975609955229</v>
       </c>
       <c r="E504" s="41">
-        <f>IF(C504&gt;0,(1-D504)/C504,1)</f>
+        <f>IF(C504&gt;x_series,(1-EXP(-C504))/C504,1-C504/2+C504^2/6-C504^3/24)</f>
         <v>0.987754790712</v>
       </c>
       <c r="F504" s="41">
-        <f>IF(C504&gt;0,(C504-1+D504)/C504^2,1/2)</f>
+        <f>IF(C504&gt;x_series,(C504-1+EXP(-C504))/C504^2,1/2-C504/6+C504^2/24-C504^3/120)</f>
         <v>0.495909878433</v>
       </c>
       <c r="G504" s="41">
@@ -36653,11 +36663,11 @@
         <v>0.875147620487</v>
       </c>
       <c r="N504" s="41">
-        <f>IF(L504&gt;0,(1-M504)/L504,1)</f>
+        <f>IF(L504&gt;x_series,(1-EXP(-L504))/L504,1-L504/2+L504^2/6-L504^3/24)</f>
         <v>0.936186667199</v>
       </c>
       <c r="O504" s="41">
-        <f>IF(L504&gt;0,(L504-1+M504)/L504^2,1/2)</f>
+        <f>IF(L504&gt;x_series,(L504-1+EXP(-L504))/L504^2,1/2-L504/6+L504^2/24-L504^3/120)</f>
         <v>0.478494615731</v>
       </c>
       <c r="P504" s="41">
@@ -36695,11 +36705,11 @@
         <v>0.972720762548</v>
       </c>
       <c r="E505" s="41">
-        <f>IF(C505&gt;0,(1-D505)/C505,1)</f>
+        <f>IF(C505&gt;x_series,(1-EXP(-C505))/C505,1-C505/2+C505^2/6-C505^3/24)</f>
         <v>0.98629750747</v>
       </c>
       <c r="F505" s="41">
-        <f>IF(C505&gt;0,(C505-1+D505)/C505^2,1/2)</f>
+        <f>IF(C505&gt;x_series,(C505-1+EXP(-C505))/C505^2,1/2-C505/6+C505^2/24-C505^3/120)</f>
         <v>0.49542199454</v>
       </c>
       <c r="G505" s="41">
@@ -36727,11 +36737,11 @@
         <v>0.861240964803</v>
       </c>
       <c r="N505" s="41">
-        <f>IF(L505&gt;0,(1-M505)/L505,1)</f>
+        <f>IF(L505&gt;x_series,(1-EXP(-L505))/L505,1-L505/2+L505^2/6-L505^3/24)</f>
         <v>0.928893794794</v>
       </c>
       <c r="O505" s="41">
-        <f>IF(L505&gt;0,(L505-1+M505)/L505^2,1/2)</f>
+        <f>IF(L505&gt;x_series,(L505-1+EXP(-L505))/L505^2,1/2-L505/6+L505^2/24-L505^3/120)</f>
         <v>0.476005852111</v>
       </c>
       <c r="P505" s="41">
@@ -36769,11 +36779,11 @@
         <v>0.969494837828</v>
       </c>
       <c r="E506" s="41">
-        <f>IF(C506&gt;0,(1-D506)/C506,1)</f>
+        <f>IF(C506&gt;x_series,(1-EXP(-C506))/C506,1-C506/2+C506^2/6-C506^3/24)</f>
         <v>0.984668665686</v>
       </c>
       <c r="F506" s="41">
-        <f>IF(C506&gt;0,(C506-1+D506)/C506^2,1/2)</f>
+        <f>IF(C506&gt;x_series,(C506-1+EXP(-C506))/C506^2,1/2-C506/6+C506^2/24-C506^3/120)</f>
         <v>0.494876389028</v>
       </c>
       <c r="G506" s="41">
@@ -36801,11 +36811,11 @@
         <v>0.845926822908</v>
       </c>
       <c r="N506" s="41">
-        <f>IF(L506&gt;0,(1-M506)/L506,1)</f>
+        <f>IF(L506&gt;x_series,(1-EXP(-L506))/L506,1-L506/2+L506^2/6-L506^3/24)</f>
         <v>0.920816088474</v>
       </c>
       <c r="O506" s="41">
-        <f>IF(L506&gt;0,(L506-1+M506)/L506^2,1/2)</f>
+        <f>IF(L506&gt;x_series,(L506-1+EXP(-L506))/L506^2,1/2-L506/6+L506^2/24-L506^3/120)</f>
         <v>0.473241488604</v>
       </c>
       <c r="P506" s="41">
@@ -36843,11 +36853,11 @@
         <v>0.965894294598</v>
       </c>
       <c r="E507" s="41">
-        <f>IF(C507&gt;0,(1-D507)/C507,1)</f>
+        <f>IF(C507&gt;x_series,(1-EXP(-C507))/C507,1-C507/2+C507^2/6-C507^3/24)</f>
         <v>0.982848524455</v>
       </c>
       <c r="F507" s="41">
-        <f>IF(C507&gt;0,(C507-1+D507)/C507^2,1/2)</f>
+        <f>IF(C507&gt;x_series,(C507-1+EXP(-C507))/C507^2,1/2-C507/6+C507^2/24-C507^3/120)</f>
         <v>0.494266347307</v>
       </c>
       <c r="G507" s="41">
@@ -36875,11 +36885,11 @@
         <v>0.829097077536</v>
       </c>
       <c r="N507" s="41">
-        <f>IF(L507&gt;0,(1-M507)/L507,1)</f>
+        <f>IF(L507&gt;x_series,(1-EXP(-L507))/L507,1-L507/2+L507^2/6-L507^3/24)</f>
         <v>0.911880909338</v>
       </c>
       <c r="O507" s="41">
-        <f>IF(L507&gt;0,(L507-1+M507)/L507^2,1/2)</f>
+        <f>IF(L507&gt;x_series,(L507-1+EXP(-L507))/L507^2,1/2-L507/6+L507^2/24-L507^3/120)</f>
         <v>0.470174034267</v>
       </c>
       <c r="P507" s="41">
@@ -36917,11 +36927,11 @@
         <v>0.96187732791</v>
       </c>
       <c r="E508" s="41">
-        <f>IF(C508&gt;0,(1-D508)/C508,1)</f>
+        <f>IF(C508&gt;x_series,(1-EXP(-C508))/C508,1-C508/2+C508^2/6-C508^3/24)</f>
         <v>0.980815186604</v>
       </c>
       <c r="F508" s="41">
-        <f>IF(C508&gt;0,(C508-1+D508)/C508^2,1/2)</f>
+        <f>IF(C508&gt;x_series,(C508-1+EXP(-C508))/C508^2,1/2-C508/6+C508^2/24-C508^3/120)</f>
         <v>0.493584402654</v>
       </c>
       <c r="G508" s="41">
@@ -36949,11 +36959,11 @@
         <v>0.810643902102</v>
       </c>
       <c r="N508" s="41">
-        <f>IF(L508&gt;0,(1-M508)/L508,1)</f>
+        <f>IF(L508&gt;x_series,(1-EXP(-L508))/L508,1-L508/2+L508^2/6-L508^3/24)</f>
         <v>0.902011811106</v>
       </c>
       <c r="O508" s="41">
-        <f>IF(L508&gt;0,(L508-1+M508)/L508^2,1/2)</f>
+        <f>IF(L508&gt;x_series,(L508-1+EXP(-L508))/L508^2,1/2-L508/6+L508^2/24-L508^3/120)</f>
         <v>0.466774002592</v>
       </c>
       <c r="P508" s="41">
@@ -36991,11 +37001,11 @@
         <v>0.957397897566</v>
       </c>
       <c r="E509" s="41">
-        <f>IF(C509&gt;0,(1-D509)/C509,1)</f>
+        <f>IF(C509&gt;x_series,(1-EXP(-C509))/C509,1-C509/2+C509^2/6-C509^3/24)</f>
         <v>0.978544392535</v>
       </c>
       <c r="F509" s="41">
-        <f>IF(C509&gt;0,(C509-1+D509)/C509^2,1/2)</f>
+        <f>IF(C509&gt;x_series,(C509-1+EXP(-C509))/C509^2,1/2-C509/6+C509^2/24-C509^3/120)</f>
         <v>0.492822259325</v>
       </c>
       <c r="G509" s="41">
@@ -37023,11 +37033,11 @@
         <v>0.790462357975</v>
       </c>
       <c r="N509" s="41">
-        <f>IF(L509&gt;0,(1-M509)/L509,1)</f>
+        <f>IF(L509&gt;x_series,(1-EXP(-L509))/L509,1-L509/2+L509^2/6-L509^3/24)</f>
         <v>0.891129115587</v>
       </c>
       <c r="O509" s="41">
-        <f>IF(L509&gt;0,(L509-1+M509)/L509^2,1/2)</f>
+        <f>IF(L509&gt;x_series,(L509-1+EXP(-L509))/L509^2,1/2-L509/6+L509^2/24-L509^3/120)</f>
         <v>0.463009958509</v>
       </c>
       <c r="P509" s="41">
@@ -37065,11 +37075,11 @@
         <v>0.952405409749</v>
       </c>
       <c r="E510" s="41">
-        <f>IF(C510&gt;0,(1-D510)/C510,1)</f>
+        <f>IF(C510&gt;x_series,(1-EXP(-C510))/C510,1-C510/2+C510^2/6-C510^3/24)</f>
         <v>0.976009302069</v>
       </c>
       <c r="F510" s="41">
-        <f>IF(C510&gt;0,(C510-1+D510)/C510^2,1/2)</f>
+        <f>IF(C510&gt;x_series,(C510-1+EXP(-C510))/C510^2,1/2-C510/6+C510^2/24-C510^3/120)</f>
         <v>0.491970709705</v>
       </c>
       <c r="G510" s="41">
@@ -37097,11 +37107,11 @@
         <v>0.768453670319</v>
       </c>
       <c r="N510" s="41">
-        <f>IF(L510&gt;0,(1-M510)/L510,1)</f>
+        <f>IF(L510&gt;x_series,(1-EXP(-L510))/L510,1-L510/2+L510^2/6-L510^3/24)</f>
         <v>0.879150741141</v>
       </c>
       <c r="O510" s="41">
-        <f>IF(L510&gt;0,(L510-1+M510)/L510^2,1/2)</f>
+        <f>IF(L510&gt;x_series,(L510-1+EXP(-L510))/L510^2,1/2-L510/6+L510^2/24-L510^3/120)</f>
         <v>0.458848627137</v>
       </c>
       <c r="P510" s="41">
@@ -37139,11 +37149,11 @@
         <v>0.94684440512</v>
       </c>
       <c r="E511" s="41">
-        <f>IF(C511&gt;0,(1-D511)/C511,1)</f>
+        <f>IF(C511&gt;x_series,(1-EXP(-C511))/C511,1-C511/2+C511^2/6-C511^3/24)</f>
         <v>0.973180265816</v>
       </c>
       <c r="F511" s="41">
-        <f>IF(C511&gt;0,(C511-1+D511)/C511^2,1/2)</f>
+        <f>IF(C511&gt;x_series,(C511-1+EXP(-C511))/C511^2,1/2-C511/6+C511^2/24-C511^3/120)</f>
         <v>0.491019545574</v>
       </c>
       <c r="G511" s="41">
@@ -37171,11 +37181,11 @@
         <v>0.744529264939</v>
       </c>
       <c r="N511" s="41">
-        <f>IF(L511&gt;0,(1-M511)/L511,1)</f>
+        <f>IF(L511&gt;x_series,(1-EXP(-L511))/L511,1-L511/2+L511^2/6-L511^3/24)</f>
         <v>0.865993334361</v>
       </c>
       <c r="O511" s="41">
-        <f>IF(L511&gt;0,(L511-1+M511)/L511^2,1/2)</f>
+        <f>IF(L511&gt;x_series,(L511-1+EXP(-L511))/L511^2,1/2-L511/6+L511^2/24-L511^3/120)</f>
         <v>0.454255080042</v>
       </c>
       <c r="P511" s="41">
@@ -37213,11 +37223,11 @@
         <v>0.940654264069</v>
       </c>
       <c r="E512" s="41">
-        <f>IF(C512&gt;0,(1-D512)/C512,1)</f>
+        <f>IF(C512&gt;x_series,(1-EXP(-C512))/C512,1-C512/2+C512^2/6-C512^3/24)</f>
         <v>0.970024588442</v>
       </c>
       <c r="F512" s="41">
-        <f>IF(C512&gt;0,(C512-1+D512)/C512^2,1/2)</f>
+        <f>IF(C512&gt;x_series,(C512-1+EXP(-C512))/C512^2,1/2-C512/6+C512^2/24-C512^3/120)</f>
         <v>0.489957463732</v>
       </c>
       <c r="G512" s="41">
@@ -37245,11 +37255,11 @@
         <v>0.718615632825</v>
       </c>
       <c r="N512" s="41">
-        <f>IF(L512&gt;0,(1-M512)/L512,1)</f>
+        <f>IF(L512&gt;x_series,(1-EXP(-L512))/L512,1-L512/2+L512^2/6-L512^3/24)</f>
         <v>0.851573757876</v>
       </c>
       <c r="O512" s="41">
-        <f>IF(L512&gt;0,(L512-1+M512)/L512^2,1/2)</f>
+        <f>IF(L512&gt;x_series,(L512-1+EXP(-L512))/L512^2,1/2-L512/6+L512^2/24-L512^3/120)</f>
         <v>0.449193016804</v>
       </c>
       <c r="P512" s="41">
@@ -37287,11 +37297,11 @@
         <v>0.9337689431</v>
       </c>
       <c r="E513" s="41">
-        <f>IF(C513&gt;0,(1-D513)/C513,1)</f>
+        <f>IF(C513&gt;x_series,(1-EXP(-C513))/C513,1-C513/2+C513^2/6-C513^3/24)</f>
         <v>0.966506287286</v>
       </c>
       <c r="F513" s="41">
-        <f>IF(C513&gt;0,(C513-1+D513)/C513^2,1/2)</f>
+        <f>IF(C513&gt;x_series,(C513-1+EXP(-C513))/C513^2,1/2-C513/6+C513^2/24-C513^3/120)</f>
         <v>0.488771966473</v>
       </c>
       <c r="G513" s="41">
@@ -37319,11 +37329,11 @@
         <v>0.690660059918</v>
       </c>
       <c r="N513" s="41">
-        <f>IF(L513&gt;0,(1-M513)/L513,1)</f>
+        <f>IF(L513&gt;x_series,(1-EXP(-L513))/L513,1-L513/2+L513^2/6-L513^3/24)</f>
         <v>0.835810987205</v>
       </c>
       <c r="O513" s="41">
-        <f>IF(L513&gt;0,(L513-1+M513)/L513^2,1/2)</f>
+        <f>IF(L513&gt;x_series,(L513-1+EXP(-L513))/L513^2,1/2-L513/6+L513^2/24-L513^3/120)</f>
         <v>0.443625161483</v>
       </c>
       <c r="P513" s="41">
@@ -37361,11 +37371,11 @@
         <v>0.926116760238</v>
       </c>
       <c r="E514" s="41">
-        <f>IF(C514&gt;0,(1-D514)/C514,1)</f>
+        <f>IF(C514&gt;x_series,(1-EXP(-C514))/C514,1-C514/2+C514^2/6-C514^3/24)</f>
         <v>0.96258585108</v>
       </c>
       <c r="F514" s="41">
-        <f>IF(C514&gt;0,(C514-1+D514)/C514^2,1/2)</f>
+        <f>IF(C514&gt;x_series,(C514-1+EXP(-C514))/C514^2,1/2-C514/6+C514^2/24-C514^3/120)</f>
         <v>0.48744925773</v>
       </c>
       <c r="G514" s="41">
@@ -37393,11 +37403,11 @@
         <v>0.660637212579</v>
       </c>
       <c r="N514" s="41">
-        <f>IF(L514&gt;0,(1-M514)/L514,1)</f>
+        <f>IF(L514&gt;x_series,(1-EXP(-L514))/L514,1-L514/2+L514^2/6-L514^3/24)</f>
         <v>0.818628465553</v>
       </c>
       <c r="O514" s="41">
-        <f>IF(L514&gt;0,(L514-1+M514)/L514^2,1/2)</f>
+        <f>IF(L514&gt;x_series,(L514-1+EXP(-L514))/L514^2,1/2-L514/6+L514^2/24-L514^3/120)</f>
         <v>0.437513794802</v>
       </c>
       <c r="P514" s="41">
@@ -37435,11 +37445,11 @@
         <v>0.917620252115</v>
       </c>
       <c r="E515" s="41">
-        <f>IF(C515&gt;0,(1-D515)/C515,1)</f>
+        <f>IF(C515&gt;x_series,(1-EXP(-C515))/C515,1-C515/2+C515^2/6-C515^3/24)</f>
         <v>0.958220005227</v>
       </c>
       <c r="F515" s="41">
-        <f>IF(C515&gt;0,(C515-1+D515)/C515^2,1/2)</f>
+        <f>IF(C515&gt;x_series,(C515-1+EXP(-C515))/C515^2,1/2-C515/6+C515^2/24-C515^3/120)</f>
         <v>0.485974136088</v>
       </c>
       <c r="G515" s="41">
@@ -37467,11 +37477,11 @@
         <v>0.62855649984</v>
       </c>
       <c r="N515" s="41">
-        <f>IF(L515&gt;0,(1-M515)/L515,1)</f>
+        <f>IF(L515&gt;x_series,(1-EXP(-L515))/L515,1-L515/2+L515^2/6-L515^3/24)</f>
         <v>0.79995695561</v>
       </c>
       <c r="O515" s="41">
-        <f>IF(L515&gt;0,(L515-1+M515)/L515^2,1/2)</f>
+        <f>IF(L515&gt;x_series,(L515-1+EXP(-L515))/L515^2,1/2-L515/6+L515^2/24-L515^3/120)</f>
         <v>0.430821443133</v>
       </c>
       <c r="P515" s="41">
@@ -37509,11 +37519,11 @@
         <v>0.908196130908</v>
       </c>
       <c r="E516" s="41">
-        <f>IF(C516&gt;0,(1-D516)/C516,1)</f>
+        <f>IF(C516&gt;x_series,(1-EXP(-C516))/C516,1-C516/2+C516^2/6-C516^3/24)</f>
         <v>0.953361492091</v>
       </c>
       <c r="F516" s="41">
-        <f>IF(C516&gt;0,(C516-1+D516)/C516^2,1/2)</f>
+        <f>IF(C516&gt;x_series,(C516-1+EXP(-C516))/C516^2,1/2-C516/6+C516^2/24-C516^3/120)</f>
         <v>0.48432988641</v>
       </c>
       <c r="G516" s="41">
@@ -37541,11 +37551,11 @@
         <v>0.594470037278</v>
       </c>
       <c r="N516" s="41">
-        <f>IF(L516&gt;0,(1-M516)/L516,1)</f>
+        <f>IF(L516&gt;x_series,(1-EXP(-L516))/L516,1-L516/2+L516^2/6-L516^3/24)</f>
         <v>0.779737909765</v>
       </c>
       <c r="O516" s="41">
-        <f>IF(L516&gt;0,(L516-1+M516)/L516^2,1/2)</f>
+        <f>IF(L516&gt;x_series,(L516-1+EXP(-L516))/L516^2,1/2-L516/6+L516^2/24-L516^3/120)</f>
         <v>0.423511744206</v>
       </c>
       <c r="P516" s="41">
@@ -37583,11 +37593,11 @@
         <v>0.897755375803</v>
       </c>
       <c r="E517" s="41">
-        <f>IF(C517&gt;0,(1-D517)/C517,1)</f>
+        <f>IF(C517&gt;x_series,(1-EXP(-C517))/C517,1-C517/2+C517^2/6-C517^3/24)</f>
         <v>0.947958877225</v>
       </c>
       <c r="F517" s="41">
-        <f>IF(C517&gt;0,(C517-1+D517)/C517^2,1/2)</f>
+        <f>IF(C517&gt;x_series,(C517-1+EXP(-C517))/C517^2,1/2-C517/6+C517^2/24-C517^3/120)</f>
         <v>0.48249817242</v>
       </c>
       <c r="G517" s="41">
@@ -37615,11 +37625,11 @@
         <v>0.558480911237</v>
       </c>
       <c r="N517" s="41">
-        <f>IF(L517&gt;0,(1-M517)/L517,1)</f>
+        <f>IF(L517&gt;x_series,(1-EXP(-L517))/L517,1-L517/2+L517^2/6-L517^3/24)</f>
         <v>0.75792735247</v>
       </c>
       <c r="O517" s="41">
-        <f>IF(L517&gt;0,(L517-1+M517)/L517^2,1/2)</f>
+        <f>IF(L517&gt;x_series,(L517-1+EXP(-L517))/L517^2,1/2-L517/6+L517^2/24-L517^3/120)</f>
         <v>0.415550506235</v>
       </c>
       <c r="P517" s="41">
@@ -37657,11 +37667,11 @@
         <v>0.886203500956</v>
       </c>
       <c r="E518" s="41">
-        <f>IF(C518&gt;0,(1-D518)/C518,1)</f>
+        <f>IF(C518&gt;x_series,(1-EXP(-C518))/C518,1-C518/2+C518^2/6-C518^3/24)</f>
         <v>0.941956395413</v>
       </c>
       <c r="F518" s="41">
-        <f>IF(C518&gt;0,(C518-1+D518)/C518^2,1/2)</f>
+        <f>IF(C518&gt;x_series,(C518-1+EXP(-C518))/C518^2,1/2-C518/6+C518^2/24-C518^3/120)</f>
         <v>0.480458933387</v>
       </c>
       <c r="G518" s="41">
@@ -37689,11 +37699,11 @@
         <v>0.52075128557</v>
       </c>
       <c r="N518" s="41">
-        <f>IF(L518&gt;0,(1-M518)/L518,1)</f>
+        <f>IF(L518&gt;x_series,(1-EXP(-L518))/L518,1-L518/2+L518^2/6-L518^3/24)</f>
         <v>0.73450022856</v>
       </c>
       <c r="O518" s="41">
-        <f>IF(L518&gt;0,(L518-1+M518)/L518^2,1/2)</f>
+        <f>IF(L518&gt;x_series,(L518-1+EXP(-L518))/L518^2,1/2-L518/6+L518^2/24-L518^3/120)</f>
         <v>0.406906971127</v>
       </c>
       <c r="P518" s="41">
@@ -37731,11 +37741,11 @@
         <v>0.87344105009</v>
       </c>
       <c r="E519" s="41">
-        <f>IF(C519&gt;0,(1-D519)/C519,1)</f>
+        <f>IF(C519&gt;x_series,(1-EXP(-C519))/C519,1-C519/2+C519^2/6-C519^3/24)</f>
         <v>0.935293853813</v>
       </c>
       <c r="F519" s="41">
-        <f>IF(C519&gt;0,(C519-1+D519)/C519^2,1/2)</f>
+        <f>IF(C519&gt;x_series,(C519-1+EXP(-C519))/C519^2,1/2-C519/6+C519^2/24-C519^3/120)</f>
         <v>0.478190288995</v>
       </c>
       <c r="G519" s="41">
@@ -37763,11 +37773,11 @@
         <v>0.481509710387</v>
       </c>
       <c r="N519" s="41">
-        <f>IF(L519&gt;0,(1-M519)/L519,1)</f>
+        <f>IF(L519&gt;x_series,(1-EXP(-L519))/L519,1-L519/2+L519^2/6-L519^3/24)</f>
         <v>0.709455117464</v>
       </c>
       <c r="O519" s="41">
-        <f>IF(L519&gt;0,(L519-1+M519)/L519^2,1/2)</f>
+        <f>IF(L519&gt;x_series,(L519-1+EXP(-L519))/L519^2,1/2-L519/6+L519^2/24-L519^3/120)</f>
         <v>0.3975552829</v>
       </c>
       <c r="P519" s="41">
@@ -37805,11 +37815,11 @@
         <v>0.859364376571</v>
       </c>
       <c r="E520" s="41">
-        <f>IF(C520&gt;0,(1-D520)/C520,1)</f>
+        <f>IF(C520&gt;x_series,(1-EXP(-C520))/C520,1-C520/2+C520^2/6-C520^3/24)</f>
         <v>0.927906613546</v>
       </c>
       <c r="F520" s="41">
-        <f>IF(C520&gt;0,(C520-1+D520)/C520^2,1/2)</f>
+        <f>IF(C520&gt;x_series,(C520-1+EXP(-C520))/C520^2,1/2-C520/6+C520^2/24-C520^3/120)</f>
         <v>0.475668457626</v>
       </c>
       <c r="G520" s="41">
@@ -37837,11 +37847,11 @@
         <v>0.441056794828</v>
       </c>
       <c r="N520" s="41">
-        <f>IF(L520&gt;0,(1-M520)/L520,1)</f>
+        <f>IF(L520&gt;x_series,(1-EXP(-L520))/L520,1-L520/2+L520^2/6-L520^3/24)</f>
         <v>0.682819144541</v>
       </c>
       <c r="O520" s="41">
-        <f>IF(L520&gt;0,(L520-1+M520)/L520^2,1/2)</f>
+        <f>IF(L520&gt;x_series,(L520-1+EXP(-L520))/L520^2,1/2-L520/6+L520^2/24-L520^3/120)</f>
         <v>0.387476148534</v>
       </c>
       <c r="P520" s="41">
@@ -37879,11 +37889,11 @@
         <v>0.84386677676</v>
       </c>
       <c r="E521" s="41">
-        <f>IF(C521&gt;0,(1-D521)/C521,1)</f>
+        <f>IF(C521&gt;x_series,(1-EXP(-C521))/C521,1-C521/2+C521^2/6-C521^3/24)</f>
         <v>0.919725675504</v>
       </c>
       <c r="F521" s="41">
-        <f>IF(C521&gt;0,(C521-1+D521)/C521^2,1/2)</f>
+        <f>IF(C521&gt;x_series,(C521-1+EXP(-C521))/C521^2,1/2-C521/6+C521^2/24-C521^3/120)</f>
         <v>0.472867694595</v>
       </c>
       <c r="G521" s="41">
@@ -37911,11 +37921,11 @@
         <v>0.399768215341</v>
       </c>
       <c r="N521" s="41">
-        <f>IF(L521&gt;0,(1-M521)/L521,1)</f>
+        <f>IF(L521&gt;x_series,(1-EXP(-L521))/L521,1-L521/2+L521^2/6-L521^3/24)</f>
         <v>0.654652838482</v>
       </c>
       <c r="O521" s="41">
-        <f>IF(L521&gt;0,(L521-1+M521)/L521^2,1/2)</f>
+        <f>IF(L521&gt;x_series,(L521-1+EXP(-L521))/L521^2,1/2-L521/6+L521^2/24-L521^3/120)</f>
         <v>0.376658659751</v>
       </c>
       <c r="P521" s="41">
@@ -37953,11 +37963,11 @@
         <v>0.826840052996</v>
       </c>
       <c r="E522" s="41">
-        <f>IF(C522&gt;0,(1-D522)/C522,1)</f>
+        <f>IF(C522&gt;x_series,(1-EXP(-C522))/C522,1-C522/2+C522^2/6-C522^3/24)</f>
         <v>0.910677901209</v>
       </c>
       <c r="F522" s="41">
-        <f>IF(C522&gt;0,(C522-1+D522)/C522^2,1/2)</f>
+        <f>IF(C522&gt;x_series,(C522-1+EXP(-C522))/C522^2,1/2-C522/6+C522^2/24-C522^3/120)</f>
         <v>0.469760258453</v>
       </c>
       <c r="G522" s="41">
@@ -37985,11 +37995,11 @@
         <v>0.358093881486</v>
       </c>
       <c r="N522" s="41">
-        <f>IF(L522&gt;0,(1-M522)/L522,1)</f>
+        <f>IF(L522&gt;x_series,(1-EXP(-L522))/L522,1-L522/2+L522^2/6-L522^3/24)</f>
         <v>0.625054591612</v>
       </c>
       <c r="O522" s="41">
-        <f>IF(L522&gt;0,(L522-1+M522)/L522^2,1/2)</f>
+        <f>IF(L522&gt;x_series,(L522-1+EXP(-L522))/L522^2,1/2-L522/6+L522^2/24-L522^3/120)</f>
         <v>0.365102220336</v>
       </c>
       <c r="P522" s="41">
@@ -38027,11 +38037,11 @@
         <v>0.808176589756</v>
       </c>
       <c r="E523" s="41">
-        <f>IF(C523&gt;0,(1-D523)/C523,1)</f>
+        <f>IF(C523&gt;x_series,(1-EXP(-C523))/C523,1-C523/2+C523^2/6-C523^3/24)</f>
         <v>0.900686404787</v>
       </c>
       <c r="F523" s="41">
-        <f>IF(C523&gt;0,(C523-1+D523)/C523^2,1/2)</f>
+        <f>IF(C523&gt;x_series,(C523-1+EXP(-C523))/C523^2,1/2-C523/6+C523^2/24-C523^3/120)</f>
         <v>0.466316415216</v>
       </c>
       <c r="G523" s="41">
@@ -38059,11 +38069,11 @@
         <v>0.31655202155</v>
       </c>
       <c r="N523" s="41">
-        <f>IF(L523&gt;0,(1-M523)/L523,1)</f>
+        <f>IF(L523&gt;x_series,(1-EXP(-L523))/L523,1-L523/2+L523^2/6-L523^3/24)</f>
         <v>0.594164286172</v>
       </c>
       <c r="O523" s="41">
-        <f>IF(L523&gt;0,(L523-1+M523)/L523^2,1/2)</f>
+        <f>IF(L523&gt;x_series,(L523-1+EXP(-L523))/L523^2,1/2-L523/6+L523^2/24-L523^3/120)</f>
         <v>0.352818495062</v>
       </c>
       <c r="P523" s="41">
@@ -38101,11 +38111,11 @@
         <v>0.787772031109</v>
       </c>
       <c r="E524" s="41">
-        <f>IF(C524&gt;0,(1-D524)/C524,1)</f>
+        <f>IF(C524&gt;x_series,(1-EXP(-C524))/C524,1-C524/2+C524^2/6-C524^3/24)</f>
         <v>0.88967115751</v>
       </c>
       <c r="F524" s="41">
-        <f>IF(C524&gt;0,(C524-1+D524)/C524^2,1/2)</f>
+        <f>IF(C524&gt;x_series,(C524-1+EXP(-C524))/C524^2,1/2-C524/6+C524^2/24-C524^3/120)</f>
         <v>0.462504492306</v>
       </c>
       <c r="G524" s="41">
@@ -38133,11 +38143,11 @@
         <v>0.275717041303</v>
       </c>
       <c r="N524" s="41">
-        <f>IF(L524&gt;0,(1-M524)/L524,1)</f>
+        <f>IF(L524&gt;x_series,(1-EXP(-L524))/L524,1-L524/2+L524^2/6-L524^3/24)</f>
         <v>0.562165567104</v>
       </c>
       <c r="O524" s="41">
-        <f>IF(L524&gt;0,(L524-1+M524)/L524^2,1/2)</f>
+        <f>IF(L524&gt;x_series,(L524-1+EXP(-L524))/L524^2,1/2-L524/6+L524^2/24-L524^3/120)</f>
         <v>0.339833264487</v>
       </c>
       <c r="P524" s="41">
@@ -38175,11 +38185,11 @@
         <v>0.765528647534</v>
       </c>
       <c r="E525" s="41">
-        <f>IF(C525&gt;0,(1-D525)/C525,1)</f>
+        <f>IF(C525&gt;x_series,(1-EXP(-C525))/C525,1-C525/2+C525^2/6-C525^3/24)</f>
         <v>0.877549851432</v>
       </c>
       <c r="F525" s="41">
-        <f>IF(C525&gt;0,(C525-1+D525)/C525^2,1/2)</f>
+        <f>IF(C525&gt;x_series,(C525-1+EXP(-C525))/C525^2,1/2-C525/6+C525^2/24-C525^3/120)</f>
         <v>0.458290996123</v>
       </c>
       <c r="G525" s="41">
@@ -38207,11 +38217,11 @@
         <v>0.236200318752</v>
       </c>
       <c r="N525" s="41">
-        <f>IF(L525&gt;0,(1-M525)/L525,1)</f>
+        <f>IF(L525&gt;x_series,(1-EXP(-L525))/L525,1-L525/2+L525^2/6-L525^3/24)</f>
         <v>0.529286189308</v>
       </c>
       <c r="O525" s="41">
-        <f>IF(L525&gt;0,(L525-1+M525)/L525^2,1/2)</f>
+        <f>IF(L525&gt;x_series,(L525-1+EXP(-L525))/L525^2,1/2-L525/6+L525^2/24-L525^3/120)</f>
         <v>0.326188037561</v>
       </c>
       <c r="P525" s="41">
@@ -38249,11 +38259,11 @@
         <v>0.741359473179</v>
       </c>
       <c r="E526" s="41">
-        <f>IF(C526&gt;0,(1-D526)/C526,1)</f>
+        <f>IF(C526&gt;x_series,(1-EXP(-C526))/C526,1-C526/2+C526^2/6-C526^3/24)</f>
         <v>0.864239072748</v>
       </c>
       <c r="F526" s="41">
-        <f>IF(C526&gt;0,(C526-1+D526)/C526^2,1/2)</f>
+        <f>IF(C526&gt;x_series,(C526-1+EXP(-C526))/C526^2,1/2-C526/6+C526^2/24-C526^3/120)</f>
         <v>0.453640809219</v>
       </c>
       <c r="G526" s="41">
@@ -38281,11 +38291,11 @@
         <v>0.198623686632</v>
       </c>
       <c r="N526" s="41">
-        <f>IF(L526&gt;0,(1-M526)/L526,1)</f>
+        <f>IF(L526&gt;x_series,(1-EXP(-L526))/L526,1-L526/2+L526^2/6-L526^3/24)</f>
         <v>0.495795868367</v>
       </c>
       <c r="O526" s="41">
-        <f>IF(L526&gt;0,(L526-1+M526)/L526^2,1/2)</f>
+        <f>IF(L526&gt;x_series,(L526-1+EXP(-L526))/L526^2,1/2-L526/6+L526^2/24-L526^3/120)</f>
         <v>0.311941245464</v>
       </c>
       <c r="P526" s="41">
@@ -38323,11 +38333,11 @@
         <v>0.715193277412</v>
       </c>
       <c r="E527" s="41">
-        <f>IF(C527&gt;0,(1-D527)/C527,1)</f>
+        <f>IF(C527&gt;x_series,(1-EXP(-C527))/C527,1-C527/2+C527^2/6-C527^3/24)</f>
         <v>0.849655837971</v>
       </c>
       <c r="F527" s="41">
-        <f>IF(C527&gt;0,(C527-1+D527)/C527^2,1/2)</f>
+        <f>IF(C527&gt;x_series,(C527-1+EXP(-C527))/C527^2,1/2-C527/6+C527^2/24-C527^3/120)</f>
         <v>0.448517485163</v>
       </c>
       <c r="G527" s="41">
@@ -38355,11 +38365,11 @@
         <v>0.163586254627</v>
       </c>
       <c r="N527" s="41">
-        <f>IF(L527&gt;0,(1-M527)/L527,1)</f>
+        <f>IF(L527&gt;x_series,(1-EXP(-L527))/L527,1-L527/2+L527^2/6-L527^3/24)</f>
         <v>0.462001144722</v>
       </c>
       <c r="O527" s="41">
-        <f>IF(L527&gt;0,(L527-1+M527)/L527^2,1/2)</f>
+        <f>IF(L527&gt;x_series,(L527-1+EXP(-L527))/L527^2,1/2-L527/6+L527^2/24-L527^3/120)</f>
         <v>0.297168821498</v>
       </c>
       <c r="P527" s="41">
@@ -38397,11 +38407,11 @@
         <v>0.686980403355</v>
       </c>
       <c r="E528" s="41">
-        <f>IF(C528&gt;0,(1-D528)/C528,1)</f>
+        <f>IF(C528&gt;x_series,(1-EXP(-C528))/C528,1-C528/2+C528^2/6-C528^3/24)</f>
         <v>0.833719545606</v>
       </c>
       <c r="F528" s="41">
-        <f>IF(C528&gt;0,(C528-1+D528)/C528^2,1/2)</f>
+        <f>IF(C528&gt;x_series,(C528-1+EXP(-C528))/C528^2,1/2-C528/6+C528^2/24-C528^3/120)</f>
         <v>0.442883660853</v>
       </c>
       <c r="G528" s="41">
@@ -38429,11 +38439,11 @@
         <v>0.131626409172</v>
       </c>
       <c r="N528" s="41">
-        <f>IF(L528&gt;0,(1-M528)/L528,1)</f>
+        <f>IF(L528&gt;x_series,(1-EXP(-L528))/L528,1-L528/2+L528^2/6-L528^3/24)</f>
         <v>0.42823695623</v>
       </c>
       <c r="O528" s="41">
-        <f>IF(L528&gt;0,(L528-1+M528)/L528^2,1/2)</f>
+        <f>IF(L528&gt;x_series,(L528-1+EXP(-L528))/L528^2,1/2-L528/6+L528^2/24-L528^3/120)</f>
         <v>0.281963970502</v>
       </c>
       <c r="P528" s="41">
@@ -38471,11 +38481,11 @@
         <v>0.656699456515</v>
       </c>
       <c r="E529" s="41">
-        <f>IF(C529&gt;0,(1-D529)/C529,1)</f>
+        <f>IF(C529&gt;x_series,(1-EXP(-C529))/C529,1-C529/2+C529^2/6-C529^3/24)</f>
         <v>0.816354391322</v>
       </c>
       <c r="F529" s="41">
-        <f>IF(C529&gt;0,(C529-1+D529)/C529^2,1/2)</f>
+        <f>IF(C529&gt;x_series,(C529-1+EXP(-C529))/C529^2,1/2-C529/6+C529^2/24-C529^3/120)</f>
         <v>0.436701607196</v>
       </c>
       <c r="G529" s="41">
@@ -38503,11 +38513,11 @@
         <v>0.103182183408</v>
       </c>
       <c r="N529" s="41">
-        <f>IF(L529&gt;0,(1-M529)/L529,1)</f>
+        <f>IF(L529&gt;x_series,(1-EXP(-L529))/L529,1-L529/2+L529^2/6-L529^3/24)</f>
         <v>0.394854917084</v>
       </c>
       <c r="O529" s="41">
-        <f>IF(L529&gt;0,(L529-1+M529)/L529^2,1/2)</f>
+        <f>IF(L529&gt;x_series,(L529-1+EXP(-L529))/L529^2,1/2-L529/6+L529^2/24-L529^3/120)</f>
         <v>0.266435955127</v>
       </c>
       <c r="P529" s="41">
@@ -38545,11 +38555,11 @@
         <v>0.624364754062</v>
       </c>
       <c r="E530" s="41">
-        <f>IF(C530&gt;0,(1-D530)/C530,1)</f>
+        <f>IF(C530&gt;x_series,(1-EXP(-C530))/C530,1-C530/2+C530^2/6-C530^3/24)</f>
         <v>0.797492283961</v>
       </c>
       <c r="F530" s="41">
-        <f>IF(C530&gt;0,(C530-1+D530)/C530^2,1/2)</f>
+        <f>IF(C530&gt;x_series,(C530-1+EXP(-C530))/C530^2,1/2-C530/6+C530^2/24-C530^3/120)</f>
         <v>0.429933939187</v>
       </c>
       <c r="G530" s="41">
@@ -38577,11 +38587,11 @@
         <v>0.07855448254</v>
       </c>
       <c r="N530" s="41">
-        <f>IF(L530&gt;0,(1-M530)/L530,1)</f>
+        <f>IF(L530&gt;x_series,(1-EXP(-L530))/L530,1-L530/2+L530^2/6-L530^3/24)</f>
         <v>0.362208716027</v>
       </c>
       <c r="O530" s="41">
-        <f>IF(L530&gt;0,(L530-1+M530)/L530^2,1/2)</f>
+        <f>IF(L530&gt;x_series,(L530-1+EXP(-L530))/L530^2,1/2-L530/6+L530^2/24-L530^3/120)</f>
         <v>0.250707782157</v>
       </c>
       <c r="P530" s="41">
@@ -38619,11 +38629,11 @@
         <v>0.590034345489</v>
       </c>
       <c r="E531" s="41">
-        <f>IF(C531&gt;0,(1-D531)/C531,1)</f>
+        <f>IF(C531&gt;x_series,(1-EXP(-C531))/C531,1-C531/2+C531^2/6-C531^3/24)</f>
         <v>0.777076280898</v>
       </c>
       <c r="F531" s="41">
-        <f>IF(C531&gt;0,(C531-1+D531)/C531^2,1/2)</f>
+        <f>IF(C531&gt;x_series,(C531-1+EXP(-C531))/C531^2,1/2-C531/6+C531^2/24-C531^3/120)</f>
         <v>0.422544505027</v>
       </c>
       <c r="G531" s="41">
@@ -38651,11 +38661,11 @@
         <v>0.057878536288</v>
       </c>
       <c r="N531" s="41">
-        <f>IF(L531&gt;0,(1-M531)/L531,1)</f>
+        <f>IF(L531&gt;x_series,(1-EXP(-L531))/L531,1-L531/2+L531^2/6-L531^3/24)</f>
         <v>0.330637537136</v>
       </c>
       <c r="O531" s="41">
-        <f>IF(L531&gt;0,(L531-1+M531)/L531^2,1/2)</f>
+        <f>IF(L531&gt;x_series,(L531-1+EXP(-L531))/L531^2,1/2-L531/6+L531^2/24-L531^3/120)</f>
         <v>0.234912763054</v>
       </c>
       <c r="P531" s="41">
@@ -38693,11 +38703,11 @@
         <v>0.55381828538</v>
       </c>
       <c r="E532" s="41">
-        <f>IF(C532&gt;0,(1-D532)/C532,1)</f>
+        <f>IF(C532&gt;x_series,(1-EXP(-C532))/C532,1-C532/2+C532^2/6-C532^3/24)</f>
         <v>0.755064532215</v>
       </c>
       <c r="F532" s="41">
-        <f>IF(C532&gt;0,(C532-1+D532)/C532^2,1/2)</f>
+        <f>IF(C532&gt;x_series,(C532-1+EXP(-C532))/C532^2,1/2-C532/6+C532^2/24-C532^3/120)</f>
         <v>0.414499470387</v>
       </c>
       <c r="G532" s="41">
@@ -38725,11 +38735,11 @@
         <v>0.041109021098</v>
       </c>
       <c r="N532" s="41">
-        <f>IF(L532&gt;0,(1-M532)/L532,1)</f>
+        <f>IF(L532&gt;x_series,(1-EXP(-L532))/L532,1-L532/2+L532^2/6-L532^3/24)</f>
         <v>0.300448898459</v>
       </c>
       <c r="O532" s="41">
-        <f>IF(L532&gt;0,(L532-1+M532)/L532^2,1/2)</f>
+        <f>IF(L532&gt;x_series,(L532-1+EXP(-L532))/L532^2,1/2-L532/6+L532^2/24-L532^3/120)</f>
         <v>0.219190046104</v>
       </c>
       <c r="P532" s="41">
@@ -38767,11 +38777,11 @@
         <v>0.515886678871</v>
       </c>
       <c r="E533" s="41">
-        <f>IF(C533&gt;0,(1-D533)/C533,1)</f>
+        <f>IF(C533&gt;x_series,(1-EXP(-C533))/C533,1-C533/2+C533^2/6-C533^3/24)</f>
         <v>0.731434681533</v>
       </c>
       <c r="F533" s="41">
-        <f>IF(C533&gt;0,(C533-1+D533)/C533^2,1/2)</f>
+        <f>IF(C533&gt;x_series,(C533-1+EXP(-C533))/C533^2,1/2-C533/6+C533^2/24-C533^3/120)</f>
         <v>0.405768607494</v>
       </c>
       <c r="G533" s="41">
@@ -38799,11 +38809,11 @@
         <v>0.028023185084</v>
       </c>
       <c r="N533" s="41">
-        <f>IF(L533&gt;0,(1-M533)/L533,1)</f>
+        <f>IF(L533&gt;x_series,(1-EXP(-L533))/L533,1-L533/2+L533^2/6-L533^3/24)</f>
         <v>0.271902688724</v>
       </c>
       <c r="O533" s="41">
-        <f>IF(L533&gt;0,(L533-1+M533)/L533^2,1/2)</f>
+        <f>IF(L533&gt;x_series,(L533-1+EXP(-L533))/L533^2,1/2-L533/6+L533^2/24-L533^3/120)</f>
         <v>0.203679361021</v>
       </c>
       <c r="P533" s="41">
@@ -38841,11 +38851,11 @@
         <v>0.476476834998</v>
       </c>
       <c r="E534" s="41">
-        <f>IF(C534&gt;0,(1-D534)/C534,1)</f>
+        <f>IF(C534&gt;x_series,(1-EXP(-C534))/C534,1-C534/2+C534^2/6-C534^3/24)</f>
         <v>0.706188615629</v>
       </c>
       <c r="F534" s="41">
-        <f>IF(C534&gt;0,(C534-1+D534)/C534^2,1/2)</f>
+        <f>IF(C534&gt;x_series,(C534-1+EXP(-C534))/C534^2,1/2-C534/6+C534^2/24-C534^3/120)</f>
         <v>0.396326788681</v>
       </c>
       <c r="G534" s="41">
@@ -38873,11 +38883,11 @@
         <v>0.01824386121</v>
       </c>
       <c r="N534" s="41">
-        <f>IF(L534&gt;0,(1-M534)/L534,1)</f>
+        <f>IF(L534&gt;x_series,(1-EXP(-L534))/L534,1-L534/2+L534^2/6-L534^3/24)</f>
         <v>0.245198334062</v>
       </c>
       <c r="O534" s="41">
-        <f>IF(L534&gt;0,(L534-1+M534)/L534^2,1/2)</f>
+        <f>IF(L534&gt;x_series,(L534-1+EXP(-L534))/L534^2,1/2-L534/6+L534^2/24-L534^3/120)</f>
         <v>0.188515359082</v>
       </c>
       <c r="P534" s="41">
@@ -38915,11 +38925,11 @@
         <v>0.435898665194</v>
       </c>
       <c r="E535" s="41">
-        <f>IF(C535&gt;0,(1-D535)/C535,1)</f>
+        <f>IF(C535&gt;x_series,(1-EXP(-C535))/C535,1-C535/2+C535^2/6-C535^3/24)</f>
         <v>0.679357384467</v>
       </c>
       <c r="F535" s="41">
-        <f>IF(C535&gt;0,(C535-1+D535)/C535^2,1/2)</f>
+        <f>IF(C535&gt;x_series,(C535-1+EXP(-C535))/C535^2,1/2-C535/6+C535^2/24-C535^3/120)</f>
         <v>0.386155669552</v>
       </c>
       <c r="G535" s="41">
@@ -38947,11 +38957,11 @@
         <v>0.011280696321</v>
       </c>
       <c r="N535" s="41">
-        <f>IF(L535&gt;0,(1-M535)/L535,1)</f>
+        <f>IF(L535&gt;x_series,(1-EXP(-L535))/L535,1-L535/2+L535^2/6-L535^3/24)</f>
         <v>0.220466834873</v>
       </c>
       <c r="O535" s="41">
-        <f>IF(L535&gt;0,(L535-1+M535)/L535^2,1/2)</f>
+        <f>IF(L535&gt;x_series,(L535-1+EXP(-L535))/L535^2,1/2-L535/6+L535^2/24-L535^3/120)</f>
         <v>0.173822043278</v>
       </c>
       <c r="P535" s="41">
@@ -38989,11 +38999,11 @@
         <v>0.39453727654</v>
       </c>
       <c r="E536" s="41">
-        <f>IF(C536&gt;0,(1-D536)/C536,1)</f>
+        <f>IF(C536&gt;x_series,(1-EXP(-C536))/C536,1-C536/2+C536^2/6-C536^3/24)</f>
         <v>0.651006029451</v>
       </c>
       <c r="F536" s="41">
-        <f>IF(C536&gt;0,(C536-1+D536)/C536^2,1/2)</f>
+        <f>IF(C536&gt;x_series,(C536-1+EXP(-C536))/C536^2,1/2-C536/6+C536^2/24-C536^3/120)</f>
         <v>0.375245527538</v>
       </c>
       <c r="G536" s="41">
@@ -39021,11 +39031,11 @@
         <v>0.006583970591</v>
       </c>
       <c r="N536" s="41">
-        <f>IF(L536&gt;0,(1-M536)/L536,1)</f>
+        <f>IF(L536&gt;x_series,(1-EXP(-L536))/L536,1-L536/2+L536^2/6-L536^3/24)</f>
         <v>0.197768830304</v>
       </c>
       <c r="O536" s="41">
-        <f>IF(L536&gt;0,(L536-1+M536)/L536^2,1/2)</f>
+        <f>IF(L536&gt;x_series,(L536-1+EXP(-L536))/L536^2,1/2-L536/6+L536^2/24-L536^3/120)</f>
         <v>0.159707831732</v>
       </c>
       <c r="P536" s="41">
@@ -39063,11 +39073,11 @@
         <v>0.352851568344</v>
       </c>
       <c r="E537" s="41">
-        <f>IF(C537&gt;0,(1-D537)/C537,1)</f>
+        <f>IF(C537&gt;x_series,(1-EXP(-C537))/C537,1-C537/2+C537^2/6-C537^3/24)</f>
         <v>0.62123796488</v>
       </c>
       <c r="F537" s="41">
-        <f>IF(C537&gt;0,(C537-1+D537)/C537^2,1/2)</f>
+        <f>IF(C537&gt;x_series,(C537-1+EXP(-C537))/C537^2,1/2-C537/6+C537^2/24-C537^3/120)</f>
         <v>0.363597197122</v>
       </c>
       <c r="G537" s="41">
@@ -39095,11 +39105,11 @@
         <v>0.003602160039</v>
       </c>
       <c r="N537" s="41">
-        <f>IF(L537&gt;0,(1-M537)/L537,1)</f>
+        <f>IF(L537&gt;x_series,(1-EXP(-L537))/L537,1-L537/2+L537^2/6-L537^3/24)</f>
         <v>0.177098932521</v>
       </c>
       <c r="O537" s="41">
-        <f>IF(L537&gt;0,(L537-1+M537)/L537^2,1/2)</f>
+        <f>IF(L537&gt;x_series,(L537-1+EXP(-L537))/L537^2,1/2-L537/6+L537^2/24-L537^3/120)</f>
         <v>0.146261758884</v>
       </c>
       <c r="P537" s="41">
@@ -39137,11 +39147,11 @@
         <v>0.311367596115</v>
       </c>
       <c r="E538" s="41">
-        <f>IF(C538&gt;0,(1-D538)/C538,1)</f>
+        <f>IF(C538&gt;x_series,(1-EXP(-C538))/C538,1-C538/2+C538^2/6-C538^3/24)</f>
         <v>0.590198464388</v>
       </c>
       <c r="F538" s="41">
-        <f>IF(C538&gt;0,(C538-1+D538)/C538^2,1/2)</f>
+        <f>IF(C538&gt;x_series,(C538-1+EXP(-C538))/C538^2,1/2-C538/6+C538^2/24-C538^3/120)</f>
         <v>0.351224013941</v>
       </c>
       <c r="G538" s="41">
@@ -39169,11 +39179,11 @@
         <v>0.001833117228</v>
       </c>
       <c r="N538" s="41">
-        <f>IF(L538&gt;0,(1-M538)/L538,1)</f>
+        <f>IF(L538&gt;x_series,(1-EXP(-L538))/L538,1-L538/2+L538^2/6-L538^3/24)</f>
         <v>0.158395506841</v>
       </c>
       <c r="O538" s="41">
-        <f>IF(L538&gt;0,(L538-1+M538)/L538^2,1/2)</f>
+        <f>IF(L538&gt;x_series,(L538-1+EXP(-L538))/L538^2,1/2-L538/6+L538^2/24-L538^3/120)</f>
         <v>0.133551185232</v>
       </c>
       <c r="P538" s="41">
@@ -39211,11 +39221,11 @@
         <v>0.270665581782</v>
       </c>
       <c r="E539" s="41">
-        <f>IF(C539&gt;0,(1-D539)/C539,1)</f>
+        <f>IF(C539&gt;x_series,(1-EXP(-C539))/C539,1-C539/2+C539^2/6-C539^3/24)</f>
         <v>0.55807672424</v>
       </c>
       <c r="F539" s="41">
-        <f>IF(C539&gt;0,(C539-1+D539)/C539^2,1/2)</f>
+        <f>IF(C539&gt;x_series,(C539-1+EXP(-C539))/C539^2,1/2-C539/6+C539^2/24-C539^3/120)</f>
         <v>0.338153647958</v>
       </c>
       <c r="G539" s="41">
@@ -39243,11 +39253,11 @@
         <v>0.0008601888562468</v>
       </c>
       <c r="N539" s="41">
-        <f>IF(L539&gt;0,(1-M539)/L539,1)</f>
+        <f>IF(L539&gt;x_series,(1-EXP(-L539))/L539,1-L539/2+L539^2/6-L539^3/24)</f>
         <v>0.141554130191</v>
       </c>
       <c r="O539" s="41">
-        <f>IF(L539&gt;0,(L539-1+M539)/L539^2,1/2)</f>
+        <f>IF(L539&gt;x_series,(L539-1+EXP(-L539))/L539^2,1/2-L539/6+L539^2/24-L539^3/120)</f>
         <v>0.121621175597</v>
       </c>
       <c r="P539" s="41">
@@ -39525,7 +39535,7 @@
         </is>
       </c>
       <c r="D551" s="41">
-        <f>IF(x_su&gt;0,(1-EXP(-x_su))/x_su,1)</f>
+        <f>IF(x_su&gt;x_series,(1-EXP(-x_su))/x_su,1-x_su/2+x_su^2/6-x_su^3/24)</f>
         <v>0.981632381646</v>
       </c>
       <c r="E551" s="51" t="inlineStr">
@@ -39551,7 +39561,7 @@
         </is>
       </c>
       <c r="D552" s="41">
-        <f>IF(x_su&gt;0,(x_su-1+EXP(-x_su))/x_su^2,1/2)</f>
+        <f>IF(x_su&gt;x_series,(x_su-1+EXP(-x_su))/x_su^2,1/2-x_su/6+x_su^2/24-x_su^3/120)</f>
         <v>0.49385853192</v>
       </c>
       <c r="E552" s="51" t="inlineStr">
@@ -39889,12 +39899,12 @@
         </is>
       </c>
       <c r="D566" s="41">
-        <f>IF(F_gap_g&gt;0,S_O2_g/F_gap_g+(y_O2_post_g-S_O2_g/F_gap_g)*IF(ABS((1/tau_L_h)-(F_gap_g/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_g/n_hs_gas))*(EXP(-(F_gap_g/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_g-S_O2_g/n_hs_gas/(1/tau_L_h)+S_O2_g/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
+        <f>y_O2_post_g*IF(ABS((1/tau_L_h)-(F_gap_g/n_hs_gas))&lt;=rate_tol_rel*(1/tau_L_h),((1/tau_L_h)*t_gap_h)*EXP(-((1/tau_L_h)*t_gap_h)),(1/tau_L_h)/((1/tau_L_h)-(F_gap_g/n_hs_gas))*(EXP(-((F_gap_g/n_hs_gas)*t_gap_h))-EXP(-((1/tau_L_h)*t_gap_h))))/(1-EXP(-((1/tau_L_h)*t_gap_h)))+S_O2_g/n_hs_gas*IF(ABS((1/tau_L_h)-(F_gap_g/n_hs_gas))&lt;=rate_tol_rel*(1/tau_L_h),(1-(1+((1/tau_L_h)*t_gap_h))*EXP(-((1/tau_L_h)*t_gap_h)))/(1/tau_L_h),(((1/tau_L_h)*t_gap_h)*IF(((F_gap_g/n_hs_gas)*t_gap_h)&gt;x_series,(1-EXP(-((F_gap_g/n_hs_gas)*t_gap_h)))/((F_gap_g/n_hs_gas)*t_gap_h),1-((F_gap_g/n_hs_gas)*t_gap_h)/2+((F_gap_g/n_hs_gas)*t_gap_h)^2/6-((F_gap_g/n_hs_gas)*t_gap_h)^3/24)-(1-EXP(-((1/tau_L_h)*t_gap_h))))/((1/tau_L_h)-(F_gap_g/n_hs_gas)))/(1-EXP(-((1/tau_L_h)*t_gap_h)))</f>
         <v>0.035988377729</v>
       </c>
       <c r="E566" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exact periodic solution of the first-order liquid (rate 1/τ, D326) driven by the exponential headspace ramp of the gap (from y_O2_post to S/F at rate F/n), maximal just before a pulse. Replaces the quasi-steady lag correction, which over-trusted gaps comparable to τ.</t>
+          <t xml:space="preserve">Exact periodic solution of the first-order liquid (rate b = 1/τ, D326) driven by the headspace ramp of the gap, y = y_post·e^(−at) + (S/F)(1 − e^(−at)) with a = F/n, maximal just before a pulse: z = y_post·G + (S/n)·H, with H = (bT·Φ(aT) − (1 − e^(−bT)))/((b − a)(1 − e^(−bT))). Written this way it stays exact as the vent flow F → 0 (no S/F terms to cancel); the coincident-rate limit (D569) is used when a = b.</t>
         </is>
       </c>
     </row>
@@ -39915,7 +39925,7 @@
         </is>
       </c>
       <c r="D567" s="41">
-        <f>IF(F_gap_l&gt;0,S_O2_l/F_gap_l+(y_O2_post_l-S_O2_l/F_gap_l)*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-(F_gap_l/n_hs_gas)*t_gap_h)-EXP(-(1/tau_L_h)*t_gap_h)),(1/tau_L_h)*t_gap_h*EXP(-(1/tau_L_h)*t_gap_h))/(1-EXP(-(1/tau_L_h)*t_gap_h)),y_O2_post_l-S_O2_l/n_hs_gas/(1/tau_L_h)+S_O2_l/n_hs_gas*t_gap_h/(1-EXP(-(1/tau_L_h)*t_gap_h)))</f>
+        <f>y_O2_post_l*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&lt;=rate_tol_rel*(1/tau_L_h),((1/tau_L_h)*t_gap_h)*EXP(-((1/tau_L_h)*t_gap_h)),(1/tau_L_h)/((1/tau_L_h)-(F_gap_l/n_hs_gas))*(EXP(-((F_gap_l/n_hs_gas)*t_gap_h))-EXP(-((1/tau_L_h)*t_gap_h))))/(1-EXP(-((1/tau_L_h)*t_gap_h)))+S_O2_l/n_hs_gas*IF(ABS((1/tau_L_h)-(F_gap_l/n_hs_gas))&lt;=rate_tol_rel*(1/tau_L_h),(1-(1+((1/tau_L_h)*t_gap_h))*EXP(-((1/tau_L_h)*t_gap_h)))/(1/tau_L_h),(((1/tau_L_h)*t_gap_h)*IF(((F_gap_l/n_hs_gas)*t_gap_h)&gt;x_series,(1-EXP(-((F_gap_l/n_hs_gas)*t_gap_h)))/((F_gap_l/n_hs_gas)*t_gap_h),1-((F_gap_l/n_hs_gas)*t_gap_h)/2+((F_gap_l/n_hs_gas)*t_gap_h)^2/6-((F_gap_l/n_hs_gas)*t_gap_h)^3/24)-(1-EXP(-((1/tau_L_h)*t_gap_h))))/((1/tau_L_h)-(F_gap_l/n_hs_gas)))/(1-EXP(-((1/tau_L_h)*t_gap_h)))</f>
         <v>0.070079461273</v>
       </c>
       <c r="E567" s="51" t="inlineStr">
@@ -39941,7 +39951,7 @@
         </is>
       </c>
       <c r="D568" s="41">
-        <f>IF(F_gap_su&gt;0,S_O2_su/F_gap_su+(y_O2_end_su*flush_ret-S_O2_su/F_gap_su)*IF(ABS((1/tau_L_h)-(F_gap_su/n_hs_gas))&gt;rate_tol_rel*(1/tau_L_h),(1/tau_L_h)/((1/tau_L_h)-(F_gap_su/n_hs_gas))*(EXP(-(F_gap_su/n_hs_gas)*t_gap_su_h)-EXP(-(1/tau_L_h)*t_gap_su_h)),(1/tau_L_h)*t_gap_su_h*EXP(-(1/tau_L_h)*t_gap_su_h))/(1-EXP(-(1/tau_L_h)*t_gap_su_h)),y_O2_end_su*flush_ret-S_O2_su/n_hs_gas/(1/tau_L_h)+S_O2_su/n_hs_gas*t_gap_su_h/(1-EXP(-(1/tau_L_h)*t_gap_su_h)))</f>
+        <f>y_O2_end_su*flush_ret*IF(ABS((1/tau_L_h)-(F_gap_su/n_hs_gas))&lt;=rate_tol_rel*(1/tau_L_h),((1/tau_L_h)*t_gap_su_h)*EXP(-((1/tau_L_h)*t_gap_su_h)),(1/tau_L_h)/((1/tau_L_h)-(F_gap_su/n_hs_gas))*(EXP(-((F_gap_su/n_hs_gas)*t_gap_su_h))-EXP(-((1/tau_L_h)*t_gap_su_h))))/(1-EXP(-((1/tau_L_h)*t_gap_su_h)))+S_O2_su/n_hs_gas*IF(ABS((1/tau_L_h)-(F_gap_su/n_hs_gas))&lt;=rate_tol_rel*(1/tau_L_h),(1-(1+((1/tau_L_h)*t_gap_su_h))*EXP(-((1/tau_L_h)*t_gap_su_h)))/(1/tau_L_h),(((1/tau_L_h)*t_gap_su_h)*IF(((F_gap_su/n_hs_gas)*t_gap_su_h)&gt;x_series,(1-EXP(-((F_gap_su/n_hs_gas)*t_gap_su_h)))/((F_gap_su/n_hs_gas)*t_gap_su_h),1-((F_gap_su/n_hs_gas)*t_gap_su_h)/2+((F_gap_su/n_hs_gas)*t_gap_su_h)^2/6-((F_gap_su/n_hs_gas)*t_gap_su_h)^3/24)-(1-EXP(-((1/tau_L_h)*t_gap_su_h))))/((1/tau_L_h)-(F_gap_su/n_hs_gas)))/(1-EXP(-((1/tau_L_h)*t_gap_su_h)))</f>
         <v>0.012412137716</v>
       </c>
       <c r="E568" s="51" t="inlineStr">
@@ -40336,6 +40346,31 @@
       <c r="E583" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">As D89 on the larger of its guard source and the start-up source (D572).</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Small-argument switch for Φ and Ψ (numerical)</t>
+        </is>
+      </c>
+      <c r="B584" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x_series</t>
+        </is>
+      </c>
+      <c r="C584" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D584" s="106">
+        <v>0.001</v>
+      </c>
+      <c r="E584" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Numerical, not a datum: below this x the exponential helpers Φ(x) = (1 − e^−x)/x and Ψ(x) = (x − 1 + e^−x)/x² (D333–D334, D355–D356, D377–D378, D551–D552, the grid columns E, F, N, O and D566–D568) use their Taylor series to x³, which are exact to ~1e-13 there, instead of the closed forms, which lose all precision as x → 0 (a near-zero vent flow).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gas model: thirteenth Codex review fixes (wrap every long Summary note, Graphite rod in both companions)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WrwcPcmd18tNqAYZEEZ7MY
</commit_message>
<xml_diff>
--- a/Media/electroPioreactorGasModel.xlsx
+++ b/Media/electroPioreactorGasModel.xlsx
@@ -10368,7 +10368,7 @@
     <xf numFmtId="0" fontId="26" fillId="17" borderId="11"/>
     <xf numFmtId="44" fontId="49" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="183">
+  <cellXfs count="189">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="45" fillId="21" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -10640,6 +10640,24 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="50" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -11388,7 +11406,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A6" s="21" t="s">
         <v>1142</v>
       </c>
@@ -11404,7 +11422,7 @@
       <c r="E6" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="22" t="inlineStr">
+      <c r="F6" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">LED channel D %, the AEP-Plugin 'electrolysis_power' setting (runtime-clamped 0–10 %); drives the electrolysis current via Gerrit's Law. The model needs 3–10 % (fit range ∩ plugin clamp), which the D6 validation enforces.</t>
         </is>
@@ -11486,7 +11504,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2" ht="92" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">Vent model</t>
@@ -11504,13 +11522,13 @@
       <c r="E11" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="22" t="inlineStr">
+      <c r="F11" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">"Outflow only" = check valve or sealed cap that holds a vacuum (no air ever enters). "Open vent" = a plain needle or tube with no forced flow (air drawn back after each pulse; Q_backdraw, Mass Transfer D385, an estimate). "Air exchange" = measured bidirectional exchange at Q_vent (Mass Transfer D142). The MEP0.3 and AEP0.1.1 caps vent through 2 × 1/16" ID tubes to 0.2 µm PTFE filters, AEP0.2 through needles to the same filters, with no check valve: Open vent (owner, T5). Anything else → #N/A throughout.</t>
         </is>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2" ht="77" customHeight="1">
       <c r="A12" s="18" t="s">
         <v>1795</v>
       </c>
@@ -11526,13 +11544,13 @@
       <c r="E12" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F12" s="22" t="inlineStr">
+      <c r="F12" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">"Growth" sizes the headline schedule (rows 18–21) on the O₂ surplus after knallgas uptake; "Lag" on the whole net electrolytic O₂ plus H₂ (no uptake yet). Anything else → #N/A. Both phases are shown either way, and the start-up schedule (rows 31 and 33) is always the lag one. If the chosen phase’s DO target is unreachable (rows 65–66), the schedule falls back to the legacy O₂ flush guard (Mass Transfer D89).</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="62" customHeight="1">
       <c r="A13" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">Added NaHCO₃ (on top of the recipe)</t>
@@ -11554,13 +11572,13 @@
           <t xml:space="preserve">input/blank</t>
         </is>
       </c>
-      <c r="F13" s="22" t="inlineStr">
+      <c r="F13" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">NaHCO₃ added to the medium; blank = none. It feeds the charge balance, ionic strength, conductivity and CO₂ storage (Chemistry D44, D185, D180, D296), so pH, DO and the schedule respond. Row 80 then shows what is still needed. After a large addition (pH up by more than 0.1) re-enter the DIC reference pH, Chemistry D291 (D310 says when).</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="62" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">N₂ dose (mean flow of timed pulses)</t>
@@ -11582,13 +11600,13 @@
           <t xml:space="preserve">input/blank</t>
         </is>
       </c>
-      <c r="F14" s="22" t="inlineStr">
+      <c r="F14" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Blank = none, the owner’s preference: fix the medium first (rows 80–81). If N₂ must be used it is pulsed apart from the CO₂ pulses (owner, T7); the balance takes its mean flow as an inert inflow with no O₂ or CO₂ (Mass Transfer D424–D425), exact for the mean-field fractions; the sawtooth of a separate N₂ flush is a model improvement (row 135).</t>
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="47" customHeight="1">
       <c r="A15" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">Solenoid command resolution</t>
@@ -11612,7 +11630,7 @@
           <t xml:space="preserve">input</t>
         </is>
       </c>
-      <c r="F15" s="22" t="inlineStr">
+      <c r="F15" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Smallest step the AEP-Plugin solenoid timer is commanded in; the pulse is rounded to it (row 19). Same solenoid as ed04, whose logged pulses (0.2, 0.25, 0.4, 0.6 s) are all 0.05 s multiples (owner, T8).</t>
         </is>
@@ -11664,7 +11682,7 @@
       </c>
       <c r="G18" s="136"/>
     </row>
-    <row r="19" spans="1:7" s="4" customFormat="1" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" s="4" customFormat="1" thickBot="1" x14ac:dyDescent="0.25" ht="32" customHeight="1">
       <c r="A19" s="25" t="s">
         <v>1710</v>
       </c>
@@ -11682,13 +11700,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D121","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F19" s="57" t="inlineStr">
+      <c r="F19" s="184" t="inlineStr">
         <is>
           <t xml:space="preserve">Pulse actually evaluated by every operating check below. Summary override wins, then Manual mode, otherwise the optimum rounded to the pulse resolution.</t>
         </is>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" thickBot="1" x14ac:dyDescent="0.25" ht="47" customHeight="1">
       <c r="A20" s="64" t="str">
         <f>"CO₂ sparge interval ("&amp;vent_model_sel&amp;", sized on "&amp;O2_phase_sel&amp;")"</f>
         <v>CO₂ sparge interval (Open vent, sized on Growth)</v>
@@ -11707,14 +11725,14 @@
         <f>HYPERLINK("#'Mass Transfer'!D91","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F20" s="22" t="inlineStr">
+      <c r="F20" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Time between doses: the shortest of the carbon-limited, headspace-O₂-dilution and pH-ceiling intervals (rows 28–30), plus the H₂ flammability screen when the schedule is sized on Lag (row 12); row 22 says which binds. Sized for the vent model in row 11 and the pulse in row 19.</t>
         </is>
       </c>
       <c r="G20" s="136"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A21" s="25" t="s">
         <v>1715</v>
       </c>
@@ -11732,13 +11750,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D122","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F21" s="22" t="inlineStr">
+      <c r="F21" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Interval actually evaluated below, in decimal minutes. Default converts the commanded pulse to the ideal delivery duty and rounds down to 0.01 min; overrides and Manual mode are evaluated directly.</t>
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="47" customHeight="1">
       <c r="A22" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve">Binding constraint on the interval</t>
@@ -11757,13 +11775,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D94","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="F22" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Which upper bound sets row 20: carbon supply, headspace-O₂ dilution, the pH ceiling (rows 28–30) or, when sized on Lag, the H₂ flammability screen; an invalid selector or an unreachable target is named here instead.</t>
         </is>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" thickBot="1" x14ac:dyDescent="0.25" ht="62" customHeight="1">
       <c r="A23" s="64" t="s">
         <v>1744</v>
       </c>
@@ -11779,13 +11797,13 @@
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F23" s="22" t="inlineStr">
+      <c r="F23" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">pH at the cycle-average dissolved CO₂ of the schedule in use, on the activity scale a probe reads; the trough just after a pulse is lower. Colour: green inside the HOB band (Chemistry pH_band_lo–pH_band_hi), red outside pH_red_lo–pH_red_hi (Chemistry D299–D300), amber between; thresholds in rows 159–162.</t>
         </is>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A24" s="64" t="s">
         <v>1749</v>
       </c>
@@ -11803,7 +11821,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D108","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F24" s="22" t="inlineStr">
+      <c r="F24" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Time-mean dissolved O₂ of the sawtooth model at the schedule in use, on the sizing phase; near the target by construction when O₂ dilution binds. Both phases, mean and peak: rows 59–62.</t>
         </is>
@@ -11827,7 +11845,7 @@
         <f>HYPERLINK("#Chemistry!D226","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F25" s="180" t="str">
+      <c r="F25" s="185" t="str">
         <f>IF(Chemistry!Cl_model_check&lt;&gt;"OK",Chemistry!Cl_model_check,"Effective chlorine on the as-Cl2 basis; zero for chloride-free medium. Lifetime and potency require measurement.")</f>
         <v>Effective chlorine on the as-Cl2 basis; zero for chloride-free medium. Lifetime and potency require measurement.</v>
       </c>
@@ -11839,7 +11857,7 @@
         </is>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A28" s="64" t="s">
         <v>1752</v>
       </c>
@@ -11857,11 +11875,11 @@
         <f>HYPERLINK("#'Mass Transfer'!D112","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F28" s="183" t="s">
         <v>1754</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="32" customHeight="1">
       <c r="A29" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve">DO-limited sparge interval</t>
@@ -11885,13 +11903,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D185","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F29" s="22" t="inlineStr">
+      <c r="F29" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Longest interval that still dilutes headspace O₂ enough to hold the DO target on the sizing phase (row 12). #N/A = the target is unreachable at this surface kLa.</t>
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="62" customHeight="1">
       <c r="A30" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve">pH-ceiling interval (longest keeping pH at or under the band ceiling)</t>
@@ -11915,13 +11933,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D432","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F30" s="22" t="inlineStr">
+      <c r="F30" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Longest interval keeping pH at or under the band ceiling, for the pulse in use. Far above the other bounds, or "no pH bound", unless N₂ dilutes the headspace; then it stops pH overshooting the band once CO₂ no longer has to dilute O₂. Row 55 warns if a long interval lets the carbon pool run dry.</t>
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="92" customHeight="1">
       <c r="A31" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve">Start-up (lag-phase) interval, same pulse</t>
@@ -11945,13 +11963,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D547","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F31" s="22" t="inlineStr">
+      <c r="F31" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Owner asked for both schedules (T4). Until uptake starts: the shortest of the lag O₂ bound (the legacy guard when the lag DO target is unreachable), the interval clearing the start-up hazard screen (Mass Transfer D581), the lag pH ceiling and the carbon bound. Sized on Growth it assumes no cathodic O₂ loss, an upper bound on the lag O₂ and H₂ sources, because the start-up DO differs from the lag reference (Electrochemistry D129); select Lag in row 12 to size and evaluate every output on the lag phase itself.</t>
         </is>
       </c>
     </row>
-    <row r="32" x14ac:dyDescent="0.2">
+    <row r="32" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A32" s="64" t="s">
         <v>1788</v>
       </c>
@@ -11971,7 +11989,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D93","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F32" s="22" t="inlineStr">
+      <c r="F32" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Delivered CO₂ duty of the schedule as run (rows 19 and 21) against the sized duty; 1 = rounding the interval has not moved the CO₂ dose. The sizing already uses the commanded pulse (Mass Transfer D320), so a ratio near 1 also means the DO target holds.</t>
         </is>
@@ -11996,7 +12014,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D556","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F33" s="22" t="inlineStr">
+      <c r="F33" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">The lag sawtooth at the start-up interval, on start-up sources that assume no cathodic O₂ loss (Mass Transfer D572) unless the schedule is sized on Lag; rows 61–62 show the lag phase at the headline schedule instead.</t>
         </is>
@@ -12018,7 +12036,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A35" s="64" t="s">
         <v>63</v>
       </c>
@@ -12034,7 +12052,7 @@
         <f>HYPERLINK("#Geometry!D90","→ Geometry")</f>
         <v>→ Geometry</v>
       </c>
-      <c r="F35" s="22" t="inlineStr">
+      <c r="F35" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Red until the vial headspace is measured (vial-geometry.md); while red, the pulse above is provisional (~4x uncertain). Once a headspace and its working fill are included on the Calibrations tab it reads OK, because the measured headspace replaces the cylinder approximation.</t>
         </is>
@@ -12056,11 +12074,11 @@
         <f>HYPERLINK("#'Mass Transfer'!D120","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F36" s="181" t="s">
+      <c r="F36" s="186" t="s">
         <v>1720</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2" ht="62" customHeight="1">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2" ht="77" customHeight="1">
       <c r="A37" s="64" t="s">
         <v>1721</v>
       </c>
@@ -12076,7 +12094,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D374","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F37" s="181" t="s">
+      <c r="F37" s="186" t="s">
         <v>1723</v>
       </c>
     </row>
@@ -12116,7 +12134,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D113","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F39" s="181" t="s">
+      <c r="F39" s="186" t="s">
         <v>1727</v>
       </c>
     </row>
@@ -12136,7 +12154,7 @@
         <f>HYPERLINK("#Biology!D44","→ Biology")</f>
         <v>→ Biology</v>
       </c>
-      <c r="F40" s="22" t="inlineStr">
+      <c r="F40" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Nominal lag-phase hazard screen, not safety certification. Predictions depend on unmeasured vent/transfer behaviour; validate mixture-specific limits, sampling and gas clearance before operation.</t>
         </is>
@@ -12158,7 +12176,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D64","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F41" s="181" t="s">
+      <c r="F41" s="186" t="s">
         <v>68</v>
       </c>
     </row>
@@ -12178,7 +12196,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D126","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F42" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Ratio of CO₂ delivered to carbon demand (should be ≥ 1), with the absorbed ratio beside it (row 77): delivered counts gas the pulse expels unabsorbed, absorbed does not.</t>
         </is>
@@ -12200,7 +12218,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D130","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F43" s="181" t="s">
+      <c r="F43" s="186" t="s">
         <v>1735</v>
       </c>
     </row>
@@ -12224,7 +12242,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A45" s="64" t="s">
         <v>73</v>
       </c>
@@ -12240,7 +12258,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D59","→ Mass")</f>
         <v>→ Mass</v>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F45" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Pulse flow against the measured no-carryover maximum for this reactor (CO2 flows column M). Reads "not measured" (amber) until one is recorded; the superficial-velocity rule of thumb is row 51.</t>
         </is>
@@ -12342,7 +12360,7 @@
         <f>HYPERLINK("#Biology!D45","→ Biology")</f>
         <v>→ Biology</v>
       </c>
-      <c r="F50" s="181" t="s">
+      <c r="F50" s="186" t="s">
         <v>898</v>
       </c>
     </row>
@@ -12361,13 +12379,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D414","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F51" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Secondary to row 45: gas velocity against the provisional 50 mm/s entrainment rule of thumb. It cannot fail at bench flows; row 45 tests the measured limit.</t>
         </is>
       </c>
     </row>
-    <row r="52" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="52" x14ac:dyDescent="0.2" ht="92" customHeight="1">
       <c r="A52" s="64" t="s">
         <v>1827</v>
       </c>
@@ -12384,7 +12402,7 @@
         <f>HYPERLINK("#Chemistry!D220","→ Chemistry")</f>
         <v>→ Chemistry</v>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F52" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">The vent model couples the two: when O₂ dilution binds, CO₂ is doing the O₂ dilution, so the DO-limited interval sets the pH (row 22 says which bound binds). Tests both band edges (rows 160–161) at the evaluated schedule, including any override in G18/G20. Red = the two targets conflict: fix the medium (rows 80–81) or measure the vent. Amber "watch" = the DIC or lag-DO reference needs re-entering first (Chemistry D310, Electrochemistry D134). #N/A = a selector (D2–D5, D11, D12) is not a listed value.</t>
         </is>
@@ -12410,11 +12428,11 @@
         <f>HYPERLINK("#'Mass Transfer'!D389","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F53" s="181" t="s">
+      <c r="F53" s="186" t="s">
         <v>1830</v>
       </c>
     </row>
-    <row r="54" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="54" x14ac:dyDescent="0.2" ht="62" customHeight="1">
       <c r="A54" s="64" t="s">
         <v>1831</v>
       </c>
@@ -12431,13 +12449,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D391","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F54" s="22" t="inlineStr">
+      <c r="F54" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">"HEADSPACE SAGS" = the check-valve model needs more vacuum than a real cap holds: switch D11 to Open vent or Air exchange. With an open vent or air exchange it reads UNVERIFIED, because the air ingress is assumed until the vent back-draw is measured (row 121); OK when an N₂ dose covers the per-cycle deficit.</t>
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="32" customHeight="1">
       <c r="A55" s="64" t="inlineStr">
         <is>
           <t xml:space="preserve">Carbon pool stays above air equilibrium through the cycle?</t>
@@ -12456,7 +12474,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D435","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F55" s="22" t="inlineStr">
+      <c r="F55" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Pulse-start dissolved CO₂ against air equilibrium at the schedule in use; WATCH = fixation empties the pool within the cycle (only reachable with a long, N₂-relaxed interval).</t>
         </is>
@@ -12469,7 +12487,7 @@
         </is>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A58" s="64" t="s">
         <v>1799</v>
       </c>
@@ -12484,7 +12502,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D386","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F58" s="22" t="inlineStr">
+      <c r="F58" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">0 for "Outflow only"; Q_backdraw (Mass Transfer D385, an estimate) for "Open vent"; the measured Q_vent (Mass Transfer D142) for "Air exchange". The single number that reconciles the O₂, CO₂ and flammability blocks — measure it.</t>
         </is>
@@ -12543,7 +12561,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D364","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F61" s="181" t="s">
+      <c r="F61" s="186" t="s">
         <v>1806</v>
       </c>
     </row>
@@ -12566,7 +12584,7 @@
         <v>1808</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A63" s="64" t="s">
         <v>1809</v>
       </c>
@@ -12578,13 +12596,13 @@
         <f>HYPERLINK("#'Mass Transfer'!D348","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F63" s="22" t="inlineStr">
+      <c r="F63" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Red = the growth-phase sawtooth peaks above the organism’s inhibition limit: its toxic DO when known, otherwise the 0.30 atm ceiling (Mass Transfer D565).</t>
         </is>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
       <c r="A64" s="64" t="s">
         <v>1811</v>
       </c>
@@ -12596,7 +12614,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D369","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F64" s="22" t="inlineStr">
+      <c r="F64" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Red = the lag-phase peak breaches that limit at the schedule in use; the culture would then be inhibited before it can take up O₂ (Mass Transfer D565).</t>
         </is>
@@ -12630,7 +12648,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D368","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F66" s="182" t="str">
+      <c r="F66" s="187" t="str">
         <f>"Same on the lag source. Currently "&amp;TEXT('Mass Transfer'!kLa_margin_l,"0.00")&amp;"×: "&amp;IF('Mass Transfer'!kLa_margin_l&lt;1,"the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).","the target can be held during lag at the kLa in use.")</f>
         <v>Same on the lag source. Currently 0.61×: the target cannot be held during lag at the kLa in use, whatever the schedule — an owner decision (target the ceiling with a margin during lag?).</v>
       </c>
@@ -12650,7 +12668,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D345","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F67" s="181" t="s">
+      <c r="F67" s="186" t="s">
         <v>1817</v>
       </c>
     </row>
@@ -12669,7 +12687,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D366","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F68" s="181" t="s">
+      <c r="F68" s="186" t="s">
         <v>1817</v>
       </c>
     </row>
@@ -12732,7 +12750,7 @@
         <v>1824</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2" ht="32" customHeight="1">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A72" s="64" t="s">
         <v>1825</v>
       </c>
@@ -12747,7 +12765,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D381","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F72" s="181" t="s">
+      <c r="F72" s="186" t="s">
         <v>1826</v>
       </c>
     </row>
@@ -12783,7 +12801,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A76" s="64" t="s">
         <v>1756</v>
       </c>
@@ -12801,13 +12819,13 @@
         <f>HYPERLINK("#Biology!D98","→ Biology")</f>
         <v>→ Biology</v>
       </c>
-      <c r="F76" s="22" t="inlineStr">
+      <c r="F76" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Dissolved CO₂ at the lowest point of the dosing cycle vs RuBisCO Km (was the in-sparge saturation peak, which a sub-second pulse never reaches); large = ample carbon. Complements the supply:demand ratio (D42).</t>
         </is>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A77" s="64" t="s">
         <v>1833</v>
       </c>
@@ -12825,7 +12843,7 @@
         <f>HYPERLINK("#'Mass Transfer'!D417","→ Mass Transfer")</f>
         <v>→ Mass Transfer</v>
       </c>
-      <c r="F77" s="22" t="inlineStr">
+      <c r="F77" s="183" t="inlineStr">
         <is>
           <t xml:space="preserve">Shown beside D42: CO₂ the liquid takes up after each pulse (incl. bicarbonate), per hour, over fixation. Informative, not pass/fail: below 1 the culture also draws on headspace CO₂ between pulses. Carbon sufficiency is row 76.</t>
         </is>
@@ -12838,7 +12856,7 @@
         </is>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2" ht="47" customHeight="1">
       <c r="A80" s="64" t="inlineStr">
         <i